<commit_message>
📊 Dados atualizados - 2026-09-14 05:36
</commit_message>
<xml_diff>
--- a/data/ativos.xlsx
+++ b/data/ativos.xlsx
@@ -1740,7 +1740,7 @@
         <v>7.37</v>
       </c>
       <c r="G6" t="n">
-        <v>464934231</v>
+        <v>464934200</v>
       </c>
       <c r="H6" t="n">
         <v>200</v>
@@ -1758,7 +1758,7 @@
         <v>1.91</v>
       </c>
       <c r="M6" t="n">
-        <v>7.238115664929348</v>
+        <v>7.238115182320043</v>
       </c>
       <c r="N6" t="n">
         <v>1.26</v>
@@ -1836,7 +1836,7 @@
         <v>35958279</v>
       </c>
       <c r="AM6" t="n">
-        <v>44448779.2543021</v>
+        <v>44448776.29063097</v>
       </c>
       <c r="AN6" t="n">
         <v>0.5199</v>
@@ -11848,7 +11848,7 @@
         <v>34.5</v>
       </c>
       <c r="G50" t="n">
-        <v>967124900</v>
+        <v>974049400</v>
       </c>
       <c r="H50" t="n">
         <v>100</v>
@@ -11866,7 +11866,7 @@
         <v>0.8</v>
       </c>
       <c r="M50" t="n">
-        <v>0.9784277868454088</v>
+        <v>0.9854332141795732</v>
       </c>
       <c r="N50" t="n">
         <v>0.06</v>
@@ -11944,7 +11944,7 @@
         <v>84709985.8</v>
       </c>
       <c r="AM50" t="n">
-        <v>330076757.6791809</v>
+        <v>332440068.2593856</v>
       </c>
       <c r="AN50" t="n">
         <v>4.4983</v>
@@ -14136,7 +14136,7 @@
         <v>376.6</v>
       </c>
       <c r="G60" t="n">
-        <v>171258852</v>
+        <v>171258900</v>
       </c>
       <c r="H60" t="n">
         <v>8</v>
@@ -14154,7 +14154,7 @@
         <v>0.83</v>
       </c>
       <c r="M60" t="n">
-        <v>12.80992104751274</v>
+        <v>12.80992463784517</v>
       </c>
       <c r="N60" t="n">
         <v>0.68</v>
@@ -14232,7 +14232,7 @@
         <v>59558607.5</v>
       </c>
       <c r="AM60" t="n">
-        <v>-25111268.62170088</v>
+        <v>-25111275.65982405</v>
       </c>
       <c r="AN60" t="n">
         <v>10.0581</v>

</xml_diff>

<commit_message>
📊 Dados atualizados - 2026-09-15 05:38
</commit_message>
<xml_diff>
--- a/data/ativos.xlsx
+++ b/data/ativos.xlsx
@@ -1047,13 +1047,13 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>25.1</v>
+        <v>25.05</v>
       </c>
       <c r="G3" t="n">
-        <v>3357546731</v>
+        <v>3350858237</v>
       </c>
       <c r="H3" t="n">
-        <v>398500</v>
+        <v>454800</v>
       </c>
       <c r="I3" t="n">
         <v>129510368</v>
@@ -1068,7 +1068,7 @@
         <v>0.88</v>
       </c>
       <c r="M3" t="n">
-        <v>0.8354324040170742</v>
+        <v>0.8337681577475935</v>
       </c>
       <c r="N3" t="n">
         <v>0.09</v>
@@ -1146,7 +1146,7 @@
         <v>506385538.88</v>
       </c>
       <c r="AM3" t="n">
-        <v>655770845.8984375</v>
+        <v>654464499.4140625</v>
       </c>
       <c r="AN3" t="n">
         <v>2.7</v>
@@ -1187,7 +1187,7 @@
         <v>40.42</v>
       </c>
       <c r="AZ3" t="n">
-        <v>45.93</v>
+        <v>45.84</v>
       </c>
       <c r="BA3" t="n">
         <v>4.87</v>
@@ -1196,19 +1196,19 @@
         <v>21.14</v>
       </c>
       <c r="BC3" t="n">
-        <v>97.20999999999999</v>
+        <v>97.59999999999999</v>
       </c>
       <c r="BD3" t="n">
-        <v>61.02</v>
+        <v>61.34</v>
       </c>
       <c r="BE3" t="n">
         <v>83</v>
       </c>
       <c r="BF3" t="n">
-        <v>-80.59999999999999</v>
+        <v>-80.56</v>
       </c>
       <c r="BG3" t="n">
-        <v>-15.79</v>
+        <v>-15.63</v>
       </c>
       <c r="BH3" t="n">
         <v>27.85</v>
@@ -1217,7 +1217,7 @@
         <v>0</v>
       </c>
       <c r="BJ3" t="n">
-        <v>25.1</v>
+        <v>25.05</v>
       </c>
       <c r="BK3" t="n">
         <v>3.91</v>
@@ -1226,7 +1226,7 @@
         <v>4.39</v>
       </c>
       <c r="BM3" t="n">
-        <v>25.32</v>
+        <v>25.09</v>
       </c>
       <c r="BN3" t="n">
         <v>27.17</v>
@@ -1235,19 +1235,19 @@
         <v>18.72</v>
       </c>
       <c r="BP3" t="n">
-        <v>24.96</v>
+        <v>24.59</v>
       </c>
       <c r="BQ3" t="n">
-        <v>5.71</v>
+        <v>5.7</v>
       </c>
       <c r="BR3" t="n">
-        <v>25</v>
+        <v>24.87</v>
       </c>
       <c r="BS3" t="n">
         <v>0.79</v>
       </c>
       <c r="BT3" t="n">
-        <v>529000</v>
+        <v>533320</v>
       </c>
     </row>
     <row r="4">
@@ -1277,13 +1277,13 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>15.62</v>
+        <v>15.87</v>
       </c>
       <c r="G4" t="n">
-        <v>241870387427</v>
+        <v>245741552427</v>
       </c>
       <c r="H4" t="n">
-        <v>22932100</v>
+        <v>29303600</v>
       </c>
       <c r="I4" t="n">
         <v>15484664889</v>
@@ -1298,7 +1298,7 @@
         <v>2.76</v>
       </c>
       <c r="M4" t="n">
-        <v>2.738705781894346</v>
+        <v>2.782539101388105</v>
       </c>
       <c r="N4" t="n">
         <v>1.76</v>
@@ -1376,7 +1376,7 @@
         <v>16258898133.45</v>
       </c>
       <c r="AM4" t="n">
-        <v>23947563111.58416</v>
+        <v>24330846774.9505</v>
       </c>
       <c r="AN4" t="n">
         <v>0.269</v>
@@ -1417,7 +1417,7 @@
         <v>9.470000000000001</v>
       </c>
       <c r="AZ4" t="n">
-        <v>19.5</v>
+        <v>19.81</v>
       </c>
       <c r="BA4" t="n">
         <v>1.13</v>
@@ -1426,19 +1426,19 @@
         <v>11.39</v>
       </c>
       <c r="BC4" t="n">
-        <v>-25.71</v>
+        <v>-26.88</v>
       </c>
       <c r="BD4" t="n">
-        <v>-39.34</v>
+        <v>-40.3</v>
       </c>
       <c r="BE4" t="n">
         <v>24.83</v>
       </c>
       <c r="BF4" t="n">
-        <v>-92.78</v>
+        <v>-92.90000000000001</v>
       </c>
       <c r="BG4" t="n">
-        <v>-27.1</v>
+        <v>-28.25</v>
       </c>
       <c r="BH4" t="n">
         <v>5.7</v>
@@ -1447,7 +1447,7 @@
         <v>0</v>
       </c>
       <c r="BJ4" t="n">
-        <v>15.62</v>
+        <v>15.87</v>
       </c>
       <c r="BK4" t="n">
         <v>1.05</v>
@@ -1456,7 +1456,7 @@
         <v>1.04</v>
       </c>
       <c r="BM4" t="n">
-        <v>15.78</v>
+        <v>15.91</v>
       </c>
       <c r="BN4" t="n">
         <v>17</v>
@@ -1465,19 +1465,19 @@
         <v>11.09</v>
       </c>
       <c r="BP4" t="n">
-        <v>15.59</v>
+        <v>15.37</v>
       </c>
       <c r="BQ4" t="n">
-        <v>15.06</v>
+        <v>15.31</v>
       </c>
       <c r="BR4" t="n">
-        <v>15.78</v>
+        <v>15.4</v>
       </c>
       <c r="BS4" t="n">
         <v>2.76</v>
       </c>
       <c r="BT4" t="n">
-        <v>30552467</v>
+        <v>28956417</v>
       </c>
     </row>
     <row r="5">
@@ -1737,13 +1737,13 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>7.37</v>
+        <v>7.49</v>
       </c>
       <c r="G6" t="n">
-        <v>464934200</v>
+        <v>472504313</v>
       </c>
       <c r="H6" t="n">
-        <v>200</v>
+        <v>900</v>
       </c>
       <c r="I6" t="n">
         <v>63084700</v>
@@ -1758,7 +1758,7 @@
         <v>1.91</v>
       </c>
       <c r="M6" t="n">
-        <v>7.238115182320043</v>
+        <v>7.355967019928846</v>
       </c>
       <c r="N6" t="n">
         <v>1.26</v>
@@ -1836,7 +1836,7 @@
         <v>35958279</v>
       </c>
       <c r="AM6" t="n">
-        <v>44448776.29063097</v>
+        <v>45172496.4627151</v>
       </c>
       <c r="AN6" t="n">
         <v>0.5199</v>
@@ -1877,7 +1877,7 @@
         <v>5.74</v>
       </c>
       <c r="AZ6" t="n">
-        <v>8.65</v>
+        <v>8.789999999999999</v>
       </c>
       <c r="BA6" t="n">
         <v>0.65</v>
@@ -1886,19 +1886,19 @@
         <v>7.95</v>
       </c>
       <c r="BC6" t="n">
-        <v>-4.53</v>
+        <v>-6.06</v>
       </c>
       <c r="BD6" t="n">
-        <v>-22.05</v>
+        <v>-23.3</v>
       </c>
       <c r="BE6" t="n">
         <v>17.33</v>
       </c>
       <c r="BF6" t="n">
-        <v>-91.2</v>
+        <v>-91.34</v>
       </c>
       <c r="BG6" t="n">
-        <v>7.92</v>
+        <v>6.19</v>
       </c>
       <c r="BH6" t="n">
         <v>3.86</v>
@@ -1907,7 +1907,7 @@
         <v>0</v>
       </c>
       <c r="BJ6" t="n">
-        <v>7.37</v>
+        <v>7.49</v>
       </c>
       <c r="BK6" t="n">
         <v>0.57</v>
@@ -1916,7 +1916,7 @@
         <v>0.5600000000000001</v>
       </c>
       <c r="BM6" t="n">
-        <v>7.37</v>
+        <v>7.49</v>
       </c>
       <c r="BN6" t="n">
         <v>8.16</v>
@@ -1925,19 +1925,19 @@
         <v>6.22</v>
       </c>
       <c r="BP6" t="n">
-        <v>7.35</v>
+        <v>7.24</v>
       </c>
       <c r="BQ6" t="n">
-        <v>13.11</v>
+        <v>13.32</v>
       </c>
       <c r="BR6" t="n">
-        <v>7.35</v>
+        <v>7.37</v>
       </c>
       <c r="BS6" t="n">
         <v>7.32</v>
       </c>
       <c r="BT6" t="n">
-        <v>270</v>
+        <v>253</v>
       </c>
     </row>
     <row r="7">
@@ -3117,13 +3117,13 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>5.07</v>
+        <v>5.06</v>
       </c>
       <c r="G12" t="n">
-        <v>486524922</v>
+        <v>485565336</v>
       </c>
       <c r="H12" t="n">
-        <v>449000</v>
+        <v>255400</v>
       </c>
       <c r="I12" t="n">
         <v>95961536</v>
@@ -3138,7 +3138,7 @@
         <v>0.32</v>
       </c>
       <c r="M12" t="n">
-        <v>0.08798728973810956</v>
+        <v>0.08781375007427578</v>
       </c>
       <c r="N12" t="n">
         <v>0.14</v>
@@ -3216,7 +3216,7 @@
         <v>362734606.08</v>
       </c>
       <c r="AM12" t="n">
-        <v>523145077.4193548</v>
+        <v>522113264.516129</v>
       </c>
       <c r="AN12" t="n">
         <v>0.4208</v>
@@ -3257,7 +3257,7 @@
         <v>30.49</v>
       </c>
       <c r="AZ12" t="n">
-        <v>6.85</v>
+        <v>6.84</v>
       </c>
       <c r="BA12" t="n">
         <v>4.41</v>
@@ -3266,19 +3266,19 @@
         <v>18.12</v>
       </c>
       <c r="BC12" t="n">
-        <v>636.63</v>
+        <v>638.09</v>
       </c>
       <c r="BD12" t="n">
-        <v>501.46</v>
+        <v>502.65</v>
       </c>
       <c r="BE12" t="n">
         <v>35.17</v>
       </c>
       <c r="BF12" t="n">
-        <v>-12.99</v>
+        <v>-12.81</v>
       </c>
       <c r="BG12" t="n">
-        <v>257.37</v>
+        <v>258.08</v>
       </c>
       <c r="BH12" t="n">
         <v>16.4</v>
@@ -3287,7 +3287,7 @@
         <v>0</v>
       </c>
       <c r="BJ12" t="n">
-        <v>5.07</v>
+        <v>5.06</v>
       </c>
       <c r="BK12" t="n">
         <v>3.78</v>
@@ -3296,7 +3296,7 @@
         <v>3.43</v>
       </c>
       <c r="BM12" t="n">
-        <v>5.1</v>
+        <v>5.08</v>
       </c>
       <c r="BN12" t="n">
         <v>8.23</v>
@@ -3305,19 +3305,19 @@
         <v>4.42</v>
       </c>
       <c r="BP12" t="n">
+        <v>4.99</v>
+      </c>
+      <c r="BQ12" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="BR12" t="n">
         <v>5.04</v>
-      </c>
-      <c r="BQ12" t="n">
-        <v>1.48</v>
-      </c>
-      <c r="BR12" t="n">
-        <v>5.1</v>
       </c>
       <c r="BS12" t="n">
         <v>0.09</v>
       </c>
       <c r="BT12" t="n">
-        <v>482027</v>
+        <v>491947</v>
       </c>
     </row>
     <row r="13">
@@ -3347,13 +3347,13 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>28.63</v>
+        <v>28.44</v>
       </c>
       <c r="G13" t="n">
-        <v>14434985043</v>
+        <v>14339192309</v>
       </c>
       <c r="H13" t="n">
-        <v>3688300</v>
+        <v>4292700</v>
       </c>
       <c r="I13" t="n">
         <v>504190947</v>
@@ -3368,7 +3368,7 @@
         <v>1.13</v>
       </c>
       <c r="M13" t="n">
-        <v>4.992452360939528</v>
+        <v>4.959321695435232</v>
       </c>
       <c r="N13" t="n">
         <v>0.57</v>
@@ -3446,7 +3446,7 @@
         <v>932753251.95</v>
       </c>
       <c r="AM13" t="n">
-        <v>1502079609.05307</v>
+        <v>1492111582.622269</v>
       </c>
       <c r="AN13" t="n">
         <v>2.6301</v>
@@ -3487,7 +3487,7 @@
         <v>26.6</v>
       </c>
       <c r="AZ13" t="n">
-        <v>51.82</v>
+        <v>51.48</v>
       </c>
       <c r="BA13" t="n">
         <v>2.6</v>
@@ -3496,19 +3496,19 @@
         <v>8.69</v>
       </c>
       <c r="BC13" t="n">
-        <v>13.77</v>
+        <v>14.53</v>
       </c>
       <c r="BD13" t="n">
-        <v>-7.1</v>
+        <v>-6.48</v>
       </c>
       <c r="BE13" t="n">
         <v>81</v>
       </c>
       <c r="BF13" t="n">
-        <v>-90.90000000000001</v>
+        <v>-90.84</v>
       </c>
       <c r="BG13" t="n">
-        <v>-69.63</v>
+        <v>-69.43000000000001</v>
       </c>
       <c r="BH13" t="n">
         <v>25.49</v>
@@ -3517,7 +3517,7 @@
         <v>0</v>
       </c>
       <c r="BJ13" t="n">
-        <v>28.63</v>
+        <v>28.44</v>
       </c>
       <c r="BK13" t="n">
         <v>1.85</v>
@@ -3526,7 +3526,7 @@
         <v>1.96</v>
       </c>
       <c r="BM13" t="n">
-        <v>29.21</v>
+        <v>28.48</v>
       </c>
       <c r="BN13" t="n">
         <v>32.43</v>
@@ -3535,19 +3535,19 @@
         <v>21.06</v>
       </c>
       <c r="BP13" t="n">
-        <v>28.47</v>
+        <v>27.8</v>
       </c>
       <c r="BQ13" t="n">
-        <v>14.63</v>
+        <v>14.53</v>
       </c>
       <c r="BR13" t="n">
-        <v>29.08</v>
+        <v>27.91</v>
       </c>
       <c r="BS13" t="n">
         <v>5.01</v>
       </c>
       <c r="BT13" t="n">
-        <v>4550534</v>
+        <v>4560105</v>
       </c>
     </row>
     <row r="14">
@@ -3577,13 +3577,13 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>10</v>
+        <v>9.9</v>
       </c>
       <c r="G14" t="n">
-        <v>7974653792</v>
+        <v>7789191837</v>
       </c>
       <c r="H14" t="n">
-        <v>2700</v>
+        <v>11700</v>
       </c>
       <c r="I14" t="n">
         <v>339510689</v>
@@ -3598,7 +3598,7 @@
         <v>1.92</v>
       </c>
       <c r="M14" t="n">
-        <v>3.311218025310331</v>
+        <v>3.234210924510375</v>
       </c>
       <c r="N14" t="n">
         <v>1.11</v>
@@ -3676,7 +3676,7 @@
         <v>349696009.67</v>
       </c>
       <c r="AM14" t="n">
-        <v>885089211.0987792</v>
+        <v>864505198.3351831</v>
       </c>
       <c r="AN14" t="n">
         <v>0.1489</v>
@@ -3717,7 +3717,7 @@
         <v>9.050000000000001</v>
       </c>
       <c r="AZ14" t="n">
-        <v>8.029999999999999</v>
+        <v>7.95</v>
       </c>
       <c r="BA14" t="n">
         <v>1.42</v>
@@ -3726,19 +3726,19 @@
         <v>5.94</v>
       </c>
       <c r="BC14" t="n">
-        <v>10.83</v>
+        <v>11.95</v>
       </c>
       <c r="BD14" t="n">
-        <v>-9.51</v>
+        <v>-8.6</v>
       </c>
       <c r="BE14" t="n">
         <v>-19.67</v>
       </c>
       <c r="BF14" t="n">
-        <v>-85.79000000000001</v>
+        <v>-85.64</v>
       </c>
       <c r="BG14" t="n">
-        <v>-40.58</v>
+        <v>-39.98</v>
       </c>
       <c r="BH14" t="n">
         <v>5.3</v>
@@ -3747,7 +3747,7 @@
         <v>0</v>
       </c>
       <c r="BJ14" t="n">
-        <v>10</v>
+        <v>9.9</v>
       </c>
       <c r="BK14" t="n">
         <v>1.03</v>
@@ -3756,7 +3756,7 @@
         <v>1.01</v>
       </c>
       <c r="BM14" t="n">
-        <v>10</v>
+        <v>9.9</v>
       </c>
       <c r="BN14" t="n">
         <v>13.49</v>
@@ -3765,19 +3765,19 @@
         <v>7.65</v>
       </c>
       <c r="BP14" t="n">
+        <v>9.56</v>
+      </c>
+      <c r="BQ14" t="n">
         <v>9.77</v>
       </c>
-      <c r="BQ14" t="n">
-        <v>9.869999999999999</v>
-      </c>
       <c r="BR14" t="n">
-        <v>9.77</v>
+        <v>9.75</v>
       </c>
       <c r="BS14" t="n">
         <v>1.44</v>
       </c>
       <c r="BT14" t="n">
-        <v>12497</v>
+        <v>12490</v>
       </c>
     </row>
     <row r="15">
@@ -3807,13 +3807,13 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>13.33</v>
+        <v>13.02</v>
       </c>
       <c r="G15" t="n">
-        <v>7974653792</v>
+        <v>7789191837</v>
       </c>
       <c r="H15" t="n">
-        <v>1699500</v>
+        <v>967500</v>
       </c>
       <c r="I15" t="n">
         <v>343551533</v>
@@ -3828,7 +3828,7 @@
         <v>2.56</v>
       </c>
       <c r="M15" t="n">
-        <v>3.272271566904433</v>
+        <v>3.196170221577339</v>
       </c>
       <c r="N15" t="n">
         <v>1.47</v>
@@ -3906,7 +3906,7 @@
         <v>353858078.99</v>
       </c>
       <c r="AM15" t="n">
-        <v>665108739.9499583</v>
+        <v>649640686.9891577</v>
       </c>
       <c r="AN15" t="n">
         <v>0.1638</v>
@@ -3947,7 +3947,7 @@
         <v>9.050000000000001</v>
       </c>
       <c r="AZ15" t="n">
-        <v>8.859999999999999</v>
+        <v>8.66</v>
       </c>
       <c r="BA15" t="n">
         <v>1.42</v>
@@ -3956,19 +3956,19 @@
         <v>6.19</v>
       </c>
       <c r="BC15" t="n">
-        <v>-16.86</v>
+        <v>-14.88</v>
       </c>
       <c r="BD15" t="n">
-        <v>-32.12</v>
+        <v>-30.5</v>
       </c>
       <c r="BE15" t="n">
         <v>-33.5</v>
       </c>
       <c r="BF15" t="n">
-        <v>-89.34</v>
+        <v>-89.08</v>
       </c>
       <c r="BG15" t="n">
-        <v>-53.58</v>
+        <v>-52.47</v>
       </c>
       <c r="BH15" t="n">
         <v>5.3</v>
@@ -3977,7 +3977,7 @@
         <v>0</v>
       </c>
       <c r="BJ15" t="n">
-        <v>13.33</v>
+        <v>13.02</v>
       </c>
       <c r="BK15" t="n">
         <v>1.03</v>
@@ -3986,7 +3986,7 @@
         <v>1.01</v>
       </c>
       <c r="BM15" t="n">
-        <v>13.41</v>
+        <v>13.21</v>
       </c>
       <c r="BN15" t="n">
         <v>16.22</v>
@@ -3995,19 +3995,19 @@
         <v>7.84</v>
       </c>
       <c r="BP15" t="n">
+        <v>12.86</v>
+      </c>
+      <c r="BQ15" t="n">
+        <v>12.85</v>
+      </c>
+      <c r="BR15" t="n">
         <v>13.16</v>
-      </c>
-      <c r="BQ15" t="n">
-        <v>13.16</v>
-      </c>
-      <c r="BR15" t="n">
-        <v>13.3</v>
       </c>
       <c r="BS15" t="n">
         <v>1.92</v>
       </c>
       <c r="BT15" t="n">
-        <v>2338760</v>
+        <v>2373813</v>
       </c>
     </row>
     <row r="16">
@@ -4037,13 +4037,13 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>4.35</v>
+        <v>4.32</v>
       </c>
       <c r="G16" t="n">
-        <v>953979774</v>
+        <v>947400661</v>
       </c>
       <c r="H16" t="n">
-        <v>47600</v>
+        <v>63200</v>
       </c>
       <c r="I16" t="n">
         <v>219305733</v>
@@ -4058,7 +4058,7 @@
         <v>2.69</v>
       </c>
       <c r="M16" t="n">
-        <v>0.4513124221540528</v>
+        <v>0.448199950061269</v>
       </c>
       <c r="N16" t="n">
         <v>0.39</v>
@@ -4136,7 +4136,7 @@
         <v>17544458.64</v>
       </c>
       <c r="AM16" t="n">
-        <v>267971846.6292135</v>
+        <v>266123781.1797753</v>
       </c>
       <c r="AN16" t="n">
         <v>0.0077</v>
@@ -4186,16 +4186,16 @@
         <v>0</v>
       </c>
       <c r="BC16" t="n">
-        <v>-60.02</v>
+        <v>-59.75</v>
       </c>
       <c r="BD16" t="n">
-        <v>-67.36</v>
+        <v>-67.13</v>
       </c>
       <c r="BE16" t="n">
         <v>-97.17</v>
       </c>
       <c r="BF16" t="n">
-        <v>-98.16</v>
+        <v>-98.15000000000001</v>
       </c>
       <c r="BG16" t="n">
         <v>-100</v>
@@ -4207,7 +4207,7 @@
         <v>0</v>
       </c>
       <c r="BJ16" t="n">
-        <v>4.35</v>
+        <v>4.32</v>
       </c>
       <c r="BK16" t="n">
         <v>0.08</v>
@@ -4216,28 +4216,28 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="BM16" t="n">
-        <v>4.44</v>
+        <v>4.36</v>
       </c>
       <c r="BN16" t="n">
         <v>5.54</v>
       </c>
       <c r="BO16" t="n">
-        <v>2.98</v>
+        <v>3</v>
       </c>
       <c r="BP16" t="n">
-        <v>4.33</v>
+        <v>4.28</v>
       </c>
       <c r="BQ16" t="n">
-        <v>59.36</v>
+        <v>58.95</v>
       </c>
       <c r="BR16" t="n">
-        <v>4.44</v>
+        <v>4.29</v>
       </c>
       <c r="BS16" t="n">
         <v>0.49</v>
       </c>
       <c r="BT16" t="n">
-        <v>141910</v>
+        <v>138763</v>
       </c>
     </row>
     <row r="17">
@@ -4267,13 +4267,13 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>33.74</v>
+        <v>33.4</v>
       </c>
       <c r="G17" t="n">
-        <v>11121612159</v>
+        <v>11009535622</v>
       </c>
       <c r="H17" t="n">
-        <v>541900</v>
+        <v>567600</v>
       </c>
       <c r="I17" t="n">
         <v>0</v>
@@ -4360,13 +4360,13 @@
         <v>8.039999999999999</v>
       </c>
       <c r="AK17" t="n">
-        <v>5022404334.808526</v>
+        <v>4971791736.813584</v>
       </c>
       <c r="AL17" t="n">
-        <v>1390201519.875</v>
+        <v>1376191952.75</v>
       </c>
       <c r="AM17" t="n">
-        <v>3443223578.637771</v>
+        <v>3408524960.371517</v>
       </c>
       <c r="AN17" t="n">
         <v>1.08</v>
@@ -4407,7 +4407,7 @@
         <v>42.98</v>
       </c>
       <c r="AZ17" t="n">
-        <v>18.05</v>
+        <v>17.87</v>
       </c>
       <c r="BA17" t="n">
         <v>4.55</v>
@@ -4416,19 +4416,19 @@
         <v>16.33</v>
       </c>
       <c r="BC17" t="n">
-        <v>56.01</v>
+        <v>57.6</v>
       </c>
       <c r="BD17" t="n">
-        <v>27.38</v>
+        <v>28.68</v>
       </c>
       <c r="BE17" t="n">
         <v>-46.5</v>
       </c>
       <c r="BF17" t="n">
-        <v>-86.52</v>
+        <v>-86.38</v>
       </c>
       <c r="BG17" t="n">
-        <v>-51.59</v>
+        <v>-51.1</v>
       </c>
       <c r="BH17" t="n">
         <v>29.25</v>
@@ -4437,7 +4437,7 @@
         <v>0</v>
       </c>
       <c r="BJ17" t="n">
-        <v>33.74</v>
+        <v>33.4</v>
       </c>
       <c r="BK17" t="n">
         <v>4.21</v>
@@ -4446,7 +4446,7 @@
         <v>12.62</v>
       </c>
       <c r="BM17" t="n">
-        <v>34.02</v>
+        <v>33.49</v>
       </c>
       <c r="BN17" t="n">
         <v>36.63</v>
@@ -4455,19 +4455,19 @@
         <v>29.28</v>
       </c>
       <c r="BP17" t="n">
-        <v>33.54</v>
+        <v>33.02</v>
       </c>
       <c r="BQ17" t="n">
-        <v>2.67</v>
+        <v>2.65</v>
       </c>
       <c r="BR17" t="n">
-        <v>33.92</v>
+        <v>33.3</v>
       </c>
       <c r="BS17" t="n">
         <v>2.21</v>
       </c>
       <c r="BT17" t="n">
-        <v>1076424</v>
+        <v>1072646</v>
       </c>
     </row>
     <row r="18">
@@ -4497,13 +4497,13 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>11.8</v>
+        <v>11.5</v>
       </c>
       <c r="G18" t="n">
-        <v>11121612159</v>
+        <v>11009535622</v>
       </c>
       <c r="H18" t="n">
-        <v>2900</v>
+        <v>5300</v>
       </c>
       <c r="I18" t="n">
         <v>671494278</v>
@@ -4518,7 +4518,7 @@
         <v>1.2</v>
       </c>
       <c r="M18" t="n">
-        <v>3.274639376760259</v>
+        <v>3.241639642906554</v>
       </c>
       <c r="N18" t="n">
         <v>0.33</v>
@@ -4596,7 +4596,7 @@
         <v>940091989.1999999</v>
       </c>
       <c r="AM18" t="n">
-        <v>3310003618.75</v>
+        <v>3276647506.547619</v>
       </c>
       <c r="AN18" t="n">
         <v>0.36</v>
@@ -4637,7 +4637,7 @@
         <v>14.31</v>
       </c>
       <c r="AZ18" t="n">
-        <v>6.08</v>
+        <v>5.92</v>
       </c>
       <c r="BA18" t="n">
         <v>1.51</v>
@@ -4646,19 +4646,19 @@
         <v>5.44</v>
       </c>
       <c r="BC18" t="n">
-        <v>48.52</v>
+        <v>52.39</v>
       </c>
       <c r="BD18" t="n">
-        <v>21.26</v>
+        <v>24.43</v>
       </c>
       <c r="BE18" t="n">
         <v>-48.5</v>
       </c>
       <c r="BF18" t="n">
-        <v>-87.18000000000001</v>
+        <v>-86.84999999999999</v>
       </c>
       <c r="BG18" t="n">
-        <v>-53.86</v>
+        <v>-52.66</v>
       </c>
       <c r="BH18" t="n">
         <v>9.75</v>
@@ -4667,7 +4667,7 @@
         <v>0</v>
       </c>
       <c r="BJ18" t="n">
-        <v>11.8</v>
+        <v>11.5</v>
       </c>
       <c r="BK18" t="n">
         <v>1.4</v>
@@ -4676,28 +4676,28 @@
         <v>12.62</v>
       </c>
       <c r="BM18" t="n">
-        <v>11.91</v>
+        <v>11.9</v>
       </c>
       <c r="BN18" t="n">
         <v>13.82</v>
       </c>
       <c r="BO18" t="n">
-        <v>10.11</v>
+        <v>10.19</v>
       </c>
       <c r="BP18" t="n">
-        <v>11.7</v>
+        <v>11.43</v>
       </c>
       <c r="BQ18" t="n">
-        <v>0.93</v>
+        <v>0.91</v>
       </c>
       <c r="BR18" t="n">
-        <v>11.74</v>
+        <v>11.9</v>
       </c>
       <c r="BS18" t="n">
         <v>2.3</v>
       </c>
       <c r="BT18" t="n">
-        <v>9650</v>
+        <v>9673</v>
       </c>
     </row>
     <row r="19">
@@ -4727,13 +4727,13 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>10.96</v>
+        <v>10.8</v>
       </c>
       <c r="G19" t="n">
-        <v>11121612159</v>
+        <v>11009535622</v>
       </c>
       <c r="H19" t="n">
-        <v>7900</v>
+        <v>9300</v>
       </c>
       <c r="I19" t="n">
         <v>317386323</v>
@@ -4748,7 +4748,7 @@
         <v>1.12</v>
       </c>
       <c r="M19" t="n">
-        <v>6.928154884632505</v>
+        <v>6.858337344138532</v>
       </c>
       <c r="N19" t="n">
         <v>0.3</v>
@@ -4826,7 +4826,7 @@
         <v>444340852.2</v>
       </c>
       <c r="AM19" t="n">
-        <v>3530670526.666667</v>
+        <v>3495090673.650794</v>
       </c>
       <c r="AN19" t="n">
         <v>0.36</v>
@@ -4867,7 +4867,7 @@
         <v>14.31</v>
       </c>
       <c r="AZ19" t="n">
-        <v>6.03</v>
+        <v>5.94</v>
       </c>
       <c r="BA19" t="n">
         <v>1.51</v>
@@ -4876,19 +4876,19 @@
         <v>5.25</v>
       </c>
       <c r="BC19" t="n">
-        <v>59.9</v>
+        <v>62.27</v>
       </c>
       <c r="BD19" t="n">
-        <v>30.56</v>
+        <v>32.49</v>
       </c>
       <c r="BE19" t="n">
         <v>-45</v>
       </c>
       <c r="BF19" t="n">
-        <v>-86.2</v>
+        <v>-85.98999999999999</v>
       </c>
       <c r="BG19" t="n">
-        <v>-52.1</v>
+        <v>-51.39</v>
       </c>
       <c r="BH19" t="n">
         <v>9.75</v>
@@ -4897,7 +4897,7 @@
         <v>0</v>
       </c>
       <c r="BJ19" t="n">
-        <v>10.96</v>
+        <v>10.8</v>
       </c>
       <c r="BK19" t="n">
         <v>1.4</v>
@@ -4906,7 +4906,7 @@
         <v>12.62</v>
       </c>
       <c r="BM19" t="n">
-        <v>11.13</v>
+        <v>11.15</v>
       </c>
       <c r="BN19" t="n">
         <v>11.41</v>
@@ -4915,19 +4915,19 @@
         <v>9.19</v>
       </c>
       <c r="BP19" t="n">
-        <v>10.95</v>
+        <v>10.8</v>
       </c>
       <c r="BQ19" t="n">
-        <v>0.87</v>
+        <v>0.86</v>
       </c>
       <c r="BR19" t="n">
-        <v>11.01</v>
+        <v>11.15</v>
       </c>
       <c r="BS19" t="n">
         <v>2.16</v>
       </c>
       <c r="BT19" t="n">
-        <v>13908</v>
+        <v>13907</v>
       </c>
     </row>
     <row r="20">
@@ -5417,13 +5417,13 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>4.91</v>
+        <v>4.99</v>
       </c>
       <c r="G22" t="n">
-        <v>983204392</v>
+        <v>999223502</v>
       </c>
       <c r="H22" t="n">
-        <v>1773300</v>
+        <v>893100</v>
       </c>
       <c r="I22" t="n">
         <v>200245299</v>
@@ -5438,7 +5438,7 @@
         <v>0.27</v>
       </c>
       <c r="M22" t="n">
-        <v>0.0833920612791982</v>
+        <v>0.08475074784897729</v>
       </c>
       <c r="N22" t="n">
         <v>0.08</v>
@@ -5516,7 +5516,7 @@
         <v>378463615.11</v>
       </c>
       <c r="AM22" t="n">
-        <v>222948841.723356</v>
+        <v>226581292.9705215</v>
       </c>
       <c r="AN22" t="n">
         <v>0</v>
@@ -5566,19 +5566,19 @@
         <v>172.49</v>
       </c>
       <c r="BC22" t="n">
-        <v>504.99</v>
+        <v>495.29</v>
       </c>
       <c r="BD22" t="n">
-        <v>393.97</v>
+        <v>386.05</v>
       </c>
       <c r="BE22" t="n">
         <v>-100</v>
       </c>
       <c r="BF22" t="n">
-        <v>-61.51</v>
+        <v>-62.12</v>
       </c>
       <c r="BG22" t="n">
-        <v>3413.03</v>
+        <v>3356.71</v>
       </c>
       <c r="BH22" t="n">
         <v>20.75</v>
@@ -5587,7 +5587,7 @@
         <v>0</v>
       </c>
       <c r="BJ22" t="n">
-        <v>4.91</v>
+        <v>4.99</v>
       </c>
       <c r="BK22" t="n">
         <v>1.89</v>
@@ -5596,7 +5596,7 @@
         <v>0.67</v>
       </c>
       <c r="BM22" t="n">
-        <v>5.36</v>
+        <v>5.06</v>
       </c>
       <c r="BN22" t="n">
         <v>8.82</v>
@@ -5605,19 +5605,19 @@
         <v>3.37</v>
       </c>
       <c r="BP22" t="n">
-        <v>4.89</v>
+        <v>4.77</v>
       </c>
       <c r="BQ22" t="n">
-        <v>7.31</v>
+        <v>7.43</v>
       </c>
       <c r="BR22" t="n">
-        <v>5.34</v>
+        <v>4.85</v>
       </c>
       <c r="BS22" t="n">
         <v>0.09</v>
       </c>
       <c r="BT22" t="n">
-        <v>1550707</v>
+        <v>1562667</v>
       </c>
     </row>
     <row r="23">
@@ -5877,13 +5877,13 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.93</v>
+        <v>2.9</v>
       </c>
       <c r="G24" t="n">
-        <v>1183335024</v>
+        <v>1171219848</v>
       </c>
       <c r="H24" t="n">
-        <v>4187500</v>
+        <v>3733900</v>
       </c>
       <c r="I24" t="n">
         <v>403868805</v>
@@ -5898,7 +5898,7 @@
         <v>0.49</v>
       </c>
       <c r="M24" t="n">
-        <v>0.2860603873994232</v>
+        <v>0.2831316547331177</v>
       </c>
       <c r="N24" t="n">
         <v>0.11</v>
@@ -5976,7 +5976,7 @@
         <v>153470145.9</v>
       </c>
       <c r="AM24" t="n">
-        <v>1066067589.189189</v>
+        <v>1055153016.216216</v>
       </c>
       <c r="AN24" t="n">
         <v>0.0813</v>
@@ -6017,7 +6017,7 @@
         <v>5.84</v>
       </c>
       <c r="AZ24" t="n">
-        <v>1.35</v>
+        <v>1.34</v>
       </c>
       <c r="BA24" t="n">
         <v>0.38</v>
@@ -6026,19 +6026,19 @@
         <v>1.46</v>
       </c>
       <c r="BC24" t="n">
-        <v>144.25</v>
+        <v>146.77</v>
       </c>
       <c r="BD24" t="n">
-        <v>99.43000000000001</v>
+        <v>101.49</v>
       </c>
       <c r="BE24" t="n">
         <v>-53.83</v>
       </c>
       <c r="BF24" t="n">
-        <v>-87.03</v>
+        <v>-86.90000000000001</v>
       </c>
       <c r="BG24" t="n">
-        <v>-50.25</v>
+        <v>-49.73</v>
       </c>
       <c r="BH24" t="n">
         <v>5.99</v>
@@ -6047,7 +6047,7 @@
         <v>0</v>
       </c>
       <c r="BJ24" t="n">
-        <v>2.93</v>
+        <v>2.9</v>
       </c>
       <c r="BK24" t="n">
         <v>0.38</v>
@@ -6065,19 +6065,19 @@
         <v>1.92</v>
       </c>
       <c r="BP24" t="n">
-        <v>2.86</v>
+        <v>2.87</v>
       </c>
       <c r="BQ24" t="n">
-        <v>7.2</v>
+        <v>7.12</v>
       </c>
       <c r="BR24" t="n">
-        <v>2.89</v>
+        <v>2.87</v>
       </c>
       <c r="BS24" t="n">
         <v>0.29</v>
       </c>
       <c r="BT24" t="n">
-        <v>9270327</v>
+        <v>9148997</v>
       </c>
     </row>
     <row r="25">
@@ -6107,13 +6107,13 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>3.79</v>
+        <v>3.7</v>
       </c>
       <c r="G25" t="n">
-        <v>1313212246</v>
+        <v>1282028186</v>
       </c>
       <c r="H25" t="n">
-        <v>820800</v>
+        <v>737400</v>
       </c>
       <c r="I25" t="n">
         <v>346494097</v>
@@ -6128,7 +6128,7 @@
         <v>0.97</v>
       </c>
       <c r="M25" t="n">
-        <v>0.6548275874796344</v>
+        <v>0.6392777912910751</v>
       </c>
       <c r="N25" t="n">
         <v>0.22</v>
@@ -6206,7 +6206,7 @@
         <v>62368937.46</v>
       </c>
       <c r="AM25" t="n">
-        <v>482798619.8529412</v>
+        <v>471333891.9117647</v>
       </c>
       <c r="AN25" t="n">
         <v>0.4742</v>
@@ -6247,7 +6247,7 @@
         <v>3.27</v>
       </c>
       <c r="AZ25" t="n">
-        <v>8.83</v>
+        <v>8.619999999999999</v>
       </c>
       <c r="BA25" t="n">
         <v>0.23</v>
@@ -6256,19 +6256,19 @@
         <v>2.2</v>
       </c>
       <c r="BC25" t="n">
-        <v>5.8</v>
+        <v>8.369999999999999</v>
       </c>
       <c r="BD25" t="n">
-        <v>-13.62</v>
+        <v>-11.51</v>
       </c>
       <c r="BE25" t="n">
         <v>133</v>
       </c>
       <c r="BF25" t="n">
-        <v>-93.89</v>
+        <v>-93.73999999999999</v>
       </c>
       <c r="BG25" t="n">
-        <v>-41.96</v>
+        <v>-40.55</v>
       </c>
       <c r="BH25" t="n">
         <v>3.97</v>
@@ -6277,7 +6277,7 @@
         <v>0</v>
       </c>
       <c r="BJ25" t="n">
-        <v>3.79</v>
+        <v>3.7</v>
       </c>
       <c r="BK25" t="n">
         <v>0.18</v>
@@ -6286,7 +6286,7 @@
         <v>0.24</v>
       </c>
       <c r="BM25" t="n">
-        <v>3.96</v>
+        <v>3.76</v>
       </c>
       <c r="BN25" t="n">
         <v>6.3</v>
@@ -6295,19 +6295,19 @@
         <v>2.64</v>
       </c>
       <c r="BP25" t="n">
-        <v>3.74</v>
+        <v>3.58</v>
       </c>
       <c r="BQ25" t="n">
-        <v>16.02</v>
+        <v>15.63</v>
       </c>
       <c r="BR25" t="n">
-        <v>3.86</v>
+        <v>3.72</v>
       </c>
       <c r="BS25" t="n">
         <v>0.67</v>
       </c>
       <c r="BT25" t="n">
-        <v>1171030</v>
+        <v>1176577</v>
       </c>
     </row>
     <row r="26">
@@ -6337,13 +6337,13 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>9.82</v>
+        <v>9.630000000000001</v>
       </c>
       <c r="G26" t="n">
-        <v>13300138846</v>
+        <v>13042804744</v>
       </c>
       <c r="H26" t="n">
-        <v>6420300</v>
+        <v>6288500</v>
       </c>
       <c r="I26" t="n">
         <v>1354393401</v>
@@ -6358,7 +6358,7 @@
         <v>1.94</v>
       </c>
       <c r="M26" t="n">
-        <v>0.1715041692357606</v>
+        <v>0.1681858676833815</v>
       </c>
       <c r="N26" t="n">
         <v>0.26</v>
@@ -6436,7 +6436,7 @@
         <v>961619314.7099999</v>
       </c>
       <c r="AM26" t="n">
-        <v>4750049587.857143</v>
+        <v>4658144551.428572</v>
       </c>
       <c r="AN26" t="n">
         <v>0.1043</v>
@@ -6477,7 +6477,7 @@
         <v>7.07</v>
       </c>
       <c r="AZ26" t="n">
-        <v>1.88</v>
+        <v>1.85</v>
       </c>
       <c r="BA26" t="n">
         <v>0.66</v>
@@ -6486,19 +6486,19 @@
         <v>1.19</v>
       </c>
       <c r="BC26" t="n">
-        <v>-11.86</v>
+        <v>-10.12</v>
       </c>
       <c r="BD26" t="n">
-        <v>-28.03</v>
+        <v>-26.61</v>
       </c>
       <c r="BE26" t="n">
         <v>-80.83</v>
       </c>
       <c r="BF26" t="n">
-        <v>-93.29000000000001</v>
+        <v>-93.15000000000001</v>
       </c>
       <c r="BG26" t="n">
-        <v>-87.84999999999999</v>
+        <v>-87.61</v>
       </c>
       <c r="BH26" t="n">
         <v>4.69</v>
@@ -6507,7 +6507,7 @@
         <v>0</v>
       </c>
       <c r="BJ26" t="n">
-        <v>9.82</v>
+        <v>9.630000000000001</v>
       </c>
       <c r="BK26" t="n">
         <v>0.71</v>
@@ -6516,7 +6516,7 @@
         <v>0.72</v>
       </c>
       <c r="BM26" t="n">
-        <v>10</v>
+        <v>9.82</v>
       </c>
       <c r="BN26" t="n">
         <v>10.6</v>
@@ -6525,19 +6525,19 @@
         <v>6.91</v>
       </c>
       <c r="BP26" t="n">
-        <v>9.710000000000001</v>
+        <v>9.5</v>
       </c>
       <c r="BQ26" t="n">
-        <v>13.69</v>
+        <v>13.43</v>
       </c>
       <c r="BR26" t="n">
-        <v>9.85</v>
+        <v>9.5</v>
       </c>
       <c r="BS26" t="n">
         <v>0.16</v>
       </c>
       <c r="BT26" t="n">
-        <v>11610410</v>
+        <v>11652403</v>
       </c>
     </row>
     <row r="27">
@@ -8165,13 +8165,13 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>16.43</v>
+        <v>15.77</v>
       </c>
       <c r="G34" t="n">
-        <v>3392627477</v>
+        <v>3256344240</v>
       </c>
       <c r="H34" t="n">
-        <v>2144200</v>
+        <v>2761600</v>
       </c>
       <c r="I34" t="n">
         <v>206489813</v>
@@ -8186,7 +8186,7 @@
         <v>0.45</v>
       </c>
       <c r="M34" t="n">
-        <v>0.2982515791180681</v>
+        <v>0.2862706908778672</v>
       </c>
       <c r="N34" t="n">
         <v>0.24</v>
@@ -8264,7 +8264,7 @@
         <v>324189006.41</v>
       </c>
       <c r="AM34" t="n">
-        <v>705327957.7962579</v>
+        <v>676994644.4906446</v>
       </c>
       <c r="AN34" t="n">
         <v>0</v>
@@ -8305,7 +8305,7 @@
         <v>30.28</v>
       </c>
       <c r="AZ34" t="n">
-        <v>38.34</v>
+        <v>36.8</v>
       </c>
       <c r="BA34" t="n">
         <v>2.29</v>
@@ -8314,19 +8314,19 @@
         <v>25.26</v>
       </c>
       <c r="BC34" t="n">
-        <v>125.74</v>
+        <v>135.18</v>
       </c>
       <c r="BD34" t="n">
-        <v>84.31</v>
+        <v>92.03</v>
       </c>
       <c r="BE34" t="n">
         <v>133.33</v>
       </c>
       <c r="BF34" t="n">
-        <v>-86.03</v>
+        <v>-85.45</v>
       </c>
       <c r="BG34" t="n">
-        <v>53.73</v>
+        <v>60.16</v>
       </c>
       <c r="BH34" t="n">
         <v>38.94</v>
@@ -8335,7 +8335,7 @@
         <v>0</v>
       </c>
       <c r="BJ34" t="n">
-        <v>16.43</v>
+        <v>15.77</v>
       </c>
       <c r="BK34" t="n">
         <v>1.57</v>
@@ -8344,7 +8344,7 @@
         <v>1.58</v>
       </c>
       <c r="BM34" t="n">
-        <v>17.32</v>
+        <v>16.2</v>
       </c>
       <c r="BN34" t="n">
         <v>31.12</v>
@@ -8353,19 +8353,19 @@
         <v>14.32</v>
       </c>
       <c r="BP34" t="n">
-        <v>16.35</v>
+        <v>15.69</v>
       </c>
       <c r="BQ34" t="n">
-        <v>10.42</v>
+        <v>10</v>
       </c>
       <c r="BR34" t="n">
-        <v>17.01</v>
+        <v>16.1</v>
       </c>
       <c r="BS34" t="n">
         <v>0.32</v>
       </c>
       <c r="BT34" t="n">
-        <v>3122953</v>
+        <v>3073890</v>
       </c>
     </row>
     <row r="35">
@@ -8395,13 +8395,13 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>17.28</v>
+        <v>17.37</v>
       </c>
       <c r="G35" t="n">
-        <v>87203523465</v>
+        <v>87657709235</v>
       </c>
       <c r="H35" t="n">
-        <v>32548400</v>
+        <v>38229400</v>
       </c>
       <c r="I35" t="n">
         <v>5046500000</v>
@@ -8416,7 +8416,7 @@
         <v>4.69</v>
       </c>
       <c r="M35" t="n">
-        <v>7.23966821219386</v>
+        <v>7.277374879893125</v>
       </c>
       <c r="N35" t="n">
         <v>1.79</v>
@@ -8494,7 +8494,7 @@
         <v>5349290000</v>
       </c>
       <c r="AM35" t="n">
-        <v>7206902765.702479</v>
+        <v>7244438779.752067</v>
       </c>
       <c r="AN35" t="n">
         <v>0.5305</v>
@@ -8535,7 +8535,7 @@
         <v>7.68</v>
       </c>
       <c r="AZ35" t="n">
-        <v>10.08</v>
+        <v>10.13</v>
       </c>
       <c r="BA35" t="n">
         <v>1.11</v>
@@ -8544,19 +8544,19 @@
         <v>9.119999999999999</v>
       </c>
       <c r="BC35" t="n">
-        <v>-45.56</v>
+        <v>-45.85</v>
       </c>
       <c r="BD35" t="n">
-        <v>-55.55</v>
+        <v>-55.78</v>
       </c>
       <c r="BE35" t="n">
         <v>-41.67</v>
       </c>
       <c r="BF35" t="n">
-        <v>-93.55</v>
+        <v>-93.59</v>
       </c>
       <c r="BG35" t="n">
-        <v>-47.24</v>
+        <v>-47.51</v>
       </c>
       <c r="BH35" t="n">
         <v>3.71</v>
@@ -8565,7 +8565,7 @@
         <v>0</v>
       </c>
       <c r="BJ35" t="n">
-        <v>17.28</v>
+        <v>17.37</v>
       </c>
       <c r="BK35" t="n">
         <v>1.06</v>
@@ -8574,7 +8574,7 @@
         <v>1.04</v>
       </c>
       <c r="BM35" t="n">
-        <v>17.83</v>
+        <v>17.44</v>
       </c>
       <c r="BN35" t="n">
         <v>20.08</v>
@@ -8583,19 +8583,19 @@
         <v>11.7</v>
       </c>
       <c r="BP35" t="n">
-        <v>17.2</v>
+        <v>16.81</v>
       </c>
       <c r="BQ35" t="n">
-        <v>16.54</v>
+        <v>16.62</v>
       </c>
       <c r="BR35" t="n">
-        <v>17.8</v>
+        <v>16.85</v>
       </c>
       <c r="BS35" t="n">
         <v>7.3</v>
       </c>
       <c r="BT35" t="n">
-        <v>37151143</v>
+        <v>36830480</v>
       </c>
     </row>
     <row r="36">
@@ -8855,13 +8855,13 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>15</v>
+        <v>14.9</v>
       </c>
       <c r="G37" t="n">
-        <v>203118150</v>
+        <v>199073828</v>
       </c>
       <c r="H37" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="I37" t="n">
         <v>4900000</v>
@@ -8876,7 +8876,7 @@
         <v>0.88</v>
       </c>
       <c r="M37" t="n">
-        <v>1.977526294725682</v>
+        <v>1.938151413163707</v>
       </c>
       <c r="N37" t="n">
         <v>0.5</v>
@@ -8954,7 +8954,7 @@
         <v>11319000</v>
       </c>
       <c r="AM37" t="n">
-        <v>48592858.85167465</v>
+        <v>47625317.70334928</v>
       </c>
       <c r="AN37" t="n">
         <v>0</v>
@@ -8995,7 +8995,7 @@
         <v>24.36</v>
       </c>
       <c r="AZ37" t="n">
-        <v>66.7</v>
+        <v>66.26000000000001</v>
       </c>
       <c r="BA37" t="n">
         <v>2.44</v>
@@ -9004,19 +9004,19 @@
         <v>15.53</v>
       </c>
       <c r="BC37" t="n">
-        <v>98.92</v>
+        <v>100.26</v>
       </c>
       <c r="BD37" t="n">
-        <v>62.42</v>
+        <v>63.51</v>
       </c>
       <c r="BE37" t="n">
         <v>344.67</v>
       </c>
       <c r="BF37" t="n">
-        <v>-83.7</v>
+        <v>-83.59</v>
       </c>
       <c r="BG37" t="n">
-        <v>3.56</v>
+        <v>4.25</v>
       </c>
       <c r="BH37" t="n">
         <v>17.13</v>
@@ -9025,7 +9025,7 @@
         <v>0</v>
       </c>
       <c r="BJ37" t="n">
-        <v>15</v>
+        <v>14.9</v>
       </c>
       <c r="BK37" t="n">
         <v>2.31</v>
@@ -9034,7 +9034,7 @@
         <v>2.31</v>
       </c>
       <c r="BM37" t="n">
-        <v>15</v>
+        <v>14.9</v>
       </c>
       <c r="BN37" t="n">
         <v>20.9</v>
@@ -9043,13 +9043,13 @@
         <v>13.05</v>
       </c>
       <c r="BP37" t="n">
-        <v>15</v>
+        <v>14.9</v>
       </c>
       <c r="BQ37" t="n">
-        <v>6.49</v>
+        <v>6.45</v>
       </c>
       <c r="BR37" t="n">
-        <v>15</v>
+        <v>14.9</v>
       </c>
       <c r="BS37" t="n">
         <v>0.72</v>
@@ -9315,13 +9315,13 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>69.75</v>
+        <v>69.04000000000001</v>
       </c>
       <c r="G39" t="n">
-        <v>3910067820</v>
+        <v>3870265083</v>
       </c>
       <c r="H39" t="n">
-        <v>2700</v>
+        <v>2800</v>
       </c>
       <c r="I39" t="n">
         <v>168174945</v>
@@ -9336,7 +9336,7 @@
         <v>0.53</v>
       </c>
       <c r="M39" t="n">
-        <v>0.1962682535799908</v>
+        <v>0.1942703307719169</v>
       </c>
       <c r="N39" t="n">
         <v>0.06</v>
@@ -9414,7 +9414,7 @@
         <v>2536078170.6</v>
       </c>
       <c r="AM39" t="n">
-        <v>410721409.6638656</v>
+        <v>406540449.894958</v>
       </c>
       <c r="AN39" t="n">
         <v>11.9435</v>
@@ -9455,7 +9455,7 @@
         <v>170.24</v>
       </c>
       <c r="AZ39" t="n">
-        <v>203.79</v>
+        <v>201.71</v>
       </c>
       <c r="BA39" t="n">
         <v>19.01</v>
@@ -9464,19 +9464,19 @@
         <v>91.72</v>
       </c>
       <c r="BC39" t="n">
-        <v>198.93</v>
+        <v>202.01</v>
       </c>
       <c r="BD39" t="n">
-        <v>144.08</v>
+        <v>146.59</v>
       </c>
       <c r="BE39" t="n">
         <v>192.17</v>
       </c>
       <c r="BF39" t="n">
-        <v>-72.75</v>
+        <v>-72.47</v>
       </c>
       <c r="BG39" t="n">
-        <v>31.5</v>
+        <v>32.86</v>
       </c>
       <c r="BH39" t="n">
         <v>128.13</v>
@@ -9485,7 +9485,7 @@
         <v>0</v>
       </c>
       <c r="BJ39" t="n">
-        <v>69.75</v>
+        <v>69.04000000000001</v>
       </c>
       <c r="BK39" t="n">
         <v>15.08</v>
@@ -9494,7 +9494,7 @@
         <v>15.08</v>
       </c>
       <c r="BM39" t="n">
-        <v>69.75</v>
+        <v>69.68000000000001</v>
       </c>
       <c r="BN39" t="n">
         <v>74.56</v>
@@ -9503,19 +9503,19 @@
         <v>54.98</v>
       </c>
       <c r="BP39" t="n">
-        <v>68</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="BQ39" t="n">
-        <v>4.62</v>
+        <v>4.58</v>
       </c>
       <c r="BR39" t="n">
-        <v>68</v>
+        <v>69.68000000000001</v>
       </c>
       <c r="BS39" t="n">
         <v>0.58</v>
       </c>
       <c r="BT39" t="n">
-        <v>3933</v>
+        <v>3903</v>
       </c>
     </row>
     <row r="40">
@@ -9545,13 +9545,13 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>22.49</v>
+        <v>22.12</v>
       </c>
       <c r="G40" t="n">
-        <v>128886432858</v>
+        <v>126766075009</v>
       </c>
       <c r="H40" t="n">
-        <v>22391900</v>
+        <v>29686100</v>
       </c>
       <c r="I40" t="n">
         <v>5730834040</v>
@@ -9566,7 +9566,7 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="M40" t="n">
-        <v>0.3910573877388558</v>
+        <v>0.3846239596183408</v>
       </c>
       <c r="N40" t="n">
         <v>0.05</v>
@@ -9644,7 +9644,7 @@
         <v>15358635227.2</v>
       </c>
       <c r="AM40" t="n">
-        <v>6684980957.365145</v>
+        <v>6575003890.508298</v>
       </c>
       <c r="AN40" t="n">
         <v>0.5641</v>
@@ -9685,7 +9685,7 @@
         <v>36.13</v>
       </c>
       <c r="AZ40" t="n">
-        <v>11.36</v>
+        <v>11.17</v>
       </c>
       <c r="BA40" t="n">
         <v>2.76</v>
@@ -9694,19 +9694,19 @@
         <v>27.89</v>
       </c>
       <c r="BC40" t="n">
-        <v>96.75</v>
+        <v>100.04</v>
       </c>
       <c r="BD40" t="n">
-        <v>60.64</v>
+        <v>63.33</v>
       </c>
       <c r="BE40" t="n">
         <v>-49.5</v>
       </c>
       <c r="BF40" t="n">
-        <v>-87.73</v>
+        <v>-87.52</v>
       </c>
       <c r="BG40" t="n">
-        <v>24.01</v>
+        <v>26.09</v>
       </c>
       <c r="BH40" t="n">
         <v>32.47</v>
@@ -9715,7 +9715,7 @@
         <v>0</v>
       </c>
       <c r="BJ40" t="n">
-        <v>22.49</v>
+        <v>22.12</v>
       </c>
       <c r="BK40" t="n">
         <v>2.68</v>
@@ -9724,7 +9724,7 @@
         <v>2.5</v>
       </c>
       <c r="BM40" t="n">
-        <v>22.97</v>
+        <v>22.26</v>
       </c>
       <c r="BN40" t="n">
         <v>27.36</v>
@@ -9733,19 +9733,19 @@
         <v>17.67</v>
       </c>
       <c r="BP40" t="n">
-        <v>22.29</v>
+        <v>21.83</v>
       </c>
       <c r="BQ40" t="n">
-        <v>9</v>
+        <v>8.85</v>
       </c>
       <c r="BR40" t="n">
-        <v>22.8</v>
+        <v>21.95</v>
       </c>
       <c r="BS40" t="n">
         <v>0.39</v>
       </c>
       <c r="BT40" t="n">
-        <v>30950360</v>
+        <v>31162577</v>
       </c>
     </row>
     <row r="41">
@@ -9775,13 +9775,13 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>16.32</v>
+        <v>16.17</v>
       </c>
       <c r="G41" t="n">
-        <v>195515865004</v>
+        <v>192689175097</v>
       </c>
       <c r="H41" t="n">
-        <v>5176200</v>
+        <v>6498700</v>
       </c>
       <c r="I41" t="n">
         <v>5303870781</v>
@@ -9796,7 +9796,7 @@
         <v>0.92</v>
       </c>
       <c r="M41" t="n">
-        <v>1.302911557289405</v>
+        <v>1.284074584910574</v>
       </c>
       <c r="N41" t="n">
         <v>0.07000000000000001</v>
@@ -9874,7 +9874,7 @@
         <v>12304980211.92</v>
       </c>
       <c r="AM41" t="n">
-        <v>30125711094.60709</v>
+        <v>29690165654.39137</v>
       </c>
       <c r="AN41" t="n">
         <v>1.6841</v>
@@ -9915,7 +9915,7 @@
         <v>24.4</v>
       </c>
       <c r="AZ41" t="n">
-        <v>24.43</v>
+        <v>24.2</v>
       </c>
       <c r="BA41" t="n">
         <v>2.53</v>
@@ -9924,19 +9924,19 @@
         <v>13.77</v>
       </c>
       <c r="BC41" t="n">
-        <v>83.12</v>
+        <v>84.81999999999999</v>
       </c>
       <c r="BD41" t="n">
-        <v>49.52</v>
+        <v>50.91</v>
       </c>
       <c r="BE41" t="n">
         <v>49.67</v>
       </c>
       <c r="BF41" t="n">
-        <v>-84.51000000000001</v>
+        <v>-84.37</v>
       </c>
       <c r="BG41" t="n">
-        <v>-15.62</v>
+        <v>-14.84</v>
       </c>
       <c r="BH41" t="n">
         <v>17.11</v>
@@ -9945,7 +9945,7 @@
         <v>0</v>
       </c>
       <c r="BJ41" t="n">
-        <v>16.32</v>
+        <v>16.17</v>
       </c>
       <c r="BK41" t="n">
         <v>2.32</v>
@@ -9954,28 +9954,28 @@
         <v>2.34</v>
       </c>
       <c r="BM41" t="n">
-        <v>16.38</v>
+        <v>16.2</v>
       </c>
       <c r="BN41" t="n">
         <v>18.28</v>
       </c>
       <c r="BO41" t="n">
-        <v>13.34</v>
+        <v>13.43</v>
       </c>
       <c r="BP41" t="n">
-        <v>16.17</v>
+        <v>15.92</v>
       </c>
       <c r="BQ41" t="n">
-        <v>6.98</v>
+        <v>6.92</v>
       </c>
       <c r="BR41" t="n">
-        <v>16.25</v>
+        <v>15.96</v>
       </c>
       <c r="BS41" t="n">
         <v>0.5600000000000001</v>
       </c>
       <c r="BT41" t="n">
-        <v>7409959</v>
+        <v>7349463</v>
       </c>
     </row>
     <row r="42">
@@ -10005,13 +10005,13 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>18.59</v>
+        <v>18.33</v>
       </c>
       <c r="G42" t="n">
-        <v>195515865004</v>
+        <v>192689175097</v>
       </c>
       <c r="H42" t="n">
-        <v>34171600</v>
+        <v>21528800</v>
       </c>
       <c r="I42" t="n">
         <v>5288141247</v>
@@ -10026,7 +10026,7 @@
         <v>1.05</v>
       </c>
       <c r="M42" t="n">
-        <v>1.306787057334152</v>
+        <v>1.287894054531085</v>
       </c>
       <c r="N42" t="n">
         <v>0.08</v>
@@ -10104,7 +10104,7 @@
         <v>12268487693.04</v>
       </c>
       <c r="AM42" t="n">
-        <v>26600797959.72789</v>
+        <v>26216214298.91157</v>
       </c>
       <c r="AN42" t="n">
         <v>1.8491</v>
@@ -10145,7 +10145,7 @@
         <v>24.4</v>
       </c>
       <c r="AZ42" t="n">
-        <v>26.92</v>
+        <v>26.55</v>
       </c>
       <c r="BA42" t="n">
         <v>2.53</v>
@@ -10154,19 +10154,19 @@
         <v>15.11</v>
       </c>
       <c r="BC42" t="n">
-        <v>60.76</v>
+        <v>63.04</v>
       </c>
       <c r="BD42" t="n">
-        <v>31.26</v>
+        <v>33.12</v>
       </c>
       <c r="BE42" t="n">
         <v>44.83</v>
       </c>
       <c r="BF42" t="n">
-        <v>-86.41</v>
+        <v>-86.20999999999999</v>
       </c>
       <c r="BG42" t="n">
-        <v>-18.69</v>
+        <v>-17.54</v>
       </c>
       <c r="BH42" t="n">
         <v>17.11</v>
@@ -10175,7 +10175,7 @@
         <v>0</v>
       </c>
       <c r="BJ42" t="n">
-        <v>18.59</v>
+        <v>18.33</v>
       </c>
       <c r="BK42" t="n">
         <v>2.32</v>
@@ -10184,28 +10184,28 @@
         <v>2.34</v>
       </c>
       <c r="BM42" t="n">
-        <v>18.59</v>
+        <v>18.44</v>
       </c>
       <c r="BN42" t="n">
         <v>21.33</v>
       </c>
       <c r="BO42" t="n">
-        <v>15.64</v>
+        <v>15.67</v>
       </c>
       <c r="BP42" t="n">
-        <v>18.37</v>
+        <v>18.12</v>
       </c>
       <c r="BQ42" t="n">
-        <v>7.95</v>
+        <v>7.84</v>
       </c>
       <c r="BR42" t="n">
-        <v>18.5</v>
+        <v>18.2</v>
       </c>
       <c r="BS42" t="n">
         <v>0.63</v>
       </c>
       <c r="BT42" t="n">
-        <v>40850208</v>
+        <v>40385889</v>
       </c>
     </row>
     <row r="43">
@@ -10235,13 +10235,13 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>39.5</v>
+        <v>39.77</v>
       </c>
       <c r="G43" t="n">
-        <v>76685260500</v>
+        <v>77209478888</v>
       </c>
       <c r="H43" t="n">
-        <v>9254800</v>
+        <v>5320400</v>
       </c>
       <c r="I43" t="n">
         <v>1941400000</v>
@@ -10334,7 +10334,7 @@
         <v>9182822000</v>
       </c>
       <c r="AM43" t="n">
-        <v>9340470219.244822</v>
+        <v>9404321423.629719</v>
       </c>
       <c r="AN43" t="n">
         <v>4.5901</v>
@@ -10375,7 +10375,7 @@
         <v>19.95</v>
       </c>
       <c r="AZ43" t="n">
-        <v>71.69</v>
+        <v>72.18000000000001</v>
       </c>
       <c r="BA43" t="n">
         <v>5.63</v>
@@ -10384,19 +10384,19 @@
         <v>48.62</v>
       </c>
       <c r="BC43" t="n">
-        <v>-38.14</v>
+        <v>-38.56</v>
       </c>
       <c r="BD43" t="n">
-        <v>-49.49</v>
+        <v>-49.83</v>
       </c>
       <c r="BE43" t="n">
         <v>81.5</v>
       </c>
       <c r="BF43" t="n">
-        <v>-85.75</v>
+        <v>-85.84999999999999</v>
       </c>
       <c r="BG43" t="n">
-        <v>23.08</v>
+        <v>22.25</v>
       </c>
       <c r="BH43" t="n">
         <v>5.61</v>
@@ -10405,7 +10405,7 @@
         <v>0</v>
       </c>
       <c r="BJ43" t="n">
-        <v>39.5</v>
+        <v>39.77</v>
       </c>
       <c r="BK43" t="n">
         <v>4.73</v>
@@ -10414,7 +10414,7 @@
         <v>4.73</v>
       </c>
       <c r="BM43" t="n">
-        <v>41.25</v>
+        <v>40.11</v>
       </c>
       <c r="BN43" t="n">
         <v>42.98</v>
@@ -10423,19 +10423,19 @@
         <v>28.06</v>
       </c>
       <c r="BP43" t="n">
-        <v>39.47</v>
+        <v>38.86</v>
       </c>
       <c r="BQ43" t="n">
-        <v>8.34</v>
+        <v>8.4</v>
       </c>
       <c r="BR43" t="n">
-        <v>41.03</v>
+        <v>39.06</v>
       </c>
       <c r="BS43" t="n">
         <v>0</v>
       </c>
       <c r="BT43" t="n">
-        <v>6532688</v>
+        <v>6715793</v>
       </c>
     </row>
     <row r="44">
@@ -10925,13 +10925,13 @@
         </is>
       </c>
       <c r="F46" t="n">
-        <v>4.13</v>
+        <v>4.08</v>
       </c>
       <c r="G46" t="n">
-        <v>4132234444</v>
+        <v>4082207203</v>
       </c>
       <c r="H46" t="n">
-        <v>41219100</v>
+        <v>24498800</v>
       </c>
       <c r="I46" t="n">
         <v>1000541644</v>
@@ -10946,7 +10946,7 @@
         <v>2.5</v>
       </c>
       <c r="M46" t="n">
-        <v>0.07182604270709787</v>
+        <v>0.07095647472946251</v>
       </c>
       <c r="N46" t="n">
         <v>0.08</v>
@@ -11024,7 +11024,7 @@
         <v>460249156.24</v>
       </c>
       <c r="AM46" t="n">
-        <v>4051210239.215686</v>
+        <v>4002163924.509804</v>
       </c>
       <c r="AN46" t="n">
         <v>0.0311</v>
@@ -11065,7 +11065,7 @@
         <v>3.3</v>
       </c>
       <c r="AZ46" t="n">
-        <v>3.41</v>
+        <v>3.37</v>
       </c>
       <c r="BA46" t="n">
         <v>0.42</v>
@@ -11074,19 +11074,19 @@
         <v>7.38</v>
       </c>
       <c r="BC46" t="n">
-        <v>-2.09</v>
+        <v>-0.89</v>
       </c>
       <c r="BD46" t="n">
-        <v>-20.05</v>
+        <v>-19.07</v>
       </c>
       <c r="BE46" t="n">
         <v>-17.5</v>
       </c>
       <c r="BF46" t="n">
-        <v>-89.76000000000001</v>
+        <v>-89.63</v>
       </c>
       <c r="BG46" t="n">
-        <v>78.66</v>
+        <v>80.84999999999999</v>
       </c>
       <c r="BH46" t="n">
         <v>1.58</v>
@@ -11095,7 +11095,7 @@
         <v>0</v>
       </c>
       <c r="BJ46" t="n">
-        <v>4.13</v>
+        <v>4.08</v>
       </c>
       <c r="BK46" t="n">
         <v>0.46</v>
@@ -11104,7 +11104,7 @@
         <v>0.46</v>
       </c>
       <c r="BM46" t="n">
-        <v>4.16</v>
+        <v>4.2</v>
       </c>
       <c r="BN46" t="n">
         <v>7.31</v>
@@ -11113,19 +11113,19 @@
         <v>2.97</v>
       </c>
       <c r="BP46" t="n">
-        <v>3.85</v>
+        <v>4.06</v>
       </c>
       <c r="BQ46" t="n">
-        <v>9.029999999999999</v>
+        <v>8.92</v>
       </c>
       <c r="BR46" t="n">
-        <v>3.99</v>
+        <v>4.14</v>
       </c>
       <c r="BS46" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="BT46" t="n">
-        <v>18378000</v>
+        <v>19430970</v>
       </c>
     </row>
     <row r="47">
@@ -11155,13 +11155,13 @@
         </is>
       </c>
       <c r="F47" t="n">
-        <v>9.029999999999999</v>
+        <v>8.81</v>
       </c>
       <c r="G47" t="n">
-        <v>3149333408</v>
+        <v>3060600312</v>
       </c>
       <c r="H47" t="n">
-        <v>8000</v>
+        <v>16100</v>
       </c>
       <c r="I47" t="n">
         <v>254106600</v>
@@ -11176,7 +11176,7 @@
         <v>1.22</v>
       </c>
       <c r="M47" t="n">
-        <v>0.7426490515063208</v>
+        <v>0.7217247665721741</v>
       </c>
       <c r="N47" t="n">
         <v>0.07000000000000001</v>
@@ -11254,7 +11254,7 @@
         <v>322715382</v>
       </c>
       <c r="AM47" t="n">
-        <v>558392448.2269504</v>
+        <v>542659629.7872341</v>
       </c>
       <c r="AN47" t="n">
         <v>0.4132</v>
@@ -11295,7 +11295,7 @@
         <v>11.74</v>
       </c>
       <c r="AZ47" t="n">
-        <v>11.86</v>
+        <v>11.57</v>
       </c>
       <c r="BA47" t="n">
         <v>1.46</v>
@@ -11304,19 +11304,19 @@
         <v>8.619999999999999</v>
       </c>
       <c r="BC47" t="n">
-        <v>59.17</v>
+        <v>63.15</v>
       </c>
       <c r="BD47" t="n">
-        <v>29.97</v>
+        <v>33.21</v>
       </c>
       <c r="BE47" t="n">
         <v>31.33</v>
       </c>
       <c r="BF47" t="n">
-        <v>-83.84999999999999</v>
+        <v>-83.45</v>
       </c>
       <c r="BG47" t="n">
-        <v>-4.54</v>
+        <v>-2.16</v>
       </c>
       <c r="BH47" t="n">
         <v>7.23</v>
@@ -11325,7 +11325,7 @@
         <v>0</v>
       </c>
       <c r="BJ47" t="n">
-        <v>9.029999999999999</v>
+        <v>8.81</v>
       </c>
       <c r="BK47" t="n">
         <v>1.27</v>
@@ -11334,7 +11334,7 @@
         <v>1.29</v>
       </c>
       <c r="BM47" t="n">
-        <v>9.029999999999999</v>
+        <v>9.1</v>
       </c>
       <c r="BN47" t="n">
         <v>9.25</v>
@@ -11343,19 +11343,19 @@
         <v>7.2</v>
       </c>
       <c r="BP47" t="n">
-        <v>8.9</v>
+        <v>8.789999999999999</v>
       </c>
       <c r="BQ47" t="n">
-        <v>6.98</v>
+        <v>6.81</v>
       </c>
       <c r="BR47" t="n">
-        <v>8.9</v>
+        <v>9.029999999999999</v>
       </c>
       <c r="BS47" t="n">
         <v>0.53</v>
       </c>
       <c r="BT47" t="n">
-        <v>12707</v>
+        <v>12736</v>
       </c>
     </row>
     <row r="48">
@@ -11385,13 +11385,13 @@
         </is>
       </c>
       <c r="F48" t="n">
-        <v>9.02</v>
+        <v>9.039999999999999</v>
       </c>
       <c r="G48" t="n">
-        <v>3149333408</v>
+        <v>3060600312</v>
       </c>
       <c r="H48" t="n">
-        <v>2000</v>
+        <v>1300</v>
       </c>
       <c r="I48" t="n">
         <v>93397546</v>
@@ -11406,7 +11406,7 @@
         <v>1.24</v>
       </c>
       <c r="M48" t="n">
-        <v>2.020524452232354</v>
+        <v>1.963595773377695</v>
       </c>
       <c r="N48" t="n">
         <v>0.07000000000000001</v>
@@ -11484,7 +11484,7 @@
         <v>118614883.42</v>
       </c>
       <c r="AM48" t="n">
-        <v>550582763.6363636</v>
+        <v>535069984.6153846</v>
       </c>
       <c r="AN48" t="n">
         <v>0.4132</v>
@@ -11525,7 +11525,7 @@
         <v>11.74</v>
       </c>
       <c r="AZ48" t="n">
-        <v>11.8</v>
+        <v>11.83</v>
       </c>
       <c r="BA48" t="n">
         <v>1.46</v>
@@ -11534,19 +11534,19 @@
         <v>8.24</v>
       </c>
       <c r="BC48" t="n">
-        <v>59.35</v>
+        <v>59</v>
       </c>
       <c r="BD48" t="n">
-        <v>30.11</v>
+        <v>29.82</v>
       </c>
       <c r="BE48" t="n">
         <v>30.83</v>
       </c>
       <c r="BF48" t="n">
-        <v>-83.83</v>
+        <v>-83.87</v>
       </c>
       <c r="BG48" t="n">
-        <v>-8.69</v>
+        <v>-8.890000000000001</v>
       </c>
       <c r="BH48" t="n">
         <v>7.23</v>
@@ -11555,7 +11555,7 @@
         <v>0</v>
       </c>
       <c r="BJ48" t="n">
-        <v>9.02</v>
+        <v>9.039999999999999</v>
       </c>
       <c r="BK48" t="n">
         <v>1.27</v>
@@ -11564,7 +11564,7 @@
         <v>1.29</v>
       </c>
       <c r="BM48" t="n">
-        <v>9.06</v>
+        <v>9.1</v>
       </c>
       <c r="BN48" t="n">
         <v>9.48</v>
@@ -11573,19 +11573,19 @@
         <v>7.21</v>
       </c>
       <c r="BP48" t="n">
-        <v>9</v>
+        <v>9.029999999999999</v>
       </c>
       <c r="BQ48" t="n">
-        <v>6.97</v>
+        <v>6.99</v>
       </c>
       <c r="BR48" t="n">
-        <v>9.029999999999999</v>
+        <v>9.1</v>
       </c>
       <c r="BS48" t="n">
         <v>0.54</v>
       </c>
       <c r="BT48" t="n">
-        <v>2702</v>
+        <v>2678</v>
       </c>
     </row>
     <row r="49">
@@ -11851,7 +11851,7 @@
         <v>974049400</v>
       </c>
       <c r="H50" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I50" t="n">
         <v>11540870</v>
@@ -12523,13 +12523,13 @@
         </is>
       </c>
       <c r="F53" t="n">
-        <v>6.7</v>
+        <v>6.53</v>
       </c>
       <c r="G53" t="n">
-        <v>916911053</v>
+        <v>893646200</v>
       </c>
       <c r="H53" t="n">
-        <v>51100</v>
+        <v>1600</v>
       </c>
       <c r="I53" t="n">
         <v>136852484</v>
@@ -12544,7 +12544,7 @@
         <v>2.79</v>
       </c>
       <c r="M53" t="n">
-        <v>2.38196398505093</v>
+        <v>2.321526233992972</v>
       </c>
       <c r="N53" t="n">
         <v>1.48</v>
@@ -12622,7 +12622,7 @@
         <v>39687220.36</v>
       </c>
       <c r="AM53" t="n">
-        <v>46709681.76260825</v>
+        <v>45524513.49974529</v>
       </c>
       <c r="AN53" t="n">
         <v>0</v>
@@ -12672,16 +12672,16 @@
         <v>0</v>
       </c>
       <c r="BC53" t="n">
-        <v>-41.18</v>
+        <v>-39.65</v>
       </c>
       <c r="BD53" t="n">
-        <v>-51.98</v>
+        <v>-50.73</v>
       </c>
       <c r="BE53" t="n">
         <v>-100</v>
       </c>
       <c r="BF53" t="n">
-        <v>-95.67</v>
+        <v>-95.56</v>
       </c>
       <c r="BG53" t="n">
         <v>-100</v>
@@ -12693,7 +12693,7 @@
         <v>0</v>
       </c>
       <c r="BJ53" t="n">
-        <v>6.7</v>
+        <v>6.53</v>
       </c>
       <c r="BK53" t="n">
         <v>0.29</v>
@@ -12702,7 +12702,7 @@
         <v>0.09</v>
       </c>
       <c r="BM53" t="n">
-        <v>6.78</v>
+        <v>6.7</v>
       </c>
       <c r="BN53" t="n">
         <v>10.39</v>
@@ -12711,19 +12711,19 @@
         <v>4.82</v>
       </c>
       <c r="BP53" t="n">
-        <v>6.53</v>
+        <v>6.52</v>
       </c>
       <c r="BQ53" t="n">
-        <v>78.53</v>
+        <v>76.54000000000001</v>
       </c>
       <c r="BR53" t="n">
-        <v>6.53</v>
+        <v>6.7</v>
       </c>
       <c r="BS53" t="n">
         <v>2.36</v>
       </c>
       <c r="BT53" t="n">
-        <v>44010</v>
+        <v>44250</v>
       </c>
     </row>
     <row r="54">
@@ -12753,13 +12753,13 @@
         </is>
       </c>
       <c r="F54" t="n">
-        <v>10.18</v>
+        <v>10.45</v>
       </c>
       <c r="G54" t="n">
-        <v>2374098231</v>
+        <v>2437065355</v>
       </c>
       <c r="H54" t="n">
-        <v>364200</v>
+        <v>314600</v>
       </c>
       <c r="I54" t="n">
         <v>233212121</v>
@@ -12774,7 +12774,7 @@
         <v>0.97</v>
       </c>
       <c r="M54" t="n">
-        <v>1.332561348463959</v>
+        <v>1.36790426501674</v>
       </c>
       <c r="N54" t="n">
         <v>0.5600000000000001</v>
@@ -12852,7 +12852,7 @@
         <v>233212121</v>
       </c>
       <c r="AM54" t="n">
-        <v>324774039.8084816</v>
+        <v>333387873.4610123</v>
       </c>
       <c r="AN54" t="n">
         <v>0.1531</v>
@@ -12893,7 +12893,7 @@
         <v>12.25</v>
       </c>
       <c r="AZ54" t="n">
-        <v>16.2</v>
+        <v>16.63</v>
       </c>
       <c r="BA54" t="n">
         <v>0.98</v>
@@ -12902,19 +12902,19 @@
         <v>6.52</v>
       </c>
       <c r="BC54" t="n">
-        <v>47.42</v>
+        <v>43.61</v>
       </c>
       <c r="BD54" t="n">
-        <v>20.37</v>
+        <v>17.26</v>
       </c>
       <c r="BE54" t="n">
         <v>59.17</v>
       </c>
       <c r="BF54" t="n">
-        <v>-90.34</v>
+        <v>-90.59</v>
       </c>
       <c r="BG54" t="n">
-        <v>-35.99</v>
+        <v>-37.64</v>
       </c>
       <c r="BH54" t="n">
         <v>10.01</v>
@@ -12923,7 +12923,7 @@
         <v>0</v>
       </c>
       <c r="BJ54" t="n">
-        <v>10.18</v>
+        <v>10.45</v>
       </c>
       <c r="BK54" t="n">
         <v>1</v>
@@ -12932,7 +12932,7 @@
         <v>1</v>
       </c>
       <c r="BM54" t="n">
-        <v>10.18</v>
+        <v>10.45</v>
       </c>
       <c r="BN54" t="n">
         <v>11.75</v>
@@ -12941,19 +12941,19 @@
         <v>8.279999999999999</v>
       </c>
       <c r="BP54" t="n">
-        <v>9.880000000000001</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="BQ54" t="n">
-        <v>10.15</v>
+        <v>10.42</v>
       </c>
       <c r="BR54" t="n">
-        <v>10</v>
+        <v>10.12</v>
       </c>
       <c r="BS54" t="n">
         <v>1.26</v>
       </c>
       <c r="BT54" t="n">
-        <v>279180</v>
+        <v>277960</v>
       </c>
     </row>
     <row r="55">
@@ -12983,13 +12983,13 @@
         </is>
       </c>
       <c r="F55" t="n">
-        <v>51.03</v>
+        <v>49.53</v>
       </c>
       <c r="G55" t="n">
-        <v>6579775784</v>
+        <v>5087404482</v>
       </c>
       <c r="H55" t="n">
-        <v>5300</v>
+        <v>9600</v>
       </c>
       <c r="I55" t="n">
         <v>84052790</v>
@@ -13004,7 +13004,7 @@
         <v>2</v>
       </c>
       <c r="M55" t="n">
-        <v>1.015727609880742</v>
+        <v>0.7853485232071301</v>
       </c>
       <c r="N55" t="n">
         <v>0.16</v>
@@ -13082,7 +13082,7 @@
         <v>579123723.1</v>
       </c>
       <c r="AM55" t="n">
-        <v>330974637.0221328</v>
+        <v>255905658.0482897</v>
       </c>
       <c r="AN55" t="n">
         <v>3.1953</v>
@@ -13123,7 +13123,7 @@
         <v>51.21</v>
       </c>
       <c r="AZ55" t="n">
-        <v>53.67</v>
+        <v>52.09</v>
       </c>
       <c r="BA55" t="n">
         <v>9.380000000000001</v>
@@ -13132,19 +13132,19 @@
         <v>16.08</v>
       </c>
       <c r="BC55" t="n">
-        <v>22.9</v>
+        <v>26.62</v>
       </c>
       <c r="BD55" t="n">
-        <v>0.34</v>
+        <v>3.38</v>
       </c>
       <c r="BE55" t="n">
         <v>5.17</v>
       </c>
       <c r="BF55" t="n">
-        <v>-81.62</v>
+        <v>-81.06999999999999</v>
       </c>
       <c r="BG55" t="n">
-        <v>-68.5</v>
+        <v>-67.54000000000001</v>
       </c>
       <c r="BH55" t="n">
         <v>25.37</v>
@@ -13153,7 +13153,7 @@
         <v>0</v>
       </c>
       <c r="BJ55" t="n">
-        <v>51.03</v>
+        <v>49.53</v>
       </c>
       <c r="BK55" t="n">
         <v>6.89</v>
@@ -13162,7 +13162,7 @@
         <v>7.03</v>
       </c>
       <c r="BM55" t="n">
-        <v>51.86</v>
+        <v>50.93</v>
       </c>
       <c r="BN55" t="n">
         <v>73.67</v>
@@ -13171,19 +13171,19 @@
         <v>34.46</v>
       </c>
       <c r="BP55" t="n">
-        <v>51.03</v>
+        <v>49.31</v>
       </c>
       <c r="BQ55" t="n">
-        <v>7.26</v>
+        <v>7.04</v>
       </c>
       <c r="BR55" t="n">
-        <v>51.5</v>
+        <v>50.93</v>
       </c>
       <c r="BS55" t="n">
         <v>0.66</v>
       </c>
       <c r="BT55" t="n">
-        <v>6564</v>
+        <v>6645</v>
       </c>
     </row>
     <row r="56">
@@ -13213,13 +13213,13 @@
         </is>
       </c>
       <c r="F56" t="n">
-        <v>58.72</v>
+        <v>58.71</v>
       </c>
       <c r="G56" t="n">
-        <v>6579775784</v>
+        <v>5087404482</v>
       </c>
       <c r="H56" t="n">
-        <v>23000</v>
+        <v>46600</v>
       </c>
       <c r="I56" t="n">
         <v>39675836</v>
@@ -13234,7 +13234,7 @@
         <v>2.41</v>
       </c>
       <c r="M56" t="n">
-        <v>2.151806945933237</v>
+        <v>1.663751571559552</v>
       </c>
       <c r="N56" t="n">
         <v>0.19</v>
@@ -13312,7 +13312,7 @@
         <v>273366510.04</v>
       </c>
       <c r="AM56" t="n">
-        <v>273701155.7404326</v>
+        <v>211622482.6123128</v>
       </c>
       <c r="AN56" t="n">
         <v>3.5102</v>
@@ -13353,7 +13353,7 @@
         <v>51.21</v>
       </c>
       <c r="AZ56" t="n">
-        <v>56.08</v>
+        <v>56.07</v>
       </c>
       <c r="BA56" t="n">
         <v>9.380000000000001</v>
@@ -13362,10 +13362,10 @@
         <v>17.68</v>
       </c>
       <c r="BC56" t="n">
-        <v>6.8</v>
+        <v>6.82</v>
       </c>
       <c r="BD56" t="n">
-        <v>-12.8</v>
+        <v>-12.78</v>
       </c>
       <c r="BE56" t="n">
         <v>-4.5</v>
@@ -13374,7 +13374,7 @@
         <v>-84.03</v>
       </c>
       <c r="BG56" t="n">
-        <v>-69.90000000000001</v>
+        <v>-69.89</v>
       </c>
       <c r="BH56" t="n">
         <v>25.37</v>
@@ -13383,7 +13383,7 @@
         <v>0</v>
       </c>
       <c r="BJ56" t="n">
-        <v>58.72</v>
+        <v>58.71</v>
       </c>
       <c r="BK56" t="n">
         <v>6.89</v>
@@ -13392,28 +13392,28 @@
         <v>7.03</v>
       </c>
       <c r="BM56" t="n">
-        <v>61.25</v>
+        <v>60.76</v>
       </c>
       <c r="BN56" t="n">
         <v>86.77</v>
       </c>
       <c r="BO56" t="n">
-        <v>46.08</v>
+        <v>46.32</v>
       </c>
       <c r="BP56" t="n">
-        <v>58.72</v>
+        <v>57</v>
       </c>
       <c r="BQ56" t="n">
         <v>8.35</v>
       </c>
       <c r="BR56" t="n">
-        <v>61.25</v>
+        <v>58.65</v>
       </c>
       <c r="BS56" t="n">
         <v>0.79</v>
       </c>
       <c r="BT56" t="n">
-        <v>32888</v>
+        <v>33006</v>
       </c>
     </row>
     <row r="57">
@@ -13443,13 +13443,13 @@
         </is>
       </c>
       <c r="F57" t="n">
-        <v>6.09</v>
+        <v>6.08</v>
       </c>
       <c r="G57" t="n">
-        <v>1424195255</v>
+        <v>1421857230</v>
       </c>
       <c r="H57" t="n">
-        <v>960500</v>
+        <v>1303700</v>
       </c>
       <c r="I57" t="n">
         <v>233858065</v>
@@ -13464,7 +13464,7 @@
         <v>0.77</v>
       </c>
       <c r="M57" t="n">
-        <v>0.4262998919879031</v>
+        <v>0.4256000583088722</v>
       </c>
       <c r="N57" t="n">
         <v>0.08</v>
@@ -13542,7 +13542,7 @@
         <v>229180903.7</v>
       </c>
       <c r="AM57" t="n">
-        <v>106521709.4240838</v>
+        <v>106346838.4442782</v>
       </c>
       <c r="AN57" t="n">
         <v>0.347</v>
@@ -13583,7 +13583,7 @@
         <v>10.72</v>
       </c>
       <c r="AZ57" t="n">
-        <v>9.289999999999999</v>
+        <v>9.27</v>
       </c>
       <c r="BA57" t="n">
         <v>1.13</v>
@@ -13592,19 +13592,19 @@
         <v>6.26</v>
       </c>
       <c r="BC57" t="n">
-        <v>115.62</v>
+        <v>115.98</v>
       </c>
       <c r="BD57" t="n">
-        <v>76.05</v>
+        <v>76.34</v>
       </c>
       <c r="BE57" t="n">
         <v>52.5</v>
       </c>
       <c r="BF57" t="n">
-        <v>-81.48999999999999</v>
+        <v>-81.45999999999999</v>
       </c>
       <c r="BG57" t="n">
-        <v>2.86</v>
+        <v>3.02</v>
       </c>
       <c r="BH57" t="n">
         <v>7.82</v>
@@ -13613,7 +13613,7 @@
         <v>0</v>
       </c>
       <c r="BJ57" t="n">
-        <v>6.09</v>
+        <v>6.08</v>
       </c>
       <c r="BK57" t="n">
         <v>0.98</v>
@@ -13622,28 +13622,28 @@
         <v>1.04</v>
       </c>
       <c r="BM57" t="n">
-        <v>6.11</v>
+        <v>6.08</v>
       </c>
       <c r="BN57" t="n">
         <v>6.11</v>
       </c>
       <c r="BO57" t="n">
-        <v>3.39</v>
+        <v>3.4</v>
       </c>
       <c r="BP57" t="n">
-        <v>5.96</v>
+        <v>5.85</v>
       </c>
       <c r="BQ57" t="n">
-        <v>5.88</v>
+        <v>5.87</v>
       </c>
       <c r="BR57" t="n">
-        <v>5.99</v>
+        <v>6.06</v>
       </c>
       <c r="BS57" t="n">
         <v>0.42</v>
       </c>
       <c r="BT57" t="n">
-        <v>1266570</v>
+        <v>1281513</v>
       </c>
     </row>
     <row r="58">
@@ -14133,13 +14133,13 @@
         </is>
       </c>
       <c r="F60" t="n">
-        <v>376.6</v>
+        <v>376.99</v>
       </c>
       <c r="G60" t="n">
-        <v>171258900</v>
+        <v>171436235</v>
       </c>
       <c r="H60" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I60" t="n">
         <v>454750</v>
@@ -14154,7 +14154,7 @@
         <v>0.83</v>
       </c>
       <c r="M60" t="n">
-        <v>12.80992463784517</v>
+        <v>12.82318904620965</v>
       </c>
       <c r="N60" t="n">
         <v>0.68</v>
@@ -14232,7 +14232,7 @@
         <v>59558607.5</v>
       </c>
       <c r="AM60" t="n">
-        <v>-25111275.65982405</v>
+        <v>-25137277.85923754</v>
       </c>
       <c r="AN60" t="n">
         <v>10.0581</v>
@@ -14273,7 +14273,7 @@
         <v>944.87</v>
       </c>
       <c r="AZ60" t="n">
-        <v>2165.45</v>
+        <v>2167.69</v>
       </c>
       <c r="BA60" t="n">
         <v>231.1</v>
@@ -14282,19 +14282,19 @@
         <v>727.97</v>
       </c>
       <c r="BC60" t="n">
-        <v>207.28</v>
+        <v>206.96</v>
       </c>
       <c r="BD60" t="n">
-        <v>150.89</v>
+        <v>150.63</v>
       </c>
       <c r="BE60" t="n">
         <v>475</v>
       </c>
       <c r="BF60" t="n">
-        <v>-38.64</v>
+        <v>-38.7</v>
       </c>
       <c r="BG60" t="n">
-        <v>93.3</v>
+        <v>93.09999999999999</v>
       </c>
       <c r="BH60" t="n">
         <v>454.44</v>
@@ -14303,7 +14303,7 @@
         <v>0</v>
       </c>
       <c r="BJ60" t="n">
-        <v>376.6</v>
+        <v>376.99</v>
       </c>
       <c r="BK60" t="n">
         <v>130.97</v>
@@ -14321,13 +14321,13 @@
         <v>306.27</v>
       </c>
       <c r="BP60" t="n">
-        <v>371.25</v>
+        <v>369.01</v>
       </c>
       <c r="BQ60" t="n">
         <v>2.88</v>
       </c>
       <c r="BR60" t="n">
-        <v>377</v>
+        <v>376.6</v>
       </c>
       <c r="BS60" t="n">
         <v>12.82</v>
@@ -14363,13 +14363,13 @@
         </is>
       </c>
       <c r="F61" t="n">
-        <v>26.27</v>
+        <v>26.9</v>
       </c>
       <c r="G61" t="n">
-        <v>2248932444</v>
+        <v>2302865120</v>
       </c>
       <c r="H61" t="n">
-        <v>369800</v>
+        <v>586000</v>
       </c>
       <c r="I61" t="n">
         <v>85608392</v>
@@ -14384,7 +14384,7 @@
         <v>2.37</v>
       </c>
       <c r="M61" t="n">
-        <v>1.192686088916857</v>
+        <v>1.221288438700584</v>
       </c>
       <c r="N61" t="n">
         <v>1.1</v>
@@ -14462,7 +14462,7 @@
         <v>160087693.04</v>
       </c>
       <c r="AM61" t="n">
-        <v>176525309.5761381</v>
+        <v>180758643.6420722</v>
       </c>
       <c r="AN61" t="n">
         <v>0.38</v>
@@ -14503,7 +14503,7 @@
         <v>17.56</v>
       </c>
       <c r="AZ61" t="n">
-        <v>33.1</v>
+        <v>33.89</v>
       </c>
       <c r="BA61" t="n">
         <v>2.52</v>
@@ -14512,19 +14512,19 @@
         <v>11.76</v>
       </c>
       <c r="BC61" t="n">
-        <v>-18.14</v>
+        <v>-20.06</v>
       </c>
       <c r="BD61" t="n">
-        <v>-33.16</v>
+        <v>-34.73</v>
       </c>
       <c r="BE61" t="n">
         <v>26</v>
       </c>
       <c r="BF61" t="n">
-        <v>-90.40000000000001</v>
+        <v>-90.62</v>
       </c>
       <c r="BG61" t="n">
-        <v>-55.25</v>
+        <v>-56.3</v>
       </c>
       <c r="BH61" t="n">
         <v>10.99</v>
@@ -14533,7 +14533,7 @@
         <v>0</v>
       </c>
       <c r="BJ61" t="n">
-        <v>26.27</v>
+        <v>26.9</v>
       </c>
       <c r="BK61" t="n">
         <v>1.87</v>
@@ -14542,7 +14542,7 @@
         <v>1.86</v>
       </c>
       <c r="BM61" t="n">
-        <v>26.54</v>
+        <v>27.08</v>
       </c>
       <c r="BN61" t="n">
         <v>28.25</v>
@@ -14551,19 +14551,19 @@
         <v>19.35</v>
       </c>
       <c r="BP61" t="n">
-        <v>25.91</v>
+        <v>25.72</v>
       </c>
       <c r="BQ61" t="n">
-        <v>14.11</v>
+        <v>14.45</v>
       </c>
       <c r="BR61" t="n">
-        <v>26.05</v>
+        <v>25.92</v>
       </c>
       <c r="BS61" t="n">
         <v>1.19</v>
       </c>
       <c r="BT61" t="n">
-        <v>480755</v>
+        <v>488191</v>
       </c>
     </row>
     <row r="62">
@@ -14823,13 +14823,13 @@
         </is>
       </c>
       <c r="F63" t="n">
-        <v>1.34</v>
+        <v>1.6</v>
       </c>
       <c r="G63" t="n">
-        <v>349083006</v>
+        <v>416815526</v>
       </c>
       <c r="H63" t="n">
-        <v>200</v>
+        <v>149200</v>
       </c>
       <c r="I63" t="n">
         <v>122894462</v>
@@ -14844,7 +14844,7 @@
         <v>-0.22</v>
       </c>
       <c r="M63" t="n">
-        <v>0.429354082561069</v>
+        <v>0.5126615867486239</v>
       </c>
       <c r="N63" t="n">
         <v>0.37</v>
@@ -14922,7 +14922,7 @@
         <v>31952560.12</v>
       </c>
       <c r="AM63" t="n">
-        <v>198342617.0454545</v>
+        <v>236827003.4090909</v>
       </c>
       <c r="AN63" t="n">
         <v>0</v>
@@ -14981,7 +14981,7 @@
         <v>-100</v>
       </c>
       <c r="BF63" t="n">
-        <v>-78.42</v>
+        <v>-81.93000000000001</v>
       </c>
       <c r="BG63" t="n">
         <v>-100</v>
@@ -14993,7 +14993,7 @@
         <v>0</v>
       </c>
       <c r="BJ63" t="n">
-        <v>1.34</v>
+        <v>1.6</v>
       </c>
       <c r="BK63" t="n">
         <v>0.26</v>
@@ -15002,28 +15002,28 @@
         <v>0.26</v>
       </c>
       <c r="BM63" t="n">
-        <v>1.34</v>
+        <v>2.12</v>
       </c>
       <c r="BN63" t="n">
-        <v>1.54</v>
+        <v>2.12</v>
       </c>
       <c r="BO63" t="n">
         <v>1.16</v>
       </c>
       <c r="BP63" t="n">
-        <v>1.34</v>
+        <v>1.21</v>
       </c>
       <c r="BQ63" t="n">
-        <v>5.13</v>
+        <v>6.13</v>
       </c>
       <c r="BR63" t="n">
-        <v>1.34</v>
+        <v>1.3</v>
       </c>
       <c r="BS63" t="n">
         <v>0.19</v>
       </c>
       <c r="BT63" t="n">
-        <v>15137</v>
+        <v>15143</v>
       </c>
     </row>
     <row r="64">
@@ -15053,13 +15053,13 @@
         </is>
       </c>
       <c r="F64" t="n">
-        <v>60.82</v>
+        <v>60.48</v>
       </c>
       <c r="G64" t="n">
-        <v>234645444242</v>
+        <v>230376543536</v>
       </c>
       <c r="H64" t="n">
-        <v>7839100</v>
+        <v>8470300</v>
       </c>
       <c r="I64" t="n">
         <v>0</v>
@@ -15146,13 +15146,13 @@
         <v>41.22</v>
       </c>
       <c r="AK64" t="n">
-        <v>67276292091.72118</v>
+        <v>66052335616.729</v>
       </c>
       <c r="AL64" t="n">
-        <v>18756630235.17186</v>
+        <v>18415391169.94405</v>
       </c>
       <c r="AM64" t="n">
-        <v>20894518632.41318</v>
+        <v>20514384998.75334</v>
       </c>
       <c r="AN64" t="n">
         <v>1.4201</v>
@@ -15193,7 +15193,7 @@
         <v>38.98</v>
       </c>
       <c r="AZ64" t="n">
-        <v>24.33</v>
+        <v>24.19</v>
       </c>
       <c r="BA64" t="n">
         <v>6.69</v>
@@ -15202,19 +15202,19 @@
         <v>10.4</v>
       </c>
       <c r="BC64" t="n">
-        <v>-21.51</v>
+        <v>-21.06</v>
       </c>
       <c r="BD64" t="n">
-        <v>-35.91</v>
+        <v>-35.55</v>
       </c>
       <c r="BE64" t="n">
         <v>-60</v>
       </c>
       <c r="BF64" t="n">
-        <v>-88.98999999999999</v>
+        <v>-88.93000000000001</v>
       </c>
       <c r="BG64" t="n">
-        <v>-82.90000000000001</v>
+        <v>-82.81</v>
       </c>
       <c r="BH64" t="n">
         <v>21.37</v>
@@ -15223,7 +15223,7 @@
         <v>0</v>
       </c>
       <c r="BJ64" t="n">
-        <v>60.82</v>
+        <v>60.48</v>
       </c>
       <c r="BK64" t="n">
         <v>4.74</v>
@@ -15232,7 +15232,7 @@
         <v>1.57</v>
       </c>
       <c r="BM64" t="n">
-        <v>61.07</v>
+        <v>61</v>
       </c>
       <c r="BN64" t="n">
         <v>64.72</v>
@@ -15241,19 +15241,19 @@
         <v>44.12</v>
       </c>
       <c r="BP64" t="n">
-        <v>60.33</v>
+        <v>59.09</v>
       </c>
       <c r="BQ64" t="n">
-        <v>38.74</v>
+        <v>38.52</v>
       </c>
       <c r="BR64" t="n">
-        <v>61.02</v>
+        <v>59.12</v>
       </c>
       <c r="BS64" t="n">
         <v>3.49</v>
       </c>
       <c r="BT64" t="n">
-        <v>12253994</v>
+        <v>12354237</v>
       </c>
     </row>
     <row r="65">
@@ -15283,13 +15283,13 @@
         </is>
       </c>
       <c r="F65" t="n">
-        <v>23.69</v>
+        <v>23.56</v>
       </c>
       <c r="G65" t="n">
-        <v>234645444242</v>
+        <v>230376543536</v>
       </c>
       <c r="H65" t="n">
-        <v>7900</v>
+        <v>8200</v>
       </c>
       <c r="I65" t="n">
         <v>7298813414</v>
@@ -15304,7 +15304,7 @@
         <v>3.29</v>
       </c>
       <c r="M65" t="n">
-        <v>5.672774857493353</v>
+        <v>5.569570157856582</v>
       </c>
       <c r="N65" t="n">
         <v>0.29</v>
@@ -15382,7 +15382,7 @@
         <v>11532125194.12</v>
       </c>
       <c r="AM65" t="n">
-        <v>17576437770.93633</v>
+        <v>17256669927.79026</v>
       </c>
       <c r="AN65" t="n">
         <v>0.4734</v>
@@ -15423,7 +15423,7 @@
         <v>12.99</v>
       </c>
       <c r="AZ65" t="n">
-        <v>7.98</v>
+        <v>7.93</v>
       </c>
       <c r="BA65" t="n">
         <v>2.23</v>
@@ -15432,19 +15432,19 @@
         <v>3.47</v>
       </c>
       <c r="BC65" t="n">
-        <v>-32.84</v>
+        <v>-32.47</v>
       </c>
       <c r="BD65" t="n">
-        <v>-45.17</v>
+        <v>-44.86</v>
       </c>
       <c r="BE65" t="n">
         <v>-66.33</v>
       </c>
       <c r="BF65" t="n">
-        <v>-90.58</v>
+        <v>-90.53</v>
       </c>
       <c r="BG65" t="n">
-        <v>-85.37</v>
+        <v>-85.29000000000001</v>
       </c>
       <c r="BH65" t="n">
         <v>7.12</v>
@@ -15453,7 +15453,7 @@
         <v>0</v>
       </c>
       <c r="BJ65" t="n">
-        <v>23.69</v>
+        <v>23.56</v>
       </c>
       <c r="BK65" t="n">
         <v>1.58</v>
@@ -15462,7 +15462,7 @@
         <v>1.57</v>
       </c>
       <c r="BM65" t="n">
-        <v>23.9</v>
+        <v>23.69</v>
       </c>
       <c r="BN65" t="n">
         <v>46.43</v>
@@ -15471,19 +15471,19 @@
         <v>20.44</v>
       </c>
       <c r="BP65" t="n">
-        <v>23.44</v>
+        <v>23.41</v>
       </c>
       <c r="BQ65" t="n">
-        <v>15.09</v>
+        <v>15.01</v>
       </c>
       <c r="BR65" t="n">
-        <v>23.89</v>
+        <v>23.69</v>
       </c>
       <c r="BS65" t="n">
         <v>4.14</v>
       </c>
       <c r="BT65" t="n">
-        <v>11943</v>
+        <v>12007</v>
       </c>
     </row>
     <row r="66">
@@ -15513,13 +15513,13 @@
         </is>
       </c>
       <c r="F66" t="n">
-        <v>19.76</v>
+        <v>20.17</v>
       </c>
       <c r="G66" t="n">
-        <v>234645444242</v>
+        <v>230376543536</v>
       </c>
       <c r="H66" t="n">
-        <v>2000</v>
+        <v>200</v>
       </c>
       <c r="I66" t="n">
         <v>2972355254</v>
@@ -15534,7 +15534,7 @@
         <v>2.75</v>
       </c>
       <c r="M66" t="n">
-        <v>13.92987098993464</v>
+        <v>13.67644507623102</v>
       </c>
       <c r="N66" t="n">
         <v>0.25</v>
@@ -15612,7 +15612,7 @@
         <v>4696321301.320001</v>
       </c>
       <c r="AM66" t="n">
-        <v>21044434461.16592</v>
+        <v>20661573411.30045</v>
       </c>
       <c r="AN66" t="n">
         <v>0.4734</v>
@@ -15653,7 +15653,7 @@
         <v>12.99</v>
       </c>
       <c r="AZ66" t="n">
-        <v>7.94</v>
+        <v>8.1</v>
       </c>
       <c r="BA66" t="n">
         <v>2.23</v>
@@ -15662,19 +15662,19 @@
         <v>3.47</v>
       </c>
       <c r="BC66" t="n">
-        <v>-19.49</v>
+        <v>-21.12</v>
       </c>
       <c r="BD66" t="n">
-        <v>-34.26</v>
+        <v>-35.6</v>
       </c>
       <c r="BE66" t="n">
         <v>-59.83</v>
       </c>
       <c r="BF66" t="n">
-        <v>-88.70999999999999</v>
+        <v>-88.94</v>
       </c>
       <c r="BG66" t="n">
-        <v>-82.45999999999999</v>
+        <v>-82.81999999999999</v>
       </c>
       <c r="BH66" t="n">
         <v>7.12</v>
@@ -15683,7 +15683,7 @@
         <v>0</v>
       </c>
       <c r="BJ66" t="n">
-        <v>19.76</v>
+        <v>20.17</v>
       </c>
       <c r="BK66" t="n">
         <v>1.58</v>
@@ -15692,28 +15692,28 @@
         <v>1.57</v>
       </c>
       <c r="BM66" t="n">
-        <v>20.2</v>
+        <v>21.33</v>
       </c>
       <c r="BN66" t="n">
-        <v>21.16</v>
+        <v>21.33</v>
       </c>
       <c r="BO66" t="n">
         <v>9.48</v>
       </c>
       <c r="BP66" t="n">
-        <v>19.55</v>
+        <v>20.17</v>
       </c>
       <c r="BQ66" t="n">
-        <v>12.59</v>
+        <v>12.85</v>
       </c>
       <c r="BR66" t="n">
-        <v>19.57</v>
+        <v>21.33</v>
       </c>
       <c r="BS66" t="n">
         <v>3.46</v>
       </c>
       <c r="BT66" t="n">
-        <v>7070</v>
+        <v>7113</v>
       </c>
     </row>
     <row r="67">
@@ -15973,13 +15973,13 @@
         </is>
       </c>
       <c r="F68" t="n">
-        <v>19.23</v>
+        <v>18.78</v>
       </c>
       <c r="G68" t="n">
-        <v>8419842135</v>
+        <v>8068099400</v>
       </c>
       <c r="H68" t="n">
-        <v>18400</v>
+        <v>64300</v>
       </c>
       <c r="I68" t="n">
         <v>137989898</v>
@@ -16072,7 +16072,7 @@
         <v>205604948.02</v>
       </c>
       <c r="AM68" t="n">
-        <v>583900286.7545077</v>
+        <v>559507586.6851594</v>
       </c>
       <c r="AN68" t="n">
         <v>0.1911</v>
@@ -16113,7 +16113,7 @@
         <v>21.39</v>
       </c>
       <c r="AZ68" t="n">
-        <v>35.58</v>
+        <v>34.74</v>
       </c>
       <c r="BA68" t="n">
         <v>1.24</v>
@@ -16122,19 +16122,19 @@
         <v>63.25</v>
       </c>
       <c r="BC68" t="n">
-        <v>36.26</v>
+        <v>39.53</v>
       </c>
       <c r="BD68" t="n">
-        <v>11.26</v>
+        <v>13.92</v>
       </c>
       <c r="BE68" t="n">
         <v>85</v>
       </c>
       <c r="BF68" t="n">
-        <v>-93.55</v>
+        <v>-93.40000000000001</v>
       </c>
       <c r="BG68" t="n">
-        <v>228.91</v>
+        <v>236.79</v>
       </c>
       <c r="BH68" t="n">
         <v>20.48</v>
@@ -16143,7 +16143,7 @@
         <v>0</v>
       </c>
       <c r="BJ68" t="n">
-        <v>19.23</v>
+        <v>18.78</v>
       </c>
       <c r="BK68" t="n">
         <v>1.49</v>
@@ -16152,7 +16152,7 @@
         <v>1.49</v>
       </c>
       <c r="BM68" t="n">
-        <v>19.33</v>
+        <v>19.43</v>
       </c>
       <c r="BN68" t="n">
         <v>22.11</v>
@@ -16161,13 +16161,13 @@
         <v>15.07</v>
       </c>
       <c r="BP68" t="n">
-        <v>19.1</v>
+        <v>18.78</v>
       </c>
       <c r="BQ68" t="n">
-        <v>12.93</v>
+        <v>12.63</v>
       </c>
       <c r="BR68" t="n">
-        <v>19.33</v>
+        <v>19.43</v>
       </c>
       <c r="BS68" t="n">
         <v>0</v>
@@ -16203,13 +16203,13 @@
         </is>
       </c>
       <c r="F69" t="n">
-        <v>22.54</v>
+        <v>21.64</v>
       </c>
       <c r="G69" t="n">
-        <v>8419842135</v>
+        <v>8068099400</v>
       </c>
       <c r="H69" t="n">
-        <v>1582700</v>
+        <v>1983400</v>
       </c>
       <c r="I69" t="n">
         <v>255106712</v>
@@ -16302,7 +16302,7 @@
         <v>380109000.88</v>
       </c>
       <c r="AM69" t="n">
-        <v>501181079.4642857</v>
+        <v>480244011.9047619</v>
       </c>
       <c r="AN69" t="n">
         <v>0.8856000000000001</v>
@@ -16343,7 +16343,7 @@
         <v>21.39</v>
       </c>
       <c r="AZ69" t="n">
-        <v>39.41</v>
+        <v>37.83</v>
       </c>
       <c r="BA69" t="n">
         <v>1.24</v>
@@ -16352,19 +16352,19 @@
         <v>69.59</v>
       </c>
       <c r="BC69" t="n">
-        <v>16.25</v>
+        <v>21.09</v>
       </c>
       <c r="BD69" t="n">
-        <v>-5.08</v>
+        <v>-1.13</v>
       </c>
       <c r="BE69" t="n">
         <v>74.83</v>
       </c>
       <c r="BF69" t="n">
-        <v>-94.5</v>
+        <v>-94.27</v>
       </c>
       <c r="BG69" t="n">
-        <v>208.73</v>
+        <v>221.57</v>
       </c>
       <c r="BH69" t="n">
         <v>20.48</v>
@@ -16373,7 +16373,7 @@
         <v>0</v>
       </c>
       <c r="BJ69" t="n">
-        <v>22.54</v>
+        <v>21.64</v>
       </c>
       <c r="BK69" t="n">
         <v>1.49</v>
@@ -16382,28 +16382,28 @@
         <v>1.49</v>
       </c>
       <c r="BM69" t="n">
-        <v>22.61</v>
+        <v>22.15</v>
       </c>
       <c r="BN69" t="n">
         <v>25.63</v>
       </c>
       <c r="BO69" t="n">
-        <v>16.71</v>
+        <v>16.73</v>
       </c>
       <c r="BP69" t="n">
-        <v>22.26</v>
+        <v>21.64</v>
       </c>
       <c r="BQ69" t="n">
-        <v>15.16</v>
+        <v>14.56</v>
       </c>
       <c r="BR69" t="n">
-        <v>22.47</v>
+        <v>22</v>
       </c>
       <c r="BS69" t="n">
         <v>0</v>
       </c>
       <c r="BT69" t="n">
-        <v>1918823</v>
+        <v>1923390</v>
       </c>
     </row>
     <row r="70">
@@ -16433,13 +16433,13 @@
         </is>
       </c>
       <c r="F70" t="n">
-        <v>18.29</v>
+        <v>17.75</v>
       </c>
       <c r="G70" t="n">
-        <v>8496751613</v>
+        <v>8245890300</v>
       </c>
       <c r="H70" t="n">
-        <v>2814000</v>
+        <v>4184800</v>
       </c>
       <c r="I70" t="n">
         <v>464557268</v>
@@ -16454,7 +16454,7 @@
         <v>0.68</v>
       </c>
       <c r="M70" t="n">
-        <v>0.6706332687132415</v>
+        <v>0.6508332380670019</v>
       </c>
       <c r="N70" t="n">
         <v>0.2</v>
@@ -16532,7 +16532,7 @@
         <v>55746872.16</v>
       </c>
       <c r="AM70" t="n">
-        <v>2804208453.135314</v>
+        <v>2721415940.594059</v>
       </c>
       <c r="AN70" t="n">
         <v>0.1236</v>
@@ -16573,7 +16573,7 @@
         <v>6.9</v>
       </c>
       <c r="AZ70" t="n">
-        <v>2.1</v>
+        <v>2.04</v>
       </c>
       <c r="BA70" t="n">
         <v>0.12</v>
@@ -16582,19 +16582,19 @@
         <v>1.07</v>
       </c>
       <c r="BC70" t="n">
-        <v>-53.8</v>
+        <v>-52.4</v>
       </c>
       <c r="BD70" t="n">
-        <v>-62.28</v>
+        <v>-61.13</v>
       </c>
       <c r="BE70" t="n">
         <v>-88.5</v>
       </c>
       <c r="BF70" t="n">
-        <v>-99.34</v>
+        <v>-99.31999999999999</v>
       </c>
       <c r="BG70" t="n">
-        <v>-94.15000000000001</v>
+        <v>-93.97</v>
       </c>
       <c r="BH70" t="n">
         <v>26.44</v>
@@ -16603,7 +16603,7 @@
         <v>0</v>
       </c>
       <c r="BJ70" t="n">
-        <v>18.29</v>
+        <v>17.75</v>
       </c>
       <c r="BK70" t="n">
         <v>0.12</v>
@@ -16612,7 +16612,7 @@
         <v>0.1</v>
       </c>
       <c r="BM70" t="n">
-        <v>18.64</v>
+        <v>18.6</v>
       </c>
       <c r="BN70" t="n">
         <v>22.15</v>
@@ -16621,19 +16621,19 @@
         <v>13.21</v>
       </c>
       <c r="BP70" t="n">
-        <v>18.29</v>
+        <v>17.72</v>
       </c>
       <c r="BQ70" t="n">
-        <v>183.43</v>
+        <v>178.02</v>
       </c>
       <c r="BR70" t="n">
-        <v>18.5</v>
+        <v>18.45</v>
       </c>
       <c r="BS70" t="n">
         <v>0.67</v>
       </c>
       <c r="BT70" t="n">
-        <v>6063490</v>
+        <v>5779190</v>
       </c>
     </row>
     <row r="71">

</xml_diff>

<commit_message>
📊 Dados atualizados - 2026-09-16 05:32
</commit_message>
<xml_diff>
--- a/data/ativos.xlsx
+++ b/data/ativos.xlsx
@@ -1047,13 +1047,13 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>25.05</v>
+        <v>24.69</v>
       </c>
       <c r="G3" t="n">
-        <v>3350858237</v>
+        <v>3302704832</v>
       </c>
       <c r="H3" t="n">
-        <v>454800</v>
+        <v>410100</v>
       </c>
       <c r="I3" t="n">
         <v>129510368</v>
@@ -1068,7 +1068,7 @@
         <v>0.88</v>
       </c>
       <c r="M3" t="n">
-        <v>0.8337681577475935</v>
+        <v>0.8217865181387306</v>
       </c>
       <c r="N3" t="n">
         <v>0.09</v>
@@ -1146,7 +1146,7 @@
         <v>506385538.88</v>
       </c>
       <c r="AM3" t="n">
-        <v>654464499.4140625</v>
+        <v>645059537.5</v>
       </c>
       <c r="AN3" t="n">
         <v>2.7</v>
@@ -1187,7 +1187,7 @@
         <v>40.42</v>
       </c>
       <c r="AZ3" t="n">
-        <v>45.84</v>
+        <v>45.18</v>
       </c>
       <c r="BA3" t="n">
         <v>4.87</v>
@@ -1196,19 +1196,19 @@
         <v>21.14</v>
       </c>
       <c r="BC3" t="n">
-        <v>97.59999999999999</v>
+        <v>100.48</v>
       </c>
       <c r="BD3" t="n">
-        <v>61.34</v>
+        <v>63.69</v>
       </c>
       <c r="BE3" t="n">
         <v>83</v>
       </c>
       <c r="BF3" t="n">
-        <v>-80.56</v>
+        <v>-80.28</v>
       </c>
       <c r="BG3" t="n">
-        <v>-15.63</v>
+        <v>-14.4</v>
       </c>
       <c r="BH3" t="n">
         <v>27.85</v>
@@ -1217,7 +1217,7 @@
         <v>0</v>
       </c>
       <c r="BJ3" t="n">
-        <v>25.05</v>
+        <v>24.69</v>
       </c>
       <c r="BK3" t="n">
         <v>3.91</v>
@@ -1226,7 +1226,7 @@
         <v>4.39</v>
       </c>
       <c r="BM3" t="n">
-        <v>25.09</v>
+        <v>25.05</v>
       </c>
       <c r="BN3" t="n">
         <v>27.17</v>
@@ -1235,19 +1235,19 @@
         <v>18.72</v>
       </c>
       <c r="BP3" t="n">
-        <v>24.59</v>
+        <v>24.53</v>
       </c>
       <c r="BQ3" t="n">
-        <v>5.7</v>
+        <v>5.62</v>
       </c>
       <c r="BR3" t="n">
-        <v>24.87</v>
+        <v>25.02</v>
       </c>
       <c r="BS3" t="n">
         <v>0.79</v>
       </c>
       <c r="BT3" t="n">
-        <v>533320</v>
+        <v>531937</v>
       </c>
     </row>
     <row r="4">
@@ -1277,13 +1277,13 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>15.87</v>
+        <v>15.73</v>
       </c>
       <c r="G4" t="n">
-        <v>245741552427</v>
+        <v>243573694711</v>
       </c>
       <c r="H4" t="n">
-        <v>29303600</v>
+        <v>20798700</v>
       </c>
       <c r="I4" t="n">
         <v>15484664889</v>
@@ -1298,7 +1298,7 @@
         <v>2.76</v>
       </c>
       <c r="M4" t="n">
-        <v>2.782539101388105</v>
+        <v>2.75799238227837</v>
       </c>
       <c r="N4" t="n">
         <v>1.76</v>
@@ -1376,7 +1376,7 @@
         <v>16258898133.45</v>
       </c>
       <c r="AM4" t="n">
-        <v>24330846774.9505</v>
+        <v>24116207397.12872</v>
       </c>
       <c r="AN4" t="n">
         <v>0.269</v>
@@ -1417,7 +1417,7 @@
         <v>9.470000000000001</v>
       </c>
       <c r="AZ4" t="n">
-        <v>19.81</v>
+        <v>19.64</v>
       </c>
       <c r="BA4" t="n">
         <v>1.13</v>
@@ -1426,19 +1426,19 @@
         <v>11.39</v>
       </c>
       <c r="BC4" t="n">
-        <v>-26.88</v>
+        <v>-26.23</v>
       </c>
       <c r="BD4" t="n">
-        <v>-40.3</v>
+        <v>-39.76</v>
       </c>
       <c r="BE4" t="n">
         <v>24.83</v>
       </c>
       <c r="BF4" t="n">
-        <v>-92.90000000000001</v>
+        <v>-92.83</v>
       </c>
       <c r="BG4" t="n">
-        <v>-28.25</v>
+        <v>-27.61</v>
       </c>
       <c r="BH4" t="n">
         <v>5.7</v>
@@ -1447,7 +1447,7 @@
         <v>0</v>
       </c>
       <c r="BJ4" t="n">
-        <v>15.87</v>
+        <v>15.73</v>
       </c>
       <c r="BK4" t="n">
         <v>1.05</v>
@@ -1456,7 +1456,7 @@
         <v>1.04</v>
       </c>
       <c r="BM4" t="n">
-        <v>15.91</v>
+        <v>15.95</v>
       </c>
       <c r="BN4" t="n">
         <v>17</v>
@@ -1465,19 +1465,19 @@
         <v>11.09</v>
       </c>
       <c r="BP4" t="n">
-        <v>15.37</v>
+        <v>15.71</v>
       </c>
       <c r="BQ4" t="n">
-        <v>15.31</v>
+        <v>15.17</v>
       </c>
       <c r="BR4" t="n">
-        <v>15.4</v>
+        <v>15.95</v>
       </c>
       <c r="BS4" t="n">
         <v>2.76</v>
       </c>
       <c r="BT4" t="n">
-        <v>28956417</v>
+        <v>28658427</v>
       </c>
     </row>
     <row r="5">
@@ -1737,13 +1737,13 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>7.49</v>
+        <v>7.32</v>
       </c>
       <c r="G6" t="n">
-        <v>472504313</v>
+        <v>461779941</v>
       </c>
       <c r="H6" t="n">
-        <v>900</v>
+        <v>100</v>
       </c>
       <c r="I6" t="n">
         <v>63084700</v>
@@ -1758,7 +1758,7 @@
         <v>1.91</v>
       </c>
       <c r="M6" t="n">
-        <v>7.355967019928846</v>
+        <v>7.189009545529139</v>
       </c>
       <c r="N6" t="n">
         <v>1.26</v>
@@ -1836,7 +1836,7 @@
         <v>35958279</v>
       </c>
       <c r="AM6" t="n">
-        <v>45172496.4627151</v>
+        <v>44147221.89292543</v>
       </c>
       <c r="AN6" t="n">
         <v>0.5199</v>
@@ -1877,7 +1877,7 @@
         <v>5.74</v>
       </c>
       <c r="AZ6" t="n">
-        <v>8.789999999999999</v>
+        <v>8.59</v>
       </c>
       <c r="BA6" t="n">
         <v>0.65</v>
@@ -1886,19 +1886,19 @@
         <v>7.95</v>
       </c>
       <c r="BC6" t="n">
-        <v>-6.06</v>
+        <v>-3.88</v>
       </c>
       <c r="BD6" t="n">
-        <v>-23.3</v>
+        <v>-21.52</v>
       </c>
       <c r="BE6" t="n">
         <v>17.33</v>
       </c>
       <c r="BF6" t="n">
-        <v>-91.34</v>
+        <v>-91.14</v>
       </c>
       <c r="BG6" t="n">
-        <v>6.19</v>
+        <v>8.66</v>
       </c>
       <c r="BH6" t="n">
         <v>3.86</v>
@@ -1907,7 +1907,7 @@
         <v>0</v>
       </c>
       <c r="BJ6" t="n">
-        <v>7.49</v>
+        <v>7.32</v>
       </c>
       <c r="BK6" t="n">
         <v>0.57</v>
@@ -1916,7 +1916,7 @@
         <v>0.5600000000000001</v>
       </c>
       <c r="BM6" t="n">
-        <v>7.49</v>
+        <v>7.32</v>
       </c>
       <c r="BN6" t="n">
         <v>8.16</v>
@@ -1925,19 +1925,19 @@
         <v>6.22</v>
       </c>
       <c r="BP6" t="n">
-        <v>7.24</v>
+        <v>7.32</v>
       </c>
       <c r="BQ6" t="n">
-        <v>13.32</v>
+        <v>13.02</v>
       </c>
       <c r="BR6" t="n">
-        <v>7.37</v>
+        <v>7.32</v>
       </c>
       <c r="BS6" t="n">
         <v>7.32</v>
       </c>
       <c r="BT6" t="n">
-        <v>253</v>
+        <v>283</v>
       </c>
     </row>
     <row r="7">
@@ -3117,13 +3117,13 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>5.06</v>
+        <v>5.05</v>
       </c>
       <c r="G12" t="n">
-        <v>485565336</v>
+        <v>484605795</v>
       </c>
       <c r="H12" t="n">
-        <v>255400</v>
+        <v>260900</v>
       </c>
       <c r="I12" t="n">
         <v>95961536</v>
@@ -3138,7 +3138,7 @@
         <v>0.32</v>
       </c>
       <c r="M12" t="n">
-        <v>0.08781375007427578</v>
+        <v>0.08764021854862333</v>
       </c>
       <c r="N12" t="n">
         <v>0.14</v>
@@ -3216,7 +3216,7 @@
         <v>362734606.08</v>
       </c>
       <c r="AM12" t="n">
-        <v>522113264.516129</v>
+        <v>521081500</v>
       </c>
       <c r="AN12" t="n">
         <v>0.4208</v>
@@ -3257,7 +3257,7 @@
         <v>30.49</v>
       </c>
       <c r="AZ12" t="n">
-        <v>6.84</v>
+        <v>6.83</v>
       </c>
       <c r="BA12" t="n">
         <v>4.41</v>
@@ -3266,19 +3266,19 @@
         <v>18.12</v>
       </c>
       <c r="BC12" t="n">
-        <v>638.09</v>
+        <v>639.55</v>
       </c>
       <c r="BD12" t="n">
-        <v>502.65</v>
+        <v>503.84</v>
       </c>
       <c r="BE12" t="n">
         <v>35.17</v>
       </c>
       <c r="BF12" t="n">
-        <v>-12.81</v>
+        <v>-12.64</v>
       </c>
       <c r="BG12" t="n">
-        <v>258.08</v>
+        <v>258.79</v>
       </c>
       <c r="BH12" t="n">
         <v>16.4</v>
@@ -3287,7 +3287,7 @@
         <v>0</v>
       </c>
       <c r="BJ12" t="n">
-        <v>5.06</v>
+        <v>5.05</v>
       </c>
       <c r="BK12" t="n">
         <v>3.78</v>
@@ -3296,7 +3296,7 @@
         <v>3.43</v>
       </c>
       <c r="BM12" t="n">
-        <v>5.08</v>
+        <v>5.1</v>
       </c>
       <c r="BN12" t="n">
         <v>8.23</v>
@@ -3305,19 +3305,19 @@
         <v>4.42</v>
       </c>
       <c r="BP12" t="n">
-        <v>4.99</v>
+        <v>5.04</v>
       </c>
       <c r="BQ12" t="n">
         <v>1.47</v>
       </c>
       <c r="BR12" t="n">
-        <v>5.04</v>
+        <v>5.05</v>
       </c>
       <c r="BS12" t="n">
         <v>0.09</v>
       </c>
       <c r="BT12" t="n">
-        <v>491947</v>
+        <v>497557</v>
       </c>
     </row>
     <row r="13">
@@ -3347,13 +3347,13 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>28.44</v>
+        <v>28.53</v>
       </c>
       <c r="G13" t="n">
-        <v>14339192309</v>
+        <v>14384566723</v>
       </c>
       <c r="H13" t="n">
-        <v>4292700</v>
+        <v>2870100</v>
       </c>
       <c r="I13" t="n">
         <v>504190947</v>
@@ -3368,7 +3368,7 @@
         <v>1.13</v>
       </c>
       <c r="M13" t="n">
-        <v>4.959321695435232</v>
+        <v>4.975014791037738</v>
       </c>
       <c r="N13" t="n">
         <v>0.57</v>
@@ -3446,7 +3446,7 @@
         <v>932753251.95</v>
       </c>
       <c r="AM13" t="n">
-        <v>1492111582.622269</v>
+        <v>1496833165.764828</v>
       </c>
       <c r="AN13" t="n">
         <v>2.6301</v>
@@ -3487,7 +3487,7 @@
         <v>26.6</v>
       </c>
       <c r="AZ13" t="n">
-        <v>51.48</v>
+        <v>51.64</v>
       </c>
       <c r="BA13" t="n">
         <v>2.6</v>
@@ -3496,19 +3496,19 @@
         <v>8.69</v>
       </c>
       <c r="BC13" t="n">
-        <v>14.53</v>
+        <v>14.17</v>
       </c>
       <c r="BD13" t="n">
-        <v>-6.48</v>
+        <v>-6.78</v>
       </c>
       <c r="BE13" t="n">
         <v>81</v>
       </c>
       <c r="BF13" t="n">
-        <v>-90.84</v>
+        <v>-90.87</v>
       </c>
       <c r="BG13" t="n">
-        <v>-69.43000000000001</v>
+        <v>-69.53</v>
       </c>
       <c r="BH13" t="n">
         <v>25.49</v>
@@ -3517,7 +3517,7 @@
         <v>0</v>
       </c>
       <c r="BJ13" t="n">
-        <v>28.44</v>
+        <v>28.53</v>
       </c>
       <c r="BK13" t="n">
         <v>1.85</v>
@@ -3526,7 +3526,7 @@
         <v>1.96</v>
       </c>
       <c r="BM13" t="n">
-        <v>28.48</v>
+        <v>28.67</v>
       </c>
       <c r="BN13" t="n">
         <v>32.43</v>
@@ -3535,19 +3535,19 @@
         <v>21.06</v>
       </c>
       <c r="BP13" t="n">
-        <v>27.8</v>
+        <v>28.25</v>
       </c>
       <c r="BQ13" t="n">
-        <v>14.53</v>
+        <v>14.58</v>
       </c>
       <c r="BR13" t="n">
-        <v>27.91</v>
+        <v>28.51</v>
       </c>
       <c r="BS13" t="n">
         <v>5.01</v>
       </c>
       <c r="BT13" t="n">
-        <v>4560105</v>
+        <v>4629999</v>
       </c>
     </row>
     <row r="14">
@@ -3577,13 +3577,13 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>9.9</v>
+        <v>9.77</v>
       </c>
       <c r="G14" t="n">
-        <v>7789191837</v>
+        <v>7816145214</v>
       </c>
       <c r="H14" t="n">
-        <v>11700</v>
+        <v>3600</v>
       </c>
       <c r="I14" t="n">
         <v>339510689</v>
@@ -3598,7 +3598,7 @@
         <v>1.92</v>
       </c>
       <c r="M14" t="n">
-        <v>3.234210924510375</v>
+        <v>3.245402445809384</v>
       </c>
       <c r="N14" t="n">
         <v>1.11</v>
@@ -3676,7 +3676,7 @@
         <v>349696009.67</v>
       </c>
       <c r="AM14" t="n">
-        <v>864505198.3351831</v>
+        <v>867496694.1176471</v>
       </c>
       <c r="AN14" t="n">
         <v>0.1489</v>
@@ -3717,7 +3717,7 @@
         <v>9.050000000000001</v>
       </c>
       <c r="AZ14" t="n">
-        <v>7.95</v>
+        <v>7.85</v>
       </c>
       <c r="BA14" t="n">
         <v>1.42</v>
@@ -3726,19 +3726,19 @@
         <v>5.94</v>
       </c>
       <c r="BC14" t="n">
-        <v>11.95</v>
+        <v>13.44</v>
       </c>
       <c r="BD14" t="n">
-        <v>-8.6</v>
+        <v>-7.38</v>
       </c>
       <c r="BE14" t="n">
         <v>-19.67</v>
       </c>
       <c r="BF14" t="n">
-        <v>-85.64</v>
+        <v>-85.45</v>
       </c>
       <c r="BG14" t="n">
-        <v>-39.98</v>
+        <v>-39.18</v>
       </c>
       <c r="BH14" t="n">
         <v>5.3</v>
@@ -3747,7 +3747,7 @@
         <v>0</v>
       </c>
       <c r="BJ14" t="n">
-        <v>9.9</v>
+        <v>9.77</v>
       </c>
       <c r="BK14" t="n">
         <v>1.03</v>
@@ -3756,7 +3756,7 @@
         <v>1.01</v>
       </c>
       <c r="BM14" t="n">
-        <v>9.9</v>
+        <v>9.859999999999999</v>
       </c>
       <c r="BN14" t="n">
         <v>13.49</v>
@@ -3765,19 +3765,19 @@
         <v>7.65</v>
       </c>
       <c r="BP14" t="n">
-        <v>9.56</v>
+        <v>9.77</v>
       </c>
       <c r="BQ14" t="n">
-        <v>9.77</v>
+        <v>9.65</v>
       </c>
       <c r="BR14" t="n">
-        <v>9.75</v>
+        <v>9.789999999999999</v>
       </c>
       <c r="BS14" t="n">
         <v>1.44</v>
       </c>
       <c r="BT14" t="n">
-        <v>12490</v>
+        <v>12717</v>
       </c>
     </row>
     <row r="15">
@@ -3807,13 +3807,13 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>13.02</v>
+        <v>12.99</v>
       </c>
       <c r="G15" t="n">
-        <v>7789191837</v>
+        <v>7816145214</v>
       </c>
       <c r="H15" t="n">
-        <v>967500</v>
+        <v>667800</v>
       </c>
       <c r="I15" t="n">
         <v>343551533</v>
@@ -3828,7 +3828,7 @@
         <v>2.56</v>
       </c>
       <c r="M15" t="n">
-        <v>3.196170221577339</v>
+        <v>3.207230108500284</v>
       </c>
       <c r="N15" t="n">
         <v>1.47</v>
@@ -3906,7 +3906,7 @@
         <v>353858078.99</v>
       </c>
       <c r="AM15" t="n">
-        <v>649640686.9891577</v>
+        <v>651888675.0625521</v>
       </c>
       <c r="AN15" t="n">
         <v>0.1638</v>
@@ -3947,7 +3947,7 @@
         <v>9.050000000000001</v>
       </c>
       <c r="AZ15" t="n">
-        <v>8.66</v>
+        <v>8.640000000000001</v>
       </c>
       <c r="BA15" t="n">
         <v>1.42</v>
@@ -3956,19 +3956,19 @@
         <v>6.19</v>
       </c>
       <c r="BC15" t="n">
-        <v>-14.88</v>
+        <v>-14.68</v>
       </c>
       <c r="BD15" t="n">
-        <v>-30.5</v>
+        <v>-30.34</v>
       </c>
       <c r="BE15" t="n">
         <v>-33.5</v>
       </c>
       <c r="BF15" t="n">
-        <v>-89.08</v>
+        <v>-89.06</v>
       </c>
       <c r="BG15" t="n">
-        <v>-52.47</v>
+        <v>-52.36</v>
       </c>
       <c r="BH15" t="n">
         <v>5.3</v>
@@ -3977,7 +3977,7 @@
         <v>0</v>
       </c>
       <c r="BJ15" t="n">
-        <v>13.02</v>
+        <v>12.99</v>
       </c>
       <c r="BK15" t="n">
         <v>1.03</v>
@@ -3986,7 +3986,7 @@
         <v>1.01</v>
       </c>
       <c r="BM15" t="n">
-        <v>13.21</v>
+        <v>13.23</v>
       </c>
       <c r="BN15" t="n">
         <v>16.22</v>
@@ -3995,19 +3995,19 @@
         <v>7.84</v>
       </c>
       <c r="BP15" t="n">
-        <v>12.86</v>
+        <v>12.98</v>
       </c>
       <c r="BQ15" t="n">
-        <v>12.85</v>
+        <v>12.82</v>
       </c>
       <c r="BR15" t="n">
-        <v>13.16</v>
+        <v>13.04</v>
       </c>
       <c r="BS15" t="n">
         <v>1.92</v>
       </c>
       <c r="BT15" t="n">
-        <v>2373813</v>
+        <v>2361563</v>
       </c>
     </row>
     <row r="16">
@@ -4037,13 +4037,13 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>4.32</v>
+        <v>4.25</v>
       </c>
       <c r="G16" t="n">
-        <v>947400661</v>
+        <v>932049225</v>
       </c>
       <c r="H16" t="n">
-        <v>63200</v>
+        <v>222400</v>
       </c>
       <c r="I16" t="n">
         <v>219305733</v>
@@ -4058,7 +4058,7 @@
         <v>2.69</v>
       </c>
       <c r="M16" t="n">
-        <v>0.448199950061269</v>
+        <v>0.4409374336499903</v>
       </c>
       <c r="N16" t="n">
         <v>0.39</v>
@@ -4136,7 +4136,7 @@
         <v>17544458.64</v>
       </c>
       <c r="AM16" t="n">
-        <v>266123781.1797753</v>
+        <v>261811580.0561798</v>
       </c>
       <c r="AN16" t="n">
         <v>0.0077</v>
@@ -4186,16 +4186,16 @@
         <v>0</v>
       </c>
       <c r="BC16" t="n">
-        <v>-59.75</v>
+        <v>-59.08</v>
       </c>
       <c r="BD16" t="n">
-        <v>-67.13</v>
+        <v>-66.59</v>
       </c>
       <c r="BE16" t="n">
         <v>-97.17</v>
       </c>
       <c r="BF16" t="n">
-        <v>-98.15000000000001</v>
+        <v>-98.12</v>
       </c>
       <c r="BG16" t="n">
         <v>-100</v>
@@ -4207,7 +4207,7 @@
         <v>0</v>
       </c>
       <c r="BJ16" t="n">
-        <v>4.32</v>
+        <v>4.25</v>
       </c>
       <c r="BK16" t="n">
         <v>0.08</v>
@@ -4216,28 +4216,28 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="BM16" t="n">
-        <v>4.36</v>
+        <v>4.35</v>
       </c>
       <c r="BN16" t="n">
         <v>5.54</v>
       </c>
       <c r="BO16" t="n">
-        <v>3</v>
+        <v>3.08</v>
       </c>
       <c r="BP16" t="n">
-        <v>4.28</v>
+        <v>4.13</v>
       </c>
       <c r="BQ16" t="n">
-        <v>58.95</v>
+        <v>58</v>
       </c>
       <c r="BR16" t="n">
-        <v>4.29</v>
+        <v>4.32</v>
       </c>
       <c r="BS16" t="n">
         <v>0.49</v>
       </c>
       <c r="BT16" t="n">
-        <v>138763</v>
+        <v>139897</v>
       </c>
     </row>
     <row r="17">
@@ -4267,13 +4267,13 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>33.4</v>
+        <v>33.41</v>
       </c>
       <c r="G17" t="n">
-        <v>11009535622</v>
+        <v>11012834678</v>
       </c>
       <c r="H17" t="n">
-        <v>567600</v>
+        <v>529900</v>
       </c>
       <c r="I17" t="n">
         <v>0</v>
@@ -4360,13 +4360,13 @@
         <v>8.039999999999999</v>
       </c>
       <c r="AK17" t="n">
-        <v>4971791736.813584</v>
+        <v>4973281556.177746</v>
       </c>
       <c r="AL17" t="n">
-        <v>1376191952.75</v>
+        <v>1376604334.75</v>
       </c>
       <c r="AM17" t="n">
-        <v>3408524960.371517</v>
+        <v>3409546339.93808</v>
       </c>
       <c r="AN17" t="n">
         <v>1.08</v>
@@ -4416,19 +4416,19 @@
         <v>16.33</v>
       </c>
       <c r="BC17" t="n">
-        <v>57.6</v>
+        <v>57.55</v>
       </c>
       <c r="BD17" t="n">
-        <v>28.68</v>
+        <v>28.64</v>
       </c>
       <c r="BE17" t="n">
         <v>-46.5</v>
       </c>
       <c r="BF17" t="n">
-        <v>-86.38</v>
+        <v>-86.39</v>
       </c>
       <c r="BG17" t="n">
-        <v>-51.1</v>
+        <v>-51.11</v>
       </c>
       <c r="BH17" t="n">
         <v>29.25</v>
@@ -4437,7 +4437,7 @@
         <v>0</v>
       </c>
       <c r="BJ17" t="n">
-        <v>33.4</v>
+        <v>33.41</v>
       </c>
       <c r="BK17" t="n">
         <v>4.21</v>
@@ -4446,7 +4446,7 @@
         <v>12.62</v>
       </c>
       <c r="BM17" t="n">
-        <v>33.49</v>
+        <v>33.61</v>
       </c>
       <c r="BN17" t="n">
         <v>36.63</v>
@@ -4455,19 +4455,19 @@
         <v>29.28</v>
       </c>
       <c r="BP17" t="n">
-        <v>33.02</v>
+        <v>33.33</v>
       </c>
       <c r="BQ17" t="n">
         <v>2.65</v>
       </c>
       <c r="BR17" t="n">
-        <v>33.3</v>
+        <v>33.44</v>
       </c>
       <c r="BS17" t="n">
         <v>2.21</v>
       </c>
       <c r="BT17" t="n">
-        <v>1072646</v>
+        <v>1076550</v>
       </c>
     </row>
     <row r="18">
@@ -4497,13 +4497,13 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>11.5</v>
+        <v>11.7</v>
       </c>
       <c r="G18" t="n">
-        <v>11009535622</v>
+        <v>11012834678</v>
       </c>
       <c r="H18" t="n">
-        <v>5300</v>
+        <v>1500</v>
       </c>
       <c r="I18" t="n">
         <v>671494278</v>
@@ -4518,7 +4518,7 @@
         <v>1.2</v>
       </c>
       <c r="M18" t="n">
-        <v>3.241639642906554</v>
+        <v>3.242611014550277</v>
       </c>
       <c r="N18" t="n">
         <v>0.33</v>
@@ -4596,7 +4596,7 @@
         <v>940091989.1999999</v>
       </c>
       <c r="AM18" t="n">
-        <v>3276647506.547619</v>
+        <v>3277629368.452381</v>
       </c>
       <c r="AN18" t="n">
         <v>0.36</v>
@@ -4637,7 +4637,7 @@
         <v>14.31</v>
       </c>
       <c r="AZ18" t="n">
-        <v>5.92</v>
+        <v>6.03</v>
       </c>
       <c r="BA18" t="n">
         <v>1.51</v>
@@ -4646,19 +4646,19 @@
         <v>5.44</v>
       </c>
       <c r="BC18" t="n">
-        <v>52.39</v>
+        <v>49.79</v>
       </c>
       <c r="BD18" t="n">
-        <v>24.43</v>
+        <v>22.3</v>
       </c>
       <c r="BE18" t="n">
         <v>-48.5</v>
       </c>
       <c r="BF18" t="n">
-        <v>-86.84999999999999</v>
+        <v>-87.06999999999999</v>
       </c>
       <c r="BG18" t="n">
-        <v>-52.66</v>
+        <v>-53.47</v>
       </c>
       <c r="BH18" t="n">
         <v>9.75</v>
@@ -4667,7 +4667,7 @@
         <v>0</v>
       </c>
       <c r="BJ18" t="n">
-        <v>11.5</v>
+        <v>11.7</v>
       </c>
       <c r="BK18" t="n">
         <v>1.4</v>
@@ -4676,7 +4676,7 @@
         <v>12.62</v>
       </c>
       <c r="BM18" t="n">
-        <v>11.9</v>
+        <v>11.89</v>
       </c>
       <c r="BN18" t="n">
         <v>13.82</v>
@@ -4685,19 +4685,19 @@
         <v>10.19</v>
       </c>
       <c r="BP18" t="n">
-        <v>11.43</v>
+        <v>11.48</v>
       </c>
       <c r="BQ18" t="n">
-        <v>0.91</v>
+        <v>0.93</v>
       </c>
       <c r="BR18" t="n">
-        <v>11.9</v>
+        <v>11.64</v>
       </c>
       <c r="BS18" t="n">
         <v>2.3</v>
       </c>
       <c r="BT18" t="n">
-        <v>9673</v>
+        <v>9782</v>
       </c>
     </row>
     <row r="19">
@@ -4727,13 +4727,13 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>10.8</v>
+        <v>10.92</v>
       </c>
       <c r="G19" t="n">
-        <v>11009535622</v>
+        <v>11012834678</v>
       </c>
       <c r="H19" t="n">
-        <v>9300</v>
+        <v>2100</v>
       </c>
       <c r="I19" t="n">
         <v>317386323</v>
@@ -4748,7 +4748,7 @@
         <v>1.12</v>
       </c>
       <c r="M19" t="n">
-        <v>6.858337344138532</v>
+        <v>6.860392475230528</v>
       </c>
       <c r="N19" t="n">
         <v>0.3</v>
@@ -4826,7 +4826,7 @@
         <v>444340852.2</v>
       </c>
       <c r="AM19" t="n">
-        <v>3495090673.650794</v>
+        <v>3496137993.015873</v>
       </c>
       <c r="AN19" t="n">
         <v>0.36</v>
@@ -4867,7 +4867,7 @@
         <v>14.31</v>
       </c>
       <c r="AZ19" t="n">
-        <v>5.94</v>
+        <v>6.01</v>
       </c>
       <c r="BA19" t="n">
         <v>1.51</v>
@@ -4876,19 +4876,19 @@
         <v>5.25</v>
       </c>
       <c r="BC19" t="n">
-        <v>62.27</v>
+        <v>60.49</v>
       </c>
       <c r="BD19" t="n">
-        <v>32.49</v>
+        <v>31.04</v>
       </c>
       <c r="BE19" t="n">
         <v>-45</v>
       </c>
       <c r="BF19" t="n">
-        <v>-85.98999999999999</v>
+        <v>-86.15000000000001</v>
       </c>
       <c r="BG19" t="n">
-        <v>-51.39</v>
+        <v>-51.92</v>
       </c>
       <c r="BH19" t="n">
         <v>9.75</v>
@@ -4897,7 +4897,7 @@
         <v>0</v>
       </c>
       <c r="BJ19" t="n">
-        <v>10.8</v>
+        <v>10.92</v>
       </c>
       <c r="BK19" t="n">
         <v>1.4</v>
@@ -4906,7 +4906,7 @@
         <v>12.62</v>
       </c>
       <c r="BM19" t="n">
-        <v>11.15</v>
+        <v>10.97</v>
       </c>
       <c r="BN19" t="n">
         <v>11.41</v>
@@ -4915,19 +4915,19 @@
         <v>9.19</v>
       </c>
       <c r="BP19" t="n">
-        <v>10.8</v>
+        <v>10.84</v>
       </c>
       <c r="BQ19" t="n">
-        <v>0.86</v>
+        <v>0.87</v>
       </c>
       <c r="BR19" t="n">
-        <v>11.15</v>
+        <v>10.97</v>
       </c>
       <c r="BS19" t="n">
         <v>2.16</v>
       </c>
       <c r="BT19" t="n">
-        <v>13907</v>
+        <v>13995</v>
       </c>
     </row>
     <row r="20">
@@ -5417,13 +5417,13 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>4.99</v>
+        <v>4.98</v>
       </c>
       <c r="G22" t="n">
-        <v>999223502</v>
+        <v>997221597</v>
       </c>
       <c r="H22" t="n">
-        <v>893100</v>
+        <v>1121600</v>
       </c>
       <c r="I22" t="n">
         <v>200245299</v>
@@ -5438,7 +5438,7 @@
         <v>0.27</v>
       </c>
       <c r="M22" t="n">
-        <v>0.08475074784897729</v>
+        <v>0.08458095305778891</v>
       </c>
       <c r="N22" t="n">
         <v>0.08</v>
@@ -5516,7 +5516,7 @@
         <v>378463615.11</v>
       </c>
       <c r="AM22" t="n">
-        <v>226581292.9705215</v>
+        <v>226127346.2585034</v>
       </c>
       <c r="AN22" t="n">
         <v>0</v>
@@ -5566,19 +5566,19 @@
         <v>172.49</v>
       </c>
       <c r="BC22" t="n">
-        <v>495.29</v>
+        <v>496.49</v>
       </c>
       <c r="BD22" t="n">
-        <v>386.05</v>
+        <v>387.03</v>
       </c>
       <c r="BE22" t="n">
         <v>-100</v>
       </c>
       <c r="BF22" t="n">
-        <v>-62.12</v>
+        <v>-62.05</v>
       </c>
       <c r="BG22" t="n">
-        <v>3356.71</v>
+        <v>3363.65</v>
       </c>
       <c r="BH22" t="n">
         <v>20.75</v>
@@ -5587,7 +5587,7 @@
         <v>0</v>
       </c>
       <c r="BJ22" t="n">
-        <v>4.99</v>
+        <v>4.98</v>
       </c>
       <c r="BK22" t="n">
         <v>1.89</v>
@@ -5596,7 +5596,7 @@
         <v>0.67</v>
       </c>
       <c r="BM22" t="n">
-        <v>5.06</v>
+        <v>5.04</v>
       </c>
       <c r="BN22" t="n">
         <v>8.82</v>
@@ -5605,19 +5605,19 @@
         <v>3.37</v>
       </c>
       <c r="BP22" t="n">
-        <v>4.77</v>
+        <v>4.83</v>
       </c>
       <c r="BQ22" t="n">
-        <v>7.43</v>
+        <v>7.42</v>
       </c>
       <c r="BR22" t="n">
-        <v>4.85</v>
+        <v>5</v>
       </c>
       <c r="BS22" t="n">
         <v>0.09</v>
       </c>
       <c r="BT22" t="n">
-        <v>1562667</v>
+        <v>1564023</v>
       </c>
     </row>
     <row r="23">
@@ -5877,13 +5877,13 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.9</v>
+        <v>2.93</v>
       </c>
       <c r="G24" t="n">
-        <v>1171219848</v>
+        <v>1183335024</v>
       </c>
       <c r="H24" t="n">
-        <v>3733900</v>
+        <v>5463100</v>
       </c>
       <c r="I24" t="n">
         <v>403868805</v>
@@ -5898,7 +5898,7 @@
         <v>0.49</v>
       </c>
       <c r="M24" t="n">
-        <v>0.2831316547331177</v>
+        <v>0.2860603873994232</v>
       </c>
       <c r="N24" t="n">
         <v>0.11</v>
@@ -5976,7 +5976,7 @@
         <v>153470145.9</v>
       </c>
       <c r="AM24" t="n">
-        <v>1055153016.216216</v>
+        <v>1066067589.189189</v>
       </c>
       <c r="AN24" t="n">
         <v>0.0813</v>
@@ -6017,7 +6017,7 @@
         <v>5.84</v>
       </c>
       <c r="AZ24" t="n">
-        <v>1.34</v>
+        <v>1.35</v>
       </c>
       <c r="BA24" t="n">
         <v>0.38</v>
@@ -6026,19 +6026,19 @@
         <v>1.46</v>
       </c>
       <c r="BC24" t="n">
-        <v>146.77</v>
+        <v>144.25</v>
       </c>
       <c r="BD24" t="n">
-        <v>101.49</v>
+        <v>99.43000000000001</v>
       </c>
       <c r="BE24" t="n">
         <v>-53.83</v>
       </c>
       <c r="BF24" t="n">
-        <v>-86.90000000000001</v>
+        <v>-87.03</v>
       </c>
       <c r="BG24" t="n">
-        <v>-49.73</v>
+        <v>-50.25</v>
       </c>
       <c r="BH24" t="n">
         <v>5.99</v>
@@ -6047,7 +6047,7 @@
         <v>0</v>
       </c>
       <c r="BJ24" t="n">
-        <v>2.9</v>
+        <v>2.93</v>
       </c>
       <c r="BK24" t="n">
         <v>0.38</v>
@@ -6056,7 +6056,7 @@
         <v>0.41</v>
       </c>
       <c r="BM24" t="n">
-        <v>2.95</v>
+        <v>2.96</v>
       </c>
       <c r="BN24" t="n">
         <v>5.29</v>
@@ -6065,19 +6065,19 @@
         <v>1.92</v>
       </c>
       <c r="BP24" t="n">
-        <v>2.87</v>
+        <v>2.84</v>
       </c>
       <c r="BQ24" t="n">
-        <v>7.12</v>
+        <v>7.2</v>
       </c>
       <c r="BR24" t="n">
-        <v>2.87</v>
+        <v>2.94</v>
       </c>
       <c r="BS24" t="n">
         <v>0.29</v>
       </c>
       <c r="BT24" t="n">
-        <v>9148997</v>
+        <v>9102590</v>
       </c>
     </row>
     <row r="25">
@@ -6107,13 +6107,13 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>3.7</v>
+        <v>3.76</v>
       </c>
       <c r="G25" t="n">
-        <v>1282028186</v>
+        <v>1302817436</v>
       </c>
       <c r="H25" t="n">
-        <v>737400</v>
+        <v>1003800</v>
       </c>
       <c r="I25" t="n">
         <v>346494097</v>
@@ -6128,7 +6128,7 @@
         <v>0.97</v>
       </c>
       <c r="M25" t="n">
-        <v>0.6392777912910751</v>
+        <v>0.6496442605838165</v>
       </c>
       <c r="N25" t="n">
         <v>0.22</v>
@@ -6206,7 +6206,7 @@
         <v>62368937.46</v>
       </c>
       <c r="AM25" t="n">
-        <v>471333891.9117647</v>
+        <v>478976998.5294117</v>
       </c>
       <c r="AN25" t="n">
         <v>0.4742</v>
@@ -6247,7 +6247,7 @@
         <v>3.27</v>
       </c>
       <c r="AZ25" t="n">
-        <v>8.619999999999999</v>
+        <v>8.76</v>
       </c>
       <c r="BA25" t="n">
         <v>0.23</v>
@@ -6256,19 +6256,19 @@
         <v>2.2</v>
       </c>
       <c r="BC25" t="n">
-        <v>8.369999999999999</v>
+        <v>6.64</v>
       </c>
       <c r="BD25" t="n">
-        <v>-11.51</v>
+        <v>-12.93</v>
       </c>
       <c r="BE25" t="n">
         <v>133</v>
       </c>
       <c r="BF25" t="n">
-        <v>-93.73999999999999</v>
+        <v>-93.84</v>
       </c>
       <c r="BG25" t="n">
-        <v>-40.55</v>
+        <v>-41.5</v>
       </c>
       <c r="BH25" t="n">
         <v>3.97</v>
@@ -6277,7 +6277,7 @@
         <v>0</v>
       </c>
       <c r="BJ25" t="n">
-        <v>3.7</v>
+        <v>3.76</v>
       </c>
       <c r="BK25" t="n">
         <v>0.18</v>
@@ -6286,7 +6286,7 @@
         <v>0.24</v>
       </c>
       <c r="BM25" t="n">
-        <v>3.76</v>
+        <v>3.86</v>
       </c>
       <c r="BN25" t="n">
         <v>6.3</v>
@@ -6295,19 +6295,19 @@
         <v>2.64</v>
       </c>
       <c r="BP25" t="n">
-        <v>3.58</v>
+        <v>3.66</v>
       </c>
       <c r="BQ25" t="n">
-        <v>15.63</v>
+        <v>15.89</v>
       </c>
       <c r="BR25" t="n">
-        <v>3.72</v>
+        <v>3.73</v>
       </c>
       <c r="BS25" t="n">
         <v>0.67</v>
       </c>
       <c r="BT25" t="n">
-        <v>1176577</v>
+        <v>1186897</v>
       </c>
     </row>
     <row r="26">
@@ -6337,13 +6337,13 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>9.630000000000001</v>
+        <v>9.65</v>
       </c>
       <c r="G26" t="n">
-        <v>13042804744</v>
+        <v>13069891933</v>
       </c>
       <c r="H26" t="n">
-        <v>6288500</v>
+        <v>7799400</v>
       </c>
       <c r="I26" t="n">
         <v>1354393401</v>
@@ -6358,7 +6358,7 @@
         <v>1.94</v>
       </c>
       <c r="M26" t="n">
-        <v>0.1681858676833815</v>
+        <v>0.1685351547021237</v>
       </c>
       <c r="N26" t="n">
         <v>0.26</v>
@@ -6436,7 +6436,7 @@
         <v>961619314.7099999</v>
       </c>
       <c r="AM26" t="n">
-        <v>4658144551.428572</v>
+        <v>4667818547.5</v>
       </c>
       <c r="AN26" t="n">
         <v>0.1043</v>
@@ -6486,19 +6486,19 @@
         <v>1.19</v>
       </c>
       <c r="BC26" t="n">
-        <v>-10.12</v>
+        <v>-10.3</v>
       </c>
       <c r="BD26" t="n">
-        <v>-26.61</v>
+        <v>-26.76</v>
       </c>
       <c r="BE26" t="n">
         <v>-80.83</v>
       </c>
       <c r="BF26" t="n">
-        <v>-93.15000000000001</v>
+        <v>-93.17</v>
       </c>
       <c r="BG26" t="n">
-        <v>-87.61</v>
+        <v>-87.63</v>
       </c>
       <c r="BH26" t="n">
         <v>4.69</v>
@@ -6507,7 +6507,7 @@
         <v>0</v>
       </c>
       <c r="BJ26" t="n">
-        <v>9.630000000000001</v>
+        <v>9.65</v>
       </c>
       <c r="BK26" t="n">
         <v>0.71</v>
@@ -6525,19 +6525,19 @@
         <v>6.91</v>
       </c>
       <c r="BP26" t="n">
-        <v>9.5</v>
+        <v>9.48</v>
       </c>
       <c r="BQ26" t="n">
-        <v>13.43</v>
+        <v>13.45</v>
       </c>
       <c r="BR26" t="n">
-        <v>9.5</v>
+        <v>9.75</v>
       </c>
       <c r="BS26" t="n">
         <v>0.16</v>
       </c>
       <c r="BT26" t="n">
-        <v>11652403</v>
+        <v>11736210</v>
       </c>
     </row>
     <row r="27">
@@ -8165,13 +8165,13 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>15.77</v>
+        <v>15.3</v>
       </c>
       <c r="G34" t="n">
-        <v>3256344240</v>
+        <v>3159292449</v>
       </c>
       <c r="H34" t="n">
-        <v>2761600</v>
+        <v>2631800</v>
       </c>
       <c r="I34" t="n">
         <v>206489813</v>
@@ -8186,7 +8186,7 @@
         <v>0.45</v>
       </c>
       <c r="M34" t="n">
-        <v>0.2862706908778672</v>
+        <v>0.2777387049412377</v>
       </c>
       <c r="N34" t="n">
         <v>0.24</v>
@@ -8264,7 +8264,7 @@
         <v>324189006.41</v>
       </c>
       <c r="AM34" t="n">
-        <v>676994644.4906446</v>
+        <v>656817556.9646571</v>
       </c>
       <c r="AN34" t="n">
         <v>0</v>
@@ -8305,7 +8305,7 @@
         <v>30.28</v>
       </c>
       <c r="AZ34" t="n">
-        <v>36.8</v>
+        <v>35.7</v>
       </c>
       <c r="BA34" t="n">
         <v>2.29</v>
@@ -8314,19 +8314,19 @@
         <v>25.26</v>
       </c>
       <c r="BC34" t="n">
-        <v>135.18</v>
+        <v>142.41</v>
       </c>
       <c r="BD34" t="n">
-        <v>92.03</v>
+        <v>97.93000000000001</v>
       </c>
       <c r="BE34" t="n">
         <v>133.33</v>
       </c>
       <c r="BF34" t="n">
-        <v>-85.45</v>
+        <v>-85</v>
       </c>
       <c r="BG34" t="n">
-        <v>60.16</v>
+        <v>65.08</v>
       </c>
       <c r="BH34" t="n">
         <v>38.94</v>
@@ -8335,7 +8335,7 @@
         <v>0</v>
       </c>
       <c r="BJ34" t="n">
-        <v>15.77</v>
+        <v>15.3</v>
       </c>
       <c r="BK34" t="n">
         <v>1.57</v>
@@ -8344,7 +8344,7 @@
         <v>1.58</v>
       </c>
       <c r="BM34" t="n">
-        <v>16.2</v>
+        <v>15.99</v>
       </c>
       <c r="BN34" t="n">
         <v>31.12</v>
@@ -8353,19 +8353,19 @@
         <v>14.32</v>
       </c>
       <c r="BP34" t="n">
-        <v>15.69</v>
+        <v>15.3</v>
       </c>
       <c r="BQ34" t="n">
-        <v>10</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="BR34" t="n">
-        <v>16.1</v>
+        <v>15.82</v>
       </c>
       <c r="BS34" t="n">
         <v>0.32</v>
       </c>
       <c r="BT34" t="n">
-        <v>3073890</v>
+        <v>3104737</v>
       </c>
     </row>
     <row r="35">
@@ -8395,13 +8395,13 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>17.37</v>
+        <v>17.42</v>
       </c>
       <c r="G35" t="n">
-        <v>87657709235</v>
+        <v>87910012965</v>
       </c>
       <c r="H35" t="n">
-        <v>38229400</v>
+        <v>28718200</v>
       </c>
       <c r="I35" t="n">
         <v>5046500000</v>
@@ -8416,7 +8416,7 @@
         <v>4.69</v>
       </c>
       <c r="M35" t="n">
-        <v>7.277374879893125</v>
+        <v>7.298321227257541</v>
       </c>
       <c r="N35" t="n">
         <v>1.79</v>
@@ -8494,7 +8494,7 @@
         <v>5349290000</v>
       </c>
       <c r="AM35" t="n">
-        <v>7244438779.752067</v>
+        <v>7265290327.68595</v>
       </c>
       <c r="AN35" t="n">
         <v>0.5305</v>
@@ -8535,7 +8535,7 @@
         <v>7.68</v>
       </c>
       <c r="AZ35" t="n">
-        <v>10.13</v>
+        <v>10.16</v>
       </c>
       <c r="BA35" t="n">
         <v>1.11</v>
@@ -8544,19 +8544,19 @@
         <v>9.119999999999999</v>
       </c>
       <c r="BC35" t="n">
-        <v>-45.85</v>
+        <v>-46</v>
       </c>
       <c r="BD35" t="n">
-        <v>-55.78</v>
+        <v>-55.91</v>
       </c>
       <c r="BE35" t="n">
         <v>-41.67</v>
       </c>
       <c r="BF35" t="n">
-        <v>-93.59</v>
+        <v>-93.59999999999999</v>
       </c>
       <c r="BG35" t="n">
-        <v>-47.51</v>
+        <v>-47.66</v>
       </c>
       <c r="BH35" t="n">
         <v>3.71</v>
@@ -8565,7 +8565,7 @@
         <v>0</v>
       </c>
       <c r="BJ35" t="n">
-        <v>17.37</v>
+        <v>17.42</v>
       </c>
       <c r="BK35" t="n">
         <v>1.06</v>
@@ -8574,7 +8574,7 @@
         <v>1.04</v>
       </c>
       <c r="BM35" t="n">
-        <v>17.44</v>
+        <v>17.61</v>
       </c>
       <c r="BN35" t="n">
         <v>20.08</v>
@@ -8583,19 +8583,19 @@
         <v>11.7</v>
       </c>
       <c r="BP35" t="n">
-        <v>16.81</v>
+        <v>17.2</v>
       </c>
       <c r="BQ35" t="n">
-        <v>16.62</v>
+        <v>16.67</v>
       </c>
       <c r="BR35" t="n">
-        <v>16.85</v>
+        <v>17.56</v>
       </c>
       <c r="BS35" t="n">
         <v>7.3</v>
       </c>
       <c r="BT35" t="n">
-        <v>36830480</v>
+        <v>37288447</v>
       </c>
     </row>
     <row r="36">
@@ -8858,10 +8858,10 @@
         <v>14.9</v>
       </c>
       <c r="G37" t="n">
-        <v>199073828</v>
+        <v>199919850</v>
       </c>
       <c r="H37" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="I37" t="n">
         <v>4900000</v>
@@ -8876,7 +8876,7 @@
         <v>0.88</v>
       </c>
       <c r="M37" t="n">
-        <v>1.938151413163707</v>
+        <v>1.946388150013252</v>
       </c>
       <c r="N37" t="n">
         <v>0.5</v>
@@ -8954,7 +8954,7 @@
         <v>11319000</v>
       </c>
       <c r="AM37" t="n">
-        <v>47625317.70334928</v>
+        <v>47827715.31100479</v>
       </c>
       <c r="AN37" t="n">
         <v>0</v>
@@ -9055,7 +9055,7 @@
         <v>0.72</v>
       </c>
       <c r="BT37" t="n">
-        <v>850</v>
+        <v>843</v>
       </c>
     </row>
     <row r="38">
@@ -9315,13 +9315,13 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>69.04000000000001</v>
+        <v>69.97</v>
       </c>
       <c r="G39" t="n">
-        <v>3870265083</v>
+        <v>3922400019</v>
       </c>
       <c r="H39" t="n">
-        <v>2800</v>
+        <v>4000</v>
       </c>
       <c r="I39" t="n">
         <v>168174945</v>
@@ -9336,7 +9336,7 @@
         <v>0.53</v>
       </c>
       <c r="M39" t="n">
-        <v>0.1942703307719169</v>
+        <v>0.1968872758762667</v>
       </c>
       <c r="N39" t="n">
         <v>0.06</v>
@@ -9414,7 +9414,7 @@
         <v>2536078170.6</v>
       </c>
       <c r="AM39" t="n">
-        <v>406540449.894958</v>
+        <v>412016808.7184874</v>
       </c>
       <c r="AN39" t="n">
         <v>11.9435</v>
@@ -9455,7 +9455,7 @@
         <v>170.24</v>
       </c>
       <c r="AZ39" t="n">
-        <v>201.71</v>
+        <v>204.43</v>
       </c>
       <c r="BA39" t="n">
         <v>19.01</v>
@@ -9464,19 +9464,19 @@
         <v>91.72</v>
       </c>
       <c r="BC39" t="n">
-        <v>202.01</v>
+        <v>197.99</v>
       </c>
       <c r="BD39" t="n">
-        <v>146.59</v>
+        <v>143.31</v>
       </c>
       <c r="BE39" t="n">
         <v>192.17</v>
       </c>
       <c r="BF39" t="n">
-        <v>-72.47</v>
+        <v>-72.83</v>
       </c>
       <c r="BG39" t="n">
-        <v>32.86</v>
+        <v>31.09</v>
       </c>
       <c r="BH39" t="n">
         <v>128.13</v>
@@ -9485,7 +9485,7 @@
         <v>0</v>
       </c>
       <c r="BJ39" t="n">
-        <v>69.04000000000001</v>
+        <v>69.97</v>
       </c>
       <c r="BK39" t="n">
         <v>15.08</v>
@@ -9494,7 +9494,7 @@
         <v>15.08</v>
       </c>
       <c r="BM39" t="n">
-        <v>69.68000000000001</v>
+        <v>70.33</v>
       </c>
       <c r="BN39" t="n">
         <v>74.56</v>
@@ -9503,19 +9503,19 @@
         <v>54.98</v>
       </c>
       <c r="BP39" t="n">
-        <v>68.90000000000001</v>
+        <v>69.69</v>
       </c>
       <c r="BQ39" t="n">
-        <v>4.58</v>
+        <v>4.64</v>
       </c>
       <c r="BR39" t="n">
-        <v>69.68000000000001</v>
+        <v>69.69</v>
       </c>
       <c r="BS39" t="n">
         <v>0.58</v>
       </c>
       <c r="BT39" t="n">
-        <v>3903</v>
+        <v>3830</v>
       </c>
     </row>
     <row r="40">
@@ -9545,13 +9545,13 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>22.12</v>
+        <v>22.04</v>
       </c>
       <c r="G40" t="n">
-        <v>126766075009</v>
+        <v>126307520486</v>
       </c>
       <c r="H40" t="n">
-        <v>29686100</v>
+        <v>21989500</v>
       </c>
       <c r="I40" t="n">
         <v>5730834040</v>
@@ -9566,7 +9566,7 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="M40" t="n">
-        <v>0.3846239596183408</v>
+        <v>0.3832326484467625</v>
       </c>
       <c r="N40" t="n">
         <v>0.05</v>
@@ -9644,7 +9644,7 @@
         <v>15358635227.2</v>
       </c>
       <c r="AM40" t="n">
-        <v>6575003890.508298</v>
+        <v>6551219942.219916</v>
       </c>
       <c r="AN40" t="n">
         <v>0.5641</v>
@@ -9685,7 +9685,7 @@
         <v>36.13</v>
       </c>
       <c r="AZ40" t="n">
-        <v>11.17</v>
+        <v>11.13</v>
       </c>
       <c r="BA40" t="n">
         <v>2.76</v>
@@ -9694,19 +9694,19 @@
         <v>27.89</v>
       </c>
       <c r="BC40" t="n">
-        <v>100.04</v>
+        <v>100.77</v>
       </c>
       <c r="BD40" t="n">
-        <v>63.33</v>
+        <v>63.92</v>
       </c>
       <c r="BE40" t="n">
         <v>-49.5</v>
       </c>
       <c r="BF40" t="n">
-        <v>-87.52</v>
+        <v>-87.48</v>
       </c>
       <c r="BG40" t="n">
-        <v>26.09</v>
+        <v>26.54</v>
       </c>
       <c r="BH40" t="n">
         <v>32.47</v>
@@ -9715,7 +9715,7 @@
         <v>0</v>
       </c>
       <c r="BJ40" t="n">
-        <v>22.12</v>
+        <v>22.04</v>
       </c>
       <c r="BK40" t="n">
         <v>2.68</v>
@@ -9724,7 +9724,7 @@
         <v>2.5</v>
       </c>
       <c r="BM40" t="n">
-        <v>22.26</v>
+        <v>22.33</v>
       </c>
       <c r="BN40" t="n">
         <v>27.36</v>
@@ -9733,19 +9733,19 @@
         <v>17.67</v>
       </c>
       <c r="BP40" t="n">
-        <v>21.83</v>
+        <v>21.92</v>
       </c>
       <c r="BQ40" t="n">
-        <v>8.85</v>
+        <v>8.82</v>
       </c>
       <c r="BR40" t="n">
-        <v>21.95</v>
+        <v>22.28</v>
       </c>
       <c r="BS40" t="n">
         <v>0.39</v>
       </c>
       <c r="BT40" t="n">
-        <v>31162577</v>
+        <v>31195740</v>
       </c>
     </row>
     <row r="41">
@@ -9775,13 +9775,13 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>16.17</v>
+        <v>16.09</v>
       </c>
       <c r="G41" t="n">
-        <v>192689175097</v>
+        <v>191758302038</v>
       </c>
       <c r="H41" t="n">
-        <v>6498700</v>
+        <v>5032900</v>
       </c>
       <c r="I41" t="n">
         <v>5303870781</v>
@@ -9796,7 +9796,7 @@
         <v>0.92</v>
       </c>
       <c r="M41" t="n">
-        <v>1.284074584910574</v>
+        <v>1.277871276207643</v>
       </c>
       <c r="N41" t="n">
         <v>0.07000000000000001</v>
@@ -9874,7 +9874,7 @@
         <v>12304980211.92</v>
       </c>
       <c r="AM41" t="n">
-        <v>29690165654.39137</v>
+        <v>29546733750.07704</v>
       </c>
       <c r="AN41" t="n">
         <v>1.6841</v>
@@ -9915,7 +9915,7 @@
         <v>24.4</v>
       </c>
       <c r="AZ41" t="n">
-        <v>24.2</v>
+        <v>24.08</v>
       </c>
       <c r="BA41" t="n">
         <v>2.53</v>
@@ -9924,19 +9924,19 @@
         <v>13.77</v>
       </c>
       <c r="BC41" t="n">
-        <v>84.81999999999999</v>
+        <v>85.73999999999999</v>
       </c>
       <c r="BD41" t="n">
-        <v>50.91</v>
+        <v>51.66</v>
       </c>
       <c r="BE41" t="n">
         <v>49.67</v>
       </c>
       <c r="BF41" t="n">
-        <v>-84.37</v>
+        <v>-84.29000000000001</v>
       </c>
       <c r="BG41" t="n">
-        <v>-14.84</v>
+        <v>-14.42</v>
       </c>
       <c r="BH41" t="n">
         <v>17.11</v>
@@ -9945,7 +9945,7 @@
         <v>0</v>
       </c>
       <c r="BJ41" t="n">
-        <v>16.17</v>
+        <v>16.09</v>
       </c>
       <c r="BK41" t="n">
         <v>2.32</v>
@@ -9954,7 +9954,7 @@
         <v>2.34</v>
       </c>
       <c r="BM41" t="n">
-        <v>16.2</v>
+        <v>16.31</v>
       </c>
       <c r="BN41" t="n">
         <v>18.28</v>
@@ -9963,19 +9963,19 @@
         <v>13.43</v>
       </c>
       <c r="BP41" t="n">
-        <v>15.92</v>
+        <v>16.01</v>
       </c>
       <c r="BQ41" t="n">
-        <v>6.92</v>
+        <v>6.88</v>
       </c>
       <c r="BR41" t="n">
-        <v>15.96</v>
+        <v>16.31</v>
       </c>
       <c r="BS41" t="n">
         <v>0.5600000000000001</v>
       </c>
       <c r="BT41" t="n">
-        <v>7349463</v>
+        <v>6933868</v>
       </c>
     </row>
     <row r="42">
@@ -10005,13 +10005,13 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>18.33</v>
+        <v>18.2</v>
       </c>
       <c r="G42" t="n">
-        <v>192689175097</v>
+        <v>191758302038</v>
       </c>
       <c r="H42" t="n">
-        <v>21528800</v>
+        <v>24044300</v>
       </c>
       <c r="I42" t="n">
         <v>5288141247</v>
@@ -10026,7 +10026,7 @@
         <v>1.05</v>
       </c>
       <c r="M42" t="n">
-        <v>1.287894054531085</v>
+        <v>1.281672294135848</v>
       </c>
       <c r="N42" t="n">
         <v>0.08</v>
@@ -10104,7 +10104,7 @@
         <v>12268487693.04</v>
       </c>
       <c r="AM42" t="n">
-        <v>26216214298.91157</v>
+        <v>26089564903.12925</v>
       </c>
       <c r="AN42" t="n">
         <v>1.8491</v>
@@ -10145,7 +10145,7 @@
         <v>24.4</v>
       </c>
       <c r="AZ42" t="n">
-        <v>26.55</v>
+        <v>26.36</v>
       </c>
       <c r="BA42" t="n">
         <v>2.53</v>
@@ -10154,19 +10154,19 @@
         <v>15.11</v>
       </c>
       <c r="BC42" t="n">
-        <v>63.04</v>
+        <v>64.20999999999999</v>
       </c>
       <c r="BD42" t="n">
-        <v>33.12</v>
+        <v>34.07</v>
       </c>
       <c r="BE42" t="n">
         <v>44.83</v>
       </c>
       <c r="BF42" t="n">
-        <v>-86.20999999999999</v>
+        <v>-86.11</v>
       </c>
       <c r="BG42" t="n">
-        <v>-17.54</v>
+        <v>-16.95</v>
       </c>
       <c r="BH42" t="n">
         <v>17.11</v>
@@ -10175,7 +10175,7 @@
         <v>0</v>
       </c>
       <c r="BJ42" t="n">
-        <v>18.33</v>
+        <v>18.2</v>
       </c>
       <c r="BK42" t="n">
         <v>2.32</v>
@@ -10184,7 +10184,7 @@
         <v>2.34</v>
       </c>
       <c r="BM42" t="n">
-        <v>18.44</v>
+        <v>18.46</v>
       </c>
       <c r="BN42" t="n">
         <v>21.33</v>
@@ -10193,19 +10193,19 @@
         <v>15.67</v>
       </c>
       <c r="BP42" t="n">
-        <v>18.12</v>
+        <v>18.14</v>
       </c>
       <c r="BQ42" t="n">
-        <v>7.84</v>
+        <v>7.79</v>
       </c>
       <c r="BR42" t="n">
-        <v>18.2</v>
+        <v>18.45</v>
       </c>
       <c r="BS42" t="n">
         <v>0.63</v>
       </c>
       <c r="BT42" t="n">
-        <v>40385889</v>
+        <v>40260834</v>
       </c>
     </row>
     <row r="43">
@@ -10235,13 +10235,13 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>39.77</v>
+        <v>40.16</v>
       </c>
       <c r="G43" t="n">
-        <v>77209478888</v>
+        <v>77966623703</v>
       </c>
       <c r="H43" t="n">
-        <v>5320400</v>
+        <v>5465900</v>
       </c>
       <c r="I43" t="n">
         <v>1941400000</v>
@@ -10334,7 +10334,7 @@
         <v>9182822000</v>
       </c>
       <c r="AM43" t="n">
-        <v>9404321423.629719</v>
+        <v>9496543690.986601</v>
       </c>
       <c r="AN43" t="n">
         <v>4.5901</v>
@@ -10375,7 +10375,7 @@
         <v>19.95</v>
       </c>
       <c r="AZ43" t="n">
-        <v>72.18000000000001</v>
+        <v>72.89</v>
       </c>
       <c r="BA43" t="n">
         <v>5.63</v>
@@ -10384,19 +10384,19 @@
         <v>48.62</v>
       </c>
       <c r="BC43" t="n">
-        <v>-38.56</v>
+        <v>-39.16</v>
       </c>
       <c r="BD43" t="n">
-        <v>-49.83</v>
+        <v>-50.32</v>
       </c>
       <c r="BE43" t="n">
         <v>81.5</v>
       </c>
       <c r="BF43" t="n">
-        <v>-85.84999999999999</v>
+        <v>-85.98</v>
       </c>
       <c r="BG43" t="n">
-        <v>22.25</v>
+        <v>21.06</v>
       </c>
       <c r="BH43" t="n">
         <v>5.61</v>
@@ -10405,7 +10405,7 @@
         <v>0</v>
       </c>
       <c r="BJ43" t="n">
-        <v>39.77</v>
+        <v>40.16</v>
       </c>
       <c r="BK43" t="n">
         <v>4.73</v>
@@ -10414,7 +10414,7 @@
         <v>4.73</v>
       </c>
       <c r="BM43" t="n">
-        <v>40.11</v>
+        <v>40.6</v>
       </c>
       <c r="BN43" t="n">
         <v>42.98</v>
@@ -10423,19 +10423,19 @@
         <v>28.06</v>
       </c>
       <c r="BP43" t="n">
-        <v>38.86</v>
+        <v>39.78</v>
       </c>
       <c r="BQ43" t="n">
-        <v>8.4</v>
+        <v>8.48</v>
       </c>
       <c r="BR43" t="n">
-        <v>39.06</v>
+        <v>40</v>
       </c>
       <c r="BS43" t="n">
         <v>0</v>
       </c>
       <c r="BT43" t="n">
-        <v>6715793</v>
+        <v>6777434</v>
       </c>
     </row>
     <row r="44">
@@ -10925,13 +10925,13 @@
         </is>
       </c>
       <c r="F46" t="n">
-        <v>4.08</v>
+        <v>4.04</v>
       </c>
       <c r="G46" t="n">
-        <v>4082207203</v>
+        <v>4042185601</v>
       </c>
       <c r="H46" t="n">
-        <v>24498800</v>
+        <v>18773700</v>
       </c>
       <c r="I46" t="n">
         <v>1000541644</v>
@@ -10946,7 +10946,7 @@
         <v>2.5</v>
       </c>
       <c r="M46" t="n">
-        <v>0.07095647472946251</v>
+        <v>0.07026082366381874</v>
       </c>
       <c r="N46" t="n">
         <v>0.08</v>
@@ -11024,7 +11024,7 @@
         <v>460249156.24</v>
       </c>
       <c r="AM46" t="n">
-        <v>4002163924.509804</v>
+        <v>3962927059.803922</v>
       </c>
       <c r="AN46" t="n">
         <v>0.0311</v>
@@ -11065,7 +11065,7 @@
         <v>3.3</v>
       </c>
       <c r="AZ46" t="n">
-        <v>3.37</v>
+        <v>3.33</v>
       </c>
       <c r="BA46" t="n">
         <v>0.42</v>
@@ -11074,19 +11074,19 @@
         <v>7.38</v>
       </c>
       <c r="BC46" t="n">
-        <v>-0.89</v>
+        <v>0.1</v>
       </c>
       <c r="BD46" t="n">
-        <v>-19.07</v>
+        <v>-18.27</v>
       </c>
       <c r="BE46" t="n">
         <v>-17.5</v>
       </c>
       <c r="BF46" t="n">
-        <v>-89.63</v>
+        <v>-89.53</v>
       </c>
       <c r="BG46" t="n">
-        <v>80.84999999999999</v>
+        <v>82.64</v>
       </c>
       <c r="BH46" t="n">
         <v>1.58</v>
@@ -11095,7 +11095,7 @@
         <v>0</v>
       </c>
       <c r="BJ46" t="n">
-        <v>4.08</v>
+        <v>4.04</v>
       </c>
       <c r="BK46" t="n">
         <v>0.46</v>
@@ -11104,7 +11104,7 @@
         <v>0.46</v>
       </c>
       <c r="BM46" t="n">
-        <v>4.2</v>
+        <v>4.12</v>
       </c>
       <c r="BN46" t="n">
         <v>7.31</v>
@@ -11113,19 +11113,19 @@
         <v>2.97</v>
       </c>
       <c r="BP46" t="n">
-        <v>4.06</v>
+        <v>3.98</v>
       </c>
       <c r="BQ46" t="n">
-        <v>8.92</v>
+        <v>8.83</v>
       </c>
       <c r="BR46" t="n">
-        <v>4.14</v>
+        <v>4.1</v>
       </c>
       <c r="BS46" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="BT46" t="n">
-        <v>19430970</v>
+        <v>20065343</v>
       </c>
     </row>
     <row r="47">
@@ -11155,13 +11155,13 @@
         </is>
       </c>
       <c r="F47" t="n">
-        <v>8.81</v>
+        <v>8.83</v>
       </c>
       <c r="G47" t="n">
-        <v>3060600312</v>
+        <v>3089991365</v>
       </c>
       <c r="H47" t="n">
-        <v>16100</v>
+        <v>9100</v>
       </c>
       <c r="I47" t="n">
         <v>254106600</v>
@@ -11176,7 +11176,7 @@
         <v>1.22</v>
       </c>
       <c r="M47" t="n">
-        <v>0.7217247665721741</v>
+        <v>0.7286555150212827</v>
       </c>
       <c r="N47" t="n">
         <v>0.07000000000000001</v>
@@ -11254,7 +11254,7 @@
         <v>322715382</v>
       </c>
       <c r="AM47" t="n">
-        <v>542659629.7872341</v>
+        <v>547870809.3971632</v>
       </c>
       <c r="AN47" t="n">
         <v>0.4132</v>
@@ -11295,7 +11295,7 @@
         <v>11.74</v>
       </c>
       <c r="AZ47" t="n">
-        <v>11.57</v>
+        <v>11.6</v>
       </c>
       <c r="BA47" t="n">
         <v>1.46</v>
@@ -11304,19 +11304,19 @@
         <v>8.619999999999999</v>
       </c>
       <c r="BC47" t="n">
-        <v>63.15</v>
+        <v>62.78</v>
       </c>
       <c r="BD47" t="n">
-        <v>33.21</v>
+        <v>32.91</v>
       </c>
       <c r="BE47" t="n">
         <v>31.33</v>
       </c>
       <c r="BF47" t="n">
-        <v>-83.45</v>
+        <v>-83.48</v>
       </c>
       <c r="BG47" t="n">
-        <v>-2.16</v>
+        <v>-2.38</v>
       </c>
       <c r="BH47" t="n">
         <v>7.23</v>
@@ -11325,7 +11325,7 @@
         <v>0</v>
       </c>
       <c r="BJ47" t="n">
-        <v>8.81</v>
+        <v>8.83</v>
       </c>
       <c r="BK47" t="n">
         <v>1.27</v>
@@ -11334,7 +11334,7 @@
         <v>1.29</v>
       </c>
       <c r="BM47" t="n">
-        <v>9.1</v>
+        <v>8.93</v>
       </c>
       <c r="BN47" t="n">
         <v>9.25</v>
@@ -11343,19 +11343,19 @@
         <v>7.2</v>
       </c>
       <c r="BP47" t="n">
-        <v>8.789999999999999</v>
+        <v>8.82</v>
       </c>
       <c r="BQ47" t="n">
-        <v>6.81</v>
+        <v>6.83</v>
       </c>
       <c r="BR47" t="n">
-        <v>9.029999999999999</v>
+        <v>8.869999999999999</v>
       </c>
       <c r="BS47" t="n">
         <v>0.53</v>
       </c>
       <c r="BT47" t="n">
-        <v>12736</v>
+        <v>12944</v>
       </c>
     </row>
     <row r="48">
@@ -11385,13 +11385,13 @@
         </is>
       </c>
       <c r="F48" t="n">
-        <v>9.039999999999999</v>
+        <v>9.130000000000001</v>
       </c>
       <c r="G48" t="n">
-        <v>3060600312</v>
+        <v>3089991365</v>
       </c>
       <c r="H48" t="n">
-        <v>1300</v>
+        <v>2100</v>
       </c>
       <c r="I48" t="n">
         <v>93397546</v>
@@ -11406,7 +11406,7 @@
         <v>1.24</v>
       </c>
       <c r="M48" t="n">
-        <v>1.963595773377695</v>
+        <v>1.982452253010021</v>
       </c>
       <c r="N48" t="n">
         <v>0.07000000000000001</v>
@@ -11484,7 +11484,7 @@
         <v>118614883.42</v>
       </c>
       <c r="AM48" t="n">
-        <v>535069984.6153846</v>
+        <v>540208280.5944057</v>
       </c>
       <c r="AN48" t="n">
         <v>0.4132</v>
@@ -11525,7 +11525,7 @@
         <v>11.74</v>
       </c>
       <c r="AZ48" t="n">
-        <v>11.83</v>
+        <v>11.95</v>
       </c>
       <c r="BA48" t="n">
         <v>1.46</v>
@@ -11534,19 +11534,19 @@
         <v>8.24</v>
       </c>
       <c r="BC48" t="n">
-        <v>59</v>
+        <v>57.43</v>
       </c>
       <c r="BD48" t="n">
-        <v>29.82</v>
+        <v>28.54</v>
       </c>
       <c r="BE48" t="n">
         <v>30.83</v>
       </c>
       <c r="BF48" t="n">
-        <v>-83.87</v>
+        <v>-84.03</v>
       </c>
       <c r="BG48" t="n">
-        <v>-8.890000000000001</v>
+        <v>-9.789999999999999</v>
       </c>
       <c r="BH48" t="n">
         <v>7.23</v>
@@ -11555,7 +11555,7 @@
         <v>0</v>
       </c>
       <c r="BJ48" t="n">
-        <v>9.039999999999999</v>
+        <v>9.130000000000001</v>
       </c>
       <c r="BK48" t="n">
         <v>1.27</v>
@@ -11564,7 +11564,7 @@
         <v>1.29</v>
       </c>
       <c r="BM48" t="n">
-        <v>9.1</v>
+        <v>9.140000000000001</v>
       </c>
       <c r="BN48" t="n">
         <v>9.48</v>
@@ -11573,10 +11573,10 @@
         <v>7.21</v>
       </c>
       <c r="BP48" t="n">
-        <v>9.029999999999999</v>
+        <v>9.06</v>
       </c>
       <c r="BQ48" t="n">
-        <v>6.99</v>
+        <v>7.06</v>
       </c>
       <c r="BR48" t="n">
         <v>9.1</v>
@@ -11585,7 +11585,7 @@
         <v>0.54</v>
       </c>
       <c r="BT48" t="n">
-        <v>2678</v>
+        <v>2641</v>
       </c>
     </row>
     <row r="49">
@@ -11845,13 +11845,13 @@
         </is>
       </c>
       <c r="F50" t="n">
-        <v>34.5</v>
+        <v>34.3</v>
       </c>
       <c r="G50" t="n">
         <v>974049400</v>
       </c>
       <c r="H50" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="I50" t="n">
         <v>11540870</v>
@@ -11985,7 +11985,7 @@
         <v>68.48999999999999</v>
       </c>
       <c r="AZ50" t="n">
-        <v>76.06999999999999</v>
+        <v>75.63</v>
       </c>
       <c r="BA50" t="n">
         <v>9.210000000000001</v>
@@ -11994,19 +11994,19 @@
         <v>30.53</v>
       </c>
       <c r="BC50" t="n">
-        <v>143.12</v>
+        <v>144.54</v>
       </c>
       <c r="BD50" t="n">
-        <v>98.51000000000001</v>
+        <v>99.67</v>
       </c>
       <c r="BE50" t="n">
         <v>120.5</v>
       </c>
       <c r="BF50" t="n">
-        <v>-73.29000000000001</v>
+        <v>-73.14</v>
       </c>
       <c r="BG50" t="n">
-        <v>-11.51</v>
+        <v>-10.99</v>
       </c>
       <c r="BH50" t="n">
         <v>42.6</v>
@@ -12015,7 +12015,7 @@
         <v>0</v>
       </c>
       <c r="BJ50" t="n">
-        <v>34.5</v>
+        <v>34.3</v>
       </c>
       <c r="BK50" t="n">
         <v>7.34</v>
@@ -12024,7 +12024,7 @@
         <v>7.6</v>
       </c>
       <c r="BM50" t="n">
-        <v>34.5</v>
+        <v>34.3</v>
       </c>
       <c r="BN50" t="n">
         <v>39.22</v>
@@ -12033,13 +12033,13 @@
         <v>23.5</v>
       </c>
       <c r="BP50" t="n">
-        <v>34.5</v>
+        <v>34.3</v>
       </c>
       <c r="BQ50" t="n">
-        <v>4.54</v>
+        <v>4.51</v>
       </c>
       <c r="BR50" t="n">
-        <v>34.5</v>
+        <v>34.3</v>
       </c>
       <c r="BS50" t="n">
         <v>0.4</v>
@@ -12523,13 +12523,13 @@
         </is>
       </c>
       <c r="F53" t="n">
-        <v>6.53</v>
+        <v>6.5</v>
       </c>
       <c r="G53" t="n">
-        <v>893646200</v>
+        <v>889540600</v>
       </c>
       <c r="H53" t="n">
-        <v>1600</v>
+        <v>20600</v>
       </c>
       <c r="I53" t="n">
         <v>136852484</v>
@@ -12544,7 +12544,7 @@
         <v>2.79</v>
       </c>
       <c r="M53" t="n">
-        <v>2.321526233992972</v>
+        <v>2.310860650559303</v>
       </c>
       <c r="N53" t="n">
         <v>1.48</v>
@@ -12622,7 +12622,7 @@
         <v>39687220.36</v>
       </c>
       <c r="AM53" t="n">
-        <v>45524513.49974529</v>
+        <v>45315364.2384106</v>
       </c>
       <c r="AN53" t="n">
         <v>0</v>
@@ -12672,16 +12672,16 @@
         <v>0</v>
       </c>
       <c r="BC53" t="n">
-        <v>-39.65</v>
+        <v>-39.37</v>
       </c>
       <c r="BD53" t="n">
-        <v>-50.73</v>
+        <v>-50.5</v>
       </c>
       <c r="BE53" t="n">
         <v>-100</v>
       </c>
       <c r="BF53" t="n">
-        <v>-95.56</v>
+        <v>-95.54000000000001</v>
       </c>
       <c r="BG53" t="n">
         <v>-100</v>
@@ -12693,7 +12693,7 @@
         <v>0</v>
       </c>
       <c r="BJ53" t="n">
-        <v>6.53</v>
+        <v>6.5</v>
       </c>
       <c r="BK53" t="n">
         <v>0.29</v>
@@ -12702,7 +12702,7 @@
         <v>0.09</v>
       </c>
       <c r="BM53" t="n">
-        <v>6.7</v>
+        <v>6.69</v>
       </c>
       <c r="BN53" t="n">
         <v>10.39</v>
@@ -12711,19 +12711,19 @@
         <v>4.82</v>
       </c>
       <c r="BP53" t="n">
-        <v>6.52</v>
+        <v>6.48</v>
       </c>
       <c r="BQ53" t="n">
-        <v>76.54000000000001</v>
+        <v>76.18000000000001</v>
       </c>
       <c r="BR53" t="n">
-        <v>6.7</v>
+        <v>6.55</v>
       </c>
       <c r="BS53" t="n">
         <v>2.36</v>
       </c>
       <c r="BT53" t="n">
-        <v>44250</v>
+        <v>38900</v>
       </c>
     </row>
     <row r="54">
@@ -12753,13 +12753,13 @@
         </is>
       </c>
       <c r="F54" t="n">
-        <v>10.45</v>
+        <v>10.37</v>
       </c>
       <c r="G54" t="n">
-        <v>2437065355</v>
+        <v>2418409450</v>
       </c>
       <c r="H54" t="n">
-        <v>314600</v>
+        <v>193700</v>
       </c>
       <c r="I54" t="n">
         <v>233212121</v>
@@ -12774,7 +12774,7 @@
         <v>0.97</v>
       </c>
       <c r="M54" t="n">
-        <v>1.36790426501674</v>
+        <v>1.35743286261266</v>
       </c>
       <c r="N54" t="n">
         <v>0.5600000000000001</v>
@@ -12852,7 +12852,7 @@
         <v>233212121</v>
       </c>
       <c r="AM54" t="n">
-        <v>333387873.4610123</v>
+        <v>330835766.0738714</v>
       </c>
       <c r="AN54" t="n">
         <v>0.1531</v>
@@ -12893,7 +12893,7 @@
         <v>12.25</v>
       </c>
       <c r="AZ54" t="n">
-        <v>16.63</v>
+        <v>16.51</v>
       </c>
       <c r="BA54" t="n">
         <v>0.98</v>
@@ -12902,19 +12902,19 @@
         <v>6.52</v>
       </c>
       <c r="BC54" t="n">
-        <v>43.61</v>
+        <v>44.72</v>
       </c>
       <c r="BD54" t="n">
-        <v>17.26</v>
+        <v>18.16</v>
       </c>
       <c r="BE54" t="n">
         <v>59.17</v>
       </c>
       <c r="BF54" t="n">
-        <v>-90.59</v>
+        <v>-90.52</v>
       </c>
       <c r="BG54" t="n">
-        <v>-37.64</v>
+        <v>-37.16</v>
       </c>
       <c r="BH54" t="n">
         <v>10.01</v>
@@ -12923,7 +12923,7 @@
         <v>0</v>
       </c>
       <c r="BJ54" t="n">
-        <v>10.45</v>
+        <v>10.37</v>
       </c>
       <c r="BK54" t="n">
         <v>1</v>
@@ -12932,7 +12932,7 @@
         <v>1</v>
       </c>
       <c r="BM54" t="n">
-        <v>10.45</v>
+        <v>10.5</v>
       </c>
       <c r="BN54" t="n">
         <v>11.75</v>
@@ -12941,19 +12941,19 @@
         <v>8.279999999999999</v>
       </c>
       <c r="BP54" t="n">
-        <v>9.949999999999999</v>
+        <v>10.26</v>
       </c>
       <c r="BQ54" t="n">
-        <v>10.42</v>
+        <v>10.34</v>
       </c>
       <c r="BR54" t="n">
-        <v>10.12</v>
+        <v>10.39</v>
       </c>
       <c r="BS54" t="n">
         <v>1.26</v>
       </c>
       <c r="BT54" t="n">
-        <v>277960</v>
+        <v>263377</v>
       </c>
     </row>
     <row r="55">
@@ -12983,13 +12983,13 @@
         </is>
       </c>
       <c r="F55" t="n">
-        <v>49.53</v>
+        <v>49.52</v>
       </c>
       <c r="G55" t="n">
-        <v>5087404482</v>
+        <v>6578755376</v>
       </c>
       <c r="H55" t="n">
-        <v>9600</v>
+        <v>13600</v>
       </c>
       <c r="I55" t="n">
         <v>84052790</v>
@@ -13004,7 +13004,7 @@
         <v>2</v>
       </c>
       <c r="M55" t="n">
-        <v>0.7853485232071301</v>
+        <v>1.015570088315727</v>
       </c>
       <c r="N55" t="n">
         <v>0.16</v>
@@ -13082,7 +13082,7 @@
         <v>579123723.1</v>
       </c>
       <c r="AM55" t="n">
-        <v>255905658.0482897</v>
+        <v>330923308.6519115</v>
       </c>
       <c r="AN55" t="n">
         <v>3.1953</v>
@@ -13123,7 +13123,7 @@
         <v>51.21</v>
       </c>
       <c r="AZ55" t="n">
-        <v>52.09</v>
+        <v>52.08</v>
       </c>
       <c r="BA55" t="n">
         <v>9.380000000000001</v>
@@ -13132,16 +13132,16 @@
         <v>16.08</v>
       </c>
       <c r="BC55" t="n">
-        <v>26.62</v>
+        <v>26.64</v>
       </c>
       <c r="BD55" t="n">
-        <v>3.38</v>
+        <v>3.4</v>
       </c>
       <c r="BE55" t="n">
         <v>5.17</v>
       </c>
       <c r="BF55" t="n">
-        <v>-81.06999999999999</v>
+        <v>-81.06</v>
       </c>
       <c r="BG55" t="n">
         <v>-67.54000000000001</v>
@@ -13153,7 +13153,7 @@
         <v>0</v>
       </c>
       <c r="BJ55" t="n">
-        <v>49.53</v>
+        <v>49.52</v>
       </c>
       <c r="BK55" t="n">
         <v>6.89</v>
@@ -13162,28 +13162,28 @@
         <v>7.03</v>
       </c>
       <c r="BM55" t="n">
-        <v>50.93</v>
+        <v>49.65</v>
       </c>
       <c r="BN55" t="n">
         <v>73.67</v>
       </c>
       <c r="BO55" t="n">
-        <v>34.46</v>
+        <v>35.58</v>
       </c>
       <c r="BP55" t="n">
-        <v>49.31</v>
+        <v>49.24</v>
       </c>
       <c r="BQ55" t="n">
         <v>7.04</v>
       </c>
       <c r="BR55" t="n">
-        <v>50.93</v>
+        <v>49.65</v>
       </c>
       <c r="BS55" t="n">
         <v>0.66</v>
       </c>
       <c r="BT55" t="n">
-        <v>6645</v>
+        <v>6860</v>
       </c>
     </row>
     <row r="56">
@@ -13213,13 +13213,13 @@
         </is>
       </c>
       <c r="F56" t="n">
-        <v>58.71</v>
+        <v>59.49</v>
       </c>
       <c r="G56" t="n">
-        <v>5087404482</v>
+        <v>6578755376</v>
       </c>
       <c r="H56" t="n">
-        <v>46600</v>
+        <v>49500</v>
       </c>
       <c r="I56" t="n">
         <v>39675836</v>
@@ -13234,7 +13234,7 @@
         <v>2.41</v>
       </c>
       <c r="M56" t="n">
-        <v>1.663751571559552</v>
+        <v>2.151473238358061</v>
       </c>
       <c r="N56" t="n">
         <v>0.19</v>
@@ -13312,7 +13312,7 @@
         <v>273366510.04</v>
       </c>
       <c r="AM56" t="n">
-        <v>211622482.6123128</v>
+        <v>273658709.484193</v>
       </c>
       <c r="AN56" t="n">
         <v>3.5102</v>
@@ -13353,7 +13353,7 @@
         <v>51.21</v>
       </c>
       <c r="AZ56" t="n">
-        <v>56.07</v>
+        <v>56.81</v>
       </c>
       <c r="BA56" t="n">
         <v>9.380000000000001</v>
@@ -13362,19 +13362,19 @@
         <v>17.68</v>
       </c>
       <c r="BC56" t="n">
-        <v>6.82</v>
+        <v>5.42</v>
       </c>
       <c r="BD56" t="n">
-        <v>-12.78</v>
+        <v>-13.93</v>
       </c>
       <c r="BE56" t="n">
         <v>-4.5</v>
       </c>
       <c r="BF56" t="n">
-        <v>-84.03</v>
+        <v>-84.23999999999999</v>
       </c>
       <c r="BG56" t="n">
-        <v>-69.89</v>
+        <v>-70.28</v>
       </c>
       <c r="BH56" t="n">
         <v>25.37</v>
@@ -13383,7 +13383,7 @@
         <v>0</v>
       </c>
       <c r="BJ56" t="n">
-        <v>58.71</v>
+        <v>59.49</v>
       </c>
       <c r="BK56" t="n">
         <v>6.89</v>
@@ -13392,28 +13392,28 @@
         <v>7.03</v>
       </c>
       <c r="BM56" t="n">
-        <v>60.76</v>
+        <v>60.77</v>
       </c>
       <c r="BN56" t="n">
         <v>86.77</v>
       </c>
       <c r="BO56" t="n">
-        <v>46.32</v>
+        <v>46.42</v>
       </c>
       <c r="BP56" t="n">
-        <v>57</v>
+        <v>58.1</v>
       </c>
       <c r="BQ56" t="n">
-        <v>8.35</v>
+        <v>8.460000000000001</v>
       </c>
       <c r="BR56" t="n">
-        <v>58.65</v>
+        <v>58.7</v>
       </c>
       <c r="BS56" t="n">
         <v>0.79</v>
       </c>
       <c r="BT56" t="n">
-        <v>33006</v>
+        <v>33970</v>
       </c>
     </row>
     <row r="57">
@@ -13443,13 +13443,13 @@
         </is>
       </c>
       <c r="F57" t="n">
-        <v>6.08</v>
+        <v>6.16</v>
       </c>
       <c r="G57" t="n">
-        <v>1421857230</v>
+        <v>1440565244</v>
       </c>
       <c r="H57" t="n">
-        <v>1303700</v>
+        <v>1377200</v>
       </c>
       <c r="I57" t="n">
         <v>233858065</v>
@@ -13464,7 +13464,7 @@
         <v>0.77</v>
       </c>
       <c r="M57" t="n">
-        <v>0.4256000583088722</v>
+        <v>0.4311998693737589</v>
       </c>
       <c r="N57" t="n">
         <v>0.08</v>
@@ -13542,7 +13542,7 @@
         <v>229180903.7</v>
       </c>
       <c r="AM57" t="n">
-        <v>106346838.4442782</v>
+        <v>107746091.5482423</v>
       </c>
       <c r="AN57" t="n">
         <v>0.347</v>
@@ -13583,7 +13583,7 @@
         <v>10.72</v>
       </c>
       <c r="AZ57" t="n">
-        <v>9.27</v>
+        <v>9.390000000000001</v>
       </c>
       <c r="BA57" t="n">
         <v>1.13</v>
@@ -13592,19 +13592,19 @@
         <v>6.26</v>
       </c>
       <c r="BC57" t="n">
-        <v>115.98</v>
+        <v>113.17</v>
       </c>
       <c r="BD57" t="n">
-        <v>76.34</v>
+        <v>74.05</v>
       </c>
       <c r="BE57" t="n">
         <v>52.5</v>
       </c>
       <c r="BF57" t="n">
-        <v>-81.45999999999999</v>
+        <v>-81.7</v>
       </c>
       <c r="BG57" t="n">
-        <v>3.02</v>
+        <v>1.69</v>
       </c>
       <c r="BH57" t="n">
         <v>7.82</v>
@@ -13613,7 +13613,7 @@
         <v>0</v>
       </c>
       <c r="BJ57" t="n">
-        <v>6.08</v>
+        <v>6.16</v>
       </c>
       <c r="BK57" t="n">
         <v>0.98</v>
@@ -13622,28 +13622,28 @@
         <v>1.04</v>
       </c>
       <c r="BM57" t="n">
-        <v>6.08</v>
+        <v>6.18</v>
       </c>
       <c r="BN57" t="n">
-        <v>6.11</v>
+        <v>6.18</v>
       </c>
       <c r="BO57" t="n">
-        <v>3.4</v>
+        <v>3.42</v>
       </c>
       <c r="BP57" t="n">
-        <v>5.85</v>
+        <v>5.93</v>
       </c>
       <c r="BQ57" t="n">
-        <v>5.87</v>
+        <v>5.95</v>
       </c>
       <c r="BR57" t="n">
-        <v>6.06</v>
+        <v>6.03</v>
       </c>
       <c r="BS57" t="n">
         <v>0.42</v>
       </c>
       <c r="BT57" t="n">
-        <v>1281513</v>
+        <v>1305155</v>
       </c>
     </row>
     <row r="58">
@@ -14088,7 +14088,7 @@
         <v>25.98</v>
       </c>
       <c r="BO59" t="n">
-        <v>15.73</v>
+        <v>15.82</v>
       </c>
       <c r="BP59" t="n">
         <v>20</v>
@@ -14103,7 +14103,7 @@
         <v>1.42</v>
       </c>
       <c r="BT59" t="n">
-        <v>113</v>
+        <v>103</v>
       </c>
     </row>
     <row r="60">
@@ -14133,10 +14133,10 @@
         </is>
       </c>
       <c r="F60" t="n">
-        <v>376.99</v>
+        <v>373.01</v>
       </c>
       <c r="G60" t="n">
-        <v>171436235</v>
+        <v>169626264</v>
       </c>
       <c r="H60" t="n">
         <v>9</v>
@@ -14154,7 +14154,7 @@
         <v>0.83</v>
       </c>
       <c r="M60" t="n">
-        <v>12.82318904620965</v>
+        <v>12.68780576331641</v>
       </c>
       <c r="N60" t="n">
         <v>0.68</v>
@@ -14232,7 +14232,7 @@
         <v>59558607.5</v>
       </c>
       <c r="AM60" t="n">
-        <v>-25137277.85923754</v>
+        <v>-24871886.2170088</v>
       </c>
       <c r="AN60" t="n">
         <v>10.0581</v>
@@ -14273,7 +14273,7 @@
         <v>944.87</v>
       </c>
       <c r="AZ60" t="n">
-        <v>2167.69</v>
+        <v>2144.81</v>
       </c>
       <c r="BA60" t="n">
         <v>231.1</v>
@@ -14282,19 +14282,19 @@
         <v>727.97</v>
       </c>
       <c r="BC60" t="n">
-        <v>206.96</v>
+        <v>210.24</v>
       </c>
       <c r="BD60" t="n">
-        <v>150.63</v>
+        <v>153.31</v>
       </c>
       <c r="BE60" t="n">
         <v>475</v>
       </c>
       <c r="BF60" t="n">
-        <v>-38.7</v>
+        <v>-38.05</v>
       </c>
       <c r="BG60" t="n">
-        <v>93.09999999999999</v>
+        <v>95.16</v>
       </c>
       <c r="BH60" t="n">
         <v>454.44</v>
@@ -14303,7 +14303,7 @@
         <v>0</v>
       </c>
       <c r="BJ60" t="n">
-        <v>376.99</v>
+        <v>373.01</v>
       </c>
       <c r="BK60" t="n">
         <v>130.97</v>
@@ -14321,19 +14321,19 @@
         <v>306.27</v>
       </c>
       <c r="BP60" t="n">
-        <v>369.01</v>
+        <v>372</v>
       </c>
       <c r="BQ60" t="n">
-        <v>2.88</v>
+        <v>2.85</v>
       </c>
       <c r="BR60" t="n">
-        <v>376.6</v>
+        <v>372</v>
       </c>
       <c r="BS60" t="n">
         <v>12.82</v>
       </c>
       <c r="BT60" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="61">
@@ -14363,13 +14363,13 @@
         </is>
       </c>
       <c r="F61" t="n">
-        <v>26.9</v>
+        <v>27.65</v>
       </c>
       <c r="G61" t="n">
-        <v>2302865120</v>
+        <v>2367072227</v>
       </c>
       <c r="H61" t="n">
-        <v>586000</v>
+        <v>433400</v>
       </c>
       <c r="I61" t="n">
         <v>85608392</v>
@@ -14384,7 +14384,7 @@
         <v>2.37</v>
       </c>
       <c r="M61" t="n">
-        <v>1.221288438700584</v>
+        <v>1.255339672001435</v>
       </c>
       <c r="N61" t="n">
         <v>1.1</v>
@@ -14462,7 +14462,7 @@
         <v>160087693.04</v>
       </c>
       <c r="AM61" t="n">
-        <v>180758643.6420722</v>
+        <v>185798447.9591837</v>
       </c>
       <c r="AN61" t="n">
         <v>0.38</v>
@@ -14503,7 +14503,7 @@
         <v>17.56</v>
       </c>
       <c r="AZ61" t="n">
-        <v>33.89</v>
+        <v>34.84</v>
       </c>
       <c r="BA61" t="n">
         <v>2.52</v>
@@ -14512,19 +14512,19 @@
         <v>11.76</v>
       </c>
       <c r="BC61" t="n">
-        <v>-20.06</v>
+        <v>-22.23</v>
       </c>
       <c r="BD61" t="n">
-        <v>-34.73</v>
+        <v>-36.5</v>
       </c>
       <c r="BE61" t="n">
         <v>26</v>
       </c>
       <c r="BF61" t="n">
-        <v>-90.62</v>
+        <v>-90.88</v>
       </c>
       <c r="BG61" t="n">
-        <v>-56.3</v>
+        <v>-57.48</v>
       </c>
       <c r="BH61" t="n">
         <v>10.99</v>
@@ -14533,7 +14533,7 @@
         <v>0</v>
       </c>
       <c r="BJ61" t="n">
-        <v>26.9</v>
+        <v>27.65</v>
       </c>
       <c r="BK61" t="n">
         <v>1.87</v>
@@ -14542,7 +14542,7 @@
         <v>1.86</v>
       </c>
       <c r="BM61" t="n">
-        <v>27.08</v>
+        <v>27.78</v>
       </c>
       <c r="BN61" t="n">
         <v>28.25</v>
@@ -14551,19 +14551,19 @@
         <v>19.35</v>
       </c>
       <c r="BP61" t="n">
-        <v>25.72</v>
+        <v>26.76</v>
       </c>
       <c r="BQ61" t="n">
-        <v>14.45</v>
+        <v>14.85</v>
       </c>
       <c r="BR61" t="n">
-        <v>25.92</v>
+        <v>26.93</v>
       </c>
       <c r="BS61" t="n">
         <v>1.19</v>
       </c>
       <c r="BT61" t="n">
-        <v>488191</v>
+        <v>500434</v>
       </c>
     </row>
     <row r="62">
@@ -14804,7 +14804,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Bombril SA Preference Shares</t>
+          <t>Bombril S.A Em Recuperacao Judicial Preference Shares</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -14823,13 +14823,13 @@
         </is>
       </c>
       <c r="F63" t="n">
-        <v>1.6</v>
+        <v>1.42</v>
       </c>
       <c r="G63" t="n">
-        <v>416815526</v>
+        <v>369923762</v>
       </c>
       <c r="H63" t="n">
-        <v>149200</v>
+        <v>61000</v>
       </c>
       <c r="I63" t="n">
         <v>122894462</v>
@@ -14844,7 +14844,7 @@
         <v>-0.22</v>
       </c>
       <c r="M63" t="n">
-        <v>0.5126615867486239</v>
+        <v>0.4549871369305478</v>
       </c>
       <c r="N63" t="n">
         <v>0.37</v>
@@ -14922,7 +14922,7 @@
         <v>31952560.12</v>
       </c>
       <c r="AM63" t="n">
-        <v>236827003.4090909</v>
+        <v>210183955.6818182</v>
       </c>
       <c r="AN63" t="n">
         <v>0</v>
@@ -14981,7 +14981,7 @@
         <v>-100</v>
       </c>
       <c r="BF63" t="n">
-        <v>-81.93000000000001</v>
+        <v>-79.64</v>
       </c>
       <c r="BG63" t="n">
         <v>-100</v>
@@ -14993,7 +14993,7 @@
         <v>0</v>
       </c>
       <c r="BJ63" t="n">
-        <v>1.6</v>
+        <v>1.42</v>
       </c>
       <c r="BK63" t="n">
         <v>0.26</v>
@@ -15002,7 +15002,7 @@
         <v>0.26</v>
       </c>
       <c r="BM63" t="n">
-        <v>2.12</v>
+        <v>1.88</v>
       </c>
       <c r="BN63" t="n">
         <v>2.12</v>
@@ -15011,19 +15011,19 @@
         <v>1.16</v>
       </c>
       <c r="BP63" t="n">
-        <v>1.21</v>
+        <v>1.41</v>
       </c>
       <c r="BQ63" t="n">
-        <v>6.13</v>
+        <v>5.44</v>
       </c>
       <c r="BR63" t="n">
-        <v>1.3</v>
+        <v>1.65</v>
       </c>
       <c r="BS63" t="n">
         <v>0.19</v>
       </c>
       <c r="BT63" t="n">
-        <v>15143</v>
+        <v>20063</v>
       </c>
     </row>
     <row r="64">
@@ -15053,13 +15053,13 @@
         </is>
       </c>
       <c r="F64" t="n">
-        <v>60.48</v>
+        <v>60.2</v>
       </c>
       <c r="G64" t="n">
-        <v>230376543536</v>
+        <v>230868267125</v>
       </c>
       <c r="H64" t="n">
-        <v>8470300</v>
+        <v>5207200</v>
       </c>
       <c r="I64" t="n">
         <v>0</v>
@@ -15146,13 +15146,13 @@
         <v>41.22</v>
       </c>
       <c r="AK64" t="n">
-        <v>66052335616.729</v>
+        <v>66193319985.33168</v>
       </c>
       <c r="AL64" t="n">
-        <v>18415391169.94405</v>
+        <v>18454697611.91047</v>
       </c>
       <c r="AM64" t="n">
-        <v>20514384998.75334</v>
+        <v>20558171605.07569</v>
       </c>
       <c r="AN64" t="n">
         <v>1.4201</v>
@@ -15193,7 +15193,7 @@
         <v>38.98</v>
       </c>
       <c r="AZ64" t="n">
-        <v>24.19</v>
+        <v>24.08</v>
       </c>
       <c r="BA64" t="n">
         <v>6.69</v>
@@ -15202,19 +15202,19 @@
         <v>10.4</v>
       </c>
       <c r="BC64" t="n">
-        <v>-21.06</v>
+        <v>-20.7</v>
       </c>
       <c r="BD64" t="n">
-        <v>-35.55</v>
+        <v>-35.25</v>
       </c>
       <c r="BE64" t="n">
         <v>-60</v>
       </c>
       <c r="BF64" t="n">
-        <v>-88.93000000000001</v>
+        <v>-88.88</v>
       </c>
       <c r="BG64" t="n">
-        <v>-82.81</v>
+        <v>-82.73</v>
       </c>
       <c r="BH64" t="n">
         <v>21.37</v>
@@ -15223,7 +15223,7 @@
         <v>0</v>
       </c>
       <c r="BJ64" t="n">
-        <v>60.48</v>
+        <v>60.2</v>
       </c>
       <c r="BK64" t="n">
         <v>4.74</v>
@@ -15232,7 +15232,7 @@
         <v>1.57</v>
       </c>
       <c r="BM64" t="n">
-        <v>61</v>
+        <v>60.98</v>
       </c>
       <c r="BN64" t="n">
         <v>64.72</v>
@@ -15241,19 +15241,19 @@
         <v>44.12</v>
       </c>
       <c r="BP64" t="n">
-        <v>59.09</v>
+        <v>60.06</v>
       </c>
       <c r="BQ64" t="n">
-        <v>38.52</v>
+        <v>38.34</v>
       </c>
       <c r="BR64" t="n">
-        <v>59.12</v>
+        <v>60.98</v>
       </c>
       <c r="BS64" t="n">
         <v>3.49</v>
       </c>
       <c r="BT64" t="n">
-        <v>12354237</v>
+        <v>12462611</v>
       </c>
     </row>
     <row r="65">
@@ -15283,13 +15283,13 @@
         </is>
       </c>
       <c r="F65" t="n">
-        <v>23.56</v>
+        <v>23.55</v>
       </c>
       <c r="G65" t="n">
-        <v>230376543536</v>
+        <v>230868267125</v>
       </c>
       <c r="H65" t="n">
-        <v>8200</v>
+        <v>5700</v>
       </c>
       <c r="I65" t="n">
         <v>7298813414</v>
@@ -15304,7 +15304,7 @@
         <v>3.29</v>
       </c>
       <c r="M65" t="n">
-        <v>5.569570157856582</v>
+        <v>5.58145803925793</v>
       </c>
       <c r="N65" t="n">
         <v>0.29</v>
@@ -15382,7 +15382,7 @@
         <v>11532125194.12</v>
       </c>
       <c r="AM65" t="n">
-        <v>17256669927.79026</v>
+        <v>17293503155.43071</v>
       </c>
       <c r="AN65" t="n">
         <v>0.4734</v>
@@ -15432,10 +15432,10 @@
         <v>3.47</v>
       </c>
       <c r="BC65" t="n">
-        <v>-32.47</v>
+        <v>-32.44</v>
       </c>
       <c r="BD65" t="n">
-        <v>-44.86</v>
+        <v>-44.84</v>
       </c>
       <c r="BE65" t="n">
         <v>-66.33</v>
@@ -15444,7 +15444,7 @@
         <v>-90.53</v>
       </c>
       <c r="BG65" t="n">
-        <v>-85.29000000000001</v>
+        <v>-85.28</v>
       </c>
       <c r="BH65" t="n">
         <v>7.12</v>
@@ -15453,7 +15453,7 @@
         <v>0</v>
       </c>
       <c r="BJ65" t="n">
-        <v>23.56</v>
+        <v>23.55</v>
       </c>
       <c r="BK65" t="n">
         <v>1.58</v>
@@ -15462,7 +15462,7 @@
         <v>1.57</v>
       </c>
       <c r="BM65" t="n">
-        <v>23.69</v>
+        <v>23.9</v>
       </c>
       <c r="BN65" t="n">
         <v>46.43</v>
@@ -15471,19 +15471,19 @@
         <v>20.44</v>
       </c>
       <c r="BP65" t="n">
-        <v>23.41</v>
+        <v>23.55</v>
       </c>
       <c r="BQ65" t="n">
-        <v>15.01</v>
+        <v>15</v>
       </c>
       <c r="BR65" t="n">
-        <v>23.69</v>
+        <v>23.89</v>
       </c>
       <c r="BS65" t="n">
         <v>4.14</v>
       </c>
       <c r="BT65" t="n">
-        <v>12007</v>
+        <v>12089</v>
       </c>
     </row>
     <row r="66">
@@ -15973,13 +15973,13 @@
         </is>
       </c>
       <c r="F68" t="n">
-        <v>18.78</v>
+        <v>18.7</v>
       </c>
       <c r="G68" t="n">
-        <v>8068099400</v>
+        <v>8051979740</v>
       </c>
       <c r="H68" t="n">
-        <v>64300</v>
+        <v>44000</v>
       </c>
       <c r="I68" t="n">
         <v>137989898</v>
@@ -16072,7 +16072,7 @@
         <v>205604948.02</v>
       </c>
       <c r="AM68" t="n">
-        <v>559507586.6851594</v>
+        <v>558389718.446602</v>
       </c>
       <c r="AN68" t="n">
         <v>0.1911</v>
@@ -16113,7 +16113,7 @@
         <v>21.39</v>
       </c>
       <c r="AZ68" t="n">
-        <v>34.74</v>
+        <v>34.6</v>
       </c>
       <c r="BA68" t="n">
         <v>1.24</v>
@@ -16122,19 +16122,19 @@
         <v>63.25</v>
       </c>
       <c r="BC68" t="n">
-        <v>39.53</v>
+        <v>40.12</v>
       </c>
       <c r="BD68" t="n">
-        <v>13.92</v>
+        <v>14.41</v>
       </c>
       <c r="BE68" t="n">
         <v>85</v>
       </c>
       <c r="BF68" t="n">
-        <v>-93.40000000000001</v>
+        <v>-93.37</v>
       </c>
       <c r="BG68" t="n">
-        <v>236.79</v>
+        <v>238.23</v>
       </c>
       <c r="BH68" t="n">
         <v>20.48</v>
@@ -16143,7 +16143,7 @@
         <v>0</v>
       </c>
       <c r="BJ68" t="n">
-        <v>18.78</v>
+        <v>18.7</v>
       </c>
       <c r="BK68" t="n">
         <v>1.49</v>
@@ -16152,7 +16152,7 @@
         <v>1.49</v>
       </c>
       <c r="BM68" t="n">
-        <v>19.43</v>
+        <v>18.84</v>
       </c>
       <c r="BN68" t="n">
         <v>22.11</v>
@@ -16161,19 +16161,19 @@
         <v>15.07</v>
       </c>
       <c r="BP68" t="n">
-        <v>18.78</v>
+        <v>18.58</v>
       </c>
       <c r="BQ68" t="n">
-        <v>12.63</v>
+        <v>12.58</v>
       </c>
       <c r="BR68" t="n">
-        <v>19.43</v>
+        <v>18.82</v>
       </c>
       <c r="BS68" t="n">
         <v>0</v>
       </c>
       <c r="BT68" t="n">
-        <v>32337</v>
+        <v>32470</v>
       </c>
     </row>
     <row r="69">
@@ -16203,13 +16203,13 @@
         </is>
       </c>
       <c r="F69" t="n">
-        <v>21.64</v>
+        <v>21.48</v>
       </c>
       <c r="G69" t="n">
-        <v>8068099400</v>
+        <v>8051979740</v>
       </c>
       <c r="H69" t="n">
-        <v>1983400</v>
+        <v>1004500</v>
       </c>
       <c r="I69" t="n">
         <v>255106712</v>
@@ -16302,7 +16302,7 @@
         <v>380109000.88</v>
       </c>
       <c r="AM69" t="n">
-        <v>480244011.9047619</v>
+        <v>479284508.3333333</v>
       </c>
       <c r="AN69" t="n">
         <v>0.8856000000000001</v>
@@ -16343,7 +16343,7 @@
         <v>21.39</v>
       </c>
       <c r="AZ69" t="n">
-        <v>37.83</v>
+        <v>37.55</v>
       </c>
       <c r="BA69" t="n">
         <v>1.24</v>
@@ -16352,19 +16352,19 @@
         <v>69.59</v>
       </c>
       <c r="BC69" t="n">
-        <v>21.09</v>
+        <v>21.99</v>
       </c>
       <c r="BD69" t="n">
-        <v>-1.13</v>
+        <v>-0.4</v>
       </c>
       <c r="BE69" t="n">
         <v>74.83</v>
       </c>
       <c r="BF69" t="n">
-        <v>-94.27</v>
+        <v>-94.23</v>
       </c>
       <c r="BG69" t="n">
-        <v>221.57</v>
+        <v>223.96</v>
       </c>
       <c r="BH69" t="n">
         <v>20.48</v>
@@ -16373,7 +16373,7 @@
         <v>0</v>
       </c>
       <c r="BJ69" t="n">
-        <v>21.64</v>
+        <v>21.48</v>
       </c>
       <c r="BK69" t="n">
         <v>1.49</v>
@@ -16382,7 +16382,7 @@
         <v>1.49</v>
       </c>
       <c r="BM69" t="n">
-        <v>22.15</v>
+        <v>21.8</v>
       </c>
       <c r="BN69" t="n">
         <v>25.63</v>
@@ -16391,19 +16391,19 @@
         <v>16.73</v>
       </c>
       <c r="BP69" t="n">
-        <v>21.64</v>
+        <v>21.36</v>
       </c>
       <c r="BQ69" t="n">
-        <v>14.56</v>
+        <v>14.45</v>
       </c>
       <c r="BR69" t="n">
-        <v>22</v>
+        <v>21.8</v>
       </c>
       <c r="BS69" t="n">
         <v>0</v>
       </c>
       <c r="BT69" t="n">
-        <v>1923390</v>
+        <v>1934300</v>
       </c>
     </row>
     <row r="70">
@@ -16433,13 +16433,13 @@
         </is>
       </c>
       <c r="F70" t="n">
-        <v>17.75</v>
+        <v>17.91</v>
       </c>
       <c r="G70" t="n">
-        <v>8245890300</v>
+        <v>8320219381</v>
       </c>
       <c r="H70" t="n">
-        <v>4184800</v>
+        <v>2729900</v>
       </c>
       <c r="I70" t="n">
         <v>464557268</v>
@@ -16454,7 +16454,7 @@
         <v>0.68</v>
       </c>
       <c r="M70" t="n">
-        <v>0.6508332380670019</v>
+        <v>0.656699898271028</v>
       </c>
       <c r="N70" t="n">
         <v>0.2</v>
@@ -16532,7 +16532,7 @@
         <v>55746872.16</v>
       </c>
       <c r="AM70" t="n">
-        <v>2721415940.594059</v>
+        <v>2745946990.429043</v>
       </c>
       <c r="AN70" t="n">
         <v>0.1236</v>
@@ -16573,7 +16573,7 @@
         <v>6.9</v>
       </c>
       <c r="AZ70" t="n">
-        <v>2.04</v>
+        <v>2.06</v>
       </c>
       <c r="BA70" t="n">
         <v>0.12</v>
@@ -16582,19 +16582,19 @@
         <v>1.07</v>
       </c>
       <c r="BC70" t="n">
-        <v>-52.4</v>
+        <v>-52.82</v>
       </c>
       <c r="BD70" t="n">
-        <v>-61.13</v>
+        <v>-61.48</v>
       </c>
       <c r="BE70" t="n">
         <v>-88.5</v>
       </c>
       <c r="BF70" t="n">
-        <v>-99.31999999999999</v>
+        <v>-99.33</v>
       </c>
       <c r="BG70" t="n">
-        <v>-93.97</v>
+        <v>-94.03</v>
       </c>
       <c r="BH70" t="n">
         <v>26.44</v>
@@ -16603,7 +16603,7 @@
         <v>0</v>
       </c>
       <c r="BJ70" t="n">
-        <v>17.75</v>
+        <v>17.91</v>
       </c>
       <c r="BK70" t="n">
         <v>0.12</v>
@@ -16612,7 +16612,7 @@
         <v>0.1</v>
       </c>
       <c r="BM70" t="n">
-        <v>18.6</v>
+        <v>18.1</v>
       </c>
       <c r="BN70" t="n">
         <v>22.15</v>
@@ -16621,19 +16621,19 @@
         <v>13.21</v>
       </c>
       <c r="BP70" t="n">
-        <v>17.72</v>
+        <v>17.57</v>
       </c>
       <c r="BQ70" t="n">
-        <v>178.02</v>
+        <v>179.62</v>
       </c>
       <c r="BR70" t="n">
-        <v>18.45</v>
+        <v>17.71</v>
       </c>
       <c r="BS70" t="n">
         <v>0.67</v>
       </c>
       <c r="BT70" t="n">
-        <v>5779190</v>
+        <v>5622153</v>
       </c>
     </row>
     <row r="71">

</xml_diff>

<commit_message>
📊 Dados atualizados - 2026-09-17 05:39
</commit_message>
<xml_diff>
--- a/data/ativos.xlsx
+++ b/data/ativos.xlsx
@@ -1047,13 +1047,13 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>24.69</v>
+        <v>24.66</v>
       </c>
       <c r="G3" t="n">
-        <v>3302704832</v>
+        <v>3299651007</v>
       </c>
       <c r="H3" t="n">
-        <v>410100</v>
+        <v>488500</v>
       </c>
       <c r="I3" t="n">
         <v>129510368</v>
@@ -1068,7 +1068,7 @@
         <v>0.88</v>
       </c>
       <c r="M3" t="n">
-        <v>0.8217865181387306</v>
+        <v>0.8210266584657016</v>
       </c>
       <c r="N3" t="n">
         <v>0.09</v>
@@ -1146,7 +1146,7 @@
         <v>506385538.88</v>
       </c>
       <c r="AM3" t="n">
-        <v>645059537.5</v>
+        <v>644463087.3046875</v>
       </c>
       <c r="AN3" t="n">
         <v>2.7</v>
@@ -1187,7 +1187,7 @@
         <v>40.42</v>
       </c>
       <c r="AZ3" t="n">
-        <v>45.18</v>
+        <v>45.13</v>
       </c>
       <c r="BA3" t="n">
         <v>4.87</v>
@@ -1196,19 +1196,19 @@
         <v>21.14</v>
       </c>
       <c r="BC3" t="n">
-        <v>100.48</v>
+        <v>100.72</v>
       </c>
       <c r="BD3" t="n">
-        <v>63.69</v>
+        <v>63.89</v>
       </c>
       <c r="BE3" t="n">
         <v>83</v>
       </c>
       <c r="BF3" t="n">
-        <v>-80.28</v>
+        <v>-80.26000000000001</v>
       </c>
       <c r="BG3" t="n">
-        <v>-14.4</v>
+        <v>-14.29</v>
       </c>
       <c r="BH3" t="n">
         <v>27.85</v>
@@ -1217,7 +1217,7 @@
         <v>0</v>
       </c>
       <c r="BJ3" t="n">
-        <v>24.69</v>
+        <v>24.66</v>
       </c>
       <c r="BK3" t="n">
         <v>3.91</v>
@@ -1226,7 +1226,7 @@
         <v>4.39</v>
       </c>
       <c r="BM3" t="n">
-        <v>25.05</v>
+        <v>24.8</v>
       </c>
       <c r="BN3" t="n">
         <v>27.17</v>
@@ -1235,19 +1235,19 @@
         <v>18.72</v>
       </c>
       <c r="BP3" t="n">
-        <v>24.53</v>
+        <v>24.34</v>
       </c>
       <c r="BQ3" t="n">
-        <v>5.62</v>
+        <v>5.61</v>
       </c>
       <c r="BR3" t="n">
-        <v>25.02</v>
+        <v>24.74</v>
       </c>
       <c r="BS3" t="n">
         <v>0.79</v>
       </c>
       <c r="BT3" t="n">
-        <v>531937</v>
+        <v>527580</v>
       </c>
     </row>
     <row r="4">
@@ -1277,13 +1277,13 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>15.73</v>
+        <v>15.63</v>
       </c>
       <c r="G4" t="n">
-        <v>243573694711</v>
+        <v>242095728872</v>
       </c>
       <c r="H4" t="n">
-        <v>20798700</v>
+        <v>32094600</v>
       </c>
       <c r="I4" t="n">
         <v>15484664889</v>
@@ -1298,7 +1298,7 @@
         <v>2.76</v>
       </c>
       <c r="M4" t="n">
-        <v>2.75799238227837</v>
+        <v>2.741257329956459</v>
       </c>
       <c r="N4" t="n">
         <v>1.76</v>
@@ -1376,7 +1376,7 @@
         <v>16258898133.45</v>
       </c>
       <c r="AM4" t="n">
-        <v>24116207397.12872</v>
+        <v>23969874145.74258</v>
       </c>
       <c r="AN4" t="n">
         <v>0.269</v>
@@ -1417,7 +1417,7 @@
         <v>9.470000000000001</v>
       </c>
       <c r="AZ4" t="n">
-        <v>19.64</v>
+        <v>19.51</v>
       </c>
       <c r="BA4" t="n">
         <v>1.13</v>
@@ -1426,19 +1426,19 @@
         <v>11.39</v>
       </c>
       <c r="BC4" t="n">
-        <v>-26.23</v>
+        <v>-25.76</v>
       </c>
       <c r="BD4" t="n">
-        <v>-39.76</v>
+        <v>-39.38</v>
       </c>
       <c r="BE4" t="n">
         <v>24.83</v>
       </c>
       <c r="BF4" t="n">
-        <v>-92.83</v>
+        <v>-92.79000000000001</v>
       </c>
       <c r="BG4" t="n">
-        <v>-27.61</v>
+        <v>-27.15</v>
       </c>
       <c r="BH4" t="n">
         <v>5.7</v>
@@ -1447,7 +1447,7 @@
         <v>0</v>
       </c>
       <c r="BJ4" t="n">
-        <v>15.73</v>
+        <v>15.63</v>
       </c>
       <c r="BK4" t="n">
         <v>1.05</v>
@@ -1456,7 +1456,7 @@
         <v>1.04</v>
       </c>
       <c r="BM4" t="n">
-        <v>15.95</v>
+        <v>15.77</v>
       </c>
       <c r="BN4" t="n">
         <v>17</v>
@@ -1465,19 +1465,19 @@
         <v>11.09</v>
       </c>
       <c r="BP4" t="n">
-        <v>15.71</v>
+        <v>15.52</v>
       </c>
       <c r="BQ4" t="n">
-        <v>15.17</v>
+        <v>15.07</v>
       </c>
       <c r="BR4" t="n">
-        <v>15.95</v>
+        <v>15.7</v>
       </c>
       <c r="BS4" t="n">
         <v>2.76</v>
       </c>
       <c r="BT4" t="n">
-        <v>28658427</v>
+        <v>28204413</v>
       </c>
     </row>
     <row r="5">
@@ -1743,7 +1743,7 @@
         <v>461779941</v>
       </c>
       <c r="H6" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I6" t="n">
         <v>63084700</v>
@@ -3117,13 +3117,13 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>5.05</v>
+        <v>5.13</v>
       </c>
       <c r="G12" t="n">
-        <v>484605795</v>
+        <v>492426043</v>
       </c>
       <c r="H12" t="n">
-        <v>260900</v>
+        <v>526500</v>
       </c>
       <c r="I12" t="n">
         <v>95961536</v>
@@ -3138,7 +3138,7 @@
         <v>0.32</v>
       </c>
       <c r="M12" t="n">
-        <v>0.08764021854862333</v>
+        <v>0.08905449846623026</v>
       </c>
       <c r="N12" t="n">
         <v>0.14</v>
@@ -3216,7 +3216,7 @@
         <v>362734606.08</v>
       </c>
       <c r="AM12" t="n">
-        <v>521081500</v>
+        <v>529490368.8172043</v>
       </c>
       <c r="AN12" t="n">
         <v>0.4208</v>
@@ -3257,7 +3257,7 @@
         <v>30.49</v>
       </c>
       <c r="AZ12" t="n">
-        <v>6.83</v>
+        <v>6.93</v>
       </c>
       <c r="BA12" t="n">
         <v>4.41</v>
@@ -3266,19 +3266,19 @@
         <v>18.12</v>
       </c>
       <c r="BC12" t="n">
-        <v>639.55</v>
+        <v>628.02</v>
       </c>
       <c r="BD12" t="n">
-        <v>503.84</v>
+        <v>494.42</v>
       </c>
       <c r="BE12" t="n">
         <v>35.17</v>
       </c>
       <c r="BF12" t="n">
-        <v>-12.64</v>
+        <v>-14</v>
       </c>
       <c r="BG12" t="n">
-        <v>258.79</v>
+        <v>253.19</v>
       </c>
       <c r="BH12" t="n">
         <v>16.4</v>
@@ -3287,7 +3287,7 @@
         <v>0</v>
       </c>
       <c r="BJ12" t="n">
-        <v>5.05</v>
+        <v>5.13</v>
       </c>
       <c r="BK12" t="n">
         <v>3.78</v>
@@ -3296,7 +3296,7 @@
         <v>3.43</v>
       </c>
       <c r="BM12" t="n">
-        <v>5.1</v>
+        <v>5.13</v>
       </c>
       <c r="BN12" t="n">
         <v>8.23</v>
@@ -3305,19 +3305,19 @@
         <v>4.42</v>
       </c>
       <c r="BP12" t="n">
-        <v>5.04</v>
+        <v>5.03</v>
       </c>
       <c r="BQ12" t="n">
-        <v>1.47</v>
+        <v>1.5</v>
       </c>
       <c r="BR12" t="n">
-        <v>5.05</v>
+        <v>5.06</v>
       </c>
       <c r="BS12" t="n">
         <v>0.09</v>
       </c>
       <c r="BT12" t="n">
-        <v>497557</v>
+        <v>495810</v>
       </c>
     </row>
     <row r="13">
@@ -3347,13 +3347,13 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>28.53</v>
+        <v>28.46</v>
       </c>
       <c r="G13" t="n">
-        <v>14384566723</v>
+        <v>14353453326</v>
       </c>
       <c r="H13" t="n">
-        <v>2870100</v>
+        <v>9049300</v>
       </c>
       <c r="I13" t="n">
         <v>504190947</v>
@@ -3368,7 +3368,7 @@
         <v>1.13</v>
       </c>
       <c r="M13" t="n">
-        <v>4.975014791037738</v>
+        <v>4.964253979589248</v>
       </c>
       <c r="N13" t="n">
         <v>0.57</v>
@@ -3446,7 +3446,7 @@
         <v>932753251.95</v>
       </c>
       <c r="AM13" t="n">
-        <v>1496833165.764828</v>
+        <v>1493595559.417274</v>
       </c>
       <c r="AN13" t="n">
         <v>2.6301</v>
@@ -3487,7 +3487,7 @@
         <v>26.6</v>
       </c>
       <c r="AZ13" t="n">
-        <v>51.64</v>
+        <v>51.51</v>
       </c>
       <c r="BA13" t="n">
         <v>2.6</v>
@@ -3496,19 +3496,19 @@
         <v>8.69</v>
       </c>
       <c r="BC13" t="n">
-        <v>14.17</v>
+        <v>14.45</v>
       </c>
       <c r="BD13" t="n">
-        <v>-6.78</v>
+        <v>-6.55</v>
       </c>
       <c r="BE13" t="n">
         <v>81</v>
       </c>
       <c r="BF13" t="n">
-        <v>-90.87</v>
+        <v>-90.84999999999999</v>
       </c>
       <c r="BG13" t="n">
-        <v>-69.53</v>
+        <v>-69.45</v>
       </c>
       <c r="BH13" t="n">
         <v>25.49</v>
@@ -3517,7 +3517,7 @@
         <v>0</v>
       </c>
       <c r="BJ13" t="n">
-        <v>28.53</v>
+        <v>28.46</v>
       </c>
       <c r="BK13" t="n">
         <v>1.85</v>
@@ -3526,7 +3526,7 @@
         <v>1.96</v>
       </c>
       <c r="BM13" t="n">
-        <v>28.67</v>
+        <v>28.82</v>
       </c>
       <c r="BN13" t="n">
         <v>32.43</v>
@@ -3535,19 +3535,19 @@
         <v>21.06</v>
       </c>
       <c r="BP13" t="n">
-        <v>28.25</v>
+        <v>28.4</v>
       </c>
       <c r="BQ13" t="n">
-        <v>14.58</v>
+        <v>14.54</v>
       </c>
       <c r="BR13" t="n">
-        <v>28.51</v>
+        <v>28.53</v>
       </c>
       <c r="BS13" t="n">
         <v>5.01</v>
       </c>
       <c r="BT13" t="n">
-        <v>4629999</v>
+        <v>4510147</v>
       </c>
     </row>
     <row r="14">
@@ -3577,13 +3577,13 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>9.77</v>
+        <v>9.6</v>
       </c>
       <c r="G14" t="n">
-        <v>7816145214</v>
+        <v>7925797696</v>
       </c>
       <c r="H14" t="n">
-        <v>3600</v>
+        <v>16800</v>
       </c>
       <c r="I14" t="n">
         <v>339510689</v>
@@ -3598,7 +3598,7 @@
         <v>1.92</v>
       </c>
       <c r="M14" t="n">
-        <v>3.245402445809384</v>
+        <v>3.290932105702915</v>
       </c>
       <c r="N14" t="n">
         <v>1.11</v>
@@ -3676,7 +3676,7 @@
         <v>349696009.67</v>
       </c>
       <c r="AM14" t="n">
-        <v>867496694.1176471</v>
+        <v>879666780.9100999</v>
       </c>
       <c r="AN14" t="n">
         <v>0.1489</v>
@@ -3717,7 +3717,7 @@
         <v>9.050000000000001</v>
       </c>
       <c r="AZ14" t="n">
-        <v>7.85</v>
+        <v>7.71</v>
       </c>
       <c r="BA14" t="n">
         <v>1.42</v>
@@ -3726,19 +3726,19 @@
         <v>5.94</v>
       </c>
       <c r="BC14" t="n">
-        <v>13.44</v>
+        <v>15.45</v>
       </c>
       <c r="BD14" t="n">
-        <v>-7.38</v>
+        <v>-5.74</v>
       </c>
       <c r="BE14" t="n">
         <v>-19.67</v>
       </c>
       <c r="BF14" t="n">
-        <v>-85.45</v>
+        <v>-85.2</v>
       </c>
       <c r="BG14" t="n">
-        <v>-39.18</v>
+        <v>-38.1</v>
       </c>
       <c r="BH14" t="n">
         <v>5.3</v>
@@ -3747,7 +3747,7 @@
         <v>0</v>
       </c>
       <c r="BJ14" t="n">
-        <v>9.77</v>
+        <v>9.6</v>
       </c>
       <c r="BK14" t="n">
         <v>1.03</v>
@@ -3765,19 +3765,19 @@
         <v>7.65</v>
       </c>
       <c r="BP14" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="BQ14" t="n">
+        <v>9.48</v>
+      </c>
+      <c r="BR14" t="n">
         <v>9.77</v>
-      </c>
-      <c r="BQ14" t="n">
-        <v>9.65</v>
-      </c>
-      <c r="BR14" t="n">
-        <v>9.789999999999999</v>
       </c>
       <c r="BS14" t="n">
         <v>1.44</v>
       </c>
       <c r="BT14" t="n">
-        <v>12717</v>
+        <v>12590</v>
       </c>
     </row>
     <row r="15">
@@ -3807,13 +3807,13 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>12.99</v>
+        <v>13.23</v>
       </c>
       <c r="G15" t="n">
-        <v>7816145214</v>
+        <v>7925797696</v>
       </c>
       <c r="H15" t="n">
-        <v>667800</v>
+        <v>2706900</v>
       </c>
       <c r="I15" t="n">
         <v>343551533</v>
@@ -3828,7 +3828,7 @@
         <v>2.56</v>
       </c>
       <c r="M15" t="n">
-        <v>3.207230108500284</v>
+        <v>3.252224249744266</v>
       </c>
       <c r="N15" t="n">
         <v>1.47</v>
@@ -3906,7 +3906,7 @@
         <v>353858078.99</v>
       </c>
       <c r="AM15" t="n">
-        <v>651888675.0625521</v>
+        <v>661034003.0025021</v>
       </c>
       <c r="AN15" t="n">
         <v>0.1638</v>
@@ -3947,7 +3947,7 @@
         <v>9.050000000000001</v>
       </c>
       <c r="AZ15" t="n">
-        <v>8.640000000000001</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="BA15" t="n">
         <v>1.42</v>
@@ -3956,19 +3956,19 @@
         <v>6.19</v>
       </c>
       <c r="BC15" t="n">
-        <v>-14.68</v>
+        <v>-16.23</v>
       </c>
       <c r="BD15" t="n">
-        <v>-30.34</v>
+        <v>-31.6</v>
       </c>
       <c r="BE15" t="n">
         <v>-33.5</v>
       </c>
       <c r="BF15" t="n">
-        <v>-89.06</v>
+        <v>-89.26000000000001</v>
       </c>
       <c r="BG15" t="n">
-        <v>-52.36</v>
+        <v>-53.22</v>
       </c>
       <c r="BH15" t="n">
         <v>5.3</v>
@@ -3977,7 +3977,7 @@
         <v>0</v>
       </c>
       <c r="BJ15" t="n">
-        <v>12.99</v>
+        <v>13.23</v>
       </c>
       <c r="BK15" t="n">
         <v>1.03</v>
@@ -3986,7 +3986,7 @@
         <v>1.01</v>
       </c>
       <c r="BM15" t="n">
-        <v>13.23</v>
+        <v>13.35</v>
       </c>
       <c r="BN15" t="n">
         <v>16.22</v>
@@ -3995,19 +3995,19 @@
         <v>7.84</v>
       </c>
       <c r="BP15" t="n">
-        <v>12.98</v>
+        <v>12.97</v>
       </c>
       <c r="BQ15" t="n">
-        <v>12.82</v>
+        <v>13.06</v>
       </c>
       <c r="BR15" t="n">
-        <v>13.04</v>
+        <v>13.01</v>
       </c>
       <c r="BS15" t="n">
         <v>1.92</v>
       </c>
       <c r="BT15" t="n">
-        <v>2361563</v>
+        <v>2332907</v>
       </c>
     </row>
     <row r="16">
@@ -4037,13 +4037,13 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>4.25</v>
+        <v>4.22</v>
       </c>
       <c r="G16" t="n">
-        <v>932049225</v>
+        <v>925739665</v>
       </c>
       <c r="H16" t="n">
-        <v>222400</v>
+        <v>68800</v>
       </c>
       <c r="I16" t="n">
         <v>219305733</v>
@@ -4058,7 +4058,7 @@
         <v>2.69</v>
       </c>
       <c r="M16" t="n">
-        <v>0.4409374336499903</v>
+        <v>0.4379524827276175</v>
       </c>
       <c r="N16" t="n">
         <v>0.39</v>
@@ -4136,7 +4136,7 @@
         <v>17544458.64</v>
       </c>
       <c r="AM16" t="n">
-        <v>261811580.0561798</v>
+        <v>260039231.741573</v>
       </c>
       <c r="AN16" t="n">
         <v>0.0077</v>
@@ -4186,16 +4186,16 @@
         <v>0</v>
       </c>
       <c r="BC16" t="n">
-        <v>-59.08</v>
+        <v>-58.79</v>
       </c>
       <c r="BD16" t="n">
-        <v>-66.59</v>
+        <v>-66.34999999999999</v>
       </c>
       <c r="BE16" t="n">
         <v>-97.17</v>
       </c>
       <c r="BF16" t="n">
-        <v>-98.12</v>
+        <v>-98.09999999999999</v>
       </c>
       <c r="BG16" t="n">
         <v>-100</v>
@@ -4207,7 +4207,7 @@
         <v>0</v>
       </c>
       <c r="BJ16" t="n">
-        <v>4.25</v>
+        <v>4.22</v>
       </c>
       <c r="BK16" t="n">
         <v>0.08</v>
@@ -4216,28 +4216,28 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="BM16" t="n">
-        <v>4.35</v>
+        <v>4.3</v>
       </c>
       <c r="BN16" t="n">
         <v>5.54</v>
       </c>
       <c r="BO16" t="n">
-        <v>3.08</v>
+        <v>3.1</v>
       </c>
       <c r="BP16" t="n">
-        <v>4.13</v>
+        <v>4.17</v>
       </c>
       <c r="BQ16" t="n">
-        <v>58</v>
+        <v>57.59</v>
       </c>
       <c r="BR16" t="n">
-        <v>4.32</v>
+        <v>4.26</v>
       </c>
       <c r="BS16" t="n">
         <v>0.49</v>
       </c>
       <c r="BT16" t="n">
-        <v>139897</v>
+        <v>145277</v>
       </c>
     </row>
     <row r="17">
@@ -4267,13 +4267,13 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>33.41</v>
+        <v>32.97</v>
       </c>
       <c r="G17" t="n">
-        <v>11012834678</v>
+        <v>10870961118</v>
       </c>
       <c r="H17" t="n">
-        <v>529900</v>
+        <v>1773100</v>
       </c>
       <c r="I17" t="n">
         <v>0</v>
@@ -4360,13 +4360,13 @@
         <v>8.039999999999999</v>
       </c>
       <c r="AK17" t="n">
-        <v>4973281556.177746</v>
+        <v>4909212932.622832</v>
       </c>
       <c r="AL17" t="n">
-        <v>1376604334.75</v>
+        <v>1358870139.75</v>
       </c>
       <c r="AM17" t="n">
-        <v>3409546339.93808</v>
+        <v>3365622637.151703</v>
       </c>
       <c r="AN17" t="n">
         <v>1.08</v>
@@ -4407,7 +4407,7 @@
         <v>42.98</v>
       </c>
       <c r="AZ17" t="n">
-        <v>17.87</v>
+        <v>17.64</v>
       </c>
       <c r="BA17" t="n">
         <v>4.55</v>
@@ -4416,19 +4416,19 @@
         <v>16.33</v>
       </c>
       <c r="BC17" t="n">
-        <v>57.55</v>
+        <v>59.65</v>
       </c>
       <c r="BD17" t="n">
-        <v>28.64</v>
+        <v>30.36</v>
       </c>
       <c r="BE17" t="n">
         <v>-46.5</v>
       </c>
       <c r="BF17" t="n">
-        <v>-86.39</v>
+        <v>-86.2</v>
       </c>
       <c r="BG17" t="n">
-        <v>-51.11</v>
+        <v>-50.46</v>
       </c>
       <c r="BH17" t="n">
         <v>29.25</v>
@@ -4437,7 +4437,7 @@
         <v>0</v>
       </c>
       <c r="BJ17" t="n">
-        <v>33.41</v>
+        <v>32.97</v>
       </c>
       <c r="BK17" t="n">
         <v>4.21</v>
@@ -4446,7 +4446,7 @@
         <v>12.62</v>
       </c>
       <c r="BM17" t="n">
-        <v>33.61</v>
+        <v>33.4</v>
       </c>
       <c r="BN17" t="n">
         <v>36.63</v>
@@ -4455,19 +4455,19 @@
         <v>29.28</v>
       </c>
       <c r="BP17" t="n">
-        <v>33.33</v>
+        <v>32.9</v>
       </c>
       <c r="BQ17" t="n">
-        <v>2.65</v>
+        <v>2.61</v>
       </c>
       <c r="BR17" t="n">
-        <v>33.44</v>
+        <v>33.37</v>
       </c>
       <c r="BS17" t="n">
         <v>2.21</v>
       </c>
       <c r="BT17" t="n">
-        <v>1076550</v>
+        <v>1070251</v>
       </c>
     </row>
     <row r="18">
@@ -4497,13 +4497,13 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>11.7</v>
+        <v>11.35</v>
       </c>
       <c r="G18" t="n">
-        <v>11012834678</v>
+        <v>10870961118</v>
       </c>
       <c r="H18" t="n">
-        <v>1500</v>
+        <v>10600</v>
       </c>
       <c r="I18" t="n">
         <v>671494278</v>
@@ -4518,7 +4518,7 @@
         <v>1.2</v>
       </c>
       <c r="M18" t="n">
-        <v>3.242611014550277</v>
+        <v>3.200837866965625</v>
       </c>
       <c r="N18" t="n">
         <v>0.33</v>
@@ -4596,7 +4596,7 @@
         <v>940091989.1999999</v>
       </c>
       <c r="AM18" t="n">
-        <v>3277629368.452381</v>
+        <v>3235405094.642857</v>
       </c>
       <c r="AN18" t="n">
         <v>0.36</v>
@@ -4637,7 +4637,7 @@
         <v>14.31</v>
       </c>
       <c r="AZ18" t="n">
-        <v>6.03</v>
+        <v>5.85</v>
       </c>
       <c r="BA18" t="n">
         <v>1.51</v>
@@ -4646,19 +4646,19 @@
         <v>5.44</v>
       </c>
       <c r="BC18" t="n">
-        <v>49.79</v>
+        <v>54.41</v>
       </c>
       <c r="BD18" t="n">
-        <v>22.3</v>
+        <v>26.07</v>
       </c>
       <c r="BE18" t="n">
         <v>-48.5</v>
       </c>
       <c r="BF18" t="n">
-        <v>-87.06999999999999</v>
+        <v>-86.67</v>
       </c>
       <c r="BG18" t="n">
-        <v>-53.47</v>
+        <v>-52.03</v>
       </c>
       <c r="BH18" t="n">
         <v>9.75</v>
@@ -4667,7 +4667,7 @@
         <v>0</v>
       </c>
       <c r="BJ18" t="n">
-        <v>11.7</v>
+        <v>11.35</v>
       </c>
       <c r="BK18" t="n">
         <v>1.4</v>
@@ -4676,7 +4676,7 @@
         <v>12.62</v>
       </c>
       <c r="BM18" t="n">
-        <v>11.89</v>
+        <v>11.57</v>
       </c>
       <c r="BN18" t="n">
         <v>13.82</v>
@@ -4685,19 +4685,19 @@
         <v>10.19</v>
       </c>
       <c r="BP18" t="n">
-        <v>11.48</v>
+        <v>11.35</v>
       </c>
       <c r="BQ18" t="n">
-        <v>0.93</v>
+        <v>0.9</v>
       </c>
       <c r="BR18" t="n">
-        <v>11.64</v>
+        <v>11.56</v>
       </c>
       <c r="BS18" t="n">
         <v>2.3</v>
       </c>
       <c r="BT18" t="n">
-        <v>9782</v>
+        <v>9698</v>
       </c>
     </row>
     <row r="19">
@@ -4727,13 +4727,13 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>10.92</v>
+        <v>10.8</v>
       </c>
       <c r="G19" t="n">
-        <v>11012834678</v>
+        <v>10870961118</v>
       </c>
       <c r="H19" t="n">
-        <v>2100</v>
+        <v>8800</v>
       </c>
       <c r="I19" t="n">
         <v>317386323</v>
@@ -4748,7 +4748,7 @@
         <v>1.12</v>
       </c>
       <c r="M19" t="n">
-        <v>6.860392475230528</v>
+        <v>6.772013022354284</v>
       </c>
       <c r="N19" t="n">
         <v>0.3</v>
@@ -4826,7 +4826,7 @@
         <v>444340852.2</v>
       </c>
       <c r="AM19" t="n">
-        <v>3496137993.015873</v>
+        <v>3451098767.619048</v>
       </c>
       <c r="AN19" t="n">
         <v>0.36</v>
@@ -4867,7 +4867,7 @@
         <v>14.31</v>
       </c>
       <c r="AZ19" t="n">
-        <v>6.01</v>
+        <v>5.94</v>
       </c>
       <c r="BA19" t="n">
         <v>1.51</v>
@@ -4876,19 +4876,19 @@
         <v>5.25</v>
       </c>
       <c r="BC19" t="n">
-        <v>60.49</v>
+        <v>62.27</v>
       </c>
       <c r="BD19" t="n">
-        <v>31.04</v>
+        <v>32.49</v>
       </c>
       <c r="BE19" t="n">
         <v>-45</v>
       </c>
       <c r="BF19" t="n">
-        <v>-86.15000000000001</v>
+        <v>-85.98999999999999</v>
       </c>
       <c r="BG19" t="n">
-        <v>-51.92</v>
+        <v>-51.39</v>
       </c>
       <c r="BH19" t="n">
         <v>9.75</v>
@@ -4897,7 +4897,7 @@
         <v>0</v>
       </c>
       <c r="BJ19" t="n">
-        <v>10.92</v>
+        <v>10.8</v>
       </c>
       <c r="BK19" t="n">
         <v>1.4</v>
@@ -4906,7 +4906,7 @@
         <v>12.62</v>
       </c>
       <c r="BM19" t="n">
-        <v>10.97</v>
+        <v>10.9</v>
       </c>
       <c r="BN19" t="n">
         <v>11.41</v>
@@ -4915,19 +4915,19 @@
         <v>9.19</v>
       </c>
       <c r="BP19" t="n">
-        <v>10.84</v>
+        <v>10.8</v>
       </c>
       <c r="BQ19" t="n">
-        <v>0.87</v>
+        <v>0.86</v>
       </c>
       <c r="BR19" t="n">
-        <v>10.97</v>
+        <v>10.9</v>
       </c>
       <c r="BS19" t="n">
         <v>2.16</v>
       </c>
       <c r="BT19" t="n">
-        <v>13995</v>
+        <v>13726</v>
       </c>
     </row>
     <row r="20">
@@ -5417,13 +5417,13 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>4.98</v>
+        <v>5.01</v>
       </c>
       <c r="G22" t="n">
-        <v>997221597</v>
+        <v>1003521081</v>
       </c>
       <c r="H22" t="n">
-        <v>1121600</v>
+        <v>757500</v>
       </c>
       <c r="I22" t="n">
         <v>200245299</v>
@@ -5438,7 +5438,7 @@
         <v>0.27</v>
       </c>
       <c r="M22" t="n">
-        <v>0.08458095305778891</v>
+        <v>0.08511525392140358</v>
       </c>
       <c r="N22" t="n">
         <v>0.08</v>
@@ -5516,7 +5516,7 @@
         <v>378463615.11</v>
       </c>
       <c r="AM22" t="n">
-        <v>226127346.2585034</v>
+        <v>227555800.6802721</v>
       </c>
       <c r="AN22" t="n">
         <v>0</v>
@@ -5566,19 +5566,19 @@
         <v>172.49</v>
       </c>
       <c r="BC22" t="n">
-        <v>496.49</v>
+        <v>492.92</v>
       </c>
       <c r="BD22" t="n">
-        <v>387.03</v>
+        <v>384.11</v>
       </c>
       <c r="BE22" t="n">
         <v>-100</v>
       </c>
       <c r="BF22" t="n">
-        <v>-62.05</v>
+        <v>-62.28</v>
       </c>
       <c r="BG22" t="n">
-        <v>3363.65</v>
+        <v>3342.91</v>
       </c>
       <c r="BH22" t="n">
         <v>20.75</v>
@@ -5587,7 +5587,7 @@
         <v>0</v>
       </c>
       <c r="BJ22" t="n">
-        <v>4.98</v>
+        <v>5.01</v>
       </c>
       <c r="BK22" t="n">
         <v>1.89</v>
@@ -5596,7 +5596,7 @@
         <v>0.67</v>
       </c>
       <c r="BM22" t="n">
-        <v>5.04</v>
+        <v>5.09</v>
       </c>
       <c r="BN22" t="n">
         <v>8.82</v>
@@ -5605,19 +5605,19 @@
         <v>3.37</v>
       </c>
       <c r="BP22" t="n">
-        <v>4.83</v>
+        <v>4.94</v>
       </c>
       <c r="BQ22" t="n">
-        <v>7.42</v>
+        <v>7.46</v>
       </c>
       <c r="BR22" t="n">
-        <v>5</v>
+        <v>4.97</v>
       </c>
       <c r="BS22" t="n">
         <v>0.09</v>
       </c>
       <c r="BT22" t="n">
-        <v>1564023</v>
+        <v>1577207</v>
       </c>
     </row>
     <row r="23">
@@ -5880,10 +5880,10 @@
         <v>2.93</v>
       </c>
       <c r="G24" t="n">
-        <v>1183335024</v>
+        <v>1183679885</v>
       </c>
       <c r="H24" t="n">
-        <v>5463100</v>
+        <v>5331500</v>
       </c>
       <c r="I24" t="n">
         <v>403868805</v>
@@ -5898,7 +5898,7 @@
         <v>0.49</v>
       </c>
       <c r="M24" t="n">
-        <v>0.2860603873994232</v>
+        <v>0.2861437543827864</v>
       </c>
       <c r="N24" t="n">
         <v>0.11</v>
@@ -5976,7 +5976,7 @@
         <v>153470145.9</v>
       </c>
       <c r="AM24" t="n">
-        <v>1066067589.189189</v>
+        <v>1066378274.774775</v>
       </c>
       <c r="AN24" t="n">
         <v>0.0813</v>
@@ -6056,7 +6056,7 @@
         <v>0.41</v>
       </c>
       <c r="BM24" t="n">
-        <v>2.96</v>
+        <v>3.01</v>
       </c>
       <c r="BN24" t="n">
         <v>5.29</v>
@@ -6065,7 +6065,7 @@
         <v>1.92</v>
       </c>
       <c r="BP24" t="n">
-        <v>2.84</v>
+        <v>2.9</v>
       </c>
       <c r="BQ24" t="n">
         <v>7.2</v>
@@ -6077,7 +6077,7 @@
         <v>0.29</v>
       </c>
       <c r="BT24" t="n">
-        <v>9102590</v>
+        <v>8821017</v>
       </c>
     </row>
     <row r="25">
@@ -6107,13 +6107,13 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>3.76</v>
+        <v>3.85</v>
       </c>
       <c r="G25" t="n">
-        <v>1302817436</v>
+        <v>1334390331</v>
       </c>
       <c r="H25" t="n">
-        <v>1003800</v>
+        <v>1568000</v>
       </c>
       <c r="I25" t="n">
         <v>346494097</v>
@@ -6128,7 +6128,7 @@
         <v>0.97</v>
       </c>
       <c r="M25" t="n">
-        <v>0.6496442605838165</v>
+        <v>0.6653879476576864</v>
       </c>
       <c r="N25" t="n">
         <v>0.22</v>
@@ -6206,7 +6206,7 @@
         <v>62368937.46</v>
       </c>
       <c r="AM25" t="n">
-        <v>478976998.5294117</v>
+        <v>490584680.5147058</v>
       </c>
       <c r="AN25" t="n">
         <v>0.4742</v>
@@ -6247,7 +6247,7 @@
         <v>3.27</v>
       </c>
       <c r="AZ25" t="n">
-        <v>8.76</v>
+        <v>8.970000000000001</v>
       </c>
       <c r="BA25" t="n">
         <v>0.23</v>
@@ -6256,19 +6256,19 @@
         <v>2.2</v>
       </c>
       <c r="BC25" t="n">
-        <v>6.64</v>
+        <v>4.15</v>
       </c>
       <c r="BD25" t="n">
-        <v>-12.93</v>
+        <v>-14.96</v>
       </c>
       <c r="BE25" t="n">
         <v>133</v>
       </c>
       <c r="BF25" t="n">
-        <v>-93.84</v>
+        <v>-93.98</v>
       </c>
       <c r="BG25" t="n">
-        <v>-41.5</v>
+        <v>-42.86</v>
       </c>
       <c r="BH25" t="n">
         <v>3.97</v>
@@ -6277,7 +6277,7 @@
         <v>0</v>
       </c>
       <c r="BJ25" t="n">
-        <v>3.76</v>
+        <v>3.85</v>
       </c>
       <c r="BK25" t="n">
         <v>0.18</v>
@@ -6286,7 +6286,7 @@
         <v>0.24</v>
       </c>
       <c r="BM25" t="n">
-        <v>3.86</v>
+        <v>4</v>
       </c>
       <c r="BN25" t="n">
         <v>6.3</v>
@@ -6295,19 +6295,19 @@
         <v>2.64</v>
       </c>
       <c r="BP25" t="n">
-        <v>3.66</v>
+        <v>3.74</v>
       </c>
       <c r="BQ25" t="n">
-        <v>15.89</v>
+        <v>16.27</v>
       </c>
       <c r="BR25" t="n">
-        <v>3.73</v>
+        <v>3.78</v>
       </c>
       <c r="BS25" t="n">
         <v>0.67</v>
       </c>
       <c r="BT25" t="n">
-        <v>1186897</v>
+        <v>1186133</v>
       </c>
     </row>
     <row r="26">
@@ -6337,13 +6337,13 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>9.65</v>
+        <v>10.1</v>
       </c>
       <c r="G26" t="n">
-        <v>13069891933</v>
+        <v>13683349216</v>
       </c>
       <c r="H26" t="n">
-        <v>7799400</v>
+        <v>16505300</v>
       </c>
       <c r="I26" t="n">
         <v>1354393401</v>
@@ -6358,7 +6358,7 @@
         <v>1.94</v>
       </c>
       <c r="M26" t="n">
-        <v>0.1685351547021237</v>
+        <v>0.1764456346528036</v>
       </c>
       <c r="N26" t="n">
         <v>0.26</v>
@@ -6436,7 +6436,7 @@
         <v>961619314.7099999</v>
       </c>
       <c r="AM26" t="n">
-        <v>4667818547.5</v>
+        <v>4886910434.285714</v>
       </c>
       <c r="AN26" t="n">
         <v>0.1043</v>
@@ -6477,7 +6477,7 @@
         <v>7.07</v>
       </c>
       <c r="AZ26" t="n">
-        <v>1.85</v>
+        <v>1.94</v>
       </c>
       <c r="BA26" t="n">
         <v>0.66</v>
@@ -6486,19 +6486,19 @@
         <v>1.19</v>
       </c>
       <c r="BC26" t="n">
-        <v>-10.3</v>
+        <v>-14.3</v>
       </c>
       <c r="BD26" t="n">
-        <v>-26.76</v>
+        <v>-30.03</v>
       </c>
       <c r="BE26" t="n">
         <v>-80.83</v>
       </c>
       <c r="BF26" t="n">
-        <v>-93.17</v>
+        <v>-93.47</v>
       </c>
       <c r="BG26" t="n">
-        <v>-87.63</v>
+        <v>-88.18000000000001</v>
       </c>
       <c r="BH26" t="n">
         <v>4.69</v>
@@ -6507,7 +6507,7 @@
         <v>0</v>
       </c>
       <c r="BJ26" t="n">
-        <v>9.65</v>
+        <v>10.1</v>
       </c>
       <c r="BK26" t="n">
         <v>0.71</v>
@@ -6516,7 +6516,7 @@
         <v>0.72</v>
       </c>
       <c r="BM26" t="n">
-        <v>9.82</v>
+        <v>10.19</v>
       </c>
       <c r="BN26" t="n">
         <v>10.6</v>
@@ -6525,19 +6525,19 @@
         <v>6.91</v>
       </c>
       <c r="BP26" t="n">
-        <v>9.48</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="BQ26" t="n">
-        <v>13.45</v>
+        <v>14.08</v>
       </c>
       <c r="BR26" t="n">
-        <v>9.75</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="BS26" t="n">
         <v>0.16</v>
       </c>
       <c r="BT26" t="n">
-        <v>11736210</v>
+        <v>11796480</v>
       </c>
     </row>
     <row r="27">
@@ -8165,13 +8165,13 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>15.3</v>
+        <v>15.03</v>
       </c>
       <c r="G34" t="n">
-        <v>3159292449</v>
+        <v>3104444941</v>
       </c>
       <c r="H34" t="n">
-        <v>2631800</v>
+        <v>3684600</v>
       </c>
       <c r="I34" t="n">
         <v>206489813</v>
@@ -8186,7 +8186,7 @@
         <v>0.45</v>
       </c>
       <c r="M34" t="n">
-        <v>0.2777387049412377</v>
+        <v>0.2729169684014641</v>
       </c>
       <c r="N34" t="n">
         <v>0.24</v>
@@ -8264,7 +8264,7 @@
         <v>324189006.41</v>
       </c>
       <c r="AM34" t="n">
-        <v>656817556.9646571</v>
+        <v>645414748.6486487</v>
       </c>
       <c r="AN34" t="n">
         <v>0</v>
@@ -8305,7 +8305,7 @@
         <v>30.28</v>
       </c>
       <c r="AZ34" t="n">
-        <v>35.7</v>
+        <v>35.07</v>
       </c>
       <c r="BA34" t="n">
         <v>2.29</v>
@@ -8314,19 +8314,19 @@
         <v>25.26</v>
       </c>
       <c r="BC34" t="n">
-        <v>142.41</v>
+        <v>146.76</v>
       </c>
       <c r="BD34" t="n">
-        <v>97.93000000000001</v>
+        <v>101.48</v>
       </c>
       <c r="BE34" t="n">
         <v>133.33</v>
       </c>
       <c r="BF34" t="n">
-        <v>-85</v>
+        <v>-84.73</v>
       </c>
       <c r="BG34" t="n">
-        <v>65.08</v>
+        <v>68.05</v>
       </c>
       <c r="BH34" t="n">
         <v>38.94</v>
@@ -8335,7 +8335,7 @@
         <v>0</v>
       </c>
       <c r="BJ34" t="n">
-        <v>15.3</v>
+        <v>15.03</v>
       </c>
       <c r="BK34" t="n">
         <v>1.57</v>
@@ -8344,7 +8344,7 @@
         <v>1.58</v>
       </c>
       <c r="BM34" t="n">
-        <v>15.99</v>
+        <v>15.38</v>
       </c>
       <c r="BN34" t="n">
         <v>31.12</v>
@@ -8353,19 +8353,19 @@
         <v>14.32</v>
       </c>
       <c r="BP34" t="n">
-        <v>15.3</v>
+        <v>14.96</v>
       </c>
       <c r="BQ34" t="n">
-        <v>9.699999999999999</v>
+        <v>9.529999999999999</v>
       </c>
       <c r="BR34" t="n">
-        <v>15.82</v>
+        <v>15.34</v>
       </c>
       <c r="BS34" t="n">
         <v>0.32</v>
       </c>
       <c r="BT34" t="n">
-        <v>3104737</v>
+        <v>3064873</v>
       </c>
     </row>
     <row r="35">
@@ -8395,13 +8395,13 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>17.42</v>
+        <v>17.58</v>
       </c>
       <c r="G35" t="n">
-        <v>87910012965</v>
+        <v>88743294634</v>
       </c>
       <c r="H35" t="n">
-        <v>28718200</v>
+        <v>30862100</v>
       </c>
       <c r="I35" t="n">
         <v>5046500000</v>
@@ -8416,7 +8416,7 @@
         <v>4.69</v>
       </c>
       <c r="M35" t="n">
-        <v>7.298321227257541</v>
+        <v>7.36750057427423</v>
       </c>
       <c r="N35" t="n">
         <v>1.79</v>
@@ -8494,7 +8494,7 @@
         <v>5349290000</v>
       </c>
       <c r="AM35" t="n">
-        <v>7265290327.68595</v>
+        <v>7334156581.322314</v>
       </c>
       <c r="AN35" t="n">
         <v>0.5305</v>
@@ -8535,7 +8535,7 @@
         <v>7.68</v>
       </c>
       <c r="AZ35" t="n">
-        <v>10.16</v>
+        <v>10.26</v>
       </c>
       <c r="BA35" t="n">
         <v>1.11</v>
@@ -8544,19 +8544,19 @@
         <v>9.119999999999999</v>
       </c>
       <c r="BC35" t="n">
-        <v>-46</v>
+        <v>-46.49</v>
       </c>
       <c r="BD35" t="n">
-        <v>-55.91</v>
+        <v>-56.31</v>
       </c>
       <c r="BE35" t="n">
         <v>-41.67</v>
       </c>
       <c r="BF35" t="n">
-        <v>-93.59999999999999</v>
+        <v>-93.66</v>
       </c>
       <c r="BG35" t="n">
-        <v>-47.66</v>
+        <v>-48.14</v>
       </c>
       <c r="BH35" t="n">
         <v>3.71</v>
@@ -8565,7 +8565,7 @@
         <v>0</v>
       </c>
       <c r="BJ35" t="n">
-        <v>17.42</v>
+        <v>17.58</v>
       </c>
       <c r="BK35" t="n">
         <v>1.06</v>
@@ -8574,7 +8574,7 @@
         <v>1.04</v>
       </c>
       <c r="BM35" t="n">
-        <v>17.61</v>
+        <v>17.76</v>
       </c>
       <c r="BN35" t="n">
         <v>20.08</v>
@@ -8583,19 +8583,19 @@
         <v>11.7</v>
       </c>
       <c r="BP35" t="n">
-        <v>17.2</v>
+        <v>17.32</v>
       </c>
       <c r="BQ35" t="n">
-        <v>16.67</v>
+        <v>16.82</v>
       </c>
       <c r="BR35" t="n">
-        <v>17.56</v>
+        <v>17.37</v>
       </c>
       <c r="BS35" t="n">
         <v>7.3</v>
       </c>
       <c r="BT35" t="n">
-        <v>37288447</v>
+        <v>37224647</v>
       </c>
     </row>
     <row r="36">
@@ -8858,10 +8858,10 @@
         <v>14.9</v>
       </c>
       <c r="G37" t="n">
-        <v>199919850</v>
+        <v>199978109</v>
       </c>
       <c r="H37" t="n">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="I37" t="n">
         <v>4900000</v>
@@ -8876,7 +8876,7 @@
         <v>0.88</v>
       </c>
       <c r="M37" t="n">
-        <v>1.946388150013252</v>
+        <v>1.946955350454987</v>
       </c>
       <c r="N37" t="n">
         <v>0.5</v>
@@ -8954,7 +8954,7 @@
         <v>11319000</v>
       </c>
       <c r="AM37" t="n">
-        <v>47827715.31100479</v>
+        <v>47841652.8708134</v>
       </c>
       <c r="AN37" t="n">
         <v>0</v>
@@ -9043,13 +9043,13 @@
         <v>13.05</v>
       </c>
       <c r="BP37" t="n">
-        <v>14.9</v>
+        <v>14.8</v>
       </c>
       <c r="BQ37" t="n">
         <v>6.45</v>
       </c>
       <c r="BR37" t="n">
-        <v>14.9</v>
+        <v>14.8</v>
       </c>
       <c r="BS37" t="n">
         <v>0.72</v>
@@ -9315,10 +9315,10 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>69.97</v>
+        <v>69.06</v>
       </c>
       <c r="G39" t="n">
-        <v>3922400019</v>
+        <v>3872514501</v>
       </c>
       <c r="H39" t="n">
         <v>4000</v>
@@ -9336,7 +9336,7 @@
         <v>0.53</v>
       </c>
       <c r="M39" t="n">
-        <v>0.1968872758762667</v>
+        <v>0.1943832416887489</v>
       </c>
       <c r="N39" t="n">
         <v>0.06</v>
@@ -9414,7 +9414,7 @@
         <v>2536078170.6</v>
       </c>
       <c r="AM39" t="n">
-        <v>412016808.7184874</v>
+        <v>406776733.2983193</v>
       </c>
       <c r="AN39" t="n">
         <v>11.9435</v>
@@ -9455,7 +9455,7 @@
         <v>170.24</v>
       </c>
       <c r="AZ39" t="n">
-        <v>204.43</v>
+        <v>201.77</v>
       </c>
       <c r="BA39" t="n">
         <v>19.01</v>
@@ -9464,19 +9464,19 @@
         <v>91.72</v>
       </c>
       <c r="BC39" t="n">
-        <v>197.99</v>
+        <v>201.92</v>
       </c>
       <c r="BD39" t="n">
-        <v>143.31</v>
+        <v>146.52</v>
       </c>
       <c r="BE39" t="n">
         <v>192.17</v>
       </c>
       <c r="BF39" t="n">
-        <v>-72.83</v>
+        <v>-72.47</v>
       </c>
       <c r="BG39" t="n">
-        <v>31.09</v>
+        <v>32.82</v>
       </c>
       <c r="BH39" t="n">
         <v>128.13</v>
@@ -9485,7 +9485,7 @@
         <v>0</v>
       </c>
       <c r="BJ39" t="n">
-        <v>69.97</v>
+        <v>69.06</v>
       </c>
       <c r="BK39" t="n">
         <v>15.08</v>
@@ -9494,7 +9494,7 @@
         <v>15.08</v>
       </c>
       <c r="BM39" t="n">
-        <v>70.33</v>
+        <v>70.37</v>
       </c>
       <c r="BN39" t="n">
         <v>74.56</v>
@@ -9503,19 +9503,19 @@
         <v>54.98</v>
       </c>
       <c r="BP39" t="n">
-        <v>69.69</v>
+        <v>69.06</v>
       </c>
       <c r="BQ39" t="n">
-        <v>4.64</v>
+        <v>4.58</v>
       </c>
       <c r="BR39" t="n">
-        <v>69.69</v>
+        <v>69.16</v>
       </c>
       <c r="BS39" t="n">
         <v>0.58</v>
       </c>
       <c r="BT39" t="n">
-        <v>3830</v>
+        <v>3887</v>
       </c>
     </row>
     <row r="40">
@@ -9545,13 +9545,13 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>22.04</v>
+        <v>22.71</v>
       </c>
       <c r="G40" t="n">
-        <v>126307520486</v>
+        <v>130185160591</v>
       </c>
       <c r="H40" t="n">
-        <v>21989500</v>
+        <v>32049800</v>
       </c>
       <c r="I40" t="n">
         <v>5730834040</v>
@@ -9566,7 +9566,7 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="M40" t="n">
-        <v>0.3832326484467625</v>
+        <v>0.3949978884059084</v>
       </c>
       <c r="N40" t="n">
         <v>0.05</v>
@@ -9644,7 +9644,7 @@
         <v>15358635227.2</v>
       </c>
       <c r="AM40" t="n">
-        <v>6551219942.219916</v>
+        <v>6752342354.304979</v>
       </c>
       <c r="AN40" t="n">
         <v>0.5641</v>
@@ -9685,7 +9685,7 @@
         <v>36.13</v>
       </c>
       <c r="AZ40" t="n">
-        <v>11.13</v>
+        <v>11.47</v>
       </c>
       <c r="BA40" t="n">
         <v>2.76</v>
@@ -9694,19 +9694,19 @@
         <v>27.89</v>
       </c>
       <c r="BC40" t="n">
-        <v>100.77</v>
+        <v>94.84</v>
       </c>
       <c r="BD40" t="n">
-        <v>63.92</v>
+        <v>59.09</v>
       </c>
       <c r="BE40" t="n">
         <v>-49.5</v>
       </c>
       <c r="BF40" t="n">
-        <v>-87.48</v>
+        <v>-87.84999999999999</v>
       </c>
       <c r="BG40" t="n">
-        <v>26.54</v>
+        <v>22.81</v>
       </c>
       <c r="BH40" t="n">
         <v>32.47</v>
@@ -9715,7 +9715,7 @@
         <v>0</v>
       </c>
       <c r="BJ40" t="n">
-        <v>22.04</v>
+        <v>22.71</v>
       </c>
       <c r="BK40" t="n">
         <v>2.68</v>
@@ -9724,7 +9724,7 @@
         <v>2.5</v>
       </c>
       <c r="BM40" t="n">
-        <v>22.33</v>
+        <v>22.74</v>
       </c>
       <c r="BN40" t="n">
         <v>27.36</v>
@@ -9733,19 +9733,19 @@
         <v>17.67</v>
       </c>
       <c r="BP40" t="n">
-        <v>21.92</v>
+        <v>21.51</v>
       </c>
       <c r="BQ40" t="n">
-        <v>8.82</v>
+        <v>9.09</v>
       </c>
       <c r="BR40" t="n">
-        <v>22.28</v>
+        <v>21.95</v>
       </c>
       <c r="BS40" t="n">
         <v>0.39</v>
       </c>
       <c r="BT40" t="n">
-        <v>31195740</v>
+        <v>31648024</v>
       </c>
     </row>
     <row r="41">
@@ -9778,10 +9778,10 @@
         <v>16.09</v>
       </c>
       <c r="G41" t="n">
-        <v>191758302038</v>
+        <v>192114033541</v>
       </c>
       <c r="H41" t="n">
-        <v>5032900</v>
+        <v>5050400</v>
       </c>
       <c r="I41" t="n">
         <v>5303870781</v>
@@ -9796,7 +9796,7 @@
         <v>0.92</v>
       </c>
       <c r="M41" t="n">
-        <v>1.277871276207643</v>
+        <v>1.280241859722904</v>
       </c>
       <c r="N41" t="n">
         <v>0.07000000000000001</v>
@@ -9874,7 +9874,7 @@
         <v>12304980211.92</v>
       </c>
       <c r="AM41" t="n">
-        <v>29546733750.07704</v>
+        <v>29601546000.15408</v>
       </c>
       <c r="AN41" t="n">
         <v>1.6841</v>
@@ -9954,7 +9954,7 @@
         <v>2.34</v>
       </c>
       <c r="BM41" t="n">
-        <v>16.31</v>
+        <v>16.14</v>
       </c>
       <c r="BN41" t="n">
         <v>18.28</v>
@@ -9963,19 +9963,19 @@
         <v>13.43</v>
       </c>
       <c r="BP41" t="n">
-        <v>16.01</v>
+        <v>15.89</v>
       </c>
       <c r="BQ41" t="n">
         <v>6.88</v>
       </c>
       <c r="BR41" t="n">
-        <v>16.31</v>
+        <v>16.07</v>
       </c>
       <c r="BS41" t="n">
         <v>0.5600000000000001</v>
       </c>
       <c r="BT41" t="n">
-        <v>6933868</v>
+        <v>6971226</v>
       </c>
     </row>
     <row r="42">
@@ -10005,13 +10005,13 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>18.2</v>
+        <v>18.21</v>
       </c>
       <c r="G42" t="n">
-        <v>191758302038</v>
+        <v>192114033541</v>
       </c>
       <c r="H42" t="n">
-        <v>24044300</v>
+        <v>34375100</v>
       </c>
       <c r="I42" t="n">
         <v>5288141247</v>
@@ -10026,7 +10026,7 @@
         <v>1.05</v>
       </c>
       <c r="M42" t="n">
-        <v>1.281672294135848</v>
+        <v>1.284049928932886</v>
       </c>
       <c r="N42" t="n">
         <v>0.08</v>
@@ -10104,7 +10104,7 @@
         <v>12268487693.04</v>
       </c>
       <c r="AM42" t="n">
-        <v>26089564903.12925</v>
+        <v>26137963747.07483</v>
       </c>
       <c r="AN42" t="n">
         <v>1.8491</v>
@@ -10145,7 +10145,7 @@
         <v>24.4</v>
       </c>
       <c r="AZ42" t="n">
-        <v>26.36</v>
+        <v>26.37</v>
       </c>
       <c r="BA42" t="n">
         <v>2.53</v>
@@ -10154,19 +10154,19 @@
         <v>15.11</v>
       </c>
       <c r="BC42" t="n">
-        <v>64.20999999999999</v>
+        <v>64.12</v>
       </c>
       <c r="BD42" t="n">
-        <v>34.07</v>
+        <v>34</v>
       </c>
       <c r="BE42" t="n">
         <v>44.83</v>
       </c>
       <c r="BF42" t="n">
-        <v>-86.11</v>
+        <v>-86.12</v>
       </c>
       <c r="BG42" t="n">
-        <v>-16.95</v>
+        <v>-17</v>
       </c>
       <c r="BH42" t="n">
         <v>17.11</v>
@@ -10175,7 +10175,7 @@
         <v>0</v>
       </c>
       <c r="BJ42" t="n">
-        <v>18.2</v>
+        <v>18.21</v>
       </c>
       <c r="BK42" t="n">
         <v>2.32</v>
@@ -10184,7 +10184,7 @@
         <v>2.34</v>
       </c>
       <c r="BM42" t="n">
-        <v>18.46</v>
+        <v>18.25</v>
       </c>
       <c r="BN42" t="n">
         <v>21.33</v>
@@ -10193,19 +10193,19 @@
         <v>15.67</v>
       </c>
       <c r="BP42" t="n">
-        <v>18.14</v>
+        <v>17.97</v>
       </c>
       <c r="BQ42" t="n">
         <v>7.79</v>
       </c>
       <c r="BR42" t="n">
-        <v>18.45</v>
+        <v>18.21</v>
       </c>
       <c r="BS42" t="n">
         <v>0.63</v>
       </c>
       <c r="BT42" t="n">
-        <v>40260834</v>
+        <v>40428097</v>
       </c>
     </row>
     <row r="43">
@@ -10235,13 +10235,13 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>40.16</v>
+        <v>40.59</v>
       </c>
       <c r="G43" t="n">
-        <v>77966623703</v>
+        <v>78824359646</v>
       </c>
       <c r="H43" t="n">
-        <v>5465900</v>
+        <v>6868600</v>
       </c>
       <c r="I43" t="n">
         <v>1941400000</v>
@@ -10334,7 +10334,7 @@
         <v>9182822000</v>
       </c>
       <c r="AM43" t="n">
-        <v>9496543690.986601</v>
+        <v>9601018227.2838</v>
       </c>
       <c r="AN43" t="n">
         <v>4.5901</v>
@@ -10375,7 +10375,7 @@
         <v>19.95</v>
       </c>
       <c r="AZ43" t="n">
-        <v>72.89</v>
+        <v>73.67</v>
       </c>
       <c r="BA43" t="n">
         <v>5.63</v>
@@ -10384,19 +10384,19 @@
         <v>48.62</v>
       </c>
       <c r="BC43" t="n">
-        <v>-39.16</v>
+        <v>-39.8</v>
       </c>
       <c r="BD43" t="n">
-        <v>-50.32</v>
+        <v>-50.85</v>
       </c>
       <c r="BE43" t="n">
         <v>81.5</v>
       </c>
       <c r="BF43" t="n">
-        <v>-85.98</v>
+        <v>-86.13</v>
       </c>
       <c r="BG43" t="n">
-        <v>21.06</v>
+        <v>19.78</v>
       </c>
       <c r="BH43" t="n">
         <v>5.61</v>
@@ -10405,7 +10405,7 @@
         <v>0</v>
       </c>
       <c r="BJ43" t="n">
-        <v>40.16</v>
+        <v>40.59</v>
       </c>
       <c r="BK43" t="n">
         <v>4.73</v>
@@ -10414,7 +10414,7 @@
         <v>4.73</v>
       </c>
       <c r="BM43" t="n">
-        <v>40.6</v>
+        <v>40.95</v>
       </c>
       <c r="BN43" t="n">
         <v>42.98</v>
@@ -10423,19 +10423,19 @@
         <v>28.06</v>
       </c>
       <c r="BP43" t="n">
-        <v>39.78</v>
+        <v>40.01</v>
       </c>
       <c r="BQ43" t="n">
-        <v>8.48</v>
+        <v>8.57</v>
       </c>
       <c r="BR43" t="n">
-        <v>40</v>
+        <v>40.16</v>
       </c>
       <c r="BS43" t="n">
         <v>0</v>
       </c>
       <c r="BT43" t="n">
-        <v>6777434</v>
+        <v>6773488</v>
       </c>
     </row>
     <row r="44">
@@ -10925,13 +10925,13 @@
         </is>
       </c>
       <c r="F46" t="n">
-        <v>4.04</v>
+        <v>4</v>
       </c>
       <c r="G46" t="n">
-        <v>4042185601</v>
+        <v>4003328000</v>
       </c>
       <c r="H46" t="n">
-        <v>18773700</v>
+        <v>13869800</v>
       </c>
       <c r="I46" t="n">
         <v>1000541644</v>
@@ -10946,7 +10946,7 @@
         <v>2.5</v>
       </c>
       <c r="M46" t="n">
-        <v>0.07026082366381874</v>
+        <v>0.06958540513499498</v>
       </c>
       <c r="N46" t="n">
         <v>0.08</v>
@@ -11024,7 +11024,7 @@
         <v>460249156.24</v>
       </c>
       <c r="AM46" t="n">
-        <v>3962927059.803922</v>
+        <v>3924831372.549019</v>
       </c>
       <c r="AN46" t="n">
         <v>0.0311</v>
@@ -11065,7 +11065,7 @@
         <v>3.3</v>
       </c>
       <c r="AZ46" t="n">
-        <v>3.33</v>
+        <v>3.3</v>
       </c>
       <c r="BA46" t="n">
         <v>0.42</v>
@@ -11074,19 +11074,19 @@
         <v>7.38</v>
       </c>
       <c r="BC46" t="n">
-        <v>0.1</v>
+        <v>1.1</v>
       </c>
       <c r="BD46" t="n">
-        <v>-18.27</v>
+        <v>-17.45</v>
       </c>
       <c r="BE46" t="n">
         <v>-17.5</v>
       </c>
       <c r="BF46" t="n">
-        <v>-89.53</v>
+        <v>-89.42</v>
       </c>
       <c r="BG46" t="n">
-        <v>82.64</v>
+        <v>84.47</v>
       </c>
       <c r="BH46" t="n">
         <v>1.58</v>
@@ -11095,7 +11095,7 @@
         <v>0</v>
       </c>
       <c r="BJ46" t="n">
-        <v>4.04</v>
+        <v>4</v>
       </c>
       <c r="BK46" t="n">
         <v>0.46</v>
@@ -11104,7 +11104,7 @@
         <v>0.46</v>
       </c>
       <c r="BM46" t="n">
-        <v>4.12</v>
+        <v>4.04</v>
       </c>
       <c r="BN46" t="n">
         <v>7.31</v>
@@ -11113,19 +11113,19 @@
         <v>2.97</v>
       </c>
       <c r="BP46" t="n">
-        <v>3.98</v>
+        <v>3.94</v>
       </c>
       <c r="BQ46" t="n">
-        <v>8.83</v>
+        <v>8.74</v>
       </c>
       <c r="BR46" t="n">
-        <v>4.1</v>
+        <v>4.03</v>
       </c>
       <c r="BS46" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="BT46" t="n">
-        <v>20065343</v>
+        <v>20476617</v>
       </c>
     </row>
     <row r="47">
@@ -11155,13 +11155,13 @@
         </is>
       </c>
       <c r="F47" t="n">
-        <v>8.83</v>
+        <v>8.99</v>
       </c>
       <c r="G47" t="n">
-        <v>3089991365</v>
+        <v>3153507624</v>
       </c>
       <c r="H47" t="n">
-        <v>9100</v>
+        <v>8600</v>
       </c>
       <c r="I47" t="n">
         <v>254106600</v>
@@ -11176,7 +11176,7 @@
         <v>1.22</v>
       </c>
       <c r="M47" t="n">
-        <v>0.7286555150212827</v>
+        <v>0.7436333796645614</v>
       </c>
       <c r="N47" t="n">
         <v>0.07000000000000001</v>
@@ -11254,7 +11254,7 @@
         <v>322715382</v>
       </c>
       <c r="AM47" t="n">
-        <v>547870809.3971632</v>
+        <v>559132557.4468086</v>
       </c>
       <c r="AN47" t="n">
         <v>0.4132</v>
@@ -11295,7 +11295,7 @@
         <v>11.74</v>
       </c>
       <c r="AZ47" t="n">
-        <v>11.6</v>
+        <v>11.81</v>
       </c>
       <c r="BA47" t="n">
         <v>1.46</v>
@@ -11304,19 +11304,19 @@
         <v>8.619999999999999</v>
       </c>
       <c r="BC47" t="n">
-        <v>62.78</v>
+        <v>59.88</v>
       </c>
       <c r="BD47" t="n">
-        <v>32.91</v>
+        <v>30.54</v>
       </c>
       <c r="BE47" t="n">
         <v>31.33</v>
       </c>
       <c r="BF47" t="n">
-        <v>-83.48</v>
+        <v>-83.78</v>
       </c>
       <c r="BG47" t="n">
-        <v>-2.38</v>
+        <v>-4.12</v>
       </c>
       <c r="BH47" t="n">
         <v>7.23</v>
@@ -11325,7 +11325,7 @@
         <v>0</v>
       </c>
       <c r="BJ47" t="n">
-        <v>8.83</v>
+        <v>8.99</v>
       </c>
       <c r="BK47" t="n">
         <v>1.27</v>
@@ -11334,7 +11334,7 @@
         <v>1.29</v>
       </c>
       <c r="BM47" t="n">
-        <v>8.93</v>
+        <v>9.050000000000001</v>
       </c>
       <c r="BN47" t="n">
         <v>9.25</v>
@@ -11343,19 +11343,19 @@
         <v>7.2</v>
       </c>
       <c r="BP47" t="n">
-        <v>8.82</v>
+        <v>8.84</v>
       </c>
       <c r="BQ47" t="n">
-        <v>6.83</v>
+        <v>6.95</v>
       </c>
       <c r="BR47" t="n">
-        <v>8.869999999999999</v>
+        <v>8.84</v>
       </c>
       <c r="BS47" t="n">
         <v>0.53</v>
       </c>
       <c r="BT47" t="n">
-        <v>12944</v>
+        <v>12614</v>
       </c>
     </row>
     <row r="48">
@@ -11385,13 +11385,13 @@
         </is>
       </c>
       <c r="F48" t="n">
-        <v>9.130000000000001</v>
+        <v>9.140000000000001</v>
       </c>
       <c r="G48" t="n">
-        <v>3089991365</v>
+        <v>3153507624</v>
       </c>
       <c r="H48" t="n">
-        <v>2100</v>
+        <v>3800</v>
       </c>
       <c r="I48" t="n">
         <v>93397546</v>
@@ -11406,7 +11406,7 @@
         <v>1.24</v>
       </c>
       <c r="M48" t="n">
-        <v>1.982452253010021</v>
+        <v>2.023202512762711</v>
       </c>
       <c r="N48" t="n">
         <v>0.07000000000000001</v>
@@ -11484,7 +11484,7 @@
         <v>118614883.42</v>
       </c>
       <c r="AM48" t="n">
-        <v>540208280.5944057</v>
+        <v>551312521.6783217</v>
       </c>
       <c r="AN48" t="n">
         <v>0.4132</v>
@@ -11525,7 +11525,7 @@
         <v>11.74</v>
       </c>
       <c r="AZ48" t="n">
-        <v>11.95</v>
+        <v>11.96</v>
       </c>
       <c r="BA48" t="n">
         <v>1.46</v>
@@ -11534,19 +11534,19 @@
         <v>8.24</v>
       </c>
       <c r="BC48" t="n">
-        <v>57.43</v>
+        <v>57.26</v>
       </c>
       <c r="BD48" t="n">
-        <v>28.54</v>
+        <v>28.4</v>
       </c>
       <c r="BE48" t="n">
         <v>30.83</v>
       </c>
       <c r="BF48" t="n">
-        <v>-84.03</v>
+        <v>-84.04000000000001</v>
       </c>
       <c r="BG48" t="n">
-        <v>-9.789999999999999</v>
+        <v>-9.890000000000001</v>
       </c>
       <c r="BH48" t="n">
         <v>7.23</v>
@@ -11555,7 +11555,7 @@
         <v>0</v>
       </c>
       <c r="BJ48" t="n">
-        <v>9.130000000000001</v>
+        <v>9.140000000000001</v>
       </c>
       <c r="BK48" t="n">
         <v>1.27</v>
@@ -11573,19 +11573,19 @@
         <v>7.21</v>
       </c>
       <c r="BP48" t="n">
-        <v>9.06</v>
+        <v>9.01</v>
       </c>
       <c r="BQ48" t="n">
-        <v>7.06</v>
+        <v>7.07</v>
       </c>
       <c r="BR48" t="n">
-        <v>9.1</v>
+        <v>9.029999999999999</v>
       </c>
       <c r="BS48" t="n">
         <v>0.54</v>
       </c>
       <c r="BT48" t="n">
-        <v>2641</v>
+        <v>2651</v>
       </c>
     </row>
     <row r="49">
@@ -11845,13 +11845,13 @@
         </is>
       </c>
       <c r="F50" t="n">
-        <v>34.3</v>
+        <v>33.01</v>
       </c>
       <c r="G50" t="n">
-        <v>974049400</v>
+        <v>972024300</v>
       </c>
       <c r="H50" t="n">
-        <v>100</v>
+        <v>600</v>
       </c>
       <c r="I50" t="n">
         <v>11540870</v>
@@ -11866,7 +11866,7 @@
         <v>0.8</v>
       </c>
       <c r="M50" t="n">
-        <v>0.9854332141795732</v>
+        <v>0.9833844466303759</v>
       </c>
       <c r="N50" t="n">
         <v>0.06</v>
@@ -11944,7 +11944,7 @@
         <v>84709985.8</v>
       </c>
       <c r="AM50" t="n">
-        <v>332440068.2593856</v>
+        <v>331748907.8498293</v>
       </c>
       <c r="AN50" t="n">
         <v>4.4983</v>
@@ -11985,7 +11985,7 @@
         <v>68.48999999999999</v>
       </c>
       <c r="AZ50" t="n">
-        <v>75.63</v>
+        <v>72.79000000000001</v>
       </c>
       <c r="BA50" t="n">
         <v>9.210000000000001</v>
@@ -11994,19 +11994,19 @@
         <v>30.53</v>
       </c>
       <c r="BC50" t="n">
-        <v>144.54</v>
+        <v>154.1</v>
       </c>
       <c r="BD50" t="n">
-        <v>99.67</v>
+        <v>107.47</v>
       </c>
       <c r="BE50" t="n">
         <v>120.5</v>
       </c>
       <c r="BF50" t="n">
-        <v>-73.14</v>
+        <v>-72.09</v>
       </c>
       <c r="BG50" t="n">
-        <v>-10.99</v>
+        <v>-7.51</v>
       </c>
       <c r="BH50" t="n">
         <v>42.6</v>
@@ -12015,7 +12015,7 @@
         <v>0</v>
       </c>
       <c r="BJ50" t="n">
-        <v>34.3</v>
+        <v>33.01</v>
       </c>
       <c r="BK50" t="n">
         <v>7.34</v>
@@ -12024,7 +12024,7 @@
         <v>7.6</v>
       </c>
       <c r="BM50" t="n">
-        <v>34.3</v>
+        <v>33.8</v>
       </c>
       <c r="BN50" t="n">
         <v>39.22</v>
@@ -12033,19 +12033,19 @@
         <v>23.5</v>
       </c>
       <c r="BP50" t="n">
-        <v>34.3</v>
+        <v>33.01</v>
       </c>
       <c r="BQ50" t="n">
-        <v>4.51</v>
+        <v>4.34</v>
       </c>
       <c r="BR50" t="n">
-        <v>34.3</v>
+        <v>33.8</v>
       </c>
       <c r="BS50" t="n">
         <v>0.4</v>
       </c>
       <c r="BT50" t="n">
-        <v>727</v>
+        <v>670</v>
       </c>
     </row>
     <row r="51">
@@ -12523,13 +12523,13 @@
         </is>
       </c>
       <c r="F53" t="n">
-        <v>6.5</v>
+        <v>6.61</v>
       </c>
       <c r="G53" t="n">
-        <v>889540600</v>
+        <v>904858121</v>
       </c>
       <c r="H53" t="n">
-        <v>20600</v>
+        <v>22500</v>
       </c>
       <c r="I53" t="n">
         <v>136852484</v>
@@ -12544,7 +12544,7 @@
         <v>2.79</v>
       </c>
       <c r="M53" t="n">
-        <v>2.310860650559303</v>
+        <v>2.350652714623625</v>
       </c>
       <c r="N53" t="n">
         <v>1.48</v>
@@ -12622,7 +12622,7 @@
         <v>39687220.36</v>
       </c>
       <c r="AM53" t="n">
-        <v>45315364.2384106</v>
+        <v>46095676.05705553</v>
       </c>
       <c r="AN53" t="n">
         <v>0</v>
@@ -12672,16 +12672,16 @@
         <v>0</v>
       </c>
       <c r="BC53" t="n">
-        <v>-39.37</v>
+        <v>-40.38</v>
       </c>
       <c r="BD53" t="n">
-        <v>-50.5</v>
+        <v>-51.32</v>
       </c>
       <c r="BE53" t="n">
         <v>-100</v>
       </c>
       <c r="BF53" t="n">
-        <v>-95.54000000000001</v>
+        <v>-95.61</v>
       </c>
       <c r="BG53" t="n">
         <v>-100</v>
@@ -12693,7 +12693,7 @@
         <v>0</v>
       </c>
       <c r="BJ53" t="n">
-        <v>6.5</v>
+        <v>6.61</v>
       </c>
       <c r="BK53" t="n">
         <v>0.29</v>
@@ -12702,7 +12702,7 @@
         <v>0.09</v>
       </c>
       <c r="BM53" t="n">
-        <v>6.69</v>
+        <v>6.73</v>
       </c>
       <c r="BN53" t="n">
         <v>10.39</v>
@@ -12711,19 +12711,19 @@
         <v>4.82</v>
       </c>
       <c r="BP53" t="n">
-        <v>6.48</v>
+        <v>6.43</v>
       </c>
       <c r="BQ53" t="n">
-        <v>76.18000000000001</v>
+        <v>77.47</v>
       </c>
       <c r="BR53" t="n">
-        <v>6.55</v>
+        <v>6.51</v>
       </c>
       <c r="BS53" t="n">
         <v>2.36</v>
       </c>
       <c r="BT53" t="n">
-        <v>38900</v>
+        <v>38050</v>
       </c>
     </row>
     <row r="54">
@@ -12753,13 +12753,13 @@
         </is>
       </c>
       <c r="F54" t="n">
-        <v>10.37</v>
+        <v>10.55</v>
       </c>
       <c r="G54" t="n">
-        <v>2418409450</v>
+        <v>2461104044</v>
       </c>
       <c r="H54" t="n">
-        <v>193700</v>
+        <v>273200</v>
       </c>
       <c r="I54" t="n">
         <v>233212121</v>
@@ -12774,7 +12774,7 @@
         <v>0.97</v>
       </c>
       <c r="M54" t="n">
-        <v>1.35743286261266</v>
+        <v>1.38139697875995</v>
       </c>
       <c r="N54" t="n">
         <v>0.5600000000000001</v>
@@ -12852,7 +12852,7 @@
         <v>233212121</v>
       </c>
       <c r="AM54" t="n">
-        <v>330835766.0738714</v>
+        <v>336676339.8084816</v>
       </c>
       <c r="AN54" t="n">
         <v>0.1531</v>
@@ -12893,7 +12893,7 @@
         <v>12.25</v>
       </c>
       <c r="AZ54" t="n">
-        <v>16.51</v>
+        <v>16.79</v>
       </c>
       <c r="BA54" t="n">
         <v>0.98</v>
@@ -12902,19 +12902,19 @@
         <v>6.52</v>
       </c>
       <c r="BC54" t="n">
-        <v>44.72</v>
+        <v>42.25</v>
       </c>
       <c r="BD54" t="n">
-        <v>18.16</v>
+        <v>16.15</v>
       </c>
       <c r="BE54" t="n">
         <v>59.17</v>
       </c>
       <c r="BF54" t="n">
-        <v>-90.52</v>
+        <v>-90.68000000000001</v>
       </c>
       <c r="BG54" t="n">
-        <v>-37.16</v>
+        <v>-38.23</v>
       </c>
       <c r="BH54" t="n">
         <v>10.01</v>
@@ -12923,7 +12923,7 @@
         <v>0</v>
       </c>
       <c r="BJ54" t="n">
-        <v>10.37</v>
+        <v>10.55</v>
       </c>
       <c r="BK54" t="n">
         <v>1</v>
@@ -12932,7 +12932,7 @@
         <v>1</v>
       </c>
       <c r="BM54" t="n">
-        <v>10.5</v>
+        <v>10.63</v>
       </c>
       <c r="BN54" t="n">
         <v>11.75</v>
@@ -12944,16 +12944,16 @@
         <v>10.26</v>
       </c>
       <c r="BQ54" t="n">
-        <v>10.34</v>
+        <v>10.52</v>
       </c>
       <c r="BR54" t="n">
-        <v>10.39</v>
+        <v>10.31</v>
       </c>
       <c r="BS54" t="n">
         <v>1.26</v>
       </c>
       <c r="BT54" t="n">
-        <v>263377</v>
+        <v>264583</v>
       </c>
     </row>
     <row r="55">
@@ -12983,13 +12983,13 @@
         </is>
       </c>
       <c r="F55" t="n">
-        <v>49.52</v>
+        <v>49.23</v>
       </c>
       <c r="G55" t="n">
-        <v>6578755376</v>
+        <v>6562892176</v>
       </c>
       <c r="H55" t="n">
-        <v>13600</v>
+        <v>15900</v>
       </c>
       <c r="I55" t="n">
         <v>84052790</v>
@@ -13004,7 +13004,7 @@
         <v>2</v>
       </c>
       <c r="M55" t="n">
-        <v>1.015570088315727</v>
+        <v>1.013121267755574</v>
       </c>
       <c r="N55" t="n">
         <v>0.16</v>
@@ -13082,7 +13082,7 @@
         <v>579123723.1</v>
       </c>
       <c r="AM55" t="n">
-        <v>330923308.6519115</v>
+        <v>330125360.9657948</v>
       </c>
       <c r="AN55" t="n">
         <v>3.1953</v>
@@ -13123,7 +13123,7 @@
         <v>51.21</v>
       </c>
       <c r="AZ55" t="n">
-        <v>52.08</v>
+        <v>51.77</v>
       </c>
       <c r="BA55" t="n">
         <v>9.380000000000001</v>
@@ -13132,19 +13132,19 @@
         <v>16.08</v>
       </c>
       <c r="BC55" t="n">
-        <v>26.64</v>
+        <v>27.39</v>
       </c>
       <c r="BD55" t="n">
-        <v>3.4</v>
+        <v>4.01</v>
       </c>
       <c r="BE55" t="n">
         <v>5.17</v>
       </c>
       <c r="BF55" t="n">
-        <v>-81.06</v>
+        <v>-80.95</v>
       </c>
       <c r="BG55" t="n">
-        <v>-67.54000000000001</v>
+        <v>-67.34</v>
       </c>
       <c r="BH55" t="n">
         <v>25.37</v>
@@ -13153,7 +13153,7 @@
         <v>0</v>
       </c>
       <c r="BJ55" t="n">
-        <v>49.52</v>
+        <v>49.23</v>
       </c>
       <c r="BK55" t="n">
         <v>6.89</v>
@@ -13162,7 +13162,7 @@
         <v>7.03</v>
       </c>
       <c r="BM55" t="n">
-        <v>49.65</v>
+        <v>49.52</v>
       </c>
       <c r="BN55" t="n">
         <v>73.67</v>
@@ -13171,19 +13171,19 @@
         <v>35.58</v>
       </c>
       <c r="BP55" t="n">
-        <v>49.24</v>
+        <v>49.1</v>
       </c>
       <c r="BQ55" t="n">
-        <v>7.04</v>
+        <v>7</v>
       </c>
       <c r="BR55" t="n">
-        <v>49.65</v>
+        <v>49.52</v>
       </c>
       <c r="BS55" t="n">
         <v>0.66</v>
       </c>
       <c r="BT55" t="n">
-        <v>6860</v>
+        <v>7180</v>
       </c>
     </row>
     <row r="56">
@@ -13213,13 +13213,13 @@
         </is>
       </c>
       <c r="F56" t="n">
-        <v>59.49</v>
+        <v>59.84</v>
       </c>
       <c r="G56" t="n">
-        <v>6578755376</v>
+        <v>6562892176</v>
       </c>
       <c r="H56" t="n">
-        <v>49500</v>
+        <v>16200</v>
       </c>
       <c r="I56" t="n">
         <v>39675836</v>
@@ -13234,7 +13234,7 @@
         <v>2.41</v>
       </c>
       <c r="M56" t="n">
-        <v>2.151473238358061</v>
+        <v>2.146285440921599</v>
       </c>
       <c r="N56" t="n">
         <v>0.19</v>
@@ -13312,7 +13312,7 @@
         <v>273366510.04</v>
       </c>
       <c r="AM56" t="n">
-        <v>273658709.484193</v>
+        <v>272998842.5956739</v>
       </c>
       <c r="AN56" t="n">
         <v>3.5102</v>
@@ -13353,7 +13353,7 @@
         <v>51.21</v>
       </c>
       <c r="AZ56" t="n">
-        <v>56.81</v>
+        <v>57.15</v>
       </c>
       <c r="BA56" t="n">
         <v>9.380000000000001</v>
@@ -13362,19 +13362,19 @@
         <v>17.68</v>
       </c>
       <c r="BC56" t="n">
-        <v>5.42</v>
+        <v>4.8</v>
       </c>
       <c r="BD56" t="n">
-        <v>-13.93</v>
+        <v>-14.43</v>
       </c>
       <c r="BE56" t="n">
         <v>-4.5</v>
       </c>
       <c r="BF56" t="n">
-        <v>-84.23999999999999</v>
+        <v>-84.33</v>
       </c>
       <c r="BG56" t="n">
-        <v>-70.28</v>
+        <v>-70.45999999999999</v>
       </c>
       <c r="BH56" t="n">
         <v>25.37</v>
@@ -13383,7 +13383,7 @@
         <v>0</v>
       </c>
       <c r="BJ56" t="n">
-        <v>59.49</v>
+        <v>59.84</v>
       </c>
       <c r="BK56" t="n">
         <v>6.89</v>
@@ -13392,7 +13392,7 @@
         <v>7.03</v>
       </c>
       <c r="BM56" t="n">
-        <v>60.77</v>
+        <v>60.55</v>
       </c>
       <c r="BN56" t="n">
         <v>86.77</v>
@@ -13401,19 +13401,19 @@
         <v>46.42</v>
       </c>
       <c r="BP56" t="n">
-        <v>58.1</v>
+        <v>58.58</v>
       </c>
       <c r="BQ56" t="n">
-        <v>8.460000000000001</v>
+        <v>8.51</v>
       </c>
       <c r="BR56" t="n">
-        <v>58.7</v>
+        <v>59.99</v>
       </c>
       <c r="BS56" t="n">
         <v>0.79</v>
       </c>
       <c r="BT56" t="n">
-        <v>33970</v>
+        <v>35013</v>
       </c>
     </row>
     <row r="57">
@@ -13443,13 +13443,13 @@
         </is>
       </c>
       <c r="F57" t="n">
-        <v>6.16</v>
+        <v>6.03</v>
       </c>
       <c r="G57" t="n">
-        <v>1440565244</v>
+        <v>1410574432</v>
       </c>
       <c r="H57" t="n">
-        <v>1377200</v>
+        <v>1147700</v>
       </c>
       <c r="I57" t="n">
         <v>233858065</v>
@@ -13464,7 +13464,7 @@
         <v>0.77</v>
       </c>
       <c r="M57" t="n">
-        <v>0.4311998693737589</v>
+        <v>0.4222228138251294</v>
       </c>
       <c r="N57" t="n">
         <v>0.08</v>
@@ -13542,7 +13542,7 @@
         <v>229180903.7</v>
       </c>
       <c r="AM57" t="n">
-        <v>107746091.5482423</v>
+        <v>105502949.289454</v>
       </c>
       <c r="AN57" t="n">
         <v>0.347</v>
@@ -13583,7 +13583,7 @@
         <v>10.72</v>
       </c>
       <c r="AZ57" t="n">
-        <v>9.390000000000001</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="BA57" t="n">
         <v>1.13</v>
@@ -13592,19 +13592,19 @@
         <v>6.26</v>
       </c>
       <c r="BC57" t="n">
-        <v>113.17</v>
+        <v>117.77</v>
       </c>
       <c r="BD57" t="n">
-        <v>74.05</v>
+        <v>77.81</v>
       </c>
       <c r="BE57" t="n">
         <v>52.5</v>
       </c>
       <c r="BF57" t="n">
-        <v>-81.7</v>
+        <v>-81.3</v>
       </c>
       <c r="BG57" t="n">
-        <v>1.69</v>
+        <v>3.88</v>
       </c>
       <c r="BH57" t="n">
         <v>7.82</v>
@@ -13613,7 +13613,7 @@
         <v>0</v>
       </c>
       <c r="BJ57" t="n">
-        <v>6.16</v>
+        <v>6.03</v>
       </c>
       <c r="BK57" t="n">
         <v>0.98</v>
@@ -13622,28 +13622,28 @@
         <v>1.04</v>
       </c>
       <c r="BM57" t="n">
-        <v>6.18</v>
+        <v>6.16</v>
       </c>
       <c r="BN57" t="n">
         <v>6.18</v>
       </c>
       <c r="BO57" t="n">
-        <v>3.42</v>
+        <v>3.43</v>
       </c>
       <c r="BP57" t="n">
-        <v>5.93</v>
+        <v>5.98</v>
       </c>
       <c r="BQ57" t="n">
-        <v>5.95</v>
+        <v>5.82</v>
       </c>
       <c r="BR57" t="n">
-        <v>6.03</v>
+        <v>6.15</v>
       </c>
       <c r="BS57" t="n">
         <v>0.42</v>
       </c>
       <c r="BT57" t="n">
-        <v>1305155</v>
+        <v>1300412</v>
       </c>
     </row>
     <row r="58">
@@ -14133,13 +14133,13 @@
         </is>
       </c>
       <c r="F60" t="n">
-        <v>373.01</v>
+        <v>376</v>
       </c>
       <c r="G60" t="n">
-        <v>169626264</v>
+        <v>171035782</v>
       </c>
       <c r="H60" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="I60" t="n">
         <v>454750</v>
@@ -14154,7 +14154,7 @@
         <v>0.83</v>
       </c>
       <c r="M60" t="n">
-        <v>12.68780576331641</v>
+        <v>12.79323572552968</v>
       </c>
       <c r="N60" t="n">
         <v>0.68</v>
@@ -14232,7 +14232,7 @@
         <v>59558607.5</v>
       </c>
       <c r="AM60" t="n">
-        <v>-24871886.2170088</v>
+        <v>-25078560.41055718</v>
       </c>
       <c r="AN60" t="n">
         <v>10.0581</v>
@@ -14273,7 +14273,7 @@
         <v>944.87</v>
       </c>
       <c r="AZ60" t="n">
-        <v>2144.81</v>
+        <v>2162</v>
       </c>
       <c r="BA60" t="n">
         <v>231.1</v>
@@ -14282,19 +14282,19 @@
         <v>727.97</v>
       </c>
       <c r="BC60" t="n">
-        <v>210.24</v>
+        <v>207.77</v>
       </c>
       <c r="BD60" t="n">
-        <v>153.31</v>
+        <v>151.29</v>
       </c>
       <c r="BE60" t="n">
         <v>475</v>
       </c>
       <c r="BF60" t="n">
-        <v>-38.05</v>
+        <v>-38.54</v>
       </c>
       <c r="BG60" t="n">
-        <v>95.16</v>
+        <v>93.61</v>
       </c>
       <c r="BH60" t="n">
         <v>454.44</v>
@@ -14303,7 +14303,7 @@
         <v>0</v>
       </c>
       <c r="BJ60" t="n">
-        <v>373.01</v>
+        <v>376</v>
       </c>
       <c r="BK60" t="n">
         <v>130.97</v>
@@ -14312,7 +14312,7 @@
         <v>130.97</v>
       </c>
       <c r="BM60" t="n">
-        <v>377</v>
+        <v>377.09</v>
       </c>
       <c r="BN60" t="n">
         <v>405</v>
@@ -14321,13 +14321,13 @@
         <v>306.27</v>
       </c>
       <c r="BP60" t="n">
-        <v>372</v>
+        <v>376</v>
       </c>
       <c r="BQ60" t="n">
-        <v>2.85</v>
+        <v>2.87</v>
       </c>
       <c r="BR60" t="n">
-        <v>372</v>
+        <v>377</v>
       </c>
       <c r="BS60" t="n">
         <v>12.82</v>
@@ -14363,13 +14363,13 @@
         </is>
       </c>
       <c r="F61" t="n">
-        <v>27.65</v>
+        <v>27.45</v>
       </c>
       <c r="G61" t="n">
-        <v>2367072227</v>
+        <v>2350634150</v>
       </c>
       <c r="H61" t="n">
-        <v>433400</v>
+        <v>560200</v>
       </c>
       <c r="I61" t="n">
         <v>85608392</v>
@@ -14384,7 +14384,7 @@
         <v>2.37</v>
       </c>
       <c r="M61" t="n">
-        <v>1.255339672001435</v>
+        <v>1.246621995390583</v>
       </c>
       <c r="N61" t="n">
         <v>1.1</v>
@@ -14462,7 +14462,7 @@
         <v>160087693.04</v>
       </c>
       <c r="AM61" t="n">
-        <v>185798447.9591837</v>
+        <v>184508175.0392465</v>
       </c>
       <c r="AN61" t="n">
         <v>0.38</v>
@@ -14503,7 +14503,7 @@
         <v>17.56</v>
       </c>
       <c r="AZ61" t="n">
-        <v>34.84</v>
+        <v>34.59</v>
       </c>
       <c r="BA61" t="n">
         <v>2.52</v>
@@ -14512,19 +14512,19 @@
         <v>11.76</v>
       </c>
       <c r="BC61" t="n">
-        <v>-22.23</v>
+        <v>-21.66</v>
       </c>
       <c r="BD61" t="n">
-        <v>-36.5</v>
+        <v>-36.04</v>
       </c>
       <c r="BE61" t="n">
         <v>26</v>
       </c>
       <c r="BF61" t="n">
-        <v>-90.88</v>
+        <v>-90.81</v>
       </c>
       <c r="BG61" t="n">
-        <v>-57.48</v>
+        <v>-57.17</v>
       </c>
       <c r="BH61" t="n">
         <v>10.99</v>
@@ -14533,7 +14533,7 @@
         <v>0</v>
       </c>
       <c r="BJ61" t="n">
-        <v>27.65</v>
+        <v>27.45</v>
       </c>
       <c r="BK61" t="n">
         <v>1.87</v>
@@ -14542,7 +14542,7 @@
         <v>1.86</v>
       </c>
       <c r="BM61" t="n">
-        <v>27.78</v>
+        <v>28</v>
       </c>
       <c r="BN61" t="n">
         <v>28.25</v>
@@ -14551,19 +14551,19 @@
         <v>19.35</v>
       </c>
       <c r="BP61" t="n">
-        <v>26.76</v>
+        <v>26.88</v>
       </c>
       <c r="BQ61" t="n">
-        <v>14.85</v>
+        <v>14.74</v>
       </c>
       <c r="BR61" t="n">
-        <v>26.93</v>
+        <v>27.6</v>
       </c>
       <c r="BS61" t="n">
         <v>1.19</v>
       </c>
       <c r="BT61" t="n">
-        <v>500434</v>
+        <v>504287</v>
       </c>
     </row>
     <row r="62">
@@ -14593,13 +14593,13 @@
         </is>
       </c>
       <c r="F62" t="n">
-        <v>109.25</v>
+        <v>115.24</v>
       </c>
       <c r="G62" t="n">
-        <v>10782950000</v>
+        <v>11377473281</v>
       </c>
       <c r="H62" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="I62" t="n">
         <v>98699749</v>
@@ -14614,7 +14614,7 @@
         <v>0.64</v>
       </c>
       <c r="M62" t="n">
-        <v>1.010777786066382</v>
+        <v>1.06650751918525</v>
       </c>
       <c r="N62" t="n">
         <v>0.13</v>
@@ -14692,7 +14692,7 @@
         <v>2757670987.06</v>
       </c>
       <c r="AM62" t="n">
-        <v>4365566801.619432</v>
+        <v>4606264486.234818</v>
       </c>
       <c r="AN62" t="n">
         <v>6.9319</v>
@@ -14733,7 +14733,7 @@
         <v>267.2</v>
       </c>
       <c r="AZ62" t="n">
-        <v>115.44</v>
+        <v>121.77</v>
       </c>
       <c r="BA62" t="n">
         <v>34.09</v>
@@ -14742,19 +14742,19 @@
         <v>76.01000000000001</v>
       </c>
       <c r="BC62" t="n">
-        <v>199.54</v>
+        <v>183.97</v>
       </c>
       <c r="BD62" t="n">
-        <v>144.57</v>
+        <v>131.86</v>
       </c>
       <c r="BE62" t="n">
         <v>5.67</v>
       </c>
       <c r="BF62" t="n">
-        <v>-68.79000000000001</v>
+        <v>-70.42</v>
       </c>
       <c r="BG62" t="n">
-        <v>-30.43</v>
+        <v>-34.04</v>
       </c>
       <c r="BH62" t="n">
         <v>170.35</v>
@@ -14763,7 +14763,7 @@
         <v>0</v>
       </c>
       <c r="BJ62" t="n">
-        <v>109.25</v>
+        <v>115.24</v>
       </c>
       <c r="BK62" t="n">
         <v>27.94</v>
@@ -14772,28 +14772,28 @@
         <v>32.73</v>
       </c>
       <c r="BM62" t="n">
-        <v>109.25</v>
+        <v>115.24</v>
       </c>
       <c r="BN62" t="n">
         <v>122.2</v>
       </c>
       <c r="BO62" t="n">
-        <v>90.42</v>
+        <v>91.36</v>
       </c>
       <c r="BP62" t="n">
-        <v>109.25</v>
+        <v>115.24</v>
       </c>
       <c r="BQ62" t="n">
-        <v>3.34</v>
+        <v>3.52</v>
       </c>
       <c r="BR62" t="n">
-        <v>109.25</v>
+        <v>115.24</v>
       </c>
       <c r="BS62" t="n">
         <v>1.01</v>
       </c>
       <c r="BT62" t="n">
-        <v>214</v>
+        <v>156</v>
       </c>
     </row>
     <row r="63">
@@ -14823,13 +14823,13 @@
         </is>
       </c>
       <c r="F63" t="n">
-        <v>1.42</v>
+        <v>1.41</v>
       </c>
       <c r="G63" t="n">
-        <v>369923762</v>
+        <v>367425687</v>
       </c>
       <c r="H63" t="n">
-        <v>61000</v>
+        <v>20300</v>
       </c>
       <c r="I63" t="n">
         <v>122894462</v>
@@ -14844,7 +14844,7 @@
         <v>-0.22</v>
       </c>
       <c r="M63" t="n">
-        <v>0.4549871369305478</v>
+        <v>0.451914633596502</v>
       </c>
       <c r="N63" t="n">
         <v>0.37</v>
@@ -14922,7 +14922,7 @@
         <v>31952560.12</v>
       </c>
       <c r="AM63" t="n">
-        <v>210183955.6818182</v>
+        <v>208764594.8863636</v>
       </c>
       <c r="AN63" t="n">
         <v>0</v>
@@ -14981,7 +14981,7 @@
         <v>-100</v>
       </c>
       <c r="BF63" t="n">
-        <v>-79.64</v>
+        <v>-79.48999999999999</v>
       </c>
       <c r="BG63" t="n">
         <v>-100</v>
@@ -14993,7 +14993,7 @@
         <v>0</v>
       </c>
       <c r="BJ63" t="n">
-        <v>1.42</v>
+        <v>1.41</v>
       </c>
       <c r="BK63" t="n">
         <v>0.26</v>
@@ -15002,7 +15002,7 @@
         <v>0.26</v>
       </c>
       <c r="BM63" t="n">
-        <v>1.88</v>
+        <v>1.52</v>
       </c>
       <c r="BN63" t="n">
         <v>2.12</v>
@@ -15011,19 +15011,19 @@
         <v>1.16</v>
       </c>
       <c r="BP63" t="n">
-        <v>1.41</v>
+        <v>1.36</v>
       </c>
       <c r="BQ63" t="n">
-        <v>5.44</v>
+        <v>5.4</v>
       </c>
       <c r="BR63" t="n">
-        <v>1.65</v>
+        <v>1.51</v>
       </c>
       <c r="BS63" t="n">
         <v>0.19</v>
       </c>
       <c r="BT63" t="n">
-        <v>20063</v>
+        <v>22040</v>
       </c>
     </row>
     <row r="64">
@@ -15053,13 +15053,13 @@
         </is>
       </c>
       <c r="F64" t="n">
-        <v>60.2</v>
+        <v>60.83</v>
       </c>
       <c r="G64" t="n">
-        <v>230868267125</v>
+        <v>234363823664</v>
       </c>
       <c r="H64" t="n">
-        <v>5207200</v>
+        <v>10448200</v>
       </c>
       <c r="I64" t="n">
         <v>0</v>
@@ -15146,13 +15146,13 @@
         <v>41.22</v>
       </c>
       <c r="AK64" t="n">
-        <v>66193319985.33168</v>
+        <v>67195547339.45985</v>
       </c>
       <c r="AL64" t="n">
-        <v>18454697611.91047</v>
+        <v>18734118598.24141</v>
       </c>
       <c r="AM64" t="n">
-        <v>20558171605.07569</v>
+        <v>20869441109.88424</v>
       </c>
       <c r="AN64" t="n">
         <v>1.4201</v>
@@ -15193,7 +15193,7 @@
         <v>38.98</v>
       </c>
       <c r="AZ64" t="n">
-        <v>24.08</v>
+        <v>24.33</v>
       </c>
       <c r="BA64" t="n">
         <v>6.69</v>
@@ -15202,19 +15202,19 @@
         <v>10.4</v>
       </c>
       <c r="BC64" t="n">
-        <v>-20.7</v>
+        <v>-21.52</v>
       </c>
       <c r="BD64" t="n">
-        <v>-35.25</v>
+        <v>-35.92</v>
       </c>
       <c r="BE64" t="n">
         <v>-60</v>
       </c>
       <c r="BF64" t="n">
-        <v>-88.88</v>
+        <v>-89</v>
       </c>
       <c r="BG64" t="n">
-        <v>-82.73</v>
+        <v>-82.91</v>
       </c>
       <c r="BH64" t="n">
         <v>21.37</v>
@@ -15223,7 +15223,7 @@
         <v>0</v>
       </c>
       <c r="BJ64" t="n">
-        <v>60.2</v>
+        <v>60.83</v>
       </c>
       <c r="BK64" t="n">
         <v>4.74</v>
@@ -15232,7 +15232,7 @@
         <v>1.57</v>
       </c>
       <c r="BM64" t="n">
-        <v>60.98</v>
+        <v>61.2</v>
       </c>
       <c r="BN64" t="n">
         <v>64.72</v>
@@ -15241,19 +15241,19 @@
         <v>44.12</v>
       </c>
       <c r="BP64" t="n">
-        <v>60.06</v>
+        <v>59.81</v>
       </c>
       <c r="BQ64" t="n">
-        <v>38.34</v>
+        <v>38.74</v>
       </c>
       <c r="BR64" t="n">
-        <v>60.98</v>
+        <v>60.17</v>
       </c>
       <c r="BS64" t="n">
         <v>3.49</v>
       </c>
       <c r="BT64" t="n">
-        <v>12462611</v>
+        <v>12430983</v>
       </c>
     </row>
     <row r="65">
@@ -15283,13 +15283,13 @@
         </is>
       </c>
       <c r="F65" t="n">
-        <v>23.55</v>
+        <v>23.75</v>
       </c>
       <c r="G65" t="n">
-        <v>230868267125</v>
+        <v>234363823664</v>
       </c>
       <c r="H65" t="n">
-        <v>5700</v>
+        <v>2400</v>
       </c>
       <c r="I65" t="n">
         <v>7298813414</v>
@@ -15304,7 +15304,7 @@
         <v>3.29</v>
       </c>
       <c r="M65" t="n">
-        <v>5.58145803925793</v>
+        <v>5.665966414485257</v>
       </c>
       <c r="N65" t="n">
         <v>0.29</v>
@@ -15382,7 +15382,7 @@
         <v>11532125194.12</v>
       </c>
       <c r="AM65" t="n">
-        <v>17293503155.43071</v>
+        <v>17555342596.55431</v>
       </c>
       <c r="AN65" t="n">
         <v>0.4734</v>
@@ -15423,7 +15423,7 @@
         <v>12.99</v>
       </c>
       <c r="AZ65" t="n">
-        <v>7.93</v>
+        <v>8</v>
       </c>
       <c r="BA65" t="n">
         <v>2.23</v>
@@ -15432,19 +15432,19 @@
         <v>3.47</v>
       </c>
       <c r="BC65" t="n">
-        <v>-32.44</v>
+        <v>-33.01</v>
       </c>
       <c r="BD65" t="n">
-        <v>-44.84</v>
+        <v>-45.3</v>
       </c>
       <c r="BE65" t="n">
         <v>-66.33</v>
       </c>
       <c r="BF65" t="n">
-        <v>-90.53</v>
+        <v>-90.61</v>
       </c>
       <c r="BG65" t="n">
-        <v>-85.28</v>
+        <v>-85.41</v>
       </c>
       <c r="BH65" t="n">
         <v>7.12</v>
@@ -15453,7 +15453,7 @@
         <v>0</v>
       </c>
       <c r="BJ65" t="n">
-        <v>23.55</v>
+        <v>23.75</v>
       </c>
       <c r="BK65" t="n">
         <v>1.58</v>
@@ -15471,10 +15471,10 @@
         <v>20.44</v>
       </c>
       <c r="BP65" t="n">
-        <v>23.55</v>
+        <v>23.53</v>
       </c>
       <c r="BQ65" t="n">
-        <v>15</v>
+        <v>15.13</v>
       </c>
       <c r="BR65" t="n">
         <v>23.89</v>
@@ -15483,7 +15483,7 @@
         <v>4.14</v>
       </c>
       <c r="BT65" t="n">
-        <v>12089</v>
+        <v>11757</v>
       </c>
     </row>
     <row r="66">
@@ -15513,13 +15513,13 @@
         </is>
       </c>
       <c r="F66" t="n">
-        <v>20.17</v>
+        <v>21</v>
       </c>
       <c r="G66" t="n">
-        <v>230376543536</v>
+        <v>234363823664</v>
       </c>
       <c r="H66" t="n">
-        <v>200</v>
+        <v>2000</v>
       </c>
       <c r="I66" t="n">
         <v>2972355254</v>
@@ -15534,7 +15534,7 @@
         <v>2.75</v>
       </c>
       <c r="M66" t="n">
-        <v>13.67644507623102</v>
+        <v>13.91315241126237</v>
       </c>
       <c r="N66" t="n">
         <v>0.25</v>
@@ -15612,7 +15612,7 @@
         <v>4696321301.320001</v>
       </c>
       <c r="AM66" t="n">
-        <v>20661573411.30045</v>
+        <v>21019177010.22422</v>
       </c>
       <c r="AN66" t="n">
         <v>0.4734</v>
@@ -15653,7 +15653,7 @@
         <v>12.99</v>
       </c>
       <c r="AZ66" t="n">
-        <v>8.1</v>
+        <v>8.44</v>
       </c>
       <c r="BA66" t="n">
         <v>2.23</v>
@@ -15662,19 +15662,19 @@
         <v>3.47</v>
       </c>
       <c r="BC66" t="n">
-        <v>-21.12</v>
+        <v>-24.24</v>
       </c>
       <c r="BD66" t="n">
-        <v>-35.6</v>
+        <v>-38.14</v>
       </c>
       <c r="BE66" t="n">
         <v>-59.83</v>
       </c>
       <c r="BF66" t="n">
-        <v>-88.94</v>
+        <v>-89.37</v>
       </c>
       <c r="BG66" t="n">
-        <v>-82.81999999999999</v>
+        <v>-83.5</v>
       </c>
       <c r="BH66" t="n">
         <v>7.12</v>
@@ -15683,7 +15683,7 @@
         <v>0</v>
       </c>
       <c r="BJ66" t="n">
-        <v>20.17</v>
+        <v>21</v>
       </c>
       <c r="BK66" t="n">
         <v>1.58</v>
@@ -15692,7 +15692,7 @@
         <v>1.57</v>
       </c>
       <c r="BM66" t="n">
-        <v>21.33</v>
+        <v>21.04</v>
       </c>
       <c r="BN66" t="n">
         <v>21.33</v>
@@ -15704,16 +15704,16 @@
         <v>20.17</v>
       </c>
       <c r="BQ66" t="n">
-        <v>12.85</v>
+        <v>13.37</v>
       </c>
       <c r="BR66" t="n">
-        <v>21.33</v>
+        <v>20.17</v>
       </c>
       <c r="BS66" t="n">
         <v>3.46</v>
       </c>
       <c r="BT66" t="n">
-        <v>7113</v>
+        <v>7015</v>
       </c>
     </row>
     <row r="67">
@@ -15973,13 +15973,13 @@
         </is>
       </c>
       <c r="F68" t="n">
-        <v>18.7</v>
+        <v>18.43</v>
       </c>
       <c r="G68" t="n">
-        <v>8051979740</v>
+        <v>7825980923</v>
       </c>
       <c r="H68" t="n">
-        <v>44000</v>
+        <v>70000</v>
       </c>
       <c r="I68" t="n">
         <v>137989898</v>
@@ -16072,7 +16072,7 @@
         <v>205604948.02</v>
       </c>
       <c r="AM68" t="n">
-        <v>558389718.446602</v>
+        <v>542717123.6477115</v>
       </c>
       <c r="AN68" t="n">
         <v>0.1911</v>
@@ -16113,7 +16113,7 @@
         <v>21.39</v>
       </c>
       <c r="AZ68" t="n">
-        <v>34.6</v>
+        <v>34.1</v>
       </c>
       <c r="BA68" t="n">
         <v>1.24</v>
@@ -16122,19 +16122,19 @@
         <v>63.25</v>
       </c>
       <c r="BC68" t="n">
-        <v>40.12</v>
+        <v>42.18</v>
       </c>
       <c r="BD68" t="n">
-        <v>14.41</v>
+        <v>16.09</v>
       </c>
       <c r="BE68" t="n">
         <v>85</v>
       </c>
       <c r="BF68" t="n">
-        <v>-93.37</v>
+        <v>-93.27</v>
       </c>
       <c r="BG68" t="n">
-        <v>238.23</v>
+        <v>243.18</v>
       </c>
       <c r="BH68" t="n">
         <v>20.48</v>
@@ -16143,7 +16143,7 @@
         <v>0</v>
       </c>
       <c r="BJ68" t="n">
-        <v>18.7</v>
+        <v>18.43</v>
       </c>
       <c r="BK68" t="n">
         <v>1.49</v>
@@ -16152,28 +16152,28 @@
         <v>1.49</v>
       </c>
       <c r="BM68" t="n">
-        <v>18.84</v>
+        <v>18.7</v>
       </c>
       <c r="BN68" t="n">
         <v>22.11</v>
       </c>
       <c r="BO68" t="n">
-        <v>15.07</v>
+        <v>15.39</v>
       </c>
       <c r="BP68" t="n">
-        <v>18.58</v>
+        <v>18.33</v>
       </c>
       <c r="BQ68" t="n">
-        <v>12.58</v>
+        <v>12.4</v>
       </c>
       <c r="BR68" t="n">
-        <v>18.82</v>
+        <v>18.7</v>
       </c>
       <c r="BS68" t="n">
         <v>0</v>
       </c>
       <c r="BT68" t="n">
-        <v>32470</v>
+        <v>32887</v>
       </c>
     </row>
     <row r="69">
@@ -16203,13 +16203,13 @@
         </is>
       </c>
       <c r="F69" t="n">
-        <v>21.48</v>
+        <v>20.85</v>
       </c>
       <c r="G69" t="n">
-        <v>8051979740</v>
+        <v>7825980923</v>
       </c>
       <c r="H69" t="n">
-        <v>1004500</v>
+        <v>3739600</v>
       </c>
       <c r="I69" t="n">
         <v>255106712</v>
@@ -16302,7 +16302,7 @@
         <v>380109000.88</v>
       </c>
       <c r="AM69" t="n">
-        <v>479284508.3333333</v>
+        <v>465832197.797619</v>
       </c>
       <c r="AN69" t="n">
         <v>0.8856000000000001</v>
@@ -16343,7 +16343,7 @@
         <v>21.39</v>
       </c>
       <c r="AZ69" t="n">
-        <v>37.55</v>
+        <v>36.45</v>
       </c>
       <c r="BA69" t="n">
         <v>1.24</v>
@@ -16352,19 +16352,19 @@
         <v>69.59</v>
       </c>
       <c r="BC69" t="n">
-        <v>21.99</v>
+        <v>25.67</v>
       </c>
       <c r="BD69" t="n">
-        <v>-0.4</v>
+        <v>2.61</v>
       </c>
       <c r="BE69" t="n">
         <v>74.83</v>
       </c>
       <c r="BF69" t="n">
-        <v>-94.23</v>
+        <v>-94.06</v>
       </c>
       <c r="BG69" t="n">
-        <v>223.96</v>
+        <v>233.75</v>
       </c>
       <c r="BH69" t="n">
         <v>20.48</v>
@@ -16373,7 +16373,7 @@
         <v>0</v>
       </c>
       <c r="BJ69" t="n">
-        <v>21.48</v>
+        <v>20.85</v>
       </c>
       <c r="BK69" t="n">
         <v>1.49</v>
@@ -16382,7 +16382,7 @@
         <v>1.49</v>
       </c>
       <c r="BM69" t="n">
-        <v>21.8</v>
+        <v>21.61</v>
       </c>
       <c r="BN69" t="n">
         <v>25.63</v>
@@ -16391,19 +16391,19 @@
         <v>16.73</v>
       </c>
       <c r="BP69" t="n">
-        <v>21.36</v>
+        <v>20.83</v>
       </c>
       <c r="BQ69" t="n">
-        <v>14.45</v>
+        <v>14.02</v>
       </c>
       <c r="BR69" t="n">
-        <v>21.8</v>
+        <v>21.48</v>
       </c>
       <c r="BS69" t="n">
         <v>0</v>
       </c>
       <c r="BT69" t="n">
-        <v>1934300</v>
+        <v>1878750</v>
       </c>
     </row>
     <row r="70">
@@ -16433,13 +16433,13 @@
         </is>
       </c>
       <c r="F70" t="n">
-        <v>17.91</v>
+        <v>17.73</v>
       </c>
       <c r="G70" t="n">
-        <v>8320219381</v>
+        <v>8238997812</v>
       </c>
       <c r="H70" t="n">
-        <v>2729900</v>
+        <v>3314100</v>
       </c>
       <c r="I70" t="n">
         <v>464557268</v>
@@ -16454,7 +16454,7 @@
         <v>0.68</v>
       </c>
       <c r="M70" t="n">
-        <v>0.656699898271028</v>
+        <v>0.6502892264296681</v>
       </c>
       <c r="N70" t="n">
         <v>0.2</v>
@@ -16532,7 +16532,7 @@
         <v>55746872.16</v>
       </c>
       <c r="AM70" t="n">
-        <v>2745946990.429043</v>
+        <v>2719141192.079208</v>
       </c>
       <c r="AN70" t="n">
         <v>0.1236</v>
@@ -16573,7 +16573,7 @@
         <v>6.9</v>
       </c>
       <c r="AZ70" t="n">
-        <v>2.06</v>
+        <v>2.04</v>
       </c>
       <c r="BA70" t="n">
         <v>0.12</v>
@@ -16582,19 +16582,19 @@
         <v>1.07</v>
       </c>
       <c r="BC70" t="n">
-        <v>-52.82</v>
+        <v>-52.35</v>
       </c>
       <c r="BD70" t="n">
-        <v>-61.48</v>
+        <v>-61.09</v>
       </c>
       <c r="BE70" t="n">
         <v>-88.5</v>
       </c>
       <c r="BF70" t="n">
-        <v>-99.33</v>
+        <v>-99.31999999999999</v>
       </c>
       <c r="BG70" t="n">
-        <v>-94.03</v>
+        <v>-93.97</v>
       </c>
       <c r="BH70" t="n">
         <v>26.44</v>
@@ -16603,7 +16603,7 @@
         <v>0</v>
       </c>
       <c r="BJ70" t="n">
-        <v>17.91</v>
+        <v>17.73</v>
       </c>
       <c r="BK70" t="n">
         <v>0.12</v>
@@ -16612,7 +16612,7 @@
         <v>0.1</v>
       </c>
       <c r="BM70" t="n">
-        <v>18.1</v>
+        <v>17.81</v>
       </c>
       <c r="BN70" t="n">
         <v>22.15</v>
@@ -16621,19 +16621,19 @@
         <v>13.21</v>
       </c>
       <c r="BP70" t="n">
-        <v>17.57</v>
+        <v>17.55</v>
       </c>
       <c r="BQ70" t="n">
-        <v>179.62</v>
+        <v>177.82</v>
       </c>
       <c r="BR70" t="n">
-        <v>17.71</v>
+        <v>17.8</v>
       </c>
       <c r="BS70" t="n">
         <v>0.67</v>
       </c>
       <c r="BT70" t="n">
-        <v>5622153</v>
+        <v>5387240</v>
       </c>
     </row>
     <row r="71">

</xml_diff>

<commit_message>
📊 Dados atualizados - 2026-09-18 05:26
</commit_message>
<xml_diff>
--- a/data/ativos.xlsx
+++ b/data/ativos.xlsx
@@ -1047,13 +1047,13 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>24.66</v>
+        <v>24.97</v>
       </c>
       <c r="G3" t="n">
-        <v>3299651007</v>
+        <v>3340159401</v>
       </c>
       <c r="H3" t="n">
-        <v>488500</v>
+        <v>332600</v>
       </c>
       <c r="I3" t="n">
         <v>129510368</v>
@@ -1068,7 +1068,7 @@
         <v>0.88</v>
       </c>
       <c r="M3" t="n">
-        <v>0.8210266584657016</v>
+        <v>0.8311060490724889</v>
       </c>
       <c r="N3" t="n">
         <v>0.09</v>
@@ -1146,7 +1146,7 @@
         <v>506385538.88</v>
       </c>
       <c r="AM3" t="n">
-        <v>644463087.3046875</v>
+        <v>652374883.0078125</v>
       </c>
       <c r="AN3" t="n">
         <v>2.7</v>
@@ -1187,7 +1187,7 @@
         <v>40.42</v>
       </c>
       <c r="AZ3" t="n">
-        <v>45.13</v>
+        <v>45.7</v>
       </c>
       <c r="BA3" t="n">
         <v>4.87</v>
@@ -1196,19 +1196,19 @@
         <v>21.14</v>
       </c>
       <c r="BC3" t="n">
-        <v>100.72</v>
+        <v>98.23</v>
       </c>
       <c r="BD3" t="n">
-        <v>63.89</v>
+        <v>61.86</v>
       </c>
       <c r="BE3" t="n">
         <v>83</v>
       </c>
       <c r="BF3" t="n">
-        <v>-80.26000000000001</v>
+        <v>-80.5</v>
       </c>
       <c r="BG3" t="n">
-        <v>-14.29</v>
+        <v>-15.36</v>
       </c>
       <c r="BH3" t="n">
         <v>27.85</v>
@@ -1217,7 +1217,7 @@
         <v>0</v>
       </c>
       <c r="BJ3" t="n">
-        <v>24.66</v>
+        <v>24.97</v>
       </c>
       <c r="BK3" t="n">
         <v>3.91</v>
@@ -1226,7 +1226,7 @@
         <v>4.39</v>
       </c>
       <c r="BM3" t="n">
-        <v>24.8</v>
+        <v>25.04</v>
       </c>
       <c r="BN3" t="n">
         <v>27.17</v>
@@ -1235,19 +1235,19 @@
         <v>18.72</v>
       </c>
       <c r="BP3" t="n">
-        <v>24.34</v>
+        <v>24.51</v>
       </c>
       <c r="BQ3" t="n">
-        <v>5.61</v>
+        <v>5.68</v>
       </c>
       <c r="BR3" t="n">
-        <v>24.74</v>
+        <v>24.78</v>
       </c>
       <c r="BS3" t="n">
         <v>0.79</v>
       </c>
       <c r="BT3" t="n">
-        <v>527580</v>
+        <v>520900</v>
       </c>
     </row>
     <row r="4">
@@ -1277,13 +1277,13 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>15.63</v>
+        <v>15.55</v>
       </c>
       <c r="G4" t="n">
-        <v>242095728872</v>
+        <v>240786465953</v>
       </c>
       <c r="H4" t="n">
-        <v>32094600</v>
+        <v>18516700</v>
       </c>
       <c r="I4" t="n">
         <v>15484664889</v>
@@ -1298,7 +1298,7 @@
         <v>2.76</v>
       </c>
       <c r="M4" t="n">
-        <v>2.741257329956459</v>
+        <v>2.726432505948736</v>
       </c>
       <c r="N4" t="n">
         <v>1.76</v>
@@ -1376,7 +1376,7 @@
         <v>16258898133.45</v>
       </c>
       <c r="AM4" t="n">
-        <v>23969874145.74258</v>
+        <v>23840244153.76238</v>
       </c>
       <c r="AN4" t="n">
         <v>0.269</v>
@@ -1417,7 +1417,7 @@
         <v>9.470000000000001</v>
       </c>
       <c r="AZ4" t="n">
-        <v>19.51</v>
+        <v>19.41</v>
       </c>
       <c r="BA4" t="n">
         <v>1.13</v>
@@ -1426,19 +1426,19 @@
         <v>11.39</v>
       </c>
       <c r="BC4" t="n">
-        <v>-25.76</v>
+        <v>-25.37</v>
       </c>
       <c r="BD4" t="n">
-        <v>-39.38</v>
+        <v>-39.07</v>
       </c>
       <c r="BE4" t="n">
         <v>24.83</v>
       </c>
       <c r="BF4" t="n">
-        <v>-92.79000000000001</v>
+        <v>-92.75</v>
       </c>
       <c r="BG4" t="n">
-        <v>-27.15</v>
+        <v>-26.77</v>
       </c>
       <c r="BH4" t="n">
         <v>5.7</v>
@@ -1447,7 +1447,7 @@
         <v>0</v>
       </c>
       <c r="BJ4" t="n">
-        <v>15.63</v>
+        <v>15.55</v>
       </c>
       <c r="BK4" t="n">
         <v>1.05</v>
@@ -1456,7 +1456,7 @@
         <v>1.04</v>
       </c>
       <c r="BM4" t="n">
-        <v>15.77</v>
+        <v>15.73</v>
       </c>
       <c r="BN4" t="n">
         <v>17</v>
@@ -1465,19 +1465,19 @@
         <v>11.09</v>
       </c>
       <c r="BP4" t="n">
-        <v>15.52</v>
+        <v>15.44</v>
       </c>
       <c r="BQ4" t="n">
-        <v>15.07</v>
+        <v>15</v>
       </c>
       <c r="BR4" t="n">
-        <v>15.7</v>
+        <v>15.63</v>
       </c>
       <c r="BS4" t="n">
         <v>2.76</v>
       </c>
       <c r="BT4" t="n">
-        <v>28204413</v>
+        <v>28327710</v>
       </c>
     </row>
     <row r="5">
@@ -3117,13 +3117,13 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>5.13</v>
+        <v>5.06</v>
       </c>
       <c r="G12" t="n">
-        <v>492426043</v>
+        <v>485565336</v>
       </c>
       <c r="H12" t="n">
-        <v>526500</v>
+        <v>351900</v>
       </c>
       <c r="I12" t="n">
         <v>95961536</v>
@@ -3138,7 +3138,7 @@
         <v>0.32</v>
       </c>
       <c r="M12" t="n">
-        <v>0.08905449846623026</v>
+        <v>0.08781375007427578</v>
       </c>
       <c r="N12" t="n">
         <v>0.14</v>
@@ -3216,7 +3216,7 @@
         <v>362734606.08</v>
       </c>
       <c r="AM12" t="n">
-        <v>529490368.8172043</v>
+        <v>522113264.516129</v>
       </c>
       <c r="AN12" t="n">
         <v>0.4208</v>
@@ -3257,7 +3257,7 @@
         <v>30.49</v>
       </c>
       <c r="AZ12" t="n">
-        <v>6.93</v>
+        <v>6.84</v>
       </c>
       <c r="BA12" t="n">
         <v>4.41</v>
@@ -3266,19 +3266,19 @@
         <v>18.12</v>
       </c>
       <c r="BC12" t="n">
-        <v>628.02</v>
+        <v>638.09</v>
       </c>
       <c r="BD12" t="n">
-        <v>494.42</v>
+        <v>502.65</v>
       </c>
       <c r="BE12" t="n">
         <v>35.17</v>
       </c>
       <c r="BF12" t="n">
-        <v>-14</v>
+        <v>-12.81</v>
       </c>
       <c r="BG12" t="n">
-        <v>253.19</v>
+        <v>258.08</v>
       </c>
       <c r="BH12" t="n">
         <v>16.4</v>
@@ -3287,7 +3287,7 @@
         <v>0</v>
       </c>
       <c r="BJ12" t="n">
-        <v>5.13</v>
+        <v>5.06</v>
       </c>
       <c r="BK12" t="n">
         <v>3.78</v>
@@ -3296,7 +3296,7 @@
         <v>3.43</v>
       </c>
       <c r="BM12" t="n">
-        <v>5.13</v>
+        <v>5.15</v>
       </c>
       <c r="BN12" t="n">
         <v>8.23</v>
@@ -3305,19 +3305,19 @@
         <v>4.42</v>
       </c>
       <c r="BP12" t="n">
-        <v>5.03</v>
+        <v>5.04</v>
       </c>
       <c r="BQ12" t="n">
-        <v>1.5</v>
+        <v>1.47</v>
       </c>
       <c r="BR12" t="n">
-        <v>5.06</v>
+        <v>5.15</v>
       </c>
       <c r="BS12" t="n">
         <v>0.09</v>
       </c>
       <c r="BT12" t="n">
-        <v>495810</v>
+        <v>505573</v>
       </c>
     </row>
     <row r="13">
@@ -3347,13 +3347,13 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>28.46</v>
+        <v>28.29</v>
       </c>
       <c r="G13" t="n">
-        <v>14353453326</v>
+        <v>14263555364</v>
       </c>
       <c r="H13" t="n">
-        <v>9049300</v>
+        <v>5922600</v>
       </c>
       <c r="I13" t="n">
         <v>504190947</v>
@@ -3368,7 +3368,7 @@
         <v>1.13</v>
       </c>
       <c r="M13" t="n">
-        <v>4.964253979589248</v>
+        <v>4.933162067038345</v>
       </c>
       <c r="N13" t="n">
         <v>0.57</v>
@@ -3446,7 +3446,7 @@
         <v>932753251.95</v>
       </c>
       <c r="AM13" t="n">
-        <v>1493595559.417274</v>
+        <v>1484240932.778356</v>
       </c>
       <c r="AN13" t="n">
         <v>2.6301</v>
@@ -3487,7 +3487,7 @@
         <v>26.6</v>
       </c>
       <c r="AZ13" t="n">
-        <v>51.51</v>
+        <v>51.2</v>
       </c>
       <c r="BA13" t="n">
         <v>2.6</v>
@@ -3496,19 +3496,19 @@
         <v>8.69</v>
       </c>
       <c r="BC13" t="n">
-        <v>14.45</v>
+        <v>15.14</v>
       </c>
       <c r="BD13" t="n">
-        <v>-6.55</v>
+        <v>-5.99</v>
       </c>
       <c r="BE13" t="n">
         <v>81</v>
       </c>
       <c r="BF13" t="n">
-        <v>-90.84999999999999</v>
+        <v>-90.79000000000001</v>
       </c>
       <c r="BG13" t="n">
-        <v>-69.45</v>
+        <v>-69.27</v>
       </c>
       <c r="BH13" t="n">
         <v>25.49</v>
@@ -3517,7 +3517,7 @@
         <v>0</v>
       </c>
       <c r="BJ13" t="n">
-        <v>28.46</v>
+        <v>28.29</v>
       </c>
       <c r="BK13" t="n">
         <v>1.85</v>
@@ -3526,7 +3526,7 @@
         <v>1.96</v>
       </c>
       <c r="BM13" t="n">
-        <v>28.82</v>
+        <v>28.76</v>
       </c>
       <c r="BN13" t="n">
         <v>32.43</v>
@@ -3535,19 +3535,19 @@
         <v>21.06</v>
       </c>
       <c r="BP13" t="n">
-        <v>28.4</v>
+        <v>27.82</v>
       </c>
       <c r="BQ13" t="n">
-        <v>14.54</v>
+        <v>14.45</v>
       </c>
       <c r="BR13" t="n">
-        <v>28.53</v>
+        <v>28.76</v>
       </c>
       <c r="BS13" t="n">
         <v>5.01</v>
       </c>
       <c r="BT13" t="n">
-        <v>4510147</v>
+        <v>4708622</v>
       </c>
     </row>
     <row r="14">
@@ -3577,13 +3577,13 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>9.6</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="G14" t="n">
-        <v>7925797696</v>
+        <v>7556726851</v>
       </c>
       <c r="H14" t="n">
-        <v>16800</v>
+        <v>8000</v>
       </c>
       <c r="I14" t="n">
         <v>339510689</v>
@@ -3598,7 +3598,7 @@
         <v>1.92</v>
       </c>
       <c r="M14" t="n">
-        <v>3.290932105702915</v>
+        <v>3.137687329634206</v>
       </c>
       <c r="N14" t="n">
         <v>1.11</v>
@@ -3676,7 +3676,7 @@
         <v>349696009.67</v>
       </c>
       <c r="AM14" t="n">
-        <v>879666780.9100999</v>
+        <v>838704422.9744729</v>
       </c>
       <c r="AN14" t="n">
         <v>0.1489</v>
@@ -3717,7 +3717,7 @@
         <v>9.050000000000001</v>
       </c>
       <c r="AZ14" t="n">
-        <v>7.71</v>
+        <v>7.73</v>
       </c>
       <c r="BA14" t="n">
         <v>1.42</v>
@@ -3726,19 +3726,19 @@
         <v>5.94</v>
       </c>
       <c r="BC14" t="n">
-        <v>15.45</v>
+        <v>15.21</v>
       </c>
       <c r="BD14" t="n">
-        <v>-5.74</v>
+        <v>-5.94</v>
       </c>
       <c r="BE14" t="n">
         <v>-19.67</v>
       </c>
       <c r="BF14" t="n">
-        <v>-85.2</v>
+        <v>-85.23</v>
       </c>
       <c r="BG14" t="n">
-        <v>-38.1</v>
+        <v>-38.23</v>
       </c>
       <c r="BH14" t="n">
         <v>5.3</v>
@@ -3747,7 +3747,7 @@
         <v>0</v>
       </c>
       <c r="BJ14" t="n">
-        <v>9.6</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="BK14" t="n">
         <v>1.03</v>
@@ -3756,7 +3756,7 @@
         <v>1.01</v>
       </c>
       <c r="BM14" t="n">
-        <v>9.859999999999999</v>
+        <v>9.99</v>
       </c>
       <c r="BN14" t="n">
         <v>13.49</v>
@@ -3765,19 +3765,19 @@
         <v>7.65</v>
       </c>
       <c r="BP14" t="n">
-        <v>9.6</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="BQ14" t="n">
-        <v>9.48</v>
+        <v>9.5</v>
       </c>
       <c r="BR14" t="n">
-        <v>9.77</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="BS14" t="n">
         <v>1.44</v>
       </c>
       <c r="BT14" t="n">
-        <v>12590</v>
+        <v>12437</v>
       </c>
     </row>
     <row r="15">
@@ -3807,13 +3807,13 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>13.23</v>
+        <v>12.81</v>
       </c>
       <c r="G15" t="n">
-        <v>7925797696</v>
+        <v>7556726851</v>
       </c>
       <c r="H15" t="n">
-        <v>2706900</v>
+        <v>3949400</v>
       </c>
       <c r="I15" t="n">
         <v>343551533</v>
@@ -3828,7 +3828,7 @@
         <v>2.56</v>
       </c>
       <c r="M15" t="n">
-        <v>3.252224249744266</v>
+        <v>3.100781934658634</v>
       </c>
       <c r="N15" t="n">
         <v>1.47</v>
@@ -3906,7 +3906,7 @@
         <v>353858078.99</v>
       </c>
       <c r="AM15" t="n">
-        <v>661034003.0025021</v>
+        <v>630252447.9566305</v>
       </c>
       <c r="AN15" t="n">
         <v>0.1638</v>
@@ -3947,7 +3947,7 @@
         <v>9.050000000000001</v>
       </c>
       <c r="AZ15" t="n">
-        <v>8.800000000000001</v>
+        <v>8.52</v>
       </c>
       <c r="BA15" t="n">
         <v>1.42</v>
@@ -3956,19 +3956,19 @@
         <v>6.19</v>
       </c>
       <c r="BC15" t="n">
-        <v>-16.23</v>
+        <v>-13.48</v>
       </c>
       <c r="BD15" t="n">
-        <v>-31.6</v>
+        <v>-29.36</v>
       </c>
       <c r="BE15" t="n">
         <v>-33.5</v>
       </c>
       <c r="BF15" t="n">
-        <v>-89.26000000000001</v>
+        <v>-88.91</v>
       </c>
       <c r="BG15" t="n">
-        <v>-53.22</v>
+        <v>-51.69</v>
       </c>
       <c r="BH15" t="n">
         <v>5.3</v>
@@ -3977,7 +3977,7 @@
         <v>0</v>
       </c>
       <c r="BJ15" t="n">
-        <v>13.23</v>
+        <v>12.81</v>
       </c>
       <c r="BK15" t="n">
         <v>1.03</v>
@@ -3986,7 +3986,7 @@
         <v>1.01</v>
       </c>
       <c r="BM15" t="n">
-        <v>13.35</v>
+        <v>13.52</v>
       </c>
       <c r="BN15" t="n">
         <v>16.22</v>
@@ -3995,19 +3995,19 @@
         <v>7.84</v>
       </c>
       <c r="BP15" t="n">
-        <v>12.97</v>
+        <v>12.81</v>
       </c>
       <c r="BQ15" t="n">
-        <v>13.06</v>
+        <v>12.65</v>
       </c>
       <c r="BR15" t="n">
-        <v>13.01</v>
+        <v>13.38</v>
       </c>
       <c r="BS15" t="n">
         <v>1.92</v>
       </c>
       <c r="BT15" t="n">
-        <v>2332907</v>
+        <v>2389933</v>
       </c>
     </row>
     <row r="16">
@@ -4037,13 +4037,13 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>4.22</v>
+        <v>4.35</v>
       </c>
       <c r="G16" t="n">
-        <v>925739665</v>
+        <v>953979774</v>
       </c>
       <c r="H16" t="n">
-        <v>68800</v>
+        <v>62200</v>
       </c>
       <c r="I16" t="n">
         <v>219305733</v>
@@ -4058,7 +4058,7 @@
         <v>2.69</v>
       </c>
       <c r="M16" t="n">
-        <v>0.4379524827276175</v>
+        <v>0.4513124221540528</v>
       </c>
       <c r="N16" t="n">
         <v>0.39</v>
@@ -4136,7 +4136,7 @@
         <v>17544458.64</v>
       </c>
       <c r="AM16" t="n">
-        <v>260039231.741573</v>
+        <v>267971846.6292135</v>
       </c>
       <c r="AN16" t="n">
         <v>0.0077</v>
@@ -4186,16 +4186,16 @@
         <v>0</v>
       </c>
       <c r="BC16" t="n">
-        <v>-58.79</v>
+        <v>-60.02</v>
       </c>
       <c r="BD16" t="n">
-        <v>-66.34999999999999</v>
+        <v>-67.36</v>
       </c>
       <c r="BE16" t="n">
         <v>-97.17</v>
       </c>
       <c r="BF16" t="n">
-        <v>-98.09999999999999</v>
+        <v>-98.16</v>
       </c>
       <c r="BG16" t="n">
         <v>-100</v>
@@ -4207,7 +4207,7 @@
         <v>0</v>
       </c>
       <c r="BJ16" t="n">
-        <v>4.22</v>
+        <v>4.35</v>
       </c>
       <c r="BK16" t="n">
         <v>0.08</v>
@@ -4216,28 +4216,28 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="BM16" t="n">
-        <v>4.3</v>
+        <v>4.38</v>
       </c>
       <c r="BN16" t="n">
         <v>5.54</v>
       </c>
       <c r="BO16" t="n">
-        <v>3.1</v>
+        <v>3.13</v>
       </c>
       <c r="BP16" t="n">
-        <v>4.17</v>
+        <v>4.2</v>
       </c>
       <c r="BQ16" t="n">
-        <v>57.59</v>
+        <v>59.36</v>
       </c>
       <c r="BR16" t="n">
-        <v>4.26</v>
+        <v>4.2</v>
       </c>
       <c r="BS16" t="n">
         <v>0.49</v>
       </c>
       <c r="BT16" t="n">
-        <v>145277</v>
+        <v>145310</v>
       </c>
     </row>
     <row r="17">
@@ -4267,13 +4267,13 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>32.97</v>
+        <v>33.4</v>
       </c>
       <c r="G17" t="n">
-        <v>10870961118</v>
+        <v>11009538962</v>
       </c>
       <c r="H17" t="n">
-        <v>1773100</v>
+        <v>646500</v>
       </c>
       <c r="I17" t="n">
         <v>0</v>
@@ -4360,13 +4360,13 @@
         <v>8.039999999999999</v>
       </c>
       <c r="AK17" t="n">
-        <v>4909212932.622832</v>
+        <v>4971793245.122832</v>
       </c>
       <c r="AL17" t="n">
-        <v>1358870139.75</v>
+        <v>1376192370.25</v>
       </c>
       <c r="AM17" t="n">
-        <v>3365622637.151703</v>
+        <v>3408525994.427245</v>
       </c>
       <c r="AN17" t="n">
         <v>1.08</v>
@@ -4407,7 +4407,7 @@
         <v>42.98</v>
       </c>
       <c r="AZ17" t="n">
-        <v>17.64</v>
+        <v>17.87</v>
       </c>
       <c r="BA17" t="n">
         <v>4.55</v>
@@ -4416,19 +4416,19 @@
         <v>16.33</v>
       </c>
       <c r="BC17" t="n">
-        <v>59.65</v>
+        <v>57.6</v>
       </c>
       <c r="BD17" t="n">
-        <v>30.36</v>
+        <v>28.68</v>
       </c>
       <c r="BE17" t="n">
         <v>-46.5</v>
       </c>
       <c r="BF17" t="n">
-        <v>-86.2</v>
+        <v>-86.38</v>
       </c>
       <c r="BG17" t="n">
-        <v>-50.46</v>
+        <v>-51.1</v>
       </c>
       <c r="BH17" t="n">
         <v>29.25</v>
@@ -4437,7 +4437,7 @@
         <v>0</v>
       </c>
       <c r="BJ17" t="n">
-        <v>32.97</v>
+        <v>33.4</v>
       </c>
       <c r="BK17" t="n">
         <v>4.21</v>
@@ -4446,7 +4446,7 @@
         <v>12.62</v>
       </c>
       <c r="BM17" t="n">
-        <v>33.4</v>
+        <v>33.48</v>
       </c>
       <c r="BN17" t="n">
         <v>36.63</v>
@@ -4455,19 +4455,19 @@
         <v>29.28</v>
       </c>
       <c r="BP17" t="n">
-        <v>32.9</v>
+        <v>32.82</v>
       </c>
       <c r="BQ17" t="n">
-        <v>2.61</v>
+        <v>2.65</v>
       </c>
       <c r="BR17" t="n">
-        <v>33.37</v>
+        <v>33</v>
       </c>
       <c r="BS17" t="n">
         <v>2.21</v>
       </c>
       <c r="BT17" t="n">
-        <v>1070251</v>
+        <v>1084652</v>
       </c>
     </row>
     <row r="18">
@@ -4497,13 +4497,13 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>11.35</v>
+        <v>11.3</v>
       </c>
       <c r="G18" t="n">
-        <v>10870961118</v>
+        <v>11009538962</v>
       </c>
       <c r="H18" t="n">
-        <v>10600</v>
+        <v>5500</v>
       </c>
       <c r="I18" t="n">
         <v>671494278</v>
@@ -4518,7 +4518,7 @@
         <v>1.2</v>
       </c>
       <c r="M18" t="n">
-        <v>3.200837866965625</v>
+        <v>3.241640626333719</v>
       </c>
       <c r="N18" t="n">
         <v>0.33</v>
@@ -4596,7 +4596,7 @@
         <v>940091989.1999999</v>
       </c>
       <c r="AM18" t="n">
-        <v>3235405094.642857</v>
+        <v>3276648500.595238</v>
       </c>
       <c r="AN18" t="n">
         <v>0.36</v>
@@ -4637,7 +4637,7 @@
         <v>14.31</v>
       </c>
       <c r="AZ18" t="n">
-        <v>5.85</v>
+        <v>5.82</v>
       </c>
       <c r="BA18" t="n">
         <v>1.51</v>
@@ -4646,19 +4646,19 @@
         <v>5.44</v>
       </c>
       <c r="BC18" t="n">
-        <v>54.41</v>
+        <v>55.09</v>
       </c>
       <c r="BD18" t="n">
-        <v>26.07</v>
+        <v>26.63</v>
       </c>
       <c r="BE18" t="n">
         <v>-48.5</v>
       </c>
       <c r="BF18" t="n">
-        <v>-86.67</v>
+        <v>-86.61</v>
       </c>
       <c r="BG18" t="n">
-        <v>-52.03</v>
+        <v>-51.82</v>
       </c>
       <c r="BH18" t="n">
         <v>9.75</v>
@@ -4667,7 +4667,7 @@
         <v>0</v>
       </c>
       <c r="BJ18" t="n">
-        <v>11.35</v>
+        <v>11.3</v>
       </c>
       <c r="BK18" t="n">
         <v>1.4</v>
@@ -4676,7 +4676,7 @@
         <v>12.62</v>
       </c>
       <c r="BM18" t="n">
-        <v>11.57</v>
+        <v>11.44</v>
       </c>
       <c r="BN18" t="n">
         <v>13.82</v>
@@ -4685,19 +4685,19 @@
         <v>10.19</v>
       </c>
       <c r="BP18" t="n">
-        <v>11.35</v>
+        <v>11.25</v>
       </c>
       <c r="BQ18" t="n">
         <v>0.9</v>
       </c>
       <c r="BR18" t="n">
-        <v>11.56</v>
+        <v>11.28</v>
       </c>
       <c r="BS18" t="n">
         <v>2.3</v>
       </c>
       <c r="BT18" t="n">
-        <v>9698</v>
+        <v>9951</v>
       </c>
     </row>
     <row r="19">
@@ -4727,13 +4727,13 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>10.8</v>
+        <v>10.91</v>
       </c>
       <c r="G19" t="n">
-        <v>10870961118</v>
+        <v>11009538962</v>
       </c>
       <c r="H19" t="n">
-        <v>8800</v>
+        <v>4600</v>
       </c>
       <c r="I19" t="n">
         <v>317386323</v>
@@ -4748,7 +4748,7 @@
         <v>1.12</v>
       </c>
       <c r="M19" t="n">
-        <v>6.772013022354284</v>
+        <v>6.858339424775492</v>
       </c>
       <c r="N19" t="n">
         <v>0.3</v>
@@ -4826,7 +4826,7 @@
         <v>444340852.2</v>
       </c>
       <c r="AM19" t="n">
-        <v>3451098767.619048</v>
+        <v>3495091733.968254</v>
       </c>
       <c r="AN19" t="n">
         <v>0.36</v>
@@ -4867,7 +4867,7 @@
         <v>14.31</v>
       </c>
       <c r="AZ19" t="n">
-        <v>5.94</v>
+        <v>6</v>
       </c>
       <c r="BA19" t="n">
         <v>1.51</v>
@@ -4876,19 +4876,19 @@
         <v>5.25</v>
       </c>
       <c r="BC19" t="n">
-        <v>62.27</v>
+        <v>60.63</v>
       </c>
       <c r="BD19" t="n">
-        <v>32.49</v>
+        <v>31.16</v>
       </c>
       <c r="BE19" t="n">
         <v>-45</v>
       </c>
       <c r="BF19" t="n">
-        <v>-85.98999999999999</v>
+        <v>-86.14</v>
       </c>
       <c r="BG19" t="n">
-        <v>-51.39</v>
+        <v>-51.88</v>
       </c>
       <c r="BH19" t="n">
         <v>9.75</v>
@@ -4897,7 +4897,7 @@
         <v>0</v>
       </c>
       <c r="BJ19" t="n">
-        <v>10.8</v>
+        <v>10.91</v>
       </c>
       <c r="BK19" t="n">
         <v>1.4</v>
@@ -4906,7 +4906,7 @@
         <v>12.62</v>
       </c>
       <c r="BM19" t="n">
-        <v>10.9</v>
+        <v>11.03</v>
       </c>
       <c r="BN19" t="n">
         <v>11.41</v>
@@ -4921,13 +4921,13 @@
         <v>0.86</v>
       </c>
       <c r="BR19" t="n">
-        <v>10.9</v>
+        <v>10.88</v>
       </c>
       <c r="BS19" t="n">
         <v>2.16</v>
       </c>
       <c r="BT19" t="n">
-        <v>13726</v>
+        <v>13684</v>
       </c>
     </row>
     <row r="20">
@@ -5417,13 +5417,13 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>5.01</v>
+        <v>4.94</v>
       </c>
       <c r="G22" t="n">
-        <v>1003521081</v>
+        <v>989211793</v>
       </c>
       <c r="H22" t="n">
-        <v>757500</v>
+        <v>1005200</v>
       </c>
       <c r="I22" t="n">
         <v>200245299</v>
@@ -5438,7 +5438,7 @@
         <v>0.27</v>
       </c>
       <c r="M22" t="n">
-        <v>0.08511525392140358</v>
+        <v>0.08390158865356404</v>
       </c>
       <c r="N22" t="n">
         <v>0.08</v>
@@ -5516,7 +5516,7 @@
         <v>378463615.11</v>
       </c>
       <c r="AM22" t="n">
-        <v>227555800.6802721</v>
+        <v>224311064.1723356</v>
       </c>
       <c r="AN22" t="n">
         <v>0</v>
@@ -5566,19 +5566,19 @@
         <v>172.49</v>
       </c>
       <c r="BC22" t="n">
-        <v>492.92</v>
+        <v>501.32</v>
       </c>
       <c r="BD22" t="n">
-        <v>384.11</v>
+        <v>390.97</v>
       </c>
       <c r="BE22" t="n">
         <v>-100</v>
       </c>
       <c r="BF22" t="n">
-        <v>-62.28</v>
+        <v>-61.74</v>
       </c>
       <c r="BG22" t="n">
-        <v>3342.91</v>
+        <v>3391.69</v>
       </c>
       <c r="BH22" t="n">
         <v>20.75</v>
@@ -5587,7 +5587,7 @@
         <v>0</v>
       </c>
       <c r="BJ22" t="n">
-        <v>5.01</v>
+        <v>4.94</v>
       </c>
       <c r="BK22" t="n">
         <v>1.89</v>
@@ -5596,7 +5596,7 @@
         <v>0.67</v>
       </c>
       <c r="BM22" t="n">
-        <v>5.09</v>
+        <v>5.08</v>
       </c>
       <c r="BN22" t="n">
         <v>8.82</v>
@@ -5605,19 +5605,19 @@
         <v>3.37</v>
       </c>
       <c r="BP22" t="n">
-        <v>4.94</v>
+        <v>4.85</v>
       </c>
       <c r="BQ22" t="n">
-        <v>7.46</v>
+        <v>7.36</v>
       </c>
       <c r="BR22" t="n">
-        <v>4.97</v>
+        <v>5.05</v>
       </c>
       <c r="BS22" t="n">
         <v>0.09</v>
       </c>
       <c r="BT22" t="n">
-        <v>1577207</v>
+        <v>1563307</v>
       </c>
     </row>
     <row r="23">
@@ -5877,13 +5877,13 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.93</v>
+        <v>2.86</v>
       </c>
       <c r="G24" t="n">
-        <v>1183679885</v>
+        <v>1155065011</v>
       </c>
       <c r="H24" t="n">
-        <v>5331500</v>
+        <v>4726300</v>
       </c>
       <c r="I24" t="n">
         <v>403868805</v>
@@ -5898,7 +5898,7 @@
         <v>0.49</v>
       </c>
       <c r="M24" t="n">
-        <v>0.2861437543827864</v>
+        <v>0.2792263710756008</v>
       </c>
       <c r="N24" t="n">
         <v>0.11</v>
@@ -5976,7 +5976,7 @@
         <v>153470145.9</v>
       </c>
       <c r="AM24" t="n">
-        <v>1066378274.774775</v>
+        <v>1040599109.009009</v>
       </c>
       <c r="AN24" t="n">
         <v>0.0813</v>
@@ -6017,7 +6017,7 @@
         <v>5.84</v>
       </c>
       <c r="AZ24" t="n">
-        <v>1.35</v>
+        <v>1.32</v>
       </c>
       <c r="BA24" t="n">
         <v>0.38</v>
@@ -6026,19 +6026,19 @@
         <v>1.46</v>
       </c>
       <c r="BC24" t="n">
-        <v>144.25</v>
+        <v>150.22</v>
       </c>
       <c r="BD24" t="n">
-        <v>99.43000000000001</v>
+        <v>104.31</v>
       </c>
       <c r="BE24" t="n">
         <v>-53.83</v>
       </c>
       <c r="BF24" t="n">
-        <v>-87.03</v>
+        <v>-86.70999999999999</v>
       </c>
       <c r="BG24" t="n">
-        <v>-50.25</v>
+        <v>-49.03</v>
       </c>
       <c r="BH24" t="n">
         <v>5.99</v>
@@ -6047,7 +6047,7 @@
         <v>0</v>
       </c>
       <c r="BJ24" t="n">
-        <v>2.93</v>
+        <v>2.86</v>
       </c>
       <c r="BK24" t="n">
         <v>0.38</v>
@@ -6056,7 +6056,7 @@
         <v>0.41</v>
       </c>
       <c r="BM24" t="n">
-        <v>3.01</v>
+        <v>2.98</v>
       </c>
       <c r="BN24" t="n">
         <v>5.29</v>
@@ -6065,19 +6065,19 @@
         <v>1.92</v>
       </c>
       <c r="BP24" t="n">
-        <v>2.9</v>
+        <v>2.83</v>
       </c>
       <c r="BQ24" t="n">
-        <v>7.2</v>
+        <v>7.02</v>
       </c>
       <c r="BR24" t="n">
-        <v>2.94</v>
+        <v>2.93</v>
       </c>
       <c r="BS24" t="n">
         <v>0.29</v>
       </c>
       <c r="BT24" t="n">
-        <v>8821017</v>
+        <v>8653000</v>
       </c>
     </row>
     <row r="25">
@@ -6107,13 +6107,13 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>3.85</v>
+        <v>3.97</v>
       </c>
       <c r="G25" t="n">
-        <v>1334390331</v>
+        <v>1375581189</v>
       </c>
       <c r="H25" t="n">
-        <v>1568000</v>
+        <v>1312100</v>
       </c>
       <c r="I25" t="n">
         <v>346494097</v>
@@ -6128,7 +6128,7 @@
         <v>0.97</v>
       </c>
       <c r="M25" t="n">
-        <v>0.6653879476576864</v>
+        <v>0.6859275902421313</v>
       </c>
       <c r="N25" t="n">
         <v>0.22</v>
@@ -6206,7 +6206,7 @@
         <v>62368937.46</v>
       </c>
       <c r="AM25" t="n">
-        <v>490584680.5147058</v>
+        <v>505728378.3088235</v>
       </c>
       <c r="AN25" t="n">
         <v>0.4742</v>
@@ -6247,7 +6247,7 @@
         <v>3.27</v>
       </c>
       <c r="AZ25" t="n">
-        <v>8.970000000000001</v>
+        <v>9.25</v>
       </c>
       <c r="BA25" t="n">
         <v>0.23</v>
@@ -6256,19 +6256,19 @@
         <v>2.2</v>
       </c>
       <c r="BC25" t="n">
-        <v>4.15</v>
+        <v>1</v>
       </c>
       <c r="BD25" t="n">
-        <v>-14.96</v>
+        <v>-17.53</v>
       </c>
       <c r="BE25" t="n">
         <v>133</v>
       </c>
       <c r="BF25" t="n">
-        <v>-93.98</v>
+        <v>-94.16</v>
       </c>
       <c r="BG25" t="n">
-        <v>-42.86</v>
+        <v>-44.59</v>
       </c>
       <c r="BH25" t="n">
         <v>3.97</v>
@@ -6277,7 +6277,7 @@
         <v>0</v>
       </c>
       <c r="BJ25" t="n">
-        <v>3.85</v>
+        <v>3.97</v>
       </c>
       <c r="BK25" t="n">
         <v>0.18</v>
@@ -6286,7 +6286,7 @@
         <v>0.24</v>
       </c>
       <c r="BM25" t="n">
-        <v>4</v>
+        <v>4.06</v>
       </c>
       <c r="BN25" t="n">
         <v>6.3</v>
@@ -6295,19 +6295,19 @@
         <v>2.64</v>
       </c>
       <c r="BP25" t="n">
-        <v>3.74</v>
+        <v>3.85</v>
       </c>
       <c r="BQ25" t="n">
-        <v>16.27</v>
+        <v>16.78</v>
       </c>
       <c r="BR25" t="n">
-        <v>3.78</v>
+        <v>3.91</v>
       </c>
       <c r="BS25" t="n">
         <v>0.67</v>
       </c>
       <c r="BT25" t="n">
-        <v>1186133</v>
+        <v>1228043</v>
       </c>
     </row>
     <row r="26">
@@ -6337,13 +6337,13 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>10.1</v>
+        <v>10.21</v>
       </c>
       <c r="G26" t="n">
-        <v>13683349216</v>
+        <v>13828352581</v>
       </c>
       <c r="H26" t="n">
-        <v>16505300</v>
+        <v>9755800</v>
       </c>
       <c r="I26" t="n">
         <v>1354393401</v>
@@ -6358,7 +6358,7 @@
         <v>1.94</v>
       </c>
       <c r="M26" t="n">
-        <v>0.1764456346528036</v>
+        <v>0.1783154408208944</v>
       </c>
       <c r="N26" t="n">
         <v>0.26</v>
@@ -6436,7 +6436,7 @@
         <v>961619314.7099999</v>
       </c>
       <c r="AM26" t="n">
-        <v>4886910434.285714</v>
+        <v>4938697350.357143</v>
       </c>
       <c r="AN26" t="n">
         <v>0.1043</v>
@@ -6477,7 +6477,7 @@
         <v>7.07</v>
       </c>
       <c r="AZ26" t="n">
-        <v>1.94</v>
+        <v>1.96</v>
       </c>
       <c r="BA26" t="n">
         <v>0.66</v>
@@ -6486,19 +6486,19 @@
         <v>1.19</v>
       </c>
       <c r="BC26" t="n">
-        <v>-14.3</v>
+        <v>-15.22</v>
       </c>
       <c r="BD26" t="n">
-        <v>-30.03</v>
+        <v>-30.78</v>
       </c>
       <c r="BE26" t="n">
         <v>-80.83</v>
       </c>
       <c r="BF26" t="n">
-        <v>-93.47</v>
+        <v>-93.54000000000001</v>
       </c>
       <c r="BG26" t="n">
-        <v>-88.18000000000001</v>
+        <v>-88.31</v>
       </c>
       <c r="BH26" t="n">
         <v>4.69</v>
@@ -6507,7 +6507,7 @@
         <v>0</v>
       </c>
       <c r="BJ26" t="n">
-        <v>10.1</v>
+        <v>10.21</v>
       </c>
       <c r="BK26" t="n">
         <v>0.71</v>
@@ -6516,28 +6516,28 @@
         <v>0.72</v>
       </c>
       <c r="BM26" t="n">
-        <v>10.19</v>
+        <v>10.28</v>
       </c>
       <c r="BN26" t="n">
-        <v>10.6</v>
+        <v>10.41</v>
       </c>
       <c r="BO26" t="n">
         <v>6.91</v>
       </c>
       <c r="BP26" t="n">
-        <v>9.619999999999999</v>
+        <v>9.880000000000001</v>
       </c>
       <c r="BQ26" t="n">
-        <v>14.08</v>
+        <v>14.24</v>
       </c>
       <c r="BR26" t="n">
-        <v>9.619999999999999</v>
+        <v>10.14</v>
       </c>
       <c r="BS26" t="n">
         <v>0.16</v>
       </c>
       <c r="BT26" t="n">
-        <v>11796480</v>
+        <v>12155697</v>
       </c>
     </row>
     <row r="27">
@@ -8165,13 +8165,13 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>15.03</v>
+        <v>14.81</v>
       </c>
       <c r="G34" t="n">
-        <v>3104444941</v>
+        <v>3058114024</v>
       </c>
       <c r="H34" t="n">
-        <v>3684600</v>
+        <v>2608300</v>
       </c>
       <c r="I34" t="n">
         <v>206489813</v>
@@ -8186,7 +8186,7 @@
         <v>0.45</v>
       </c>
       <c r="M34" t="n">
-        <v>0.2729169684014641</v>
+        <v>0.2688439396793548</v>
       </c>
       <c r="N34" t="n">
         <v>0.24</v>
@@ -8264,7 +8264,7 @@
         <v>324189006.41</v>
       </c>
       <c r="AM34" t="n">
-        <v>645414748.6486487</v>
+        <v>635782541.3721415</v>
       </c>
       <c r="AN34" t="n">
         <v>0</v>
@@ -8305,7 +8305,7 @@
         <v>30.28</v>
       </c>
       <c r="AZ34" t="n">
-        <v>35.07</v>
+        <v>34.56</v>
       </c>
       <c r="BA34" t="n">
         <v>2.29</v>
@@ -8314,19 +8314,19 @@
         <v>25.26</v>
       </c>
       <c r="BC34" t="n">
-        <v>146.76</v>
+        <v>150.43</v>
       </c>
       <c r="BD34" t="n">
-        <v>101.48</v>
+        <v>104.47</v>
       </c>
       <c r="BE34" t="n">
         <v>133.33</v>
       </c>
       <c r="BF34" t="n">
-        <v>-84.73</v>
+        <v>-84.5</v>
       </c>
       <c r="BG34" t="n">
-        <v>68.05</v>
+        <v>70.55</v>
       </c>
       <c r="BH34" t="n">
         <v>38.94</v>
@@ -8335,7 +8335,7 @@
         <v>0</v>
       </c>
       <c r="BJ34" t="n">
-        <v>15.03</v>
+        <v>14.81</v>
       </c>
       <c r="BK34" t="n">
         <v>1.57</v>
@@ -8344,28 +8344,28 @@
         <v>1.58</v>
       </c>
       <c r="BM34" t="n">
-        <v>15.38</v>
+        <v>15.2</v>
       </c>
       <c r="BN34" t="n">
-        <v>31.12</v>
+        <v>30.87</v>
       </c>
       <c r="BO34" t="n">
         <v>14.32</v>
       </c>
       <c r="BP34" t="n">
-        <v>14.96</v>
+        <v>14.68</v>
       </c>
       <c r="BQ34" t="n">
-        <v>9.529999999999999</v>
+        <v>9.390000000000001</v>
       </c>
       <c r="BR34" t="n">
-        <v>15.34</v>
+        <v>15.2</v>
       </c>
       <c r="BS34" t="n">
         <v>0.32</v>
       </c>
       <c r="BT34" t="n">
-        <v>3064873</v>
+        <v>3121040</v>
       </c>
     </row>
     <row r="35">
@@ -8395,13 +8395,13 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>17.58</v>
+        <v>17.6</v>
       </c>
       <c r="G35" t="n">
-        <v>88743294634</v>
+        <v>88818384325</v>
       </c>
       <c r="H35" t="n">
-        <v>30862100</v>
+        <v>31853100</v>
       </c>
       <c r="I35" t="n">
         <v>5046500000</v>
@@ -8416,7 +8416,7 @@
         <v>4.69</v>
       </c>
       <c r="M35" t="n">
-        <v>7.36750057427423</v>
+        <v>7.373734547712406</v>
       </c>
       <c r="N35" t="n">
         <v>1.79</v>
@@ -8494,7 +8494,7 @@
         <v>5349290000</v>
       </c>
       <c r="AM35" t="n">
-        <v>7334156581.322314</v>
+        <v>7340362340.909091</v>
       </c>
       <c r="AN35" t="n">
         <v>0.5305</v>
@@ -8535,7 +8535,7 @@
         <v>7.68</v>
       </c>
       <c r="AZ35" t="n">
-        <v>10.26</v>
+        <v>10.27</v>
       </c>
       <c r="BA35" t="n">
         <v>1.11</v>
@@ -8544,19 +8544,19 @@
         <v>9.119999999999999</v>
       </c>
       <c r="BC35" t="n">
-        <v>-46.49</v>
+        <v>-46.55</v>
       </c>
       <c r="BD35" t="n">
-        <v>-56.31</v>
+        <v>-56.36</v>
       </c>
       <c r="BE35" t="n">
         <v>-41.67</v>
       </c>
       <c r="BF35" t="n">
-        <v>-93.66</v>
+        <v>-93.67</v>
       </c>
       <c r="BG35" t="n">
-        <v>-48.14</v>
+        <v>-48.2</v>
       </c>
       <c r="BH35" t="n">
         <v>3.71</v>
@@ -8565,7 +8565,7 @@
         <v>0</v>
       </c>
       <c r="BJ35" t="n">
-        <v>17.58</v>
+        <v>17.6</v>
       </c>
       <c r="BK35" t="n">
         <v>1.06</v>
@@ -8574,7 +8574,7 @@
         <v>1.04</v>
       </c>
       <c r="BM35" t="n">
-        <v>17.76</v>
+        <v>17.79</v>
       </c>
       <c r="BN35" t="n">
         <v>20.08</v>
@@ -8583,19 +8583,19 @@
         <v>11.7</v>
       </c>
       <c r="BP35" t="n">
-        <v>17.32</v>
+        <v>17.24</v>
       </c>
       <c r="BQ35" t="n">
-        <v>16.82</v>
+        <v>16.84</v>
       </c>
       <c r="BR35" t="n">
-        <v>17.37</v>
+        <v>17.73</v>
       </c>
       <c r="BS35" t="n">
         <v>7.3</v>
       </c>
       <c r="BT35" t="n">
-        <v>37224647</v>
+        <v>36985797</v>
       </c>
     </row>
     <row r="36">
@@ -9315,13 +9315,13 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>69.06</v>
+        <v>69.62</v>
       </c>
       <c r="G39" t="n">
-        <v>3872514501</v>
+        <v>3902779696</v>
       </c>
       <c r="H39" t="n">
-        <v>4000</v>
+        <v>1000</v>
       </c>
       <c r="I39" t="n">
         <v>168174945</v>
@@ -9336,7 +9336,7 @@
         <v>0.53</v>
       </c>
       <c r="M39" t="n">
-        <v>0.1943832416887489</v>
+        <v>0.1959024217235617</v>
       </c>
       <c r="N39" t="n">
         <v>0.06</v>
@@ -9414,7 +9414,7 @@
         <v>2536078170.6</v>
       </c>
       <c r="AM39" t="n">
-        <v>406776733.2983193</v>
+        <v>409955850.4201681</v>
       </c>
       <c r="AN39" t="n">
         <v>11.9435</v>
@@ -9455,7 +9455,7 @@
         <v>170.24</v>
       </c>
       <c r="AZ39" t="n">
-        <v>201.77</v>
+        <v>203.41</v>
       </c>
       <c r="BA39" t="n">
         <v>19.01</v>
@@ -9464,19 +9464,19 @@
         <v>91.72</v>
       </c>
       <c r="BC39" t="n">
-        <v>201.92</v>
+        <v>199.49</v>
       </c>
       <c r="BD39" t="n">
-        <v>146.52</v>
+        <v>144.53</v>
       </c>
       <c r="BE39" t="n">
         <v>192.17</v>
       </c>
       <c r="BF39" t="n">
-        <v>-72.47</v>
+        <v>-72.69</v>
       </c>
       <c r="BG39" t="n">
-        <v>32.82</v>
+        <v>31.75</v>
       </c>
       <c r="BH39" t="n">
         <v>128.13</v>
@@ -9485,7 +9485,7 @@
         <v>0</v>
       </c>
       <c r="BJ39" t="n">
-        <v>69.06</v>
+        <v>69.62</v>
       </c>
       <c r="BK39" t="n">
         <v>15.08</v>
@@ -9494,7 +9494,7 @@
         <v>15.08</v>
       </c>
       <c r="BM39" t="n">
-        <v>70.37</v>
+        <v>69.89</v>
       </c>
       <c r="BN39" t="n">
         <v>74.56</v>
@@ -9503,19 +9503,19 @@
         <v>54.98</v>
       </c>
       <c r="BP39" t="n">
-        <v>69.06</v>
+        <v>69.41</v>
       </c>
       <c r="BQ39" t="n">
-        <v>4.58</v>
+        <v>4.62</v>
       </c>
       <c r="BR39" t="n">
-        <v>69.16</v>
+        <v>69.89</v>
       </c>
       <c r="BS39" t="n">
         <v>0.58</v>
       </c>
       <c r="BT39" t="n">
-        <v>3887</v>
+        <v>3817</v>
       </c>
     </row>
     <row r="40">
@@ -9545,13 +9545,13 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>22.71</v>
+        <v>22.78</v>
       </c>
       <c r="G40" t="n">
-        <v>130185160591</v>
+        <v>130548356895</v>
       </c>
       <c r="H40" t="n">
-        <v>32049800</v>
+        <v>30659600</v>
       </c>
       <c r="I40" t="n">
         <v>5730834040</v>
@@ -9566,7 +9566,7 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="M40" t="n">
-        <v>0.3949978884059084</v>
+        <v>0.3960998709399051</v>
       </c>
       <c r="N40" t="n">
         <v>0.05</v>
@@ -9644,7 +9644,7 @@
         <v>15358635227.2</v>
       </c>
       <c r="AM40" t="n">
-        <v>6752342354.304979</v>
+        <v>6771180336.877593</v>
       </c>
       <c r="AN40" t="n">
         <v>0.5641</v>
@@ -9685,7 +9685,7 @@
         <v>36.13</v>
       </c>
       <c r="AZ40" t="n">
-        <v>11.47</v>
+        <v>11.5</v>
       </c>
       <c r="BA40" t="n">
         <v>2.76</v>
@@ -9694,19 +9694,19 @@
         <v>27.89</v>
       </c>
       <c r="BC40" t="n">
-        <v>94.84</v>
+        <v>94.23999999999999</v>
       </c>
       <c r="BD40" t="n">
-        <v>59.09</v>
+        <v>58.6</v>
       </c>
       <c r="BE40" t="n">
         <v>-49.5</v>
       </c>
       <c r="BF40" t="n">
-        <v>-87.84999999999999</v>
+        <v>-87.89</v>
       </c>
       <c r="BG40" t="n">
-        <v>22.81</v>
+        <v>22.43</v>
       </c>
       <c r="BH40" t="n">
         <v>32.47</v>
@@ -9715,7 +9715,7 @@
         <v>0</v>
       </c>
       <c r="BJ40" t="n">
-        <v>22.71</v>
+        <v>22.78</v>
       </c>
       <c r="BK40" t="n">
         <v>2.68</v>
@@ -9724,7 +9724,7 @@
         <v>2.5</v>
       </c>
       <c r="BM40" t="n">
-        <v>22.74</v>
+        <v>23.03</v>
       </c>
       <c r="BN40" t="n">
         <v>27.36</v>
@@ -9733,19 +9733,19 @@
         <v>17.67</v>
       </c>
       <c r="BP40" t="n">
-        <v>21.51</v>
+        <v>22.3</v>
       </c>
       <c r="BQ40" t="n">
-        <v>9.09</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="BR40" t="n">
-        <v>21.95</v>
+        <v>22.79</v>
       </c>
       <c r="BS40" t="n">
         <v>0.39</v>
       </c>
       <c r="BT40" t="n">
-        <v>31648024</v>
+        <v>32342306</v>
       </c>
     </row>
     <row r="41">
@@ -9775,13 +9775,13 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>16.09</v>
+        <v>16.03</v>
       </c>
       <c r="G41" t="n">
-        <v>192114033541</v>
+        <v>191375773977</v>
       </c>
       <c r="H41" t="n">
-        <v>5050400</v>
+        <v>5695800</v>
       </c>
       <c r="I41" t="n">
         <v>5303870781</v>
@@ -9796,7 +9796,7 @@
         <v>0.92</v>
       </c>
       <c r="M41" t="n">
-        <v>1.280241859722904</v>
+        <v>1.275322121275104</v>
       </c>
       <c r="N41" t="n">
         <v>0.07000000000000001</v>
@@ -9874,7 +9874,7 @@
         <v>12304980211.92</v>
       </c>
       <c r="AM41" t="n">
-        <v>29601546000.15408</v>
+        <v>29487792600.46225</v>
       </c>
       <c r="AN41" t="n">
         <v>1.6841</v>
@@ -9915,7 +9915,7 @@
         <v>24.4</v>
       </c>
       <c r="AZ41" t="n">
-        <v>24.08</v>
+        <v>23.99</v>
       </c>
       <c r="BA41" t="n">
         <v>2.53</v>
@@ -9924,19 +9924,19 @@
         <v>13.77</v>
       </c>
       <c r="BC41" t="n">
-        <v>85.73999999999999</v>
+        <v>86.43000000000001</v>
       </c>
       <c r="BD41" t="n">
-        <v>51.66</v>
+        <v>52.22</v>
       </c>
       <c r="BE41" t="n">
         <v>49.67</v>
       </c>
       <c r="BF41" t="n">
-        <v>-84.29000000000001</v>
+        <v>-84.23</v>
       </c>
       <c r="BG41" t="n">
-        <v>-14.42</v>
+        <v>-14.1</v>
       </c>
       <c r="BH41" t="n">
         <v>17.11</v>
@@ -9945,7 +9945,7 @@
         <v>0</v>
       </c>
       <c r="BJ41" t="n">
-        <v>16.09</v>
+        <v>16.03</v>
       </c>
       <c r="BK41" t="n">
         <v>2.32</v>
@@ -9963,19 +9963,19 @@
         <v>13.43</v>
       </c>
       <c r="BP41" t="n">
-        <v>15.89</v>
+        <v>15.74</v>
       </c>
       <c r="BQ41" t="n">
-        <v>6.88</v>
+        <v>6.86</v>
       </c>
       <c r="BR41" t="n">
-        <v>16.07</v>
+        <v>16.09</v>
       </c>
       <c r="BS41" t="n">
         <v>0.5600000000000001</v>
       </c>
       <c r="BT41" t="n">
-        <v>6971226</v>
+        <v>6988188</v>
       </c>
     </row>
     <row r="42">
@@ -10005,13 +10005,13 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>18.21</v>
+        <v>18.15</v>
       </c>
       <c r="G42" t="n">
-        <v>192114033541</v>
+        <v>191375773977</v>
       </c>
       <c r="H42" t="n">
-        <v>34375100</v>
+        <v>40269400</v>
       </c>
       <c r="I42" t="n">
         <v>5288141247</v>
@@ -10026,7 +10026,7 @@
         <v>1.05</v>
       </c>
       <c r="M42" t="n">
-        <v>1.284049928932886</v>
+        <v>1.279115556762277</v>
       </c>
       <c r="N42" t="n">
         <v>0.08</v>
@@ -10104,7 +10104,7 @@
         <v>12268487693.04</v>
       </c>
       <c r="AM42" t="n">
-        <v>26137963747.07483</v>
+        <v>26037520268.97959</v>
       </c>
       <c r="AN42" t="n">
         <v>1.8491</v>
@@ -10145,7 +10145,7 @@
         <v>24.4</v>
       </c>
       <c r="AZ42" t="n">
-        <v>26.37</v>
+        <v>26.29</v>
       </c>
       <c r="BA42" t="n">
         <v>2.53</v>
@@ -10154,19 +10154,19 @@
         <v>15.11</v>
       </c>
       <c r="BC42" t="n">
-        <v>64.12</v>
+        <v>64.66</v>
       </c>
       <c r="BD42" t="n">
-        <v>34</v>
+        <v>34.44</v>
       </c>
       <c r="BE42" t="n">
         <v>44.83</v>
       </c>
       <c r="BF42" t="n">
-        <v>-86.12</v>
+        <v>-86.08</v>
       </c>
       <c r="BG42" t="n">
-        <v>-17</v>
+        <v>-16.72</v>
       </c>
       <c r="BH42" t="n">
         <v>17.11</v>
@@ -10175,7 +10175,7 @@
         <v>0</v>
       </c>
       <c r="BJ42" t="n">
-        <v>18.21</v>
+        <v>18.15</v>
       </c>
       <c r="BK42" t="n">
         <v>2.32</v>
@@ -10184,7 +10184,7 @@
         <v>2.34</v>
       </c>
       <c r="BM42" t="n">
-        <v>18.25</v>
+        <v>18.26</v>
       </c>
       <c r="BN42" t="n">
         <v>21.33</v>
@@ -10193,19 +10193,19 @@
         <v>15.67</v>
       </c>
       <c r="BP42" t="n">
-        <v>17.97</v>
+        <v>17.85</v>
       </c>
       <c r="BQ42" t="n">
-        <v>7.79</v>
+        <v>7.76</v>
       </c>
       <c r="BR42" t="n">
-        <v>18.21</v>
+        <v>18.19</v>
       </c>
       <c r="BS42" t="n">
         <v>0.63</v>
       </c>
       <c r="BT42" t="n">
-        <v>40428097</v>
+        <v>40515008</v>
       </c>
     </row>
     <row r="43">
@@ -10235,13 +10235,13 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>40.59</v>
+        <v>40.41</v>
       </c>
       <c r="G43" t="n">
-        <v>78824359646</v>
+        <v>78451973703</v>
       </c>
       <c r="H43" t="n">
-        <v>6868600</v>
+        <v>5078700</v>
       </c>
       <c r="I43" t="n">
         <v>1941400000</v>
@@ -10334,7 +10334,7 @@
         <v>9182822000</v>
       </c>
       <c r="AM43" t="n">
-        <v>9601018227.2838</v>
+        <v>9555660621.559072</v>
       </c>
       <c r="AN43" t="n">
         <v>4.5901</v>
@@ -10375,7 +10375,7 @@
         <v>19.95</v>
       </c>
       <c r="AZ43" t="n">
-        <v>73.67</v>
+        <v>73.34</v>
       </c>
       <c r="BA43" t="n">
         <v>5.63</v>
@@ -10384,19 +10384,19 @@
         <v>48.62</v>
       </c>
       <c r="BC43" t="n">
-        <v>-39.8</v>
+        <v>-39.53</v>
       </c>
       <c r="BD43" t="n">
-        <v>-50.85</v>
+        <v>-50.63</v>
       </c>
       <c r="BE43" t="n">
         <v>81.5</v>
       </c>
       <c r="BF43" t="n">
-        <v>-86.13</v>
+        <v>-86.06999999999999</v>
       </c>
       <c r="BG43" t="n">
-        <v>19.78</v>
+        <v>20.31</v>
       </c>
       <c r="BH43" t="n">
         <v>5.61</v>
@@ -10405,7 +10405,7 @@
         <v>0</v>
       </c>
       <c r="BJ43" t="n">
-        <v>40.59</v>
+        <v>40.41</v>
       </c>
       <c r="BK43" t="n">
         <v>4.73</v>
@@ -10414,7 +10414,7 @@
         <v>4.73</v>
       </c>
       <c r="BM43" t="n">
-        <v>40.95</v>
+        <v>41.05</v>
       </c>
       <c r="BN43" t="n">
         <v>42.98</v>
@@ -10423,19 +10423,19 @@
         <v>28.06</v>
       </c>
       <c r="BP43" t="n">
-        <v>40.01</v>
+        <v>40.06</v>
       </c>
       <c r="BQ43" t="n">
-        <v>8.57</v>
+        <v>8.539999999999999</v>
       </c>
       <c r="BR43" t="n">
-        <v>40.16</v>
+        <v>40.63</v>
       </c>
       <c r="BS43" t="n">
         <v>0</v>
       </c>
       <c r="BT43" t="n">
-        <v>6773488</v>
+        <v>6705721</v>
       </c>
     </row>
     <row r="44">
@@ -10925,13 +10925,13 @@
         </is>
       </c>
       <c r="F46" t="n">
-        <v>4</v>
+        <v>3.81</v>
       </c>
       <c r="G46" t="n">
-        <v>4003328000</v>
+        <v>3812061152</v>
       </c>
       <c r="H46" t="n">
-        <v>13869800</v>
+        <v>29974200</v>
       </c>
       <c r="I46" t="n">
         <v>1000541644</v>
@@ -10946,7 +10946,7 @@
         <v>2.5</v>
       </c>
       <c r="M46" t="n">
-        <v>0.06958540513499498</v>
+        <v>0.06626082590816831</v>
       </c>
       <c r="N46" t="n">
         <v>0.08</v>
@@ -11024,7 +11024,7 @@
         <v>460249156.24</v>
       </c>
       <c r="AM46" t="n">
-        <v>3924831372.549019</v>
+        <v>3737314854.901961</v>
       </c>
       <c r="AN46" t="n">
         <v>0.0311</v>
@@ -11065,7 +11065,7 @@
         <v>3.3</v>
       </c>
       <c r="AZ46" t="n">
-        <v>3.3</v>
+        <v>3.14</v>
       </c>
       <c r="BA46" t="n">
         <v>0.42</v>
@@ -11074,19 +11074,19 @@
         <v>7.38</v>
       </c>
       <c r="BC46" t="n">
-        <v>1.1</v>
+        <v>6.14</v>
       </c>
       <c r="BD46" t="n">
-        <v>-17.45</v>
+        <v>-13.34</v>
       </c>
       <c r="BE46" t="n">
         <v>-17.5</v>
       </c>
       <c r="BF46" t="n">
-        <v>-89.42</v>
+        <v>-88.90000000000001</v>
       </c>
       <c r="BG46" t="n">
-        <v>84.47</v>
+        <v>93.66</v>
       </c>
       <c r="BH46" t="n">
         <v>1.58</v>
@@ -11095,7 +11095,7 @@
         <v>0</v>
       </c>
       <c r="BJ46" t="n">
-        <v>4</v>
+        <v>3.81</v>
       </c>
       <c r="BK46" t="n">
         <v>0.46</v>
@@ -11104,7 +11104,7 @@
         <v>0.46</v>
       </c>
       <c r="BM46" t="n">
-        <v>4.04</v>
+        <v>4.05</v>
       </c>
       <c r="BN46" t="n">
         <v>7.31</v>
@@ -11113,19 +11113,19 @@
         <v>2.97</v>
       </c>
       <c r="BP46" t="n">
-        <v>3.94</v>
+        <v>3.78</v>
       </c>
       <c r="BQ46" t="n">
-        <v>8.74</v>
+        <v>8.33</v>
       </c>
       <c r="BR46" t="n">
-        <v>4.03</v>
+        <v>4.01</v>
       </c>
       <c r="BS46" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="BT46" t="n">
-        <v>20476617</v>
+        <v>20775803</v>
       </c>
     </row>
     <row r="47">
@@ -11155,13 +11155,13 @@
         </is>
       </c>
       <c r="F47" t="n">
-        <v>8.99</v>
+        <v>8.82</v>
       </c>
       <c r="G47" t="n">
-        <v>3153507624</v>
+        <v>3078731143</v>
       </c>
       <c r="H47" t="n">
-        <v>8600</v>
+        <v>12100</v>
       </c>
       <c r="I47" t="n">
         <v>254106600</v>
@@ -11176,7 +11176,7 @@
         <v>1.22</v>
       </c>
       <c r="M47" t="n">
-        <v>0.7436333796645614</v>
+        <v>0.7260002251219001</v>
       </c>
       <c r="N47" t="n">
         <v>0.07000000000000001</v>
@@ -11254,7 +11254,7 @@
         <v>322715382</v>
       </c>
       <c r="AM47" t="n">
-        <v>559132557.4468086</v>
+        <v>545874316.1347518</v>
       </c>
       <c r="AN47" t="n">
         <v>0.4132</v>
@@ -11295,7 +11295,7 @@
         <v>11.74</v>
       </c>
       <c r="AZ47" t="n">
-        <v>11.81</v>
+        <v>11.58</v>
       </c>
       <c r="BA47" t="n">
         <v>1.46</v>
@@ -11304,19 +11304,19 @@
         <v>8.619999999999999</v>
       </c>
       <c r="BC47" t="n">
-        <v>59.88</v>
+        <v>62.96</v>
       </c>
       <c r="BD47" t="n">
-        <v>30.54</v>
+        <v>33.06</v>
       </c>
       <c r="BE47" t="n">
         <v>31.33</v>
       </c>
       <c r="BF47" t="n">
-        <v>-83.78</v>
+        <v>-83.45999999999999</v>
       </c>
       <c r="BG47" t="n">
-        <v>-4.12</v>
+        <v>-2.27</v>
       </c>
       <c r="BH47" t="n">
         <v>7.23</v>
@@ -11325,7 +11325,7 @@
         <v>0</v>
       </c>
       <c r="BJ47" t="n">
-        <v>8.99</v>
+        <v>8.82</v>
       </c>
       <c r="BK47" t="n">
         <v>1.27</v>
@@ -11334,7 +11334,7 @@
         <v>1.29</v>
       </c>
       <c r="BM47" t="n">
-        <v>9.050000000000001</v>
+        <v>9.029999999999999</v>
       </c>
       <c r="BN47" t="n">
         <v>9.25</v>
@@ -11343,19 +11343,19 @@
         <v>7.2</v>
       </c>
       <c r="BP47" t="n">
-        <v>8.84</v>
+        <v>8.81</v>
       </c>
       <c r="BQ47" t="n">
-        <v>6.95</v>
+        <v>6.82</v>
       </c>
       <c r="BR47" t="n">
-        <v>8.84</v>
+        <v>8.99</v>
       </c>
       <c r="BS47" t="n">
         <v>0.53</v>
       </c>
       <c r="BT47" t="n">
-        <v>12614</v>
+        <v>12172</v>
       </c>
     </row>
     <row r="48">
@@ -11385,13 +11385,13 @@
         </is>
       </c>
       <c r="F48" t="n">
-        <v>9.140000000000001</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="G48" t="n">
-        <v>3153507624</v>
+        <v>3078731143</v>
       </c>
       <c r="H48" t="n">
-        <v>3800</v>
+        <v>3100</v>
       </c>
       <c r="I48" t="n">
         <v>93397546</v>
@@ -11406,7 +11406,7 @@
         <v>1.24</v>
       </c>
       <c r="M48" t="n">
-        <v>2.023202512762711</v>
+        <v>1.975228008720493</v>
       </c>
       <c r="N48" t="n">
         <v>0.07000000000000001</v>
@@ -11484,7 +11484,7 @@
         <v>118614883.42</v>
       </c>
       <c r="AM48" t="n">
-        <v>551312521.6783217</v>
+        <v>538239710.3146853</v>
       </c>
       <c r="AN48" t="n">
         <v>0.4132</v>
@@ -11525,7 +11525,7 @@
         <v>11.74</v>
       </c>
       <c r="AZ48" t="n">
-        <v>11.96</v>
+        <v>11.93</v>
       </c>
       <c r="BA48" t="n">
         <v>1.46</v>
@@ -11534,19 +11534,19 @@
         <v>8.24</v>
       </c>
       <c r="BC48" t="n">
-        <v>57.26</v>
+        <v>57.6</v>
       </c>
       <c r="BD48" t="n">
-        <v>28.4</v>
+        <v>28.68</v>
       </c>
       <c r="BE48" t="n">
         <v>30.83</v>
       </c>
       <c r="BF48" t="n">
-        <v>-84.04000000000001</v>
+        <v>-84.01000000000001</v>
       </c>
       <c r="BG48" t="n">
-        <v>-9.890000000000001</v>
+        <v>-9.69</v>
       </c>
       <c r="BH48" t="n">
         <v>7.23</v>
@@ -11555,7 +11555,7 @@
         <v>0</v>
       </c>
       <c r="BJ48" t="n">
-        <v>9.140000000000001</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="BK48" t="n">
         <v>1.27</v>
@@ -11564,7 +11564,7 @@
         <v>1.29</v>
       </c>
       <c r="BM48" t="n">
-        <v>9.140000000000001</v>
+        <v>9.15</v>
       </c>
       <c r="BN48" t="n">
         <v>9.48</v>
@@ -11573,19 +11573,19 @@
         <v>7.21</v>
       </c>
       <c r="BP48" t="n">
-        <v>9.01</v>
+        <v>9.1</v>
       </c>
       <c r="BQ48" t="n">
-        <v>7.07</v>
+        <v>7.05</v>
       </c>
       <c r="BR48" t="n">
-        <v>9.029999999999999</v>
+        <v>9.130000000000001</v>
       </c>
       <c r="BS48" t="n">
         <v>0.54</v>
       </c>
       <c r="BT48" t="n">
-        <v>2651</v>
+        <v>2577</v>
       </c>
     </row>
     <row r="49">
@@ -11845,13 +11845,13 @@
         </is>
       </c>
       <c r="F50" t="n">
-        <v>33.01</v>
+        <v>32.96</v>
       </c>
       <c r="G50" t="n">
-        <v>972024300</v>
+        <v>956853500</v>
       </c>
       <c r="H50" t="n">
-        <v>600</v>
+        <v>300</v>
       </c>
       <c r="I50" t="n">
         <v>11540870</v>
@@ -11866,7 +11866,7 @@
         <v>0.8</v>
       </c>
       <c r="M50" t="n">
-        <v>0.9833844466303759</v>
+        <v>0.9680363439513173</v>
       </c>
       <c r="N50" t="n">
         <v>0.06</v>
@@ -11944,7 +11944,7 @@
         <v>84709985.8</v>
       </c>
       <c r="AM50" t="n">
-        <v>331748907.8498293</v>
+        <v>326571160.4095563</v>
       </c>
       <c r="AN50" t="n">
         <v>4.4983</v>
@@ -11985,7 +11985,7 @@
         <v>68.48999999999999</v>
       </c>
       <c r="AZ50" t="n">
-        <v>72.79000000000001</v>
+        <v>72.68000000000001</v>
       </c>
       <c r="BA50" t="n">
         <v>9.210000000000001</v>
@@ -11994,19 +11994,19 @@
         <v>30.53</v>
       </c>
       <c r="BC50" t="n">
-        <v>154.1</v>
+        <v>154.48</v>
       </c>
       <c r="BD50" t="n">
-        <v>107.47</v>
+        <v>107.78</v>
       </c>
       <c r="BE50" t="n">
         <v>120.5</v>
       </c>
       <c r="BF50" t="n">
-        <v>-72.09</v>
+        <v>-72.05</v>
       </c>
       <c r="BG50" t="n">
-        <v>-7.51</v>
+        <v>-7.37</v>
       </c>
       <c r="BH50" t="n">
         <v>42.6</v>
@@ -12015,7 +12015,7 @@
         <v>0</v>
       </c>
       <c r="BJ50" t="n">
-        <v>33.01</v>
+        <v>32.96</v>
       </c>
       <c r="BK50" t="n">
         <v>7.34</v>
@@ -12024,7 +12024,7 @@
         <v>7.6</v>
       </c>
       <c r="BM50" t="n">
-        <v>33.8</v>
+        <v>33.49</v>
       </c>
       <c r="BN50" t="n">
         <v>39.22</v>
@@ -12033,19 +12033,19 @@
         <v>23.5</v>
       </c>
       <c r="BP50" t="n">
-        <v>33.01</v>
+        <v>32.96</v>
       </c>
       <c r="BQ50" t="n">
         <v>4.34</v>
       </c>
       <c r="BR50" t="n">
-        <v>33.8</v>
+        <v>33.49</v>
       </c>
       <c r="BS50" t="n">
         <v>0.4</v>
       </c>
       <c r="BT50" t="n">
-        <v>670</v>
+        <v>543</v>
       </c>
     </row>
     <row r="51">
@@ -12523,13 +12523,13 @@
         </is>
       </c>
       <c r="F53" t="n">
-        <v>6.61</v>
+        <v>6.26</v>
       </c>
       <c r="G53" t="n">
-        <v>904858121</v>
+        <v>856696055</v>
       </c>
       <c r="H53" t="n">
-        <v>22500</v>
+        <v>195700</v>
       </c>
       <c r="I53" t="n">
         <v>136852484</v>
@@ -12544,7 +12544,7 @@
         <v>2.79</v>
       </c>
       <c r="M53" t="n">
-        <v>2.350652714623625</v>
+        <v>2.225536645532411</v>
       </c>
       <c r="N53" t="n">
         <v>1.48</v>
@@ -12622,7 +12622,7 @@
         <v>39687220.36</v>
       </c>
       <c r="AM53" t="n">
-        <v>46095676.05705553</v>
+        <v>43642183.138054</v>
       </c>
       <c r="AN53" t="n">
         <v>0</v>
@@ -12672,16 +12672,16 @@
         <v>0</v>
       </c>
       <c r="BC53" t="n">
-        <v>-40.38</v>
+        <v>-37.05</v>
       </c>
       <c r="BD53" t="n">
-        <v>-51.32</v>
+        <v>-48.6</v>
       </c>
       <c r="BE53" t="n">
         <v>-100</v>
       </c>
       <c r="BF53" t="n">
-        <v>-95.61</v>
+        <v>-95.37</v>
       </c>
       <c r="BG53" t="n">
         <v>-100</v>
@@ -12693,7 +12693,7 @@
         <v>0</v>
       </c>
       <c r="BJ53" t="n">
-        <v>6.61</v>
+        <v>6.26</v>
       </c>
       <c r="BK53" t="n">
         <v>0.29</v>
@@ -12702,7 +12702,7 @@
         <v>0.09</v>
       </c>
       <c r="BM53" t="n">
-        <v>6.73</v>
+        <v>6.56</v>
       </c>
       <c r="BN53" t="n">
         <v>10.39</v>
@@ -12711,19 +12711,19 @@
         <v>4.82</v>
       </c>
       <c r="BP53" t="n">
-        <v>6.43</v>
+        <v>6.26</v>
       </c>
       <c r="BQ53" t="n">
-        <v>77.47</v>
+        <v>73.37</v>
       </c>
       <c r="BR53" t="n">
-        <v>6.51</v>
+        <v>6.56</v>
       </c>
       <c r="BS53" t="n">
         <v>2.36</v>
       </c>
       <c r="BT53" t="n">
-        <v>38050</v>
+        <v>37217</v>
       </c>
     </row>
     <row r="54">
@@ -12753,13 +12753,13 @@
         </is>
       </c>
       <c r="F54" t="n">
-        <v>10.55</v>
+        <v>10.69</v>
       </c>
       <c r="G54" t="n">
-        <v>2461104044</v>
+        <v>2493037251</v>
       </c>
       <c r="H54" t="n">
-        <v>273200</v>
+        <v>344100</v>
       </c>
       <c r="I54" t="n">
         <v>233212121</v>
@@ -12774,7 +12774,7 @@
         <v>0.97</v>
       </c>
       <c r="M54" t="n">
-        <v>1.38139697875995</v>
+        <v>1.399320818989078</v>
       </c>
       <c r="N54" t="n">
         <v>0.5600000000000001</v>
@@ -12852,7 +12852,7 @@
         <v>233212121</v>
       </c>
       <c r="AM54" t="n">
-        <v>336676339.8084816</v>
+        <v>341044767.5786594</v>
       </c>
       <c r="AN54" t="n">
         <v>0.1531</v>
@@ -12893,7 +12893,7 @@
         <v>12.25</v>
       </c>
       <c r="AZ54" t="n">
-        <v>16.79</v>
+        <v>17.01</v>
       </c>
       <c r="BA54" t="n">
         <v>0.98</v>
@@ -12902,19 +12902,19 @@
         <v>6.52</v>
       </c>
       <c r="BC54" t="n">
-        <v>42.25</v>
+        <v>40.39</v>
       </c>
       <c r="BD54" t="n">
-        <v>16.15</v>
+        <v>14.63</v>
       </c>
       <c r="BE54" t="n">
         <v>59.17</v>
       </c>
       <c r="BF54" t="n">
-        <v>-90.68000000000001</v>
+        <v>-90.8</v>
       </c>
       <c r="BG54" t="n">
-        <v>-38.23</v>
+        <v>-39.04</v>
       </c>
       <c r="BH54" t="n">
         <v>10.01</v>
@@ -12923,7 +12923,7 @@
         <v>0</v>
       </c>
       <c r="BJ54" t="n">
-        <v>10.55</v>
+        <v>10.69</v>
       </c>
       <c r="BK54" t="n">
         <v>1</v>
@@ -12932,7 +12932,7 @@
         <v>1</v>
       </c>
       <c r="BM54" t="n">
-        <v>10.63</v>
+        <v>10.96</v>
       </c>
       <c r="BN54" t="n">
         <v>11.75</v>
@@ -12941,19 +12941,19 @@
         <v>8.279999999999999</v>
       </c>
       <c r="BP54" t="n">
-        <v>10.26</v>
+        <v>10.58</v>
       </c>
       <c r="BQ54" t="n">
-        <v>10.52</v>
+        <v>10.66</v>
       </c>
       <c r="BR54" t="n">
-        <v>10.31</v>
+        <v>10.58</v>
       </c>
       <c r="BS54" t="n">
         <v>1.26</v>
       </c>
       <c r="BT54" t="n">
-        <v>264583</v>
+        <v>265840</v>
       </c>
     </row>
     <row r="55">
@@ -12983,13 +12983,13 @@
         </is>
       </c>
       <c r="F55" t="n">
-        <v>49.23</v>
+        <v>49.2</v>
       </c>
       <c r="G55" t="n">
-        <v>6562892176</v>
+        <v>6427234179</v>
       </c>
       <c r="H55" t="n">
-        <v>15900</v>
+        <v>8900</v>
       </c>
       <c r="I55" t="n">
         <v>84052790</v>
@@ -13004,7 +13004,7 @@
         <v>2</v>
       </c>
       <c r="M55" t="n">
-        <v>1.013121267755574</v>
+        <v>0.9921795856105552</v>
       </c>
       <c r="N55" t="n">
         <v>0.16</v>
@@ -13082,7 +13082,7 @@
         <v>579123723.1</v>
       </c>
       <c r="AM55" t="n">
-        <v>330125360.9657948</v>
+        <v>323301518.0583501</v>
       </c>
       <c r="AN55" t="n">
         <v>3.1953</v>
@@ -13123,7 +13123,7 @@
         <v>51.21</v>
       </c>
       <c r="AZ55" t="n">
-        <v>51.77</v>
+        <v>51.74</v>
       </c>
       <c r="BA55" t="n">
         <v>9.380000000000001</v>
@@ -13132,19 +13132,19 @@
         <v>16.08</v>
       </c>
       <c r="BC55" t="n">
-        <v>27.39</v>
+        <v>27.47</v>
       </c>
       <c r="BD55" t="n">
-        <v>4.01</v>
+        <v>4.08</v>
       </c>
       <c r="BE55" t="n">
         <v>5.17</v>
       </c>
       <c r="BF55" t="n">
-        <v>-80.95</v>
+        <v>-80.94</v>
       </c>
       <c r="BG55" t="n">
-        <v>-67.34</v>
+        <v>-67.31999999999999</v>
       </c>
       <c r="BH55" t="n">
         <v>25.37</v>
@@ -13153,7 +13153,7 @@
         <v>0</v>
       </c>
       <c r="BJ55" t="n">
-        <v>49.23</v>
+        <v>49.2</v>
       </c>
       <c r="BK55" t="n">
         <v>6.89</v>
@@ -13162,7 +13162,7 @@
         <v>7.03</v>
       </c>
       <c r="BM55" t="n">
-        <v>49.52</v>
+        <v>49.93</v>
       </c>
       <c r="BN55" t="n">
         <v>73.67</v>
@@ -13171,19 +13171,19 @@
         <v>35.58</v>
       </c>
       <c r="BP55" t="n">
-        <v>49.1</v>
+        <v>49.01</v>
       </c>
       <c r="BQ55" t="n">
         <v>7</v>
       </c>
       <c r="BR55" t="n">
-        <v>49.52</v>
+        <v>49.87</v>
       </c>
       <c r="BS55" t="n">
         <v>0.66</v>
       </c>
       <c r="BT55" t="n">
-        <v>7180</v>
+        <v>7594</v>
       </c>
     </row>
     <row r="56">
@@ -13213,13 +13213,13 @@
         </is>
       </c>
       <c r="F56" t="n">
-        <v>59.84</v>
+        <v>59.06</v>
       </c>
       <c r="G56" t="n">
-        <v>6562892176</v>
+        <v>6427234179</v>
       </c>
       <c r="H56" t="n">
-        <v>16200</v>
+        <v>18000</v>
       </c>
       <c r="I56" t="n">
         <v>39675836</v>
@@ -13234,7 +13234,7 @@
         <v>2.41</v>
       </c>
       <c r="M56" t="n">
-        <v>2.146285440921599</v>
+        <v>2.101920734615675</v>
       </c>
       <c r="N56" t="n">
         <v>0.19</v>
@@ -13312,7 +13312,7 @@
         <v>273366510.04</v>
       </c>
       <c r="AM56" t="n">
-        <v>272998842.5956739</v>
+        <v>267355831.0732113</v>
       </c>
       <c r="AN56" t="n">
         <v>3.5102</v>
@@ -13353,7 +13353,7 @@
         <v>51.21</v>
       </c>
       <c r="AZ56" t="n">
-        <v>57.15</v>
+        <v>56.4</v>
       </c>
       <c r="BA56" t="n">
         <v>9.380000000000001</v>
@@ -13362,19 +13362,19 @@
         <v>17.68</v>
       </c>
       <c r="BC56" t="n">
-        <v>4.8</v>
+        <v>6.19</v>
       </c>
       <c r="BD56" t="n">
-        <v>-14.43</v>
+        <v>-13.3</v>
       </c>
       <c r="BE56" t="n">
         <v>-4.5</v>
       </c>
       <c r="BF56" t="n">
-        <v>-84.33</v>
+        <v>-84.12</v>
       </c>
       <c r="BG56" t="n">
-        <v>-70.45999999999999</v>
+        <v>-70.06999999999999</v>
       </c>
       <c r="BH56" t="n">
         <v>25.37</v>
@@ -13383,7 +13383,7 @@
         <v>0</v>
       </c>
       <c r="BJ56" t="n">
-        <v>59.84</v>
+        <v>59.06</v>
       </c>
       <c r="BK56" t="n">
         <v>6.89</v>
@@ -13392,7 +13392,7 @@
         <v>7.03</v>
       </c>
       <c r="BM56" t="n">
-        <v>60.55</v>
+        <v>60.46</v>
       </c>
       <c r="BN56" t="n">
         <v>86.77</v>
@@ -13401,19 +13401,19 @@
         <v>46.42</v>
       </c>
       <c r="BP56" t="n">
-        <v>58.58</v>
+        <v>59</v>
       </c>
       <c r="BQ56" t="n">
-        <v>8.51</v>
+        <v>8.4</v>
       </c>
       <c r="BR56" t="n">
-        <v>59.99</v>
+        <v>60.4</v>
       </c>
       <c r="BS56" t="n">
         <v>0.79</v>
       </c>
       <c r="BT56" t="n">
-        <v>35013</v>
+        <v>34553</v>
       </c>
     </row>
     <row r="57">
@@ -13443,13 +13443,13 @@
         </is>
       </c>
       <c r="F57" t="n">
-        <v>6.03</v>
+        <v>6.05</v>
       </c>
       <c r="G57" t="n">
-        <v>1410574432</v>
+        <v>1414840944</v>
       </c>
       <c r="H57" t="n">
-        <v>1147700</v>
+        <v>740400</v>
       </c>
       <c r="I57" t="n">
         <v>233858065</v>
@@ -13464,7 +13464,7 @@
         <v>0.77</v>
       </c>
       <c r="M57" t="n">
-        <v>0.4222228138251294</v>
+        <v>0.4234998954600946</v>
       </c>
       <c r="N57" t="n">
         <v>0.08</v>
@@ -13542,7 +13542,7 @@
         <v>229180903.7</v>
       </c>
       <c r="AM57" t="n">
-        <v>105502949.289454</v>
+        <v>105822060.1346298</v>
       </c>
       <c r="AN57" t="n">
         <v>0.347</v>
@@ -13583,7 +13583,7 @@
         <v>10.72</v>
       </c>
       <c r="AZ57" t="n">
-        <v>9.199999999999999</v>
+        <v>9.23</v>
       </c>
       <c r="BA57" t="n">
         <v>1.13</v>
@@ -13592,19 +13592,19 @@
         <v>6.26</v>
       </c>
       <c r="BC57" t="n">
-        <v>117.77</v>
+        <v>117.05</v>
       </c>
       <c r="BD57" t="n">
-        <v>77.81</v>
+        <v>77.22</v>
       </c>
       <c r="BE57" t="n">
         <v>52.5</v>
       </c>
       <c r="BF57" t="n">
-        <v>-81.3</v>
+        <v>-81.36</v>
       </c>
       <c r="BG57" t="n">
-        <v>3.88</v>
+        <v>3.54</v>
       </c>
       <c r="BH57" t="n">
         <v>7.82</v>
@@ -13613,7 +13613,7 @@
         <v>0</v>
       </c>
       <c r="BJ57" t="n">
-        <v>6.03</v>
+        <v>6.05</v>
       </c>
       <c r="BK57" t="n">
         <v>0.98</v>
@@ -13622,7 +13622,7 @@
         <v>1.04</v>
       </c>
       <c r="BM57" t="n">
-        <v>6.16</v>
+        <v>6.07</v>
       </c>
       <c r="BN57" t="n">
         <v>6.18</v>
@@ -13631,19 +13631,19 @@
         <v>3.43</v>
       </c>
       <c r="BP57" t="n">
-        <v>5.98</v>
+        <v>5.97</v>
       </c>
       <c r="BQ57" t="n">
-        <v>5.82</v>
+        <v>5.84</v>
       </c>
       <c r="BR57" t="n">
-        <v>6.15</v>
+        <v>6.03</v>
       </c>
       <c r="BS57" t="n">
         <v>0.42</v>
       </c>
       <c r="BT57" t="n">
-        <v>1300412</v>
+        <v>1286956</v>
       </c>
     </row>
     <row r="58">
@@ -14133,13 +14133,13 @@
         </is>
       </c>
       <c r="F60" t="n">
-        <v>376</v>
+        <v>380</v>
       </c>
       <c r="G60" t="n">
-        <v>171035782</v>
+        <v>172805000</v>
       </c>
       <c r="H60" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="I60" t="n">
         <v>454750</v>
@@ -14154,7 +14154,7 @@
         <v>0.83</v>
       </c>
       <c r="M60" t="n">
-        <v>12.79323572552968</v>
+        <v>12.92557074139116</v>
       </c>
       <c r="N60" t="n">
         <v>0.68</v>
@@ -14232,7 +14232,7 @@
         <v>59558607.5</v>
       </c>
       <c r="AM60" t="n">
-        <v>-25078560.41055718</v>
+        <v>-25337976.53958944</v>
       </c>
       <c r="AN60" t="n">
         <v>10.0581</v>
@@ -14273,7 +14273,7 @@
         <v>944.87</v>
       </c>
       <c r="AZ60" t="n">
-        <v>2162</v>
+        <v>2185</v>
       </c>
       <c r="BA60" t="n">
         <v>231.1</v>
@@ -14282,19 +14282,19 @@
         <v>727.97</v>
       </c>
       <c r="BC60" t="n">
-        <v>207.77</v>
+        <v>204.53</v>
       </c>
       <c r="BD60" t="n">
-        <v>151.29</v>
+        <v>148.65</v>
       </c>
       <c r="BE60" t="n">
         <v>475</v>
       </c>
       <c r="BF60" t="n">
-        <v>-38.54</v>
+        <v>-39.19</v>
       </c>
       <c r="BG60" t="n">
-        <v>93.61</v>
+        <v>91.56999999999999</v>
       </c>
       <c r="BH60" t="n">
         <v>454.44</v>
@@ -14303,7 +14303,7 @@
         <v>0</v>
       </c>
       <c r="BJ60" t="n">
-        <v>376</v>
+        <v>380</v>
       </c>
       <c r="BK60" t="n">
         <v>130.97</v>
@@ -14312,7 +14312,7 @@
         <v>130.97</v>
       </c>
       <c r="BM60" t="n">
-        <v>377.09</v>
+        <v>380</v>
       </c>
       <c r="BN60" t="n">
         <v>405</v>
@@ -14321,19 +14321,19 @@
         <v>306.27</v>
       </c>
       <c r="BP60" t="n">
-        <v>376</v>
+        <v>377.09</v>
       </c>
       <c r="BQ60" t="n">
-        <v>2.87</v>
+        <v>2.9</v>
       </c>
       <c r="BR60" t="n">
-        <v>377</v>
+        <v>377.09</v>
       </c>
       <c r="BS60" t="n">
         <v>12.82</v>
       </c>
       <c r="BT60" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="61">
@@ -14363,13 +14363,13 @@
         </is>
       </c>
       <c r="F61" t="n">
-        <v>27.45</v>
+        <v>27.64</v>
       </c>
       <c r="G61" t="n">
-        <v>2350634150</v>
+        <v>2366215294</v>
       </c>
       <c r="H61" t="n">
-        <v>560200</v>
+        <v>369500</v>
       </c>
       <c r="I61" t="n">
         <v>85608392</v>
@@ -14384,7 +14384,7 @@
         <v>2.37</v>
       </c>
       <c r="M61" t="n">
-        <v>1.246621995390583</v>
+        <v>1.254885211009972</v>
       </c>
       <c r="N61" t="n">
         <v>1.1</v>
@@ -14462,7 +14462,7 @@
         <v>160087693.04</v>
       </c>
       <c r="AM61" t="n">
-        <v>184508175.0392465</v>
+        <v>185731184.7723705</v>
       </c>
       <c r="AN61" t="n">
         <v>0.38</v>
@@ -14503,7 +14503,7 @@
         <v>17.56</v>
       </c>
       <c r="AZ61" t="n">
-        <v>34.59</v>
+        <v>34.83</v>
       </c>
       <c r="BA61" t="n">
         <v>2.52</v>
@@ -14512,19 +14512,19 @@
         <v>11.76</v>
       </c>
       <c r="BC61" t="n">
-        <v>-21.66</v>
+        <v>-22.2</v>
       </c>
       <c r="BD61" t="n">
-        <v>-36.04</v>
+        <v>-36.48</v>
       </c>
       <c r="BE61" t="n">
         <v>26</v>
       </c>
       <c r="BF61" t="n">
-        <v>-90.81</v>
+        <v>-90.87</v>
       </c>
       <c r="BG61" t="n">
-        <v>-57.17</v>
+        <v>-57.47</v>
       </c>
       <c r="BH61" t="n">
         <v>10.99</v>
@@ -14533,7 +14533,7 @@
         <v>0</v>
       </c>
       <c r="BJ61" t="n">
-        <v>27.45</v>
+        <v>27.64</v>
       </c>
       <c r="BK61" t="n">
         <v>1.87</v>
@@ -14542,7 +14542,7 @@
         <v>1.86</v>
       </c>
       <c r="BM61" t="n">
-        <v>28</v>
+        <v>28.07</v>
       </c>
       <c r="BN61" t="n">
         <v>28.25</v>
@@ -14551,19 +14551,19 @@
         <v>19.35</v>
       </c>
       <c r="BP61" t="n">
-        <v>26.88</v>
+        <v>27.49</v>
       </c>
       <c r="BQ61" t="n">
-        <v>14.74</v>
+        <v>14.84</v>
       </c>
       <c r="BR61" t="n">
-        <v>27.6</v>
+        <v>27.61</v>
       </c>
       <c r="BS61" t="n">
         <v>1.19</v>
       </c>
       <c r="BT61" t="n">
-        <v>504287</v>
+        <v>509514</v>
       </c>
     </row>
     <row r="62">
@@ -14823,13 +14823,13 @@
         </is>
       </c>
       <c r="F63" t="n">
-        <v>1.41</v>
+        <v>1.38</v>
       </c>
       <c r="G63" t="n">
-        <v>367425687</v>
+        <v>359503384</v>
       </c>
       <c r="H63" t="n">
-        <v>20300</v>
+        <v>31900</v>
       </c>
       <c r="I63" t="n">
         <v>122894462</v>
@@ -14844,7 +14844,7 @@
         <v>-0.22</v>
       </c>
       <c r="M63" t="n">
-        <v>0.451914633596502</v>
+        <v>0.4421706097458084</v>
       </c>
       <c r="N63" t="n">
         <v>0.37</v>
@@ -14922,7 +14922,7 @@
         <v>31952560.12</v>
       </c>
       <c r="AM63" t="n">
-        <v>208764594.8863636</v>
+        <v>204263286.3636364</v>
       </c>
       <c r="AN63" t="n">
         <v>0</v>
@@ -14981,7 +14981,7 @@
         <v>-100</v>
       </c>
       <c r="BF63" t="n">
-        <v>-79.48999999999999</v>
+        <v>-79.05</v>
       </c>
       <c r="BG63" t="n">
         <v>-100</v>
@@ -14993,7 +14993,7 @@
         <v>0</v>
       </c>
       <c r="BJ63" t="n">
-        <v>1.41</v>
+        <v>1.38</v>
       </c>
       <c r="BK63" t="n">
         <v>0.26</v>
@@ -15002,7 +15002,7 @@
         <v>0.26</v>
       </c>
       <c r="BM63" t="n">
-        <v>1.52</v>
+        <v>1.44</v>
       </c>
       <c r="BN63" t="n">
         <v>2.12</v>
@@ -15011,19 +15011,19 @@
         <v>1.16</v>
       </c>
       <c r="BP63" t="n">
-        <v>1.36</v>
+        <v>1.34</v>
       </c>
       <c r="BQ63" t="n">
-        <v>5.4</v>
+        <v>5.29</v>
       </c>
       <c r="BR63" t="n">
-        <v>1.51</v>
+        <v>1.37</v>
       </c>
       <c r="BS63" t="n">
         <v>0.19</v>
       </c>
       <c r="BT63" t="n">
-        <v>22040</v>
+        <v>22640</v>
       </c>
     </row>
     <row r="64">
@@ -15053,13 +15053,13 @@
         </is>
       </c>
       <c r="F64" t="n">
-        <v>60.83</v>
+        <v>61.14</v>
       </c>
       <c r="G64" t="n">
-        <v>234363823664</v>
+        <v>236998752694</v>
       </c>
       <c r="H64" t="n">
-        <v>10448200</v>
+        <v>7134900</v>
       </c>
       <c r="I64" t="n">
         <v>0</v>
@@ -15146,13 +15146,13 @@
         <v>41.22</v>
       </c>
       <c r="AK64" t="n">
-        <v>67195547339.45985</v>
+        <v>67951020157.76189</v>
       </c>
       <c r="AL64" t="n">
-        <v>18734118598.24141</v>
+        <v>18944744419.98401</v>
       </c>
       <c r="AM64" t="n">
-        <v>20869441109.88424</v>
+        <v>21104074149.065</v>
       </c>
       <c r="AN64" t="n">
         <v>1.4201</v>
@@ -15193,7 +15193,7 @@
         <v>38.98</v>
       </c>
       <c r="AZ64" t="n">
-        <v>24.33</v>
+        <v>24.46</v>
       </c>
       <c r="BA64" t="n">
         <v>6.69</v>
@@ -15202,19 +15202,19 @@
         <v>10.4</v>
       </c>
       <c r="BC64" t="n">
-        <v>-21.52</v>
+        <v>-21.92</v>
       </c>
       <c r="BD64" t="n">
-        <v>-35.92</v>
+        <v>-36.25</v>
       </c>
       <c r="BE64" t="n">
         <v>-60</v>
       </c>
       <c r="BF64" t="n">
-        <v>-89</v>
+        <v>-89.05</v>
       </c>
       <c r="BG64" t="n">
-        <v>-82.91</v>
+        <v>-82.98999999999999</v>
       </c>
       <c r="BH64" t="n">
         <v>21.37</v>
@@ -15223,7 +15223,7 @@
         <v>0</v>
       </c>
       <c r="BJ64" t="n">
-        <v>60.83</v>
+        <v>61.14</v>
       </c>
       <c r="BK64" t="n">
         <v>4.74</v>
@@ -15232,7 +15232,7 @@
         <v>1.57</v>
       </c>
       <c r="BM64" t="n">
-        <v>61.2</v>
+        <v>61.67</v>
       </c>
       <c r="BN64" t="n">
         <v>64.72</v>
@@ -15241,19 +15241,19 @@
         <v>44.12</v>
       </c>
       <c r="BP64" t="n">
-        <v>59.81</v>
+        <v>59.85</v>
       </c>
       <c r="BQ64" t="n">
-        <v>38.74</v>
+        <v>38.94</v>
       </c>
       <c r="BR64" t="n">
-        <v>60.17</v>
+        <v>60.83</v>
       </c>
       <c r="BS64" t="n">
         <v>3.49</v>
       </c>
       <c r="BT64" t="n">
-        <v>12430983</v>
+        <v>12583835</v>
       </c>
     </row>
     <row r="65">
@@ -15283,13 +15283,13 @@
         </is>
       </c>
       <c r="F65" t="n">
-        <v>23.75</v>
+        <v>23.89</v>
       </c>
       <c r="G65" t="n">
-        <v>234363823664</v>
+        <v>236998752694</v>
       </c>
       <c r="H65" t="n">
-        <v>2400</v>
+        <v>9900</v>
       </c>
       <c r="I65" t="n">
         <v>7298813414</v>
@@ -15304,7 +15304,7 @@
         <v>3.29</v>
       </c>
       <c r="M65" t="n">
-        <v>5.665966414485257</v>
+        <v>5.729668308212404</v>
       </c>
       <c r="N65" t="n">
         <v>0.29</v>
@@ -15382,7 +15382,7 @@
         <v>11532125194.12</v>
       </c>
       <c r="AM65" t="n">
-        <v>17555342596.55431</v>
+        <v>17752715557.603</v>
       </c>
       <c r="AN65" t="n">
         <v>0.4734</v>
@@ -15423,7 +15423,7 @@
         <v>12.99</v>
       </c>
       <c r="AZ65" t="n">
-        <v>8</v>
+        <v>8.039999999999999</v>
       </c>
       <c r="BA65" t="n">
         <v>2.23</v>
@@ -15432,19 +15432,19 @@
         <v>3.47</v>
       </c>
       <c r="BC65" t="n">
-        <v>-33.01</v>
+        <v>-33.4</v>
       </c>
       <c r="BD65" t="n">
-        <v>-45.3</v>
+        <v>-45.63</v>
       </c>
       <c r="BE65" t="n">
         <v>-66.33</v>
       </c>
       <c r="BF65" t="n">
-        <v>-90.61</v>
+        <v>-90.66</v>
       </c>
       <c r="BG65" t="n">
-        <v>-85.41</v>
+        <v>-85.48999999999999</v>
       </c>
       <c r="BH65" t="n">
         <v>7.12</v>
@@ -15453,7 +15453,7 @@
         <v>0</v>
       </c>
       <c r="BJ65" t="n">
-        <v>23.75</v>
+        <v>23.89</v>
       </c>
       <c r="BK65" t="n">
         <v>1.58</v>
@@ -15471,19 +15471,19 @@
         <v>20.44</v>
       </c>
       <c r="BP65" t="n">
-        <v>23.53</v>
+        <v>23.63</v>
       </c>
       <c r="BQ65" t="n">
-        <v>15.13</v>
+        <v>15.22</v>
       </c>
       <c r="BR65" t="n">
-        <v>23.89</v>
+        <v>23.67</v>
       </c>
       <c r="BS65" t="n">
         <v>4.14</v>
       </c>
       <c r="BT65" t="n">
-        <v>11757</v>
+        <v>11504</v>
       </c>
     </row>
     <row r="66">
@@ -15513,13 +15513,13 @@
         </is>
       </c>
       <c r="F66" t="n">
-        <v>21</v>
+        <v>20.21</v>
       </c>
       <c r="G66" t="n">
-        <v>234363823664</v>
+        <v>236998752694</v>
       </c>
       <c r="H66" t="n">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="I66" t="n">
         <v>2972355254</v>
@@ -15534,7 +15534,7 @@
         <v>2.75</v>
       </c>
       <c r="M66" t="n">
-        <v>13.91315241126237</v>
+        <v>14.06957659232458</v>
       </c>
       <c r="N66" t="n">
         <v>0.25</v>
@@ -15612,7 +15612,7 @@
         <v>4696321301.320001</v>
       </c>
       <c r="AM66" t="n">
-        <v>21019177010.22422</v>
+        <v>21255493515.15695</v>
       </c>
       <c r="AN66" t="n">
         <v>0.4734</v>
@@ -15653,7 +15653,7 @@
         <v>12.99</v>
       </c>
       <c r="AZ66" t="n">
-        <v>8.44</v>
+        <v>8.119999999999999</v>
       </c>
       <c r="BA66" t="n">
         <v>2.23</v>
@@ -15662,19 +15662,19 @@
         <v>3.47</v>
       </c>
       <c r="BC66" t="n">
-        <v>-24.24</v>
+        <v>-21.28</v>
       </c>
       <c r="BD66" t="n">
-        <v>-38.14</v>
+        <v>-35.72</v>
       </c>
       <c r="BE66" t="n">
         <v>-59.83</v>
       </c>
       <c r="BF66" t="n">
-        <v>-89.37</v>
+        <v>-88.95999999999999</v>
       </c>
       <c r="BG66" t="n">
-        <v>-83.5</v>
+        <v>-82.84999999999999</v>
       </c>
       <c r="BH66" t="n">
         <v>7.12</v>
@@ -15683,7 +15683,7 @@
         <v>0</v>
       </c>
       <c r="BJ66" t="n">
-        <v>21</v>
+        <v>20.21</v>
       </c>
       <c r="BK66" t="n">
         <v>1.58</v>
@@ -15692,7 +15692,7 @@
         <v>1.57</v>
       </c>
       <c r="BM66" t="n">
-        <v>21.04</v>
+        <v>20.99</v>
       </c>
       <c r="BN66" t="n">
         <v>21.33</v>
@@ -15701,19 +15701,19 @@
         <v>9.48</v>
       </c>
       <c r="BP66" t="n">
-        <v>20.17</v>
+        <v>20.21</v>
       </c>
       <c r="BQ66" t="n">
-        <v>13.37</v>
+        <v>12.87</v>
       </c>
       <c r="BR66" t="n">
-        <v>20.17</v>
+        <v>20.97</v>
       </c>
       <c r="BS66" t="n">
         <v>3.46</v>
       </c>
       <c r="BT66" t="n">
-        <v>7015</v>
+        <v>6330</v>
       </c>
     </row>
     <row r="67">
@@ -15973,13 +15973,13 @@
         </is>
       </c>
       <c r="F68" t="n">
-        <v>18.43</v>
+        <v>18.51</v>
       </c>
       <c r="G68" t="n">
-        <v>7825980923</v>
+        <v>8054439710</v>
       </c>
       <c r="H68" t="n">
-        <v>70000</v>
+        <v>46100</v>
       </c>
       <c r="I68" t="n">
         <v>137989898</v>
@@ -16072,7 +16072,7 @@
         <v>205604948.02</v>
       </c>
       <c r="AM68" t="n">
-        <v>542717123.6477115</v>
+        <v>558560312.7600554</v>
       </c>
       <c r="AN68" t="n">
         <v>0.1911</v>
@@ -16113,7 +16113,7 @@
         <v>21.39</v>
       </c>
       <c r="AZ68" t="n">
-        <v>34.1</v>
+        <v>34.24</v>
       </c>
       <c r="BA68" t="n">
         <v>1.24</v>
@@ -16122,19 +16122,19 @@
         <v>63.25</v>
       </c>
       <c r="BC68" t="n">
-        <v>42.18</v>
+        <v>41.56</v>
       </c>
       <c r="BD68" t="n">
-        <v>16.09</v>
+        <v>15.58</v>
       </c>
       <c r="BE68" t="n">
         <v>85</v>
       </c>
       <c r="BF68" t="n">
-        <v>-93.27</v>
+        <v>-93.3</v>
       </c>
       <c r="BG68" t="n">
-        <v>243.18</v>
+        <v>241.7</v>
       </c>
       <c r="BH68" t="n">
         <v>20.48</v>
@@ -16143,7 +16143,7 @@
         <v>0</v>
       </c>
       <c r="BJ68" t="n">
-        <v>18.43</v>
+        <v>18.51</v>
       </c>
       <c r="BK68" t="n">
         <v>1.49</v>
@@ -16152,7 +16152,7 @@
         <v>1.49</v>
       </c>
       <c r="BM68" t="n">
-        <v>18.7</v>
+        <v>18.65</v>
       </c>
       <c r="BN68" t="n">
         <v>22.11</v>
@@ -16161,19 +16161,19 @@
         <v>15.39</v>
       </c>
       <c r="BP68" t="n">
-        <v>18.33</v>
+        <v>18.43</v>
       </c>
       <c r="BQ68" t="n">
-        <v>12.4</v>
+        <v>12.45</v>
       </c>
       <c r="BR68" t="n">
-        <v>18.7</v>
+        <v>18.5</v>
       </c>
       <c r="BS68" t="n">
         <v>0</v>
       </c>
       <c r="BT68" t="n">
-        <v>32887</v>
+        <v>34380</v>
       </c>
     </row>
     <row r="69">
@@ -16203,13 +16203,13 @@
         </is>
       </c>
       <c r="F69" t="n">
-        <v>20.85</v>
+        <v>21.36</v>
       </c>
       <c r="G69" t="n">
-        <v>7825980923</v>
+        <v>8054439710</v>
       </c>
       <c r="H69" t="n">
-        <v>3739600</v>
+        <v>3324400</v>
       </c>
       <c r="I69" t="n">
         <v>255106712</v>
@@ -16302,7 +16302,7 @@
         <v>380109000.88</v>
       </c>
       <c r="AM69" t="n">
-        <v>465832197.797619</v>
+        <v>479430935.1190476</v>
       </c>
       <c r="AN69" t="n">
         <v>0.8856000000000001</v>
@@ -16343,7 +16343,7 @@
         <v>21.39</v>
       </c>
       <c r="AZ69" t="n">
-        <v>36.45</v>
+        <v>37.34</v>
       </c>
       <c r="BA69" t="n">
         <v>1.24</v>
@@ -16352,19 +16352,19 @@
         <v>69.59</v>
       </c>
       <c r="BC69" t="n">
-        <v>25.67</v>
+        <v>22.67</v>
       </c>
       <c r="BD69" t="n">
-        <v>2.61</v>
+        <v>0.16</v>
       </c>
       <c r="BE69" t="n">
         <v>74.83</v>
       </c>
       <c r="BF69" t="n">
-        <v>-94.06</v>
+        <v>-94.2</v>
       </c>
       <c r="BG69" t="n">
-        <v>233.75</v>
+        <v>225.78</v>
       </c>
       <c r="BH69" t="n">
         <v>20.48</v>
@@ -16373,7 +16373,7 @@
         <v>0</v>
       </c>
       <c r="BJ69" t="n">
-        <v>20.85</v>
+        <v>21.36</v>
       </c>
       <c r="BK69" t="n">
         <v>1.49</v>
@@ -16382,7 +16382,7 @@
         <v>1.49</v>
       </c>
       <c r="BM69" t="n">
-        <v>21.61</v>
+        <v>21.36</v>
       </c>
       <c r="BN69" t="n">
         <v>25.63</v>
@@ -16391,19 +16391,19 @@
         <v>16.73</v>
       </c>
       <c r="BP69" t="n">
-        <v>20.83</v>
+        <v>20.81</v>
       </c>
       <c r="BQ69" t="n">
-        <v>14.02</v>
+        <v>14.37</v>
       </c>
       <c r="BR69" t="n">
-        <v>21.48</v>
+        <v>21.05</v>
       </c>
       <c r="BS69" t="n">
         <v>0</v>
       </c>
       <c r="BT69" t="n">
-        <v>1878750</v>
+        <v>1944550</v>
       </c>
     </row>
     <row r="70">
@@ -16433,13 +16433,13 @@
         </is>
       </c>
       <c r="F70" t="n">
-        <v>17.73</v>
+        <v>17.52</v>
       </c>
       <c r="G70" t="n">
-        <v>8238997812</v>
+        <v>8139044108</v>
       </c>
       <c r="H70" t="n">
-        <v>3314100</v>
+        <v>2811000</v>
       </c>
       <c r="I70" t="n">
         <v>464557268</v>
@@ -16454,7 +16454,7 @@
         <v>0.68</v>
       </c>
       <c r="M70" t="n">
-        <v>0.6502892264296681</v>
+        <v>0.6424000609830807</v>
       </c>
       <c r="N70" t="n">
         <v>0.2</v>
@@ -16532,7 +16532,7 @@
         <v>55746872.16</v>
       </c>
       <c r="AM70" t="n">
-        <v>2719141192.079208</v>
+        <v>2686153170.957096</v>
       </c>
       <c r="AN70" t="n">
         <v>0.1236</v>
@@ -16573,7 +16573,7 @@
         <v>6.9</v>
       </c>
       <c r="AZ70" t="n">
-        <v>2.04</v>
+        <v>2.01</v>
       </c>
       <c r="BA70" t="n">
         <v>0.12</v>
@@ -16582,10 +16582,10 @@
         <v>1.07</v>
       </c>
       <c r="BC70" t="n">
-        <v>-52.35</v>
+        <v>-51.77</v>
       </c>
       <c r="BD70" t="n">
-        <v>-61.09</v>
+        <v>-60.62</v>
       </c>
       <c r="BE70" t="n">
         <v>-88.5</v>
@@ -16594,7 +16594,7 @@
         <v>-99.31999999999999</v>
       </c>
       <c r="BG70" t="n">
-        <v>-93.97</v>
+        <v>-93.90000000000001</v>
       </c>
       <c r="BH70" t="n">
         <v>26.44</v>
@@ -16603,7 +16603,7 @@
         <v>0</v>
       </c>
       <c r="BJ70" t="n">
-        <v>17.73</v>
+        <v>17.52</v>
       </c>
       <c r="BK70" t="n">
         <v>0.12</v>
@@ -16612,7 +16612,7 @@
         <v>0.1</v>
       </c>
       <c r="BM70" t="n">
-        <v>17.81</v>
+        <v>17.79</v>
       </c>
       <c r="BN70" t="n">
         <v>22.15</v>
@@ -16621,19 +16621,19 @@
         <v>13.21</v>
       </c>
       <c r="BP70" t="n">
-        <v>17.55</v>
+        <v>17.5</v>
       </c>
       <c r="BQ70" t="n">
-        <v>177.82</v>
+        <v>175.71</v>
       </c>
       <c r="BR70" t="n">
-        <v>17.8</v>
+        <v>17.61</v>
       </c>
       <c r="BS70" t="n">
         <v>0.67</v>
       </c>
       <c r="BT70" t="n">
-        <v>5387240</v>
+        <v>5101400</v>
       </c>
     </row>
     <row r="71">

</xml_diff>

<commit_message>
📊 Dados atualizados - 2026-09-19 05:21
</commit_message>
<xml_diff>
--- a/data/ativos.xlsx
+++ b/data/ativos.xlsx
@@ -1047,13 +1047,13 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>24.97</v>
+        <v>24.8</v>
       </c>
       <c r="G3" t="n">
-        <v>3340159401</v>
+        <v>3317416537</v>
       </c>
       <c r="H3" t="n">
-        <v>332600</v>
+        <v>0</v>
       </c>
       <c r="I3" t="n">
         <v>129510368</v>
@@ -1068,7 +1068,7 @@
         <v>0.88</v>
       </c>
       <c r="M3" t="n">
-        <v>0.8311060490724889</v>
+        <v>0.8254471179933391</v>
       </c>
       <c r="N3" t="n">
         <v>0.09</v>
@@ -1146,7 +1146,7 @@
         <v>506385538.88</v>
       </c>
       <c r="AM3" t="n">
-        <v>652374883.0078125</v>
+        <v>647932917.3828125</v>
       </c>
       <c r="AN3" t="n">
         <v>2.7</v>
@@ -1187,7 +1187,7 @@
         <v>40.42</v>
       </c>
       <c r="AZ3" t="n">
-        <v>45.7</v>
+        <v>45.38</v>
       </c>
       <c r="BA3" t="n">
         <v>4.87</v>
@@ -1196,25 +1196,25 @@
         <v>21.14</v>
       </c>
       <c r="BC3" t="n">
-        <v>98.23</v>
+        <v>99.59</v>
       </c>
       <c r="BD3" t="n">
-        <v>61.86</v>
+        <v>62.97</v>
       </c>
       <c r="BE3" t="n">
         <v>83</v>
       </c>
       <c r="BF3" t="n">
-        <v>-80.5</v>
+        <v>-80.37</v>
       </c>
       <c r="BG3" t="n">
-        <v>-15.36</v>
+        <v>-14.77</v>
       </c>
       <c r="BH3" t="n">
         <v>27.85</v>
       </c>
       <c r="BI3" t="n">
-        <v>0</v>
+        <v>-0.68</v>
       </c>
       <c r="BJ3" t="n">
         <v>24.97</v>
@@ -1226,7 +1226,7 @@
         <v>4.39</v>
       </c>
       <c r="BM3" t="n">
-        <v>25.04</v>
+        <v>24.95</v>
       </c>
       <c r="BN3" t="n">
         <v>27.17</v>
@@ -1235,19 +1235,19 @@
         <v>18.72</v>
       </c>
       <c r="BP3" t="n">
-        <v>24.51</v>
+        <v>24.7</v>
       </c>
       <c r="BQ3" t="n">
-        <v>5.68</v>
+        <v>5.65</v>
       </c>
       <c r="BR3" t="n">
-        <v>24.78</v>
+        <v>24.95</v>
       </c>
       <c r="BS3" t="n">
         <v>0.79</v>
       </c>
       <c r="BT3" t="n">
-        <v>520900</v>
+        <v>514897</v>
       </c>
     </row>
     <row r="4">
@@ -1277,13 +1277,13 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>15.55</v>
+        <v>15.38</v>
       </c>
       <c r="G4" t="n">
-        <v>240786465953</v>
+        <v>238154072572</v>
       </c>
       <c r="H4" t="n">
-        <v>18516700</v>
+        <v>0</v>
       </c>
       <c r="I4" t="n">
         <v>15484664889</v>
@@ -1298,7 +1298,7 @@
         <v>2.76</v>
       </c>
       <c r="M4" t="n">
-        <v>2.726432505948736</v>
+        <v>2.69662583532048</v>
       </c>
       <c r="N4" t="n">
         <v>1.76</v>
@@ -1376,7 +1376,7 @@
         <v>16258898133.45</v>
       </c>
       <c r="AM4" t="n">
-        <v>23840244153.76238</v>
+        <v>23579611145.74258</v>
       </c>
       <c r="AN4" t="n">
         <v>0.269</v>
@@ -1417,7 +1417,7 @@
         <v>9.470000000000001</v>
       </c>
       <c r="AZ4" t="n">
-        <v>19.41</v>
+        <v>19.2</v>
       </c>
       <c r="BA4" t="n">
         <v>1.13</v>
@@ -1426,19 +1426,19 @@
         <v>11.39</v>
       </c>
       <c r="BC4" t="n">
-        <v>-25.37</v>
+        <v>-24.55</v>
       </c>
       <c r="BD4" t="n">
-        <v>-39.07</v>
+        <v>-38.39</v>
       </c>
       <c r="BE4" t="n">
         <v>24.83</v>
       </c>
       <c r="BF4" t="n">
-        <v>-92.75</v>
+        <v>-92.67</v>
       </c>
       <c r="BG4" t="n">
-        <v>-26.77</v>
+        <v>-25.96</v>
       </c>
       <c r="BH4" t="n">
         <v>5.7</v>
@@ -1447,7 +1447,7 @@
         <v>0</v>
       </c>
       <c r="BJ4" t="n">
-        <v>15.55</v>
+        <v>15.38</v>
       </c>
       <c r="BK4" t="n">
         <v>1.05</v>
@@ -1456,7 +1456,7 @@
         <v>1.04</v>
       </c>
       <c r="BM4" t="n">
-        <v>15.73</v>
+        <v>15.53</v>
       </c>
       <c r="BN4" t="n">
         <v>17</v>
@@ -1465,19 +1465,19 @@
         <v>11.09</v>
       </c>
       <c r="BP4" t="n">
-        <v>15.44</v>
+        <v>15.29</v>
       </c>
       <c r="BQ4" t="n">
-        <v>15</v>
+        <v>14.83</v>
       </c>
       <c r="BR4" t="n">
-        <v>15.63</v>
+        <v>15.47</v>
       </c>
       <c r="BS4" t="n">
         <v>2.76</v>
       </c>
       <c r="BT4" t="n">
-        <v>28327710</v>
+        <v>27757920</v>
       </c>
     </row>
     <row r="5">
@@ -3117,13 +3117,13 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>5.06</v>
+        <v>5.05</v>
       </c>
       <c r="G12" t="n">
-        <v>485565336</v>
+        <v>484605795</v>
       </c>
       <c r="H12" t="n">
-        <v>351900</v>
+        <v>370400</v>
       </c>
       <c r="I12" t="n">
         <v>95961536</v>
@@ -3138,7 +3138,7 @@
         <v>0.32</v>
       </c>
       <c r="M12" t="n">
-        <v>0.08781375007427578</v>
+        <v>0.08764021854862333</v>
       </c>
       <c r="N12" t="n">
         <v>0.14</v>
@@ -3216,7 +3216,7 @@
         <v>362734606.08</v>
       </c>
       <c r="AM12" t="n">
-        <v>522113264.516129</v>
+        <v>521081500</v>
       </c>
       <c r="AN12" t="n">
         <v>0.4208</v>
@@ -3257,7 +3257,7 @@
         <v>30.49</v>
       </c>
       <c r="AZ12" t="n">
-        <v>6.84</v>
+        <v>6.83</v>
       </c>
       <c r="BA12" t="n">
         <v>4.41</v>
@@ -3266,19 +3266,19 @@
         <v>18.12</v>
       </c>
       <c r="BC12" t="n">
-        <v>638.09</v>
+        <v>639.55</v>
       </c>
       <c r="BD12" t="n">
-        <v>502.65</v>
+        <v>503.84</v>
       </c>
       <c r="BE12" t="n">
         <v>35.17</v>
       </c>
       <c r="BF12" t="n">
-        <v>-12.81</v>
+        <v>-12.64</v>
       </c>
       <c r="BG12" t="n">
-        <v>258.08</v>
+        <v>258.79</v>
       </c>
       <c r="BH12" t="n">
         <v>16.4</v>
@@ -3287,7 +3287,7 @@
         <v>0</v>
       </c>
       <c r="BJ12" t="n">
-        <v>5.06</v>
+        <v>5.05</v>
       </c>
       <c r="BK12" t="n">
         <v>3.78</v>
@@ -3296,7 +3296,7 @@
         <v>3.43</v>
       </c>
       <c r="BM12" t="n">
-        <v>5.15</v>
+        <v>5.07</v>
       </c>
       <c r="BN12" t="n">
         <v>8.23</v>
@@ -3305,19 +3305,19 @@
         <v>4.42</v>
       </c>
       <c r="BP12" t="n">
-        <v>5.04</v>
+        <v>4.96</v>
       </c>
       <c r="BQ12" t="n">
         <v>1.47</v>
       </c>
       <c r="BR12" t="n">
-        <v>5.15</v>
+        <v>5.07</v>
       </c>
       <c r="BS12" t="n">
         <v>0.09</v>
       </c>
       <c r="BT12" t="n">
-        <v>505573</v>
+        <v>509497</v>
       </c>
     </row>
     <row r="13">
@@ -3347,13 +3347,13 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>28.29</v>
+        <v>28.87</v>
       </c>
       <c r="G13" t="n">
-        <v>14263555364</v>
+        <v>14555988819</v>
       </c>
       <c r="H13" t="n">
-        <v>5922600</v>
+        <v>0</v>
       </c>
       <c r="I13" t="n">
         <v>504190947</v>
@@ -3368,7 +3368,7 @@
         <v>1.13</v>
       </c>
       <c r="M13" t="n">
-        <v>4.933162067038345</v>
+        <v>5.034302462299124</v>
       </c>
       <c r="N13" t="n">
         <v>0.57</v>
@@ -3446,7 +3446,7 @@
         <v>932753251.95</v>
       </c>
       <c r="AM13" t="n">
-        <v>1484240932.778356</v>
+        <v>1514671052.965661</v>
       </c>
       <c r="AN13" t="n">
         <v>2.6301</v>
@@ -3487,7 +3487,7 @@
         <v>26.6</v>
       </c>
       <c r="AZ13" t="n">
-        <v>51.2</v>
+        <v>52.25</v>
       </c>
       <c r="BA13" t="n">
         <v>2.6</v>
@@ -3496,19 +3496,19 @@
         <v>8.69</v>
       </c>
       <c r="BC13" t="n">
-        <v>15.14</v>
+        <v>12.83</v>
       </c>
       <c r="BD13" t="n">
-        <v>-5.99</v>
+        <v>-7.88</v>
       </c>
       <c r="BE13" t="n">
         <v>81</v>
       </c>
       <c r="BF13" t="n">
-        <v>-90.79000000000001</v>
+        <v>-90.98</v>
       </c>
       <c r="BG13" t="n">
-        <v>-69.27</v>
+        <v>-69.89</v>
       </c>
       <c r="BH13" t="n">
         <v>25.49</v>
@@ -3517,7 +3517,7 @@
         <v>0</v>
       </c>
       <c r="BJ13" t="n">
-        <v>28.29</v>
+        <v>28.87</v>
       </c>
       <c r="BK13" t="n">
         <v>1.85</v>
@@ -3526,7 +3526,7 @@
         <v>1.96</v>
       </c>
       <c r="BM13" t="n">
-        <v>28.76</v>
+        <v>28.87</v>
       </c>
       <c r="BN13" t="n">
         <v>32.43</v>
@@ -3535,19 +3535,19 @@
         <v>21.06</v>
       </c>
       <c r="BP13" t="n">
-        <v>27.82</v>
+        <v>28.05</v>
       </c>
       <c r="BQ13" t="n">
-        <v>14.45</v>
+        <v>14.75</v>
       </c>
       <c r="BR13" t="n">
-        <v>28.76</v>
+        <v>28.15</v>
       </c>
       <c r="BS13" t="n">
         <v>5.01</v>
       </c>
       <c r="BT13" t="n">
-        <v>4708622</v>
+        <v>4784913</v>
       </c>
     </row>
     <row r="14">
@@ -3577,13 +3577,13 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>9.619999999999999</v>
+        <v>9.539999999999999</v>
       </c>
       <c r="G14" t="n">
-        <v>7556726851</v>
+        <v>7732824181</v>
       </c>
       <c r="H14" t="n">
-        <v>8000</v>
+        <v>14800</v>
       </c>
       <c r="I14" t="n">
         <v>339510689</v>
@@ -3598,7 +3598,7 @@
         <v>1.92</v>
       </c>
       <c r="M14" t="n">
-        <v>3.137687329634206</v>
+        <v>3.210806071652822</v>
       </c>
       <c r="N14" t="n">
         <v>1.11</v>
@@ -3676,7 +3676,7 @@
         <v>349696009.67</v>
       </c>
       <c r="AM14" t="n">
-        <v>838704422.9744729</v>
+        <v>858249076.6925639</v>
       </c>
       <c r="AN14" t="n">
         <v>0.1489</v>
@@ -3717,7 +3717,7 @@
         <v>9.050000000000001</v>
       </c>
       <c r="AZ14" t="n">
-        <v>7.73</v>
+        <v>7.66</v>
       </c>
       <c r="BA14" t="n">
         <v>1.42</v>
@@ -3726,19 +3726,19 @@
         <v>5.94</v>
       </c>
       <c r="BC14" t="n">
-        <v>15.21</v>
+        <v>16.17</v>
       </c>
       <c r="BD14" t="n">
-        <v>-5.94</v>
+        <v>-5.15</v>
       </c>
       <c r="BE14" t="n">
         <v>-19.67</v>
       </c>
       <c r="BF14" t="n">
-        <v>-85.23</v>
+        <v>-85.09999999999999</v>
       </c>
       <c r="BG14" t="n">
-        <v>-38.23</v>
+        <v>-37.71</v>
       </c>
       <c r="BH14" t="n">
         <v>5.3</v>
@@ -3747,7 +3747,7 @@
         <v>0</v>
       </c>
       <c r="BJ14" t="n">
-        <v>9.619999999999999</v>
+        <v>9.539999999999999</v>
       </c>
       <c r="BK14" t="n">
         <v>1.03</v>
@@ -3756,7 +3756,7 @@
         <v>1.01</v>
       </c>
       <c r="BM14" t="n">
-        <v>9.99</v>
+        <v>9.75</v>
       </c>
       <c r="BN14" t="n">
         <v>13.49</v>
@@ -3765,19 +3765,19 @@
         <v>7.65</v>
       </c>
       <c r="BP14" t="n">
-        <v>9.619999999999999</v>
+        <v>9.539999999999999</v>
       </c>
       <c r="BQ14" t="n">
-        <v>9.5</v>
+        <v>9.42</v>
       </c>
       <c r="BR14" t="n">
-        <v>9.699999999999999</v>
+        <v>9.640000000000001</v>
       </c>
       <c r="BS14" t="n">
         <v>1.44</v>
       </c>
       <c r="BT14" t="n">
-        <v>12437</v>
+        <v>12083</v>
       </c>
     </row>
     <row r="15">
@@ -3807,13 +3807,13 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>12.81</v>
+        <v>12.92</v>
       </c>
       <c r="G15" t="n">
-        <v>7556726851</v>
+        <v>7732824181</v>
       </c>
       <c r="H15" t="n">
-        <v>3949400</v>
+        <v>0</v>
       </c>
       <c r="I15" t="n">
         <v>343551533</v>
@@ -3828,7 +3828,7 @@
         <v>2.56</v>
       </c>
       <c r="M15" t="n">
-        <v>3.100781934658634</v>
+        <v>3.173040655977026</v>
       </c>
       <c r="N15" t="n">
         <v>1.47</v>
@@ -3906,7 +3906,7 @@
         <v>353858078.99</v>
       </c>
       <c r="AM15" t="n">
-        <v>630252447.9566305</v>
+        <v>644939464.6371976</v>
       </c>
       <c r="AN15" t="n">
         <v>0.1638</v>
@@ -3947,7 +3947,7 @@
         <v>9.050000000000001</v>
       </c>
       <c r="AZ15" t="n">
-        <v>8.52</v>
+        <v>8.59</v>
       </c>
       <c r="BA15" t="n">
         <v>1.42</v>
@@ -3956,19 +3956,19 @@
         <v>6.19</v>
       </c>
       <c r="BC15" t="n">
-        <v>-13.48</v>
+        <v>-14.22</v>
       </c>
       <c r="BD15" t="n">
-        <v>-29.36</v>
+        <v>-29.96</v>
       </c>
       <c r="BE15" t="n">
         <v>-33.5</v>
       </c>
       <c r="BF15" t="n">
-        <v>-88.91</v>
+        <v>-89</v>
       </c>
       <c r="BG15" t="n">
-        <v>-51.69</v>
+        <v>-52.1</v>
       </c>
       <c r="BH15" t="n">
         <v>5.3</v>
@@ -3977,7 +3977,7 @@
         <v>0</v>
       </c>
       <c r="BJ15" t="n">
-        <v>12.81</v>
+        <v>12.92</v>
       </c>
       <c r="BK15" t="n">
         <v>1.03</v>
@@ -3986,7 +3986,7 @@
         <v>1.01</v>
       </c>
       <c r="BM15" t="n">
-        <v>13.52</v>
+        <v>13.17</v>
       </c>
       <c r="BN15" t="n">
         <v>16.22</v>
@@ -3995,19 +3995,19 @@
         <v>7.84</v>
       </c>
       <c r="BP15" t="n">
-        <v>12.81</v>
+        <v>12.68</v>
       </c>
       <c r="BQ15" t="n">
-        <v>12.65</v>
+        <v>12.76</v>
       </c>
       <c r="BR15" t="n">
-        <v>13.38</v>
+        <v>12.76</v>
       </c>
       <c r="BS15" t="n">
         <v>1.92</v>
       </c>
       <c r="BT15" t="n">
-        <v>2389933</v>
+        <v>2482773</v>
       </c>
     </row>
     <row r="16">
@@ -4043,7 +4043,7 @@
         <v>953979774</v>
       </c>
       <c r="H16" t="n">
-        <v>62200</v>
+        <v>113400</v>
       </c>
       <c r="I16" t="n">
         <v>219305733</v>
@@ -4216,28 +4216,28 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="BM16" t="n">
-        <v>4.38</v>
+        <v>4.39</v>
       </c>
       <c r="BN16" t="n">
         <v>5.54</v>
       </c>
       <c r="BO16" t="n">
-        <v>3.13</v>
+        <v>3.14</v>
       </c>
       <c r="BP16" t="n">
-        <v>4.2</v>
+        <v>4.23</v>
       </c>
       <c r="BQ16" t="n">
         <v>59.36</v>
       </c>
       <c r="BR16" t="n">
-        <v>4.2</v>
+        <v>4.35</v>
       </c>
       <c r="BS16" t="n">
         <v>0.49</v>
       </c>
       <c r="BT16" t="n">
-        <v>145310</v>
+        <v>144607</v>
       </c>
     </row>
     <row r="17">
@@ -4267,13 +4267,13 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>33.4</v>
+        <v>32.7</v>
       </c>
       <c r="G17" t="n">
-        <v>11009538962</v>
+        <v>10778799881</v>
       </c>
       <c r="H17" t="n">
-        <v>646500</v>
+        <v>0</v>
       </c>
       <c r="I17" t="n">
         <v>0</v>
@@ -4360,13 +4360,13 @@
         <v>8.039999999999999</v>
       </c>
       <c r="AK17" t="n">
-        <v>4971793245.122832</v>
+        <v>4867593876.896676</v>
       </c>
       <c r="AL17" t="n">
-        <v>1376192370.25</v>
+        <v>1347349985.125</v>
       </c>
       <c r="AM17" t="n">
-        <v>3408525994.427245</v>
+        <v>3337089746.439629</v>
       </c>
       <c r="AN17" t="n">
         <v>1.08</v>
@@ -4407,7 +4407,7 @@
         <v>42.98</v>
       </c>
       <c r="AZ17" t="n">
-        <v>17.87</v>
+        <v>17.49</v>
       </c>
       <c r="BA17" t="n">
         <v>4.55</v>
@@ -4416,19 +4416,19 @@
         <v>16.33</v>
       </c>
       <c r="BC17" t="n">
-        <v>57.6</v>
+        <v>60.97</v>
       </c>
       <c r="BD17" t="n">
-        <v>28.68</v>
+        <v>31.43</v>
       </c>
       <c r="BE17" t="n">
         <v>-46.5</v>
       </c>
       <c r="BF17" t="n">
-        <v>-86.38</v>
+        <v>-86.09</v>
       </c>
       <c r="BG17" t="n">
-        <v>-51.1</v>
+        <v>-50.05</v>
       </c>
       <c r="BH17" t="n">
         <v>29.25</v>
@@ -4437,7 +4437,7 @@
         <v>0</v>
       </c>
       <c r="BJ17" t="n">
-        <v>33.4</v>
+        <v>32.7</v>
       </c>
       <c r="BK17" t="n">
         <v>4.21</v>
@@ -4446,28 +4446,28 @@
         <v>12.62</v>
       </c>
       <c r="BM17" t="n">
-        <v>33.48</v>
+        <v>33.41</v>
       </c>
       <c r="BN17" t="n">
         <v>36.63</v>
       </c>
       <c r="BO17" t="n">
-        <v>29.28</v>
+        <v>29.52</v>
       </c>
       <c r="BP17" t="n">
-        <v>32.82</v>
+        <v>32.7</v>
       </c>
       <c r="BQ17" t="n">
-        <v>2.65</v>
+        <v>2.59</v>
       </c>
       <c r="BR17" t="n">
-        <v>33</v>
+        <v>33.25</v>
       </c>
       <c r="BS17" t="n">
         <v>2.21</v>
       </c>
       <c r="BT17" t="n">
-        <v>1084652</v>
+        <v>1069405</v>
       </c>
     </row>
     <row r="18">
@@ -4497,13 +4497,13 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>11.3</v>
+        <v>11.37</v>
       </c>
       <c r="G18" t="n">
-        <v>11009538962</v>
+        <v>10778799881</v>
       </c>
       <c r="H18" t="n">
-        <v>5500</v>
+        <v>0</v>
       </c>
       <c r="I18" t="n">
         <v>671494278</v>
@@ -4518,7 +4518,7 @@
         <v>1.2</v>
       </c>
       <c r="M18" t="n">
-        <v>3.241640626333719</v>
+        <v>3.173701979526239</v>
       </c>
       <c r="N18" t="n">
         <v>0.33</v>
@@ -4596,7 +4596,7 @@
         <v>940091989.1999999</v>
       </c>
       <c r="AM18" t="n">
-        <v>3276648500.595238</v>
+        <v>3207976155.059524</v>
       </c>
       <c r="AN18" t="n">
         <v>0.36</v>
@@ -4637,7 +4637,7 @@
         <v>14.31</v>
       </c>
       <c r="AZ18" t="n">
-        <v>5.82</v>
+        <v>5.86</v>
       </c>
       <c r="BA18" t="n">
         <v>1.51</v>
@@ -4646,25 +4646,25 @@
         <v>5.44</v>
       </c>
       <c r="BC18" t="n">
-        <v>55.09</v>
+        <v>54.13</v>
       </c>
       <c r="BD18" t="n">
-        <v>26.63</v>
+        <v>25.85</v>
       </c>
       <c r="BE18" t="n">
         <v>-48.5</v>
       </c>
       <c r="BF18" t="n">
-        <v>-86.61</v>
+        <v>-86.7</v>
       </c>
       <c r="BG18" t="n">
-        <v>-51.82</v>
+        <v>-52.12</v>
       </c>
       <c r="BH18" t="n">
         <v>9.75</v>
       </c>
       <c r="BI18" t="n">
-        <v>0</v>
+        <v>0.62</v>
       </c>
       <c r="BJ18" t="n">
         <v>11.3</v>
@@ -4676,7 +4676,7 @@
         <v>12.62</v>
       </c>
       <c r="BM18" t="n">
-        <v>11.44</v>
+        <v>11.37</v>
       </c>
       <c r="BN18" t="n">
         <v>13.82</v>
@@ -4685,19 +4685,19 @@
         <v>10.19</v>
       </c>
       <c r="BP18" t="n">
-        <v>11.25</v>
+        <v>11.3</v>
       </c>
       <c r="BQ18" t="n">
         <v>0.9</v>
       </c>
       <c r="BR18" t="n">
-        <v>11.28</v>
+        <v>11.3</v>
       </c>
       <c r="BS18" t="n">
         <v>2.3</v>
       </c>
       <c r="BT18" t="n">
-        <v>9951</v>
+        <v>10071</v>
       </c>
     </row>
     <row r="19">
@@ -4727,13 +4727,13 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>10.91</v>
+        <v>10.9</v>
       </c>
       <c r="G19" t="n">
-        <v>11009538962</v>
+        <v>10778799881</v>
       </c>
       <c r="H19" t="n">
-        <v>4600</v>
+        <v>6600</v>
       </c>
       <c r="I19" t="n">
         <v>317386323</v>
@@ -4748,7 +4748,7 @@
         <v>1.12</v>
       </c>
       <c r="M19" t="n">
-        <v>6.858339424775492</v>
+        <v>6.714601622355173</v>
       </c>
       <c r="N19" t="n">
         <v>0.3</v>
@@ -4826,7 +4826,7 @@
         <v>444340852.2</v>
       </c>
       <c r="AM19" t="n">
-        <v>3495091733.968254</v>
+        <v>3421841232.063492</v>
       </c>
       <c r="AN19" t="n">
         <v>0.36</v>
@@ -4876,19 +4876,19 @@
         <v>5.25</v>
       </c>
       <c r="BC19" t="n">
-        <v>60.63</v>
+        <v>60.78</v>
       </c>
       <c r="BD19" t="n">
-        <v>31.16</v>
+        <v>31.28</v>
       </c>
       <c r="BE19" t="n">
         <v>-45</v>
       </c>
       <c r="BF19" t="n">
-        <v>-86.14</v>
+        <v>-86.12</v>
       </c>
       <c r="BG19" t="n">
-        <v>-51.88</v>
+        <v>-51.83</v>
       </c>
       <c r="BH19" t="n">
         <v>9.75</v>
@@ -4897,7 +4897,7 @@
         <v>0</v>
       </c>
       <c r="BJ19" t="n">
-        <v>10.91</v>
+        <v>10.9</v>
       </c>
       <c r="BK19" t="n">
         <v>1.4</v>
@@ -4915,19 +4915,19 @@
         <v>9.19</v>
       </c>
       <c r="BP19" t="n">
-        <v>10.8</v>
+        <v>10.84</v>
       </c>
       <c r="BQ19" t="n">
         <v>0.86</v>
       </c>
       <c r="BR19" t="n">
-        <v>10.88</v>
+        <v>10.91</v>
       </c>
       <c r="BS19" t="n">
         <v>2.16</v>
       </c>
       <c r="BT19" t="n">
-        <v>13684</v>
+        <v>13511</v>
       </c>
     </row>
     <row r="20">
@@ -5417,13 +5417,13 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>4.94</v>
+        <v>4.74</v>
       </c>
       <c r="G22" t="n">
-        <v>989211793</v>
+        <v>949162676</v>
       </c>
       <c r="H22" t="n">
-        <v>1005200</v>
+        <v>0</v>
       </c>
       <c r="I22" t="n">
         <v>200245299</v>
@@ -5438,7 +5438,7 @@
         <v>0.27</v>
       </c>
       <c r="M22" t="n">
-        <v>0.08390158865356404</v>
+        <v>0.08050475840522867</v>
       </c>
       <c r="N22" t="n">
         <v>0.08</v>
@@ -5516,7 +5516,7 @@
         <v>378463615.11</v>
       </c>
       <c r="AM22" t="n">
-        <v>224311064.1723356</v>
+        <v>215229631.7460317</v>
       </c>
       <c r="AN22" t="n">
         <v>0</v>
@@ -5566,19 +5566,19 @@
         <v>172.49</v>
       </c>
       <c r="BC22" t="n">
-        <v>501.32</v>
+        <v>526.6900000000001</v>
       </c>
       <c r="BD22" t="n">
-        <v>390.97</v>
+        <v>411.69</v>
       </c>
       <c r="BE22" t="n">
         <v>-100</v>
       </c>
       <c r="BF22" t="n">
-        <v>-61.74</v>
+        <v>-60.13</v>
       </c>
       <c r="BG22" t="n">
-        <v>3391.69</v>
+        <v>3539.02</v>
       </c>
       <c r="BH22" t="n">
         <v>20.75</v>
@@ -5587,7 +5587,7 @@
         <v>0</v>
       </c>
       <c r="BJ22" t="n">
-        <v>4.94</v>
+        <v>4.74</v>
       </c>
       <c r="BK22" t="n">
         <v>1.89</v>
@@ -5596,28 +5596,28 @@
         <v>0.67</v>
       </c>
       <c r="BM22" t="n">
-        <v>5.08</v>
+        <v>4.95</v>
       </c>
       <c r="BN22" t="n">
-        <v>8.82</v>
+        <v>8.279999999999999</v>
       </c>
       <c r="BO22" t="n">
         <v>3.37</v>
       </c>
       <c r="BP22" t="n">
-        <v>4.85</v>
+        <v>4.66</v>
       </c>
       <c r="BQ22" t="n">
-        <v>7.36</v>
+        <v>7.06</v>
       </c>
       <c r="BR22" t="n">
-        <v>5.05</v>
+        <v>4.94</v>
       </c>
       <c r="BS22" t="n">
         <v>0.09</v>
       </c>
       <c r="BT22" t="n">
-        <v>1563307</v>
+        <v>1561730</v>
       </c>
     </row>
     <row r="23">
@@ -5877,13 +5877,13 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.86</v>
+        <v>2.87</v>
       </c>
       <c r="G24" t="n">
-        <v>1155065011</v>
+        <v>1159103409</v>
       </c>
       <c r="H24" t="n">
-        <v>4726300</v>
+        <v>0</v>
       </c>
       <c r="I24" t="n">
         <v>403868805</v>
@@ -5898,7 +5898,7 @@
         <v>0.49</v>
       </c>
       <c r="M24" t="n">
-        <v>0.2792263710756008</v>
+        <v>0.2802026167481476</v>
       </c>
       <c r="N24" t="n">
         <v>0.11</v>
@@ -5976,7 +5976,7 @@
         <v>153470145.9</v>
       </c>
       <c r="AM24" t="n">
-        <v>1040599109.009009</v>
+        <v>1044237305.405405</v>
       </c>
       <c r="AN24" t="n">
         <v>0.0813</v>
@@ -6026,19 +6026,19 @@
         <v>1.46</v>
       </c>
       <c r="BC24" t="n">
-        <v>150.22</v>
+        <v>149.35</v>
       </c>
       <c r="BD24" t="n">
-        <v>104.31</v>
+        <v>103.6</v>
       </c>
       <c r="BE24" t="n">
         <v>-53.83</v>
       </c>
       <c r="BF24" t="n">
-        <v>-86.70999999999999</v>
+        <v>-86.76000000000001</v>
       </c>
       <c r="BG24" t="n">
-        <v>-49.03</v>
+        <v>-49.21</v>
       </c>
       <c r="BH24" t="n">
         <v>5.99</v>
@@ -6047,7 +6047,7 @@
         <v>0</v>
       </c>
       <c r="BJ24" t="n">
-        <v>2.86</v>
+        <v>2.87</v>
       </c>
       <c r="BK24" t="n">
         <v>0.38</v>
@@ -6056,7 +6056,7 @@
         <v>0.41</v>
       </c>
       <c r="BM24" t="n">
-        <v>2.98</v>
+        <v>2.91</v>
       </c>
       <c r="BN24" t="n">
         <v>5.29</v>
@@ -6065,19 +6065,19 @@
         <v>1.92</v>
       </c>
       <c r="BP24" t="n">
-        <v>2.83</v>
+        <v>2.75</v>
       </c>
       <c r="BQ24" t="n">
-        <v>7.02</v>
+        <v>7.05</v>
       </c>
       <c r="BR24" t="n">
-        <v>2.93</v>
+        <v>2.86</v>
       </c>
       <c r="BS24" t="n">
         <v>0.29</v>
       </c>
       <c r="BT24" t="n">
-        <v>8653000</v>
+        <v>8506603</v>
       </c>
     </row>
     <row r="25">
@@ -6107,13 +6107,13 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>3.97</v>
+        <v>4.07</v>
       </c>
       <c r="G25" t="n">
-        <v>1375581189</v>
+        <v>1410231453</v>
       </c>
       <c r="H25" t="n">
-        <v>1312100</v>
+        <v>0</v>
       </c>
       <c r="I25" t="n">
         <v>346494097</v>
@@ -6128,7 +6128,7 @@
         <v>0.97</v>
       </c>
       <c r="M25" t="n">
-        <v>0.6859275902421313</v>
+        <v>0.7032057940128967</v>
       </c>
       <c r="N25" t="n">
         <v>0.22</v>
@@ -6206,7 +6206,7 @@
         <v>62368937.46</v>
       </c>
       <c r="AM25" t="n">
-        <v>505728378.3088235</v>
+        <v>518467445.9558823</v>
       </c>
       <c r="AN25" t="n">
         <v>0.4742</v>
@@ -6247,7 +6247,7 @@
         <v>3.27</v>
       </c>
       <c r="AZ25" t="n">
-        <v>9.25</v>
+        <v>9.48</v>
       </c>
       <c r="BA25" t="n">
         <v>0.23</v>
@@ -6256,25 +6256,25 @@
         <v>2.2</v>
       </c>
       <c r="BC25" t="n">
-        <v>1</v>
+        <v>-1.48</v>
       </c>
       <c r="BD25" t="n">
-        <v>-17.53</v>
+        <v>-19.56</v>
       </c>
       <c r="BE25" t="n">
         <v>133</v>
       </c>
       <c r="BF25" t="n">
-        <v>-94.16</v>
+        <v>-94.31</v>
       </c>
       <c r="BG25" t="n">
-        <v>-44.59</v>
+        <v>-45.95</v>
       </c>
       <c r="BH25" t="n">
         <v>3.97</v>
       </c>
       <c r="BI25" t="n">
-        <v>0</v>
+        <v>2.52</v>
       </c>
       <c r="BJ25" t="n">
         <v>3.97</v>
@@ -6286,7 +6286,7 @@
         <v>0.24</v>
       </c>
       <c r="BM25" t="n">
-        <v>4.06</v>
+        <v>4.1</v>
       </c>
       <c r="BN25" t="n">
         <v>6.3</v>
@@ -6298,16 +6298,16 @@
         <v>3.85</v>
       </c>
       <c r="BQ25" t="n">
-        <v>16.78</v>
+        <v>17.2</v>
       </c>
       <c r="BR25" t="n">
-        <v>3.91</v>
+        <v>3.97</v>
       </c>
       <c r="BS25" t="n">
         <v>0.67</v>
       </c>
       <c r="BT25" t="n">
-        <v>1228043</v>
+        <v>1255643</v>
       </c>
     </row>
     <row r="26">
@@ -6337,13 +6337,13 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>10.21</v>
+        <v>10.26</v>
       </c>
       <c r="G26" t="n">
-        <v>13828352581</v>
+        <v>13896072489</v>
       </c>
       <c r="H26" t="n">
-        <v>9755800</v>
+        <v>0</v>
       </c>
       <c r="I26" t="n">
         <v>1354393401</v>
@@ -6358,7 +6358,7 @@
         <v>1.94</v>
       </c>
       <c r="M26" t="n">
-        <v>0.1783154408208944</v>
+        <v>0.1791886833258593</v>
       </c>
       <c r="N26" t="n">
         <v>0.26</v>
@@ -6436,7 +6436,7 @@
         <v>961619314.7099999</v>
       </c>
       <c r="AM26" t="n">
-        <v>4938697350.357143</v>
+        <v>4962883031.785714</v>
       </c>
       <c r="AN26" t="n">
         <v>0.1043</v>
@@ -6477,7 +6477,7 @@
         <v>7.07</v>
       </c>
       <c r="AZ26" t="n">
-        <v>1.96</v>
+        <v>1.97</v>
       </c>
       <c r="BA26" t="n">
         <v>0.66</v>
@@ -6486,19 +6486,19 @@
         <v>1.19</v>
       </c>
       <c r="BC26" t="n">
-        <v>-15.22</v>
+        <v>-15.64</v>
       </c>
       <c r="BD26" t="n">
-        <v>-30.78</v>
+        <v>-31.12</v>
       </c>
       <c r="BE26" t="n">
         <v>-80.83</v>
       </c>
       <c r="BF26" t="n">
-        <v>-93.54000000000001</v>
+        <v>-93.56999999999999</v>
       </c>
       <c r="BG26" t="n">
-        <v>-88.31</v>
+        <v>-88.37</v>
       </c>
       <c r="BH26" t="n">
         <v>4.69</v>
@@ -6507,7 +6507,7 @@
         <v>0</v>
       </c>
       <c r="BJ26" t="n">
-        <v>10.21</v>
+        <v>10.26</v>
       </c>
       <c r="BK26" t="n">
         <v>0.71</v>
@@ -6516,28 +6516,28 @@
         <v>0.72</v>
       </c>
       <c r="BM26" t="n">
-        <v>10.28</v>
+        <v>10.3</v>
       </c>
       <c r="BN26" t="n">
-        <v>10.41</v>
+        <v>10.35</v>
       </c>
       <c r="BO26" t="n">
         <v>6.91</v>
       </c>
       <c r="BP26" t="n">
-        <v>9.880000000000001</v>
+        <v>10.04</v>
       </c>
       <c r="BQ26" t="n">
-        <v>14.24</v>
+        <v>14.31</v>
       </c>
       <c r="BR26" t="n">
-        <v>10.14</v>
+        <v>10.1</v>
       </c>
       <c r="BS26" t="n">
         <v>0.16</v>
       </c>
       <c r="BT26" t="n">
-        <v>12155697</v>
+        <v>12192447</v>
       </c>
     </row>
     <row r="27">
@@ -8165,13 +8165,13 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>14.81</v>
+        <v>14.3</v>
       </c>
       <c r="G34" t="n">
-        <v>3058114024</v>
+        <v>2952804179</v>
       </c>
       <c r="H34" t="n">
-        <v>2608300</v>
+        <v>0</v>
       </c>
       <c r="I34" t="n">
         <v>206489813</v>
@@ -8186,7 +8186,7 @@
         <v>0.45</v>
       </c>
       <c r="M34" t="n">
-        <v>0.2688439396793548</v>
+        <v>0.2595859743469208</v>
       </c>
       <c r="N34" t="n">
         <v>0.24</v>
@@ -8264,7 +8264,7 @@
         <v>324189006.41</v>
       </c>
       <c r="AM34" t="n">
-        <v>635782541.3721415</v>
+        <v>613888602.7027028</v>
       </c>
       <c r="AN34" t="n">
         <v>0</v>
@@ -8305,7 +8305,7 @@
         <v>30.28</v>
       </c>
       <c r="AZ34" t="n">
-        <v>34.56</v>
+        <v>33.37</v>
       </c>
       <c r="BA34" t="n">
         <v>2.29</v>
@@ -8314,19 +8314,19 @@
         <v>25.26</v>
       </c>
       <c r="BC34" t="n">
-        <v>150.43</v>
+        <v>159.36</v>
       </c>
       <c r="BD34" t="n">
-        <v>104.47</v>
+        <v>111.77</v>
       </c>
       <c r="BE34" t="n">
         <v>133.33</v>
       </c>
       <c r="BF34" t="n">
-        <v>-84.5</v>
+        <v>-83.95</v>
       </c>
       <c r="BG34" t="n">
-        <v>70.55</v>
+        <v>76.63</v>
       </c>
       <c r="BH34" t="n">
         <v>38.94</v>
@@ -8335,7 +8335,7 @@
         <v>0</v>
       </c>
       <c r="BJ34" t="n">
-        <v>14.81</v>
+        <v>14.3</v>
       </c>
       <c r="BK34" t="n">
         <v>1.57</v>
@@ -8344,28 +8344,28 @@
         <v>1.58</v>
       </c>
       <c r="BM34" t="n">
-        <v>15.2</v>
+        <v>14.81</v>
       </c>
       <c r="BN34" t="n">
-        <v>30.87</v>
+        <v>29.87</v>
       </c>
       <c r="BO34" t="n">
-        <v>14.32</v>
+        <v>14.3</v>
       </c>
       <c r="BP34" t="n">
-        <v>14.68</v>
+        <v>14.3</v>
       </c>
       <c r="BQ34" t="n">
-        <v>9.390000000000001</v>
+        <v>9.07</v>
       </c>
       <c r="BR34" t="n">
-        <v>15.2</v>
+        <v>14.74</v>
       </c>
       <c r="BS34" t="n">
         <v>0.32</v>
       </c>
       <c r="BT34" t="n">
-        <v>3121040</v>
+        <v>3111263</v>
       </c>
     </row>
     <row r="35">
@@ -8395,13 +8395,13 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>17.6</v>
+        <v>17.59</v>
       </c>
       <c r="G35" t="n">
-        <v>88818384325</v>
+        <v>88767935770</v>
       </c>
       <c r="H35" t="n">
-        <v>31853100</v>
+        <v>0</v>
       </c>
       <c r="I35" t="n">
         <v>5046500000</v>
@@ -8416,7 +8416,7 @@
         <v>4.69</v>
       </c>
       <c r="M35" t="n">
-        <v>7.373734547712406</v>
+        <v>7.369546290340773</v>
       </c>
       <c r="N35" t="n">
         <v>1.79</v>
@@ -8494,7 +8494,7 @@
         <v>5349290000</v>
       </c>
       <c r="AM35" t="n">
-        <v>7340362340.909091</v>
+        <v>7336193038.842976</v>
       </c>
       <c r="AN35" t="n">
         <v>0.5305</v>
@@ -8535,7 +8535,7 @@
         <v>7.68</v>
       </c>
       <c r="AZ35" t="n">
-        <v>10.27</v>
+        <v>10.26</v>
       </c>
       <c r="BA35" t="n">
         <v>1.11</v>
@@ -8544,10 +8544,10 @@
         <v>9.119999999999999</v>
       </c>
       <c r="BC35" t="n">
-        <v>-46.55</v>
+        <v>-46.52</v>
       </c>
       <c r="BD35" t="n">
-        <v>-56.36</v>
+        <v>-56.34</v>
       </c>
       <c r="BE35" t="n">
         <v>-41.67</v>
@@ -8556,13 +8556,13 @@
         <v>-93.67</v>
       </c>
       <c r="BG35" t="n">
-        <v>-48.2</v>
+        <v>-48.17</v>
       </c>
       <c r="BH35" t="n">
         <v>3.71</v>
       </c>
       <c r="BI35" t="n">
-        <v>0</v>
+        <v>-0.06</v>
       </c>
       <c r="BJ35" t="n">
         <v>17.6</v>
@@ -8574,7 +8574,7 @@
         <v>1.04</v>
       </c>
       <c r="BM35" t="n">
-        <v>17.79</v>
+        <v>17.7</v>
       </c>
       <c r="BN35" t="n">
         <v>20.08</v>
@@ -8583,19 +8583,19 @@
         <v>11.7</v>
       </c>
       <c r="BP35" t="n">
-        <v>17.24</v>
+        <v>17.39</v>
       </c>
       <c r="BQ35" t="n">
-        <v>16.84</v>
+        <v>16.83</v>
       </c>
       <c r="BR35" t="n">
-        <v>17.73</v>
+        <v>17.44</v>
       </c>
       <c r="BS35" t="n">
         <v>7.3</v>
       </c>
       <c r="BT35" t="n">
-        <v>36985797</v>
+        <v>36804613</v>
       </c>
     </row>
     <row r="36">
@@ -9315,13 +9315,13 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>69.62</v>
+        <v>69.61</v>
       </c>
       <c r="G39" t="n">
-        <v>3902779696</v>
+        <v>3902218993</v>
       </c>
       <c r="H39" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="I39" t="n">
         <v>168174945</v>
@@ -9336,7 +9336,7 @@
         <v>0.53</v>
       </c>
       <c r="M39" t="n">
-        <v>0.1959024217235617</v>
+        <v>0.1958742768924096</v>
       </c>
       <c r="N39" t="n">
         <v>0.06</v>
@@ -9414,7 +9414,7 @@
         <v>2536078170.6</v>
       </c>
       <c r="AM39" t="n">
-        <v>409955850.4201681</v>
+        <v>409896953.0462185</v>
       </c>
       <c r="AN39" t="n">
         <v>11.9435</v>
@@ -9455,7 +9455,7 @@
         <v>170.24</v>
       </c>
       <c r="AZ39" t="n">
-        <v>203.41</v>
+        <v>203.38</v>
       </c>
       <c r="BA39" t="n">
         <v>19.01</v>
@@ -9464,10 +9464,10 @@
         <v>91.72</v>
       </c>
       <c r="BC39" t="n">
-        <v>199.49</v>
+        <v>199.53</v>
       </c>
       <c r="BD39" t="n">
-        <v>144.53</v>
+        <v>144.57</v>
       </c>
       <c r="BE39" t="n">
         <v>192.17</v>
@@ -9476,13 +9476,13 @@
         <v>-72.69</v>
       </c>
       <c r="BG39" t="n">
-        <v>31.75</v>
+        <v>31.77</v>
       </c>
       <c r="BH39" t="n">
         <v>128.13</v>
       </c>
       <c r="BI39" t="n">
-        <v>0</v>
+        <v>-0.01</v>
       </c>
       <c r="BJ39" t="n">
         <v>69.62</v>
@@ -9494,7 +9494,7 @@
         <v>15.08</v>
       </c>
       <c r="BM39" t="n">
-        <v>69.89</v>
+        <v>69.61</v>
       </c>
       <c r="BN39" t="n">
         <v>74.56</v>
@@ -9503,19 +9503,19 @@
         <v>54.98</v>
       </c>
       <c r="BP39" t="n">
-        <v>69.41</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="BQ39" t="n">
         <v>4.62</v>
       </c>
       <c r="BR39" t="n">
-        <v>69.89</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="BS39" t="n">
         <v>0.58</v>
       </c>
       <c r="BT39" t="n">
-        <v>3817</v>
+        <v>3630</v>
       </c>
     </row>
     <row r="40">
@@ -9545,13 +9545,13 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>22.78</v>
+        <v>23.2</v>
       </c>
       <c r="G40" t="n">
-        <v>130548356895</v>
+        <v>132955353172</v>
       </c>
       <c r="H40" t="n">
-        <v>30659600</v>
+        <v>0</v>
       </c>
       <c r="I40" t="n">
         <v>5730834040</v>
@@ -9566,7 +9566,7 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="M40" t="n">
-        <v>0.3960998709399051</v>
+        <v>0.4034029955241491</v>
       </c>
       <c r="N40" t="n">
         <v>0.05</v>
@@ -9644,7 +9644,7 @@
         <v>15358635227.2</v>
       </c>
       <c r="AM40" t="n">
-        <v>6771180336.877593</v>
+        <v>6896024542.116182</v>
       </c>
       <c r="AN40" t="n">
         <v>0.5641</v>
@@ -9685,7 +9685,7 @@
         <v>36.13</v>
       </c>
       <c r="AZ40" t="n">
-        <v>11.5</v>
+        <v>11.72</v>
       </c>
       <c r="BA40" t="n">
         <v>2.76</v>
@@ -9694,19 +9694,19 @@
         <v>27.89</v>
       </c>
       <c r="BC40" t="n">
-        <v>94.23999999999999</v>
+        <v>90.73</v>
       </c>
       <c r="BD40" t="n">
-        <v>58.6</v>
+        <v>55.73</v>
       </c>
       <c r="BE40" t="n">
         <v>-49.5</v>
       </c>
       <c r="BF40" t="n">
-        <v>-87.89</v>
+        <v>-88.11</v>
       </c>
       <c r="BG40" t="n">
-        <v>22.43</v>
+        <v>20.22</v>
       </c>
       <c r="BH40" t="n">
         <v>32.47</v>
@@ -9715,7 +9715,7 @@
         <v>0</v>
       </c>
       <c r="BJ40" t="n">
-        <v>22.78</v>
+        <v>23.2</v>
       </c>
       <c r="BK40" t="n">
         <v>2.68</v>
@@ -9724,7 +9724,7 @@
         <v>2.5</v>
       </c>
       <c r="BM40" t="n">
-        <v>23.03</v>
+        <v>23.23</v>
       </c>
       <c r="BN40" t="n">
         <v>27.36</v>
@@ -9736,16 +9736,16 @@
         <v>22.3</v>
       </c>
       <c r="BQ40" t="n">
-        <v>9.119999999999999</v>
+        <v>9.279999999999999</v>
       </c>
       <c r="BR40" t="n">
-        <v>22.79</v>
+        <v>22.59</v>
       </c>
       <c r="BS40" t="n">
         <v>0.39</v>
       </c>
       <c r="BT40" t="n">
-        <v>32342306</v>
+        <v>32908031</v>
       </c>
     </row>
     <row r="41">
@@ -9775,13 +9775,13 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>16.03</v>
+        <v>15.79</v>
       </c>
       <c r="G41" t="n">
-        <v>191375773977</v>
+        <v>189650037887</v>
       </c>
       <c r="H41" t="n">
-        <v>5695800</v>
+        <v>0</v>
       </c>
       <c r="I41" t="n">
         <v>5303870781</v>
@@ -9796,7 +9796,7 @@
         <v>0.92</v>
       </c>
       <c r="M41" t="n">
-        <v>1.275322121275104</v>
+        <v>1.263821870405711</v>
       </c>
       <c r="N41" t="n">
         <v>0.07000000000000001</v>
@@ -9874,7 +9874,7 @@
         <v>12304980211.92</v>
       </c>
       <c r="AM41" t="n">
-        <v>29487792600.46225</v>
+        <v>29221885652.85054</v>
       </c>
       <c r="AN41" t="n">
         <v>1.6841</v>
@@ -9915,7 +9915,7 @@
         <v>24.4</v>
       </c>
       <c r="AZ41" t="n">
-        <v>23.99</v>
+        <v>23.63</v>
       </c>
       <c r="BA41" t="n">
         <v>2.53</v>
@@ -9924,25 +9924,25 @@
         <v>13.77</v>
       </c>
       <c r="BC41" t="n">
-        <v>86.43000000000001</v>
+        <v>89.27</v>
       </c>
       <c r="BD41" t="n">
-        <v>52.22</v>
+        <v>54.54</v>
       </c>
       <c r="BE41" t="n">
         <v>49.67</v>
       </c>
       <c r="BF41" t="n">
-        <v>-84.23</v>
+        <v>-84</v>
       </c>
       <c r="BG41" t="n">
-        <v>-14.1</v>
+        <v>-12.79</v>
       </c>
       <c r="BH41" t="n">
         <v>17.11</v>
       </c>
       <c r="BI41" t="n">
-        <v>0</v>
+        <v>-1.5</v>
       </c>
       <c r="BJ41" t="n">
         <v>16.03</v>
@@ -9954,7 +9954,7 @@
         <v>2.34</v>
       </c>
       <c r="BM41" t="n">
-        <v>16.14</v>
+        <v>15.95</v>
       </c>
       <c r="BN41" t="n">
         <v>18.28</v>
@@ -9963,19 +9963,19 @@
         <v>13.43</v>
       </c>
       <c r="BP41" t="n">
-        <v>15.74</v>
+        <v>15.77</v>
       </c>
       <c r="BQ41" t="n">
-        <v>6.86</v>
+        <v>6.76</v>
       </c>
       <c r="BR41" t="n">
-        <v>16.09</v>
+        <v>15.91</v>
       </c>
       <c r="BS41" t="n">
         <v>0.5600000000000001</v>
       </c>
       <c r="BT41" t="n">
-        <v>6988188</v>
+        <v>7020174</v>
       </c>
     </row>
     <row r="42">
@@ -10005,13 +10005,13 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>18.15</v>
+        <v>17.99</v>
       </c>
       <c r="G42" t="n">
-        <v>191375773977</v>
+        <v>189650037887</v>
       </c>
       <c r="H42" t="n">
-        <v>40269400</v>
+        <v>0</v>
       </c>
       <c r="I42" t="n">
         <v>5288141247</v>
@@ -10026,7 +10026,7 @@
         <v>1.05</v>
       </c>
       <c r="M42" t="n">
-        <v>1.279115556762277</v>
+        <v>1.267581098488314</v>
       </c>
       <c r="N42" t="n">
         <v>0.08</v>
@@ -10104,7 +10104,7 @@
         <v>12268487693.04</v>
       </c>
       <c r="AM42" t="n">
-        <v>26037520268.97959</v>
+        <v>25802726243.12925</v>
       </c>
       <c r="AN42" t="n">
         <v>1.8491</v>
@@ -10145,7 +10145,7 @@
         <v>24.4</v>
       </c>
       <c r="AZ42" t="n">
-        <v>26.29</v>
+        <v>26.06</v>
       </c>
       <c r="BA42" t="n">
         <v>2.53</v>
@@ -10154,25 +10154,25 @@
         <v>15.11</v>
       </c>
       <c r="BC42" t="n">
-        <v>64.66</v>
+        <v>66.12</v>
       </c>
       <c r="BD42" t="n">
-        <v>34.44</v>
+        <v>35.64</v>
       </c>
       <c r="BE42" t="n">
         <v>44.83</v>
       </c>
       <c r="BF42" t="n">
-        <v>-86.08</v>
+        <v>-85.95</v>
       </c>
       <c r="BG42" t="n">
-        <v>-16.72</v>
+        <v>-15.98</v>
       </c>
       <c r="BH42" t="n">
         <v>17.11</v>
       </c>
       <c r="BI42" t="n">
-        <v>0</v>
+        <v>-0.88</v>
       </c>
       <c r="BJ42" t="n">
         <v>18.15</v>
@@ -10184,7 +10184,7 @@
         <v>2.34</v>
       </c>
       <c r="BM42" t="n">
-        <v>18.26</v>
+        <v>18.11</v>
       </c>
       <c r="BN42" t="n">
         <v>21.33</v>
@@ -10193,19 +10193,19 @@
         <v>15.67</v>
       </c>
       <c r="BP42" t="n">
-        <v>17.85</v>
+        <v>17.9</v>
       </c>
       <c r="BQ42" t="n">
-        <v>7.76</v>
+        <v>7.7</v>
       </c>
       <c r="BR42" t="n">
-        <v>18.19</v>
+        <v>18.09</v>
       </c>
       <c r="BS42" t="n">
         <v>0.63</v>
       </c>
       <c r="BT42" t="n">
-        <v>40515008</v>
+        <v>40611854</v>
       </c>
     </row>
     <row r="43">
@@ -10235,13 +10235,13 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>40.41</v>
+        <v>40.86</v>
       </c>
       <c r="G43" t="n">
-        <v>78451973703</v>
+        <v>79325605184</v>
       </c>
       <c r="H43" t="n">
-        <v>5078700</v>
+        <v>0</v>
       </c>
       <c r="I43" t="n">
         <v>1941400000</v>
@@ -10334,7 +10334,7 @@
         <v>9182822000</v>
       </c>
       <c r="AM43" t="n">
-        <v>9555660621.559072</v>
+        <v>9662071276.979292</v>
       </c>
       <c r="AN43" t="n">
         <v>4.5901</v>
@@ -10375,7 +10375,7 @@
         <v>19.95</v>
       </c>
       <c r="AZ43" t="n">
-        <v>73.34</v>
+        <v>74.16</v>
       </c>
       <c r="BA43" t="n">
         <v>5.63</v>
@@ -10384,25 +10384,25 @@
         <v>48.62</v>
       </c>
       <c r="BC43" t="n">
-        <v>-39.53</v>
+        <v>-40.2</v>
       </c>
       <c r="BD43" t="n">
-        <v>-50.63</v>
+        <v>-51.17</v>
       </c>
       <c r="BE43" t="n">
         <v>81.5</v>
       </c>
       <c r="BF43" t="n">
-        <v>-86.06999999999999</v>
+        <v>-86.22</v>
       </c>
       <c r="BG43" t="n">
-        <v>20.31</v>
+        <v>18.98</v>
       </c>
       <c r="BH43" t="n">
         <v>5.61</v>
       </c>
       <c r="BI43" t="n">
-        <v>0</v>
+        <v>1.11</v>
       </c>
       <c r="BJ43" t="n">
         <v>40.41</v>
@@ -10414,7 +10414,7 @@
         <v>4.73</v>
       </c>
       <c r="BM43" t="n">
-        <v>41.05</v>
+        <v>40.86</v>
       </c>
       <c r="BN43" t="n">
         <v>42.98</v>
@@ -10423,19 +10423,19 @@
         <v>28.06</v>
       </c>
       <c r="BP43" t="n">
-        <v>40.06</v>
+        <v>39.95</v>
       </c>
       <c r="BQ43" t="n">
-        <v>8.539999999999999</v>
+        <v>8.630000000000001</v>
       </c>
       <c r="BR43" t="n">
-        <v>40.63</v>
+        <v>40.32</v>
       </c>
       <c r="BS43" t="n">
         <v>0</v>
       </c>
       <c r="BT43" t="n">
-        <v>6705721</v>
+        <v>6637224</v>
       </c>
     </row>
     <row r="44">
@@ -10925,13 +10925,13 @@
         </is>
       </c>
       <c r="F46" t="n">
-        <v>3.81</v>
+        <v>3.98</v>
       </c>
       <c r="G46" t="n">
-        <v>3812061152</v>
+        <v>3982157179</v>
       </c>
       <c r="H46" t="n">
-        <v>29974200</v>
+        <v>0</v>
       </c>
       <c r="I46" t="n">
         <v>1000541644</v>
@@ -10946,7 +10946,7 @@
         <v>2.5</v>
       </c>
       <c r="M46" t="n">
-        <v>0.06626082590816831</v>
+        <v>0.0692174162626554</v>
       </c>
       <c r="N46" t="n">
         <v>0.08</v>
@@ -11024,7 +11024,7 @@
         <v>460249156.24</v>
       </c>
       <c r="AM46" t="n">
-        <v>3737314854.901961</v>
+        <v>3904075665.686275</v>
       </c>
       <c r="AN46" t="n">
         <v>0.0311</v>
@@ -11065,7 +11065,7 @@
         <v>3.3</v>
       </c>
       <c r="AZ46" t="n">
-        <v>3.14</v>
+        <v>3.28</v>
       </c>
       <c r="BA46" t="n">
         <v>0.42</v>
@@ -11074,19 +11074,19 @@
         <v>7.38</v>
       </c>
       <c r="BC46" t="n">
-        <v>6.14</v>
+        <v>1.61</v>
       </c>
       <c r="BD46" t="n">
-        <v>-13.34</v>
+        <v>-17.04</v>
       </c>
       <c r="BE46" t="n">
         <v>-17.5</v>
       </c>
       <c r="BF46" t="n">
-        <v>-88.90000000000001</v>
+        <v>-89.37</v>
       </c>
       <c r="BG46" t="n">
-        <v>93.66</v>
+        <v>85.39</v>
       </c>
       <c r="BH46" t="n">
         <v>1.58</v>
@@ -11095,7 +11095,7 @@
         <v>0</v>
       </c>
       <c r="BJ46" t="n">
-        <v>3.81</v>
+        <v>3.98</v>
       </c>
       <c r="BK46" t="n">
         <v>0.46</v>
@@ -11104,7 +11104,7 @@
         <v>0.46</v>
       </c>
       <c r="BM46" t="n">
-        <v>4.05</v>
+        <v>4.01</v>
       </c>
       <c r="BN46" t="n">
         <v>7.31</v>
@@ -11113,19 +11113,19 @@
         <v>2.97</v>
       </c>
       <c r="BP46" t="n">
-        <v>3.78</v>
+        <v>3.8</v>
       </c>
       <c r="BQ46" t="n">
-        <v>8.33</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="BR46" t="n">
-        <v>4.01</v>
+        <v>3.81</v>
       </c>
       <c r="BS46" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="BT46" t="n">
-        <v>20775803</v>
+        <v>21479160</v>
       </c>
     </row>
     <row r="47">
@@ -11155,13 +11155,13 @@
         </is>
       </c>
       <c r="F47" t="n">
-        <v>8.82</v>
+        <v>8.93</v>
       </c>
       <c r="G47" t="n">
-        <v>3078731143</v>
+        <v>3131580544</v>
       </c>
       <c r="H47" t="n">
-        <v>12100</v>
+        <v>0</v>
       </c>
       <c r="I47" t="n">
         <v>254106600</v>
@@ -11176,7 +11176,7 @@
         <v>1.22</v>
       </c>
       <c r="M47" t="n">
-        <v>0.7260002251219001</v>
+        <v>0.7384627219238034</v>
       </c>
       <c r="N47" t="n">
         <v>0.07000000000000001</v>
@@ -11254,7 +11254,7 @@
         <v>322715382</v>
       </c>
       <c r="AM47" t="n">
-        <v>545874316.1347518</v>
+        <v>555244777.3049645</v>
       </c>
       <c r="AN47" t="n">
         <v>0.4132</v>
@@ -11295,7 +11295,7 @@
         <v>11.74</v>
       </c>
       <c r="AZ47" t="n">
-        <v>11.58</v>
+        <v>11.73</v>
       </c>
       <c r="BA47" t="n">
         <v>1.46</v>
@@ -11304,25 +11304,25 @@
         <v>8.619999999999999</v>
       </c>
       <c r="BC47" t="n">
-        <v>62.96</v>
+        <v>60.96</v>
       </c>
       <c r="BD47" t="n">
-        <v>33.06</v>
+        <v>31.42</v>
       </c>
       <c r="BE47" t="n">
         <v>31.33</v>
       </c>
       <c r="BF47" t="n">
-        <v>-83.45999999999999</v>
+        <v>-83.67</v>
       </c>
       <c r="BG47" t="n">
-        <v>-2.27</v>
+        <v>-3.47</v>
       </c>
       <c r="BH47" t="n">
         <v>7.23</v>
       </c>
       <c r="BI47" t="n">
-        <v>0</v>
+        <v>1.25</v>
       </c>
       <c r="BJ47" t="n">
         <v>8.82</v>
@@ -11334,28 +11334,28 @@
         <v>1.29</v>
       </c>
       <c r="BM47" t="n">
-        <v>9.029999999999999</v>
+        <v>8.93</v>
       </c>
       <c r="BN47" t="n">
-        <v>9.25</v>
+        <v>9.24</v>
       </c>
       <c r="BO47" t="n">
-        <v>7.2</v>
+        <v>7.19</v>
       </c>
       <c r="BP47" t="n">
-        <v>8.81</v>
+        <v>8.83</v>
       </c>
       <c r="BQ47" t="n">
-        <v>6.82</v>
+        <v>6.9</v>
       </c>
       <c r="BR47" t="n">
-        <v>8.99</v>
+        <v>8.83</v>
       </c>
       <c r="BS47" t="n">
         <v>0.53</v>
       </c>
       <c r="BT47" t="n">
-        <v>12172</v>
+        <v>12261</v>
       </c>
     </row>
     <row r="48">
@@ -11385,13 +11385,13 @@
         </is>
       </c>
       <c r="F48" t="n">
-        <v>9.119999999999999</v>
+        <v>9.06</v>
       </c>
       <c r="G48" t="n">
-        <v>3078731143</v>
+        <v>3131580544</v>
       </c>
       <c r="H48" t="n">
-        <v>3100</v>
+        <v>0</v>
       </c>
       <c r="I48" t="n">
         <v>93397546</v>
@@ -11406,7 +11406,7 @@
         <v>1.24</v>
       </c>
       <c r="M48" t="n">
-        <v>1.975228008720493</v>
+        <v>2.009134709971964</v>
       </c>
       <c r="N48" t="n">
         <v>0.07000000000000001</v>
@@ -11484,7 +11484,7 @@
         <v>118614883.42</v>
       </c>
       <c r="AM48" t="n">
-        <v>538239710.3146853</v>
+        <v>547479116.0839161</v>
       </c>
       <c r="AN48" t="n">
         <v>0.4132</v>
@@ -11525,7 +11525,7 @@
         <v>11.74</v>
       </c>
       <c r="AZ48" t="n">
-        <v>11.93</v>
+        <v>11.85</v>
       </c>
       <c r="BA48" t="n">
         <v>1.46</v>
@@ -11534,25 +11534,25 @@
         <v>8.24</v>
       </c>
       <c r="BC48" t="n">
-        <v>57.6</v>
+        <v>58.65</v>
       </c>
       <c r="BD48" t="n">
-        <v>28.68</v>
+        <v>29.54</v>
       </c>
       <c r="BE48" t="n">
         <v>30.83</v>
       </c>
       <c r="BF48" t="n">
-        <v>-84.01000000000001</v>
+        <v>-83.90000000000001</v>
       </c>
       <c r="BG48" t="n">
-        <v>-9.69</v>
+        <v>-9.09</v>
       </c>
       <c r="BH48" t="n">
         <v>7.23</v>
       </c>
       <c r="BI48" t="n">
-        <v>0</v>
+        <v>-0.66</v>
       </c>
       <c r="BJ48" t="n">
         <v>9.119999999999999</v>
@@ -11564,28 +11564,28 @@
         <v>1.29</v>
       </c>
       <c r="BM48" t="n">
-        <v>9.15</v>
+        <v>9.19</v>
       </c>
       <c r="BN48" t="n">
         <v>9.48</v>
       </c>
       <c r="BO48" t="n">
-        <v>7.21</v>
+        <v>7.2</v>
       </c>
       <c r="BP48" t="n">
-        <v>9.1</v>
+        <v>9.039999999999999</v>
       </c>
       <c r="BQ48" t="n">
-        <v>7.05</v>
+        <v>7.01</v>
       </c>
       <c r="BR48" t="n">
-        <v>9.130000000000001</v>
+        <v>9.19</v>
       </c>
       <c r="BS48" t="n">
         <v>0.54</v>
       </c>
       <c r="BT48" t="n">
-        <v>2577</v>
+        <v>2480</v>
       </c>
     </row>
     <row r="49">
@@ -11845,13 +11845,13 @@
         </is>
       </c>
       <c r="F50" t="n">
-        <v>32.96</v>
+        <v>33.44</v>
       </c>
       <c r="G50" t="n">
-        <v>956853500</v>
+        <v>956276500</v>
       </c>
       <c r="H50" t="n">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="I50" t="n">
         <v>11540870</v>
@@ -11866,7 +11866,7 @@
         <v>0.8</v>
       </c>
       <c r="M50" t="n">
-        <v>0.9680363439513173</v>
+        <v>0.9674526004937661</v>
       </c>
       <c r="N50" t="n">
         <v>0.06</v>
@@ -11944,7 +11944,7 @@
         <v>84709985.8</v>
       </c>
       <c r="AM50" t="n">
-        <v>326571160.4095563</v>
+        <v>326374232.0819113</v>
       </c>
       <c r="AN50" t="n">
         <v>4.4983</v>
@@ -11985,7 +11985,7 @@
         <v>68.48999999999999</v>
       </c>
       <c r="AZ50" t="n">
-        <v>72.68000000000001</v>
+        <v>73.73999999999999</v>
       </c>
       <c r="BA50" t="n">
         <v>9.210000000000001</v>
@@ -11994,19 +11994,19 @@
         <v>30.53</v>
       </c>
       <c r="BC50" t="n">
-        <v>154.48</v>
+        <v>150.83</v>
       </c>
       <c r="BD50" t="n">
-        <v>107.78</v>
+        <v>104.8</v>
       </c>
       <c r="BE50" t="n">
         <v>120.5</v>
       </c>
       <c r="BF50" t="n">
-        <v>-72.05</v>
+        <v>-72.45</v>
       </c>
       <c r="BG50" t="n">
-        <v>-7.37</v>
+        <v>-8.699999999999999</v>
       </c>
       <c r="BH50" t="n">
         <v>42.6</v>
@@ -12015,7 +12015,7 @@
         <v>0</v>
       </c>
       <c r="BJ50" t="n">
-        <v>32.96</v>
+        <v>33.44</v>
       </c>
       <c r="BK50" t="n">
         <v>7.34</v>
@@ -12024,7 +12024,7 @@
         <v>7.6</v>
       </c>
       <c r="BM50" t="n">
-        <v>33.49</v>
+        <v>33.44</v>
       </c>
       <c r="BN50" t="n">
         <v>39.22</v>
@@ -12033,19 +12033,19 @@
         <v>23.5</v>
       </c>
       <c r="BP50" t="n">
-        <v>32.96</v>
+        <v>33.44</v>
       </c>
       <c r="BQ50" t="n">
-        <v>4.34</v>
+        <v>4.4</v>
       </c>
       <c r="BR50" t="n">
-        <v>33.49</v>
+        <v>33.44</v>
       </c>
       <c r="BS50" t="n">
         <v>0.4</v>
       </c>
       <c r="BT50" t="n">
-        <v>543</v>
+        <v>530</v>
       </c>
     </row>
     <row r="51">
@@ -12529,7 +12529,7 @@
         <v>856696055</v>
       </c>
       <c r="H53" t="n">
-        <v>195700</v>
+        <v>0</v>
       </c>
       <c r="I53" t="n">
         <v>136852484</v>
@@ -12702,7 +12702,7 @@
         <v>0.09</v>
       </c>
       <c r="BM53" t="n">
-        <v>6.56</v>
+        <v>6.36</v>
       </c>
       <c r="BN53" t="n">
         <v>10.39</v>
@@ -12717,13 +12717,13 @@
         <v>73.37</v>
       </c>
       <c r="BR53" t="n">
-        <v>6.56</v>
+        <v>6.35</v>
       </c>
       <c r="BS53" t="n">
         <v>2.36</v>
       </c>
       <c r="BT53" t="n">
-        <v>37217</v>
+        <v>42807</v>
       </c>
     </row>
     <row r="54">
@@ -12753,13 +12753,13 @@
         </is>
       </c>
       <c r="F54" t="n">
-        <v>10.69</v>
+        <v>10.55</v>
       </c>
       <c r="G54" t="n">
-        <v>2493037251</v>
+        <v>2460387699</v>
       </c>
       <c r="H54" t="n">
-        <v>344100</v>
+        <v>0</v>
       </c>
       <c r="I54" t="n">
         <v>233212121</v>
@@ -12774,7 +12774,7 @@
         <v>0.97</v>
       </c>
       <c r="M54" t="n">
-        <v>1.399320818989078</v>
+        <v>1.38099490034268</v>
       </c>
       <c r="N54" t="n">
         <v>0.5600000000000001</v>
@@ -12852,7 +12852,7 @@
         <v>233212121</v>
       </c>
       <c r="AM54" t="n">
-        <v>341044767.5786594</v>
+        <v>336578344.5964432</v>
       </c>
       <c r="AN54" t="n">
         <v>0.1531</v>
@@ -12893,7 +12893,7 @@
         <v>12.25</v>
       </c>
       <c r="AZ54" t="n">
-        <v>17.01</v>
+        <v>16.79</v>
       </c>
       <c r="BA54" t="n">
         <v>0.98</v>
@@ -12902,25 +12902,25 @@
         <v>6.52</v>
       </c>
       <c r="BC54" t="n">
-        <v>40.39</v>
+        <v>42.25</v>
       </c>
       <c r="BD54" t="n">
-        <v>14.63</v>
+        <v>16.15</v>
       </c>
       <c r="BE54" t="n">
         <v>59.17</v>
       </c>
       <c r="BF54" t="n">
-        <v>-90.8</v>
+        <v>-90.68000000000001</v>
       </c>
       <c r="BG54" t="n">
-        <v>-39.04</v>
+        <v>-38.23</v>
       </c>
       <c r="BH54" t="n">
         <v>10.01</v>
       </c>
       <c r="BI54" t="n">
-        <v>0</v>
+        <v>-1.31</v>
       </c>
       <c r="BJ54" t="n">
         <v>10.69</v>
@@ -12932,7 +12932,7 @@
         <v>1</v>
       </c>
       <c r="BM54" t="n">
-        <v>10.96</v>
+        <v>10.69</v>
       </c>
       <c r="BN54" t="n">
         <v>11.75</v>
@@ -12941,19 +12941,19 @@
         <v>8.279999999999999</v>
       </c>
       <c r="BP54" t="n">
-        <v>10.58</v>
+        <v>10.29</v>
       </c>
       <c r="BQ54" t="n">
-        <v>10.66</v>
+        <v>10.52</v>
       </c>
       <c r="BR54" t="n">
-        <v>10.58</v>
+        <v>10.69</v>
       </c>
       <c r="BS54" t="n">
         <v>1.26</v>
       </c>
       <c r="BT54" t="n">
-        <v>265840</v>
+        <v>270133</v>
       </c>
     </row>
     <row r="55">
@@ -12983,13 +12983,13 @@
         </is>
       </c>
       <c r="F55" t="n">
-        <v>49.2</v>
+        <v>49.72</v>
       </c>
       <c r="G55" t="n">
-        <v>6427234179</v>
+        <v>6690365323</v>
       </c>
       <c r="H55" t="n">
-        <v>8900</v>
+        <v>0</v>
       </c>
       <c r="I55" t="n">
         <v>84052790</v>
@@ -13004,7 +13004,7 @@
         <v>2</v>
       </c>
       <c r="M55" t="n">
-        <v>0.9921795856105552</v>
+        <v>1.032799445124647</v>
       </c>
       <c r="N55" t="n">
         <v>0.16</v>
@@ -13082,7 +13082,7 @@
         <v>579123723.1</v>
       </c>
       <c r="AM55" t="n">
-        <v>323301518.0583501</v>
+        <v>336537491.0965795</v>
       </c>
       <c r="AN55" t="n">
         <v>3.1953</v>
@@ -13123,7 +13123,7 @@
         <v>51.21</v>
       </c>
       <c r="AZ55" t="n">
-        <v>51.74</v>
+        <v>52.29</v>
       </c>
       <c r="BA55" t="n">
         <v>9.380000000000001</v>
@@ -13132,25 +13132,25 @@
         <v>16.08</v>
       </c>
       <c r="BC55" t="n">
-        <v>27.47</v>
+        <v>26.13</v>
       </c>
       <c r="BD55" t="n">
-        <v>4.08</v>
+        <v>2.99</v>
       </c>
       <c r="BE55" t="n">
         <v>5.17</v>
       </c>
       <c r="BF55" t="n">
-        <v>-80.94</v>
+        <v>-81.14</v>
       </c>
       <c r="BG55" t="n">
-        <v>-67.31999999999999</v>
+        <v>-67.67</v>
       </c>
       <c r="BH55" t="n">
         <v>25.37</v>
       </c>
       <c r="BI55" t="n">
-        <v>0</v>
+        <v>1.06</v>
       </c>
       <c r="BJ55" t="n">
         <v>49.2</v>
@@ -13162,7 +13162,7 @@
         <v>7.03</v>
       </c>
       <c r="BM55" t="n">
-        <v>49.93</v>
+        <v>49.99</v>
       </c>
       <c r="BN55" t="n">
         <v>73.67</v>
@@ -13171,19 +13171,19 @@
         <v>35.58</v>
       </c>
       <c r="BP55" t="n">
-        <v>49.01</v>
+        <v>49.16</v>
       </c>
       <c r="BQ55" t="n">
-        <v>7</v>
+        <v>7.07</v>
       </c>
       <c r="BR55" t="n">
-        <v>49.87</v>
+        <v>49.16</v>
       </c>
       <c r="BS55" t="n">
         <v>0.66</v>
       </c>
       <c r="BT55" t="n">
-        <v>7594</v>
+        <v>7501</v>
       </c>
     </row>
     <row r="56">
@@ -13213,13 +13213,13 @@
         </is>
       </c>
       <c r="F56" t="n">
-        <v>59.06</v>
+        <v>60.99</v>
       </c>
       <c r="G56" t="n">
-        <v>6427234179</v>
+        <v>6690365323</v>
       </c>
       <c r="H56" t="n">
-        <v>18000</v>
+        <v>20500</v>
       </c>
       <c r="I56" t="n">
         <v>39675836</v>
@@ -13234,7 +13234,7 @@
         <v>2.41</v>
       </c>
       <c r="M56" t="n">
-        <v>2.101920734615675</v>
+        <v>2.187973427281495</v>
       </c>
       <c r="N56" t="n">
         <v>0.19</v>
@@ -13312,7 +13312,7 @@
         <v>273366510.04</v>
       </c>
       <c r="AM56" t="n">
-        <v>267355831.0732113</v>
+        <v>278301386.1480865</v>
       </c>
       <c r="AN56" t="n">
         <v>3.5102</v>
@@ -13353,7 +13353,7 @@
         <v>51.21</v>
       </c>
       <c r="AZ56" t="n">
-        <v>56.4</v>
+        <v>58.25</v>
       </c>
       <c r="BA56" t="n">
         <v>9.380000000000001</v>
@@ -13362,19 +13362,19 @@
         <v>17.68</v>
       </c>
       <c r="BC56" t="n">
-        <v>6.19</v>
+        <v>2.83</v>
       </c>
       <c r="BD56" t="n">
-        <v>-13.3</v>
+        <v>-16.04</v>
       </c>
       <c r="BE56" t="n">
         <v>-4.5</v>
       </c>
       <c r="BF56" t="n">
-        <v>-84.12</v>
+        <v>-84.62</v>
       </c>
       <c r="BG56" t="n">
-        <v>-70.06999999999999</v>
+        <v>-71.02</v>
       </c>
       <c r="BH56" t="n">
         <v>25.37</v>
@@ -13383,7 +13383,7 @@
         <v>0</v>
       </c>
       <c r="BJ56" t="n">
-        <v>59.06</v>
+        <v>60.99</v>
       </c>
       <c r="BK56" t="n">
         <v>6.89</v>
@@ -13392,7 +13392,7 @@
         <v>7.03</v>
       </c>
       <c r="BM56" t="n">
-        <v>60.46</v>
+        <v>60.99</v>
       </c>
       <c r="BN56" t="n">
         <v>86.77</v>
@@ -13401,19 +13401,19 @@
         <v>46.42</v>
       </c>
       <c r="BP56" t="n">
-        <v>59</v>
+        <v>58.92</v>
       </c>
       <c r="BQ56" t="n">
-        <v>8.4</v>
+        <v>8.67</v>
       </c>
       <c r="BR56" t="n">
-        <v>60.4</v>
+        <v>59.63</v>
       </c>
       <c r="BS56" t="n">
         <v>0.79</v>
       </c>
       <c r="BT56" t="n">
-        <v>34553</v>
+        <v>32592</v>
       </c>
     </row>
     <row r="57">
@@ -13443,13 +13443,13 @@
         </is>
       </c>
       <c r="F57" t="n">
-        <v>6.05</v>
+        <v>6.07</v>
       </c>
       <c r="G57" t="n">
-        <v>1414840944</v>
+        <v>1419518100</v>
       </c>
       <c r="H57" t="n">
-        <v>740400</v>
+        <v>884100</v>
       </c>
       <c r="I57" t="n">
         <v>233858065</v>
@@ -13464,7 +13464,7 @@
         <v>0.77</v>
       </c>
       <c r="M57" t="n">
-        <v>0.4234998954600946</v>
+        <v>0.4248998938736623</v>
       </c>
       <c r="N57" t="n">
         <v>0.08</v>
@@ -13542,7 +13542,7 @@
         <v>229180903.7</v>
       </c>
       <c r="AM57" t="n">
-        <v>105822060.1346298</v>
+        <v>106171884.8167539</v>
       </c>
       <c r="AN57" t="n">
         <v>0.347</v>
@@ -13583,7 +13583,7 @@
         <v>10.72</v>
       </c>
       <c r="AZ57" t="n">
-        <v>9.23</v>
+        <v>9.26</v>
       </c>
       <c r="BA57" t="n">
         <v>1.13</v>
@@ -13592,19 +13592,19 @@
         <v>6.26</v>
       </c>
       <c r="BC57" t="n">
-        <v>117.05</v>
+        <v>116.33</v>
       </c>
       <c r="BD57" t="n">
-        <v>77.22</v>
+        <v>76.63</v>
       </c>
       <c r="BE57" t="n">
         <v>52.5</v>
       </c>
       <c r="BF57" t="n">
-        <v>-81.36</v>
+        <v>-81.43000000000001</v>
       </c>
       <c r="BG57" t="n">
-        <v>3.54</v>
+        <v>3.19</v>
       </c>
       <c r="BH57" t="n">
         <v>7.82</v>
@@ -13613,7 +13613,7 @@
         <v>0</v>
       </c>
       <c r="BJ57" t="n">
-        <v>6.05</v>
+        <v>6.07</v>
       </c>
       <c r="BK57" t="n">
         <v>0.98</v>
@@ -13631,10 +13631,10 @@
         <v>3.43</v>
       </c>
       <c r="BP57" t="n">
-        <v>5.97</v>
+        <v>5.94</v>
       </c>
       <c r="BQ57" t="n">
-        <v>5.84</v>
+        <v>5.86</v>
       </c>
       <c r="BR57" t="n">
         <v>6.03</v>
@@ -13643,7 +13643,7 @@
         <v>0.42</v>
       </c>
       <c r="BT57" t="n">
-        <v>1286956</v>
+        <v>1286880</v>
       </c>
     </row>
     <row r="58">
@@ -13909,7 +13909,7 @@
         <v>94446470</v>
       </c>
       <c r="H59" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I59" t="n">
         <v>710143</v>
@@ -14088,7 +14088,7 @@
         <v>25.98</v>
       </c>
       <c r="BO59" t="n">
-        <v>15.82</v>
+        <v>15.85</v>
       </c>
       <c r="BP59" t="n">
         <v>20</v>
@@ -14133,13 +14133,13 @@
         </is>
       </c>
       <c r="F60" t="n">
-        <v>380</v>
+        <v>376.92</v>
       </c>
       <c r="G60" t="n">
-        <v>172805000</v>
+        <v>171404376</v>
       </c>
       <c r="H60" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="I60" t="n">
         <v>454750</v>
@@ -14154,7 +14154,7 @@
         <v>0.83</v>
       </c>
       <c r="M60" t="n">
-        <v>12.92557074139116</v>
+        <v>12.82080603785775</v>
       </c>
       <c r="N60" t="n">
         <v>0.68</v>
@@ -14232,7 +14232,7 @@
         <v>59558607.5</v>
       </c>
       <c r="AM60" t="n">
-        <v>-25337976.53958944</v>
+        <v>-25132606.4516129</v>
       </c>
       <c r="AN60" t="n">
         <v>10.0581</v>
@@ -14273,7 +14273,7 @@
         <v>944.87</v>
       </c>
       <c r="AZ60" t="n">
-        <v>2185</v>
+        <v>2167.29</v>
       </c>
       <c r="BA60" t="n">
         <v>231.1</v>
@@ -14282,19 +14282,19 @@
         <v>727.97</v>
       </c>
       <c r="BC60" t="n">
-        <v>204.53</v>
+        <v>207.02</v>
       </c>
       <c r="BD60" t="n">
-        <v>148.65</v>
+        <v>150.68</v>
       </c>
       <c r="BE60" t="n">
         <v>475</v>
       </c>
       <c r="BF60" t="n">
-        <v>-39.19</v>
+        <v>-38.69</v>
       </c>
       <c r="BG60" t="n">
-        <v>91.56999999999999</v>
+        <v>93.14</v>
       </c>
       <c r="BH60" t="n">
         <v>454.44</v>
@@ -14303,7 +14303,7 @@
         <v>0</v>
       </c>
       <c r="BJ60" t="n">
-        <v>380</v>
+        <v>376.92</v>
       </c>
       <c r="BK60" t="n">
         <v>130.97</v>
@@ -14321,13 +14321,13 @@
         <v>306.27</v>
       </c>
       <c r="BP60" t="n">
-        <v>377.09</v>
+        <v>376.92</v>
       </c>
       <c r="BQ60" t="n">
-        <v>2.9</v>
+        <v>2.88</v>
       </c>
       <c r="BR60" t="n">
-        <v>377.09</v>
+        <v>380</v>
       </c>
       <c r="BS60" t="n">
         <v>12.82</v>
@@ -14363,13 +14363,13 @@
         </is>
       </c>
       <c r="F61" t="n">
-        <v>27.64</v>
+        <v>27.52</v>
       </c>
       <c r="G61" t="n">
-        <v>2366215294</v>
+        <v>2355942931</v>
       </c>
       <c r="H61" t="n">
-        <v>369500</v>
+        <v>0</v>
       </c>
       <c r="I61" t="n">
         <v>85608392</v>
@@ -14384,7 +14384,7 @@
         <v>2.37</v>
       </c>
       <c r="M61" t="n">
-        <v>1.254885211009972</v>
+        <v>1.24943742422425</v>
       </c>
       <c r="N61" t="n">
         <v>1.1</v>
@@ -14462,7 +14462,7 @@
         <v>160087693.04</v>
       </c>
       <c r="AM61" t="n">
-        <v>185731184.7723705</v>
+        <v>184924876.844584</v>
       </c>
       <c r="AN61" t="n">
         <v>0.38</v>
@@ -14503,7 +14503,7 @@
         <v>17.56</v>
       </c>
       <c r="AZ61" t="n">
-        <v>34.83</v>
+        <v>34.68</v>
       </c>
       <c r="BA61" t="n">
         <v>2.52</v>
@@ -14512,19 +14512,19 @@
         <v>11.76</v>
       </c>
       <c r="BC61" t="n">
-        <v>-22.2</v>
+        <v>-21.86</v>
       </c>
       <c r="BD61" t="n">
-        <v>-36.48</v>
+        <v>-36.2</v>
       </c>
       <c r="BE61" t="n">
         <v>26</v>
       </c>
       <c r="BF61" t="n">
-        <v>-90.87</v>
+        <v>-90.83</v>
       </c>
       <c r="BG61" t="n">
-        <v>-57.47</v>
+        <v>-57.28</v>
       </c>
       <c r="BH61" t="n">
         <v>10.99</v>
@@ -14533,7 +14533,7 @@
         <v>0</v>
       </c>
       <c r="BJ61" t="n">
-        <v>27.64</v>
+        <v>27.52</v>
       </c>
       <c r="BK61" t="n">
         <v>1.87</v>
@@ -14542,7 +14542,7 @@
         <v>1.86</v>
       </c>
       <c r="BM61" t="n">
-        <v>28.07</v>
+        <v>27.71</v>
       </c>
       <c r="BN61" t="n">
         <v>28.25</v>
@@ -14551,19 +14551,19 @@
         <v>19.35</v>
       </c>
       <c r="BP61" t="n">
-        <v>27.49</v>
+        <v>27.34</v>
       </c>
       <c r="BQ61" t="n">
-        <v>14.84</v>
+        <v>14.78</v>
       </c>
       <c r="BR61" t="n">
-        <v>27.61</v>
+        <v>27.64</v>
       </c>
       <c r="BS61" t="n">
         <v>1.19</v>
       </c>
       <c r="BT61" t="n">
-        <v>509514</v>
+        <v>511550</v>
       </c>
     </row>
     <row r="62">
@@ -14823,13 +14823,13 @@
         </is>
       </c>
       <c r="F63" t="n">
-        <v>1.38</v>
+        <v>1.35</v>
       </c>
       <c r="G63" t="n">
-        <v>359503384</v>
+        <v>346664076</v>
       </c>
       <c r="H63" t="n">
-        <v>31900</v>
+        <v>30200</v>
       </c>
       <c r="I63" t="n">
         <v>122894462</v>
@@ -14844,7 +14844,7 @@
         <v>-0.22</v>
       </c>
       <c r="M63" t="n">
-        <v>0.4421706097458084</v>
+        <v>0.4263789234926569</v>
       </c>
       <c r="N63" t="n">
         <v>0.37</v>
@@ -14922,7 +14922,7 @@
         <v>31952560.12</v>
       </c>
       <c r="AM63" t="n">
-        <v>204263286.3636364</v>
+        <v>196968225</v>
       </c>
       <c r="AN63" t="n">
         <v>0</v>
@@ -14981,7 +14981,7 @@
         <v>-100</v>
       </c>
       <c r="BF63" t="n">
-        <v>-79.05</v>
+        <v>-78.58</v>
       </c>
       <c r="BG63" t="n">
         <v>-100</v>
@@ -14993,7 +14993,7 @@
         <v>0</v>
       </c>
       <c r="BJ63" t="n">
-        <v>1.38</v>
+        <v>1.35</v>
       </c>
       <c r="BK63" t="n">
         <v>0.26</v>
@@ -15002,7 +15002,7 @@
         <v>0.26</v>
       </c>
       <c r="BM63" t="n">
-        <v>1.44</v>
+        <v>1.43</v>
       </c>
       <c r="BN63" t="n">
         <v>2.12</v>
@@ -15011,10 +15011,10 @@
         <v>1.16</v>
       </c>
       <c r="BP63" t="n">
-        <v>1.34</v>
+        <v>1.35</v>
       </c>
       <c r="BQ63" t="n">
-        <v>5.29</v>
+        <v>5.17</v>
       </c>
       <c r="BR63" t="n">
         <v>1.37</v>
@@ -15023,7 +15023,7 @@
         <v>0.19</v>
       </c>
       <c r="BT63" t="n">
-        <v>22640</v>
+        <v>23603</v>
       </c>
     </row>
     <row r="64">
@@ -15053,13 +15053,13 @@
         </is>
       </c>
       <c r="F64" t="n">
-        <v>61.14</v>
+        <v>61.4</v>
       </c>
       <c r="G64" t="n">
-        <v>236998752694</v>
+        <v>235466795451</v>
       </c>
       <c r="H64" t="n">
-        <v>7134900</v>
+        <v>0</v>
       </c>
       <c r="I64" t="n">
         <v>0</v>
@@ -15146,13 +15146,13 @@
         <v>41.22</v>
       </c>
       <c r="AK64" t="n">
-        <v>67951020157.76189</v>
+        <v>67511785535.99014</v>
       </c>
       <c r="AL64" t="n">
-        <v>18944744419.98401</v>
+        <v>18822285807.43405</v>
       </c>
       <c r="AM64" t="n">
-        <v>21104074149.065</v>
+        <v>20967657653.69546</v>
       </c>
       <c r="AN64" t="n">
         <v>1.4201</v>
@@ -15193,7 +15193,7 @@
         <v>38.98</v>
       </c>
       <c r="AZ64" t="n">
-        <v>24.46</v>
+        <v>24.56</v>
       </c>
       <c r="BA64" t="n">
         <v>6.69</v>
@@ -15202,25 +15202,25 @@
         <v>10.4</v>
       </c>
       <c r="BC64" t="n">
-        <v>-21.92</v>
+        <v>-22.25</v>
       </c>
       <c r="BD64" t="n">
-        <v>-36.25</v>
+        <v>-36.52</v>
       </c>
       <c r="BE64" t="n">
         <v>-60</v>
       </c>
       <c r="BF64" t="n">
-        <v>-89.05</v>
+        <v>-89.09999999999999</v>
       </c>
       <c r="BG64" t="n">
-        <v>-82.98999999999999</v>
+        <v>-83.06999999999999</v>
       </c>
       <c r="BH64" t="n">
         <v>21.37</v>
       </c>
       <c r="BI64" t="n">
-        <v>0</v>
+        <v>0.43</v>
       </c>
       <c r="BJ64" t="n">
         <v>61.14</v>
@@ -15232,7 +15232,7 @@
         <v>1.57</v>
       </c>
       <c r="BM64" t="n">
-        <v>61.67</v>
+        <v>61.6</v>
       </c>
       <c r="BN64" t="n">
         <v>64.72</v>
@@ -15241,19 +15241,19 @@
         <v>44.12</v>
       </c>
       <c r="BP64" t="n">
-        <v>59.85</v>
+        <v>60.48</v>
       </c>
       <c r="BQ64" t="n">
-        <v>38.94</v>
+        <v>39.11</v>
       </c>
       <c r="BR64" t="n">
-        <v>60.83</v>
+        <v>60.62</v>
       </c>
       <c r="BS64" t="n">
         <v>3.49</v>
       </c>
       <c r="BT64" t="n">
-        <v>12583835</v>
+        <v>12665342</v>
       </c>
     </row>
     <row r="65">
@@ -15283,13 +15283,13 @@
         </is>
       </c>
       <c r="F65" t="n">
-        <v>23.89</v>
+        <v>23.75</v>
       </c>
       <c r="G65" t="n">
-        <v>236998752694</v>
+        <v>235466795451</v>
       </c>
       <c r="H65" t="n">
-        <v>9900</v>
+        <v>3900</v>
       </c>
       <c r="I65" t="n">
         <v>7298813414</v>
@@ -15304,7 +15304,7 @@
         <v>3.29</v>
       </c>
       <c r="M65" t="n">
-        <v>5.729668308212404</v>
+        <v>5.692631797408119</v>
       </c>
       <c r="N65" t="n">
         <v>0.29</v>
@@ -15382,7 +15382,7 @@
         <v>11532125194.12</v>
       </c>
       <c r="AM65" t="n">
-        <v>17752715557.603</v>
+        <v>17637962206.06742</v>
       </c>
       <c r="AN65" t="n">
         <v>0.4734</v>
@@ -15423,7 +15423,7 @@
         <v>12.99</v>
       </c>
       <c r="AZ65" t="n">
-        <v>8.039999999999999</v>
+        <v>8</v>
       </c>
       <c r="BA65" t="n">
         <v>2.23</v>
@@ -15432,19 +15432,19 @@
         <v>3.47</v>
       </c>
       <c r="BC65" t="n">
-        <v>-33.4</v>
+        <v>-33.01</v>
       </c>
       <c r="BD65" t="n">
-        <v>-45.63</v>
+        <v>-45.3</v>
       </c>
       <c r="BE65" t="n">
         <v>-66.33</v>
       </c>
       <c r="BF65" t="n">
-        <v>-90.66</v>
+        <v>-90.61</v>
       </c>
       <c r="BG65" t="n">
-        <v>-85.48999999999999</v>
+        <v>-85.41</v>
       </c>
       <c r="BH65" t="n">
         <v>7.12</v>
@@ -15453,7 +15453,7 @@
         <v>0</v>
       </c>
       <c r="BJ65" t="n">
-        <v>23.89</v>
+        <v>23.75</v>
       </c>
       <c r="BK65" t="n">
         <v>1.58</v>
@@ -15462,7 +15462,7 @@
         <v>1.57</v>
       </c>
       <c r="BM65" t="n">
-        <v>23.9</v>
+        <v>24.08</v>
       </c>
       <c r="BN65" t="n">
         <v>46.43</v>
@@ -15471,19 +15471,19 @@
         <v>20.44</v>
       </c>
       <c r="BP65" t="n">
-        <v>23.63</v>
+        <v>23.66</v>
       </c>
       <c r="BQ65" t="n">
-        <v>15.22</v>
+        <v>15.13</v>
       </c>
       <c r="BR65" t="n">
-        <v>23.67</v>
+        <v>23.66</v>
       </c>
       <c r="BS65" t="n">
         <v>4.14</v>
       </c>
       <c r="BT65" t="n">
-        <v>11504</v>
+        <v>11531</v>
       </c>
     </row>
     <row r="66">
@@ -15513,13 +15513,13 @@
         </is>
       </c>
       <c r="F66" t="n">
-        <v>20.21</v>
+        <v>20.91</v>
       </c>
       <c r="G66" t="n">
-        <v>236998752694</v>
+        <v>235466795451</v>
       </c>
       <c r="H66" t="n">
-        <v>1500</v>
+        <v>600</v>
       </c>
       <c r="I66" t="n">
         <v>2972355254</v>
@@ -15534,7 +15534,7 @@
         <v>2.75</v>
       </c>
       <c r="M66" t="n">
-        <v>14.06957659232458</v>
+        <v>13.97863100918734</v>
       </c>
       <c r="N66" t="n">
         <v>0.25</v>
@@ -15612,7 +15612,7 @@
         <v>4696321301.320001</v>
       </c>
       <c r="AM66" t="n">
-        <v>21255493515.15695</v>
+        <v>21118098246.72646</v>
       </c>
       <c r="AN66" t="n">
         <v>0.4734</v>
@@ -15653,7 +15653,7 @@
         <v>12.99</v>
       </c>
       <c r="AZ66" t="n">
-        <v>8.119999999999999</v>
+        <v>8.4</v>
       </c>
       <c r="BA66" t="n">
         <v>2.23</v>
@@ -15662,19 +15662,19 @@
         <v>3.47</v>
       </c>
       <c r="BC66" t="n">
-        <v>-21.28</v>
+        <v>-23.91</v>
       </c>
       <c r="BD66" t="n">
-        <v>-35.72</v>
+        <v>-37.88</v>
       </c>
       <c r="BE66" t="n">
         <v>-59.83</v>
       </c>
       <c r="BF66" t="n">
-        <v>-88.95999999999999</v>
+        <v>-89.33</v>
       </c>
       <c r="BG66" t="n">
-        <v>-82.84999999999999</v>
+        <v>-83.43000000000001</v>
       </c>
       <c r="BH66" t="n">
         <v>7.12</v>
@@ -15683,7 +15683,7 @@
         <v>0</v>
       </c>
       <c r="BJ66" t="n">
-        <v>20.21</v>
+        <v>20.91</v>
       </c>
       <c r="BK66" t="n">
         <v>1.58</v>
@@ -15692,7 +15692,7 @@
         <v>1.57</v>
       </c>
       <c r="BM66" t="n">
-        <v>20.99</v>
+        <v>21</v>
       </c>
       <c r="BN66" t="n">
         <v>21.33</v>
@@ -15701,19 +15701,19 @@
         <v>9.48</v>
       </c>
       <c r="BP66" t="n">
-        <v>20.21</v>
+        <v>20.91</v>
       </c>
       <c r="BQ66" t="n">
-        <v>12.87</v>
+        <v>13.32</v>
       </c>
       <c r="BR66" t="n">
-        <v>20.97</v>
+        <v>20.99</v>
       </c>
       <c r="BS66" t="n">
         <v>3.46</v>
       </c>
       <c r="BT66" t="n">
-        <v>6330</v>
+        <v>6009</v>
       </c>
     </row>
     <row r="67">
@@ -15976,10 +15976,10 @@
         <v>18.51</v>
       </c>
       <c r="G68" t="n">
-        <v>8054439710</v>
+        <v>7943322285</v>
       </c>
       <c r="H68" t="n">
-        <v>46100</v>
+        <v>0</v>
       </c>
       <c r="I68" t="n">
         <v>137989898</v>
@@ -16072,7 +16072,7 @@
         <v>205604948.02</v>
       </c>
       <c r="AM68" t="n">
-        <v>558560312.7600554</v>
+        <v>550854527.3925104</v>
       </c>
       <c r="AN68" t="n">
         <v>0.1911</v>
@@ -16152,7 +16152,7 @@
         <v>1.49</v>
       </c>
       <c r="BM68" t="n">
-        <v>18.65</v>
+        <v>18.62</v>
       </c>
       <c r="BN68" t="n">
         <v>22.11</v>
@@ -16161,19 +16161,19 @@
         <v>15.39</v>
       </c>
       <c r="BP68" t="n">
-        <v>18.43</v>
+        <v>18.5</v>
       </c>
       <c r="BQ68" t="n">
         <v>12.45</v>
       </c>
       <c r="BR68" t="n">
-        <v>18.5</v>
+        <v>18.62</v>
       </c>
       <c r="BS68" t="n">
         <v>0</v>
       </c>
       <c r="BT68" t="n">
-        <v>34380</v>
+        <v>35050</v>
       </c>
     </row>
     <row r="69">
@@ -16203,13 +16203,13 @@
         </is>
       </c>
       <c r="F69" t="n">
-        <v>21.36</v>
+        <v>21.2</v>
       </c>
       <c r="G69" t="n">
-        <v>8054439710</v>
+        <v>7943322285</v>
       </c>
       <c r="H69" t="n">
-        <v>3324400</v>
+        <v>0</v>
       </c>
       <c r="I69" t="n">
         <v>255106712</v>
@@ -16302,7 +16302,7 @@
         <v>380109000.88</v>
       </c>
       <c r="AM69" t="n">
-        <v>479430935.1190476</v>
+        <v>472816802.6785714</v>
       </c>
       <c r="AN69" t="n">
         <v>0.8856000000000001</v>
@@ -16343,7 +16343,7 @@
         <v>21.39</v>
       </c>
       <c r="AZ69" t="n">
-        <v>37.34</v>
+        <v>37.06</v>
       </c>
       <c r="BA69" t="n">
         <v>1.24</v>
@@ -16352,25 +16352,25 @@
         <v>69.59</v>
       </c>
       <c r="BC69" t="n">
-        <v>22.67</v>
+        <v>23.6</v>
       </c>
       <c r="BD69" t="n">
-        <v>0.16</v>
+        <v>0.92</v>
       </c>
       <c r="BE69" t="n">
         <v>74.83</v>
       </c>
       <c r="BF69" t="n">
-        <v>-94.2</v>
+        <v>-94.15000000000001</v>
       </c>
       <c r="BG69" t="n">
-        <v>225.78</v>
+        <v>228.24</v>
       </c>
       <c r="BH69" t="n">
         <v>20.48</v>
       </c>
       <c r="BI69" t="n">
-        <v>0</v>
+        <v>-0.75</v>
       </c>
       <c r="BJ69" t="n">
         <v>21.36</v>
@@ -16382,7 +16382,7 @@
         <v>1.49</v>
       </c>
       <c r="BM69" t="n">
-        <v>21.36</v>
+        <v>21.28</v>
       </c>
       <c r="BN69" t="n">
         <v>25.63</v>
@@ -16391,19 +16391,19 @@
         <v>16.73</v>
       </c>
       <c r="BP69" t="n">
-        <v>20.81</v>
+        <v>21</v>
       </c>
       <c r="BQ69" t="n">
-        <v>14.37</v>
+        <v>14.26</v>
       </c>
       <c r="BR69" t="n">
-        <v>21.05</v>
+        <v>21.12</v>
       </c>
       <c r="BS69" t="n">
         <v>0</v>
       </c>
       <c r="BT69" t="n">
-        <v>1944550</v>
+        <v>2014377</v>
       </c>
     </row>
     <row r="70">
@@ -16433,13 +16433,13 @@
         </is>
       </c>
       <c r="F70" t="n">
-        <v>17.52</v>
+        <v>17.35</v>
       </c>
       <c r="G70" t="n">
-        <v>8139044108</v>
+        <v>8060067597</v>
       </c>
       <c r="H70" t="n">
-        <v>2811000</v>
+        <v>0</v>
       </c>
       <c r="I70" t="n">
         <v>464557268</v>
@@ -16454,7 +16454,7 @@
         <v>0.68</v>
       </c>
       <c r="M70" t="n">
-        <v>0.6424000609830807</v>
+        <v>0.6361665875174727</v>
       </c>
       <c r="N70" t="n">
         <v>0.2</v>
@@ -16532,7 +16532,7 @@
         <v>55746872.16</v>
       </c>
       <c r="AM70" t="n">
-        <v>2686153170.957096</v>
+        <v>2660088315.841584</v>
       </c>
       <c r="AN70" t="n">
         <v>0.1236</v>
@@ -16573,7 +16573,7 @@
         <v>6.9</v>
       </c>
       <c r="AZ70" t="n">
-        <v>2.01</v>
+        <v>2</v>
       </c>
       <c r="BA70" t="n">
         <v>0.12</v>
@@ -16582,19 +16582,19 @@
         <v>1.07</v>
       </c>
       <c r="BC70" t="n">
-        <v>-51.77</v>
+        <v>-51.3</v>
       </c>
       <c r="BD70" t="n">
-        <v>-60.62</v>
+        <v>-60.24</v>
       </c>
       <c r="BE70" t="n">
         <v>-88.5</v>
       </c>
       <c r="BF70" t="n">
-        <v>-99.31999999999999</v>
+        <v>-99.31</v>
       </c>
       <c r="BG70" t="n">
-        <v>-93.90000000000001</v>
+        <v>-93.84</v>
       </c>
       <c r="BH70" t="n">
         <v>26.44</v>
@@ -16603,7 +16603,7 @@
         <v>0</v>
       </c>
       <c r="BJ70" t="n">
-        <v>17.52</v>
+        <v>17.35</v>
       </c>
       <c r="BK70" t="n">
         <v>0.12</v>
@@ -16612,7 +16612,7 @@
         <v>0.1</v>
       </c>
       <c r="BM70" t="n">
-        <v>17.79</v>
+        <v>17.54</v>
       </c>
       <c r="BN70" t="n">
         <v>22.15</v>
@@ -16621,19 +16621,19 @@
         <v>13.21</v>
       </c>
       <c r="BP70" t="n">
+        <v>17.34</v>
+      </c>
+      <c r="BQ70" t="n">
+        <v>174</v>
+      </c>
+      <c r="BR70" t="n">
         <v>17.5</v>
-      </c>
-      <c r="BQ70" t="n">
-        <v>175.71</v>
-      </c>
-      <c r="BR70" t="n">
-        <v>17.61</v>
       </c>
       <c r="BS70" t="n">
         <v>0.67</v>
       </c>
       <c r="BT70" t="n">
-        <v>5101400</v>
+        <v>4576120</v>
       </c>
     </row>
     <row r="71">

</xml_diff>

<commit_message>
📊 Dados atualizados - 2026-09-21 05:43
</commit_message>
<xml_diff>
--- a/data/ativos.xlsx
+++ b/data/ativos.xlsx
@@ -11158,7 +11158,7 @@
         <v>8.93</v>
       </c>
       <c r="G47" t="n">
-        <v>3131580544</v>
+        <v>3115354000</v>
       </c>
       <c r="H47" t="n">
         <v>0</v>
@@ -11176,7 +11176,7 @@
         <v>1.22</v>
       </c>
       <c r="M47" t="n">
-        <v>0.7384627219238034</v>
+        <v>0.7346363161579945</v>
       </c>
       <c r="N47" t="n">
         <v>0.07000000000000001</v>
@@ -11254,7 +11254,7 @@
         <v>322715382</v>
       </c>
       <c r="AM47" t="n">
-        <v>555244777.3049645</v>
+        <v>552367730.4964539</v>
       </c>
       <c r="AN47" t="n">
         <v>0.4132</v>
@@ -11388,7 +11388,7 @@
         <v>9.06</v>
       </c>
       <c r="G48" t="n">
-        <v>3131580544</v>
+        <v>3115354000</v>
       </c>
       <c r="H48" t="n">
         <v>0</v>
@@ -11406,7 +11406,7 @@
         <v>1.24</v>
       </c>
       <c r="M48" t="n">
-        <v>2.009134709971964</v>
+        <v>1.998724212041215</v>
       </c>
       <c r="N48" t="n">
         <v>0.07000000000000001</v>
@@ -11484,7 +11484,7 @@
         <v>118614883.42</v>
       </c>
       <c r="AM48" t="n">
-        <v>547479116.0839161</v>
+        <v>544642307.6923077</v>
       </c>
       <c r="AN48" t="n">
         <v>0.4132</v>
@@ -11848,7 +11848,7 @@
         <v>33.44</v>
       </c>
       <c r="G50" t="n">
-        <v>956276500</v>
+        <v>961816100</v>
       </c>
       <c r="H50" t="n">
         <v>100</v>
@@ -11866,7 +11866,7 @@
         <v>0.8</v>
       </c>
       <c r="M50" t="n">
-        <v>0.9674526004937661</v>
+        <v>0.9730569423610977</v>
       </c>
       <c r="N50" t="n">
         <v>0.06</v>
@@ -11944,7 +11944,7 @@
         <v>84709985.8</v>
       </c>
       <c r="AM50" t="n">
-        <v>326374232.0819113</v>
+        <v>328264880.546075</v>
       </c>
       <c r="AN50" t="n">
         <v>4.4983</v>
@@ -13906,7 +13906,7 @@
         <v>20</v>
       </c>
       <c r="G59" t="n">
-        <v>94446470</v>
+        <v>96504000</v>
       </c>
       <c r="H59" t="n">
         <v>0</v>
@@ -13924,7 +13924,7 @@
         <v>0.61</v>
       </c>
       <c r="M59" t="n">
-        <v>10.03244621711721</v>
+        <v>10.25100450802109</v>
       </c>
       <c r="N59" t="n">
         <v>0.15</v>
@@ -14002,7 +14002,7 @@
         <v>1881878.95</v>
       </c>
       <c r="AM59" t="n">
-        <v>15953795.60810811</v>
+        <v>16301351.35135135</v>
       </c>
       <c r="AN59" t="n">
         <v>1.4</v>
@@ -14136,7 +14136,7 @@
         <v>376.92</v>
       </c>
       <c r="G60" t="n">
-        <v>171404376</v>
+        <v>171404400</v>
       </c>
       <c r="H60" t="n">
         <v>14</v>
@@ -14154,7 +14154,7 @@
         <v>0.83</v>
       </c>
       <c r="M60" t="n">
-        <v>12.82080603785775</v>
+        <v>12.82080783302397</v>
       </c>
       <c r="N60" t="n">
         <v>0.68</v>
@@ -14232,7 +14232,7 @@
         <v>59558607.5</v>
       </c>
       <c r="AM60" t="n">
-        <v>-25132606.4516129</v>
+        <v>-25132609.97067448</v>
       </c>
       <c r="AN60" t="n">
         <v>10.0581</v>

</xml_diff>

<commit_message>
📊 Dados atualizados - 2026-09-22 05:41
</commit_message>
<xml_diff>
--- a/data/ativos.xlsx
+++ b/data/ativos.xlsx
@@ -1047,13 +1047,13 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>24.8</v>
+        <v>25.28</v>
       </c>
       <c r="G3" t="n">
-        <v>3317416537</v>
+        <v>3381624795</v>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>583300</v>
       </c>
       <c r="I3" t="n">
         <v>129510368</v>
@@ -1068,7 +1068,7 @@
         <v>0.88</v>
       </c>
       <c r="M3" t="n">
-        <v>0.8254471179933391</v>
+        <v>0.8414235625930282</v>
       </c>
       <c r="N3" t="n">
         <v>0.09</v>
@@ -1146,7 +1146,7 @@
         <v>506385538.88</v>
       </c>
       <c r="AM3" t="n">
-        <v>647932917.3828125</v>
+        <v>660473592.7734375</v>
       </c>
       <c r="AN3" t="n">
         <v>2.7</v>
@@ -1187,7 +1187,7 @@
         <v>40.42</v>
       </c>
       <c r="AZ3" t="n">
-        <v>45.38</v>
+        <v>46.26</v>
       </c>
       <c r="BA3" t="n">
         <v>4.87</v>
@@ -1196,28 +1196,28 @@
         <v>21.14</v>
       </c>
       <c r="BC3" t="n">
-        <v>99.59</v>
+        <v>95.8</v>
       </c>
       <c r="BD3" t="n">
-        <v>62.97</v>
+        <v>59.87</v>
       </c>
       <c r="BE3" t="n">
         <v>83</v>
       </c>
       <c r="BF3" t="n">
-        <v>-80.37</v>
+        <v>-80.73999999999999</v>
       </c>
       <c r="BG3" t="n">
-        <v>-14.77</v>
+        <v>-16.39</v>
       </c>
       <c r="BH3" t="n">
         <v>27.85</v>
       </c>
       <c r="BI3" t="n">
-        <v>-0.68</v>
+        <v>0</v>
       </c>
       <c r="BJ3" t="n">
-        <v>24.97</v>
+        <v>25.28</v>
       </c>
       <c r="BK3" t="n">
         <v>3.91</v>
@@ -1226,7 +1226,7 @@
         <v>4.39</v>
       </c>
       <c r="BM3" t="n">
-        <v>24.95</v>
+        <v>25.4</v>
       </c>
       <c r="BN3" t="n">
         <v>27.17</v>
@@ -1235,19 +1235,19 @@
         <v>18.72</v>
       </c>
       <c r="BP3" t="n">
-        <v>24.7</v>
+        <v>24.85</v>
       </c>
       <c r="BQ3" t="n">
-        <v>5.65</v>
+        <v>5.75</v>
       </c>
       <c r="BR3" t="n">
-        <v>24.95</v>
+        <v>24.85</v>
       </c>
       <c r="BS3" t="n">
         <v>0.79</v>
       </c>
       <c r="BT3" t="n">
-        <v>514897</v>
+        <v>515463</v>
       </c>
     </row>
     <row r="4">
@@ -1277,13 +1277,13 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>15.38</v>
+        <v>15.5</v>
       </c>
       <c r="G4" t="n">
-        <v>238154072572</v>
+        <v>240012230000</v>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
+        <v>18020800</v>
       </c>
       <c r="I4" t="n">
         <v>15484664889</v>
@@ -1298,7 +1298,7 @@
         <v>2.76</v>
       </c>
       <c r="M4" t="n">
-        <v>2.69662583532048</v>
+        <v>2.717665808613074</v>
       </c>
       <c r="N4" t="n">
         <v>1.76</v>
@@ -1376,7 +1376,7 @@
         <v>16258898133.45</v>
       </c>
       <c r="AM4" t="n">
-        <v>23579611145.74258</v>
+        <v>23763587128.71287</v>
       </c>
       <c r="AN4" t="n">
         <v>0.269</v>
@@ -1417,7 +1417,7 @@
         <v>9.470000000000001</v>
       </c>
       <c r="AZ4" t="n">
-        <v>19.2</v>
+        <v>19.35</v>
       </c>
       <c r="BA4" t="n">
         <v>1.13</v>
@@ -1426,28 +1426,28 @@
         <v>11.39</v>
       </c>
       <c r="BC4" t="n">
-        <v>-24.55</v>
+        <v>-25.13</v>
       </c>
       <c r="BD4" t="n">
-        <v>-38.39</v>
+        <v>-38.87</v>
       </c>
       <c r="BE4" t="n">
         <v>24.83</v>
       </c>
       <c r="BF4" t="n">
-        <v>-92.67</v>
+        <v>-92.73</v>
       </c>
       <c r="BG4" t="n">
-        <v>-25.96</v>
+        <v>-26.54</v>
       </c>
       <c r="BH4" t="n">
         <v>5.7</v>
       </c>
       <c r="BI4" t="n">
-        <v>0</v>
+        <v>0.38</v>
       </c>
       <c r="BJ4" t="n">
-        <v>15.38</v>
+        <v>15.44</v>
       </c>
       <c r="BK4" t="n">
         <v>1.05</v>
@@ -1456,7 +1456,7 @@
         <v>1.04</v>
       </c>
       <c r="BM4" t="n">
-        <v>15.53</v>
+        <v>15.62</v>
       </c>
       <c r="BN4" t="n">
         <v>17</v>
@@ -1465,19 +1465,19 @@
         <v>11.09</v>
       </c>
       <c r="BP4" t="n">
-        <v>15.29</v>
+        <v>15.42</v>
       </c>
       <c r="BQ4" t="n">
-        <v>14.83</v>
+        <v>14.95</v>
       </c>
       <c r="BR4" t="n">
-        <v>15.47</v>
+        <v>15.48</v>
       </c>
       <c r="BS4" t="n">
         <v>2.76</v>
       </c>
       <c r="BT4" t="n">
-        <v>27757920</v>
+        <v>28016813</v>
       </c>
     </row>
     <row r="5">
@@ -1737,13 +1737,13 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>7.32</v>
+        <v>7.38</v>
       </c>
       <c r="G6" t="n">
-        <v>461779941</v>
+        <v>465565019</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="I6" t="n">
         <v>63084700</v>
@@ -1758,7 +1758,7 @@
         <v>1.91</v>
       </c>
       <c r="M6" t="n">
-        <v>7.189009545529139</v>
+        <v>7.247935799046444</v>
       </c>
       <c r="N6" t="n">
         <v>1.26</v>
@@ -1836,7 +1836,7 @@
         <v>35958279</v>
       </c>
       <c r="AM6" t="n">
-        <v>44147221.89292543</v>
+        <v>44509084.03441682</v>
       </c>
       <c r="AN6" t="n">
         <v>0.5199</v>
@@ -1877,7 +1877,7 @@
         <v>5.74</v>
       </c>
       <c r="AZ6" t="n">
-        <v>8.59</v>
+        <v>8.66</v>
       </c>
       <c r="BA6" t="n">
         <v>0.65</v>
@@ -1886,19 +1886,19 @@
         <v>7.95</v>
       </c>
       <c r="BC6" t="n">
-        <v>-3.88</v>
+        <v>-4.66</v>
       </c>
       <c r="BD6" t="n">
-        <v>-21.52</v>
+        <v>-22.16</v>
       </c>
       <c r="BE6" t="n">
         <v>17.33</v>
       </c>
       <c r="BF6" t="n">
-        <v>-91.14</v>
+        <v>-91.20999999999999</v>
       </c>
       <c r="BG6" t="n">
-        <v>8.66</v>
+        <v>7.77</v>
       </c>
       <c r="BH6" t="n">
         <v>3.86</v>
@@ -1907,7 +1907,7 @@
         <v>0</v>
       </c>
       <c r="BJ6" t="n">
-        <v>7.32</v>
+        <v>7.38</v>
       </c>
       <c r="BK6" t="n">
         <v>0.57</v>
@@ -1916,7 +1916,7 @@
         <v>0.5600000000000001</v>
       </c>
       <c r="BM6" t="n">
-        <v>7.32</v>
+        <v>7.38</v>
       </c>
       <c r="BN6" t="n">
         <v>8.16</v>
@@ -1925,19 +1925,19 @@
         <v>6.22</v>
       </c>
       <c r="BP6" t="n">
-        <v>7.32</v>
+        <v>7.37</v>
       </c>
       <c r="BQ6" t="n">
-        <v>13.02</v>
+        <v>13.12</v>
       </c>
       <c r="BR6" t="n">
-        <v>7.32</v>
+        <v>7.37</v>
       </c>
       <c r="BS6" t="n">
         <v>7.32</v>
       </c>
       <c r="BT6" t="n">
-        <v>283</v>
+        <v>230</v>
       </c>
     </row>
     <row r="7">
@@ -3117,13 +3117,13 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>5.05</v>
+        <v>5.01</v>
       </c>
       <c r="G12" t="n">
-        <v>484605795</v>
+        <v>480767337</v>
       </c>
       <c r="H12" t="n">
-        <v>370400</v>
+        <v>457100</v>
       </c>
       <c r="I12" t="n">
         <v>95961536</v>
@@ -3138,7 +3138,7 @@
         <v>0.32</v>
       </c>
       <c r="M12" t="n">
-        <v>0.08764021854862333</v>
+        <v>0.08694603927656219</v>
       </c>
       <c r="N12" t="n">
         <v>0.14</v>
@@ -3216,7 +3216,7 @@
         <v>362734606.08</v>
       </c>
       <c r="AM12" t="n">
-        <v>521081500</v>
+        <v>516954125.8064516</v>
       </c>
       <c r="AN12" t="n">
         <v>0.4208</v>
@@ -3257,7 +3257,7 @@
         <v>30.49</v>
       </c>
       <c r="AZ12" t="n">
-        <v>6.83</v>
+        <v>6.77</v>
       </c>
       <c r="BA12" t="n">
         <v>4.41</v>
@@ -3266,19 +3266,19 @@
         <v>18.12</v>
       </c>
       <c r="BC12" t="n">
-        <v>639.55</v>
+        <v>645.45</v>
       </c>
       <c r="BD12" t="n">
-        <v>503.84</v>
+        <v>508.66</v>
       </c>
       <c r="BE12" t="n">
         <v>35.17</v>
       </c>
       <c r="BF12" t="n">
-        <v>-12.64</v>
+        <v>-11.94</v>
       </c>
       <c r="BG12" t="n">
-        <v>258.79</v>
+        <v>261.65</v>
       </c>
       <c r="BH12" t="n">
         <v>16.4</v>
@@ -3287,7 +3287,7 @@
         <v>0</v>
       </c>
       <c r="BJ12" t="n">
-        <v>5.05</v>
+        <v>5.01</v>
       </c>
       <c r="BK12" t="n">
         <v>3.78</v>
@@ -3296,7 +3296,7 @@
         <v>3.43</v>
       </c>
       <c r="BM12" t="n">
-        <v>5.07</v>
+        <v>5.08</v>
       </c>
       <c r="BN12" t="n">
         <v>8.23</v>
@@ -3308,16 +3308,16 @@
         <v>4.96</v>
       </c>
       <c r="BQ12" t="n">
-        <v>1.47</v>
+        <v>1.46</v>
       </c>
       <c r="BR12" t="n">
-        <v>5.07</v>
+        <v>5.05</v>
       </c>
       <c r="BS12" t="n">
         <v>0.09</v>
       </c>
       <c r="BT12" t="n">
-        <v>509497</v>
+        <v>514337</v>
       </c>
     </row>
     <row r="13">
@@ -3347,13 +3347,13 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>28.87</v>
+        <v>29.7</v>
       </c>
       <c r="G13" t="n">
-        <v>14555988819</v>
+        <v>14974467144</v>
       </c>
       <c r="H13" t="n">
-        <v>0</v>
+        <v>5891600</v>
       </c>
       <c r="I13" t="n">
         <v>504190947</v>
@@ -3368,7 +3368,7 @@
         <v>1.13</v>
       </c>
       <c r="M13" t="n">
-        <v>5.034302462299124</v>
+        <v>5.179036460666611</v>
       </c>
       <c r="N13" t="n">
         <v>0.57</v>
@@ -3446,7 +3446,7 @@
         <v>932753251.95</v>
       </c>
       <c r="AM13" t="n">
-        <v>1514671052.965661</v>
+        <v>1558217184.599376</v>
       </c>
       <c r="AN13" t="n">
         <v>2.6301</v>
@@ -3487,7 +3487,7 @@
         <v>26.6</v>
       </c>
       <c r="AZ13" t="n">
-        <v>52.25</v>
+        <v>53.76</v>
       </c>
       <c r="BA13" t="n">
         <v>2.6</v>
@@ -3496,19 +3496,19 @@
         <v>8.69</v>
       </c>
       <c r="BC13" t="n">
-        <v>12.83</v>
+        <v>9.67</v>
       </c>
       <c r="BD13" t="n">
-        <v>-7.88</v>
+        <v>-10.45</v>
       </c>
       <c r="BE13" t="n">
         <v>81</v>
       </c>
       <c r="BF13" t="n">
-        <v>-90.98</v>
+        <v>-91.23</v>
       </c>
       <c r="BG13" t="n">
-        <v>-69.89</v>
+        <v>-70.73</v>
       </c>
       <c r="BH13" t="n">
         <v>25.49</v>
@@ -3517,7 +3517,7 @@
         <v>0</v>
       </c>
       <c r="BJ13" t="n">
-        <v>28.87</v>
+        <v>29.7</v>
       </c>
       <c r="BK13" t="n">
         <v>1.85</v>
@@ -3526,7 +3526,7 @@
         <v>1.96</v>
       </c>
       <c r="BM13" t="n">
-        <v>28.87</v>
+        <v>29.87</v>
       </c>
       <c r="BN13" t="n">
         <v>32.43</v>
@@ -3535,19 +3535,19 @@
         <v>21.06</v>
       </c>
       <c r="BP13" t="n">
-        <v>28.05</v>
+        <v>29.01</v>
       </c>
       <c r="BQ13" t="n">
-        <v>14.75</v>
+        <v>15.17</v>
       </c>
       <c r="BR13" t="n">
-        <v>28.15</v>
+        <v>29.01</v>
       </c>
       <c r="BS13" t="n">
         <v>5.01</v>
       </c>
       <c r="BT13" t="n">
-        <v>4784913</v>
+        <v>4780353</v>
       </c>
     </row>
     <row r="14">
@@ -3577,13 +3577,13 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>9.539999999999999</v>
+        <v>9.640000000000001</v>
       </c>
       <c r="G14" t="n">
-        <v>7732824181</v>
+        <v>7832120285</v>
       </c>
       <c r="H14" t="n">
-        <v>14800</v>
+        <v>9300</v>
       </c>
       <c r="I14" t="n">
         <v>339510689</v>
@@ -3598,7 +3598,7 @@
         <v>1.92</v>
       </c>
       <c r="M14" t="n">
-        <v>3.210806071652822</v>
+        <v>3.252035579288342</v>
       </c>
       <c r="N14" t="n">
         <v>1.11</v>
@@ -3676,7 +3676,7 @@
         <v>349696009.67</v>
       </c>
       <c r="AM14" t="n">
-        <v>858249076.6925639</v>
+        <v>869269731.964484</v>
       </c>
       <c r="AN14" t="n">
         <v>0.1489</v>
@@ -3717,7 +3717,7 @@
         <v>9.050000000000001</v>
       </c>
       <c r="AZ14" t="n">
-        <v>7.66</v>
+        <v>7.74</v>
       </c>
       <c r="BA14" t="n">
         <v>1.42</v>
@@ -3726,19 +3726,19 @@
         <v>5.94</v>
       </c>
       <c r="BC14" t="n">
-        <v>16.17</v>
+        <v>14.97</v>
       </c>
       <c r="BD14" t="n">
-        <v>-5.15</v>
+        <v>-6.13</v>
       </c>
       <c r="BE14" t="n">
         <v>-19.67</v>
       </c>
       <c r="BF14" t="n">
-        <v>-85.09999999999999</v>
+        <v>-85.26000000000001</v>
       </c>
       <c r="BG14" t="n">
-        <v>-37.71</v>
+        <v>-38.36</v>
       </c>
       <c r="BH14" t="n">
         <v>5.3</v>
@@ -3747,7 +3747,7 @@
         <v>0</v>
       </c>
       <c r="BJ14" t="n">
-        <v>9.539999999999999</v>
+        <v>9.640000000000001</v>
       </c>
       <c r="BK14" t="n">
         <v>1.03</v>
@@ -3756,7 +3756,7 @@
         <v>1.01</v>
       </c>
       <c r="BM14" t="n">
-        <v>9.75</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="BN14" t="n">
         <v>13.49</v>
@@ -3768,16 +3768,16 @@
         <v>9.539999999999999</v>
       </c>
       <c r="BQ14" t="n">
-        <v>9.42</v>
+        <v>9.52</v>
       </c>
       <c r="BR14" t="n">
-        <v>9.640000000000001</v>
+        <v>9.539999999999999</v>
       </c>
       <c r="BS14" t="n">
         <v>1.44</v>
       </c>
       <c r="BT14" t="n">
-        <v>12083</v>
+        <v>12480</v>
       </c>
     </row>
     <row r="15">
@@ -3807,13 +3807,13 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>12.92</v>
+        <v>13.18</v>
       </c>
       <c r="G15" t="n">
-        <v>7732824181</v>
+        <v>7832120285</v>
       </c>
       <c r="H15" t="n">
-        <v>0</v>
+        <v>1214600</v>
       </c>
       <c r="I15" t="n">
         <v>343551533</v>
@@ -3828,7 +3828,7 @@
         <v>2.56</v>
       </c>
       <c r="M15" t="n">
-        <v>3.173040655977026</v>
+        <v>3.213785223239563</v>
       </c>
       <c r="N15" t="n">
         <v>1.47</v>
@@ -3906,7 +3906,7 @@
         <v>353858078.99</v>
       </c>
       <c r="AM15" t="n">
-        <v>644939464.6371976</v>
+        <v>653221041.2844037</v>
       </c>
       <c r="AN15" t="n">
         <v>0.1638</v>
@@ -3947,7 +3947,7 @@
         <v>9.050000000000001</v>
       </c>
       <c r="AZ15" t="n">
-        <v>8.59</v>
+        <v>8.76</v>
       </c>
       <c r="BA15" t="n">
         <v>1.42</v>
@@ -3956,19 +3956,19 @@
         <v>6.19</v>
       </c>
       <c r="BC15" t="n">
-        <v>-14.22</v>
+        <v>-15.91</v>
       </c>
       <c r="BD15" t="n">
-        <v>-29.96</v>
+        <v>-31.34</v>
       </c>
       <c r="BE15" t="n">
         <v>-33.5</v>
       </c>
       <c r="BF15" t="n">
-        <v>-89</v>
+        <v>-89.22</v>
       </c>
       <c r="BG15" t="n">
-        <v>-52.1</v>
+        <v>-53.05</v>
       </c>
       <c r="BH15" t="n">
         <v>5.3</v>
@@ -3977,7 +3977,7 @@
         <v>0</v>
       </c>
       <c r="BJ15" t="n">
-        <v>12.92</v>
+        <v>13.18</v>
       </c>
       <c r="BK15" t="n">
         <v>1.03</v>
@@ -3986,7 +3986,7 @@
         <v>1.01</v>
       </c>
       <c r="BM15" t="n">
-        <v>13.17</v>
+        <v>13.28</v>
       </c>
       <c r="BN15" t="n">
         <v>16.22</v>
@@ -3995,19 +3995,19 @@
         <v>7.84</v>
       </c>
       <c r="BP15" t="n">
-        <v>12.68</v>
+        <v>12.9</v>
       </c>
       <c r="BQ15" t="n">
-        <v>12.76</v>
+        <v>13.01</v>
       </c>
       <c r="BR15" t="n">
-        <v>12.76</v>
+        <v>13</v>
       </c>
       <c r="BS15" t="n">
         <v>1.92</v>
       </c>
       <c r="BT15" t="n">
-        <v>2482773</v>
+        <v>2560813</v>
       </c>
     </row>
     <row r="16">
@@ -4037,13 +4037,13 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>4.35</v>
+        <v>4.4</v>
       </c>
       <c r="G16" t="n">
-        <v>953979774</v>
+        <v>964945100</v>
       </c>
       <c r="H16" t="n">
-        <v>113400</v>
+        <v>61400</v>
       </c>
       <c r="I16" t="n">
         <v>219305733</v>
@@ -4058,7 +4058,7 @@
         <v>2.69</v>
       </c>
       <c r="M16" t="n">
-        <v>0.4513124221540528</v>
+        <v>0.4564999407699022</v>
       </c>
       <c r="N16" t="n">
         <v>0.39</v>
@@ -4136,7 +4136,7 @@
         <v>17544458.64</v>
       </c>
       <c r="AM16" t="n">
-        <v>267971846.6292135</v>
+        <v>271051994.3820224</v>
       </c>
       <c r="AN16" t="n">
         <v>0.0077</v>
@@ -4186,16 +4186,16 @@
         <v>0</v>
       </c>
       <c r="BC16" t="n">
-        <v>-60.02</v>
+        <v>-60.48</v>
       </c>
       <c r="BD16" t="n">
-        <v>-67.36</v>
+        <v>-67.73</v>
       </c>
       <c r="BE16" t="n">
         <v>-97.17</v>
       </c>
       <c r="BF16" t="n">
-        <v>-98.16</v>
+        <v>-98.18000000000001</v>
       </c>
       <c r="BG16" t="n">
         <v>-100</v>
@@ -4207,7 +4207,7 @@
         <v>0</v>
       </c>
       <c r="BJ16" t="n">
-        <v>4.35</v>
+        <v>4.4</v>
       </c>
       <c r="BK16" t="n">
         <v>0.08</v>
@@ -4216,19 +4216,19 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="BM16" t="n">
-        <v>4.39</v>
+        <v>4.44</v>
       </c>
       <c r="BN16" t="n">
         <v>5.54</v>
       </c>
       <c r="BO16" t="n">
-        <v>3.14</v>
+        <v>3.19</v>
       </c>
       <c r="BP16" t="n">
-        <v>4.23</v>
+        <v>4.28</v>
       </c>
       <c r="BQ16" t="n">
-        <v>59.36</v>
+        <v>60.04</v>
       </c>
       <c r="BR16" t="n">
         <v>4.35</v>
@@ -4237,7 +4237,7 @@
         <v>0.49</v>
       </c>
       <c r="BT16" t="n">
-        <v>144607</v>
+        <v>140537</v>
       </c>
     </row>
     <row r="17">
@@ -4267,13 +4267,13 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>32.7</v>
+        <v>32.65</v>
       </c>
       <c r="G17" t="n">
-        <v>10778799881</v>
+        <v>10762318787</v>
       </c>
       <c r="H17" t="n">
-        <v>0</v>
+        <v>1650300</v>
       </c>
       <c r="I17" t="n">
         <v>0</v>
@@ -4360,13 +4360,13 @@
         <v>8.039999999999999</v>
       </c>
       <c r="AK17" t="n">
-        <v>4867593876.896676</v>
+        <v>4860151186.325868</v>
       </c>
       <c r="AL17" t="n">
-        <v>1347349985.125</v>
+        <v>1345289848.375</v>
       </c>
       <c r="AM17" t="n">
-        <v>3337089746.439629</v>
+        <v>3331987240.557276</v>
       </c>
       <c r="AN17" t="n">
         <v>1.08</v>
@@ -4407,7 +4407,7 @@
         <v>42.98</v>
       </c>
       <c r="AZ17" t="n">
-        <v>17.49</v>
+        <v>17.47</v>
       </c>
       <c r="BA17" t="n">
         <v>4.55</v>
@@ -4416,19 +4416,19 @@
         <v>16.33</v>
       </c>
       <c r="BC17" t="n">
-        <v>60.97</v>
+        <v>61.22</v>
       </c>
       <c r="BD17" t="n">
-        <v>31.43</v>
+        <v>31.63</v>
       </c>
       <c r="BE17" t="n">
         <v>-46.5</v>
       </c>
       <c r="BF17" t="n">
-        <v>-86.09</v>
+        <v>-86.06999999999999</v>
       </c>
       <c r="BG17" t="n">
-        <v>-50.05</v>
+        <v>-49.97</v>
       </c>
       <c r="BH17" t="n">
         <v>29.25</v>
@@ -4437,7 +4437,7 @@
         <v>0</v>
       </c>
       <c r="BJ17" t="n">
-        <v>32.7</v>
+        <v>32.65</v>
       </c>
       <c r="BK17" t="n">
         <v>4.21</v>
@@ -4446,28 +4446,28 @@
         <v>12.62</v>
       </c>
       <c r="BM17" t="n">
-        <v>33.41</v>
+        <v>33.26</v>
       </c>
       <c r="BN17" t="n">
         <v>36.63</v>
       </c>
       <c r="BO17" t="n">
-        <v>29.52</v>
+        <v>29.53</v>
       </c>
       <c r="BP17" t="n">
-        <v>32.7</v>
+        <v>32.65</v>
       </c>
       <c r="BQ17" t="n">
         <v>2.59</v>
       </c>
       <c r="BR17" t="n">
-        <v>33.25</v>
+        <v>32.81</v>
       </c>
       <c r="BS17" t="n">
         <v>2.21</v>
       </c>
       <c r="BT17" t="n">
-        <v>1069405</v>
+        <v>1146901</v>
       </c>
     </row>
     <row r="18">
@@ -4497,13 +4497,13 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>11.37</v>
+        <v>11.2</v>
       </c>
       <c r="G18" t="n">
-        <v>10778799881</v>
+        <v>10762318787</v>
       </c>
       <c r="H18" t="n">
-        <v>0</v>
+        <v>8500</v>
       </c>
       <c r="I18" t="n">
         <v>671494278</v>
@@ -4518,7 +4518,7 @@
         <v>1.2</v>
       </c>
       <c r="M18" t="n">
-        <v>3.173701979526239</v>
+        <v>3.168849298223123</v>
       </c>
       <c r="N18" t="n">
         <v>0.33</v>
@@ -4596,7 +4596,7 @@
         <v>940091989.1999999</v>
       </c>
       <c r="AM18" t="n">
-        <v>3207976155.059524</v>
+        <v>3203071067.559524</v>
       </c>
       <c r="AN18" t="n">
         <v>0.36</v>
@@ -4637,7 +4637,7 @@
         <v>14.31</v>
       </c>
       <c r="AZ18" t="n">
-        <v>5.86</v>
+        <v>5.77</v>
       </c>
       <c r="BA18" t="n">
         <v>1.51</v>
@@ -4646,28 +4646,28 @@
         <v>5.44</v>
       </c>
       <c r="BC18" t="n">
-        <v>54.13</v>
+        <v>56.47</v>
       </c>
       <c r="BD18" t="n">
-        <v>25.85</v>
+        <v>27.76</v>
       </c>
       <c r="BE18" t="n">
         <v>-48.5</v>
       </c>
       <c r="BF18" t="n">
-        <v>-86.7</v>
+        <v>-86.5</v>
       </c>
       <c r="BG18" t="n">
-        <v>-52.12</v>
+        <v>-51.39</v>
       </c>
       <c r="BH18" t="n">
         <v>9.75</v>
       </c>
       <c r="BI18" t="n">
-        <v>0.62</v>
+        <v>0</v>
       </c>
       <c r="BJ18" t="n">
-        <v>11.3</v>
+        <v>11.2</v>
       </c>
       <c r="BK18" t="n">
         <v>1.4</v>
@@ -4676,7 +4676,7 @@
         <v>12.62</v>
       </c>
       <c r="BM18" t="n">
-        <v>11.37</v>
+        <v>11.39</v>
       </c>
       <c r="BN18" t="n">
         <v>13.82</v>
@@ -4685,19 +4685,19 @@
         <v>10.19</v>
       </c>
       <c r="BP18" t="n">
-        <v>11.3</v>
+        <v>11.2</v>
       </c>
       <c r="BQ18" t="n">
-        <v>0.9</v>
+        <v>0.89</v>
       </c>
       <c r="BR18" t="n">
-        <v>11.3</v>
+        <v>11.39</v>
       </c>
       <c r="BS18" t="n">
         <v>2.3</v>
       </c>
       <c r="BT18" t="n">
-        <v>10071</v>
+        <v>10003</v>
       </c>
     </row>
     <row r="19">
@@ -4727,13 +4727,13 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>10.9</v>
+        <v>10.91</v>
       </c>
       <c r="G19" t="n">
-        <v>10778799881</v>
+        <v>10762318787</v>
       </c>
       <c r="H19" t="n">
-        <v>6600</v>
+        <v>8800</v>
       </c>
       <c r="I19" t="n">
         <v>317386323</v>
@@ -4748,7 +4748,7 @@
         <v>1.12</v>
       </c>
       <c r="M19" t="n">
-        <v>6.714601622355173</v>
+        <v>6.70433480399577</v>
       </c>
       <c r="N19" t="n">
         <v>0.3</v>
@@ -4826,7 +4826,7 @@
         <v>444340852.2</v>
       </c>
       <c r="AM19" t="n">
-        <v>3421841232.063492</v>
+        <v>3416609138.730159</v>
       </c>
       <c r="AN19" t="n">
         <v>0.36</v>
@@ -4876,19 +4876,19 @@
         <v>5.25</v>
       </c>
       <c r="BC19" t="n">
-        <v>60.78</v>
+        <v>60.63</v>
       </c>
       <c r="BD19" t="n">
-        <v>31.28</v>
+        <v>31.16</v>
       </c>
       <c r="BE19" t="n">
         <v>-45</v>
       </c>
       <c r="BF19" t="n">
-        <v>-86.12</v>
+        <v>-86.14</v>
       </c>
       <c r="BG19" t="n">
-        <v>-51.83</v>
+        <v>-51.88</v>
       </c>
       <c r="BH19" t="n">
         <v>9.75</v>
@@ -4897,7 +4897,7 @@
         <v>0</v>
       </c>
       <c r="BJ19" t="n">
-        <v>10.9</v>
+        <v>10.91</v>
       </c>
       <c r="BK19" t="n">
         <v>1.4</v>
@@ -4906,7 +4906,7 @@
         <v>12.62</v>
       </c>
       <c r="BM19" t="n">
-        <v>11.03</v>
+        <v>10.99</v>
       </c>
       <c r="BN19" t="n">
         <v>11.41</v>
@@ -4915,19 +4915,19 @@
         <v>9.19</v>
       </c>
       <c r="BP19" t="n">
-        <v>10.84</v>
+        <v>10.75</v>
       </c>
       <c r="BQ19" t="n">
         <v>0.86</v>
       </c>
       <c r="BR19" t="n">
-        <v>10.91</v>
+        <v>10.75</v>
       </c>
       <c r="BS19" t="n">
         <v>2.16</v>
       </c>
       <c r="BT19" t="n">
-        <v>13511</v>
+        <v>13312</v>
       </c>
     </row>
     <row r="20">
@@ -5417,13 +5417,13 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>4.74</v>
+        <v>5.02</v>
       </c>
       <c r="G22" t="n">
-        <v>949162676</v>
+        <v>1005230900</v>
       </c>
       <c r="H22" t="n">
-        <v>0</v>
+        <v>829100</v>
       </c>
       <c r="I22" t="n">
         <v>200245299</v>
@@ -5438,7 +5438,7 @@
         <v>0.27</v>
       </c>
       <c r="M22" t="n">
-        <v>0.08050475840522867</v>
+        <v>0.0852602749688933</v>
       </c>
       <c r="N22" t="n">
         <v>0.08</v>
@@ -5516,7 +5516,7 @@
         <v>378463615.11</v>
       </c>
       <c r="AM22" t="n">
-        <v>215229631.7460317</v>
+        <v>227943514.739229</v>
       </c>
       <c r="AN22" t="n">
         <v>0</v>
@@ -5566,19 +5566,19 @@
         <v>172.49</v>
       </c>
       <c r="BC22" t="n">
-        <v>526.6900000000001</v>
+        <v>491.74</v>
       </c>
       <c r="BD22" t="n">
-        <v>411.69</v>
+        <v>383.15</v>
       </c>
       <c r="BE22" t="n">
         <v>-100</v>
       </c>
       <c r="BF22" t="n">
-        <v>-60.13</v>
+        <v>-62.35</v>
       </c>
       <c r="BG22" t="n">
-        <v>3539.02</v>
+        <v>3336.05</v>
       </c>
       <c r="BH22" t="n">
         <v>20.75</v>
@@ -5587,7 +5587,7 @@
         <v>0</v>
       </c>
       <c r="BJ22" t="n">
-        <v>4.74</v>
+        <v>5.02</v>
       </c>
       <c r="BK22" t="n">
         <v>1.89</v>
@@ -5596,28 +5596,28 @@
         <v>0.67</v>
       </c>
       <c r="BM22" t="n">
-        <v>4.95</v>
+        <v>5.02</v>
       </c>
       <c r="BN22" t="n">
-        <v>8.279999999999999</v>
+        <v>7.89</v>
       </c>
       <c r="BO22" t="n">
         <v>3.37</v>
       </c>
       <c r="BP22" t="n">
-        <v>4.66</v>
+        <v>4.8</v>
       </c>
       <c r="BQ22" t="n">
-        <v>7.06</v>
+        <v>7.48</v>
       </c>
       <c r="BR22" t="n">
-        <v>4.94</v>
+        <v>4.87</v>
       </c>
       <c r="BS22" t="n">
         <v>0.09</v>
       </c>
       <c r="BT22" t="n">
-        <v>1561730</v>
+        <v>1565410</v>
       </c>
     </row>
     <row r="23">
@@ -5877,13 +5877,13 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.87</v>
+        <v>2.96</v>
       </c>
       <c r="G24" t="n">
-        <v>1159103409</v>
+        <v>1195451959</v>
       </c>
       <c r="H24" t="n">
-        <v>0</v>
+        <v>4018900</v>
       </c>
       <c r="I24" t="n">
         <v>403868805</v>
@@ -5898,7 +5898,7 @@
         <v>0.49</v>
       </c>
       <c r="M24" t="n">
-        <v>0.2802026167481476</v>
+        <v>0.2889895452878435</v>
       </c>
       <c r="N24" t="n">
         <v>0.11</v>
@@ -5976,7 +5976,7 @@
         <v>153470145.9</v>
       </c>
       <c r="AM24" t="n">
-        <v>1044237305.405405</v>
+        <v>1076983746.846847</v>
       </c>
       <c r="AN24" t="n">
         <v>0.0813</v>
@@ -6017,7 +6017,7 @@
         <v>5.84</v>
       </c>
       <c r="AZ24" t="n">
-        <v>1.32</v>
+        <v>1.37</v>
       </c>
       <c r="BA24" t="n">
         <v>0.38</v>
@@ -6026,19 +6026,19 @@
         <v>1.46</v>
       </c>
       <c r="BC24" t="n">
-        <v>149.35</v>
+        <v>141.77</v>
       </c>
       <c r="BD24" t="n">
-        <v>103.6</v>
+        <v>97.41</v>
       </c>
       <c r="BE24" t="n">
         <v>-53.83</v>
       </c>
       <c r="BF24" t="n">
-        <v>-86.76000000000001</v>
+        <v>-87.16</v>
       </c>
       <c r="BG24" t="n">
-        <v>-49.21</v>
+        <v>-50.75</v>
       </c>
       <c r="BH24" t="n">
         <v>5.99</v>
@@ -6047,7 +6047,7 @@
         <v>0</v>
       </c>
       <c r="BJ24" t="n">
-        <v>2.87</v>
+        <v>2.96</v>
       </c>
       <c r="BK24" t="n">
         <v>0.38</v>
@@ -6056,7 +6056,7 @@
         <v>0.41</v>
       </c>
       <c r="BM24" t="n">
-        <v>2.91</v>
+        <v>2.97</v>
       </c>
       <c r="BN24" t="n">
         <v>5.29</v>
@@ -6065,19 +6065,19 @@
         <v>1.92</v>
       </c>
       <c r="BP24" t="n">
-        <v>2.75</v>
+        <v>2.86</v>
       </c>
       <c r="BQ24" t="n">
-        <v>7.05</v>
+        <v>7.27</v>
       </c>
       <c r="BR24" t="n">
-        <v>2.86</v>
+        <v>2.88</v>
       </c>
       <c r="BS24" t="n">
         <v>0.29</v>
       </c>
       <c r="BT24" t="n">
-        <v>8506603</v>
+        <v>8447850</v>
       </c>
     </row>
     <row r="25">
@@ -6107,13 +6107,13 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>4.07</v>
+        <v>4.54</v>
       </c>
       <c r="G25" t="n">
-        <v>1410231453</v>
+        <v>1573083200</v>
       </c>
       <c r="H25" t="n">
-        <v>0</v>
+        <v>1673400</v>
       </c>
       <c r="I25" t="n">
         <v>346494097</v>
@@ -6128,7 +6128,7 @@
         <v>0.97</v>
       </c>
       <c r="M25" t="n">
-        <v>0.7032057940128967</v>
+        <v>0.7844111109216257</v>
       </c>
       <c r="N25" t="n">
         <v>0.22</v>
@@ -6206,7 +6206,7 @@
         <v>62368937.46</v>
       </c>
       <c r="AM25" t="n">
-        <v>518467445.9558823</v>
+        <v>578339411.7647059</v>
       </c>
       <c r="AN25" t="n">
         <v>0.4742</v>
@@ -6247,7 +6247,7 @@
         <v>3.27</v>
       </c>
       <c r="AZ25" t="n">
-        <v>9.48</v>
+        <v>10.58</v>
       </c>
       <c r="BA25" t="n">
         <v>0.23</v>
@@ -6256,28 +6256,28 @@
         <v>2.2</v>
       </c>
       <c r="BC25" t="n">
-        <v>-1.48</v>
+        <v>-11.68</v>
       </c>
       <c r="BD25" t="n">
-        <v>-19.56</v>
+        <v>-27.89</v>
       </c>
       <c r="BE25" t="n">
         <v>133</v>
       </c>
       <c r="BF25" t="n">
-        <v>-94.31</v>
+        <v>-94.90000000000001</v>
       </c>
       <c r="BG25" t="n">
-        <v>-45.95</v>
+        <v>-51.55</v>
       </c>
       <c r="BH25" t="n">
         <v>3.97</v>
       </c>
       <c r="BI25" t="n">
-        <v>2.52</v>
+        <v>0</v>
       </c>
       <c r="BJ25" t="n">
-        <v>3.97</v>
+        <v>4.54</v>
       </c>
       <c r="BK25" t="n">
         <v>0.18</v>
@@ -6286,7 +6286,7 @@
         <v>0.24</v>
       </c>
       <c r="BM25" t="n">
-        <v>4.1</v>
+        <v>4.54</v>
       </c>
       <c r="BN25" t="n">
         <v>6.3</v>
@@ -6295,19 +6295,19 @@
         <v>2.64</v>
       </c>
       <c r="BP25" t="n">
-        <v>3.85</v>
+        <v>4.07</v>
       </c>
       <c r="BQ25" t="n">
-        <v>17.2</v>
+        <v>19.18</v>
       </c>
       <c r="BR25" t="n">
-        <v>3.97</v>
+        <v>4.12</v>
       </c>
       <c r="BS25" t="n">
         <v>0.67</v>
       </c>
       <c r="BT25" t="n">
-        <v>1255643</v>
+        <v>1266297</v>
       </c>
     </row>
     <row r="26">
@@ -6337,13 +6337,13 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>10.26</v>
+        <v>10.22</v>
       </c>
       <c r="G26" t="n">
-        <v>13896072489</v>
+        <v>13841896821</v>
       </c>
       <c r="H26" t="n">
-        <v>0</v>
+        <v>6225700</v>
       </c>
       <c r="I26" t="n">
         <v>1354393401</v>
@@ -6358,7 +6358,7 @@
         <v>1.94</v>
       </c>
       <c r="M26" t="n">
-        <v>0.1791886833258593</v>
+        <v>0.1784900926539336</v>
       </c>
       <c r="N26" t="n">
         <v>0.26</v>
@@ -6436,7 +6436,7 @@
         <v>961619314.7099999</v>
       </c>
       <c r="AM26" t="n">
-        <v>4962883031.785714</v>
+        <v>4943534578.928572</v>
       </c>
       <c r="AN26" t="n">
         <v>0.1043</v>
@@ -6477,7 +6477,7 @@
         <v>7.07</v>
       </c>
       <c r="AZ26" t="n">
-        <v>1.97</v>
+        <v>1.96</v>
       </c>
       <c r="BA26" t="n">
         <v>0.66</v>
@@ -6486,19 +6486,19 @@
         <v>1.19</v>
       </c>
       <c r="BC26" t="n">
-        <v>-15.64</v>
+        <v>-15.31</v>
       </c>
       <c r="BD26" t="n">
-        <v>-31.12</v>
+        <v>-30.85</v>
       </c>
       <c r="BE26" t="n">
         <v>-80.83</v>
       </c>
       <c r="BF26" t="n">
-        <v>-93.56999999999999</v>
+        <v>-93.55</v>
       </c>
       <c r="BG26" t="n">
-        <v>-88.37</v>
+        <v>-88.31999999999999</v>
       </c>
       <c r="BH26" t="n">
         <v>4.69</v>
@@ -6507,7 +6507,7 @@
         <v>0</v>
       </c>
       <c r="BJ26" t="n">
-        <v>10.26</v>
+        <v>10.22</v>
       </c>
       <c r="BK26" t="n">
         <v>0.71</v>
@@ -6516,28 +6516,28 @@
         <v>0.72</v>
       </c>
       <c r="BM26" t="n">
-        <v>10.3</v>
+        <v>10.39</v>
       </c>
       <c r="BN26" t="n">
-        <v>10.35</v>
+        <v>10.39</v>
       </c>
       <c r="BO26" t="n">
         <v>6.91</v>
       </c>
       <c r="BP26" t="n">
-        <v>10.04</v>
+        <v>10.15</v>
       </c>
       <c r="BQ26" t="n">
-        <v>14.31</v>
+        <v>14.25</v>
       </c>
       <c r="BR26" t="n">
-        <v>10.1</v>
+        <v>10.31</v>
       </c>
       <c r="BS26" t="n">
         <v>0.16</v>
       </c>
       <c r="BT26" t="n">
-        <v>12192447</v>
+        <v>12150707</v>
       </c>
     </row>
     <row r="27">
@@ -8165,13 +8165,13 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>14.3</v>
+        <v>14.98</v>
       </c>
       <c r="G34" t="n">
-        <v>2952804179</v>
+        <v>3093215611</v>
       </c>
       <c r="H34" t="n">
-        <v>0</v>
+        <v>2960200</v>
       </c>
       <c r="I34" t="n">
         <v>206489813</v>
@@ -8186,7 +8186,7 @@
         <v>0.45</v>
       </c>
       <c r="M34" t="n">
-        <v>0.2595859743469208</v>
+        <v>0.2719297791425067</v>
       </c>
       <c r="N34" t="n">
         <v>0.24</v>
@@ -8264,7 +8264,7 @@
         <v>324189006.41</v>
       </c>
       <c r="AM34" t="n">
-        <v>613888602.7027028</v>
+        <v>643080168.6070687</v>
       </c>
       <c r="AN34" t="n">
         <v>0</v>
@@ -8305,7 +8305,7 @@
         <v>30.28</v>
       </c>
       <c r="AZ34" t="n">
-        <v>33.37</v>
+        <v>34.95</v>
       </c>
       <c r="BA34" t="n">
         <v>2.29</v>
@@ -8314,19 +8314,19 @@
         <v>25.26</v>
       </c>
       <c r="BC34" t="n">
-        <v>159.36</v>
+        <v>147.59</v>
       </c>
       <c r="BD34" t="n">
-        <v>111.77</v>
+        <v>102.15</v>
       </c>
       <c r="BE34" t="n">
         <v>133.33</v>
       </c>
       <c r="BF34" t="n">
-        <v>-83.95</v>
+        <v>-84.68000000000001</v>
       </c>
       <c r="BG34" t="n">
-        <v>76.63</v>
+        <v>68.61</v>
       </c>
       <c r="BH34" t="n">
         <v>38.94</v>
@@ -8335,7 +8335,7 @@
         <v>0</v>
       </c>
       <c r="BJ34" t="n">
-        <v>14.3</v>
+        <v>14.98</v>
       </c>
       <c r="BK34" t="n">
         <v>1.57</v>
@@ -8344,28 +8344,28 @@
         <v>1.58</v>
       </c>
       <c r="BM34" t="n">
-        <v>14.81</v>
+        <v>15.07</v>
       </c>
       <c r="BN34" t="n">
-        <v>29.87</v>
+        <v>29.39</v>
       </c>
       <c r="BO34" t="n">
         <v>14.3</v>
       </c>
       <c r="BP34" t="n">
-        <v>14.3</v>
+        <v>14.31</v>
       </c>
       <c r="BQ34" t="n">
-        <v>9.07</v>
+        <v>9.5</v>
       </c>
       <c r="BR34" t="n">
-        <v>14.74</v>
+        <v>14.45</v>
       </c>
       <c r="BS34" t="n">
         <v>0.32</v>
       </c>
       <c r="BT34" t="n">
-        <v>3111263</v>
+        <v>3242083</v>
       </c>
     </row>
     <row r="35">
@@ -8395,13 +8395,13 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>17.59</v>
+        <v>18.23</v>
       </c>
       <c r="G35" t="n">
-        <v>88767935770</v>
+        <v>91997692689</v>
       </c>
       <c r="H35" t="n">
-        <v>0</v>
+        <v>49189900</v>
       </c>
       <c r="I35" t="n">
         <v>5046500000</v>
@@ -8416,7 +8416,7 @@
         <v>4.69</v>
       </c>
       <c r="M35" t="n">
-        <v>7.369546290340773</v>
+        <v>7.637681883611637</v>
       </c>
       <c r="N35" t="n">
         <v>1.79</v>
@@ -8494,7 +8494,7 @@
         <v>5349290000</v>
       </c>
       <c r="AM35" t="n">
-        <v>7336193038.842976</v>
+        <v>7603115098.264463</v>
       </c>
       <c r="AN35" t="n">
         <v>0.5305</v>
@@ -8535,7 +8535,7 @@
         <v>7.68</v>
       </c>
       <c r="AZ35" t="n">
-        <v>10.26</v>
+        <v>10.63</v>
       </c>
       <c r="BA35" t="n">
         <v>1.11</v>
@@ -8544,28 +8544,28 @@
         <v>9.119999999999999</v>
       </c>
       <c r="BC35" t="n">
-        <v>-46.52</v>
+        <v>-48.4</v>
       </c>
       <c r="BD35" t="n">
-        <v>-56.34</v>
+        <v>-57.87</v>
       </c>
       <c r="BE35" t="n">
         <v>-41.67</v>
       </c>
       <c r="BF35" t="n">
-        <v>-93.67</v>
+        <v>-93.89</v>
       </c>
       <c r="BG35" t="n">
-        <v>-48.17</v>
+        <v>-49.99</v>
       </c>
       <c r="BH35" t="n">
         <v>3.71</v>
       </c>
       <c r="BI35" t="n">
-        <v>-0.06</v>
+        <v>0</v>
       </c>
       <c r="BJ35" t="n">
-        <v>17.6</v>
+        <v>18.23</v>
       </c>
       <c r="BK35" t="n">
         <v>1.06</v>
@@ -8574,7 +8574,7 @@
         <v>1.04</v>
       </c>
       <c r="BM35" t="n">
-        <v>17.7</v>
+        <v>18.38</v>
       </c>
       <c r="BN35" t="n">
         <v>20.08</v>
@@ -8583,19 +8583,19 @@
         <v>11.7</v>
       </c>
       <c r="BP35" t="n">
-        <v>17.39</v>
+        <v>17.75</v>
       </c>
       <c r="BQ35" t="n">
-        <v>16.83</v>
+        <v>17.45</v>
       </c>
       <c r="BR35" t="n">
-        <v>17.44</v>
+        <v>17.78</v>
       </c>
       <c r="BS35" t="n">
         <v>7.3</v>
       </c>
       <c r="BT35" t="n">
-        <v>36804613</v>
+        <v>38258820</v>
       </c>
     </row>
     <row r="36">
@@ -8855,13 +8855,13 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>14.9</v>
+        <v>14.8</v>
       </c>
       <c r="G37" t="n">
-        <v>199978109</v>
+        <v>198578114</v>
       </c>
       <c r="H37" t="n">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="I37" t="n">
         <v>4900000</v>
@@ -8876,7 +8876,7 @@
         <v>0.88</v>
       </c>
       <c r="M37" t="n">
-        <v>1.946955350454987</v>
+        <v>1.933325219789734</v>
       </c>
       <c r="N37" t="n">
         <v>0.5</v>
@@ -8954,7 +8954,7 @@
         <v>11319000</v>
       </c>
       <c r="AM37" t="n">
-        <v>47841652.8708134</v>
+        <v>47506725.83732058</v>
       </c>
       <c r="AN37" t="n">
         <v>0</v>
@@ -8995,7 +8995,7 @@
         <v>24.36</v>
       </c>
       <c r="AZ37" t="n">
-        <v>66.26000000000001</v>
+        <v>65.81</v>
       </c>
       <c r="BA37" t="n">
         <v>2.44</v>
@@ -9004,19 +9004,19 @@
         <v>15.53</v>
       </c>
       <c r="BC37" t="n">
-        <v>100.26</v>
+        <v>101.61</v>
       </c>
       <c r="BD37" t="n">
-        <v>63.51</v>
+        <v>64.61</v>
       </c>
       <c r="BE37" t="n">
         <v>344.67</v>
       </c>
       <c r="BF37" t="n">
-        <v>-83.59</v>
+        <v>-83.48</v>
       </c>
       <c r="BG37" t="n">
-        <v>4.25</v>
+        <v>4.95</v>
       </c>
       <c r="BH37" t="n">
         <v>17.13</v>
@@ -9025,7 +9025,7 @@
         <v>0</v>
       </c>
       <c r="BJ37" t="n">
-        <v>14.9</v>
+        <v>14.8</v>
       </c>
       <c r="BK37" t="n">
         <v>2.31</v>
@@ -9040,22 +9040,22 @@
         <v>20.9</v>
       </c>
       <c r="BO37" t="n">
-        <v>13.05</v>
+        <v>13.2</v>
       </c>
       <c r="BP37" t="n">
         <v>14.8</v>
       </c>
       <c r="BQ37" t="n">
-        <v>6.45</v>
+        <v>6.4</v>
       </c>
       <c r="BR37" t="n">
-        <v>14.8</v>
+        <v>14.9</v>
       </c>
       <c r="BS37" t="n">
         <v>0.72</v>
       </c>
       <c r="BT37" t="n">
-        <v>843</v>
+        <v>837</v>
       </c>
     </row>
     <row r="38">
@@ -9315,13 +9315,13 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>69.61</v>
+        <v>69.89</v>
       </c>
       <c r="G39" t="n">
-        <v>3902218993</v>
+        <v>3917915251</v>
       </c>
       <c r="H39" t="n">
-        <v>0</v>
+        <v>1500</v>
       </c>
       <c r="I39" t="n">
         <v>168174945</v>
@@ -9336,7 +9336,7 @@
         <v>0.53</v>
       </c>
       <c r="M39" t="n">
-        <v>0.1958742768924096</v>
+        <v>0.1966621601944954</v>
       </c>
       <c r="N39" t="n">
         <v>0.06</v>
@@ -9414,7 +9414,7 @@
         <v>2536078170.6</v>
       </c>
       <c r="AM39" t="n">
-        <v>409896953.0462185</v>
+        <v>411545719.6428571</v>
       </c>
       <c r="AN39" t="n">
         <v>11.9435</v>
@@ -9455,7 +9455,7 @@
         <v>170.24</v>
       </c>
       <c r="AZ39" t="n">
-        <v>203.38</v>
+        <v>204.2</v>
       </c>
       <c r="BA39" t="n">
         <v>19.01</v>
@@ -9464,28 +9464,28 @@
         <v>91.72</v>
       </c>
       <c r="BC39" t="n">
-        <v>199.53</v>
+        <v>198.33</v>
       </c>
       <c r="BD39" t="n">
-        <v>144.57</v>
+        <v>143.59</v>
       </c>
       <c r="BE39" t="n">
         <v>192.17</v>
       </c>
       <c r="BF39" t="n">
-        <v>-72.69</v>
+        <v>-72.8</v>
       </c>
       <c r="BG39" t="n">
-        <v>31.77</v>
+        <v>31.24</v>
       </c>
       <c r="BH39" t="n">
         <v>128.13</v>
       </c>
       <c r="BI39" t="n">
-        <v>-0.01</v>
+        <v>0</v>
       </c>
       <c r="BJ39" t="n">
-        <v>69.62</v>
+        <v>69.89</v>
       </c>
       <c r="BK39" t="n">
         <v>15.08</v>
@@ -9494,7 +9494,7 @@
         <v>15.08</v>
       </c>
       <c r="BM39" t="n">
-        <v>69.61</v>
+        <v>69.89</v>
       </c>
       <c r="BN39" t="n">
         <v>74.56</v>
@@ -9503,19 +9503,19 @@
         <v>54.98</v>
       </c>
       <c r="BP39" t="n">
-        <v>69.59999999999999</v>
+        <v>69.58</v>
       </c>
       <c r="BQ39" t="n">
-        <v>4.62</v>
+        <v>4.63</v>
       </c>
       <c r="BR39" t="n">
-        <v>69.59999999999999</v>
+        <v>69.58</v>
       </c>
       <c r="BS39" t="n">
         <v>0.58</v>
       </c>
       <c r="BT39" t="n">
-        <v>3630</v>
+        <v>3547</v>
       </c>
     </row>
     <row r="40">
@@ -9545,13 +9545,13 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>23.2</v>
+        <v>22.99</v>
       </c>
       <c r="G40" t="n">
-        <v>132955353172</v>
+        <v>131751803378</v>
       </c>
       <c r="H40" t="n">
-        <v>0</v>
+        <v>57775600</v>
       </c>
       <c r="I40" t="n">
         <v>5730834040</v>
@@ -9566,7 +9566,7 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="M40" t="n">
-        <v>0.4034029955241491</v>
+        <v>0.3997512765028474</v>
       </c>
       <c r="N40" t="n">
         <v>0.05</v>
@@ -9644,7 +9644,7 @@
         <v>15358635227.2</v>
       </c>
       <c r="AM40" t="n">
-        <v>6896024542.116182</v>
+        <v>6833599760.26971</v>
       </c>
       <c r="AN40" t="n">
         <v>0.5641</v>
@@ -9685,7 +9685,7 @@
         <v>36.13</v>
       </c>
       <c r="AZ40" t="n">
-        <v>11.72</v>
+        <v>11.61</v>
       </c>
       <c r="BA40" t="n">
         <v>2.76</v>
@@ -9694,19 +9694,19 @@
         <v>27.89</v>
       </c>
       <c r="BC40" t="n">
-        <v>90.73</v>
+        <v>92.47</v>
       </c>
       <c r="BD40" t="n">
-        <v>55.73</v>
+        <v>57.15</v>
       </c>
       <c r="BE40" t="n">
         <v>-49.5</v>
       </c>
       <c r="BF40" t="n">
-        <v>-88.11</v>
+        <v>-88</v>
       </c>
       <c r="BG40" t="n">
-        <v>20.22</v>
+        <v>21.31</v>
       </c>
       <c r="BH40" t="n">
         <v>32.47</v>
@@ -9715,7 +9715,7 @@
         <v>0</v>
       </c>
       <c r="BJ40" t="n">
-        <v>23.2</v>
+        <v>22.99</v>
       </c>
       <c r="BK40" t="n">
         <v>2.68</v>
@@ -9724,7 +9724,7 @@
         <v>2.5</v>
       </c>
       <c r="BM40" t="n">
-        <v>23.23</v>
+        <v>23.38</v>
       </c>
       <c r="BN40" t="n">
         <v>27.36</v>
@@ -9733,19 +9733,19 @@
         <v>17.67</v>
       </c>
       <c r="BP40" t="n">
-        <v>22.3</v>
+        <v>22.83</v>
       </c>
       <c r="BQ40" t="n">
-        <v>9.279999999999999</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="BR40" t="n">
-        <v>22.59</v>
+        <v>23.2</v>
       </c>
       <c r="BS40" t="n">
         <v>0.39</v>
       </c>
       <c r="BT40" t="n">
-        <v>32908031</v>
+        <v>34132289</v>
       </c>
     </row>
     <row r="41">
@@ -9775,13 +9775,13 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>15.79</v>
+        <v>16.02</v>
       </c>
       <c r="G41" t="n">
-        <v>189650037887</v>
+        <v>190883571996</v>
       </c>
       <c r="H41" t="n">
-        <v>0</v>
+        <v>6190700</v>
       </c>
       <c r="I41" t="n">
         <v>5303870781</v>
@@ -9796,7 +9796,7 @@
         <v>0.92</v>
       </c>
       <c r="M41" t="n">
-        <v>1.263821870405711</v>
+        <v>1.272042102799097</v>
       </c>
       <c r="N41" t="n">
         <v>0.07000000000000001</v>
@@ -9874,7 +9874,7 @@
         <v>12304980211.92</v>
       </c>
       <c r="AM41" t="n">
-        <v>29221885652.85054</v>
+        <v>29411952541.75655</v>
       </c>
       <c r="AN41" t="n">
         <v>1.6841</v>
@@ -9915,7 +9915,7 @@
         <v>24.4</v>
       </c>
       <c r="AZ41" t="n">
-        <v>23.63</v>
+        <v>23.98</v>
       </c>
       <c r="BA41" t="n">
         <v>2.53</v>
@@ -9924,28 +9924,28 @@
         <v>13.77</v>
       </c>
       <c r="BC41" t="n">
-        <v>89.27</v>
+        <v>86.55</v>
       </c>
       <c r="BD41" t="n">
-        <v>54.54</v>
+        <v>52.32</v>
       </c>
       <c r="BE41" t="n">
         <v>49.67</v>
       </c>
       <c r="BF41" t="n">
-        <v>-84</v>
+        <v>-84.22</v>
       </c>
       <c r="BG41" t="n">
-        <v>-12.79</v>
+        <v>-14.04</v>
       </c>
       <c r="BH41" t="n">
         <v>17.11</v>
       </c>
       <c r="BI41" t="n">
-        <v>-1.5</v>
+        <v>0</v>
       </c>
       <c r="BJ41" t="n">
-        <v>16.03</v>
+        <v>16.02</v>
       </c>
       <c r="BK41" t="n">
         <v>2.32</v>
@@ -9954,7 +9954,7 @@
         <v>2.34</v>
       </c>
       <c r="BM41" t="n">
-        <v>15.95</v>
+        <v>16.08</v>
       </c>
       <c r="BN41" t="n">
         <v>18.28</v>
@@ -9963,19 +9963,19 @@
         <v>13.43</v>
       </c>
       <c r="BP41" t="n">
-        <v>15.77</v>
+        <v>15.89</v>
       </c>
       <c r="BQ41" t="n">
-        <v>6.76</v>
+        <v>6.85</v>
       </c>
       <c r="BR41" t="n">
-        <v>15.91</v>
+        <v>15.96</v>
       </c>
       <c r="BS41" t="n">
         <v>0.5600000000000001</v>
       </c>
       <c r="BT41" t="n">
-        <v>7020174</v>
+        <v>7180531</v>
       </c>
     </row>
     <row r="42">
@@ -10005,13 +10005,13 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>17.99</v>
+        <v>18.16</v>
       </c>
       <c r="G42" t="n">
-        <v>189650037887</v>
+        <v>190883571996</v>
       </c>
       <c r="H42" t="n">
-        <v>0</v>
+        <v>54948000</v>
       </c>
       <c r="I42" t="n">
         <v>5288141247</v>
@@ -10026,7 +10026,7 @@
         <v>1.05</v>
       </c>
       <c r="M42" t="n">
-        <v>1.267581098488314</v>
+        <v>1.27582578189745</v>
       </c>
       <c r="N42" t="n">
         <v>0.08</v>
@@ -10104,7 +10104,7 @@
         <v>12268487693.04</v>
       </c>
       <c r="AM42" t="n">
-        <v>25802726243.12925</v>
+        <v>25970554013.06123</v>
       </c>
       <c r="AN42" t="n">
         <v>1.8491</v>
@@ -10145,7 +10145,7 @@
         <v>24.4</v>
       </c>
       <c r="AZ42" t="n">
-        <v>26.06</v>
+        <v>26.3</v>
       </c>
       <c r="BA42" t="n">
         <v>2.53</v>
@@ -10154,28 +10154,28 @@
         <v>15.11</v>
       </c>
       <c r="BC42" t="n">
-        <v>66.12</v>
+        <v>64.56999999999999</v>
       </c>
       <c r="BD42" t="n">
-        <v>35.64</v>
+        <v>34.37</v>
       </c>
       <c r="BE42" t="n">
         <v>44.83</v>
       </c>
       <c r="BF42" t="n">
-        <v>-85.95</v>
+        <v>-86.08</v>
       </c>
       <c r="BG42" t="n">
-        <v>-15.98</v>
+        <v>-16.77</v>
       </c>
       <c r="BH42" t="n">
         <v>17.11</v>
       </c>
       <c r="BI42" t="n">
-        <v>-0.88</v>
+        <v>0</v>
       </c>
       <c r="BJ42" t="n">
-        <v>18.15</v>
+        <v>18.16</v>
       </c>
       <c r="BK42" t="n">
         <v>2.32</v>
@@ -10184,7 +10184,7 @@
         <v>2.34</v>
       </c>
       <c r="BM42" t="n">
-        <v>18.11</v>
+        <v>18.23</v>
       </c>
       <c r="BN42" t="n">
         <v>21.33</v>
@@ -10193,19 +10193,19 @@
         <v>15.67</v>
       </c>
       <c r="BP42" t="n">
-        <v>17.9</v>
+        <v>18.01</v>
       </c>
       <c r="BQ42" t="n">
-        <v>7.7</v>
+        <v>7.77</v>
       </c>
       <c r="BR42" t="n">
-        <v>18.09</v>
+        <v>18.15</v>
       </c>
       <c r="BS42" t="n">
         <v>0.63</v>
       </c>
       <c r="BT42" t="n">
-        <v>40611854</v>
+        <v>40434852</v>
       </c>
     </row>
     <row r="43">
@@ -10235,13 +10235,13 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>40.86</v>
+        <v>39.82</v>
       </c>
       <c r="G43" t="n">
-        <v>79325605184</v>
+        <v>77306507587</v>
       </c>
       <c r="H43" t="n">
-        <v>0</v>
+        <v>8742900</v>
       </c>
       <c r="I43" t="n">
         <v>1941400000</v>
@@ -10334,7 +10334,7 @@
         <v>9182822000</v>
       </c>
       <c r="AM43" t="n">
-        <v>9662071276.979292</v>
+        <v>9416139779.171741</v>
       </c>
       <c r="AN43" t="n">
         <v>4.5901</v>
@@ -10375,7 +10375,7 @@
         <v>19.95</v>
       </c>
       <c r="AZ43" t="n">
-        <v>74.16</v>
+        <v>72.27</v>
       </c>
       <c r="BA43" t="n">
         <v>5.63</v>
@@ -10384,28 +10384,28 @@
         <v>48.62</v>
       </c>
       <c r="BC43" t="n">
-        <v>-40.2</v>
+        <v>-38.64</v>
       </c>
       <c r="BD43" t="n">
-        <v>-51.17</v>
+        <v>-49.9</v>
       </c>
       <c r="BE43" t="n">
         <v>81.5</v>
       </c>
       <c r="BF43" t="n">
-        <v>-86.22</v>
+        <v>-85.86</v>
       </c>
       <c r="BG43" t="n">
-        <v>18.98</v>
+        <v>22.09</v>
       </c>
       <c r="BH43" t="n">
         <v>5.61</v>
       </c>
       <c r="BI43" t="n">
-        <v>1.11</v>
+        <v>0</v>
       </c>
       <c r="BJ43" t="n">
-        <v>40.41</v>
+        <v>39.82</v>
       </c>
       <c r="BK43" t="n">
         <v>4.73</v>
@@ -10414,7 +10414,7 @@
         <v>4.73</v>
       </c>
       <c r="BM43" t="n">
-        <v>40.86</v>
+        <v>41.21</v>
       </c>
       <c r="BN43" t="n">
         <v>42.98</v>
@@ -10423,19 +10423,19 @@
         <v>28.06</v>
       </c>
       <c r="BP43" t="n">
-        <v>39.95</v>
+        <v>39.7</v>
       </c>
       <c r="BQ43" t="n">
-        <v>8.630000000000001</v>
+        <v>8.41</v>
       </c>
       <c r="BR43" t="n">
-        <v>40.32</v>
+        <v>40.92</v>
       </c>
       <c r="BS43" t="n">
         <v>0</v>
       </c>
       <c r="BT43" t="n">
-        <v>6637224</v>
+        <v>6584443</v>
       </c>
     </row>
     <row r="44">
@@ -10925,16 +10925,16 @@
         </is>
       </c>
       <c r="F46" t="n">
-        <v>3.98</v>
+        <v>3.92</v>
       </c>
       <c r="G46" t="n">
-        <v>3982157179</v>
+        <v>3922124716</v>
       </c>
       <c r="H46" t="n">
-        <v>0</v>
+        <v>19463500</v>
       </c>
       <c r="I46" t="n">
-        <v>1000541644</v>
+        <v>1000542188</v>
       </c>
       <c r="J46" t="n">
         <v>4.95</v>
@@ -10946,7 +10946,7 @@
         <v>2.5</v>
       </c>
       <c r="M46" t="n">
-        <v>0.0692174162626554</v>
+        <v>0.0681739015547508</v>
       </c>
       <c r="N46" t="n">
         <v>0.08</v>
@@ -11018,13 +11018,13 @@
         <v>-8.029999999999999</v>
       </c>
       <c r="AK46" t="n">
-        <v>57531144530</v>
+        <v>57531175810</v>
       </c>
       <c r="AL46" t="n">
-        <v>460249156.24</v>
+        <v>460249406.48</v>
       </c>
       <c r="AM46" t="n">
-        <v>3904075665.686275</v>
+        <v>3845220309.803922</v>
       </c>
       <c r="AN46" t="n">
         <v>0.0311</v>
@@ -11065,7 +11065,7 @@
         <v>3.3</v>
       </c>
       <c r="AZ46" t="n">
-        <v>3.28</v>
+        <v>3.23</v>
       </c>
       <c r="BA46" t="n">
         <v>0.42</v>
@@ -11074,19 +11074,19 @@
         <v>7.38</v>
       </c>
       <c r="BC46" t="n">
-        <v>1.61</v>
+        <v>3.16</v>
       </c>
       <c r="BD46" t="n">
-        <v>-17.04</v>
+        <v>-15.77</v>
       </c>
       <c r="BE46" t="n">
         <v>-17.5</v>
       </c>
       <c r="BF46" t="n">
-        <v>-89.37</v>
+        <v>-89.20999999999999</v>
       </c>
       <c r="BG46" t="n">
-        <v>85.39</v>
+        <v>88.23</v>
       </c>
       <c r="BH46" t="n">
         <v>1.58</v>
@@ -11095,7 +11095,7 @@
         <v>0</v>
       </c>
       <c r="BJ46" t="n">
-        <v>3.98</v>
+        <v>3.92</v>
       </c>
       <c r="BK46" t="n">
         <v>0.46</v>
@@ -11104,7 +11104,7 @@
         <v>0.46</v>
       </c>
       <c r="BM46" t="n">
-        <v>4.01</v>
+        <v>4.02</v>
       </c>
       <c r="BN46" t="n">
         <v>7.31</v>
@@ -11113,19 +11113,19 @@
         <v>2.97</v>
       </c>
       <c r="BP46" t="n">
-        <v>3.8</v>
+        <v>3.86</v>
       </c>
       <c r="BQ46" t="n">
-        <v>8.699999999999999</v>
+        <v>8.57</v>
       </c>
       <c r="BR46" t="n">
-        <v>3.81</v>
+        <v>4</v>
       </c>
       <c r="BS46" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="BT46" t="n">
-        <v>21479160</v>
+        <v>22327503</v>
       </c>
     </row>
     <row r="47">
@@ -11155,13 +11155,13 @@
         </is>
       </c>
       <c r="F47" t="n">
-        <v>8.93</v>
+        <v>9</v>
       </c>
       <c r="G47" t="n">
-        <v>3115354000</v>
+        <v>3139774200</v>
       </c>
       <c r="H47" t="n">
-        <v>0</v>
+        <v>3900</v>
       </c>
       <c r="I47" t="n">
         <v>254106600</v>
@@ -11176,7 +11176,7 @@
         <v>1.22</v>
       </c>
       <c r="M47" t="n">
-        <v>0.7346363161579945</v>
+        <v>0.7403948802787467</v>
       </c>
       <c r="N47" t="n">
         <v>0.07000000000000001</v>
@@ -11254,7 +11254,7 @@
         <v>322715382</v>
       </c>
       <c r="AM47" t="n">
-        <v>552367730.4964539</v>
+        <v>556697553.1914893</v>
       </c>
       <c r="AN47" t="n">
         <v>0.4132</v>
@@ -11295,7 +11295,7 @@
         <v>11.74</v>
       </c>
       <c r="AZ47" t="n">
-        <v>11.73</v>
+        <v>11.82</v>
       </c>
       <c r="BA47" t="n">
         <v>1.46</v>
@@ -11304,28 +11304,28 @@
         <v>8.619999999999999</v>
       </c>
       <c r="BC47" t="n">
-        <v>60.96</v>
+        <v>59.71</v>
       </c>
       <c r="BD47" t="n">
-        <v>31.42</v>
+        <v>30.4</v>
       </c>
       <c r="BE47" t="n">
         <v>31.33</v>
       </c>
       <c r="BF47" t="n">
-        <v>-83.67</v>
+        <v>-83.79000000000001</v>
       </c>
       <c r="BG47" t="n">
-        <v>-3.47</v>
+        <v>-4.23</v>
       </c>
       <c r="BH47" t="n">
         <v>7.23</v>
       </c>
       <c r="BI47" t="n">
-        <v>1.25</v>
+        <v>0</v>
       </c>
       <c r="BJ47" t="n">
-        <v>8.82</v>
+        <v>9</v>
       </c>
       <c r="BK47" t="n">
         <v>1.27</v>
@@ -11334,7 +11334,7 @@
         <v>1.29</v>
       </c>
       <c r="BM47" t="n">
-        <v>8.93</v>
+        <v>9.029999999999999</v>
       </c>
       <c r="BN47" t="n">
         <v>9.24</v>
@@ -11343,19 +11343,19 @@
         <v>7.19</v>
       </c>
       <c r="BP47" t="n">
-        <v>8.83</v>
+        <v>8.94</v>
       </c>
       <c r="BQ47" t="n">
-        <v>6.9</v>
+        <v>6.96</v>
       </c>
       <c r="BR47" t="n">
-        <v>8.83</v>
+        <v>8.98</v>
       </c>
       <c r="BS47" t="n">
         <v>0.53</v>
       </c>
       <c r="BT47" t="n">
-        <v>12261</v>
+        <v>11766</v>
       </c>
     </row>
     <row r="48">
@@ -11385,13 +11385,13 @@
         </is>
       </c>
       <c r="F48" t="n">
-        <v>9.06</v>
+        <v>9.15</v>
       </c>
       <c r="G48" t="n">
-        <v>3115354000</v>
+        <v>3139774200</v>
       </c>
       <c r="H48" t="n">
-        <v>0</v>
+        <v>1900</v>
       </c>
       <c r="I48" t="n">
         <v>93397546</v>
@@ -11406,7 +11406,7 @@
         <v>1.24</v>
       </c>
       <c r="M48" t="n">
-        <v>1.998724212041215</v>
+        <v>2.014391531069129</v>
       </c>
       <c r="N48" t="n">
         <v>0.07000000000000001</v>
@@ -11484,7 +11484,7 @@
         <v>118614883.42</v>
       </c>
       <c r="AM48" t="n">
-        <v>544642307.6923077</v>
+        <v>548911573.4265734</v>
       </c>
       <c r="AN48" t="n">
         <v>0.4132</v>
@@ -11525,7 +11525,7 @@
         <v>11.74</v>
       </c>
       <c r="AZ48" t="n">
-        <v>11.85</v>
+        <v>11.97</v>
       </c>
       <c r="BA48" t="n">
         <v>1.46</v>
@@ -11534,28 +11534,28 @@
         <v>8.24</v>
       </c>
       <c r="BC48" t="n">
-        <v>58.65</v>
+        <v>57.09</v>
       </c>
       <c r="BD48" t="n">
-        <v>29.54</v>
+        <v>28.26</v>
       </c>
       <c r="BE48" t="n">
         <v>30.83</v>
       </c>
       <c r="BF48" t="n">
-        <v>-83.90000000000001</v>
+        <v>-84.06</v>
       </c>
       <c r="BG48" t="n">
-        <v>-9.09</v>
+        <v>-9.99</v>
       </c>
       <c r="BH48" t="n">
         <v>7.23</v>
       </c>
       <c r="BI48" t="n">
-        <v>-0.66</v>
+        <v>0</v>
       </c>
       <c r="BJ48" t="n">
-        <v>9.119999999999999</v>
+        <v>9.15</v>
       </c>
       <c r="BK48" t="n">
         <v>1.27</v>
@@ -11564,7 +11564,7 @@
         <v>1.29</v>
       </c>
       <c r="BM48" t="n">
-        <v>9.19</v>
+        <v>9.289999999999999</v>
       </c>
       <c r="BN48" t="n">
         <v>9.48</v>
@@ -11573,19 +11573,19 @@
         <v>7.2</v>
       </c>
       <c r="BP48" t="n">
-        <v>9.039999999999999</v>
+        <v>9.08</v>
       </c>
       <c r="BQ48" t="n">
-        <v>7.01</v>
+        <v>7.08</v>
       </c>
       <c r="BR48" t="n">
-        <v>9.19</v>
+        <v>9.140000000000001</v>
       </c>
       <c r="BS48" t="n">
         <v>0.54</v>
       </c>
       <c r="BT48" t="n">
-        <v>2480</v>
+        <v>2453</v>
       </c>
     </row>
     <row r="49">
@@ -11851,7 +11851,7 @@
         <v>961816100</v>
       </c>
       <c r="H50" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="I50" t="n">
         <v>11540870</v>
@@ -12045,7 +12045,7 @@
         <v>0.4</v>
       </c>
       <c r="BT50" t="n">
-        <v>530</v>
+        <v>493</v>
       </c>
     </row>
     <row r="51">
@@ -12523,13 +12523,13 @@
         </is>
       </c>
       <c r="F53" t="n">
-        <v>6.26</v>
+        <v>6.47</v>
       </c>
       <c r="G53" t="n">
-        <v>856696055</v>
+        <v>885434999</v>
       </c>
       <c r="H53" t="n">
-        <v>0</v>
+        <v>11800</v>
       </c>
       <c r="I53" t="n">
         <v>136852484</v>
@@ -12544,7 +12544,7 @@
         <v>2.79</v>
       </c>
       <c r="M53" t="n">
-        <v>2.225536645532411</v>
+        <v>2.30019506452782</v>
       </c>
       <c r="N53" t="n">
         <v>1.48</v>
@@ -12622,7 +12622,7 @@
         <v>39687220.36</v>
       </c>
       <c r="AM53" t="n">
-        <v>43642183.138054</v>
+        <v>45106214.92613347</v>
       </c>
       <c r="AN53" t="n">
         <v>0</v>
@@ -12672,16 +12672,16 @@
         <v>0</v>
       </c>
       <c r="BC53" t="n">
-        <v>-37.05</v>
+        <v>-39.09</v>
       </c>
       <c r="BD53" t="n">
-        <v>-48.6</v>
+        <v>-50.27</v>
       </c>
       <c r="BE53" t="n">
         <v>-100</v>
       </c>
       <c r="BF53" t="n">
-        <v>-95.37</v>
+        <v>-95.52</v>
       </c>
       <c r="BG53" t="n">
         <v>-100</v>
@@ -12693,7 +12693,7 @@
         <v>0</v>
       </c>
       <c r="BJ53" t="n">
-        <v>6.26</v>
+        <v>6.47</v>
       </c>
       <c r="BK53" t="n">
         <v>0.29</v>
@@ -12702,7 +12702,7 @@
         <v>0.09</v>
       </c>
       <c r="BM53" t="n">
-        <v>6.36</v>
+        <v>6.47</v>
       </c>
       <c r="BN53" t="n">
         <v>10.39</v>
@@ -12711,19 +12711,19 @@
         <v>4.82</v>
       </c>
       <c r="BP53" t="n">
-        <v>6.26</v>
+        <v>6.29</v>
       </c>
       <c r="BQ53" t="n">
-        <v>73.37</v>
+        <v>75.83</v>
       </c>
       <c r="BR53" t="n">
-        <v>6.35</v>
+        <v>6.29</v>
       </c>
       <c r="BS53" t="n">
         <v>2.36</v>
       </c>
       <c r="BT53" t="n">
-        <v>42807</v>
+        <v>42190</v>
       </c>
     </row>
     <row r="54">
@@ -12753,13 +12753,13 @@
         </is>
       </c>
       <c r="F54" t="n">
-        <v>10.55</v>
+        <v>10.56</v>
       </c>
       <c r="G54" t="n">
-        <v>2460387699</v>
+        <v>2462719873</v>
       </c>
       <c r="H54" t="n">
-        <v>0</v>
+        <v>281200</v>
       </c>
       <c r="I54" t="n">
         <v>233212121</v>
@@ -12774,7 +12774,7 @@
         <v>0.97</v>
       </c>
       <c r="M54" t="n">
-        <v>1.38099490034268</v>
+        <v>1.382303929973262</v>
       </c>
       <c r="N54" t="n">
         <v>0.5600000000000001</v>
@@ -12852,7 +12852,7 @@
         <v>233212121</v>
       </c>
       <c r="AM54" t="n">
-        <v>336578344.5964432</v>
+        <v>336897383.4473324</v>
       </c>
       <c r="AN54" t="n">
         <v>0.1531</v>
@@ -12893,7 +12893,7 @@
         <v>12.25</v>
       </c>
       <c r="AZ54" t="n">
-        <v>16.79</v>
+        <v>16.81</v>
       </c>
       <c r="BA54" t="n">
         <v>0.98</v>
@@ -12902,28 +12902,28 @@
         <v>6.52</v>
       </c>
       <c r="BC54" t="n">
-        <v>42.25</v>
+        <v>42.12</v>
       </c>
       <c r="BD54" t="n">
-        <v>16.15</v>
+        <v>16.04</v>
       </c>
       <c r="BE54" t="n">
         <v>59.17</v>
       </c>
       <c r="BF54" t="n">
-        <v>-90.68000000000001</v>
+        <v>-90.69</v>
       </c>
       <c r="BG54" t="n">
-        <v>-38.23</v>
+        <v>-38.29</v>
       </c>
       <c r="BH54" t="n">
         <v>10.01</v>
       </c>
       <c r="BI54" t="n">
-        <v>-1.31</v>
+        <v>0</v>
       </c>
       <c r="BJ54" t="n">
-        <v>10.69</v>
+        <v>10.56</v>
       </c>
       <c r="BK54" t="n">
         <v>1</v>
@@ -12932,7 +12932,7 @@
         <v>1</v>
       </c>
       <c r="BM54" t="n">
-        <v>10.69</v>
+        <v>10.78</v>
       </c>
       <c r="BN54" t="n">
         <v>11.75</v>
@@ -12941,19 +12941,19 @@
         <v>8.279999999999999</v>
       </c>
       <c r="BP54" t="n">
-        <v>10.29</v>
+        <v>10.53</v>
       </c>
       <c r="BQ54" t="n">
-        <v>10.52</v>
+        <v>10.53</v>
       </c>
       <c r="BR54" t="n">
-        <v>10.69</v>
+        <v>10.55</v>
       </c>
       <c r="BS54" t="n">
         <v>1.26</v>
       </c>
       <c r="BT54" t="n">
-        <v>270133</v>
+        <v>273040</v>
       </c>
     </row>
     <row r="55">
@@ -12983,13 +12983,13 @@
         </is>
       </c>
       <c r="F55" t="n">
-        <v>49.72</v>
+        <v>50.1</v>
       </c>
       <c r="G55" t="n">
-        <v>6690365323</v>
+        <v>6684404349</v>
       </c>
       <c r="H55" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="I55" t="n">
         <v>84052790</v>
@@ -13004,7 +13004,7 @@
         <v>2</v>
       </c>
       <c r="M55" t="n">
-        <v>1.032799445124647</v>
+        <v>1.031879242662991</v>
       </c>
       <c r="N55" t="n">
         <v>0.16</v>
@@ -13082,7 +13082,7 @@
         <v>579123723.1</v>
       </c>
       <c r="AM55" t="n">
-        <v>336537491.0965795</v>
+        <v>336237643.3098592</v>
       </c>
       <c r="AN55" t="n">
         <v>3.1953</v>
@@ -13123,7 +13123,7 @@
         <v>51.21</v>
       </c>
       <c r="AZ55" t="n">
-        <v>52.29</v>
+        <v>52.69</v>
       </c>
       <c r="BA55" t="n">
         <v>9.380000000000001</v>
@@ -13132,28 +13132,28 @@
         <v>16.08</v>
       </c>
       <c r="BC55" t="n">
-        <v>26.13</v>
+        <v>25.18</v>
       </c>
       <c r="BD55" t="n">
-        <v>2.99</v>
+        <v>2.21</v>
       </c>
       <c r="BE55" t="n">
         <v>5.17</v>
       </c>
       <c r="BF55" t="n">
-        <v>-81.14</v>
+        <v>-81.28</v>
       </c>
       <c r="BG55" t="n">
-        <v>-67.67</v>
+        <v>-67.91</v>
       </c>
       <c r="BH55" t="n">
         <v>25.37</v>
       </c>
       <c r="BI55" t="n">
-        <v>1.06</v>
+        <v>0</v>
       </c>
       <c r="BJ55" t="n">
-        <v>49.2</v>
+        <v>50.1</v>
       </c>
       <c r="BK55" t="n">
         <v>6.89</v>
@@ -13162,7 +13162,7 @@
         <v>7.03</v>
       </c>
       <c r="BM55" t="n">
-        <v>49.99</v>
+        <v>50.5</v>
       </c>
       <c r="BN55" t="n">
         <v>73.67</v>
@@ -13171,19 +13171,19 @@
         <v>35.58</v>
       </c>
       <c r="BP55" t="n">
-        <v>49.16</v>
+        <v>49.8</v>
       </c>
       <c r="BQ55" t="n">
-        <v>7.07</v>
+        <v>7.13</v>
       </c>
       <c r="BR55" t="n">
-        <v>49.16</v>
+        <v>50</v>
       </c>
       <c r="BS55" t="n">
         <v>0.66</v>
       </c>
       <c r="BT55" t="n">
-        <v>7501</v>
+        <v>7645</v>
       </c>
     </row>
     <row r="56">
@@ -13213,13 +13213,13 @@
         </is>
       </c>
       <c r="F56" t="n">
-        <v>60.99</v>
+        <v>61.78</v>
       </c>
       <c r="G56" t="n">
-        <v>6690365323</v>
+        <v>6684404349</v>
       </c>
       <c r="H56" t="n">
-        <v>20500</v>
+        <v>28100</v>
       </c>
       <c r="I56" t="n">
         <v>39675836</v>
@@ -13234,7 +13234,7 @@
         <v>2.41</v>
       </c>
       <c r="M56" t="n">
-        <v>2.187973427281495</v>
+        <v>2.186023989233937</v>
       </c>
       <c r="N56" t="n">
         <v>0.19</v>
@@ -13312,7 +13312,7 @@
         <v>273366510.04</v>
       </c>
       <c r="AM56" t="n">
-        <v>278301386.1480865</v>
+        <v>278053425.499168</v>
       </c>
       <c r="AN56" t="n">
         <v>3.5102</v>
@@ -13353,7 +13353,7 @@
         <v>51.21</v>
       </c>
       <c r="AZ56" t="n">
-        <v>58.25</v>
+        <v>59</v>
       </c>
       <c r="BA56" t="n">
         <v>9.380000000000001</v>
@@ -13362,19 +13362,19 @@
         <v>17.68</v>
       </c>
       <c r="BC56" t="n">
-        <v>2.83</v>
+        <v>1.51</v>
       </c>
       <c r="BD56" t="n">
-        <v>-16.04</v>
+        <v>-17.12</v>
       </c>
       <c r="BE56" t="n">
         <v>-4.5</v>
       </c>
       <c r="BF56" t="n">
-        <v>-84.62</v>
+        <v>-84.81999999999999</v>
       </c>
       <c r="BG56" t="n">
-        <v>-71.02</v>
+        <v>-71.39</v>
       </c>
       <c r="BH56" t="n">
         <v>25.37</v>
@@ -13383,7 +13383,7 @@
         <v>0</v>
       </c>
       <c r="BJ56" t="n">
-        <v>60.99</v>
+        <v>61.78</v>
       </c>
       <c r="BK56" t="n">
         <v>6.89</v>
@@ -13392,7 +13392,7 @@
         <v>7.03</v>
       </c>
       <c r="BM56" t="n">
-        <v>60.99</v>
+        <v>63.45</v>
       </c>
       <c r="BN56" t="n">
         <v>86.77</v>
@@ -13401,19 +13401,19 @@
         <v>46.42</v>
       </c>
       <c r="BP56" t="n">
-        <v>58.92</v>
+        <v>60.94</v>
       </c>
       <c r="BQ56" t="n">
-        <v>8.67</v>
+        <v>8.789999999999999</v>
       </c>
       <c r="BR56" t="n">
-        <v>59.63</v>
+        <v>61.41</v>
       </c>
       <c r="BS56" t="n">
         <v>0.79</v>
       </c>
       <c r="BT56" t="n">
-        <v>32592</v>
+        <v>32225</v>
       </c>
     </row>
     <row r="57">
@@ -13443,13 +13443,13 @@
         </is>
       </c>
       <c r="F57" t="n">
-        <v>6.07</v>
+        <v>6.17</v>
       </c>
       <c r="G57" t="n">
-        <v>1419518100</v>
+        <v>1442903260</v>
       </c>
       <c r="H57" t="n">
-        <v>884100</v>
+        <v>1628700</v>
       </c>
       <c r="I57" t="n">
         <v>233858065</v>
@@ -13464,7 +13464,7 @@
         <v>0.77</v>
       </c>
       <c r="M57" t="n">
-        <v>0.4248998938736623</v>
+        <v>0.4318997003588481</v>
       </c>
       <c r="N57" t="n">
         <v>0.08</v>
@@ -13542,7 +13542,7 @@
         <v>229180903.7</v>
       </c>
       <c r="AM57" t="n">
-        <v>106171884.8167539</v>
+        <v>107920961.854899</v>
       </c>
       <c r="AN57" t="n">
         <v>0.347</v>
@@ -13583,7 +13583,7 @@
         <v>10.72</v>
       </c>
       <c r="AZ57" t="n">
-        <v>9.26</v>
+        <v>9.41</v>
       </c>
       <c r="BA57" t="n">
         <v>1.13</v>
@@ -13592,19 +13592,19 @@
         <v>6.26</v>
       </c>
       <c r="BC57" t="n">
-        <v>116.33</v>
+        <v>112.82</v>
       </c>
       <c r="BD57" t="n">
-        <v>76.63</v>
+        <v>73.77</v>
       </c>
       <c r="BE57" t="n">
         <v>52.5</v>
       </c>
       <c r="BF57" t="n">
-        <v>-81.43000000000001</v>
+        <v>-81.73</v>
       </c>
       <c r="BG57" t="n">
-        <v>3.19</v>
+        <v>1.52</v>
       </c>
       <c r="BH57" t="n">
         <v>7.82</v>
@@ -13613,7 +13613,7 @@
         <v>0</v>
       </c>
       <c r="BJ57" t="n">
-        <v>6.07</v>
+        <v>6.17</v>
       </c>
       <c r="BK57" t="n">
         <v>0.98</v>
@@ -13622,28 +13622,28 @@
         <v>1.04</v>
       </c>
       <c r="BM57" t="n">
-        <v>6.07</v>
+        <v>6.21</v>
       </c>
       <c r="BN57" t="n">
-        <v>6.18</v>
+        <v>6.21</v>
       </c>
       <c r="BO57" t="n">
         <v>3.43</v>
       </c>
       <c r="BP57" t="n">
-        <v>5.94</v>
+        <v>6.04</v>
       </c>
       <c r="BQ57" t="n">
-        <v>5.86</v>
+        <v>5.96</v>
       </c>
       <c r="BR57" t="n">
-        <v>6.03</v>
+        <v>6.07</v>
       </c>
       <c r="BS57" t="n">
         <v>0.42</v>
       </c>
       <c r="BT57" t="n">
-        <v>1286880</v>
+        <v>1288511</v>
       </c>
     </row>
     <row r="58">
@@ -14103,7 +14103,7 @@
         <v>1.42</v>
       </c>
       <c r="BT59" t="n">
-        <v>103</v>
+        <v>137</v>
       </c>
     </row>
     <row r="60">
@@ -14133,13 +14133,13 @@
         </is>
       </c>
       <c r="F60" t="n">
-        <v>376.92</v>
+        <v>373.89</v>
       </c>
       <c r="G60" t="n">
-        <v>171404400</v>
+        <v>170026484</v>
       </c>
       <c r="H60" t="n">
-        <v>14</v>
+        <v>36</v>
       </c>
       <c r="I60" t="n">
         <v>454750</v>
@@ -14154,7 +14154,7 @@
         <v>0.83</v>
       </c>
       <c r="M60" t="n">
-        <v>12.82080783302397</v>
+        <v>12.71774165592438</v>
       </c>
       <c r="N60" t="n">
         <v>0.68</v>
@@ -14232,7 +14232,7 @@
         <v>59558607.5</v>
       </c>
       <c r="AM60" t="n">
-        <v>-25132609.97067448</v>
+        <v>-24930569.50146627</v>
       </c>
       <c r="AN60" t="n">
         <v>10.0581</v>
@@ -14273,7 +14273,7 @@
         <v>944.87</v>
       </c>
       <c r="AZ60" t="n">
-        <v>2167.29</v>
+        <v>2149.87</v>
       </c>
       <c r="BA60" t="n">
         <v>231.1</v>
@@ -14282,19 +14282,19 @@
         <v>727.97</v>
       </c>
       <c r="BC60" t="n">
-        <v>207.02</v>
+        <v>209.51</v>
       </c>
       <c r="BD60" t="n">
-        <v>150.68</v>
+        <v>152.71</v>
       </c>
       <c r="BE60" t="n">
         <v>475</v>
       </c>
       <c r="BF60" t="n">
-        <v>-38.69</v>
+        <v>-38.19</v>
       </c>
       <c r="BG60" t="n">
-        <v>93.14</v>
+        <v>94.7</v>
       </c>
       <c r="BH60" t="n">
         <v>454.44</v>
@@ -14303,7 +14303,7 @@
         <v>0</v>
       </c>
       <c r="BJ60" t="n">
-        <v>376.92</v>
+        <v>373.89</v>
       </c>
       <c r="BK60" t="n">
         <v>130.97</v>
@@ -14312,7 +14312,7 @@
         <v>130.97</v>
       </c>
       <c r="BM60" t="n">
-        <v>380</v>
+        <v>387</v>
       </c>
       <c r="BN60" t="n">
         <v>405</v>
@@ -14321,19 +14321,19 @@
         <v>306.27</v>
       </c>
       <c r="BP60" t="n">
-        <v>376.92</v>
+        <v>370.01</v>
       </c>
       <c r="BQ60" t="n">
-        <v>2.88</v>
+        <v>2.85</v>
       </c>
       <c r="BR60" t="n">
-        <v>380</v>
+        <v>377</v>
       </c>
       <c r="BS60" t="n">
         <v>12.82</v>
       </c>
       <c r="BT60" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="61">
@@ -14363,13 +14363,13 @@
         </is>
       </c>
       <c r="F61" t="n">
-        <v>27.52</v>
+        <v>27.66</v>
       </c>
       <c r="G61" t="n">
-        <v>2355942931</v>
+        <v>2367928054</v>
       </c>
       <c r="H61" t="n">
-        <v>0</v>
+        <v>516500</v>
       </c>
       <c r="I61" t="n">
         <v>85608392</v>
@@ -14384,7 +14384,7 @@
         <v>2.37</v>
       </c>
       <c r="M61" t="n">
-        <v>1.24943742422425</v>
+        <v>1.255793546443125</v>
       </c>
       <c r="N61" t="n">
         <v>1.1</v>
@@ -14462,7 +14462,7 @@
         <v>160087693.04</v>
       </c>
       <c r="AM61" t="n">
-        <v>184924876.844584</v>
+        <v>185865624.33281</v>
       </c>
       <c r="AN61" t="n">
         <v>0.38</v>
@@ -14503,7 +14503,7 @@
         <v>17.56</v>
       </c>
       <c r="AZ61" t="n">
-        <v>34.68</v>
+        <v>34.85</v>
       </c>
       <c r="BA61" t="n">
         <v>2.52</v>
@@ -14512,19 +14512,19 @@
         <v>11.76</v>
       </c>
       <c r="BC61" t="n">
-        <v>-21.86</v>
+        <v>-22.26</v>
       </c>
       <c r="BD61" t="n">
-        <v>-36.2</v>
+        <v>-36.52</v>
       </c>
       <c r="BE61" t="n">
         <v>26</v>
       </c>
       <c r="BF61" t="n">
-        <v>-90.83</v>
+        <v>-90.88</v>
       </c>
       <c r="BG61" t="n">
-        <v>-57.28</v>
+        <v>-57.5</v>
       </c>
       <c r="BH61" t="n">
         <v>10.99</v>
@@ -14533,7 +14533,7 @@
         <v>0</v>
       </c>
       <c r="BJ61" t="n">
-        <v>27.52</v>
+        <v>27.66</v>
       </c>
       <c r="BK61" t="n">
         <v>1.87</v>
@@ -14542,7 +14542,7 @@
         <v>1.86</v>
       </c>
       <c r="BM61" t="n">
-        <v>27.71</v>
+        <v>27.93</v>
       </c>
       <c r="BN61" t="n">
         <v>28.25</v>
@@ -14551,19 +14551,19 @@
         <v>19.35</v>
       </c>
       <c r="BP61" t="n">
-        <v>27.34</v>
+        <v>27.58</v>
       </c>
       <c r="BQ61" t="n">
-        <v>14.78</v>
+        <v>14.86</v>
       </c>
       <c r="BR61" t="n">
-        <v>27.64</v>
+        <v>27.7</v>
       </c>
       <c r="BS61" t="n">
         <v>1.19</v>
       </c>
       <c r="BT61" t="n">
-        <v>511550</v>
+        <v>523762</v>
       </c>
     </row>
     <row r="62">
@@ -14593,13 +14593,13 @@
         </is>
       </c>
       <c r="F62" t="n">
-        <v>115.24</v>
+        <v>105</v>
       </c>
       <c r="G62" t="n">
-        <v>11377473281</v>
+        <v>10363473750</v>
       </c>
       <c r="H62" t="n">
-        <v>100</v>
+        <v>600</v>
       </c>
       <c r="I62" t="n">
         <v>98699749</v>
@@ -14614,7 +14614,7 @@
         <v>0.64</v>
       </c>
       <c r="M62" t="n">
-        <v>1.06650751918525</v>
+        <v>0.9714567027559305</v>
       </c>
       <c r="N62" t="n">
         <v>0.13</v>
@@ -14692,7 +14692,7 @@
         <v>2757670987.06</v>
       </c>
       <c r="AM62" t="n">
-        <v>4606264486.234818</v>
+        <v>4195738360.323886</v>
       </c>
       <c r="AN62" t="n">
         <v>6.9319</v>
@@ -14733,7 +14733,7 @@
         <v>267.2</v>
       </c>
       <c r="AZ62" t="n">
-        <v>121.77</v>
+        <v>110.95</v>
       </c>
       <c r="BA62" t="n">
         <v>34.09</v>
@@ -14742,19 +14742,19 @@
         <v>76.01000000000001</v>
       </c>
       <c r="BC62" t="n">
-        <v>183.97</v>
+        <v>211.66</v>
       </c>
       <c r="BD62" t="n">
-        <v>131.86</v>
+        <v>154.47</v>
       </c>
       <c r="BE62" t="n">
         <v>5.67</v>
       </c>
       <c r="BF62" t="n">
-        <v>-70.42</v>
+        <v>-67.53</v>
       </c>
       <c r="BG62" t="n">
-        <v>-34.04</v>
+        <v>-27.61</v>
       </c>
       <c r="BH62" t="n">
         <v>170.35</v>
@@ -14763,7 +14763,7 @@
         <v>0</v>
       </c>
       <c r="BJ62" t="n">
-        <v>115.24</v>
+        <v>105</v>
       </c>
       <c r="BK62" t="n">
         <v>27.94</v>
@@ -14772,28 +14772,28 @@
         <v>32.73</v>
       </c>
       <c r="BM62" t="n">
-        <v>115.24</v>
+        <v>114.5</v>
       </c>
       <c r="BN62" t="n">
         <v>122.2</v>
       </c>
       <c r="BO62" t="n">
-        <v>91.36</v>
+        <v>91.84999999999999</v>
       </c>
       <c r="BP62" t="n">
-        <v>115.24</v>
+        <v>105</v>
       </c>
       <c r="BQ62" t="n">
-        <v>3.52</v>
+        <v>3.21</v>
       </c>
       <c r="BR62" t="n">
-        <v>115.24</v>
+        <v>114.5</v>
       </c>
       <c r="BS62" t="n">
         <v>1.01</v>
       </c>
       <c r="BT62" t="n">
-        <v>156</v>
+        <v>142</v>
       </c>
     </row>
     <row r="63">
@@ -14823,13 +14823,13 @@
         </is>
       </c>
       <c r="F63" t="n">
-        <v>1.35</v>
+        <v>1.43</v>
       </c>
       <c r="G63" t="n">
-        <v>346664076</v>
+        <v>372528857</v>
       </c>
       <c r="H63" t="n">
-        <v>30200</v>
+        <v>64700</v>
       </c>
       <c r="I63" t="n">
         <v>122894462</v>
@@ -14844,7 +14844,7 @@
         <v>-0.22</v>
       </c>
       <c r="M63" t="n">
-        <v>0.4263789234926569</v>
+        <v>0.4581912693417068</v>
       </c>
       <c r="N63" t="n">
         <v>0.37</v>
@@ -14922,7 +14922,7 @@
         <v>31952560.12</v>
       </c>
       <c r="AM63" t="n">
-        <v>196968225</v>
+        <v>211664123.2954545</v>
       </c>
       <c r="AN63" t="n">
         <v>0</v>
@@ -14981,7 +14981,7 @@
         <v>-100</v>
       </c>
       <c r="BF63" t="n">
-        <v>-78.58</v>
+        <v>-79.78</v>
       </c>
       <c r="BG63" t="n">
         <v>-100</v>
@@ -14993,7 +14993,7 @@
         <v>0</v>
       </c>
       <c r="BJ63" t="n">
-        <v>1.35</v>
+        <v>1.43</v>
       </c>
       <c r="BK63" t="n">
         <v>0.26</v>
@@ -15002,7 +15002,7 @@
         <v>0.26</v>
       </c>
       <c r="BM63" t="n">
-        <v>1.43</v>
+        <v>1.5</v>
       </c>
       <c r="BN63" t="n">
         <v>2.12</v>
@@ -15011,19 +15011,19 @@
         <v>1.16</v>
       </c>
       <c r="BP63" t="n">
-        <v>1.35</v>
+        <v>1.4</v>
       </c>
       <c r="BQ63" t="n">
-        <v>5.17</v>
+        <v>5.48</v>
       </c>
       <c r="BR63" t="n">
-        <v>1.37</v>
+        <v>1.41</v>
       </c>
       <c r="BS63" t="n">
         <v>0.19</v>
       </c>
       <c r="BT63" t="n">
-        <v>23603</v>
+        <v>24607</v>
       </c>
     </row>
     <row r="64">
@@ -15053,13 +15053,13 @@
         </is>
       </c>
       <c r="F64" t="n">
-        <v>61.4</v>
+        <v>63.5</v>
       </c>
       <c r="G64" t="n">
-        <v>235466795451</v>
+        <v>243585047500</v>
       </c>
       <c r="H64" t="n">
-        <v>0</v>
+        <v>13763400</v>
       </c>
       <c r="I64" t="n">
         <v>0</v>
@@ -15146,13 +15146,13 @@
         <v>41.22</v>
       </c>
       <c r="AK64" t="n">
-        <v>67511785535.99014</v>
+        <v>69839407527.063</v>
       </c>
       <c r="AL64" t="n">
-        <v>18822285807.43405</v>
+        <v>19471226818.54517</v>
       </c>
       <c r="AM64" t="n">
-        <v>20967657653.69546</v>
+        <v>21690565227.07035</v>
       </c>
       <c r="AN64" t="n">
         <v>1.4201</v>
@@ -15193,7 +15193,7 @@
         <v>38.98</v>
       </c>
       <c r="AZ64" t="n">
-        <v>24.56</v>
+        <v>25.4</v>
       </c>
       <c r="BA64" t="n">
         <v>6.69</v>
@@ -15202,28 +15202,28 @@
         <v>10.4</v>
       </c>
       <c r="BC64" t="n">
-        <v>-22.25</v>
+        <v>-24.82</v>
       </c>
       <c r="BD64" t="n">
-        <v>-36.52</v>
+        <v>-38.61</v>
       </c>
       <c r="BE64" t="n">
         <v>-60</v>
       </c>
       <c r="BF64" t="n">
-        <v>-89.09999999999999</v>
+        <v>-89.45999999999999</v>
       </c>
       <c r="BG64" t="n">
-        <v>-83.06999999999999</v>
+        <v>-83.63</v>
       </c>
       <c r="BH64" t="n">
         <v>21.37</v>
       </c>
       <c r="BI64" t="n">
-        <v>0.43</v>
+        <v>0</v>
       </c>
       <c r="BJ64" t="n">
-        <v>61.14</v>
+        <v>63.5</v>
       </c>
       <c r="BK64" t="n">
         <v>4.74</v>
@@ -15232,7 +15232,7 @@
         <v>1.57</v>
       </c>
       <c r="BM64" t="n">
-        <v>61.6</v>
+        <v>63.77</v>
       </c>
       <c r="BN64" t="n">
         <v>64.72</v>
@@ -15241,19 +15241,19 @@
         <v>44.12</v>
       </c>
       <c r="BP64" t="n">
-        <v>60.48</v>
+        <v>61.68</v>
       </c>
       <c r="BQ64" t="n">
-        <v>39.11</v>
+        <v>40.44</v>
       </c>
       <c r="BR64" t="n">
-        <v>60.62</v>
+        <v>61.7</v>
       </c>
       <c r="BS64" t="n">
         <v>3.49</v>
       </c>
       <c r="BT64" t="n">
-        <v>12665342</v>
+        <v>12175841</v>
       </c>
     </row>
     <row r="65">
@@ -15283,13 +15283,13 @@
         </is>
       </c>
       <c r="F65" t="n">
-        <v>23.75</v>
+        <v>24.11</v>
       </c>
       <c r="G65" t="n">
-        <v>235466795451</v>
+        <v>243585047500</v>
       </c>
       <c r="H65" t="n">
-        <v>3900</v>
+        <v>6200</v>
       </c>
       <c r="I65" t="n">
         <v>7298813414</v>
@@ -15304,7 +15304,7 @@
         <v>3.29</v>
       </c>
       <c r="M65" t="n">
-        <v>5.692631797408119</v>
+        <v>5.888898195245635</v>
       </c>
       <c r="N65" t="n">
         <v>0.29</v>
@@ -15382,7 +15382,7 @@
         <v>11532125194.12</v>
       </c>
       <c r="AM65" t="n">
-        <v>17637962206.06742</v>
+        <v>18246070973.78277</v>
       </c>
       <c r="AN65" t="n">
         <v>0.4734</v>
@@ -15423,7 +15423,7 @@
         <v>12.99</v>
       </c>
       <c r="AZ65" t="n">
-        <v>8</v>
+        <v>8.119999999999999</v>
       </c>
       <c r="BA65" t="n">
         <v>2.23</v>
@@ -15432,19 +15432,19 @@
         <v>3.47</v>
       </c>
       <c r="BC65" t="n">
-        <v>-33.01</v>
+        <v>-34.01</v>
       </c>
       <c r="BD65" t="n">
-        <v>-45.3</v>
+        <v>-46.12</v>
       </c>
       <c r="BE65" t="n">
         <v>-66.33</v>
       </c>
       <c r="BF65" t="n">
-        <v>-90.61</v>
+        <v>-90.75</v>
       </c>
       <c r="BG65" t="n">
-        <v>-85.41</v>
+        <v>-85.63</v>
       </c>
       <c r="BH65" t="n">
         <v>7.12</v>
@@ -15453,7 +15453,7 @@
         <v>0</v>
       </c>
       <c r="BJ65" t="n">
-        <v>23.75</v>
+        <v>24.11</v>
       </c>
       <c r="BK65" t="n">
         <v>1.58</v>
@@ -15462,7 +15462,7 @@
         <v>1.57</v>
       </c>
       <c r="BM65" t="n">
-        <v>24.08</v>
+        <v>24.29</v>
       </c>
       <c r="BN65" t="n">
         <v>46.43</v>
@@ -15471,19 +15471,19 @@
         <v>20.44</v>
       </c>
       <c r="BP65" t="n">
-        <v>23.66</v>
+        <v>23.85</v>
       </c>
       <c r="BQ65" t="n">
-        <v>15.13</v>
+        <v>15.36</v>
       </c>
       <c r="BR65" t="n">
-        <v>23.66</v>
+        <v>23.91</v>
       </c>
       <c r="BS65" t="n">
         <v>4.14</v>
       </c>
       <c r="BT65" t="n">
-        <v>11531</v>
+        <v>11230</v>
       </c>
     </row>
     <row r="66">
@@ -15513,13 +15513,13 @@
         </is>
       </c>
       <c r="F66" t="n">
-        <v>20.91</v>
+        <v>20.35</v>
       </c>
       <c r="G66" t="n">
-        <v>235466795451</v>
+        <v>243585047500</v>
       </c>
       <c r="H66" t="n">
-        <v>600</v>
+        <v>5500</v>
       </c>
       <c r="I66" t="n">
         <v>2972355254</v>
@@ -15534,7 +15534,7 @@
         <v>2.75</v>
       </c>
       <c r="M66" t="n">
-        <v>13.97863100918734</v>
+        <v>14.46057603084185</v>
       </c>
       <c r="N66" t="n">
         <v>0.25</v>
@@ -15612,7 +15612,7 @@
         <v>4696321301.320001</v>
       </c>
       <c r="AM66" t="n">
-        <v>21118098246.72646</v>
+        <v>21846192600.89686</v>
       </c>
       <c r="AN66" t="n">
         <v>0.4734</v>
@@ -15653,7 +15653,7 @@
         <v>12.99</v>
       </c>
       <c r="AZ66" t="n">
-        <v>8.4</v>
+        <v>8.17</v>
       </c>
       <c r="BA66" t="n">
         <v>2.23</v>
@@ -15662,19 +15662,19 @@
         <v>3.47</v>
       </c>
       <c r="BC66" t="n">
-        <v>-23.91</v>
+        <v>-21.82</v>
       </c>
       <c r="BD66" t="n">
-        <v>-37.88</v>
+        <v>-36.17</v>
       </c>
       <c r="BE66" t="n">
         <v>-59.83</v>
       </c>
       <c r="BF66" t="n">
-        <v>-89.33</v>
+        <v>-89.04000000000001</v>
       </c>
       <c r="BG66" t="n">
-        <v>-83.43000000000001</v>
+        <v>-82.97</v>
       </c>
       <c r="BH66" t="n">
         <v>7.12</v>
@@ -15683,7 +15683,7 @@
         <v>0</v>
       </c>
       <c r="BJ66" t="n">
-        <v>20.91</v>
+        <v>20.35</v>
       </c>
       <c r="BK66" t="n">
         <v>1.58</v>
@@ -15701,19 +15701,19 @@
         <v>9.48</v>
       </c>
       <c r="BP66" t="n">
+        <v>19.51</v>
+      </c>
+      <c r="BQ66" t="n">
+        <v>12.96</v>
+      </c>
+      <c r="BR66" t="n">
         <v>20.91</v>
-      </c>
-      <c r="BQ66" t="n">
-        <v>13.32</v>
-      </c>
-      <c r="BR66" t="n">
-        <v>20.99</v>
       </c>
       <c r="BS66" t="n">
         <v>3.46</v>
       </c>
       <c r="BT66" t="n">
-        <v>6009</v>
+        <v>5614</v>
       </c>
     </row>
     <row r="67">
@@ -15973,13 +15973,13 @@
         </is>
       </c>
       <c r="F68" t="n">
-        <v>18.51</v>
+        <v>18.5</v>
       </c>
       <c r="G68" t="n">
-        <v>7943322285</v>
+        <v>7853534567</v>
       </c>
       <c r="H68" t="n">
-        <v>0</v>
+        <v>31600</v>
       </c>
       <c r="I68" t="n">
         <v>137989898</v>
@@ -16072,7 +16072,7 @@
         <v>205604948.02</v>
       </c>
       <c r="AM68" t="n">
-        <v>550854527.3925104</v>
+        <v>544627917.2676837</v>
       </c>
       <c r="AN68" t="n">
         <v>0.1911</v>
@@ -16113,7 +16113,7 @@
         <v>21.39</v>
       </c>
       <c r="AZ68" t="n">
-        <v>34.24</v>
+        <v>34.22</v>
       </c>
       <c r="BA68" t="n">
         <v>1.24</v>
@@ -16122,10 +16122,10 @@
         <v>63.25</v>
       </c>
       <c r="BC68" t="n">
-        <v>41.56</v>
+        <v>41.64</v>
       </c>
       <c r="BD68" t="n">
-        <v>15.58</v>
+        <v>15.65</v>
       </c>
       <c r="BE68" t="n">
         <v>85</v>
@@ -16134,7 +16134,7 @@
         <v>-93.3</v>
       </c>
       <c r="BG68" t="n">
-        <v>241.7</v>
+        <v>241.88</v>
       </c>
       <c r="BH68" t="n">
         <v>20.48</v>
@@ -16143,7 +16143,7 @@
         <v>0</v>
       </c>
       <c r="BJ68" t="n">
-        <v>18.51</v>
+        <v>18.5</v>
       </c>
       <c r="BK68" t="n">
         <v>1.49</v>
@@ -16152,7 +16152,7 @@
         <v>1.49</v>
       </c>
       <c r="BM68" t="n">
-        <v>18.62</v>
+        <v>18.69</v>
       </c>
       <c r="BN68" t="n">
         <v>22.11</v>
@@ -16161,19 +16161,19 @@
         <v>15.39</v>
       </c>
       <c r="BP68" t="n">
-        <v>18.5</v>
+        <v>18.47</v>
       </c>
       <c r="BQ68" t="n">
-        <v>12.45</v>
+        <v>12.44</v>
       </c>
       <c r="BR68" t="n">
-        <v>18.62</v>
+        <v>18.61</v>
       </c>
       <c r="BS68" t="n">
         <v>0</v>
       </c>
       <c r="BT68" t="n">
-        <v>35050</v>
+        <v>34920</v>
       </c>
     </row>
     <row r="69">
@@ -16203,13 +16203,13 @@
         </is>
       </c>
       <c r="F69" t="n">
-        <v>21.2</v>
+        <v>20.91</v>
       </c>
       <c r="G69" t="n">
-        <v>7943322285</v>
+        <v>7853534567</v>
       </c>
       <c r="H69" t="n">
-        <v>0</v>
+        <v>1387800</v>
       </c>
       <c r="I69" t="n">
         <v>255106712</v>
@@ -16302,7 +16302,7 @@
         <v>380109000.88</v>
       </c>
       <c r="AM69" t="n">
-        <v>472816802.6785714</v>
+        <v>467472295.6547619</v>
       </c>
       <c r="AN69" t="n">
         <v>0.8856000000000001</v>
@@ -16343,7 +16343,7 @@
         <v>21.39</v>
       </c>
       <c r="AZ69" t="n">
-        <v>37.06</v>
+        <v>36.56</v>
       </c>
       <c r="BA69" t="n">
         <v>1.24</v>
@@ -16352,28 +16352,28 @@
         <v>69.59</v>
       </c>
       <c r="BC69" t="n">
-        <v>23.6</v>
+        <v>25.31</v>
       </c>
       <c r="BD69" t="n">
-        <v>0.92</v>
+        <v>2.32</v>
       </c>
       <c r="BE69" t="n">
         <v>74.83</v>
       </c>
       <c r="BF69" t="n">
-        <v>-94.15000000000001</v>
+        <v>-94.06999999999999</v>
       </c>
       <c r="BG69" t="n">
-        <v>228.24</v>
+        <v>232.79</v>
       </c>
       <c r="BH69" t="n">
         <v>20.48</v>
       </c>
       <c r="BI69" t="n">
-        <v>-0.75</v>
+        <v>0</v>
       </c>
       <c r="BJ69" t="n">
-        <v>21.36</v>
+        <v>20.91</v>
       </c>
       <c r="BK69" t="n">
         <v>1.49</v>
@@ -16382,7 +16382,7 @@
         <v>1.49</v>
       </c>
       <c r="BM69" t="n">
-        <v>21.28</v>
+        <v>21.35</v>
       </c>
       <c r="BN69" t="n">
         <v>25.63</v>
@@ -16391,19 +16391,19 @@
         <v>16.73</v>
       </c>
       <c r="BP69" t="n">
-        <v>21</v>
+        <v>20.86</v>
       </c>
       <c r="BQ69" t="n">
-        <v>14.26</v>
+        <v>14.06</v>
       </c>
       <c r="BR69" t="n">
-        <v>21.12</v>
+        <v>21.35</v>
       </c>
       <c r="BS69" t="n">
         <v>0</v>
       </c>
       <c r="BT69" t="n">
-        <v>2014377</v>
+        <v>2035450</v>
       </c>
     </row>
     <row r="70">
@@ -16433,13 +16433,13 @@
         </is>
       </c>
       <c r="F70" t="n">
-        <v>17.35</v>
+        <v>17.4</v>
       </c>
       <c r="G70" t="n">
-        <v>8060067597</v>
+        <v>8083295102</v>
       </c>
       <c r="H70" t="n">
-        <v>0</v>
+        <v>2112600</v>
       </c>
       <c r="I70" t="n">
         <v>464557268</v>
@@ -16454,7 +16454,7 @@
         <v>0.68</v>
       </c>
       <c r="M70" t="n">
-        <v>0.6361665875174727</v>
+        <v>0.6379998925629409</v>
       </c>
       <c r="N70" t="n">
         <v>0.2</v>
@@ -16532,7 +16532,7 @@
         <v>55746872.16</v>
       </c>
       <c r="AM70" t="n">
-        <v>2660088315.841584</v>
+        <v>2667754159.075908</v>
       </c>
       <c r="AN70" t="n">
         <v>0.1236</v>
@@ -16582,10 +16582,10 @@
         <v>1.07</v>
       </c>
       <c r="BC70" t="n">
-        <v>-51.3</v>
+        <v>-51.44</v>
       </c>
       <c r="BD70" t="n">
-        <v>-60.24</v>
+        <v>-60.35</v>
       </c>
       <c r="BE70" t="n">
         <v>-88.5</v>
@@ -16594,7 +16594,7 @@
         <v>-99.31</v>
       </c>
       <c r="BG70" t="n">
-        <v>-93.84</v>
+        <v>-93.84999999999999</v>
       </c>
       <c r="BH70" t="n">
         <v>26.44</v>
@@ -16603,7 +16603,7 @@
         <v>0</v>
       </c>
       <c r="BJ70" t="n">
-        <v>17.35</v>
+        <v>17.4</v>
       </c>
       <c r="BK70" t="n">
         <v>0.12</v>
@@ -16612,7 +16612,7 @@
         <v>0.1</v>
       </c>
       <c r="BM70" t="n">
-        <v>17.54</v>
+        <v>17.41</v>
       </c>
       <c r="BN70" t="n">
         <v>22.15</v>
@@ -16621,19 +16621,19 @@
         <v>13.21</v>
       </c>
       <c r="BP70" t="n">
-        <v>17.34</v>
+        <v>17.08</v>
       </c>
       <c r="BQ70" t="n">
-        <v>174</v>
+        <v>174.51</v>
       </c>
       <c r="BR70" t="n">
-        <v>17.5</v>
+        <v>17.31</v>
       </c>
       <c r="BS70" t="n">
         <v>0.67</v>
       </c>
       <c r="BT70" t="n">
-        <v>4576120</v>
+        <v>4561720</v>
       </c>
     </row>
     <row r="71">

</xml_diff>

<commit_message>
📊 Dados atualizados - 2026-09-23 05:25
</commit_message>
<xml_diff>
--- a/data/ativos.xlsx
+++ b/data/ativos.xlsx
@@ -1047,13 +1047,13 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>25.28</v>
+        <v>25.25</v>
       </c>
       <c r="G3" t="n">
-        <v>3381624795</v>
+        <v>3377611700</v>
       </c>
       <c r="H3" t="n">
-        <v>583300</v>
+        <v>448200</v>
       </c>
       <c r="I3" t="n">
         <v>129510368</v>
@@ -1068,7 +1068,7 @@
         <v>0.88</v>
       </c>
       <c r="M3" t="n">
-        <v>0.8414235625930282</v>
+        <v>0.840425015179691</v>
       </c>
       <c r="N3" t="n">
         <v>0.09</v>
@@ -1146,7 +1146,7 @@
         <v>506385538.88</v>
       </c>
       <c r="AM3" t="n">
-        <v>660473592.7734375</v>
+        <v>659689785.15625</v>
       </c>
       <c r="AN3" t="n">
         <v>2.7</v>
@@ -1187,7 +1187,7 @@
         <v>40.42</v>
       </c>
       <c r="AZ3" t="n">
-        <v>46.26</v>
+        <v>46.21</v>
       </c>
       <c r="BA3" t="n">
         <v>4.87</v>
@@ -1196,19 +1196,19 @@
         <v>21.14</v>
       </c>
       <c r="BC3" t="n">
-        <v>95.8</v>
+        <v>96.03</v>
       </c>
       <c r="BD3" t="n">
-        <v>59.87</v>
+        <v>60.06</v>
       </c>
       <c r="BE3" t="n">
         <v>83</v>
       </c>
       <c r="BF3" t="n">
-        <v>-80.73999999999999</v>
+        <v>-80.72</v>
       </c>
       <c r="BG3" t="n">
-        <v>-16.39</v>
+        <v>-16.29</v>
       </c>
       <c r="BH3" t="n">
         <v>27.85</v>
@@ -1217,7 +1217,7 @@
         <v>0</v>
       </c>
       <c r="BJ3" t="n">
-        <v>25.28</v>
+        <v>25.25</v>
       </c>
       <c r="BK3" t="n">
         <v>3.91</v>
@@ -1226,7 +1226,7 @@
         <v>4.39</v>
       </c>
       <c r="BM3" t="n">
-        <v>25.4</v>
+        <v>25.29</v>
       </c>
       <c r="BN3" t="n">
         <v>27.17</v>
@@ -1235,13 +1235,13 @@
         <v>18.72</v>
       </c>
       <c r="BP3" t="n">
-        <v>24.85</v>
+        <v>24.88</v>
       </c>
       <c r="BQ3" t="n">
         <v>5.75</v>
       </c>
       <c r="BR3" t="n">
-        <v>24.85</v>
+        <v>25.16</v>
       </c>
       <c r="BS3" t="n">
         <v>0.79</v>
@@ -1277,13 +1277,13 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>15.5</v>
+        <v>15.6</v>
       </c>
       <c r="G4" t="n">
-        <v>240012230000</v>
+        <v>241560701906</v>
       </c>
       <c r="H4" t="n">
-        <v>18020800</v>
+        <v>24129900</v>
       </c>
       <c r="I4" t="n">
         <v>15484664889</v>
@@ -1298,7 +1298,7 @@
         <v>2.76</v>
       </c>
       <c r="M4" t="n">
-        <v>2.717665808613074</v>
+        <v>2.735199203284397</v>
       </c>
       <c r="N4" t="n">
         <v>1.76</v>
@@ -1376,7 +1376,7 @@
         <v>16258898133.45</v>
       </c>
       <c r="AM4" t="n">
-        <v>23763587128.71287</v>
+        <v>23916901178.81188</v>
       </c>
       <c r="AN4" t="n">
         <v>0.269</v>
@@ -1417,7 +1417,7 @@
         <v>9.470000000000001</v>
       </c>
       <c r="AZ4" t="n">
-        <v>19.35</v>
+        <v>19.47</v>
       </c>
       <c r="BA4" t="n">
         <v>1.13</v>
@@ -1426,28 +1426,28 @@
         <v>11.39</v>
       </c>
       <c r="BC4" t="n">
-        <v>-25.13</v>
+        <v>-25.61</v>
       </c>
       <c r="BD4" t="n">
-        <v>-38.87</v>
+        <v>-39.26</v>
       </c>
       <c r="BE4" t="n">
         <v>24.83</v>
       </c>
       <c r="BF4" t="n">
-        <v>-92.73</v>
+        <v>-92.77</v>
       </c>
       <c r="BG4" t="n">
-        <v>-26.54</v>
+        <v>-27.01</v>
       </c>
       <c r="BH4" t="n">
         <v>5.7</v>
       </c>
       <c r="BI4" t="n">
-        <v>0.38</v>
+        <v>0</v>
       </c>
       <c r="BJ4" t="n">
-        <v>15.44</v>
+        <v>15.6</v>
       </c>
       <c r="BK4" t="n">
         <v>1.05</v>
@@ -1456,7 +1456,7 @@
         <v>1.04</v>
       </c>
       <c r="BM4" t="n">
-        <v>15.62</v>
+        <v>15.61</v>
       </c>
       <c r="BN4" t="n">
         <v>17</v>
@@ -1465,13 +1465,13 @@
         <v>11.09</v>
       </c>
       <c r="BP4" t="n">
-        <v>15.42</v>
+        <v>15.31</v>
       </c>
       <c r="BQ4" t="n">
-        <v>14.95</v>
+        <v>15.04</v>
       </c>
       <c r="BR4" t="n">
-        <v>15.48</v>
+        <v>15.34</v>
       </c>
       <c r="BS4" t="n">
         <v>2.76</v>
@@ -3117,13 +3117,13 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>5.01</v>
+        <v>4.96</v>
       </c>
       <c r="G12" t="n">
-        <v>480767337</v>
+        <v>475969192</v>
       </c>
       <c r="H12" t="n">
-        <v>457100</v>
+        <v>344200</v>
       </c>
       <c r="I12" t="n">
         <v>95961536</v>
@@ -3138,7 +3138,7 @@
         <v>0.32</v>
       </c>
       <c r="M12" t="n">
-        <v>0.08694603927656219</v>
+        <v>0.0860783020749714</v>
       </c>
       <c r="N12" t="n">
         <v>0.14</v>
@@ -3216,7 +3216,7 @@
         <v>362734606.08</v>
       </c>
       <c r="AM12" t="n">
-        <v>516954125.8064516</v>
+        <v>511794830.1075268</v>
       </c>
       <c r="AN12" t="n">
         <v>0.4208</v>
@@ -3257,7 +3257,7 @@
         <v>30.49</v>
       </c>
       <c r="AZ12" t="n">
-        <v>6.77</v>
+        <v>6.7</v>
       </c>
       <c r="BA12" t="n">
         <v>4.41</v>
@@ -3266,19 +3266,19 @@
         <v>18.12</v>
       </c>
       <c r="BC12" t="n">
-        <v>645.45</v>
+        <v>652.97</v>
       </c>
       <c r="BD12" t="n">
-        <v>508.66</v>
+        <v>514.8</v>
       </c>
       <c r="BE12" t="n">
         <v>35.17</v>
       </c>
       <c r="BF12" t="n">
-        <v>-11.94</v>
+        <v>-11.06</v>
       </c>
       <c r="BG12" t="n">
-        <v>261.65</v>
+        <v>265.3</v>
       </c>
       <c r="BH12" t="n">
         <v>16.4</v>
@@ -3287,7 +3287,7 @@
         <v>0</v>
       </c>
       <c r="BJ12" t="n">
-        <v>5.01</v>
+        <v>4.96</v>
       </c>
       <c r="BK12" t="n">
         <v>3.78</v>
@@ -3296,7 +3296,7 @@
         <v>3.43</v>
       </c>
       <c r="BM12" t="n">
-        <v>5.08</v>
+        <v>5.02</v>
       </c>
       <c r="BN12" t="n">
         <v>8.23</v>
@@ -3308,10 +3308,10 @@
         <v>4.96</v>
       </c>
       <c r="BQ12" t="n">
-        <v>1.46</v>
+        <v>1.45</v>
       </c>
       <c r="BR12" t="n">
-        <v>5.05</v>
+        <v>5</v>
       </c>
       <c r="BS12" t="n">
         <v>0.09</v>
@@ -3347,13 +3347,13 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>29.7</v>
+        <v>29.72</v>
       </c>
       <c r="G13" t="n">
-        <v>14974467144</v>
+        <v>14984553201</v>
       </c>
       <c r="H13" t="n">
-        <v>5891600</v>
+        <v>11646700</v>
       </c>
       <c r="I13" t="n">
         <v>504190947</v>
@@ -3368,7 +3368,7 @@
         <v>1.13</v>
       </c>
       <c r="M13" t="n">
-        <v>5.179036460666611</v>
+        <v>5.182524802284717</v>
       </c>
       <c r="N13" t="n">
         <v>0.57</v>
@@ -3446,7 +3446,7 @@
         <v>932753251.95</v>
       </c>
       <c r="AM13" t="n">
-        <v>1558217184.599376</v>
+        <v>1559266722.268471</v>
       </c>
       <c r="AN13" t="n">
         <v>2.6301</v>
@@ -3487,7 +3487,7 @@
         <v>26.6</v>
       </c>
       <c r="AZ13" t="n">
-        <v>53.76</v>
+        <v>53.79</v>
       </c>
       <c r="BA13" t="n">
         <v>2.6</v>
@@ -3496,28 +3496,28 @@
         <v>8.69</v>
       </c>
       <c r="BC13" t="n">
-        <v>9.67</v>
+        <v>9.6</v>
       </c>
       <c r="BD13" t="n">
-        <v>-10.45</v>
+        <v>-10.51</v>
       </c>
       <c r="BE13" t="n">
         <v>81</v>
       </c>
       <c r="BF13" t="n">
-        <v>-91.23</v>
+        <v>-91.23999999999999</v>
       </c>
       <c r="BG13" t="n">
-        <v>-70.73</v>
+        <v>-70.75</v>
       </c>
       <c r="BH13" t="n">
         <v>25.49</v>
       </c>
       <c r="BI13" t="n">
-        <v>0</v>
+        <v>0.99</v>
       </c>
       <c r="BJ13" t="n">
-        <v>29.7</v>
+        <v>29.43</v>
       </c>
       <c r="BK13" t="n">
         <v>1.85</v>
@@ -3526,7 +3526,7 @@
         <v>1.96</v>
       </c>
       <c r="BM13" t="n">
-        <v>29.87</v>
+        <v>29.83</v>
       </c>
       <c r="BN13" t="n">
         <v>32.43</v>
@@ -3535,13 +3535,13 @@
         <v>21.06</v>
       </c>
       <c r="BP13" t="n">
-        <v>29.01</v>
+        <v>29.43</v>
       </c>
       <c r="BQ13" t="n">
-        <v>15.17</v>
+        <v>15.18</v>
       </c>
       <c r="BR13" t="n">
-        <v>29.01</v>
+        <v>29.69</v>
       </c>
       <c r="BS13" t="n">
         <v>5.01</v>
@@ -3577,13 +3577,13 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>9.640000000000001</v>
+        <v>10.2</v>
       </c>
       <c r="G14" t="n">
-        <v>7832120285</v>
+        <v>8167853032</v>
       </c>
       <c r="H14" t="n">
-        <v>9300</v>
+        <v>19400</v>
       </c>
       <c r="I14" t="n">
         <v>339510689</v>
@@ -3598,7 +3598,7 @@
         <v>1.92</v>
       </c>
       <c r="M14" t="n">
-        <v>3.252035579288342</v>
+        <v>3.391437784393292</v>
       </c>
       <c r="N14" t="n">
         <v>1.11</v>
@@ -3676,7 +3676,7 @@
         <v>349696009.67</v>
       </c>
       <c r="AM14" t="n">
-        <v>869269731.964484</v>
+        <v>906531968.0355161</v>
       </c>
       <c r="AN14" t="n">
         <v>0.1489</v>
@@ -3717,7 +3717,7 @@
         <v>9.050000000000001</v>
       </c>
       <c r="AZ14" t="n">
-        <v>7.74</v>
+        <v>8.19</v>
       </c>
       <c r="BA14" t="n">
         <v>1.42</v>
@@ -3726,19 +3726,19 @@
         <v>5.94</v>
       </c>
       <c r="BC14" t="n">
-        <v>14.97</v>
+        <v>8.65</v>
       </c>
       <c r="BD14" t="n">
-        <v>-6.13</v>
+        <v>-11.28</v>
       </c>
       <c r="BE14" t="n">
         <v>-19.67</v>
       </c>
       <c r="BF14" t="n">
-        <v>-85.26000000000001</v>
+        <v>-86.06999999999999</v>
       </c>
       <c r="BG14" t="n">
-        <v>-38.36</v>
+        <v>-41.74</v>
       </c>
       <c r="BH14" t="n">
         <v>5.3</v>
@@ -3747,7 +3747,7 @@
         <v>0</v>
       </c>
       <c r="BJ14" t="n">
-        <v>9.640000000000001</v>
+        <v>10.2</v>
       </c>
       <c r="BK14" t="n">
         <v>1.03</v>
@@ -3756,7 +3756,7 @@
         <v>1.01</v>
       </c>
       <c r="BM14" t="n">
-        <v>9.699999999999999</v>
+        <v>10.2</v>
       </c>
       <c r="BN14" t="n">
         <v>13.49</v>
@@ -3765,13 +3765,13 @@
         <v>7.65</v>
       </c>
       <c r="BP14" t="n">
-        <v>9.539999999999999</v>
+        <v>9.640000000000001</v>
       </c>
       <c r="BQ14" t="n">
-        <v>9.52</v>
+        <v>10.07</v>
       </c>
       <c r="BR14" t="n">
-        <v>9.539999999999999</v>
+        <v>9.66</v>
       </c>
       <c r="BS14" t="n">
         <v>1.44</v>
@@ -3807,13 +3807,13 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>13.18</v>
+        <v>13.8</v>
       </c>
       <c r="G15" t="n">
-        <v>7832120285</v>
+        <v>8167853032</v>
       </c>
       <c r="H15" t="n">
-        <v>1214600</v>
+        <v>2427800</v>
       </c>
       <c r="I15" t="n">
         <v>343551533</v>
@@ -3828,7 +3828,7 @@
         <v>2.56</v>
       </c>
       <c r="M15" t="n">
-        <v>3.213785223239563</v>
+        <v>3.351547783313195</v>
       </c>
       <c r="N15" t="n">
         <v>1.47</v>
@@ -3906,7 +3906,7 @@
         <v>353858078.99</v>
       </c>
       <c r="AM15" t="n">
-        <v>653221041.2844037</v>
+        <v>681222104.4203503</v>
       </c>
       <c r="AN15" t="n">
         <v>0.1638</v>
@@ -3947,7 +3947,7 @@
         <v>9.050000000000001</v>
       </c>
       <c r="AZ15" t="n">
-        <v>8.76</v>
+        <v>9.18</v>
       </c>
       <c r="BA15" t="n">
         <v>1.42</v>
@@ -3956,19 +3956,19 @@
         <v>6.19</v>
       </c>
       <c r="BC15" t="n">
-        <v>-15.91</v>
+        <v>-19.69</v>
       </c>
       <c r="BD15" t="n">
-        <v>-31.34</v>
+        <v>-34.43</v>
       </c>
       <c r="BE15" t="n">
         <v>-33.5</v>
       </c>
       <c r="BF15" t="n">
-        <v>-89.22</v>
+        <v>-89.7</v>
       </c>
       <c r="BG15" t="n">
-        <v>-53.05</v>
+        <v>-55.16</v>
       </c>
       <c r="BH15" t="n">
         <v>5.3</v>
@@ -3977,7 +3977,7 @@
         <v>0</v>
       </c>
       <c r="BJ15" t="n">
-        <v>13.18</v>
+        <v>13.8</v>
       </c>
       <c r="BK15" t="n">
         <v>1.03</v>
@@ -3986,7 +3986,7 @@
         <v>1.01</v>
       </c>
       <c r="BM15" t="n">
-        <v>13.28</v>
+        <v>13.8</v>
       </c>
       <c r="BN15" t="n">
         <v>16.22</v>
@@ -3995,13 +3995,13 @@
         <v>7.84</v>
       </c>
       <c r="BP15" t="n">
-        <v>12.9</v>
+        <v>13.09</v>
       </c>
       <c r="BQ15" t="n">
-        <v>13.01</v>
+        <v>13.62</v>
       </c>
       <c r="BR15" t="n">
-        <v>13</v>
+        <v>13.09</v>
       </c>
       <c r="BS15" t="n">
         <v>1.92</v>
@@ -4037,13 +4037,13 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>4.4</v>
+        <v>4.41</v>
       </c>
       <c r="G16" t="n">
-        <v>964945100</v>
+        <v>967138103</v>
       </c>
       <c r="H16" t="n">
-        <v>61400</v>
+        <v>147600</v>
       </c>
       <c r="I16" t="n">
         <v>219305733</v>
@@ -4058,7 +4058,7 @@
         <v>2.69</v>
       </c>
       <c r="M16" t="n">
-        <v>0.4564999407699022</v>
+        <v>0.4575374150672568</v>
       </c>
       <c r="N16" t="n">
         <v>0.39</v>
@@ -4136,7 +4136,7 @@
         <v>17544458.64</v>
       </c>
       <c r="AM16" t="n">
-        <v>271051994.3820224</v>
+        <v>271668006.4606742</v>
       </c>
       <c r="AN16" t="n">
         <v>0.0077</v>
@@ -4186,16 +4186,16 @@
         <v>0</v>
       </c>
       <c r="BC16" t="n">
-        <v>-60.48</v>
+        <v>-60.57</v>
       </c>
       <c r="BD16" t="n">
-        <v>-67.73</v>
+        <v>-67.8</v>
       </c>
       <c r="BE16" t="n">
         <v>-97.17</v>
       </c>
       <c r="BF16" t="n">
-        <v>-98.18000000000001</v>
+        <v>-98.19</v>
       </c>
       <c r="BG16" t="n">
         <v>-100</v>
@@ -4207,7 +4207,7 @@
         <v>0</v>
       </c>
       <c r="BJ16" t="n">
-        <v>4.4</v>
+        <v>4.41</v>
       </c>
       <c r="BK16" t="n">
         <v>0.08</v>
@@ -4216,7 +4216,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="BM16" t="n">
-        <v>4.44</v>
+        <v>4.51</v>
       </c>
       <c r="BN16" t="n">
         <v>5.54</v>
@@ -4225,13 +4225,13 @@
         <v>3.19</v>
       </c>
       <c r="BP16" t="n">
-        <v>4.28</v>
+        <v>4.33</v>
       </c>
       <c r="BQ16" t="n">
-        <v>60.04</v>
+        <v>60.18</v>
       </c>
       <c r="BR16" t="n">
-        <v>4.35</v>
+        <v>4.33</v>
       </c>
       <c r="BS16" t="n">
         <v>0.49</v>
@@ -4267,13 +4267,13 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>32.65</v>
+        <v>32.57</v>
       </c>
       <c r="G17" t="n">
-        <v>10762318787</v>
+        <v>10735948032</v>
       </c>
       <c r="H17" t="n">
-        <v>1650300</v>
+        <v>1641000</v>
       </c>
       <c r="I17" t="n">
         <v>0</v>
@@ -4360,13 +4360,13 @@
         <v>8.039999999999999</v>
       </c>
       <c r="AK17" t="n">
-        <v>4860151186.325868</v>
+        <v>4848242427.745665</v>
       </c>
       <c r="AL17" t="n">
-        <v>1345289848.375</v>
+        <v>1341993504</v>
       </c>
       <c r="AM17" t="n">
-        <v>3331987240.557276</v>
+        <v>3323822920.123839</v>
       </c>
       <c r="AN17" t="n">
         <v>1.08</v>
@@ -4407,7 +4407,7 @@
         <v>42.98</v>
       </c>
       <c r="AZ17" t="n">
-        <v>17.47</v>
+        <v>17.42</v>
       </c>
       <c r="BA17" t="n">
         <v>4.55</v>
@@ -4416,19 +4416,19 @@
         <v>16.33</v>
       </c>
       <c r="BC17" t="n">
-        <v>61.22</v>
+        <v>61.61</v>
       </c>
       <c r="BD17" t="n">
-        <v>31.63</v>
+        <v>31.96</v>
       </c>
       <c r="BE17" t="n">
         <v>-46.5</v>
       </c>
       <c r="BF17" t="n">
-        <v>-86.06999999999999</v>
+        <v>-86.03</v>
       </c>
       <c r="BG17" t="n">
-        <v>-49.97</v>
+        <v>-49.85</v>
       </c>
       <c r="BH17" t="n">
         <v>29.25</v>
@@ -4437,7 +4437,7 @@
         <v>0</v>
       </c>
       <c r="BJ17" t="n">
-        <v>32.65</v>
+        <v>32.57</v>
       </c>
       <c r="BK17" t="n">
         <v>4.21</v>
@@ -4446,7 +4446,7 @@
         <v>12.62</v>
       </c>
       <c r="BM17" t="n">
-        <v>33.26</v>
+        <v>32.85</v>
       </c>
       <c r="BN17" t="n">
         <v>36.63</v>
@@ -4455,13 +4455,13 @@
         <v>29.53</v>
       </c>
       <c r="BP17" t="n">
-        <v>32.65</v>
+        <v>32.26</v>
       </c>
       <c r="BQ17" t="n">
-        <v>2.59</v>
+        <v>2.58</v>
       </c>
       <c r="BR17" t="n">
-        <v>32.81</v>
+        <v>32.6</v>
       </c>
       <c r="BS17" t="n">
         <v>2.21</v>
@@ -4497,13 +4497,13 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>11.2</v>
+        <v>11.06</v>
       </c>
       <c r="G18" t="n">
-        <v>10762318787</v>
+        <v>10735948032</v>
       </c>
       <c r="H18" t="n">
-        <v>8500</v>
+        <v>5300</v>
       </c>
       <c r="I18" t="n">
         <v>671494278</v>
@@ -4518,7 +4518,7 @@
         <v>1.2</v>
       </c>
       <c r="M18" t="n">
-        <v>3.168849298223123</v>
+        <v>3.161084712344446</v>
       </c>
       <c r="N18" t="n">
         <v>0.33</v>
@@ -4596,7 +4596,7 @@
         <v>940091989.1999999</v>
       </c>
       <c r="AM18" t="n">
-        <v>3203071067.559524</v>
+        <v>3195222628.571429</v>
       </c>
       <c r="AN18" t="n">
         <v>0.36</v>
@@ -4637,7 +4637,7 @@
         <v>14.31</v>
       </c>
       <c r="AZ18" t="n">
-        <v>5.77</v>
+        <v>5.7</v>
       </c>
       <c r="BA18" t="n">
         <v>1.51</v>
@@ -4646,19 +4646,19 @@
         <v>5.44</v>
       </c>
       <c r="BC18" t="n">
-        <v>56.47</v>
+        <v>58.45</v>
       </c>
       <c r="BD18" t="n">
-        <v>27.76</v>
+        <v>29.38</v>
       </c>
       <c r="BE18" t="n">
         <v>-48.5</v>
       </c>
       <c r="BF18" t="n">
-        <v>-86.5</v>
+        <v>-86.31999999999999</v>
       </c>
       <c r="BG18" t="n">
-        <v>-51.39</v>
+        <v>-50.77</v>
       </c>
       <c r="BH18" t="n">
         <v>9.75</v>
@@ -4667,7 +4667,7 @@
         <v>0</v>
       </c>
       <c r="BJ18" t="n">
-        <v>11.2</v>
+        <v>11.06</v>
       </c>
       <c r="BK18" t="n">
         <v>1.4</v>
@@ -4676,7 +4676,7 @@
         <v>12.62</v>
       </c>
       <c r="BM18" t="n">
-        <v>11.39</v>
+        <v>11.19</v>
       </c>
       <c r="BN18" t="n">
         <v>13.82</v>
@@ -4685,13 +4685,13 @@
         <v>10.19</v>
       </c>
       <c r="BP18" t="n">
-        <v>11.2</v>
+        <v>11.05</v>
       </c>
       <c r="BQ18" t="n">
-        <v>0.89</v>
+        <v>0.88</v>
       </c>
       <c r="BR18" t="n">
-        <v>11.39</v>
+        <v>11.1</v>
       </c>
       <c r="BS18" t="n">
         <v>2.3</v>
@@ -4727,13 +4727,13 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>10.91</v>
+        <v>10.8</v>
       </c>
       <c r="G19" t="n">
-        <v>10762318787</v>
+        <v>10735948032</v>
       </c>
       <c r="H19" t="n">
-        <v>8800</v>
+        <v>9600</v>
       </c>
       <c r="I19" t="n">
         <v>317386323</v>
@@ -4748,7 +4748,7 @@
         <v>1.12</v>
       </c>
       <c r="M19" t="n">
-        <v>6.70433480399577</v>
+        <v>6.687907268809978</v>
       </c>
       <c r="N19" t="n">
         <v>0.3</v>
@@ -4826,7 +4826,7 @@
         <v>444340852.2</v>
       </c>
       <c r="AM19" t="n">
-        <v>3416609138.730159</v>
+        <v>3408237470.476191</v>
       </c>
       <c r="AN19" t="n">
         <v>0.36</v>
@@ -4867,7 +4867,7 @@
         <v>14.31</v>
       </c>
       <c r="AZ19" t="n">
-        <v>6</v>
+        <v>5.94</v>
       </c>
       <c r="BA19" t="n">
         <v>1.51</v>
@@ -4876,19 +4876,19 @@
         <v>5.25</v>
       </c>
       <c r="BC19" t="n">
-        <v>60.63</v>
+        <v>62.27</v>
       </c>
       <c r="BD19" t="n">
-        <v>31.16</v>
+        <v>32.49</v>
       </c>
       <c r="BE19" t="n">
         <v>-45</v>
       </c>
       <c r="BF19" t="n">
-        <v>-86.14</v>
+        <v>-85.98999999999999</v>
       </c>
       <c r="BG19" t="n">
-        <v>-51.88</v>
+        <v>-51.39</v>
       </c>
       <c r="BH19" t="n">
         <v>9.75</v>
@@ -4897,7 +4897,7 @@
         <v>0</v>
       </c>
       <c r="BJ19" t="n">
-        <v>10.91</v>
+        <v>10.8</v>
       </c>
       <c r="BK19" t="n">
         <v>1.4</v>
@@ -4906,7 +4906,7 @@
         <v>12.62</v>
       </c>
       <c r="BM19" t="n">
-        <v>10.99</v>
+        <v>10.89</v>
       </c>
       <c r="BN19" t="n">
         <v>11.41</v>
@@ -4915,13 +4915,13 @@
         <v>9.19</v>
       </c>
       <c r="BP19" t="n">
-        <v>10.75</v>
+        <v>10.63</v>
       </c>
       <c r="BQ19" t="n">
         <v>0.86</v>
       </c>
       <c r="BR19" t="n">
-        <v>10.75</v>
+        <v>10.77</v>
       </c>
       <c r="BS19" t="n">
         <v>2.16</v>
@@ -5417,13 +5417,13 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>5.02</v>
+        <v>5.12</v>
       </c>
       <c r="G22" t="n">
-        <v>1005230900</v>
+        <v>1025255401</v>
       </c>
       <c r="H22" t="n">
-        <v>829100</v>
+        <v>1500800</v>
       </c>
       <c r="I22" t="n">
         <v>200245299</v>
@@ -5438,7 +5438,7 @@
         <v>0.27</v>
       </c>
       <c r="M22" t="n">
-        <v>0.0852602749688933</v>
+        <v>0.08695868521610603</v>
       </c>
       <c r="N22" t="n">
         <v>0.08</v>
@@ -5516,7 +5516,7 @@
         <v>378463615.11</v>
       </c>
       <c r="AM22" t="n">
-        <v>227943514.739229</v>
+        <v>232484217.9138322</v>
       </c>
       <c r="AN22" t="n">
         <v>0</v>
@@ -5566,19 +5566,19 @@
         <v>172.49</v>
       </c>
       <c r="BC22" t="n">
-        <v>491.74</v>
+        <v>480.18</v>
       </c>
       <c r="BD22" t="n">
-        <v>383.15</v>
+        <v>373.71</v>
       </c>
       <c r="BE22" t="n">
         <v>-100</v>
       </c>
       <c r="BF22" t="n">
-        <v>-62.35</v>
+        <v>-63.09</v>
       </c>
       <c r="BG22" t="n">
-        <v>3336.05</v>
+        <v>3268.94</v>
       </c>
       <c r="BH22" t="n">
         <v>20.75</v>
@@ -5587,7 +5587,7 @@
         <v>0</v>
       </c>
       <c r="BJ22" t="n">
-        <v>5.02</v>
+        <v>5.12</v>
       </c>
       <c r="BK22" t="n">
         <v>1.89</v>
@@ -5596,7 +5596,7 @@
         <v>0.67</v>
       </c>
       <c r="BM22" t="n">
-        <v>5.02</v>
+        <v>5.41</v>
       </c>
       <c r="BN22" t="n">
         <v>7.89</v>
@@ -5605,13 +5605,13 @@
         <v>3.37</v>
       </c>
       <c r="BP22" t="n">
-        <v>4.8</v>
+        <v>4.95</v>
       </c>
       <c r="BQ22" t="n">
-        <v>7.48</v>
+        <v>7.63</v>
       </c>
       <c r="BR22" t="n">
-        <v>4.87</v>
+        <v>5.01</v>
       </c>
       <c r="BS22" t="n">
         <v>0.09</v>
@@ -5877,13 +5877,13 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.96</v>
+        <v>3</v>
       </c>
       <c r="G24" t="n">
-        <v>1195451959</v>
+        <v>1211606700</v>
       </c>
       <c r="H24" t="n">
-        <v>4018900</v>
+        <v>3762700</v>
       </c>
       <c r="I24" t="n">
         <v>403868805</v>
@@ -5898,7 +5898,7 @@
         <v>0.49</v>
       </c>
       <c r="M24" t="n">
-        <v>0.2889895452878435</v>
+        <v>0.292894805738241</v>
       </c>
       <c r="N24" t="n">
         <v>0.11</v>
@@ -5976,7 +5976,7 @@
         <v>153470145.9</v>
       </c>
       <c r="AM24" t="n">
-        <v>1076983746.846847</v>
+        <v>1091537567.567568</v>
       </c>
       <c r="AN24" t="n">
         <v>0.0813</v>
@@ -6017,7 +6017,7 @@
         <v>5.84</v>
       </c>
       <c r="AZ24" t="n">
-        <v>1.37</v>
+        <v>1.38</v>
       </c>
       <c r="BA24" t="n">
         <v>0.38</v>
@@ -6026,19 +6026,19 @@
         <v>1.46</v>
       </c>
       <c r="BC24" t="n">
-        <v>141.77</v>
+        <v>138.55</v>
       </c>
       <c r="BD24" t="n">
-        <v>97.41</v>
+        <v>94.77</v>
       </c>
       <c r="BE24" t="n">
         <v>-53.83</v>
       </c>
       <c r="BF24" t="n">
-        <v>-87.16</v>
+        <v>-87.33</v>
       </c>
       <c r="BG24" t="n">
-        <v>-50.75</v>
+        <v>-51.41</v>
       </c>
       <c r="BH24" t="n">
         <v>5.99</v>
@@ -6047,7 +6047,7 @@
         <v>0</v>
       </c>
       <c r="BJ24" t="n">
-        <v>2.96</v>
+        <v>3</v>
       </c>
       <c r="BK24" t="n">
         <v>0.38</v>
@@ -6056,7 +6056,7 @@
         <v>0.41</v>
       </c>
       <c r="BM24" t="n">
-        <v>2.97</v>
+        <v>3.03</v>
       </c>
       <c r="BN24" t="n">
         <v>5.29</v>
@@ -6065,13 +6065,13 @@
         <v>1.92</v>
       </c>
       <c r="BP24" t="n">
-        <v>2.86</v>
+        <v>2.89</v>
       </c>
       <c r="BQ24" t="n">
-        <v>7.27</v>
+        <v>7.37</v>
       </c>
       <c r="BR24" t="n">
-        <v>2.88</v>
+        <v>2.93</v>
       </c>
       <c r="BS24" t="n">
         <v>0.29</v>
@@ -6107,13 +6107,13 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>4.54</v>
+        <v>4.52</v>
       </c>
       <c r="G25" t="n">
-        <v>1573083200</v>
+        <v>1566152873</v>
       </c>
       <c r="H25" t="n">
-        <v>1673400</v>
+        <v>619300</v>
       </c>
       <c r="I25" t="n">
         <v>346494097</v>
@@ -6128,7 +6128,7 @@
         <v>0.97</v>
       </c>
       <c r="M25" t="n">
-        <v>0.7844111109216257</v>
+        <v>0.7809553334388326</v>
       </c>
       <c r="N25" t="n">
         <v>0.22</v>
@@ -6206,7 +6206,7 @@
         <v>62368937.46</v>
       </c>
       <c r="AM25" t="n">
-        <v>578339411.7647059</v>
+        <v>575791497.4264705</v>
       </c>
       <c r="AN25" t="n">
         <v>0.4742</v>
@@ -6247,7 +6247,7 @@
         <v>3.27</v>
       </c>
       <c r="AZ25" t="n">
-        <v>10.58</v>
+        <v>10.53</v>
       </c>
       <c r="BA25" t="n">
         <v>0.23</v>
@@ -6256,19 +6256,19 @@
         <v>2.2</v>
       </c>
       <c r="BC25" t="n">
-        <v>-11.68</v>
+        <v>-11.29</v>
       </c>
       <c r="BD25" t="n">
-        <v>-27.89</v>
+        <v>-27.57</v>
       </c>
       <c r="BE25" t="n">
         <v>133</v>
       </c>
       <c r="BF25" t="n">
-        <v>-94.90000000000001</v>
+        <v>-94.87</v>
       </c>
       <c r="BG25" t="n">
-        <v>-51.55</v>
+        <v>-51.33</v>
       </c>
       <c r="BH25" t="n">
         <v>3.97</v>
@@ -6277,7 +6277,7 @@
         <v>0</v>
       </c>
       <c r="BJ25" t="n">
-        <v>4.54</v>
+        <v>4.52</v>
       </c>
       <c r="BK25" t="n">
         <v>0.18</v>
@@ -6286,7 +6286,7 @@
         <v>0.24</v>
       </c>
       <c r="BM25" t="n">
-        <v>4.54</v>
+        <v>4.58</v>
       </c>
       <c r="BN25" t="n">
         <v>6.3</v>
@@ -6295,13 +6295,13 @@
         <v>2.64</v>
       </c>
       <c r="BP25" t="n">
-        <v>4.07</v>
+        <v>4.42</v>
       </c>
       <c r="BQ25" t="n">
-        <v>19.18</v>
+        <v>19.1</v>
       </c>
       <c r="BR25" t="n">
-        <v>4.12</v>
+        <v>4.52</v>
       </c>
       <c r="BS25" t="n">
         <v>0.67</v>
@@ -6337,13 +6337,13 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>10.22</v>
+        <v>10.34</v>
       </c>
       <c r="G26" t="n">
-        <v>13841896821</v>
+        <v>14004423826</v>
       </c>
       <c r="H26" t="n">
-        <v>6225700</v>
+        <v>15338300</v>
       </c>
       <c r="I26" t="n">
         <v>1354393401</v>
@@ -6358,7 +6358,7 @@
         <v>1.94</v>
       </c>
       <c r="M26" t="n">
-        <v>0.1784900926539336</v>
+        <v>0.1805858646826056</v>
       </c>
       <c r="N26" t="n">
         <v>0.26</v>
@@ -6436,7 +6436,7 @@
         <v>961619314.7099999</v>
       </c>
       <c r="AM26" t="n">
-        <v>4943534578.928572</v>
+        <v>5001579937.857143</v>
       </c>
       <c r="AN26" t="n">
         <v>0.1043</v>
@@ -6477,7 +6477,7 @@
         <v>7.07</v>
       </c>
       <c r="AZ26" t="n">
-        <v>1.96</v>
+        <v>1.98</v>
       </c>
       <c r="BA26" t="n">
         <v>0.66</v>
@@ -6486,19 +6486,19 @@
         <v>1.19</v>
       </c>
       <c r="BC26" t="n">
-        <v>-15.31</v>
+        <v>-16.29</v>
       </c>
       <c r="BD26" t="n">
-        <v>-30.85</v>
+        <v>-31.65</v>
       </c>
       <c r="BE26" t="n">
         <v>-80.83</v>
       </c>
       <c r="BF26" t="n">
-        <v>-93.55</v>
+        <v>-93.62</v>
       </c>
       <c r="BG26" t="n">
-        <v>-88.31999999999999</v>
+        <v>-88.45999999999999</v>
       </c>
       <c r="BH26" t="n">
         <v>4.69</v>
@@ -6507,7 +6507,7 @@
         <v>0</v>
       </c>
       <c r="BJ26" t="n">
-        <v>10.22</v>
+        <v>10.34</v>
       </c>
       <c r="BK26" t="n">
         <v>0.71</v>
@@ -6516,22 +6516,22 @@
         <v>0.72</v>
       </c>
       <c r="BM26" t="n">
-        <v>10.39</v>
+        <v>10.4</v>
       </c>
       <c r="BN26" t="n">
-        <v>10.39</v>
+        <v>10.4</v>
       </c>
       <c r="BO26" t="n">
         <v>6.91</v>
       </c>
       <c r="BP26" t="n">
+        <v>10.04</v>
+      </c>
+      <c r="BQ26" t="n">
+        <v>14.42</v>
+      </c>
+      <c r="BR26" t="n">
         <v>10.15</v>
-      </c>
-      <c r="BQ26" t="n">
-        <v>14.25</v>
-      </c>
-      <c r="BR26" t="n">
-        <v>10.31</v>
       </c>
       <c r="BS26" t="n">
         <v>0.16</v>
@@ -8165,13 +8165,13 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>14.98</v>
+        <v>14.87</v>
       </c>
       <c r="G34" t="n">
-        <v>3093215611</v>
+        <v>3070501815</v>
       </c>
       <c r="H34" t="n">
-        <v>2960200</v>
+        <v>2444800</v>
       </c>
       <c r="I34" t="n">
         <v>206489813</v>
@@ -8186,7 +8186,7 @@
         <v>0.45</v>
       </c>
       <c r="M34" t="n">
-        <v>0.2719297791425067</v>
+        <v>0.2699329711903539</v>
       </c>
       <c r="N34" t="n">
         <v>0.24</v>
@@ -8264,7 +8264,7 @@
         <v>324189006.41</v>
       </c>
       <c r="AM34" t="n">
-        <v>643080168.6070687</v>
+        <v>638357965.6964657</v>
       </c>
       <c r="AN34" t="n">
         <v>0</v>
@@ -8305,7 +8305,7 @@
         <v>30.28</v>
       </c>
       <c r="AZ34" t="n">
-        <v>34.95</v>
+        <v>34.7</v>
       </c>
       <c r="BA34" t="n">
         <v>2.29</v>
@@ -8314,19 +8314,19 @@
         <v>25.26</v>
       </c>
       <c r="BC34" t="n">
-        <v>147.59</v>
+        <v>149.42</v>
       </c>
       <c r="BD34" t="n">
-        <v>102.15</v>
+        <v>103.65</v>
       </c>
       <c r="BE34" t="n">
         <v>133.33</v>
       </c>
       <c r="BF34" t="n">
-        <v>-84.68000000000001</v>
+        <v>-84.56999999999999</v>
       </c>
       <c r="BG34" t="n">
-        <v>68.61</v>
+        <v>69.86</v>
       </c>
       <c r="BH34" t="n">
         <v>38.94</v>
@@ -8335,7 +8335,7 @@
         <v>0</v>
       </c>
       <c r="BJ34" t="n">
-        <v>14.98</v>
+        <v>14.87</v>
       </c>
       <c r="BK34" t="n">
         <v>1.57</v>
@@ -8344,7 +8344,7 @@
         <v>1.58</v>
       </c>
       <c r="BM34" t="n">
-        <v>15.07</v>
+        <v>15.09</v>
       </c>
       <c r="BN34" t="n">
         <v>29.39</v>
@@ -8353,13 +8353,13 @@
         <v>14.3</v>
       </c>
       <c r="BP34" t="n">
-        <v>14.31</v>
+        <v>14.61</v>
       </c>
       <c r="BQ34" t="n">
-        <v>9.5</v>
+        <v>9.43</v>
       </c>
       <c r="BR34" t="n">
-        <v>14.45</v>
+        <v>14.92</v>
       </c>
       <c r="BS34" t="n">
         <v>0.32</v>
@@ -8395,13 +8395,13 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>18.23</v>
+        <v>18.43</v>
       </c>
       <c r="G35" t="n">
-        <v>91997692689</v>
+        <v>93006996540</v>
       </c>
       <c r="H35" t="n">
-        <v>49189900</v>
+        <v>83679100</v>
       </c>
       <c r="I35" t="n">
         <v>5046500000</v>
@@ -8416,7 +8416,7 @@
         <v>4.69</v>
       </c>
       <c r="M35" t="n">
-        <v>7.637681883611637</v>
+        <v>7.721474656153245</v>
       </c>
       <c r="N35" t="n">
         <v>1.79</v>
@@ -8494,7 +8494,7 @@
         <v>5349290000</v>
       </c>
       <c r="AM35" t="n">
-        <v>7603115098.264463</v>
+        <v>7686528639.669422</v>
       </c>
       <c r="AN35" t="n">
         <v>0.5305</v>
@@ -8535,7 +8535,7 @@
         <v>7.68</v>
       </c>
       <c r="AZ35" t="n">
-        <v>10.63</v>
+        <v>10.75</v>
       </c>
       <c r="BA35" t="n">
         <v>1.11</v>
@@ -8544,28 +8544,28 @@
         <v>9.119999999999999</v>
       </c>
       <c r="BC35" t="n">
-        <v>-48.4</v>
+        <v>-48.96</v>
       </c>
       <c r="BD35" t="n">
-        <v>-57.87</v>
+        <v>-58.33</v>
       </c>
       <c r="BE35" t="n">
         <v>-41.67</v>
       </c>
       <c r="BF35" t="n">
-        <v>-93.89</v>
+        <v>-93.95</v>
       </c>
       <c r="BG35" t="n">
-        <v>-49.99</v>
+        <v>-50.53</v>
       </c>
       <c r="BH35" t="n">
         <v>3.71</v>
       </c>
       <c r="BI35" t="n">
-        <v>0</v>
+        <v>1.03</v>
       </c>
       <c r="BJ35" t="n">
-        <v>18.23</v>
+        <v>18.24</v>
       </c>
       <c r="BK35" t="n">
         <v>1.06</v>
@@ -8574,7 +8574,7 @@
         <v>1.04</v>
       </c>
       <c r="BM35" t="n">
-        <v>18.38</v>
+        <v>18.53</v>
       </c>
       <c r="BN35" t="n">
         <v>20.08</v>
@@ -8583,13 +8583,13 @@
         <v>11.7</v>
       </c>
       <c r="BP35" t="n">
-        <v>17.75</v>
+        <v>18.03</v>
       </c>
       <c r="BQ35" t="n">
-        <v>17.45</v>
+        <v>17.64</v>
       </c>
       <c r="BR35" t="n">
-        <v>17.78</v>
+        <v>18.12</v>
       </c>
       <c r="BS35" t="n">
         <v>7.3</v>
@@ -9315,13 +9315,13 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>69.89</v>
+        <v>69.51000000000001</v>
       </c>
       <c r="G39" t="n">
-        <v>3917915251</v>
+        <v>3896613942</v>
       </c>
       <c r="H39" t="n">
-        <v>1500</v>
+        <v>1900</v>
       </c>
       <c r="I39" t="n">
         <v>168174945</v>
@@ -9336,7 +9336,7 @@
         <v>0.53</v>
       </c>
       <c r="M39" t="n">
-        <v>0.1966621601944954</v>
+        <v>0.1955929279180083</v>
       </c>
       <c r="N39" t="n">
         <v>0.06</v>
@@ -9414,7 +9414,7 @@
         <v>2536078170.6</v>
       </c>
       <c r="AM39" t="n">
-        <v>411545719.6428571</v>
+        <v>409308187.1848739</v>
       </c>
       <c r="AN39" t="n">
         <v>11.9435</v>
@@ -9455,7 +9455,7 @@
         <v>170.24</v>
       </c>
       <c r="AZ39" t="n">
-        <v>204.2</v>
+        <v>203.09</v>
       </c>
       <c r="BA39" t="n">
         <v>19.01</v>
@@ -9464,19 +9464,19 @@
         <v>91.72</v>
       </c>
       <c r="BC39" t="n">
-        <v>198.33</v>
+        <v>199.96</v>
       </c>
       <c r="BD39" t="n">
-        <v>143.59</v>
+        <v>144.92</v>
       </c>
       <c r="BE39" t="n">
         <v>192.17</v>
       </c>
       <c r="BF39" t="n">
-        <v>-72.8</v>
+        <v>-72.65000000000001</v>
       </c>
       <c r="BG39" t="n">
-        <v>31.24</v>
+        <v>31.96</v>
       </c>
       <c r="BH39" t="n">
         <v>128.13</v>
@@ -9485,7 +9485,7 @@
         <v>0</v>
       </c>
       <c r="BJ39" t="n">
-        <v>69.89</v>
+        <v>69.51000000000001</v>
       </c>
       <c r="BK39" t="n">
         <v>15.08</v>
@@ -9503,13 +9503,13 @@
         <v>54.98</v>
       </c>
       <c r="BP39" t="n">
-        <v>69.58</v>
+        <v>69.05</v>
       </c>
       <c r="BQ39" t="n">
-        <v>4.63</v>
+        <v>4.61</v>
       </c>
       <c r="BR39" t="n">
-        <v>69.58</v>
+        <v>69.89</v>
       </c>
       <c r="BS39" t="n">
         <v>0.58</v>
@@ -9545,13 +9545,13 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>22.99</v>
+        <v>22.67</v>
       </c>
       <c r="G40" t="n">
-        <v>131751803378</v>
+        <v>129918029887</v>
       </c>
       <c r="H40" t="n">
-        <v>57775600</v>
+        <v>51731400</v>
       </c>
       <c r="I40" t="n">
         <v>5730834040</v>
@@ -9566,7 +9566,7 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="M40" t="n">
-        <v>0.3997512765028474</v>
+        <v>0.39418738079099</v>
       </c>
       <c r="N40" t="n">
         <v>0.05</v>
@@ -9644,7 +9644,7 @@
         <v>15358635227.2</v>
       </c>
       <c r="AM40" t="n">
-        <v>6833599760.26971</v>
+        <v>6738487027.334024</v>
       </c>
       <c r="AN40" t="n">
         <v>0.5641</v>
@@ -9685,7 +9685,7 @@
         <v>36.13</v>
       </c>
       <c r="AZ40" t="n">
-        <v>11.61</v>
+        <v>11.45</v>
       </c>
       <c r="BA40" t="n">
         <v>2.76</v>
@@ -9694,19 +9694,19 @@
         <v>27.89</v>
       </c>
       <c r="BC40" t="n">
-        <v>92.47</v>
+        <v>95.19</v>
       </c>
       <c r="BD40" t="n">
-        <v>57.15</v>
+        <v>59.37</v>
       </c>
       <c r="BE40" t="n">
         <v>-49.5</v>
       </c>
       <c r="BF40" t="n">
-        <v>-88</v>
+        <v>-87.83</v>
       </c>
       <c r="BG40" t="n">
-        <v>21.31</v>
+        <v>23.03</v>
       </c>
       <c r="BH40" t="n">
         <v>32.47</v>
@@ -9715,7 +9715,7 @@
         <v>0</v>
       </c>
       <c r="BJ40" t="n">
-        <v>22.99</v>
+        <v>22.67</v>
       </c>
       <c r="BK40" t="n">
         <v>2.68</v>
@@ -9724,7 +9724,7 @@
         <v>2.5</v>
       </c>
       <c r="BM40" t="n">
-        <v>23.38</v>
+        <v>22.89</v>
       </c>
       <c r="BN40" t="n">
         <v>27.36</v>
@@ -9733,13 +9733,13 @@
         <v>17.67</v>
       </c>
       <c r="BP40" t="n">
-        <v>22.83</v>
+        <v>22.3</v>
       </c>
       <c r="BQ40" t="n">
-        <v>9.199999999999999</v>
+        <v>9.07</v>
       </c>
       <c r="BR40" t="n">
-        <v>23.2</v>
+        <v>22.84</v>
       </c>
       <c r="BS40" t="n">
         <v>0.39</v>
@@ -9775,13 +9775,13 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>16.02</v>
+        <v>16.3</v>
       </c>
       <c r="G41" t="n">
-        <v>190883571996</v>
+        <v>194181247715</v>
       </c>
       <c r="H41" t="n">
-        <v>6190700</v>
+        <v>8101200</v>
       </c>
       <c r="I41" t="n">
         <v>5303870781</v>
@@ -9796,7 +9796,7 @@
         <v>0.92</v>
       </c>
       <c r="M41" t="n">
-        <v>1.272042102799097</v>
+        <v>1.294017709772935</v>
       </c>
       <c r="N41" t="n">
         <v>0.07000000000000001</v>
@@ -9874,7 +9874,7 @@
         <v>12304980211.92</v>
       </c>
       <c r="AM41" t="n">
-        <v>29411952541.75655</v>
+        <v>29920068985.36209</v>
       </c>
       <c r="AN41" t="n">
         <v>1.6841</v>
@@ -9915,7 +9915,7 @@
         <v>24.4</v>
       </c>
       <c r="AZ41" t="n">
-        <v>23.98</v>
+        <v>24.4</v>
       </c>
       <c r="BA41" t="n">
         <v>2.53</v>
@@ -9924,19 +9924,19 @@
         <v>13.77</v>
       </c>
       <c r="BC41" t="n">
-        <v>86.55</v>
+        <v>83.34999999999999</v>
       </c>
       <c r="BD41" t="n">
-        <v>52.32</v>
+        <v>49.7</v>
       </c>
       <c r="BE41" t="n">
         <v>49.67</v>
       </c>
       <c r="BF41" t="n">
-        <v>-84.22</v>
+        <v>-84.5</v>
       </c>
       <c r="BG41" t="n">
-        <v>-14.04</v>
+        <v>-15.52</v>
       </c>
       <c r="BH41" t="n">
         <v>17.11</v>
@@ -9945,7 +9945,7 @@
         <v>0</v>
       </c>
       <c r="BJ41" t="n">
-        <v>16.02</v>
+        <v>16.3</v>
       </c>
       <c r="BK41" t="n">
         <v>2.32</v>
@@ -9954,7 +9954,7 @@
         <v>2.34</v>
       </c>
       <c r="BM41" t="n">
-        <v>16.08</v>
+        <v>16.3</v>
       </c>
       <c r="BN41" t="n">
         <v>18.28</v>
@@ -9963,13 +9963,13 @@
         <v>13.43</v>
       </c>
       <c r="BP41" t="n">
-        <v>15.89</v>
+        <v>15.82</v>
       </c>
       <c r="BQ41" t="n">
-        <v>6.85</v>
+        <v>6.97</v>
       </c>
       <c r="BR41" t="n">
-        <v>15.96</v>
+        <v>15.95</v>
       </c>
       <c r="BS41" t="n">
         <v>0.5600000000000001</v>
@@ -10005,13 +10005,13 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>18.16</v>
+        <v>18.43</v>
       </c>
       <c r="G42" t="n">
-        <v>190883571996</v>
+        <v>194181247715</v>
       </c>
       <c r="H42" t="n">
-        <v>54948000</v>
+        <v>44514900</v>
       </c>
       <c r="I42" t="n">
         <v>5288141247</v>
@@ -10026,7 +10026,7 @@
         <v>1.05</v>
       </c>
       <c r="M42" t="n">
-        <v>1.27582578189745</v>
+        <v>1.297866755139116</v>
       </c>
       <c r="N42" t="n">
         <v>0.08</v>
@@ -10104,7 +10104,7 @@
         <v>12268487693.04</v>
       </c>
       <c r="AM42" t="n">
-        <v>25970554013.06123</v>
+        <v>26419217376.19048</v>
       </c>
       <c r="AN42" t="n">
         <v>1.8491</v>
@@ -10145,7 +10145,7 @@
         <v>24.4</v>
       </c>
       <c r="AZ42" t="n">
-        <v>26.3</v>
+        <v>26.69</v>
       </c>
       <c r="BA42" t="n">
         <v>2.53</v>
@@ -10154,19 +10154,19 @@
         <v>15.11</v>
       </c>
       <c r="BC42" t="n">
-        <v>64.56999999999999</v>
+        <v>62.16</v>
       </c>
       <c r="BD42" t="n">
-        <v>34.37</v>
+        <v>32.4</v>
       </c>
       <c r="BE42" t="n">
         <v>44.83</v>
       </c>
       <c r="BF42" t="n">
-        <v>-86.08</v>
+        <v>-86.29000000000001</v>
       </c>
       <c r="BG42" t="n">
-        <v>-16.77</v>
+        <v>-17.99</v>
       </c>
       <c r="BH42" t="n">
         <v>17.11</v>
@@ -10175,7 +10175,7 @@
         <v>0</v>
       </c>
       <c r="BJ42" t="n">
-        <v>18.16</v>
+        <v>18.43</v>
       </c>
       <c r="BK42" t="n">
         <v>2.32</v>
@@ -10184,7 +10184,7 @@
         <v>2.34</v>
       </c>
       <c r="BM42" t="n">
-        <v>18.23</v>
+        <v>18.44</v>
       </c>
       <c r="BN42" t="n">
         <v>21.33</v>
@@ -10193,13 +10193,13 @@
         <v>15.67</v>
       </c>
       <c r="BP42" t="n">
-        <v>18.01</v>
+        <v>17.92</v>
       </c>
       <c r="BQ42" t="n">
-        <v>7.77</v>
+        <v>7.88</v>
       </c>
       <c r="BR42" t="n">
-        <v>18.15</v>
+        <v>18.05</v>
       </c>
       <c r="BS42" t="n">
         <v>0.63</v>
@@ -10235,13 +10235,13 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>39.82</v>
+        <v>39.35</v>
       </c>
       <c r="G43" t="n">
-        <v>77306507587</v>
+        <v>76394087037</v>
       </c>
       <c r="H43" t="n">
-        <v>8742900</v>
+        <v>7846600</v>
       </c>
       <c r="I43" t="n">
         <v>1941400000</v>
@@ -10334,7 +10334,7 @@
         <v>9182822000</v>
       </c>
       <c r="AM43" t="n">
-        <v>9416139779.171741</v>
+        <v>9305004511.205845</v>
       </c>
       <c r="AN43" t="n">
         <v>4.5901</v>
@@ -10375,7 +10375,7 @@
         <v>19.95</v>
       </c>
       <c r="AZ43" t="n">
-        <v>72.27</v>
+        <v>71.42</v>
       </c>
       <c r="BA43" t="n">
         <v>5.63</v>
@@ -10384,19 +10384,19 @@
         <v>48.62</v>
       </c>
       <c r="BC43" t="n">
-        <v>-38.64</v>
+        <v>-37.9</v>
       </c>
       <c r="BD43" t="n">
-        <v>-49.9</v>
+        <v>-49.3</v>
       </c>
       <c r="BE43" t="n">
         <v>81.5</v>
       </c>
       <c r="BF43" t="n">
-        <v>-85.86</v>
+        <v>-85.7</v>
       </c>
       <c r="BG43" t="n">
-        <v>22.09</v>
+        <v>23.55</v>
       </c>
       <c r="BH43" t="n">
         <v>5.61</v>
@@ -10405,7 +10405,7 @@
         <v>0</v>
       </c>
       <c r="BJ43" t="n">
-        <v>39.82</v>
+        <v>39.35</v>
       </c>
       <c r="BK43" t="n">
         <v>4.73</v>
@@ -10414,7 +10414,7 @@
         <v>4.73</v>
       </c>
       <c r="BM43" t="n">
-        <v>41.21</v>
+        <v>39.82</v>
       </c>
       <c r="BN43" t="n">
         <v>42.98</v>
@@ -10423,13 +10423,13 @@
         <v>28.06</v>
       </c>
       <c r="BP43" t="n">
-        <v>39.7</v>
+        <v>39.04</v>
       </c>
       <c r="BQ43" t="n">
-        <v>8.41</v>
+        <v>8.31</v>
       </c>
       <c r="BR43" t="n">
-        <v>40.92</v>
+        <v>39.72</v>
       </c>
       <c r="BS43" t="n">
         <v>0</v>
@@ -10925,13 +10925,13 @@
         </is>
       </c>
       <c r="F46" t="n">
-        <v>3.92</v>
+        <v>4.02</v>
       </c>
       <c r="G46" t="n">
-        <v>3922124716</v>
+        <v>4022178820</v>
       </c>
       <c r="H46" t="n">
-        <v>19463500</v>
+        <v>15997400</v>
       </c>
       <c r="I46" t="n">
         <v>1000542188</v>
@@ -10946,7 +10946,7 @@
         <v>2.5</v>
       </c>
       <c r="M46" t="n">
-        <v>0.0681739015547508</v>
+        <v>0.06991302999409356</v>
       </c>
       <c r="N46" t="n">
         <v>0.08</v>
@@ -11024,7 +11024,7 @@
         <v>460249406.48</v>
       </c>
       <c r="AM46" t="n">
-        <v>3845220309.803922</v>
+        <v>3943312568.627451</v>
       </c>
       <c r="AN46" t="n">
         <v>0.0311</v>
@@ -11065,7 +11065,7 @@
         <v>3.3</v>
       </c>
       <c r="AZ46" t="n">
-        <v>3.23</v>
+        <v>3.32</v>
       </c>
       <c r="BA46" t="n">
         <v>0.42</v>
@@ -11074,19 +11074,19 @@
         <v>7.38</v>
       </c>
       <c r="BC46" t="n">
-        <v>3.16</v>
+        <v>0.59</v>
       </c>
       <c r="BD46" t="n">
-        <v>-15.77</v>
+        <v>-17.87</v>
       </c>
       <c r="BE46" t="n">
         <v>-17.5</v>
       </c>
       <c r="BF46" t="n">
-        <v>-89.20999999999999</v>
+        <v>-89.48</v>
       </c>
       <c r="BG46" t="n">
-        <v>88.23</v>
+        <v>83.55</v>
       </c>
       <c r="BH46" t="n">
         <v>1.58</v>
@@ -11095,7 +11095,7 @@
         <v>0</v>
       </c>
       <c r="BJ46" t="n">
-        <v>3.92</v>
+        <v>4.02</v>
       </c>
       <c r="BK46" t="n">
         <v>0.46</v>
@@ -11113,13 +11113,13 @@
         <v>2.97</v>
       </c>
       <c r="BP46" t="n">
-        <v>3.86</v>
+        <v>3.87</v>
       </c>
       <c r="BQ46" t="n">
-        <v>8.57</v>
+        <v>8.789999999999999</v>
       </c>
       <c r="BR46" t="n">
-        <v>4</v>
+        <v>3.9</v>
       </c>
       <c r="BS46" t="n">
         <v>0.07000000000000001</v>
@@ -11158,10 +11158,10 @@
         <v>9</v>
       </c>
       <c r="G47" t="n">
-        <v>3139774200</v>
+        <v>3141546300</v>
       </c>
       <c r="H47" t="n">
-        <v>3900</v>
+        <v>7200</v>
       </c>
       <c r="I47" t="n">
         <v>254106600</v>
@@ -11176,7 +11176,7 @@
         <v>1.22</v>
       </c>
       <c r="M47" t="n">
-        <v>0.7403948802787467</v>
+        <v>0.740812761847218</v>
       </c>
       <c r="N47" t="n">
         <v>0.07000000000000001</v>
@@ -11254,7 +11254,7 @@
         <v>322715382</v>
       </c>
       <c r="AM47" t="n">
-        <v>556697553.1914893</v>
+        <v>557011755.319149</v>
       </c>
       <c r="AN47" t="n">
         <v>0.4132</v>
@@ -11334,7 +11334,7 @@
         <v>1.29</v>
       </c>
       <c r="BM47" t="n">
-        <v>9.029999999999999</v>
+        <v>9</v>
       </c>
       <c r="BN47" t="n">
         <v>9.24</v>
@@ -11343,13 +11343,13 @@
         <v>7.19</v>
       </c>
       <c r="BP47" t="n">
-        <v>8.94</v>
+        <v>8.93</v>
       </c>
       <c r="BQ47" t="n">
         <v>6.96</v>
       </c>
       <c r="BR47" t="n">
-        <v>8.98</v>
+        <v>9</v>
       </c>
       <c r="BS47" t="n">
         <v>0.53</v>
@@ -11385,13 +11385,13 @@
         </is>
       </c>
       <c r="F48" t="n">
-        <v>9.15</v>
+        <v>9.1</v>
       </c>
       <c r="G48" t="n">
-        <v>3139774200</v>
+        <v>3141546300</v>
       </c>
       <c r="H48" t="n">
-        <v>1900</v>
+        <v>1200</v>
       </c>
       <c r="I48" t="n">
         <v>93397546</v>
@@ -11406,7 +11406,7 @@
         <v>1.24</v>
       </c>
       <c r="M48" t="n">
-        <v>2.014391531069129</v>
+        <v>2.015528460989824</v>
       </c>
       <c r="N48" t="n">
         <v>0.07000000000000001</v>
@@ -11484,7 +11484,7 @@
         <v>118614883.42</v>
       </c>
       <c r="AM48" t="n">
-        <v>548911573.4265734</v>
+        <v>549221381.1188811</v>
       </c>
       <c r="AN48" t="n">
         <v>0.4132</v>
@@ -11525,7 +11525,7 @@
         <v>11.74</v>
       </c>
       <c r="AZ48" t="n">
-        <v>11.97</v>
+        <v>11.91</v>
       </c>
       <c r="BA48" t="n">
         <v>1.46</v>
@@ -11534,19 +11534,19 @@
         <v>8.24</v>
       </c>
       <c r="BC48" t="n">
-        <v>57.09</v>
+        <v>57.95</v>
       </c>
       <c r="BD48" t="n">
-        <v>28.26</v>
+        <v>28.97</v>
       </c>
       <c r="BE48" t="n">
         <v>30.83</v>
       </c>
       <c r="BF48" t="n">
-        <v>-84.06</v>
+        <v>-83.97</v>
       </c>
       <c r="BG48" t="n">
-        <v>-9.99</v>
+        <v>-9.49</v>
       </c>
       <c r="BH48" t="n">
         <v>7.23</v>
@@ -11555,7 +11555,7 @@
         <v>0</v>
       </c>
       <c r="BJ48" t="n">
-        <v>9.15</v>
+        <v>9.1</v>
       </c>
       <c r="BK48" t="n">
         <v>1.27</v>
@@ -11564,7 +11564,7 @@
         <v>1.29</v>
       </c>
       <c r="BM48" t="n">
-        <v>9.289999999999999</v>
+        <v>9.15</v>
       </c>
       <c r="BN48" t="n">
         <v>9.48</v>
@@ -11573,13 +11573,13 @@
         <v>7.2</v>
       </c>
       <c r="BP48" t="n">
-        <v>9.08</v>
+        <v>9.07</v>
       </c>
       <c r="BQ48" t="n">
-        <v>7.08</v>
+        <v>7.04</v>
       </c>
       <c r="BR48" t="n">
-        <v>9.140000000000001</v>
+        <v>9.15</v>
       </c>
       <c r="BS48" t="n">
         <v>0.54</v>
@@ -11845,13 +11845,13 @@
         </is>
       </c>
       <c r="F50" t="n">
-        <v>33.44</v>
+        <v>32.61</v>
       </c>
       <c r="G50" t="n">
         <v>961816100</v>
       </c>
       <c r="H50" t="n">
-        <v>200</v>
+        <v>600</v>
       </c>
       <c r="I50" t="n">
         <v>11540870</v>
@@ -11985,7 +11985,7 @@
         <v>68.48999999999999</v>
       </c>
       <c r="AZ50" t="n">
-        <v>73.73999999999999</v>
+        <v>71.91</v>
       </c>
       <c r="BA50" t="n">
         <v>9.210000000000001</v>
@@ -11994,19 +11994,19 @@
         <v>30.53</v>
       </c>
       <c r="BC50" t="n">
-        <v>150.83</v>
+        <v>157.21</v>
       </c>
       <c r="BD50" t="n">
-        <v>104.8</v>
+        <v>110.01</v>
       </c>
       <c r="BE50" t="n">
         <v>120.5</v>
       </c>
       <c r="BF50" t="n">
-        <v>-72.45</v>
+        <v>-71.75</v>
       </c>
       <c r="BG50" t="n">
-        <v>-8.699999999999999</v>
+        <v>-6.38</v>
       </c>
       <c r="BH50" t="n">
         <v>42.6</v>
@@ -12015,7 +12015,7 @@
         <v>0</v>
       </c>
       <c r="BJ50" t="n">
-        <v>33.44</v>
+        <v>32.61</v>
       </c>
       <c r="BK50" t="n">
         <v>7.34</v>
@@ -12024,7 +12024,7 @@
         <v>7.6</v>
       </c>
       <c r="BM50" t="n">
-        <v>33.44</v>
+        <v>33.93</v>
       </c>
       <c r="BN50" t="n">
         <v>39.22</v>
@@ -12033,13 +12033,13 @@
         <v>23.5</v>
       </c>
       <c r="BP50" t="n">
-        <v>33.44</v>
+        <v>32.61</v>
       </c>
       <c r="BQ50" t="n">
-        <v>4.4</v>
+        <v>4.29</v>
       </c>
       <c r="BR50" t="n">
-        <v>33.44</v>
+        <v>33.93</v>
       </c>
       <c r="BS50" t="n">
         <v>0.4</v>
@@ -12523,13 +12523,13 @@
         </is>
       </c>
       <c r="F53" t="n">
-        <v>6.47</v>
+        <v>6.41</v>
       </c>
       <c r="G53" t="n">
-        <v>885434999</v>
+        <v>877223863</v>
       </c>
       <c r="H53" t="n">
-        <v>11800</v>
+        <v>2900</v>
       </c>
       <c r="I53" t="n">
         <v>136852484</v>
@@ -12544,7 +12544,7 @@
         <v>2.79</v>
       </c>
       <c r="M53" t="n">
-        <v>2.30019506452782</v>
+        <v>2.27886406392055</v>
       </c>
       <c r="N53" t="n">
         <v>1.48</v>
@@ -12622,7 +12622,7 @@
         <v>39687220.36</v>
       </c>
       <c r="AM53" t="n">
-        <v>45106214.92613347</v>
+        <v>44687919.66377993</v>
       </c>
       <c r="AN53" t="n">
         <v>0</v>
@@ -12672,16 +12672,16 @@
         <v>0</v>
       </c>
       <c r="BC53" t="n">
-        <v>-39.09</v>
+        <v>-38.52</v>
       </c>
       <c r="BD53" t="n">
-        <v>-50.27</v>
+        <v>-49.8</v>
       </c>
       <c r="BE53" t="n">
         <v>-100</v>
       </c>
       <c r="BF53" t="n">
-        <v>-95.52</v>
+        <v>-95.48</v>
       </c>
       <c r="BG53" t="n">
         <v>-100</v>
@@ -12693,7 +12693,7 @@
         <v>0</v>
       </c>
       <c r="BJ53" t="n">
-        <v>6.47</v>
+        <v>6.41</v>
       </c>
       <c r="BK53" t="n">
         <v>0.29</v>
@@ -12711,13 +12711,13 @@
         <v>4.82</v>
       </c>
       <c r="BP53" t="n">
-        <v>6.29</v>
+        <v>6.38</v>
       </c>
       <c r="BQ53" t="n">
-        <v>75.83</v>
+        <v>75.13</v>
       </c>
       <c r="BR53" t="n">
-        <v>6.29</v>
+        <v>6.46</v>
       </c>
       <c r="BS53" t="n">
         <v>2.36</v>
@@ -12753,13 +12753,13 @@
         </is>
       </c>
       <c r="F54" t="n">
-        <v>10.56</v>
+        <v>10.52</v>
       </c>
       <c r="G54" t="n">
-        <v>2462719873</v>
+        <v>2453391398</v>
       </c>
       <c r="H54" t="n">
-        <v>281200</v>
+        <v>219900</v>
       </c>
       <c r="I54" t="n">
         <v>233212121</v>
@@ -12774,7 +12774,7 @@
         <v>0.97</v>
       </c>
       <c r="M54" t="n">
-        <v>1.382303929973262</v>
+        <v>1.377067935496371</v>
       </c>
       <c r="N54" t="n">
         <v>0.5600000000000001</v>
@@ -12852,7 +12852,7 @@
         <v>233212121</v>
       </c>
       <c r="AM54" t="n">
-        <v>336897383.4473324</v>
+        <v>335621258.2763338</v>
       </c>
       <c r="AN54" t="n">
         <v>0.1531</v>
@@ -12893,7 +12893,7 @@
         <v>12.25</v>
       </c>
       <c r="AZ54" t="n">
-        <v>16.81</v>
+        <v>16.74</v>
       </c>
       <c r="BA54" t="n">
         <v>0.98</v>
@@ -12902,19 +12902,19 @@
         <v>6.52</v>
       </c>
       <c r="BC54" t="n">
-        <v>42.12</v>
+        <v>42.66</v>
       </c>
       <c r="BD54" t="n">
-        <v>16.04</v>
+        <v>16.48</v>
       </c>
       <c r="BE54" t="n">
         <v>59.17</v>
       </c>
       <c r="BF54" t="n">
-        <v>-90.69</v>
+        <v>-90.65000000000001</v>
       </c>
       <c r="BG54" t="n">
-        <v>-38.29</v>
+        <v>-38.06</v>
       </c>
       <c r="BH54" t="n">
         <v>10.01</v>
@@ -12923,7 +12923,7 @@
         <v>0</v>
       </c>
       <c r="BJ54" t="n">
-        <v>10.56</v>
+        <v>10.52</v>
       </c>
       <c r="BK54" t="n">
         <v>1</v>
@@ -12932,7 +12932,7 @@
         <v>1</v>
       </c>
       <c r="BM54" t="n">
-        <v>10.78</v>
+        <v>10.62</v>
       </c>
       <c r="BN54" t="n">
         <v>11.75</v>
@@ -12941,13 +12941,13 @@
         <v>8.279999999999999</v>
       </c>
       <c r="BP54" t="n">
-        <v>10.53</v>
+        <v>10.37</v>
       </c>
       <c r="BQ54" t="n">
-        <v>10.53</v>
+        <v>10.49</v>
       </c>
       <c r="BR54" t="n">
-        <v>10.55</v>
+        <v>10.49</v>
       </c>
       <c r="BS54" t="n">
         <v>1.26</v>
@@ -12983,13 +12983,13 @@
         </is>
       </c>
       <c r="F55" t="n">
-        <v>50.1</v>
+        <v>50.44</v>
       </c>
       <c r="G55" t="n">
-        <v>6684404349</v>
+        <v>6482124212</v>
       </c>
       <c r="H55" t="n">
-        <v>5000</v>
+        <v>2200</v>
       </c>
       <c r="I55" t="n">
         <v>84052790</v>
@@ -13004,7 +13004,7 @@
         <v>2</v>
       </c>
       <c r="M55" t="n">
-        <v>1.031879242662991</v>
+        <v>1.00065302359015</v>
       </c>
       <c r="N55" t="n">
         <v>0.16</v>
@@ -13082,7 +13082,7 @@
         <v>579123723.1</v>
       </c>
       <c r="AM55" t="n">
-        <v>336237643.3098592</v>
+        <v>326062586.1167002</v>
       </c>
       <c r="AN55" t="n">
         <v>3.1953</v>
@@ -13123,7 +13123,7 @@
         <v>51.21</v>
       </c>
       <c r="AZ55" t="n">
-        <v>52.69</v>
+        <v>53.05</v>
       </c>
       <c r="BA55" t="n">
         <v>9.380000000000001</v>
@@ -13132,19 +13132,19 @@
         <v>16.08</v>
       </c>
       <c r="BC55" t="n">
-        <v>25.18</v>
+        <v>24.33</v>
       </c>
       <c r="BD55" t="n">
-        <v>2.21</v>
+        <v>1.52</v>
       </c>
       <c r="BE55" t="n">
         <v>5.17</v>
       </c>
       <c r="BF55" t="n">
-        <v>-81.28</v>
+        <v>-81.41</v>
       </c>
       <c r="BG55" t="n">
-        <v>-67.91</v>
+        <v>-68.13</v>
       </c>
       <c r="BH55" t="n">
         <v>25.37</v>
@@ -13153,7 +13153,7 @@
         <v>0</v>
       </c>
       <c r="BJ55" t="n">
-        <v>50.1</v>
+        <v>50.44</v>
       </c>
       <c r="BK55" t="n">
         <v>6.89</v>
@@ -13162,7 +13162,7 @@
         <v>7.03</v>
       </c>
       <c r="BM55" t="n">
-        <v>50.5</v>
+        <v>50.58</v>
       </c>
       <c r="BN55" t="n">
         <v>73.67</v>
@@ -13171,13 +13171,13 @@
         <v>35.58</v>
       </c>
       <c r="BP55" t="n">
-        <v>49.8</v>
+        <v>49.41</v>
       </c>
       <c r="BQ55" t="n">
-        <v>7.13</v>
+        <v>7.17</v>
       </c>
       <c r="BR55" t="n">
-        <v>50</v>
+        <v>50.07</v>
       </c>
       <c r="BS55" t="n">
         <v>0.66</v>
@@ -13213,13 +13213,13 @@
         </is>
       </c>
       <c r="F56" t="n">
-        <v>61.78</v>
+        <v>60.11</v>
       </c>
       <c r="G56" t="n">
-        <v>6684404349</v>
+        <v>6482124212</v>
       </c>
       <c r="H56" t="n">
-        <v>28100</v>
+        <v>21900</v>
       </c>
       <c r="I56" t="n">
         <v>39675836</v>
@@ -13234,7 +13234,7 @@
         <v>2.41</v>
       </c>
       <c r="M56" t="n">
-        <v>2.186023989233937</v>
+        <v>2.119871612905345</v>
       </c>
       <c r="N56" t="n">
         <v>0.19</v>
@@ -13312,7 +13312,7 @@
         <v>273366510.04</v>
       </c>
       <c r="AM56" t="n">
-        <v>278053425.499168</v>
+        <v>269639110.3161398</v>
       </c>
       <c r="AN56" t="n">
         <v>3.5102</v>
@@ -13353,7 +13353,7 @@
         <v>51.21</v>
       </c>
       <c r="AZ56" t="n">
-        <v>59</v>
+        <v>57.41</v>
       </c>
       <c r="BA56" t="n">
         <v>9.380000000000001</v>
@@ -13362,19 +13362,19 @@
         <v>17.68</v>
       </c>
       <c r="BC56" t="n">
-        <v>1.51</v>
+        <v>4.33</v>
       </c>
       <c r="BD56" t="n">
-        <v>-17.12</v>
+        <v>-14.81</v>
       </c>
       <c r="BE56" t="n">
         <v>-4.5</v>
       </c>
       <c r="BF56" t="n">
-        <v>-84.81999999999999</v>
+        <v>-84.40000000000001</v>
       </c>
       <c r="BG56" t="n">
-        <v>-71.39</v>
+        <v>-70.59</v>
       </c>
       <c r="BH56" t="n">
         <v>25.37</v>
@@ -13383,7 +13383,7 @@
         <v>0</v>
       </c>
       <c r="BJ56" t="n">
-        <v>61.78</v>
+        <v>60.11</v>
       </c>
       <c r="BK56" t="n">
         <v>6.89</v>
@@ -13392,7 +13392,7 @@
         <v>7.03</v>
       </c>
       <c r="BM56" t="n">
-        <v>63.45</v>
+        <v>61.25</v>
       </c>
       <c r="BN56" t="n">
         <v>86.77</v>
@@ -13401,13 +13401,13 @@
         <v>46.42</v>
       </c>
       <c r="BP56" t="n">
-        <v>60.94</v>
+        <v>60.11</v>
       </c>
       <c r="BQ56" t="n">
-        <v>8.789999999999999</v>
+        <v>8.550000000000001</v>
       </c>
       <c r="BR56" t="n">
-        <v>61.41</v>
+        <v>61.25</v>
       </c>
       <c r="BS56" t="n">
         <v>0.79</v>
@@ -13443,13 +13443,13 @@
         </is>
       </c>
       <c r="F57" t="n">
-        <v>6.17</v>
+        <v>6.12</v>
       </c>
       <c r="G57" t="n">
-        <v>1442903260</v>
+        <v>1431210933</v>
       </c>
       <c r="H57" t="n">
-        <v>1628700</v>
+        <v>1412400</v>
       </c>
       <c r="I57" t="n">
         <v>233858065</v>
@@ -13464,7 +13464,7 @@
         <v>0.77</v>
       </c>
       <c r="M57" t="n">
-        <v>0.4318997003588481</v>
+        <v>0.4283998728459504</v>
       </c>
       <c r="N57" t="n">
         <v>0.08</v>
@@ -13542,7 +13542,7 @@
         <v>229180903.7</v>
       </c>
       <c r="AM57" t="n">
-        <v>107920961.854899</v>
+        <v>107046442.2587883</v>
       </c>
       <c r="AN57" t="n">
         <v>0.347</v>
@@ -13583,7 +13583,7 @@
         <v>10.72</v>
       </c>
       <c r="AZ57" t="n">
-        <v>9.41</v>
+        <v>9.33</v>
       </c>
       <c r="BA57" t="n">
         <v>1.13</v>
@@ -13592,19 +13592,19 @@
         <v>6.26</v>
       </c>
       <c r="BC57" t="n">
-        <v>112.82</v>
+        <v>114.56</v>
       </c>
       <c r="BD57" t="n">
-        <v>73.77</v>
+        <v>75.19</v>
       </c>
       <c r="BE57" t="n">
         <v>52.5</v>
       </c>
       <c r="BF57" t="n">
-        <v>-81.73</v>
+        <v>-81.58</v>
       </c>
       <c r="BG57" t="n">
-        <v>1.52</v>
+        <v>2.35</v>
       </c>
       <c r="BH57" t="n">
         <v>7.82</v>
@@ -13613,7 +13613,7 @@
         <v>0</v>
       </c>
       <c r="BJ57" t="n">
-        <v>6.17</v>
+        <v>6.12</v>
       </c>
       <c r="BK57" t="n">
         <v>0.98</v>
@@ -13622,10 +13622,10 @@
         <v>1.04</v>
       </c>
       <c r="BM57" t="n">
-        <v>6.21</v>
+        <v>6.16</v>
       </c>
       <c r="BN57" t="n">
-        <v>6.21</v>
+        <v>6.18</v>
       </c>
       <c r="BO57" t="n">
         <v>3.43</v>
@@ -13634,10 +13634,10 @@
         <v>6.04</v>
       </c>
       <c r="BQ57" t="n">
-        <v>5.96</v>
+        <v>5.91</v>
       </c>
       <c r="BR57" t="n">
-        <v>6.07</v>
+        <v>6.14</v>
       </c>
       <c r="BS57" t="n">
         <v>0.42</v>
@@ -14133,13 +14133,13 @@
         </is>
       </c>
       <c r="F60" t="n">
-        <v>373.89</v>
+        <v>373.9</v>
       </c>
       <c r="G60" t="n">
-        <v>170026484</v>
+        <v>170031022</v>
       </c>
       <c r="H60" t="n">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="I60" t="n">
         <v>454750</v>
@@ -14154,7 +14154,7 @@
         <v>0.83</v>
       </c>
       <c r="M60" t="n">
-        <v>12.71774165592438</v>
+        <v>12.71808109193621</v>
       </c>
       <c r="N60" t="n">
         <v>0.68</v>
@@ -14232,7 +14232,7 @@
         <v>59558607.5</v>
       </c>
       <c r="AM60" t="n">
-        <v>-24930569.50146627</v>
+        <v>-24931234.8973607</v>
       </c>
       <c r="AN60" t="n">
         <v>10.0581</v>
@@ -14273,7 +14273,7 @@
         <v>944.87</v>
       </c>
       <c r="AZ60" t="n">
-        <v>2149.87</v>
+        <v>2149.92</v>
       </c>
       <c r="BA60" t="n">
         <v>231.1</v>
@@ -14282,7 +14282,7 @@
         <v>727.97</v>
       </c>
       <c r="BC60" t="n">
-        <v>209.51</v>
+        <v>209.5</v>
       </c>
       <c r="BD60" t="n">
         <v>152.71</v>
@@ -14303,7 +14303,7 @@
         <v>0</v>
       </c>
       <c r="BJ60" t="n">
-        <v>373.89</v>
+        <v>373.9</v>
       </c>
       <c r="BK60" t="n">
         <v>130.97</v>
@@ -14312,7 +14312,7 @@
         <v>130.97</v>
       </c>
       <c r="BM60" t="n">
-        <v>387</v>
+        <v>375.5</v>
       </c>
       <c r="BN60" t="n">
         <v>405</v>
@@ -14321,13 +14321,13 @@
         <v>306.27</v>
       </c>
       <c r="BP60" t="n">
-        <v>370.01</v>
+        <v>369.83</v>
       </c>
       <c r="BQ60" t="n">
         <v>2.85</v>
       </c>
       <c r="BR60" t="n">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="BS60" t="n">
         <v>12.82</v>
@@ -14363,13 +14363,13 @@
         </is>
       </c>
       <c r="F61" t="n">
-        <v>27.66</v>
+        <v>28.55</v>
       </c>
       <c r="G61" t="n">
-        <v>2367928054</v>
+        <v>2444119183</v>
       </c>
       <c r="H61" t="n">
-        <v>516500</v>
+        <v>1229100</v>
       </c>
       <c r="I61" t="n">
         <v>85608392</v>
@@ -14384,7 +14384,7 @@
         <v>2.37</v>
       </c>
       <c r="M61" t="n">
-        <v>1.255793546443125</v>
+        <v>1.296200318064749</v>
       </c>
       <c r="N61" t="n">
         <v>1.1</v>
@@ -14462,7 +14462,7 @@
         <v>160087693.04</v>
       </c>
       <c r="AM61" t="n">
-        <v>185865624.33281</v>
+        <v>191846089.7174254</v>
       </c>
       <c r="AN61" t="n">
         <v>0.38</v>
@@ -14503,7 +14503,7 @@
         <v>17.56</v>
       </c>
       <c r="AZ61" t="n">
-        <v>34.85</v>
+        <v>35.97</v>
       </c>
       <c r="BA61" t="n">
         <v>2.52</v>
@@ -14512,19 +14512,19 @@
         <v>11.76</v>
       </c>
       <c r="BC61" t="n">
-        <v>-22.26</v>
+        <v>-24.68</v>
       </c>
       <c r="BD61" t="n">
-        <v>-36.52</v>
+        <v>-38.5</v>
       </c>
       <c r="BE61" t="n">
         <v>26</v>
       </c>
       <c r="BF61" t="n">
-        <v>-90.88</v>
+        <v>-91.16</v>
       </c>
       <c r="BG61" t="n">
-        <v>-57.5</v>
+        <v>-58.82</v>
       </c>
       <c r="BH61" t="n">
         <v>10.99</v>
@@ -14533,7 +14533,7 @@
         <v>0</v>
       </c>
       <c r="BJ61" t="n">
-        <v>27.66</v>
+        <v>28.55</v>
       </c>
       <c r="BK61" t="n">
         <v>1.87</v>
@@ -14542,22 +14542,22 @@
         <v>1.86</v>
       </c>
       <c r="BM61" t="n">
-        <v>27.93</v>
+        <v>28.68</v>
       </c>
       <c r="BN61" t="n">
-        <v>28.25</v>
+        <v>28.68</v>
       </c>
       <c r="BO61" t="n">
         <v>19.35</v>
       </c>
       <c r="BP61" t="n">
-        <v>27.58</v>
+        <v>27.53</v>
       </c>
       <c r="BQ61" t="n">
-        <v>14.86</v>
+        <v>15.33</v>
       </c>
       <c r="BR61" t="n">
-        <v>27.7</v>
+        <v>27.54</v>
       </c>
       <c r="BS61" t="n">
         <v>1.19</v>
@@ -14823,13 +14823,13 @@
         </is>
       </c>
       <c r="F63" t="n">
-        <v>1.43</v>
+        <v>1.34</v>
       </c>
       <c r="G63" t="n">
-        <v>372528857</v>
+        <v>349083006</v>
       </c>
       <c r="H63" t="n">
-        <v>64700</v>
+        <v>22300</v>
       </c>
       <c r="I63" t="n">
         <v>122894462</v>
@@ -14844,7 +14844,7 @@
         <v>-0.22</v>
       </c>
       <c r="M63" t="n">
-        <v>0.4581912693417068</v>
+        <v>0.429354082561069</v>
       </c>
       <c r="N63" t="n">
         <v>0.37</v>
@@ -14922,7 +14922,7 @@
         <v>31952560.12</v>
       </c>
       <c r="AM63" t="n">
-        <v>211664123.2954545</v>
+        <v>198342617.0454545</v>
       </c>
       <c r="AN63" t="n">
         <v>0</v>
@@ -14981,7 +14981,7 @@
         <v>-100</v>
       </c>
       <c r="BF63" t="n">
-        <v>-79.78</v>
+        <v>-78.42</v>
       </c>
       <c r="BG63" t="n">
         <v>-100</v>
@@ -14993,7 +14993,7 @@
         <v>0</v>
       </c>
       <c r="BJ63" t="n">
-        <v>1.43</v>
+        <v>1.34</v>
       </c>
       <c r="BK63" t="n">
         <v>0.26</v>
@@ -15002,7 +15002,7 @@
         <v>0.26</v>
       </c>
       <c r="BM63" t="n">
-        <v>1.5</v>
+        <v>1.46</v>
       </c>
       <c r="BN63" t="n">
         <v>2.12</v>
@@ -15011,13 +15011,13 @@
         <v>1.16</v>
       </c>
       <c r="BP63" t="n">
+        <v>1.34</v>
+      </c>
+      <c r="BQ63" t="n">
+        <v>5.13</v>
+      </c>
+      <c r="BR63" t="n">
         <v>1.4</v>
-      </c>
-      <c r="BQ63" t="n">
-        <v>5.48</v>
-      </c>
-      <c r="BR63" t="n">
-        <v>1.41</v>
       </c>
       <c r="BS63" t="n">
         <v>0.19</v>
@@ -15053,13 +15053,13 @@
         </is>
       </c>
       <c r="F64" t="n">
-        <v>63.5</v>
+        <v>63.95</v>
       </c>
       <c r="G64" t="n">
-        <v>243585047500</v>
+        <v>238167580941</v>
       </c>
       <c r="H64" t="n">
-        <v>13763400</v>
+        <v>11722500</v>
       </c>
       <c r="I64" t="n">
         <v>0</v>
@@ -15146,13 +15146,13 @@
         <v>41.22</v>
       </c>
       <c r="AK64" t="n">
-        <v>69839407527.063</v>
+        <v>68286140367.76318</v>
       </c>
       <c r="AL64" t="n">
-        <v>19471226818.54517</v>
+        <v>19038175934.53238</v>
       </c>
       <c r="AM64" t="n">
-        <v>21690565227.07035</v>
+        <v>21208155025.91273</v>
       </c>
       <c r="AN64" t="n">
         <v>1.4201</v>
@@ -15193,7 +15193,7 @@
         <v>38.98</v>
       </c>
       <c r="AZ64" t="n">
-        <v>25.4</v>
+        <v>25.58</v>
       </c>
       <c r="BA64" t="n">
         <v>6.69</v>
@@ -15202,19 +15202,19 @@
         <v>10.4</v>
       </c>
       <c r="BC64" t="n">
-        <v>-24.82</v>
+        <v>-25.35</v>
       </c>
       <c r="BD64" t="n">
-        <v>-38.61</v>
+        <v>-39.05</v>
       </c>
       <c r="BE64" t="n">
         <v>-60</v>
       </c>
       <c r="BF64" t="n">
-        <v>-89.45999999999999</v>
+        <v>-89.53</v>
       </c>
       <c r="BG64" t="n">
-        <v>-83.63</v>
+        <v>-83.73999999999999</v>
       </c>
       <c r="BH64" t="n">
         <v>21.37</v>
@@ -15223,7 +15223,7 @@
         <v>0</v>
       </c>
       <c r="BJ64" t="n">
-        <v>63.5</v>
+        <v>63.95</v>
       </c>
       <c r="BK64" t="n">
         <v>4.74</v>
@@ -15232,7 +15232,7 @@
         <v>1.57</v>
       </c>
       <c r="BM64" t="n">
-        <v>63.77</v>
+        <v>64</v>
       </c>
       <c r="BN64" t="n">
         <v>64.72</v>
@@ -15241,13 +15241,13 @@
         <v>44.12</v>
       </c>
       <c r="BP64" t="n">
-        <v>61.68</v>
+        <v>62.82</v>
       </c>
       <c r="BQ64" t="n">
-        <v>40.44</v>
+        <v>40.73</v>
       </c>
       <c r="BR64" t="n">
-        <v>61.7</v>
+        <v>63.1</v>
       </c>
       <c r="BS64" t="n">
         <v>3.49</v>
@@ -15283,13 +15283,13 @@
         </is>
       </c>
       <c r="F65" t="n">
-        <v>24.11</v>
+        <v>24.27</v>
       </c>
       <c r="G65" t="n">
-        <v>243585047500</v>
+        <v>238167580941</v>
       </c>
       <c r="H65" t="n">
-        <v>6200</v>
+        <v>4700</v>
       </c>
       <c r="I65" t="n">
         <v>7298813414</v>
@@ -15304,7 +15304,7 @@
         <v>3.29</v>
       </c>
       <c r="M65" t="n">
-        <v>5.888898195245635</v>
+        <v>5.757925833150631</v>
       </c>
       <c r="N65" t="n">
         <v>0.29</v>
@@ -15382,7 +15382,7 @@
         <v>11532125194.12</v>
       </c>
       <c r="AM65" t="n">
-        <v>18246070973.78277</v>
+        <v>17840268235.2809</v>
       </c>
       <c r="AN65" t="n">
         <v>0.4734</v>
@@ -15423,7 +15423,7 @@
         <v>12.99</v>
       </c>
       <c r="AZ65" t="n">
-        <v>8.119999999999999</v>
+        <v>8.17</v>
       </c>
       <c r="BA65" t="n">
         <v>2.23</v>
@@ -15432,19 +15432,19 @@
         <v>3.47</v>
       </c>
       <c r="BC65" t="n">
-        <v>-34.01</v>
+        <v>-34.45</v>
       </c>
       <c r="BD65" t="n">
-        <v>-46.12</v>
+        <v>-46.48</v>
       </c>
       <c r="BE65" t="n">
         <v>-66.33</v>
       </c>
       <c r="BF65" t="n">
-        <v>-90.75</v>
+        <v>-90.81</v>
       </c>
       <c r="BG65" t="n">
-        <v>-85.63</v>
+        <v>-85.72</v>
       </c>
       <c r="BH65" t="n">
         <v>7.12</v>
@@ -15453,7 +15453,7 @@
         <v>0</v>
       </c>
       <c r="BJ65" t="n">
-        <v>24.11</v>
+        <v>24.27</v>
       </c>
       <c r="BK65" t="n">
         <v>1.58</v>
@@ -15462,7 +15462,7 @@
         <v>1.57</v>
       </c>
       <c r="BM65" t="n">
-        <v>24.29</v>
+        <v>24.85</v>
       </c>
       <c r="BN65" t="n">
         <v>46.43</v>
@@ -15471,13 +15471,13 @@
         <v>20.44</v>
       </c>
       <c r="BP65" t="n">
-        <v>23.85</v>
+        <v>24.11</v>
       </c>
       <c r="BQ65" t="n">
-        <v>15.36</v>
+        <v>15.46</v>
       </c>
       <c r="BR65" t="n">
-        <v>23.91</v>
+        <v>24.11</v>
       </c>
       <c r="BS65" t="n">
         <v>4.14</v>
@@ -15513,13 +15513,13 @@
         </is>
       </c>
       <c r="F66" t="n">
-        <v>20.35</v>
+        <v>20.3</v>
       </c>
       <c r="G66" t="n">
-        <v>243585047500</v>
+        <v>238167580941</v>
       </c>
       <c r="H66" t="n">
-        <v>5500</v>
+        <v>1800</v>
       </c>
       <c r="I66" t="n">
         <v>2972355254</v>
@@ -15534,7 +15534,7 @@
         <v>2.75</v>
       </c>
       <c r="M66" t="n">
-        <v>14.46057603084185</v>
+        <v>14.13896479946705</v>
       </c>
       <c r="N66" t="n">
         <v>0.25</v>
@@ -15612,7 +15612,7 @@
         <v>4696321301.320001</v>
       </c>
       <c r="AM66" t="n">
-        <v>21846192600.89686</v>
+        <v>21360321160.6278</v>
       </c>
       <c r="AN66" t="n">
         <v>0.4734</v>
@@ -15653,7 +15653,7 @@
         <v>12.99</v>
       </c>
       <c r="AZ66" t="n">
-        <v>8.17</v>
+        <v>8.15</v>
       </c>
       <c r="BA66" t="n">
         <v>2.23</v>
@@ -15662,19 +15662,19 @@
         <v>3.47</v>
       </c>
       <c r="BC66" t="n">
-        <v>-21.82</v>
+        <v>-21.63</v>
       </c>
       <c r="BD66" t="n">
-        <v>-36.17</v>
+        <v>-36.01</v>
       </c>
       <c r="BE66" t="n">
         <v>-59.83</v>
       </c>
       <c r="BF66" t="n">
-        <v>-89.04000000000001</v>
+        <v>-89.01000000000001</v>
       </c>
       <c r="BG66" t="n">
-        <v>-82.97</v>
+        <v>-82.93000000000001</v>
       </c>
       <c r="BH66" t="n">
         <v>7.12</v>
@@ -15683,7 +15683,7 @@
         <v>0</v>
       </c>
       <c r="BJ66" t="n">
-        <v>20.35</v>
+        <v>20.3</v>
       </c>
       <c r="BK66" t="n">
         <v>1.58</v>
@@ -15692,7 +15692,7 @@
         <v>1.57</v>
       </c>
       <c r="BM66" t="n">
-        <v>21</v>
+        <v>20.83</v>
       </c>
       <c r="BN66" t="n">
         <v>21.33</v>
@@ -15701,13 +15701,13 @@
         <v>9.48</v>
       </c>
       <c r="BP66" t="n">
-        <v>19.51</v>
+        <v>20.12</v>
       </c>
       <c r="BQ66" t="n">
-        <v>12.96</v>
+        <v>12.93</v>
       </c>
       <c r="BR66" t="n">
-        <v>20.91</v>
+        <v>20.83</v>
       </c>
       <c r="BS66" t="n">
         <v>3.46</v>
@@ -15973,13 +15973,13 @@
         </is>
       </c>
       <c r="F68" t="n">
-        <v>18.5</v>
+        <v>18.63</v>
       </c>
       <c r="G68" t="n">
-        <v>7853534567</v>
+        <v>8041741852</v>
       </c>
       <c r="H68" t="n">
-        <v>31600</v>
+        <v>45200</v>
       </c>
       <c r="I68" t="n">
         <v>137989898</v>
@@ -16072,7 +16072,7 @@
         <v>205604948.02</v>
       </c>
       <c r="AM68" t="n">
-        <v>544627917.2676837</v>
+        <v>557679740.0832177</v>
       </c>
       <c r="AN68" t="n">
         <v>0.1911</v>
@@ -16113,7 +16113,7 @@
         <v>21.39</v>
       </c>
       <c r="AZ68" t="n">
-        <v>34.22</v>
+        <v>34.47</v>
       </c>
       <c r="BA68" t="n">
         <v>1.24</v>
@@ -16122,19 +16122,19 @@
         <v>63.25</v>
       </c>
       <c r="BC68" t="n">
-        <v>41.64</v>
+        <v>40.65</v>
       </c>
       <c r="BD68" t="n">
-        <v>15.65</v>
+        <v>14.84</v>
       </c>
       <c r="BE68" t="n">
         <v>85</v>
       </c>
       <c r="BF68" t="n">
-        <v>-93.3</v>
+        <v>-93.34999999999999</v>
       </c>
       <c r="BG68" t="n">
-        <v>241.88</v>
+        <v>239.5</v>
       </c>
       <c r="BH68" t="n">
         <v>20.48</v>
@@ -16143,7 +16143,7 @@
         <v>0</v>
       </c>
       <c r="BJ68" t="n">
-        <v>18.5</v>
+        <v>18.63</v>
       </c>
       <c r="BK68" t="n">
         <v>1.49</v>
@@ -16152,7 +16152,7 @@
         <v>1.49</v>
       </c>
       <c r="BM68" t="n">
-        <v>18.69</v>
+        <v>18.65</v>
       </c>
       <c r="BN68" t="n">
         <v>22.11</v>
@@ -16161,13 +16161,13 @@
         <v>15.39</v>
       </c>
       <c r="BP68" t="n">
-        <v>18.47</v>
+        <v>18.39</v>
       </c>
       <c r="BQ68" t="n">
-        <v>12.44</v>
+        <v>12.53</v>
       </c>
       <c r="BR68" t="n">
-        <v>18.61</v>
+        <v>18.5</v>
       </c>
       <c r="BS68" t="n">
         <v>0</v>
@@ -16203,13 +16203,13 @@
         </is>
       </c>
       <c r="F69" t="n">
-        <v>20.91</v>
+        <v>21.32</v>
       </c>
       <c r="G69" t="n">
-        <v>7853534567</v>
+        <v>8041741852</v>
       </c>
       <c r="H69" t="n">
-        <v>1387800</v>
+        <v>3330000</v>
       </c>
       <c r="I69" t="n">
         <v>255106712</v>
@@ -16302,7 +16302,7 @@
         <v>380109000.88</v>
       </c>
       <c r="AM69" t="n">
-        <v>467472295.6547619</v>
+        <v>478675110.2380952</v>
       </c>
       <c r="AN69" t="n">
         <v>0.8856000000000001</v>
@@ -16343,7 +16343,7 @@
         <v>21.39</v>
       </c>
       <c r="AZ69" t="n">
-        <v>36.56</v>
+        <v>37.27</v>
       </c>
       <c r="BA69" t="n">
         <v>1.24</v>
@@ -16352,19 +16352,19 @@
         <v>69.59</v>
       </c>
       <c r="BC69" t="n">
-        <v>25.31</v>
+        <v>22.9</v>
       </c>
       <c r="BD69" t="n">
-        <v>2.32</v>
+        <v>0.35</v>
       </c>
       <c r="BE69" t="n">
         <v>74.83</v>
       </c>
       <c r="BF69" t="n">
-        <v>-94.06999999999999</v>
+        <v>-94.19</v>
       </c>
       <c r="BG69" t="n">
-        <v>232.79</v>
+        <v>226.39</v>
       </c>
       <c r="BH69" t="n">
         <v>20.48</v>
@@ -16373,7 +16373,7 @@
         <v>0</v>
       </c>
       <c r="BJ69" t="n">
-        <v>20.91</v>
+        <v>21.32</v>
       </c>
       <c r="BK69" t="n">
         <v>1.49</v>
@@ -16382,7 +16382,7 @@
         <v>1.49</v>
       </c>
       <c r="BM69" t="n">
-        <v>21.35</v>
+        <v>21.32</v>
       </c>
       <c r="BN69" t="n">
         <v>25.63</v>
@@ -16391,13 +16391,13 @@
         <v>16.73</v>
       </c>
       <c r="BP69" t="n">
-        <v>20.86</v>
+        <v>20.72</v>
       </c>
       <c r="BQ69" t="n">
-        <v>14.06</v>
+        <v>14.34</v>
       </c>
       <c r="BR69" t="n">
-        <v>21.35</v>
+        <v>20.85</v>
       </c>
       <c r="BS69" t="n">
         <v>0</v>
@@ -16433,13 +16433,13 @@
         </is>
       </c>
       <c r="F70" t="n">
-        <v>17.4</v>
+        <v>17.89</v>
       </c>
       <c r="G70" t="n">
-        <v>8083295102</v>
+        <v>8310928024</v>
       </c>
       <c r="H70" t="n">
-        <v>2112600</v>
+        <v>3016800</v>
       </c>
       <c r="I70" t="n">
         <v>464557268</v>
@@ -16454,7 +16454,7 @@
         <v>0.68</v>
       </c>
       <c r="M70" t="n">
-        <v>0.6379998925629409</v>
+        <v>0.6559665482333314</v>
       </c>
       <c r="N70" t="n">
         <v>0.2</v>
@@ -16532,7 +16532,7 @@
         <v>55746872.16</v>
       </c>
       <c r="AM70" t="n">
-        <v>2667754159.075908</v>
+        <v>2742880535.973598</v>
       </c>
       <c r="AN70" t="n">
         <v>0.1236</v>
@@ -16573,7 +16573,7 @@
         <v>6.9</v>
       </c>
       <c r="AZ70" t="n">
-        <v>2</v>
+        <v>2.06</v>
       </c>
       <c r="BA70" t="n">
         <v>0.12</v>
@@ -16582,19 +16582,19 @@
         <v>1.07</v>
       </c>
       <c r="BC70" t="n">
-        <v>-51.44</v>
+        <v>-52.77</v>
       </c>
       <c r="BD70" t="n">
-        <v>-60.35</v>
+        <v>-61.44</v>
       </c>
       <c r="BE70" t="n">
         <v>-88.5</v>
       </c>
       <c r="BF70" t="n">
-        <v>-99.31</v>
+        <v>-99.33</v>
       </c>
       <c r="BG70" t="n">
-        <v>-93.84999999999999</v>
+        <v>-94.02</v>
       </c>
       <c r="BH70" t="n">
         <v>26.44</v>
@@ -16603,7 +16603,7 @@
         <v>0</v>
       </c>
       <c r="BJ70" t="n">
-        <v>17.4</v>
+        <v>17.89</v>
       </c>
       <c r="BK70" t="n">
         <v>0.12</v>
@@ -16612,7 +16612,7 @@
         <v>0.1</v>
       </c>
       <c r="BM70" t="n">
-        <v>17.41</v>
+        <v>17.89</v>
       </c>
       <c r="BN70" t="n">
         <v>22.15</v>
@@ -16621,13 +16621,13 @@
         <v>13.21</v>
       </c>
       <c r="BP70" t="n">
-        <v>17.08</v>
+        <v>17.18</v>
       </c>
       <c r="BQ70" t="n">
-        <v>174.51</v>
+        <v>179.42</v>
       </c>
       <c r="BR70" t="n">
-        <v>17.31</v>
+        <v>17.18</v>
       </c>
       <c r="BS70" t="n">
         <v>0.67</v>

</xml_diff>

<commit_message>
📊 Dados atualizados - 2026-09-24 05:42
</commit_message>
<xml_diff>
--- a/data/ativos.xlsx
+++ b/data/ativos.xlsx
@@ -1047,13 +1047,13 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>25.25</v>
+        <v>24.93</v>
       </c>
       <c r="G3" t="n">
-        <v>3377611700</v>
+        <v>3334806364</v>
       </c>
       <c r="H3" t="n">
-        <v>448200</v>
+        <v>329000</v>
       </c>
       <c r="I3" t="n">
         <v>129510368</v>
@@ -1068,7 +1068,7 @@
         <v>0.88</v>
       </c>
       <c r="M3" t="n">
-        <v>0.840425015179691</v>
+        <v>0.8297740942471362</v>
       </c>
       <c r="N3" t="n">
         <v>0.09</v>
@@ -1146,7 +1146,7 @@
         <v>506385538.88</v>
       </c>
       <c r="AM3" t="n">
-        <v>659689785.15625</v>
+        <v>651329367.96875</v>
       </c>
       <c r="AN3" t="n">
         <v>2.7</v>
@@ -1187,7 +1187,7 @@
         <v>40.42</v>
       </c>
       <c r="AZ3" t="n">
-        <v>46.21</v>
+        <v>45.62</v>
       </c>
       <c r="BA3" t="n">
         <v>4.87</v>
@@ -1196,19 +1196,19 @@
         <v>21.14</v>
       </c>
       <c r="BC3" t="n">
-        <v>96.03</v>
+        <v>98.55</v>
       </c>
       <c r="BD3" t="n">
-        <v>60.06</v>
+        <v>62.12</v>
       </c>
       <c r="BE3" t="n">
         <v>83</v>
       </c>
       <c r="BF3" t="n">
-        <v>-80.72</v>
+        <v>-80.47</v>
       </c>
       <c r="BG3" t="n">
-        <v>-16.29</v>
+        <v>-15.22</v>
       </c>
       <c r="BH3" t="n">
         <v>27.85</v>
@@ -1217,7 +1217,7 @@
         <v>0</v>
       </c>
       <c r="BJ3" t="n">
-        <v>25.25</v>
+        <v>24.93</v>
       </c>
       <c r="BK3" t="n">
         <v>3.91</v>
@@ -1226,7 +1226,7 @@
         <v>4.39</v>
       </c>
       <c r="BM3" t="n">
-        <v>25.29</v>
+        <v>25.41</v>
       </c>
       <c r="BN3" t="n">
         <v>27.17</v>
@@ -1235,19 +1235,19 @@
         <v>18.72</v>
       </c>
       <c r="BP3" t="n">
-        <v>24.88</v>
+        <v>24.81</v>
       </c>
       <c r="BQ3" t="n">
-        <v>5.75</v>
+        <v>5.68</v>
       </c>
       <c r="BR3" t="n">
-        <v>25.16</v>
+        <v>25.15</v>
       </c>
       <c r="BS3" t="n">
         <v>0.79</v>
       </c>
       <c r="BT3" t="n">
-        <v>515463</v>
+        <v>526857</v>
       </c>
     </row>
     <row r="4">
@@ -1277,13 +1277,13 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>15.6</v>
+        <v>15.3</v>
       </c>
       <c r="G4" t="n">
-        <v>241560701906</v>
+        <v>236915300953</v>
       </c>
       <c r="H4" t="n">
-        <v>24129900</v>
+        <v>20586000</v>
       </c>
       <c r="I4" t="n">
         <v>15484664889</v>
@@ -1298,7 +1298,7 @@
         <v>2.76</v>
       </c>
       <c r="M4" t="n">
-        <v>2.735199203284397</v>
+        <v>2.682599186454977</v>
       </c>
       <c r="N4" t="n">
         <v>1.76</v>
@@ -1376,7 +1376,7 @@
         <v>16258898133.45</v>
       </c>
       <c r="AM4" t="n">
-        <v>23916901178.81188</v>
+        <v>23456960490.39604</v>
       </c>
       <c r="AN4" t="n">
         <v>0.269</v>
@@ -1417,7 +1417,7 @@
         <v>9.470000000000001</v>
       </c>
       <c r="AZ4" t="n">
-        <v>19.47</v>
+        <v>19.1</v>
       </c>
       <c r="BA4" t="n">
         <v>1.13</v>
@@ -1426,19 +1426,19 @@
         <v>11.39</v>
       </c>
       <c r="BC4" t="n">
-        <v>-25.61</v>
+        <v>-24.15</v>
       </c>
       <c r="BD4" t="n">
-        <v>-39.26</v>
+        <v>-38.07</v>
       </c>
       <c r="BE4" t="n">
         <v>24.83</v>
       </c>
       <c r="BF4" t="n">
-        <v>-92.77</v>
+        <v>-92.63</v>
       </c>
       <c r="BG4" t="n">
-        <v>-27.01</v>
+        <v>-25.58</v>
       </c>
       <c r="BH4" t="n">
         <v>5.7</v>
@@ -1447,7 +1447,7 @@
         <v>0</v>
       </c>
       <c r="BJ4" t="n">
-        <v>15.6</v>
+        <v>15.3</v>
       </c>
       <c r="BK4" t="n">
         <v>1.05</v>
@@ -1456,28 +1456,28 @@
         <v>1.04</v>
       </c>
       <c r="BM4" t="n">
-        <v>15.61</v>
+        <v>15.58</v>
       </c>
       <c r="BN4" t="n">
-        <v>17</v>
+        <v>16.94</v>
       </c>
       <c r="BO4" t="n">
-        <v>11.09</v>
+        <v>11.04</v>
       </c>
       <c r="BP4" t="n">
-        <v>15.31</v>
+        <v>15.3</v>
       </c>
       <c r="BQ4" t="n">
-        <v>15.04</v>
+        <v>14.76</v>
       </c>
       <c r="BR4" t="n">
-        <v>15.34</v>
+        <v>15.45</v>
       </c>
       <c r="BS4" t="n">
         <v>2.76</v>
       </c>
       <c r="BT4" t="n">
-        <v>28016813</v>
+        <v>27943700</v>
       </c>
     </row>
     <row r="5">
@@ -1737,10 +1737,10 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>7.38</v>
+        <v>7.33</v>
       </c>
       <c r="G6" t="n">
-        <v>465565019</v>
+        <v>462410846</v>
       </c>
       <c r="H6" t="n">
         <v>200</v>
@@ -1758,7 +1758,7 @@
         <v>1.91</v>
       </c>
       <c r="M6" t="n">
-        <v>7.247935799046444</v>
+        <v>7.198831501107158</v>
       </c>
       <c r="N6" t="n">
         <v>1.26</v>
@@ -1836,7 +1836,7 @@
         <v>35958279</v>
       </c>
       <c r="AM6" t="n">
-        <v>44509084.03441682</v>
+        <v>44207537.8585086</v>
       </c>
       <c r="AN6" t="n">
         <v>0.5199</v>
@@ -1877,7 +1877,7 @@
         <v>5.74</v>
       </c>
       <c r="AZ6" t="n">
-        <v>8.66</v>
+        <v>8.6</v>
       </c>
       <c r="BA6" t="n">
         <v>0.65</v>
@@ -1886,19 +1886,19 @@
         <v>7.95</v>
       </c>
       <c r="BC6" t="n">
-        <v>-4.66</v>
+        <v>-4.01</v>
       </c>
       <c r="BD6" t="n">
-        <v>-22.16</v>
+        <v>-21.63</v>
       </c>
       <c r="BE6" t="n">
         <v>17.33</v>
       </c>
       <c r="BF6" t="n">
-        <v>-91.20999999999999</v>
+        <v>-91.15000000000001</v>
       </c>
       <c r="BG6" t="n">
-        <v>7.77</v>
+        <v>8.51</v>
       </c>
       <c r="BH6" t="n">
         <v>3.86</v>
@@ -1907,7 +1907,7 @@
         <v>0</v>
       </c>
       <c r="BJ6" t="n">
-        <v>7.38</v>
+        <v>7.33</v>
       </c>
       <c r="BK6" t="n">
         <v>0.57</v>
@@ -1916,7 +1916,7 @@
         <v>0.5600000000000001</v>
       </c>
       <c r="BM6" t="n">
-        <v>7.38</v>
+        <v>7.33</v>
       </c>
       <c r="BN6" t="n">
         <v>8.16</v>
@@ -1925,19 +1925,19 @@
         <v>6.22</v>
       </c>
       <c r="BP6" t="n">
-        <v>7.37</v>
+        <v>7.33</v>
       </c>
       <c r="BQ6" t="n">
-        <v>13.12</v>
+        <v>13.03</v>
       </c>
       <c r="BR6" t="n">
-        <v>7.37</v>
+        <v>7.33</v>
       </c>
       <c r="BS6" t="n">
         <v>7.32</v>
       </c>
       <c r="BT6" t="n">
-        <v>230</v>
+        <v>237</v>
       </c>
     </row>
     <row r="7">
@@ -3117,13 +3117,13 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>4.96</v>
+        <v>4.94</v>
       </c>
       <c r="G12" t="n">
-        <v>475969192</v>
+        <v>474049963</v>
       </c>
       <c r="H12" t="n">
-        <v>344200</v>
+        <v>305500</v>
       </c>
       <c r="I12" t="n">
         <v>95961536</v>
@@ -3138,7 +3138,7 @@
         <v>0.32</v>
       </c>
       <c r="M12" t="n">
-        <v>0.0860783020749714</v>
+        <v>0.08573121243894083</v>
       </c>
       <c r="N12" t="n">
         <v>0.14</v>
@@ -3216,7 +3216,7 @@
         <v>362734606.08</v>
       </c>
       <c r="AM12" t="n">
-        <v>511794830.1075268</v>
+        <v>509731143.0107527</v>
       </c>
       <c r="AN12" t="n">
         <v>0.4208</v>
@@ -3257,7 +3257,7 @@
         <v>30.49</v>
       </c>
       <c r="AZ12" t="n">
-        <v>6.7</v>
+        <v>6.68</v>
       </c>
       <c r="BA12" t="n">
         <v>4.41</v>
@@ -3266,19 +3266,19 @@
         <v>18.12</v>
       </c>
       <c r="BC12" t="n">
-        <v>652.97</v>
+        <v>656.02</v>
       </c>
       <c r="BD12" t="n">
-        <v>514.8</v>
+        <v>517.29</v>
       </c>
       <c r="BE12" t="n">
         <v>35.17</v>
       </c>
       <c r="BF12" t="n">
-        <v>-11.06</v>
+        <v>-10.7</v>
       </c>
       <c r="BG12" t="n">
-        <v>265.3</v>
+        <v>266.78</v>
       </c>
       <c r="BH12" t="n">
         <v>16.4</v>
@@ -3287,7 +3287,7 @@
         <v>0</v>
       </c>
       <c r="BJ12" t="n">
-        <v>4.96</v>
+        <v>4.94</v>
       </c>
       <c r="BK12" t="n">
         <v>3.78</v>
@@ -3296,7 +3296,7 @@
         <v>3.43</v>
       </c>
       <c r="BM12" t="n">
-        <v>5.02</v>
+        <v>5</v>
       </c>
       <c r="BN12" t="n">
         <v>8.23</v>
@@ -3305,19 +3305,19 @@
         <v>4.42</v>
       </c>
       <c r="BP12" t="n">
+        <v>4.92</v>
+      </c>
+      <c r="BQ12" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="BR12" t="n">
         <v>4.96</v>
-      </c>
-      <c r="BQ12" t="n">
-        <v>1.45</v>
-      </c>
-      <c r="BR12" t="n">
-        <v>5</v>
       </c>
       <c r="BS12" t="n">
         <v>0.09</v>
       </c>
       <c r="BT12" t="n">
-        <v>514337</v>
+        <v>525237</v>
       </c>
     </row>
     <row r="13">
@@ -3347,13 +3347,13 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>29.72</v>
+        <v>29.34</v>
       </c>
       <c r="G13" t="n">
-        <v>14984553201</v>
+        <v>14792955214</v>
       </c>
       <c r="H13" t="n">
-        <v>11646700</v>
+        <v>2837400</v>
       </c>
       <c r="I13" t="n">
         <v>504190947</v>
@@ -3368,7 +3368,7 @@
         <v>1.13</v>
       </c>
       <c r="M13" t="n">
-        <v>5.182524802284717</v>
+        <v>5.11625914148216</v>
       </c>
       <c r="N13" t="n">
         <v>0.57</v>
@@ -3446,7 +3446,7 @@
         <v>932753251.95</v>
       </c>
       <c r="AM13" t="n">
-        <v>1559266722.268471</v>
+        <v>1539329366.701353</v>
       </c>
       <c r="AN13" t="n">
         <v>2.6301</v>
@@ -3487,7 +3487,7 @@
         <v>26.6</v>
       </c>
       <c r="AZ13" t="n">
-        <v>53.79</v>
+        <v>53.11</v>
       </c>
       <c r="BA13" t="n">
         <v>2.6</v>
@@ -3496,28 +3496,28 @@
         <v>8.69</v>
       </c>
       <c r="BC13" t="n">
-        <v>9.6</v>
+        <v>11.02</v>
       </c>
       <c r="BD13" t="n">
-        <v>-10.51</v>
+        <v>-9.35</v>
       </c>
       <c r="BE13" t="n">
         <v>81</v>
       </c>
       <c r="BF13" t="n">
-        <v>-91.23999999999999</v>
+        <v>-91.12</v>
       </c>
       <c r="BG13" t="n">
-        <v>-70.75</v>
+        <v>-70.37</v>
       </c>
       <c r="BH13" t="n">
         <v>25.49</v>
       </c>
       <c r="BI13" t="n">
-        <v>0.99</v>
+        <v>0</v>
       </c>
       <c r="BJ13" t="n">
-        <v>29.43</v>
+        <v>29.34</v>
       </c>
       <c r="BK13" t="n">
         <v>1.85</v>
@@ -3526,28 +3526,28 @@
         <v>1.96</v>
       </c>
       <c r="BM13" t="n">
-        <v>29.83</v>
+        <v>29.7</v>
       </c>
       <c r="BN13" t="n">
-        <v>32.43</v>
+        <v>32.11</v>
       </c>
       <c r="BO13" t="n">
-        <v>21.06</v>
+        <v>20.85</v>
       </c>
       <c r="BP13" t="n">
-        <v>29.43</v>
+        <v>29.06</v>
       </c>
       <c r="BQ13" t="n">
-        <v>15.18</v>
+        <v>14.99</v>
       </c>
       <c r="BR13" t="n">
-        <v>29.69</v>
+        <v>29.15</v>
       </c>
       <c r="BS13" t="n">
         <v>5.01</v>
       </c>
       <c r="BT13" t="n">
-        <v>4780353</v>
+        <v>5061107</v>
       </c>
     </row>
     <row r="14">
@@ -3577,13 +3577,13 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>10.2</v>
+        <v>10.19</v>
       </c>
       <c r="G14" t="n">
-        <v>8167853032</v>
+        <v>7877048150</v>
       </c>
       <c r="H14" t="n">
-        <v>19400</v>
+        <v>9500</v>
       </c>
       <c r="I14" t="n">
         <v>339510689</v>
@@ -3598,7 +3598,7 @@
         <v>1.92</v>
       </c>
       <c r="M14" t="n">
-        <v>3.391437784393292</v>
+        <v>3.27069042754971</v>
       </c>
       <c r="N14" t="n">
         <v>1.11</v>
@@ -3676,7 +3676,7 @@
         <v>349696009.67</v>
       </c>
       <c r="AM14" t="n">
-        <v>906531968.0355161</v>
+        <v>874256176.4705882</v>
       </c>
       <c r="AN14" t="n">
         <v>0.1489</v>
@@ -3726,19 +3726,19 @@
         <v>5.94</v>
       </c>
       <c r="BC14" t="n">
-        <v>8.65</v>
+        <v>8.76</v>
       </c>
       <c r="BD14" t="n">
-        <v>-11.28</v>
+        <v>-11.2</v>
       </c>
       <c r="BE14" t="n">
         <v>-19.67</v>
       </c>
       <c r="BF14" t="n">
-        <v>-86.06999999999999</v>
+        <v>-86.05</v>
       </c>
       <c r="BG14" t="n">
-        <v>-41.74</v>
+        <v>-41.69</v>
       </c>
       <c r="BH14" t="n">
         <v>5.3</v>
@@ -3747,7 +3747,7 @@
         <v>0</v>
       </c>
       <c r="BJ14" t="n">
-        <v>10.2</v>
+        <v>10.19</v>
       </c>
       <c r="BK14" t="n">
         <v>1.03</v>
@@ -3756,7 +3756,7 @@
         <v>1.01</v>
       </c>
       <c r="BM14" t="n">
-        <v>10.2</v>
+        <v>10.19</v>
       </c>
       <c r="BN14" t="n">
         <v>13.49</v>
@@ -3765,19 +3765,19 @@
         <v>7.65</v>
       </c>
       <c r="BP14" t="n">
-        <v>9.640000000000001</v>
+        <v>9.880000000000001</v>
       </c>
       <c r="BQ14" t="n">
-        <v>10.07</v>
+        <v>10.06</v>
       </c>
       <c r="BR14" t="n">
-        <v>9.66</v>
+        <v>9.93</v>
       </c>
       <c r="BS14" t="n">
         <v>1.44</v>
       </c>
       <c r="BT14" t="n">
-        <v>12480</v>
+        <v>10950</v>
       </c>
     </row>
     <row r="15">
@@ -3807,13 +3807,13 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>13.8</v>
+        <v>13.25</v>
       </c>
       <c r="G15" t="n">
-        <v>8167853032</v>
+        <v>7877048150</v>
       </c>
       <c r="H15" t="n">
-        <v>2427800</v>
+        <v>1438400</v>
       </c>
       <c r="I15" t="n">
         <v>343551533</v>
@@ -3828,7 +3828,7 @@
         <v>2.56</v>
       </c>
       <c r="M15" t="n">
-        <v>3.351547783313195</v>
+        <v>3.232220653671503</v>
       </c>
       <c r="N15" t="n">
         <v>1.47</v>
@@ -3906,7 +3906,7 @@
         <v>353858078.99</v>
       </c>
       <c r="AM15" t="n">
-        <v>681222104.4203503</v>
+        <v>656968152.6271893</v>
       </c>
       <c r="AN15" t="n">
         <v>0.1638</v>
@@ -3947,7 +3947,7 @@
         <v>9.050000000000001</v>
       </c>
       <c r="AZ15" t="n">
-        <v>9.18</v>
+        <v>8.81</v>
       </c>
       <c r="BA15" t="n">
         <v>1.42</v>
@@ -3956,19 +3956,19 @@
         <v>6.19</v>
       </c>
       <c r="BC15" t="n">
-        <v>-19.69</v>
+        <v>-16.36</v>
       </c>
       <c r="BD15" t="n">
-        <v>-34.43</v>
+        <v>-31.71</v>
       </c>
       <c r="BE15" t="n">
         <v>-33.5</v>
       </c>
       <c r="BF15" t="n">
-        <v>-89.7</v>
+        <v>-89.27</v>
       </c>
       <c r="BG15" t="n">
-        <v>-55.16</v>
+        <v>-53.3</v>
       </c>
       <c r="BH15" t="n">
         <v>5.3</v>
@@ -3977,7 +3977,7 @@
         <v>0</v>
       </c>
       <c r="BJ15" t="n">
-        <v>13.8</v>
+        <v>13.25</v>
       </c>
       <c r="BK15" t="n">
         <v>1.03</v>
@@ -3986,7 +3986,7 @@
         <v>1.01</v>
       </c>
       <c r="BM15" t="n">
-        <v>13.8</v>
+        <v>13.91</v>
       </c>
       <c r="BN15" t="n">
         <v>16.22</v>
@@ -3995,19 +3995,19 @@
         <v>7.84</v>
       </c>
       <c r="BP15" t="n">
-        <v>13.09</v>
+        <v>13.18</v>
       </c>
       <c r="BQ15" t="n">
-        <v>13.62</v>
+        <v>13.08</v>
       </c>
       <c r="BR15" t="n">
-        <v>13.09</v>
+        <v>13.7</v>
       </c>
       <c r="BS15" t="n">
         <v>1.92</v>
       </c>
       <c r="BT15" t="n">
-        <v>2560813</v>
+        <v>2374237</v>
       </c>
     </row>
     <row r="16">
@@ -4037,13 +4037,13 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>4.41</v>
+        <v>4.49</v>
       </c>
       <c r="G16" t="n">
-        <v>967138103</v>
+        <v>984682542</v>
       </c>
       <c r="H16" t="n">
-        <v>147600</v>
+        <v>86400</v>
       </c>
       <c r="I16" t="n">
         <v>219305733</v>
@@ -4058,7 +4058,7 @@
         <v>2.69</v>
       </c>
       <c r="M16" t="n">
-        <v>0.4575374150672568</v>
+        <v>0.46583740577589</v>
       </c>
       <c r="N16" t="n">
         <v>0.39</v>
@@ -4136,7 +4136,7 @@
         <v>17544458.64</v>
       </c>
       <c r="AM16" t="n">
-        <v>271668006.4606742</v>
+        <v>276596219.6629214</v>
       </c>
       <c r="AN16" t="n">
         <v>0.0077</v>
@@ -4177,7 +4177,7 @@
         <v>1.42</v>
       </c>
       <c r="AZ16" t="n">
-        <v>0.12</v>
+        <v>0.13</v>
       </c>
       <c r="BA16" t="n">
         <v>0.08</v>
@@ -4186,16 +4186,16 @@
         <v>0</v>
       </c>
       <c r="BC16" t="n">
-        <v>-60.57</v>
+        <v>-61.27</v>
       </c>
       <c r="BD16" t="n">
-        <v>-67.8</v>
+        <v>-68.38</v>
       </c>
       <c r="BE16" t="n">
         <v>-97.17</v>
       </c>
       <c r="BF16" t="n">
-        <v>-98.19</v>
+        <v>-98.22</v>
       </c>
       <c r="BG16" t="n">
         <v>-100</v>
@@ -4207,7 +4207,7 @@
         <v>0</v>
       </c>
       <c r="BJ16" t="n">
-        <v>4.41</v>
+        <v>4.49</v>
       </c>
       <c r="BK16" t="n">
         <v>0.08</v>
@@ -4216,28 +4216,28 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="BM16" t="n">
-        <v>4.51</v>
+        <v>4.5</v>
       </c>
       <c r="BN16" t="n">
         <v>5.54</v>
       </c>
       <c r="BO16" t="n">
-        <v>3.19</v>
+        <v>3.22</v>
       </c>
       <c r="BP16" t="n">
-        <v>4.33</v>
+        <v>4.37</v>
       </c>
       <c r="BQ16" t="n">
-        <v>60.18</v>
+        <v>61.27</v>
       </c>
       <c r="BR16" t="n">
-        <v>4.33</v>
+        <v>4.39</v>
       </c>
       <c r="BS16" t="n">
         <v>0.49</v>
       </c>
       <c r="BT16" t="n">
-        <v>140537</v>
+        <v>138393</v>
       </c>
     </row>
     <row r="17">
@@ -4267,13 +4267,13 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>32.57</v>
+        <v>32.25</v>
       </c>
       <c r="G17" t="n">
-        <v>10735948032</v>
+        <v>10630467525</v>
       </c>
       <c r="H17" t="n">
-        <v>1641000</v>
+        <v>1066400</v>
       </c>
       <c r="I17" t="n">
         <v>0</v>
@@ -4360,13 +4360,13 @@
         <v>8.039999999999999</v>
       </c>
       <c r="AK17" t="n">
-        <v>4848242427.745665</v>
+        <v>4800608528.269508</v>
       </c>
       <c r="AL17" t="n">
-        <v>1341993504</v>
+        <v>1328808440.625</v>
       </c>
       <c r="AM17" t="n">
-        <v>3323822920.123839</v>
+        <v>3291166416.408669</v>
       </c>
       <c r="AN17" t="n">
         <v>1.08</v>
@@ -4407,7 +4407,7 @@
         <v>42.98</v>
       </c>
       <c r="AZ17" t="n">
-        <v>17.42</v>
+        <v>17.25</v>
       </c>
       <c r="BA17" t="n">
         <v>4.55</v>
@@ -4416,19 +4416,19 @@
         <v>16.33</v>
       </c>
       <c r="BC17" t="n">
-        <v>61.61</v>
+        <v>63.22</v>
       </c>
       <c r="BD17" t="n">
-        <v>31.96</v>
+        <v>33.27</v>
       </c>
       <c r="BE17" t="n">
         <v>-46.5</v>
       </c>
       <c r="BF17" t="n">
-        <v>-86.03</v>
+        <v>-85.90000000000001</v>
       </c>
       <c r="BG17" t="n">
-        <v>-49.85</v>
+        <v>-49.35</v>
       </c>
       <c r="BH17" t="n">
         <v>29.25</v>
@@ -4437,7 +4437,7 @@
         <v>0</v>
       </c>
       <c r="BJ17" t="n">
-        <v>32.57</v>
+        <v>32.25</v>
       </c>
       <c r="BK17" t="n">
         <v>4.21</v>
@@ -4446,7 +4446,7 @@
         <v>12.62</v>
       </c>
       <c r="BM17" t="n">
-        <v>32.85</v>
+        <v>32.59</v>
       </c>
       <c r="BN17" t="n">
         <v>36.63</v>
@@ -4455,19 +4455,19 @@
         <v>29.53</v>
       </c>
       <c r="BP17" t="n">
-        <v>32.26</v>
+        <v>31.96</v>
       </c>
       <c r="BQ17" t="n">
-        <v>2.58</v>
+        <v>2.56</v>
       </c>
       <c r="BR17" t="n">
-        <v>32.6</v>
+        <v>32.3</v>
       </c>
       <c r="BS17" t="n">
         <v>2.21</v>
       </c>
       <c r="BT17" t="n">
-        <v>1146901</v>
+        <v>1170310</v>
       </c>
     </row>
     <row r="18">
@@ -4497,13 +4497,13 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>11.06</v>
+        <v>11.09</v>
       </c>
       <c r="G18" t="n">
-        <v>10735948032</v>
+        <v>10630467525</v>
       </c>
       <c r="H18" t="n">
-        <v>5300</v>
+        <v>15500</v>
       </c>
       <c r="I18" t="n">
         <v>671494278</v>
@@ -4518,7 +4518,7 @@
         <v>1.2</v>
       </c>
       <c r="M18" t="n">
-        <v>3.161084712344446</v>
+        <v>3.130027108755625</v>
       </c>
       <c r="N18" t="n">
         <v>0.33</v>
@@ -4596,7 +4596,7 @@
         <v>940091989.1999999</v>
       </c>
       <c r="AM18" t="n">
-        <v>3195222628.571429</v>
+        <v>3163829620.535715</v>
       </c>
       <c r="AN18" t="n">
         <v>0.36</v>
@@ -4637,7 +4637,7 @@
         <v>14.31</v>
       </c>
       <c r="AZ18" t="n">
-        <v>5.7</v>
+        <v>5.71</v>
       </c>
       <c r="BA18" t="n">
         <v>1.51</v>
@@ -4646,19 +4646,19 @@
         <v>5.44</v>
       </c>
       <c r="BC18" t="n">
-        <v>58.45</v>
+        <v>58.03</v>
       </c>
       <c r="BD18" t="n">
-        <v>29.38</v>
+        <v>29.03</v>
       </c>
       <c r="BE18" t="n">
         <v>-48.5</v>
       </c>
       <c r="BF18" t="n">
-        <v>-86.31999999999999</v>
+        <v>-86.36</v>
       </c>
       <c r="BG18" t="n">
-        <v>-50.77</v>
+        <v>-50.91</v>
       </c>
       <c r="BH18" t="n">
         <v>9.75</v>
@@ -4667,7 +4667,7 @@
         <v>0</v>
       </c>
       <c r="BJ18" t="n">
-        <v>11.06</v>
+        <v>11.09</v>
       </c>
       <c r="BK18" t="n">
         <v>1.4</v>
@@ -4676,7 +4676,7 @@
         <v>12.62</v>
       </c>
       <c r="BM18" t="n">
-        <v>11.19</v>
+        <v>11.91</v>
       </c>
       <c r="BN18" t="n">
         <v>13.82</v>
@@ -4685,19 +4685,19 @@
         <v>10.19</v>
       </c>
       <c r="BP18" t="n">
-        <v>11.05</v>
+        <v>11</v>
       </c>
       <c r="BQ18" t="n">
         <v>0.88</v>
       </c>
       <c r="BR18" t="n">
-        <v>11.1</v>
+        <v>11.04</v>
       </c>
       <c r="BS18" t="n">
         <v>2.3</v>
       </c>
       <c r="BT18" t="n">
-        <v>10003</v>
+        <v>9693</v>
       </c>
     </row>
     <row r="19">
@@ -4727,13 +4727,13 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>10.8</v>
+        <v>10.79</v>
       </c>
       <c r="G19" t="n">
-        <v>10735948032</v>
+        <v>10630467525</v>
       </c>
       <c r="H19" t="n">
-        <v>9600</v>
+        <v>15000</v>
       </c>
       <c r="I19" t="n">
         <v>317386323</v>
@@ -4748,7 +4748,7 @@
         <v>1.12</v>
       </c>
       <c r="M19" t="n">
-        <v>6.687907268809978</v>
+        <v>6.622198693528095</v>
       </c>
       <c r="N19" t="n">
         <v>0.3</v>
@@ -4826,7 +4826,7 @@
         <v>444340852.2</v>
       </c>
       <c r="AM19" t="n">
-        <v>3408237470.476191</v>
+        <v>3374751595.238095</v>
       </c>
       <c r="AN19" t="n">
         <v>0.36</v>
@@ -4867,7 +4867,7 @@
         <v>14.31</v>
       </c>
       <c r="AZ19" t="n">
-        <v>5.94</v>
+        <v>5.93</v>
       </c>
       <c r="BA19" t="n">
         <v>1.51</v>
@@ -4876,19 +4876,19 @@
         <v>5.25</v>
       </c>
       <c r="BC19" t="n">
-        <v>62.27</v>
+        <v>62.42</v>
       </c>
       <c r="BD19" t="n">
-        <v>32.49</v>
+        <v>32.61</v>
       </c>
       <c r="BE19" t="n">
         <v>-45</v>
       </c>
       <c r="BF19" t="n">
-        <v>-85.98999999999999</v>
+        <v>-85.98</v>
       </c>
       <c r="BG19" t="n">
-        <v>-51.39</v>
+        <v>-51.34</v>
       </c>
       <c r="BH19" t="n">
         <v>9.75</v>
@@ -4897,7 +4897,7 @@
         <v>0</v>
       </c>
       <c r="BJ19" t="n">
-        <v>10.8</v>
+        <v>10.79</v>
       </c>
       <c r="BK19" t="n">
         <v>1.4</v>
@@ -4906,7 +4906,7 @@
         <v>12.62</v>
       </c>
       <c r="BM19" t="n">
-        <v>10.89</v>
+        <v>10.79</v>
       </c>
       <c r="BN19" t="n">
         <v>11.41</v>
@@ -4915,19 +4915,19 @@
         <v>9.19</v>
       </c>
       <c r="BP19" t="n">
-        <v>10.63</v>
+        <v>10.51</v>
       </c>
       <c r="BQ19" t="n">
-        <v>0.86</v>
+        <v>0.85</v>
       </c>
       <c r="BR19" t="n">
-        <v>10.77</v>
+        <v>10.66</v>
       </c>
       <c r="BS19" t="n">
         <v>2.16</v>
       </c>
       <c r="BT19" t="n">
-        <v>13312</v>
+        <v>12713</v>
       </c>
     </row>
     <row r="20">
@@ -5417,13 +5417,13 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>5.12</v>
+        <v>5.15</v>
       </c>
       <c r="G22" t="n">
-        <v>1025255401</v>
+        <v>1031263314</v>
       </c>
       <c r="H22" t="n">
-        <v>1500800</v>
+        <v>823100</v>
       </c>
       <c r="I22" t="n">
         <v>200245299</v>
@@ -5438,7 +5438,7 @@
         <v>0.27</v>
       </c>
       <c r="M22" t="n">
-        <v>0.08695868521610603</v>
+        <v>0.08746825601657506</v>
       </c>
       <c r="N22" t="n">
         <v>0.08</v>
@@ -5516,7 +5516,7 @@
         <v>378463615.11</v>
       </c>
       <c r="AM22" t="n">
-        <v>232484217.9138322</v>
+        <v>233846556.462585</v>
       </c>
       <c r="AN22" t="n">
         <v>0</v>
@@ -5566,19 +5566,19 @@
         <v>172.49</v>
       </c>
       <c r="BC22" t="n">
-        <v>480.18</v>
+        <v>476.8</v>
       </c>
       <c r="BD22" t="n">
-        <v>373.71</v>
+        <v>370.95</v>
       </c>
       <c r="BE22" t="n">
         <v>-100</v>
       </c>
       <c r="BF22" t="n">
-        <v>-63.09</v>
+        <v>-63.3</v>
       </c>
       <c r="BG22" t="n">
-        <v>3268.94</v>
+        <v>3249.31</v>
       </c>
       <c r="BH22" t="n">
         <v>20.75</v>
@@ -5587,7 +5587,7 @@
         <v>0</v>
       </c>
       <c r="BJ22" t="n">
-        <v>5.12</v>
+        <v>5.15</v>
       </c>
       <c r="BK22" t="n">
         <v>1.89</v>
@@ -5596,7 +5596,7 @@
         <v>0.67</v>
       </c>
       <c r="BM22" t="n">
-        <v>5.41</v>
+        <v>5.32</v>
       </c>
       <c r="BN22" t="n">
         <v>7.89</v>
@@ -5605,19 +5605,19 @@
         <v>3.37</v>
       </c>
       <c r="BP22" t="n">
-        <v>4.95</v>
+        <v>5.06</v>
       </c>
       <c r="BQ22" t="n">
-        <v>7.63</v>
+        <v>7.67</v>
       </c>
       <c r="BR22" t="n">
-        <v>5.01</v>
+        <v>5.08</v>
       </c>
       <c r="BS22" t="n">
         <v>0.09</v>
       </c>
       <c r="BT22" t="n">
-        <v>1565410</v>
+        <v>1522243</v>
       </c>
     </row>
     <row r="23">
@@ -5877,13 +5877,13 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>3</v>
+        <v>2.99</v>
       </c>
       <c r="G24" t="n">
-        <v>1211606700</v>
+        <v>1207567117</v>
       </c>
       <c r="H24" t="n">
-        <v>3762700</v>
+        <v>3723300</v>
       </c>
       <c r="I24" t="n">
         <v>403868805</v>
@@ -5898,7 +5898,7 @@
         <v>0.49</v>
       </c>
       <c r="M24" t="n">
-        <v>0.292894805738241</v>
+        <v>0.2919182736028141</v>
       </c>
       <c r="N24" t="n">
         <v>0.11</v>
@@ -5976,7 +5976,7 @@
         <v>153470145.9</v>
       </c>
       <c r="AM24" t="n">
-        <v>1091537567.567568</v>
+        <v>1087898303.603604</v>
       </c>
       <c r="AN24" t="n">
         <v>0.0813</v>
@@ -6026,19 +6026,19 @@
         <v>1.46</v>
       </c>
       <c r="BC24" t="n">
-        <v>138.55</v>
+        <v>139.35</v>
       </c>
       <c r="BD24" t="n">
-        <v>94.77</v>
+        <v>95.42</v>
       </c>
       <c r="BE24" t="n">
         <v>-53.83</v>
       </c>
       <c r="BF24" t="n">
-        <v>-87.33</v>
+        <v>-87.29000000000001</v>
       </c>
       <c r="BG24" t="n">
-        <v>-51.41</v>
+        <v>-51.24</v>
       </c>
       <c r="BH24" t="n">
         <v>5.99</v>
@@ -6047,7 +6047,7 @@
         <v>0</v>
       </c>
       <c r="BJ24" t="n">
-        <v>3</v>
+        <v>2.99</v>
       </c>
       <c r="BK24" t="n">
         <v>0.38</v>
@@ -6056,7 +6056,7 @@
         <v>0.41</v>
       </c>
       <c r="BM24" t="n">
-        <v>3.03</v>
+        <v>3.07</v>
       </c>
       <c r="BN24" t="n">
         <v>5.29</v>
@@ -6065,19 +6065,19 @@
         <v>1.92</v>
       </c>
       <c r="BP24" t="n">
-        <v>2.89</v>
+        <v>2.95</v>
       </c>
       <c r="BQ24" t="n">
-        <v>7.37</v>
+        <v>7.34</v>
       </c>
       <c r="BR24" t="n">
-        <v>2.93</v>
+        <v>2.96</v>
       </c>
       <c r="BS24" t="n">
         <v>0.29</v>
       </c>
       <c r="BT24" t="n">
-        <v>8447850</v>
+        <v>8138913</v>
       </c>
     </row>
     <row r="25">
@@ -6107,13 +6107,13 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>4.52</v>
+        <v>4.49</v>
       </c>
       <c r="G25" t="n">
-        <v>1566152873</v>
+        <v>1555757980</v>
       </c>
       <c r="H25" t="n">
-        <v>619300</v>
+        <v>873100</v>
       </c>
       <c r="I25" t="n">
         <v>346494097</v>
@@ -6128,7 +6128,7 @@
         <v>0.97</v>
       </c>
       <c r="M25" t="n">
-        <v>0.7809553334388326</v>
+        <v>0.7757719651554249</v>
       </c>
       <c r="N25" t="n">
         <v>0.22</v>
@@ -6206,7 +6206,7 @@
         <v>62368937.46</v>
       </c>
       <c r="AM25" t="n">
-        <v>575791497.4264705</v>
+        <v>571969845.5882353</v>
       </c>
       <c r="AN25" t="n">
         <v>0.4742</v>
@@ -6247,7 +6247,7 @@
         <v>3.27</v>
       </c>
       <c r="AZ25" t="n">
-        <v>10.53</v>
+        <v>10.46</v>
       </c>
       <c r="BA25" t="n">
         <v>0.23</v>
@@ -6256,19 +6256,19 @@
         <v>2.2</v>
       </c>
       <c r="BC25" t="n">
-        <v>-11.29</v>
+        <v>-10.69</v>
       </c>
       <c r="BD25" t="n">
-        <v>-27.57</v>
+        <v>-27.08</v>
       </c>
       <c r="BE25" t="n">
         <v>133</v>
       </c>
       <c r="BF25" t="n">
-        <v>-94.87</v>
+        <v>-94.84</v>
       </c>
       <c r="BG25" t="n">
-        <v>-51.33</v>
+        <v>-51.01</v>
       </c>
       <c r="BH25" t="n">
         <v>3.97</v>
@@ -6277,7 +6277,7 @@
         <v>0</v>
       </c>
       <c r="BJ25" t="n">
-        <v>4.52</v>
+        <v>4.49</v>
       </c>
       <c r="BK25" t="n">
         <v>0.18</v>
@@ -6286,7 +6286,7 @@
         <v>0.24</v>
       </c>
       <c r="BM25" t="n">
-        <v>4.58</v>
+        <v>4.75</v>
       </c>
       <c r="BN25" t="n">
         <v>6.3</v>
@@ -6295,19 +6295,19 @@
         <v>2.64</v>
       </c>
       <c r="BP25" t="n">
-        <v>4.42</v>
+        <v>4.46</v>
       </c>
       <c r="BQ25" t="n">
-        <v>19.1</v>
+        <v>18.97</v>
       </c>
       <c r="BR25" t="n">
-        <v>4.52</v>
+        <v>4.51</v>
       </c>
       <c r="BS25" t="n">
         <v>0.67</v>
       </c>
       <c r="BT25" t="n">
-        <v>1266297</v>
+        <v>1261540</v>
       </c>
     </row>
     <row r="26">
@@ -6337,13 +6337,13 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>10.34</v>
+        <v>10.29</v>
       </c>
       <c r="G26" t="n">
-        <v>14004423826</v>
+        <v>13936703918</v>
       </c>
       <c r="H26" t="n">
-        <v>15338300</v>
+        <v>18073500</v>
       </c>
       <c r="I26" t="n">
         <v>1354393401</v>
@@ -6358,7 +6358,7 @@
         <v>1.94</v>
       </c>
       <c r="M26" t="n">
-        <v>0.1805858646826056</v>
+        <v>0.1797126221776407</v>
       </c>
       <c r="N26" t="n">
         <v>0.26</v>
@@ -6436,7 +6436,7 @@
         <v>961619314.7099999</v>
       </c>
       <c r="AM26" t="n">
-        <v>5001579937.857143</v>
+        <v>4977394256.428572</v>
       </c>
       <c r="AN26" t="n">
         <v>0.1043</v>
@@ -6477,7 +6477,7 @@
         <v>7.07</v>
       </c>
       <c r="AZ26" t="n">
-        <v>1.98</v>
+        <v>1.97</v>
       </c>
       <c r="BA26" t="n">
         <v>0.66</v>
@@ -6486,19 +6486,19 @@
         <v>1.19</v>
       </c>
       <c r="BC26" t="n">
-        <v>-16.29</v>
+        <v>-15.88</v>
       </c>
       <c r="BD26" t="n">
-        <v>-31.65</v>
+        <v>-31.32</v>
       </c>
       <c r="BE26" t="n">
         <v>-80.83</v>
       </c>
       <c r="BF26" t="n">
-        <v>-93.62</v>
+        <v>-93.59</v>
       </c>
       <c r="BG26" t="n">
-        <v>-88.45999999999999</v>
+        <v>-88.40000000000001</v>
       </c>
       <c r="BH26" t="n">
         <v>4.69</v>
@@ -6507,7 +6507,7 @@
         <v>0</v>
       </c>
       <c r="BJ26" t="n">
-        <v>10.34</v>
+        <v>10.29</v>
       </c>
       <c r="BK26" t="n">
         <v>0.71</v>
@@ -6516,28 +6516,28 @@
         <v>0.72</v>
       </c>
       <c r="BM26" t="n">
-        <v>10.4</v>
+        <v>10.55</v>
       </c>
       <c r="BN26" t="n">
-        <v>10.4</v>
+        <v>10.55</v>
       </c>
       <c r="BO26" t="n">
         <v>6.91</v>
       </c>
       <c r="BP26" t="n">
-        <v>10.04</v>
+        <v>10.16</v>
       </c>
       <c r="BQ26" t="n">
-        <v>14.42</v>
+        <v>14.35</v>
       </c>
       <c r="BR26" t="n">
-        <v>10.15</v>
+        <v>10.19</v>
       </c>
       <c r="BS26" t="n">
         <v>0.16</v>
       </c>
       <c r="BT26" t="n">
-        <v>12150707</v>
+        <v>11997927</v>
       </c>
     </row>
     <row r="27">
@@ -8165,13 +8165,13 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>14.87</v>
+        <v>14.9</v>
       </c>
       <c r="G34" t="n">
-        <v>3070501815</v>
+        <v>3076696451</v>
       </c>
       <c r="H34" t="n">
-        <v>2444800</v>
+        <v>2532500</v>
       </c>
       <c r="I34" t="n">
         <v>206489813</v>
@@ -8186,7 +8186,7 @@
         <v>0.45</v>
       </c>
       <c r="M34" t="n">
-        <v>0.2699329711903539</v>
+        <v>0.2704775520444521</v>
       </c>
       <c r="N34" t="n">
         <v>0.24</v>
@@ -8264,7 +8264,7 @@
         <v>324189006.41</v>
       </c>
       <c r="AM34" t="n">
-        <v>638357965.6964657</v>
+        <v>639645831.8087319</v>
       </c>
       <c r="AN34" t="n">
         <v>0</v>
@@ -8305,7 +8305,7 @@
         <v>30.28</v>
       </c>
       <c r="AZ34" t="n">
-        <v>34.7</v>
+        <v>34.77</v>
       </c>
       <c r="BA34" t="n">
         <v>2.29</v>
@@ -8314,19 +8314,19 @@
         <v>25.26</v>
       </c>
       <c r="BC34" t="n">
-        <v>149.42</v>
+        <v>148.92</v>
       </c>
       <c r="BD34" t="n">
-        <v>103.65</v>
+        <v>103.24</v>
       </c>
       <c r="BE34" t="n">
         <v>133.33</v>
       </c>
       <c r="BF34" t="n">
-        <v>-84.56999999999999</v>
+        <v>-84.59999999999999</v>
       </c>
       <c r="BG34" t="n">
-        <v>69.86</v>
+        <v>69.52</v>
       </c>
       <c r="BH34" t="n">
         <v>38.94</v>
@@ -8335,7 +8335,7 @@
         <v>0</v>
       </c>
       <c r="BJ34" t="n">
-        <v>14.87</v>
+        <v>14.9</v>
       </c>
       <c r="BK34" t="n">
         <v>1.57</v>
@@ -8344,7 +8344,7 @@
         <v>1.58</v>
       </c>
       <c r="BM34" t="n">
-        <v>15.09</v>
+        <v>15.41</v>
       </c>
       <c r="BN34" t="n">
         <v>29.39</v>
@@ -8353,19 +8353,19 @@
         <v>14.3</v>
       </c>
       <c r="BP34" t="n">
-        <v>14.61</v>
+        <v>14.58</v>
       </c>
       <c r="BQ34" t="n">
-        <v>9.43</v>
+        <v>9.449999999999999</v>
       </c>
       <c r="BR34" t="n">
-        <v>14.92</v>
+        <v>14.7</v>
       </c>
       <c r="BS34" t="n">
         <v>0.32</v>
       </c>
       <c r="BT34" t="n">
-        <v>3242083</v>
+        <v>3144380</v>
       </c>
     </row>
     <row r="35">
@@ -8395,13 +8395,13 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>18.43</v>
+        <v>18.04</v>
       </c>
       <c r="G35" t="n">
-        <v>93006996540</v>
+        <v>91038846580</v>
       </c>
       <c r="H35" t="n">
-        <v>83679100</v>
+        <v>46402400</v>
       </c>
       <c r="I35" t="n">
         <v>5046500000</v>
@@ -8416,7 +8416,7 @@
         <v>4.69</v>
       </c>
       <c r="M35" t="n">
-        <v>7.721474656153245</v>
+        <v>7.55807813114974</v>
       </c>
       <c r="N35" t="n">
         <v>1.79</v>
@@ -8494,7 +8494,7 @@
         <v>5349290000</v>
       </c>
       <c r="AM35" t="n">
-        <v>7686528639.669422</v>
+        <v>7523871618.181818</v>
       </c>
       <c r="AN35" t="n">
         <v>0.5305</v>
@@ -8535,7 +8535,7 @@
         <v>7.68</v>
       </c>
       <c r="AZ35" t="n">
-        <v>10.75</v>
+        <v>10.52</v>
       </c>
       <c r="BA35" t="n">
         <v>1.11</v>
@@ -8544,28 +8544,28 @@
         <v>9.119999999999999</v>
       </c>
       <c r="BC35" t="n">
-        <v>-48.96</v>
+        <v>-47.86</v>
       </c>
       <c r="BD35" t="n">
-        <v>-58.33</v>
+        <v>-57.43</v>
       </c>
       <c r="BE35" t="n">
         <v>-41.67</v>
       </c>
       <c r="BF35" t="n">
-        <v>-93.95</v>
+        <v>-93.81999999999999</v>
       </c>
       <c r="BG35" t="n">
-        <v>-50.53</v>
+        <v>-49.46</v>
       </c>
       <c r="BH35" t="n">
         <v>3.71</v>
       </c>
       <c r="BI35" t="n">
-        <v>1.03</v>
+        <v>0</v>
       </c>
       <c r="BJ35" t="n">
-        <v>18.24</v>
+        <v>18.04</v>
       </c>
       <c r="BK35" t="n">
         <v>1.06</v>
@@ -8574,7 +8574,7 @@
         <v>1.04</v>
       </c>
       <c r="BM35" t="n">
-        <v>18.53</v>
+        <v>18.49</v>
       </c>
       <c r="BN35" t="n">
         <v>20.08</v>
@@ -8583,19 +8583,19 @@
         <v>11.7</v>
       </c>
       <c r="BP35" t="n">
-        <v>18.03</v>
+        <v>17.97</v>
       </c>
       <c r="BQ35" t="n">
-        <v>17.64</v>
+        <v>17.26</v>
       </c>
       <c r="BR35" t="n">
-        <v>18.12</v>
+        <v>18.04</v>
       </c>
       <c r="BS35" t="n">
         <v>7.3</v>
       </c>
       <c r="BT35" t="n">
-        <v>38258820</v>
+        <v>41082773</v>
       </c>
     </row>
     <row r="36">
@@ -8855,10 +8855,10 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>14.8</v>
+        <v>15</v>
       </c>
       <c r="G37" t="n">
-        <v>198578114</v>
+        <v>202125000</v>
       </c>
       <c r="H37" t="n">
         <v>500</v>
@@ -8876,7 +8876,7 @@
         <v>0.88</v>
       </c>
       <c r="M37" t="n">
-        <v>1.933325219789734</v>
+        <v>1.967857142857143</v>
       </c>
       <c r="N37" t="n">
         <v>0.5</v>
@@ -8954,7 +8954,7 @@
         <v>11319000</v>
       </c>
       <c r="AM37" t="n">
-        <v>47506725.83732058</v>
+        <v>48355263.15789474</v>
       </c>
       <c r="AN37" t="n">
         <v>0</v>
@@ -8995,7 +8995,7 @@
         <v>24.36</v>
       </c>
       <c r="AZ37" t="n">
-        <v>65.81</v>
+        <v>66.7</v>
       </c>
       <c r="BA37" t="n">
         <v>2.44</v>
@@ -9004,19 +9004,19 @@
         <v>15.53</v>
       </c>
       <c r="BC37" t="n">
-        <v>101.61</v>
+        <v>98.92</v>
       </c>
       <c r="BD37" t="n">
-        <v>64.61</v>
+        <v>62.42</v>
       </c>
       <c r="BE37" t="n">
         <v>344.67</v>
       </c>
       <c r="BF37" t="n">
-        <v>-83.48</v>
+        <v>-83.7</v>
       </c>
       <c r="BG37" t="n">
-        <v>4.95</v>
+        <v>3.56</v>
       </c>
       <c r="BH37" t="n">
         <v>17.13</v>
@@ -9025,7 +9025,7 @@
         <v>0</v>
       </c>
       <c r="BJ37" t="n">
-        <v>14.8</v>
+        <v>15</v>
       </c>
       <c r="BK37" t="n">
         <v>2.31</v>
@@ -9034,7 +9034,7 @@
         <v>2.31</v>
       </c>
       <c r="BM37" t="n">
-        <v>14.9</v>
+        <v>15</v>
       </c>
       <c r="BN37" t="n">
         <v>20.9</v>
@@ -9043,19 +9043,19 @@
         <v>13.2</v>
       </c>
       <c r="BP37" t="n">
-        <v>14.8</v>
+        <v>14.99</v>
       </c>
       <c r="BQ37" t="n">
-        <v>6.4</v>
+        <v>6.49</v>
       </c>
       <c r="BR37" t="n">
-        <v>14.9</v>
+        <v>14.99</v>
       </c>
       <c r="BS37" t="n">
         <v>0.72</v>
       </c>
       <c r="BT37" t="n">
-        <v>837</v>
+        <v>853</v>
       </c>
     </row>
     <row r="38">
@@ -9315,13 +9315,13 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>69.51000000000001</v>
+        <v>69.44</v>
       </c>
       <c r="G39" t="n">
-        <v>3896613942</v>
+        <v>3892689877</v>
       </c>
       <c r="H39" t="n">
-        <v>1900</v>
+        <v>1600</v>
       </c>
       <c r="I39" t="n">
         <v>168174945</v>
@@ -9336,7 +9336,7 @@
         <v>0.53</v>
       </c>
       <c r="M39" t="n">
-        <v>0.1955929279180083</v>
+        <v>0.195395957067389</v>
       </c>
       <c r="N39" t="n">
         <v>0.06</v>
@@ -9414,7 +9414,7 @@
         <v>2536078170.6</v>
       </c>
       <c r="AM39" t="n">
-        <v>409308187.1848739</v>
+        <v>408895995.4831933</v>
       </c>
       <c r="AN39" t="n">
         <v>11.9435</v>
@@ -9455,7 +9455,7 @@
         <v>170.24</v>
       </c>
       <c r="AZ39" t="n">
-        <v>203.09</v>
+        <v>202.88</v>
       </c>
       <c r="BA39" t="n">
         <v>19.01</v>
@@ -9464,19 +9464,19 @@
         <v>91.72</v>
       </c>
       <c r="BC39" t="n">
-        <v>199.96</v>
+        <v>200.27</v>
       </c>
       <c r="BD39" t="n">
-        <v>144.92</v>
+        <v>145.17</v>
       </c>
       <c r="BE39" t="n">
         <v>192.17</v>
       </c>
       <c r="BF39" t="n">
-        <v>-72.65000000000001</v>
+        <v>-72.62</v>
       </c>
       <c r="BG39" t="n">
-        <v>31.96</v>
+        <v>32.09</v>
       </c>
       <c r="BH39" t="n">
         <v>128.13</v>
@@ -9485,7 +9485,7 @@
         <v>0</v>
       </c>
       <c r="BJ39" t="n">
-        <v>69.51000000000001</v>
+        <v>69.44</v>
       </c>
       <c r="BK39" t="n">
         <v>15.08</v>
@@ -9494,7 +9494,7 @@
         <v>15.08</v>
       </c>
       <c r="BM39" t="n">
-        <v>69.89</v>
+        <v>69.5</v>
       </c>
       <c r="BN39" t="n">
         <v>74.56</v>
@@ -9503,19 +9503,19 @@
         <v>54.98</v>
       </c>
       <c r="BP39" t="n">
-        <v>69.05</v>
+        <v>69.03</v>
       </c>
       <c r="BQ39" t="n">
-        <v>4.61</v>
+        <v>4.6</v>
       </c>
       <c r="BR39" t="n">
-        <v>69.89</v>
+        <v>69.45</v>
       </c>
       <c r="BS39" t="n">
         <v>0.58</v>
       </c>
       <c r="BT39" t="n">
-        <v>3547</v>
+        <v>3030</v>
       </c>
     </row>
     <row r="40">
@@ -9545,13 +9545,13 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>22.67</v>
+        <v>22.17</v>
       </c>
       <c r="G40" t="n">
-        <v>129918029887</v>
+        <v>127052568047</v>
       </c>
       <c r="H40" t="n">
-        <v>51731400</v>
+        <v>39523600</v>
       </c>
       <c r="I40" t="n">
         <v>5730834040</v>
@@ -9566,7 +9566,7 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="M40" t="n">
-        <v>0.39418738079099</v>
+        <v>0.385493214950817</v>
       </c>
       <c r="N40" t="n">
         <v>0.05</v>
@@ -9644,7 +9644,7 @@
         <v>15358635227.2</v>
       </c>
       <c r="AM40" t="n">
-        <v>6738487027.334024</v>
+        <v>6589863487.914937</v>
       </c>
       <c r="AN40" t="n">
         <v>0.5641</v>
@@ -9685,7 +9685,7 @@
         <v>36.13</v>
       </c>
       <c r="AZ40" t="n">
-        <v>11.45</v>
+        <v>11.2</v>
       </c>
       <c r="BA40" t="n">
         <v>2.76</v>
@@ -9694,19 +9694,19 @@
         <v>27.89</v>
       </c>
       <c r="BC40" t="n">
-        <v>95.19</v>
+        <v>99.59</v>
       </c>
       <c r="BD40" t="n">
-        <v>59.37</v>
+        <v>62.96</v>
       </c>
       <c r="BE40" t="n">
         <v>-49.5</v>
       </c>
       <c r="BF40" t="n">
-        <v>-87.83</v>
+        <v>-87.55</v>
       </c>
       <c r="BG40" t="n">
-        <v>23.03</v>
+        <v>25.8</v>
       </c>
       <c r="BH40" t="n">
         <v>32.47</v>
@@ -9715,7 +9715,7 @@
         <v>0</v>
       </c>
       <c r="BJ40" t="n">
-        <v>22.67</v>
+        <v>22.17</v>
       </c>
       <c r="BK40" t="n">
         <v>2.68</v>
@@ -9724,7 +9724,7 @@
         <v>2.5</v>
       </c>
       <c r="BM40" t="n">
-        <v>22.89</v>
+        <v>23.07</v>
       </c>
       <c r="BN40" t="n">
         <v>27.36</v>
@@ -9733,19 +9733,19 @@
         <v>17.67</v>
       </c>
       <c r="BP40" t="n">
-        <v>22.3</v>
+        <v>22.12</v>
       </c>
       <c r="BQ40" t="n">
-        <v>9.07</v>
+        <v>8.869999999999999</v>
       </c>
       <c r="BR40" t="n">
-        <v>22.84</v>
+        <v>22.43</v>
       </c>
       <c r="BS40" t="n">
         <v>0.39</v>
       </c>
       <c r="BT40" t="n">
-        <v>34132289</v>
+        <v>36599027</v>
       </c>
     </row>
     <row r="41">
@@ -9775,13 +9775,13 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>16.3</v>
+        <v>15.95</v>
       </c>
       <c r="G41" t="n">
-        <v>194181247715</v>
+        <v>190196133343</v>
       </c>
       <c r="H41" t="n">
-        <v>8101200</v>
+        <v>8581200</v>
       </c>
       <c r="I41" t="n">
         <v>5303870781</v>
@@ -9796,7 +9796,7 @@
         <v>0.92</v>
       </c>
       <c r="M41" t="n">
-        <v>1.294017709772935</v>
+        <v>1.267461033299173</v>
       </c>
       <c r="N41" t="n">
         <v>0.07000000000000001</v>
@@ -9874,7 +9874,7 @@
         <v>12304980211.92</v>
       </c>
       <c r="AM41" t="n">
-        <v>29920068985.36209</v>
+        <v>29306029790.90909</v>
       </c>
       <c r="AN41" t="n">
         <v>1.6841</v>
@@ -9915,7 +9915,7 @@
         <v>24.4</v>
       </c>
       <c r="AZ41" t="n">
-        <v>24.4</v>
+        <v>23.87</v>
       </c>
       <c r="BA41" t="n">
         <v>2.53</v>
@@ -9924,19 +9924,19 @@
         <v>13.77</v>
       </c>
       <c r="BC41" t="n">
-        <v>83.34999999999999</v>
+        <v>87.37</v>
       </c>
       <c r="BD41" t="n">
-        <v>49.7</v>
+        <v>52.99</v>
       </c>
       <c r="BE41" t="n">
         <v>49.67</v>
       </c>
       <c r="BF41" t="n">
-        <v>-84.5</v>
+        <v>-84.16</v>
       </c>
       <c r="BG41" t="n">
-        <v>-15.52</v>
+        <v>-13.67</v>
       </c>
       <c r="BH41" t="n">
         <v>17.11</v>
@@ -9945,7 +9945,7 @@
         <v>0</v>
       </c>
       <c r="BJ41" t="n">
-        <v>16.3</v>
+        <v>15.95</v>
       </c>
       <c r="BK41" t="n">
         <v>2.32</v>
@@ -9954,7 +9954,7 @@
         <v>2.34</v>
       </c>
       <c r="BM41" t="n">
-        <v>16.3</v>
+        <v>16.44</v>
       </c>
       <c r="BN41" t="n">
         <v>18.28</v>
@@ -9963,19 +9963,19 @@
         <v>13.43</v>
       </c>
       <c r="BP41" t="n">
-        <v>15.82</v>
+        <v>15.88</v>
       </c>
       <c r="BQ41" t="n">
-        <v>6.97</v>
+        <v>6.82</v>
       </c>
       <c r="BR41" t="n">
-        <v>15.95</v>
+        <v>16.17</v>
       </c>
       <c r="BS41" t="n">
         <v>0.5600000000000001</v>
       </c>
       <c r="BT41" t="n">
-        <v>7180531</v>
+        <v>7202383</v>
       </c>
     </row>
     <row r="42">
@@ -10005,13 +10005,13 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>18.43</v>
+        <v>18.03</v>
       </c>
       <c r="G42" t="n">
-        <v>194181247715</v>
+        <v>190196133343</v>
       </c>
       <c r="H42" t="n">
-        <v>44514900</v>
+        <v>39576500</v>
       </c>
       <c r="I42" t="n">
         <v>5288141247</v>
@@ -10026,7 +10026,7 @@
         <v>1.05</v>
       </c>
       <c r="M42" t="n">
-        <v>1.297866755139116</v>
+        <v>1.271231086042803</v>
       </c>
       <c r="N42" t="n">
         <v>0.08</v>
@@ -10104,7 +10104,7 @@
         <v>12268487693.04</v>
       </c>
       <c r="AM42" t="n">
-        <v>26419217376.19048</v>
+        <v>25877024944.62585</v>
       </c>
       <c r="AN42" t="n">
         <v>1.8491</v>
@@ -10145,7 +10145,7 @@
         <v>24.4</v>
       </c>
       <c r="AZ42" t="n">
-        <v>26.69</v>
+        <v>26.11</v>
       </c>
       <c r="BA42" t="n">
         <v>2.53</v>
@@ -10154,19 +10154,19 @@
         <v>15.11</v>
       </c>
       <c r="BC42" t="n">
-        <v>62.16</v>
+        <v>65.75</v>
       </c>
       <c r="BD42" t="n">
-        <v>32.4</v>
+        <v>35.34</v>
       </c>
       <c r="BE42" t="n">
         <v>44.83</v>
       </c>
       <c r="BF42" t="n">
-        <v>-86.29000000000001</v>
+        <v>-85.98</v>
       </c>
       <c r="BG42" t="n">
-        <v>-17.99</v>
+        <v>-16.17</v>
       </c>
       <c r="BH42" t="n">
         <v>17.11</v>
@@ -10175,7 +10175,7 @@
         <v>0</v>
       </c>
       <c r="BJ42" t="n">
-        <v>18.43</v>
+        <v>18.03</v>
       </c>
       <c r="BK42" t="n">
         <v>2.32</v>
@@ -10184,7 +10184,7 @@
         <v>2.34</v>
       </c>
       <c r="BM42" t="n">
-        <v>18.44</v>
+        <v>18.66</v>
       </c>
       <c r="BN42" t="n">
         <v>21.33</v>
@@ -10193,19 +10193,19 @@
         <v>15.67</v>
       </c>
       <c r="BP42" t="n">
-        <v>17.92</v>
+        <v>18.03</v>
       </c>
       <c r="BQ42" t="n">
-        <v>7.88</v>
+        <v>7.71</v>
       </c>
       <c r="BR42" t="n">
-        <v>18.05</v>
+        <v>18.18</v>
       </c>
       <c r="BS42" t="n">
         <v>0.63</v>
       </c>
       <c r="BT42" t="n">
-        <v>40434852</v>
+        <v>41807093</v>
       </c>
     </row>
     <row r="43">
@@ -10235,13 +10235,13 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>39.35</v>
+        <v>38.86</v>
       </c>
       <c r="G43" t="n">
-        <v>76394087037</v>
+        <v>75442805184</v>
       </c>
       <c r="H43" t="n">
-        <v>7846600</v>
+        <v>6633900</v>
       </c>
       <c r="I43" t="n">
         <v>1941400000</v>
@@ -10334,7 +10334,7 @@
         <v>9182822000</v>
       </c>
       <c r="AM43" t="n">
-        <v>9305004511.205845</v>
+        <v>9189135832.399511</v>
       </c>
       <c r="AN43" t="n">
         <v>4.5901</v>
@@ -10375,7 +10375,7 @@
         <v>19.95</v>
       </c>
       <c r="AZ43" t="n">
-        <v>71.42</v>
+        <v>70.53</v>
       </c>
       <c r="BA43" t="n">
         <v>5.63</v>
@@ -10384,19 +10384,19 @@
         <v>48.62</v>
       </c>
       <c r="BC43" t="n">
-        <v>-37.9</v>
+        <v>-37.12</v>
       </c>
       <c r="BD43" t="n">
-        <v>-49.3</v>
+        <v>-48.66</v>
       </c>
       <c r="BE43" t="n">
         <v>81.5</v>
       </c>
       <c r="BF43" t="n">
-        <v>-85.7</v>
+        <v>-85.52</v>
       </c>
       <c r="BG43" t="n">
-        <v>23.55</v>
+        <v>25.11</v>
       </c>
       <c r="BH43" t="n">
         <v>5.61</v>
@@ -10405,7 +10405,7 @@
         <v>0</v>
       </c>
       <c r="BJ43" t="n">
-        <v>39.35</v>
+        <v>38.86</v>
       </c>
       <c r="BK43" t="n">
         <v>4.73</v>
@@ -10414,7 +10414,7 @@
         <v>4.73</v>
       </c>
       <c r="BM43" t="n">
-        <v>39.82</v>
+        <v>39.23</v>
       </c>
       <c r="BN43" t="n">
         <v>42.98</v>
@@ -10423,19 +10423,19 @@
         <v>28.06</v>
       </c>
       <c r="BP43" t="n">
-        <v>39.04</v>
+        <v>38.67</v>
       </c>
       <c r="BQ43" t="n">
-        <v>8.31</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="BR43" t="n">
-        <v>39.72</v>
+        <v>39.14</v>
       </c>
       <c r="BS43" t="n">
         <v>0</v>
       </c>
       <c r="BT43" t="n">
-        <v>6584443</v>
+        <v>6641470</v>
       </c>
     </row>
     <row r="44">
@@ -10931,7 +10931,7 @@
         <v>4022178820</v>
       </c>
       <c r="H46" t="n">
-        <v>15997400</v>
+        <v>10047200</v>
       </c>
       <c r="I46" t="n">
         <v>1000542188</v>
@@ -11104,7 +11104,7 @@
         <v>0.46</v>
       </c>
       <c r="BM46" t="n">
-        <v>4.02</v>
+        <v>4.06</v>
       </c>
       <c r="BN46" t="n">
         <v>7.31</v>
@@ -11113,19 +11113,19 @@
         <v>2.97</v>
       </c>
       <c r="BP46" t="n">
-        <v>3.87</v>
+        <v>3.92</v>
       </c>
       <c r="BQ46" t="n">
         <v>8.789999999999999</v>
       </c>
       <c r="BR46" t="n">
-        <v>3.9</v>
+        <v>3.99</v>
       </c>
       <c r="BS46" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="BT46" t="n">
-        <v>22327503</v>
+        <v>22859087</v>
       </c>
     </row>
     <row r="47">
@@ -11155,13 +11155,13 @@
         </is>
       </c>
       <c r="F47" t="n">
-        <v>9</v>
+        <v>8.98</v>
       </c>
       <c r="G47" t="n">
-        <v>3141546300</v>
+        <v>3129905204</v>
       </c>
       <c r="H47" t="n">
-        <v>7200</v>
+        <v>3800</v>
       </c>
       <c r="I47" t="n">
         <v>254106600</v>
@@ -11176,7 +11176,7 @@
         <v>1.22</v>
       </c>
       <c r="M47" t="n">
-        <v>0.740812761847218</v>
+        <v>0.738067657476581</v>
       </c>
       <c r="N47" t="n">
         <v>0.07000000000000001</v>
@@ -11254,7 +11254,7 @@
         <v>322715382</v>
       </c>
       <c r="AM47" t="n">
-        <v>557011755.319149</v>
+        <v>554947731.2056738</v>
       </c>
       <c r="AN47" t="n">
         <v>0.4132</v>
@@ -11295,7 +11295,7 @@
         <v>11.74</v>
       </c>
       <c r="AZ47" t="n">
-        <v>11.82</v>
+        <v>11.79</v>
       </c>
       <c r="BA47" t="n">
         <v>1.46</v>
@@ -11304,19 +11304,19 @@
         <v>8.619999999999999</v>
       </c>
       <c r="BC47" t="n">
-        <v>59.71</v>
+        <v>60.06</v>
       </c>
       <c r="BD47" t="n">
-        <v>30.4</v>
+        <v>30.69</v>
       </c>
       <c r="BE47" t="n">
         <v>31.33</v>
       </c>
       <c r="BF47" t="n">
-        <v>-83.79000000000001</v>
+        <v>-83.76000000000001</v>
       </c>
       <c r="BG47" t="n">
-        <v>-4.23</v>
+        <v>-4.01</v>
       </c>
       <c r="BH47" t="n">
         <v>7.23</v>
@@ -11325,7 +11325,7 @@
         <v>0</v>
       </c>
       <c r="BJ47" t="n">
-        <v>9</v>
+        <v>8.98</v>
       </c>
       <c r="BK47" t="n">
         <v>1.27</v>
@@ -11343,19 +11343,19 @@
         <v>7.19</v>
       </c>
       <c r="BP47" t="n">
-        <v>8.93</v>
+        <v>8.92</v>
       </c>
       <c r="BQ47" t="n">
-        <v>6.96</v>
+        <v>6.94</v>
       </c>
       <c r="BR47" t="n">
-        <v>9</v>
+        <v>8.99</v>
       </c>
       <c r="BS47" t="n">
         <v>0.53</v>
       </c>
       <c r="BT47" t="n">
-        <v>11766</v>
+        <v>11413</v>
       </c>
     </row>
     <row r="48">
@@ -11385,13 +11385,13 @@
         </is>
       </c>
       <c r="F48" t="n">
-        <v>9.1</v>
+        <v>9.19</v>
       </c>
       <c r="G48" t="n">
-        <v>3141546300</v>
+        <v>3129905204</v>
       </c>
       <c r="H48" t="n">
-        <v>1200</v>
+        <v>3700</v>
       </c>
       <c r="I48" t="n">
         <v>93397546</v>
@@ -11406,7 +11406,7 @@
         <v>1.24</v>
       </c>
       <c r="M48" t="n">
-        <v>2.015528460989824</v>
+        <v>2.008059858567789</v>
       </c>
       <c r="N48" t="n">
         <v>0.07000000000000001</v>
@@ -11484,7 +11484,7 @@
         <v>118614883.42</v>
       </c>
       <c r="AM48" t="n">
-        <v>549221381.1188811</v>
+        <v>547186224.4755245</v>
       </c>
       <c r="AN48" t="n">
         <v>0.4132</v>
@@ -11525,7 +11525,7 @@
         <v>11.74</v>
       </c>
       <c r="AZ48" t="n">
-        <v>11.91</v>
+        <v>12.02</v>
       </c>
       <c r="BA48" t="n">
         <v>1.46</v>
@@ -11534,19 +11534,19 @@
         <v>8.24</v>
       </c>
       <c r="BC48" t="n">
-        <v>57.95</v>
+        <v>56.4</v>
       </c>
       <c r="BD48" t="n">
-        <v>28.97</v>
+        <v>27.7</v>
       </c>
       <c r="BE48" t="n">
         <v>30.83</v>
       </c>
       <c r="BF48" t="n">
-        <v>-83.97</v>
+        <v>-84.13</v>
       </c>
       <c r="BG48" t="n">
-        <v>-9.49</v>
+        <v>-10.38</v>
       </c>
       <c r="BH48" t="n">
         <v>7.23</v>
@@ -11555,7 +11555,7 @@
         <v>0</v>
       </c>
       <c r="BJ48" t="n">
-        <v>9.1</v>
+        <v>9.19</v>
       </c>
       <c r="BK48" t="n">
         <v>1.27</v>
@@ -11564,7 +11564,7 @@
         <v>1.29</v>
       </c>
       <c r="BM48" t="n">
-        <v>9.15</v>
+        <v>9.35</v>
       </c>
       <c r="BN48" t="n">
         <v>9.48</v>
@@ -11573,19 +11573,19 @@
         <v>7.2</v>
       </c>
       <c r="BP48" t="n">
-        <v>9.07</v>
+        <v>9.09</v>
       </c>
       <c r="BQ48" t="n">
-        <v>7.04</v>
+        <v>7.11</v>
       </c>
       <c r="BR48" t="n">
-        <v>9.15</v>
+        <v>9.09</v>
       </c>
       <c r="BS48" t="n">
         <v>0.54</v>
       </c>
       <c r="BT48" t="n">
-        <v>2453</v>
+        <v>2420</v>
       </c>
     </row>
     <row r="49">
@@ -11845,13 +11845,13 @@
         </is>
       </c>
       <c r="F50" t="n">
-        <v>32.61</v>
+        <v>33.31</v>
       </c>
       <c r="G50" t="n">
-        <v>961816100</v>
+        <v>952237200</v>
       </c>
       <c r="H50" t="n">
-        <v>600</v>
+        <v>1200</v>
       </c>
       <c r="I50" t="n">
         <v>11540870</v>
@@ -11866,7 +11866,7 @@
         <v>0.8</v>
       </c>
       <c r="M50" t="n">
-        <v>0.9730569423610977</v>
+        <v>0.9633660927847777</v>
       </c>
       <c r="N50" t="n">
         <v>0.06</v>
@@ -11944,7 +11944,7 @@
         <v>84709985.8</v>
       </c>
       <c r="AM50" t="n">
-        <v>328264880.546075</v>
+        <v>324995631.3993174</v>
       </c>
       <c r="AN50" t="n">
         <v>4.4983</v>
@@ -11985,7 +11985,7 @@
         <v>68.48999999999999</v>
       </c>
       <c r="AZ50" t="n">
-        <v>71.91</v>
+        <v>73.45</v>
       </c>
       <c r="BA50" t="n">
         <v>9.210000000000001</v>
@@ -11994,19 +11994,19 @@
         <v>30.53</v>
       </c>
       <c r="BC50" t="n">
-        <v>157.21</v>
+        <v>151.81</v>
       </c>
       <c r="BD50" t="n">
-        <v>110.01</v>
+        <v>105.6</v>
       </c>
       <c r="BE50" t="n">
         <v>120.5</v>
       </c>
       <c r="BF50" t="n">
-        <v>-71.75</v>
+        <v>-72.34</v>
       </c>
       <c r="BG50" t="n">
-        <v>-6.38</v>
+        <v>-8.35</v>
       </c>
       <c r="BH50" t="n">
         <v>42.6</v>
@@ -12015,7 +12015,7 @@
         <v>0</v>
       </c>
       <c r="BJ50" t="n">
-        <v>32.61</v>
+        <v>33.31</v>
       </c>
       <c r="BK50" t="n">
         <v>7.34</v>
@@ -12024,7 +12024,7 @@
         <v>7.6</v>
       </c>
       <c r="BM50" t="n">
-        <v>33.93</v>
+        <v>33.8</v>
       </c>
       <c r="BN50" t="n">
         <v>39.22</v>
@@ -12033,19 +12033,19 @@
         <v>23.5</v>
       </c>
       <c r="BP50" t="n">
-        <v>32.61</v>
+        <v>33.07</v>
       </c>
       <c r="BQ50" t="n">
-        <v>4.29</v>
+        <v>4.38</v>
       </c>
       <c r="BR50" t="n">
-        <v>33.93</v>
+        <v>33.09</v>
       </c>
       <c r="BS50" t="n">
         <v>0.4</v>
       </c>
       <c r="BT50" t="n">
-        <v>493</v>
+        <v>487</v>
       </c>
     </row>
     <row r="51">
@@ -12523,13 +12523,13 @@
         </is>
       </c>
       <c r="F53" t="n">
-        <v>6.41</v>
+        <v>6.26</v>
       </c>
       <c r="G53" t="n">
-        <v>877223863</v>
+        <v>856696055</v>
       </c>
       <c r="H53" t="n">
-        <v>2900</v>
+        <v>5200</v>
       </c>
       <c r="I53" t="n">
         <v>136852484</v>
@@ -12544,7 +12544,7 @@
         <v>2.79</v>
       </c>
       <c r="M53" t="n">
-        <v>2.27886406392055</v>
+        <v>2.225536645532411</v>
       </c>
       <c r="N53" t="n">
         <v>1.48</v>
@@ -12622,7 +12622,7 @@
         <v>39687220.36</v>
       </c>
       <c r="AM53" t="n">
-        <v>44687919.66377993</v>
+        <v>43642183.138054</v>
       </c>
       <c r="AN53" t="n">
         <v>0</v>
@@ -12672,16 +12672,16 @@
         <v>0</v>
       </c>
       <c r="BC53" t="n">
-        <v>-38.52</v>
+        <v>-37.05</v>
       </c>
       <c r="BD53" t="n">
-        <v>-49.8</v>
+        <v>-48.6</v>
       </c>
       <c r="BE53" t="n">
         <v>-100</v>
       </c>
       <c r="BF53" t="n">
-        <v>-95.48</v>
+        <v>-95.37</v>
       </c>
       <c r="BG53" t="n">
         <v>-100</v>
@@ -12693,7 +12693,7 @@
         <v>0</v>
       </c>
       <c r="BJ53" t="n">
-        <v>6.41</v>
+        <v>6.26</v>
       </c>
       <c r="BK53" t="n">
         <v>0.29</v>
@@ -12702,7 +12702,7 @@
         <v>0.09</v>
       </c>
       <c r="BM53" t="n">
-        <v>6.47</v>
+        <v>6.44</v>
       </c>
       <c r="BN53" t="n">
         <v>10.39</v>
@@ -12711,19 +12711,19 @@
         <v>4.82</v>
       </c>
       <c r="BP53" t="n">
-        <v>6.38</v>
+        <v>6.22</v>
       </c>
       <c r="BQ53" t="n">
-        <v>75.13</v>
+        <v>73.37</v>
       </c>
       <c r="BR53" t="n">
-        <v>6.46</v>
+        <v>6.42</v>
       </c>
       <c r="BS53" t="n">
         <v>2.36</v>
       </c>
       <c r="BT53" t="n">
-        <v>42190</v>
+        <v>36310</v>
       </c>
     </row>
     <row r="54">
@@ -12753,13 +12753,13 @@
         </is>
       </c>
       <c r="F54" t="n">
-        <v>10.52</v>
+        <v>10.26</v>
       </c>
       <c r="G54" t="n">
-        <v>2453391398</v>
+        <v>2392756199</v>
       </c>
       <c r="H54" t="n">
-        <v>219900</v>
+        <v>175700</v>
       </c>
       <c r="I54" t="n">
         <v>233212121</v>
@@ -12774,7 +12774,7 @@
         <v>0.97</v>
       </c>
       <c r="M54" t="n">
-        <v>1.377067935496371</v>
+        <v>1.34303390881257</v>
       </c>
       <c r="N54" t="n">
         <v>0.5600000000000001</v>
@@ -12852,7 +12852,7 @@
         <v>233212121</v>
       </c>
       <c r="AM54" t="n">
-        <v>335621258.2763338</v>
+        <v>327326429.4117647</v>
       </c>
       <c r="AN54" t="n">
         <v>0.1531</v>
@@ -12893,7 +12893,7 @@
         <v>12.25</v>
       </c>
       <c r="AZ54" t="n">
-        <v>16.74</v>
+        <v>16.33</v>
       </c>
       <c r="BA54" t="n">
         <v>0.98</v>
@@ -12902,19 +12902,19 @@
         <v>6.52</v>
       </c>
       <c r="BC54" t="n">
-        <v>42.66</v>
+        <v>46.27</v>
       </c>
       <c r="BD54" t="n">
-        <v>16.48</v>
+        <v>19.43</v>
       </c>
       <c r="BE54" t="n">
         <v>59.17</v>
       </c>
       <c r="BF54" t="n">
-        <v>-90.65000000000001</v>
+        <v>-90.42</v>
       </c>
       <c r="BG54" t="n">
-        <v>-38.06</v>
+        <v>-36.49</v>
       </c>
       <c r="BH54" t="n">
         <v>10.01</v>
@@ -12923,7 +12923,7 @@
         <v>0</v>
       </c>
       <c r="BJ54" t="n">
-        <v>10.52</v>
+        <v>10.26</v>
       </c>
       <c r="BK54" t="n">
         <v>1</v>
@@ -12932,7 +12932,7 @@
         <v>1</v>
       </c>
       <c r="BM54" t="n">
-        <v>10.62</v>
+        <v>10.58</v>
       </c>
       <c r="BN54" t="n">
         <v>11.75</v>
@@ -12941,19 +12941,19 @@
         <v>8.279999999999999</v>
       </c>
       <c r="BP54" t="n">
-        <v>10.37</v>
+        <v>10.25</v>
       </c>
       <c r="BQ54" t="n">
-        <v>10.49</v>
+        <v>10.23</v>
       </c>
       <c r="BR54" t="n">
-        <v>10.49</v>
+        <v>10.46</v>
       </c>
       <c r="BS54" t="n">
         <v>1.26</v>
       </c>
       <c r="BT54" t="n">
-        <v>273040</v>
+        <v>277350</v>
       </c>
     </row>
     <row r="55">
@@ -12983,13 +12983,13 @@
         </is>
       </c>
       <c r="F55" t="n">
-        <v>50.44</v>
+        <v>50.03</v>
       </c>
       <c r="G55" t="n">
-        <v>6482124212</v>
+        <v>6525984600</v>
       </c>
       <c r="H55" t="n">
-        <v>2200</v>
+        <v>700</v>
       </c>
       <c r="I55" t="n">
         <v>84052790</v>
@@ -13004,7 +13004,7 @@
         <v>2</v>
       </c>
       <c r="M55" t="n">
-        <v>1.00065302359015</v>
+        <v>1.007423802494199</v>
       </c>
       <c r="N55" t="n">
         <v>0.16</v>
@@ -13082,7 +13082,7 @@
         <v>579123723.1</v>
       </c>
       <c r="AM55" t="n">
-        <v>326062586.1167002</v>
+        <v>328268843.0583501</v>
       </c>
       <c r="AN55" t="n">
         <v>3.1953</v>
@@ -13123,7 +13123,7 @@
         <v>51.21</v>
       </c>
       <c r="AZ55" t="n">
-        <v>53.05</v>
+        <v>52.61</v>
       </c>
       <c r="BA55" t="n">
         <v>9.380000000000001</v>
@@ -13132,19 +13132,19 @@
         <v>16.08</v>
       </c>
       <c r="BC55" t="n">
-        <v>24.33</v>
+        <v>25.35</v>
       </c>
       <c r="BD55" t="n">
-        <v>1.52</v>
+        <v>2.35</v>
       </c>
       <c r="BE55" t="n">
         <v>5.17</v>
       </c>
       <c r="BF55" t="n">
-        <v>-81.41</v>
+        <v>-81.26000000000001</v>
       </c>
       <c r="BG55" t="n">
-        <v>-68.13</v>
+        <v>-67.87</v>
       </c>
       <c r="BH55" t="n">
         <v>25.37</v>
@@ -13153,7 +13153,7 @@
         <v>0</v>
       </c>
       <c r="BJ55" t="n">
-        <v>50.44</v>
+        <v>50.03</v>
       </c>
       <c r="BK55" t="n">
         <v>6.89</v>
@@ -13162,7 +13162,7 @@
         <v>7.03</v>
       </c>
       <c r="BM55" t="n">
-        <v>50.58</v>
+        <v>50.98</v>
       </c>
       <c r="BN55" t="n">
         <v>73.67</v>
@@ -13171,19 +13171,19 @@
         <v>35.58</v>
       </c>
       <c r="BP55" t="n">
-        <v>49.41</v>
+        <v>50.03</v>
       </c>
       <c r="BQ55" t="n">
-        <v>7.17</v>
+        <v>7.12</v>
       </c>
       <c r="BR55" t="n">
-        <v>50.07</v>
+        <v>50.98</v>
       </c>
       <c r="BS55" t="n">
         <v>0.66</v>
       </c>
       <c r="BT55" t="n">
-        <v>7645</v>
+        <v>7090</v>
       </c>
     </row>
     <row r="56">
@@ -13213,13 +13213,13 @@
         </is>
       </c>
       <c r="F56" t="n">
-        <v>60.11</v>
+        <v>59.25</v>
       </c>
       <c r="G56" t="n">
-        <v>6482124212</v>
+        <v>6525984600</v>
       </c>
       <c r="H56" t="n">
-        <v>21900</v>
+        <v>17800</v>
       </c>
       <c r="I56" t="n">
         <v>39675836</v>
@@ -13234,7 +13234,7 @@
         <v>2.41</v>
       </c>
       <c r="M56" t="n">
-        <v>2.119871612905345</v>
+        <v>2.134215428051634</v>
       </c>
       <c r="N56" t="n">
         <v>0.19</v>
@@ -13312,7 +13312,7 @@
         <v>273366510.04</v>
       </c>
       <c r="AM56" t="n">
-        <v>269639110.3161398</v>
+        <v>271463585.6905158</v>
       </c>
       <c r="AN56" t="n">
         <v>3.5102</v>
@@ -13353,7 +13353,7 @@
         <v>51.21</v>
       </c>
       <c r="AZ56" t="n">
-        <v>57.41</v>
+        <v>56.58</v>
       </c>
       <c r="BA56" t="n">
         <v>9.380000000000001</v>
@@ -13362,19 +13362,19 @@
         <v>17.68</v>
       </c>
       <c r="BC56" t="n">
-        <v>4.33</v>
+        <v>5.85</v>
       </c>
       <c r="BD56" t="n">
-        <v>-14.81</v>
+        <v>-13.58</v>
       </c>
       <c r="BE56" t="n">
         <v>-4.5</v>
       </c>
       <c r="BF56" t="n">
-        <v>-84.40000000000001</v>
+        <v>-84.17</v>
       </c>
       <c r="BG56" t="n">
-        <v>-70.59</v>
+        <v>-70.16</v>
       </c>
       <c r="BH56" t="n">
         <v>25.37</v>
@@ -13383,7 +13383,7 @@
         <v>0</v>
       </c>
       <c r="BJ56" t="n">
-        <v>60.11</v>
+        <v>59.25</v>
       </c>
       <c r="BK56" t="n">
         <v>6.89</v>
@@ -13392,7 +13392,7 @@
         <v>7.03</v>
       </c>
       <c r="BM56" t="n">
-        <v>61.25</v>
+        <v>60.5</v>
       </c>
       <c r="BN56" t="n">
         <v>86.77</v>
@@ -13401,19 +13401,19 @@
         <v>46.42</v>
       </c>
       <c r="BP56" t="n">
+        <v>58.42</v>
+      </c>
+      <c r="BQ56" t="n">
+        <v>8.43</v>
+      </c>
+      <c r="BR56" t="n">
         <v>60.11</v>
-      </c>
-      <c r="BQ56" t="n">
-        <v>8.550000000000001</v>
-      </c>
-      <c r="BR56" t="n">
-        <v>61.25</v>
       </c>
       <c r="BS56" t="n">
         <v>0.79</v>
       </c>
       <c r="BT56" t="n">
-        <v>32225</v>
+        <v>31633</v>
       </c>
     </row>
     <row r="57">
@@ -13443,13 +13443,13 @@
         </is>
       </c>
       <c r="F57" t="n">
-        <v>6.12</v>
+        <v>6.03</v>
       </c>
       <c r="G57" t="n">
-        <v>1431210933</v>
+        <v>1410163789</v>
       </c>
       <c r="H57" t="n">
-        <v>1412400</v>
+        <v>1477600</v>
       </c>
       <c r="I57" t="n">
         <v>233858065</v>
@@ -13464,7 +13464,7 @@
         <v>0.77</v>
       </c>
       <c r="M57" t="n">
-        <v>0.4283998728459504</v>
+        <v>0.4220998973458538</v>
       </c>
       <c r="N57" t="n">
         <v>0.08</v>
@@ -13542,7 +13542,7 @@
         <v>229180903.7</v>
       </c>
       <c r="AM57" t="n">
-        <v>107046442.2587883</v>
+        <v>105472235.5272999</v>
       </c>
       <c r="AN57" t="n">
         <v>0.347</v>
@@ -13583,7 +13583,7 @@
         <v>10.72</v>
       </c>
       <c r="AZ57" t="n">
-        <v>9.33</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="BA57" t="n">
         <v>1.13</v>
@@ -13592,19 +13592,19 @@
         <v>6.26</v>
       </c>
       <c r="BC57" t="n">
-        <v>114.56</v>
+        <v>117.77</v>
       </c>
       <c r="BD57" t="n">
-        <v>75.19</v>
+        <v>77.81</v>
       </c>
       <c r="BE57" t="n">
         <v>52.5</v>
       </c>
       <c r="BF57" t="n">
-        <v>-81.58</v>
+        <v>-81.3</v>
       </c>
       <c r="BG57" t="n">
-        <v>2.35</v>
+        <v>3.88</v>
       </c>
       <c r="BH57" t="n">
         <v>7.82</v>
@@ -13613,7 +13613,7 @@
         <v>0</v>
       </c>
       <c r="BJ57" t="n">
-        <v>6.12</v>
+        <v>6.03</v>
       </c>
       <c r="BK57" t="n">
         <v>0.98</v>
@@ -13622,28 +13622,28 @@
         <v>1.04</v>
       </c>
       <c r="BM57" t="n">
-        <v>6.16</v>
+        <v>6.22</v>
       </c>
       <c r="BN57" t="n">
-        <v>6.18</v>
+        <v>6.22</v>
       </c>
       <c r="BO57" t="n">
         <v>3.43</v>
       </c>
       <c r="BP57" t="n">
-        <v>6.04</v>
+        <v>6.03</v>
       </c>
       <c r="BQ57" t="n">
-        <v>5.91</v>
+        <v>5.82</v>
       </c>
       <c r="BR57" t="n">
-        <v>6.14</v>
+        <v>6.1</v>
       </c>
       <c r="BS57" t="n">
         <v>0.42</v>
       </c>
       <c r="BT57" t="n">
-        <v>1288511</v>
+        <v>1328663</v>
       </c>
     </row>
     <row r="58">
@@ -14133,13 +14133,13 @@
         </is>
       </c>
       <c r="F60" t="n">
-        <v>373.9</v>
+        <v>374.49</v>
       </c>
       <c r="G60" t="n">
-        <v>170031022</v>
+        <v>170299285</v>
       </c>
       <c r="H60" t="n">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="I60" t="n">
         <v>454750</v>
@@ -14154,7 +14154,7 @@
         <v>0.83</v>
       </c>
       <c r="M60" t="n">
-        <v>12.71808109193621</v>
+        <v>12.73814678670082</v>
       </c>
       <c r="N60" t="n">
         <v>0.68</v>
@@ -14232,7 +14232,7 @@
         <v>59558607.5</v>
       </c>
       <c r="AM60" t="n">
-        <v>-24931234.8973607</v>
+        <v>-24970569.64809384</v>
       </c>
       <c r="AN60" t="n">
         <v>10.0581</v>
@@ -14273,7 +14273,7 @@
         <v>944.87</v>
       </c>
       <c r="AZ60" t="n">
-        <v>2149.92</v>
+        <v>2153.32</v>
       </c>
       <c r="BA60" t="n">
         <v>231.1</v>
@@ -14282,19 +14282,19 @@
         <v>727.97</v>
       </c>
       <c r="BC60" t="n">
-        <v>209.5</v>
+        <v>209.01</v>
       </c>
       <c r="BD60" t="n">
-        <v>152.71</v>
+        <v>152.31</v>
       </c>
       <c r="BE60" t="n">
         <v>475</v>
       </c>
       <c r="BF60" t="n">
-        <v>-38.19</v>
+        <v>-38.29</v>
       </c>
       <c r="BG60" t="n">
-        <v>94.7</v>
+        <v>94.39</v>
       </c>
       <c r="BH60" t="n">
         <v>454.44</v>
@@ -14303,7 +14303,7 @@
         <v>0</v>
       </c>
       <c r="BJ60" t="n">
-        <v>373.9</v>
+        <v>374.49</v>
       </c>
       <c r="BK60" t="n">
         <v>130.97</v>
@@ -14312,22 +14312,22 @@
         <v>130.97</v>
       </c>
       <c r="BM60" t="n">
-        <v>375.5</v>
+        <v>374.49</v>
       </c>
       <c r="BN60" t="n">
         <v>405</v>
       </c>
       <c r="BO60" t="n">
-        <v>306.27</v>
+        <v>309.24</v>
       </c>
       <c r="BP60" t="n">
         <v>369.83</v>
       </c>
       <c r="BQ60" t="n">
-        <v>2.85</v>
+        <v>2.86</v>
       </c>
       <c r="BR60" t="n">
-        <v>375</v>
+        <v>369.83</v>
       </c>
       <c r="BS60" t="n">
         <v>12.82</v>
@@ -14363,13 +14363,13 @@
         </is>
       </c>
       <c r="F61" t="n">
-        <v>28.55</v>
+        <v>27.82</v>
       </c>
       <c r="G61" t="n">
-        <v>2444119183</v>
+        <v>2381625661</v>
       </c>
       <c r="H61" t="n">
-        <v>1229100</v>
+        <v>508600</v>
       </c>
       <c r="I61" t="n">
         <v>85608392</v>
@@ -14384,7 +14384,7 @@
         <v>2.37</v>
       </c>
       <c r="M61" t="n">
-        <v>1.296200318064749</v>
+        <v>1.263057857722877</v>
       </c>
       <c r="N61" t="n">
         <v>1.1</v>
@@ -14462,7 +14462,7 @@
         <v>160087693.04</v>
       </c>
       <c r="AM61" t="n">
-        <v>191846089.7174254</v>
+        <v>186940789.7174254</v>
       </c>
       <c r="AN61" t="n">
         <v>0.38</v>
@@ -14503,7 +14503,7 @@
         <v>17.56</v>
       </c>
       <c r="AZ61" t="n">
-        <v>35.97</v>
+        <v>35.05</v>
       </c>
       <c r="BA61" t="n">
         <v>2.52</v>
@@ -14512,19 +14512,19 @@
         <v>11.76</v>
       </c>
       <c r="BC61" t="n">
-        <v>-24.68</v>
+        <v>-22.7</v>
       </c>
       <c r="BD61" t="n">
-        <v>-38.5</v>
+        <v>-36.89</v>
       </c>
       <c r="BE61" t="n">
         <v>26</v>
       </c>
       <c r="BF61" t="n">
-        <v>-91.16</v>
+        <v>-90.93000000000001</v>
       </c>
       <c r="BG61" t="n">
-        <v>-58.82</v>
+        <v>-57.74</v>
       </c>
       <c r="BH61" t="n">
         <v>10.99</v>
@@ -14533,7 +14533,7 @@
         <v>0</v>
       </c>
       <c r="BJ61" t="n">
-        <v>28.55</v>
+        <v>27.82</v>
       </c>
       <c r="BK61" t="n">
         <v>1.87</v>
@@ -14542,7 +14542,7 @@
         <v>1.86</v>
       </c>
       <c r="BM61" t="n">
-        <v>28.68</v>
+        <v>28.61</v>
       </c>
       <c r="BN61" t="n">
         <v>28.68</v>
@@ -14551,19 +14551,19 @@
         <v>19.35</v>
       </c>
       <c r="BP61" t="n">
-        <v>27.53</v>
+        <v>27.6</v>
       </c>
       <c r="BQ61" t="n">
-        <v>15.33</v>
+        <v>14.94</v>
       </c>
       <c r="BR61" t="n">
-        <v>27.54</v>
+        <v>28.51</v>
       </c>
       <c r="BS61" t="n">
         <v>1.19</v>
       </c>
       <c r="BT61" t="n">
-        <v>523762</v>
+        <v>564890</v>
       </c>
     </row>
     <row r="62">
@@ -14593,13 +14593,13 @@
         </is>
       </c>
       <c r="F62" t="n">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="G62" t="n">
-        <v>10363473750</v>
+        <v>10856968100</v>
       </c>
       <c r="H62" t="n">
-        <v>600</v>
+        <v>200</v>
       </c>
       <c r="I62" t="n">
         <v>98699749</v>
@@ -14614,7 +14614,7 @@
         <v>0.64</v>
       </c>
       <c r="M62" t="n">
-        <v>0.9714567027559305</v>
+        <v>1.017716133294815</v>
       </c>
       <c r="N62" t="n">
         <v>0.13</v>
@@ -14692,7 +14692,7 @@
         <v>2757670987.06</v>
       </c>
       <c r="AM62" t="n">
-        <v>4195738360.323886</v>
+        <v>4395533643.724696</v>
       </c>
       <c r="AN62" t="n">
         <v>6.9319</v>
@@ -14733,7 +14733,7 @@
         <v>267.2</v>
       </c>
       <c r="AZ62" t="n">
-        <v>110.95</v>
+        <v>116.23</v>
       </c>
       <c r="BA62" t="n">
         <v>34.09</v>
@@ -14742,19 +14742,19 @@
         <v>76.01000000000001</v>
       </c>
       <c r="BC62" t="n">
-        <v>211.66</v>
+        <v>197.5</v>
       </c>
       <c r="BD62" t="n">
-        <v>154.47</v>
+        <v>142.91</v>
       </c>
       <c r="BE62" t="n">
         <v>5.67</v>
       </c>
       <c r="BF62" t="n">
-        <v>-67.53</v>
+        <v>-69.01000000000001</v>
       </c>
       <c r="BG62" t="n">
-        <v>-27.61</v>
+        <v>-30.9</v>
       </c>
       <c r="BH62" t="n">
         <v>170.35</v>
@@ -14763,7 +14763,7 @@
         <v>0</v>
       </c>
       <c r="BJ62" t="n">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="BK62" t="n">
         <v>27.94</v>
@@ -14772,7 +14772,7 @@
         <v>32.73</v>
       </c>
       <c r="BM62" t="n">
-        <v>114.5</v>
+        <v>110</v>
       </c>
       <c r="BN62" t="n">
         <v>122.2</v>
@@ -14781,19 +14781,19 @@
         <v>91.84999999999999</v>
       </c>
       <c r="BP62" t="n">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="BQ62" t="n">
-        <v>3.21</v>
+        <v>3.36</v>
       </c>
       <c r="BR62" t="n">
-        <v>114.5</v>
+        <v>110</v>
       </c>
       <c r="BS62" t="n">
         <v>1.01</v>
       </c>
       <c r="BT62" t="n">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="63">
@@ -14823,13 +14823,13 @@
         </is>
       </c>
       <c r="F63" t="n">
-        <v>1.34</v>
+        <v>1.35</v>
       </c>
       <c r="G63" t="n">
-        <v>349083006</v>
+        <v>351688101</v>
       </c>
       <c r="H63" t="n">
-        <v>22300</v>
+        <v>2400</v>
       </c>
       <c r="I63" t="n">
         <v>122894462</v>
@@ -14844,7 +14844,7 @@
         <v>-0.22</v>
       </c>
       <c r="M63" t="n">
-        <v>0.429354082561069</v>
+        <v>0.4325582149722281</v>
       </c>
       <c r="N63" t="n">
         <v>0.37</v>
@@ -14922,7 +14922,7 @@
         <v>31952560.12</v>
       </c>
       <c r="AM63" t="n">
-        <v>198342617.0454545</v>
+        <v>199822784.6590909</v>
       </c>
       <c r="AN63" t="n">
         <v>0</v>
@@ -14981,7 +14981,7 @@
         <v>-100</v>
       </c>
       <c r="BF63" t="n">
-        <v>-78.42</v>
+        <v>-78.58</v>
       </c>
       <c r="BG63" t="n">
         <v>-100</v>
@@ -14993,7 +14993,7 @@
         <v>0</v>
       </c>
       <c r="BJ63" t="n">
-        <v>1.34</v>
+        <v>1.35</v>
       </c>
       <c r="BK63" t="n">
         <v>0.26</v>
@@ -15002,7 +15002,7 @@
         <v>0.26</v>
       </c>
       <c r="BM63" t="n">
-        <v>1.46</v>
+        <v>1.36</v>
       </c>
       <c r="BN63" t="n">
         <v>2.12</v>
@@ -15011,19 +15011,19 @@
         <v>1.16</v>
       </c>
       <c r="BP63" t="n">
-        <v>1.34</v>
+        <v>1.35</v>
       </c>
       <c r="BQ63" t="n">
-        <v>5.13</v>
+        <v>5.17</v>
       </c>
       <c r="BR63" t="n">
-        <v>1.4</v>
+        <v>1.36</v>
       </c>
       <c r="BS63" t="n">
         <v>0.19</v>
       </c>
       <c r="BT63" t="n">
-        <v>24607</v>
+        <v>27227</v>
       </c>
     </row>
     <row r="64">
@@ -15053,13 +15053,13 @@
         </is>
       </c>
       <c r="F64" t="n">
-        <v>63.95</v>
+        <v>63.65</v>
       </c>
       <c r="G64" t="n">
-        <v>238167580941</v>
+        <v>236396551217</v>
       </c>
       <c r="H64" t="n">
-        <v>11722500</v>
+        <v>11058500</v>
       </c>
       <c r="I64" t="n">
         <v>0</v>
@@ -15146,13 +15146,13 @@
         <v>41.22</v>
       </c>
       <c r="AK64" t="n">
-        <v>68286140367.76318</v>
+        <v>67778360157.49811</v>
       </c>
       <c r="AL64" t="n">
-        <v>19038175934.53238</v>
+        <v>18896606811.91047</v>
       </c>
       <c r="AM64" t="n">
-        <v>21208155025.91273</v>
+        <v>21050449796.70525</v>
       </c>
       <c r="AN64" t="n">
         <v>1.4201</v>
@@ -15193,7 +15193,7 @@
         <v>38.98</v>
       </c>
       <c r="AZ64" t="n">
-        <v>25.58</v>
+        <v>25.46</v>
       </c>
       <c r="BA64" t="n">
         <v>6.69</v>
@@ -15202,19 +15202,19 @@
         <v>10.4</v>
       </c>
       <c r="BC64" t="n">
-        <v>-25.35</v>
+        <v>-25</v>
       </c>
       <c r="BD64" t="n">
-        <v>-39.05</v>
+        <v>-38.76</v>
       </c>
       <c r="BE64" t="n">
         <v>-60</v>
       </c>
       <c r="BF64" t="n">
-        <v>-89.53</v>
+        <v>-89.48</v>
       </c>
       <c r="BG64" t="n">
-        <v>-83.73999999999999</v>
+        <v>-83.66</v>
       </c>
       <c r="BH64" t="n">
         <v>21.37</v>
@@ -15223,7 +15223,7 @@
         <v>0</v>
       </c>
       <c r="BJ64" t="n">
-        <v>63.95</v>
+        <v>63.65</v>
       </c>
       <c r="BK64" t="n">
         <v>4.74</v>
@@ -15232,7 +15232,7 @@
         <v>1.57</v>
       </c>
       <c r="BM64" t="n">
-        <v>64</v>
+        <v>64.31999999999999</v>
       </c>
       <c r="BN64" t="n">
         <v>64.72</v>
@@ -15241,19 +15241,19 @@
         <v>44.12</v>
       </c>
       <c r="BP64" t="n">
-        <v>62.82</v>
+        <v>63.07</v>
       </c>
       <c r="BQ64" t="n">
-        <v>40.73</v>
+        <v>40.54</v>
       </c>
       <c r="BR64" t="n">
-        <v>63.1</v>
+        <v>63.58</v>
       </c>
       <c r="BS64" t="n">
         <v>3.49</v>
       </c>
       <c r="BT64" t="n">
-        <v>12175841</v>
+        <v>12220037</v>
       </c>
     </row>
     <row r="65">
@@ -15283,13 +15283,13 @@
         </is>
       </c>
       <c r="F65" t="n">
-        <v>24.27</v>
+        <v>24.42</v>
       </c>
       <c r="G65" t="n">
-        <v>238167580941</v>
+        <v>236396551217</v>
       </c>
       <c r="H65" t="n">
-        <v>4700</v>
+        <v>2800</v>
       </c>
       <c r="I65" t="n">
         <v>7298813414</v>
@@ -15304,7 +15304,7 @@
         <v>3.29</v>
       </c>
       <c r="M65" t="n">
-        <v>5.757925833150631</v>
+        <v>5.715109519701055</v>
       </c>
       <c r="N65" t="n">
         <v>0.29</v>
@@ -15382,7 +15382,7 @@
         <v>11532125194.12</v>
       </c>
       <c r="AM65" t="n">
-        <v>17840268235.2809</v>
+        <v>17707606832.73408</v>
       </c>
       <c r="AN65" t="n">
         <v>0.4734</v>
@@ -15423,7 +15423,7 @@
         <v>12.99</v>
       </c>
       <c r="AZ65" t="n">
-        <v>8.17</v>
+        <v>8.220000000000001</v>
       </c>
       <c r="BA65" t="n">
         <v>2.23</v>
@@ -15432,19 +15432,19 @@
         <v>3.47</v>
       </c>
       <c r="BC65" t="n">
-        <v>-34.45</v>
+        <v>-34.85</v>
       </c>
       <c r="BD65" t="n">
-        <v>-46.48</v>
+        <v>-46.81</v>
       </c>
       <c r="BE65" t="n">
         <v>-66.33</v>
       </c>
       <c r="BF65" t="n">
-        <v>-90.81</v>
+        <v>-90.86</v>
       </c>
       <c r="BG65" t="n">
-        <v>-85.72</v>
+        <v>-85.81</v>
       </c>
       <c r="BH65" t="n">
         <v>7.12</v>
@@ -15453,7 +15453,7 @@
         <v>0</v>
       </c>
       <c r="BJ65" t="n">
-        <v>24.27</v>
+        <v>24.42</v>
       </c>
       <c r="BK65" t="n">
         <v>1.58</v>
@@ -15462,7 +15462,7 @@
         <v>1.57</v>
       </c>
       <c r="BM65" t="n">
-        <v>24.85</v>
+        <v>24.89</v>
       </c>
       <c r="BN65" t="n">
         <v>46.43</v>
@@ -15471,19 +15471,19 @@
         <v>20.44</v>
       </c>
       <c r="BP65" t="n">
-        <v>24.11</v>
+        <v>24.05</v>
       </c>
       <c r="BQ65" t="n">
-        <v>15.46</v>
+        <v>15.55</v>
       </c>
       <c r="BR65" t="n">
-        <v>24.11</v>
+        <v>24.27</v>
       </c>
       <c r="BS65" t="n">
         <v>4.14</v>
       </c>
       <c r="BT65" t="n">
-        <v>11230</v>
+        <v>10510</v>
       </c>
     </row>
     <row r="66">
@@ -15513,13 +15513,13 @@
         </is>
       </c>
       <c r="F66" t="n">
-        <v>20.3</v>
+        <v>20.59</v>
       </c>
       <c r="G66" t="n">
-        <v>238167580941</v>
+        <v>236396551217</v>
       </c>
       <c r="H66" t="n">
-        <v>1800</v>
+        <v>900</v>
       </c>
       <c r="I66" t="n">
         <v>2972355254</v>
@@ -15534,7 +15534,7 @@
         <v>2.75</v>
       </c>
       <c r="M66" t="n">
-        <v>14.13896479946705</v>
+        <v>14.03382653158227</v>
       </c>
       <c r="N66" t="n">
         <v>0.25</v>
@@ -15612,7 +15612,7 @@
         <v>4696321301.320001</v>
       </c>
       <c r="AM66" t="n">
-        <v>21360321160.6278</v>
+        <v>21201484414.08072</v>
       </c>
       <c r="AN66" t="n">
         <v>0.4734</v>
@@ -15653,7 +15653,7 @@
         <v>12.99</v>
       </c>
       <c r="AZ66" t="n">
-        <v>8.15</v>
+        <v>8.27</v>
       </c>
       <c r="BA66" t="n">
         <v>2.23</v>
@@ -15662,19 +15662,19 @@
         <v>3.47</v>
       </c>
       <c r="BC66" t="n">
-        <v>-21.63</v>
+        <v>-22.73</v>
       </c>
       <c r="BD66" t="n">
-        <v>-36.01</v>
+        <v>-36.91</v>
       </c>
       <c r="BE66" t="n">
         <v>-59.83</v>
       </c>
       <c r="BF66" t="n">
-        <v>-89.01000000000001</v>
+        <v>-89.16</v>
       </c>
       <c r="BG66" t="n">
-        <v>-82.93000000000001</v>
+        <v>-83.17</v>
       </c>
       <c r="BH66" t="n">
         <v>7.12</v>
@@ -15683,7 +15683,7 @@
         <v>0</v>
       </c>
       <c r="BJ66" t="n">
-        <v>20.3</v>
+        <v>20.59</v>
       </c>
       <c r="BK66" t="n">
         <v>1.58</v>
@@ -15692,7 +15692,7 @@
         <v>1.57</v>
       </c>
       <c r="BM66" t="n">
-        <v>20.83</v>
+        <v>20.59</v>
       </c>
       <c r="BN66" t="n">
         <v>21.33</v>
@@ -15701,19 +15701,19 @@
         <v>9.48</v>
       </c>
       <c r="BP66" t="n">
-        <v>20.12</v>
+        <v>20.03</v>
       </c>
       <c r="BQ66" t="n">
-        <v>12.93</v>
+        <v>13.11</v>
       </c>
       <c r="BR66" t="n">
-        <v>20.83</v>
+        <v>20.03</v>
       </c>
       <c r="BS66" t="n">
         <v>3.46</v>
       </c>
       <c r="BT66" t="n">
-        <v>5614</v>
+        <v>5560</v>
       </c>
     </row>
     <row r="67">
@@ -15973,13 +15973,13 @@
         </is>
       </c>
       <c r="F68" t="n">
-        <v>18.63</v>
+        <v>18.11</v>
       </c>
       <c r="G68" t="n">
-        <v>8041741852</v>
+        <v>7727860905</v>
       </c>
       <c r="H68" t="n">
-        <v>45200</v>
+        <v>112800</v>
       </c>
       <c r="I68" t="n">
         <v>137989898</v>
@@ -16072,7 +16072,7 @@
         <v>205604948.02</v>
       </c>
       <c r="AM68" t="n">
-        <v>557679740.0832177</v>
+        <v>535912684.1192788</v>
       </c>
       <c r="AN68" t="n">
         <v>0.1911</v>
@@ -16113,7 +16113,7 @@
         <v>21.39</v>
       </c>
       <c r="AZ68" t="n">
-        <v>34.47</v>
+        <v>33.5</v>
       </c>
       <c r="BA68" t="n">
         <v>1.24</v>
@@ -16122,19 +16122,19 @@
         <v>63.25</v>
       </c>
       <c r="BC68" t="n">
-        <v>40.65</v>
+        <v>44.69</v>
       </c>
       <c r="BD68" t="n">
-        <v>14.84</v>
+        <v>18.14</v>
       </c>
       <c r="BE68" t="n">
         <v>85</v>
       </c>
       <c r="BF68" t="n">
-        <v>-93.34999999999999</v>
+        <v>-93.16</v>
       </c>
       <c r="BG68" t="n">
-        <v>239.5</v>
+        <v>249.25</v>
       </c>
       <c r="BH68" t="n">
         <v>20.48</v>
@@ -16143,7 +16143,7 @@
         <v>0</v>
       </c>
       <c r="BJ68" t="n">
-        <v>18.63</v>
+        <v>18.11</v>
       </c>
       <c r="BK68" t="n">
         <v>1.49</v>
@@ -16152,7 +16152,7 @@
         <v>1.49</v>
       </c>
       <c r="BM68" t="n">
-        <v>18.65</v>
+        <v>18.8</v>
       </c>
       <c r="BN68" t="n">
         <v>22.11</v>
@@ -16161,19 +16161,19 @@
         <v>15.39</v>
       </c>
       <c r="BP68" t="n">
-        <v>18.39</v>
+        <v>18.11</v>
       </c>
       <c r="BQ68" t="n">
-        <v>12.53</v>
+        <v>12.18</v>
       </c>
       <c r="BR68" t="n">
-        <v>18.5</v>
+        <v>18.8</v>
       </c>
       <c r="BS68" t="n">
         <v>0</v>
       </c>
       <c r="BT68" t="n">
-        <v>34920</v>
+        <v>36243</v>
       </c>
     </row>
     <row r="69">
@@ -16203,13 +16203,13 @@
         </is>
       </c>
       <c r="F69" t="n">
-        <v>21.32</v>
+        <v>20.57</v>
       </c>
       <c r="G69" t="n">
-        <v>8041741852</v>
+        <v>7727860905</v>
       </c>
       <c r="H69" t="n">
-        <v>3330000</v>
+        <v>3737300</v>
       </c>
       <c r="I69" t="n">
         <v>255106712</v>
@@ -16302,7 +16302,7 @@
         <v>380109000.88</v>
       </c>
       <c r="AM69" t="n">
-        <v>478675110.2380952</v>
+        <v>459991720.5357143</v>
       </c>
       <c r="AN69" t="n">
         <v>0.8856000000000001</v>
@@ -16343,7 +16343,7 @@
         <v>21.39</v>
       </c>
       <c r="AZ69" t="n">
-        <v>37.27</v>
+        <v>35.96</v>
       </c>
       <c r="BA69" t="n">
         <v>1.24</v>
@@ -16352,19 +16352,19 @@
         <v>69.59</v>
       </c>
       <c r="BC69" t="n">
-        <v>22.9</v>
+        <v>27.38</v>
       </c>
       <c r="BD69" t="n">
-        <v>0.35</v>
+        <v>4.01</v>
       </c>
       <c r="BE69" t="n">
         <v>74.83</v>
       </c>
       <c r="BF69" t="n">
-        <v>-94.19</v>
+        <v>-93.97</v>
       </c>
       <c r="BG69" t="n">
-        <v>226.39</v>
+        <v>238.29</v>
       </c>
       <c r="BH69" t="n">
         <v>20.48</v>
@@ -16373,7 +16373,7 @@
         <v>0</v>
       </c>
       <c r="BJ69" t="n">
-        <v>21.32</v>
+        <v>20.57</v>
       </c>
       <c r="BK69" t="n">
         <v>1.49</v>
@@ -16382,7 +16382,7 @@
         <v>1.49</v>
       </c>
       <c r="BM69" t="n">
-        <v>21.32</v>
+        <v>21.15</v>
       </c>
       <c r="BN69" t="n">
         <v>25.63</v>
@@ -16391,19 +16391,19 @@
         <v>16.73</v>
       </c>
       <c r="BP69" t="n">
-        <v>20.72</v>
+        <v>20.57</v>
       </c>
       <c r="BQ69" t="n">
-        <v>14.34</v>
+        <v>13.84</v>
       </c>
       <c r="BR69" t="n">
-        <v>20.85</v>
+        <v>21.14</v>
       </c>
       <c r="BS69" t="n">
         <v>0</v>
       </c>
       <c r="BT69" t="n">
-        <v>2035450</v>
+        <v>2027813</v>
       </c>
     </row>
     <row r="70">
@@ -16433,13 +16433,13 @@
         </is>
       </c>
       <c r="F70" t="n">
-        <v>17.89</v>
+        <v>17.6</v>
       </c>
       <c r="G70" t="n">
-        <v>8310928024</v>
+        <v>8176206897</v>
       </c>
       <c r="H70" t="n">
-        <v>3016800</v>
+        <v>2251900</v>
       </c>
       <c r="I70" t="n">
         <v>464557268</v>
@@ -16454,7 +16454,7 @@
         <v>0.68</v>
       </c>
       <c r="M70" t="n">
-        <v>0.6559665482333314</v>
+        <v>0.6453332528423601</v>
       </c>
       <c r="N70" t="n">
         <v>0.2</v>
@@ -16532,7 +16532,7 @@
         <v>55746872.16</v>
       </c>
       <c r="AM70" t="n">
-        <v>2742880535.973598</v>
+        <v>2698418117.821783</v>
       </c>
       <c r="AN70" t="n">
         <v>0.1236</v>
@@ -16573,7 +16573,7 @@
         <v>6.9</v>
       </c>
       <c r="AZ70" t="n">
-        <v>2.06</v>
+        <v>2.02</v>
       </c>
       <c r="BA70" t="n">
         <v>0.12</v>
@@ -16582,19 +16582,19 @@
         <v>1.07</v>
       </c>
       <c r="BC70" t="n">
-        <v>-52.77</v>
+        <v>-51.99</v>
       </c>
       <c r="BD70" t="n">
-        <v>-61.44</v>
+        <v>-60.8</v>
       </c>
       <c r="BE70" t="n">
         <v>-88.5</v>
       </c>
       <c r="BF70" t="n">
-        <v>-99.33</v>
+        <v>-99.31999999999999</v>
       </c>
       <c r="BG70" t="n">
-        <v>-94.02</v>
+        <v>-93.92</v>
       </c>
       <c r="BH70" t="n">
         <v>26.44</v>
@@ -16603,7 +16603,7 @@
         <v>0</v>
       </c>
       <c r="BJ70" t="n">
-        <v>17.89</v>
+        <v>17.6</v>
       </c>
       <c r="BK70" t="n">
         <v>0.12</v>
@@ -16612,7 +16612,7 @@
         <v>0.1</v>
       </c>
       <c r="BM70" t="n">
-        <v>17.89</v>
+        <v>18.02</v>
       </c>
       <c r="BN70" t="n">
         <v>22.15</v>
@@ -16621,19 +16621,19 @@
         <v>13.21</v>
       </c>
       <c r="BP70" t="n">
-        <v>17.18</v>
+        <v>17.57</v>
       </c>
       <c r="BQ70" t="n">
-        <v>179.42</v>
+        <v>176.51</v>
       </c>
       <c r="BR70" t="n">
-        <v>17.18</v>
+        <v>17.8</v>
       </c>
       <c r="BS70" t="n">
         <v>0.67</v>
       </c>
       <c r="BT70" t="n">
-        <v>4561720</v>
+        <v>4292827</v>
       </c>
     </row>
     <row r="71">

</xml_diff>

<commit_message>
📊 Dados atualizados - 2026-09-25 05:40
</commit_message>
<xml_diff>
--- a/data/ativos.xlsx
+++ b/data/ativos.xlsx
@@ -1047,13 +1047,13 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>24.93</v>
+        <v>24.76</v>
       </c>
       <c r="G3" t="n">
-        <v>3334806364</v>
+        <v>3312068474</v>
       </c>
       <c r="H3" t="n">
-        <v>329000</v>
+        <v>309400</v>
       </c>
       <c r="I3" t="n">
         <v>129510368</v>
@@ -1068,7 +1068,7 @@
         <v>0.88</v>
       </c>
       <c r="M3" t="n">
-        <v>0.8297740942471362</v>
+        <v>0.8241164008099646</v>
       </c>
       <c r="N3" t="n">
         <v>0.09</v>
@@ -1146,7 +1146,7 @@
         <v>506385538.88</v>
       </c>
       <c r="AM3" t="n">
-        <v>651329367.96875</v>
+        <v>646888373.828125</v>
       </c>
       <c r="AN3" t="n">
         <v>2.7</v>
@@ -1187,7 +1187,7 @@
         <v>40.42</v>
       </c>
       <c r="AZ3" t="n">
-        <v>45.62</v>
+        <v>45.31</v>
       </c>
       <c r="BA3" t="n">
         <v>4.87</v>
@@ -1196,19 +1196,19 @@
         <v>21.14</v>
       </c>
       <c r="BC3" t="n">
-        <v>98.55</v>
+        <v>99.91</v>
       </c>
       <c r="BD3" t="n">
-        <v>62.12</v>
+        <v>63.23</v>
       </c>
       <c r="BE3" t="n">
         <v>83</v>
       </c>
       <c r="BF3" t="n">
-        <v>-80.47</v>
+        <v>-80.34</v>
       </c>
       <c r="BG3" t="n">
-        <v>-15.22</v>
+        <v>-14.64</v>
       </c>
       <c r="BH3" t="n">
         <v>27.85</v>
@@ -1217,7 +1217,7 @@
         <v>0</v>
       </c>
       <c r="BJ3" t="n">
-        <v>24.93</v>
+        <v>24.76</v>
       </c>
       <c r="BK3" t="n">
         <v>3.91</v>
@@ -1226,7 +1226,7 @@
         <v>4.39</v>
       </c>
       <c r="BM3" t="n">
-        <v>25.41</v>
+        <v>25.04</v>
       </c>
       <c r="BN3" t="n">
         <v>27.17</v>
@@ -1235,19 +1235,19 @@
         <v>18.72</v>
       </c>
       <c r="BP3" t="n">
-        <v>24.81</v>
+        <v>24.62</v>
       </c>
       <c r="BQ3" t="n">
-        <v>5.68</v>
+        <v>5.64</v>
       </c>
       <c r="BR3" t="n">
-        <v>25.15</v>
+        <v>24.9</v>
       </c>
       <c r="BS3" t="n">
         <v>0.79</v>
       </c>
       <c r="BT3" t="n">
-        <v>526857</v>
+        <v>522973</v>
       </c>
     </row>
     <row r="4">
@@ -1277,13 +1277,13 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>15.3</v>
+        <v>15.34</v>
       </c>
       <c r="G4" t="n">
-        <v>236915300953</v>
+        <v>237534686762</v>
       </c>
       <c r="H4" t="n">
-        <v>20586000</v>
+        <v>15784900</v>
       </c>
       <c r="I4" t="n">
         <v>15484664889</v>
@@ -1298,7 +1298,7 @@
         <v>2.76</v>
       </c>
       <c r="M4" t="n">
-        <v>2.682599186454977</v>
+        <v>2.689612510882067</v>
       </c>
       <c r="N4" t="n">
         <v>1.76</v>
@@ -1376,7 +1376,7 @@
         <v>16258898133.45</v>
       </c>
       <c r="AM4" t="n">
-        <v>23456960490.39604</v>
+        <v>23518285818.0198</v>
       </c>
       <c r="AN4" t="n">
         <v>0.269</v>
@@ -1417,7 +1417,7 @@
         <v>9.470000000000001</v>
       </c>
       <c r="AZ4" t="n">
-        <v>19.1</v>
+        <v>19.15</v>
       </c>
       <c r="BA4" t="n">
         <v>1.13</v>
@@ -1426,19 +1426,19 @@
         <v>11.39</v>
       </c>
       <c r="BC4" t="n">
-        <v>-24.15</v>
+        <v>-24.35</v>
       </c>
       <c r="BD4" t="n">
-        <v>-38.07</v>
+        <v>-38.23</v>
       </c>
       <c r="BE4" t="n">
         <v>24.83</v>
       </c>
       <c r="BF4" t="n">
-        <v>-92.63</v>
+        <v>-92.65000000000001</v>
       </c>
       <c r="BG4" t="n">
-        <v>-25.58</v>
+        <v>-25.77</v>
       </c>
       <c r="BH4" t="n">
         <v>5.7</v>
@@ -1447,7 +1447,7 @@
         <v>0</v>
       </c>
       <c r="BJ4" t="n">
-        <v>15.3</v>
+        <v>15.34</v>
       </c>
       <c r="BK4" t="n">
         <v>1.05</v>
@@ -1456,7 +1456,7 @@
         <v>1.04</v>
       </c>
       <c r="BM4" t="n">
-        <v>15.58</v>
+        <v>15.55</v>
       </c>
       <c r="BN4" t="n">
         <v>16.94</v>
@@ -1465,19 +1465,19 @@
         <v>11.04</v>
       </c>
       <c r="BP4" t="n">
-        <v>15.3</v>
+        <v>15.31</v>
       </c>
       <c r="BQ4" t="n">
-        <v>14.76</v>
+        <v>14.79</v>
       </c>
       <c r="BR4" t="n">
-        <v>15.45</v>
+        <v>15.35</v>
       </c>
       <c r="BS4" t="n">
         <v>2.76</v>
       </c>
       <c r="BT4" t="n">
-        <v>27943700</v>
+        <v>27496667</v>
       </c>
     </row>
     <row r="5">
@@ -3117,13 +3117,13 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>4.94</v>
+        <v>4.89</v>
       </c>
       <c r="G12" t="n">
-        <v>474049963</v>
+        <v>469251868</v>
       </c>
       <c r="H12" t="n">
-        <v>305500</v>
+        <v>571400</v>
       </c>
       <c r="I12" t="n">
         <v>95961536</v>
@@ -3138,7 +3138,7 @@
         <v>0.32</v>
       </c>
       <c r="M12" t="n">
-        <v>0.08573121243894083</v>
+        <v>0.08486348427977373</v>
       </c>
       <c r="N12" t="n">
         <v>0.14</v>
@@ -3216,7 +3216,7 @@
         <v>362734606.08</v>
       </c>
       <c r="AM12" t="n">
-        <v>509731143.0107527</v>
+        <v>504571901.0752688</v>
       </c>
       <c r="AN12" t="n">
         <v>0.4208</v>
@@ -3257,7 +3257,7 @@
         <v>30.49</v>
       </c>
       <c r="AZ12" t="n">
-        <v>6.68</v>
+        <v>6.61</v>
       </c>
       <c r="BA12" t="n">
         <v>4.41</v>
@@ -3266,19 +3266,19 @@
         <v>18.12</v>
       </c>
       <c r="BC12" t="n">
-        <v>656.02</v>
+        <v>663.75</v>
       </c>
       <c r="BD12" t="n">
-        <v>517.29</v>
+        <v>523.6</v>
       </c>
       <c r="BE12" t="n">
         <v>35.17</v>
       </c>
       <c r="BF12" t="n">
-        <v>-10.7</v>
+        <v>-9.779999999999999</v>
       </c>
       <c r="BG12" t="n">
-        <v>266.78</v>
+        <v>270.53</v>
       </c>
       <c r="BH12" t="n">
         <v>16.4</v>
@@ -3287,7 +3287,7 @@
         <v>0</v>
       </c>
       <c r="BJ12" t="n">
-        <v>4.94</v>
+        <v>4.89</v>
       </c>
       <c r="BK12" t="n">
         <v>3.78</v>
@@ -3296,7 +3296,7 @@
         <v>3.43</v>
       </c>
       <c r="BM12" t="n">
-        <v>5</v>
+        <v>4.96</v>
       </c>
       <c r="BN12" t="n">
         <v>8.23</v>
@@ -3305,19 +3305,19 @@
         <v>4.42</v>
       </c>
       <c r="BP12" t="n">
-        <v>4.92</v>
+        <v>4.84</v>
       </c>
       <c r="BQ12" t="n">
-        <v>1.44</v>
+        <v>1.43</v>
       </c>
       <c r="BR12" t="n">
-        <v>4.96</v>
+        <v>4.95</v>
       </c>
       <c r="BS12" t="n">
         <v>0.09</v>
       </c>
       <c r="BT12" t="n">
-        <v>525237</v>
+        <v>521930</v>
       </c>
     </row>
     <row r="13">
@@ -3347,13 +3347,13 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>29.34</v>
+        <v>29.12</v>
       </c>
       <c r="G13" t="n">
-        <v>14792955214</v>
+        <v>14682036519</v>
       </c>
       <c r="H13" t="n">
-        <v>2837400</v>
+        <v>3664800</v>
       </c>
       <c r="I13" t="n">
         <v>504190947</v>
@@ -3368,7 +3368,7 @@
         <v>1.13</v>
       </c>
       <c r="M13" t="n">
-        <v>5.11625914148216</v>
+        <v>5.077897044183444</v>
       </c>
       <c r="N13" t="n">
         <v>0.57</v>
@@ -3446,7 +3446,7 @@
         <v>932753251.95</v>
       </c>
       <c r="AM13" t="n">
-        <v>1539329366.701353</v>
+        <v>1527787358.896982</v>
       </c>
       <c r="AN13" t="n">
         <v>2.6301</v>
@@ -3487,7 +3487,7 @@
         <v>26.6</v>
       </c>
       <c r="AZ13" t="n">
-        <v>53.11</v>
+        <v>52.71</v>
       </c>
       <c r="BA13" t="n">
         <v>2.6</v>
@@ -3496,19 +3496,19 @@
         <v>8.69</v>
       </c>
       <c r="BC13" t="n">
-        <v>11.02</v>
+        <v>11.86</v>
       </c>
       <c r="BD13" t="n">
-        <v>-9.35</v>
+        <v>-8.67</v>
       </c>
       <c r="BE13" t="n">
         <v>81</v>
       </c>
       <c r="BF13" t="n">
-        <v>-91.12</v>
+        <v>-91.06</v>
       </c>
       <c r="BG13" t="n">
-        <v>-70.37</v>
+        <v>-70.14</v>
       </c>
       <c r="BH13" t="n">
         <v>25.49</v>
@@ -3517,7 +3517,7 @@
         <v>0</v>
       </c>
       <c r="BJ13" t="n">
-        <v>29.34</v>
+        <v>29.12</v>
       </c>
       <c r="BK13" t="n">
         <v>1.85</v>
@@ -3526,7 +3526,7 @@
         <v>1.96</v>
       </c>
       <c r="BM13" t="n">
-        <v>29.7</v>
+        <v>29.49</v>
       </c>
       <c r="BN13" t="n">
         <v>32.11</v>
@@ -3535,19 +3535,19 @@
         <v>20.85</v>
       </c>
       <c r="BP13" t="n">
-        <v>29.06</v>
+        <v>28.87</v>
       </c>
       <c r="BQ13" t="n">
-        <v>14.99</v>
+        <v>14.88</v>
       </c>
       <c r="BR13" t="n">
-        <v>29.15</v>
+        <v>29.49</v>
       </c>
       <c r="BS13" t="n">
         <v>5.01</v>
       </c>
       <c r="BT13" t="n">
-        <v>5061107</v>
+        <v>4984300</v>
       </c>
     </row>
     <row r="14">
@@ -3577,13 +3577,13 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>10.19</v>
+        <v>10.18</v>
       </c>
       <c r="G14" t="n">
-        <v>7877048150</v>
+        <v>8047950317</v>
       </c>
       <c r="H14" t="n">
-        <v>9500</v>
+        <v>2800</v>
       </c>
       <c r="I14" t="n">
         <v>339510689</v>
@@ -3598,7 +3598,7 @@
         <v>1.92</v>
       </c>
       <c r="M14" t="n">
-        <v>3.27069042754971</v>
+        <v>3.341652045532762</v>
       </c>
       <c r="N14" t="n">
         <v>1.11</v>
@@ -3676,7 +3676,7 @@
         <v>349696009.67</v>
       </c>
       <c r="AM14" t="n">
-        <v>874256176.4705882</v>
+        <v>893224230.5216427</v>
       </c>
       <c r="AN14" t="n">
         <v>0.1489</v>
@@ -3717,7 +3717,7 @@
         <v>9.050000000000001</v>
       </c>
       <c r="AZ14" t="n">
-        <v>8.19</v>
+        <v>8.18</v>
       </c>
       <c r="BA14" t="n">
         <v>1.42</v>
@@ -3726,19 +3726,19 @@
         <v>5.94</v>
       </c>
       <c r="BC14" t="n">
-        <v>8.76</v>
+        <v>8.869999999999999</v>
       </c>
       <c r="BD14" t="n">
-        <v>-11.2</v>
+        <v>-11.11</v>
       </c>
       <c r="BE14" t="n">
         <v>-19.67</v>
       </c>
       <c r="BF14" t="n">
-        <v>-86.05</v>
+        <v>-86.04000000000001</v>
       </c>
       <c r="BG14" t="n">
-        <v>-41.69</v>
+        <v>-41.63</v>
       </c>
       <c r="BH14" t="n">
         <v>5.3</v>
@@ -3747,7 +3747,7 @@
         <v>0</v>
       </c>
       <c r="BJ14" t="n">
-        <v>10.19</v>
+        <v>10.18</v>
       </c>
       <c r="BK14" t="n">
         <v>1.03</v>
@@ -3756,7 +3756,7 @@
         <v>1.01</v>
       </c>
       <c r="BM14" t="n">
-        <v>10.19</v>
+        <v>10.18</v>
       </c>
       <c r="BN14" t="n">
         <v>13.49</v>
@@ -3765,19 +3765,19 @@
         <v>7.65</v>
       </c>
       <c r="BP14" t="n">
-        <v>9.880000000000001</v>
+        <v>9.93</v>
       </c>
       <c r="BQ14" t="n">
-        <v>10.06</v>
+        <v>10.05</v>
       </c>
       <c r="BR14" t="n">
-        <v>9.93</v>
+        <v>9.960000000000001</v>
       </c>
       <c r="BS14" t="n">
         <v>1.44</v>
       </c>
       <c r="BT14" t="n">
-        <v>10950</v>
+        <v>11173</v>
       </c>
     </row>
     <row r="15">
@@ -3807,13 +3807,13 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>13.25</v>
+        <v>13.31</v>
       </c>
       <c r="G15" t="n">
-        <v>7877048150</v>
+        <v>8047950317</v>
       </c>
       <c r="H15" t="n">
-        <v>1438400</v>
+        <v>814300</v>
       </c>
       <c r="I15" t="n">
         <v>343551533</v>
@@ -3828,7 +3828,7 @@
         <v>2.56</v>
       </c>
       <c r="M15" t="n">
-        <v>3.232220653671503</v>
+        <v>3.302347622989903</v>
       </c>
       <c r="N15" t="n">
         <v>1.47</v>
@@ -3906,7 +3906,7 @@
         <v>353858078.99</v>
       </c>
       <c r="AM15" t="n">
-        <v>656968152.6271893</v>
+        <v>671221877.9816513</v>
       </c>
       <c r="AN15" t="n">
         <v>0.1638</v>
@@ -3947,7 +3947,7 @@
         <v>9.050000000000001</v>
       </c>
       <c r="AZ15" t="n">
-        <v>8.81</v>
+        <v>8.85</v>
       </c>
       <c r="BA15" t="n">
         <v>1.42</v>
@@ -3956,19 +3956,19 @@
         <v>6.19</v>
       </c>
       <c r="BC15" t="n">
-        <v>-16.36</v>
+        <v>-16.73</v>
       </c>
       <c r="BD15" t="n">
-        <v>-31.71</v>
+        <v>-32.01</v>
       </c>
       <c r="BE15" t="n">
         <v>-33.5</v>
       </c>
       <c r="BF15" t="n">
-        <v>-89.27</v>
+        <v>-89.31999999999999</v>
       </c>
       <c r="BG15" t="n">
-        <v>-53.3</v>
+        <v>-53.51</v>
       </c>
       <c r="BH15" t="n">
         <v>5.3</v>
@@ -3977,7 +3977,7 @@
         <v>0</v>
       </c>
       <c r="BJ15" t="n">
-        <v>13.25</v>
+        <v>13.31</v>
       </c>
       <c r="BK15" t="n">
         <v>1.03</v>
@@ -3986,7 +3986,7 @@
         <v>1.01</v>
       </c>
       <c r="BM15" t="n">
-        <v>13.91</v>
+        <v>13.5</v>
       </c>
       <c r="BN15" t="n">
         <v>16.22</v>
@@ -3995,19 +3995,19 @@
         <v>7.84</v>
       </c>
       <c r="BP15" t="n">
-        <v>13.18</v>
+        <v>13.13</v>
       </c>
       <c r="BQ15" t="n">
-        <v>13.08</v>
+        <v>13.14</v>
       </c>
       <c r="BR15" t="n">
-        <v>13.7</v>
+        <v>13.19</v>
       </c>
       <c r="BS15" t="n">
         <v>1.92</v>
       </c>
       <c r="BT15" t="n">
-        <v>2374237</v>
+        <v>2361077</v>
       </c>
     </row>
     <row r="16">
@@ -4037,13 +4037,13 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>4.49</v>
+        <v>4.38</v>
       </c>
       <c r="G16" t="n">
-        <v>984682542</v>
+        <v>960558991</v>
       </c>
       <c r="H16" t="n">
-        <v>86400</v>
+        <v>66600</v>
       </c>
       <c r="I16" t="n">
         <v>219305733</v>
@@ -4058,7 +4058,7 @@
         <v>2.69</v>
       </c>
       <c r="M16" t="n">
-        <v>0.46583740577589</v>
+        <v>0.4544249434475568</v>
       </c>
       <c r="N16" t="n">
         <v>0.39</v>
@@ -4136,7 +4136,7 @@
         <v>17544458.64</v>
       </c>
       <c r="AM16" t="n">
-        <v>276596219.6629214</v>
+        <v>269819941.2921348</v>
       </c>
       <c r="AN16" t="n">
         <v>0.0077</v>
@@ -4177,7 +4177,7 @@
         <v>1.42</v>
       </c>
       <c r="AZ16" t="n">
-        <v>0.13</v>
+        <v>0.12</v>
       </c>
       <c r="BA16" t="n">
         <v>0.08</v>
@@ -4186,16 +4186,16 @@
         <v>0</v>
       </c>
       <c r="BC16" t="n">
-        <v>-61.27</v>
+        <v>-60.3</v>
       </c>
       <c r="BD16" t="n">
-        <v>-68.38</v>
+        <v>-67.58</v>
       </c>
       <c r="BE16" t="n">
         <v>-97.17</v>
       </c>
       <c r="BF16" t="n">
-        <v>-98.22</v>
+        <v>-98.17</v>
       </c>
       <c r="BG16" t="n">
         <v>-100</v>
@@ -4207,7 +4207,7 @@
         <v>0</v>
       </c>
       <c r="BJ16" t="n">
-        <v>4.49</v>
+        <v>4.38</v>
       </c>
       <c r="BK16" t="n">
         <v>0.08</v>
@@ -4216,7 +4216,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="BM16" t="n">
-        <v>4.5</v>
+        <v>4.49</v>
       </c>
       <c r="BN16" t="n">
         <v>5.54</v>
@@ -4225,19 +4225,19 @@
         <v>3.22</v>
       </c>
       <c r="BP16" t="n">
-        <v>4.37</v>
+        <v>4.35</v>
       </c>
       <c r="BQ16" t="n">
-        <v>61.27</v>
+        <v>59.77</v>
       </c>
       <c r="BR16" t="n">
-        <v>4.39</v>
+        <v>4.49</v>
       </c>
       <c r="BS16" t="n">
         <v>0.49</v>
       </c>
       <c r="BT16" t="n">
-        <v>138393</v>
+        <v>136167</v>
       </c>
     </row>
     <row r="17">
@@ -4267,13 +4267,13 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>32.25</v>
+        <v>32.05</v>
       </c>
       <c r="G17" t="n">
-        <v>10630467525</v>
+        <v>10564541893</v>
       </c>
       <c r="H17" t="n">
-        <v>1066400</v>
+        <v>1269000</v>
       </c>
       <c r="I17" t="n">
         <v>0</v>
@@ -4360,13 +4360,13 @@
         <v>8.039999999999999</v>
       </c>
       <c r="AK17" t="n">
-        <v>4800608528.269508</v>
+        <v>4770837198.78974</v>
       </c>
       <c r="AL17" t="n">
-        <v>1328808440.625</v>
+        <v>1320567736.625</v>
       </c>
       <c r="AM17" t="n">
-        <v>3291166416.408669</v>
+        <v>3270756004.024768</v>
       </c>
       <c r="AN17" t="n">
         <v>1.08</v>
@@ -4407,7 +4407,7 @@
         <v>42.98</v>
       </c>
       <c r="AZ17" t="n">
-        <v>17.25</v>
+        <v>17.15</v>
       </c>
       <c r="BA17" t="n">
         <v>4.55</v>
@@ -4416,19 +4416,19 @@
         <v>16.33</v>
       </c>
       <c r="BC17" t="n">
-        <v>63.22</v>
+        <v>64.23999999999999</v>
       </c>
       <c r="BD17" t="n">
-        <v>33.27</v>
+        <v>34.1</v>
       </c>
       <c r="BE17" t="n">
         <v>-46.5</v>
       </c>
       <c r="BF17" t="n">
-        <v>-85.90000000000001</v>
+        <v>-85.81</v>
       </c>
       <c r="BG17" t="n">
-        <v>-49.35</v>
+        <v>-49.04</v>
       </c>
       <c r="BH17" t="n">
         <v>29.25</v>
@@ -4437,7 +4437,7 @@
         <v>0</v>
       </c>
       <c r="BJ17" t="n">
-        <v>32.25</v>
+        <v>32.05</v>
       </c>
       <c r="BK17" t="n">
         <v>4.21</v>
@@ -4446,7 +4446,7 @@
         <v>12.62</v>
       </c>
       <c r="BM17" t="n">
-        <v>32.59</v>
+        <v>32.29</v>
       </c>
       <c r="BN17" t="n">
         <v>36.63</v>
@@ -4455,19 +4455,19 @@
         <v>29.53</v>
       </c>
       <c r="BP17" t="n">
-        <v>31.96</v>
+        <v>31.63</v>
       </c>
       <c r="BQ17" t="n">
-        <v>2.56</v>
+        <v>2.54</v>
       </c>
       <c r="BR17" t="n">
-        <v>32.3</v>
+        <v>32.29</v>
       </c>
       <c r="BS17" t="n">
         <v>2.21</v>
       </c>
       <c r="BT17" t="n">
-        <v>1170310</v>
+        <v>1176323</v>
       </c>
     </row>
     <row r="18">
@@ -4497,13 +4497,13 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>11.09</v>
+        <v>10.98</v>
       </c>
       <c r="G18" t="n">
-        <v>10630467525</v>
+        <v>10564541893</v>
       </c>
       <c r="H18" t="n">
-        <v>15500</v>
+        <v>17700</v>
       </c>
       <c r="I18" t="n">
         <v>671494278</v>
@@ -4518,7 +4518,7 @@
         <v>1.2</v>
       </c>
       <c r="M18" t="n">
-        <v>3.130027108755625</v>
+        <v>3.110616013727436</v>
       </c>
       <c r="N18" t="n">
         <v>0.33</v>
@@ -4596,7 +4596,7 @@
         <v>940091989.1999999</v>
       </c>
       <c r="AM18" t="n">
-        <v>3163829620.535715</v>
+        <v>3144208896.726191</v>
       </c>
       <c r="AN18" t="n">
         <v>0.36</v>
@@ -4637,7 +4637,7 @@
         <v>14.31</v>
       </c>
       <c r="AZ18" t="n">
-        <v>5.71</v>
+        <v>5.65</v>
       </c>
       <c r="BA18" t="n">
         <v>1.51</v>
@@ -4646,19 +4646,19 @@
         <v>5.44</v>
       </c>
       <c r="BC18" t="n">
-        <v>58.03</v>
+        <v>59.61</v>
       </c>
       <c r="BD18" t="n">
-        <v>29.03</v>
+        <v>30.32</v>
       </c>
       <c r="BE18" t="n">
         <v>-48.5</v>
       </c>
       <c r="BF18" t="n">
-        <v>-86.36</v>
+        <v>-86.22</v>
       </c>
       <c r="BG18" t="n">
-        <v>-50.91</v>
+        <v>-50.41</v>
       </c>
       <c r="BH18" t="n">
         <v>9.75</v>
@@ -4667,7 +4667,7 @@
         <v>0</v>
       </c>
       <c r="BJ18" t="n">
-        <v>11.09</v>
+        <v>10.98</v>
       </c>
       <c r="BK18" t="n">
         <v>1.4</v>
@@ -4676,7 +4676,7 @@
         <v>12.62</v>
       </c>
       <c r="BM18" t="n">
-        <v>11.91</v>
+        <v>11.07</v>
       </c>
       <c r="BN18" t="n">
         <v>13.82</v>
@@ -4685,10 +4685,10 @@
         <v>10.19</v>
       </c>
       <c r="BP18" t="n">
-        <v>11</v>
+        <v>10.9</v>
       </c>
       <c r="BQ18" t="n">
-        <v>0.88</v>
+        <v>0.87</v>
       </c>
       <c r="BR18" t="n">
         <v>11.04</v>
@@ -4697,7 +4697,7 @@
         <v>2.3</v>
       </c>
       <c r="BT18" t="n">
-        <v>9693</v>
+        <v>10050</v>
       </c>
     </row>
     <row r="19">
@@ -4727,13 +4727,13 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>10.79</v>
+        <v>10.4</v>
       </c>
       <c r="G19" t="n">
-        <v>10630467525</v>
+        <v>10564541893</v>
       </c>
       <c r="H19" t="n">
-        <v>15000</v>
+        <v>34300</v>
       </c>
       <c r="I19" t="n">
         <v>317386323</v>
@@ -4748,7 +4748,7 @@
         <v>1.12</v>
       </c>
       <c r="M19" t="n">
-        <v>6.622198693528095</v>
+        <v>6.581130637671312</v>
       </c>
       <c r="N19" t="n">
         <v>0.3</v>
@@ -4826,7 +4826,7 @@
         <v>444340852.2</v>
       </c>
       <c r="AM19" t="n">
-        <v>3374751595.238095</v>
+        <v>3353822823.174603</v>
       </c>
       <c r="AN19" t="n">
         <v>0.36</v>
@@ -4867,7 +4867,7 @@
         <v>14.31</v>
       </c>
       <c r="AZ19" t="n">
-        <v>5.93</v>
+        <v>5.72</v>
       </c>
       <c r="BA19" t="n">
         <v>1.51</v>
@@ -4876,19 +4876,19 @@
         <v>5.25</v>
       </c>
       <c r="BC19" t="n">
-        <v>62.42</v>
+        <v>68.51000000000001</v>
       </c>
       <c r="BD19" t="n">
-        <v>32.61</v>
+        <v>37.59</v>
       </c>
       <c r="BE19" t="n">
         <v>-45</v>
       </c>
       <c r="BF19" t="n">
-        <v>-85.98</v>
+        <v>-85.45999999999999</v>
       </c>
       <c r="BG19" t="n">
-        <v>-51.34</v>
+        <v>-49.52</v>
       </c>
       <c r="BH19" t="n">
         <v>9.75</v>
@@ -4897,7 +4897,7 @@
         <v>0</v>
       </c>
       <c r="BJ19" t="n">
-        <v>10.79</v>
+        <v>10.4</v>
       </c>
       <c r="BK19" t="n">
         <v>1.4</v>
@@ -4906,7 +4906,7 @@
         <v>12.62</v>
       </c>
       <c r="BM19" t="n">
-        <v>10.79</v>
+        <v>10.62</v>
       </c>
       <c r="BN19" t="n">
         <v>11.41</v>
@@ -4915,19 +4915,19 @@
         <v>9.19</v>
       </c>
       <c r="BP19" t="n">
-        <v>10.51</v>
+        <v>10.38</v>
       </c>
       <c r="BQ19" t="n">
-        <v>0.85</v>
+        <v>0.82</v>
       </c>
       <c r="BR19" t="n">
-        <v>10.66</v>
+        <v>10.58</v>
       </c>
       <c r="BS19" t="n">
         <v>2.16</v>
       </c>
       <c r="BT19" t="n">
-        <v>12713</v>
+        <v>12600</v>
       </c>
     </row>
     <row r="20">
@@ -5417,13 +5417,13 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>5.15</v>
+        <v>5.25</v>
       </c>
       <c r="G22" t="n">
-        <v>1031263314</v>
+        <v>1051287300</v>
       </c>
       <c r="H22" t="n">
-        <v>823100</v>
+        <v>1959500</v>
       </c>
       <c r="I22" t="n">
         <v>200245299</v>
@@ -5438,7 +5438,7 @@
         <v>0.27</v>
       </c>
       <c r="M22" t="n">
-        <v>0.08746825601657506</v>
+        <v>0.08916662258323478</v>
       </c>
       <c r="N22" t="n">
         <v>0.08</v>
@@ -5516,7 +5516,7 @@
         <v>378463615.11</v>
       </c>
       <c r="AM22" t="n">
-        <v>233846556.462585</v>
+        <v>238387142.8571428</v>
       </c>
       <c r="AN22" t="n">
         <v>0</v>
@@ -5566,19 +5566,19 @@
         <v>172.49</v>
       </c>
       <c r="BC22" t="n">
-        <v>476.8</v>
+        <v>465.81</v>
       </c>
       <c r="BD22" t="n">
-        <v>370.95</v>
+        <v>361.98</v>
       </c>
       <c r="BE22" t="n">
         <v>-100</v>
       </c>
       <c r="BF22" t="n">
-        <v>-63.3</v>
+        <v>-64</v>
       </c>
       <c r="BG22" t="n">
-        <v>3249.31</v>
+        <v>3185.52</v>
       </c>
       <c r="BH22" t="n">
         <v>20.75</v>
@@ -5587,7 +5587,7 @@
         <v>0</v>
       </c>
       <c r="BJ22" t="n">
-        <v>5.15</v>
+        <v>5.25</v>
       </c>
       <c r="BK22" t="n">
         <v>1.89</v>
@@ -5596,7 +5596,7 @@
         <v>0.67</v>
       </c>
       <c r="BM22" t="n">
-        <v>5.32</v>
+        <v>5.34</v>
       </c>
       <c r="BN22" t="n">
         <v>7.89</v>
@@ -5605,19 +5605,19 @@
         <v>3.37</v>
       </c>
       <c r="BP22" t="n">
-        <v>5.06</v>
+        <v>4.87</v>
       </c>
       <c r="BQ22" t="n">
-        <v>7.67</v>
+        <v>7.82</v>
       </c>
       <c r="BR22" t="n">
-        <v>5.08</v>
+        <v>5.13</v>
       </c>
       <c r="BS22" t="n">
         <v>0.09</v>
       </c>
       <c r="BT22" t="n">
-        <v>1522243</v>
+        <v>1501080</v>
       </c>
     </row>
     <row r="23">
@@ -5877,13 +5877,13 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.99</v>
+        <v>3</v>
       </c>
       <c r="G24" t="n">
-        <v>1207567117</v>
+        <v>1211606400</v>
       </c>
       <c r="H24" t="n">
-        <v>3723300</v>
+        <v>5591000</v>
       </c>
       <c r="I24" t="n">
         <v>403868805</v>
@@ -5898,7 +5898,7 @@
         <v>0.49</v>
       </c>
       <c r="M24" t="n">
-        <v>0.2919182736028141</v>
+        <v>0.2928947332159929</v>
       </c>
       <c r="N24" t="n">
         <v>0.11</v>
@@ -5976,7 +5976,7 @@
         <v>153470145.9</v>
       </c>
       <c r="AM24" t="n">
-        <v>1087898303.603604</v>
+        <v>1091537297.297297</v>
       </c>
       <c r="AN24" t="n">
         <v>0.0813</v>
@@ -6026,19 +6026,19 @@
         <v>1.46</v>
       </c>
       <c r="BC24" t="n">
-        <v>139.35</v>
+        <v>138.55</v>
       </c>
       <c r="BD24" t="n">
-        <v>95.42</v>
+        <v>94.77</v>
       </c>
       <c r="BE24" t="n">
         <v>-53.83</v>
       </c>
       <c r="BF24" t="n">
-        <v>-87.29000000000001</v>
+        <v>-87.33</v>
       </c>
       <c r="BG24" t="n">
-        <v>-51.24</v>
+        <v>-51.41</v>
       </c>
       <c r="BH24" t="n">
         <v>5.99</v>
@@ -6047,7 +6047,7 @@
         <v>0</v>
       </c>
       <c r="BJ24" t="n">
-        <v>2.99</v>
+        <v>3</v>
       </c>
       <c r="BK24" t="n">
         <v>0.38</v>
@@ -6056,7 +6056,7 @@
         <v>0.41</v>
       </c>
       <c r="BM24" t="n">
-        <v>3.07</v>
+        <v>3.05</v>
       </c>
       <c r="BN24" t="n">
         <v>5.29</v>
@@ -6065,19 +6065,19 @@
         <v>1.92</v>
       </c>
       <c r="BP24" t="n">
-        <v>2.95</v>
+        <v>2.92</v>
       </c>
       <c r="BQ24" t="n">
-        <v>7.34</v>
+        <v>7.37</v>
       </c>
       <c r="BR24" t="n">
-        <v>2.96</v>
+        <v>3.01</v>
       </c>
       <c r="BS24" t="n">
         <v>0.29</v>
       </c>
       <c r="BT24" t="n">
-        <v>8138913</v>
+        <v>7900803</v>
       </c>
     </row>
     <row r="25">
@@ -6107,13 +6107,13 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>4.49</v>
+        <v>4.67</v>
       </c>
       <c r="G25" t="n">
-        <v>1555757980</v>
+        <v>1618127940</v>
       </c>
       <c r="H25" t="n">
-        <v>873100</v>
+        <v>1032900</v>
       </c>
       <c r="I25" t="n">
         <v>346494097</v>
@@ -6128,7 +6128,7 @@
         <v>0.97</v>
       </c>
       <c r="M25" t="n">
-        <v>0.7757719651554249</v>
+        <v>0.8068724750405584</v>
       </c>
       <c r="N25" t="n">
         <v>0.22</v>
@@ -6206,7 +6206,7 @@
         <v>62368937.46</v>
       </c>
       <c r="AM25" t="n">
-        <v>571969845.5882353</v>
+        <v>594899977.9411764</v>
       </c>
       <c r="AN25" t="n">
         <v>0.4742</v>
@@ -6247,7 +6247,7 @@
         <v>3.27</v>
       </c>
       <c r="AZ25" t="n">
-        <v>10.46</v>
+        <v>10.88</v>
       </c>
       <c r="BA25" t="n">
         <v>0.23</v>
@@ -6256,19 +6256,19 @@
         <v>2.2</v>
       </c>
       <c r="BC25" t="n">
-        <v>-10.69</v>
+        <v>-14.14</v>
       </c>
       <c r="BD25" t="n">
-        <v>-27.08</v>
+        <v>-29.89</v>
       </c>
       <c r="BE25" t="n">
         <v>133</v>
       </c>
       <c r="BF25" t="n">
-        <v>-94.84</v>
+        <v>-95.04000000000001</v>
       </c>
       <c r="BG25" t="n">
-        <v>-51.01</v>
+        <v>-52.9</v>
       </c>
       <c r="BH25" t="n">
         <v>3.97</v>
@@ -6277,7 +6277,7 @@
         <v>0</v>
       </c>
       <c r="BJ25" t="n">
-        <v>4.49</v>
+        <v>4.67</v>
       </c>
       <c r="BK25" t="n">
         <v>0.18</v>
@@ -6286,7 +6286,7 @@
         <v>0.24</v>
       </c>
       <c r="BM25" t="n">
-        <v>4.75</v>
+        <v>4.67</v>
       </c>
       <c r="BN25" t="n">
         <v>6.3</v>
@@ -6295,19 +6295,19 @@
         <v>2.64</v>
       </c>
       <c r="BP25" t="n">
-        <v>4.46</v>
+        <v>4.45</v>
       </c>
       <c r="BQ25" t="n">
-        <v>18.97</v>
+        <v>19.73</v>
       </c>
       <c r="BR25" t="n">
-        <v>4.51</v>
+        <v>4.45</v>
       </c>
       <c r="BS25" t="n">
         <v>0.67</v>
       </c>
       <c r="BT25" t="n">
-        <v>1261540</v>
+        <v>1257897</v>
       </c>
     </row>
     <row r="26">
@@ -6337,13 +6337,13 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>10.29</v>
+        <v>10.24</v>
       </c>
       <c r="G26" t="n">
-        <v>13936703918</v>
+        <v>13868984010</v>
       </c>
       <c r="H26" t="n">
-        <v>18073500</v>
+        <v>8212300</v>
       </c>
       <c r="I26" t="n">
         <v>1354393401</v>
@@ -6358,7 +6358,7 @@
         <v>1.94</v>
       </c>
       <c r="M26" t="n">
-        <v>0.1797126221776407</v>
+        <v>0.1788393796726758</v>
       </c>
       <c r="N26" t="n">
         <v>0.26</v>
@@ -6436,7 +6436,7 @@
         <v>961619314.7099999</v>
       </c>
       <c r="AM26" t="n">
-        <v>4977394256.428572</v>
+        <v>4953208575</v>
       </c>
       <c r="AN26" t="n">
         <v>0.1043</v>
@@ -6477,7 +6477,7 @@
         <v>7.07</v>
       </c>
       <c r="AZ26" t="n">
-        <v>1.97</v>
+        <v>1.96</v>
       </c>
       <c r="BA26" t="n">
         <v>0.66</v>
@@ -6486,19 +6486,19 @@
         <v>1.19</v>
       </c>
       <c r="BC26" t="n">
-        <v>-15.88</v>
+        <v>-15.47</v>
       </c>
       <c r="BD26" t="n">
-        <v>-31.32</v>
+        <v>-30.98</v>
       </c>
       <c r="BE26" t="n">
         <v>-80.83</v>
       </c>
       <c r="BF26" t="n">
-        <v>-93.59</v>
+        <v>-93.56</v>
       </c>
       <c r="BG26" t="n">
-        <v>-88.40000000000001</v>
+        <v>-88.34999999999999</v>
       </c>
       <c r="BH26" t="n">
         <v>4.69</v>
@@ -6507,7 +6507,7 @@
         <v>0</v>
       </c>
       <c r="BJ26" t="n">
-        <v>10.29</v>
+        <v>10.24</v>
       </c>
       <c r="BK26" t="n">
         <v>0.71</v>
@@ -6516,7 +6516,7 @@
         <v>0.72</v>
       </c>
       <c r="BM26" t="n">
-        <v>10.55</v>
+        <v>10.4</v>
       </c>
       <c r="BN26" t="n">
         <v>10.55</v>
@@ -6528,16 +6528,16 @@
         <v>10.16</v>
       </c>
       <c r="BQ26" t="n">
-        <v>14.35</v>
+        <v>14.28</v>
       </c>
       <c r="BR26" t="n">
-        <v>10.19</v>
+        <v>10.35</v>
       </c>
       <c r="BS26" t="n">
         <v>0.16</v>
       </c>
       <c r="BT26" t="n">
-        <v>11997927</v>
+        <v>12125420</v>
       </c>
     </row>
     <row r="27">
@@ -8165,13 +8165,13 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>14.9</v>
+        <v>14.5</v>
       </c>
       <c r="G34" t="n">
-        <v>3076696451</v>
+        <v>2994100650</v>
       </c>
       <c r="H34" t="n">
-        <v>2532500</v>
+        <v>2993900</v>
       </c>
       <c r="I34" t="n">
         <v>206489813</v>
@@ -8186,7 +8186,7 @@
         <v>0.45</v>
       </c>
       <c r="M34" t="n">
-        <v>0.2704775520444521</v>
+        <v>0.2632164164662674</v>
       </c>
       <c r="N34" t="n">
         <v>0.24</v>
@@ -8264,7 +8264,7 @@
         <v>324189006.41</v>
       </c>
       <c r="AM34" t="n">
-        <v>639645831.8087319</v>
+        <v>622474147.6091477</v>
       </c>
       <c r="AN34" t="n">
         <v>0</v>
@@ -8305,7 +8305,7 @@
         <v>30.28</v>
       </c>
       <c r="AZ34" t="n">
-        <v>34.77</v>
+        <v>33.83</v>
       </c>
       <c r="BA34" t="n">
         <v>2.29</v>
@@ -8314,19 +8314,19 @@
         <v>25.26</v>
       </c>
       <c r="BC34" t="n">
-        <v>148.92</v>
+        <v>155.78</v>
       </c>
       <c r="BD34" t="n">
-        <v>103.24</v>
+        <v>108.85</v>
       </c>
       <c r="BE34" t="n">
         <v>133.33</v>
       </c>
       <c r="BF34" t="n">
-        <v>-84.59999999999999</v>
+        <v>-84.17</v>
       </c>
       <c r="BG34" t="n">
-        <v>69.52</v>
+        <v>74.19</v>
       </c>
       <c r="BH34" t="n">
         <v>38.94</v>
@@ -8335,7 +8335,7 @@
         <v>0</v>
       </c>
       <c r="BJ34" t="n">
-        <v>14.9</v>
+        <v>14.5</v>
       </c>
       <c r="BK34" t="n">
         <v>1.57</v>
@@ -8344,28 +8344,28 @@
         <v>1.58</v>
       </c>
       <c r="BM34" t="n">
-        <v>15.41</v>
+        <v>14.94</v>
       </c>
       <c r="BN34" t="n">
-        <v>29.39</v>
+        <v>28.86</v>
       </c>
       <c r="BO34" t="n">
         <v>14.3</v>
       </c>
       <c r="BP34" t="n">
-        <v>14.58</v>
+        <v>14.41</v>
       </c>
       <c r="BQ34" t="n">
-        <v>9.449999999999999</v>
+        <v>9.19</v>
       </c>
       <c r="BR34" t="n">
-        <v>14.7</v>
+        <v>14.93</v>
       </c>
       <c r="BS34" t="n">
         <v>0.32</v>
       </c>
       <c r="BT34" t="n">
-        <v>3144380</v>
+        <v>3185590</v>
       </c>
     </row>
     <row r="35">
@@ -8395,13 +8395,13 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>18.04</v>
+        <v>17.82</v>
       </c>
       <c r="G35" t="n">
-        <v>91038846580</v>
+        <v>89928628459</v>
       </c>
       <c r="H35" t="n">
-        <v>46402400</v>
+        <v>43921400</v>
       </c>
       <c r="I35" t="n">
         <v>5046500000</v>
@@ -8416,7 +8416,7 @@
         <v>4.69</v>
       </c>
       <c r="M35" t="n">
-        <v>7.55807813114974</v>
+        <v>7.46590741923543</v>
       </c>
       <c r="N35" t="n">
         <v>1.79</v>
@@ -8494,7 +8494,7 @@
         <v>5349290000</v>
       </c>
       <c r="AM35" t="n">
-        <v>7523871618.181818</v>
+        <v>7432118054.462811</v>
       </c>
       <c r="AN35" t="n">
         <v>0.5305</v>
@@ -8535,7 +8535,7 @@
         <v>7.68</v>
       </c>
       <c r="AZ35" t="n">
-        <v>10.52</v>
+        <v>10.4</v>
       </c>
       <c r="BA35" t="n">
         <v>1.11</v>
@@ -8544,19 +8544,19 @@
         <v>9.119999999999999</v>
       </c>
       <c r="BC35" t="n">
-        <v>-47.86</v>
+        <v>-47.21</v>
       </c>
       <c r="BD35" t="n">
-        <v>-57.43</v>
+        <v>-56.9</v>
       </c>
       <c r="BE35" t="n">
         <v>-41.67</v>
       </c>
       <c r="BF35" t="n">
-        <v>-93.81999999999999</v>
+        <v>-93.75</v>
       </c>
       <c r="BG35" t="n">
-        <v>-49.46</v>
+        <v>-48.84</v>
       </c>
       <c r="BH35" t="n">
         <v>3.71</v>
@@ -8565,7 +8565,7 @@
         <v>0</v>
       </c>
       <c r="BJ35" t="n">
-        <v>18.04</v>
+        <v>17.82</v>
       </c>
       <c r="BK35" t="n">
         <v>1.06</v>
@@ -8574,7 +8574,7 @@
         <v>1.04</v>
       </c>
       <c r="BM35" t="n">
-        <v>18.49</v>
+        <v>18.09</v>
       </c>
       <c r="BN35" t="n">
         <v>20.08</v>
@@ -8583,19 +8583,19 @@
         <v>11.7</v>
       </c>
       <c r="BP35" t="n">
-        <v>17.97</v>
+        <v>17.7</v>
       </c>
       <c r="BQ35" t="n">
-        <v>17.26</v>
+        <v>17.05</v>
       </c>
       <c r="BR35" t="n">
-        <v>18.04</v>
+        <v>18</v>
       </c>
       <c r="BS35" t="n">
         <v>7.3</v>
       </c>
       <c r="BT35" t="n">
-        <v>41082773</v>
+        <v>41235613</v>
       </c>
     </row>
     <row r="36">
@@ -8855,13 +8855,13 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>15</v>
+        <v>14.95</v>
       </c>
       <c r="G37" t="n">
-        <v>202125000</v>
+        <v>199741864</v>
       </c>
       <c r="H37" t="n">
-        <v>500</v>
+        <v>200</v>
       </c>
       <c r="I37" t="n">
         <v>4900000</v>
@@ -8876,7 +8876,7 @@
         <v>0.88</v>
       </c>
       <c r="M37" t="n">
-        <v>1.967857142857143</v>
+        <v>1.94465530636982</v>
       </c>
       <c r="N37" t="n">
         <v>0.5</v>
@@ -8954,7 +8954,7 @@
         <v>11319000</v>
       </c>
       <c r="AM37" t="n">
-        <v>48355263.15789474</v>
+        <v>47785134.92822967</v>
       </c>
       <c r="AN37" t="n">
         <v>0</v>
@@ -8995,7 +8995,7 @@
         <v>24.36</v>
       </c>
       <c r="AZ37" t="n">
-        <v>66.7</v>
+        <v>66.48</v>
       </c>
       <c r="BA37" t="n">
         <v>2.44</v>
@@ -9004,19 +9004,19 @@
         <v>15.53</v>
       </c>
       <c r="BC37" t="n">
-        <v>98.92</v>
+        <v>99.59</v>
       </c>
       <c r="BD37" t="n">
-        <v>62.42</v>
+        <v>62.96</v>
       </c>
       <c r="BE37" t="n">
         <v>344.67</v>
       </c>
       <c r="BF37" t="n">
-        <v>-83.7</v>
+        <v>-83.65000000000001</v>
       </c>
       <c r="BG37" t="n">
-        <v>3.56</v>
+        <v>3.9</v>
       </c>
       <c r="BH37" t="n">
         <v>17.13</v>
@@ -9025,7 +9025,7 @@
         <v>0</v>
       </c>
       <c r="BJ37" t="n">
-        <v>15</v>
+        <v>14.95</v>
       </c>
       <c r="BK37" t="n">
         <v>2.31</v>
@@ -9034,7 +9034,7 @@
         <v>2.31</v>
       </c>
       <c r="BM37" t="n">
-        <v>15</v>
+        <v>14.95</v>
       </c>
       <c r="BN37" t="n">
         <v>20.9</v>
@@ -9043,19 +9043,19 @@
         <v>13.2</v>
       </c>
       <c r="BP37" t="n">
-        <v>14.99</v>
+        <v>14.85</v>
       </c>
       <c r="BQ37" t="n">
-        <v>6.49</v>
+        <v>6.47</v>
       </c>
       <c r="BR37" t="n">
-        <v>14.99</v>
+        <v>14.85</v>
       </c>
       <c r="BS37" t="n">
         <v>0.72</v>
       </c>
       <c r="BT37" t="n">
-        <v>853</v>
+        <v>850</v>
       </c>
     </row>
     <row r="38">
@@ -9315,13 +9315,13 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>69.44</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="G39" t="n">
-        <v>3892689877</v>
+        <v>3845599294</v>
       </c>
       <c r="H39" t="n">
-        <v>1600</v>
+        <v>3400</v>
       </c>
       <c r="I39" t="n">
         <v>168174945</v>
@@ -9336,7 +9336,7 @@
         <v>0.53</v>
       </c>
       <c r="M39" t="n">
-        <v>0.195395957067389</v>
+        <v>0.1930322163572666</v>
       </c>
       <c r="N39" t="n">
         <v>0.06</v>
@@ -9414,7 +9414,7 @@
         <v>2536078170.6</v>
       </c>
       <c r="AM39" t="n">
-        <v>408895995.4831933</v>
+        <v>403949505.6722689</v>
       </c>
       <c r="AN39" t="n">
         <v>11.9435</v>
@@ -9455,7 +9455,7 @@
         <v>170.24</v>
       </c>
       <c r="AZ39" t="n">
-        <v>202.88</v>
+        <v>200.43</v>
       </c>
       <c r="BA39" t="n">
         <v>19.01</v>
@@ -9464,19 +9464,19 @@
         <v>91.72</v>
       </c>
       <c r="BC39" t="n">
-        <v>200.27</v>
+        <v>203.94</v>
       </c>
       <c r="BD39" t="n">
-        <v>145.17</v>
+        <v>148.17</v>
       </c>
       <c r="BE39" t="n">
         <v>192.17</v>
       </c>
       <c r="BF39" t="n">
-        <v>-72.62</v>
+        <v>-72.29000000000001</v>
       </c>
       <c r="BG39" t="n">
-        <v>32.09</v>
+        <v>33.71</v>
       </c>
       <c r="BH39" t="n">
         <v>128.13</v>
@@ -9485,7 +9485,7 @@
         <v>0</v>
       </c>
       <c r="BJ39" t="n">
-        <v>69.44</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="BK39" t="n">
         <v>15.08</v>
@@ -9494,7 +9494,7 @@
         <v>15.08</v>
       </c>
       <c r="BM39" t="n">
-        <v>69.5</v>
+        <v>68.81999999999999</v>
       </c>
       <c r="BN39" t="n">
         <v>74.56</v>
@@ -9503,19 +9503,19 @@
         <v>54.98</v>
       </c>
       <c r="BP39" t="n">
-        <v>69.03</v>
+        <v>68.09</v>
       </c>
       <c r="BQ39" t="n">
-        <v>4.6</v>
+        <v>4.55</v>
       </c>
       <c r="BR39" t="n">
-        <v>69.45</v>
+        <v>68.81999999999999</v>
       </c>
       <c r="BS39" t="n">
         <v>0.58</v>
       </c>
       <c r="BT39" t="n">
-        <v>3030</v>
+        <v>3080</v>
       </c>
     </row>
     <row r="40">
@@ -9545,13 +9545,13 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>22.17</v>
+        <v>21.54</v>
       </c>
       <c r="G40" t="n">
-        <v>127052568047</v>
+        <v>123442169606</v>
       </c>
       <c r="H40" t="n">
-        <v>39523600</v>
+        <v>36947000</v>
       </c>
       <c r="I40" t="n">
         <v>5730834040</v>
@@ -9566,7 +9566,7 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="M40" t="n">
-        <v>0.385493214950817</v>
+        <v>0.3745388192729615</v>
       </c>
       <c r="N40" t="n">
         <v>0.05</v>
@@ -9644,7 +9644,7 @@
         <v>15358635227.2</v>
       </c>
       <c r="AM40" t="n">
-        <v>6589863487.914937</v>
+        <v>6402602157.987552</v>
       </c>
       <c r="AN40" t="n">
         <v>0.5641</v>
@@ -9685,7 +9685,7 @@
         <v>36.13</v>
       </c>
       <c r="AZ40" t="n">
-        <v>11.2</v>
+        <v>10.88</v>
       </c>
       <c r="BA40" t="n">
         <v>2.76</v>
@@ -9694,19 +9694,19 @@
         <v>27.89</v>
       </c>
       <c r="BC40" t="n">
-        <v>99.59</v>
+        <v>105.43</v>
       </c>
       <c r="BD40" t="n">
-        <v>62.96</v>
+        <v>67.73</v>
       </c>
       <c r="BE40" t="n">
         <v>-49.5</v>
       </c>
       <c r="BF40" t="n">
-        <v>-87.55</v>
+        <v>-87.19</v>
       </c>
       <c r="BG40" t="n">
-        <v>25.8</v>
+        <v>29.48</v>
       </c>
       <c r="BH40" t="n">
         <v>32.47</v>
@@ -9715,7 +9715,7 @@
         <v>0</v>
       </c>
       <c r="BJ40" t="n">
-        <v>22.17</v>
+        <v>21.54</v>
       </c>
       <c r="BK40" t="n">
         <v>2.68</v>
@@ -9724,7 +9724,7 @@
         <v>2.5</v>
       </c>
       <c r="BM40" t="n">
-        <v>23.07</v>
+        <v>22.24</v>
       </c>
       <c r="BN40" t="n">
         <v>27.36</v>
@@ -9733,19 +9733,19 @@
         <v>17.67</v>
       </c>
       <c r="BP40" t="n">
-        <v>22.12</v>
+        <v>21.48</v>
       </c>
       <c r="BQ40" t="n">
-        <v>8.869999999999999</v>
+        <v>8.619999999999999</v>
       </c>
       <c r="BR40" t="n">
-        <v>22.43</v>
+        <v>22.17</v>
       </c>
       <c r="BS40" t="n">
         <v>0.39</v>
       </c>
       <c r="BT40" t="n">
-        <v>36599027</v>
+        <v>37323550</v>
       </c>
     </row>
     <row r="41">
@@ -9775,13 +9775,13 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>15.95</v>
+        <v>15.63</v>
       </c>
       <c r="G41" t="n">
-        <v>190196133343</v>
+        <v>187579718444</v>
       </c>
       <c r="H41" t="n">
-        <v>8581200</v>
+        <v>8898100</v>
       </c>
       <c r="I41" t="n">
         <v>5303870781</v>
@@ -9796,7 +9796,7 @@
         <v>0.92</v>
       </c>
       <c r="M41" t="n">
-        <v>1.267461033299173</v>
+        <v>1.250025326941013</v>
       </c>
       <c r="N41" t="n">
         <v>0.07000000000000001</v>
@@ -9874,7 +9874,7 @@
         <v>12304980211.92</v>
       </c>
       <c r="AM41" t="n">
-        <v>29306029790.90909</v>
+        <v>28902884197.84283</v>
       </c>
       <c r="AN41" t="n">
         <v>1.6841</v>
@@ -9915,7 +9915,7 @@
         <v>24.4</v>
       </c>
       <c r="AZ41" t="n">
-        <v>23.87</v>
+        <v>23.39</v>
       </c>
       <c r="BA41" t="n">
         <v>2.53</v>
@@ -9924,19 +9924,19 @@
         <v>13.77</v>
       </c>
       <c r="BC41" t="n">
-        <v>87.37</v>
+        <v>91.20999999999999</v>
       </c>
       <c r="BD41" t="n">
-        <v>52.99</v>
+        <v>56.12</v>
       </c>
       <c r="BE41" t="n">
         <v>49.67</v>
       </c>
       <c r="BF41" t="n">
-        <v>-84.16</v>
+        <v>-83.83</v>
       </c>
       <c r="BG41" t="n">
-        <v>-13.67</v>
+        <v>-11.9</v>
       </c>
       <c r="BH41" t="n">
         <v>17.11</v>
@@ -9945,7 +9945,7 @@
         <v>0</v>
       </c>
       <c r="BJ41" t="n">
-        <v>15.95</v>
+        <v>15.63</v>
       </c>
       <c r="BK41" t="n">
         <v>2.32</v>
@@ -9954,7 +9954,7 @@
         <v>2.34</v>
       </c>
       <c r="BM41" t="n">
-        <v>16.44</v>
+        <v>15.95</v>
       </c>
       <c r="BN41" t="n">
         <v>18.28</v>
@@ -9963,19 +9963,19 @@
         <v>13.43</v>
       </c>
       <c r="BP41" t="n">
-        <v>15.88</v>
+        <v>15.57</v>
       </c>
       <c r="BQ41" t="n">
-        <v>6.82</v>
+        <v>6.69</v>
       </c>
       <c r="BR41" t="n">
-        <v>16.17</v>
+        <v>15.95</v>
       </c>
       <c r="BS41" t="n">
         <v>0.5600000000000001</v>
       </c>
       <c r="BT41" t="n">
-        <v>7202383</v>
+        <v>7174877</v>
       </c>
     </row>
     <row r="42">
@@ -10005,13 +10005,13 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>18.03</v>
+        <v>17.78</v>
       </c>
       <c r="G42" t="n">
-        <v>190196133343</v>
+        <v>187579718444</v>
       </c>
       <c r="H42" t="n">
-        <v>39576500</v>
+        <v>34713200</v>
       </c>
       <c r="I42" t="n">
         <v>5288141247</v>
@@ -10026,7 +10026,7 @@
         <v>1.05</v>
       </c>
       <c r="M42" t="n">
-        <v>1.271231086042803</v>
+        <v>1.25374351731502</v>
       </c>
       <c r="N42" t="n">
         <v>0.08</v>
@@ -10104,7 +10104,7 @@
         <v>12268487693.04</v>
       </c>
       <c r="AM42" t="n">
-        <v>25877024944.62585</v>
+        <v>25521050128.43538</v>
       </c>
       <c r="AN42" t="n">
         <v>1.8491</v>
@@ -10145,7 +10145,7 @@
         <v>24.4</v>
       </c>
       <c r="AZ42" t="n">
-        <v>26.11</v>
+        <v>25.75</v>
       </c>
       <c r="BA42" t="n">
         <v>2.53</v>
@@ -10154,19 +10154,19 @@
         <v>15.11</v>
       </c>
       <c r="BC42" t="n">
-        <v>65.75</v>
+        <v>68.08</v>
       </c>
       <c r="BD42" t="n">
-        <v>35.34</v>
+        <v>37.24</v>
       </c>
       <c r="BE42" t="n">
         <v>44.83</v>
       </c>
       <c r="BF42" t="n">
-        <v>-85.98</v>
+        <v>-85.79000000000001</v>
       </c>
       <c r="BG42" t="n">
-        <v>-16.17</v>
+        <v>-14.99</v>
       </c>
       <c r="BH42" t="n">
         <v>17.11</v>
@@ -10175,7 +10175,7 @@
         <v>0</v>
       </c>
       <c r="BJ42" t="n">
-        <v>18.03</v>
+        <v>17.78</v>
       </c>
       <c r="BK42" t="n">
         <v>2.32</v>
@@ -10184,7 +10184,7 @@
         <v>2.34</v>
       </c>
       <c r="BM42" t="n">
-        <v>18.66</v>
+        <v>18.1</v>
       </c>
       <c r="BN42" t="n">
         <v>21.33</v>
@@ -10193,19 +10193,19 @@
         <v>15.67</v>
       </c>
       <c r="BP42" t="n">
-        <v>18.03</v>
+        <v>17.66</v>
       </c>
       <c r="BQ42" t="n">
-        <v>7.71</v>
+        <v>7.61</v>
       </c>
       <c r="BR42" t="n">
-        <v>18.18</v>
+        <v>18.08</v>
       </c>
       <c r="BS42" t="n">
         <v>0.63</v>
       </c>
       <c r="BT42" t="n">
-        <v>41807093</v>
+        <v>41398077</v>
       </c>
     </row>
     <row r="43">
@@ -10235,13 +10235,13 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>38.86</v>
+        <v>38.77</v>
       </c>
       <c r="G43" t="n">
-        <v>75442805184</v>
+        <v>75268040118</v>
       </c>
       <c r="H43" t="n">
-        <v>6633900</v>
+        <v>3910900</v>
       </c>
       <c r="I43" t="n">
         <v>1941400000</v>
@@ -10334,7 +10334,7 @@
         <v>9182822000</v>
       </c>
       <c r="AM43" t="n">
-        <v>9189135832.399511</v>
+        <v>9167848979.049938</v>
       </c>
       <c r="AN43" t="n">
         <v>4.5901</v>
@@ -10375,7 +10375,7 @@
         <v>19.95</v>
       </c>
       <c r="AZ43" t="n">
-        <v>70.53</v>
+        <v>70.37</v>
       </c>
       <c r="BA43" t="n">
         <v>5.63</v>
@@ -10384,19 +10384,19 @@
         <v>48.62</v>
       </c>
       <c r="BC43" t="n">
-        <v>-37.12</v>
+        <v>-36.98</v>
       </c>
       <c r="BD43" t="n">
-        <v>-48.66</v>
+        <v>-48.54</v>
       </c>
       <c r="BE43" t="n">
         <v>81.5</v>
       </c>
       <c r="BF43" t="n">
-        <v>-85.52</v>
+        <v>-85.48</v>
       </c>
       <c r="BG43" t="n">
-        <v>25.11</v>
+        <v>25.4</v>
       </c>
       <c r="BH43" t="n">
         <v>5.61</v>
@@ -10405,7 +10405,7 @@
         <v>0</v>
       </c>
       <c r="BJ43" t="n">
-        <v>38.86</v>
+        <v>38.77</v>
       </c>
       <c r="BK43" t="n">
         <v>4.73</v>
@@ -10423,19 +10423,19 @@
         <v>28.06</v>
       </c>
       <c r="BP43" t="n">
-        <v>38.67</v>
+        <v>38.69</v>
       </c>
       <c r="BQ43" t="n">
-        <v>8.210000000000001</v>
+        <v>8.19</v>
       </c>
       <c r="BR43" t="n">
-        <v>39.14</v>
+        <v>38.88</v>
       </c>
       <c r="BS43" t="n">
         <v>0</v>
       </c>
       <c r="BT43" t="n">
-        <v>6641470</v>
+        <v>6596033</v>
       </c>
     </row>
     <row r="44">
@@ -10925,13 +10925,13 @@
         </is>
       </c>
       <c r="F46" t="n">
-        <v>4.02</v>
+        <v>4.05</v>
       </c>
       <c r="G46" t="n">
-        <v>4022178820</v>
+        <v>4052195290</v>
       </c>
       <c r="H46" t="n">
-        <v>10047200</v>
+        <v>18284500</v>
       </c>
       <c r="I46" t="n">
         <v>1000542188</v>
@@ -10946,7 +10946,7 @@
         <v>2.5</v>
       </c>
       <c r="M46" t="n">
-        <v>0.06991302999409356</v>
+        <v>0.07043477267668936</v>
       </c>
       <c r="N46" t="n">
         <v>0.08</v>
@@ -11024,7 +11024,7 @@
         <v>460249406.48</v>
       </c>
       <c r="AM46" t="n">
-        <v>3943312568.627451</v>
+        <v>3972740480.392157</v>
       </c>
       <c r="AN46" t="n">
         <v>0.0311</v>
@@ -11065,7 +11065,7 @@
         <v>3.3</v>
       </c>
       <c r="AZ46" t="n">
-        <v>3.32</v>
+        <v>3.34</v>
       </c>
       <c r="BA46" t="n">
         <v>0.42</v>
@@ -11074,19 +11074,19 @@
         <v>7.38</v>
       </c>
       <c r="BC46" t="n">
-        <v>0.59</v>
+        <v>-0.15</v>
       </c>
       <c r="BD46" t="n">
-        <v>-17.87</v>
+        <v>-18.47</v>
       </c>
       <c r="BE46" t="n">
         <v>-17.5</v>
       </c>
       <c r="BF46" t="n">
-        <v>-89.48</v>
+        <v>-89.55</v>
       </c>
       <c r="BG46" t="n">
-        <v>83.55</v>
+        <v>82.19</v>
       </c>
       <c r="BH46" t="n">
         <v>1.58</v>
@@ -11095,7 +11095,7 @@
         <v>0</v>
       </c>
       <c r="BJ46" t="n">
-        <v>4.02</v>
+        <v>4.05</v>
       </c>
       <c r="BK46" t="n">
         <v>0.46</v>
@@ -11104,7 +11104,7 @@
         <v>0.46</v>
       </c>
       <c r="BM46" t="n">
-        <v>4.06</v>
+        <v>4.11</v>
       </c>
       <c r="BN46" t="n">
         <v>7.31</v>
@@ -11113,19 +11113,19 @@
         <v>2.97</v>
       </c>
       <c r="BP46" t="n">
-        <v>3.92</v>
+        <v>3.98</v>
       </c>
       <c r="BQ46" t="n">
-        <v>8.789999999999999</v>
+        <v>8.85</v>
       </c>
       <c r="BR46" t="n">
-        <v>3.99</v>
+        <v>4.02</v>
       </c>
       <c r="BS46" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="BT46" t="n">
-        <v>22859087</v>
+        <v>22806877</v>
       </c>
     </row>
     <row r="47">
@@ -11155,13 +11155,13 @@
         </is>
       </c>
       <c r="F47" t="n">
-        <v>8.98</v>
+        <v>8.93</v>
       </c>
       <c r="G47" t="n">
-        <v>3129905204</v>
+        <v>3122716625</v>
       </c>
       <c r="H47" t="n">
-        <v>3800</v>
+        <v>4800</v>
       </c>
       <c r="I47" t="n">
         <v>254106600</v>
@@ -11176,7 +11176,7 @@
         <v>1.22</v>
       </c>
       <c r="M47" t="n">
-        <v>0.738067657476581</v>
+        <v>0.73637250784191</v>
       </c>
       <c r="N47" t="n">
         <v>0.07000000000000001</v>
@@ -11254,7 +11254,7 @@
         <v>322715382</v>
       </c>
       <c r="AM47" t="n">
-        <v>554947731.2056738</v>
+        <v>553673160.4609929</v>
       </c>
       <c r="AN47" t="n">
         <v>0.4132</v>
@@ -11295,7 +11295,7 @@
         <v>11.74</v>
       </c>
       <c r="AZ47" t="n">
-        <v>11.79</v>
+        <v>11.73</v>
       </c>
       <c r="BA47" t="n">
         <v>1.46</v>
@@ -11304,19 +11304,19 @@
         <v>8.619999999999999</v>
       </c>
       <c r="BC47" t="n">
-        <v>60.06</v>
+        <v>60.96</v>
       </c>
       <c r="BD47" t="n">
-        <v>30.69</v>
+        <v>31.42</v>
       </c>
       <c r="BE47" t="n">
         <v>31.33</v>
       </c>
       <c r="BF47" t="n">
-        <v>-83.76000000000001</v>
+        <v>-83.67</v>
       </c>
       <c r="BG47" t="n">
-        <v>-4.01</v>
+        <v>-3.47</v>
       </c>
       <c r="BH47" t="n">
         <v>7.23</v>
@@ -11325,7 +11325,7 @@
         <v>0</v>
       </c>
       <c r="BJ47" t="n">
-        <v>8.98</v>
+        <v>8.93</v>
       </c>
       <c r="BK47" t="n">
         <v>1.27</v>
@@ -11343,19 +11343,19 @@
         <v>7.19</v>
       </c>
       <c r="BP47" t="n">
-        <v>8.92</v>
+        <v>8.9</v>
       </c>
       <c r="BQ47" t="n">
-        <v>6.94</v>
+        <v>6.9</v>
       </c>
       <c r="BR47" t="n">
-        <v>8.99</v>
+        <v>8.98</v>
       </c>
       <c r="BS47" t="n">
         <v>0.53</v>
       </c>
       <c r="BT47" t="n">
-        <v>11413</v>
+        <v>11317</v>
       </c>
     </row>
     <row r="48">
@@ -11385,13 +11385,13 @@
         </is>
       </c>
       <c r="F48" t="n">
-        <v>9.19</v>
+        <v>9.109999999999999</v>
       </c>
       <c r="G48" t="n">
-        <v>3129905204</v>
+        <v>3122716625</v>
       </c>
       <c r="H48" t="n">
-        <v>3700</v>
+        <v>7700</v>
       </c>
       <c r="I48" t="n">
         <v>93397546</v>
@@ -11406,7 +11406,7 @@
         <v>1.24</v>
       </c>
       <c r="M48" t="n">
-        <v>2.008059858567789</v>
+        <v>2.003447866833473</v>
       </c>
       <c r="N48" t="n">
         <v>0.07000000000000001</v>
@@ -11484,7 +11484,7 @@
         <v>118614883.42</v>
       </c>
       <c r="AM48" t="n">
-        <v>547186224.4755245</v>
+        <v>545929479.8951049</v>
       </c>
       <c r="AN48" t="n">
         <v>0.4132</v>
@@ -11525,7 +11525,7 @@
         <v>11.74</v>
       </c>
       <c r="AZ48" t="n">
-        <v>12.02</v>
+        <v>11.92</v>
       </c>
       <c r="BA48" t="n">
         <v>1.46</v>
@@ -11534,19 +11534,19 @@
         <v>8.24</v>
       </c>
       <c r="BC48" t="n">
-        <v>56.4</v>
+        <v>57.78</v>
       </c>
       <c r="BD48" t="n">
-        <v>27.7</v>
+        <v>28.82</v>
       </c>
       <c r="BE48" t="n">
         <v>30.83</v>
       </c>
       <c r="BF48" t="n">
-        <v>-84.13</v>
+        <v>-83.98999999999999</v>
       </c>
       <c r="BG48" t="n">
-        <v>-10.38</v>
+        <v>-9.59</v>
       </c>
       <c r="BH48" t="n">
         <v>7.23</v>
@@ -11555,7 +11555,7 @@
         <v>0</v>
       </c>
       <c r="BJ48" t="n">
-        <v>9.19</v>
+        <v>9.109999999999999</v>
       </c>
       <c r="BK48" t="n">
         <v>1.27</v>
@@ -11564,7 +11564,7 @@
         <v>1.29</v>
       </c>
       <c r="BM48" t="n">
-        <v>9.35</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="BN48" t="n">
         <v>9.48</v>
@@ -11573,19 +11573,19 @@
         <v>7.2</v>
       </c>
       <c r="BP48" t="n">
-        <v>9.09</v>
+        <v>9.050000000000001</v>
       </c>
       <c r="BQ48" t="n">
-        <v>7.11</v>
+        <v>7.04</v>
       </c>
       <c r="BR48" t="n">
-        <v>9.09</v>
+        <v>9.08</v>
       </c>
       <c r="BS48" t="n">
         <v>0.54</v>
       </c>
       <c r="BT48" t="n">
-        <v>2420</v>
+        <v>2497</v>
       </c>
     </row>
     <row r="49">
@@ -11615,13 +11615,13 @@
         </is>
       </c>
       <c r="F49" t="n">
-        <v>49.9</v>
+        <v>50.49</v>
       </c>
       <c r="G49" t="n">
-        <v>996908218</v>
+        <v>971669984</v>
       </c>
       <c r="H49" t="n">
-        <v>0</v>
+        <v>2700</v>
       </c>
       <c r="I49" t="n">
         <v>11540870</v>
@@ -11636,7 +11636,7 @@
         <v>1.09</v>
       </c>
       <c r="M49" t="n">
-        <v>1.00855918550514</v>
+        <v>0.9830259897033297</v>
       </c>
       <c r="N49" t="n">
         <v>0.08</v>
@@ -11714,7 +11714,7 @@
         <v>84709985.8</v>
       </c>
       <c r="AM49" t="n">
-        <v>249227054.5</v>
+        <v>242917496</v>
       </c>
       <c r="AN49" t="n">
         <v>3.3186</v>
@@ -11755,7 +11755,7 @@
         <v>68.48999999999999</v>
       </c>
       <c r="AZ49" t="n">
-        <v>59.55</v>
+        <v>60.25</v>
       </c>
       <c r="BA49" t="n">
         <v>9.210000000000001</v>
@@ -11764,19 +11764,19 @@
         <v>27.75</v>
       </c>
       <c r="BC49" t="n">
-        <v>68.09</v>
+        <v>66.13</v>
       </c>
       <c r="BD49" t="n">
-        <v>37.25</v>
+        <v>35.64</v>
       </c>
       <c r="BE49" t="n">
         <v>19.33</v>
       </c>
       <c r="BF49" t="n">
-        <v>-81.54000000000001</v>
+        <v>-81.75</v>
       </c>
       <c r="BG49" t="n">
-        <v>-44.38</v>
+        <v>-45.03</v>
       </c>
       <c r="BH49" t="n">
         <v>42.6</v>
@@ -11785,7 +11785,7 @@
         <v>0</v>
       </c>
       <c r="BJ49" t="n">
-        <v>49.9</v>
+        <v>50.49</v>
       </c>
       <c r="BK49" t="n">
         <v>7.34</v>
@@ -11794,28 +11794,28 @@
         <v>7.6</v>
       </c>
       <c r="BM49" t="n">
-        <v>50.68</v>
+        <v>50.49</v>
       </c>
       <c r="BN49" t="n">
         <v>64.2</v>
       </c>
       <c r="BO49" t="n">
-        <v>27.62</v>
+        <v>28.48</v>
       </c>
       <c r="BP49" t="n">
-        <v>44.13</v>
+        <v>46.36</v>
       </c>
       <c r="BQ49" t="n">
-        <v>6.57</v>
+        <v>6.64</v>
       </c>
       <c r="BR49" t="n">
-        <v>48.88</v>
+        <v>49.15</v>
       </c>
       <c r="BS49" t="n">
         <v>0.54</v>
       </c>
       <c r="BT49" t="n">
-        <v>373</v>
+        <v>243</v>
       </c>
     </row>
     <row r="50">
@@ -11845,13 +11845,13 @@
         </is>
       </c>
       <c r="F50" t="n">
-        <v>33.31</v>
+        <v>33.1</v>
       </c>
       <c r="G50" t="n">
-        <v>952237200</v>
+        <v>971669984</v>
       </c>
       <c r="H50" t="n">
-        <v>1200</v>
+        <v>1000</v>
       </c>
       <c r="I50" t="n">
         <v>11540870</v>
@@ -11866,7 +11866,7 @@
         <v>0.8</v>
       </c>
       <c r="M50" t="n">
-        <v>0.9633660927847777</v>
+        <v>0.9830259897033297</v>
       </c>
       <c r="N50" t="n">
         <v>0.06</v>
@@ -11944,7 +11944,7 @@
         <v>84709985.8</v>
       </c>
       <c r="AM50" t="n">
-        <v>324995631.3993174</v>
+        <v>331627980.887372</v>
       </c>
       <c r="AN50" t="n">
         <v>4.4983</v>
@@ -11985,7 +11985,7 @@
         <v>68.48999999999999</v>
       </c>
       <c r="AZ50" t="n">
-        <v>73.45</v>
+        <v>72.98999999999999</v>
       </c>
       <c r="BA50" t="n">
         <v>9.210000000000001</v>
@@ -11994,19 +11994,19 @@
         <v>30.53</v>
       </c>
       <c r="BC50" t="n">
-        <v>151.81</v>
+        <v>153.41</v>
       </c>
       <c r="BD50" t="n">
-        <v>105.6</v>
+        <v>106.9</v>
       </c>
       <c r="BE50" t="n">
         <v>120.5</v>
       </c>
       <c r="BF50" t="n">
-        <v>-72.34</v>
+        <v>-72.16</v>
       </c>
       <c r="BG50" t="n">
-        <v>-8.35</v>
+        <v>-7.76</v>
       </c>
       <c r="BH50" t="n">
         <v>42.6</v>
@@ -12015,7 +12015,7 @@
         <v>0</v>
       </c>
       <c r="BJ50" t="n">
-        <v>33.31</v>
+        <v>33.1</v>
       </c>
       <c r="BK50" t="n">
         <v>7.34</v>
@@ -12024,7 +12024,7 @@
         <v>7.6</v>
       </c>
       <c r="BM50" t="n">
-        <v>33.8</v>
+        <v>33.98</v>
       </c>
       <c r="BN50" t="n">
         <v>39.22</v>
@@ -12033,19 +12033,19 @@
         <v>23.5</v>
       </c>
       <c r="BP50" t="n">
-        <v>33.07</v>
+        <v>32.65</v>
       </c>
       <c r="BQ50" t="n">
-        <v>4.38</v>
+        <v>4.35</v>
       </c>
       <c r="BR50" t="n">
-        <v>33.09</v>
+        <v>33.98</v>
       </c>
       <c r="BS50" t="n">
         <v>0.4</v>
       </c>
       <c r="BT50" t="n">
-        <v>487</v>
+        <v>520</v>
       </c>
     </row>
     <row r="51">
@@ -12523,13 +12523,13 @@
         </is>
       </c>
       <c r="F53" t="n">
-        <v>6.26</v>
+        <v>6</v>
       </c>
       <c r="G53" t="n">
-        <v>856696055</v>
+        <v>821114400</v>
       </c>
       <c r="H53" t="n">
-        <v>5200</v>
+        <v>27200</v>
       </c>
       <c r="I53" t="n">
         <v>136852484</v>
@@ -12544,7 +12544,7 @@
         <v>2.79</v>
       </c>
       <c r="M53" t="n">
-        <v>2.225536645532411</v>
+        <v>2.133102138977818</v>
       </c>
       <c r="N53" t="n">
         <v>1.48</v>
@@ -12622,7 +12622,7 @@
         <v>39687220.36</v>
       </c>
       <c r="AM53" t="n">
-        <v>43642183.138054</v>
+        <v>41829566.98930209</v>
       </c>
       <c r="AN53" t="n">
         <v>0</v>
@@ -12672,16 +12672,16 @@
         <v>0</v>
       </c>
       <c r="BC53" t="n">
-        <v>-37.05</v>
+        <v>-34.32</v>
       </c>
       <c r="BD53" t="n">
-        <v>-48.6</v>
+        <v>-46.37</v>
       </c>
       <c r="BE53" t="n">
         <v>-100</v>
       </c>
       <c r="BF53" t="n">
-        <v>-95.37</v>
+        <v>-95.17</v>
       </c>
       <c r="BG53" t="n">
         <v>-100</v>
@@ -12693,7 +12693,7 @@
         <v>0</v>
       </c>
       <c r="BJ53" t="n">
-        <v>6.26</v>
+        <v>6</v>
       </c>
       <c r="BK53" t="n">
         <v>0.29</v>
@@ -12702,7 +12702,7 @@
         <v>0.09</v>
       </c>
       <c r="BM53" t="n">
-        <v>6.44</v>
+        <v>6.29</v>
       </c>
       <c r="BN53" t="n">
         <v>10.39</v>
@@ -12711,19 +12711,19 @@
         <v>4.82</v>
       </c>
       <c r="BP53" t="n">
-        <v>6.22</v>
+        <v>6</v>
       </c>
       <c r="BQ53" t="n">
-        <v>73.37</v>
+        <v>70.31999999999999</v>
       </c>
       <c r="BR53" t="n">
-        <v>6.42</v>
+        <v>6.29</v>
       </c>
       <c r="BS53" t="n">
         <v>2.36</v>
       </c>
       <c r="BT53" t="n">
-        <v>36310</v>
+        <v>34953</v>
       </c>
     </row>
     <row r="54">
@@ -12753,13 +12753,13 @@
         </is>
       </c>
       <c r="F54" t="n">
-        <v>10.26</v>
+        <v>10.29</v>
       </c>
       <c r="G54" t="n">
-        <v>2392756199</v>
+        <v>2399751471</v>
       </c>
       <c r="H54" t="n">
-        <v>175700</v>
+        <v>246300</v>
       </c>
       <c r="I54" t="n">
         <v>233212121</v>
@@ -12774,7 +12774,7 @@
         <v>0.97</v>
       </c>
       <c r="M54" t="n">
-        <v>1.34303390881257</v>
+        <v>1.346960296089842</v>
       </c>
       <c r="N54" t="n">
         <v>0.5600000000000001</v>
@@ -12852,7 +12852,7 @@
         <v>233212121</v>
       </c>
       <c r="AM54" t="n">
-        <v>327326429.4117647</v>
+        <v>328283374.9658003</v>
       </c>
       <c r="AN54" t="n">
         <v>0.1531</v>
@@ -12893,7 +12893,7 @@
         <v>12.25</v>
       </c>
       <c r="AZ54" t="n">
-        <v>16.33</v>
+        <v>16.38</v>
       </c>
       <c r="BA54" t="n">
         <v>0.98</v>
@@ -12902,19 +12902,19 @@
         <v>6.52</v>
       </c>
       <c r="BC54" t="n">
-        <v>46.27</v>
+        <v>45.85</v>
       </c>
       <c r="BD54" t="n">
-        <v>19.43</v>
+        <v>19.08</v>
       </c>
       <c r="BE54" t="n">
         <v>59.17</v>
       </c>
       <c r="BF54" t="n">
-        <v>-90.42</v>
+        <v>-90.44</v>
       </c>
       <c r="BG54" t="n">
-        <v>-36.49</v>
+        <v>-36.67</v>
       </c>
       <c r="BH54" t="n">
         <v>10.01</v>
@@ -12923,7 +12923,7 @@
         <v>0</v>
       </c>
       <c r="BJ54" t="n">
-        <v>10.26</v>
+        <v>10.29</v>
       </c>
       <c r="BK54" t="n">
         <v>1</v>
@@ -12932,7 +12932,7 @@
         <v>1</v>
       </c>
       <c r="BM54" t="n">
-        <v>10.58</v>
+        <v>10.6</v>
       </c>
       <c r="BN54" t="n">
         <v>11.75</v>
@@ -12941,19 +12941,19 @@
         <v>8.279999999999999</v>
       </c>
       <c r="BP54" t="n">
+        <v>10.21</v>
+      </c>
+      <c r="BQ54" t="n">
+        <v>10.26</v>
+      </c>
+      <c r="BR54" t="n">
         <v>10.25</v>
-      </c>
-      <c r="BQ54" t="n">
-        <v>10.23</v>
-      </c>
-      <c r="BR54" t="n">
-        <v>10.46</v>
       </c>
       <c r="BS54" t="n">
         <v>1.26</v>
       </c>
       <c r="BT54" t="n">
-        <v>277350</v>
+        <v>274093</v>
       </c>
     </row>
     <row r="55">
@@ -12983,13 +12983,13 @@
         </is>
       </c>
       <c r="F55" t="n">
-        <v>50.03</v>
+        <v>49.64</v>
       </c>
       <c r="G55" t="n">
-        <v>6525984600</v>
+        <v>6373382231</v>
       </c>
       <c r="H55" t="n">
-        <v>700</v>
+        <v>4100</v>
       </c>
       <c r="I55" t="n">
         <v>84052790</v>
@@ -13004,7 +13004,7 @@
         <v>2</v>
       </c>
       <c r="M55" t="n">
-        <v>1.007423802494199</v>
+        <v>0.9838663980149425</v>
       </c>
       <c r="N55" t="n">
         <v>0.16</v>
@@ -13082,7 +13082,7 @@
         <v>579123723.1</v>
       </c>
       <c r="AM55" t="n">
-        <v>328268843.0583501</v>
+        <v>320592667.555332</v>
       </c>
       <c r="AN55" t="n">
         <v>3.1953</v>
@@ -13123,7 +13123,7 @@
         <v>51.21</v>
       </c>
       <c r="AZ55" t="n">
-        <v>52.61</v>
+        <v>52.2</v>
       </c>
       <c r="BA55" t="n">
         <v>9.380000000000001</v>
@@ -13132,19 +13132,19 @@
         <v>16.08</v>
       </c>
       <c r="BC55" t="n">
-        <v>25.35</v>
+        <v>26.34</v>
       </c>
       <c r="BD55" t="n">
-        <v>2.35</v>
+        <v>3.15</v>
       </c>
       <c r="BE55" t="n">
         <v>5.17</v>
       </c>
       <c r="BF55" t="n">
-        <v>-81.26000000000001</v>
+        <v>-81.11</v>
       </c>
       <c r="BG55" t="n">
-        <v>-67.87</v>
+        <v>-67.61</v>
       </c>
       <c r="BH55" t="n">
         <v>25.37</v>
@@ -13153,7 +13153,7 @@
         <v>0</v>
       </c>
       <c r="BJ55" t="n">
-        <v>50.03</v>
+        <v>49.64</v>
       </c>
       <c r="BK55" t="n">
         <v>6.89</v>
@@ -13162,7 +13162,7 @@
         <v>7.03</v>
       </c>
       <c r="BM55" t="n">
-        <v>50.98</v>
+        <v>50.88</v>
       </c>
       <c r="BN55" t="n">
         <v>73.67</v>
@@ -13171,19 +13171,19 @@
         <v>35.58</v>
       </c>
       <c r="BP55" t="n">
-        <v>50.03</v>
+        <v>49.62</v>
       </c>
       <c r="BQ55" t="n">
-        <v>7.12</v>
+        <v>7.06</v>
       </c>
       <c r="BR55" t="n">
-        <v>50.98</v>
+        <v>50.71</v>
       </c>
       <c r="BS55" t="n">
         <v>0.66</v>
       </c>
       <c r="BT55" t="n">
-        <v>7090</v>
+        <v>7003</v>
       </c>
     </row>
     <row r="56">
@@ -13213,13 +13213,13 @@
         </is>
       </c>
       <c r="F56" t="n">
-        <v>59.25</v>
+        <v>57.6</v>
       </c>
       <c r="G56" t="n">
-        <v>6525984600</v>
+        <v>6373382231</v>
       </c>
       <c r="H56" t="n">
-        <v>17800</v>
+        <v>56700</v>
       </c>
       <c r="I56" t="n">
         <v>39675836</v>
@@ -13234,7 +13234,7 @@
         <v>2.41</v>
       </c>
       <c r="M56" t="n">
-        <v>2.134215428051634</v>
+        <v>2.084309344871937</v>
       </c>
       <c r="N56" t="n">
         <v>0.19</v>
@@ -13312,7 +13312,7 @@
         <v>273366510.04</v>
       </c>
       <c r="AM56" t="n">
-        <v>271463585.6905158</v>
+        <v>265115733.4026622</v>
       </c>
       <c r="AN56" t="n">
         <v>3.5102</v>
@@ -13353,7 +13353,7 @@
         <v>51.21</v>
       </c>
       <c r="AZ56" t="n">
-        <v>56.58</v>
+        <v>55.01</v>
       </c>
       <c r="BA56" t="n">
         <v>9.380000000000001</v>
@@ -13362,19 +13362,19 @@
         <v>17.68</v>
       </c>
       <c r="BC56" t="n">
-        <v>5.85</v>
+        <v>8.880000000000001</v>
       </c>
       <c r="BD56" t="n">
-        <v>-13.58</v>
+        <v>-11.1</v>
       </c>
       <c r="BE56" t="n">
         <v>-4.5</v>
       </c>
       <c r="BF56" t="n">
-        <v>-84.17</v>
+        <v>-83.72</v>
       </c>
       <c r="BG56" t="n">
-        <v>-70.16</v>
+        <v>-69.31</v>
       </c>
       <c r="BH56" t="n">
         <v>25.37</v>
@@ -13383,7 +13383,7 @@
         <v>0</v>
       </c>
       <c r="BJ56" t="n">
-        <v>59.25</v>
+        <v>57.6</v>
       </c>
       <c r="BK56" t="n">
         <v>6.89</v>
@@ -13392,7 +13392,7 @@
         <v>7.03</v>
       </c>
       <c r="BM56" t="n">
-        <v>60.5</v>
+        <v>60.46</v>
       </c>
       <c r="BN56" t="n">
         <v>86.77</v>
@@ -13401,19 +13401,19 @@
         <v>46.42</v>
       </c>
       <c r="BP56" t="n">
-        <v>58.42</v>
+        <v>57.6</v>
       </c>
       <c r="BQ56" t="n">
-        <v>8.43</v>
+        <v>8.19</v>
       </c>
       <c r="BR56" t="n">
-        <v>60.11</v>
+        <v>59.63</v>
       </c>
       <c r="BS56" t="n">
         <v>0.79</v>
       </c>
       <c r="BT56" t="n">
-        <v>31633</v>
+        <v>30470</v>
       </c>
     </row>
     <row r="57">
@@ -13443,13 +13443,13 @@
         </is>
       </c>
       <c r="F57" t="n">
-        <v>6.03</v>
+        <v>6</v>
       </c>
       <c r="G57" t="n">
-        <v>1410163789</v>
+        <v>1403148000</v>
       </c>
       <c r="H57" t="n">
-        <v>1477600</v>
+        <v>894900</v>
       </c>
       <c r="I57" t="n">
         <v>233858065</v>
@@ -13464,7 +13464,7 @@
         <v>0.77</v>
       </c>
       <c r="M57" t="n">
-        <v>0.4220998973458538</v>
+        <v>0.4199998832625251</v>
       </c>
       <c r="N57" t="n">
         <v>0.08</v>
@@ -13542,7 +13542,7 @@
         <v>229180903.7</v>
       </c>
       <c r="AM57" t="n">
-        <v>105472235.5272999</v>
+        <v>104947494.3904263</v>
       </c>
       <c r="AN57" t="n">
         <v>0.347</v>
@@ -13583,7 +13583,7 @@
         <v>10.72</v>
       </c>
       <c r="AZ57" t="n">
-        <v>9.199999999999999</v>
+        <v>9.15</v>
       </c>
       <c r="BA57" t="n">
         <v>1.13</v>
@@ -13592,19 +13592,19 @@
         <v>6.26</v>
       </c>
       <c r="BC57" t="n">
-        <v>117.77</v>
+        <v>118.85</v>
       </c>
       <c r="BD57" t="n">
-        <v>77.81</v>
+        <v>78.69</v>
       </c>
       <c r="BE57" t="n">
         <v>52.5</v>
       </c>
       <c r="BF57" t="n">
-        <v>-81.3</v>
+        <v>-81.20999999999999</v>
       </c>
       <c r="BG57" t="n">
-        <v>3.88</v>
+        <v>4.4</v>
       </c>
       <c r="BH57" t="n">
         <v>7.82</v>
@@ -13613,7 +13613,7 @@
         <v>0</v>
       </c>
       <c r="BJ57" t="n">
-        <v>6.03</v>
+        <v>6</v>
       </c>
       <c r="BK57" t="n">
         <v>0.98</v>
@@ -13622,7 +13622,7 @@
         <v>1.04</v>
       </c>
       <c r="BM57" t="n">
-        <v>6.22</v>
+        <v>6.05</v>
       </c>
       <c r="BN57" t="n">
         <v>6.22</v>
@@ -13631,19 +13631,19 @@
         <v>3.43</v>
       </c>
       <c r="BP57" t="n">
-        <v>6.03</v>
+        <v>5.95</v>
       </c>
       <c r="BQ57" t="n">
-        <v>5.82</v>
+        <v>5.79</v>
       </c>
       <c r="BR57" t="n">
-        <v>6.1</v>
+        <v>6.02</v>
       </c>
       <c r="BS57" t="n">
         <v>0.42</v>
       </c>
       <c r="BT57" t="n">
-        <v>1328663</v>
+        <v>1346737</v>
       </c>
     </row>
     <row r="58">
@@ -14133,13 +14133,13 @@
         </is>
       </c>
       <c r="F60" t="n">
-        <v>374.49</v>
+        <v>370</v>
       </c>
       <c r="G60" t="n">
-        <v>170299285</v>
+        <v>168257463</v>
       </c>
       <c r="H60" t="n">
-        <v>16</v>
+        <v>58</v>
       </c>
       <c r="I60" t="n">
         <v>454750</v>
@@ -14154,7 +14154,7 @@
         <v>0.83</v>
       </c>
       <c r="M60" t="n">
-        <v>12.73814678670082</v>
+        <v>12.58542137538558</v>
       </c>
       <c r="N60" t="n">
         <v>0.68</v>
@@ -14232,7 +14232,7 @@
         <v>59558607.5</v>
       </c>
       <c r="AM60" t="n">
-        <v>-24970569.64809384</v>
+        <v>-24671182.25806452</v>
       </c>
       <c r="AN60" t="n">
         <v>10.0581</v>
@@ -14273,7 +14273,7 @@
         <v>944.87</v>
       </c>
       <c r="AZ60" t="n">
-        <v>2153.32</v>
+        <v>2127.5</v>
       </c>
       <c r="BA60" t="n">
         <v>231.1</v>
@@ -14282,19 +14282,19 @@
         <v>727.97</v>
       </c>
       <c r="BC60" t="n">
-        <v>209.01</v>
+        <v>212.76</v>
       </c>
       <c r="BD60" t="n">
-        <v>152.31</v>
+        <v>155.37</v>
       </c>
       <c r="BE60" t="n">
         <v>475</v>
       </c>
       <c r="BF60" t="n">
-        <v>-38.29</v>
+        <v>-37.54</v>
       </c>
       <c r="BG60" t="n">
-        <v>94.39</v>
+        <v>96.75</v>
       </c>
       <c r="BH60" t="n">
         <v>454.44</v>
@@ -14303,7 +14303,7 @@
         <v>0</v>
       </c>
       <c r="BJ60" t="n">
-        <v>374.49</v>
+        <v>370</v>
       </c>
       <c r="BK60" t="n">
         <v>130.97</v>
@@ -14312,7 +14312,7 @@
         <v>130.97</v>
       </c>
       <c r="BM60" t="n">
-        <v>374.49</v>
+        <v>385.05</v>
       </c>
       <c r="BN60" t="n">
         <v>405</v>
@@ -14321,13 +14321,13 @@
         <v>309.24</v>
       </c>
       <c r="BP60" t="n">
-        <v>369.83</v>
+        <v>370</v>
       </c>
       <c r="BQ60" t="n">
-        <v>2.86</v>
+        <v>2.83</v>
       </c>
       <c r="BR60" t="n">
-        <v>369.83</v>
+        <v>385.05</v>
       </c>
       <c r="BS60" t="n">
         <v>12.82</v>
@@ -14366,10 +14366,10 @@
         <v>27.82</v>
       </c>
       <c r="G61" t="n">
-        <v>2381625661</v>
+        <v>2381624827</v>
       </c>
       <c r="H61" t="n">
-        <v>508600</v>
+        <v>919400</v>
       </c>
       <c r="I61" t="n">
         <v>85608392</v>
@@ -14384,7 +14384,7 @@
         <v>2.37</v>
       </c>
       <c r="M61" t="n">
-        <v>1.263057857722877</v>
+        <v>1.263057415424043</v>
       </c>
       <c r="N61" t="n">
         <v>1.1</v>
@@ -14462,7 +14462,7 @@
         <v>160087693.04</v>
       </c>
       <c r="AM61" t="n">
-        <v>186940789.7174254</v>
+        <v>186940724.2543171</v>
       </c>
       <c r="AN61" t="n">
         <v>0.38</v>
@@ -14542,7 +14542,7 @@
         <v>1.86</v>
       </c>
       <c r="BM61" t="n">
-        <v>28.61</v>
+        <v>28.1</v>
       </c>
       <c r="BN61" t="n">
         <v>28.68</v>
@@ -14551,19 +14551,19 @@
         <v>19.35</v>
       </c>
       <c r="BP61" t="n">
-        <v>27.6</v>
+        <v>27.42</v>
       </c>
       <c r="BQ61" t="n">
         <v>14.94</v>
       </c>
       <c r="BR61" t="n">
-        <v>28.51</v>
+        <v>27.64</v>
       </c>
       <c r="BS61" t="n">
         <v>1.19</v>
       </c>
       <c r="BT61" t="n">
-        <v>564890</v>
+        <v>564603</v>
       </c>
     </row>
     <row r="62">
@@ -14593,10 +14593,10 @@
         </is>
       </c>
       <c r="F62" t="n">
-        <v>110</v>
+        <v>111.75</v>
       </c>
       <c r="G62" t="n">
-        <v>10856968100</v>
+        <v>11029693710</v>
       </c>
       <c r="H62" t="n">
         <v>200</v>
@@ -14614,7 +14614,7 @@
         <v>0.64</v>
       </c>
       <c r="M62" t="n">
-        <v>1.017716133294815</v>
+        <v>1.033907176531848</v>
       </c>
       <c r="N62" t="n">
         <v>0.13</v>
@@ -14692,7 +14692,7 @@
         <v>2757670987.06</v>
       </c>
       <c r="AM62" t="n">
-        <v>4395533643.724696</v>
+        <v>4465463040.485829</v>
       </c>
       <c r="AN62" t="n">
         <v>6.9319</v>
@@ -14733,7 +14733,7 @@
         <v>267.2</v>
       </c>
       <c r="AZ62" t="n">
-        <v>116.23</v>
+        <v>118.08</v>
       </c>
       <c r="BA62" t="n">
         <v>34.09</v>
@@ -14742,19 +14742,19 @@
         <v>76.01000000000001</v>
       </c>
       <c r="BC62" t="n">
-        <v>197.5</v>
+        <v>192.84</v>
       </c>
       <c r="BD62" t="n">
-        <v>142.91</v>
+        <v>139.1</v>
       </c>
       <c r="BE62" t="n">
         <v>5.67</v>
       </c>
       <c r="BF62" t="n">
-        <v>-69.01000000000001</v>
+        <v>-69.48999999999999</v>
       </c>
       <c r="BG62" t="n">
-        <v>-30.9</v>
+        <v>-31.98</v>
       </c>
       <c r="BH62" t="n">
         <v>170.35</v>
@@ -14763,7 +14763,7 @@
         <v>0</v>
       </c>
       <c r="BJ62" t="n">
-        <v>110</v>
+        <v>111.75</v>
       </c>
       <c r="BK62" t="n">
         <v>27.94</v>
@@ -14772,7 +14772,7 @@
         <v>32.73</v>
       </c>
       <c r="BM62" t="n">
-        <v>110</v>
+        <v>111.75</v>
       </c>
       <c r="BN62" t="n">
         <v>122.2</v>
@@ -14781,19 +14781,19 @@
         <v>91.84999999999999</v>
       </c>
       <c r="BP62" t="n">
-        <v>110</v>
+        <v>109.01</v>
       </c>
       <c r="BQ62" t="n">
-        <v>3.36</v>
+        <v>3.41</v>
       </c>
       <c r="BR62" t="n">
-        <v>110</v>
+        <v>109.01</v>
       </c>
       <c r="BS62" t="n">
         <v>1.01</v>
       </c>
       <c r="BT62" t="n">
-        <v>143</v>
+        <v>150</v>
       </c>
     </row>
     <row r="63">
@@ -14823,13 +14823,13 @@
         </is>
       </c>
       <c r="F63" t="n">
-        <v>1.35</v>
+        <v>1.38</v>
       </c>
       <c r="G63" t="n">
-        <v>351688101</v>
+        <v>359503384</v>
       </c>
       <c r="H63" t="n">
-        <v>2400</v>
+        <v>4000</v>
       </c>
       <c r="I63" t="n">
         <v>122894462</v>
@@ -14844,7 +14844,7 @@
         <v>-0.22</v>
       </c>
       <c r="M63" t="n">
-        <v>0.4325582149722281</v>
+        <v>0.4421706097458084</v>
       </c>
       <c r="N63" t="n">
         <v>0.37</v>
@@ -14922,7 +14922,7 @@
         <v>31952560.12</v>
       </c>
       <c r="AM63" t="n">
-        <v>199822784.6590909</v>
+        <v>204263286.3636364</v>
       </c>
       <c r="AN63" t="n">
         <v>0</v>
@@ -14981,7 +14981,7 @@
         <v>-100</v>
       </c>
       <c r="BF63" t="n">
-        <v>-78.58</v>
+        <v>-79.05</v>
       </c>
       <c r="BG63" t="n">
         <v>-100</v>
@@ -14993,7 +14993,7 @@
         <v>0</v>
       </c>
       <c r="BJ63" t="n">
-        <v>1.35</v>
+        <v>1.38</v>
       </c>
       <c r="BK63" t="n">
         <v>0.26</v>
@@ -15002,7 +15002,7 @@
         <v>0.26</v>
       </c>
       <c r="BM63" t="n">
-        <v>1.36</v>
+        <v>1.42</v>
       </c>
       <c r="BN63" t="n">
         <v>2.12</v>
@@ -15014,16 +15014,16 @@
         <v>1.35</v>
       </c>
       <c r="BQ63" t="n">
-        <v>5.17</v>
+        <v>5.29</v>
       </c>
       <c r="BR63" t="n">
-        <v>1.36</v>
+        <v>1.35</v>
       </c>
       <c r="BS63" t="n">
         <v>0.19</v>
       </c>
       <c r="BT63" t="n">
-        <v>27227</v>
+        <v>25973</v>
       </c>
     </row>
     <row r="64">
@@ -15053,13 +15053,13 @@
         </is>
       </c>
       <c r="F64" t="n">
-        <v>63.65</v>
+        <v>62.7</v>
       </c>
       <c r="G64" t="n">
-        <v>236396551217</v>
+        <v>235893892970</v>
       </c>
       <c r="H64" t="n">
-        <v>11058500</v>
+        <v>9817700</v>
       </c>
       <c r="I64" t="n">
         <v>0</v>
@@ -15146,13 +15146,13 @@
         <v>41.22</v>
       </c>
       <c r="AK64" t="n">
-        <v>67778360157.49811</v>
+        <v>67634240661.98978</v>
       </c>
       <c r="AL64" t="n">
-        <v>18896606811.91047</v>
+        <v>18856426296.56275</v>
       </c>
       <c r="AM64" t="n">
-        <v>21050449796.70525</v>
+        <v>21005689489.75957</v>
       </c>
       <c r="AN64" t="n">
         <v>1.4201</v>
@@ -15193,7 +15193,7 @@
         <v>38.98</v>
       </c>
       <c r="AZ64" t="n">
-        <v>25.46</v>
+        <v>25.08</v>
       </c>
       <c r="BA64" t="n">
         <v>6.69</v>
@@ -15202,19 +15202,19 @@
         <v>10.4</v>
       </c>
       <c r="BC64" t="n">
-        <v>-25</v>
+        <v>-23.86</v>
       </c>
       <c r="BD64" t="n">
-        <v>-38.76</v>
+        <v>-37.83</v>
       </c>
       <c r="BE64" t="n">
         <v>-60</v>
       </c>
       <c r="BF64" t="n">
-        <v>-89.48</v>
+        <v>-89.31999999999999</v>
       </c>
       <c r="BG64" t="n">
-        <v>-83.66</v>
+        <v>-83.42</v>
       </c>
       <c r="BH64" t="n">
         <v>21.37</v>
@@ -15223,7 +15223,7 @@
         <v>0</v>
       </c>
       <c r="BJ64" t="n">
-        <v>63.65</v>
+        <v>62.7</v>
       </c>
       <c r="BK64" t="n">
         <v>4.74</v>
@@ -15232,7 +15232,7 @@
         <v>1.57</v>
       </c>
       <c r="BM64" t="n">
-        <v>64.31999999999999</v>
+        <v>63.86</v>
       </c>
       <c r="BN64" t="n">
         <v>64.72</v>
@@ -15241,19 +15241,19 @@
         <v>44.12</v>
       </c>
       <c r="BP64" t="n">
-        <v>63.07</v>
+        <v>62.5</v>
       </c>
       <c r="BQ64" t="n">
-        <v>40.54</v>
+        <v>39.93</v>
       </c>
       <c r="BR64" t="n">
-        <v>63.58</v>
+        <v>63.83</v>
       </c>
       <c r="BS64" t="n">
         <v>3.49</v>
       </c>
       <c r="BT64" t="n">
-        <v>12220037</v>
+        <v>11307657</v>
       </c>
     </row>
     <row r="65">
@@ -15283,13 +15283,13 @@
         </is>
       </c>
       <c r="F65" t="n">
-        <v>24.42</v>
+        <v>24.3</v>
       </c>
       <c r="G65" t="n">
-        <v>236396551217</v>
+        <v>235893892970</v>
       </c>
       <c r="H65" t="n">
-        <v>2800</v>
+        <v>6800</v>
       </c>
       <c r="I65" t="n">
         <v>7298813414</v>
@@ -15304,7 +15304,7 @@
         <v>3.29</v>
       </c>
       <c r="M65" t="n">
-        <v>5.715109519701055</v>
+        <v>5.702957282632465</v>
       </c>
       <c r="N65" t="n">
         <v>0.29</v>
@@ -15382,7 +15382,7 @@
         <v>11532125194.12</v>
       </c>
       <c r="AM65" t="n">
-        <v>17707606832.73408</v>
+        <v>17669954529.58802</v>
       </c>
       <c r="AN65" t="n">
         <v>0.4734</v>
@@ -15423,7 +15423,7 @@
         <v>12.99</v>
       </c>
       <c r="AZ65" t="n">
-        <v>8.220000000000001</v>
+        <v>8.18</v>
       </c>
       <c r="BA65" t="n">
         <v>2.23</v>
@@ -15432,19 +15432,19 @@
         <v>3.47</v>
       </c>
       <c r="BC65" t="n">
-        <v>-34.85</v>
+        <v>-34.53</v>
       </c>
       <c r="BD65" t="n">
-        <v>-46.81</v>
+        <v>-46.54</v>
       </c>
       <c r="BE65" t="n">
         <v>-66.33</v>
       </c>
       <c r="BF65" t="n">
-        <v>-90.86</v>
+        <v>-90.81999999999999</v>
       </c>
       <c r="BG65" t="n">
-        <v>-85.81</v>
+        <v>-85.73999999999999</v>
       </c>
       <c r="BH65" t="n">
         <v>7.12</v>
@@ -15453,7 +15453,7 @@
         <v>0</v>
       </c>
       <c r="BJ65" t="n">
-        <v>24.42</v>
+        <v>24.3</v>
       </c>
       <c r="BK65" t="n">
         <v>1.58</v>
@@ -15462,7 +15462,7 @@
         <v>1.57</v>
       </c>
       <c r="BM65" t="n">
-        <v>24.89</v>
+        <v>24.99</v>
       </c>
       <c r="BN65" t="n">
         <v>46.43</v>
@@ -15471,19 +15471,19 @@
         <v>20.44</v>
       </c>
       <c r="BP65" t="n">
-        <v>24.05</v>
+        <v>24.14</v>
       </c>
       <c r="BQ65" t="n">
-        <v>15.55</v>
+        <v>15.48</v>
       </c>
       <c r="BR65" t="n">
-        <v>24.27</v>
+        <v>24.78</v>
       </c>
       <c r="BS65" t="n">
         <v>4.14</v>
       </c>
       <c r="BT65" t="n">
-        <v>10510</v>
+        <v>9577</v>
       </c>
     </row>
     <row r="66">
@@ -15513,13 +15513,13 @@
         </is>
       </c>
       <c r="F66" t="n">
-        <v>20.59</v>
+        <v>20.6</v>
       </c>
       <c r="G66" t="n">
-        <v>236396551217</v>
+        <v>235893892970</v>
       </c>
       <c r="H66" t="n">
-        <v>900</v>
+        <v>500</v>
       </c>
       <c r="I66" t="n">
         <v>2972355254</v>
@@ -15534,7 +15534,7 @@
         <v>2.75</v>
       </c>
       <c r="M66" t="n">
-        <v>14.03382653158227</v>
+        <v>14.00398591585945</v>
       </c>
       <c r="N66" t="n">
         <v>0.25</v>
@@ -15612,7 +15612,7 @@
         <v>4696321301.320001</v>
       </c>
       <c r="AM66" t="n">
-        <v>21201484414.08072</v>
+        <v>21156402956.95067</v>
       </c>
       <c r="AN66" t="n">
         <v>0.4734</v>
@@ -15662,19 +15662,19 @@
         <v>3.47</v>
       </c>
       <c r="BC66" t="n">
-        <v>-22.73</v>
+        <v>-22.77</v>
       </c>
       <c r="BD66" t="n">
-        <v>-36.91</v>
+        <v>-36.94</v>
       </c>
       <c r="BE66" t="n">
         <v>-59.83</v>
       </c>
       <c r="BF66" t="n">
-        <v>-89.16</v>
+        <v>-89.17</v>
       </c>
       <c r="BG66" t="n">
-        <v>-83.17</v>
+        <v>-83.18000000000001</v>
       </c>
       <c r="BH66" t="n">
         <v>7.12</v>
@@ -15683,7 +15683,7 @@
         <v>0</v>
       </c>
       <c r="BJ66" t="n">
-        <v>20.59</v>
+        <v>20.6</v>
       </c>
       <c r="BK66" t="n">
         <v>1.58</v>
@@ -15692,7 +15692,7 @@
         <v>1.57</v>
       </c>
       <c r="BM66" t="n">
-        <v>20.59</v>
+        <v>20.6</v>
       </c>
       <c r="BN66" t="n">
         <v>21.33</v>
@@ -15701,19 +15701,19 @@
         <v>9.48</v>
       </c>
       <c r="BP66" t="n">
-        <v>20.03</v>
+        <v>20.59</v>
       </c>
       <c r="BQ66" t="n">
-        <v>13.11</v>
+        <v>13.12</v>
       </c>
       <c r="BR66" t="n">
-        <v>20.03</v>
+        <v>20.59</v>
       </c>
       <c r="BS66" t="n">
         <v>3.46</v>
       </c>
       <c r="BT66" t="n">
-        <v>5560</v>
+        <v>4727</v>
       </c>
     </row>
     <row r="67">
@@ -15973,13 +15973,13 @@
         </is>
       </c>
       <c r="F68" t="n">
-        <v>18.11</v>
+        <v>17.93</v>
       </c>
       <c r="G68" t="n">
-        <v>7727860905</v>
+        <v>7663690078</v>
       </c>
       <c r="H68" t="n">
-        <v>112800</v>
+        <v>52300</v>
       </c>
       <c r="I68" t="n">
         <v>137989898</v>
@@ -16072,7 +16072,7 @@
         <v>205604948.02</v>
       </c>
       <c r="AM68" t="n">
-        <v>535912684.1192788</v>
+        <v>531462557.4202496</v>
       </c>
       <c r="AN68" t="n">
         <v>0.1911</v>
@@ -16113,7 +16113,7 @@
         <v>21.39</v>
       </c>
       <c r="AZ68" t="n">
-        <v>33.5</v>
+        <v>33.17</v>
       </c>
       <c r="BA68" t="n">
         <v>1.24</v>
@@ -16122,19 +16122,19 @@
         <v>63.25</v>
       </c>
       <c r="BC68" t="n">
-        <v>44.69</v>
+        <v>46.14</v>
       </c>
       <c r="BD68" t="n">
-        <v>18.14</v>
+        <v>19.32</v>
       </c>
       <c r="BE68" t="n">
         <v>85</v>
       </c>
       <c r="BF68" t="n">
-        <v>-93.16</v>
+        <v>-93.09</v>
       </c>
       <c r="BG68" t="n">
-        <v>249.25</v>
+        <v>252.75</v>
       </c>
       <c r="BH68" t="n">
         <v>20.48</v>
@@ -16143,7 +16143,7 @@
         <v>0</v>
       </c>
       <c r="BJ68" t="n">
-        <v>18.11</v>
+        <v>17.93</v>
       </c>
       <c r="BK68" t="n">
         <v>1.49</v>
@@ -16152,7 +16152,7 @@
         <v>1.49</v>
       </c>
       <c r="BM68" t="n">
-        <v>18.8</v>
+        <v>18.27</v>
       </c>
       <c r="BN68" t="n">
         <v>22.11</v>
@@ -16161,19 +16161,19 @@
         <v>15.39</v>
       </c>
       <c r="BP68" t="n">
-        <v>18.11</v>
+        <v>17.91</v>
       </c>
       <c r="BQ68" t="n">
-        <v>12.18</v>
+        <v>12.06</v>
       </c>
       <c r="BR68" t="n">
-        <v>18.8</v>
+        <v>18.22</v>
       </c>
       <c r="BS68" t="n">
         <v>0</v>
       </c>
       <c r="BT68" t="n">
-        <v>36243</v>
+        <v>39323</v>
       </c>
     </row>
     <row r="69">
@@ -16203,13 +16203,13 @@
         </is>
       </c>
       <c r="F69" t="n">
-        <v>20.57</v>
+        <v>20.35</v>
       </c>
       <c r="G69" t="n">
-        <v>7727860905</v>
+        <v>7663690078</v>
       </c>
       <c r="H69" t="n">
-        <v>3737300</v>
+        <v>1660000</v>
       </c>
       <c r="I69" t="n">
         <v>255106712</v>
@@ -16302,7 +16302,7 @@
         <v>380109000.88</v>
       </c>
       <c r="AM69" t="n">
-        <v>459991720.5357143</v>
+        <v>456172028.452381</v>
       </c>
       <c r="AN69" t="n">
         <v>0.8856000000000001</v>
@@ -16343,7 +16343,7 @@
         <v>21.39</v>
       </c>
       <c r="AZ69" t="n">
-        <v>35.96</v>
+        <v>35.58</v>
       </c>
       <c r="BA69" t="n">
         <v>1.24</v>
@@ -16352,19 +16352,19 @@
         <v>69.59</v>
       </c>
       <c r="BC69" t="n">
-        <v>27.38</v>
+        <v>28.76</v>
       </c>
       <c r="BD69" t="n">
-        <v>4.01</v>
+        <v>5.13</v>
       </c>
       <c r="BE69" t="n">
         <v>74.83</v>
       </c>
       <c r="BF69" t="n">
-        <v>-93.97</v>
+        <v>-93.91</v>
       </c>
       <c r="BG69" t="n">
-        <v>238.29</v>
+        <v>241.95</v>
       </c>
       <c r="BH69" t="n">
         <v>20.48</v>
@@ -16373,7 +16373,7 @@
         <v>0</v>
       </c>
       <c r="BJ69" t="n">
-        <v>20.57</v>
+        <v>20.35</v>
       </c>
       <c r="BK69" t="n">
         <v>1.49</v>
@@ -16382,7 +16382,7 @@
         <v>1.49</v>
       </c>
       <c r="BM69" t="n">
-        <v>21.15</v>
+        <v>20.63</v>
       </c>
       <c r="BN69" t="n">
         <v>25.63</v>
@@ -16391,19 +16391,19 @@
         <v>16.73</v>
       </c>
       <c r="BP69" t="n">
-        <v>20.57</v>
+        <v>20.3</v>
       </c>
       <c r="BQ69" t="n">
-        <v>13.84</v>
+        <v>13.69</v>
       </c>
       <c r="BR69" t="n">
-        <v>21.14</v>
+        <v>20.62</v>
       </c>
       <c r="BS69" t="n">
         <v>0</v>
       </c>
       <c r="BT69" t="n">
-        <v>2027813</v>
+        <v>2103810</v>
       </c>
     </row>
     <row r="70">
@@ -16433,13 +16433,13 @@
         </is>
       </c>
       <c r="F70" t="n">
-        <v>17.6</v>
+        <v>17.48</v>
       </c>
       <c r="G70" t="n">
-        <v>8176206897</v>
+        <v>8120459643</v>
       </c>
       <c r="H70" t="n">
-        <v>2251900</v>
+        <v>1398600</v>
       </c>
       <c r="I70" t="n">
         <v>464557268</v>
@@ -16454,7 +16454,7 @@
         <v>0.68</v>
       </c>
       <c r="M70" t="n">
-        <v>0.6453332528423601</v>
+        <v>0.640933222704418</v>
       </c>
       <c r="N70" t="n">
         <v>0.2</v>
@@ -16532,7 +16532,7 @@
         <v>55746872.16</v>
       </c>
       <c r="AM70" t="n">
-        <v>2698418117.821783</v>
+        <v>2680019684.158416</v>
       </c>
       <c r="AN70" t="n">
         <v>0.1236</v>
@@ -16573,7 +16573,7 @@
         <v>6.9</v>
       </c>
       <c r="AZ70" t="n">
-        <v>2.02</v>
+        <v>2.01</v>
       </c>
       <c r="BA70" t="n">
         <v>0.12</v>
@@ -16582,19 +16582,19 @@
         <v>1.07</v>
       </c>
       <c r="BC70" t="n">
-        <v>-51.99</v>
+        <v>-51.66</v>
       </c>
       <c r="BD70" t="n">
-        <v>-60.8</v>
+        <v>-60.53</v>
       </c>
       <c r="BE70" t="n">
         <v>-88.5</v>
       </c>
       <c r="BF70" t="n">
-        <v>-99.31999999999999</v>
+        <v>-99.31</v>
       </c>
       <c r="BG70" t="n">
-        <v>-93.92</v>
+        <v>-93.88</v>
       </c>
       <c r="BH70" t="n">
         <v>26.44</v>
@@ -16603,7 +16603,7 @@
         <v>0</v>
       </c>
       <c r="BJ70" t="n">
-        <v>17.6</v>
+        <v>17.48</v>
       </c>
       <c r="BK70" t="n">
         <v>0.12</v>
@@ -16612,7 +16612,7 @@
         <v>0.1</v>
       </c>
       <c r="BM70" t="n">
-        <v>18.02</v>
+        <v>17.75</v>
       </c>
       <c r="BN70" t="n">
         <v>22.15</v>
@@ -16621,19 +16621,19 @@
         <v>13.21</v>
       </c>
       <c r="BP70" t="n">
-        <v>17.57</v>
+        <v>17.48</v>
       </c>
       <c r="BQ70" t="n">
-        <v>176.51</v>
+        <v>175.31</v>
       </c>
       <c r="BR70" t="n">
-        <v>17.8</v>
+        <v>17.65</v>
       </c>
       <c r="BS70" t="n">
         <v>0.67</v>
       </c>
       <c r="BT70" t="n">
-        <v>4292827</v>
+        <v>4206477</v>
       </c>
     </row>
     <row r="71">

</xml_diff>

<commit_message>
📊 Dados atualizados - 2026-09-26 05:44
</commit_message>
<xml_diff>
--- a/data/ativos.xlsx
+++ b/data/ativos.xlsx
@@ -1047,13 +1047,13 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>24.76</v>
+        <v>24.69</v>
       </c>
       <c r="G3" t="n">
-        <v>3312068474</v>
+        <v>3302702363</v>
       </c>
       <c r="H3" t="n">
-        <v>309400</v>
+        <v>210500</v>
       </c>
       <c r="I3" t="n">
         <v>129510368</v>
@@ -1068,7 +1068,7 @@
         <v>0.88</v>
       </c>
       <c r="M3" t="n">
-        <v>0.8241164008099646</v>
+        <v>0.8217859037965425</v>
       </c>
       <c r="N3" t="n">
         <v>0.09</v>
@@ -1146,7 +1146,7 @@
         <v>506385538.88</v>
       </c>
       <c r="AM3" t="n">
-        <v>646888373.828125</v>
+        <v>645059055.2734375</v>
       </c>
       <c r="AN3" t="n">
         <v>2.7</v>
@@ -1187,7 +1187,7 @@
         <v>40.42</v>
       </c>
       <c r="AZ3" t="n">
-        <v>45.31</v>
+        <v>45.18</v>
       </c>
       <c r="BA3" t="n">
         <v>4.87</v>
@@ -1196,19 +1196,19 @@
         <v>21.14</v>
       </c>
       <c r="BC3" t="n">
-        <v>99.91</v>
+        <v>100.48</v>
       </c>
       <c r="BD3" t="n">
-        <v>63.23</v>
+        <v>63.69</v>
       </c>
       <c r="BE3" t="n">
         <v>83</v>
       </c>
       <c r="BF3" t="n">
-        <v>-80.34</v>
+        <v>-80.28</v>
       </c>
       <c r="BG3" t="n">
-        <v>-14.64</v>
+        <v>-14.4</v>
       </c>
       <c r="BH3" t="n">
         <v>27.85</v>
@@ -1217,7 +1217,7 @@
         <v>0</v>
       </c>
       <c r="BJ3" t="n">
-        <v>24.76</v>
+        <v>24.69</v>
       </c>
       <c r="BK3" t="n">
         <v>3.91</v>
@@ -1226,7 +1226,7 @@
         <v>4.39</v>
       </c>
       <c r="BM3" t="n">
-        <v>25.04</v>
+        <v>24.92</v>
       </c>
       <c r="BN3" t="n">
         <v>27.17</v>
@@ -1238,16 +1238,16 @@
         <v>24.62</v>
       </c>
       <c r="BQ3" t="n">
-        <v>5.64</v>
+        <v>5.62</v>
       </c>
       <c r="BR3" t="n">
-        <v>24.9</v>
+        <v>24.89</v>
       </c>
       <c r="BS3" t="n">
         <v>0.79</v>
       </c>
       <c r="BT3" t="n">
-        <v>522973</v>
+        <v>519427</v>
       </c>
     </row>
     <row r="4">
@@ -1277,13 +1277,13 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>15.34</v>
+        <v>15.32</v>
       </c>
       <c r="G4" t="n">
-        <v>237534686762</v>
+        <v>237224986474</v>
       </c>
       <c r="H4" t="n">
-        <v>15784900</v>
+        <v>12323400</v>
       </c>
       <c r="I4" t="n">
         <v>15484664889</v>
@@ -1298,7 +1298,7 @@
         <v>2.76</v>
       </c>
       <c r="M4" t="n">
-        <v>2.689612510882067</v>
+        <v>2.686105765064926</v>
       </c>
       <c r="N4" t="n">
         <v>1.76</v>
@@ -1376,7 +1376,7 @@
         <v>16258898133.45</v>
       </c>
       <c r="AM4" t="n">
-        <v>23518285818.0198</v>
+        <v>23487622423.16832</v>
       </c>
       <c r="AN4" t="n">
         <v>0.269</v>
@@ -1417,7 +1417,7 @@
         <v>9.470000000000001</v>
       </c>
       <c r="AZ4" t="n">
-        <v>19.15</v>
+        <v>19.12</v>
       </c>
       <c r="BA4" t="n">
         <v>1.13</v>
@@ -1426,19 +1426,19 @@
         <v>11.39</v>
       </c>
       <c r="BC4" t="n">
-        <v>-24.35</v>
+        <v>-24.25</v>
       </c>
       <c r="BD4" t="n">
-        <v>-38.23</v>
+        <v>-38.15</v>
       </c>
       <c r="BE4" t="n">
         <v>24.83</v>
       </c>
       <c r="BF4" t="n">
-        <v>-92.65000000000001</v>
+        <v>-92.64</v>
       </c>
       <c r="BG4" t="n">
-        <v>-25.77</v>
+        <v>-25.67</v>
       </c>
       <c r="BH4" t="n">
         <v>5.7</v>
@@ -1447,7 +1447,7 @@
         <v>0</v>
       </c>
       <c r="BJ4" t="n">
-        <v>15.34</v>
+        <v>15.32</v>
       </c>
       <c r="BK4" t="n">
         <v>1.05</v>
@@ -1456,7 +1456,7 @@
         <v>1.04</v>
       </c>
       <c r="BM4" t="n">
-        <v>15.55</v>
+        <v>15.39</v>
       </c>
       <c r="BN4" t="n">
         <v>16.94</v>
@@ -1465,19 +1465,19 @@
         <v>11.04</v>
       </c>
       <c r="BP4" t="n">
-        <v>15.31</v>
+        <v>15.21</v>
       </c>
       <c r="BQ4" t="n">
-        <v>14.79</v>
+        <v>14.77</v>
       </c>
       <c r="BR4" t="n">
-        <v>15.35</v>
+        <v>15.3</v>
       </c>
       <c r="BS4" t="n">
         <v>2.76</v>
       </c>
       <c r="BT4" t="n">
-        <v>27496667</v>
+        <v>27122850</v>
       </c>
     </row>
     <row r="5">
@@ -3117,13 +3117,13 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>4.89</v>
+        <v>4.97</v>
       </c>
       <c r="G12" t="n">
-        <v>469251868</v>
+        <v>476928783</v>
       </c>
       <c r="H12" t="n">
-        <v>571400</v>
+        <v>464100</v>
       </c>
       <c r="I12" t="n">
         <v>95961536</v>
@@ -3138,7 +3138,7 @@
         <v>0.32</v>
       </c>
       <c r="M12" t="n">
-        <v>0.08486348427977373</v>
+        <v>0.08625184264304754</v>
       </c>
       <c r="N12" t="n">
         <v>0.14</v>
@@ -3216,7 +3216,7 @@
         <v>362734606.08</v>
       </c>
       <c r="AM12" t="n">
-        <v>504571901.0752688</v>
+        <v>512826648.3870968</v>
       </c>
       <c r="AN12" t="n">
         <v>0.4208</v>
@@ -3257,7 +3257,7 @@
         <v>30.49</v>
       </c>
       <c r="AZ12" t="n">
-        <v>6.61</v>
+        <v>6.72</v>
       </c>
       <c r="BA12" t="n">
         <v>4.41</v>
@@ -3266,19 +3266,19 @@
         <v>18.12</v>
       </c>
       <c r="BC12" t="n">
-        <v>663.75</v>
+        <v>651.45</v>
       </c>
       <c r="BD12" t="n">
-        <v>523.6</v>
+        <v>513.5599999999999</v>
       </c>
       <c r="BE12" t="n">
         <v>35.17</v>
       </c>
       <c r="BF12" t="n">
-        <v>-9.779999999999999</v>
+        <v>-11.23</v>
       </c>
       <c r="BG12" t="n">
-        <v>270.53</v>
+        <v>264.57</v>
       </c>
       <c r="BH12" t="n">
         <v>16.4</v>
@@ -3287,7 +3287,7 @@
         <v>0</v>
       </c>
       <c r="BJ12" t="n">
-        <v>4.89</v>
+        <v>4.97</v>
       </c>
       <c r="BK12" t="n">
         <v>3.78</v>
@@ -3296,7 +3296,7 @@
         <v>3.43</v>
       </c>
       <c r="BM12" t="n">
-        <v>4.96</v>
+        <v>4.99</v>
       </c>
       <c r="BN12" t="n">
         <v>8.23</v>
@@ -3305,19 +3305,19 @@
         <v>4.42</v>
       </c>
       <c r="BP12" t="n">
-        <v>4.84</v>
+        <v>4.85</v>
       </c>
       <c r="BQ12" t="n">
-        <v>1.43</v>
+        <v>1.45</v>
       </c>
       <c r="BR12" t="n">
-        <v>4.95</v>
+        <v>4.89</v>
       </c>
       <c r="BS12" t="n">
         <v>0.09</v>
       </c>
       <c r="BT12" t="n">
-        <v>521930</v>
+        <v>535617</v>
       </c>
     </row>
     <row r="13">
@@ -3347,13 +3347,13 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>29.12</v>
+        <v>28.98</v>
       </c>
       <c r="G13" t="n">
-        <v>14682036519</v>
+        <v>14611452051</v>
       </c>
       <c r="H13" t="n">
-        <v>3664800</v>
+        <v>2778400</v>
       </c>
       <c r="I13" t="n">
         <v>504190947</v>
@@ -3368,7 +3368,7 @@
         <v>1.13</v>
       </c>
       <c r="M13" t="n">
-        <v>5.077897044183444</v>
+        <v>5.053484854433157</v>
       </c>
       <c r="N13" t="n">
         <v>0.57</v>
@@ -3446,7 +3446,7 @@
         <v>932753251.95</v>
       </c>
       <c r="AM13" t="n">
-        <v>1527787358.896982</v>
+        <v>1520442461.082206</v>
       </c>
       <c r="AN13" t="n">
         <v>2.6301</v>
@@ -3487,7 +3487,7 @@
         <v>26.6</v>
       </c>
       <c r="AZ13" t="n">
-        <v>52.71</v>
+        <v>52.45</v>
       </c>
       <c r="BA13" t="n">
         <v>2.6</v>
@@ -3496,19 +3496,19 @@
         <v>8.69</v>
       </c>
       <c r="BC13" t="n">
-        <v>11.86</v>
+        <v>12.4</v>
       </c>
       <c r="BD13" t="n">
-        <v>-8.67</v>
+        <v>-8.23</v>
       </c>
       <c r="BE13" t="n">
         <v>81</v>
       </c>
       <c r="BF13" t="n">
-        <v>-91.06</v>
+        <v>-91.01000000000001</v>
       </c>
       <c r="BG13" t="n">
-        <v>-70.14</v>
+        <v>-70</v>
       </c>
       <c r="BH13" t="n">
         <v>25.49</v>
@@ -3517,7 +3517,7 @@
         <v>0</v>
       </c>
       <c r="BJ13" t="n">
-        <v>29.12</v>
+        <v>28.98</v>
       </c>
       <c r="BK13" t="n">
         <v>1.85</v>
@@ -3526,7 +3526,7 @@
         <v>1.96</v>
       </c>
       <c r="BM13" t="n">
-        <v>29.49</v>
+        <v>29.31</v>
       </c>
       <c r="BN13" t="n">
         <v>32.11</v>
@@ -3535,19 +3535,19 @@
         <v>20.85</v>
       </c>
       <c r="BP13" t="n">
-        <v>28.87</v>
+        <v>28.59</v>
       </c>
       <c r="BQ13" t="n">
-        <v>14.88</v>
+        <v>14.81</v>
       </c>
       <c r="BR13" t="n">
-        <v>29.49</v>
+        <v>29.04</v>
       </c>
       <c r="BS13" t="n">
         <v>5.01</v>
       </c>
       <c r="BT13" t="n">
-        <v>4984300</v>
+        <v>4968973</v>
       </c>
     </row>
     <row r="14">
@@ -3577,13 +3577,13 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>10.18</v>
+        <v>10.39</v>
       </c>
       <c r="G14" t="n">
-        <v>8047950317</v>
+        <v>8372725593</v>
       </c>
       <c r="H14" t="n">
-        <v>2800</v>
+        <v>3600</v>
       </c>
       <c r="I14" t="n">
         <v>339510689</v>
@@ -3598,7 +3598,7 @@
         <v>1.92</v>
       </c>
       <c r="M14" t="n">
-        <v>3.341652045532762</v>
+        <v>3.47650451388006</v>
       </c>
       <c r="N14" t="n">
         <v>1.11</v>
@@ -3676,7 +3676,7 @@
         <v>349696009.67</v>
       </c>
       <c r="AM14" t="n">
-        <v>893224230.5216427</v>
+        <v>929270321.0876803</v>
       </c>
       <c r="AN14" t="n">
         <v>0.1489</v>
@@ -3717,7 +3717,7 @@
         <v>9.050000000000001</v>
       </c>
       <c r="AZ14" t="n">
-        <v>8.18</v>
+        <v>8.35</v>
       </c>
       <c r="BA14" t="n">
         <v>1.42</v>
@@ -3726,19 +3726,19 @@
         <v>5.94</v>
       </c>
       <c r="BC14" t="n">
-        <v>8.869999999999999</v>
+        <v>6.67</v>
       </c>
       <c r="BD14" t="n">
-        <v>-11.11</v>
+        <v>-12.91</v>
       </c>
       <c r="BE14" t="n">
         <v>-19.67</v>
       </c>
       <c r="BF14" t="n">
-        <v>-86.04000000000001</v>
+        <v>-86.31999999999999</v>
       </c>
       <c r="BG14" t="n">
-        <v>-41.63</v>
+        <v>-42.81</v>
       </c>
       <c r="BH14" t="n">
         <v>5.3</v>
@@ -3747,7 +3747,7 @@
         <v>0</v>
       </c>
       <c r="BJ14" t="n">
-        <v>10.18</v>
+        <v>10.39</v>
       </c>
       <c r="BK14" t="n">
         <v>1.03</v>
@@ -3756,7 +3756,7 @@
         <v>1.01</v>
       </c>
       <c r="BM14" t="n">
-        <v>10.18</v>
+        <v>10.39</v>
       </c>
       <c r="BN14" t="n">
         <v>13.49</v>
@@ -3765,19 +3765,19 @@
         <v>7.65</v>
       </c>
       <c r="BP14" t="n">
-        <v>9.93</v>
+        <v>10.1</v>
       </c>
       <c r="BQ14" t="n">
-        <v>10.05</v>
+        <v>10.26</v>
       </c>
       <c r="BR14" t="n">
-        <v>9.960000000000001</v>
+        <v>10.1</v>
       </c>
       <c r="BS14" t="n">
         <v>1.44</v>
       </c>
       <c r="BT14" t="n">
-        <v>11173</v>
+        <v>10950</v>
       </c>
     </row>
     <row r="15">
@@ -3807,13 +3807,13 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>13.31</v>
+        <v>13.88</v>
       </c>
       <c r="G15" t="n">
-        <v>8047950317</v>
+        <v>8372725593</v>
       </c>
       <c r="H15" t="n">
-        <v>814300</v>
+        <v>1982200</v>
       </c>
       <c r="I15" t="n">
         <v>343551533</v>
@@ -3828,7 +3828,7 @@
         <v>2.56</v>
       </c>
       <c r="M15" t="n">
-        <v>3.302347622989903</v>
+        <v>3.435613960188701</v>
       </c>
       <c r="N15" t="n">
         <v>1.47</v>
@@ -3906,7 +3906,7 @@
         <v>353858078.99</v>
       </c>
       <c r="AM15" t="n">
-        <v>671221877.9816513</v>
+        <v>698309056.9641367</v>
       </c>
       <c r="AN15" t="n">
         <v>0.1638</v>
@@ -3947,7 +3947,7 @@
         <v>9.050000000000001</v>
       </c>
       <c r="AZ15" t="n">
-        <v>8.85</v>
+        <v>9.23</v>
       </c>
       <c r="BA15" t="n">
         <v>1.42</v>
@@ -3956,19 +3956,19 @@
         <v>6.19</v>
       </c>
       <c r="BC15" t="n">
-        <v>-16.73</v>
+        <v>-20.15</v>
       </c>
       <c r="BD15" t="n">
-        <v>-32.01</v>
+        <v>-34.81</v>
       </c>
       <c r="BE15" t="n">
         <v>-33.5</v>
       </c>
       <c r="BF15" t="n">
-        <v>-89.31999999999999</v>
+        <v>-89.76000000000001</v>
       </c>
       <c r="BG15" t="n">
-        <v>-53.51</v>
+        <v>-55.42</v>
       </c>
       <c r="BH15" t="n">
         <v>5.3</v>
@@ -3977,7 +3977,7 @@
         <v>0</v>
       </c>
       <c r="BJ15" t="n">
-        <v>13.31</v>
+        <v>13.88</v>
       </c>
       <c r="BK15" t="n">
         <v>1.03</v>
@@ -3986,7 +3986,7 @@
         <v>1.01</v>
       </c>
       <c r="BM15" t="n">
-        <v>13.5</v>
+        <v>13.93</v>
       </c>
       <c r="BN15" t="n">
         <v>16.22</v>
@@ -3995,19 +3995,19 @@
         <v>7.84</v>
       </c>
       <c r="BP15" t="n">
-        <v>13.13</v>
+        <v>13.31</v>
       </c>
       <c r="BQ15" t="n">
-        <v>13.14</v>
+        <v>13.7</v>
       </c>
       <c r="BR15" t="n">
-        <v>13.19</v>
+        <v>13.32</v>
       </c>
       <c r="BS15" t="n">
         <v>1.92</v>
       </c>
       <c r="BT15" t="n">
-        <v>2361077</v>
+        <v>2353290</v>
       </c>
     </row>
     <row r="16">
@@ -4037,13 +4037,13 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>4.38</v>
+        <v>4.5</v>
       </c>
       <c r="G16" t="n">
-        <v>960558991</v>
+        <v>986875650</v>
       </c>
       <c r="H16" t="n">
-        <v>66600</v>
+        <v>58800</v>
       </c>
       <c r="I16" t="n">
         <v>219305733</v>
@@ -4058,7 +4058,7 @@
         <v>2.69</v>
       </c>
       <c r="M16" t="n">
-        <v>0.4544249434475568</v>
+        <v>0.4668749297470486</v>
       </c>
       <c r="N16" t="n">
         <v>0.39</v>
@@ -4136,7 +4136,7 @@
         <v>17544458.64</v>
       </c>
       <c r="AM16" t="n">
-        <v>269819941.2921348</v>
+        <v>277212261.2359551</v>
       </c>
       <c r="AN16" t="n">
         <v>0.0077</v>
@@ -4177,7 +4177,7 @@
         <v>1.42</v>
       </c>
       <c r="AZ16" t="n">
-        <v>0.12</v>
+        <v>0.13</v>
       </c>
       <c r="BA16" t="n">
         <v>0.08</v>
@@ -4186,16 +4186,16 @@
         <v>0</v>
       </c>
       <c r="BC16" t="n">
-        <v>-60.3</v>
+        <v>-61.36</v>
       </c>
       <c r="BD16" t="n">
-        <v>-67.58</v>
+        <v>-68.45</v>
       </c>
       <c r="BE16" t="n">
         <v>-97.17</v>
       </c>
       <c r="BF16" t="n">
-        <v>-98.17</v>
+        <v>-98.22</v>
       </c>
       <c r="BG16" t="n">
         <v>-100</v>
@@ -4207,7 +4207,7 @@
         <v>0</v>
       </c>
       <c r="BJ16" t="n">
-        <v>4.38</v>
+        <v>4.5</v>
       </c>
       <c r="BK16" t="n">
         <v>0.08</v>
@@ -4216,7 +4216,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="BM16" t="n">
-        <v>4.49</v>
+        <v>4.5</v>
       </c>
       <c r="BN16" t="n">
         <v>5.54</v>
@@ -4228,16 +4228,16 @@
         <v>4.35</v>
       </c>
       <c r="BQ16" t="n">
-        <v>59.77</v>
+        <v>61.41</v>
       </c>
       <c r="BR16" t="n">
-        <v>4.49</v>
+        <v>4.39</v>
       </c>
       <c r="BS16" t="n">
         <v>0.49</v>
       </c>
       <c r="BT16" t="n">
-        <v>136167</v>
+        <v>134720</v>
       </c>
     </row>
     <row r="17">
@@ -4267,13 +4267,13 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>32.05</v>
+        <v>32.11</v>
       </c>
       <c r="G17" t="n">
-        <v>10564541893</v>
+        <v>10584316749</v>
       </c>
       <c r="H17" t="n">
-        <v>1269000</v>
+        <v>986500</v>
       </c>
       <c r="I17" t="n">
         <v>0</v>
@@ -4360,13 +4360,13 @@
         <v>8.039999999999999</v>
       </c>
       <c r="AK17" t="n">
-        <v>4770837198.78974</v>
+        <v>4779767318.009394</v>
       </c>
       <c r="AL17" t="n">
-        <v>1320567736.625</v>
+        <v>1323039593.625</v>
       </c>
       <c r="AM17" t="n">
-        <v>3270756004.024768</v>
+        <v>3276878250.464396</v>
       </c>
       <c r="AN17" t="n">
         <v>1.08</v>
@@ -4407,7 +4407,7 @@
         <v>42.98</v>
       </c>
       <c r="AZ17" t="n">
-        <v>17.15</v>
+        <v>17.18</v>
       </c>
       <c r="BA17" t="n">
         <v>4.55</v>
@@ -4416,19 +4416,19 @@
         <v>16.33</v>
       </c>
       <c r="BC17" t="n">
-        <v>64.23999999999999</v>
+        <v>63.93</v>
       </c>
       <c r="BD17" t="n">
-        <v>34.1</v>
+        <v>33.85</v>
       </c>
       <c r="BE17" t="n">
         <v>-46.5</v>
       </c>
       <c r="BF17" t="n">
-        <v>-85.81</v>
+        <v>-85.83</v>
       </c>
       <c r="BG17" t="n">
-        <v>-49.04</v>
+        <v>-49.13</v>
       </c>
       <c r="BH17" t="n">
         <v>29.25</v>
@@ -4437,7 +4437,7 @@
         <v>0</v>
       </c>
       <c r="BJ17" t="n">
-        <v>32.05</v>
+        <v>32.11</v>
       </c>
       <c r="BK17" t="n">
         <v>4.21</v>
@@ -4446,7 +4446,7 @@
         <v>12.62</v>
       </c>
       <c r="BM17" t="n">
-        <v>32.29</v>
+        <v>32.21</v>
       </c>
       <c r="BN17" t="n">
         <v>36.63</v>
@@ -4455,19 +4455,19 @@
         <v>29.53</v>
       </c>
       <c r="BP17" t="n">
-        <v>31.63</v>
+        <v>31.84</v>
       </c>
       <c r="BQ17" t="n">
         <v>2.54</v>
       </c>
       <c r="BR17" t="n">
-        <v>32.29</v>
+        <v>31.91</v>
       </c>
       <c r="BS17" t="n">
         <v>2.21</v>
       </c>
       <c r="BT17" t="n">
-        <v>1176323</v>
+        <v>1174540</v>
       </c>
     </row>
     <row r="18">
@@ -4497,13 +4497,13 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>10.98</v>
+        <v>11.2</v>
       </c>
       <c r="G18" t="n">
-        <v>10564541893</v>
+        <v>10584316749</v>
       </c>
       <c r="H18" t="n">
-        <v>17700</v>
+        <v>3500</v>
       </c>
       <c r="I18" t="n">
         <v>671494278</v>
@@ -4518,7 +4518,7 @@
         <v>1.2</v>
       </c>
       <c r="M18" t="n">
-        <v>3.110616013727436</v>
+        <v>3.116438507912775</v>
       </c>
       <c r="N18" t="n">
         <v>0.33</v>
@@ -4596,7 +4596,7 @@
         <v>940091989.1999999</v>
       </c>
       <c r="AM18" t="n">
-        <v>3144208896.726191</v>
+        <v>3150094270.535715</v>
       </c>
       <c r="AN18" t="n">
         <v>0.36</v>
@@ -4637,7 +4637,7 @@
         <v>14.31</v>
       </c>
       <c r="AZ18" t="n">
-        <v>5.65</v>
+        <v>5.77</v>
       </c>
       <c r="BA18" t="n">
         <v>1.51</v>
@@ -4646,19 +4646,19 @@
         <v>5.44</v>
       </c>
       <c r="BC18" t="n">
-        <v>59.61</v>
+        <v>56.47</v>
       </c>
       <c r="BD18" t="n">
-        <v>30.32</v>
+        <v>27.76</v>
       </c>
       <c r="BE18" t="n">
         <v>-48.5</v>
       </c>
       <c r="BF18" t="n">
-        <v>-86.22</v>
+        <v>-86.5</v>
       </c>
       <c r="BG18" t="n">
-        <v>-50.41</v>
+        <v>-51.39</v>
       </c>
       <c r="BH18" t="n">
         <v>9.75</v>
@@ -4667,7 +4667,7 @@
         <v>0</v>
       </c>
       <c r="BJ18" t="n">
-        <v>10.98</v>
+        <v>11.2</v>
       </c>
       <c r="BK18" t="n">
         <v>1.4</v>
@@ -4676,7 +4676,7 @@
         <v>12.62</v>
       </c>
       <c r="BM18" t="n">
-        <v>11.07</v>
+        <v>11.2</v>
       </c>
       <c r="BN18" t="n">
         <v>13.82</v>
@@ -4685,19 +4685,19 @@
         <v>10.19</v>
       </c>
       <c r="BP18" t="n">
-        <v>10.9</v>
+        <v>10.99</v>
       </c>
       <c r="BQ18" t="n">
-        <v>0.87</v>
+        <v>0.89</v>
       </c>
       <c r="BR18" t="n">
-        <v>11.04</v>
+        <v>11.18</v>
       </c>
       <c r="BS18" t="n">
         <v>2.3</v>
       </c>
       <c r="BT18" t="n">
-        <v>10050</v>
+        <v>10457</v>
       </c>
     </row>
     <row r="19">
@@ -4727,13 +4727,13 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>10.4</v>
+        <v>10.53</v>
       </c>
       <c r="G19" t="n">
-        <v>10564541893</v>
+        <v>10584316749</v>
       </c>
       <c r="H19" t="n">
-        <v>34300</v>
+        <v>3900</v>
       </c>
       <c r="I19" t="n">
         <v>317386323</v>
@@ -4748,7 +4748,7 @@
         <v>1.12</v>
       </c>
       <c r="M19" t="n">
-        <v>6.581130637671312</v>
+        <v>6.593449289250835</v>
       </c>
       <c r="N19" t="n">
         <v>0.3</v>
@@ -4826,7 +4826,7 @@
         <v>444340852.2</v>
       </c>
       <c r="AM19" t="n">
-        <v>3353822823.174603</v>
+        <v>3360100555.238095</v>
       </c>
       <c r="AN19" t="n">
         <v>0.36</v>
@@ -4867,7 +4867,7 @@
         <v>14.31</v>
       </c>
       <c r="AZ19" t="n">
-        <v>5.72</v>
+        <v>5.79</v>
       </c>
       <c r="BA19" t="n">
         <v>1.51</v>
@@ -4876,19 +4876,19 @@
         <v>5.25</v>
       </c>
       <c r="BC19" t="n">
-        <v>68.51000000000001</v>
+        <v>66.43000000000001</v>
       </c>
       <c r="BD19" t="n">
-        <v>37.59</v>
+        <v>35.89</v>
       </c>
       <c r="BE19" t="n">
         <v>-45</v>
       </c>
       <c r="BF19" t="n">
-        <v>-85.45999999999999</v>
+        <v>-85.64</v>
       </c>
       <c r="BG19" t="n">
-        <v>-49.52</v>
+        <v>-50.14</v>
       </c>
       <c r="BH19" t="n">
         <v>9.75</v>
@@ -4897,7 +4897,7 @@
         <v>0</v>
       </c>
       <c r="BJ19" t="n">
-        <v>10.4</v>
+        <v>10.53</v>
       </c>
       <c r="BK19" t="n">
         <v>1.4</v>
@@ -4906,7 +4906,7 @@
         <v>12.62</v>
       </c>
       <c r="BM19" t="n">
-        <v>10.62</v>
+        <v>10.57</v>
       </c>
       <c r="BN19" t="n">
         <v>11.41</v>
@@ -4915,19 +4915,19 @@
         <v>9.19</v>
       </c>
       <c r="BP19" t="n">
-        <v>10.38</v>
+        <v>10.4</v>
       </c>
       <c r="BQ19" t="n">
-        <v>0.82</v>
+        <v>0.83</v>
       </c>
       <c r="BR19" t="n">
-        <v>10.58</v>
+        <v>10.41</v>
       </c>
       <c r="BS19" t="n">
         <v>2.16</v>
       </c>
       <c r="BT19" t="n">
-        <v>12600</v>
+        <v>13273</v>
       </c>
     </row>
     <row r="20">
@@ -5417,13 +5417,13 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>5.25</v>
+        <v>5.16</v>
       </c>
       <c r="G22" t="n">
-        <v>1051287300</v>
+        <v>1033265717</v>
       </c>
       <c r="H22" t="n">
-        <v>1959500</v>
+        <v>1631500</v>
       </c>
       <c r="I22" t="n">
         <v>200245299</v>
@@ -5438,7 +5438,7 @@
         <v>0.27</v>
       </c>
       <c r="M22" t="n">
-        <v>0.08916662258323478</v>
+        <v>0.08763809304643409</v>
       </c>
       <c r="N22" t="n">
         <v>0.08</v>
@@ -5516,7 +5516,7 @@
         <v>378463615.11</v>
       </c>
       <c r="AM22" t="n">
-        <v>238387142.8571428</v>
+        <v>234300616.0997732</v>
       </c>
       <c r="AN22" t="n">
         <v>0</v>
@@ -5566,19 +5566,19 @@
         <v>172.49</v>
       </c>
       <c r="BC22" t="n">
-        <v>465.81</v>
+        <v>475.68</v>
       </c>
       <c r="BD22" t="n">
-        <v>361.98</v>
+        <v>370.04</v>
       </c>
       <c r="BE22" t="n">
         <v>-100</v>
       </c>
       <c r="BF22" t="n">
-        <v>-64</v>
+        <v>-63.37</v>
       </c>
       <c r="BG22" t="n">
-        <v>3185.52</v>
+        <v>3242.82</v>
       </c>
       <c r="BH22" t="n">
         <v>20.75</v>
@@ -5587,7 +5587,7 @@
         <v>0</v>
       </c>
       <c r="BJ22" t="n">
-        <v>5.25</v>
+        <v>5.16</v>
       </c>
       <c r="BK22" t="n">
         <v>1.89</v>
@@ -5596,7 +5596,7 @@
         <v>0.67</v>
       </c>
       <c r="BM22" t="n">
-        <v>5.34</v>
+        <v>5.29</v>
       </c>
       <c r="BN22" t="n">
         <v>7.89</v>
@@ -5605,19 +5605,19 @@
         <v>3.37</v>
       </c>
       <c r="BP22" t="n">
-        <v>4.87</v>
+        <v>5.03</v>
       </c>
       <c r="BQ22" t="n">
-        <v>7.82</v>
+        <v>7.69</v>
       </c>
       <c r="BR22" t="n">
-        <v>5.13</v>
+        <v>5.25</v>
       </c>
       <c r="BS22" t="n">
         <v>0.09</v>
       </c>
       <c r="BT22" t="n">
-        <v>1501080</v>
+        <v>1534617</v>
       </c>
     </row>
     <row r="23">
@@ -5877,13 +5877,13 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>3</v>
+        <v>2.93</v>
       </c>
       <c r="G24" t="n">
-        <v>1211606400</v>
+        <v>1183335024</v>
       </c>
       <c r="H24" t="n">
-        <v>5591000</v>
+        <v>4912300</v>
       </c>
       <c r="I24" t="n">
         <v>403868805</v>
@@ -5898,7 +5898,7 @@
         <v>0.49</v>
       </c>
       <c r="M24" t="n">
-        <v>0.2928947332159929</v>
+        <v>0.2860603873994232</v>
       </c>
       <c r="N24" t="n">
         <v>0.11</v>
@@ -5976,7 +5976,7 @@
         <v>153470145.9</v>
       </c>
       <c r="AM24" t="n">
-        <v>1091537297.297297</v>
+        <v>1066067589.189189</v>
       </c>
       <c r="AN24" t="n">
         <v>0.0813</v>
@@ -6017,7 +6017,7 @@
         <v>5.84</v>
       </c>
       <c r="AZ24" t="n">
-        <v>1.38</v>
+        <v>1.35</v>
       </c>
       <c r="BA24" t="n">
         <v>0.38</v>
@@ -6026,19 +6026,19 @@
         <v>1.46</v>
       </c>
       <c r="BC24" t="n">
-        <v>138.55</v>
+        <v>144.25</v>
       </c>
       <c r="BD24" t="n">
-        <v>94.77</v>
+        <v>99.43000000000001</v>
       </c>
       <c r="BE24" t="n">
         <v>-53.83</v>
       </c>
       <c r="BF24" t="n">
-        <v>-87.33</v>
+        <v>-87.03</v>
       </c>
       <c r="BG24" t="n">
-        <v>-51.41</v>
+        <v>-50.25</v>
       </c>
       <c r="BH24" t="n">
         <v>5.99</v>
@@ -6047,7 +6047,7 @@
         <v>0</v>
       </c>
       <c r="BJ24" t="n">
-        <v>3</v>
+        <v>2.93</v>
       </c>
       <c r="BK24" t="n">
         <v>0.38</v>
@@ -6065,19 +6065,19 @@
         <v>1.92</v>
       </c>
       <c r="BP24" t="n">
-        <v>2.92</v>
+        <v>2.9</v>
       </c>
       <c r="BQ24" t="n">
-        <v>7.37</v>
+        <v>7.2</v>
       </c>
       <c r="BR24" t="n">
-        <v>3.01</v>
+        <v>3</v>
       </c>
       <c r="BS24" t="n">
         <v>0.29</v>
       </c>
       <c r="BT24" t="n">
-        <v>7900803</v>
+        <v>7841887</v>
       </c>
     </row>
     <row r="25">
@@ -6107,13 +6107,13 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>4.67</v>
+        <v>4.22</v>
       </c>
       <c r="G25" t="n">
-        <v>1618127940</v>
+        <v>1462204607</v>
       </c>
       <c r="H25" t="n">
-        <v>1032900</v>
+        <v>3648200</v>
       </c>
       <c r="I25" t="n">
         <v>346494097</v>
@@ -6128,7 +6128,7 @@
         <v>0.97</v>
       </c>
       <c r="M25" t="n">
-        <v>0.8068724750405584</v>
+        <v>0.7291219817054744</v>
       </c>
       <c r="N25" t="n">
         <v>0.22</v>
@@ -6206,7 +6206,7 @@
         <v>62368937.46</v>
       </c>
       <c r="AM25" t="n">
-        <v>594899977.9411764</v>
+        <v>537575223.1617646</v>
       </c>
       <c r="AN25" t="n">
         <v>0.4742</v>
@@ -6247,7 +6247,7 @@
         <v>3.27</v>
       </c>
       <c r="AZ25" t="n">
-        <v>10.88</v>
+        <v>9.83</v>
       </c>
       <c r="BA25" t="n">
         <v>0.23</v>
@@ -6256,19 +6256,19 @@
         <v>2.2</v>
       </c>
       <c r="BC25" t="n">
-        <v>-14.14</v>
+        <v>-4.98</v>
       </c>
       <c r="BD25" t="n">
-        <v>-29.89</v>
+        <v>-22.42</v>
       </c>
       <c r="BE25" t="n">
         <v>133</v>
       </c>
       <c r="BF25" t="n">
-        <v>-95.04000000000001</v>
+        <v>-94.51000000000001</v>
       </c>
       <c r="BG25" t="n">
-        <v>-52.9</v>
+        <v>-47.87</v>
       </c>
       <c r="BH25" t="n">
         <v>3.97</v>
@@ -6277,7 +6277,7 @@
         <v>0</v>
       </c>
       <c r="BJ25" t="n">
-        <v>4.67</v>
+        <v>4.22</v>
       </c>
       <c r="BK25" t="n">
         <v>0.18</v>
@@ -6286,7 +6286,7 @@
         <v>0.24</v>
       </c>
       <c r="BM25" t="n">
-        <v>4.67</v>
+        <v>4.66</v>
       </c>
       <c r="BN25" t="n">
         <v>6.3</v>
@@ -6295,19 +6295,19 @@
         <v>2.64</v>
       </c>
       <c r="BP25" t="n">
-        <v>4.45</v>
+        <v>4.01</v>
       </c>
       <c r="BQ25" t="n">
-        <v>19.73</v>
+        <v>17.83</v>
       </c>
       <c r="BR25" t="n">
-        <v>4.45</v>
+        <v>4.66</v>
       </c>
       <c r="BS25" t="n">
         <v>0.67</v>
       </c>
       <c r="BT25" t="n">
-        <v>1257897</v>
+        <v>1099787</v>
       </c>
     </row>
     <row r="26">
@@ -6337,13 +6337,13 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>10.24</v>
+        <v>10.49</v>
       </c>
       <c r="G26" t="n">
-        <v>13868984010</v>
+        <v>14207582260</v>
       </c>
       <c r="H26" t="n">
-        <v>8212300</v>
+        <v>16425200</v>
       </c>
       <c r="I26" t="n">
         <v>1354393401</v>
@@ -6358,7 +6358,7 @@
         <v>1.94</v>
       </c>
       <c r="M26" t="n">
-        <v>0.1788393796726758</v>
+        <v>0.1832055755630591</v>
       </c>
       <c r="N26" t="n">
         <v>0.26</v>
@@ -6436,7 +6436,7 @@
         <v>961619314.7099999</v>
       </c>
       <c r="AM26" t="n">
-        <v>4953208575</v>
+        <v>5074136521.428572</v>
       </c>
       <c r="AN26" t="n">
         <v>0.1043</v>
@@ -6477,7 +6477,7 @@
         <v>7.07</v>
       </c>
       <c r="AZ26" t="n">
-        <v>1.96</v>
+        <v>2.01</v>
       </c>
       <c r="BA26" t="n">
         <v>0.66</v>
@@ -6486,19 +6486,19 @@
         <v>1.19</v>
       </c>
       <c r="BC26" t="n">
-        <v>-15.47</v>
+        <v>-17.49</v>
       </c>
       <c r="BD26" t="n">
-        <v>-30.98</v>
+        <v>-32.63</v>
       </c>
       <c r="BE26" t="n">
         <v>-80.83</v>
       </c>
       <c r="BF26" t="n">
-        <v>-93.56</v>
+        <v>-93.72</v>
       </c>
       <c r="BG26" t="n">
-        <v>-88.34999999999999</v>
+        <v>-88.62</v>
       </c>
       <c r="BH26" t="n">
         <v>4.69</v>
@@ -6507,7 +6507,7 @@
         <v>0</v>
       </c>
       <c r="BJ26" t="n">
-        <v>10.24</v>
+        <v>10.49</v>
       </c>
       <c r="BK26" t="n">
         <v>0.71</v>
@@ -6516,7 +6516,7 @@
         <v>0.72</v>
       </c>
       <c r="BM26" t="n">
-        <v>10.4</v>
+        <v>10.5</v>
       </c>
       <c r="BN26" t="n">
         <v>10.55</v>
@@ -6525,19 +6525,19 @@
         <v>6.91</v>
       </c>
       <c r="BP26" t="n">
-        <v>10.16</v>
+        <v>10.05</v>
       </c>
       <c r="BQ26" t="n">
-        <v>14.28</v>
+        <v>14.63</v>
       </c>
       <c r="BR26" t="n">
-        <v>10.35</v>
+        <v>10.22</v>
       </c>
       <c r="BS26" t="n">
         <v>0.16</v>
       </c>
       <c r="BT26" t="n">
-        <v>12125420</v>
+        <v>12118290</v>
       </c>
     </row>
     <row r="27">
@@ -8165,13 +8165,13 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>14.5</v>
+        <v>16.38</v>
       </c>
       <c r="G34" t="n">
-        <v>2994100650</v>
+        <v>3382301112</v>
       </c>
       <c r="H34" t="n">
-        <v>2993900</v>
+        <v>9668900</v>
       </c>
       <c r="I34" t="n">
         <v>206489813</v>
@@ -8186,7 +8186,7 @@
         <v>0.45</v>
       </c>
       <c r="M34" t="n">
-        <v>0.2632164164662674</v>
+        <v>0.2973437710287099</v>
       </c>
       <c r="N34" t="n">
         <v>0.24</v>
@@ -8264,7 +8264,7 @@
         <v>324189006.41</v>
       </c>
       <c r="AM34" t="n">
-        <v>622474147.6091477</v>
+        <v>703181104.3659045</v>
       </c>
       <c r="AN34" t="n">
         <v>0</v>
@@ -8305,7 +8305,7 @@
         <v>30.28</v>
       </c>
       <c r="AZ34" t="n">
-        <v>33.83</v>
+        <v>38.22</v>
       </c>
       <c r="BA34" t="n">
         <v>2.29</v>
@@ -8314,19 +8314,19 @@
         <v>25.26</v>
       </c>
       <c r="BC34" t="n">
-        <v>155.78</v>
+        <v>126.43</v>
       </c>
       <c r="BD34" t="n">
-        <v>108.85</v>
+        <v>84.88</v>
       </c>
       <c r="BE34" t="n">
         <v>133.33</v>
       </c>
       <c r="BF34" t="n">
-        <v>-84.17</v>
+        <v>-85.98999999999999</v>
       </c>
       <c r="BG34" t="n">
-        <v>74.19</v>
+        <v>54.2</v>
       </c>
       <c r="BH34" t="n">
         <v>38.94</v>
@@ -8335,7 +8335,7 @@
         <v>0</v>
       </c>
       <c r="BJ34" t="n">
-        <v>14.5</v>
+        <v>16.38</v>
       </c>
       <c r="BK34" t="n">
         <v>1.57</v>
@@ -8344,7 +8344,7 @@
         <v>1.58</v>
       </c>
       <c r="BM34" t="n">
-        <v>14.94</v>
+        <v>17.32</v>
       </c>
       <c r="BN34" t="n">
         <v>28.86</v>
@@ -8353,19 +8353,19 @@
         <v>14.3</v>
       </c>
       <c r="BP34" t="n">
-        <v>14.41</v>
+        <v>14.39</v>
       </c>
       <c r="BQ34" t="n">
-        <v>9.19</v>
+        <v>10.39</v>
       </c>
       <c r="BR34" t="n">
-        <v>14.93</v>
+        <v>14.5</v>
       </c>
       <c r="BS34" t="n">
         <v>0.32</v>
       </c>
       <c r="BT34" t="n">
-        <v>3185590</v>
+        <v>3203397</v>
       </c>
     </row>
     <row r="35">
@@ -8395,13 +8395,13 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>17.82</v>
+        <v>17.96</v>
       </c>
       <c r="G35" t="n">
-        <v>89928628459</v>
+        <v>90635135379</v>
       </c>
       <c r="H35" t="n">
-        <v>43921400</v>
+        <v>17058300</v>
       </c>
       <c r="I35" t="n">
         <v>5046500000</v>
@@ -8416,7 +8416,7 @@
         <v>4.69</v>
       </c>
       <c r="M35" t="n">
-        <v>7.46590741923543</v>
+        <v>7.524561880513843</v>
       </c>
       <c r="N35" t="n">
         <v>1.79</v>
@@ -8494,7 +8494,7 @@
         <v>5349290000</v>
       </c>
       <c r="AM35" t="n">
-        <v>7432118054.462811</v>
+        <v>7490507056.115703</v>
       </c>
       <c r="AN35" t="n">
         <v>0.5305</v>
@@ -8535,7 +8535,7 @@
         <v>7.68</v>
       </c>
       <c r="AZ35" t="n">
-        <v>10.4</v>
+        <v>10.48</v>
       </c>
       <c r="BA35" t="n">
         <v>1.11</v>
@@ -8544,19 +8544,19 @@
         <v>9.119999999999999</v>
       </c>
       <c r="BC35" t="n">
-        <v>-47.21</v>
+        <v>-47.62</v>
       </c>
       <c r="BD35" t="n">
-        <v>-56.9</v>
+        <v>-57.24</v>
       </c>
       <c r="BE35" t="n">
         <v>-41.67</v>
       </c>
       <c r="BF35" t="n">
-        <v>-93.75</v>
+        <v>-93.8</v>
       </c>
       <c r="BG35" t="n">
-        <v>-48.84</v>
+        <v>-49.24</v>
       </c>
       <c r="BH35" t="n">
         <v>3.71</v>
@@ -8565,7 +8565,7 @@
         <v>0</v>
       </c>
       <c r="BJ35" t="n">
-        <v>17.82</v>
+        <v>17.96</v>
       </c>
       <c r="BK35" t="n">
         <v>1.06</v>
@@ -8574,28 +8574,28 @@
         <v>1.04</v>
       </c>
       <c r="BM35" t="n">
-        <v>18.09</v>
+        <v>18.03</v>
       </c>
       <c r="BN35" t="n">
-        <v>20.08</v>
+        <v>19.88</v>
       </c>
       <c r="BO35" t="n">
-        <v>11.7</v>
+        <v>11.58</v>
       </c>
       <c r="BP35" t="n">
-        <v>17.7</v>
+        <v>17.62</v>
       </c>
       <c r="BQ35" t="n">
-        <v>17.05</v>
+        <v>17.19</v>
       </c>
       <c r="BR35" t="n">
-        <v>18</v>
+        <v>17.76</v>
       </c>
       <c r="BS35" t="n">
         <v>7.3</v>
       </c>
       <c r="BT35" t="n">
-        <v>41235613</v>
+        <v>40957743</v>
       </c>
     </row>
     <row r="36">
@@ -8858,7 +8858,7 @@
         <v>14.95</v>
       </c>
       <c r="G37" t="n">
-        <v>199741864</v>
+        <v>200164949</v>
       </c>
       <c r="H37" t="n">
         <v>200</v>
@@ -8876,7 +8876,7 @@
         <v>0.88</v>
       </c>
       <c r="M37" t="n">
-        <v>1.94465530636982</v>
+        <v>1.94877439524693</v>
       </c>
       <c r="N37" t="n">
         <v>0.5</v>
@@ -8954,7 +8954,7 @@
         <v>11319000</v>
       </c>
       <c r="AM37" t="n">
-        <v>47785134.92822967</v>
+        <v>47886351.4354067</v>
       </c>
       <c r="AN37" t="n">
         <v>0</v>
@@ -9043,19 +9043,19 @@
         <v>13.2</v>
       </c>
       <c r="BP37" t="n">
-        <v>14.85</v>
+        <v>14.75</v>
       </c>
       <c r="BQ37" t="n">
         <v>6.47</v>
       </c>
       <c r="BR37" t="n">
-        <v>14.85</v>
+        <v>14.75</v>
       </c>
       <c r="BS37" t="n">
         <v>0.72</v>
       </c>
       <c r="BT37" t="n">
-        <v>850</v>
+        <v>853</v>
       </c>
     </row>
     <row r="38">
@@ -9315,13 +9315,13 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>68.59999999999999</v>
+        <v>68.8</v>
       </c>
       <c r="G39" t="n">
-        <v>3845599294</v>
+        <v>3856811211</v>
       </c>
       <c r="H39" t="n">
-        <v>3400</v>
+        <v>900</v>
       </c>
       <c r="I39" t="n">
         <v>168174945</v>
@@ -9336,7 +9336,7 @@
         <v>0.53</v>
       </c>
       <c r="M39" t="n">
-        <v>0.1930322163572666</v>
+        <v>0.1935950054111081</v>
       </c>
       <c r="N39" t="n">
         <v>0.06</v>
@@ -9414,7 +9414,7 @@
         <v>2536078170.6</v>
       </c>
       <c r="AM39" t="n">
-        <v>403949505.6722689</v>
+        <v>405127228.0462185</v>
       </c>
       <c r="AN39" t="n">
         <v>11.9435</v>
@@ -9455,7 +9455,7 @@
         <v>170.24</v>
       </c>
       <c r="AZ39" t="n">
-        <v>200.43</v>
+        <v>201.01</v>
       </c>
       <c r="BA39" t="n">
         <v>19.01</v>
@@ -9464,19 +9464,19 @@
         <v>91.72</v>
       </c>
       <c r="BC39" t="n">
-        <v>203.94</v>
+        <v>203.06</v>
       </c>
       <c r="BD39" t="n">
-        <v>148.17</v>
+        <v>147.45</v>
       </c>
       <c r="BE39" t="n">
         <v>192.17</v>
       </c>
       <c r="BF39" t="n">
-        <v>-72.29000000000001</v>
+        <v>-72.37</v>
       </c>
       <c r="BG39" t="n">
-        <v>33.71</v>
+        <v>33.32</v>
       </c>
       <c r="BH39" t="n">
         <v>128.13</v>
@@ -9485,7 +9485,7 @@
         <v>0</v>
       </c>
       <c r="BJ39" t="n">
-        <v>68.59999999999999</v>
+        <v>68.8</v>
       </c>
       <c r="BK39" t="n">
         <v>15.08</v>
@@ -9494,7 +9494,7 @@
         <v>15.08</v>
       </c>
       <c r="BM39" t="n">
-        <v>68.81999999999999</v>
+        <v>68.89</v>
       </c>
       <c r="BN39" t="n">
         <v>74.56</v>
@@ -9503,19 +9503,19 @@
         <v>54.98</v>
       </c>
       <c r="BP39" t="n">
-        <v>68.09</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="BQ39" t="n">
-        <v>4.55</v>
+        <v>4.56</v>
       </c>
       <c r="BR39" t="n">
-        <v>68.81999999999999</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="BS39" t="n">
         <v>0.58</v>
       </c>
       <c r="BT39" t="n">
-        <v>3080</v>
+        <v>3153</v>
       </c>
     </row>
     <row r="40">
@@ -9545,13 +9545,13 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>21.54</v>
+        <v>21.59</v>
       </c>
       <c r="G40" t="n">
-        <v>123442169606</v>
+        <v>123728728524</v>
       </c>
       <c r="H40" t="n">
-        <v>36947000</v>
+        <v>43246900</v>
       </c>
       <c r="I40" t="n">
         <v>5730834040</v>
@@ -9566,7 +9566,7 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="M40" t="n">
-        <v>0.3745388192729615</v>
+        <v>0.3754082744935107</v>
       </c>
       <c r="N40" t="n">
         <v>0.05</v>
@@ -9644,7 +9644,7 @@
         <v>15358635227.2</v>
       </c>
       <c r="AM40" t="n">
-        <v>6402602157.987552</v>
+        <v>6417465172.406639</v>
       </c>
       <c r="AN40" t="n">
         <v>0.5641</v>
@@ -9685,7 +9685,7 @@
         <v>36.13</v>
       </c>
       <c r="AZ40" t="n">
-        <v>10.88</v>
+        <v>10.9</v>
       </c>
       <c r="BA40" t="n">
         <v>2.76</v>
@@ -9694,19 +9694,19 @@
         <v>27.89</v>
       </c>
       <c r="BC40" t="n">
-        <v>105.43</v>
+        <v>104.95</v>
       </c>
       <c r="BD40" t="n">
-        <v>67.73</v>
+        <v>67.34</v>
       </c>
       <c r="BE40" t="n">
         <v>-49.5</v>
       </c>
       <c r="BF40" t="n">
-        <v>-87.19</v>
+        <v>-87.22</v>
       </c>
       <c r="BG40" t="n">
-        <v>29.48</v>
+        <v>29.18</v>
       </c>
       <c r="BH40" t="n">
         <v>32.47</v>
@@ -9715,7 +9715,7 @@
         <v>0</v>
       </c>
       <c r="BJ40" t="n">
-        <v>21.54</v>
+        <v>21.59</v>
       </c>
       <c r="BK40" t="n">
         <v>2.68</v>
@@ -9724,7 +9724,7 @@
         <v>2.5</v>
       </c>
       <c r="BM40" t="n">
-        <v>22.24</v>
+        <v>21.77</v>
       </c>
       <c r="BN40" t="n">
         <v>27.36</v>
@@ -9733,19 +9733,19 @@
         <v>17.67</v>
       </c>
       <c r="BP40" t="n">
-        <v>21.48</v>
+        <v>21.27</v>
       </c>
       <c r="BQ40" t="n">
-        <v>8.619999999999999</v>
+        <v>8.640000000000001</v>
       </c>
       <c r="BR40" t="n">
-        <v>22.17</v>
+        <v>21.54</v>
       </c>
       <c r="BS40" t="n">
         <v>0.39</v>
       </c>
       <c r="BT40" t="n">
-        <v>37323550</v>
+        <v>37609030</v>
       </c>
     </row>
     <row r="41">
@@ -9775,13 +9775,13 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>15.63</v>
+        <v>15.77</v>
       </c>
       <c r="G41" t="n">
-        <v>187579718444</v>
+        <v>188077565572</v>
       </c>
       <c r="H41" t="n">
-        <v>8898100</v>
+        <v>4253600</v>
       </c>
       <c r="I41" t="n">
         <v>5303870781</v>
@@ -9796,7 +9796,7 @@
         <v>0.92</v>
       </c>
       <c r="M41" t="n">
-        <v>1.250025326941013</v>
+        <v>1.253342964498565</v>
       </c>
       <c r="N41" t="n">
         <v>0.07000000000000001</v>
@@ -9874,7 +9874,7 @@
         <v>12304980211.92</v>
       </c>
       <c r="AM41" t="n">
-        <v>28902884197.84283</v>
+        <v>28979594078.8906</v>
       </c>
       <c r="AN41" t="n">
         <v>1.6841</v>
@@ -9915,7 +9915,7 @@
         <v>24.4</v>
       </c>
       <c r="AZ41" t="n">
-        <v>23.39</v>
+        <v>23.6</v>
       </c>
       <c r="BA41" t="n">
         <v>2.53</v>
@@ -9924,19 +9924,19 @@
         <v>13.77</v>
       </c>
       <c r="BC41" t="n">
-        <v>91.20999999999999</v>
+        <v>89.51000000000001</v>
       </c>
       <c r="BD41" t="n">
-        <v>56.12</v>
+        <v>54.73</v>
       </c>
       <c r="BE41" t="n">
         <v>49.67</v>
       </c>
       <c r="BF41" t="n">
-        <v>-83.83</v>
+        <v>-83.97</v>
       </c>
       <c r="BG41" t="n">
-        <v>-11.9</v>
+        <v>-12.68</v>
       </c>
       <c r="BH41" t="n">
         <v>17.11</v>
@@ -9945,7 +9945,7 @@
         <v>0</v>
       </c>
       <c r="BJ41" t="n">
-        <v>15.63</v>
+        <v>15.77</v>
       </c>
       <c r="BK41" t="n">
         <v>2.32</v>
@@ -9954,7 +9954,7 @@
         <v>2.34</v>
       </c>
       <c r="BM41" t="n">
-        <v>15.95</v>
+        <v>15.82</v>
       </c>
       <c r="BN41" t="n">
         <v>18.28</v>
@@ -9963,19 +9963,19 @@
         <v>13.43</v>
       </c>
       <c r="BP41" t="n">
-        <v>15.57</v>
+        <v>15.58</v>
       </c>
       <c r="BQ41" t="n">
-        <v>6.69</v>
+        <v>6.75</v>
       </c>
       <c r="BR41" t="n">
-        <v>15.95</v>
+        <v>15.62</v>
       </c>
       <c r="BS41" t="n">
         <v>0.5600000000000001</v>
       </c>
       <c r="BT41" t="n">
-        <v>7174877</v>
+        <v>7279813</v>
       </c>
     </row>
     <row r="42">
@@ -10005,13 +10005,13 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>17.78</v>
+        <v>17.88</v>
       </c>
       <c r="G42" t="n">
-        <v>187579718444</v>
+        <v>188077565572</v>
       </c>
       <c r="H42" t="n">
-        <v>34713200</v>
+        <v>21337600</v>
       </c>
       <c r="I42" t="n">
         <v>5288141247</v>
@@ -10026,7 +10026,7 @@
         <v>1.05</v>
       </c>
       <c r="M42" t="n">
-        <v>1.25374351731502</v>
+        <v>1.25707102315905</v>
       </c>
       <c r="N42" t="n">
         <v>0.08</v>
@@ -10104,7 +10104,7 @@
         <v>12268487693.04</v>
       </c>
       <c r="AM42" t="n">
-        <v>25521050128.43538</v>
+        <v>25588784431.56463</v>
       </c>
       <c r="AN42" t="n">
         <v>1.8491</v>
@@ -10145,7 +10145,7 @@
         <v>24.4</v>
       </c>
       <c r="AZ42" t="n">
-        <v>25.75</v>
+        <v>25.9</v>
       </c>
       <c r="BA42" t="n">
         <v>2.53</v>
@@ -10154,19 +10154,19 @@
         <v>15.11</v>
       </c>
       <c r="BC42" t="n">
-        <v>68.08</v>
+        <v>67.14</v>
       </c>
       <c r="BD42" t="n">
-        <v>37.24</v>
+        <v>36.47</v>
       </c>
       <c r="BE42" t="n">
         <v>44.83</v>
       </c>
       <c r="BF42" t="n">
-        <v>-85.79000000000001</v>
+        <v>-85.87</v>
       </c>
       <c r="BG42" t="n">
-        <v>-14.99</v>
+        <v>-15.47</v>
       </c>
       <c r="BH42" t="n">
         <v>17.11</v>
@@ -10175,7 +10175,7 @@
         <v>0</v>
       </c>
       <c r="BJ42" t="n">
-        <v>17.78</v>
+        <v>17.88</v>
       </c>
       <c r="BK42" t="n">
         <v>2.32</v>
@@ -10184,7 +10184,7 @@
         <v>2.34</v>
       </c>
       <c r="BM42" t="n">
-        <v>18.1</v>
+        <v>17.95</v>
       </c>
       <c r="BN42" t="n">
         <v>21.33</v>
@@ -10193,19 +10193,19 @@
         <v>15.67</v>
       </c>
       <c r="BP42" t="n">
-        <v>17.66</v>
+        <v>17.65</v>
       </c>
       <c r="BQ42" t="n">
-        <v>7.61</v>
+        <v>7.65</v>
       </c>
       <c r="BR42" t="n">
-        <v>18.08</v>
+        <v>17.74</v>
       </c>
       <c r="BS42" t="n">
         <v>0.63</v>
       </c>
       <c r="BT42" t="n">
-        <v>41398077</v>
+        <v>41073393</v>
       </c>
     </row>
     <row r="43">
@@ -10235,13 +10235,13 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>38.77</v>
+        <v>38.99</v>
       </c>
       <c r="G43" t="n">
-        <v>75268040118</v>
+        <v>75695189258</v>
       </c>
       <c r="H43" t="n">
-        <v>3910900</v>
+        <v>4015300</v>
       </c>
       <c r="I43" t="n">
         <v>1941400000</v>
@@ -10334,7 +10334,7 @@
         <v>9182822000</v>
       </c>
       <c r="AM43" t="n">
-        <v>9167848979.049938</v>
+        <v>9219876888.915955</v>
       </c>
       <c r="AN43" t="n">
         <v>4.5901</v>
@@ -10375,7 +10375,7 @@
         <v>19.95</v>
       </c>
       <c r="AZ43" t="n">
-        <v>70.37</v>
+        <v>70.77</v>
       </c>
       <c r="BA43" t="n">
         <v>5.63</v>
@@ -10384,19 +10384,19 @@
         <v>48.62</v>
       </c>
       <c r="BC43" t="n">
-        <v>-36.98</v>
+        <v>-37.33</v>
       </c>
       <c r="BD43" t="n">
-        <v>-48.54</v>
+        <v>-48.83</v>
       </c>
       <c r="BE43" t="n">
         <v>81.5</v>
       </c>
       <c r="BF43" t="n">
-        <v>-85.48</v>
+        <v>-85.56</v>
       </c>
       <c r="BG43" t="n">
-        <v>25.4</v>
+        <v>24.69</v>
       </c>
       <c r="BH43" t="n">
         <v>5.61</v>
@@ -10405,7 +10405,7 @@
         <v>0</v>
       </c>
       <c r="BJ43" t="n">
-        <v>38.77</v>
+        <v>38.99</v>
       </c>
       <c r="BK43" t="n">
         <v>4.73</v>
@@ -10414,7 +10414,7 @@
         <v>4.73</v>
       </c>
       <c r="BM43" t="n">
-        <v>39.23</v>
+        <v>39.07</v>
       </c>
       <c r="BN43" t="n">
         <v>42.98</v>
@@ -10423,19 +10423,19 @@
         <v>28.06</v>
       </c>
       <c r="BP43" t="n">
-        <v>38.69</v>
+        <v>38.58</v>
       </c>
       <c r="BQ43" t="n">
-        <v>8.19</v>
+        <v>8.24</v>
       </c>
       <c r="BR43" t="n">
-        <v>38.88</v>
+        <v>38.74</v>
       </c>
       <c r="BS43" t="n">
         <v>0</v>
       </c>
       <c r="BT43" t="n">
-        <v>6596033</v>
+        <v>6572333</v>
       </c>
     </row>
     <row r="44">
@@ -10925,13 +10925,13 @@
         </is>
       </c>
       <c r="F46" t="n">
-        <v>4.05</v>
+        <v>4.09</v>
       </c>
       <c r="G46" t="n">
-        <v>4052195290</v>
+        <v>4092216932</v>
       </c>
       <c r="H46" t="n">
-        <v>18284500</v>
+        <v>24223330</v>
       </c>
       <c r="I46" t="n">
         <v>1000542188</v>
@@ -10946,7 +10946,7 @@
         <v>2.5</v>
       </c>
       <c r="M46" t="n">
-        <v>0.07043477267668936</v>
+        <v>0.07113042405937922</v>
       </c>
       <c r="N46" t="n">
         <v>0.08</v>
@@ -11024,7 +11024,7 @@
         <v>460249406.48</v>
       </c>
       <c r="AM46" t="n">
-        <v>3972740480.392157</v>
+        <v>4011977384.313725</v>
       </c>
       <c r="AN46" t="n">
         <v>0.0311</v>
@@ -11065,7 +11065,7 @@
         <v>3.3</v>
       </c>
       <c r="AZ46" t="n">
-        <v>3.34</v>
+        <v>3.37</v>
       </c>
       <c r="BA46" t="n">
         <v>0.42</v>
@@ -11074,19 +11074,19 @@
         <v>7.38</v>
       </c>
       <c r="BC46" t="n">
-        <v>-0.15</v>
+        <v>-1.13</v>
       </c>
       <c r="BD46" t="n">
-        <v>-18.47</v>
+        <v>-19.27</v>
       </c>
       <c r="BE46" t="n">
         <v>-17.5</v>
       </c>
       <c r="BF46" t="n">
-        <v>-89.55</v>
+        <v>-89.66</v>
       </c>
       <c r="BG46" t="n">
-        <v>82.19</v>
+        <v>80.41</v>
       </c>
       <c r="BH46" t="n">
         <v>1.58</v>
@@ -11095,7 +11095,7 @@
         <v>0</v>
       </c>
       <c r="BJ46" t="n">
-        <v>4.05</v>
+        <v>4.09</v>
       </c>
       <c r="BK46" t="n">
         <v>0.46</v>
@@ -11104,7 +11104,7 @@
         <v>0.46</v>
       </c>
       <c r="BM46" t="n">
-        <v>4.11</v>
+        <v>4.22</v>
       </c>
       <c r="BN46" t="n">
         <v>7.31</v>
@@ -11113,19 +11113,19 @@
         <v>2.97</v>
       </c>
       <c r="BP46" t="n">
-        <v>3.98</v>
+        <v>3.99</v>
       </c>
       <c r="BQ46" t="n">
-        <v>8.85</v>
+        <v>8.94</v>
       </c>
       <c r="BR46" t="n">
-        <v>4.02</v>
+        <v>4.06</v>
       </c>
       <c r="BS46" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="BT46" t="n">
-        <v>22806877</v>
+        <v>22964607</v>
       </c>
     </row>
     <row r="47">
@@ -11155,13 +11155,13 @@
         </is>
       </c>
       <c r="F47" t="n">
-        <v>8.93</v>
+        <v>8.960000000000001</v>
       </c>
       <c r="G47" t="n">
-        <v>3122716625</v>
+        <v>3130504845</v>
       </c>
       <c r="H47" t="n">
-        <v>4800</v>
+        <v>6700</v>
       </c>
       <c r="I47" t="n">
         <v>254106600</v>
@@ -11176,7 +11176,7 @@
         <v>1.22</v>
       </c>
       <c r="M47" t="n">
-        <v>0.73637250784191</v>
+        <v>0.7382090597234067</v>
       </c>
       <c r="N47" t="n">
         <v>0.07000000000000001</v>
@@ -11254,7 +11254,7 @@
         <v>322715382</v>
       </c>
       <c r="AM47" t="n">
-        <v>553673160.4609929</v>
+        <v>555054050.5319149</v>
       </c>
       <c r="AN47" t="n">
         <v>0.4132</v>
@@ -11295,7 +11295,7 @@
         <v>11.74</v>
       </c>
       <c r="AZ47" t="n">
-        <v>11.73</v>
+        <v>11.77</v>
       </c>
       <c r="BA47" t="n">
         <v>1.46</v>
@@ -11304,19 +11304,19 @@
         <v>8.619999999999999</v>
       </c>
       <c r="BC47" t="n">
-        <v>60.96</v>
+        <v>60.42</v>
       </c>
       <c r="BD47" t="n">
-        <v>31.42</v>
+        <v>30.98</v>
       </c>
       <c r="BE47" t="n">
         <v>31.33</v>
       </c>
       <c r="BF47" t="n">
-        <v>-83.67</v>
+        <v>-83.72</v>
       </c>
       <c r="BG47" t="n">
-        <v>-3.47</v>
+        <v>-3.8</v>
       </c>
       <c r="BH47" t="n">
         <v>7.23</v>
@@ -11325,7 +11325,7 @@
         <v>0</v>
       </c>
       <c r="BJ47" t="n">
-        <v>8.93</v>
+        <v>8.960000000000001</v>
       </c>
       <c r="BK47" t="n">
         <v>1.27</v>
@@ -11334,7 +11334,7 @@
         <v>1.29</v>
       </c>
       <c r="BM47" t="n">
-        <v>9</v>
+        <v>9.039999999999999</v>
       </c>
       <c r="BN47" t="n">
         <v>9.24</v>
@@ -11346,16 +11346,16 @@
         <v>8.9</v>
       </c>
       <c r="BQ47" t="n">
-        <v>6.9</v>
+        <v>6.93</v>
       </c>
       <c r="BR47" t="n">
-        <v>8.98</v>
+        <v>9</v>
       </c>
       <c r="BS47" t="n">
         <v>0.53</v>
       </c>
       <c r="BT47" t="n">
-        <v>11317</v>
+        <v>10820</v>
       </c>
     </row>
     <row r="48">
@@ -11385,13 +11385,13 @@
         </is>
       </c>
       <c r="F48" t="n">
-        <v>9.109999999999999</v>
+        <v>9.1</v>
       </c>
       <c r="G48" t="n">
-        <v>3122716625</v>
+        <v>3130504845</v>
       </c>
       <c r="H48" t="n">
-        <v>7700</v>
+        <v>1300</v>
       </c>
       <c r="I48" t="n">
         <v>93397546</v>
@@ -11406,7 +11406,7 @@
         <v>1.24</v>
       </c>
       <c r="M48" t="n">
-        <v>2.003447866833473</v>
+        <v>2.008444571504179</v>
       </c>
       <c r="N48" t="n">
         <v>0.07000000000000001</v>
@@ -11484,7 +11484,7 @@
         <v>118614883.42</v>
       </c>
       <c r="AM48" t="n">
-        <v>545929479.8951049</v>
+        <v>547291056.8181819</v>
       </c>
       <c r="AN48" t="n">
         <v>0.4132</v>
@@ -11525,7 +11525,7 @@
         <v>11.74</v>
       </c>
       <c r="AZ48" t="n">
-        <v>11.92</v>
+        <v>11.91</v>
       </c>
       <c r="BA48" t="n">
         <v>1.46</v>
@@ -11534,19 +11534,19 @@
         <v>8.24</v>
       </c>
       <c r="BC48" t="n">
-        <v>57.78</v>
+        <v>57.95</v>
       </c>
       <c r="BD48" t="n">
-        <v>28.82</v>
+        <v>28.97</v>
       </c>
       <c r="BE48" t="n">
         <v>30.83</v>
       </c>
       <c r="BF48" t="n">
-        <v>-83.98999999999999</v>
+        <v>-83.97</v>
       </c>
       <c r="BG48" t="n">
-        <v>-9.59</v>
+        <v>-9.49</v>
       </c>
       <c r="BH48" t="n">
         <v>7.23</v>
@@ -11555,7 +11555,7 @@
         <v>0</v>
       </c>
       <c r="BJ48" t="n">
-        <v>9.109999999999999</v>
+        <v>9.1</v>
       </c>
       <c r="BK48" t="n">
         <v>1.27</v>
@@ -11564,7 +11564,7 @@
         <v>1.29</v>
       </c>
       <c r="BM48" t="n">
-        <v>9.300000000000001</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="BN48" t="n">
         <v>9.48</v>
@@ -11573,19 +11573,19 @@
         <v>7.2</v>
       </c>
       <c r="BP48" t="n">
-        <v>9.050000000000001</v>
+        <v>9.08</v>
       </c>
       <c r="BQ48" t="n">
         <v>7.04</v>
       </c>
       <c r="BR48" t="n">
-        <v>9.08</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="BS48" t="n">
         <v>0.54</v>
       </c>
       <c r="BT48" t="n">
-        <v>2497</v>
+        <v>2680</v>
       </c>
     </row>
     <row r="49">
@@ -11615,13 +11615,13 @@
         </is>
       </c>
       <c r="F49" t="n">
-        <v>50.49</v>
+        <v>48.85</v>
       </c>
       <c r="G49" t="n">
-        <v>971669984</v>
+        <v>933365685</v>
       </c>
       <c r="H49" t="n">
-        <v>2700</v>
+        <v>1000</v>
       </c>
       <c r="I49" t="n">
         <v>11540870</v>
@@ -11636,7 +11636,7 @@
         <v>1.09</v>
       </c>
       <c r="M49" t="n">
-        <v>0.9830259897033297</v>
+        <v>0.9442740244739837</v>
       </c>
       <c r="N49" t="n">
         <v>0.08</v>
@@ -11714,7 +11714,7 @@
         <v>84709985.8</v>
       </c>
       <c r="AM49" t="n">
-        <v>242917496</v>
+        <v>233341421.25</v>
       </c>
       <c r="AN49" t="n">
         <v>3.3186</v>
@@ -11755,7 +11755,7 @@
         <v>68.48999999999999</v>
       </c>
       <c r="AZ49" t="n">
-        <v>60.25</v>
+        <v>58.29</v>
       </c>
       <c r="BA49" t="n">
         <v>9.210000000000001</v>
@@ -11764,19 +11764,19 @@
         <v>27.75</v>
       </c>
       <c r="BC49" t="n">
-        <v>66.13</v>
+        <v>71.7</v>
       </c>
       <c r="BD49" t="n">
-        <v>35.64</v>
+        <v>40.2</v>
       </c>
       <c r="BE49" t="n">
         <v>19.33</v>
       </c>
       <c r="BF49" t="n">
-        <v>-81.75</v>
+        <v>-81.14</v>
       </c>
       <c r="BG49" t="n">
-        <v>-45.03</v>
+        <v>-43.18</v>
       </c>
       <c r="BH49" t="n">
         <v>42.6</v>
@@ -11785,7 +11785,7 @@
         <v>0</v>
       </c>
       <c r="BJ49" t="n">
-        <v>50.49</v>
+        <v>48.85</v>
       </c>
       <c r="BK49" t="n">
         <v>7.34</v>
@@ -11794,7 +11794,7 @@
         <v>7.6</v>
       </c>
       <c r="BM49" t="n">
-        <v>50.49</v>
+        <v>54</v>
       </c>
       <c r="BN49" t="n">
         <v>64.2</v>
@@ -11803,19 +11803,19 @@
         <v>28.48</v>
       </c>
       <c r="BP49" t="n">
-        <v>46.36</v>
+        <v>48.85</v>
       </c>
       <c r="BQ49" t="n">
-        <v>6.64</v>
+        <v>6.43</v>
       </c>
       <c r="BR49" t="n">
-        <v>49.15</v>
+        <v>54</v>
       </c>
       <c r="BS49" t="n">
         <v>0.54</v>
       </c>
       <c r="BT49" t="n">
-        <v>243</v>
+        <v>333</v>
       </c>
     </row>
     <row r="50">
@@ -11845,13 +11845,13 @@
         </is>
       </c>
       <c r="F50" t="n">
-        <v>33.1</v>
+        <v>33.77</v>
       </c>
       <c r="G50" t="n">
-        <v>971669984</v>
+        <v>933365685</v>
       </c>
       <c r="H50" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="I50" t="n">
         <v>11540870</v>
@@ -11866,7 +11866,7 @@
         <v>0.8</v>
       </c>
       <c r="M50" t="n">
-        <v>0.9830259897033297</v>
+        <v>0.9442740244739837</v>
       </c>
       <c r="N50" t="n">
         <v>0.06</v>
@@ -11944,7 +11944,7 @@
         <v>84709985.8</v>
       </c>
       <c r="AM50" t="n">
-        <v>331627980.887372</v>
+        <v>318554841.2969283</v>
       </c>
       <c r="AN50" t="n">
         <v>4.4983</v>
@@ -11985,7 +11985,7 @@
         <v>68.48999999999999</v>
       </c>
       <c r="AZ50" t="n">
-        <v>72.98999999999999</v>
+        <v>74.45999999999999</v>
       </c>
       <c r="BA50" t="n">
         <v>9.210000000000001</v>
@@ -11994,19 +11994,19 @@
         <v>30.53</v>
       </c>
       <c r="BC50" t="n">
-        <v>153.41</v>
+        <v>148.38</v>
       </c>
       <c r="BD50" t="n">
-        <v>106.9</v>
+        <v>102.8</v>
       </c>
       <c r="BE50" t="n">
         <v>120.5</v>
       </c>
       <c r="BF50" t="n">
-        <v>-72.16</v>
+        <v>-72.72</v>
       </c>
       <c r="BG50" t="n">
-        <v>-7.76</v>
+        <v>-9.59</v>
       </c>
       <c r="BH50" t="n">
         <v>42.6</v>
@@ -12015,7 +12015,7 @@
         <v>0</v>
       </c>
       <c r="BJ50" t="n">
-        <v>33.1</v>
+        <v>33.77</v>
       </c>
       <c r="BK50" t="n">
         <v>7.34</v>
@@ -12024,7 +12024,7 @@
         <v>7.6</v>
       </c>
       <c r="BM50" t="n">
-        <v>33.98</v>
+        <v>34.27</v>
       </c>
       <c r="BN50" t="n">
         <v>39.22</v>
@@ -12033,19 +12033,19 @@
         <v>23.5</v>
       </c>
       <c r="BP50" t="n">
-        <v>32.65</v>
+        <v>33.58</v>
       </c>
       <c r="BQ50" t="n">
-        <v>4.35</v>
+        <v>4.44</v>
       </c>
       <c r="BR50" t="n">
-        <v>33.98</v>
+        <v>33.58</v>
       </c>
       <c r="BS50" t="n">
         <v>0.4</v>
       </c>
       <c r="BT50" t="n">
-        <v>520</v>
+        <v>547</v>
       </c>
     </row>
     <row r="51">
@@ -12523,13 +12523,13 @@
         </is>
       </c>
       <c r="F53" t="n">
-        <v>6</v>
+        <v>6.13</v>
       </c>
       <c r="G53" t="n">
-        <v>821114400</v>
+        <v>838905227</v>
       </c>
       <c r="H53" t="n">
-        <v>27200</v>
+        <v>21500</v>
       </c>
       <c r="I53" t="n">
         <v>136852484</v>
@@ -12544,7 +12544,7 @@
         <v>2.79</v>
       </c>
       <c r="M53" t="n">
-        <v>2.133102138977818</v>
+        <v>2.179319390956208</v>
       </c>
       <c r="N53" t="n">
         <v>1.48</v>
@@ -12622,7 +12622,7 @@
         <v>39687220.36</v>
       </c>
       <c r="AM53" t="n">
-        <v>41829566.98930209</v>
+        <v>42735875.03820683</v>
       </c>
       <c r="AN53" t="n">
         <v>0</v>
@@ -12672,16 +12672,16 @@
         <v>0</v>
       </c>
       <c r="BC53" t="n">
-        <v>-34.32</v>
+        <v>-35.71</v>
       </c>
       <c r="BD53" t="n">
-        <v>-46.37</v>
+        <v>-47.51</v>
       </c>
       <c r="BE53" t="n">
         <v>-100</v>
       </c>
       <c r="BF53" t="n">
-        <v>-95.17</v>
+        <v>-95.27</v>
       </c>
       <c r="BG53" t="n">
         <v>-100</v>
@@ -12690,19 +12690,19 @@
         <v>2.38</v>
       </c>
       <c r="BI53" t="n">
-        <v>0</v>
+        <v>16.96</v>
       </c>
       <c r="BJ53" t="n">
-        <v>6</v>
+        <v>5.24</v>
       </c>
       <c r="BK53" t="n">
         <v>0.29</v>
       </c>
       <c r="BL53" t="n">
-        <v>0.09</v>
+        <v>0.2</v>
       </c>
       <c r="BM53" t="n">
-        <v>6.29</v>
+        <v>6.2</v>
       </c>
       <c r="BN53" t="n">
         <v>10.39</v>
@@ -12711,19 +12711,19 @@
         <v>4.82</v>
       </c>
       <c r="BP53" t="n">
-        <v>6</v>
+        <v>5.91</v>
       </c>
       <c r="BQ53" t="n">
-        <v>70.31999999999999</v>
+        <v>30.11</v>
       </c>
       <c r="BR53" t="n">
-        <v>6.29</v>
+        <v>5.91</v>
       </c>
       <c r="BS53" t="n">
         <v>2.36</v>
       </c>
       <c r="BT53" t="n">
-        <v>34953</v>
+        <v>35257</v>
       </c>
     </row>
     <row r="54">
@@ -12753,13 +12753,13 @@
         </is>
       </c>
       <c r="F54" t="n">
-        <v>10.29</v>
+        <v>10.22</v>
       </c>
       <c r="G54" t="n">
-        <v>2399751471</v>
+        <v>2383427724</v>
       </c>
       <c r="H54" t="n">
-        <v>246300</v>
+        <v>191100</v>
       </c>
       <c r="I54" t="n">
         <v>233212121</v>
@@ -12774,7 +12774,7 @@
         <v>0.97</v>
       </c>
       <c r="M54" t="n">
-        <v>1.346960296089842</v>
+        <v>1.337797914335679</v>
       </c>
       <c r="N54" t="n">
         <v>0.5600000000000001</v>
@@ -12852,7 +12852,7 @@
         <v>233212121</v>
       </c>
       <c r="AM54" t="n">
-        <v>328283374.9658003</v>
+        <v>326050304.2407661</v>
       </c>
       <c r="AN54" t="n">
         <v>0.1531</v>
@@ -12893,7 +12893,7 @@
         <v>12.25</v>
       </c>
       <c r="AZ54" t="n">
-        <v>16.38</v>
+        <v>16.27</v>
       </c>
       <c r="BA54" t="n">
         <v>0.98</v>
@@ -12902,19 +12902,19 @@
         <v>6.52</v>
       </c>
       <c r="BC54" t="n">
-        <v>45.85</v>
+        <v>46.84</v>
       </c>
       <c r="BD54" t="n">
-        <v>19.08</v>
+        <v>19.9</v>
       </c>
       <c r="BE54" t="n">
         <v>59.17</v>
       </c>
       <c r="BF54" t="n">
-        <v>-90.44</v>
+        <v>-90.38</v>
       </c>
       <c r="BG54" t="n">
-        <v>-36.67</v>
+        <v>-36.24</v>
       </c>
       <c r="BH54" t="n">
         <v>10.01</v>
@@ -12923,7 +12923,7 @@
         <v>0</v>
       </c>
       <c r="BJ54" t="n">
-        <v>10.29</v>
+        <v>10.22</v>
       </c>
       <c r="BK54" t="n">
         <v>1</v>
@@ -12932,7 +12932,7 @@
         <v>1</v>
       </c>
       <c r="BM54" t="n">
-        <v>10.6</v>
+        <v>10.46</v>
       </c>
       <c r="BN54" t="n">
         <v>11.75</v>
@@ -12941,19 +12941,19 @@
         <v>8.279999999999999</v>
       </c>
       <c r="BP54" t="n">
-        <v>10.21</v>
+        <v>10.08</v>
       </c>
       <c r="BQ54" t="n">
-        <v>10.26</v>
+        <v>10.19</v>
       </c>
       <c r="BR54" t="n">
-        <v>10.25</v>
+        <v>10.35</v>
       </c>
       <c r="BS54" t="n">
         <v>1.26</v>
       </c>
       <c r="BT54" t="n">
-        <v>274093</v>
+        <v>249027</v>
       </c>
     </row>
     <row r="55">
@@ -12983,13 +12983,13 @@
         </is>
       </c>
       <c r="F55" t="n">
-        <v>49.64</v>
+        <v>50.1</v>
       </c>
       <c r="G55" t="n">
-        <v>6373382231</v>
+        <v>5145951203</v>
       </c>
       <c r="H55" t="n">
-        <v>4100</v>
+        <v>2600</v>
       </c>
       <c r="I55" t="n">
         <v>84052790</v>
@@ -13004,7 +13004,7 @@
         <v>2</v>
       </c>
       <c r="M55" t="n">
-        <v>0.9838663980149425</v>
+        <v>0.7943864483492438</v>
       </c>
       <c r="N55" t="n">
         <v>0.16</v>
@@ -13082,7 +13082,7 @@
         <v>579123723.1</v>
       </c>
       <c r="AM55" t="n">
-        <v>320592667.555332</v>
+        <v>258850664.1348089</v>
       </c>
       <c r="AN55" t="n">
         <v>3.1953</v>
@@ -13123,7 +13123,7 @@
         <v>51.21</v>
       </c>
       <c r="AZ55" t="n">
-        <v>52.2</v>
+        <v>52.69</v>
       </c>
       <c r="BA55" t="n">
         <v>9.380000000000001</v>
@@ -13132,19 +13132,19 @@
         <v>16.08</v>
       </c>
       <c r="BC55" t="n">
-        <v>26.34</v>
+        <v>25.18</v>
       </c>
       <c r="BD55" t="n">
-        <v>3.15</v>
+        <v>2.21</v>
       </c>
       <c r="BE55" t="n">
         <v>5.17</v>
       </c>
       <c r="BF55" t="n">
-        <v>-81.11</v>
+        <v>-81.28</v>
       </c>
       <c r="BG55" t="n">
-        <v>-67.61</v>
+        <v>-67.91</v>
       </c>
       <c r="BH55" t="n">
         <v>25.37</v>
@@ -13153,7 +13153,7 @@
         <v>0</v>
       </c>
       <c r="BJ55" t="n">
-        <v>49.64</v>
+        <v>50.1</v>
       </c>
       <c r="BK55" t="n">
         <v>6.89</v>
@@ -13162,7 +13162,7 @@
         <v>7.03</v>
       </c>
       <c r="BM55" t="n">
-        <v>50.88</v>
+        <v>50.2</v>
       </c>
       <c r="BN55" t="n">
         <v>73.67</v>
@@ -13171,19 +13171,19 @@
         <v>35.58</v>
       </c>
       <c r="BP55" t="n">
-        <v>49.62</v>
+        <v>49.65</v>
       </c>
       <c r="BQ55" t="n">
-        <v>7.06</v>
+        <v>7.13</v>
       </c>
       <c r="BR55" t="n">
-        <v>50.71</v>
+        <v>49.67</v>
       </c>
       <c r="BS55" t="n">
         <v>0.66</v>
       </c>
       <c r="BT55" t="n">
-        <v>7003</v>
+        <v>6423</v>
       </c>
     </row>
     <row r="56">
@@ -13213,13 +13213,13 @@
         </is>
       </c>
       <c r="F56" t="n">
-        <v>57.6</v>
+        <v>57.12</v>
       </c>
       <c r="G56" t="n">
-        <v>6373382231</v>
+        <v>5145951203</v>
       </c>
       <c r="H56" t="n">
-        <v>56700</v>
+        <v>29700</v>
       </c>
       <c r="I56" t="n">
         <v>39675836</v>
@@ -13234,7 +13234,7 @@
         <v>2.41</v>
       </c>
       <c r="M56" t="n">
-        <v>2.084309344871937</v>
+        <v>1.682898309236505</v>
       </c>
       <c r="N56" t="n">
         <v>0.19</v>
@@ -13312,7 +13312,7 @@
         <v>273366510.04</v>
       </c>
       <c r="AM56" t="n">
-        <v>265115733.4026622</v>
+        <v>214057870.3410982</v>
       </c>
       <c r="AN56" t="n">
         <v>3.5102</v>
@@ -13353,7 +13353,7 @@
         <v>51.21</v>
       </c>
       <c r="AZ56" t="n">
-        <v>55.01</v>
+        <v>54.55</v>
       </c>
       <c r="BA56" t="n">
         <v>9.380000000000001</v>
@@ -13362,19 +13362,19 @@
         <v>17.68</v>
       </c>
       <c r="BC56" t="n">
-        <v>8.880000000000001</v>
+        <v>9.789999999999999</v>
       </c>
       <c r="BD56" t="n">
-        <v>-11.1</v>
+        <v>-10.35</v>
       </c>
       <c r="BE56" t="n">
         <v>-4.5</v>
       </c>
       <c r="BF56" t="n">
-        <v>-83.72</v>
+        <v>-83.58</v>
       </c>
       <c r="BG56" t="n">
-        <v>-69.31</v>
+        <v>-69.05</v>
       </c>
       <c r="BH56" t="n">
         <v>25.37</v>
@@ -13383,7 +13383,7 @@
         <v>0</v>
       </c>
       <c r="BJ56" t="n">
-        <v>57.6</v>
+        <v>57.12</v>
       </c>
       <c r="BK56" t="n">
         <v>6.89</v>
@@ -13392,7 +13392,7 @@
         <v>7.03</v>
       </c>
       <c r="BM56" t="n">
-        <v>60.46</v>
+        <v>58.4</v>
       </c>
       <c r="BN56" t="n">
         <v>86.77</v>
@@ -13401,19 +13401,19 @@
         <v>46.42</v>
       </c>
       <c r="BP56" t="n">
-        <v>57.6</v>
+        <v>57.09</v>
       </c>
       <c r="BQ56" t="n">
-        <v>8.19</v>
+        <v>8.119999999999999</v>
       </c>
       <c r="BR56" t="n">
-        <v>59.63</v>
+        <v>58.29</v>
       </c>
       <c r="BS56" t="n">
         <v>0.79</v>
       </c>
       <c r="BT56" t="n">
-        <v>30470</v>
+        <v>30513</v>
       </c>
     </row>
     <row r="57">
@@ -13443,13 +13443,13 @@
         </is>
       </c>
       <c r="F57" t="n">
-        <v>6</v>
+        <v>5.96</v>
       </c>
       <c r="G57" t="n">
-        <v>1403148000</v>
+        <v>1393793688</v>
       </c>
       <c r="H57" t="n">
-        <v>894900</v>
+        <v>916400</v>
       </c>
       <c r="I57" t="n">
         <v>233858065</v>
@@ -13464,7 +13464,7 @@
         <v>0.77</v>
       </c>
       <c r="M57" t="n">
-        <v>0.4199998832625251</v>
+        <v>0.4171998864353899</v>
       </c>
       <c r="N57" t="n">
         <v>0.08</v>
@@ -13542,7 +13542,7 @@
         <v>229180903.7</v>
       </c>
       <c r="AM57" t="n">
-        <v>104947494.3904263</v>
+        <v>104247845.026178</v>
       </c>
       <c r="AN57" t="n">
         <v>0.347</v>
@@ -13583,7 +13583,7 @@
         <v>10.72</v>
       </c>
       <c r="AZ57" t="n">
-        <v>9.15</v>
+        <v>9.09</v>
       </c>
       <c r="BA57" t="n">
         <v>1.13</v>
@@ -13592,19 +13592,19 @@
         <v>6.26</v>
       </c>
       <c r="BC57" t="n">
-        <v>118.85</v>
+        <v>120.32</v>
       </c>
       <c r="BD57" t="n">
-        <v>78.69</v>
+        <v>79.89</v>
       </c>
       <c r="BE57" t="n">
         <v>52.5</v>
       </c>
       <c r="BF57" t="n">
-        <v>-81.20999999999999</v>
+        <v>-81.08</v>
       </c>
       <c r="BG57" t="n">
-        <v>4.4</v>
+        <v>5.1</v>
       </c>
       <c r="BH57" t="n">
         <v>7.82</v>
@@ -13613,7 +13613,7 @@
         <v>0</v>
       </c>
       <c r="BJ57" t="n">
-        <v>6</v>
+        <v>5.96</v>
       </c>
       <c r="BK57" t="n">
         <v>0.98</v>
@@ -13622,7 +13622,7 @@
         <v>1.04</v>
       </c>
       <c r="BM57" t="n">
-        <v>6.05</v>
+        <v>6.02</v>
       </c>
       <c r="BN57" t="n">
         <v>6.22</v>
@@ -13631,19 +13631,19 @@
         <v>3.43</v>
       </c>
       <c r="BP57" t="n">
-        <v>5.95</v>
+        <v>5.89</v>
       </c>
       <c r="BQ57" t="n">
-        <v>5.79</v>
+        <v>5.75</v>
       </c>
       <c r="BR57" t="n">
-        <v>6.02</v>
+        <v>5.98</v>
       </c>
       <c r="BS57" t="n">
         <v>0.42</v>
       </c>
       <c r="BT57" t="n">
-        <v>1346737</v>
+        <v>1348570</v>
       </c>
     </row>
     <row r="58">
@@ -13903,13 +13903,13 @@
         </is>
       </c>
       <c r="F59" t="n">
-        <v>20</v>
+        <v>19.05</v>
       </c>
       <c r="G59" t="n">
         <v>96504000</v>
       </c>
       <c r="H59" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="I59" t="n">
         <v>710143</v>
@@ -14043,7 +14043,7 @@
         <v>35.09</v>
       </c>
       <c r="AZ59" t="n">
-        <v>24.73</v>
+        <v>23.56</v>
       </c>
       <c r="BA59" t="n">
         <v>3.69</v>
@@ -14052,19 +14052,19 @@
         <v>22.8</v>
       </c>
       <c r="BC59" t="n">
-        <v>114.89</v>
+        <v>125.61</v>
       </c>
       <c r="BD59" t="n">
-        <v>75.45999999999999</v>
+        <v>84.20999999999999</v>
       </c>
       <c r="BE59" t="n">
         <v>23.67</v>
       </c>
       <c r="BF59" t="n">
-        <v>-81.56</v>
+        <v>-80.64</v>
       </c>
       <c r="BG59" t="n">
-        <v>13.99</v>
+        <v>19.67</v>
       </c>
       <c r="BH59" t="n">
         <v>30.98</v>
@@ -14073,7 +14073,7 @@
         <v>0</v>
       </c>
       <c r="BJ59" t="n">
-        <v>20</v>
+        <v>19.05</v>
       </c>
       <c r="BK59" t="n">
         <v>2.65</v>
@@ -14082,7 +14082,7 @@
         <v>2.65</v>
       </c>
       <c r="BM59" t="n">
-        <v>20</v>
+        <v>19.05</v>
       </c>
       <c r="BN59" t="n">
         <v>25.98</v>
@@ -14091,19 +14091,19 @@
         <v>15.85</v>
       </c>
       <c r="BP59" t="n">
-        <v>20</v>
+        <v>19.05</v>
       </c>
       <c r="BQ59" t="n">
-        <v>7.54</v>
+        <v>7.18</v>
       </c>
       <c r="BR59" t="n">
-        <v>20</v>
+        <v>19.05</v>
       </c>
       <c r="BS59" t="n">
         <v>1.42</v>
       </c>
       <c r="BT59" t="n">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
     <row r="60">
@@ -14133,13 +14133,13 @@
         </is>
       </c>
       <c r="F60" t="n">
-        <v>370</v>
+        <v>369.94</v>
       </c>
       <c r="G60" t="n">
-        <v>168257463</v>
+        <v>168230216</v>
       </c>
       <c r="H60" t="n">
-        <v>58</v>
+        <v>18</v>
       </c>
       <c r="I60" t="n">
         <v>454750</v>
@@ -14154,7 +14154,7 @@
         <v>0.83</v>
       </c>
       <c r="M60" t="n">
-        <v>12.58542137538558</v>
+        <v>12.58338333814134</v>
       </c>
       <c r="N60" t="n">
         <v>0.68</v>
@@ -14232,7 +14232,7 @@
         <v>59558607.5</v>
       </c>
       <c r="AM60" t="n">
-        <v>-24671182.25806452</v>
+        <v>-24667187.09677419</v>
       </c>
       <c r="AN60" t="n">
         <v>10.0581</v>
@@ -14273,7 +14273,7 @@
         <v>944.87</v>
       </c>
       <c r="AZ60" t="n">
-        <v>2127.5</v>
+        <v>2127.16</v>
       </c>
       <c r="BA60" t="n">
         <v>231.1</v>
@@ -14282,19 +14282,19 @@
         <v>727.97</v>
       </c>
       <c r="BC60" t="n">
-        <v>212.76</v>
+        <v>212.81</v>
       </c>
       <c r="BD60" t="n">
-        <v>155.37</v>
+        <v>155.41</v>
       </c>
       <c r="BE60" t="n">
         <v>475</v>
       </c>
       <c r="BF60" t="n">
-        <v>-37.54</v>
+        <v>-37.53</v>
       </c>
       <c r="BG60" t="n">
-        <v>96.75</v>
+        <v>96.78</v>
       </c>
       <c r="BH60" t="n">
         <v>454.44</v>
@@ -14303,7 +14303,7 @@
         <v>0</v>
       </c>
       <c r="BJ60" t="n">
-        <v>370</v>
+        <v>369.94</v>
       </c>
       <c r="BK60" t="n">
         <v>130.97</v>
@@ -14312,7 +14312,7 @@
         <v>130.97</v>
       </c>
       <c r="BM60" t="n">
-        <v>385.05</v>
+        <v>388</v>
       </c>
       <c r="BN60" t="n">
         <v>405</v>
@@ -14321,13 +14321,13 @@
         <v>309.24</v>
       </c>
       <c r="BP60" t="n">
-        <v>370</v>
+        <v>369.92</v>
       </c>
       <c r="BQ60" t="n">
-        <v>2.83</v>
+        <v>2.82</v>
       </c>
       <c r="BR60" t="n">
-        <v>385.05</v>
+        <v>386.99</v>
       </c>
       <c r="BS60" t="n">
         <v>12.82</v>
@@ -14363,13 +14363,13 @@
         </is>
       </c>
       <c r="F61" t="n">
-        <v>27.82</v>
+        <v>27.5</v>
       </c>
       <c r="G61" t="n">
-        <v>2381624827</v>
+        <v>2354230175</v>
       </c>
       <c r="H61" t="n">
-        <v>919400</v>
+        <v>436200</v>
       </c>
       <c r="I61" t="n">
         <v>85608392</v>
@@ -14384,7 +14384,7 @@
         <v>2.37</v>
       </c>
       <c r="M61" t="n">
-        <v>1.263057415424043</v>
+        <v>1.248529090912434</v>
       </c>
       <c r="N61" t="n">
         <v>1.1</v>
@@ -14462,7 +14462,7 @@
         <v>160087693.04</v>
       </c>
       <c r="AM61" t="n">
-        <v>186940724.2543171</v>
+        <v>184790437.5981162</v>
       </c>
       <c r="AN61" t="n">
         <v>0.38</v>
@@ -14503,7 +14503,7 @@
         <v>17.56</v>
       </c>
       <c r="AZ61" t="n">
-        <v>35.05</v>
+        <v>34.65</v>
       </c>
       <c r="BA61" t="n">
         <v>2.52</v>
@@ -14512,19 +14512,19 @@
         <v>11.76</v>
       </c>
       <c r="BC61" t="n">
-        <v>-22.7</v>
+        <v>-21.81</v>
       </c>
       <c r="BD61" t="n">
-        <v>-36.89</v>
+        <v>-36.15</v>
       </c>
       <c r="BE61" t="n">
         <v>26</v>
       </c>
       <c r="BF61" t="n">
-        <v>-90.93000000000001</v>
+        <v>-90.83</v>
       </c>
       <c r="BG61" t="n">
-        <v>-57.74</v>
+        <v>-57.25</v>
       </c>
       <c r="BH61" t="n">
         <v>10.99</v>
@@ -14533,7 +14533,7 @@
         <v>0</v>
       </c>
       <c r="BJ61" t="n">
-        <v>27.82</v>
+        <v>27.5</v>
       </c>
       <c r="BK61" t="n">
         <v>1.87</v>
@@ -14542,7 +14542,7 @@
         <v>1.86</v>
       </c>
       <c r="BM61" t="n">
-        <v>28.1</v>
+        <v>27.97</v>
       </c>
       <c r="BN61" t="n">
         <v>28.68</v>
@@ -14551,19 +14551,19 @@
         <v>19.35</v>
       </c>
       <c r="BP61" t="n">
-        <v>27.42</v>
+        <v>27.28</v>
       </c>
       <c r="BQ61" t="n">
-        <v>14.94</v>
+        <v>14.77</v>
       </c>
       <c r="BR61" t="n">
-        <v>27.64</v>
+        <v>27.82</v>
       </c>
       <c r="BS61" t="n">
         <v>1.19</v>
       </c>
       <c r="BT61" t="n">
-        <v>564603</v>
+        <v>573750</v>
       </c>
     </row>
     <row r="62">
@@ -14593,13 +14593,13 @@
         </is>
       </c>
       <c r="F62" t="n">
-        <v>111.75</v>
+        <v>111.5</v>
       </c>
       <c r="G62" t="n">
-        <v>11029693710</v>
+        <v>11005024355</v>
       </c>
       <c r="H62" t="n">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="I62" t="n">
         <v>98699749</v>
@@ -14614,7 +14614,7 @@
         <v>0.64</v>
       </c>
       <c r="M62" t="n">
-        <v>1.033907176531848</v>
+        <v>1.031594707677723</v>
       </c>
       <c r="N62" t="n">
         <v>0.13</v>
@@ -14692,7 +14692,7 @@
         <v>2757670987.06</v>
       </c>
       <c r="AM62" t="n">
-        <v>4465463040.485829</v>
+        <v>4455475447.368421</v>
       </c>
       <c r="AN62" t="n">
         <v>6.9319</v>
@@ -14733,7 +14733,7 @@
         <v>267.2</v>
       </c>
       <c r="AZ62" t="n">
-        <v>118.08</v>
+        <v>117.82</v>
       </c>
       <c r="BA62" t="n">
         <v>34.09</v>
@@ -14742,19 +14742,19 @@
         <v>76.01000000000001</v>
       </c>
       <c r="BC62" t="n">
-        <v>192.84</v>
+        <v>193.49</v>
       </c>
       <c r="BD62" t="n">
-        <v>139.1</v>
+        <v>139.64</v>
       </c>
       <c r="BE62" t="n">
         <v>5.67</v>
       </c>
       <c r="BF62" t="n">
-        <v>-69.48999999999999</v>
+        <v>-69.42</v>
       </c>
       <c r="BG62" t="n">
-        <v>-31.98</v>
+        <v>-31.83</v>
       </c>
       <c r="BH62" t="n">
         <v>170.35</v>
@@ -14763,7 +14763,7 @@
         <v>0</v>
       </c>
       <c r="BJ62" t="n">
-        <v>111.75</v>
+        <v>111.5</v>
       </c>
       <c r="BK62" t="n">
         <v>27.94</v>
@@ -14772,7 +14772,7 @@
         <v>32.73</v>
       </c>
       <c r="BM62" t="n">
-        <v>111.75</v>
+        <v>111.5</v>
       </c>
       <c r="BN62" t="n">
         <v>122.2</v>
@@ -14781,19 +14781,19 @@
         <v>91.84999999999999</v>
       </c>
       <c r="BP62" t="n">
-        <v>109.01</v>
+        <v>109</v>
       </c>
       <c r="BQ62" t="n">
         <v>3.41</v>
       </c>
       <c r="BR62" t="n">
-        <v>109.01</v>
+        <v>111.5</v>
       </c>
       <c r="BS62" t="n">
         <v>1.01</v>
       </c>
       <c r="BT62" t="n">
-        <v>150</v>
+        <v>157</v>
       </c>
     </row>
     <row r="63">
@@ -14823,13 +14823,13 @@
         </is>
       </c>
       <c r="F63" t="n">
-        <v>1.38</v>
+        <v>1.39</v>
       </c>
       <c r="G63" t="n">
-        <v>359503384</v>
+        <v>362108479</v>
       </c>
       <c r="H63" t="n">
-        <v>4000</v>
+        <v>7000</v>
       </c>
       <c r="I63" t="n">
         <v>122894462</v>
@@ -14844,7 +14844,7 @@
         <v>-0.22</v>
       </c>
       <c r="M63" t="n">
-        <v>0.4421706097458084</v>
+        <v>0.4453747421569674</v>
       </c>
       <c r="N63" t="n">
         <v>0.37</v>
@@ -14922,7 +14922,7 @@
         <v>31952560.12</v>
       </c>
       <c r="AM63" t="n">
-        <v>204263286.3636364</v>
+        <v>205743453.9772727</v>
       </c>
       <c r="AN63" t="n">
         <v>0</v>
@@ -14981,7 +14981,7 @@
         <v>-100</v>
       </c>
       <c r="BF63" t="n">
-        <v>-79.05</v>
+        <v>-79.2</v>
       </c>
       <c r="BG63" t="n">
         <v>-100</v>
@@ -14993,7 +14993,7 @@
         <v>0</v>
       </c>
       <c r="BJ63" t="n">
-        <v>1.38</v>
+        <v>1.39</v>
       </c>
       <c r="BK63" t="n">
         <v>0.26</v>
@@ -15002,7 +15002,7 @@
         <v>0.26</v>
       </c>
       <c r="BM63" t="n">
-        <v>1.42</v>
+        <v>1.39</v>
       </c>
       <c r="BN63" t="n">
         <v>2.12</v>
@@ -15014,16 +15014,16 @@
         <v>1.35</v>
       </c>
       <c r="BQ63" t="n">
-        <v>5.29</v>
+        <v>5.32</v>
       </c>
       <c r="BR63" t="n">
-        <v>1.35</v>
+        <v>1.36</v>
       </c>
       <c r="BS63" t="n">
         <v>0.19</v>
       </c>
       <c r="BT63" t="n">
-        <v>25973</v>
+        <v>25083</v>
       </c>
     </row>
     <row r="64">
@@ -15056,10 +15056,10 @@
         <v>62.7</v>
       </c>
       <c r="G64" t="n">
-        <v>235893892970</v>
+        <v>238621970003</v>
       </c>
       <c r="H64" t="n">
-        <v>9817700</v>
+        <v>6187000</v>
       </c>
       <c r="I64" t="n">
         <v>0</v>
@@ -15146,13 +15146,13 @@
         <v>41.22</v>
       </c>
       <c r="AK64" t="n">
-        <v>67634240661.98978</v>
+        <v>68416420379.6217</v>
       </c>
       <c r="AL64" t="n">
-        <v>18856426296.56275</v>
+        <v>19074498001.83853</v>
       </c>
       <c r="AM64" t="n">
-        <v>21005689489.75957</v>
+        <v>21248617097.32858</v>
       </c>
       <c r="AN64" t="n">
         <v>1.4201</v>
@@ -15232,7 +15232,7 @@
         <v>1.57</v>
       </c>
       <c r="BM64" t="n">
-        <v>63.86</v>
+        <v>63.1</v>
       </c>
       <c r="BN64" t="n">
         <v>64.72</v>
@@ -15241,19 +15241,19 @@
         <v>44.12</v>
       </c>
       <c r="BP64" t="n">
-        <v>62.5</v>
+        <v>61.9</v>
       </c>
       <c r="BQ64" t="n">
         <v>39.93</v>
       </c>
       <c r="BR64" t="n">
-        <v>63.83</v>
+        <v>62.6</v>
       </c>
       <c r="BS64" t="n">
         <v>3.49</v>
       </c>
       <c r="BT64" t="n">
-        <v>11307657</v>
+        <v>10886183</v>
       </c>
     </row>
     <row r="65">
@@ -15283,13 +15283,13 @@
         </is>
       </c>
       <c r="F65" t="n">
-        <v>24.3</v>
+        <v>24.1</v>
       </c>
       <c r="G65" t="n">
-        <v>235893892970</v>
+        <v>238621970003</v>
       </c>
       <c r="H65" t="n">
-        <v>6800</v>
+        <v>3600</v>
       </c>
       <c r="I65" t="n">
         <v>7298813414</v>
@@ -15304,7 +15304,7 @@
         <v>3.29</v>
       </c>
       <c r="M65" t="n">
-        <v>5.702957282632465</v>
+        <v>5.768911117159705</v>
       </c>
       <c r="N65" t="n">
         <v>0.29</v>
@@ -15382,7 +15382,7 @@
         <v>11532125194.12</v>
       </c>
       <c r="AM65" t="n">
-        <v>17669954529.58802</v>
+        <v>17874304869.13858</v>
       </c>
       <c r="AN65" t="n">
         <v>0.4734</v>
@@ -15423,7 +15423,7 @@
         <v>12.99</v>
       </c>
       <c r="AZ65" t="n">
-        <v>8.18</v>
+        <v>8.109999999999999</v>
       </c>
       <c r="BA65" t="n">
         <v>2.23</v>
@@ -15432,19 +15432,19 @@
         <v>3.47</v>
       </c>
       <c r="BC65" t="n">
-        <v>-34.53</v>
+        <v>-33.98</v>
       </c>
       <c r="BD65" t="n">
-        <v>-46.54</v>
+        <v>-46.1</v>
       </c>
       <c r="BE65" t="n">
         <v>-66.33</v>
       </c>
       <c r="BF65" t="n">
-        <v>-90.81999999999999</v>
+        <v>-90.73999999999999</v>
       </c>
       <c r="BG65" t="n">
-        <v>-85.73999999999999</v>
+        <v>-85.62</v>
       </c>
       <c r="BH65" t="n">
         <v>7.12</v>
@@ -15453,7 +15453,7 @@
         <v>0</v>
       </c>
       <c r="BJ65" t="n">
-        <v>24.3</v>
+        <v>24.1</v>
       </c>
       <c r="BK65" t="n">
         <v>1.58</v>
@@ -15462,7 +15462,7 @@
         <v>1.57</v>
       </c>
       <c r="BM65" t="n">
-        <v>24.99</v>
+        <v>24.78</v>
       </c>
       <c r="BN65" t="n">
         <v>46.43</v>
@@ -15471,19 +15471,19 @@
         <v>20.44</v>
       </c>
       <c r="BP65" t="n">
-        <v>24.14</v>
+        <v>24.1</v>
       </c>
       <c r="BQ65" t="n">
-        <v>15.48</v>
+        <v>15.35</v>
       </c>
       <c r="BR65" t="n">
-        <v>24.78</v>
+        <v>24.77</v>
       </c>
       <c r="BS65" t="n">
         <v>4.14</v>
       </c>
       <c r="BT65" t="n">
-        <v>9577</v>
+        <v>9160</v>
       </c>
     </row>
     <row r="66">
@@ -15513,13 +15513,13 @@
         </is>
       </c>
       <c r="F66" t="n">
-        <v>20.6</v>
+        <v>20.3</v>
       </c>
       <c r="G66" t="n">
-        <v>235893892970</v>
+        <v>238621970003</v>
       </c>
       <c r="H66" t="n">
-        <v>500</v>
+        <v>400</v>
       </c>
       <c r="I66" t="n">
         <v>2972355254</v>
@@ -15534,7 +15534,7 @@
         <v>2.75</v>
       </c>
       <c r="M66" t="n">
-        <v>14.00398591585945</v>
+        <v>14.16593988536034</v>
       </c>
       <c r="N66" t="n">
         <v>0.25</v>
@@ -15612,7 +15612,7 @@
         <v>4696321301.320001</v>
       </c>
       <c r="AM66" t="n">
-        <v>21156402956.95067</v>
+        <v>21401073542.86995</v>
       </c>
       <c r="AN66" t="n">
         <v>0.4734</v>
@@ -15653,7 +15653,7 @@
         <v>12.99</v>
       </c>
       <c r="AZ66" t="n">
-        <v>8.27</v>
+        <v>8.15</v>
       </c>
       <c r="BA66" t="n">
         <v>2.23</v>
@@ -15662,19 +15662,19 @@
         <v>3.47</v>
       </c>
       <c r="BC66" t="n">
-        <v>-22.77</v>
+        <v>-21.63</v>
       </c>
       <c r="BD66" t="n">
-        <v>-36.94</v>
+        <v>-36.01</v>
       </c>
       <c r="BE66" t="n">
         <v>-59.83</v>
       </c>
       <c r="BF66" t="n">
-        <v>-89.17</v>
+        <v>-89.01000000000001</v>
       </c>
       <c r="BG66" t="n">
-        <v>-83.18000000000001</v>
+        <v>-82.93000000000001</v>
       </c>
       <c r="BH66" t="n">
         <v>7.12</v>
@@ -15683,7 +15683,7 @@
         <v>0</v>
       </c>
       <c r="BJ66" t="n">
-        <v>20.6</v>
+        <v>20.3</v>
       </c>
       <c r="BK66" t="n">
         <v>1.58</v>
@@ -15692,7 +15692,7 @@
         <v>1.57</v>
       </c>
       <c r="BM66" t="n">
-        <v>20.6</v>
+        <v>20.3</v>
       </c>
       <c r="BN66" t="n">
         <v>21.33</v>
@@ -15701,19 +15701,19 @@
         <v>9.48</v>
       </c>
       <c r="BP66" t="n">
-        <v>20.59</v>
+        <v>20.3</v>
       </c>
       <c r="BQ66" t="n">
-        <v>13.12</v>
+        <v>12.93</v>
       </c>
       <c r="BR66" t="n">
-        <v>20.59</v>
+        <v>20.3</v>
       </c>
       <c r="BS66" t="n">
         <v>3.46</v>
       </c>
       <c r="BT66" t="n">
-        <v>4727</v>
+        <v>4500</v>
       </c>
     </row>
     <row r="67">
@@ -15973,13 +15973,13 @@
         </is>
       </c>
       <c r="F68" t="n">
-        <v>17.93</v>
+        <v>17.98</v>
       </c>
       <c r="G68" t="n">
-        <v>7663690078</v>
+        <v>7624144793</v>
       </c>
       <c r="H68" t="n">
-        <v>52300</v>
+        <v>76100</v>
       </c>
       <c r="I68" t="n">
         <v>137989898</v>
@@ -16072,7 +16072,7 @@
         <v>205604948.02</v>
       </c>
       <c r="AM68" t="n">
-        <v>531462557.4202496</v>
+        <v>528720165.9500694</v>
       </c>
       <c r="AN68" t="n">
         <v>0.1911</v>
@@ -16113,7 +16113,7 @@
         <v>21.39</v>
       </c>
       <c r="AZ68" t="n">
-        <v>33.17</v>
+        <v>33.26</v>
       </c>
       <c r="BA68" t="n">
         <v>1.24</v>
@@ -16122,19 +16122,19 @@
         <v>63.25</v>
       </c>
       <c r="BC68" t="n">
-        <v>46.14</v>
+        <v>45.73</v>
       </c>
       <c r="BD68" t="n">
-        <v>19.32</v>
+        <v>18.99</v>
       </c>
       <c r="BE68" t="n">
         <v>85</v>
       </c>
       <c r="BF68" t="n">
-        <v>-93.09</v>
+        <v>-93.11</v>
       </c>
       <c r="BG68" t="n">
-        <v>252.75</v>
+        <v>251.77</v>
       </c>
       <c r="BH68" t="n">
         <v>20.48</v>
@@ -16143,7 +16143,7 @@
         <v>0</v>
       </c>
       <c r="BJ68" t="n">
-        <v>17.93</v>
+        <v>17.98</v>
       </c>
       <c r="BK68" t="n">
         <v>1.49</v>
@@ -16152,7 +16152,7 @@
         <v>1.49</v>
       </c>
       <c r="BM68" t="n">
-        <v>18.27</v>
+        <v>18.13</v>
       </c>
       <c r="BN68" t="n">
         <v>22.11</v>
@@ -16161,19 +16161,19 @@
         <v>15.39</v>
       </c>
       <c r="BP68" t="n">
-        <v>17.91</v>
+        <v>17.9</v>
       </c>
       <c r="BQ68" t="n">
-        <v>12.06</v>
+        <v>12.09</v>
       </c>
       <c r="BR68" t="n">
-        <v>18.22</v>
+        <v>17.97</v>
       </c>
       <c r="BS68" t="n">
         <v>0</v>
       </c>
       <c r="BT68" t="n">
-        <v>39323</v>
+        <v>40317</v>
       </c>
     </row>
     <row r="69">
@@ -16203,13 +16203,13 @@
         </is>
       </c>
       <c r="F69" t="n">
-        <v>20.35</v>
+        <v>20.24</v>
       </c>
       <c r="G69" t="n">
-        <v>7663690078</v>
+        <v>7624144793</v>
       </c>
       <c r="H69" t="n">
-        <v>1660000</v>
+        <v>2431700</v>
       </c>
       <c r="I69" t="n">
         <v>255106712</v>
@@ -16302,7 +16302,7 @@
         <v>380109000.88</v>
       </c>
       <c r="AM69" t="n">
-        <v>456172028.452381</v>
+        <v>453818142.4404762</v>
       </c>
       <c r="AN69" t="n">
         <v>0.8856000000000001</v>
@@ -16343,7 +16343,7 @@
         <v>21.39</v>
       </c>
       <c r="AZ69" t="n">
-        <v>35.58</v>
+        <v>35.39</v>
       </c>
       <c r="BA69" t="n">
         <v>1.24</v>
@@ -16352,19 +16352,19 @@
         <v>69.59</v>
       </c>
       <c r="BC69" t="n">
-        <v>28.76</v>
+        <v>29.46</v>
       </c>
       <c r="BD69" t="n">
-        <v>5.13</v>
+        <v>5.7</v>
       </c>
       <c r="BE69" t="n">
         <v>74.83</v>
       </c>
       <c r="BF69" t="n">
-        <v>-93.91</v>
+        <v>-93.88</v>
       </c>
       <c r="BG69" t="n">
-        <v>241.95</v>
+        <v>243.81</v>
       </c>
       <c r="BH69" t="n">
         <v>20.48</v>
@@ -16373,7 +16373,7 @@
         <v>0</v>
       </c>
       <c r="BJ69" t="n">
-        <v>20.35</v>
+        <v>20.24</v>
       </c>
       <c r="BK69" t="n">
         <v>1.49</v>
@@ -16382,7 +16382,7 @@
         <v>1.49</v>
       </c>
       <c r="BM69" t="n">
-        <v>20.63</v>
+        <v>20.49</v>
       </c>
       <c r="BN69" t="n">
         <v>25.63</v>
@@ -16391,19 +16391,19 @@
         <v>16.73</v>
       </c>
       <c r="BP69" t="n">
-        <v>20.3</v>
+        <v>20.13</v>
       </c>
       <c r="BQ69" t="n">
-        <v>13.69</v>
+        <v>13.61</v>
       </c>
       <c r="BR69" t="n">
-        <v>20.62</v>
+        <v>20.38</v>
       </c>
       <c r="BS69" t="n">
         <v>0</v>
       </c>
       <c r="BT69" t="n">
-        <v>2103810</v>
+        <v>2102360</v>
       </c>
     </row>
     <row r="70">
@@ -16433,13 +16433,13 @@
         </is>
       </c>
       <c r="F70" t="n">
-        <v>17.48</v>
+        <v>17.41</v>
       </c>
       <c r="G70" t="n">
-        <v>8120459643</v>
+        <v>8087940781</v>
       </c>
       <c r="H70" t="n">
-        <v>1398600</v>
+        <v>1425800</v>
       </c>
       <c r="I70" t="n">
         <v>464557268</v>
@@ -16454,7 +16454,7 @@
         <v>0.68</v>
       </c>
       <c r="M70" t="n">
-        <v>0.640933222704418</v>
+        <v>0.6383665676212533</v>
       </c>
       <c r="N70" t="n">
         <v>0.2</v>
@@ -16532,7 +16532,7 @@
         <v>55746872.16</v>
       </c>
       <c r="AM70" t="n">
-        <v>2680019684.158416</v>
+        <v>2669287386.468647</v>
       </c>
       <c r="AN70" t="n">
         <v>0.1236</v>
@@ -16573,7 +16573,7 @@
         <v>6.9</v>
       </c>
       <c r="AZ70" t="n">
-        <v>2.01</v>
+        <v>2</v>
       </c>
       <c r="BA70" t="n">
         <v>0.12</v>
@@ -16582,10 +16582,10 @@
         <v>1.07</v>
       </c>
       <c r="BC70" t="n">
-        <v>-51.66</v>
+        <v>-51.47</v>
       </c>
       <c r="BD70" t="n">
-        <v>-60.53</v>
+        <v>-60.38</v>
       </c>
       <c r="BE70" t="n">
         <v>-88.5</v>
@@ -16594,7 +16594,7 @@
         <v>-99.31</v>
       </c>
       <c r="BG70" t="n">
-        <v>-93.88</v>
+        <v>-93.86</v>
       </c>
       <c r="BH70" t="n">
         <v>26.44</v>
@@ -16603,7 +16603,7 @@
         <v>0</v>
       </c>
       <c r="BJ70" t="n">
-        <v>17.48</v>
+        <v>17.41</v>
       </c>
       <c r="BK70" t="n">
         <v>0.12</v>
@@ -16612,7 +16612,7 @@
         <v>0.1</v>
       </c>
       <c r="BM70" t="n">
-        <v>17.75</v>
+        <v>17.53</v>
       </c>
       <c r="BN70" t="n">
         <v>22.15</v>
@@ -16621,19 +16621,19 @@
         <v>13.21</v>
       </c>
       <c r="BP70" t="n">
-        <v>17.48</v>
+        <v>17.3</v>
       </c>
       <c r="BQ70" t="n">
-        <v>175.31</v>
+        <v>174.61</v>
       </c>
       <c r="BR70" t="n">
-        <v>17.65</v>
+        <v>17.41</v>
       </c>
       <c r="BS70" t="n">
         <v>0.67</v>
       </c>
       <c r="BT70" t="n">
-        <v>4206477</v>
+        <v>4079570</v>
       </c>
     </row>
     <row r="71">

</xml_diff>

<commit_message>
📊 Dados atualizados - 2026-09-28 06:10
</commit_message>
<xml_diff>
--- a/data/ativos.xlsx
+++ b/data/ativos.xlsx
@@ -3813,7 +3813,7 @@
         <v>8372725593</v>
       </c>
       <c r="H15" t="n">
-        <v>1982200</v>
+        <v>0</v>
       </c>
       <c r="I15" t="n">
         <v>343551533</v>
@@ -8401,7 +8401,7 @@
         <v>90635135379</v>
       </c>
       <c r="H35" t="n">
-        <v>17058300</v>
+        <v>0</v>
       </c>
       <c r="I35" t="n">
         <v>5046500000</v>
@@ -8858,7 +8858,7 @@
         <v>14.95</v>
       </c>
       <c r="G37" t="n">
-        <v>200164949</v>
+        <v>200165000</v>
       </c>
       <c r="H37" t="n">
         <v>200</v>
@@ -8876,7 +8876,7 @@
         <v>0.88</v>
       </c>
       <c r="M37" t="n">
-        <v>1.94877439524693</v>
+        <v>1.948774891774891</v>
       </c>
       <c r="N37" t="n">
         <v>0.5</v>
@@ -8954,7 +8954,7 @@
         <v>11319000</v>
       </c>
       <c r="AM37" t="n">
-        <v>47886351.4354067</v>
+        <v>47886363.63636364</v>
       </c>
       <c r="AN37" t="n">
         <v>0</v>
@@ -9551,7 +9551,7 @@
         <v>123728728524</v>
       </c>
       <c r="H40" t="n">
-        <v>43246900</v>
+        <v>0</v>
       </c>
       <c r="I40" t="n">
         <v>5730834040</v>
@@ -10931,7 +10931,7 @@
         <v>4092216932</v>
       </c>
       <c r="H46" t="n">
-        <v>24223330</v>
+        <v>0</v>
       </c>
       <c r="I46" t="n">
         <v>1000542188</v>
@@ -11158,7 +11158,7 @@
         <v>8.960000000000001</v>
       </c>
       <c r="G47" t="n">
-        <v>3130504845</v>
+        <v>3126713000</v>
       </c>
       <c r="H47" t="n">
         <v>6700</v>
@@ -11176,7 +11176,7 @@
         <v>1.22</v>
       </c>
       <c r="M47" t="n">
-        <v>0.7382090597234067</v>
+        <v>0.7373148990462438</v>
       </c>
       <c r="N47" t="n">
         <v>0.07000000000000001</v>
@@ -11254,7 +11254,7 @@
         <v>322715382</v>
       </c>
       <c r="AM47" t="n">
-        <v>555054050.5319149</v>
+        <v>554381737.5886525</v>
       </c>
       <c r="AN47" t="n">
         <v>0.4132</v>
@@ -11388,7 +11388,7 @@
         <v>9.1</v>
       </c>
       <c r="G48" t="n">
-        <v>3130504845</v>
+        <v>3126713000</v>
       </c>
       <c r="H48" t="n">
         <v>1300</v>
@@ -11406,7 +11406,7 @@
         <v>1.24</v>
       </c>
       <c r="M48" t="n">
-        <v>2.008444571504179</v>
+        <v>2.006011829539764</v>
       </c>
       <c r="N48" t="n">
         <v>0.07000000000000001</v>
@@ -11484,7 +11484,7 @@
         <v>118614883.42</v>
       </c>
       <c r="AM48" t="n">
-        <v>547291056.8181819</v>
+        <v>546628146.8531469</v>
       </c>
       <c r="AN48" t="n">
         <v>0.4132</v>
@@ -11618,7 +11618,7 @@
         <v>48.85</v>
       </c>
       <c r="G49" t="n">
-        <v>933365685</v>
+        <v>953506700</v>
       </c>
       <c r="H49" t="n">
         <v>1000</v>
@@ -11636,7 +11636,7 @@
         <v>1.09</v>
       </c>
       <c r="M49" t="n">
-        <v>0.9442740244739837</v>
+        <v>0.9646504295601004</v>
       </c>
       <c r="N49" t="n">
         <v>0.08</v>
@@ -11714,7 +11714,7 @@
         <v>84709985.8</v>
       </c>
       <c r="AM49" t="n">
-        <v>233341421.25</v>
+        <v>238376675</v>
       </c>
       <c r="AN49" t="n">
         <v>3.3186</v>
@@ -11848,7 +11848,7 @@
         <v>33.77</v>
       </c>
       <c r="G50" t="n">
-        <v>933365685</v>
+        <v>953506700</v>
       </c>
       <c r="H50" t="n">
         <v>500</v>
@@ -11866,7 +11866,7 @@
         <v>0.8</v>
       </c>
       <c r="M50" t="n">
-        <v>0.9442740244739837</v>
+        <v>0.9646504295601004</v>
       </c>
       <c r="N50" t="n">
         <v>0.06</v>
@@ -11944,7 +11944,7 @@
         <v>84709985.8</v>
       </c>
       <c r="AM50" t="n">
-        <v>318554841.2969283</v>
+        <v>325428907.8498293</v>
       </c>
       <c r="AN50" t="n">
         <v>4.4983</v>
@@ -13906,7 +13906,7 @@
         <v>19.05</v>
       </c>
       <c r="G59" t="n">
-        <v>96504000</v>
+        <v>91920060</v>
       </c>
       <c r="H59" t="n">
         <v>100</v>
@@ -13924,7 +13924,7 @@
         <v>0.61</v>
       </c>
       <c r="M59" t="n">
-        <v>10.25100450802109</v>
+        <v>9.764081793890091</v>
       </c>
       <c r="N59" t="n">
         <v>0.15</v>
@@ -14002,7 +14002,7 @@
         <v>1881878.95</v>
       </c>
       <c r="AM59" t="n">
-        <v>16301351.35135135</v>
+        <v>15527037.16216216</v>
       </c>
       <c r="AN59" t="n">
         <v>1.4</v>
@@ -14596,7 +14596,7 @@
         <v>111.5</v>
       </c>
       <c r="G62" t="n">
-        <v>11005024355</v>
+        <v>11005020000</v>
       </c>
       <c r="H62" t="n">
         <v>300</v>
@@ -14614,7 +14614,7 @@
         <v>0.64</v>
       </c>
       <c r="M62" t="n">
-        <v>1.031594707677723</v>
+        <v>1.031594299446464</v>
       </c>
       <c r="N62" t="n">
         <v>0.13</v>
@@ -14692,7 +14692,7 @@
         <v>2757670987.06</v>
       </c>
       <c r="AM62" t="n">
-        <v>4455475447.368421</v>
+        <v>4455473684.210526</v>
       </c>
       <c r="AN62" t="n">
         <v>6.9319</v>
@@ -15059,7 +15059,7 @@
         <v>238621970003</v>
       </c>
       <c r="H64" t="n">
-        <v>6187000</v>
+        <v>0</v>
       </c>
       <c r="I64" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
📊 Dados atualizados - 2026-09-29 06:27
</commit_message>
<xml_diff>
--- a/data/ativos.xlsx
+++ b/data/ativos.xlsx
@@ -1047,13 +1047,13 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>24.69</v>
+        <v>25</v>
       </c>
       <c r="G3" t="n">
-        <v>3302702363</v>
+        <v>3344172500</v>
       </c>
       <c r="H3" t="n">
-        <v>210500</v>
+        <v>393900</v>
       </c>
       <c r="I3" t="n">
         <v>129510368</v>
@@ -1068,7 +1068,7 @@
         <v>0.88</v>
       </c>
       <c r="M3" t="n">
-        <v>0.8217859037965425</v>
+        <v>0.8321045974811152</v>
       </c>
       <c r="N3" t="n">
         <v>0.09</v>
@@ -1146,7 +1146,7 @@
         <v>506385538.88</v>
       </c>
       <c r="AM3" t="n">
-        <v>645059055.2734375</v>
+        <v>653158691.40625</v>
       </c>
       <c r="AN3" t="n">
         <v>2.7</v>
@@ -1187,7 +1187,7 @@
         <v>40.42</v>
       </c>
       <c r="AZ3" t="n">
-        <v>45.18</v>
+        <v>45.75</v>
       </c>
       <c r="BA3" t="n">
         <v>4.87</v>
@@ -1196,19 +1196,19 @@
         <v>21.14</v>
       </c>
       <c r="BC3" t="n">
-        <v>100.48</v>
+        <v>97.98999999999999</v>
       </c>
       <c r="BD3" t="n">
-        <v>63.69</v>
+        <v>61.66</v>
       </c>
       <c r="BE3" t="n">
         <v>83</v>
       </c>
       <c r="BF3" t="n">
-        <v>-80.28</v>
+        <v>-80.53</v>
       </c>
       <c r="BG3" t="n">
-        <v>-14.4</v>
+        <v>-15.46</v>
       </c>
       <c r="BH3" t="n">
         <v>27.85</v>
@@ -1217,7 +1217,7 @@
         <v>0</v>
       </c>
       <c r="BJ3" t="n">
-        <v>24.69</v>
+        <v>25</v>
       </c>
       <c r="BK3" t="n">
         <v>3.91</v>
@@ -1226,7 +1226,7 @@
         <v>4.39</v>
       </c>
       <c r="BM3" t="n">
-        <v>24.92</v>
+        <v>25</v>
       </c>
       <c r="BN3" t="n">
         <v>27.17</v>
@@ -1235,19 +1235,19 @@
         <v>18.72</v>
       </c>
       <c r="BP3" t="n">
-        <v>24.62</v>
+        <v>24.52</v>
       </c>
       <c r="BQ3" t="n">
-        <v>5.62</v>
+        <v>5.69</v>
       </c>
       <c r="BR3" t="n">
-        <v>24.89</v>
+        <v>24.69</v>
       </c>
       <c r="BS3" t="n">
         <v>0.79</v>
       </c>
       <c r="BT3" t="n">
-        <v>519427</v>
+        <v>511877</v>
       </c>
     </row>
     <row r="4">
@@ -1277,13 +1277,13 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>15.32</v>
+        <v>15.2</v>
       </c>
       <c r="G4" t="n">
-        <v>237224986474</v>
+        <v>235366829046</v>
       </c>
       <c r="H4" t="n">
-        <v>12323400</v>
+        <v>17925900</v>
       </c>
       <c r="I4" t="n">
         <v>15484664889</v>
@@ -1298,7 +1298,7 @@
         <v>2.76</v>
       </c>
       <c r="M4" t="n">
-        <v>2.686105765064926</v>
+        <v>2.665065791772331</v>
       </c>
       <c r="N4" t="n">
         <v>1.76</v>
@@ -1376,7 +1376,7 @@
         <v>16258898133.45</v>
       </c>
       <c r="AM4" t="n">
-        <v>23487622423.16832</v>
+        <v>23303646440.19802</v>
       </c>
       <c r="AN4" t="n">
         <v>0.269</v>
@@ -1417,7 +1417,7 @@
         <v>9.470000000000001</v>
       </c>
       <c r="AZ4" t="n">
-        <v>19.12</v>
+        <v>18.97</v>
       </c>
       <c r="BA4" t="n">
         <v>1.13</v>
@@ -1426,19 +1426,19 @@
         <v>11.39</v>
       </c>
       <c r="BC4" t="n">
-        <v>-24.25</v>
+        <v>-23.66</v>
       </c>
       <c r="BD4" t="n">
-        <v>-38.15</v>
+        <v>-37.66</v>
       </c>
       <c r="BE4" t="n">
         <v>24.83</v>
       </c>
       <c r="BF4" t="n">
-        <v>-92.64</v>
+        <v>-92.58</v>
       </c>
       <c r="BG4" t="n">
-        <v>-25.67</v>
+        <v>-25.09</v>
       </c>
       <c r="BH4" t="n">
         <v>5.7</v>
@@ -1447,7 +1447,7 @@
         <v>0</v>
       </c>
       <c r="BJ4" t="n">
-        <v>15.32</v>
+        <v>15.2</v>
       </c>
       <c r="BK4" t="n">
         <v>1.05</v>
@@ -1456,7 +1456,7 @@
         <v>1.04</v>
       </c>
       <c r="BM4" t="n">
-        <v>15.39</v>
+        <v>15.36</v>
       </c>
       <c r="BN4" t="n">
         <v>16.94</v>
@@ -1465,19 +1465,19 @@
         <v>11.04</v>
       </c>
       <c r="BP4" t="n">
-        <v>15.21</v>
+        <v>15.14</v>
       </c>
       <c r="BQ4" t="n">
-        <v>14.77</v>
+        <v>14.66</v>
       </c>
       <c r="BR4" t="n">
-        <v>15.3</v>
+        <v>15.18</v>
       </c>
       <c r="BS4" t="n">
         <v>2.76</v>
       </c>
       <c r="BT4" t="n">
-        <v>27122850</v>
+        <v>26800337</v>
       </c>
     </row>
     <row r="5">
@@ -1737,13 +1737,13 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>7.33</v>
+        <v>7.4</v>
       </c>
       <c r="G6" t="n">
-        <v>462410846</v>
+        <v>466826786</v>
       </c>
       <c r="H6" t="n">
-        <v>200</v>
+        <v>700</v>
       </c>
       <c r="I6" t="n">
         <v>63084700</v>
@@ -1758,7 +1758,7 @@
         <v>1.91</v>
       </c>
       <c r="M6" t="n">
-        <v>7.198831501107158</v>
+        <v>7.267579040776673</v>
       </c>
       <c r="N6" t="n">
         <v>1.26</v>
@@ -1836,7 +1836,7 @@
         <v>35958279</v>
       </c>
       <c r="AM6" t="n">
-        <v>44207537.8585086</v>
+        <v>44629711.85468451</v>
       </c>
       <c r="AN6" t="n">
         <v>0.5199</v>
@@ -1877,7 +1877,7 @@
         <v>5.74</v>
       </c>
       <c r="AZ6" t="n">
-        <v>8.6</v>
+        <v>8.68</v>
       </c>
       <c r="BA6" t="n">
         <v>0.65</v>
@@ -1886,19 +1886,19 @@
         <v>7.95</v>
       </c>
       <c r="BC6" t="n">
-        <v>-4.01</v>
+        <v>-4.92</v>
       </c>
       <c r="BD6" t="n">
-        <v>-21.63</v>
+        <v>-22.37</v>
       </c>
       <c r="BE6" t="n">
         <v>17.33</v>
       </c>
       <c r="BF6" t="n">
-        <v>-91.15000000000001</v>
+        <v>-91.23999999999999</v>
       </c>
       <c r="BG6" t="n">
-        <v>8.51</v>
+        <v>7.48</v>
       </c>
       <c r="BH6" t="n">
         <v>3.86</v>
@@ -1907,7 +1907,7 @@
         <v>0</v>
       </c>
       <c r="BJ6" t="n">
-        <v>7.33</v>
+        <v>7.4</v>
       </c>
       <c r="BK6" t="n">
         <v>0.57</v>
@@ -1916,7 +1916,7 @@
         <v>0.5600000000000001</v>
       </c>
       <c r="BM6" t="n">
-        <v>7.33</v>
+        <v>7.4</v>
       </c>
       <c r="BN6" t="n">
         <v>8.16</v>
@@ -1925,19 +1925,19 @@
         <v>6.22</v>
       </c>
       <c r="BP6" t="n">
-        <v>7.33</v>
+        <v>7.4</v>
       </c>
       <c r="BQ6" t="n">
-        <v>13.03</v>
+        <v>13.16</v>
       </c>
       <c r="BR6" t="n">
-        <v>7.33</v>
+        <v>7.4</v>
       </c>
       <c r="BS6" t="n">
         <v>7.32</v>
       </c>
       <c r="BT6" t="n">
-        <v>237</v>
+        <v>167</v>
       </c>
     </row>
     <row r="7">
@@ -2430,10 +2430,10 @@
         <v>23.01</v>
       </c>
       <c r="G9" t="n">
-        <v>208480200</v>
+        <v>201081285</v>
       </c>
       <c r="H9" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="I9" t="n">
         <v>8407877</v>
@@ -2448,7 +2448,7 @@
         <v>0.68</v>
       </c>
       <c r="M9" t="n">
-        <v>0.4179023311067924</v>
+        <v>0.4030710721855086</v>
       </c>
       <c r="N9" t="n">
         <v>0.36</v>
@@ -2526,7 +2526,7 @@
         <v>49438316.76</v>
       </c>
       <c r="AM9" t="n">
-        <v>62232895.52238806</v>
+        <v>60024264.17910448</v>
       </c>
       <c r="AN9" t="n">
         <v>0</v>
@@ -2594,7 +2594,7 @@
         <v>35.36</v>
       </c>
       <c r="BI9" t="n">
-        <v>-3.68</v>
+        <v>0</v>
       </c>
       <c r="BJ9" t="n">
         <v>23.01</v>
@@ -2627,7 +2627,7 @@
         <v>0.4</v>
       </c>
       <c r="BT9" t="n">
-        <v>17</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10">
@@ -3117,13 +3117,13 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>4.97</v>
+        <v>4.93</v>
       </c>
       <c r="G12" t="n">
-        <v>476928783</v>
+        <v>473090277</v>
       </c>
       <c r="H12" t="n">
-        <v>464100</v>
+        <v>237500</v>
       </c>
       <c r="I12" t="n">
         <v>95961536</v>
@@ -3138,7 +3138,7 @@
         <v>0.32</v>
       </c>
       <c r="M12" t="n">
-        <v>0.08625184264304754</v>
+        <v>0.08555765469025964</v>
       </c>
       <c r="N12" t="n">
         <v>0.14</v>
@@ -3216,7 +3216,7 @@
         <v>362734606.08</v>
       </c>
       <c r="AM12" t="n">
-        <v>512826648.3870968</v>
+        <v>508699222.5806451</v>
       </c>
       <c r="AN12" t="n">
         <v>0.4208</v>
@@ -3257,7 +3257,7 @@
         <v>30.49</v>
       </c>
       <c r="AZ12" t="n">
-        <v>6.72</v>
+        <v>6.66</v>
       </c>
       <c r="BA12" t="n">
         <v>4.41</v>
@@ -3266,19 +3266,19 @@
         <v>18.12</v>
       </c>
       <c r="BC12" t="n">
-        <v>651.45</v>
+        <v>657.55</v>
       </c>
       <c r="BD12" t="n">
-        <v>513.5599999999999</v>
+        <v>518.54</v>
       </c>
       <c r="BE12" t="n">
         <v>35.17</v>
       </c>
       <c r="BF12" t="n">
-        <v>-11.23</v>
+        <v>-10.51</v>
       </c>
       <c r="BG12" t="n">
-        <v>264.57</v>
+        <v>267.52</v>
       </c>
       <c r="BH12" t="n">
         <v>16.4</v>
@@ -3287,16 +3287,16 @@
         <v>0</v>
       </c>
       <c r="BJ12" t="n">
-        <v>4.97</v>
+        <v>4.93</v>
       </c>
       <c r="BK12" t="n">
         <v>3.78</v>
       </c>
       <c r="BL12" t="n">
-        <v>3.43</v>
+        <v>3.63</v>
       </c>
       <c r="BM12" t="n">
-        <v>4.99</v>
+        <v>4.95</v>
       </c>
       <c r="BN12" t="n">
         <v>8.23</v>
@@ -3305,19 +3305,19 @@
         <v>4.42</v>
       </c>
       <c r="BP12" t="n">
-        <v>4.85</v>
+        <v>4.87</v>
       </c>
       <c r="BQ12" t="n">
-        <v>1.45</v>
+        <v>1.36</v>
       </c>
       <c r="BR12" t="n">
-        <v>4.89</v>
+        <v>4.94</v>
       </c>
       <c r="BS12" t="n">
         <v>0.09</v>
       </c>
       <c r="BT12" t="n">
-        <v>535617</v>
+        <v>494383</v>
       </c>
     </row>
     <row r="13">
@@ -3347,13 +3347,13 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>28.98</v>
+        <v>28.57</v>
       </c>
       <c r="G13" t="n">
-        <v>14611452051</v>
+        <v>14404731002</v>
       </c>
       <c r="H13" t="n">
-        <v>2778400</v>
+        <v>3408200</v>
       </c>
       <c r="I13" t="n">
         <v>504190947</v>
@@ -3368,7 +3368,7 @@
         <v>1.13</v>
       </c>
       <c r="M13" t="n">
-        <v>5.053484854433157</v>
+        <v>4.981988764477982</v>
       </c>
       <c r="N13" t="n">
         <v>0.57</v>
@@ -3446,7 +3446,7 @@
         <v>932753251.95</v>
       </c>
       <c r="AM13" t="n">
-        <v>1520442461.082206</v>
+        <v>1498931425.806452</v>
       </c>
       <c r="AN13" t="n">
         <v>2.6301</v>
@@ -3487,7 +3487,7 @@
         <v>26.6</v>
       </c>
       <c r="AZ13" t="n">
-        <v>52.45</v>
+        <v>51.71</v>
       </c>
       <c r="BA13" t="n">
         <v>2.6</v>
@@ -3496,19 +3496,19 @@
         <v>8.69</v>
       </c>
       <c r="BC13" t="n">
-        <v>12.4</v>
+        <v>14.01</v>
       </c>
       <c r="BD13" t="n">
-        <v>-8.23</v>
+        <v>-6.91</v>
       </c>
       <c r="BE13" t="n">
         <v>81</v>
       </c>
       <c r="BF13" t="n">
-        <v>-91.01000000000001</v>
+        <v>-90.88</v>
       </c>
       <c r="BG13" t="n">
-        <v>-70</v>
+        <v>-69.56999999999999</v>
       </c>
       <c r="BH13" t="n">
         <v>25.49</v>
@@ -3517,7 +3517,7 @@
         <v>0</v>
       </c>
       <c r="BJ13" t="n">
-        <v>28.98</v>
+        <v>28.57</v>
       </c>
       <c r="BK13" t="n">
         <v>1.85</v>
@@ -3526,7 +3526,7 @@
         <v>1.96</v>
       </c>
       <c r="BM13" t="n">
-        <v>29.31</v>
+        <v>28.96</v>
       </c>
       <c r="BN13" t="n">
         <v>32.11</v>
@@ -3535,19 +3535,19 @@
         <v>20.85</v>
       </c>
       <c r="BP13" t="n">
-        <v>28.59</v>
+        <v>28.4</v>
       </c>
       <c r="BQ13" t="n">
-        <v>14.81</v>
+        <v>14.6</v>
       </c>
       <c r="BR13" t="n">
-        <v>29.04</v>
+        <v>28.96</v>
       </c>
       <c r="BS13" t="n">
         <v>5.01</v>
       </c>
       <c r="BT13" t="n">
-        <v>4968973</v>
+        <v>4921580</v>
       </c>
     </row>
     <row r="14">
@@ -3577,13 +3577,13 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>10.39</v>
+        <v>10.2</v>
       </c>
       <c r="G14" t="n">
-        <v>8372725593</v>
+        <v>8511180935</v>
       </c>
       <c r="H14" t="n">
-        <v>3600</v>
+        <v>7800</v>
       </c>
       <c r="I14" t="n">
         <v>339510689</v>
@@ -3598,7 +3598,7 @@
         <v>1.92</v>
       </c>
       <c r="M14" t="n">
-        <v>3.47650451388006</v>
+        <v>3.533993633293722</v>
       </c>
       <c r="N14" t="n">
         <v>1.11</v>
@@ -3676,7 +3676,7 @@
         <v>349696009.67</v>
       </c>
       <c r="AM14" t="n">
-        <v>929270321.0876803</v>
+        <v>944637173.6958935</v>
       </c>
       <c r="AN14" t="n">
         <v>0.1489</v>
@@ -3717,7 +3717,7 @@
         <v>9.050000000000001</v>
       </c>
       <c r="AZ14" t="n">
-        <v>8.35</v>
+        <v>8.19</v>
       </c>
       <c r="BA14" t="n">
         <v>1.42</v>
@@ -3726,19 +3726,19 @@
         <v>5.94</v>
       </c>
       <c r="BC14" t="n">
-        <v>6.67</v>
+        <v>8.65</v>
       </c>
       <c r="BD14" t="n">
-        <v>-12.91</v>
+        <v>-11.28</v>
       </c>
       <c r="BE14" t="n">
         <v>-19.67</v>
       </c>
       <c r="BF14" t="n">
-        <v>-86.31999999999999</v>
+        <v>-86.06999999999999</v>
       </c>
       <c r="BG14" t="n">
-        <v>-42.81</v>
+        <v>-41.74</v>
       </c>
       <c r="BH14" t="n">
         <v>5.3</v>
@@ -3747,7 +3747,7 @@
         <v>0</v>
       </c>
       <c r="BJ14" t="n">
-        <v>10.39</v>
+        <v>10.2</v>
       </c>
       <c r="BK14" t="n">
         <v>1.03</v>
@@ -3762,22 +3762,22 @@
         <v>13.49</v>
       </c>
       <c r="BO14" t="n">
-        <v>7.65</v>
+        <v>7.71</v>
       </c>
       <c r="BP14" t="n">
-        <v>10.1</v>
+        <v>10.05</v>
       </c>
       <c r="BQ14" t="n">
-        <v>10.26</v>
+        <v>10.07</v>
       </c>
       <c r="BR14" t="n">
-        <v>10.1</v>
+        <v>10.38</v>
       </c>
       <c r="BS14" t="n">
         <v>1.44</v>
       </c>
       <c r="BT14" t="n">
-        <v>10950</v>
+        <v>10650</v>
       </c>
     </row>
     <row r="15">
@@ -3807,13 +3807,13 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>13.88</v>
+        <v>14.24</v>
       </c>
       <c r="G15" t="n">
-        <v>8372725593</v>
+        <v>8511180935</v>
       </c>
       <c r="H15" t="n">
-        <v>0</v>
+        <v>1462200</v>
       </c>
       <c r="I15" t="n">
         <v>343551533</v>
@@ -3828,7 +3828,7 @@
         <v>2.56</v>
       </c>
       <c r="M15" t="n">
-        <v>3.435613960188701</v>
+        <v>3.492426894107805</v>
       </c>
       <c r="N15" t="n">
         <v>1.47</v>
@@ -3906,7 +3906,7 @@
         <v>353858078.99</v>
       </c>
       <c r="AM15" t="n">
-        <v>698309056.9641367</v>
+        <v>709856625.1042535</v>
       </c>
       <c r="AN15" t="n">
         <v>0.1638</v>
@@ -3947,7 +3947,7 @@
         <v>9.050000000000001</v>
       </c>
       <c r="AZ15" t="n">
-        <v>9.23</v>
+        <v>9.470000000000001</v>
       </c>
       <c r="BA15" t="n">
         <v>1.42</v>
@@ -3956,19 +3956,19 @@
         <v>6.19</v>
       </c>
       <c r="BC15" t="n">
-        <v>-20.15</v>
+        <v>-22.17</v>
       </c>
       <c r="BD15" t="n">
-        <v>-34.81</v>
+        <v>-36.45</v>
       </c>
       <c r="BE15" t="n">
         <v>-33.5</v>
       </c>
       <c r="BF15" t="n">
-        <v>-89.76000000000001</v>
+        <v>-90.02</v>
       </c>
       <c r="BG15" t="n">
-        <v>-55.42</v>
+        <v>-56.54</v>
       </c>
       <c r="BH15" t="n">
         <v>5.3</v>
@@ -3977,7 +3977,7 @@
         <v>0</v>
       </c>
       <c r="BJ15" t="n">
-        <v>13.88</v>
+        <v>14.24</v>
       </c>
       <c r="BK15" t="n">
         <v>1.03</v>
@@ -3986,7 +3986,7 @@
         <v>1.01</v>
       </c>
       <c r="BM15" t="n">
-        <v>13.93</v>
+        <v>14.3</v>
       </c>
       <c r="BN15" t="n">
         <v>16.22</v>
@@ -3995,19 +3995,19 @@
         <v>7.84</v>
       </c>
       <c r="BP15" t="n">
-        <v>13.31</v>
+        <v>13.62</v>
       </c>
       <c r="BQ15" t="n">
-        <v>13.7</v>
+        <v>14.06</v>
       </c>
       <c r="BR15" t="n">
-        <v>13.32</v>
+        <v>13.85</v>
       </c>
       <c r="BS15" t="n">
         <v>1.92</v>
       </c>
       <c r="BT15" t="n">
-        <v>2353290</v>
+        <v>2377230</v>
       </c>
     </row>
     <row r="16">
@@ -4037,13 +4037,13 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>4.5</v>
+        <v>4.41</v>
       </c>
       <c r="G16" t="n">
-        <v>986875650</v>
+        <v>967138103</v>
       </c>
       <c r="H16" t="n">
-        <v>58800</v>
+        <v>74500</v>
       </c>
       <c r="I16" t="n">
         <v>219305733</v>
@@ -4058,7 +4058,7 @@
         <v>2.69</v>
       </c>
       <c r="M16" t="n">
-        <v>0.4668749297470486</v>
+        <v>0.4575374150672568</v>
       </c>
       <c r="N16" t="n">
         <v>0.39</v>
@@ -4136,7 +4136,7 @@
         <v>17544458.64</v>
       </c>
       <c r="AM16" t="n">
-        <v>277212261.2359551</v>
+        <v>271668006.4606742</v>
       </c>
       <c r="AN16" t="n">
         <v>0.0077</v>
@@ -4177,7 +4177,7 @@
         <v>1.42</v>
       </c>
       <c r="AZ16" t="n">
-        <v>0.13</v>
+        <v>0.12</v>
       </c>
       <c r="BA16" t="n">
         <v>0.08</v>
@@ -4186,16 +4186,16 @@
         <v>0</v>
       </c>
       <c r="BC16" t="n">
-        <v>-61.36</v>
+        <v>-60.57</v>
       </c>
       <c r="BD16" t="n">
-        <v>-68.45</v>
+        <v>-67.8</v>
       </c>
       <c r="BE16" t="n">
         <v>-97.17</v>
       </c>
       <c r="BF16" t="n">
-        <v>-98.22</v>
+        <v>-98.19</v>
       </c>
       <c r="BG16" t="n">
         <v>-100</v>
@@ -4207,7 +4207,7 @@
         <v>0</v>
       </c>
       <c r="BJ16" t="n">
-        <v>4.5</v>
+        <v>4.41</v>
       </c>
       <c r="BK16" t="n">
         <v>0.08</v>
@@ -4216,7 +4216,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="BM16" t="n">
-        <v>4.5</v>
+        <v>4.48</v>
       </c>
       <c r="BN16" t="n">
         <v>5.54</v>
@@ -4225,19 +4225,19 @@
         <v>3.22</v>
       </c>
       <c r="BP16" t="n">
-        <v>4.35</v>
+        <v>4.39</v>
       </c>
       <c r="BQ16" t="n">
-        <v>61.41</v>
+        <v>60.18</v>
       </c>
       <c r="BR16" t="n">
-        <v>4.39</v>
+        <v>4.48</v>
       </c>
       <c r="BS16" t="n">
         <v>0.49</v>
       </c>
       <c r="BT16" t="n">
-        <v>134720</v>
+        <v>133407</v>
       </c>
     </row>
     <row r="17">
@@ -4267,13 +4267,13 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>32.11</v>
+        <v>31.55</v>
       </c>
       <c r="G17" t="n">
-        <v>10584316749</v>
+        <v>10399728443</v>
       </c>
       <c r="H17" t="n">
-        <v>986500</v>
+        <v>887200</v>
       </c>
       <c r="I17" t="n">
         <v>0</v>
@@ -4360,13 +4360,13 @@
         <v>8.039999999999999</v>
       </c>
       <c r="AK17" t="n">
-        <v>4779767318.009394</v>
+        <v>4696409159.591763</v>
       </c>
       <c r="AL17" t="n">
-        <v>1323039593.625</v>
+        <v>1299966055.375</v>
       </c>
       <c r="AM17" t="n">
-        <v>3276878250.464396</v>
+        <v>3219730168.111455</v>
       </c>
       <c r="AN17" t="n">
         <v>1.08</v>
@@ -4407,7 +4407,7 @@
         <v>42.98</v>
       </c>
       <c r="AZ17" t="n">
-        <v>17.18</v>
+        <v>16.88</v>
       </c>
       <c r="BA17" t="n">
         <v>4.55</v>
@@ -4416,19 +4416,19 @@
         <v>16.33</v>
       </c>
       <c r="BC17" t="n">
-        <v>63.93</v>
+        <v>66.84</v>
       </c>
       <c r="BD17" t="n">
-        <v>33.85</v>
+        <v>36.22</v>
       </c>
       <c r="BE17" t="n">
         <v>-46.5</v>
       </c>
       <c r="BF17" t="n">
-        <v>-85.83</v>
+        <v>-85.58</v>
       </c>
       <c r="BG17" t="n">
-        <v>-49.13</v>
+        <v>-48.23</v>
       </c>
       <c r="BH17" t="n">
         <v>29.25</v>
@@ -4437,7 +4437,7 @@
         <v>0</v>
       </c>
       <c r="BJ17" t="n">
-        <v>32.11</v>
+        <v>31.55</v>
       </c>
       <c r="BK17" t="n">
         <v>4.21</v>
@@ -4446,7 +4446,7 @@
         <v>12.62</v>
       </c>
       <c r="BM17" t="n">
-        <v>32.21</v>
+        <v>32.08</v>
       </c>
       <c r="BN17" t="n">
         <v>36.63</v>
@@ -4455,19 +4455,19 @@
         <v>29.53</v>
       </c>
       <c r="BP17" t="n">
-        <v>31.84</v>
+        <v>31.55</v>
       </c>
       <c r="BQ17" t="n">
-        <v>2.54</v>
+        <v>2.5</v>
       </c>
       <c r="BR17" t="n">
-        <v>31.91</v>
+        <v>32</v>
       </c>
       <c r="BS17" t="n">
         <v>2.21</v>
       </c>
       <c r="BT17" t="n">
-        <v>1174540</v>
+        <v>1153147</v>
       </c>
     </row>
     <row r="18">
@@ -4497,13 +4497,13 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>11.2</v>
+        <v>11</v>
       </c>
       <c r="G18" t="n">
-        <v>10584316749</v>
+        <v>10399728443</v>
       </c>
       <c r="H18" t="n">
-        <v>3500</v>
+        <v>4800</v>
       </c>
       <c r="I18" t="n">
         <v>671494278</v>
@@ -4518,7 +4518,7 @@
         <v>1.2</v>
       </c>
       <c r="M18" t="n">
-        <v>3.116438507912775</v>
+        <v>3.062088461653706</v>
       </c>
       <c r="N18" t="n">
         <v>0.33</v>
@@ -4596,7 +4596,7 @@
         <v>940091989.1999999</v>
       </c>
       <c r="AM18" t="n">
-        <v>3150094270.535715</v>
+        <v>3095157274.702381</v>
       </c>
       <c r="AN18" t="n">
         <v>0.36</v>
@@ -4637,7 +4637,7 @@
         <v>14.31</v>
       </c>
       <c r="AZ18" t="n">
-        <v>5.77</v>
+        <v>5.66</v>
       </c>
       <c r="BA18" t="n">
         <v>1.51</v>
@@ -4646,19 +4646,19 @@
         <v>5.44</v>
       </c>
       <c r="BC18" t="n">
-        <v>56.47</v>
+        <v>59.32</v>
       </c>
       <c r="BD18" t="n">
-        <v>27.76</v>
+        <v>30.08</v>
       </c>
       <c r="BE18" t="n">
         <v>-48.5</v>
       </c>
       <c r="BF18" t="n">
-        <v>-86.5</v>
+        <v>-86.25</v>
       </c>
       <c r="BG18" t="n">
-        <v>-51.39</v>
+        <v>-50.51</v>
       </c>
       <c r="BH18" t="n">
         <v>9.75</v>
@@ -4667,7 +4667,7 @@
         <v>0</v>
       </c>
       <c r="BJ18" t="n">
-        <v>11.2</v>
+        <v>11</v>
       </c>
       <c r="BK18" t="n">
         <v>1.4</v>
@@ -4685,19 +4685,19 @@
         <v>10.19</v>
       </c>
       <c r="BP18" t="n">
-        <v>10.99</v>
+        <v>10.96</v>
       </c>
       <c r="BQ18" t="n">
-        <v>0.89</v>
+        <v>0.87</v>
       </c>
       <c r="BR18" t="n">
-        <v>11.18</v>
+        <v>11.07</v>
       </c>
       <c r="BS18" t="n">
         <v>2.3</v>
       </c>
       <c r="BT18" t="n">
-        <v>10457</v>
+        <v>10103</v>
       </c>
     </row>
     <row r="19">
@@ -4727,13 +4727,13 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>10.53</v>
+        <v>10.52</v>
       </c>
       <c r="G19" t="n">
-        <v>10584316749</v>
+        <v>10399728443</v>
       </c>
       <c r="H19" t="n">
-        <v>3900</v>
+        <v>14100</v>
       </c>
       <c r="I19" t="n">
         <v>317386323</v>
@@ -4748,7 +4748,7 @@
         <v>1.12</v>
       </c>
       <c r="M19" t="n">
-        <v>6.593449289250835</v>
+        <v>6.47846089048483</v>
       </c>
       <c r="N19" t="n">
         <v>0.3</v>
@@ -4826,7 +4826,7 @@
         <v>444340852.2</v>
       </c>
       <c r="AM19" t="n">
-        <v>3360100555.238095</v>
+        <v>3301501093.015873</v>
       </c>
       <c r="AN19" t="n">
         <v>0.36</v>
@@ -4876,19 +4876,19 @@
         <v>5.25</v>
       </c>
       <c r="BC19" t="n">
-        <v>66.43000000000001</v>
+        <v>66.59</v>
       </c>
       <c r="BD19" t="n">
-        <v>35.89</v>
+        <v>36.02</v>
       </c>
       <c r="BE19" t="n">
         <v>-45</v>
       </c>
       <c r="BF19" t="n">
-        <v>-85.64</v>
+        <v>-85.62</v>
       </c>
       <c r="BG19" t="n">
-        <v>-50.14</v>
+        <v>-50.1</v>
       </c>
       <c r="BH19" t="n">
         <v>9.75</v>
@@ -4897,7 +4897,7 @@
         <v>0</v>
       </c>
       <c r="BJ19" t="n">
-        <v>10.53</v>
+        <v>10.52</v>
       </c>
       <c r="BK19" t="n">
         <v>1.4</v>
@@ -4906,7 +4906,7 @@
         <v>12.62</v>
       </c>
       <c r="BM19" t="n">
-        <v>10.57</v>
+        <v>10.58</v>
       </c>
       <c r="BN19" t="n">
         <v>11.41</v>
@@ -4915,19 +4915,19 @@
         <v>9.19</v>
       </c>
       <c r="BP19" t="n">
-        <v>10.4</v>
+        <v>10.34</v>
       </c>
       <c r="BQ19" t="n">
         <v>0.83</v>
       </c>
       <c r="BR19" t="n">
-        <v>10.41</v>
+        <v>10.58</v>
       </c>
       <c r="BS19" t="n">
         <v>2.16</v>
       </c>
       <c r="BT19" t="n">
-        <v>13273</v>
+        <v>12983</v>
       </c>
     </row>
     <row r="20">
@@ -5417,13 +5417,13 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>5.16</v>
+        <v>5.03</v>
       </c>
       <c r="G22" t="n">
-        <v>1033265717</v>
+        <v>1007233901</v>
       </c>
       <c r="H22" t="n">
-        <v>1631500</v>
+        <v>1465600</v>
       </c>
       <c r="I22" t="n">
         <v>200245299</v>
@@ -5438,7 +5438,7 @@
         <v>0.27</v>
       </c>
       <c r="M22" t="n">
-        <v>0.08763809304643409</v>
+        <v>0.0854301627190838</v>
       </c>
       <c r="N22" t="n">
         <v>0.08</v>
@@ -5516,7 +5516,7 @@
         <v>378463615.11</v>
       </c>
       <c r="AM22" t="n">
-        <v>234300616.0997732</v>
+        <v>228397709.9773242</v>
       </c>
       <c r="AN22" t="n">
         <v>0</v>
@@ -5566,19 +5566,19 @@
         <v>172.49</v>
       </c>
       <c r="BC22" t="n">
-        <v>475.68</v>
+        <v>490.56</v>
       </c>
       <c r="BD22" t="n">
-        <v>370.04</v>
+        <v>382.19</v>
       </c>
       <c r="BE22" t="n">
         <v>-100</v>
       </c>
       <c r="BF22" t="n">
-        <v>-63.37</v>
+        <v>-62.43</v>
       </c>
       <c r="BG22" t="n">
-        <v>3242.82</v>
+        <v>3329.22</v>
       </c>
       <c r="BH22" t="n">
         <v>20.75</v>
@@ -5587,7 +5587,7 @@
         <v>0</v>
       </c>
       <c r="BJ22" t="n">
-        <v>5.16</v>
+        <v>5.03</v>
       </c>
       <c r="BK22" t="n">
         <v>1.89</v>
@@ -5596,7 +5596,7 @@
         <v>0.67</v>
       </c>
       <c r="BM22" t="n">
-        <v>5.29</v>
+        <v>5.32</v>
       </c>
       <c r="BN22" t="n">
         <v>7.89</v>
@@ -5605,19 +5605,19 @@
         <v>3.37</v>
       </c>
       <c r="BP22" t="n">
-        <v>5.03</v>
+        <v>5.01</v>
       </c>
       <c r="BQ22" t="n">
-        <v>7.69</v>
+        <v>7.49</v>
       </c>
       <c r="BR22" t="n">
-        <v>5.25</v>
+        <v>5.16</v>
       </c>
       <c r="BS22" t="n">
         <v>0.09</v>
       </c>
       <c r="BT22" t="n">
-        <v>1534617</v>
+        <v>1516587</v>
       </c>
     </row>
     <row r="23">
@@ -5877,13 +5877,13 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.93</v>
+        <v>2.83</v>
       </c>
       <c r="G24" t="n">
-        <v>1183335024</v>
+        <v>1142948956</v>
       </c>
       <c r="H24" t="n">
-        <v>4912300</v>
+        <v>6200400</v>
       </c>
       <c r="I24" t="n">
         <v>403868805</v>
@@ -5898,7 +5898,7 @@
         <v>0.49</v>
       </c>
       <c r="M24" t="n">
-        <v>0.2860603873994232</v>
+        <v>0.2762974259191084</v>
       </c>
       <c r="N24" t="n">
         <v>0.11</v>
@@ -5976,7 +5976,7 @@
         <v>153470145.9</v>
       </c>
       <c r="AM24" t="n">
-        <v>1066067589.189189</v>
+        <v>1029683744.144144</v>
       </c>
       <c r="AN24" t="n">
         <v>0.0813</v>
@@ -6017,7 +6017,7 @@
         <v>5.84</v>
       </c>
       <c r="AZ24" t="n">
-        <v>1.35</v>
+        <v>1.31</v>
       </c>
       <c r="BA24" t="n">
         <v>0.38</v>
@@ -6026,19 +6026,19 @@
         <v>1.46</v>
       </c>
       <c r="BC24" t="n">
-        <v>144.25</v>
+        <v>152.88</v>
       </c>
       <c r="BD24" t="n">
-        <v>99.43000000000001</v>
+        <v>106.47</v>
       </c>
       <c r="BE24" t="n">
         <v>-53.83</v>
       </c>
       <c r="BF24" t="n">
-        <v>-87.03</v>
+        <v>-86.56999999999999</v>
       </c>
       <c r="BG24" t="n">
-        <v>-50.25</v>
+        <v>-48.49</v>
       </c>
       <c r="BH24" t="n">
         <v>5.99</v>
@@ -6047,7 +6047,7 @@
         <v>0</v>
       </c>
       <c r="BJ24" t="n">
-        <v>2.93</v>
+        <v>2.83</v>
       </c>
       <c r="BK24" t="n">
         <v>0.38</v>
@@ -6056,7 +6056,7 @@
         <v>0.41</v>
       </c>
       <c r="BM24" t="n">
-        <v>3.05</v>
+        <v>2.92</v>
       </c>
       <c r="BN24" t="n">
         <v>5.29</v>
@@ -6065,19 +6065,19 @@
         <v>1.92</v>
       </c>
       <c r="BP24" t="n">
-        <v>2.9</v>
+        <v>2.79</v>
       </c>
       <c r="BQ24" t="n">
-        <v>7.2</v>
+        <v>6.95</v>
       </c>
       <c r="BR24" t="n">
-        <v>3</v>
+        <v>2.92</v>
       </c>
       <c r="BS24" t="n">
         <v>0.29</v>
       </c>
       <c r="BT24" t="n">
-        <v>7841887</v>
+        <v>7743583</v>
       </c>
     </row>
     <row r="25">
@@ -6107,13 +6107,13 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>4.22</v>
+        <v>3.89</v>
       </c>
       <c r="G25" t="n">
-        <v>1462204607</v>
+        <v>1347861696</v>
       </c>
       <c r="H25" t="n">
-        <v>3648200</v>
+        <v>1645100</v>
       </c>
       <c r="I25" t="n">
         <v>346494097</v>
@@ -6128,7 +6128,7 @@
         <v>0.97</v>
       </c>
       <c r="M25" t="n">
-        <v>0.7291219817054744</v>
+        <v>0.6721053853528323</v>
       </c>
       <c r="N25" t="n">
         <v>0.22</v>
@@ -6206,7 +6206,7 @@
         <v>62368937.46</v>
       </c>
       <c r="AM25" t="n">
-        <v>537575223.1617646</v>
+        <v>495537388.2352941</v>
       </c>
       <c r="AN25" t="n">
         <v>0.4742</v>
@@ -6247,7 +6247,7 @@
         <v>3.27</v>
       </c>
       <c r="AZ25" t="n">
-        <v>9.83</v>
+        <v>9.06</v>
       </c>
       <c r="BA25" t="n">
         <v>0.23</v>
@@ -6256,19 +6256,19 @@
         <v>2.2</v>
       </c>
       <c r="BC25" t="n">
-        <v>-4.98</v>
+        <v>3.08</v>
       </c>
       <c r="BD25" t="n">
-        <v>-22.42</v>
+        <v>-15.84</v>
       </c>
       <c r="BE25" t="n">
         <v>133</v>
       </c>
       <c r="BF25" t="n">
-        <v>-94.51000000000001</v>
+        <v>-94.04000000000001</v>
       </c>
       <c r="BG25" t="n">
-        <v>-47.87</v>
+        <v>-43.45</v>
       </c>
       <c r="BH25" t="n">
         <v>3.97</v>
@@ -6277,7 +6277,7 @@
         <v>0</v>
       </c>
       <c r="BJ25" t="n">
-        <v>4.22</v>
+        <v>3.89</v>
       </c>
       <c r="BK25" t="n">
         <v>0.18</v>
@@ -6286,7 +6286,7 @@
         <v>0.24</v>
       </c>
       <c r="BM25" t="n">
-        <v>4.66</v>
+        <v>4.2</v>
       </c>
       <c r="BN25" t="n">
         <v>6.3</v>
@@ -6295,19 +6295,19 @@
         <v>2.64</v>
       </c>
       <c r="BP25" t="n">
-        <v>4.01</v>
+        <v>3.85</v>
       </c>
       <c r="BQ25" t="n">
-        <v>17.83</v>
+        <v>16.44</v>
       </c>
       <c r="BR25" t="n">
-        <v>4.66</v>
+        <v>4.17</v>
       </c>
       <c r="BS25" t="n">
         <v>0.67</v>
       </c>
       <c r="BT25" t="n">
-        <v>1099787</v>
+        <v>1133717</v>
       </c>
     </row>
     <row r="26">
@@ -6337,13 +6337,13 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>10.49</v>
+        <v>10.2</v>
       </c>
       <c r="G26" t="n">
-        <v>14207582260</v>
+        <v>13814808341</v>
       </c>
       <c r="H26" t="n">
-        <v>16425200</v>
+        <v>12189300</v>
       </c>
       <c r="I26" t="n">
         <v>1354393401</v>
@@ -6358,7 +6358,7 @@
         <v>1.94</v>
       </c>
       <c r="M26" t="n">
-        <v>0.1832055755630591</v>
+        <v>0.1781407889878552</v>
       </c>
       <c r="N26" t="n">
         <v>0.26</v>
@@ -6436,7 +6436,7 @@
         <v>961619314.7099999</v>
       </c>
       <c r="AM26" t="n">
-        <v>5074136521.428572</v>
+        <v>4933860121.785714</v>
       </c>
       <c r="AN26" t="n">
         <v>0.1043</v>
@@ -6477,7 +6477,7 @@
         <v>7.07</v>
       </c>
       <c r="AZ26" t="n">
-        <v>2.01</v>
+        <v>1.95</v>
       </c>
       <c r="BA26" t="n">
         <v>0.66</v>
@@ -6486,19 +6486,19 @@
         <v>1.19</v>
       </c>
       <c r="BC26" t="n">
-        <v>-17.49</v>
+        <v>-15.14</v>
       </c>
       <c r="BD26" t="n">
-        <v>-32.63</v>
+        <v>-30.71</v>
       </c>
       <c r="BE26" t="n">
         <v>-80.83</v>
       </c>
       <c r="BF26" t="n">
-        <v>-93.72</v>
+        <v>-93.54000000000001</v>
       </c>
       <c r="BG26" t="n">
-        <v>-88.62</v>
+        <v>-88.3</v>
       </c>
       <c r="BH26" t="n">
         <v>4.69</v>
@@ -6507,7 +6507,7 @@
         <v>0</v>
       </c>
       <c r="BJ26" t="n">
-        <v>10.49</v>
+        <v>10.2</v>
       </c>
       <c r="BK26" t="n">
         <v>0.71</v>
@@ -6516,7 +6516,7 @@
         <v>0.72</v>
       </c>
       <c r="BM26" t="n">
-        <v>10.5</v>
+        <v>10.48</v>
       </c>
       <c r="BN26" t="n">
         <v>10.55</v>
@@ -6525,19 +6525,19 @@
         <v>6.91</v>
       </c>
       <c r="BP26" t="n">
-        <v>10.05</v>
+        <v>10.19</v>
       </c>
       <c r="BQ26" t="n">
-        <v>14.63</v>
+        <v>14.22</v>
       </c>
       <c r="BR26" t="n">
-        <v>10.22</v>
+        <v>10.35</v>
       </c>
       <c r="BS26" t="n">
         <v>0.16</v>
       </c>
       <c r="BT26" t="n">
-        <v>12118290</v>
+        <v>12366230</v>
       </c>
     </row>
     <row r="27">
@@ -8165,13 +8165,13 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>16.38</v>
+        <v>15.52</v>
       </c>
       <c r="G34" t="n">
-        <v>3382301112</v>
+        <v>3204721790</v>
       </c>
       <c r="H34" t="n">
-        <v>9668900</v>
+        <v>3819600</v>
       </c>
       <c r="I34" t="n">
         <v>206489813</v>
@@ -8186,7 +8186,7 @@
         <v>0.45</v>
       </c>
       <c r="M34" t="n">
-        <v>0.2973437710287099</v>
+        <v>0.2817324746030705</v>
       </c>
       <c r="N34" t="n">
         <v>0.24</v>
@@ -8264,7 +8264,7 @@
         <v>324189006.41</v>
       </c>
       <c r="AM34" t="n">
-        <v>703181104.3659045</v>
+        <v>666262326.4033265</v>
       </c>
       <c r="AN34" t="n">
         <v>0</v>
@@ -8305,7 +8305,7 @@
         <v>30.28</v>
       </c>
       <c r="AZ34" t="n">
-        <v>38.22</v>
+        <v>36.21</v>
       </c>
       <c r="BA34" t="n">
         <v>2.29</v>
@@ -8314,19 +8314,19 @@
         <v>25.26</v>
       </c>
       <c r="BC34" t="n">
-        <v>126.43</v>
+        <v>138.97</v>
       </c>
       <c r="BD34" t="n">
-        <v>84.88</v>
+        <v>95.12</v>
       </c>
       <c r="BE34" t="n">
         <v>133.33</v>
       </c>
       <c r="BF34" t="n">
-        <v>-85.98999999999999</v>
+        <v>-85.20999999999999</v>
       </c>
       <c r="BG34" t="n">
-        <v>54.2</v>
+        <v>62.74</v>
       </c>
       <c r="BH34" t="n">
         <v>38.94</v>
@@ -8335,7 +8335,7 @@
         <v>0</v>
       </c>
       <c r="BJ34" t="n">
-        <v>16.38</v>
+        <v>15.52</v>
       </c>
       <c r="BK34" t="n">
         <v>1.57</v>
@@ -8344,7 +8344,7 @@
         <v>1.58</v>
       </c>
       <c r="BM34" t="n">
-        <v>17.32</v>
+        <v>16.22</v>
       </c>
       <c r="BN34" t="n">
         <v>28.86</v>
@@ -8353,19 +8353,19 @@
         <v>14.3</v>
       </c>
       <c r="BP34" t="n">
-        <v>14.39</v>
+        <v>15.44</v>
       </c>
       <c r="BQ34" t="n">
-        <v>10.39</v>
+        <v>9.84</v>
       </c>
       <c r="BR34" t="n">
-        <v>14.5</v>
+        <v>16.2</v>
       </c>
       <c r="BS34" t="n">
         <v>0.32</v>
       </c>
       <c r="BT34" t="n">
-        <v>3203397</v>
+        <v>3344313</v>
       </c>
     </row>
     <row r="35">
@@ -8395,13 +8395,13 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>17.96</v>
+        <v>17.66</v>
       </c>
       <c r="G35" t="n">
-        <v>90635135379</v>
+        <v>89121189229</v>
       </c>
       <c r="H35" t="n">
-        <v>0</v>
+        <v>46623800</v>
       </c>
       <c r="I35" t="n">
         <v>5046500000</v>
@@ -8416,7 +8416,7 @@
         <v>4.69</v>
       </c>
       <c r="M35" t="n">
-        <v>7.524561880513843</v>
+        <v>7.398873520896959</v>
       </c>
       <c r="N35" t="n">
         <v>1.79</v>
@@ -8494,7 +8494,7 @@
         <v>5349290000</v>
       </c>
       <c r="AM35" t="n">
-        <v>7490507056.115703</v>
+        <v>7365387539.586777</v>
       </c>
       <c r="AN35" t="n">
         <v>0.5305</v>
@@ -8535,7 +8535,7 @@
         <v>7.68</v>
       </c>
       <c r="AZ35" t="n">
-        <v>10.48</v>
+        <v>10.3</v>
       </c>
       <c r="BA35" t="n">
         <v>1.11</v>
@@ -8544,19 +8544,19 @@
         <v>9.119999999999999</v>
       </c>
       <c r="BC35" t="n">
-        <v>-47.62</v>
+        <v>-46.74</v>
       </c>
       <c r="BD35" t="n">
-        <v>-57.24</v>
+        <v>-56.51</v>
       </c>
       <c r="BE35" t="n">
         <v>-41.67</v>
       </c>
       <c r="BF35" t="n">
-        <v>-93.8</v>
+        <v>-93.69</v>
       </c>
       <c r="BG35" t="n">
-        <v>-49.24</v>
+        <v>-48.38</v>
       </c>
       <c r="BH35" t="n">
         <v>3.71</v>
@@ -8565,7 +8565,7 @@
         <v>0</v>
       </c>
       <c r="BJ35" t="n">
-        <v>17.96</v>
+        <v>17.66</v>
       </c>
       <c r="BK35" t="n">
         <v>1.06</v>
@@ -8574,7 +8574,7 @@
         <v>1.04</v>
       </c>
       <c r="BM35" t="n">
-        <v>18.03</v>
+        <v>17.98</v>
       </c>
       <c r="BN35" t="n">
         <v>19.88</v>
@@ -8586,16 +8586,16 @@
         <v>17.62</v>
       </c>
       <c r="BQ35" t="n">
-        <v>17.19</v>
+        <v>16.9</v>
       </c>
       <c r="BR35" t="n">
-        <v>17.76</v>
+        <v>17.73</v>
       </c>
       <c r="BS35" t="n">
         <v>7.3</v>
       </c>
       <c r="BT35" t="n">
-        <v>40957743</v>
+        <v>39479047</v>
       </c>
     </row>
     <row r="36">
@@ -8625,10 +8625,10 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>25.9</v>
+        <v>26</v>
       </c>
       <c r="G36" t="n">
-        <v>198305054</v>
+        <v>195746593</v>
       </c>
       <c r="H36" t="n">
         <v>100</v>
@@ -8646,7 +8646,7 @@
         <v>1.52</v>
       </c>
       <c r="M36" t="n">
-        <v>1.93066675066702</v>
+        <v>1.905757977612863</v>
       </c>
       <c r="N36" t="n">
         <v>0.87</v>
@@ -8724,7 +8724,7 @@
         <v>11319000</v>
       </c>
       <c r="AM36" t="n">
-        <v>27314745.73002755</v>
+        <v>26962340.63360882</v>
       </c>
       <c r="AN36" t="n">
         <v>0</v>
@@ -8765,7 +8765,7 @@
         <v>24.36</v>
       </c>
       <c r="AZ36" t="n">
-        <v>66.39</v>
+        <v>66.65000000000001</v>
       </c>
       <c r="BA36" t="n">
         <v>2.44</v>
@@ -8774,25 +8774,25 @@
         <v>14.49</v>
       </c>
       <c r="BC36" t="n">
-        <v>15.21</v>
+        <v>14.76</v>
       </c>
       <c r="BD36" t="n">
-        <v>-5.93</v>
+        <v>-6.3</v>
       </c>
       <c r="BE36" t="n">
         <v>156.33</v>
       </c>
       <c r="BF36" t="n">
-        <v>-90.56</v>
+        <v>-90.59999999999999</v>
       </c>
       <c r="BG36" t="n">
-        <v>-44.06</v>
+        <v>-44.28</v>
       </c>
       <c r="BH36" t="n">
         <v>17.13</v>
       </c>
       <c r="BI36" t="n">
-        <v>-0.38</v>
+        <v>0</v>
       </c>
       <c r="BJ36" t="n">
         <v>26</v>
@@ -8804,7 +8804,7 @@
         <v>2.31</v>
       </c>
       <c r="BM36" t="n">
-        <v>25.9</v>
+        <v>26</v>
       </c>
       <c r="BN36" t="n">
         <v>29.05</v>
@@ -8813,19 +8813,19 @@
         <v>17.14</v>
       </c>
       <c r="BP36" t="n">
-        <v>25.9</v>
+        <v>26</v>
       </c>
       <c r="BQ36" t="n">
-        <v>11.2</v>
+        <v>11.25</v>
       </c>
       <c r="BR36" t="n">
-        <v>25.9</v>
+        <v>26</v>
       </c>
       <c r="BS36" t="n">
         <v>1.24</v>
       </c>
       <c r="BT36" t="n">
-        <v>150</v>
+        <v>143</v>
       </c>
     </row>
     <row r="37">
@@ -8855,13 +8855,13 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>14.95</v>
+        <v>14.62</v>
       </c>
       <c r="G37" t="n">
-        <v>200165000</v>
+        <v>195746593</v>
       </c>
       <c r="H37" t="n">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="I37" t="n">
         <v>4900000</v>
@@ -8876,7 +8876,7 @@
         <v>0.88</v>
       </c>
       <c r="M37" t="n">
-        <v>1.948774891774891</v>
+        <v>1.905757977612863</v>
       </c>
       <c r="N37" t="n">
         <v>0.5</v>
@@ -8954,7 +8954,7 @@
         <v>11319000</v>
       </c>
       <c r="AM37" t="n">
-        <v>47886363.63636364</v>
+        <v>46829328.46889953</v>
       </c>
       <c r="AN37" t="n">
         <v>0</v>
@@ -8995,7 +8995,7 @@
         <v>24.36</v>
       </c>
       <c r="AZ37" t="n">
-        <v>66.48</v>
+        <v>65.01000000000001</v>
       </c>
       <c r="BA37" t="n">
         <v>2.44</v>
@@ -9004,19 +9004,19 @@
         <v>15.53</v>
       </c>
       <c r="BC37" t="n">
-        <v>99.59</v>
+        <v>104.09</v>
       </c>
       <c r="BD37" t="n">
-        <v>62.96</v>
+        <v>66.64</v>
       </c>
       <c r="BE37" t="n">
         <v>344.67</v>
       </c>
       <c r="BF37" t="n">
-        <v>-83.65000000000001</v>
+        <v>-83.28</v>
       </c>
       <c r="BG37" t="n">
-        <v>3.9</v>
+        <v>6.25</v>
       </c>
       <c r="BH37" t="n">
         <v>17.13</v>
@@ -9025,7 +9025,7 @@
         <v>0</v>
       </c>
       <c r="BJ37" t="n">
-        <v>14.95</v>
+        <v>14.62</v>
       </c>
       <c r="BK37" t="n">
         <v>2.31</v>
@@ -9034,7 +9034,7 @@
         <v>2.31</v>
       </c>
       <c r="BM37" t="n">
-        <v>14.95</v>
+        <v>14.62</v>
       </c>
       <c r="BN37" t="n">
         <v>20.9</v>
@@ -9043,19 +9043,19 @@
         <v>13.2</v>
       </c>
       <c r="BP37" t="n">
-        <v>14.75</v>
+        <v>14.56</v>
       </c>
       <c r="BQ37" t="n">
-        <v>6.47</v>
+        <v>6.32</v>
       </c>
       <c r="BR37" t="n">
-        <v>14.75</v>
+        <v>14.56</v>
       </c>
       <c r="BS37" t="n">
         <v>0.72</v>
       </c>
       <c r="BT37" t="n">
-        <v>853</v>
+        <v>860</v>
       </c>
     </row>
     <row r="38">
@@ -9315,13 +9315,13 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>68.8</v>
+        <v>68.95</v>
       </c>
       <c r="G39" t="n">
-        <v>3856811211</v>
+        <v>3865220303</v>
       </c>
       <c r="H39" t="n">
-        <v>900</v>
+        <v>2400</v>
       </c>
       <c r="I39" t="n">
         <v>168174945</v>
@@ -9336,7 +9336,7 @@
         <v>0.53</v>
       </c>
       <c r="M39" t="n">
-        <v>0.1935950054111081</v>
+        <v>0.1940171049441625</v>
       </c>
       <c r="N39" t="n">
         <v>0.06</v>
@@ -9414,7 +9414,7 @@
         <v>2536078170.6</v>
       </c>
       <c r="AM39" t="n">
-        <v>405127228.0462185</v>
+        <v>406010536.0294118</v>
       </c>
       <c r="AN39" t="n">
         <v>11.9435</v>
@@ -9455,7 +9455,7 @@
         <v>170.24</v>
       </c>
       <c r="AZ39" t="n">
-        <v>201.01</v>
+        <v>201.45</v>
       </c>
       <c r="BA39" t="n">
         <v>19.01</v>
@@ -9464,19 +9464,19 @@
         <v>91.72</v>
       </c>
       <c r="BC39" t="n">
-        <v>203.06</v>
+        <v>202.4</v>
       </c>
       <c r="BD39" t="n">
-        <v>147.45</v>
+        <v>146.91</v>
       </c>
       <c r="BE39" t="n">
         <v>192.17</v>
       </c>
       <c r="BF39" t="n">
-        <v>-72.37</v>
+        <v>-72.43000000000001</v>
       </c>
       <c r="BG39" t="n">
-        <v>33.32</v>
+        <v>33.03</v>
       </c>
       <c r="BH39" t="n">
         <v>128.13</v>
@@ -9485,7 +9485,7 @@
         <v>0</v>
       </c>
       <c r="BJ39" t="n">
-        <v>68.8</v>
+        <v>68.95</v>
       </c>
       <c r="BK39" t="n">
         <v>15.08</v>
@@ -9494,7 +9494,7 @@
         <v>15.08</v>
       </c>
       <c r="BM39" t="n">
-        <v>68.89</v>
+        <v>68.95</v>
       </c>
       <c r="BN39" t="n">
         <v>74.56</v>
@@ -9503,19 +9503,19 @@
         <v>54.98</v>
       </c>
       <c r="BP39" t="n">
-        <v>68.59999999999999</v>
+        <v>68.83</v>
       </c>
       <c r="BQ39" t="n">
-        <v>4.56</v>
+        <v>4.57</v>
       </c>
       <c r="BR39" t="n">
-        <v>68.59999999999999</v>
+        <v>68.95</v>
       </c>
       <c r="BS39" t="n">
         <v>0.58</v>
       </c>
       <c r="BT39" t="n">
-        <v>3153</v>
+        <v>3140</v>
       </c>
     </row>
     <row r="40">
@@ -9545,13 +9545,13 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>21.59</v>
+        <v>21.49</v>
       </c>
       <c r="G40" t="n">
-        <v>123728728524</v>
+        <v>123155599858</v>
       </c>
       <c r="H40" t="n">
-        <v>0</v>
+        <v>44554600</v>
       </c>
       <c r="I40" t="n">
         <v>5730834040</v>
@@ -9566,7 +9566,7 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="M40" t="n">
-        <v>0.3754082744935107</v>
+        <v>0.373669331192852</v>
       </c>
       <c r="N40" t="n">
         <v>0.05</v>
@@ -9644,7 +9644,7 @@
         <v>15358635227.2</v>
       </c>
       <c r="AM40" t="n">
-        <v>6417465172.406639</v>
+        <v>6387738581.846473</v>
       </c>
       <c r="AN40" t="n">
         <v>0.5641</v>
@@ -9685,7 +9685,7 @@
         <v>36.13</v>
       </c>
       <c r="AZ40" t="n">
-        <v>10.9</v>
+        <v>10.85</v>
       </c>
       <c r="BA40" t="n">
         <v>2.76</v>
@@ -9694,19 +9694,19 @@
         <v>27.89</v>
       </c>
       <c r="BC40" t="n">
-        <v>104.95</v>
+        <v>105.9</v>
       </c>
       <c r="BD40" t="n">
-        <v>67.34</v>
+        <v>68.12</v>
       </c>
       <c r="BE40" t="n">
         <v>-49.5</v>
       </c>
       <c r="BF40" t="n">
-        <v>-87.22</v>
+        <v>-87.16</v>
       </c>
       <c r="BG40" t="n">
-        <v>29.18</v>
+        <v>29.78</v>
       </c>
       <c r="BH40" t="n">
         <v>32.47</v>
@@ -9715,7 +9715,7 @@
         <v>0</v>
       </c>
       <c r="BJ40" t="n">
-        <v>21.59</v>
+        <v>21.49</v>
       </c>
       <c r="BK40" t="n">
         <v>2.68</v>
@@ -9724,7 +9724,7 @@
         <v>2.5</v>
       </c>
       <c r="BM40" t="n">
-        <v>21.77</v>
+        <v>21.81</v>
       </c>
       <c r="BN40" t="n">
         <v>27.36</v>
@@ -9733,19 +9733,19 @@
         <v>17.67</v>
       </c>
       <c r="BP40" t="n">
-        <v>21.27</v>
+        <v>21.18</v>
       </c>
       <c r="BQ40" t="n">
-        <v>8.640000000000001</v>
+        <v>8.6</v>
       </c>
       <c r="BR40" t="n">
-        <v>21.54</v>
+        <v>21.39</v>
       </c>
       <c r="BS40" t="n">
         <v>0.39</v>
       </c>
       <c r="BT40" t="n">
-        <v>37609030</v>
+        <v>37020600</v>
       </c>
     </row>
     <row r="41">
@@ -9775,13 +9775,13 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>15.77</v>
+        <v>15.61</v>
       </c>
       <c r="G41" t="n">
-        <v>188077565572</v>
+        <v>186051806992</v>
       </c>
       <c r="H41" t="n">
-        <v>4253600</v>
+        <v>6952700</v>
       </c>
       <c r="I41" t="n">
         <v>5303870781</v>
@@ -9796,7 +9796,7 @@
         <v>0.92</v>
       </c>
       <c r="M41" t="n">
-        <v>1.253342964498565</v>
+        <v>1.23984337321933</v>
       </c>
       <c r="N41" t="n">
         <v>0.07000000000000001</v>
@@ -9874,7 +9874,7 @@
         <v>12304980211.92</v>
       </c>
       <c r="AM41" t="n">
-        <v>28979594078.8906</v>
+        <v>28667458704.46841</v>
       </c>
       <c r="AN41" t="n">
         <v>1.6841</v>
@@ -9915,7 +9915,7 @@
         <v>24.4</v>
       </c>
       <c r="AZ41" t="n">
-        <v>23.6</v>
+        <v>23.36</v>
       </c>
       <c r="BA41" t="n">
         <v>2.53</v>
@@ -9924,19 +9924,19 @@
         <v>13.77</v>
       </c>
       <c r="BC41" t="n">
-        <v>89.51000000000001</v>
+        <v>91.45</v>
       </c>
       <c r="BD41" t="n">
-        <v>54.73</v>
+        <v>56.32</v>
       </c>
       <c r="BE41" t="n">
         <v>49.67</v>
       </c>
       <c r="BF41" t="n">
-        <v>-83.97</v>
+        <v>-83.81</v>
       </c>
       <c r="BG41" t="n">
-        <v>-12.68</v>
+        <v>-11.79</v>
       </c>
       <c r="BH41" t="n">
         <v>17.11</v>
@@ -9945,7 +9945,7 @@
         <v>0</v>
       </c>
       <c r="BJ41" t="n">
-        <v>15.77</v>
+        <v>15.61</v>
       </c>
       <c r="BK41" t="n">
         <v>2.32</v>
@@ -9954,7 +9954,7 @@
         <v>2.34</v>
       </c>
       <c r="BM41" t="n">
-        <v>15.82</v>
+        <v>15.78</v>
       </c>
       <c r="BN41" t="n">
         <v>18.28</v>
@@ -9963,19 +9963,19 @@
         <v>13.43</v>
       </c>
       <c r="BP41" t="n">
-        <v>15.58</v>
+        <v>15.46</v>
       </c>
       <c r="BQ41" t="n">
-        <v>6.75</v>
+        <v>6.68</v>
       </c>
       <c r="BR41" t="n">
-        <v>15.62</v>
+        <v>15.64</v>
       </c>
       <c r="BS41" t="n">
         <v>0.5600000000000001</v>
       </c>
       <c r="BT41" t="n">
-        <v>7279813</v>
+        <v>7215510</v>
       </c>
     </row>
     <row r="42">
@@ -10005,13 +10005,13 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>17.88</v>
+        <v>17.66</v>
       </c>
       <c r="G42" t="n">
-        <v>188077565572</v>
+        <v>186051806992</v>
       </c>
       <c r="H42" t="n">
-        <v>21337600</v>
+        <v>28163100</v>
       </c>
       <c r="I42" t="n">
         <v>5288141247</v>
@@ -10026,7 +10026,7 @@
         <v>1.05</v>
       </c>
       <c r="M42" t="n">
-        <v>1.25707102315905</v>
+        <v>1.243531277453127</v>
       </c>
       <c r="N42" t="n">
         <v>0.08</v>
@@ -10104,7 +10104,7 @@
         <v>12268487693.04</v>
       </c>
       <c r="AM42" t="n">
-        <v>25588784431.56463</v>
+        <v>25313171019.31973</v>
       </c>
       <c r="AN42" t="n">
         <v>1.8491</v>
@@ -10145,7 +10145,7 @@
         <v>24.4</v>
       </c>
       <c r="AZ42" t="n">
-        <v>25.9</v>
+        <v>25.58</v>
       </c>
       <c r="BA42" t="n">
         <v>2.53</v>
@@ -10154,19 +10154,19 @@
         <v>15.11</v>
       </c>
       <c r="BC42" t="n">
-        <v>67.14</v>
+        <v>69.23</v>
       </c>
       <c r="BD42" t="n">
-        <v>36.47</v>
+        <v>38.17</v>
       </c>
       <c r="BE42" t="n">
         <v>44.83</v>
       </c>
       <c r="BF42" t="n">
-        <v>-85.87</v>
+        <v>-85.69</v>
       </c>
       <c r="BG42" t="n">
-        <v>-15.47</v>
+        <v>-14.41</v>
       </c>
       <c r="BH42" t="n">
         <v>17.11</v>
@@ -10175,7 +10175,7 @@
         <v>0</v>
       </c>
       <c r="BJ42" t="n">
-        <v>17.88</v>
+        <v>17.66</v>
       </c>
       <c r="BK42" t="n">
         <v>2.32</v>
@@ -10184,7 +10184,7 @@
         <v>2.34</v>
       </c>
       <c r="BM42" t="n">
-        <v>17.95</v>
+        <v>17.88</v>
       </c>
       <c r="BN42" t="n">
         <v>21.33</v>
@@ -10193,19 +10193,19 @@
         <v>15.67</v>
       </c>
       <c r="BP42" t="n">
-        <v>17.65</v>
+        <v>17.54</v>
       </c>
       <c r="BQ42" t="n">
-        <v>7.65</v>
+        <v>7.56</v>
       </c>
       <c r="BR42" t="n">
-        <v>17.74</v>
+        <v>17.82</v>
       </c>
       <c r="BS42" t="n">
         <v>0.63</v>
       </c>
       <c r="BT42" t="n">
-        <v>41073393</v>
+        <v>40407127</v>
       </c>
     </row>
     <row r="43">
@@ -10235,13 +10235,13 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>38.99</v>
+        <v>38.38</v>
       </c>
       <c r="G43" t="n">
-        <v>75695189258</v>
+        <v>74510934073</v>
       </c>
       <c r="H43" t="n">
-        <v>4015300</v>
+        <v>6348300</v>
       </c>
       <c r="I43" t="n">
         <v>1941400000</v>
@@ -10334,7 +10334,7 @@
         <v>9182822000</v>
       </c>
       <c r="AM43" t="n">
-        <v>9219876888.915955</v>
+        <v>9075631433.982946</v>
       </c>
       <c r="AN43" t="n">
         <v>4.5901</v>
@@ -10375,7 +10375,7 @@
         <v>19.95</v>
       </c>
       <c r="AZ43" t="n">
-        <v>70.77</v>
+        <v>69.66</v>
       </c>
       <c r="BA43" t="n">
         <v>5.63</v>
@@ -10384,19 +10384,19 @@
         <v>48.62</v>
       </c>
       <c r="BC43" t="n">
-        <v>-37.33</v>
+        <v>-36.34</v>
       </c>
       <c r="BD43" t="n">
-        <v>-48.83</v>
+        <v>-48.02</v>
       </c>
       <c r="BE43" t="n">
         <v>81.5</v>
       </c>
       <c r="BF43" t="n">
-        <v>-85.56</v>
+        <v>-85.33</v>
       </c>
       <c r="BG43" t="n">
-        <v>24.69</v>
+        <v>26.67</v>
       </c>
       <c r="BH43" t="n">
         <v>5.61</v>
@@ -10405,7 +10405,7 @@
         <v>0</v>
       </c>
       <c r="BJ43" t="n">
-        <v>38.99</v>
+        <v>38.38</v>
       </c>
       <c r="BK43" t="n">
         <v>4.73</v>
@@ -10414,7 +10414,7 @@
         <v>4.73</v>
       </c>
       <c r="BM43" t="n">
-        <v>39.07</v>
+        <v>38.96</v>
       </c>
       <c r="BN43" t="n">
         <v>42.98</v>
@@ -10423,19 +10423,19 @@
         <v>28.06</v>
       </c>
       <c r="BP43" t="n">
-        <v>38.58</v>
+        <v>38.36</v>
       </c>
       <c r="BQ43" t="n">
-        <v>8.24</v>
+        <v>8.109999999999999</v>
       </c>
       <c r="BR43" t="n">
-        <v>38.74</v>
+        <v>38.81</v>
       </c>
       <c r="BS43" t="n">
         <v>0</v>
       </c>
       <c r="BT43" t="n">
-        <v>6572333</v>
+        <v>6287600</v>
       </c>
     </row>
     <row r="44">
@@ -10925,13 +10925,13 @@
         </is>
       </c>
       <c r="F46" t="n">
-        <v>4.09</v>
+        <v>4.01</v>
       </c>
       <c r="G46" t="n">
-        <v>4092216932</v>
+        <v>4012173649</v>
       </c>
       <c r="H46" t="n">
-        <v>0</v>
+        <v>22181100</v>
       </c>
       <c r="I46" t="n">
         <v>1000542188</v>
@@ -10946,7 +10946,7 @@
         <v>2.5</v>
       </c>
       <c r="M46" t="n">
-        <v>0.07113042405937922</v>
+        <v>0.06973912131138138</v>
       </c>
       <c r="N46" t="n">
         <v>0.08</v>
@@ -11024,7 +11024,7 @@
         <v>460249406.48</v>
       </c>
       <c r="AM46" t="n">
-        <v>4011977384.313725</v>
+        <v>3933503577.45098</v>
       </c>
       <c r="AN46" t="n">
         <v>0.0311</v>
@@ -11065,7 +11065,7 @@
         <v>3.3</v>
       </c>
       <c r="AZ46" t="n">
-        <v>3.37</v>
+        <v>3.31</v>
       </c>
       <c r="BA46" t="n">
         <v>0.42</v>
@@ -11074,19 +11074,19 @@
         <v>7.38</v>
       </c>
       <c r="BC46" t="n">
-        <v>-1.13</v>
+        <v>0.84</v>
       </c>
       <c r="BD46" t="n">
-        <v>-19.27</v>
+        <v>-17.66</v>
       </c>
       <c r="BE46" t="n">
         <v>-17.5</v>
       </c>
       <c r="BF46" t="n">
-        <v>-89.66</v>
+        <v>-89.45</v>
       </c>
       <c r="BG46" t="n">
-        <v>80.41</v>
+        <v>84.01000000000001</v>
       </c>
       <c r="BH46" t="n">
         <v>1.58</v>
@@ -11095,7 +11095,7 @@
         <v>0</v>
       </c>
       <c r="BJ46" t="n">
-        <v>4.09</v>
+        <v>4.01</v>
       </c>
       <c r="BK46" t="n">
         <v>0.46</v>
@@ -11104,7 +11104,7 @@
         <v>0.46</v>
       </c>
       <c r="BM46" t="n">
-        <v>4.22</v>
+        <v>4.17</v>
       </c>
       <c r="BN46" t="n">
         <v>7.31</v>
@@ -11116,16 +11116,16 @@
         <v>3.99</v>
       </c>
       <c r="BQ46" t="n">
-        <v>8.94</v>
+        <v>8.77</v>
       </c>
       <c r="BR46" t="n">
-        <v>4.06</v>
+        <v>4.07</v>
       </c>
       <c r="BS46" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="BT46" t="n">
-        <v>22964607</v>
+        <v>22561601</v>
       </c>
     </row>
     <row r="47">
@@ -11158,10 +11158,10 @@
         <v>8.960000000000001</v>
       </c>
       <c r="G47" t="n">
-        <v>3126713000</v>
+        <v>3126712973</v>
       </c>
       <c r="H47" t="n">
-        <v>6700</v>
+        <v>7600</v>
       </c>
       <c r="I47" t="n">
         <v>254106600</v>
@@ -11176,7 +11176,7 @@
         <v>1.22</v>
       </c>
       <c r="M47" t="n">
-        <v>0.7373148990462438</v>
+        <v>0.7373148926793331</v>
       </c>
       <c r="N47" t="n">
         <v>0.07000000000000001</v>
@@ -11254,7 +11254,7 @@
         <v>322715382</v>
       </c>
       <c r="AM47" t="n">
-        <v>554381737.5886525</v>
+        <v>554381732.8014184</v>
       </c>
       <c r="AN47" t="n">
         <v>0.4132</v>
@@ -11334,7 +11334,7 @@
         <v>1.29</v>
       </c>
       <c r="BM47" t="n">
-        <v>9.039999999999999</v>
+        <v>9.050000000000001</v>
       </c>
       <c r="BN47" t="n">
         <v>9.24</v>
@@ -11343,19 +11343,19 @@
         <v>7.19</v>
       </c>
       <c r="BP47" t="n">
-        <v>8.9</v>
+        <v>8.82</v>
       </c>
       <c r="BQ47" t="n">
         <v>6.93</v>
       </c>
       <c r="BR47" t="n">
-        <v>9</v>
+        <v>9.029999999999999</v>
       </c>
       <c r="BS47" t="n">
         <v>0.53</v>
       </c>
       <c r="BT47" t="n">
-        <v>10820</v>
+        <v>10443</v>
       </c>
     </row>
     <row r="48">
@@ -11388,10 +11388,10 @@
         <v>9.1</v>
       </c>
       <c r="G48" t="n">
-        <v>3126713000</v>
+        <v>3126712973</v>
       </c>
       <c r="H48" t="n">
-        <v>1300</v>
+        <v>1700</v>
       </c>
       <c r="I48" t="n">
         <v>93397546</v>
@@ -11406,7 +11406,7 @@
         <v>1.24</v>
       </c>
       <c r="M48" t="n">
-        <v>2.006011829539764</v>
+        <v>2.006011812217317</v>
       </c>
       <c r="N48" t="n">
         <v>0.07000000000000001</v>
@@ -11484,7 +11484,7 @@
         <v>118614883.42</v>
       </c>
       <c r="AM48" t="n">
-        <v>546628146.8531469</v>
+        <v>546628142.1328671</v>
       </c>
       <c r="AN48" t="n">
         <v>0.4132</v>
@@ -11573,19 +11573,19 @@
         <v>7.2</v>
       </c>
       <c r="BP48" t="n">
-        <v>9.08</v>
+        <v>9.1</v>
       </c>
       <c r="BQ48" t="n">
         <v>7.04</v>
       </c>
       <c r="BR48" t="n">
-        <v>9.199999999999999</v>
+        <v>9.109999999999999</v>
       </c>
       <c r="BS48" t="n">
         <v>0.54</v>
       </c>
       <c r="BT48" t="n">
-        <v>2680</v>
+        <v>2643</v>
       </c>
     </row>
     <row r="49">
@@ -11615,13 +11615,13 @@
         </is>
       </c>
       <c r="F49" t="n">
-        <v>48.85</v>
+        <v>48.76</v>
       </c>
       <c r="G49" t="n">
-        <v>953506700</v>
+        <v>951749820</v>
       </c>
       <c r="H49" t="n">
-        <v>1000</v>
+        <v>100</v>
       </c>
       <c r="I49" t="n">
         <v>11540870</v>
@@ -11636,7 +11636,7 @@
         <v>1.09</v>
       </c>
       <c r="M49" t="n">
-        <v>0.9646504295601004</v>
+        <v>0.9628730167252608</v>
       </c>
       <c r="N49" t="n">
         <v>0.08</v>
@@ -11714,7 +11714,7 @@
         <v>84709985.8</v>
       </c>
       <c r="AM49" t="n">
-        <v>238376675</v>
+        <v>237937455</v>
       </c>
       <c r="AN49" t="n">
         <v>3.3186</v>
@@ -11755,7 +11755,7 @@
         <v>68.48999999999999</v>
       </c>
       <c r="AZ49" t="n">
-        <v>58.29</v>
+        <v>58.19</v>
       </c>
       <c r="BA49" t="n">
         <v>9.210000000000001</v>
@@ -11764,19 +11764,19 @@
         <v>27.75</v>
       </c>
       <c r="BC49" t="n">
-        <v>71.7</v>
+        <v>72.02</v>
       </c>
       <c r="BD49" t="n">
-        <v>40.2</v>
+        <v>40.45</v>
       </c>
       <c r="BE49" t="n">
         <v>19.33</v>
       </c>
       <c r="BF49" t="n">
-        <v>-81.14</v>
+        <v>-81.09999999999999</v>
       </c>
       <c r="BG49" t="n">
-        <v>-43.18</v>
+        <v>-43.08</v>
       </c>
       <c r="BH49" t="n">
         <v>42.6</v>
@@ -11785,7 +11785,7 @@
         <v>0</v>
       </c>
       <c r="BJ49" t="n">
-        <v>48.85</v>
+        <v>48.76</v>
       </c>
       <c r="BK49" t="n">
         <v>7.34</v>
@@ -11794,7 +11794,7 @@
         <v>7.6</v>
       </c>
       <c r="BM49" t="n">
-        <v>54</v>
+        <v>48.76</v>
       </c>
       <c r="BN49" t="n">
         <v>64.2</v>
@@ -11803,19 +11803,19 @@
         <v>28.48</v>
       </c>
       <c r="BP49" t="n">
-        <v>48.85</v>
+        <v>48.76</v>
       </c>
       <c r="BQ49" t="n">
-        <v>6.43</v>
+        <v>6.42</v>
       </c>
       <c r="BR49" t="n">
-        <v>54</v>
+        <v>48.76</v>
       </c>
       <c r="BS49" t="n">
         <v>0.54</v>
       </c>
       <c r="BT49" t="n">
-        <v>333</v>
+        <v>367</v>
       </c>
     </row>
     <row r="50">
@@ -11851,7 +11851,7 @@
         <v>953506700</v>
       </c>
       <c r="H50" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="I50" t="n">
         <v>11540870</v>
@@ -12523,13 +12523,13 @@
         </is>
       </c>
       <c r="F53" t="n">
-        <v>6.13</v>
+        <v>5.98</v>
       </c>
       <c r="G53" t="n">
-        <v>838905227</v>
+        <v>818377354</v>
       </c>
       <c r="H53" t="n">
-        <v>21500</v>
+        <v>127700</v>
       </c>
       <c r="I53" t="n">
         <v>136852484</v>
@@ -12544,7 +12544,7 @@
         <v>2.79</v>
       </c>
       <c r="M53" t="n">
-        <v>2.179319390956208</v>
+        <v>2.125991803710185</v>
       </c>
       <c r="N53" t="n">
         <v>1.48</v>
@@ -12622,7 +12622,7 @@
         <v>39687220.36</v>
       </c>
       <c r="AM53" t="n">
-        <v>42735875.03820683</v>
+        <v>41690135.20122262</v>
       </c>
       <c r="AN53" t="n">
         <v>0</v>
@@ -12672,16 +12672,16 @@
         <v>0</v>
       </c>
       <c r="BC53" t="n">
-        <v>-35.71</v>
+        <v>-34.1</v>
       </c>
       <c r="BD53" t="n">
-        <v>-47.51</v>
+        <v>-46.19</v>
       </c>
       <c r="BE53" t="n">
         <v>-100</v>
       </c>
       <c r="BF53" t="n">
-        <v>-95.27</v>
+        <v>-95.15000000000001</v>
       </c>
       <c r="BG53" t="n">
         <v>-100</v>
@@ -12690,10 +12690,10 @@
         <v>2.38</v>
       </c>
       <c r="BI53" t="n">
-        <v>16.96</v>
+        <v>0</v>
       </c>
       <c r="BJ53" t="n">
-        <v>5.24</v>
+        <v>5.98</v>
       </c>
       <c r="BK53" t="n">
         <v>0.29</v>
@@ -12702,7 +12702,7 @@
         <v>0.2</v>
       </c>
       <c r="BM53" t="n">
-        <v>6.2</v>
+        <v>6.29</v>
       </c>
       <c r="BN53" t="n">
         <v>10.39</v>
@@ -12711,19 +12711,19 @@
         <v>4.82</v>
       </c>
       <c r="BP53" t="n">
-        <v>5.91</v>
+        <v>5.71</v>
       </c>
       <c r="BQ53" t="n">
-        <v>30.11</v>
+        <v>29.37</v>
       </c>
       <c r="BR53" t="n">
-        <v>5.91</v>
+        <v>5.94</v>
       </c>
       <c r="BS53" t="n">
         <v>2.36</v>
       </c>
       <c r="BT53" t="n">
-        <v>35257</v>
+        <v>32643</v>
       </c>
     </row>
     <row r="54">
@@ -12753,13 +12753,13 @@
         </is>
       </c>
       <c r="F54" t="n">
-        <v>10.22</v>
+        <v>10.29</v>
       </c>
       <c r="G54" t="n">
-        <v>2383427724</v>
+        <v>2399752500</v>
       </c>
       <c r="H54" t="n">
-        <v>191100</v>
+        <v>162500</v>
       </c>
       <c r="I54" t="n">
         <v>233212121</v>
@@ -12774,7 +12774,7 @@
         <v>0.97</v>
       </c>
       <c r="M54" t="n">
-        <v>1.337797914335679</v>
+        <v>1.346960873658878</v>
       </c>
       <c r="N54" t="n">
         <v>0.5600000000000001</v>
@@ -12852,7 +12852,7 @@
         <v>233212121</v>
       </c>
       <c r="AM54" t="n">
-        <v>326050304.2407661</v>
+        <v>328283515.7318742</v>
       </c>
       <c r="AN54" t="n">
         <v>0.1531</v>
@@ -12893,7 +12893,7 @@
         <v>12.25</v>
       </c>
       <c r="AZ54" t="n">
-        <v>16.27</v>
+        <v>16.38</v>
       </c>
       <c r="BA54" t="n">
         <v>0.98</v>
@@ -12902,19 +12902,19 @@
         <v>6.52</v>
       </c>
       <c r="BC54" t="n">
-        <v>46.84</v>
+        <v>45.85</v>
       </c>
       <c r="BD54" t="n">
-        <v>19.9</v>
+        <v>19.08</v>
       </c>
       <c r="BE54" t="n">
         <v>59.17</v>
       </c>
       <c r="BF54" t="n">
-        <v>-90.38</v>
+        <v>-90.44</v>
       </c>
       <c r="BG54" t="n">
-        <v>-36.24</v>
+        <v>-36.67</v>
       </c>
       <c r="BH54" t="n">
         <v>10.01</v>
@@ -12923,7 +12923,7 @@
         <v>0</v>
       </c>
       <c r="BJ54" t="n">
-        <v>10.22</v>
+        <v>10.29</v>
       </c>
       <c r="BK54" t="n">
         <v>1</v>
@@ -12932,7 +12932,7 @@
         <v>1</v>
       </c>
       <c r="BM54" t="n">
-        <v>10.46</v>
+        <v>10.35</v>
       </c>
       <c r="BN54" t="n">
         <v>11.75</v>
@@ -12941,19 +12941,19 @@
         <v>8.279999999999999</v>
       </c>
       <c r="BP54" t="n">
-        <v>10.08</v>
+        <v>10.12</v>
       </c>
       <c r="BQ54" t="n">
-        <v>10.19</v>
+        <v>10.26</v>
       </c>
       <c r="BR54" t="n">
-        <v>10.35</v>
+        <v>10.22</v>
       </c>
       <c r="BS54" t="n">
         <v>1.26</v>
       </c>
       <c r="BT54" t="n">
-        <v>249027</v>
+        <v>246663</v>
       </c>
     </row>
     <row r="55">
@@ -12983,13 +12983,13 @@
         </is>
       </c>
       <c r="F55" t="n">
-        <v>50.1</v>
+        <v>49.4</v>
       </c>
       <c r="G55" t="n">
-        <v>5145951203</v>
+        <v>6564644884</v>
       </c>
       <c r="H55" t="n">
-        <v>2600</v>
+        <v>5000</v>
       </c>
       <c r="I55" t="n">
         <v>84052790</v>
@@ -13004,7 +13004,7 @@
         <v>2</v>
       </c>
       <c r="M55" t="n">
-        <v>0.7943864483492438</v>
+        <v>1.013391835319895</v>
       </c>
       <c r="N55" t="n">
         <v>0.16</v>
@@ -13082,7 +13082,7 @@
         <v>579123723.1</v>
       </c>
       <c r="AM55" t="n">
-        <v>258850664.1348089</v>
+        <v>330213525.3521127</v>
       </c>
       <c r="AN55" t="n">
         <v>3.1953</v>
@@ -13123,7 +13123,7 @@
         <v>51.21</v>
       </c>
       <c r="AZ55" t="n">
-        <v>52.69</v>
+        <v>51.95</v>
       </c>
       <c r="BA55" t="n">
         <v>9.380000000000001</v>
@@ -13132,19 +13132,19 @@
         <v>16.08</v>
       </c>
       <c r="BC55" t="n">
-        <v>25.18</v>
+        <v>26.95</v>
       </c>
       <c r="BD55" t="n">
-        <v>2.21</v>
+        <v>3.65</v>
       </c>
       <c r="BE55" t="n">
         <v>5.17</v>
       </c>
       <c r="BF55" t="n">
-        <v>-81.28</v>
+        <v>-81.02</v>
       </c>
       <c r="BG55" t="n">
-        <v>-67.91</v>
+        <v>-67.45999999999999</v>
       </c>
       <c r="BH55" t="n">
         <v>25.37</v>
@@ -13153,7 +13153,7 @@
         <v>0</v>
       </c>
       <c r="BJ55" t="n">
-        <v>50.1</v>
+        <v>49.4</v>
       </c>
       <c r="BK55" t="n">
         <v>6.89</v>
@@ -13162,7 +13162,7 @@
         <v>7.03</v>
       </c>
       <c r="BM55" t="n">
-        <v>50.2</v>
+        <v>49.97</v>
       </c>
       <c r="BN55" t="n">
         <v>73.67</v>
@@ -13171,19 +13171,19 @@
         <v>35.58</v>
       </c>
       <c r="BP55" t="n">
-        <v>49.65</v>
+        <v>49.4</v>
       </c>
       <c r="BQ55" t="n">
-        <v>7.13</v>
+        <v>7.03</v>
       </c>
       <c r="BR55" t="n">
-        <v>49.67</v>
+        <v>49.8</v>
       </c>
       <c r="BS55" t="n">
         <v>0.66</v>
       </c>
       <c r="BT55" t="n">
-        <v>6423</v>
+        <v>6393</v>
       </c>
     </row>
     <row r="56">
@@ -13213,13 +13213,13 @@
         </is>
       </c>
       <c r="F56" t="n">
-        <v>57.12</v>
+        <v>57.89</v>
       </c>
       <c r="G56" t="n">
-        <v>5145951203</v>
+        <v>6564644884</v>
       </c>
       <c r="H56" t="n">
-        <v>29700</v>
+        <v>9700</v>
       </c>
       <c r="I56" t="n">
         <v>39675836</v>
@@ -13234,7 +13234,7 @@
         <v>2.41</v>
       </c>
       <c r="M56" t="n">
-        <v>1.682898309236505</v>
+        <v>2.146858635111249</v>
       </c>
       <c r="N56" t="n">
         <v>0.19</v>
@@ -13312,7 +13312,7 @@
         <v>273366510.04</v>
       </c>
       <c r="AM56" t="n">
-        <v>214057870.3410982</v>
+        <v>273071750.5823627</v>
       </c>
       <c r="AN56" t="n">
         <v>3.5102</v>
@@ -13353,7 +13353,7 @@
         <v>51.21</v>
       </c>
       <c r="AZ56" t="n">
-        <v>54.55</v>
+        <v>55.28</v>
       </c>
       <c r="BA56" t="n">
         <v>9.380000000000001</v>
@@ -13362,19 +13362,19 @@
         <v>17.68</v>
       </c>
       <c r="BC56" t="n">
-        <v>9.789999999999999</v>
+        <v>8.33</v>
       </c>
       <c r="BD56" t="n">
-        <v>-10.35</v>
+        <v>-11.55</v>
       </c>
       <c r="BE56" t="n">
         <v>-4.5</v>
       </c>
       <c r="BF56" t="n">
-        <v>-83.58</v>
+        <v>-83.8</v>
       </c>
       <c r="BG56" t="n">
-        <v>-69.05</v>
+        <v>-69.45999999999999</v>
       </c>
       <c r="BH56" t="n">
         <v>25.37</v>
@@ -13383,7 +13383,7 @@
         <v>0</v>
       </c>
       <c r="BJ56" t="n">
-        <v>57.12</v>
+        <v>57.89</v>
       </c>
       <c r="BK56" t="n">
         <v>6.89</v>
@@ -13392,7 +13392,7 @@
         <v>7.03</v>
       </c>
       <c r="BM56" t="n">
-        <v>58.4</v>
+        <v>58.14</v>
       </c>
       <c r="BN56" t="n">
         <v>86.77</v>
@@ -13401,19 +13401,19 @@
         <v>46.42</v>
       </c>
       <c r="BP56" t="n">
-        <v>57.09</v>
+        <v>56.5</v>
       </c>
       <c r="BQ56" t="n">
-        <v>8.119999999999999</v>
+        <v>8.23</v>
       </c>
       <c r="BR56" t="n">
-        <v>58.29</v>
+        <v>57.06</v>
       </c>
       <c r="BS56" t="n">
         <v>0.79</v>
       </c>
       <c r="BT56" t="n">
-        <v>30513</v>
+        <v>30327</v>
       </c>
     </row>
     <row r="57">
@@ -13443,13 +13443,13 @@
         </is>
       </c>
       <c r="F57" t="n">
-        <v>5.96</v>
+        <v>5.97</v>
       </c>
       <c r="G57" t="n">
-        <v>1393793688</v>
+        <v>1396132210</v>
       </c>
       <c r="H57" t="n">
-        <v>916400</v>
+        <v>1294600</v>
       </c>
       <c r="I57" t="n">
         <v>233858065</v>
@@ -13464,7 +13464,7 @@
         <v>0.77</v>
       </c>
       <c r="M57" t="n">
-        <v>0.4171998864353899</v>
+        <v>0.4178998688798696</v>
       </c>
       <c r="N57" t="n">
         <v>0.08</v>
@@ -13542,7 +13542,7 @@
         <v>229180903.7</v>
       </c>
       <c r="AM57" t="n">
-        <v>104247845.026178</v>
+        <v>104422753.1787584</v>
       </c>
       <c r="AN57" t="n">
         <v>0.347</v>
@@ -13583,7 +13583,7 @@
         <v>10.72</v>
       </c>
       <c r="AZ57" t="n">
-        <v>9.09</v>
+        <v>9.1</v>
       </c>
       <c r="BA57" t="n">
         <v>1.13</v>
@@ -13592,19 +13592,19 @@
         <v>6.26</v>
       </c>
       <c r="BC57" t="n">
-        <v>120.32</v>
+        <v>119.95</v>
       </c>
       <c r="BD57" t="n">
-        <v>79.89</v>
+        <v>79.59</v>
       </c>
       <c r="BE57" t="n">
         <v>52.5</v>
       </c>
       <c r="BF57" t="n">
-        <v>-81.08</v>
+        <v>-81.11</v>
       </c>
       <c r="BG57" t="n">
-        <v>5.1</v>
+        <v>4.92</v>
       </c>
       <c r="BH57" t="n">
         <v>7.82</v>
@@ -13613,7 +13613,7 @@
         <v>0</v>
       </c>
       <c r="BJ57" t="n">
-        <v>5.96</v>
+        <v>5.97</v>
       </c>
       <c r="BK57" t="n">
         <v>0.98</v>
@@ -13622,7 +13622,7 @@
         <v>1.04</v>
       </c>
       <c r="BM57" t="n">
-        <v>6.02</v>
+        <v>6.01</v>
       </c>
       <c r="BN57" t="n">
         <v>6.22</v>
@@ -13631,19 +13631,19 @@
         <v>3.43</v>
       </c>
       <c r="BP57" t="n">
-        <v>5.89</v>
+        <v>5.84</v>
       </c>
       <c r="BQ57" t="n">
-        <v>5.75</v>
+        <v>5.76</v>
       </c>
       <c r="BR57" t="n">
-        <v>5.98</v>
+        <v>5.94</v>
       </c>
       <c r="BS57" t="n">
         <v>0.42</v>
       </c>
       <c r="BT57" t="n">
-        <v>1348570</v>
+        <v>1346403</v>
       </c>
     </row>
     <row r="58">
@@ -13909,7 +13909,7 @@
         <v>91920060</v>
       </c>
       <c r="H59" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I59" t="n">
         <v>710143</v>
@@ -14133,13 +14133,13 @@
         </is>
       </c>
       <c r="F60" t="n">
-        <v>369.94</v>
+        <v>383.95</v>
       </c>
       <c r="G60" t="n">
-        <v>168230216</v>
+        <v>174601229</v>
       </c>
       <c r="H60" t="n">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="I60" t="n">
         <v>454750</v>
@@ -14154,7 +14154,7 @@
         <v>0.83</v>
       </c>
       <c r="M60" t="n">
-        <v>12.58338333814134</v>
+        <v>13.05992614202909</v>
       </c>
       <c r="N60" t="n">
         <v>0.68</v>
@@ -14232,7 +14232,7 @@
         <v>59558607.5</v>
       </c>
       <c r="AM60" t="n">
-        <v>-24667187.09677419</v>
+        <v>-25601353.22580645</v>
       </c>
       <c r="AN60" t="n">
         <v>10.0581</v>
@@ -14273,7 +14273,7 @@
         <v>944.87</v>
       </c>
       <c r="AZ60" t="n">
-        <v>2127.16</v>
+        <v>2207.71</v>
       </c>
       <c r="BA60" t="n">
         <v>231.1</v>
@@ -14282,19 +14282,19 @@
         <v>727.97</v>
       </c>
       <c r="BC60" t="n">
-        <v>212.81</v>
+        <v>201.4</v>
       </c>
       <c r="BD60" t="n">
-        <v>155.41</v>
+        <v>146.09</v>
       </c>
       <c r="BE60" t="n">
         <v>475</v>
       </c>
       <c r="BF60" t="n">
-        <v>-37.53</v>
+        <v>-39.81</v>
       </c>
       <c r="BG60" t="n">
-        <v>96.78</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="BH60" t="n">
         <v>454.44</v>
@@ -14303,7 +14303,7 @@
         <v>0</v>
       </c>
       <c r="BJ60" t="n">
-        <v>369.94</v>
+        <v>383.95</v>
       </c>
       <c r="BK60" t="n">
         <v>130.97</v>
@@ -14312,7 +14312,7 @@
         <v>130.97</v>
       </c>
       <c r="BM60" t="n">
-        <v>388</v>
+        <v>383.95</v>
       </c>
       <c r="BN60" t="n">
         <v>405</v>
@@ -14321,19 +14321,19 @@
         <v>309.24</v>
       </c>
       <c r="BP60" t="n">
-        <v>369.92</v>
+        <v>373</v>
       </c>
       <c r="BQ60" t="n">
-        <v>2.82</v>
+        <v>2.93</v>
       </c>
       <c r="BR60" t="n">
-        <v>386.99</v>
+        <v>374.12</v>
       </c>
       <c r="BS60" t="n">
         <v>12.82</v>
       </c>
       <c r="BT60" t="n">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="61">
@@ -14363,13 +14363,13 @@
         </is>
       </c>
       <c r="F61" t="n">
-        <v>27.5</v>
+        <v>27.31</v>
       </c>
       <c r="G61" t="n">
-        <v>2354230175</v>
+        <v>2337965358</v>
       </c>
       <c r="H61" t="n">
-        <v>436200</v>
+        <v>1413700</v>
       </c>
       <c r="I61" t="n">
         <v>85608392</v>
@@ -14384,7 +14384,7 @@
         <v>2.37</v>
       </c>
       <c r="M61" t="n">
-        <v>1.248529090912434</v>
+        <v>1.239903300028215</v>
       </c>
       <c r="N61" t="n">
         <v>1.1</v>
@@ -14462,7 +14462,7 @@
         <v>160087693.04</v>
       </c>
       <c r="AM61" t="n">
-        <v>184790437.5981162</v>
+        <v>183513764.3642072</v>
       </c>
       <c r="AN61" t="n">
         <v>0.38</v>
@@ -14503,7 +14503,7 @@
         <v>17.56</v>
       </c>
       <c r="AZ61" t="n">
-        <v>34.65</v>
+        <v>34.41</v>
       </c>
       <c r="BA61" t="n">
         <v>2.52</v>
@@ -14512,19 +14512,19 @@
         <v>11.76</v>
       </c>
       <c r="BC61" t="n">
-        <v>-21.81</v>
+        <v>-21.26</v>
       </c>
       <c r="BD61" t="n">
-        <v>-36.15</v>
+        <v>-35.71</v>
       </c>
       <c r="BE61" t="n">
         <v>26</v>
       </c>
       <c r="BF61" t="n">
-        <v>-90.83</v>
+        <v>-90.76000000000001</v>
       </c>
       <c r="BG61" t="n">
-        <v>-57.25</v>
+        <v>-56.95</v>
       </c>
       <c r="BH61" t="n">
         <v>10.99</v>
@@ -14533,7 +14533,7 @@
         <v>0</v>
       </c>
       <c r="BJ61" t="n">
-        <v>27.5</v>
+        <v>27.31</v>
       </c>
       <c r="BK61" t="n">
         <v>1.87</v>
@@ -14542,7 +14542,7 @@
         <v>1.86</v>
       </c>
       <c r="BM61" t="n">
-        <v>27.97</v>
+        <v>27.46</v>
       </c>
       <c r="BN61" t="n">
         <v>28.68</v>
@@ -14551,19 +14551,19 @@
         <v>19.35</v>
       </c>
       <c r="BP61" t="n">
-        <v>27.28</v>
+        <v>27</v>
       </c>
       <c r="BQ61" t="n">
-        <v>14.77</v>
+        <v>14.67</v>
       </c>
       <c r="BR61" t="n">
-        <v>27.82</v>
+        <v>27.46</v>
       </c>
       <c r="BS61" t="n">
         <v>1.19</v>
       </c>
       <c r="BT61" t="n">
-        <v>573750</v>
+        <v>569237</v>
       </c>
     </row>
     <row r="62">
@@ -14593,10 +14593,10 @@
         </is>
       </c>
       <c r="F62" t="n">
-        <v>111.5</v>
+        <v>110.95</v>
       </c>
       <c r="G62" t="n">
-        <v>11005020000</v>
+        <v>10950734742</v>
       </c>
       <c r="H62" t="n">
         <v>300</v>
@@ -14614,7 +14614,7 @@
         <v>0.64</v>
       </c>
       <c r="M62" t="n">
-        <v>1.031594299446464</v>
+        <v>1.026505679644157</v>
       </c>
       <c r="N62" t="n">
         <v>0.13</v>
@@ -14692,7 +14692,7 @@
         <v>2757670987.06</v>
       </c>
       <c r="AM62" t="n">
-        <v>4455473684.210526</v>
+        <v>4433495846.963562</v>
       </c>
       <c r="AN62" t="n">
         <v>6.9319</v>
@@ -14733,7 +14733,7 @@
         <v>267.2</v>
       </c>
       <c r="AZ62" t="n">
-        <v>117.82</v>
+        <v>117.24</v>
       </c>
       <c r="BA62" t="n">
         <v>34.09</v>
@@ -14742,19 +14742,19 @@
         <v>76.01000000000001</v>
       </c>
       <c r="BC62" t="n">
-        <v>193.49</v>
+        <v>194.95</v>
       </c>
       <c r="BD62" t="n">
-        <v>139.64</v>
+        <v>140.83</v>
       </c>
       <c r="BE62" t="n">
         <v>5.67</v>
       </c>
       <c r="BF62" t="n">
-        <v>-69.42</v>
+        <v>-69.27</v>
       </c>
       <c r="BG62" t="n">
-        <v>-31.83</v>
+        <v>-31.49</v>
       </c>
       <c r="BH62" t="n">
         <v>170.35</v>
@@ -14763,7 +14763,7 @@
         <v>0</v>
       </c>
       <c r="BJ62" t="n">
-        <v>111.5</v>
+        <v>110.95</v>
       </c>
       <c r="BK62" t="n">
         <v>27.94</v>
@@ -14772,7 +14772,7 @@
         <v>32.73</v>
       </c>
       <c r="BM62" t="n">
-        <v>111.5</v>
+        <v>111</v>
       </c>
       <c r="BN62" t="n">
         <v>122.2</v>
@@ -14781,19 +14781,19 @@
         <v>91.84999999999999</v>
       </c>
       <c r="BP62" t="n">
-        <v>109</v>
+        <v>110.95</v>
       </c>
       <c r="BQ62" t="n">
-        <v>3.41</v>
+        <v>3.39</v>
       </c>
       <c r="BR62" t="n">
-        <v>111.5</v>
+        <v>111</v>
       </c>
       <c r="BS62" t="n">
         <v>1.01</v>
       </c>
       <c r="BT62" t="n">
-        <v>157</v>
+        <v>167</v>
       </c>
     </row>
     <row r="63">
@@ -14823,13 +14823,13 @@
         </is>
       </c>
       <c r="F63" t="n">
-        <v>1.39</v>
+        <v>1.41</v>
       </c>
       <c r="G63" t="n">
-        <v>362108479</v>
+        <v>367318668</v>
       </c>
       <c r="H63" t="n">
-        <v>7000</v>
+        <v>62300</v>
       </c>
       <c r="I63" t="n">
         <v>122894462</v>
@@ -14844,7 +14844,7 @@
         <v>-0.22</v>
       </c>
       <c r="M63" t="n">
-        <v>0.4453747421569674</v>
+        <v>0.4517830057493372</v>
       </c>
       <c r="N63" t="n">
         <v>0.37</v>
@@ -14922,7 +14922,7 @@
         <v>31952560.12</v>
       </c>
       <c r="AM63" t="n">
-        <v>205743453.9772727</v>
+        <v>208703788.6363636</v>
       </c>
       <c r="AN63" t="n">
         <v>0</v>
@@ -14981,7 +14981,7 @@
         <v>-100</v>
       </c>
       <c r="BF63" t="n">
-        <v>-79.2</v>
+        <v>-79.48999999999999</v>
       </c>
       <c r="BG63" t="n">
         <v>-100</v>
@@ -14993,7 +14993,7 @@
         <v>0</v>
       </c>
       <c r="BJ63" t="n">
-        <v>1.39</v>
+        <v>1.41</v>
       </c>
       <c r="BK63" t="n">
         <v>0.26</v>
@@ -15002,7 +15002,7 @@
         <v>0.26</v>
       </c>
       <c r="BM63" t="n">
-        <v>1.39</v>
+        <v>1.6</v>
       </c>
       <c r="BN63" t="n">
         <v>2.12</v>
@@ -15011,10 +15011,10 @@
         <v>1.16</v>
       </c>
       <c r="BP63" t="n">
-        <v>1.35</v>
+        <v>1.36</v>
       </c>
       <c r="BQ63" t="n">
-        <v>5.32</v>
+        <v>5.4</v>
       </c>
       <c r="BR63" t="n">
         <v>1.36</v>
@@ -15023,7 +15023,7 @@
         <v>0.19</v>
       </c>
       <c r="BT63" t="n">
-        <v>25083</v>
+        <v>25317</v>
       </c>
     </row>
     <row r="64">
@@ -15053,13 +15053,13 @@
         </is>
       </c>
       <c r="F64" t="n">
-        <v>62.7</v>
+        <v>62.25</v>
       </c>
       <c r="G64" t="n">
-        <v>238621970003</v>
+        <v>234574247250</v>
       </c>
       <c r="H64" t="n">
-        <v>0</v>
+        <v>9379800</v>
       </c>
       <c r="I64" t="n">
         <v>0</v>
@@ -15146,13 +15146,13 @@
         <v>41.22</v>
       </c>
       <c r="AK64" t="n">
-        <v>68416420379.6217</v>
+        <v>67255878869.35789</v>
       </c>
       <c r="AL64" t="n">
-        <v>19074498001.83853</v>
+        <v>18750939028.77698</v>
       </c>
       <c r="AM64" t="n">
-        <v>21248617097.32858</v>
+        <v>20888178739.98219</v>
       </c>
       <c r="AN64" t="n">
         <v>1.4201</v>
@@ -15193,7 +15193,7 @@
         <v>38.98</v>
       </c>
       <c r="AZ64" t="n">
-        <v>25.08</v>
+        <v>24.9</v>
       </c>
       <c r="BA64" t="n">
         <v>6.69</v>
@@ -15202,19 +15202,19 @@
         <v>10.4</v>
       </c>
       <c r="BC64" t="n">
-        <v>-23.86</v>
+        <v>-23.31</v>
       </c>
       <c r="BD64" t="n">
-        <v>-37.83</v>
+        <v>-37.38</v>
       </c>
       <c r="BE64" t="n">
         <v>-60</v>
       </c>
       <c r="BF64" t="n">
-        <v>-89.31999999999999</v>
+        <v>-89.25</v>
       </c>
       <c r="BG64" t="n">
-        <v>-83.42</v>
+        <v>-83.3</v>
       </c>
       <c r="BH64" t="n">
         <v>21.37</v>
@@ -15223,7 +15223,7 @@
         <v>0</v>
       </c>
       <c r="BJ64" t="n">
-        <v>62.7</v>
+        <v>62.25</v>
       </c>
       <c r="BK64" t="n">
         <v>4.74</v>
@@ -15232,7 +15232,7 @@
         <v>1.57</v>
       </c>
       <c r="BM64" t="n">
-        <v>63.1</v>
+        <v>63.17</v>
       </c>
       <c r="BN64" t="n">
         <v>64.72</v>
@@ -15241,19 +15241,19 @@
         <v>44.12</v>
       </c>
       <c r="BP64" t="n">
-        <v>61.9</v>
+        <v>61.72</v>
       </c>
       <c r="BQ64" t="n">
-        <v>39.93</v>
+        <v>39.65</v>
       </c>
       <c r="BR64" t="n">
-        <v>62.6</v>
+        <v>62.1</v>
       </c>
       <c r="BS64" t="n">
         <v>3.49</v>
       </c>
       <c r="BT64" t="n">
-        <v>10886183</v>
+        <v>10566997</v>
       </c>
     </row>
     <row r="65">
@@ -15283,13 +15283,13 @@
         </is>
       </c>
       <c r="F65" t="n">
-        <v>24.1</v>
+        <v>24.32</v>
       </c>
       <c r="G65" t="n">
-        <v>238621970003</v>
+        <v>234574247250</v>
       </c>
       <c r="H65" t="n">
-        <v>3600</v>
+        <v>3100</v>
       </c>
       <c r="I65" t="n">
         <v>7298813414</v>
@@ -15304,7 +15304,7 @@
         <v>3.29</v>
       </c>
       <c r="M65" t="n">
-        <v>5.768911117159705</v>
+        <v>5.671053603081398</v>
       </c>
       <c r="N65" t="n">
         <v>0.29</v>
@@ -15382,7 +15382,7 @@
         <v>11532125194.12</v>
       </c>
       <c r="AM65" t="n">
-        <v>17874304869.13858</v>
+        <v>17571104662.92135</v>
       </c>
       <c r="AN65" t="n">
         <v>0.4734</v>
@@ -15423,7 +15423,7 @@
         <v>12.99</v>
       </c>
       <c r="AZ65" t="n">
-        <v>8.109999999999999</v>
+        <v>8.19</v>
       </c>
       <c r="BA65" t="n">
         <v>2.23</v>
@@ -15432,19 +15432,19 @@
         <v>3.47</v>
       </c>
       <c r="BC65" t="n">
-        <v>-33.98</v>
+        <v>-34.58</v>
       </c>
       <c r="BD65" t="n">
-        <v>-46.1</v>
+        <v>-46.59</v>
       </c>
       <c r="BE65" t="n">
         <v>-66.33</v>
       </c>
       <c r="BF65" t="n">
-        <v>-90.73999999999999</v>
+        <v>-90.83</v>
       </c>
       <c r="BG65" t="n">
-        <v>-85.62</v>
+        <v>-85.75</v>
       </c>
       <c r="BH65" t="n">
         <v>7.12</v>
@@ -15453,7 +15453,7 @@
         <v>0</v>
       </c>
       <c r="BJ65" t="n">
-        <v>24.1</v>
+        <v>24.32</v>
       </c>
       <c r="BK65" t="n">
         <v>1.58</v>
@@ -15462,7 +15462,7 @@
         <v>1.57</v>
       </c>
       <c r="BM65" t="n">
-        <v>24.78</v>
+        <v>24.34</v>
       </c>
       <c r="BN65" t="n">
         <v>46.43</v>
@@ -15471,19 +15471,19 @@
         <v>20.44</v>
       </c>
       <c r="BP65" t="n">
-        <v>24.1</v>
+        <v>23.9</v>
       </c>
       <c r="BQ65" t="n">
-        <v>15.35</v>
+        <v>15.49</v>
       </c>
       <c r="BR65" t="n">
-        <v>24.77</v>
+        <v>24.03</v>
       </c>
       <c r="BS65" t="n">
         <v>4.14</v>
       </c>
       <c r="BT65" t="n">
-        <v>9160</v>
+        <v>8857</v>
       </c>
     </row>
     <row r="66">
@@ -15513,13 +15513,13 @@
         </is>
       </c>
       <c r="F66" t="n">
-        <v>20.3</v>
+        <v>20.31</v>
       </c>
       <c r="G66" t="n">
-        <v>238621970003</v>
+        <v>234574247250</v>
       </c>
       <c r="H66" t="n">
-        <v>400</v>
+        <v>100</v>
       </c>
       <c r="I66" t="n">
         <v>2972355254</v>
@@ -15534,7 +15534,7 @@
         <v>2.75</v>
       </c>
       <c r="M66" t="n">
-        <v>14.16593988536034</v>
+        <v>13.92564433675314</v>
       </c>
       <c r="N66" t="n">
         <v>0.25</v>
@@ -15612,7 +15612,7 @@
         <v>4696321301.320001</v>
       </c>
       <c r="AM66" t="n">
-        <v>21401073542.86995</v>
+        <v>21038049080.71749</v>
       </c>
       <c r="AN66" t="n">
         <v>0.4734</v>
@@ -15653,7 +15653,7 @@
         <v>12.99</v>
       </c>
       <c r="AZ66" t="n">
-        <v>8.15</v>
+        <v>8.16</v>
       </c>
       <c r="BA66" t="n">
         <v>2.23</v>
@@ -15662,10 +15662,10 @@
         <v>3.47</v>
       </c>
       <c r="BC66" t="n">
-        <v>-21.63</v>
+        <v>-21.67</v>
       </c>
       <c r="BD66" t="n">
-        <v>-36.01</v>
+        <v>-36.04</v>
       </c>
       <c r="BE66" t="n">
         <v>-59.83</v>
@@ -15674,7 +15674,7 @@
         <v>-89.01000000000001</v>
       </c>
       <c r="BG66" t="n">
-        <v>-82.93000000000001</v>
+        <v>-82.94</v>
       </c>
       <c r="BH66" t="n">
         <v>7.12</v>
@@ -15683,7 +15683,7 @@
         <v>0</v>
       </c>
       <c r="BJ66" t="n">
-        <v>20.3</v>
+        <v>20.31</v>
       </c>
       <c r="BK66" t="n">
         <v>1.58</v>
@@ -15692,7 +15692,7 @@
         <v>1.57</v>
       </c>
       <c r="BM66" t="n">
-        <v>20.3</v>
+        <v>20.31</v>
       </c>
       <c r="BN66" t="n">
         <v>21.33</v>
@@ -15701,19 +15701,19 @@
         <v>9.48</v>
       </c>
       <c r="BP66" t="n">
-        <v>20.3</v>
+        <v>20.31</v>
       </c>
       <c r="BQ66" t="n">
-        <v>12.93</v>
+        <v>12.94</v>
       </c>
       <c r="BR66" t="n">
-        <v>20.3</v>
+        <v>20.31</v>
       </c>
       <c r="BS66" t="n">
         <v>3.46</v>
       </c>
       <c r="BT66" t="n">
-        <v>4500</v>
+        <v>4393</v>
       </c>
     </row>
     <row r="67">
@@ -15973,13 +15973,13 @@
         </is>
       </c>
       <c r="F68" t="n">
-        <v>17.98</v>
+        <v>17.82</v>
       </c>
       <c r="G68" t="n">
-        <v>7624144793</v>
+        <v>7776608331</v>
       </c>
       <c r="H68" t="n">
-        <v>76100</v>
+        <v>89400</v>
       </c>
       <c r="I68" t="n">
         <v>137989898</v>
@@ -16072,7 +16072,7 @@
         <v>205604948.02</v>
       </c>
       <c r="AM68" t="n">
-        <v>528720165.9500694</v>
+        <v>539293226.8377254</v>
       </c>
       <c r="AN68" t="n">
         <v>0.1911</v>
@@ -16113,7 +16113,7 @@
         <v>21.39</v>
       </c>
       <c r="AZ68" t="n">
-        <v>33.26</v>
+        <v>32.97</v>
       </c>
       <c r="BA68" t="n">
         <v>1.24</v>
@@ -16122,19 +16122,19 @@
         <v>63.25</v>
       </c>
       <c r="BC68" t="n">
-        <v>45.73</v>
+        <v>47.04</v>
       </c>
       <c r="BD68" t="n">
-        <v>18.99</v>
+        <v>20.06</v>
       </c>
       <c r="BE68" t="n">
         <v>85</v>
       </c>
       <c r="BF68" t="n">
-        <v>-93.11</v>
+        <v>-93.04000000000001</v>
       </c>
       <c r="BG68" t="n">
-        <v>251.77</v>
+        <v>254.93</v>
       </c>
       <c r="BH68" t="n">
         <v>20.48</v>
@@ -16143,7 +16143,7 @@
         <v>0</v>
       </c>
       <c r="BJ68" t="n">
-        <v>17.98</v>
+        <v>17.82</v>
       </c>
       <c r="BK68" t="n">
         <v>1.49</v>
@@ -16152,28 +16152,28 @@
         <v>1.49</v>
       </c>
       <c r="BM68" t="n">
-        <v>18.13</v>
+        <v>18.07</v>
       </c>
       <c r="BN68" t="n">
         <v>22.11</v>
       </c>
       <c r="BO68" t="n">
-        <v>15.39</v>
+        <v>15.45</v>
       </c>
       <c r="BP68" t="n">
-        <v>17.9</v>
+        <v>17.68</v>
       </c>
       <c r="BQ68" t="n">
-        <v>12.09</v>
+        <v>11.99</v>
       </c>
       <c r="BR68" t="n">
-        <v>17.97</v>
+        <v>18.05</v>
       </c>
       <c r="BS68" t="n">
         <v>0</v>
       </c>
       <c r="BT68" t="n">
-        <v>40317</v>
+        <v>40983</v>
       </c>
     </row>
     <row r="69">
@@ -16203,13 +16203,13 @@
         </is>
       </c>
       <c r="F69" t="n">
-        <v>20.24</v>
+        <v>20.59</v>
       </c>
       <c r="G69" t="n">
-        <v>7624144793</v>
+        <v>7776608331</v>
       </c>
       <c r="H69" t="n">
-        <v>2431700</v>
+        <v>2533500</v>
       </c>
       <c r="I69" t="n">
         <v>255106712</v>
@@ -16302,7 +16302,7 @@
         <v>380109000.88</v>
       </c>
       <c r="AM69" t="n">
-        <v>453818142.4404762</v>
+        <v>462893353.0357143</v>
       </c>
       <c r="AN69" t="n">
         <v>0.8856000000000001</v>
@@ -16343,7 +16343,7 @@
         <v>21.39</v>
       </c>
       <c r="AZ69" t="n">
-        <v>35.39</v>
+        <v>36</v>
       </c>
       <c r="BA69" t="n">
         <v>1.24</v>
@@ -16352,19 +16352,19 @@
         <v>69.59</v>
       </c>
       <c r="BC69" t="n">
-        <v>29.46</v>
+        <v>27.26</v>
       </c>
       <c r="BD69" t="n">
-        <v>5.7</v>
+        <v>3.91</v>
       </c>
       <c r="BE69" t="n">
         <v>74.83</v>
       </c>
       <c r="BF69" t="n">
-        <v>-93.88</v>
+        <v>-93.98</v>
       </c>
       <c r="BG69" t="n">
-        <v>243.81</v>
+        <v>237.96</v>
       </c>
       <c r="BH69" t="n">
         <v>20.48</v>
@@ -16373,7 +16373,7 @@
         <v>0</v>
       </c>
       <c r="BJ69" t="n">
-        <v>20.24</v>
+        <v>20.59</v>
       </c>
       <c r="BK69" t="n">
         <v>1.49</v>
@@ -16382,28 +16382,28 @@
         <v>1.49</v>
       </c>
       <c r="BM69" t="n">
-        <v>20.49</v>
+        <v>20.64</v>
       </c>
       <c r="BN69" t="n">
         <v>25.63</v>
       </c>
       <c r="BO69" t="n">
-        <v>16.73</v>
+        <v>16.87</v>
       </c>
       <c r="BP69" t="n">
-        <v>20.13</v>
+        <v>20.02</v>
       </c>
       <c r="BQ69" t="n">
-        <v>13.61</v>
+        <v>13.85</v>
       </c>
       <c r="BR69" t="n">
-        <v>20.38</v>
+        <v>20.15</v>
       </c>
       <c r="BS69" t="n">
         <v>0</v>
       </c>
       <c r="BT69" t="n">
-        <v>2102360</v>
+        <v>2079770</v>
       </c>
     </row>
     <row r="70">
@@ -16433,13 +16433,13 @@
         </is>
       </c>
       <c r="F70" t="n">
-        <v>17.41</v>
+        <v>17.96</v>
       </c>
       <c r="G70" t="n">
-        <v>8087940781</v>
+        <v>8343446886</v>
       </c>
       <c r="H70" t="n">
-        <v>1425800</v>
+        <v>2470500</v>
       </c>
       <c r="I70" t="n">
         <v>464557268</v>
@@ -16454,7 +16454,7 @@
         <v>0.68</v>
       </c>
       <c r="M70" t="n">
-        <v>0.6383665676212533</v>
+        <v>0.6585332033164962</v>
       </c>
       <c r="N70" t="n">
         <v>0.2</v>
@@ -16532,7 +16532,7 @@
         <v>55746872.16</v>
       </c>
       <c r="AM70" t="n">
-        <v>2669287386.468647</v>
+        <v>2753612833.663366</v>
       </c>
       <c r="AN70" t="n">
         <v>0.1236</v>
@@ -16573,7 +16573,7 @@
         <v>6.9</v>
       </c>
       <c r="AZ70" t="n">
-        <v>2</v>
+        <v>2.07</v>
       </c>
       <c r="BA70" t="n">
         <v>0.12</v>
@@ -16582,19 +16582,19 @@
         <v>1.07</v>
       </c>
       <c r="BC70" t="n">
-        <v>-51.47</v>
+        <v>-52.96</v>
       </c>
       <c r="BD70" t="n">
-        <v>-60.38</v>
+        <v>-61.59</v>
       </c>
       <c r="BE70" t="n">
         <v>-88.5</v>
       </c>
       <c r="BF70" t="n">
-        <v>-99.31</v>
+        <v>-99.33</v>
       </c>
       <c r="BG70" t="n">
-        <v>-93.86</v>
+        <v>-94.05</v>
       </c>
       <c r="BH70" t="n">
         <v>26.44</v>
@@ -16603,7 +16603,7 @@
         <v>0</v>
       </c>
       <c r="BJ70" t="n">
-        <v>17.41</v>
+        <v>17.96</v>
       </c>
       <c r="BK70" t="n">
         <v>0.12</v>
@@ -16612,7 +16612,7 @@
         <v>0.1</v>
       </c>
       <c r="BM70" t="n">
-        <v>17.53</v>
+        <v>18.03</v>
       </c>
       <c r="BN70" t="n">
         <v>22.15</v>
@@ -16621,19 +16621,19 @@
         <v>13.21</v>
       </c>
       <c r="BP70" t="n">
-        <v>17.3</v>
+        <v>17.38</v>
       </c>
       <c r="BQ70" t="n">
-        <v>174.61</v>
+        <v>180.12</v>
       </c>
       <c r="BR70" t="n">
-        <v>17.41</v>
+        <v>17.43</v>
       </c>
       <c r="BS70" t="n">
         <v>0.67</v>
       </c>
       <c r="BT70" t="n">
-        <v>4079570</v>
+        <v>3976160</v>
       </c>
     </row>
     <row r="71">

</xml_diff>

<commit_message>
📊 Dados atualizados - 2026-09-30 06:13
</commit_message>
<xml_diff>
--- a/data/ativos.xlsx
+++ b/data/ativos.xlsx
@@ -1047,13 +1047,13 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>25</v>
+        <v>25.18</v>
       </c>
       <c r="G3" t="n">
-        <v>3344172500</v>
+        <v>3368248064</v>
       </c>
       <c r="H3" t="n">
-        <v>393900</v>
+        <v>601000</v>
       </c>
       <c r="I3" t="n">
         <v>129510368</v>
@@ -1068,7 +1068,7 @@
         <v>0.88</v>
       </c>
       <c r="M3" t="n">
-        <v>0.8321045974811152</v>
+        <v>0.8380951340013906</v>
       </c>
       <c r="N3" t="n">
         <v>0.09</v>
@@ -1146,7 +1146,7 @@
         <v>506385538.88</v>
       </c>
       <c r="AM3" t="n">
-        <v>653158691.40625</v>
+        <v>657860950</v>
       </c>
       <c r="AN3" t="n">
         <v>2.7</v>
@@ -1187,7 +1187,7 @@
         <v>40.42</v>
       </c>
       <c r="AZ3" t="n">
-        <v>45.75</v>
+        <v>46.08</v>
       </c>
       <c r="BA3" t="n">
         <v>4.87</v>
@@ -1196,19 +1196,19 @@
         <v>21.14</v>
       </c>
       <c r="BC3" t="n">
-        <v>97.98999999999999</v>
+        <v>96.58</v>
       </c>
       <c r="BD3" t="n">
-        <v>61.66</v>
+        <v>60.51</v>
       </c>
       <c r="BE3" t="n">
         <v>83</v>
       </c>
       <c r="BF3" t="n">
-        <v>-80.53</v>
+        <v>-80.66</v>
       </c>
       <c r="BG3" t="n">
-        <v>-15.46</v>
+        <v>-16.06</v>
       </c>
       <c r="BH3" t="n">
         <v>27.85</v>
@@ -1217,7 +1217,7 @@
         <v>0</v>
       </c>
       <c r="BJ3" t="n">
-        <v>25</v>
+        <v>25.18</v>
       </c>
       <c r="BK3" t="n">
         <v>3.91</v>
@@ -1226,7 +1226,7 @@
         <v>4.39</v>
       </c>
       <c r="BM3" t="n">
-        <v>25</v>
+        <v>25.18</v>
       </c>
       <c r="BN3" t="n">
         <v>27.17</v>
@@ -1235,19 +1235,19 @@
         <v>18.72</v>
       </c>
       <c r="BP3" t="n">
-        <v>24.52</v>
+        <v>24.74</v>
       </c>
       <c r="BQ3" t="n">
-        <v>5.69</v>
+        <v>5.73</v>
       </c>
       <c r="BR3" t="n">
-        <v>24.69</v>
+        <v>24.98</v>
       </c>
       <c r="BS3" t="n">
         <v>0.79</v>
       </c>
       <c r="BT3" t="n">
-        <v>511877</v>
+        <v>507783</v>
       </c>
     </row>
     <row r="4">
@@ -1277,13 +1277,13 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>15.2</v>
+        <v>15.27</v>
       </c>
       <c r="G4" t="n">
-        <v>235366829046</v>
+        <v>236450765288</v>
       </c>
       <c r="H4" t="n">
-        <v>17925900</v>
+        <v>21988800</v>
       </c>
       <c r="I4" t="n">
         <v>15484664889</v>
@@ -1298,7 +1298,7 @@
         <v>2.76</v>
       </c>
       <c r="M4" t="n">
-        <v>2.665065791772331</v>
+        <v>2.677339234936456</v>
       </c>
       <c r="N4" t="n">
         <v>1.76</v>
@@ -1376,7 +1376,7 @@
         <v>16258898133.45</v>
       </c>
       <c r="AM4" t="n">
-        <v>23303646440.19802</v>
+        <v>23410966860.19802</v>
       </c>
       <c r="AN4" t="n">
         <v>0.269</v>
@@ -1417,7 +1417,7 @@
         <v>9.470000000000001</v>
       </c>
       <c r="AZ4" t="n">
-        <v>18.97</v>
+        <v>19.06</v>
       </c>
       <c r="BA4" t="n">
         <v>1.13</v>
@@ -1426,19 +1426,19 @@
         <v>11.39</v>
       </c>
       <c r="BC4" t="n">
-        <v>-23.66</v>
+        <v>-24.01</v>
       </c>
       <c r="BD4" t="n">
-        <v>-37.66</v>
+        <v>-37.95</v>
       </c>
       <c r="BE4" t="n">
         <v>24.83</v>
       </c>
       <c r="BF4" t="n">
-        <v>-92.58</v>
+        <v>-92.62</v>
       </c>
       <c r="BG4" t="n">
-        <v>-25.09</v>
+        <v>-25.43</v>
       </c>
       <c r="BH4" t="n">
         <v>5.7</v>
@@ -1447,7 +1447,7 @@
         <v>0</v>
       </c>
       <c r="BJ4" t="n">
-        <v>15.2</v>
+        <v>15.27</v>
       </c>
       <c r="BK4" t="n">
         <v>1.05</v>
@@ -1456,7 +1456,7 @@
         <v>1.04</v>
       </c>
       <c r="BM4" t="n">
-        <v>15.36</v>
+        <v>15.43</v>
       </c>
       <c r="BN4" t="n">
         <v>16.94</v>
@@ -1465,19 +1465,19 @@
         <v>11.04</v>
       </c>
       <c r="BP4" t="n">
-        <v>15.14</v>
+        <v>15.08</v>
       </c>
       <c r="BQ4" t="n">
-        <v>14.66</v>
+        <v>14.73</v>
       </c>
       <c r="BR4" t="n">
-        <v>15.18</v>
+        <v>15.12</v>
       </c>
       <c r="BS4" t="n">
         <v>2.76</v>
       </c>
       <c r="BT4" t="n">
-        <v>26800337</v>
+        <v>26280057</v>
       </c>
     </row>
     <row r="5">
@@ -1737,13 +1737,13 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>7.4</v>
+        <v>7.37</v>
       </c>
       <c r="G6" t="n">
-        <v>466826786</v>
+        <v>464934231</v>
       </c>
       <c r="H6" t="n">
-        <v>700</v>
+        <v>200</v>
       </c>
       <c r="I6" t="n">
         <v>63084700</v>
@@ -1758,7 +1758,7 @@
         <v>1.91</v>
       </c>
       <c r="M6" t="n">
-        <v>7.267579040776673</v>
+        <v>7.238115664929348</v>
       </c>
       <c r="N6" t="n">
         <v>1.26</v>
@@ -1836,7 +1836,7 @@
         <v>35958279</v>
       </c>
       <c r="AM6" t="n">
-        <v>44629711.85468451</v>
+        <v>44448779.2543021</v>
       </c>
       <c r="AN6" t="n">
         <v>0.5199</v>
@@ -1877,7 +1877,7 @@
         <v>5.74</v>
       </c>
       <c r="AZ6" t="n">
-        <v>8.68</v>
+        <v>8.65</v>
       </c>
       <c r="BA6" t="n">
         <v>0.65</v>
@@ -1886,19 +1886,19 @@
         <v>7.95</v>
       </c>
       <c r="BC6" t="n">
-        <v>-4.92</v>
+        <v>-4.53</v>
       </c>
       <c r="BD6" t="n">
-        <v>-22.37</v>
+        <v>-22.05</v>
       </c>
       <c r="BE6" t="n">
         <v>17.33</v>
       </c>
       <c r="BF6" t="n">
-        <v>-91.23999999999999</v>
+        <v>-91.2</v>
       </c>
       <c r="BG6" t="n">
-        <v>7.48</v>
+        <v>7.92</v>
       </c>
       <c r="BH6" t="n">
         <v>3.86</v>
@@ -1907,7 +1907,7 @@
         <v>0</v>
       </c>
       <c r="BJ6" t="n">
-        <v>7.4</v>
+        <v>7.37</v>
       </c>
       <c r="BK6" t="n">
         <v>0.57</v>
@@ -1916,7 +1916,7 @@
         <v>0.5600000000000001</v>
       </c>
       <c r="BM6" t="n">
-        <v>7.4</v>
+        <v>7.37</v>
       </c>
       <c r="BN6" t="n">
         <v>8.16</v>
@@ -1925,19 +1925,19 @@
         <v>6.22</v>
       </c>
       <c r="BP6" t="n">
-        <v>7.4</v>
+        <v>7.32</v>
       </c>
       <c r="BQ6" t="n">
-        <v>13.16</v>
+        <v>13.11</v>
       </c>
       <c r="BR6" t="n">
-        <v>7.4</v>
+        <v>7.32</v>
       </c>
       <c r="BS6" t="n">
         <v>7.32</v>
       </c>
       <c r="BT6" t="n">
-        <v>167</v>
+        <v>180</v>
       </c>
     </row>
     <row r="7">
@@ -2433,7 +2433,7 @@
         <v>201081285</v>
       </c>
       <c r="H9" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I9" t="n">
         <v>8407877</v>
@@ -2609,7 +2609,7 @@
         <v>23.01</v>
       </c>
       <c r="BN9" t="n">
-        <v>34.04</v>
+        <v>29.5</v>
       </c>
       <c r="BO9" t="n">
         <v>21.5</v>
@@ -3120,10 +3120,10 @@
         <v>4.93</v>
       </c>
       <c r="G12" t="n">
-        <v>473090277</v>
+        <v>473090375</v>
       </c>
       <c r="H12" t="n">
-        <v>237500</v>
+        <v>198700</v>
       </c>
       <c r="I12" t="n">
         <v>95961536</v>
@@ -3138,7 +3138,7 @@
         <v>0.32</v>
       </c>
       <c r="M12" t="n">
-        <v>0.08555765469025964</v>
+        <v>0.0855576724134101</v>
       </c>
       <c r="N12" t="n">
         <v>0.14</v>
@@ -3216,7 +3216,7 @@
         <v>362734606.08</v>
       </c>
       <c r="AM12" t="n">
-        <v>508699222.5806451</v>
+        <v>508699327.9569892</v>
       </c>
       <c r="AN12" t="n">
         <v>0.4208</v>
@@ -3305,19 +3305,19 @@
         <v>4.42</v>
       </c>
       <c r="BP12" t="n">
-        <v>4.87</v>
+        <v>4.9</v>
       </c>
       <c r="BQ12" t="n">
         <v>1.36</v>
       </c>
       <c r="BR12" t="n">
-        <v>4.94</v>
+        <v>4.95</v>
       </c>
       <c r="BS12" t="n">
         <v>0.09</v>
       </c>
       <c r="BT12" t="n">
-        <v>494383</v>
+        <v>479890</v>
       </c>
     </row>
     <row r="13">
@@ -3347,13 +3347,13 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>28.57</v>
+        <v>28.77</v>
       </c>
       <c r="G13" t="n">
-        <v>14404731002</v>
+        <v>14505578177</v>
       </c>
       <c r="H13" t="n">
-        <v>3408200</v>
+        <v>2658500</v>
       </c>
       <c r="I13" t="n">
         <v>504190947</v>
@@ -3368,7 +3368,7 @@
         <v>1.13</v>
       </c>
       <c r="M13" t="n">
-        <v>4.981988764477982</v>
+        <v>5.016867547893624</v>
       </c>
       <c r="N13" t="n">
         <v>0.57</v>
@@ -3446,7 +3446,7 @@
         <v>932753251.95</v>
       </c>
       <c r="AM13" t="n">
-        <v>1498931425.806452</v>
+        <v>1509425408.636837</v>
       </c>
       <c r="AN13" t="n">
         <v>2.6301</v>
@@ -3487,7 +3487,7 @@
         <v>26.6</v>
       </c>
       <c r="AZ13" t="n">
-        <v>51.71</v>
+        <v>52.07</v>
       </c>
       <c r="BA13" t="n">
         <v>2.6</v>
@@ -3496,19 +3496,19 @@
         <v>8.69</v>
       </c>
       <c r="BC13" t="n">
-        <v>14.01</v>
+        <v>13.22</v>
       </c>
       <c r="BD13" t="n">
-        <v>-6.91</v>
+        <v>-7.56</v>
       </c>
       <c r="BE13" t="n">
         <v>81</v>
       </c>
       <c r="BF13" t="n">
-        <v>-90.88</v>
+        <v>-90.95</v>
       </c>
       <c r="BG13" t="n">
-        <v>-69.56999999999999</v>
+        <v>-69.78</v>
       </c>
       <c r="BH13" t="n">
         <v>25.49</v>
@@ -3517,7 +3517,7 @@
         <v>0</v>
       </c>
       <c r="BJ13" t="n">
-        <v>28.57</v>
+        <v>28.77</v>
       </c>
       <c r="BK13" t="n">
         <v>1.85</v>
@@ -3526,7 +3526,7 @@
         <v>1.96</v>
       </c>
       <c r="BM13" t="n">
-        <v>28.96</v>
+        <v>28.88</v>
       </c>
       <c r="BN13" t="n">
         <v>32.11</v>
@@ -3535,19 +3535,19 @@
         <v>20.85</v>
       </c>
       <c r="BP13" t="n">
-        <v>28.4</v>
+        <v>28.37</v>
       </c>
       <c r="BQ13" t="n">
-        <v>14.6</v>
+        <v>14.7</v>
       </c>
       <c r="BR13" t="n">
-        <v>28.96</v>
+        <v>28.57</v>
       </c>
       <c r="BS13" t="n">
         <v>5.01</v>
       </c>
       <c r="BT13" t="n">
-        <v>4921580</v>
+        <v>4844347</v>
       </c>
     </row>
     <row r="14">
@@ -3577,13 +3577,13 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>10.2</v>
+        <v>9.93</v>
       </c>
       <c r="G14" t="n">
-        <v>8511180935</v>
+        <v>8220231737</v>
       </c>
       <c r="H14" t="n">
-        <v>7800</v>
+        <v>3300</v>
       </c>
       <c r="I14" t="n">
         <v>339510689</v>
@@ -3598,7 +3598,7 @@
         <v>1.92</v>
       </c>
       <c r="M14" t="n">
-        <v>3.533993633293722</v>
+        <v>3.413186353881337</v>
       </c>
       <c r="N14" t="n">
         <v>1.11</v>
@@ -3676,7 +3676,7 @@
         <v>349696009.67</v>
       </c>
       <c r="AM14" t="n">
-        <v>944637173.6958935</v>
+        <v>912345364.8168702</v>
       </c>
       <c r="AN14" t="n">
         <v>0.1489</v>
@@ -3717,7 +3717,7 @@
         <v>9.050000000000001</v>
       </c>
       <c r="AZ14" t="n">
-        <v>8.19</v>
+        <v>7.98</v>
       </c>
       <c r="BA14" t="n">
         <v>1.42</v>
@@ -3726,19 +3726,19 @@
         <v>5.94</v>
       </c>
       <c r="BC14" t="n">
-        <v>8.65</v>
+        <v>11.61</v>
       </c>
       <c r="BD14" t="n">
-        <v>-11.28</v>
+        <v>-8.869999999999999</v>
       </c>
       <c r="BE14" t="n">
         <v>-19.67</v>
       </c>
       <c r="BF14" t="n">
-        <v>-86.06999999999999</v>
+        <v>-85.69</v>
       </c>
       <c r="BG14" t="n">
-        <v>-41.74</v>
+        <v>-40.16</v>
       </c>
       <c r="BH14" t="n">
         <v>5.3</v>
@@ -3747,7 +3747,7 @@
         <v>0</v>
       </c>
       <c r="BJ14" t="n">
-        <v>10.2</v>
+        <v>9.93</v>
       </c>
       <c r="BK14" t="n">
         <v>1.03</v>
@@ -3756,28 +3756,28 @@
         <v>1.01</v>
       </c>
       <c r="BM14" t="n">
-        <v>10.39</v>
+        <v>10.29</v>
       </c>
       <c r="BN14" t="n">
         <v>13.49</v>
       </c>
       <c r="BO14" t="n">
-        <v>7.71</v>
+        <v>7.77</v>
       </c>
       <c r="BP14" t="n">
-        <v>10.05</v>
+        <v>9.93</v>
       </c>
       <c r="BQ14" t="n">
-        <v>10.07</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="BR14" t="n">
-        <v>10.38</v>
+        <v>10.2</v>
       </c>
       <c r="BS14" t="n">
         <v>1.44</v>
       </c>
       <c r="BT14" t="n">
-        <v>10650</v>
+        <v>10457</v>
       </c>
     </row>
     <row r="15">
@@ -3807,13 +3807,13 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>14.24</v>
+        <v>14.01</v>
       </c>
       <c r="G15" t="n">
-        <v>8511180935</v>
+        <v>8220231737</v>
       </c>
       <c r="H15" t="n">
-        <v>1462200</v>
+        <v>1491500</v>
       </c>
       <c r="I15" t="n">
         <v>343551533</v>
@@ -3828,7 +3828,7 @@
         <v>2.56</v>
       </c>
       <c r="M15" t="n">
-        <v>3.492426894107805</v>
+        <v>3.37304054670497</v>
       </c>
       <c r="N15" t="n">
         <v>1.47</v>
@@ -3906,7 +3906,7 @@
         <v>353858078.99</v>
       </c>
       <c r="AM15" t="n">
-        <v>709856625.1042535</v>
+        <v>685590636.9474562</v>
       </c>
       <c r="AN15" t="n">
         <v>0.1638</v>
@@ -3947,7 +3947,7 @@
         <v>9.050000000000001</v>
       </c>
       <c r="AZ15" t="n">
-        <v>9.470000000000001</v>
+        <v>9.32</v>
       </c>
       <c r="BA15" t="n">
         <v>1.42</v>
@@ -3956,19 +3956,19 @@
         <v>6.19</v>
       </c>
       <c r="BC15" t="n">
-        <v>-22.17</v>
+        <v>-20.89</v>
       </c>
       <c r="BD15" t="n">
-        <v>-36.45</v>
+        <v>-35.41</v>
       </c>
       <c r="BE15" t="n">
         <v>-33.5</v>
       </c>
       <c r="BF15" t="n">
-        <v>-90.02</v>
+        <v>-89.86</v>
       </c>
       <c r="BG15" t="n">
-        <v>-56.54</v>
+        <v>-55.83</v>
       </c>
       <c r="BH15" t="n">
         <v>5.3</v>
@@ -3977,7 +3977,7 @@
         <v>0</v>
       </c>
       <c r="BJ15" t="n">
-        <v>14.24</v>
+        <v>14.01</v>
       </c>
       <c r="BK15" t="n">
         <v>1.03</v>
@@ -3986,7 +3986,7 @@
         <v>1.01</v>
       </c>
       <c r="BM15" t="n">
-        <v>14.3</v>
+        <v>14.34</v>
       </c>
       <c r="BN15" t="n">
         <v>16.22</v>
@@ -3995,19 +3995,19 @@
         <v>7.84</v>
       </c>
       <c r="BP15" t="n">
-        <v>13.62</v>
+        <v>13.91</v>
       </c>
       <c r="BQ15" t="n">
-        <v>14.06</v>
+        <v>13.83</v>
       </c>
       <c r="BR15" t="n">
-        <v>13.85</v>
+        <v>14.14</v>
       </c>
       <c r="BS15" t="n">
         <v>1.92</v>
       </c>
       <c r="BT15" t="n">
-        <v>2377230</v>
+        <v>2346800</v>
       </c>
     </row>
     <row r="16">
@@ -4037,13 +4037,13 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>4.41</v>
+        <v>4.44</v>
       </c>
       <c r="G16" t="n">
-        <v>967138103</v>
+        <v>973717320</v>
       </c>
       <c r="H16" t="n">
-        <v>74500</v>
+        <v>46200</v>
       </c>
       <c r="I16" t="n">
         <v>219305733</v>
@@ -4058,7 +4058,7 @@
         <v>2.69</v>
       </c>
       <c r="M16" t="n">
-        <v>0.4575374150672568</v>
+        <v>0.4606499363607608</v>
       </c>
       <c r="N16" t="n">
         <v>0.39</v>
@@ -4136,7 +4136,7 @@
         <v>17544458.64</v>
       </c>
       <c r="AM16" t="n">
-        <v>271668006.4606742</v>
+        <v>273516101.1235955</v>
       </c>
       <c r="AN16" t="n">
         <v>0.0077</v>
@@ -4177,7 +4177,7 @@
         <v>1.42</v>
       </c>
       <c r="AZ16" t="n">
-        <v>0.12</v>
+        <v>0.13</v>
       </c>
       <c r="BA16" t="n">
         <v>0.08</v>
@@ -4186,16 +4186,16 @@
         <v>0</v>
       </c>
       <c r="BC16" t="n">
-        <v>-60.57</v>
+        <v>-60.83</v>
       </c>
       <c r="BD16" t="n">
-        <v>-67.8</v>
+        <v>-68.02</v>
       </c>
       <c r="BE16" t="n">
         <v>-97.17</v>
       </c>
       <c r="BF16" t="n">
-        <v>-98.19</v>
+        <v>-98.2</v>
       </c>
       <c r="BG16" t="n">
         <v>-100</v>
@@ -4207,7 +4207,7 @@
         <v>0</v>
       </c>
       <c r="BJ16" t="n">
-        <v>4.41</v>
+        <v>4.44</v>
       </c>
       <c r="BK16" t="n">
         <v>0.08</v>
@@ -4225,19 +4225,19 @@
         <v>3.22</v>
       </c>
       <c r="BP16" t="n">
-        <v>4.39</v>
+        <v>4.36</v>
       </c>
       <c r="BQ16" t="n">
-        <v>60.18</v>
+        <v>60.59</v>
       </c>
       <c r="BR16" t="n">
-        <v>4.48</v>
+        <v>4.38</v>
       </c>
       <c r="BS16" t="n">
         <v>0.49</v>
       </c>
       <c r="BT16" t="n">
-        <v>133407</v>
+        <v>127940</v>
       </c>
     </row>
     <row r="17">
@@ -4267,13 +4267,13 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>31.55</v>
+        <v>31.79</v>
       </c>
       <c r="G17" t="n">
-        <v>10399728443</v>
+        <v>10478839452</v>
       </c>
       <c r="H17" t="n">
-        <v>887200</v>
+        <v>663800</v>
       </c>
       <c r="I17" t="n">
         <v>0</v>
@@ -4360,13 +4360,13 @@
         <v>8.039999999999999</v>
       </c>
       <c r="AK17" t="n">
-        <v>4696409159.591763</v>
+        <v>4732134868.135839</v>
       </c>
       <c r="AL17" t="n">
-        <v>1299966055.375</v>
+        <v>1309854931.5</v>
       </c>
       <c r="AM17" t="n">
-        <v>3219730168.111455</v>
+        <v>3244222740.557276</v>
       </c>
       <c r="AN17" t="n">
         <v>1.08</v>
@@ -4407,7 +4407,7 @@
         <v>42.98</v>
       </c>
       <c r="AZ17" t="n">
-        <v>16.88</v>
+        <v>17.01</v>
       </c>
       <c r="BA17" t="n">
         <v>4.55</v>
@@ -4416,19 +4416,19 @@
         <v>16.33</v>
       </c>
       <c r="BC17" t="n">
-        <v>66.84</v>
+        <v>65.58</v>
       </c>
       <c r="BD17" t="n">
-        <v>36.22</v>
+        <v>35.19</v>
       </c>
       <c r="BE17" t="n">
         <v>-46.5</v>
       </c>
       <c r="BF17" t="n">
-        <v>-85.58</v>
+        <v>-85.69</v>
       </c>
       <c r="BG17" t="n">
-        <v>-48.23</v>
+        <v>-48.62</v>
       </c>
       <c r="BH17" t="n">
         <v>29.25</v>
@@ -4437,7 +4437,7 @@
         <v>0</v>
       </c>
       <c r="BJ17" t="n">
-        <v>31.55</v>
+        <v>31.79</v>
       </c>
       <c r="BK17" t="n">
         <v>4.21</v>
@@ -4446,7 +4446,7 @@
         <v>12.62</v>
       </c>
       <c r="BM17" t="n">
-        <v>32.08</v>
+        <v>31.93</v>
       </c>
       <c r="BN17" t="n">
         <v>36.63</v>
@@ -4455,19 +4455,19 @@
         <v>29.53</v>
       </c>
       <c r="BP17" t="n">
-        <v>31.55</v>
+        <v>31.36</v>
       </c>
       <c r="BQ17" t="n">
-        <v>2.5</v>
+        <v>2.52</v>
       </c>
       <c r="BR17" t="n">
-        <v>32</v>
+        <v>31.61</v>
       </c>
       <c r="BS17" t="n">
         <v>2.21</v>
       </c>
       <c r="BT17" t="n">
-        <v>1153147</v>
+        <v>1125857</v>
       </c>
     </row>
     <row r="18">
@@ -4497,13 +4497,13 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>11</v>
+        <v>10.91</v>
       </c>
       <c r="G18" t="n">
-        <v>10399728443</v>
+        <v>10478839452</v>
       </c>
       <c r="H18" t="n">
-        <v>4800</v>
+        <v>12300</v>
       </c>
       <c r="I18" t="n">
         <v>671494278</v>
@@ -4518,7 +4518,7 @@
         <v>1.2</v>
       </c>
       <c r="M18" t="n">
-        <v>3.062088461653706</v>
+        <v>3.085381849474013</v>
       </c>
       <c r="N18" t="n">
         <v>0.33</v>
@@ -4596,7 +4596,7 @@
         <v>940091989.1999999</v>
       </c>
       <c r="AM18" t="n">
-        <v>3095157274.702381</v>
+        <v>3118702217.857143</v>
       </c>
       <c r="AN18" t="n">
         <v>0.36</v>
@@ -4637,7 +4637,7 @@
         <v>14.31</v>
       </c>
       <c r="AZ18" t="n">
-        <v>5.66</v>
+        <v>5.62</v>
       </c>
       <c r="BA18" t="n">
         <v>1.51</v>
@@ -4646,19 +4646,19 @@
         <v>5.44</v>
       </c>
       <c r="BC18" t="n">
-        <v>59.32</v>
+        <v>60.63</v>
       </c>
       <c r="BD18" t="n">
-        <v>30.08</v>
+        <v>31.16</v>
       </c>
       <c r="BE18" t="n">
         <v>-48.5</v>
       </c>
       <c r="BF18" t="n">
-        <v>-86.25</v>
+        <v>-86.14</v>
       </c>
       <c r="BG18" t="n">
-        <v>-50.51</v>
+        <v>-50.1</v>
       </c>
       <c r="BH18" t="n">
         <v>9.75</v>
@@ -4667,7 +4667,7 @@
         <v>0</v>
       </c>
       <c r="BJ18" t="n">
-        <v>11</v>
+        <v>10.91</v>
       </c>
       <c r="BK18" t="n">
         <v>1.4</v>
@@ -4676,7 +4676,7 @@
         <v>12.62</v>
       </c>
       <c r="BM18" t="n">
-        <v>11.2</v>
+        <v>11.26</v>
       </c>
       <c r="BN18" t="n">
         <v>13.82</v>
@@ -4685,19 +4685,19 @@
         <v>10.19</v>
       </c>
       <c r="BP18" t="n">
-        <v>10.96</v>
+        <v>10.9</v>
       </c>
       <c r="BQ18" t="n">
-        <v>0.87</v>
+        <v>0.86</v>
       </c>
       <c r="BR18" t="n">
-        <v>11.07</v>
+        <v>10.95</v>
       </c>
       <c r="BS18" t="n">
         <v>2.3</v>
       </c>
       <c r="BT18" t="n">
-        <v>10103</v>
+        <v>9557</v>
       </c>
     </row>
     <row r="19">
@@ -4727,13 +4727,13 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>10.52</v>
+        <v>10.4</v>
       </c>
       <c r="G19" t="n">
-        <v>10399728443</v>
+        <v>10478839452</v>
       </c>
       <c r="H19" t="n">
-        <v>14100</v>
+        <v>26000</v>
       </c>
       <c r="I19" t="n">
         <v>317386323</v>
@@ -4748,7 +4748,7 @@
         <v>1.12</v>
       </c>
       <c r="M19" t="n">
-        <v>6.47846089048483</v>
+        <v>6.527742713623035</v>
       </c>
       <c r="N19" t="n">
         <v>0.3</v>
@@ -4826,7 +4826,7 @@
         <v>444340852.2</v>
       </c>
       <c r="AM19" t="n">
-        <v>3301501093.015873</v>
+        <v>3326615699.047619</v>
       </c>
       <c r="AN19" t="n">
         <v>0.36</v>
@@ -4867,7 +4867,7 @@
         <v>14.31</v>
       </c>
       <c r="AZ19" t="n">
-        <v>5.79</v>
+        <v>5.72</v>
       </c>
       <c r="BA19" t="n">
         <v>1.51</v>
@@ -4876,19 +4876,19 @@
         <v>5.25</v>
       </c>
       <c r="BC19" t="n">
-        <v>66.59</v>
+        <v>68.51000000000001</v>
       </c>
       <c r="BD19" t="n">
-        <v>36.02</v>
+        <v>37.59</v>
       </c>
       <c r="BE19" t="n">
         <v>-45</v>
       </c>
       <c r="BF19" t="n">
-        <v>-85.62</v>
+        <v>-85.45999999999999</v>
       </c>
       <c r="BG19" t="n">
-        <v>-50.1</v>
+        <v>-49.52</v>
       </c>
       <c r="BH19" t="n">
         <v>9.75</v>
@@ -4897,7 +4897,7 @@
         <v>0</v>
       </c>
       <c r="BJ19" t="n">
-        <v>10.52</v>
+        <v>10.4</v>
       </c>
       <c r="BK19" t="n">
         <v>1.4</v>
@@ -4906,7 +4906,7 @@
         <v>12.62</v>
       </c>
       <c r="BM19" t="n">
-        <v>10.58</v>
+        <v>10.49</v>
       </c>
       <c r="BN19" t="n">
         <v>11.41</v>
@@ -4915,19 +4915,19 @@
         <v>9.19</v>
       </c>
       <c r="BP19" t="n">
-        <v>10.34</v>
+        <v>10.25</v>
       </c>
       <c r="BQ19" t="n">
-        <v>0.83</v>
+        <v>0.82</v>
       </c>
       <c r="BR19" t="n">
-        <v>10.58</v>
+        <v>10.32</v>
       </c>
       <c r="BS19" t="n">
         <v>2.16</v>
       </c>
       <c r="BT19" t="n">
-        <v>12983</v>
+        <v>11927</v>
       </c>
     </row>
     <row r="20">
@@ -5417,13 +5417,13 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>5.03</v>
+        <v>5.08</v>
       </c>
       <c r="G22" t="n">
-        <v>1007233901</v>
+        <v>1017246108</v>
       </c>
       <c r="H22" t="n">
-        <v>1465600</v>
+        <v>1192700</v>
       </c>
       <c r="I22" t="n">
         <v>200245299</v>
@@ -5438,7 +5438,7 @@
         <v>0.27</v>
       </c>
       <c r="M22" t="n">
-        <v>0.0854301627190838</v>
+        <v>0.08627936415316773</v>
       </c>
       <c r="N22" t="n">
         <v>0.08</v>
@@ -5516,7 +5516,7 @@
         <v>378463615.11</v>
       </c>
       <c r="AM22" t="n">
-        <v>228397709.9773242</v>
+        <v>230668051.7006803</v>
       </c>
       <c r="AN22" t="n">
         <v>0</v>
@@ -5566,19 +5566,19 @@
         <v>172.49</v>
       </c>
       <c r="BC22" t="n">
-        <v>490.56</v>
+        <v>484.75</v>
       </c>
       <c r="BD22" t="n">
-        <v>382.19</v>
+        <v>377.44</v>
       </c>
       <c r="BE22" t="n">
         <v>-100</v>
       </c>
       <c r="BF22" t="n">
-        <v>-62.43</v>
+        <v>-62.8</v>
       </c>
       <c r="BG22" t="n">
-        <v>3329.22</v>
+        <v>3295.47</v>
       </c>
       <c r="BH22" t="n">
         <v>20.75</v>
@@ -5587,7 +5587,7 @@
         <v>0</v>
       </c>
       <c r="BJ22" t="n">
-        <v>5.03</v>
+        <v>5.08</v>
       </c>
       <c r="BK22" t="n">
         <v>1.89</v>
@@ -5596,7 +5596,7 @@
         <v>0.67</v>
       </c>
       <c r="BM22" t="n">
-        <v>5.32</v>
+        <v>5.22</v>
       </c>
       <c r="BN22" t="n">
         <v>7.89</v>
@@ -5605,19 +5605,19 @@
         <v>3.37</v>
       </c>
       <c r="BP22" t="n">
-        <v>5.01</v>
+        <v>5.03</v>
       </c>
       <c r="BQ22" t="n">
-        <v>7.49</v>
+        <v>7.57</v>
       </c>
       <c r="BR22" t="n">
-        <v>5.16</v>
+        <v>5.03</v>
       </c>
       <c r="BS22" t="n">
         <v>0.09</v>
       </c>
       <c r="BT22" t="n">
-        <v>1516587</v>
+        <v>1532727</v>
       </c>
     </row>
     <row r="23">
@@ -5877,13 +5877,13 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.83</v>
+        <v>2.86</v>
       </c>
       <c r="G24" t="n">
-        <v>1142948956</v>
+        <v>1155065011</v>
       </c>
       <c r="H24" t="n">
-        <v>6200400</v>
+        <v>3842300</v>
       </c>
       <c r="I24" t="n">
         <v>403868805</v>
@@ -5898,7 +5898,7 @@
         <v>0.49</v>
       </c>
       <c r="M24" t="n">
-        <v>0.2762974259191084</v>
+        <v>0.2792263710756008</v>
       </c>
       <c r="N24" t="n">
         <v>0.11</v>
@@ -5976,7 +5976,7 @@
         <v>153470145.9</v>
       </c>
       <c r="AM24" t="n">
-        <v>1029683744.144144</v>
+        <v>1040599109.009009</v>
       </c>
       <c r="AN24" t="n">
         <v>0.0813</v>
@@ -6017,7 +6017,7 @@
         <v>5.84</v>
       </c>
       <c r="AZ24" t="n">
-        <v>1.31</v>
+        <v>1.32</v>
       </c>
       <c r="BA24" t="n">
         <v>0.38</v>
@@ -6026,19 +6026,19 @@
         <v>1.46</v>
       </c>
       <c r="BC24" t="n">
-        <v>152.88</v>
+        <v>150.22</v>
       </c>
       <c r="BD24" t="n">
-        <v>106.47</v>
+        <v>104.31</v>
       </c>
       <c r="BE24" t="n">
         <v>-53.83</v>
       </c>
       <c r="BF24" t="n">
-        <v>-86.56999999999999</v>
+        <v>-86.70999999999999</v>
       </c>
       <c r="BG24" t="n">
-        <v>-48.49</v>
+        <v>-49.03</v>
       </c>
       <c r="BH24" t="n">
         <v>5.99</v>
@@ -6047,7 +6047,7 @@
         <v>0</v>
       </c>
       <c r="BJ24" t="n">
-        <v>2.83</v>
+        <v>2.86</v>
       </c>
       <c r="BK24" t="n">
         <v>0.38</v>
@@ -6056,7 +6056,7 @@
         <v>0.41</v>
       </c>
       <c r="BM24" t="n">
-        <v>2.92</v>
+        <v>2.89</v>
       </c>
       <c r="BN24" t="n">
         <v>5.29</v>
@@ -6065,19 +6065,19 @@
         <v>1.92</v>
       </c>
       <c r="BP24" t="n">
-        <v>2.79</v>
+        <v>2.83</v>
       </c>
       <c r="BQ24" t="n">
-        <v>6.95</v>
+        <v>7.02</v>
       </c>
       <c r="BR24" t="n">
-        <v>2.92</v>
+        <v>2.83</v>
       </c>
       <c r="BS24" t="n">
         <v>0.29</v>
       </c>
       <c r="BT24" t="n">
-        <v>7743583</v>
+        <v>7454537</v>
       </c>
     </row>
     <row r="25">
@@ -6107,13 +6107,13 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>3.89</v>
+        <v>3.94</v>
       </c>
       <c r="G25" t="n">
-        <v>1347861696</v>
+        <v>1365186379</v>
       </c>
       <c r="H25" t="n">
-        <v>1645100</v>
+        <v>576400</v>
       </c>
       <c r="I25" t="n">
         <v>346494097</v>
@@ -6128,7 +6128,7 @@
         <v>0.97</v>
       </c>
       <c r="M25" t="n">
-        <v>0.6721053853528323</v>
+        <v>0.6807442633463135</v>
       </c>
       <c r="N25" t="n">
         <v>0.22</v>
@@ -6206,7 +6206,7 @@
         <v>62368937.46</v>
       </c>
       <c r="AM25" t="n">
-        <v>495537388.2352941</v>
+        <v>501906756.9852941</v>
       </c>
       <c r="AN25" t="n">
         <v>0.4742</v>
@@ -6247,7 +6247,7 @@
         <v>3.27</v>
       </c>
       <c r="AZ25" t="n">
-        <v>9.06</v>
+        <v>9.18</v>
       </c>
       <c r="BA25" t="n">
         <v>0.23</v>
@@ -6256,19 +6256,19 @@
         <v>2.2</v>
       </c>
       <c r="BC25" t="n">
-        <v>3.08</v>
+        <v>1.77</v>
       </c>
       <c r="BD25" t="n">
-        <v>-15.84</v>
+        <v>-16.9</v>
       </c>
       <c r="BE25" t="n">
         <v>133</v>
       </c>
       <c r="BF25" t="n">
-        <v>-94.04000000000001</v>
+        <v>-94.12</v>
       </c>
       <c r="BG25" t="n">
-        <v>-43.45</v>
+        <v>-44.17</v>
       </c>
       <c r="BH25" t="n">
         <v>3.97</v>
@@ -6277,7 +6277,7 @@
         <v>0</v>
       </c>
       <c r="BJ25" t="n">
-        <v>3.89</v>
+        <v>3.94</v>
       </c>
       <c r="BK25" t="n">
         <v>0.18</v>
@@ -6286,7 +6286,7 @@
         <v>0.24</v>
       </c>
       <c r="BM25" t="n">
-        <v>4.2</v>
+        <v>4.04</v>
       </c>
       <c r="BN25" t="n">
         <v>6.3</v>
@@ -6295,19 +6295,19 @@
         <v>2.64</v>
       </c>
       <c r="BP25" t="n">
-        <v>3.85</v>
+        <v>3.86</v>
       </c>
       <c r="BQ25" t="n">
-        <v>16.44</v>
+        <v>16.65</v>
       </c>
       <c r="BR25" t="n">
-        <v>4.17</v>
+        <v>3.89</v>
       </c>
       <c r="BS25" t="n">
         <v>0.67</v>
       </c>
       <c r="BT25" t="n">
-        <v>1133717</v>
+        <v>1153343</v>
       </c>
     </row>
     <row r="26">
@@ -6337,13 +6337,13 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>10.2</v>
+        <v>10.54</v>
       </c>
       <c r="G26" t="n">
-        <v>13814808341</v>
+        <v>14275302168</v>
       </c>
       <c r="H26" t="n">
-        <v>12189300</v>
+        <v>26249600</v>
       </c>
       <c r="I26" t="n">
         <v>1354393401</v>
@@ -6358,7 +6358,7 @@
         <v>1.94</v>
       </c>
       <c r="M26" t="n">
-        <v>0.1781407889878552</v>
+        <v>0.184078818068024</v>
       </c>
       <c r="N26" t="n">
         <v>0.26</v>
@@ -6436,7 +6436,7 @@
         <v>961619314.7099999</v>
       </c>
       <c r="AM26" t="n">
-        <v>4933860121.785714</v>
+        <v>5098322202.857143</v>
       </c>
       <c r="AN26" t="n">
         <v>0.1043</v>
@@ -6477,7 +6477,7 @@
         <v>7.07</v>
       </c>
       <c r="AZ26" t="n">
-        <v>1.95</v>
+        <v>2.02</v>
       </c>
       <c r="BA26" t="n">
         <v>0.66</v>
@@ -6486,19 +6486,19 @@
         <v>1.19</v>
       </c>
       <c r="BC26" t="n">
-        <v>-15.14</v>
+        <v>-17.88</v>
       </c>
       <c r="BD26" t="n">
-        <v>-30.71</v>
+        <v>-32.95</v>
       </c>
       <c r="BE26" t="n">
         <v>-80.83</v>
       </c>
       <c r="BF26" t="n">
-        <v>-93.54000000000001</v>
+        <v>-93.75</v>
       </c>
       <c r="BG26" t="n">
-        <v>-88.3</v>
+        <v>-88.68000000000001</v>
       </c>
       <c r="BH26" t="n">
         <v>4.69</v>
@@ -6507,7 +6507,7 @@
         <v>0</v>
       </c>
       <c r="BJ26" t="n">
-        <v>10.2</v>
+        <v>10.54</v>
       </c>
       <c r="BK26" t="n">
         <v>0.71</v>
@@ -6516,7 +6516,7 @@
         <v>0.72</v>
       </c>
       <c r="BM26" t="n">
-        <v>10.48</v>
+        <v>10.55</v>
       </c>
       <c r="BN26" t="n">
         <v>10.55</v>
@@ -6528,16 +6528,16 @@
         <v>10.19</v>
       </c>
       <c r="BQ26" t="n">
-        <v>14.22</v>
+        <v>14.7</v>
       </c>
       <c r="BR26" t="n">
-        <v>10.35</v>
+        <v>10.2</v>
       </c>
       <c r="BS26" t="n">
         <v>0.16</v>
       </c>
       <c r="BT26" t="n">
-        <v>12366230</v>
+        <v>12398140</v>
       </c>
     </row>
     <row r="27">
@@ -8165,13 +8165,13 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>15.52</v>
+        <v>17.15</v>
       </c>
       <c r="G34" t="n">
-        <v>3204721790</v>
+        <v>3541299991</v>
       </c>
       <c r="H34" t="n">
-        <v>3819600</v>
+        <v>6522400</v>
       </c>
       <c r="I34" t="n">
         <v>206489813</v>
@@ -8186,7 +8186,7 @@
         <v>0.45</v>
       </c>
       <c r="M34" t="n">
-        <v>0.2817324746030705</v>
+        <v>0.3113216295060238</v>
       </c>
       <c r="N34" t="n">
         <v>0.24</v>
@@ -8264,7 +8264,7 @@
         <v>324189006.41</v>
       </c>
       <c r="AM34" t="n">
-        <v>666262326.4033265</v>
+        <v>736237004.3659045</v>
       </c>
       <c r="AN34" t="n">
         <v>0</v>
@@ -8305,7 +8305,7 @@
         <v>30.28</v>
       </c>
       <c r="AZ34" t="n">
-        <v>36.21</v>
+        <v>40.02</v>
       </c>
       <c r="BA34" t="n">
         <v>2.29</v>
@@ -8314,19 +8314,19 @@
         <v>25.26</v>
       </c>
       <c r="BC34" t="n">
-        <v>138.97</v>
+        <v>116.26</v>
       </c>
       <c r="BD34" t="n">
-        <v>95.12</v>
+        <v>76.58</v>
       </c>
       <c r="BE34" t="n">
         <v>133.33</v>
       </c>
       <c r="BF34" t="n">
-        <v>-85.20999999999999</v>
+        <v>-86.62</v>
       </c>
       <c r="BG34" t="n">
-        <v>62.74</v>
+        <v>47.28</v>
       </c>
       <c r="BH34" t="n">
         <v>38.94</v>
@@ -8335,7 +8335,7 @@
         <v>0</v>
       </c>
       <c r="BJ34" t="n">
-        <v>15.52</v>
+        <v>17.15</v>
       </c>
       <c r="BK34" t="n">
         <v>1.57</v>
@@ -8344,7 +8344,7 @@
         <v>1.58</v>
       </c>
       <c r="BM34" t="n">
-        <v>16.22</v>
+        <v>17.19</v>
       </c>
       <c r="BN34" t="n">
         <v>28.86</v>
@@ -8353,19 +8353,19 @@
         <v>14.3</v>
       </c>
       <c r="BP34" t="n">
-        <v>15.44</v>
+        <v>15.4</v>
       </c>
       <c r="BQ34" t="n">
-        <v>9.84</v>
+        <v>10.87</v>
       </c>
       <c r="BR34" t="n">
-        <v>16.2</v>
+        <v>15.52</v>
       </c>
       <c r="BS34" t="n">
         <v>0.32</v>
       </c>
       <c r="BT34" t="n">
-        <v>3344313</v>
+        <v>3354970</v>
       </c>
     </row>
     <row r="35">
@@ -8395,13 +8395,13 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>17.66</v>
+        <v>17.9</v>
       </c>
       <c r="G35" t="n">
-        <v>89121189229</v>
+        <v>90332348074</v>
       </c>
       <c r="H35" t="n">
-        <v>46623800</v>
+        <v>56307100</v>
       </c>
       <c r="I35" t="n">
         <v>5046500000</v>
@@ -8416,7 +8416,7 @@
         <v>4.69</v>
       </c>
       <c r="M35" t="n">
-        <v>7.398873520896959</v>
+        <v>7.499424368404665</v>
       </c>
       <c r="N35" t="n">
         <v>1.79</v>
@@ -8494,7 +8494,7 @@
         <v>5349290000</v>
       </c>
       <c r="AM35" t="n">
-        <v>7365387539.586777</v>
+        <v>7465483311.900826</v>
       </c>
       <c r="AN35" t="n">
         <v>0.5305</v>
@@ -8535,7 +8535,7 @@
         <v>7.68</v>
       </c>
       <c r="AZ35" t="n">
-        <v>10.3</v>
+        <v>10.44</v>
       </c>
       <c r="BA35" t="n">
         <v>1.11</v>
@@ -8544,19 +8544,19 @@
         <v>9.119999999999999</v>
       </c>
       <c r="BC35" t="n">
-        <v>-46.74</v>
+        <v>-47.45</v>
       </c>
       <c r="BD35" t="n">
-        <v>-56.51</v>
+        <v>-57.09</v>
       </c>
       <c r="BE35" t="n">
         <v>-41.67</v>
       </c>
       <c r="BF35" t="n">
-        <v>-93.69</v>
+        <v>-93.78</v>
       </c>
       <c r="BG35" t="n">
-        <v>-48.38</v>
+        <v>-49.07</v>
       </c>
       <c r="BH35" t="n">
         <v>3.71</v>
@@ -8565,7 +8565,7 @@
         <v>0</v>
       </c>
       <c r="BJ35" t="n">
-        <v>17.66</v>
+        <v>17.9</v>
       </c>
       <c r="BK35" t="n">
         <v>1.06</v>
@@ -8574,7 +8574,7 @@
         <v>1.04</v>
       </c>
       <c r="BM35" t="n">
-        <v>17.98</v>
+        <v>18.05</v>
       </c>
       <c r="BN35" t="n">
         <v>19.88</v>
@@ -8583,19 +8583,19 @@
         <v>11.58</v>
       </c>
       <c r="BP35" t="n">
-        <v>17.62</v>
+        <v>17.53</v>
       </c>
       <c r="BQ35" t="n">
-        <v>16.9</v>
+        <v>17.13</v>
       </c>
       <c r="BR35" t="n">
-        <v>17.73</v>
+        <v>17.69</v>
       </c>
       <c r="BS35" t="n">
         <v>7.3</v>
       </c>
       <c r="BT35" t="n">
-        <v>39479047</v>
+        <v>39461233</v>
       </c>
     </row>
     <row r="36">
@@ -8625,13 +8625,13 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="G36" t="n">
-        <v>195746593</v>
+        <v>197807652</v>
       </c>
       <c r="H36" t="n">
-        <v>100</v>
+        <v>4600</v>
       </c>
       <c r="I36" t="n">
         <v>4900000</v>
@@ -8646,7 +8646,7 @@
         <v>1.52</v>
       </c>
       <c r="M36" t="n">
-        <v>1.905757977612863</v>
+        <v>1.925824123191094</v>
       </c>
       <c r="N36" t="n">
         <v>0.87</v>
@@ -8724,7 +8724,7 @@
         <v>11319000</v>
       </c>
       <c r="AM36" t="n">
-        <v>26962340.63360882</v>
+        <v>27246233.05785124</v>
       </c>
       <c r="AN36" t="n">
         <v>0</v>
@@ -8765,7 +8765,7 @@
         <v>24.36</v>
       </c>
       <c r="AZ36" t="n">
-        <v>66.65000000000001</v>
+        <v>56.39</v>
       </c>
       <c r="BA36" t="n">
         <v>2.44</v>
@@ -8774,19 +8774,19 @@
         <v>14.49</v>
       </c>
       <c r="BC36" t="n">
-        <v>14.76</v>
+        <v>35.63</v>
       </c>
       <c r="BD36" t="n">
-        <v>-6.3</v>
+        <v>10.74</v>
       </c>
       <c r="BE36" t="n">
         <v>156.33</v>
       </c>
       <c r="BF36" t="n">
-        <v>-90.59999999999999</v>
+        <v>-88.89</v>
       </c>
       <c r="BG36" t="n">
-        <v>-44.28</v>
+        <v>-34.15</v>
       </c>
       <c r="BH36" t="n">
         <v>17.13</v>
@@ -8795,7 +8795,7 @@
         <v>0</v>
       </c>
       <c r="BJ36" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="BK36" t="n">
         <v>2.31</v>
@@ -8804,7 +8804,7 @@
         <v>2.31</v>
       </c>
       <c r="BM36" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="BN36" t="n">
         <v>29.05</v>
@@ -8813,19 +8813,19 @@
         <v>17.14</v>
       </c>
       <c r="BP36" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="BQ36" t="n">
-        <v>11.25</v>
+        <v>9.52</v>
       </c>
       <c r="BR36" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="BS36" t="n">
         <v>1.24</v>
       </c>
       <c r="BT36" t="n">
-        <v>143</v>
+        <v>147</v>
       </c>
     </row>
     <row r="37">
@@ -8855,13 +8855,13 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>14.62</v>
+        <v>14.47</v>
       </c>
       <c r="G37" t="n">
-        <v>195746593</v>
+        <v>197807652</v>
       </c>
       <c r="H37" t="n">
-        <v>300</v>
+        <v>12000</v>
       </c>
       <c r="I37" t="n">
         <v>4900000</v>
@@ -8876,7 +8876,7 @@
         <v>0.88</v>
       </c>
       <c r="M37" t="n">
-        <v>1.905757977612863</v>
+        <v>1.925824123191094</v>
       </c>
       <c r="N37" t="n">
         <v>0.5</v>
@@ -8954,7 +8954,7 @@
         <v>11319000</v>
       </c>
       <c r="AM37" t="n">
-        <v>46829328.46889953</v>
+        <v>47322404.784689</v>
       </c>
       <c r="AN37" t="n">
         <v>0</v>
@@ -8995,7 +8995,7 @@
         <v>24.36</v>
       </c>
       <c r="AZ37" t="n">
-        <v>65.01000000000001</v>
+        <v>64.34</v>
       </c>
       <c r="BA37" t="n">
         <v>2.44</v>
@@ -9004,19 +9004,19 @@
         <v>15.53</v>
       </c>
       <c r="BC37" t="n">
-        <v>104.09</v>
+        <v>106.21</v>
       </c>
       <c r="BD37" t="n">
-        <v>66.64</v>
+        <v>68.37</v>
       </c>
       <c r="BE37" t="n">
         <v>344.67</v>
       </c>
       <c r="BF37" t="n">
-        <v>-83.28</v>
+        <v>-83.09999999999999</v>
       </c>
       <c r="BG37" t="n">
-        <v>6.25</v>
+        <v>7.35</v>
       </c>
       <c r="BH37" t="n">
         <v>17.13</v>
@@ -9025,7 +9025,7 @@
         <v>0</v>
       </c>
       <c r="BJ37" t="n">
-        <v>14.62</v>
+        <v>14.47</v>
       </c>
       <c r="BK37" t="n">
         <v>2.31</v>
@@ -9034,28 +9034,28 @@
         <v>2.31</v>
       </c>
       <c r="BM37" t="n">
-        <v>14.62</v>
+        <v>14.51</v>
       </c>
       <c r="BN37" t="n">
         <v>20.9</v>
       </c>
       <c r="BO37" t="n">
-        <v>13.2</v>
+        <v>13.42</v>
       </c>
       <c r="BP37" t="n">
-        <v>14.56</v>
+        <v>14.2</v>
       </c>
       <c r="BQ37" t="n">
-        <v>6.32</v>
+        <v>6.26</v>
       </c>
       <c r="BR37" t="n">
-        <v>14.56</v>
+        <v>14.51</v>
       </c>
       <c r="BS37" t="n">
         <v>0.72</v>
       </c>
       <c r="BT37" t="n">
-        <v>860</v>
+        <v>870</v>
       </c>
     </row>
     <row r="38">
@@ -9315,13 +9315,13 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>68.95</v>
+        <v>68.53</v>
       </c>
       <c r="G39" t="n">
-        <v>3865220303</v>
+        <v>3841675915</v>
       </c>
       <c r="H39" t="n">
-        <v>2400</v>
+        <v>700</v>
       </c>
       <c r="I39" t="n">
         <v>168174945</v>
@@ -9336,7 +9336,7 @@
         <v>0.53</v>
       </c>
       <c r="M39" t="n">
-        <v>0.1940171049441625</v>
+        <v>0.1928352799408383</v>
       </c>
       <c r="N39" t="n">
         <v>0.06</v>
@@ -9414,7 +9414,7 @@
         <v>2536078170.6</v>
       </c>
       <c r="AM39" t="n">
-        <v>406010536.0294118</v>
+        <v>403537386.0294118</v>
       </c>
       <c r="AN39" t="n">
         <v>11.9435</v>
@@ -9455,7 +9455,7 @@
         <v>170.24</v>
       </c>
       <c r="AZ39" t="n">
-        <v>201.45</v>
+        <v>200.22</v>
       </c>
       <c r="BA39" t="n">
         <v>19.01</v>
@@ -9464,19 +9464,19 @@
         <v>91.72</v>
       </c>
       <c r="BC39" t="n">
-        <v>202.4</v>
+        <v>204.25</v>
       </c>
       <c r="BD39" t="n">
-        <v>146.91</v>
+        <v>148.42</v>
       </c>
       <c r="BE39" t="n">
         <v>192.17</v>
       </c>
       <c r="BF39" t="n">
-        <v>-72.43000000000001</v>
+        <v>-72.26000000000001</v>
       </c>
       <c r="BG39" t="n">
-        <v>33.03</v>
+        <v>33.84</v>
       </c>
       <c r="BH39" t="n">
         <v>128.13</v>
@@ -9485,7 +9485,7 @@
         <v>0</v>
       </c>
       <c r="BJ39" t="n">
-        <v>68.95</v>
+        <v>68.53</v>
       </c>
       <c r="BK39" t="n">
         <v>15.08</v>
@@ -9494,7 +9494,7 @@
         <v>15.08</v>
       </c>
       <c r="BM39" t="n">
-        <v>68.95</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="BN39" t="n">
         <v>74.56</v>
@@ -9503,19 +9503,19 @@
         <v>54.98</v>
       </c>
       <c r="BP39" t="n">
-        <v>68.83</v>
+        <v>68.33</v>
       </c>
       <c r="BQ39" t="n">
-        <v>4.57</v>
+        <v>4.54</v>
       </c>
       <c r="BR39" t="n">
-        <v>68.95</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="BS39" t="n">
         <v>0.58</v>
       </c>
       <c r="BT39" t="n">
-        <v>3140</v>
+        <v>3183</v>
       </c>
     </row>
     <row r="40">
@@ -9545,13 +9545,13 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>21.49</v>
+        <v>22.04</v>
       </c>
       <c r="G40" t="n">
-        <v>123155599858</v>
+        <v>126307542526</v>
       </c>
       <c r="H40" t="n">
-        <v>44554600</v>
+        <v>37276500</v>
       </c>
       <c r="I40" t="n">
         <v>5730834040</v>
@@ -9566,7 +9566,7 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="M40" t="n">
-        <v>0.373669331192852</v>
+        <v>0.3832327153188501</v>
       </c>
       <c r="N40" t="n">
         <v>0.05</v>
@@ -9644,7 +9644,7 @@
         <v>15358635227.2</v>
       </c>
       <c r="AM40" t="n">
-        <v>6387738581.846473</v>
+        <v>6551221085.373444</v>
       </c>
       <c r="AN40" t="n">
         <v>0.5641</v>
@@ -9685,7 +9685,7 @@
         <v>36.13</v>
       </c>
       <c r="AZ40" t="n">
-        <v>10.85</v>
+        <v>11.13</v>
       </c>
       <c r="BA40" t="n">
         <v>2.76</v>
@@ -9694,19 +9694,19 @@
         <v>27.89</v>
       </c>
       <c r="BC40" t="n">
-        <v>105.9</v>
+        <v>100.77</v>
       </c>
       <c r="BD40" t="n">
-        <v>68.12</v>
+        <v>63.92</v>
       </c>
       <c r="BE40" t="n">
         <v>-49.5</v>
       </c>
       <c r="BF40" t="n">
-        <v>-87.16</v>
+        <v>-87.48</v>
       </c>
       <c r="BG40" t="n">
-        <v>29.78</v>
+        <v>26.54</v>
       </c>
       <c r="BH40" t="n">
         <v>32.47</v>
@@ -9715,7 +9715,7 @@
         <v>0</v>
       </c>
       <c r="BJ40" t="n">
-        <v>21.49</v>
+        <v>22.04</v>
       </c>
       <c r="BK40" t="n">
         <v>2.68</v>
@@ -9724,7 +9724,7 @@
         <v>2.5</v>
       </c>
       <c r="BM40" t="n">
-        <v>21.81</v>
+        <v>22.18</v>
       </c>
       <c r="BN40" t="n">
         <v>27.36</v>
@@ -9733,19 +9733,19 @@
         <v>17.67</v>
       </c>
       <c r="BP40" t="n">
-        <v>21.18</v>
+        <v>21.34</v>
       </c>
       <c r="BQ40" t="n">
-        <v>8.6</v>
+        <v>8.82</v>
       </c>
       <c r="BR40" t="n">
-        <v>21.39</v>
+        <v>21.47</v>
       </c>
       <c r="BS40" t="n">
         <v>0.39</v>
       </c>
       <c r="BT40" t="n">
-        <v>37020600</v>
+        <v>37052397</v>
       </c>
     </row>
     <row r="41">
@@ -9775,13 +9775,13 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>15.61</v>
+        <v>15.65</v>
       </c>
       <c r="G41" t="n">
-        <v>186051806992</v>
+        <v>187508242841</v>
       </c>
       <c r="H41" t="n">
-        <v>6952700</v>
+        <v>8434600</v>
       </c>
       <c r="I41" t="n">
         <v>5303870781</v>
@@ -9796,7 +9796,7 @@
         <v>0.92</v>
       </c>
       <c r="M41" t="n">
-        <v>1.23984337321933</v>
+        <v>1.249549015777154</v>
       </c>
       <c r="N41" t="n">
         <v>0.07000000000000001</v>
@@ -9874,7 +9874,7 @@
         <v>12304980211.92</v>
       </c>
       <c r="AM41" t="n">
-        <v>28667458704.46841</v>
+        <v>28891871007.85824</v>
       </c>
       <c r="AN41" t="n">
         <v>1.6841</v>
@@ -9915,7 +9915,7 @@
         <v>24.4</v>
       </c>
       <c r="AZ41" t="n">
-        <v>23.36</v>
+        <v>23.42</v>
       </c>
       <c r="BA41" t="n">
         <v>2.53</v>
@@ -9924,19 +9924,19 @@
         <v>13.77</v>
       </c>
       <c r="BC41" t="n">
-        <v>91.45</v>
+        <v>90.95999999999999</v>
       </c>
       <c r="BD41" t="n">
-        <v>56.32</v>
+        <v>55.92</v>
       </c>
       <c r="BE41" t="n">
         <v>49.67</v>
       </c>
       <c r="BF41" t="n">
-        <v>-83.81</v>
+        <v>-83.84999999999999</v>
       </c>
       <c r="BG41" t="n">
-        <v>-11.79</v>
+        <v>-12.01</v>
       </c>
       <c r="BH41" t="n">
         <v>17.11</v>
@@ -9945,7 +9945,7 @@
         <v>0</v>
       </c>
       <c r="BJ41" t="n">
-        <v>15.61</v>
+        <v>15.65</v>
       </c>
       <c r="BK41" t="n">
         <v>2.32</v>
@@ -9954,7 +9954,7 @@
         <v>2.34</v>
       </c>
       <c r="BM41" t="n">
-        <v>15.78</v>
+        <v>15.67</v>
       </c>
       <c r="BN41" t="n">
         <v>18.28</v>
@@ -9963,19 +9963,19 @@
         <v>13.43</v>
       </c>
       <c r="BP41" t="n">
-        <v>15.46</v>
+        <v>15.45</v>
       </c>
       <c r="BQ41" t="n">
-        <v>6.68</v>
+        <v>6.7</v>
       </c>
       <c r="BR41" t="n">
-        <v>15.64</v>
+        <v>15.61</v>
       </c>
       <c r="BS41" t="n">
         <v>0.5600000000000001</v>
       </c>
       <c r="BT41" t="n">
-        <v>7215510</v>
+        <v>7209050</v>
       </c>
     </row>
     <row r="42">
@@ -10005,13 +10005,13 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>17.66</v>
+        <v>17.78</v>
       </c>
       <c r="G42" t="n">
-        <v>186051806992</v>
+        <v>187508242841</v>
       </c>
       <c r="H42" t="n">
-        <v>28163100</v>
+        <v>41812200</v>
       </c>
       <c r="I42" t="n">
         <v>5288141247</v>
@@ -10026,7 +10026,7 @@
         <v>1.05</v>
       </c>
       <c r="M42" t="n">
-        <v>1.243531277453127</v>
+        <v>1.253265789367399</v>
       </c>
       <c r="N42" t="n">
         <v>0.08</v>
@@ -10104,7 +10104,7 @@
         <v>12268487693.04</v>
       </c>
       <c r="AM42" t="n">
-        <v>25313171019.31973</v>
+        <v>25511325556.59864</v>
       </c>
       <c r="AN42" t="n">
         <v>1.8491</v>
@@ -10145,7 +10145,7 @@
         <v>24.4</v>
       </c>
       <c r="AZ42" t="n">
-        <v>25.58</v>
+        <v>25.75</v>
       </c>
       <c r="BA42" t="n">
         <v>2.53</v>
@@ -10154,19 +10154,19 @@
         <v>15.11</v>
       </c>
       <c r="BC42" t="n">
-        <v>69.23</v>
+        <v>68.08</v>
       </c>
       <c r="BD42" t="n">
-        <v>38.17</v>
+        <v>37.24</v>
       </c>
       <c r="BE42" t="n">
         <v>44.83</v>
       </c>
       <c r="BF42" t="n">
-        <v>-85.69</v>
+        <v>-85.79000000000001</v>
       </c>
       <c r="BG42" t="n">
-        <v>-14.41</v>
+        <v>-14.99</v>
       </c>
       <c r="BH42" t="n">
         <v>17.11</v>
@@ -10175,7 +10175,7 @@
         <v>0</v>
       </c>
       <c r="BJ42" t="n">
-        <v>17.66</v>
+        <v>17.78</v>
       </c>
       <c r="BK42" t="n">
         <v>2.32</v>
@@ -10184,7 +10184,7 @@
         <v>2.34</v>
       </c>
       <c r="BM42" t="n">
-        <v>17.88</v>
+        <v>17.78</v>
       </c>
       <c r="BN42" t="n">
         <v>21.33</v>
@@ -10193,19 +10193,19 @@
         <v>15.67</v>
       </c>
       <c r="BP42" t="n">
-        <v>17.54</v>
+        <v>17.49</v>
       </c>
       <c r="BQ42" t="n">
-        <v>7.56</v>
+        <v>7.61</v>
       </c>
       <c r="BR42" t="n">
-        <v>17.82</v>
+        <v>17.63</v>
       </c>
       <c r="BS42" t="n">
         <v>0.63</v>
       </c>
       <c r="BT42" t="n">
-        <v>40407127</v>
+        <v>39949597</v>
       </c>
     </row>
     <row r="43">
@@ -10235,13 +10235,13 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>38.38</v>
+        <v>38.76</v>
       </c>
       <c r="G43" t="n">
-        <v>74510934073</v>
+        <v>75248621981</v>
       </c>
       <c r="H43" t="n">
-        <v>6348300</v>
+        <v>4567700</v>
       </c>
       <c r="I43" t="n">
         <v>1941400000</v>
@@ -10334,7 +10334,7 @@
         <v>9182822000</v>
       </c>
       <c r="AM43" t="n">
-        <v>9075631433.982946</v>
+        <v>9165483797.929354</v>
       </c>
       <c r="AN43" t="n">
         <v>4.5901</v>
@@ -10375,7 +10375,7 @@
         <v>19.95</v>
       </c>
       <c r="AZ43" t="n">
-        <v>69.66</v>
+        <v>70.34999999999999</v>
       </c>
       <c r="BA43" t="n">
         <v>5.63</v>
@@ -10384,19 +10384,19 @@
         <v>48.62</v>
       </c>
       <c r="BC43" t="n">
-        <v>-36.34</v>
+        <v>-36.96</v>
       </c>
       <c r="BD43" t="n">
-        <v>-48.02</v>
+        <v>-48.53</v>
       </c>
       <c r="BE43" t="n">
         <v>81.5</v>
       </c>
       <c r="BF43" t="n">
-        <v>-85.33</v>
+        <v>-85.48</v>
       </c>
       <c r="BG43" t="n">
-        <v>26.67</v>
+        <v>25.43</v>
       </c>
       <c r="BH43" t="n">
         <v>5.61</v>
@@ -10405,7 +10405,7 @@
         <v>0</v>
       </c>
       <c r="BJ43" t="n">
-        <v>38.38</v>
+        <v>38.76</v>
       </c>
       <c r="BK43" t="n">
         <v>4.73</v>
@@ -10414,7 +10414,7 @@
         <v>4.73</v>
       </c>
       <c r="BM43" t="n">
-        <v>38.96</v>
+        <v>38.97</v>
       </c>
       <c r="BN43" t="n">
         <v>42.98</v>
@@ -10423,19 +10423,19 @@
         <v>28.06</v>
       </c>
       <c r="BP43" t="n">
-        <v>38.36</v>
+        <v>38.24</v>
       </c>
       <c r="BQ43" t="n">
-        <v>8.109999999999999</v>
+        <v>8.19</v>
       </c>
       <c r="BR43" t="n">
-        <v>38.81</v>
+        <v>38.44</v>
       </c>
       <c r="BS43" t="n">
         <v>0</v>
       </c>
       <c r="BT43" t="n">
-        <v>6287600</v>
+        <v>6273510</v>
       </c>
     </row>
     <row r="44">
@@ -10925,13 +10925,13 @@
         </is>
       </c>
       <c r="F46" t="n">
-        <v>4.01</v>
+        <v>3.92</v>
       </c>
       <c r="G46" t="n">
-        <v>4012173649</v>
+        <v>3922124716</v>
       </c>
       <c r="H46" t="n">
-        <v>22181100</v>
+        <v>15110100</v>
       </c>
       <c r="I46" t="n">
         <v>1000542188</v>
@@ -10946,7 +10946,7 @@
         <v>2.5</v>
       </c>
       <c r="M46" t="n">
-        <v>0.06973912131138138</v>
+        <v>0.0681739015547508</v>
       </c>
       <c r="N46" t="n">
         <v>0.08</v>
@@ -11024,7 +11024,7 @@
         <v>460249406.48</v>
       </c>
       <c r="AM46" t="n">
-        <v>3933503577.45098</v>
+        <v>3845220309.803922</v>
       </c>
       <c r="AN46" t="n">
         <v>0.0311</v>
@@ -11065,7 +11065,7 @@
         <v>3.3</v>
       </c>
       <c r="AZ46" t="n">
-        <v>3.31</v>
+        <v>3.23</v>
       </c>
       <c r="BA46" t="n">
         <v>0.42</v>
@@ -11074,19 +11074,19 @@
         <v>7.38</v>
       </c>
       <c r="BC46" t="n">
-        <v>0.84</v>
+        <v>3.16</v>
       </c>
       <c r="BD46" t="n">
-        <v>-17.66</v>
+        <v>-15.77</v>
       </c>
       <c r="BE46" t="n">
         <v>-17.5</v>
       </c>
       <c r="BF46" t="n">
-        <v>-89.45</v>
+        <v>-89.20999999999999</v>
       </c>
       <c r="BG46" t="n">
-        <v>84.01000000000001</v>
+        <v>88.23</v>
       </c>
       <c r="BH46" t="n">
         <v>1.58</v>
@@ -11095,7 +11095,7 @@
         <v>0</v>
       </c>
       <c r="BJ46" t="n">
-        <v>4.01</v>
+        <v>3.92</v>
       </c>
       <c r="BK46" t="n">
         <v>0.46</v>
@@ -11104,7 +11104,7 @@
         <v>0.46</v>
       </c>
       <c r="BM46" t="n">
-        <v>4.17</v>
+        <v>4.02</v>
       </c>
       <c r="BN46" t="n">
         <v>7.31</v>
@@ -11113,19 +11113,19 @@
         <v>2.97</v>
       </c>
       <c r="BP46" t="n">
-        <v>3.99</v>
+        <v>3.9</v>
       </c>
       <c r="BQ46" t="n">
-        <v>8.77</v>
+        <v>8.57</v>
       </c>
       <c r="BR46" t="n">
-        <v>4.07</v>
+        <v>4.02</v>
       </c>
       <c r="BS46" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="BT46" t="n">
-        <v>22561601</v>
+        <v>22182524</v>
       </c>
     </row>
     <row r="47">
@@ -11155,13 +11155,13 @@
         </is>
       </c>
       <c r="F47" t="n">
-        <v>8.960000000000001</v>
+        <v>9.06</v>
       </c>
       <c r="G47" t="n">
-        <v>3126712973</v>
+        <v>3161609456</v>
       </c>
       <c r="H47" t="n">
-        <v>7600</v>
+        <v>4500</v>
       </c>
       <c r="I47" t="n">
         <v>254106600</v>
@@ -11176,7 +11176,7 @@
         <v>1.22</v>
       </c>
       <c r="M47" t="n">
-        <v>0.7373148926793331</v>
+        <v>0.7455438848638457</v>
       </c>
       <c r="N47" t="n">
         <v>0.07000000000000001</v>
@@ -11254,7 +11254,7 @@
         <v>322715382</v>
       </c>
       <c r="AM47" t="n">
-        <v>554381732.8014184</v>
+        <v>560569052.4822695</v>
       </c>
       <c r="AN47" t="n">
         <v>0.4132</v>
@@ -11295,7 +11295,7 @@
         <v>11.74</v>
       </c>
       <c r="AZ47" t="n">
-        <v>11.77</v>
+        <v>11.9</v>
       </c>
       <c r="BA47" t="n">
         <v>1.46</v>
@@ -11304,19 +11304,19 @@
         <v>8.619999999999999</v>
       </c>
       <c r="BC47" t="n">
-        <v>60.42</v>
+        <v>58.65</v>
       </c>
       <c r="BD47" t="n">
-        <v>30.98</v>
+        <v>29.54</v>
       </c>
       <c r="BE47" t="n">
         <v>31.33</v>
       </c>
       <c r="BF47" t="n">
-        <v>-83.72</v>
+        <v>-83.90000000000001</v>
       </c>
       <c r="BG47" t="n">
-        <v>-3.8</v>
+        <v>-4.86</v>
       </c>
       <c r="BH47" t="n">
         <v>7.23</v>
@@ -11325,16 +11325,16 @@
         <v>0</v>
       </c>
       <c r="BJ47" t="n">
-        <v>8.960000000000001</v>
+        <v>9.06</v>
       </c>
       <c r="BK47" t="n">
         <v>1.27</v>
       </c>
       <c r="BL47" t="n">
-        <v>1.29</v>
+        <v>1.28</v>
       </c>
       <c r="BM47" t="n">
-        <v>9.050000000000001</v>
+        <v>9.07</v>
       </c>
       <c r="BN47" t="n">
         <v>9.24</v>
@@ -11343,19 +11343,19 @@
         <v>7.19</v>
       </c>
       <c r="BP47" t="n">
-        <v>8.82</v>
+        <v>8.94</v>
       </c>
       <c r="BQ47" t="n">
-        <v>6.93</v>
+        <v>7.06</v>
       </c>
       <c r="BR47" t="n">
-        <v>9.029999999999999</v>
+        <v>8.94</v>
       </c>
       <c r="BS47" t="n">
         <v>0.53</v>
       </c>
       <c r="BT47" t="n">
-        <v>10443</v>
+        <v>10267</v>
       </c>
     </row>
     <row r="48">
@@ -11385,13 +11385,13 @@
         </is>
       </c>
       <c r="F48" t="n">
-        <v>9.1</v>
+        <v>9.130000000000001</v>
       </c>
       <c r="G48" t="n">
-        <v>3126712973</v>
+        <v>3161609456</v>
       </c>
       <c r="H48" t="n">
-        <v>1700</v>
+        <v>1400</v>
       </c>
       <c r="I48" t="n">
         <v>93397546</v>
@@ -11406,7 +11406,7 @@
         <v>1.24</v>
       </c>
       <c r="M48" t="n">
-        <v>2.006011812217317</v>
+        <v>2.028400422143247</v>
       </c>
       <c r="N48" t="n">
         <v>0.07000000000000001</v>
@@ -11484,7 +11484,7 @@
         <v>118614883.42</v>
       </c>
       <c r="AM48" t="n">
-        <v>546628142.1328671</v>
+        <v>552728925.874126</v>
       </c>
       <c r="AN48" t="n">
         <v>0.4132</v>
@@ -11525,7 +11525,7 @@
         <v>11.74</v>
       </c>
       <c r="AZ48" t="n">
-        <v>11.91</v>
+        <v>11.95</v>
       </c>
       <c r="BA48" t="n">
         <v>1.46</v>
@@ -11534,19 +11534,19 @@
         <v>8.24</v>
       </c>
       <c r="BC48" t="n">
-        <v>57.95</v>
+        <v>57.43</v>
       </c>
       <c r="BD48" t="n">
-        <v>28.97</v>
+        <v>28.54</v>
       </c>
       <c r="BE48" t="n">
         <v>30.83</v>
       </c>
       <c r="BF48" t="n">
-        <v>-83.97</v>
+        <v>-84.03</v>
       </c>
       <c r="BG48" t="n">
-        <v>-9.49</v>
+        <v>-9.789999999999999</v>
       </c>
       <c r="BH48" t="n">
         <v>7.23</v>
@@ -11555,16 +11555,16 @@
         <v>0</v>
       </c>
       <c r="BJ48" t="n">
-        <v>9.1</v>
+        <v>9.130000000000001</v>
       </c>
       <c r="BK48" t="n">
         <v>1.27</v>
       </c>
       <c r="BL48" t="n">
-        <v>1.29</v>
+        <v>1.28</v>
       </c>
       <c r="BM48" t="n">
-        <v>9.199999999999999</v>
+        <v>9.16</v>
       </c>
       <c r="BN48" t="n">
         <v>9.48</v>
@@ -11576,7 +11576,7 @@
         <v>9.1</v>
       </c>
       <c r="BQ48" t="n">
-        <v>7.04</v>
+        <v>7.12</v>
       </c>
       <c r="BR48" t="n">
         <v>9.109999999999999</v>
@@ -11585,7 +11585,7 @@
         <v>0.54</v>
       </c>
       <c r="BT48" t="n">
-        <v>2643</v>
+        <v>2647</v>
       </c>
     </row>
     <row r="49">
@@ -11845,13 +11845,13 @@
         </is>
       </c>
       <c r="F50" t="n">
-        <v>33.77</v>
+        <v>34.25</v>
       </c>
       <c r="G50" t="n">
-        <v>953506700</v>
+        <v>952468000</v>
       </c>
       <c r="H50" t="n">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="I50" t="n">
         <v>11540870</v>
@@ -11866,7 +11866,7 @@
         <v>0.8</v>
       </c>
       <c r="M50" t="n">
-        <v>0.9646504295601004</v>
+        <v>0.9635995901677982</v>
       </c>
       <c r="N50" t="n">
         <v>0.06</v>
@@ -11944,7 +11944,7 @@
         <v>84709985.8</v>
       </c>
       <c r="AM50" t="n">
-        <v>325428907.8498293</v>
+        <v>325074402.7303754</v>
       </c>
       <c r="AN50" t="n">
         <v>4.4983</v>
@@ -11985,7 +11985,7 @@
         <v>68.48999999999999</v>
       </c>
       <c r="AZ50" t="n">
-        <v>74.45999999999999</v>
+        <v>75.52</v>
       </c>
       <c r="BA50" t="n">
         <v>9.210000000000001</v>
@@ -11994,19 +11994,19 @@
         <v>30.53</v>
       </c>
       <c r="BC50" t="n">
-        <v>148.38</v>
+        <v>144.9</v>
       </c>
       <c r="BD50" t="n">
-        <v>102.8</v>
+        <v>99.95999999999999</v>
       </c>
       <c r="BE50" t="n">
         <v>120.5</v>
       </c>
       <c r="BF50" t="n">
-        <v>-72.72</v>
+        <v>-73.09999999999999</v>
       </c>
       <c r="BG50" t="n">
-        <v>-9.59</v>
+        <v>-10.86</v>
       </c>
       <c r="BH50" t="n">
         <v>42.6</v>
@@ -12015,7 +12015,7 @@
         <v>0</v>
       </c>
       <c r="BJ50" t="n">
-        <v>33.77</v>
+        <v>34.25</v>
       </c>
       <c r="BK50" t="n">
         <v>7.34</v>
@@ -12024,7 +12024,7 @@
         <v>7.6</v>
       </c>
       <c r="BM50" t="n">
-        <v>34.27</v>
+        <v>34.3</v>
       </c>
       <c r="BN50" t="n">
         <v>39.22</v>
@@ -12033,19 +12033,19 @@
         <v>23.5</v>
       </c>
       <c r="BP50" t="n">
-        <v>33.58</v>
+        <v>34.25</v>
       </c>
       <c r="BQ50" t="n">
-        <v>4.44</v>
+        <v>4.51</v>
       </c>
       <c r="BR50" t="n">
-        <v>33.58</v>
+        <v>34.26</v>
       </c>
       <c r="BS50" t="n">
         <v>0.4</v>
       </c>
       <c r="BT50" t="n">
-        <v>547</v>
+        <v>503</v>
       </c>
     </row>
     <row r="51">
@@ -12523,13 +12523,13 @@
         </is>
       </c>
       <c r="F53" t="n">
-        <v>5.98</v>
+        <v>5.88</v>
       </c>
       <c r="G53" t="n">
-        <v>818377354</v>
+        <v>804692127</v>
       </c>
       <c r="H53" t="n">
-        <v>127700</v>
+        <v>39600</v>
       </c>
       <c r="I53" t="n">
         <v>136852484</v>
@@ -12544,7 +12544,7 @@
         <v>2.79</v>
       </c>
       <c r="M53" t="n">
-        <v>2.125991803710185</v>
+        <v>2.090440135165465</v>
       </c>
       <c r="N53" t="n">
         <v>1.48</v>
@@ -12622,7 +12622,7 @@
         <v>39687220.36</v>
       </c>
       <c r="AM53" t="n">
-        <v>41690135.20122262</v>
+        <v>40992976.41365258</v>
       </c>
       <c r="AN53" t="n">
         <v>0</v>
@@ -12672,16 +12672,16 @@
         <v>0</v>
       </c>
       <c r="BC53" t="n">
-        <v>-34.1</v>
+        <v>-32.98</v>
       </c>
       <c r="BD53" t="n">
-        <v>-46.19</v>
+        <v>-45.28</v>
       </c>
       <c r="BE53" t="n">
         <v>-100</v>
       </c>
       <c r="BF53" t="n">
-        <v>-95.15000000000001</v>
+        <v>-95.06999999999999</v>
       </c>
       <c r="BG53" t="n">
         <v>-100</v>
@@ -12693,7 +12693,7 @@
         <v>0</v>
       </c>
       <c r="BJ53" t="n">
-        <v>5.98</v>
+        <v>5.88</v>
       </c>
       <c r="BK53" t="n">
         <v>0.29</v>
@@ -12702,7 +12702,7 @@
         <v>0.2</v>
       </c>
       <c r="BM53" t="n">
-        <v>6.29</v>
+        <v>6.3</v>
       </c>
       <c r="BN53" t="n">
         <v>10.39</v>
@@ -12711,19 +12711,19 @@
         <v>4.82</v>
       </c>
       <c r="BP53" t="n">
-        <v>5.71</v>
+        <v>5.77</v>
       </c>
       <c r="BQ53" t="n">
-        <v>29.37</v>
+        <v>28.88</v>
       </c>
       <c r="BR53" t="n">
-        <v>5.94</v>
+        <v>6.04</v>
       </c>
       <c r="BS53" t="n">
         <v>2.36</v>
       </c>
       <c r="BT53" t="n">
-        <v>32643</v>
+        <v>35577</v>
       </c>
     </row>
     <row r="54">
@@ -12753,13 +12753,13 @@
         </is>
       </c>
       <c r="F54" t="n">
-        <v>10.29</v>
+        <v>10.51</v>
       </c>
       <c r="G54" t="n">
-        <v>2399752500</v>
+        <v>2451059224</v>
       </c>
       <c r="H54" t="n">
-        <v>162500</v>
+        <v>159400</v>
       </c>
       <c r="I54" t="n">
         <v>233212121</v>
@@ -12774,7 +12774,7 @@
         <v>0.97</v>
       </c>
       <c r="M54" t="n">
-        <v>1.346960873658878</v>
+        <v>1.375758905865789</v>
       </c>
       <c r="N54" t="n">
         <v>0.5600000000000001</v>
@@ -12852,7 +12852,7 @@
         <v>233212121</v>
       </c>
       <c r="AM54" t="n">
-        <v>328283515.7318742</v>
+        <v>335302219.4254446</v>
       </c>
       <c r="AN54" t="n">
         <v>0.1531</v>
@@ -12893,7 +12893,7 @@
         <v>12.25</v>
       </c>
       <c r="AZ54" t="n">
-        <v>16.38</v>
+        <v>16.73</v>
       </c>
       <c r="BA54" t="n">
         <v>0.98</v>
@@ -12902,28 +12902,28 @@
         <v>6.52</v>
       </c>
       <c r="BC54" t="n">
-        <v>45.85</v>
+        <v>42.79</v>
       </c>
       <c r="BD54" t="n">
-        <v>19.08</v>
+        <v>16.59</v>
       </c>
       <c r="BE54" t="n">
         <v>59.17</v>
       </c>
       <c r="BF54" t="n">
-        <v>-90.44</v>
+        <v>-90.64</v>
       </c>
       <c r="BG54" t="n">
-        <v>-36.67</v>
+        <v>-38</v>
       </c>
       <c r="BH54" t="n">
         <v>10.01</v>
       </c>
       <c r="BI54" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="BJ54" t="n">
-        <v>10.29</v>
+        <v>10.45</v>
       </c>
       <c r="BK54" t="n">
         <v>1</v>
@@ -12932,28 +12932,28 @@
         <v>1</v>
       </c>
       <c r="BM54" t="n">
-        <v>10.35</v>
+        <v>10.55</v>
       </c>
       <c r="BN54" t="n">
-        <v>11.75</v>
+        <v>11.66</v>
       </c>
       <c r="BO54" t="n">
-        <v>8.279999999999999</v>
+        <v>8.220000000000001</v>
       </c>
       <c r="BP54" t="n">
-        <v>10.12</v>
+        <v>10.13</v>
       </c>
       <c r="BQ54" t="n">
-        <v>10.26</v>
+        <v>10.48</v>
       </c>
       <c r="BR54" t="n">
-        <v>10.22</v>
+        <v>10.13</v>
       </c>
       <c r="BS54" t="n">
         <v>1.26</v>
       </c>
       <c r="BT54" t="n">
-        <v>246663</v>
+        <v>242710</v>
       </c>
     </row>
     <row r="55">
@@ -12983,13 +12983,13 @@
         </is>
       </c>
       <c r="F55" t="n">
-        <v>49.4</v>
+        <v>49.3</v>
       </c>
       <c r="G55" t="n">
-        <v>6564644884</v>
+        <v>6504739356</v>
       </c>
       <c r="H55" t="n">
-        <v>5000</v>
+        <v>1700</v>
       </c>
       <c r="I55" t="n">
         <v>84052790</v>
@@ -13004,7 +13004,7 @@
         <v>2</v>
       </c>
       <c r="M55" t="n">
-        <v>1.013391835319895</v>
+        <v>1.004144149567131</v>
       </c>
       <c r="N55" t="n">
         <v>0.16</v>
@@ -13082,7 +13082,7 @@
         <v>579123723.1</v>
       </c>
       <c r="AM55" t="n">
-        <v>330213525.3521127</v>
+        <v>327200168.8128773</v>
       </c>
       <c r="AN55" t="n">
         <v>3.1953</v>
@@ -13123,7 +13123,7 @@
         <v>51.21</v>
       </c>
       <c r="AZ55" t="n">
-        <v>51.95</v>
+        <v>51.85</v>
       </c>
       <c r="BA55" t="n">
         <v>9.380000000000001</v>
@@ -13132,19 +13132,19 @@
         <v>16.08</v>
       </c>
       <c r="BC55" t="n">
-        <v>26.95</v>
+        <v>27.21</v>
       </c>
       <c r="BD55" t="n">
-        <v>3.65</v>
+        <v>3.86</v>
       </c>
       <c r="BE55" t="n">
         <v>5.17</v>
       </c>
       <c r="BF55" t="n">
-        <v>-81.02</v>
+        <v>-80.98</v>
       </c>
       <c r="BG55" t="n">
-        <v>-67.45999999999999</v>
+        <v>-67.39</v>
       </c>
       <c r="BH55" t="n">
         <v>25.37</v>
@@ -13153,7 +13153,7 @@
         <v>0</v>
       </c>
       <c r="BJ55" t="n">
-        <v>49.4</v>
+        <v>49.3</v>
       </c>
       <c r="BK55" t="n">
         <v>6.89</v>
@@ -13162,7 +13162,7 @@
         <v>7.03</v>
       </c>
       <c r="BM55" t="n">
-        <v>49.97</v>
+        <v>49.76</v>
       </c>
       <c r="BN55" t="n">
         <v>73.67</v>
@@ -13171,19 +13171,19 @@
         <v>35.58</v>
       </c>
       <c r="BP55" t="n">
-        <v>49.4</v>
+        <v>49.12</v>
       </c>
       <c r="BQ55" t="n">
-        <v>7.03</v>
+        <v>7.01</v>
       </c>
       <c r="BR55" t="n">
-        <v>49.8</v>
+        <v>49.76</v>
       </c>
       <c r="BS55" t="n">
         <v>0.66</v>
       </c>
       <c r="BT55" t="n">
-        <v>6393</v>
+        <v>6143</v>
       </c>
     </row>
     <row r="56">
@@ -13213,13 +13213,13 @@
         </is>
       </c>
       <c r="F56" t="n">
-        <v>57.89</v>
+        <v>58.39</v>
       </c>
       <c r="G56" t="n">
-        <v>6564644884</v>
+        <v>6504739356</v>
       </c>
       <c r="H56" t="n">
-        <v>9700</v>
+        <v>15100</v>
       </c>
       <c r="I56" t="n">
         <v>39675836</v>
@@ -13234,7 +13234,7 @@
         <v>2.41</v>
       </c>
       <c r="M56" t="n">
-        <v>2.146858635111249</v>
+        <v>2.127267522057875</v>
       </c>
       <c r="N56" t="n">
         <v>0.19</v>
@@ -13312,7 +13312,7 @@
         <v>273366510.04</v>
       </c>
       <c r="AM56" t="n">
-        <v>273071750.5823627</v>
+        <v>270579840.0998336</v>
       </c>
       <c r="AN56" t="n">
         <v>3.5102</v>
@@ -13353,7 +13353,7 @@
         <v>51.21</v>
       </c>
       <c r="AZ56" t="n">
-        <v>55.28</v>
+        <v>55.76</v>
       </c>
       <c r="BA56" t="n">
         <v>9.380000000000001</v>
@@ -13362,19 +13362,19 @@
         <v>17.68</v>
       </c>
       <c r="BC56" t="n">
-        <v>8.33</v>
+        <v>7.4</v>
       </c>
       <c r="BD56" t="n">
-        <v>-11.55</v>
+        <v>-12.3</v>
       </c>
       <c r="BE56" t="n">
         <v>-4.5</v>
       </c>
       <c r="BF56" t="n">
-        <v>-83.8</v>
+        <v>-83.94</v>
       </c>
       <c r="BG56" t="n">
-        <v>-69.45999999999999</v>
+        <v>-69.73</v>
       </c>
       <c r="BH56" t="n">
         <v>25.37</v>
@@ -13383,7 +13383,7 @@
         <v>0</v>
       </c>
       <c r="BJ56" t="n">
-        <v>57.89</v>
+        <v>58.39</v>
       </c>
       <c r="BK56" t="n">
         <v>6.89</v>
@@ -13392,7 +13392,7 @@
         <v>7.03</v>
       </c>
       <c r="BM56" t="n">
-        <v>58.14</v>
+        <v>58.39</v>
       </c>
       <c r="BN56" t="n">
         <v>86.77</v>
@@ -13401,19 +13401,19 @@
         <v>46.42</v>
       </c>
       <c r="BP56" t="n">
-        <v>56.5</v>
+        <v>57</v>
       </c>
       <c r="BQ56" t="n">
-        <v>8.23</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="BR56" t="n">
-        <v>57.06</v>
+        <v>58.08</v>
       </c>
       <c r="BS56" t="n">
         <v>0.79</v>
       </c>
       <c r="BT56" t="n">
-        <v>30327</v>
+        <v>29643</v>
       </c>
     </row>
     <row r="57">
@@ -13443,13 +13443,13 @@
         </is>
       </c>
       <c r="F57" t="n">
-        <v>5.97</v>
+        <v>6.08</v>
       </c>
       <c r="G57" t="n">
-        <v>1396132210</v>
+        <v>1421857230</v>
       </c>
       <c r="H57" t="n">
-        <v>1294600</v>
+        <v>1984400</v>
       </c>
       <c r="I57" t="n">
         <v>233858065</v>
@@ -13464,7 +13464,7 @@
         <v>0.77</v>
       </c>
       <c r="M57" t="n">
-        <v>0.4178998688798696</v>
+        <v>0.4256000583088722</v>
       </c>
       <c r="N57" t="n">
         <v>0.08</v>
@@ -13542,7 +13542,7 @@
         <v>229180903.7</v>
       </c>
       <c r="AM57" t="n">
-        <v>104422753.1787584</v>
+        <v>106346838.4442782</v>
       </c>
       <c r="AN57" t="n">
         <v>0.347</v>
@@ -13583,7 +13583,7 @@
         <v>10.72</v>
       </c>
       <c r="AZ57" t="n">
-        <v>9.1</v>
+        <v>9.27</v>
       </c>
       <c r="BA57" t="n">
         <v>1.13</v>
@@ -13592,19 +13592,19 @@
         <v>6.26</v>
       </c>
       <c r="BC57" t="n">
-        <v>119.95</v>
+        <v>115.98</v>
       </c>
       <c r="BD57" t="n">
-        <v>79.59</v>
+        <v>76.34</v>
       </c>
       <c r="BE57" t="n">
         <v>52.5</v>
       </c>
       <c r="BF57" t="n">
-        <v>-81.11</v>
+        <v>-81.45999999999999</v>
       </c>
       <c r="BG57" t="n">
-        <v>4.92</v>
+        <v>3.02</v>
       </c>
       <c r="BH57" t="n">
         <v>7.82</v>
@@ -13613,7 +13613,7 @@
         <v>0</v>
       </c>
       <c r="BJ57" t="n">
-        <v>5.97</v>
+        <v>6.08</v>
       </c>
       <c r="BK57" t="n">
         <v>0.98</v>
@@ -13622,7 +13622,7 @@
         <v>1.04</v>
       </c>
       <c r="BM57" t="n">
-        <v>6.01</v>
+        <v>6.08</v>
       </c>
       <c r="BN57" t="n">
         <v>6.22</v>
@@ -13631,19 +13631,19 @@
         <v>3.43</v>
       </c>
       <c r="BP57" t="n">
-        <v>5.84</v>
+        <v>5.91</v>
       </c>
       <c r="BQ57" t="n">
-        <v>5.76</v>
+        <v>5.87</v>
       </c>
       <c r="BR57" t="n">
-        <v>5.94</v>
+        <v>5.95</v>
       </c>
       <c r="BS57" t="n">
         <v>0.42</v>
       </c>
       <c r="BT57" t="n">
-        <v>1346403</v>
+        <v>1346880</v>
       </c>
     </row>
     <row r="58">
@@ -14133,13 +14133,13 @@
         </is>
       </c>
       <c r="F60" t="n">
-        <v>383.95</v>
+        <v>379.81</v>
       </c>
       <c r="G60" t="n">
-        <v>174601229</v>
+        <v>172718596</v>
       </c>
       <c r="H60" t="n">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="I60" t="n">
         <v>454750</v>
@@ -14154,7 +14154,7 @@
         <v>0.83</v>
       </c>
       <c r="M60" t="n">
-        <v>13.05992614202909</v>
+        <v>12.91910784382257</v>
       </c>
       <c r="N60" t="n">
         <v>0.68</v>
@@ -14232,7 +14232,7 @@
         <v>59558607.5</v>
       </c>
       <c r="AM60" t="n">
-        <v>-25601353.22580645</v>
+        <v>-25325307.3313783</v>
       </c>
       <c r="AN60" t="n">
         <v>10.0581</v>
@@ -14273,7 +14273,7 @@
         <v>944.87</v>
       </c>
       <c r="AZ60" t="n">
-        <v>2207.71</v>
+        <v>2183.91</v>
       </c>
       <c r="BA60" t="n">
         <v>231.1</v>
@@ -14282,19 +14282,19 @@
         <v>727.97</v>
       </c>
       <c r="BC60" t="n">
-        <v>201.4</v>
+        <v>204.68</v>
       </c>
       <c r="BD60" t="n">
-        <v>146.09</v>
+        <v>148.77</v>
       </c>
       <c r="BE60" t="n">
         <v>475</v>
       </c>
       <c r="BF60" t="n">
-        <v>-39.81</v>
+        <v>-39.15</v>
       </c>
       <c r="BG60" t="n">
-        <v>89.59999999999999</v>
+        <v>91.67</v>
       </c>
       <c r="BH60" t="n">
         <v>454.44</v>
@@ -14303,7 +14303,7 @@
         <v>0</v>
       </c>
       <c r="BJ60" t="n">
-        <v>383.95</v>
+        <v>379.81</v>
       </c>
       <c r="BK60" t="n">
         <v>130.97</v>
@@ -14321,19 +14321,19 @@
         <v>309.24</v>
       </c>
       <c r="BP60" t="n">
-        <v>373</v>
+        <v>379.76</v>
       </c>
       <c r="BQ60" t="n">
-        <v>2.93</v>
+        <v>2.9</v>
       </c>
       <c r="BR60" t="n">
-        <v>374.12</v>
+        <v>383.95</v>
       </c>
       <c r="BS60" t="n">
         <v>12.82</v>
       </c>
       <c r="BT60" t="n">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="61">
@@ -14363,13 +14363,13 @@
         </is>
       </c>
       <c r="F61" t="n">
-        <v>27.31</v>
+        <v>27.64</v>
       </c>
       <c r="G61" t="n">
-        <v>2337965358</v>
+        <v>2366215570</v>
       </c>
       <c r="H61" t="n">
-        <v>1413700</v>
+        <v>2082900</v>
       </c>
       <c r="I61" t="n">
         <v>85608392</v>
@@ -14384,7 +14384,7 @@
         <v>2.37</v>
       </c>
       <c r="M61" t="n">
-        <v>1.239903300028215</v>
+        <v>1.254885357382248</v>
       </c>
       <c r="N61" t="n">
         <v>1.1</v>
@@ -14462,7 +14462,7 @@
         <v>160087693.04</v>
       </c>
       <c r="AM61" t="n">
-        <v>183513764.3642072</v>
+        <v>185731206.4364207</v>
       </c>
       <c r="AN61" t="n">
         <v>0.38</v>
@@ -14503,7 +14503,7 @@
         <v>17.56</v>
       </c>
       <c r="AZ61" t="n">
-        <v>34.41</v>
+        <v>34.83</v>
       </c>
       <c r="BA61" t="n">
         <v>2.52</v>
@@ -14512,19 +14512,19 @@
         <v>11.76</v>
       </c>
       <c r="BC61" t="n">
-        <v>-21.26</v>
+        <v>-22.2</v>
       </c>
       <c r="BD61" t="n">
-        <v>-35.71</v>
+        <v>-36.48</v>
       </c>
       <c r="BE61" t="n">
         <v>26</v>
       </c>
       <c r="BF61" t="n">
-        <v>-90.76000000000001</v>
+        <v>-90.87</v>
       </c>
       <c r="BG61" t="n">
-        <v>-56.95</v>
+        <v>-57.47</v>
       </c>
       <c r="BH61" t="n">
         <v>10.99</v>
@@ -14533,7 +14533,7 @@
         <v>0</v>
       </c>
       <c r="BJ61" t="n">
-        <v>27.31</v>
+        <v>27.64</v>
       </c>
       <c r="BK61" t="n">
         <v>1.87</v>
@@ -14542,7 +14542,7 @@
         <v>1.86</v>
       </c>
       <c r="BM61" t="n">
-        <v>27.46</v>
+        <v>27.81</v>
       </c>
       <c r="BN61" t="n">
         <v>28.68</v>
@@ -14551,19 +14551,19 @@
         <v>19.35</v>
       </c>
       <c r="BP61" t="n">
-        <v>27</v>
+        <v>27.09</v>
       </c>
       <c r="BQ61" t="n">
-        <v>14.67</v>
+        <v>14.84</v>
       </c>
       <c r="BR61" t="n">
-        <v>27.46</v>
+        <v>27.19</v>
       </c>
       <c r="BS61" t="n">
         <v>1.19</v>
       </c>
       <c r="BT61" t="n">
-        <v>569237</v>
+        <v>589013</v>
       </c>
     </row>
     <row r="62">
@@ -14593,13 +14593,13 @@
         </is>
       </c>
       <c r="F62" t="n">
-        <v>110.95</v>
+        <v>108.02</v>
       </c>
       <c r="G62" t="n">
-        <v>10950734742</v>
+        <v>10661548824</v>
       </c>
       <c r="H62" t="n">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="I62" t="n">
         <v>98699749</v>
@@ -14614,7 +14614,7 @@
         <v>0.64</v>
       </c>
       <c r="M62" t="n">
-        <v>1.026505679644157</v>
+        <v>0.9993978193686657</v>
       </c>
       <c r="N62" t="n">
         <v>0.13</v>
@@ -14692,7 +14692,7 @@
         <v>2757670987.06</v>
       </c>
       <c r="AM62" t="n">
-        <v>4433495846.963562</v>
+        <v>4316416527.935223</v>
       </c>
       <c r="AN62" t="n">
         <v>6.9319</v>
@@ -14733,7 +14733,7 @@
         <v>267.2</v>
       </c>
       <c r="AZ62" t="n">
-        <v>117.24</v>
+        <v>114.14</v>
       </c>
       <c r="BA62" t="n">
         <v>34.09</v>
@@ -14742,19 +14742,19 @@
         <v>76.01000000000001</v>
       </c>
       <c r="BC62" t="n">
-        <v>194.95</v>
+        <v>202.95</v>
       </c>
       <c r="BD62" t="n">
-        <v>140.83</v>
+        <v>147.36</v>
       </c>
       <c r="BE62" t="n">
         <v>5.67</v>
       </c>
       <c r="BF62" t="n">
-        <v>-69.27</v>
+        <v>-68.44</v>
       </c>
       <c r="BG62" t="n">
-        <v>-31.49</v>
+        <v>-29.64</v>
       </c>
       <c r="BH62" t="n">
         <v>170.35</v>
@@ -14763,7 +14763,7 @@
         <v>0</v>
       </c>
       <c r="BJ62" t="n">
-        <v>110.95</v>
+        <v>108.02</v>
       </c>
       <c r="BK62" t="n">
         <v>27.94</v>
@@ -14772,7 +14772,7 @@
         <v>32.73</v>
       </c>
       <c r="BM62" t="n">
-        <v>111</v>
+        <v>109.14</v>
       </c>
       <c r="BN62" t="n">
         <v>122.2</v>
@@ -14781,19 +14781,19 @@
         <v>91.84999999999999</v>
       </c>
       <c r="BP62" t="n">
-        <v>110.95</v>
+        <v>108.02</v>
       </c>
       <c r="BQ62" t="n">
-        <v>3.39</v>
+        <v>3.3</v>
       </c>
       <c r="BR62" t="n">
-        <v>111</v>
+        <v>109.14</v>
       </c>
       <c r="BS62" t="n">
         <v>1.01</v>
       </c>
       <c r="BT62" t="n">
-        <v>167</v>
+        <v>173</v>
       </c>
     </row>
     <row r="63">
@@ -14823,13 +14823,13 @@
         </is>
       </c>
       <c r="F63" t="n">
-        <v>1.41</v>
+        <v>1.44</v>
       </c>
       <c r="G63" t="n">
-        <v>367318668</v>
+        <v>375133982</v>
       </c>
       <c r="H63" t="n">
-        <v>62300</v>
+        <v>24100</v>
       </c>
       <c r="I63" t="n">
         <v>122894462</v>
@@ -14844,7 +14844,7 @@
         <v>-0.22</v>
       </c>
       <c r="M63" t="n">
-        <v>0.4517830057493372</v>
+        <v>0.4613954386513177</v>
       </c>
       <c r="N63" t="n">
         <v>0.37</v>
@@ -14922,7 +14922,7 @@
         <v>31952560.12</v>
       </c>
       <c r="AM63" t="n">
-        <v>208703788.6363636</v>
+        <v>213144307.9545455</v>
       </c>
       <c r="AN63" t="n">
         <v>0</v>
@@ -14981,7 +14981,7 @@
         <v>-100</v>
       </c>
       <c r="BF63" t="n">
-        <v>-79.48999999999999</v>
+        <v>-79.92</v>
       </c>
       <c r="BG63" t="n">
         <v>-100</v>
@@ -14993,7 +14993,7 @@
         <v>0</v>
       </c>
       <c r="BJ63" t="n">
-        <v>1.41</v>
+        <v>1.44</v>
       </c>
       <c r="BK63" t="n">
         <v>0.26</v>
@@ -15002,7 +15002,7 @@
         <v>0.26</v>
       </c>
       <c r="BM63" t="n">
-        <v>1.6</v>
+        <v>1.55</v>
       </c>
       <c r="BN63" t="n">
         <v>2.12</v>
@@ -15011,19 +15011,19 @@
         <v>1.16</v>
       </c>
       <c r="BP63" t="n">
-        <v>1.36</v>
+        <v>1.41</v>
       </c>
       <c r="BQ63" t="n">
-        <v>5.4</v>
+        <v>5.52</v>
       </c>
       <c r="BR63" t="n">
-        <v>1.36</v>
+        <v>1.41</v>
       </c>
       <c r="BS63" t="n">
         <v>0.19</v>
       </c>
       <c r="BT63" t="n">
-        <v>25317</v>
+        <v>27353</v>
       </c>
     </row>
     <row r="64">
@@ -15053,13 +15053,13 @@
         </is>
       </c>
       <c r="F64" t="n">
-        <v>62.25</v>
+        <v>62.85</v>
       </c>
       <c r="G64" t="n">
-        <v>234574247250</v>
+        <v>240198552918</v>
       </c>
       <c r="H64" t="n">
-        <v>9379800</v>
+        <v>11437000</v>
       </c>
       <c r="I64" t="n">
         <v>0</v>
@@ -15146,13 +15146,13 @@
         <v>41.22</v>
       </c>
       <c r="AK64" t="n">
-        <v>67255878869.35789</v>
+        <v>68868449836.4006</v>
       </c>
       <c r="AL64" t="n">
-        <v>18750939028.77698</v>
+        <v>19200523814.38849</v>
       </c>
       <c r="AM64" t="n">
-        <v>20888178739.98219</v>
+        <v>21389007383.61531</v>
       </c>
       <c r="AN64" t="n">
         <v>1.4201</v>
@@ -15193,7 +15193,7 @@
         <v>38.98</v>
       </c>
       <c r="AZ64" t="n">
-        <v>24.9</v>
+        <v>25.14</v>
       </c>
       <c r="BA64" t="n">
         <v>6.69</v>
@@ -15202,19 +15202,19 @@
         <v>10.4</v>
       </c>
       <c r="BC64" t="n">
-        <v>-23.31</v>
+        <v>-24.04</v>
       </c>
       <c r="BD64" t="n">
-        <v>-37.38</v>
+        <v>-37.98</v>
       </c>
       <c r="BE64" t="n">
         <v>-60</v>
       </c>
       <c r="BF64" t="n">
-        <v>-89.25</v>
+        <v>-89.34999999999999</v>
       </c>
       <c r="BG64" t="n">
-        <v>-83.3</v>
+        <v>-83.45999999999999</v>
       </c>
       <c r="BH64" t="n">
         <v>21.37</v>
@@ -15223,7 +15223,7 @@
         <v>0</v>
       </c>
       <c r="BJ64" t="n">
-        <v>62.25</v>
+        <v>62.85</v>
       </c>
       <c r="BK64" t="n">
         <v>4.74</v>
@@ -15232,7 +15232,7 @@
         <v>1.57</v>
       </c>
       <c r="BM64" t="n">
-        <v>63.17</v>
+        <v>63.01</v>
       </c>
       <c r="BN64" t="n">
         <v>64.72</v>
@@ -15241,19 +15241,19 @@
         <v>44.12</v>
       </c>
       <c r="BP64" t="n">
-        <v>61.72</v>
+        <v>61.79</v>
       </c>
       <c r="BQ64" t="n">
-        <v>39.65</v>
+        <v>40.03</v>
       </c>
       <c r="BR64" t="n">
-        <v>62.1</v>
+        <v>62.13</v>
       </c>
       <c r="BS64" t="n">
         <v>3.49</v>
       </c>
       <c r="BT64" t="n">
-        <v>10566997</v>
+        <v>10323167</v>
       </c>
     </row>
     <row r="65">
@@ -15283,13 +15283,13 @@
         </is>
       </c>
       <c r="F65" t="n">
-        <v>24.32</v>
+        <v>24.2</v>
       </c>
       <c r="G65" t="n">
-        <v>234574247250</v>
+        <v>240198552918</v>
       </c>
       <c r="H65" t="n">
-        <v>3100</v>
+        <v>1700</v>
       </c>
       <c r="I65" t="n">
         <v>7298813414</v>
@@ -15304,7 +15304,7 @@
         <v>3.29</v>
       </c>
       <c r="M65" t="n">
-        <v>5.671053603081398</v>
+        <v>5.807026495661329</v>
       </c>
       <c r="N65" t="n">
         <v>0.29</v>
@@ -15382,7 +15382,7 @@
         <v>11532125194.12</v>
       </c>
       <c r="AM65" t="n">
-        <v>17571104662.92135</v>
+        <v>17992400967.64045</v>
       </c>
       <c r="AN65" t="n">
         <v>0.4734</v>
@@ -15423,7 +15423,7 @@
         <v>12.99</v>
       </c>
       <c r="AZ65" t="n">
-        <v>8.19</v>
+        <v>8.15</v>
       </c>
       <c r="BA65" t="n">
         <v>2.23</v>
@@ -15432,19 +15432,19 @@
         <v>3.47</v>
       </c>
       <c r="BC65" t="n">
-        <v>-34.58</v>
+        <v>-34.26</v>
       </c>
       <c r="BD65" t="n">
-        <v>-46.59</v>
+        <v>-46.32</v>
       </c>
       <c r="BE65" t="n">
         <v>-66.33</v>
       </c>
       <c r="BF65" t="n">
-        <v>-90.83</v>
+        <v>-90.78</v>
       </c>
       <c r="BG65" t="n">
-        <v>-85.75</v>
+        <v>-85.68000000000001</v>
       </c>
       <c r="BH65" t="n">
         <v>7.12</v>
@@ -15453,7 +15453,7 @@
         <v>0</v>
       </c>
       <c r="BJ65" t="n">
-        <v>24.32</v>
+        <v>24.2</v>
       </c>
       <c r="BK65" t="n">
         <v>1.58</v>
@@ -15462,7 +15462,7 @@
         <v>1.57</v>
       </c>
       <c r="BM65" t="n">
-        <v>24.34</v>
+        <v>24.27</v>
       </c>
       <c r="BN65" t="n">
         <v>46.43</v>
@@ -15471,19 +15471,19 @@
         <v>20.44</v>
       </c>
       <c r="BP65" t="n">
-        <v>23.9</v>
+        <v>23.75</v>
       </c>
       <c r="BQ65" t="n">
-        <v>15.49</v>
+        <v>15.41</v>
       </c>
       <c r="BR65" t="n">
-        <v>24.03</v>
+        <v>23.95</v>
       </c>
       <c r="BS65" t="n">
         <v>4.14</v>
       </c>
       <c r="BT65" t="n">
-        <v>8857</v>
+        <v>8443</v>
       </c>
     </row>
     <row r="66">
@@ -15513,13 +15513,13 @@
         </is>
       </c>
       <c r="F66" t="n">
-        <v>20.31</v>
+        <v>20.74</v>
       </c>
       <c r="G66" t="n">
-        <v>234574247250</v>
+        <v>240198552918</v>
       </c>
       <c r="H66" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="I66" t="n">
         <v>2972355254</v>
@@ -15534,7 +15534,7 @@
         <v>2.75</v>
       </c>
       <c r="M66" t="n">
-        <v>13.92564433675314</v>
+        <v>14.25953469893889</v>
       </c>
       <c r="N66" t="n">
         <v>0.25</v>
@@ -15612,7 +15612,7 @@
         <v>4696321301.320001</v>
       </c>
       <c r="AM66" t="n">
-        <v>21038049080.71749</v>
+        <v>21542471113.72197</v>
       </c>
       <c r="AN66" t="n">
         <v>0.4734</v>
@@ -15653,7 +15653,7 @@
         <v>12.99</v>
       </c>
       <c r="AZ66" t="n">
-        <v>8.16</v>
+        <v>8.33</v>
       </c>
       <c r="BA66" t="n">
         <v>2.23</v>
@@ -15662,19 +15662,19 @@
         <v>3.47</v>
       </c>
       <c r="BC66" t="n">
-        <v>-21.67</v>
+        <v>-23.29</v>
       </c>
       <c r="BD66" t="n">
-        <v>-36.04</v>
+        <v>-37.37</v>
       </c>
       <c r="BE66" t="n">
         <v>-59.83</v>
       </c>
       <c r="BF66" t="n">
-        <v>-89.01000000000001</v>
+        <v>-89.23999999999999</v>
       </c>
       <c r="BG66" t="n">
-        <v>-82.94</v>
+        <v>-83.29000000000001</v>
       </c>
       <c r="BH66" t="n">
         <v>7.12</v>
@@ -15683,7 +15683,7 @@
         <v>0</v>
       </c>
       <c r="BJ66" t="n">
-        <v>20.31</v>
+        <v>20.74</v>
       </c>
       <c r="BK66" t="n">
         <v>1.58</v>
@@ -15692,7 +15692,7 @@
         <v>1.57</v>
       </c>
       <c r="BM66" t="n">
-        <v>20.31</v>
+        <v>20.74</v>
       </c>
       <c r="BN66" t="n">
         <v>21.33</v>
@@ -15701,19 +15701,19 @@
         <v>9.48</v>
       </c>
       <c r="BP66" t="n">
-        <v>20.31</v>
+        <v>20.3</v>
       </c>
       <c r="BQ66" t="n">
-        <v>12.94</v>
+        <v>13.21</v>
       </c>
       <c r="BR66" t="n">
-        <v>20.31</v>
+        <v>20.3</v>
       </c>
       <c r="BS66" t="n">
         <v>3.46</v>
       </c>
       <c r="BT66" t="n">
-        <v>4393</v>
+        <v>4343</v>
       </c>
     </row>
     <row r="67">
@@ -15973,13 +15973,13 @@
         </is>
       </c>
       <c r="F68" t="n">
-        <v>17.82</v>
+        <v>17.83</v>
       </c>
       <c r="G68" t="n">
-        <v>7776608331</v>
+        <v>7580539738</v>
       </c>
       <c r="H68" t="n">
-        <v>89400</v>
+        <v>37000</v>
       </c>
       <c r="I68" t="n">
         <v>137989898</v>
@@ -16072,7 +16072,7 @@
         <v>205604948.02</v>
       </c>
       <c r="AM68" t="n">
-        <v>539293226.8377254</v>
+        <v>525696237.0319002</v>
       </c>
       <c r="AN68" t="n">
         <v>0.1911</v>
@@ -16113,7 +16113,7 @@
         <v>21.39</v>
       </c>
       <c r="AZ68" t="n">
-        <v>32.97</v>
+        <v>32.99</v>
       </c>
       <c r="BA68" t="n">
         <v>1.24</v>
@@ -16122,19 +16122,19 @@
         <v>63.25</v>
       </c>
       <c r="BC68" t="n">
-        <v>47.04</v>
+        <v>46.96</v>
       </c>
       <c r="BD68" t="n">
-        <v>20.06</v>
+        <v>19.99</v>
       </c>
       <c r="BE68" t="n">
         <v>85</v>
       </c>
       <c r="BF68" t="n">
-        <v>-93.04000000000001</v>
+        <v>-93.05</v>
       </c>
       <c r="BG68" t="n">
-        <v>254.93</v>
+        <v>254.73</v>
       </c>
       <c r="BH68" t="n">
         <v>20.48</v>
@@ -16143,7 +16143,7 @@
         <v>0</v>
       </c>
       <c r="BJ68" t="n">
-        <v>17.82</v>
+        <v>17.83</v>
       </c>
       <c r="BK68" t="n">
         <v>1.49</v>
@@ -16152,7 +16152,7 @@
         <v>1.49</v>
       </c>
       <c r="BM68" t="n">
-        <v>18.07</v>
+        <v>18.12</v>
       </c>
       <c r="BN68" t="n">
         <v>22.11</v>
@@ -16161,19 +16161,19 @@
         <v>15.45</v>
       </c>
       <c r="BP68" t="n">
-        <v>17.68</v>
+        <v>17.78</v>
       </c>
       <c r="BQ68" t="n">
         <v>11.99</v>
       </c>
       <c r="BR68" t="n">
-        <v>18.05</v>
+        <v>18.12</v>
       </c>
       <c r="BS68" t="n">
         <v>0</v>
       </c>
       <c r="BT68" t="n">
-        <v>40983</v>
+        <v>42227</v>
       </c>
     </row>
     <row r="69">
@@ -16203,13 +16203,13 @@
         </is>
       </c>
       <c r="F69" t="n">
-        <v>20.59</v>
+        <v>20.24</v>
       </c>
       <c r="G69" t="n">
-        <v>7776608331</v>
+        <v>7580539738</v>
       </c>
       <c r="H69" t="n">
-        <v>2533500</v>
+        <v>1790900</v>
       </c>
       <c r="I69" t="n">
         <v>255106712</v>
@@ -16302,7 +16302,7 @@
         <v>380109000.88</v>
       </c>
       <c r="AM69" t="n">
-        <v>462893353.0357143</v>
+        <v>451222603.452381</v>
       </c>
       <c r="AN69" t="n">
         <v>0.8856000000000001</v>
@@ -16343,7 +16343,7 @@
         <v>21.39</v>
       </c>
       <c r="AZ69" t="n">
-        <v>36</v>
+        <v>35.39</v>
       </c>
       <c r="BA69" t="n">
         <v>1.24</v>
@@ -16352,19 +16352,19 @@
         <v>69.59</v>
       </c>
       <c r="BC69" t="n">
-        <v>27.26</v>
+        <v>29.46</v>
       </c>
       <c r="BD69" t="n">
-        <v>3.91</v>
+        <v>5.7</v>
       </c>
       <c r="BE69" t="n">
         <v>74.83</v>
       </c>
       <c r="BF69" t="n">
-        <v>-93.98</v>
+        <v>-93.88</v>
       </c>
       <c r="BG69" t="n">
-        <v>237.96</v>
+        <v>243.81</v>
       </c>
       <c r="BH69" t="n">
         <v>20.48</v>
@@ -16373,7 +16373,7 @@
         <v>0</v>
       </c>
       <c r="BJ69" t="n">
-        <v>20.59</v>
+        <v>20.24</v>
       </c>
       <c r="BK69" t="n">
         <v>1.49</v>
@@ -16382,7 +16382,7 @@
         <v>1.49</v>
       </c>
       <c r="BM69" t="n">
-        <v>20.64</v>
+        <v>20.62</v>
       </c>
       <c r="BN69" t="n">
         <v>25.63</v>
@@ -16391,19 +16391,19 @@
         <v>16.87</v>
       </c>
       <c r="BP69" t="n">
-        <v>20.02</v>
+        <v>20.09</v>
       </c>
       <c r="BQ69" t="n">
-        <v>13.85</v>
+        <v>13.61</v>
       </c>
       <c r="BR69" t="n">
-        <v>20.15</v>
+        <v>20.53</v>
       </c>
       <c r="BS69" t="n">
         <v>0</v>
       </c>
       <c r="BT69" t="n">
-        <v>2079770</v>
+        <v>2099263</v>
       </c>
     </row>
     <row r="70">
@@ -16433,13 +16433,13 @@
         </is>
       </c>
       <c r="F70" t="n">
-        <v>17.96</v>
+        <v>18.23</v>
       </c>
       <c r="G70" t="n">
-        <v>8343446886</v>
+        <v>8468877543</v>
       </c>
       <c r="H70" t="n">
-        <v>2470500</v>
+        <v>3499500</v>
       </c>
       <c r="I70" t="n">
         <v>464557268</v>
@@ -16454,7 +16454,7 @@
         <v>0.68</v>
       </c>
       <c r="M70" t="n">
-        <v>0.6585332033164962</v>
+        <v>0.6684332186790801</v>
       </c>
       <c r="N70" t="n">
         <v>0.2</v>
@@ -16532,7 +16532,7 @@
         <v>55746872.16</v>
       </c>
       <c r="AM70" t="n">
-        <v>2753612833.663366</v>
+        <v>2795009090.09901</v>
       </c>
       <c r="AN70" t="n">
         <v>0.1236</v>
@@ -16573,7 +16573,7 @@
         <v>6.9</v>
       </c>
       <c r="AZ70" t="n">
-        <v>2.07</v>
+        <v>2.1</v>
       </c>
       <c r="BA70" t="n">
         <v>0.12</v>
@@ -16582,19 +16582,19 @@
         <v>1.07</v>
       </c>
       <c r="BC70" t="n">
-        <v>-52.96</v>
+        <v>-53.65</v>
       </c>
       <c r="BD70" t="n">
-        <v>-61.59</v>
+        <v>-62.16</v>
       </c>
       <c r="BE70" t="n">
         <v>-88.5</v>
       </c>
       <c r="BF70" t="n">
-        <v>-99.33</v>
+        <v>-99.34</v>
       </c>
       <c r="BG70" t="n">
-        <v>-94.05</v>
+        <v>-94.13</v>
       </c>
       <c r="BH70" t="n">
         <v>26.44</v>
@@ -16603,7 +16603,7 @@
         <v>0</v>
       </c>
       <c r="BJ70" t="n">
-        <v>17.96</v>
+        <v>18.23</v>
       </c>
       <c r="BK70" t="n">
         <v>0.12</v>
@@ -16612,7 +16612,7 @@
         <v>0.1</v>
       </c>
       <c r="BM70" t="n">
-        <v>18.03</v>
+        <v>18.42</v>
       </c>
       <c r="BN70" t="n">
         <v>22.15</v>
@@ -16621,19 +16621,19 @@
         <v>13.21</v>
       </c>
       <c r="BP70" t="n">
-        <v>17.38</v>
+        <v>17.62</v>
       </c>
       <c r="BQ70" t="n">
-        <v>180.12</v>
+        <v>182.83</v>
       </c>
       <c r="BR70" t="n">
-        <v>17.43</v>
+        <v>17.75</v>
       </c>
       <c r="BS70" t="n">
         <v>0.67</v>
       </c>
       <c r="BT70" t="n">
-        <v>3976160</v>
+        <v>3827607</v>
       </c>
     </row>
     <row r="71">

</xml_diff>

<commit_message>
📊 Dados atualizados - 2026-10-01 06:44
</commit_message>
<xml_diff>
--- a/data/ativos.xlsx
+++ b/data/ativos.xlsx
@@ -1047,13 +1047,13 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>25.18</v>
+        <v>25.88</v>
       </c>
       <c r="G3" t="n">
-        <v>3368248064</v>
+        <v>3461884671</v>
       </c>
       <c r="H3" t="n">
-        <v>601000</v>
+        <v>0</v>
       </c>
       <c r="I3" t="n">
         <v>129510368</v>
@@ -1068,7 +1068,7 @@
         <v>0.88</v>
       </c>
       <c r="M3" t="n">
-        <v>0.8380951340013906</v>
+        <v>0.8613940072434954</v>
       </c>
       <c r="N3" t="n">
         <v>0.09</v>
@@ -1146,7 +1146,7 @@
         <v>506385538.88</v>
       </c>
       <c r="AM3" t="n">
-        <v>657860950</v>
+        <v>676149349.8046875</v>
       </c>
       <c r="AN3" t="n">
         <v>2.7</v>
@@ -1187,7 +1187,7 @@
         <v>40.42</v>
       </c>
       <c r="AZ3" t="n">
-        <v>46.08</v>
+        <v>47.36</v>
       </c>
       <c r="BA3" t="n">
         <v>4.87</v>
@@ -1196,25 +1196,25 @@
         <v>21.14</v>
       </c>
       <c r="BC3" t="n">
-        <v>96.58</v>
+        <v>91.26000000000001</v>
       </c>
       <c r="BD3" t="n">
-        <v>60.51</v>
+        <v>56.16</v>
       </c>
       <c r="BE3" t="n">
         <v>83</v>
       </c>
       <c r="BF3" t="n">
-        <v>-80.66</v>
+        <v>-81.19</v>
       </c>
       <c r="BG3" t="n">
-        <v>-16.06</v>
+        <v>-18.33</v>
       </c>
       <c r="BH3" t="n">
         <v>27.85</v>
       </c>
       <c r="BI3" t="n">
-        <v>0</v>
+        <v>2.78</v>
       </c>
       <c r="BJ3" t="n">
         <v>25.18</v>
@@ -1226,7 +1226,7 @@
         <v>4.39</v>
       </c>
       <c r="BM3" t="n">
-        <v>25.18</v>
+        <v>26.11</v>
       </c>
       <c r="BN3" t="n">
         <v>27.17</v>
@@ -1235,19 +1235,19 @@
         <v>18.72</v>
       </c>
       <c r="BP3" t="n">
-        <v>24.74</v>
+        <v>25.24</v>
       </c>
       <c r="BQ3" t="n">
-        <v>5.73</v>
+        <v>5.89</v>
       </c>
       <c r="BR3" t="n">
-        <v>24.98</v>
+        <v>25.31</v>
       </c>
       <c r="BS3" t="n">
         <v>0.79</v>
       </c>
       <c r="BT3" t="n">
-        <v>507783</v>
+        <v>516447</v>
       </c>
     </row>
     <row r="4">
@@ -1277,13 +1277,13 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>15.27</v>
+        <v>15.36</v>
       </c>
       <c r="G4" t="n">
-        <v>236450765288</v>
+        <v>237844372283</v>
       </c>
       <c r="H4" t="n">
-        <v>21988800</v>
+        <v>0</v>
       </c>
       <c r="I4" t="n">
         <v>15484664889</v>
@@ -1298,7 +1298,7 @@
         <v>2.76</v>
       </c>
       <c r="M4" t="n">
-        <v>2.677339234936456</v>
+        <v>2.693119089492016</v>
       </c>
       <c r="N4" t="n">
         <v>1.76</v>
@@ -1376,7 +1376,7 @@
         <v>16258898133.45</v>
       </c>
       <c r="AM4" t="n">
-        <v>23410966860.19802</v>
+        <v>23548947750.79208</v>
       </c>
       <c r="AN4" t="n">
         <v>0.269</v>
@@ -1417,7 +1417,7 @@
         <v>9.470000000000001</v>
       </c>
       <c r="AZ4" t="n">
-        <v>19.06</v>
+        <v>19.17</v>
       </c>
       <c r="BA4" t="n">
         <v>1.13</v>
@@ -1426,25 +1426,25 @@
         <v>11.39</v>
       </c>
       <c r="BC4" t="n">
-        <v>-24.01</v>
+        <v>-24.45</v>
       </c>
       <c r="BD4" t="n">
-        <v>-37.95</v>
+        <v>-38.31</v>
       </c>
       <c r="BE4" t="n">
         <v>24.83</v>
       </c>
       <c r="BF4" t="n">
-        <v>-92.62</v>
+        <v>-92.66</v>
       </c>
       <c r="BG4" t="n">
-        <v>-25.43</v>
+        <v>-25.87</v>
       </c>
       <c r="BH4" t="n">
         <v>5.7</v>
       </c>
       <c r="BI4" t="n">
-        <v>0</v>
+        <v>0.59</v>
       </c>
       <c r="BJ4" t="n">
         <v>15.27</v>
@@ -1456,7 +1456,7 @@
         <v>1.04</v>
       </c>
       <c r="BM4" t="n">
-        <v>15.43</v>
+        <v>15.59</v>
       </c>
       <c r="BN4" t="n">
         <v>16.94</v>
@@ -1465,19 +1465,19 @@
         <v>11.04</v>
       </c>
       <c r="BP4" t="n">
-        <v>15.08</v>
+        <v>15.31</v>
       </c>
       <c r="BQ4" t="n">
-        <v>14.73</v>
+        <v>14.81</v>
       </c>
       <c r="BR4" t="n">
-        <v>15.12</v>
+        <v>15.59</v>
       </c>
       <c r="BS4" t="n">
         <v>2.76</v>
       </c>
       <c r="BT4" t="n">
-        <v>26280057</v>
+        <v>25861960</v>
       </c>
     </row>
     <row r="5">
@@ -3117,13 +3117,13 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>4.93</v>
+        <v>5.32</v>
       </c>
       <c r="G12" t="n">
-        <v>473090375</v>
+        <v>510515409</v>
       </c>
       <c r="H12" t="n">
-        <v>198700</v>
+        <v>3154300</v>
       </c>
       <c r="I12" t="n">
         <v>95961536</v>
@@ -3138,7 +3138,7 @@
         <v>0.32</v>
       </c>
       <c r="M12" t="n">
-        <v>0.0855576724134101</v>
+        <v>0.09232593270412673</v>
       </c>
       <c r="N12" t="n">
         <v>0.14</v>
@@ -3216,7 +3216,7 @@
         <v>362734606.08</v>
       </c>
       <c r="AM12" t="n">
-        <v>508699327.9569892</v>
+        <v>548941300</v>
       </c>
       <c r="AN12" t="n">
         <v>0.4208</v>
@@ -3257,7 +3257,7 @@
         <v>30.49</v>
       </c>
       <c r="AZ12" t="n">
-        <v>6.66</v>
+        <v>7.19</v>
       </c>
       <c r="BA12" t="n">
         <v>4.41</v>
@@ -3266,25 +3266,25 @@
         <v>18.12</v>
       </c>
       <c r="BC12" t="n">
-        <v>657.55</v>
+        <v>602.02</v>
       </c>
       <c r="BD12" t="n">
-        <v>518.54</v>
+        <v>473.19</v>
       </c>
       <c r="BE12" t="n">
         <v>35.17</v>
       </c>
       <c r="BF12" t="n">
-        <v>-10.51</v>
+        <v>-17.07</v>
       </c>
       <c r="BG12" t="n">
-        <v>267.52</v>
+        <v>240.58</v>
       </c>
       <c r="BH12" t="n">
         <v>16.4</v>
       </c>
       <c r="BI12" t="n">
-        <v>0</v>
+        <v>7.91</v>
       </c>
       <c r="BJ12" t="n">
         <v>4.93</v>
@@ -3296,7 +3296,7 @@
         <v>3.63</v>
       </c>
       <c r="BM12" t="n">
-        <v>4.95</v>
+        <v>5.45</v>
       </c>
       <c r="BN12" t="n">
         <v>8.23</v>
@@ -3305,19 +3305,19 @@
         <v>4.42</v>
       </c>
       <c r="BP12" t="n">
-        <v>4.9</v>
+        <v>5.22</v>
       </c>
       <c r="BQ12" t="n">
-        <v>1.36</v>
+        <v>1.46</v>
       </c>
       <c r="BR12" t="n">
-        <v>4.95</v>
+        <v>5.26</v>
       </c>
       <c r="BS12" t="n">
         <v>0.09</v>
       </c>
       <c r="BT12" t="n">
-        <v>479890</v>
+        <v>470260</v>
       </c>
     </row>
     <row r="13">
@@ -3347,13 +3347,13 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>28.77</v>
+        <v>29.49</v>
       </c>
       <c r="G13" t="n">
-        <v>14505578177</v>
+        <v>14868586576</v>
       </c>
       <c r="H13" t="n">
-        <v>2658500</v>
+        <v>0</v>
       </c>
       <c r="I13" t="n">
         <v>504190947</v>
@@ -3368,7 +3368,7 @@
         <v>1.13</v>
       </c>
       <c r="M13" t="n">
-        <v>5.016867547893624</v>
+        <v>5.142416838954876</v>
       </c>
       <c r="N13" t="n">
         <v>0.57</v>
@@ -3446,7 +3446,7 @@
         <v>932753251.95</v>
       </c>
       <c r="AM13" t="n">
-        <v>1509425408.636837</v>
+        <v>1547199435.587929</v>
       </c>
       <c r="AN13" t="n">
         <v>2.6301</v>
@@ -3487,7 +3487,7 @@
         <v>26.6</v>
       </c>
       <c r="AZ13" t="n">
-        <v>52.07</v>
+        <v>53.38</v>
       </c>
       <c r="BA13" t="n">
         <v>2.6</v>
@@ -3496,25 +3496,25 @@
         <v>8.69</v>
       </c>
       <c r="BC13" t="n">
-        <v>13.22</v>
+        <v>10.46</v>
       </c>
       <c r="BD13" t="n">
-        <v>-7.56</v>
+        <v>-9.81</v>
       </c>
       <c r="BE13" t="n">
         <v>81</v>
       </c>
       <c r="BF13" t="n">
-        <v>-90.95</v>
+        <v>-91.17</v>
       </c>
       <c r="BG13" t="n">
-        <v>-69.78</v>
+        <v>-70.52</v>
       </c>
       <c r="BH13" t="n">
         <v>25.49</v>
       </c>
       <c r="BI13" t="n">
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="BJ13" t="n">
         <v>28.77</v>
@@ -3526,7 +3526,7 @@
         <v>1.96</v>
       </c>
       <c r="BM13" t="n">
-        <v>28.88</v>
+        <v>29.76</v>
       </c>
       <c r="BN13" t="n">
         <v>32.11</v>
@@ -3535,19 +3535,19 @@
         <v>20.85</v>
       </c>
       <c r="BP13" t="n">
-        <v>28.37</v>
+        <v>29.01</v>
       </c>
       <c r="BQ13" t="n">
-        <v>14.7</v>
+        <v>15.07</v>
       </c>
       <c r="BR13" t="n">
-        <v>28.57</v>
+        <v>29.32</v>
       </c>
       <c r="BS13" t="n">
         <v>5.01</v>
       </c>
       <c r="BT13" t="n">
-        <v>4844347</v>
+        <v>4821963</v>
       </c>
     </row>
     <row r="14">
@@ -3577,13 +3577,13 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>9.93</v>
+        <v>10.21</v>
       </c>
       <c r="G14" t="n">
-        <v>8220231737</v>
+        <v>8283810124</v>
       </c>
       <c r="H14" t="n">
-        <v>3300</v>
+        <v>3900</v>
       </c>
       <c r="I14" t="n">
         <v>339510689</v>
@@ -3598,7 +3598,7 @@
         <v>1.92</v>
       </c>
       <c r="M14" t="n">
-        <v>3.413186353881337</v>
+        <v>3.439585230440184</v>
       </c>
       <c r="N14" t="n">
         <v>1.11</v>
@@ -3676,7 +3676,7 @@
         <v>349696009.67</v>
       </c>
       <c r="AM14" t="n">
-        <v>912345364.8168702</v>
+        <v>919401789.5671476</v>
       </c>
       <c r="AN14" t="n">
         <v>0.1489</v>
@@ -3717,7 +3717,7 @@
         <v>9.050000000000001</v>
       </c>
       <c r="AZ14" t="n">
-        <v>7.98</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="BA14" t="n">
         <v>1.42</v>
@@ -3726,25 +3726,25 @@
         <v>5.94</v>
       </c>
       <c r="BC14" t="n">
-        <v>11.61</v>
+        <v>8.550000000000001</v>
       </c>
       <c r="BD14" t="n">
-        <v>-8.869999999999999</v>
+        <v>-11.37</v>
       </c>
       <c r="BE14" t="n">
         <v>-19.67</v>
       </c>
       <c r="BF14" t="n">
-        <v>-85.69</v>
+        <v>-86.08</v>
       </c>
       <c r="BG14" t="n">
-        <v>-40.16</v>
+        <v>-41.8</v>
       </c>
       <c r="BH14" t="n">
         <v>5.3</v>
       </c>
       <c r="BI14" t="n">
-        <v>0</v>
+        <v>2.82</v>
       </c>
       <c r="BJ14" t="n">
         <v>9.93</v>
@@ -3756,7 +3756,7 @@
         <v>1.01</v>
       </c>
       <c r="BM14" t="n">
-        <v>10.29</v>
+        <v>10.42</v>
       </c>
       <c r="BN14" t="n">
         <v>13.49</v>
@@ -3765,19 +3765,19 @@
         <v>7.77</v>
       </c>
       <c r="BP14" t="n">
-        <v>9.93</v>
+        <v>10.21</v>
       </c>
       <c r="BQ14" t="n">
-        <v>9.800000000000001</v>
+        <v>10.08</v>
       </c>
       <c r="BR14" t="n">
-        <v>10.2</v>
+        <v>10.3</v>
       </c>
       <c r="BS14" t="n">
         <v>1.44</v>
       </c>
       <c r="BT14" t="n">
-        <v>10457</v>
+        <v>10220</v>
       </c>
     </row>
     <row r="15">
@@ -3807,13 +3807,13 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>14.01</v>
+        <v>14.18</v>
       </c>
       <c r="G15" t="n">
-        <v>8220231737</v>
+        <v>8283810124</v>
       </c>
       <c r="H15" t="n">
-        <v>1491500</v>
+        <v>0</v>
       </c>
       <c r="I15" t="n">
         <v>343551533</v>
@@ -3828,7 +3828,7 @@
         <v>2.56</v>
       </c>
       <c r="M15" t="n">
-        <v>3.37304054670497</v>
+        <v>3.39912892037938</v>
       </c>
       <c r="N15" t="n">
         <v>1.47</v>
@@ -3906,7 +3906,7 @@
         <v>353858078.99</v>
       </c>
       <c r="AM15" t="n">
-        <v>685590636.9474562</v>
+        <v>690893254.7122602</v>
       </c>
       <c r="AN15" t="n">
         <v>0.1638</v>
@@ -3947,7 +3947,7 @@
         <v>9.050000000000001</v>
       </c>
       <c r="AZ15" t="n">
-        <v>9.32</v>
+        <v>9.43</v>
       </c>
       <c r="BA15" t="n">
         <v>1.42</v>
@@ -3956,25 +3956,25 @@
         <v>6.19</v>
       </c>
       <c r="BC15" t="n">
-        <v>-20.89</v>
+        <v>-21.84</v>
       </c>
       <c r="BD15" t="n">
-        <v>-35.41</v>
+        <v>-36.18</v>
       </c>
       <c r="BE15" t="n">
         <v>-33.5</v>
       </c>
       <c r="BF15" t="n">
-        <v>-89.86</v>
+        <v>-89.98</v>
       </c>
       <c r="BG15" t="n">
-        <v>-55.83</v>
+        <v>-56.36</v>
       </c>
       <c r="BH15" t="n">
         <v>5.3</v>
       </c>
       <c r="BI15" t="n">
-        <v>0</v>
+        <v>1.21</v>
       </c>
       <c r="BJ15" t="n">
         <v>14.01</v>
@@ -3986,7 +3986,7 @@
         <v>1.01</v>
       </c>
       <c r="BM15" t="n">
-        <v>14.34</v>
+        <v>14.38</v>
       </c>
       <c r="BN15" t="n">
         <v>16.22</v>
@@ -3995,19 +3995,19 @@
         <v>7.84</v>
       </c>
       <c r="BP15" t="n">
-        <v>13.91</v>
+        <v>13.9</v>
       </c>
       <c r="BQ15" t="n">
-        <v>13.83</v>
+        <v>14</v>
       </c>
       <c r="BR15" t="n">
-        <v>14.14</v>
+        <v>14.18</v>
       </c>
       <c r="BS15" t="n">
         <v>1.92</v>
       </c>
       <c r="BT15" t="n">
-        <v>2346800</v>
+        <v>2350630</v>
       </c>
     </row>
     <row r="16">
@@ -4037,13 +4037,13 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>4.44</v>
+        <v>4.43</v>
       </c>
       <c r="G16" t="n">
-        <v>973717320</v>
+        <v>971524213</v>
       </c>
       <c r="H16" t="n">
-        <v>46200</v>
+        <v>113800</v>
       </c>
       <c r="I16" t="n">
         <v>219305733</v>
@@ -4058,7 +4058,7 @@
         <v>2.69</v>
       </c>
       <c r="M16" t="n">
-        <v>0.4606499363607608</v>
+        <v>0.4596124128626861</v>
       </c>
       <c r="N16" t="n">
         <v>0.39</v>
@@ -4136,7 +4136,7 @@
         <v>17544458.64</v>
       </c>
       <c r="AM16" t="n">
-        <v>273516101.1235955</v>
+        <v>272900059.8314607</v>
       </c>
       <c r="AN16" t="n">
         <v>0.0077</v>
@@ -4186,16 +4186,16 @@
         <v>0</v>
       </c>
       <c r="BC16" t="n">
-        <v>-60.83</v>
+        <v>-60.75</v>
       </c>
       <c r="BD16" t="n">
-        <v>-68.02</v>
+        <v>-67.95</v>
       </c>
       <c r="BE16" t="n">
         <v>-97.17</v>
       </c>
       <c r="BF16" t="n">
-        <v>-98.2</v>
+        <v>-98.19</v>
       </c>
       <c r="BG16" t="n">
         <v>-100</v>
@@ -4204,7 +4204,7 @@
         <v>1.68</v>
       </c>
       <c r="BI16" t="n">
-        <v>0</v>
+        <v>-0.23</v>
       </c>
       <c r="BJ16" t="n">
         <v>4.44</v>
@@ -4216,7 +4216,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="BM16" t="n">
-        <v>4.48</v>
+        <v>4.44</v>
       </c>
       <c r="BN16" t="n">
         <v>5.54</v>
@@ -4225,19 +4225,19 @@
         <v>3.22</v>
       </c>
       <c r="BP16" t="n">
-        <v>4.36</v>
+        <v>4.32</v>
       </c>
       <c r="BQ16" t="n">
-        <v>60.59</v>
+        <v>60.45</v>
       </c>
       <c r="BR16" t="n">
-        <v>4.38</v>
+        <v>4.42</v>
       </c>
       <c r="BS16" t="n">
         <v>0.49</v>
       </c>
       <c r="BT16" t="n">
-        <v>127940</v>
+        <v>126800</v>
       </c>
     </row>
     <row r="17">
@@ -4267,13 +4267,13 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>31.79</v>
+        <v>32.53</v>
       </c>
       <c r="G17" t="n">
-        <v>10478839452</v>
+        <v>10722762654</v>
       </c>
       <c r="H17" t="n">
-        <v>663800</v>
+        <v>0</v>
       </c>
       <c r="I17" t="n">
         <v>0</v>
@@ -4360,13 +4360,13 @@
         <v>8.039999999999999</v>
       </c>
       <c r="AK17" t="n">
-        <v>4732134868.135839</v>
+        <v>4842288048.229769</v>
       </c>
       <c r="AL17" t="n">
-        <v>1309854931.5</v>
+        <v>1340345331.75</v>
       </c>
       <c r="AM17" t="n">
-        <v>3244222740.557276</v>
+        <v>3319740759.752322</v>
       </c>
       <c r="AN17" t="n">
         <v>1.08</v>
@@ -4407,7 +4407,7 @@
         <v>42.98</v>
       </c>
       <c r="AZ17" t="n">
-        <v>17.01</v>
+        <v>17.4</v>
       </c>
       <c r="BA17" t="n">
         <v>4.55</v>
@@ -4416,25 +4416,25 @@
         <v>16.33</v>
       </c>
       <c r="BC17" t="n">
-        <v>65.58</v>
+        <v>61.81</v>
       </c>
       <c r="BD17" t="n">
-        <v>35.19</v>
+        <v>32.12</v>
       </c>
       <c r="BE17" t="n">
         <v>-46.5</v>
       </c>
       <c r="BF17" t="n">
-        <v>-85.69</v>
+        <v>-86.02</v>
       </c>
       <c r="BG17" t="n">
-        <v>-48.62</v>
+        <v>-49.79</v>
       </c>
       <c r="BH17" t="n">
         <v>29.25</v>
       </c>
       <c r="BI17" t="n">
-        <v>0</v>
+        <v>2.33</v>
       </c>
       <c r="BJ17" t="n">
         <v>31.79</v>
@@ -4446,7 +4446,7 @@
         <v>12.62</v>
       </c>
       <c r="BM17" t="n">
-        <v>31.93</v>
+        <v>32.6</v>
       </c>
       <c r="BN17" t="n">
         <v>36.63</v>
@@ -4455,19 +4455,19 @@
         <v>29.53</v>
       </c>
       <c r="BP17" t="n">
-        <v>31.36</v>
+        <v>31.95</v>
       </c>
       <c r="BQ17" t="n">
-        <v>2.52</v>
+        <v>2.58</v>
       </c>
       <c r="BR17" t="n">
-        <v>31.61</v>
+        <v>32.13</v>
       </c>
       <c r="BS17" t="n">
         <v>2.21</v>
       </c>
       <c r="BT17" t="n">
-        <v>1125857</v>
+        <v>1118950</v>
       </c>
     </row>
     <row r="18">
@@ -4497,13 +4497,13 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>10.91</v>
+        <v>11.5</v>
       </c>
       <c r="G18" t="n">
-        <v>10478839452</v>
+        <v>10722762654</v>
       </c>
       <c r="H18" t="n">
-        <v>12300</v>
+        <v>3200</v>
       </c>
       <c r="I18" t="n">
         <v>671494278</v>
@@ -4518,7 +4518,7 @@
         <v>1.2</v>
       </c>
       <c r="M18" t="n">
-        <v>3.085381849474013</v>
+        <v>3.157202419257888</v>
       </c>
       <c r="N18" t="n">
         <v>0.33</v>
@@ -4596,7 +4596,7 @@
         <v>940091989.1999999</v>
       </c>
       <c r="AM18" t="n">
-        <v>3118702217.857143</v>
+        <v>3191298408.928572</v>
       </c>
       <c r="AN18" t="n">
         <v>0.36</v>
@@ -4637,7 +4637,7 @@
         <v>14.31</v>
       </c>
       <c r="AZ18" t="n">
-        <v>5.62</v>
+        <v>5.92</v>
       </c>
       <c r="BA18" t="n">
         <v>1.51</v>
@@ -4646,25 +4646,25 @@
         <v>5.44</v>
       </c>
       <c r="BC18" t="n">
-        <v>60.63</v>
+        <v>52.39</v>
       </c>
       <c r="BD18" t="n">
-        <v>31.16</v>
+        <v>24.43</v>
       </c>
       <c r="BE18" t="n">
         <v>-48.5</v>
       </c>
       <c r="BF18" t="n">
-        <v>-86.14</v>
+        <v>-86.84999999999999</v>
       </c>
       <c r="BG18" t="n">
-        <v>-50.1</v>
+        <v>-52.66</v>
       </c>
       <c r="BH18" t="n">
         <v>9.75</v>
       </c>
       <c r="BI18" t="n">
-        <v>0</v>
+        <v>5.41</v>
       </c>
       <c r="BJ18" t="n">
         <v>10.91</v>
@@ -4676,7 +4676,7 @@
         <v>12.62</v>
       </c>
       <c r="BM18" t="n">
-        <v>11.26</v>
+        <v>11.5</v>
       </c>
       <c r="BN18" t="n">
         <v>13.82</v>
@@ -4685,19 +4685,19 @@
         <v>10.19</v>
       </c>
       <c r="BP18" t="n">
-        <v>10.9</v>
+        <v>11.17</v>
       </c>
       <c r="BQ18" t="n">
-        <v>0.86</v>
+        <v>0.91</v>
       </c>
       <c r="BR18" t="n">
-        <v>10.95</v>
+        <v>11.19</v>
       </c>
       <c r="BS18" t="n">
         <v>2.3</v>
       </c>
       <c r="BT18" t="n">
-        <v>9557</v>
+        <v>9603</v>
       </c>
     </row>
     <row r="19">
@@ -4727,13 +4727,13 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>10.4</v>
+        <v>10.5</v>
       </c>
       <c r="G19" t="n">
-        <v>10478839452</v>
+        <v>10722762654</v>
       </c>
       <c r="H19" t="n">
-        <v>26000</v>
+        <v>16500</v>
       </c>
       <c r="I19" t="n">
         <v>317386323</v>
@@ -4748,7 +4748,7 @@
         <v>1.12</v>
       </c>
       <c r="M19" t="n">
-        <v>6.527742713623035</v>
+        <v>6.67969350090561</v>
       </c>
       <c r="N19" t="n">
         <v>0.3</v>
@@ -4826,7 +4826,7 @@
         <v>444340852.2</v>
       </c>
       <c r="AM19" t="n">
-        <v>3326615699.047619</v>
+        <v>3404051636.190476</v>
       </c>
       <c r="AN19" t="n">
         <v>0.36</v>
@@ -4867,7 +4867,7 @@
         <v>14.31</v>
       </c>
       <c r="AZ19" t="n">
-        <v>5.72</v>
+        <v>5.78</v>
       </c>
       <c r="BA19" t="n">
         <v>1.51</v>
@@ -4876,25 +4876,25 @@
         <v>5.25</v>
       </c>
       <c r="BC19" t="n">
-        <v>68.51000000000001</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="BD19" t="n">
-        <v>37.59</v>
+        <v>36.28</v>
       </c>
       <c r="BE19" t="n">
         <v>-45</v>
       </c>
       <c r="BF19" t="n">
-        <v>-85.45999999999999</v>
+        <v>-85.59</v>
       </c>
       <c r="BG19" t="n">
-        <v>-49.52</v>
+        <v>-50</v>
       </c>
       <c r="BH19" t="n">
         <v>9.75</v>
       </c>
       <c r="BI19" t="n">
-        <v>0</v>
+        <v>0.96</v>
       </c>
       <c r="BJ19" t="n">
         <v>10.4</v>
@@ -4906,7 +4906,7 @@
         <v>12.62</v>
       </c>
       <c r="BM19" t="n">
-        <v>10.49</v>
+        <v>10.52</v>
       </c>
       <c r="BN19" t="n">
         <v>11.41</v>
@@ -4915,19 +4915,19 @@
         <v>9.19</v>
       </c>
       <c r="BP19" t="n">
-        <v>10.25</v>
+        <v>10.27</v>
       </c>
       <c r="BQ19" t="n">
-        <v>0.82</v>
+        <v>0.83</v>
       </c>
       <c r="BR19" t="n">
-        <v>10.32</v>
+        <v>10.43</v>
       </c>
       <c r="BS19" t="n">
         <v>2.16</v>
       </c>
       <c r="BT19" t="n">
-        <v>11927</v>
+        <v>11533</v>
       </c>
     </row>
     <row r="20">
@@ -5417,13 +5417,13 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>5.08</v>
+        <v>5.49</v>
       </c>
       <c r="G22" t="n">
-        <v>1017246108</v>
+        <v>1099346102</v>
       </c>
       <c r="H22" t="n">
-        <v>1192700</v>
+        <v>0</v>
       </c>
       <c r="I22" t="n">
         <v>200245299</v>
@@ -5438,7 +5438,7 @@
         <v>0.27</v>
       </c>
       <c r="M22" t="n">
-        <v>0.08627936415316773</v>
+        <v>0.09324280714261869</v>
       </c>
       <c r="N22" t="n">
         <v>0.08</v>
@@ -5516,7 +5516,7 @@
         <v>378463615.11</v>
       </c>
       <c r="AM22" t="n">
-        <v>230668051.7006803</v>
+        <v>249284830.3854875</v>
       </c>
       <c r="AN22" t="n">
         <v>0</v>
@@ -5566,25 +5566,25 @@
         <v>172.49</v>
       </c>
       <c r="BC22" t="n">
-        <v>484.75</v>
+        <v>441.08</v>
       </c>
       <c r="BD22" t="n">
-        <v>377.44</v>
+        <v>341.79</v>
       </c>
       <c r="BE22" t="n">
         <v>-100</v>
       </c>
       <c r="BF22" t="n">
-        <v>-62.8</v>
+        <v>-65.56999999999999</v>
       </c>
       <c r="BG22" t="n">
-        <v>3295.47</v>
+        <v>3041.89</v>
       </c>
       <c r="BH22" t="n">
         <v>20.75</v>
       </c>
       <c r="BI22" t="n">
-        <v>0</v>
+        <v>8.07</v>
       </c>
       <c r="BJ22" t="n">
         <v>5.08</v>
@@ -5596,7 +5596,7 @@
         <v>0.67</v>
       </c>
       <c r="BM22" t="n">
-        <v>5.22</v>
+        <v>5.52</v>
       </c>
       <c r="BN22" t="n">
         <v>7.89</v>
@@ -5605,19 +5605,19 @@
         <v>3.37</v>
       </c>
       <c r="BP22" t="n">
-        <v>5.03</v>
+        <v>5.12</v>
       </c>
       <c r="BQ22" t="n">
-        <v>7.57</v>
+        <v>8.18</v>
       </c>
       <c r="BR22" t="n">
-        <v>5.03</v>
+        <v>5.14</v>
       </c>
       <c r="BS22" t="n">
         <v>0.09</v>
       </c>
       <c r="BT22" t="n">
-        <v>1532727</v>
+        <v>1530817</v>
       </c>
     </row>
     <row r="23">
@@ -5877,13 +5877,13 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.86</v>
+        <v>2.99</v>
       </c>
       <c r="G24" t="n">
-        <v>1155065011</v>
+        <v>1207567715</v>
       </c>
       <c r="H24" t="n">
-        <v>3842300</v>
+        <v>0</v>
       </c>
       <c r="I24" t="n">
         <v>403868805</v>
@@ -5898,7 +5898,7 @@
         <v>0.49</v>
       </c>
       <c r="M24" t="n">
-        <v>0.2792263710756008</v>
+        <v>0.2919184181638287</v>
       </c>
       <c r="N24" t="n">
         <v>0.11</v>
@@ -5976,7 +5976,7 @@
         <v>153470145.9</v>
       </c>
       <c r="AM24" t="n">
-        <v>1040599109.009009</v>
+        <v>1087898842.342342</v>
       </c>
       <c r="AN24" t="n">
         <v>0.0813</v>
@@ -6017,7 +6017,7 @@
         <v>5.84</v>
       </c>
       <c r="AZ24" t="n">
-        <v>1.32</v>
+        <v>1.38</v>
       </c>
       <c r="BA24" t="n">
         <v>0.38</v>
@@ -6026,25 +6026,25 @@
         <v>1.46</v>
       </c>
       <c r="BC24" t="n">
-        <v>150.22</v>
+        <v>139.35</v>
       </c>
       <c r="BD24" t="n">
-        <v>104.31</v>
+        <v>95.42</v>
       </c>
       <c r="BE24" t="n">
         <v>-53.83</v>
       </c>
       <c r="BF24" t="n">
-        <v>-86.70999999999999</v>
+        <v>-87.29000000000001</v>
       </c>
       <c r="BG24" t="n">
-        <v>-49.03</v>
+        <v>-51.24</v>
       </c>
       <c r="BH24" t="n">
         <v>5.99</v>
       </c>
       <c r="BI24" t="n">
-        <v>0</v>
+        <v>4.55</v>
       </c>
       <c r="BJ24" t="n">
         <v>2.86</v>
@@ -6056,7 +6056,7 @@
         <v>0.41</v>
       </c>
       <c r="BM24" t="n">
-        <v>2.89</v>
+        <v>2.99</v>
       </c>
       <c r="BN24" t="n">
         <v>5.29</v>
@@ -6065,19 +6065,19 @@
         <v>1.92</v>
       </c>
       <c r="BP24" t="n">
-        <v>2.83</v>
+        <v>2.85</v>
       </c>
       <c r="BQ24" t="n">
-        <v>7.02</v>
+        <v>7.34</v>
       </c>
       <c r="BR24" t="n">
-        <v>2.83</v>
+        <v>2.89</v>
       </c>
       <c r="BS24" t="n">
         <v>0.29</v>
       </c>
       <c r="BT24" t="n">
-        <v>7454537</v>
+        <v>7235407</v>
       </c>
     </row>
     <row r="25">
@@ -6107,13 +6107,13 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>3.94</v>
+        <v>4.31</v>
       </c>
       <c r="G25" t="n">
-        <v>1365186379</v>
+        <v>1493389551</v>
       </c>
       <c r="H25" t="n">
-        <v>576400</v>
+        <v>0</v>
       </c>
       <c r="I25" t="n">
         <v>346494097</v>
@@ -6128,7 +6128,7 @@
         <v>0.97</v>
       </c>
       <c r="M25" t="n">
-        <v>0.6807442633463135</v>
+        <v>0.7446722186967973</v>
       </c>
       <c r="N25" t="n">
         <v>0.22</v>
@@ -6206,7 +6206,7 @@
         <v>62368937.46</v>
       </c>
       <c r="AM25" t="n">
-        <v>501906756.9852941</v>
+        <v>549040276.1029412</v>
       </c>
       <c r="AN25" t="n">
         <v>0.4742</v>
@@ -6247,7 +6247,7 @@
         <v>3.27</v>
       </c>
       <c r="AZ25" t="n">
-        <v>9.18</v>
+        <v>10.04</v>
       </c>
       <c r="BA25" t="n">
         <v>0.23</v>
@@ -6256,25 +6256,25 @@
         <v>2.2</v>
       </c>
       <c r="BC25" t="n">
-        <v>1.77</v>
+        <v>-6.97</v>
       </c>
       <c r="BD25" t="n">
-        <v>-16.9</v>
+        <v>-24.04</v>
       </c>
       <c r="BE25" t="n">
         <v>133</v>
       </c>
       <c r="BF25" t="n">
-        <v>-94.12</v>
+        <v>-94.62</v>
       </c>
       <c r="BG25" t="n">
-        <v>-44.17</v>
+        <v>-48.96</v>
       </c>
       <c r="BH25" t="n">
         <v>3.97</v>
       </c>
       <c r="BI25" t="n">
-        <v>0</v>
+        <v>9.390000000000001</v>
       </c>
       <c r="BJ25" t="n">
         <v>3.94</v>
@@ -6286,7 +6286,7 @@
         <v>0.24</v>
       </c>
       <c r="BM25" t="n">
-        <v>4.04</v>
+        <v>4.44</v>
       </c>
       <c r="BN25" t="n">
         <v>6.3</v>
@@ -6295,19 +6295,19 @@
         <v>2.64</v>
       </c>
       <c r="BP25" t="n">
-        <v>3.86</v>
+        <v>4.01</v>
       </c>
       <c r="BQ25" t="n">
-        <v>16.65</v>
+        <v>18.21</v>
       </c>
       <c r="BR25" t="n">
-        <v>3.89</v>
+        <v>4.01</v>
       </c>
       <c r="BS25" t="n">
         <v>0.67</v>
       </c>
       <c r="BT25" t="n">
-        <v>1153343</v>
+        <v>1159540</v>
       </c>
     </row>
     <row r="26">
@@ -6337,13 +6337,13 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>10.54</v>
+        <v>10.93</v>
       </c>
       <c r="G26" t="n">
-        <v>14275302168</v>
+        <v>14803515903</v>
       </c>
       <c r="H26" t="n">
-        <v>26249600</v>
+        <v>0</v>
       </c>
       <c r="I26" t="n">
         <v>1354393401</v>
@@ -6358,7 +6358,7 @@
         <v>1.94</v>
       </c>
       <c r="M26" t="n">
-        <v>0.184078818068024</v>
+        <v>0.1908900896531577</v>
       </c>
       <c r="N26" t="n">
         <v>0.26</v>
@@ -6436,7 +6436,7 @@
         <v>961619314.7099999</v>
       </c>
       <c r="AM26" t="n">
-        <v>5098322202.857143</v>
+        <v>5286969965.357143</v>
       </c>
       <c r="AN26" t="n">
         <v>0.1043</v>
@@ -6477,7 +6477,7 @@
         <v>7.07</v>
       </c>
       <c r="AZ26" t="n">
-        <v>2.02</v>
+        <v>2.09</v>
       </c>
       <c r="BA26" t="n">
         <v>0.66</v>
@@ -6486,25 +6486,25 @@
         <v>1.19</v>
       </c>
       <c r="BC26" t="n">
-        <v>-17.88</v>
+        <v>-20.81</v>
       </c>
       <c r="BD26" t="n">
-        <v>-32.95</v>
+        <v>-35.34</v>
       </c>
       <c r="BE26" t="n">
         <v>-80.83</v>
       </c>
       <c r="BF26" t="n">
-        <v>-93.75</v>
+        <v>-93.97</v>
       </c>
       <c r="BG26" t="n">
-        <v>-88.68000000000001</v>
+        <v>-89.08</v>
       </c>
       <c r="BH26" t="n">
         <v>4.69</v>
       </c>
       <c r="BI26" t="n">
-        <v>0</v>
+        <v>3.7</v>
       </c>
       <c r="BJ26" t="n">
         <v>10.54</v>
@@ -6516,28 +6516,28 @@
         <v>0.72</v>
       </c>
       <c r="BM26" t="n">
-        <v>10.55</v>
+        <v>11</v>
       </c>
       <c r="BN26" t="n">
-        <v>10.55</v>
+        <v>11</v>
       </c>
       <c r="BO26" t="n">
         <v>6.91</v>
       </c>
       <c r="BP26" t="n">
-        <v>10.19</v>
+        <v>10.53</v>
       </c>
       <c r="BQ26" t="n">
-        <v>14.7</v>
+        <v>15.24</v>
       </c>
       <c r="BR26" t="n">
-        <v>10.2</v>
+        <v>10.6</v>
       </c>
       <c r="BS26" t="n">
         <v>0.16</v>
       </c>
       <c r="BT26" t="n">
-        <v>12398140</v>
+        <v>12864177</v>
       </c>
     </row>
     <row r="27">
@@ -8165,13 +8165,13 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>17.15</v>
+        <v>17.38</v>
       </c>
       <c r="G34" t="n">
-        <v>3541299991</v>
+        <v>3588790812</v>
       </c>
       <c r="H34" t="n">
-        <v>6522400</v>
+        <v>0</v>
       </c>
       <c r="I34" t="n">
         <v>206489813</v>
@@ -8186,7 +8186,7 @@
         <v>0.45</v>
       </c>
       <c r="M34" t="n">
-        <v>0.3113216295060238</v>
+        <v>0.3154966273367283</v>
       </c>
       <c r="N34" t="n">
         <v>0.24</v>
@@ -8264,7 +8264,7 @@
         <v>324189006.41</v>
       </c>
       <c r="AM34" t="n">
-        <v>736237004.3659045</v>
+        <v>746110355.925156</v>
       </c>
       <c r="AN34" t="n">
         <v>0</v>
@@ -8305,7 +8305,7 @@
         <v>30.28</v>
       </c>
       <c r="AZ34" t="n">
-        <v>40.02</v>
+        <v>40.55</v>
       </c>
       <c r="BA34" t="n">
         <v>2.29</v>
@@ -8314,25 +8314,25 @@
         <v>25.26</v>
       </c>
       <c r="BC34" t="n">
-        <v>116.26</v>
+        <v>113.4</v>
       </c>
       <c r="BD34" t="n">
-        <v>76.58</v>
+        <v>74.23999999999999</v>
       </c>
       <c r="BE34" t="n">
         <v>133.33</v>
       </c>
       <c r="BF34" t="n">
-        <v>-86.62</v>
+        <v>-86.8</v>
       </c>
       <c r="BG34" t="n">
-        <v>47.28</v>
+        <v>45.33</v>
       </c>
       <c r="BH34" t="n">
         <v>38.94</v>
       </c>
       <c r="BI34" t="n">
-        <v>0</v>
+        <v>1.34</v>
       </c>
       <c r="BJ34" t="n">
         <v>17.15</v>
@@ -8344,7 +8344,7 @@
         <v>1.58</v>
       </c>
       <c r="BM34" t="n">
-        <v>17.19</v>
+        <v>18.19</v>
       </c>
       <c r="BN34" t="n">
         <v>28.86</v>
@@ -8353,19 +8353,19 @@
         <v>14.3</v>
       </c>
       <c r="BP34" t="n">
-        <v>15.4</v>
+        <v>16.69</v>
       </c>
       <c r="BQ34" t="n">
-        <v>10.87</v>
+        <v>11.02</v>
       </c>
       <c r="BR34" t="n">
-        <v>15.52</v>
+        <v>17.46</v>
       </c>
       <c r="BS34" t="n">
         <v>0.32</v>
       </c>
       <c r="BT34" t="n">
-        <v>3354970</v>
+        <v>3517930</v>
       </c>
     </row>
     <row r="35">
@@ -8395,13 +8395,13 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>17.9</v>
+        <v>18.34</v>
       </c>
       <c r="G35" t="n">
-        <v>90332348074</v>
+        <v>92552792430</v>
       </c>
       <c r="H35" t="n">
-        <v>56307100</v>
+        <v>0</v>
       </c>
       <c r="I35" t="n">
         <v>5046500000</v>
@@ -8416,7 +8416,7 @@
         <v>4.69</v>
       </c>
       <c r="M35" t="n">
-        <v>7.499424368404665</v>
+        <v>7.683766465860515</v>
       </c>
       <c r="N35" t="n">
         <v>1.79</v>
@@ -8494,7 +8494,7 @@
         <v>5349290000</v>
       </c>
       <c r="AM35" t="n">
-        <v>7465483311.900826</v>
+        <v>7648991109.917356</v>
       </c>
       <c r="AN35" t="n">
         <v>0.5305</v>
@@ -8535,7 +8535,7 @@
         <v>7.68</v>
       </c>
       <c r="AZ35" t="n">
-        <v>10.44</v>
+        <v>10.7</v>
       </c>
       <c r="BA35" t="n">
         <v>1.11</v>
@@ -8544,25 +8544,25 @@
         <v>9.119999999999999</v>
       </c>
       <c r="BC35" t="n">
-        <v>-47.45</v>
+        <v>-48.71</v>
       </c>
       <c r="BD35" t="n">
-        <v>-57.09</v>
+        <v>-58.12</v>
       </c>
       <c r="BE35" t="n">
         <v>-41.67</v>
       </c>
       <c r="BF35" t="n">
-        <v>-93.78</v>
+        <v>-93.92</v>
       </c>
       <c r="BG35" t="n">
-        <v>-49.07</v>
+        <v>-50.29</v>
       </c>
       <c r="BH35" t="n">
         <v>3.71</v>
       </c>
       <c r="BI35" t="n">
-        <v>0</v>
+        <v>2.46</v>
       </c>
       <c r="BJ35" t="n">
         <v>17.9</v>
@@ -8574,7 +8574,7 @@
         <v>1.04</v>
       </c>
       <c r="BM35" t="n">
-        <v>18.05</v>
+        <v>18.6</v>
       </c>
       <c r="BN35" t="n">
         <v>19.88</v>
@@ -8583,19 +8583,19 @@
         <v>11.58</v>
       </c>
       <c r="BP35" t="n">
-        <v>17.53</v>
+        <v>18.09</v>
       </c>
       <c r="BQ35" t="n">
-        <v>17.13</v>
+        <v>17.55</v>
       </c>
       <c r="BR35" t="n">
-        <v>17.69</v>
+        <v>18.42</v>
       </c>
       <c r="BS35" t="n">
         <v>7.3</v>
       </c>
       <c r="BT35" t="n">
-        <v>39461233</v>
+        <v>40165373</v>
       </c>
     </row>
     <row r="36">
@@ -8825,7 +8825,7 @@
         <v>1.24</v>
       </c>
       <c r="BT36" t="n">
-        <v>147</v>
+        <v>300</v>
       </c>
     </row>
     <row r="37">
@@ -8855,13 +8855,13 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>14.47</v>
+        <v>14.5</v>
       </c>
       <c r="G37" t="n">
-        <v>197807652</v>
+        <v>179073405</v>
       </c>
       <c r="H37" t="n">
-        <v>12000</v>
+        <v>300</v>
       </c>
       <c r="I37" t="n">
         <v>4900000</v>
@@ -8876,7 +8876,7 @@
         <v>0.88</v>
       </c>
       <c r="M37" t="n">
-        <v>1.925824123191094</v>
+        <v>1.743430447124304</v>
       </c>
       <c r="N37" t="n">
         <v>0.5</v>
@@ -8954,7 +8954,7 @@
         <v>11319000</v>
       </c>
       <c r="AM37" t="n">
-        <v>47322404.784689</v>
+        <v>42840527.51196173</v>
       </c>
       <c r="AN37" t="n">
         <v>0</v>
@@ -8995,7 +8995,7 @@
         <v>24.36</v>
       </c>
       <c r="AZ37" t="n">
-        <v>64.34</v>
+        <v>64.48</v>
       </c>
       <c r="BA37" t="n">
         <v>2.44</v>
@@ -9004,25 +9004,25 @@
         <v>15.53</v>
       </c>
       <c r="BC37" t="n">
-        <v>106.21</v>
+        <v>105.78</v>
       </c>
       <c r="BD37" t="n">
-        <v>68.37</v>
+        <v>68.02</v>
       </c>
       <c r="BE37" t="n">
         <v>344.67</v>
       </c>
       <c r="BF37" t="n">
-        <v>-83.09999999999999</v>
+        <v>-83.14</v>
       </c>
       <c r="BG37" t="n">
-        <v>7.35</v>
+        <v>7.13</v>
       </c>
       <c r="BH37" t="n">
         <v>17.13</v>
       </c>
       <c r="BI37" t="n">
-        <v>0</v>
+        <v>0.21</v>
       </c>
       <c r="BJ37" t="n">
         <v>14.47</v>
@@ -9034,7 +9034,7 @@
         <v>2.31</v>
       </c>
       <c r="BM37" t="n">
-        <v>14.51</v>
+        <v>14.5</v>
       </c>
       <c r="BN37" t="n">
         <v>20.9</v>
@@ -9043,19 +9043,19 @@
         <v>13.42</v>
       </c>
       <c r="BP37" t="n">
-        <v>14.2</v>
+        <v>14.5</v>
       </c>
       <c r="BQ37" t="n">
-        <v>6.26</v>
+        <v>6.27</v>
       </c>
       <c r="BR37" t="n">
-        <v>14.51</v>
+        <v>14.5</v>
       </c>
       <c r="BS37" t="n">
         <v>0.72</v>
       </c>
       <c r="BT37" t="n">
-        <v>870</v>
+        <v>1223</v>
       </c>
     </row>
     <row r="38">
@@ -9315,13 +9315,13 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>68.53</v>
+        <v>69.37</v>
       </c>
       <c r="G39" t="n">
-        <v>3841675915</v>
+        <v>3888765118</v>
       </c>
       <c r="H39" t="n">
-        <v>700</v>
+        <v>1200</v>
       </c>
       <c r="I39" t="n">
         <v>168174945</v>
@@ -9336,7 +9336,7 @@
         <v>0.53</v>
       </c>
       <c r="M39" t="n">
-        <v>0.1928352799408383</v>
+        <v>0.1951989513810139</v>
       </c>
       <c r="N39" t="n">
         <v>0.06</v>
@@ -9414,7 +9414,7 @@
         <v>2536078170.6</v>
       </c>
       <c r="AM39" t="n">
-        <v>403537386.0294118</v>
+        <v>408483730.8823529</v>
       </c>
       <c r="AN39" t="n">
         <v>11.9435</v>
@@ -9455,7 +9455,7 @@
         <v>170.24</v>
       </c>
       <c r="AZ39" t="n">
-        <v>200.22</v>
+        <v>202.68</v>
       </c>
       <c r="BA39" t="n">
         <v>19.01</v>
@@ -9464,25 +9464,25 @@
         <v>91.72</v>
       </c>
       <c r="BC39" t="n">
-        <v>204.25</v>
+        <v>200.57</v>
       </c>
       <c r="BD39" t="n">
-        <v>148.42</v>
+        <v>145.41</v>
       </c>
       <c r="BE39" t="n">
         <v>192.17</v>
       </c>
       <c r="BF39" t="n">
-        <v>-72.26000000000001</v>
+        <v>-72.59999999999999</v>
       </c>
       <c r="BG39" t="n">
-        <v>33.84</v>
+        <v>32.22</v>
       </c>
       <c r="BH39" t="n">
         <v>128.13</v>
       </c>
       <c r="BI39" t="n">
-        <v>0</v>
+        <v>1.23</v>
       </c>
       <c r="BJ39" t="n">
         <v>68.53</v>
@@ -9494,7 +9494,7 @@
         <v>15.08</v>
       </c>
       <c r="BM39" t="n">
-        <v>68.90000000000001</v>
+        <v>69.41</v>
       </c>
       <c r="BN39" t="n">
         <v>74.56</v>
@@ -9503,19 +9503,19 @@
         <v>54.98</v>
       </c>
       <c r="BP39" t="n">
-        <v>68.33</v>
+        <v>68.51000000000001</v>
       </c>
       <c r="BQ39" t="n">
-        <v>4.54</v>
+        <v>4.6</v>
       </c>
       <c r="BR39" t="n">
-        <v>68.90000000000001</v>
+        <v>68.51000000000001</v>
       </c>
       <c r="BS39" t="n">
         <v>0.58</v>
       </c>
       <c r="BT39" t="n">
-        <v>3183</v>
+        <v>3113</v>
       </c>
     </row>
     <row r="40">
@@ -9545,13 +9545,13 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>22.04</v>
+        <v>23.07</v>
       </c>
       <c r="G40" t="n">
-        <v>126307542526</v>
+        <v>132210338631</v>
       </c>
       <c r="H40" t="n">
-        <v>37276500</v>
+        <v>0</v>
       </c>
       <c r="I40" t="n">
         <v>5730834040</v>
@@ -9566,7 +9566,7 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="M40" t="n">
-        <v>0.3832327153188501</v>
+        <v>0.401142529206861</v>
       </c>
       <c r="N40" t="n">
         <v>0.05</v>
@@ -9644,7 +9644,7 @@
         <v>15358635227.2</v>
       </c>
       <c r="AM40" t="n">
-        <v>6551221085.373444</v>
+        <v>6857382709.076763</v>
       </c>
       <c r="AN40" t="n">
         <v>0.5641</v>
@@ -9685,7 +9685,7 @@
         <v>36.13</v>
       </c>
       <c r="AZ40" t="n">
-        <v>11.13</v>
+        <v>11.65</v>
       </c>
       <c r="BA40" t="n">
         <v>2.76</v>
@@ -9694,25 +9694,25 @@
         <v>27.89</v>
       </c>
       <c r="BC40" t="n">
-        <v>100.77</v>
+        <v>91.8</v>
       </c>
       <c r="BD40" t="n">
-        <v>63.92</v>
+        <v>56.61</v>
       </c>
       <c r="BE40" t="n">
         <v>-49.5</v>
       </c>
       <c r="BF40" t="n">
-        <v>-87.48</v>
+        <v>-88.04000000000001</v>
       </c>
       <c r="BG40" t="n">
-        <v>26.54</v>
+        <v>20.89</v>
       </c>
       <c r="BH40" t="n">
         <v>32.47</v>
       </c>
       <c r="BI40" t="n">
-        <v>0</v>
+        <v>4.67</v>
       </c>
       <c r="BJ40" t="n">
         <v>22.04</v>
@@ -9724,7 +9724,7 @@
         <v>2.5</v>
       </c>
       <c r="BM40" t="n">
-        <v>22.18</v>
+        <v>23.07</v>
       </c>
       <c r="BN40" t="n">
         <v>27.36</v>
@@ -9733,19 +9733,19 @@
         <v>17.67</v>
       </c>
       <c r="BP40" t="n">
-        <v>21.34</v>
+        <v>22.23</v>
       </c>
       <c r="BQ40" t="n">
-        <v>8.82</v>
+        <v>9.23</v>
       </c>
       <c r="BR40" t="n">
-        <v>21.47</v>
+        <v>22.5</v>
       </c>
       <c r="BS40" t="n">
         <v>0.39</v>
       </c>
       <c r="BT40" t="n">
-        <v>37052397</v>
+        <v>37410833</v>
       </c>
     </row>
     <row r="41">
@@ -9775,13 +9775,13 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>15.65</v>
+        <v>16.22</v>
       </c>
       <c r="G41" t="n">
-        <v>187508242841</v>
+        <v>194821269309</v>
       </c>
       <c r="H41" t="n">
-        <v>8434600</v>
+        <v>0</v>
       </c>
       <c r="I41" t="n">
         <v>5303870781</v>
@@ -9796,7 +9796,7 @@
         <v>0.92</v>
       </c>
       <c r="M41" t="n">
-        <v>1.249549015777154</v>
+        <v>1.298282793487345</v>
       </c>
       <c r="N41" t="n">
         <v>0.07000000000000001</v>
@@ -9874,7 +9874,7 @@
         <v>12304980211.92</v>
       </c>
       <c r="AM41" t="n">
-        <v>28891871007.85824</v>
+        <v>30018685563.79045</v>
       </c>
       <c r="AN41" t="n">
         <v>1.6841</v>
@@ -9915,7 +9915,7 @@
         <v>24.4</v>
       </c>
       <c r="AZ41" t="n">
-        <v>23.42</v>
+        <v>24.28</v>
       </c>
       <c r="BA41" t="n">
         <v>2.53</v>
@@ -9924,25 +9924,25 @@
         <v>13.77</v>
       </c>
       <c r="BC41" t="n">
-        <v>90.95999999999999</v>
+        <v>84.25</v>
       </c>
       <c r="BD41" t="n">
-        <v>55.92</v>
+        <v>50.44</v>
       </c>
       <c r="BE41" t="n">
         <v>49.67</v>
       </c>
       <c r="BF41" t="n">
-        <v>-83.84999999999999</v>
+        <v>-84.42</v>
       </c>
       <c r="BG41" t="n">
-        <v>-12.01</v>
+        <v>-15.1</v>
       </c>
       <c r="BH41" t="n">
         <v>17.11</v>
       </c>
       <c r="BI41" t="n">
-        <v>0</v>
+        <v>3.64</v>
       </c>
       <c r="BJ41" t="n">
         <v>15.65</v>
@@ -9954,7 +9954,7 @@
         <v>2.34</v>
       </c>
       <c r="BM41" t="n">
-        <v>15.67</v>
+        <v>16.31</v>
       </c>
       <c r="BN41" t="n">
         <v>18.28</v>
@@ -9963,19 +9963,19 @@
         <v>13.43</v>
       </c>
       <c r="BP41" t="n">
-        <v>15.45</v>
+        <v>15.87</v>
       </c>
       <c r="BQ41" t="n">
-        <v>6.7</v>
+        <v>6.94</v>
       </c>
       <c r="BR41" t="n">
-        <v>15.61</v>
+        <v>15.98</v>
       </c>
       <c r="BS41" t="n">
         <v>0.5600000000000001</v>
       </c>
       <c r="BT41" t="n">
-        <v>7209050</v>
+        <v>7317057</v>
       </c>
     </row>
     <row r="42">
@@ -10005,13 +10005,13 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>17.78</v>
+        <v>18.51</v>
       </c>
       <c r="G42" t="n">
-        <v>187508242841</v>
+        <v>194821269309</v>
       </c>
       <c r="H42" t="n">
-        <v>41812200</v>
+        <v>0</v>
       </c>
       <c r="I42" t="n">
         <v>5288141247</v>
@@ -10026,7 +10026,7 @@
         <v>1.05</v>
       </c>
       <c r="M42" t="n">
-        <v>1.253265789367399</v>
+        <v>1.302144525311048</v>
       </c>
       <c r="N42" t="n">
         <v>0.08</v>
@@ -10104,7 +10104,7 @@
         <v>12268487693.04</v>
       </c>
       <c r="AM42" t="n">
-        <v>25511325556.59864</v>
+        <v>26506295144.08163</v>
       </c>
       <c r="AN42" t="n">
         <v>1.8491</v>
@@ -10145,7 +10145,7 @@
         <v>24.4</v>
       </c>
       <c r="AZ42" t="n">
-        <v>25.75</v>
+        <v>26.81</v>
       </c>
       <c r="BA42" t="n">
         <v>2.53</v>
@@ -10154,25 +10154,25 @@
         <v>15.11</v>
       </c>
       <c r="BC42" t="n">
-        <v>68.08</v>
+        <v>61.46</v>
       </c>
       <c r="BD42" t="n">
-        <v>37.24</v>
+        <v>31.83</v>
       </c>
       <c r="BE42" t="n">
         <v>44.83</v>
       </c>
       <c r="BF42" t="n">
-        <v>-85.79000000000001</v>
+        <v>-86.34999999999999</v>
       </c>
       <c r="BG42" t="n">
-        <v>-14.99</v>
+        <v>-18.34</v>
       </c>
       <c r="BH42" t="n">
         <v>17.11</v>
       </c>
       <c r="BI42" t="n">
-        <v>0</v>
+        <v>4.11</v>
       </c>
       <c r="BJ42" t="n">
         <v>17.78</v>
@@ -10184,7 +10184,7 @@
         <v>2.34</v>
       </c>
       <c r="BM42" t="n">
-        <v>17.78</v>
+        <v>18.54</v>
       </c>
       <c r="BN42" t="n">
         <v>21.33</v>
@@ -10193,19 +10193,19 @@
         <v>15.67</v>
       </c>
       <c r="BP42" t="n">
-        <v>17.49</v>
+        <v>17.97</v>
       </c>
       <c r="BQ42" t="n">
-        <v>7.61</v>
+        <v>7.92</v>
       </c>
       <c r="BR42" t="n">
-        <v>17.63</v>
+        <v>18.15</v>
       </c>
       <c r="BS42" t="n">
         <v>0.63</v>
       </c>
       <c r="BT42" t="n">
-        <v>39949597</v>
+        <v>40003400</v>
       </c>
     </row>
     <row r="43">
@@ -10235,13 +10235,13 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>38.76</v>
+        <v>39.18</v>
       </c>
       <c r="G43" t="n">
-        <v>75248621981</v>
+        <v>76064013412</v>
       </c>
       <c r="H43" t="n">
-        <v>4567700</v>
+        <v>0</v>
       </c>
       <c r="I43" t="n">
         <v>1941400000</v>
@@ -10334,7 +10334,7 @@
         <v>9182822000</v>
       </c>
       <c r="AM43" t="n">
-        <v>9165483797.929354</v>
+        <v>9264800659.196102</v>
       </c>
       <c r="AN43" t="n">
         <v>4.5901</v>
@@ -10375,7 +10375,7 @@
         <v>19.95</v>
       </c>
       <c r="AZ43" t="n">
-        <v>70.34999999999999</v>
+        <v>71.11</v>
       </c>
       <c r="BA43" t="n">
         <v>5.63</v>
@@ -10384,25 +10384,25 @@
         <v>48.62</v>
       </c>
       <c r="BC43" t="n">
-        <v>-36.96</v>
+        <v>-37.64</v>
       </c>
       <c r="BD43" t="n">
-        <v>-48.53</v>
+        <v>-49.08</v>
       </c>
       <c r="BE43" t="n">
         <v>81.5</v>
       </c>
       <c r="BF43" t="n">
-        <v>-85.48</v>
+        <v>-85.63</v>
       </c>
       <c r="BG43" t="n">
-        <v>25.43</v>
+        <v>24.09</v>
       </c>
       <c r="BH43" t="n">
         <v>5.61</v>
       </c>
       <c r="BI43" t="n">
-        <v>0</v>
+        <v>1.08</v>
       </c>
       <c r="BJ43" t="n">
         <v>38.76</v>
@@ -10414,7 +10414,7 @@
         <v>4.73</v>
       </c>
       <c r="BM43" t="n">
-        <v>38.97</v>
+        <v>39.49</v>
       </c>
       <c r="BN43" t="n">
         <v>42.98</v>
@@ -10423,19 +10423,19 @@
         <v>28.06</v>
       </c>
       <c r="BP43" t="n">
-        <v>38.24</v>
+        <v>38.92</v>
       </c>
       <c r="BQ43" t="n">
-        <v>8.19</v>
+        <v>8.279999999999999</v>
       </c>
       <c r="BR43" t="n">
-        <v>38.44</v>
+        <v>39.09</v>
       </c>
       <c r="BS43" t="n">
         <v>0</v>
       </c>
       <c r="BT43" t="n">
-        <v>6273510</v>
+        <v>6310687</v>
       </c>
     </row>
     <row r="44">
@@ -10925,13 +10925,13 @@
         </is>
       </c>
       <c r="F46" t="n">
-        <v>3.92</v>
+        <v>3.94</v>
       </c>
       <c r="G46" t="n">
-        <v>3922124716</v>
+        <v>3942135537</v>
       </c>
       <c r="H46" t="n">
-        <v>15110100</v>
+        <v>0</v>
       </c>
       <c r="I46" t="n">
         <v>1000542188</v>
@@ -10946,7 +10946,7 @@
         <v>2.5</v>
       </c>
       <c r="M46" t="n">
-        <v>0.0681739015547508</v>
+        <v>0.06852172724609572</v>
       </c>
       <c r="N46" t="n">
         <v>0.08</v>
@@ -11024,7 +11024,7 @@
         <v>460249406.48</v>
       </c>
       <c r="AM46" t="n">
-        <v>3845220309.803922</v>
+        <v>3864838761.764706</v>
       </c>
       <c r="AN46" t="n">
         <v>0.0311</v>
@@ -11065,7 +11065,7 @@
         <v>3.3</v>
       </c>
       <c r="AZ46" t="n">
-        <v>3.23</v>
+        <v>3.25</v>
       </c>
       <c r="BA46" t="n">
         <v>0.42</v>
@@ -11074,25 +11074,25 @@
         <v>7.38</v>
       </c>
       <c r="BC46" t="n">
-        <v>3.16</v>
+        <v>2.64</v>
       </c>
       <c r="BD46" t="n">
-        <v>-15.77</v>
+        <v>-16.2</v>
       </c>
       <c r="BE46" t="n">
         <v>-17.5</v>
       </c>
       <c r="BF46" t="n">
-        <v>-89.20999999999999</v>
+        <v>-89.26000000000001</v>
       </c>
       <c r="BG46" t="n">
-        <v>88.23</v>
+        <v>87.27</v>
       </c>
       <c r="BH46" t="n">
         <v>1.58</v>
       </c>
       <c r="BI46" t="n">
-        <v>0</v>
+        <v>0.51</v>
       </c>
       <c r="BJ46" t="n">
         <v>3.92</v>
@@ -11104,7 +11104,7 @@
         <v>0.46</v>
       </c>
       <c r="BM46" t="n">
-        <v>4.02</v>
+        <v>4.06</v>
       </c>
       <c r="BN46" t="n">
         <v>7.31</v>
@@ -11113,19 +11113,19 @@
         <v>2.97</v>
       </c>
       <c r="BP46" t="n">
-        <v>3.9</v>
+        <v>3.91</v>
       </c>
       <c r="BQ46" t="n">
-        <v>8.57</v>
+        <v>8.609999999999999</v>
       </c>
       <c r="BR46" t="n">
-        <v>4.02</v>
+        <v>3.96</v>
       </c>
       <c r="BS46" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="BT46" t="n">
-        <v>22182524</v>
+        <v>21865118</v>
       </c>
     </row>
     <row r="47">
@@ -11155,13 +11155,13 @@
         </is>
       </c>
       <c r="F47" t="n">
-        <v>9.06</v>
+        <v>9.130000000000001</v>
       </c>
       <c r="G47" t="n">
-        <v>3161609456</v>
+        <v>3179300680</v>
       </c>
       <c r="H47" t="n">
-        <v>4500</v>
+        <v>13500</v>
       </c>
       <c r="I47" t="n">
         <v>254106600</v>
@@ -11176,7 +11176,7 @@
         <v>1.22</v>
       </c>
       <c r="M47" t="n">
-        <v>0.7455438848638457</v>
+        <v>0.7497156790251789</v>
       </c>
       <c r="N47" t="n">
         <v>0.07000000000000001</v>
@@ -11254,7 +11254,7 @@
         <v>322715382</v>
       </c>
       <c r="AM47" t="n">
-        <v>560569052.4822695</v>
+        <v>563705794.3262411</v>
       </c>
       <c r="AN47" t="n">
         <v>0.4132</v>
@@ -11295,7 +11295,7 @@
         <v>11.74</v>
       </c>
       <c r="AZ47" t="n">
-        <v>11.9</v>
+        <v>11.99</v>
       </c>
       <c r="BA47" t="n">
         <v>1.46</v>
@@ -11304,25 +11304,25 @@
         <v>8.619999999999999</v>
       </c>
       <c r="BC47" t="n">
-        <v>58.65</v>
+        <v>57.43</v>
       </c>
       <c r="BD47" t="n">
-        <v>29.54</v>
+        <v>28.54</v>
       </c>
       <c r="BE47" t="n">
         <v>31.33</v>
       </c>
       <c r="BF47" t="n">
-        <v>-83.90000000000001</v>
+        <v>-84.03</v>
       </c>
       <c r="BG47" t="n">
-        <v>-4.86</v>
+        <v>-5.59</v>
       </c>
       <c r="BH47" t="n">
         <v>7.23</v>
       </c>
       <c r="BI47" t="n">
-        <v>0</v>
+        <v>0.77</v>
       </c>
       <c r="BJ47" t="n">
         <v>9.06</v>
@@ -11334,7 +11334,7 @@
         <v>1.28</v>
       </c>
       <c r="BM47" t="n">
-        <v>9.07</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="BN47" t="n">
         <v>9.24</v>
@@ -11343,19 +11343,19 @@
         <v>7.19</v>
       </c>
       <c r="BP47" t="n">
-        <v>8.94</v>
+        <v>9.06</v>
       </c>
       <c r="BQ47" t="n">
-        <v>7.06</v>
+        <v>7.12</v>
       </c>
       <c r="BR47" t="n">
-        <v>8.94</v>
+        <v>9.09</v>
       </c>
       <c r="BS47" t="n">
         <v>0.53</v>
       </c>
       <c r="BT47" t="n">
-        <v>10267</v>
+        <v>10017</v>
       </c>
     </row>
     <row r="48">
@@ -11385,13 +11385,13 @@
         </is>
       </c>
       <c r="F48" t="n">
-        <v>9.130000000000001</v>
+        <v>9.35</v>
       </c>
       <c r="G48" t="n">
-        <v>3161609456</v>
+        <v>3179300680</v>
       </c>
       <c r="H48" t="n">
-        <v>1400</v>
+        <v>4700</v>
       </c>
       <c r="I48" t="n">
         <v>93397546</v>
@@ -11406,7 +11406,7 @@
         <v>1.24</v>
       </c>
       <c r="M48" t="n">
-        <v>2.028400422143247</v>
+        <v>2.039750617899313</v>
       </c>
       <c r="N48" t="n">
         <v>0.07000000000000001</v>
@@ -11484,7 +11484,7 @@
         <v>118614883.42</v>
       </c>
       <c r="AM48" t="n">
-        <v>552728925.874126</v>
+        <v>555821797.2027972</v>
       </c>
       <c r="AN48" t="n">
         <v>0.4132</v>
@@ -11525,7 +11525,7 @@
         <v>11.74</v>
       </c>
       <c r="AZ48" t="n">
-        <v>11.95</v>
+        <v>12.23</v>
       </c>
       <c r="BA48" t="n">
         <v>1.46</v>
@@ -11534,25 +11534,25 @@
         <v>8.24</v>
       </c>
       <c r="BC48" t="n">
-        <v>57.43</v>
+        <v>53.73</v>
       </c>
       <c r="BD48" t="n">
-        <v>28.54</v>
+        <v>25.52</v>
       </c>
       <c r="BE48" t="n">
         <v>30.83</v>
       </c>
       <c r="BF48" t="n">
-        <v>-84.03</v>
+        <v>-84.40000000000001</v>
       </c>
       <c r="BG48" t="n">
-        <v>-9.789999999999999</v>
+        <v>-11.91</v>
       </c>
       <c r="BH48" t="n">
         <v>7.23</v>
       </c>
       <c r="BI48" t="n">
-        <v>0</v>
+        <v>2.41</v>
       </c>
       <c r="BJ48" t="n">
         <v>9.130000000000001</v>
@@ -11564,7 +11564,7 @@
         <v>1.28</v>
       </c>
       <c r="BM48" t="n">
-        <v>9.16</v>
+        <v>9.35</v>
       </c>
       <c r="BN48" t="n">
         <v>9.48</v>
@@ -11573,19 +11573,19 @@
         <v>7.2</v>
       </c>
       <c r="BP48" t="n">
-        <v>9.1</v>
+        <v>9.18</v>
       </c>
       <c r="BQ48" t="n">
-        <v>7.12</v>
+        <v>7.29</v>
       </c>
       <c r="BR48" t="n">
-        <v>9.109999999999999</v>
+        <v>9.18</v>
       </c>
       <c r="BS48" t="n">
         <v>0.54</v>
       </c>
       <c r="BT48" t="n">
-        <v>2647</v>
+        <v>2573</v>
       </c>
     </row>
     <row r="49">
@@ -11845,13 +11845,13 @@
         </is>
       </c>
       <c r="F50" t="n">
-        <v>34.25</v>
+        <v>34.6</v>
       </c>
       <c r="G50" t="n">
-        <v>952468000</v>
+        <v>958007600</v>
       </c>
       <c r="H50" t="n">
-        <v>600</v>
+        <v>100</v>
       </c>
       <c r="I50" t="n">
         <v>11540870</v>
@@ -11866,7 +11866,7 @@
         <v>0.8</v>
       </c>
       <c r="M50" t="n">
-        <v>0.9635995901677982</v>
+        <v>0.9692039320351298</v>
       </c>
       <c r="N50" t="n">
         <v>0.06</v>
@@ -11944,7 +11944,7 @@
         <v>84709985.8</v>
       </c>
       <c r="AM50" t="n">
-        <v>325074402.7303754</v>
+        <v>326965051.1945392</v>
       </c>
       <c r="AN50" t="n">
         <v>4.4983</v>
@@ -11985,7 +11985,7 @@
         <v>68.48999999999999</v>
       </c>
       <c r="AZ50" t="n">
-        <v>75.52</v>
+        <v>76.29000000000001</v>
       </c>
       <c r="BA50" t="n">
         <v>9.210000000000001</v>
@@ -11994,25 +11994,25 @@
         <v>30.53</v>
       </c>
       <c r="BC50" t="n">
-        <v>144.9</v>
+        <v>142.42</v>
       </c>
       <c r="BD50" t="n">
-        <v>99.95999999999999</v>
+        <v>97.93000000000001</v>
       </c>
       <c r="BE50" t="n">
         <v>120.5</v>
       </c>
       <c r="BF50" t="n">
-        <v>-73.09999999999999</v>
+        <v>-73.37</v>
       </c>
       <c r="BG50" t="n">
-        <v>-10.86</v>
+        <v>-11.76</v>
       </c>
       <c r="BH50" t="n">
         <v>42.6</v>
       </c>
       <c r="BI50" t="n">
-        <v>0</v>
+        <v>1.02</v>
       </c>
       <c r="BJ50" t="n">
         <v>34.25</v>
@@ -12024,7 +12024,7 @@
         <v>7.6</v>
       </c>
       <c r="BM50" t="n">
-        <v>34.3</v>
+        <v>34.6</v>
       </c>
       <c r="BN50" t="n">
         <v>39.22</v>
@@ -12033,19 +12033,19 @@
         <v>23.5</v>
       </c>
       <c r="BP50" t="n">
-        <v>34.25</v>
+        <v>34.6</v>
       </c>
       <c r="BQ50" t="n">
-        <v>4.51</v>
+        <v>4.55</v>
       </c>
       <c r="BR50" t="n">
-        <v>34.26</v>
+        <v>34.6</v>
       </c>
       <c r="BS50" t="n">
         <v>0.4</v>
       </c>
       <c r="BT50" t="n">
-        <v>503</v>
+        <v>510</v>
       </c>
     </row>
     <row r="51">
@@ -12523,13 +12523,13 @@
         </is>
       </c>
       <c r="F53" t="n">
-        <v>5.88</v>
+        <v>6.1</v>
       </c>
       <c r="G53" t="n">
-        <v>804692127</v>
+        <v>834799626</v>
       </c>
       <c r="H53" t="n">
-        <v>39600</v>
+        <v>55200</v>
       </c>
       <c r="I53" t="n">
         <v>136852484</v>
@@ -12544,7 +12544,7 @@
         <v>2.79</v>
       </c>
       <c r="M53" t="n">
-        <v>2.090440135165465</v>
+        <v>2.168653804924725</v>
       </c>
       <c r="N53" t="n">
         <v>1.48</v>
@@ -12622,7 +12622,7 @@
         <v>39687220.36</v>
       </c>
       <c r="AM53" t="n">
-        <v>40992976.41365258</v>
+        <v>42526725.7259297</v>
       </c>
       <c r="AN53" t="n">
         <v>0</v>
@@ -12672,16 +12672,16 @@
         <v>0</v>
       </c>
       <c r="BC53" t="n">
-        <v>-32.98</v>
+        <v>-35.4</v>
       </c>
       <c r="BD53" t="n">
-        <v>-45.28</v>
+        <v>-47.25</v>
       </c>
       <c r="BE53" t="n">
         <v>-100</v>
       </c>
       <c r="BF53" t="n">
-        <v>-95.06999999999999</v>
+        <v>-95.25</v>
       </c>
       <c r="BG53" t="n">
         <v>-100</v>
@@ -12690,7 +12690,7 @@
         <v>2.38</v>
       </c>
       <c r="BI53" t="n">
-        <v>0</v>
+        <v>3.74</v>
       </c>
       <c r="BJ53" t="n">
         <v>5.88</v>
@@ -12702,7 +12702,7 @@
         <v>0.2</v>
       </c>
       <c r="BM53" t="n">
-        <v>6.3</v>
+        <v>6.1</v>
       </c>
       <c r="BN53" t="n">
         <v>10.39</v>
@@ -12711,19 +12711,19 @@
         <v>4.82</v>
       </c>
       <c r="BP53" t="n">
-        <v>5.77</v>
+        <v>5.78</v>
       </c>
       <c r="BQ53" t="n">
-        <v>28.88</v>
+        <v>29.96</v>
       </c>
       <c r="BR53" t="n">
-        <v>6.04</v>
+        <v>5.98</v>
       </c>
       <c r="BS53" t="n">
         <v>2.36</v>
       </c>
       <c r="BT53" t="n">
-        <v>35577</v>
+        <v>34733</v>
       </c>
     </row>
     <row r="54">
@@ -12753,13 +12753,13 @@
         </is>
       </c>
       <c r="F54" t="n">
-        <v>10.51</v>
+        <v>10.71</v>
       </c>
       <c r="G54" t="n">
-        <v>2451059224</v>
+        <v>2497700528</v>
       </c>
       <c r="H54" t="n">
-        <v>159400</v>
+        <v>287200</v>
       </c>
       <c r="I54" t="n">
         <v>233212121</v>
@@ -12774,7 +12774,7 @@
         <v>0.97</v>
       </c>
       <c r="M54" t="n">
-        <v>1.375758905865789</v>
+        <v>1.40193827710696</v>
       </c>
       <c r="N54" t="n">
         <v>0.5600000000000001</v>
@@ -12852,7 +12852,7 @@
         <v>233212121</v>
       </c>
       <c r="AM54" t="n">
-        <v>335302219.4254446</v>
+        <v>341682698.7688099</v>
       </c>
       <c r="AN54" t="n">
         <v>0.1531</v>
@@ -12893,7 +12893,7 @@
         <v>12.25</v>
       </c>
       <c r="AZ54" t="n">
-        <v>16.73</v>
+        <v>17.05</v>
       </c>
       <c r="BA54" t="n">
         <v>0.98</v>
@@ -12902,25 +12902,25 @@
         <v>6.52</v>
       </c>
       <c r="BC54" t="n">
-        <v>42.79</v>
+        <v>40.13</v>
       </c>
       <c r="BD54" t="n">
-        <v>16.59</v>
+        <v>14.41</v>
       </c>
       <c r="BE54" t="n">
         <v>59.17</v>
       </c>
       <c r="BF54" t="n">
-        <v>-90.64</v>
+        <v>-90.81999999999999</v>
       </c>
       <c r="BG54" t="n">
-        <v>-38</v>
+        <v>-39.16</v>
       </c>
       <c r="BH54" t="n">
         <v>10.01</v>
       </c>
       <c r="BI54" t="n">
-        <v>0.6</v>
+        <v>2.51</v>
       </c>
       <c r="BJ54" t="n">
         <v>10.45</v>
@@ -12932,28 +12932,28 @@
         <v>1</v>
       </c>
       <c r="BM54" t="n">
-        <v>10.55</v>
+        <v>10.73</v>
       </c>
       <c r="BN54" t="n">
-        <v>11.66</v>
+        <v>11.68</v>
       </c>
       <c r="BO54" t="n">
-        <v>8.220000000000001</v>
+        <v>8.23</v>
       </c>
       <c r="BP54" t="n">
-        <v>10.13</v>
+        <v>10.39</v>
       </c>
       <c r="BQ54" t="n">
-        <v>10.48</v>
+        <v>10.68</v>
       </c>
       <c r="BR54" t="n">
-        <v>10.13</v>
+        <v>10.5</v>
       </c>
       <c r="BS54" t="n">
         <v>1.26</v>
       </c>
       <c r="BT54" t="n">
-        <v>242710</v>
+        <v>240917</v>
       </c>
     </row>
     <row r="55">
@@ -12983,13 +12983,13 @@
         </is>
       </c>
       <c r="F55" t="n">
-        <v>49.3</v>
+        <v>49.48</v>
       </c>
       <c r="G55" t="n">
-        <v>6504739356</v>
+        <v>6599884943</v>
       </c>
       <c r="H55" t="n">
-        <v>1700</v>
+        <v>2900</v>
       </c>
       <c r="I55" t="n">
         <v>84052790</v>
@@ -13004,7 +13004,7 @@
         <v>2</v>
       </c>
       <c r="M55" t="n">
-        <v>1.004144149567131</v>
+        <v>1.018831884050305</v>
       </c>
       <c r="N55" t="n">
         <v>0.16</v>
@@ -13082,7 +13082,7 @@
         <v>579123723.1</v>
       </c>
       <c r="AM55" t="n">
-        <v>327200168.8128773</v>
+        <v>331986164.1348089</v>
       </c>
       <c r="AN55" t="n">
         <v>3.1953</v>
@@ -13123,7 +13123,7 @@
         <v>51.21</v>
       </c>
       <c r="AZ55" t="n">
-        <v>51.85</v>
+        <v>52.04</v>
       </c>
       <c r="BA55" t="n">
         <v>9.380000000000001</v>
@@ -13132,25 +13132,25 @@
         <v>16.08</v>
       </c>
       <c r="BC55" t="n">
-        <v>27.21</v>
+        <v>26.75</v>
       </c>
       <c r="BD55" t="n">
-        <v>3.86</v>
+        <v>3.49</v>
       </c>
       <c r="BE55" t="n">
         <v>5.17</v>
       </c>
       <c r="BF55" t="n">
-        <v>-80.98</v>
+        <v>-81.05</v>
       </c>
       <c r="BG55" t="n">
-        <v>-67.39</v>
+        <v>-67.51000000000001</v>
       </c>
       <c r="BH55" t="n">
         <v>25.37</v>
       </c>
       <c r="BI55" t="n">
-        <v>0</v>
+        <v>0.37</v>
       </c>
       <c r="BJ55" t="n">
         <v>49.3</v>
@@ -13162,7 +13162,7 @@
         <v>7.03</v>
       </c>
       <c r="BM55" t="n">
-        <v>49.76</v>
+        <v>49.61</v>
       </c>
       <c r="BN55" t="n">
         <v>73.67</v>
@@ -13171,19 +13171,19 @@
         <v>35.58</v>
       </c>
       <c r="BP55" t="n">
-        <v>49.12</v>
+        <v>49.4</v>
       </c>
       <c r="BQ55" t="n">
-        <v>7.01</v>
+        <v>7.04</v>
       </c>
       <c r="BR55" t="n">
-        <v>49.76</v>
+        <v>49.42</v>
       </c>
       <c r="BS55" t="n">
         <v>0.66</v>
       </c>
       <c r="BT55" t="n">
-        <v>6143</v>
+        <v>5943</v>
       </c>
     </row>
     <row r="56">
@@ -13213,13 +13213,13 @@
         </is>
       </c>
       <c r="F56" t="n">
-        <v>58.39</v>
+        <v>59.65</v>
       </c>
       <c r="G56" t="n">
-        <v>6504739356</v>
+        <v>6599884943</v>
       </c>
       <c r="H56" t="n">
-        <v>15100</v>
+        <v>17600</v>
       </c>
       <c r="I56" t="n">
         <v>39675836</v>
@@ -13234,7 +13234,7 @@
         <v>2.41</v>
       </c>
       <c r="M56" t="n">
-        <v>2.127267522057875</v>
+        <v>2.158383314100417</v>
       </c>
       <c r="N56" t="n">
         <v>0.19</v>
@@ -13312,7 +13312,7 @@
         <v>273366510.04</v>
       </c>
       <c r="AM56" t="n">
-        <v>270579840.0998336</v>
+        <v>274537643.2196339</v>
       </c>
       <c r="AN56" t="n">
         <v>3.5102</v>
@@ -13353,7 +13353,7 @@
         <v>51.21</v>
       </c>
       <c r="AZ56" t="n">
-        <v>55.76</v>
+        <v>56.97</v>
       </c>
       <c r="BA56" t="n">
         <v>9.380000000000001</v>
@@ -13362,25 +13362,25 @@
         <v>17.68</v>
       </c>
       <c r="BC56" t="n">
-        <v>7.4</v>
+        <v>5.14</v>
       </c>
       <c r="BD56" t="n">
-        <v>-12.3</v>
+        <v>-14.16</v>
       </c>
       <c r="BE56" t="n">
         <v>-4.5</v>
       </c>
       <c r="BF56" t="n">
-        <v>-83.94</v>
+        <v>-84.28</v>
       </c>
       <c r="BG56" t="n">
-        <v>-69.73</v>
+        <v>-70.36</v>
       </c>
       <c r="BH56" t="n">
         <v>25.37</v>
       </c>
       <c r="BI56" t="n">
-        <v>0</v>
+        <v>2.16</v>
       </c>
       <c r="BJ56" t="n">
         <v>58.39</v>
@@ -13392,7 +13392,7 @@
         <v>7.03</v>
       </c>
       <c r="BM56" t="n">
-        <v>58.39</v>
+        <v>59.94</v>
       </c>
       <c r="BN56" t="n">
         <v>86.77</v>
@@ -13401,19 +13401,19 @@
         <v>46.42</v>
       </c>
       <c r="BP56" t="n">
-        <v>57</v>
+        <v>57.57</v>
       </c>
       <c r="BQ56" t="n">
-        <v>8.300000000000001</v>
+        <v>8.48</v>
       </c>
       <c r="BR56" t="n">
-        <v>58.08</v>
+        <v>57.57</v>
       </c>
       <c r="BS56" t="n">
         <v>0.79</v>
       </c>
       <c r="BT56" t="n">
-        <v>29643</v>
+        <v>29353</v>
       </c>
     </row>
     <row r="57">
@@ -13443,13 +13443,13 @@
         </is>
       </c>
       <c r="F57" t="n">
-        <v>6.08</v>
+        <v>6.38</v>
       </c>
       <c r="G57" t="n">
-        <v>1421857230</v>
+        <v>1492014066</v>
       </c>
       <c r="H57" t="n">
-        <v>1984400</v>
+        <v>2314300</v>
       </c>
       <c r="I57" t="n">
         <v>233858065</v>
@@ -13464,7 +13464,7 @@
         <v>0.77</v>
       </c>
       <c r="M57" t="n">
-        <v>0.4256000583088722</v>
+        <v>0.44659988365165</v>
       </c>
       <c r="N57" t="n">
         <v>0.08</v>
@@ -13542,7 +13542,7 @@
         <v>229180903.7</v>
       </c>
       <c r="AM57" t="n">
-        <v>106346838.4442782</v>
+        <v>111594170.9798055</v>
       </c>
       <c r="AN57" t="n">
         <v>0.347</v>
@@ -13583,7 +13583,7 @@
         <v>10.72</v>
       </c>
       <c r="AZ57" t="n">
-        <v>9.27</v>
+        <v>9.73</v>
       </c>
       <c r="BA57" t="n">
         <v>1.13</v>
@@ -13592,25 +13592,25 @@
         <v>6.26</v>
       </c>
       <c r="BC57" t="n">
-        <v>115.98</v>
+        <v>105.82</v>
       </c>
       <c r="BD57" t="n">
-        <v>76.34</v>
+        <v>68.05</v>
       </c>
       <c r="BE57" t="n">
         <v>52.5</v>
       </c>
       <c r="BF57" t="n">
-        <v>-81.45999999999999</v>
+        <v>-82.33</v>
       </c>
       <c r="BG57" t="n">
-        <v>3.02</v>
+        <v>-1.82</v>
       </c>
       <c r="BH57" t="n">
         <v>7.82</v>
       </c>
       <c r="BI57" t="n">
-        <v>0</v>
+        <v>4.93</v>
       </c>
       <c r="BJ57" t="n">
         <v>6.08</v>
@@ -13622,28 +13622,28 @@
         <v>1.04</v>
       </c>
       <c r="BM57" t="n">
-        <v>6.08</v>
+        <v>6.38</v>
       </c>
       <c r="BN57" t="n">
-        <v>6.22</v>
+        <v>6.38</v>
       </c>
       <c r="BO57" t="n">
         <v>3.43</v>
       </c>
       <c r="BP57" t="n">
-        <v>5.91</v>
+        <v>6.1</v>
       </c>
       <c r="BQ57" t="n">
-        <v>5.87</v>
+        <v>6.16</v>
       </c>
       <c r="BR57" t="n">
-        <v>5.95</v>
+        <v>6.12</v>
       </c>
       <c r="BS57" t="n">
         <v>0.42</v>
       </c>
       <c r="BT57" t="n">
-        <v>1346880</v>
+        <v>1306047</v>
       </c>
     </row>
     <row r="58">
@@ -13676,7 +13676,7 @@
         <v>19.5</v>
       </c>
       <c r="G58" t="n">
-        <v>93644010</v>
+        <v>91920060</v>
       </c>
       <c r="H58" t="n">
         <v>0</v>
@@ -13694,7 +13694,7 @@
         <v>0.63</v>
       </c>
       <c r="M58" t="n">
-        <v>1.716607744826809</v>
+        <v>1.685005660276028</v>
       </c>
       <c r="N58" t="n">
         <v>0.16</v>
@@ -13772,7 +13772,7 @@
         <v>10904901.05</v>
       </c>
       <c r="AM58" t="n">
-        <v>15276347.47145188</v>
+        <v>14995115.82381729</v>
       </c>
       <c r="AN58" t="n">
         <v>0.5117</v>
@@ -13852,22 +13852,22 @@
         <v>2.65</v>
       </c>
       <c r="BM58" t="n">
-        <v>0</v>
+        <v>19.5</v>
       </c>
       <c r="BN58" t="n">
-        <v>22.46</v>
+        <v>21.49</v>
       </c>
       <c r="BO58" t="n">
         <v>19.5</v>
       </c>
       <c r="BP58" t="n">
-        <v>0</v>
+        <v>19.5</v>
       </c>
       <c r="BQ58" t="n">
         <v>7.35</v>
       </c>
       <c r="BR58" t="n">
-        <v>0</v>
+        <v>19.5</v>
       </c>
       <c r="BS58" t="n">
         <v>1.47</v>
@@ -13903,13 +13903,13 @@
         </is>
       </c>
       <c r="F59" t="n">
-        <v>19.05</v>
+        <v>20.45</v>
       </c>
       <c r="G59" t="n">
         <v>91920060</v>
       </c>
       <c r="H59" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="I59" t="n">
         <v>710143</v>
@@ -14043,7 +14043,7 @@
         <v>35.09</v>
       </c>
       <c r="AZ59" t="n">
-        <v>23.56</v>
+        <v>25.29</v>
       </c>
       <c r="BA59" t="n">
         <v>3.69</v>
@@ -14052,25 +14052,25 @@
         <v>22.8</v>
       </c>
       <c r="BC59" t="n">
-        <v>125.61</v>
+        <v>110.17</v>
       </c>
       <c r="BD59" t="n">
-        <v>84.20999999999999</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="BE59" t="n">
         <v>23.67</v>
       </c>
       <c r="BF59" t="n">
-        <v>-80.64</v>
+        <v>-81.97</v>
       </c>
       <c r="BG59" t="n">
-        <v>19.67</v>
+        <v>11.48</v>
       </c>
       <c r="BH59" t="n">
         <v>30.98</v>
       </c>
       <c r="BI59" t="n">
-        <v>0</v>
+        <v>7.35</v>
       </c>
       <c r="BJ59" t="n">
         <v>19.05</v>
@@ -14082,7 +14082,7 @@
         <v>2.65</v>
       </c>
       <c r="BM59" t="n">
-        <v>19.05</v>
+        <v>20.45</v>
       </c>
       <c r="BN59" t="n">
         <v>25.98</v>
@@ -14091,19 +14091,19 @@
         <v>15.85</v>
       </c>
       <c r="BP59" t="n">
-        <v>19.05</v>
+        <v>20.45</v>
       </c>
       <c r="BQ59" t="n">
-        <v>7.18</v>
+        <v>7.71</v>
       </c>
       <c r="BR59" t="n">
-        <v>19.05</v>
+        <v>20.45</v>
       </c>
       <c r="BS59" t="n">
         <v>1.42</v>
       </c>
       <c r="BT59" t="n">
-        <v>133</v>
+        <v>130</v>
       </c>
     </row>
     <row r="60">
@@ -14133,13 +14133,13 @@
         </is>
       </c>
       <c r="F60" t="n">
-        <v>379.81</v>
+        <v>378</v>
       </c>
       <c r="G60" t="n">
-        <v>172718596</v>
+        <v>171895500</v>
       </c>
       <c r="H60" t="n">
-        <v>21</v>
+        <v>64</v>
       </c>
       <c r="I60" t="n">
         <v>454750</v>
@@ -14154,7 +14154,7 @@
         <v>0.83</v>
       </c>
       <c r="M60" t="n">
-        <v>12.91910784382257</v>
+        <v>12.85754142169963</v>
       </c>
       <c r="N60" t="n">
         <v>0.68</v>
@@ -14232,7 +14232,7 @@
         <v>59558607.5</v>
       </c>
       <c r="AM60" t="n">
-        <v>-25325307.3313783</v>
+        <v>-25204618.76832844</v>
       </c>
       <c r="AN60" t="n">
         <v>10.0581</v>
@@ -14273,7 +14273,7 @@
         <v>944.87</v>
       </c>
       <c r="AZ60" t="n">
-        <v>2183.91</v>
+        <v>2173.5</v>
       </c>
       <c r="BA60" t="n">
         <v>231.1</v>
@@ -14282,25 +14282,25 @@
         <v>727.97</v>
       </c>
       <c r="BC60" t="n">
-        <v>204.68</v>
+        <v>206.14</v>
       </c>
       <c r="BD60" t="n">
-        <v>148.77</v>
+        <v>149.96</v>
       </c>
       <c r="BE60" t="n">
         <v>475</v>
       </c>
       <c r="BF60" t="n">
-        <v>-39.15</v>
+        <v>-38.86</v>
       </c>
       <c r="BG60" t="n">
-        <v>91.67</v>
+        <v>92.59</v>
       </c>
       <c r="BH60" t="n">
         <v>454.44</v>
       </c>
       <c r="BI60" t="n">
-        <v>0</v>
+        <v>-0.48</v>
       </c>
       <c r="BJ60" t="n">
         <v>379.81</v>
@@ -14312,7 +14312,7 @@
         <v>130.97</v>
       </c>
       <c r="BM60" t="n">
-        <v>383.95</v>
+        <v>380</v>
       </c>
       <c r="BN60" t="n">
         <v>405</v>
@@ -14321,19 +14321,19 @@
         <v>309.24</v>
       </c>
       <c r="BP60" t="n">
-        <v>379.76</v>
+        <v>378</v>
       </c>
       <c r="BQ60" t="n">
-        <v>2.9</v>
+        <v>2.89</v>
       </c>
       <c r="BR60" t="n">
-        <v>383.95</v>
+        <v>379.81</v>
       </c>
       <c r="BS60" t="n">
         <v>12.82</v>
       </c>
       <c r="BT60" t="n">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="61">
@@ -14363,13 +14363,13 @@
         </is>
       </c>
       <c r="F61" t="n">
-        <v>27.64</v>
+        <v>28.15</v>
       </c>
       <c r="G61" t="n">
-        <v>2366215570</v>
+        <v>2409876145</v>
       </c>
       <c r="H61" t="n">
-        <v>2082900</v>
+        <v>0</v>
       </c>
       <c r="I61" t="n">
         <v>85608392</v>
@@ -14384,7 +14384,7 @@
         <v>2.37</v>
       </c>
       <c r="M61" t="n">
-        <v>1.254885357382248</v>
+        <v>1.278040059327848</v>
       </c>
       <c r="N61" t="n">
         <v>1.1</v>
@@ -14462,7 +14462,7 @@
         <v>160087693.04</v>
       </c>
       <c r="AM61" t="n">
-        <v>185731206.4364207</v>
+        <v>189158253.1397174</v>
       </c>
       <c r="AN61" t="n">
         <v>0.38</v>
@@ -14503,7 +14503,7 @@
         <v>17.56</v>
       </c>
       <c r="AZ61" t="n">
-        <v>34.83</v>
+        <v>35.47</v>
       </c>
       <c r="BA61" t="n">
         <v>2.52</v>
@@ -14512,25 +14512,25 @@
         <v>11.76</v>
       </c>
       <c r="BC61" t="n">
-        <v>-22.2</v>
+        <v>-23.61</v>
       </c>
       <c r="BD61" t="n">
-        <v>-36.48</v>
+        <v>-37.63</v>
       </c>
       <c r="BE61" t="n">
         <v>26</v>
       </c>
       <c r="BF61" t="n">
-        <v>-90.87</v>
+        <v>-91.04000000000001</v>
       </c>
       <c r="BG61" t="n">
-        <v>-57.47</v>
+        <v>-58.24</v>
       </c>
       <c r="BH61" t="n">
         <v>10.99</v>
       </c>
       <c r="BI61" t="n">
-        <v>0</v>
+        <v>1.85</v>
       </c>
       <c r="BJ61" t="n">
         <v>27.64</v>
@@ -14542,7 +14542,7 @@
         <v>1.86</v>
       </c>
       <c r="BM61" t="n">
-        <v>27.81</v>
+        <v>28.65</v>
       </c>
       <c r="BN61" t="n">
         <v>28.68</v>
@@ -14551,19 +14551,19 @@
         <v>19.35</v>
       </c>
       <c r="BP61" t="n">
-        <v>27.09</v>
+        <v>27.78</v>
       </c>
       <c r="BQ61" t="n">
-        <v>14.84</v>
+        <v>15.12</v>
       </c>
       <c r="BR61" t="n">
-        <v>27.19</v>
+        <v>27.86</v>
       </c>
       <c r="BS61" t="n">
         <v>1.19</v>
       </c>
       <c r="BT61" t="n">
-        <v>589013</v>
+        <v>642187</v>
       </c>
     </row>
     <row r="62">
@@ -14593,13 +14593,13 @@
         </is>
       </c>
       <c r="F62" t="n">
-        <v>108.02</v>
+        <v>110</v>
       </c>
       <c r="G62" t="n">
-        <v>10661548824</v>
+        <v>10856974700</v>
       </c>
       <c r="H62" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="I62" t="n">
         <v>98699749</v>
@@ -14614,7 +14614,7 @@
         <v>0.64</v>
       </c>
       <c r="M62" t="n">
-        <v>0.9993978193686657</v>
+        <v>1.017716751969055</v>
       </c>
       <c r="N62" t="n">
         <v>0.13</v>
@@ -14692,7 +14692,7 @@
         <v>2757670987.06</v>
       </c>
       <c r="AM62" t="n">
-        <v>4316416527.935223</v>
+        <v>4395536315.789474</v>
       </c>
       <c r="AN62" t="n">
         <v>6.9319</v>
@@ -14733,7 +14733,7 @@
         <v>267.2</v>
       </c>
       <c r="AZ62" t="n">
-        <v>114.14</v>
+        <v>116.23</v>
       </c>
       <c r="BA62" t="n">
         <v>34.09</v>
@@ -14742,25 +14742,25 @@
         <v>76.01000000000001</v>
       </c>
       <c r="BC62" t="n">
-        <v>202.95</v>
+        <v>197.5</v>
       </c>
       <c r="BD62" t="n">
-        <v>147.36</v>
+        <v>142.91</v>
       </c>
       <c r="BE62" t="n">
         <v>5.67</v>
       </c>
       <c r="BF62" t="n">
-        <v>-68.44</v>
+        <v>-69.01000000000001</v>
       </c>
       <c r="BG62" t="n">
-        <v>-29.64</v>
+        <v>-30.9</v>
       </c>
       <c r="BH62" t="n">
         <v>170.35</v>
       </c>
       <c r="BI62" t="n">
-        <v>0</v>
+        <v>1.83</v>
       </c>
       <c r="BJ62" t="n">
         <v>108.02</v>
@@ -14772,7 +14772,7 @@
         <v>32.73</v>
       </c>
       <c r="BM62" t="n">
-        <v>109.14</v>
+        <v>110</v>
       </c>
       <c r="BN62" t="n">
         <v>122.2</v>
@@ -14781,19 +14781,19 @@
         <v>91.84999999999999</v>
       </c>
       <c r="BP62" t="n">
-        <v>108.02</v>
+        <v>110</v>
       </c>
       <c r="BQ62" t="n">
-        <v>3.3</v>
+        <v>3.36</v>
       </c>
       <c r="BR62" t="n">
-        <v>109.14</v>
+        <v>110</v>
       </c>
       <c r="BS62" t="n">
         <v>1.01</v>
       </c>
       <c r="BT62" t="n">
-        <v>173</v>
+        <v>157</v>
       </c>
     </row>
     <row r="63">
@@ -14823,13 +14823,13 @@
         </is>
       </c>
       <c r="F63" t="n">
-        <v>1.44</v>
+        <v>1.6</v>
       </c>
       <c r="G63" t="n">
-        <v>375133982</v>
+        <v>416815526</v>
       </c>
       <c r="H63" t="n">
-        <v>24100</v>
+        <v>117200</v>
       </c>
       <c r="I63" t="n">
         <v>122894462</v>
@@ -14844,7 +14844,7 @@
         <v>-0.22</v>
       </c>
       <c r="M63" t="n">
-        <v>0.4613954386513177</v>
+        <v>0.5126615867486239</v>
       </c>
       <c r="N63" t="n">
         <v>0.37</v>
@@ -14922,7 +14922,7 @@
         <v>31952560.12</v>
       </c>
       <c r="AM63" t="n">
-        <v>213144307.9545455</v>
+        <v>236827003.4090909</v>
       </c>
       <c r="AN63" t="n">
         <v>0</v>
@@ -14981,7 +14981,7 @@
         <v>-100</v>
       </c>
       <c r="BF63" t="n">
-        <v>-79.92</v>
+        <v>-81.93000000000001</v>
       </c>
       <c r="BG63" t="n">
         <v>-100</v>
@@ -14990,7 +14990,7 @@
         <v>-5.91</v>
       </c>
       <c r="BI63" t="n">
-        <v>0</v>
+        <v>11.11</v>
       </c>
       <c r="BJ63" t="n">
         <v>1.44</v>
@@ -15002,7 +15002,7 @@
         <v>0.26</v>
       </c>
       <c r="BM63" t="n">
-        <v>1.55</v>
+        <v>1.6</v>
       </c>
       <c r="BN63" t="n">
         <v>2.12</v>
@@ -15011,19 +15011,19 @@
         <v>1.16</v>
       </c>
       <c r="BP63" t="n">
-        <v>1.41</v>
+        <v>1.46</v>
       </c>
       <c r="BQ63" t="n">
-        <v>5.52</v>
+        <v>6.13</v>
       </c>
       <c r="BR63" t="n">
-        <v>1.41</v>
+        <v>1.54</v>
       </c>
       <c r="BS63" t="n">
         <v>0.19</v>
       </c>
       <c r="BT63" t="n">
-        <v>27353</v>
+        <v>27770</v>
       </c>
     </row>
     <row r="64">
@@ -15053,13 +15053,13 @@
         </is>
       </c>
       <c r="F64" t="n">
-        <v>62.85</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="G64" t="n">
-        <v>240198552918</v>
+        <v>243047964214</v>
       </c>
       <c r="H64" t="n">
-        <v>11437000</v>
+        <v>0</v>
       </c>
       <c r="I64" t="n">
         <v>0</v>
@@ -15146,13 +15146,13 @@
         <v>41.22</v>
       </c>
       <c r="AK64" t="n">
-        <v>68868449836.4006</v>
+        <v>69685417867.71443</v>
       </c>
       <c r="AL64" t="n">
-        <v>19200523814.38849</v>
+        <v>19428294501.51878</v>
       </c>
       <c r="AM64" t="n">
-        <v>21389007383.61531</v>
+        <v>21642739466.96349</v>
       </c>
       <c r="AN64" t="n">
         <v>1.4201</v>
@@ -15193,7 +15193,7 @@
         <v>38.98</v>
       </c>
       <c r="AZ64" t="n">
-        <v>25.14</v>
+        <v>25.64</v>
       </c>
       <c r="BA64" t="n">
         <v>6.69</v>
@@ -15202,25 +15202,25 @@
         <v>10.4</v>
       </c>
       <c r="BC64" t="n">
-        <v>-24.04</v>
+        <v>-25.52</v>
       </c>
       <c r="BD64" t="n">
-        <v>-37.98</v>
+        <v>-39.19</v>
       </c>
       <c r="BE64" t="n">
         <v>-60</v>
       </c>
       <c r="BF64" t="n">
-        <v>-89.34999999999999</v>
+        <v>-89.56</v>
       </c>
       <c r="BG64" t="n">
-        <v>-83.45999999999999</v>
+        <v>-83.78</v>
       </c>
       <c r="BH64" t="n">
         <v>21.37</v>
       </c>
       <c r="BI64" t="n">
-        <v>0</v>
+        <v>1.99</v>
       </c>
       <c r="BJ64" t="n">
         <v>62.85</v>
@@ -15232,7 +15232,7 @@
         <v>1.57</v>
       </c>
       <c r="BM64" t="n">
-        <v>63.01</v>
+        <v>64.64</v>
       </c>
       <c r="BN64" t="n">
         <v>64.72</v>
@@ -15241,19 +15241,19 @@
         <v>44.12</v>
       </c>
       <c r="BP64" t="n">
-        <v>61.79</v>
+        <v>63.23</v>
       </c>
       <c r="BQ64" t="n">
-        <v>40.03</v>
+        <v>40.83</v>
       </c>
       <c r="BR64" t="n">
-        <v>62.13</v>
+        <v>64</v>
       </c>
       <c r="BS64" t="n">
         <v>3.49</v>
       </c>
       <c r="BT64" t="n">
-        <v>10323167</v>
+        <v>10222830</v>
       </c>
     </row>
     <row r="65">
@@ -15283,13 +15283,13 @@
         </is>
       </c>
       <c r="F65" t="n">
-        <v>24.2</v>
+        <v>24.8</v>
       </c>
       <c r="G65" t="n">
-        <v>240198552918</v>
+        <v>243047964214</v>
       </c>
       <c r="H65" t="n">
-        <v>1700</v>
+        <v>2800</v>
       </c>
       <c r="I65" t="n">
         <v>7298813414</v>
@@ -15304,7 +15304,7 @@
         <v>3.29</v>
       </c>
       <c r="M65" t="n">
-        <v>5.807026495661329</v>
+        <v>5.875913700400474</v>
       </c>
       <c r="N65" t="n">
         <v>0.29</v>
@@ -15382,7 +15382,7 @@
         <v>11532125194.12</v>
       </c>
       <c r="AM65" t="n">
-        <v>17992400967.64045</v>
+        <v>18205840016.02996</v>
       </c>
       <c r="AN65" t="n">
         <v>0.4734</v>
@@ -15423,7 +15423,7 @@
         <v>12.99</v>
       </c>
       <c r="AZ65" t="n">
-        <v>8.15</v>
+        <v>8.35</v>
       </c>
       <c r="BA65" t="n">
         <v>2.23</v>
@@ -15432,25 +15432,25 @@
         <v>3.47</v>
       </c>
       <c r="BC65" t="n">
-        <v>-34.26</v>
+        <v>-35.85</v>
       </c>
       <c r="BD65" t="n">
-        <v>-46.32</v>
+        <v>-47.62</v>
       </c>
       <c r="BE65" t="n">
         <v>-66.33</v>
       </c>
       <c r="BF65" t="n">
-        <v>-90.78</v>
+        <v>-91</v>
       </c>
       <c r="BG65" t="n">
-        <v>-85.68000000000001</v>
+        <v>-86.03</v>
       </c>
       <c r="BH65" t="n">
         <v>7.12</v>
       </c>
       <c r="BI65" t="n">
-        <v>0</v>
+        <v>2.48</v>
       </c>
       <c r="BJ65" t="n">
         <v>24.2</v>
@@ -15462,7 +15462,7 @@
         <v>1.57</v>
       </c>
       <c r="BM65" t="n">
-        <v>24.27</v>
+        <v>24.8</v>
       </c>
       <c r="BN65" t="n">
         <v>46.43</v>
@@ -15471,19 +15471,19 @@
         <v>20.44</v>
       </c>
       <c r="BP65" t="n">
-        <v>23.75</v>
+        <v>24.21</v>
       </c>
       <c r="BQ65" t="n">
-        <v>15.41</v>
+        <v>15.8</v>
       </c>
       <c r="BR65" t="n">
-        <v>23.95</v>
+        <v>24.5</v>
       </c>
       <c r="BS65" t="n">
         <v>4.14</v>
       </c>
       <c r="BT65" t="n">
-        <v>8443</v>
+        <v>8357</v>
       </c>
     </row>
     <row r="66">
@@ -15513,13 +15513,13 @@
         </is>
       </c>
       <c r="F66" t="n">
-        <v>20.74</v>
+        <v>20.79</v>
       </c>
       <c r="G66" t="n">
-        <v>240198552918</v>
+        <v>243047964214</v>
       </c>
       <c r="H66" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="I66" t="n">
         <v>2972355254</v>
@@ -15534,7 +15534,7 @@
         <v>2.75</v>
       </c>
       <c r="M66" t="n">
-        <v>14.25953469893889</v>
+        <v>14.42869175152418</v>
       </c>
       <c r="N66" t="n">
         <v>0.25</v>
@@ -15612,7 +15612,7 @@
         <v>4696321301.320001</v>
       </c>
       <c r="AM66" t="n">
-        <v>21542471113.72197</v>
+        <v>21798023696.32287</v>
       </c>
       <c r="AN66" t="n">
         <v>0.4734</v>
@@ -15653,7 +15653,7 @@
         <v>12.99</v>
       </c>
       <c r="AZ66" t="n">
-        <v>8.33</v>
+        <v>8.35</v>
       </c>
       <c r="BA66" t="n">
         <v>2.23</v>
@@ -15662,25 +15662,25 @@
         <v>3.47</v>
       </c>
       <c r="BC66" t="n">
-        <v>-23.29</v>
+        <v>-23.47</v>
       </c>
       <c r="BD66" t="n">
-        <v>-37.37</v>
+        <v>-37.52</v>
       </c>
       <c r="BE66" t="n">
         <v>-59.83</v>
       </c>
       <c r="BF66" t="n">
-        <v>-89.23999999999999</v>
+        <v>-89.27</v>
       </c>
       <c r="BG66" t="n">
-        <v>-83.29000000000001</v>
+        <v>-83.33</v>
       </c>
       <c r="BH66" t="n">
         <v>7.12</v>
       </c>
       <c r="BI66" t="n">
-        <v>0</v>
+        <v>0.24</v>
       </c>
       <c r="BJ66" t="n">
         <v>20.74</v>
@@ -15692,7 +15692,7 @@
         <v>1.57</v>
       </c>
       <c r="BM66" t="n">
-        <v>20.74</v>
+        <v>20.79</v>
       </c>
       <c r="BN66" t="n">
         <v>21.33</v>
@@ -15701,19 +15701,19 @@
         <v>9.48</v>
       </c>
       <c r="BP66" t="n">
-        <v>20.3</v>
+        <v>20.79</v>
       </c>
       <c r="BQ66" t="n">
-        <v>13.21</v>
+        <v>13.24</v>
       </c>
       <c r="BR66" t="n">
-        <v>20.3</v>
+        <v>20.79</v>
       </c>
       <c r="BS66" t="n">
         <v>3.46</v>
       </c>
       <c r="BT66" t="n">
-        <v>4343</v>
+        <v>4297</v>
       </c>
     </row>
     <row r="67">
@@ -15973,13 +15973,13 @@
         </is>
       </c>
       <c r="F68" t="n">
-        <v>17.83</v>
+        <v>17.98</v>
       </c>
       <c r="G68" t="n">
-        <v>7580539738</v>
+        <v>7619953007</v>
       </c>
       <c r="H68" t="n">
-        <v>37000</v>
+        <v>82100</v>
       </c>
       <c r="I68" t="n">
         <v>137989898</v>
@@ -16072,7 +16072,7 @@
         <v>205604948.02</v>
       </c>
       <c r="AM68" t="n">
-        <v>525696237.0319002</v>
+        <v>528429473.4396671</v>
       </c>
       <c r="AN68" t="n">
         <v>0.1911</v>
@@ -16113,7 +16113,7 @@
         <v>21.39</v>
       </c>
       <c r="AZ68" t="n">
-        <v>32.99</v>
+        <v>33.26</v>
       </c>
       <c r="BA68" t="n">
         <v>1.24</v>
@@ -16122,25 +16122,25 @@
         <v>63.25</v>
       </c>
       <c r="BC68" t="n">
-        <v>46.96</v>
+        <v>45.73</v>
       </c>
       <c r="BD68" t="n">
-        <v>19.99</v>
+        <v>18.99</v>
       </c>
       <c r="BE68" t="n">
         <v>85</v>
       </c>
       <c r="BF68" t="n">
-        <v>-93.05</v>
+        <v>-93.11</v>
       </c>
       <c r="BG68" t="n">
-        <v>254.73</v>
+        <v>251.77</v>
       </c>
       <c r="BH68" t="n">
         <v>20.48</v>
       </c>
       <c r="BI68" t="n">
-        <v>0</v>
+        <v>0.84</v>
       </c>
       <c r="BJ68" t="n">
         <v>17.83</v>
@@ -16152,7 +16152,7 @@
         <v>1.49</v>
       </c>
       <c r="BM68" t="n">
-        <v>18.12</v>
+        <v>18.08</v>
       </c>
       <c r="BN68" t="n">
         <v>22.11</v>
@@ -16161,19 +16161,19 @@
         <v>15.45</v>
       </c>
       <c r="BP68" t="n">
-        <v>17.78</v>
+        <v>17.85</v>
       </c>
       <c r="BQ68" t="n">
-        <v>11.99</v>
+        <v>12.09</v>
       </c>
       <c r="BR68" t="n">
-        <v>18.12</v>
+        <v>17.89</v>
       </c>
       <c r="BS68" t="n">
         <v>0</v>
       </c>
       <c r="BT68" t="n">
-        <v>42227</v>
+        <v>41707</v>
       </c>
     </row>
     <row r="69">
@@ -16203,13 +16203,13 @@
         </is>
       </c>
       <c r="F69" t="n">
-        <v>20.24</v>
+        <v>20.23</v>
       </c>
       <c r="G69" t="n">
-        <v>7580539738</v>
+        <v>7619953007</v>
       </c>
       <c r="H69" t="n">
-        <v>1790900</v>
+        <v>0</v>
       </c>
       <c r="I69" t="n">
         <v>255106712</v>
@@ -16302,7 +16302,7 @@
         <v>380109000.88</v>
       </c>
       <c r="AM69" t="n">
-        <v>451222603.452381</v>
+        <v>453568631.3690476</v>
       </c>
       <c r="AN69" t="n">
         <v>0.8856000000000001</v>
@@ -16343,7 +16343,7 @@
         <v>21.39</v>
       </c>
       <c r="AZ69" t="n">
-        <v>35.39</v>
+        <v>35.37</v>
       </c>
       <c r="BA69" t="n">
         <v>1.24</v>
@@ -16352,25 +16352,25 @@
         <v>69.59</v>
       </c>
       <c r="BC69" t="n">
-        <v>29.46</v>
+        <v>29.52</v>
       </c>
       <c r="BD69" t="n">
-        <v>5.7</v>
+        <v>5.76</v>
       </c>
       <c r="BE69" t="n">
         <v>74.83</v>
       </c>
       <c r="BF69" t="n">
-        <v>-93.88</v>
+        <v>-93.87</v>
       </c>
       <c r="BG69" t="n">
-        <v>243.81</v>
+        <v>243.98</v>
       </c>
       <c r="BH69" t="n">
         <v>20.48</v>
       </c>
       <c r="BI69" t="n">
-        <v>0</v>
+        <v>-0.05</v>
       </c>
       <c r="BJ69" t="n">
         <v>20.24</v>
@@ -16382,28 +16382,28 @@
         <v>1.49</v>
       </c>
       <c r="BM69" t="n">
-        <v>20.62</v>
+        <v>20.56</v>
       </c>
       <c r="BN69" t="n">
         <v>25.63</v>
       </c>
       <c r="BO69" t="n">
-        <v>16.87</v>
+        <v>16.97</v>
       </c>
       <c r="BP69" t="n">
-        <v>20.09</v>
+        <v>20.21</v>
       </c>
       <c r="BQ69" t="n">
         <v>13.61</v>
       </c>
       <c r="BR69" t="n">
-        <v>20.53</v>
+        <v>20.5</v>
       </c>
       <c r="BS69" t="n">
         <v>0</v>
       </c>
       <c r="BT69" t="n">
-        <v>2099263</v>
+        <v>2104557</v>
       </c>
     </row>
     <row r="70">
@@ -16433,13 +16433,13 @@
         </is>
       </c>
       <c r="F70" t="n">
-        <v>18.23</v>
+        <v>18.12</v>
       </c>
       <c r="G70" t="n">
-        <v>8468877543</v>
+        <v>8417776853</v>
       </c>
       <c r="H70" t="n">
-        <v>3499500</v>
+        <v>0</v>
       </c>
       <c r="I70" t="n">
         <v>464557268</v>
@@ -16454,7 +16454,7 @@
         <v>0.68</v>
       </c>
       <c r="M70" t="n">
-        <v>0.6684332186790801</v>
+        <v>0.6643999334509031</v>
       </c>
       <c r="N70" t="n">
         <v>0.2</v>
@@ -16532,7 +16532,7 @@
         <v>55746872.16</v>
       </c>
       <c r="AM70" t="n">
-        <v>2795009090.09901</v>
+        <v>2778144175.907591</v>
       </c>
       <c r="AN70" t="n">
         <v>0.1236</v>
@@ -16573,7 +16573,7 @@
         <v>6.9</v>
       </c>
       <c r="AZ70" t="n">
-        <v>2.1</v>
+        <v>2.08</v>
       </c>
       <c r="BA70" t="n">
         <v>0.12</v>
@@ -16582,10 +16582,10 @@
         <v>1.07</v>
       </c>
       <c r="BC70" t="n">
-        <v>-53.65</v>
+        <v>-53.37</v>
       </c>
       <c r="BD70" t="n">
-        <v>-62.16</v>
+        <v>-61.93</v>
       </c>
       <c r="BE70" t="n">
         <v>-88.5</v>
@@ -16594,13 +16594,13 @@
         <v>-99.34</v>
       </c>
       <c r="BG70" t="n">
-        <v>-94.13</v>
+        <v>-94.09999999999999</v>
       </c>
       <c r="BH70" t="n">
         <v>26.44</v>
       </c>
       <c r="BI70" t="n">
-        <v>0</v>
+        <v>-0.6</v>
       </c>
       <c r="BJ70" t="n">
         <v>18.23</v>
@@ -16612,7 +16612,7 @@
         <v>0.1</v>
       </c>
       <c r="BM70" t="n">
-        <v>18.42</v>
+        <v>18.59</v>
       </c>
       <c r="BN70" t="n">
         <v>22.15</v>
@@ -16621,19 +16621,19 @@
         <v>13.21</v>
       </c>
       <c r="BP70" t="n">
-        <v>17.62</v>
+        <v>18.12</v>
       </c>
       <c r="BQ70" t="n">
-        <v>182.83</v>
+        <v>181.73</v>
       </c>
       <c r="BR70" t="n">
-        <v>17.75</v>
+        <v>18.49</v>
       </c>
       <c r="BS70" t="n">
         <v>0.67</v>
       </c>
       <c r="BT70" t="n">
-        <v>3827607</v>
+        <v>3798633</v>
       </c>
     </row>
     <row r="71">

</xml_diff>

<commit_message>
📊 Dados atualizados - 2026-10-02 06:30
</commit_message>
<xml_diff>
--- a/data/ativos.xlsx
+++ b/data/ativos.xlsx
@@ -1047,13 +1047,13 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>25.88</v>
+        <v>25.61</v>
       </c>
       <c r="G3" t="n">
-        <v>3461884671</v>
+        <v>3425767829</v>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>707800</v>
       </c>
       <c r="I3" t="n">
         <v>129510368</v>
@@ -1068,7 +1068,7 @@
         <v>0.88</v>
       </c>
       <c r="M3" t="n">
-        <v>0.8613940072434954</v>
+        <v>0.8524073325804212</v>
       </c>
       <c r="N3" t="n">
         <v>0.09</v>
@@ -1146,7 +1146,7 @@
         <v>506385538.88</v>
       </c>
       <c r="AM3" t="n">
-        <v>676149349.8046875</v>
+        <v>669095279.1015625</v>
       </c>
       <c r="AN3" t="n">
         <v>2.7</v>
@@ -1187,7 +1187,7 @@
         <v>40.42</v>
       </c>
       <c r="AZ3" t="n">
-        <v>47.36</v>
+        <v>46.87</v>
       </c>
       <c r="BA3" t="n">
         <v>4.87</v>
@@ -1196,28 +1196,28 @@
         <v>21.14</v>
       </c>
       <c r="BC3" t="n">
-        <v>91.26000000000001</v>
+        <v>93.28</v>
       </c>
       <c r="BD3" t="n">
-        <v>56.16</v>
+        <v>57.81</v>
       </c>
       <c r="BE3" t="n">
         <v>83</v>
       </c>
       <c r="BF3" t="n">
-        <v>-81.19</v>
+        <v>-80.98999999999999</v>
       </c>
       <c r="BG3" t="n">
-        <v>-18.33</v>
+        <v>-17.47</v>
       </c>
       <c r="BH3" t="n">
         <v>27.85</v>
       </c>
       <c r="BI3" t="n">
-        <v>2.78</v>
+        <v>0</v>
       </c>
       <c r="BJ3" t="n">
-        <v>25.18</v>
+        <v>25.61</v>
       </c>
       <c r="BK3" t="n">
         <v>3.91</v>
@@ -1226,7 +1226,7 @@
         <v>4.39</v>
       </c>
       <c r="BM3" t="n">
-        <v>26.11</v>
+        <v>25.9</v>
       </c>
       <c r="BN3" t="n">
         <v>27.17</v>
@@ -1235,19 +1235,19 @@
         <v>18.72</v>
       </c>
       <c r="BP3" t="n">
-        <v>25.24</v>
+        <v>25.43</v>
       </c>
       <c r="BQ3" t="n">
-        <v>5.89</v>
+        <v>5.83</v>
       </c>
       <c r="BR3" t="n">
-        <v>25.31</v>
+        <v>25.88</v>
       </c>
       <c r="BS3" t="n">
         <v>0.79</v>
       </c>
       <c r="BT3" t="n">
-        <v>516447</v>
+        <v>551093</v>
       </c>
     </row>
     <row r="4">
@@ -1277,13 +1277,13 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>15.36</v>
+        <v>15.42</v>
       </c>
       <c r="G4" t="n">
-        <v>237844372283</v>
+        <v>238773458381</v>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
+        <v>25111800</v>
       </c>
       <c r="I4" t="n">
         <v>15484664889</v>
@@ -1298,7 +1298,7 @@
         <v>2.76</v>
       </c>
       <c r="M4" t="n">
-        <v>2.693119089492016</v>
+        <v>2.703639159747571</v>
       </c>
       <c r="N4" t="n">
         <v>1.76</v>
@@ -1376,7 +1376,7 @@
         <v>16258898133.45</v>
       </c>
       <c r="AM4" t="n">
-        <v>23548947750.79208</v>
+        <v>23640936473.36634</v>
       </c>
       <c r="AN4" t="n">
         <v>0.269</v>
@@ -1417,7 +1417,7 @@
         <v>9.470000000000001</v>
       </c>
       <c r="AZ4" t="n">
-        <v>19.17</v>
+        <v>19.25</v>
       </c>
       <c r="BA4" t="n">
         <v>1.13</v>
@@ -1426,28 +1426,28 @@
         <v>11.39</v>
       </c>
       <c r="BC4" t="n">
-        <v>-24.45</v>
+        <v>-24.74</v>
       </c>
       <c r="BD4" t="n">
-        <v>-38.31</v>
+        <v>-38.55</v>
       </c>
       <c r="BE4" t="n">
         <v>24.83</v>
       </c>
       <c r="BF4" t="n">
-        <v>-92.66</v>
+        <v>-92.69</v>
       </c>
       <c r="BG4" t="n">
-        <v>-25.87</v>
+        <v>-26.16</v>
       </c>
       <c r="BH4" t="n">
         <v>5.7</v>
       </c>
       <c r="BI4" t="n">
-        <v>0.59</v>
+        <v>0</v>
       </c>
       <c r="BJ4" t="n">
-        <v>15.27</v>
+        <v>15.42</v>
       </c>
       <c r="BK4" t="n">
         <v>1.05</v>
@@ -1456,7 +1456,7 @@
         <v>1.04</v>
       </c>
       <c r="BM4" t="n">
-        <v>15.59</v>
+        <v>15.45</v>
       </c>
       <c r="BN4" t="n">
         <v>16.94</v>
@@ -1465,19 +1465,19 @@
         <v>11.04</v>
       </c>
       <c r="BP4" t="n">
-        <v>15.31</v>
+        <v>15.23</v>
       </c>
       <c r="BQ4" t="n">
-        <v>14.81</v>
+        <v>14.87</v>
       </c>
       <c r="BR4" t="n">
-        <v>15.59</v>
+        <v>15.36</v>
       </c>
       <c r="BS4" t="n">
         <v>2.76</v>
       </c>
       <c r="BT4" t="n">
-        <v>25861960</v>
+        <v>26042500</v>
       </c>
     </row>
     <row r="5">
@@ -1737,13 +1737,13 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>7.37</v>
+        <v>7</v>
       </c>
       <c r="G6" t="n">
-        <v>464934231</v>
+        <v>441592830</v>
       </c>
       <c r="H6" t="n">
-        <v>200</v>
+        <v>1800</v>
       </c>
       <c r="I6" t="n">
         <v>63084700</v>
@@ -1758,7 +1758,7 @@
         <v>1.91</v>
       </c>
       <c r="M6" t="n">
-        <v>7.238115664929348</v>
+        <v>6.874735752342318</v>
       </c>
       <c r="N6" t="n">
         <v>1.26</v>
@@ -1836,7 +1836,7 @@
         <v>35958279</v>
       </c>
       <c r="AM6" t="n">
-        <v>44448779.2543021</v>
+        <v>42217287.76290631</v>
       </c>
       <c r="AN6" t="n">
         <v>0.5199</v>
@@ -1877,7 +1877,7 @@
         <v>5.74</v>
       </c>
       <c r="AZ6" t="n">
-        <v>8.65</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="BA6" t="n">
         <v>0.65</v>
@@ -1886,19 +1886,19 @@
         <v>7.95</v>
       </c>
       <c r="BC6" t="n">
-        <v>-4.53</v>
+        <v>0.51</v>
       </c>
       <c r="BD6" t="n">
-        <v>-22.05</v>
+        <v>-17.93</v>
       </c>
       <c r="BE6" t="n">
         <v>17.33</v>
       </c>
       <c r="BF6" t="n">
-        <v>-91.2</v>
+        <v>-90.73999999999999</v>
       </c>
       <c r="BG6" t="n">
-        <v>7.92</v>
+        <v>13.62</v>
       </c>
       <c r="BH6" t="n">
         <v>3.86</v>
@@ -1907,7 +1907,7 @@
         <v>0</v>
       </c>
       <c r="BJ6" t="n">
-        <v>7.37</v>
+        <v>7</v>
       </c>
       <c r="BK6" t="n">
         <v>0.57</v>
@@ -1916,7 +1916,7 @@
         <v>0.5600000000000001</v>
       </c>
       <c r="BM6" t="n">
-        <v>7.37</v>
+        <v>7.33</v>
       </c>
       <c r="BN6" t="n">
         <v>8.16</v>
@@ -1925,19 +1925,19 @@
         <v>6.22</v>
       </c>
       <c r="BP6" t="n">
-        <v>7.32</v>
+        <v>7</v>
       </c>
       <c r="BQ6" t="n">
-        <v>13.11</v>
+        <v>12.45</v>
       </c>
       <c r="BR6" t="n">
-        <v>7.32</v>
+        <v>7.33</v>
       </c>
       <c r="BS6" t="n">
         <v>7.32</v>
       </c>
       <c r="BT6" t="n">
-        <v>180</v>
+        <v>167</v>
       </c>
     </row>
     <row r="7">
@@ -3117,13 +3117,13 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>5.32</v>
+        <v>5.3</v>
       </c>
       <c r="G12" t="n">
-        <v>510515409</v>
+        <v>508596180</v>
       </c>
       <c r="H12" t="n">
-        <v>3154300</v>
+        <v>1009200</v>
       </c>
       <c r="I12" t="n">
         <v>95961536</v>
@@ -3138,7 +3138,7 @@
         <v>0.32</v>
       </c>
       <c r="M12" t="n">
-        <v>0.09232593270412673</v>
+        <v>0.09197884306809616</v>
       </c>
       <c r="N12" t="n">
         <v>0.14</v>
@@ -3216,7 +3216,7 @@
         <v>362734606.08</v>
       </c>
       <c r="AM12" t="n">
-        <v>548941300</v>
+        <v>546877612.9032258</v>
       </c>
       <c r="AN12" t="n">
         <v>0.4208</v>
@@ -3257,7 +3257,7 @@
         <v>30.49</v>
       </c>
       <c r="AZ12" t="n">
-        <v>7.19</v>
+        <v>7.16</v>
       </c>
       <c r="BA12" t="n">
         <v>4.41</v>
@@ -3266,28 +3266,28 @@
         <v>18.12</v>
       </c>
       <c r="BC12" t="n">
-        <v>602.02</v>
+        <v>604.67</v>
       </c>
       <c r="BD12" t="n">
-        <v>473.19</v>
+        <v>475.36</v>
       </c>
       <c r="BE12" t="n">
         <v>35.17</v>
       </c>
       <c r="BF12" t="n">
-        <v>-17.07</v>
+        <v>-16.76</v>
       </c>
       <c r="BG12" t="n">
-        <v>240.58</v>
+        <v>241.87</v>
       </c>
       <c r="BH12" t="n">
         <v>16.4</v>
       </c>
       <c r="BI12" t="n">
-        <v>7.91</v>
+        <v>0</v>
       </c>
       <c r="BJ12" t="n">
-        <v>4.93</v>
+        <v>5.3</v>
       </c>
       <c r="BK12" t="n">
         <v>3.78</v>
@@ -3296,7 +3296,7 @@
         <v>3.63</v>
       </c>
       <c r="BM12" t="n">
-        <v>5.45</v>
+        <v>5.39</v>
       </c>
       <c r="BN12" t="n">
         <v>8.23</v>
@@ -3305,19 +3305,19 @@
         <v>4.42</v>
       </c>
       <c r="BP12" t="n">
-        <v>5.22</v>
+        <v>5.2</v>
       </c>
       <c r="BQ12" t="n">
         <v>1.46</v>
       </c>
       <c r="BR12" t="n">
-        <v>5.26</v>
+        <v>5.39</v>
       </c>
       <c r="BS12" t="n">
         <v>0.09</v>
       </c>
       <c r="BT12" t="n">
-        <v>470260</v>
+        <v>560840</v>
       </c>
     </row>
     <row r="13">
@@ -3347,13 +3347,13 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>29.49</v>
+        <v>29.73</v>
       </c>
       <c r="G13" t="n">
-        <v>14868586576</v>
+        <v>14989595226</v>
       </c>
       <c r="H13" t="n">
-        <v>0</v>
+        <v>5757100</v>
       </c>
       <c r="I13" t="n">
         <v>504190947</v>
@@ -3368,7 +3368,7 @@
         <v>1.13</v>
       </c>
       <c r="M13" t="n">
-        <v>5.142416838954876</v>
+        <v>5.184268626025453</v>
       </c>
       <c r="N13" t="n">
         <v>0.57</v>
@@ -3446,7 +3446,7 @@
         <v>932753251.95</v>
       </c>
       <c r="AM13" t="n">
-        <v>1547199435.587929</v>
+        <v>1559791386.680541</v>
       </c>
       <c r="AN13" t="n">
         <v>2.6301</v>
@@ -3487,7 +3487,7 @@
         <v>26.6</v>
       </c>
       <c r="AZ13" t="n">
-        <v>53.38</v>
+        <v>53.81</v>
       </c>
       <c r="BA13" t="n">
         <v>2.6</v>
@@ -3496,28 +3496,28 @@
         <v>8.69</v>
       </c>
       <c r="BC13" t="n">
-        <v>10.46</v>
+        <v>9.56</v>
       </c>
       <c r="BD13" t="n">
-        <v>-9.81</v>
+        <v>-10.54</v>
       </c>
       <c r="BE13" t="n">
         <v>81</v>
       </c>
       <c r="BF13" t="n">
-        <v>-91.17</v>
+        <v>-91.23999999999999</v>
       </c>
       <c r="BG13" t="n">
-        <v>-70.52</v>
+        <v>-70.76000000000001</v>
       </c>
       <c r="BH13" t="n">
         <v>25.49</v>
       </c>
       <c r="BI13" t="n">
-        <v>2.5</v>
+        <v>0</v>
       </c>
       <c r="BJ13" t="n">
-        <v>28.77</v>
+        <v>29.73</v>
       </c>
       <c r="BK13" t="n">
         <v>1.85</v>
@@ -3526,7 +3526,7 @@
         <v>1.96</v>
       </c>
       <c r="BM13" t="n">
-        <v>29.76</v>
+        <v>29.73</v>
       </c>
       <c r="BN13" t="n">
         <v>32.11</v>
@@ -3535,19 +3535,19 @@
         <v>20.85</v>
       </c>
       <c r="BP13" t="n">
-        <v>29.01</v>
+        <v>29.13</v>
       </c>
       <c r="BQ13" t="n">
-        <v>15.07</v>
+        <v>15.19</v>
       </c>
       <c r="BR13" t="n">
-        <v>29.32</v>
+        <v>29.5</v>
       </c>
       <c r="BS13" t="n">
         <v>5.01</v>
       </c>
       <c r="BT13" t="n">
-        <v>4821963</v>
+        <v>5099753</v>
       </c>
     </row>
     <row r="14">
@@ -3577,13 +3577,13 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>10.21</v>
+        <v>10.65</v>
       </c>
       <c r="G14" t="n">
-        <v>8283810124</v>
+        <v>8567288036</v>
       </c>
       <c r="H14" t="n">
-        <v>3900</v>
+        <v>8900</v>
       </c>
       <c r="I14" t="n">
         <v>339510689</v>
@@ -3598,7 +3598,7 @@
         <v>1.92</v>
       </c>
       <c r="M14" t="n">
-        <v>3.439585230440184</v>
+        <v>3.557290299083212</v>
       </c>
       <c r="N14" t="n">
         <v>1.11</v>
@@ -3676,7 +3676,7 @@
         <v>349696009.67</v>
       </c>
       <c r="AM14" t="n">
-        <v>919401789.5671476</v>
+        <v>950864376.9145395</v>
       </c>
       <c r="AN14" t="n">
         <v>0.1489</v>
@@ -3717,7 +3717,7 @@
         <v>9.050000000000001</v>
       </c>
       <c r="AZ14" t="n">
-        <v>8.199999999999999</v>
+        <v>8.56</v>
       </c>
       <c r="BA14" t="n">
         <v>1.42</v>
@@ -3726,28 +3726,28 @@
         <v>5.94</v>
       </c>
       <c r="BC14" t="n">
-        <v>8.550000000000001</v>
+        <v>4.06</v>
       </c>
       <c r="BD14" t="n">
-        <v>-11.37</v>
+        <v>-15.03</v>
       </c>
       <c r="BE14" t="n">
         <v>-19.67</v>
       </c>
       <c r="BF14" t="n">
-        <v>-86.08</v>
+        <v>-86.66</v>
       </c>
       <c r="BG14" t="n">
-        <v>-41.8</v>
+        <v>-44.2</v>
       </c>
       <c r="BH14" t="n">
         <v>5.3</v>
       </c>
       <c r="BI14" t="n">
-        <v>2.82</v>
+        <v>0</v>
       </c>
       <c r="BJ14" t="n">
-        <v>9.93</v>
+        <v>10.65</v>
       </c>
       <c r="BK14" t="n">
         <v>1.03</v>
@@ -3756,28 +3756,28 @@
         <v>1.01</v>
       </c>
       <c r="BM14" t="n">
-        <v>10.42</v>
+        <v>10.65</v>
       </c>
       <c r="BN14" t="n">
         <v>13.49</v>
       </c>
       <c r="BO14" t="n">
-        <v>7.77</v>
+        <v>7.81</v>
       </c>
       <c r="BP14" t="n">
-        <v>10.21</v>
+        <v>10.35</v>
       </c>
       <c r="BQ14" t="n">
-        <v>10.08</v>
+        <v>10.51</v>
       </c>
       <c r="BR14" t="n">
-        <v>10.3</v>
+        <v>10.39</v>
       </c>
       <c r="BS14" t="n">
         <v>1.44</v>
       </c>
       <c r="BT14" t="n">
-        <v>10220</v>
+        <v>9753</v>
       </c>
     </row>
     <row r="15">
@@ -3807,13 +3807,13 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>14.18</v>
+        <v>14.57</v>
       </c>
       <c r="G15" t="n">
-        <v>8283810124</v>
+        <v>8567288036</v>
       </c>
       <c r="H15" t="n">
-        <v>0</v>
+        <v>2677700</v>
       </c>
       <c r="I15" t="n">
         <v>343551533</v>
@@ -3828,7 +3828,7 @@
         <v>2.56</v>
       </c>
       <c r="M15" t="n">
-        <v>3.39912892037938</v>
+        <v>3.515449545133472</v>
       </c>
       <c r="N15" t="n">
         <v>1.47</v>
@@ -3906,7 +3906,7 @@
         <v>353858078.99</v>
       </c>
       <c r="AM15" t="n">
-        <v>690893254.7122602</v>
+        <v>714536116.4303586</v>
       </c>
       <c r="AN15" t="n">
         <v>0.1638</v>
@@ -3947,7 +3947,7 @@
         <v>9.050000000000001</v>
       </c>
       <c r="AZ15" t="n">
-        <v>9.43</v>
+        <v>9.69</v>
       </c>
       <c r="BA15" t="n">
         <v>1.42</v>
@@ -3956,28 +3956,28 @@
         <v>6.19</v>
       </c>
       <c r="BC15" t="n">
-        <v>-21.84</v>
+        <v>-23.93</v>
       </c>
       <c r="BD15" t="n">
-        <v>-36.18</v>
+        <v>-37.89</v>
       </c>
       <c r="BE15" t="n">
         <v>-33.5</v>
       </c>
       <c r="BF15" t="n">
-        <v>-89.98</v>
+        <v>-90.25</v>
       </c>
       <c r="BG15" t="n">
-        <v>-56.36</v>
+        <v>-57.53</v>
       </c>
       <c r="BH15" t="n">
         <v>5.3</v>
       </c>
       <c r="BI15" t="n">
-        <v>1.21</v>
+        <v>0</v>
       </c>
       <c r="BJ15" t="n">
-        <v>14.01</v>
+        <v>14.57</v>
       </c>
       <c r="BK15" t="n">
         <v>1.03</v>
@@ -3986,7 +3986,7 @@
         <v>1.01</v>
       </c>
       <c r="BM15" t="n">
-        <v>14.38</v>
+        <v>14.65</v>
       </c>
       <c r="BN15" t="n">
         <v>16.22</v>
@@ -3995,19 +3995,19 @@
         <v>7.84</v>
       </c>
       <c r="BP15" t="n">
-        <v>13.9</v>
+        <v>14.19</v>
       </c>
       <c r="BQ15" t="n">
-        <v>14</v>
+        <v>14.38</v>
       </c>
       <c r="BR15" t="n">
-        <v>14.18</v>
+        <v>14.19</v>
       </c>
       <c r="BS15" t="n">
         <v>1.92</v>
       </c>
       <c r="BT15" t="n">
-        <v>2350630</v>
+        <v>2359873</v>
       </c>
     </row>
     <row r="16">
@@ -4037,13 +4037,13 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>4.43</v>
+        <v>4.49</v>
       </c>
       <c r="G16" t="n">
-        <v>971524213</v>
+        <v>984682542</v>
       </c>
       <c r="H16" t="n">
-        <v>113800</v>
+        <v>122500</v>
       </c>
       <c r="I16" t="n">
         <v>219305733</v>
@@ -4058,7 +4058,7 @@
         <v>2.69</v>
       </c>
       <c r="M16" t="n">
-        <v>0.4596124128626861</v>
+        <v>0.46583740577589</v>
       </c>
       <c r="N16" t="n">
         <v>0.39</v>
@@ -4136,7 +4136,7 @@
         <v>17544458.64</v>
       </c>
       <c r="AM16" t="n">
-        <v>272900059.8314607</v>
+        <v>276596219.6629214</v>
       </c>
       <c r="AN16" t="n">
         <v>0.0077</v>
@@ -4186,16 +4186,16 @@
         <v>0</v>
       </c>
       <c r="BC16" t="n">
-        <v>-60.75</v>
+        <v>-61.27</v>
       </c>
       <c r="BD16" t="n">
-        <v>-67.95</v>
+        <v>-68.38</v>
       </c>
       <c r="BE16" t="n">
         <v>-97.17</v>
       </c>
       <c r="BF16" t="n">
-        <v>-98.19</v>
+        <v>-98.22</v>
       </c>
       <c r="BG16" t="n">
         <v>-100</v>
@@ -4204,10 +4204,10 @@
         <v>1.68</v>
       </c>
       <c r="BI16" t="n">
-        <v>-0.23</v>
+        <v>0</v>
       </c>
       <c r="BJ16" t="n">
-        <v>4.44</v>
+        <v>4.49</v>
       </c>
       <c r="BK16" t="n">
         <v>0.08</v>
@@ -4216,7 +4216,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="BM16" t="n">
-        <v>4.44</v>
+        <v>4.49</v>
       </c>
       <c r="BN16" t="n">
         <v>5.54</v>
@@ -4225,19 +4225,19 @@
         <v>3.22</v>
       </c>
       <c r="BP16" t="n">
-        <v>4.32</v>
+        <v>4.35</v>
       </c>
       <c r="BQ16" t="n">
-        <v>60.45</v>
+        <v>61.27</v>
       </c>
       <c r="BR16" t="n">
-        <v>4.42</v>
+        <v>4.35</v>
       </c>
       <c r="BS16" t="n">
         <v>0.49</v>
       </c>
       <c r="BT16" t="n">
-        <v>126800</v>
+        <v>129167</v>
       </c>
     </row>
     <row r="17">
@@ -4267,13 +4267,13 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>32.53</v>
+        <v>32.66</v>
       </c>
       <c r="G17" t="n">
-        <v>10722762654</v>
+        <v>10765611237</v>
       </c>
       <c r="H17" t="n">
-        <v>0</v>
+        <v>940000</v>
       </c>
       <c r="I17" t="n">
         <v>0</v>
@@ -4360,13 +4360,13 @@
         <v>8.039999999999999</v>
       </c>
       <c r="AK17" t="n">
-        <v>4842288048.229769</v>
+        <v>4861638022.489162</v>
       </c>
       <c r="AL17" t="n">
-        <v>1340345331.75</v>
+        <v>1345701404.625</v>
       </c>
       <c r="AM17" t="n">
-        <v>3319740759.752322</v>
+        <v>3333006574.922601</v>
       </c>
       <c r="AN17" t="n">
         <v>1.08</v>
@@ -4407,7 +4407,7 @@
         <v>42.98</v>
       </c>
       <c r="AZ17" t="n">
-        <v>17.4</v>
+        <v>17.47</v>
       </c>
       <c r="BA17" t="n">
         <v>4.55</v>
@@ -4416,28 +4416,28 @@
         <v>16.33</v>
       </c>
       <c r="BC17" t="n">
-        <v>61.81</v>
+        <v>61.17</v>
       </c>
       <c r="BD17" t="n">
-        <v>32.12</v>
+        <v>31.59</v>
       </c>
       <c r="BE17" t="n">
         <v>-46.5</v>
       </c>
       <c r="BF17" t="n">
-        <v>-86.02</v>
+        <v>-86.06999999999999</v>
       </c>
       <c r="BG17" t="n">
-        <v>-49.79</v>
+        <v>-49.99</v>
       </c>
       <c r="BH17" t="n">
         <v>29.25</v>
       </c>
       <c r="BI17" t="n">
-        <v>2.33</v>
+        <v>0</v>
       </c>
       <c r="BJ17" t="n">
-        <v>31.79</v>
+        <v>32.66</v>
       </c>
       <c r="BK17" t="n">
         <v>4.21</v>
@@ -4446,7 +4446,7 @@
         <v>12.62</v>
       </c>
       <c r="BM17" t="n">
-        <v>32.6</v>
+        <v>32.79</v>
       </c>
       <c r="BN17" t="n">
         <v>36.63</v>
@@ -4455,19 +4455,19 @@
         <v>29.53</v>
       </c>
       <c r="BP17" t="n">
-        <v>31.95</v>
+        <v>32.1</v>
       </c>
       <c r="BQ17" t="n">
-        <v>2.58</v>
+        <v>2.59</v>
       </c>
       <c r="BR17" t="n">
-        <v>32.13</v>
+        <v>32.65</v>
       </c>
       <c r="BS17" t="n">
         <v>2.21</v>
       </c>
       <c r="BT17" t="n">
-        <v>1118950</v>
+        <v>1120500</v>
       </c>
     </row>
     <row r="18">
@@ -4500,10 +4500,10 @@
         <v>11.5</v>
       </c>
       <c r="G18" t="n">
-        <v>10722762654</v>
+        <v>10765611237</v>
       </c>
       <c r="H18" t="n">
-        <v>3200</v>
+        <v>7200</v>
       </c>
       <c r="I18" t="n">
         <v>671494278</v>
@@ -4518,7 +4518,7 @@
         <v>1.2</v>
       </c>
       <c r="M18" t="n">
-        <v>3.157202419257888</v>
+        <v>3.169818724801022</v>
       </c>
       <c r="N18" t="n">
         <v>0.33</v>
@@ -4596,7 +4596,7 @@
         <v>940091989.1999999</v>
       </c>
       <c r="AM18" t="n">
-        <v>3191298408.928572</v>
+        <v>3204050963.392857</v>
       </c>
       <c r="AN18" t="n">
         <v>0.36</v>
@@ -4664,10 +4664,10 @@
         <v>9.75</v>
       </c>
       <c r="BI18" t="n">
-        <v>5.41</v>
+        <v>0</v>
       </c>
       <c r="BJ18" t="n">
-        <v>10.91</v>
+        <v>11.5</v>
       </c>
       <c r="BK18" t="n">
         <v>1.4</v>
@@ -4676,7 +4676,7 @@
         <v>12.62</v>
       </c>
       <c r="BM18" t="n">
-        <v>11.5</v>
+        <v>11.59</v>
       </c>
       <c r="BN18" t="n">
         <v>13.82</v>
@@ -4685,19 +4685,19 @@
         <v>10.19</v>
       </c>
       <c r="BP18" t="n">
-        <v>11.17</v>
+        <v>11.1</v>
       </c>
       <c r="BQ18" t="n">
         <v>0.91</v>
       </c>
       <c r="BR18" t="n">
-        <v>11.19</v>
+        <v>11.5</v>
       </c>
       <c r="BS18" t="n">
         <v>2.3</v>
       </c>
       <c r="BT18" t="n">
-        <v>9603</v>
+        <v>9433</v>
       </c>
     </row>
     <row r="19">
@@ -4727,13 +4727,13 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>10.5</v>
+        <v>10.6</v>
       </c>
       <c r="G19" t="n">
-        <v>10722762654</v>
+        <v>10765611237</v>
       </c>
       <c r="H19" t="n">
-        <v>16500</v>
+        <v>10400</v>
       </c>
       <c r="I19" t="n">
         <v>317386323</v>
@@ -4748,7 +4748,7 @@
         <v>1.12</v>
       </c>
       <c r="M19" t="n">
-        <v>6.67969350090561</v>
+        <v>6.706385819911789</v>
       </c>
       <c r="N19" t="n">
         <v>0.3</v>
@@ -4826,7 +4826,7 @@
         <v>444340852.2</v>
       </c>
       <c r="AM19" t="n">
-        <v>3404051636.190476</v>
+        <v>3417654360.952381</v>
       </c>
       <c r="AN19" t="n">
         <v>0.36</v>
@@ -4867,7 +4867,7 @@
         <v>14.31</v>
       </c>
       <c r="AZ19" t="n">
-        <v>5.78</v>
+        <v>5.83</v>
       </c>
       <c r="BA19" t="n">
         <v>1.51</v>
@@ -4876,28 +4876,28 @@
         <v>5.25</v>
       </c>
       <c r="BC19" t="n">
-        <v>66.90000000000001</v>
+        <v>65.33</v>
       </c>
       <c r="BD19" t="n">
-        <v>36.28</v>
+        <v>34.99</v>
       </c>
       <c r="BE19" t="n">
         <v>-45</v>
       </c>
       <c r="BF19" t="n">
-        <v>-85.59</v>
+        <v>-85.73</v>
       </c>
       <c r="BG19" t="n">
-        <v>-50</v>
+        <v>-50.47</v>
       </c>
       <c r="BH19" t="n">
         <v>9.75</v>
       </c>
       <c r="BI19" t="n">
-        <v>0.96</v>
+        <v>0</v>
       </c>
       <c r="BJ19" t="n">
-        <v>10.4</v>
+        <v>10.6</v>
       </c>
       <c r="BK19" t="n">
         <v>1.4</v>
@@ -4906,7 +4906,7 @@
         <v>12.62</v>
       </c>
       <c r="BM19" t="n">
-        <v>10.52</v>
+        <v>10.7</v>
       </c>
       <c r="BN19" t="n">
         <v>11.41</v>
@@ -4915,10 +4915,10 @@
         <v>9.19</v>
       </c>
       <c r="BP19" t="n">
-        <v>10.27</v>
+        <v>10.43</v>
       </c>
       <c r="BQ19" t="n">
-        <v>0.83</v>
+        <v>0.84</v>
       </c>
       <c r="BR19" t="n">
         <v>10.43</v>
@@ -4927,7 +4927,7 @@
         <v>2.16</v>
       </c>
       <c r="BT19" t="n">
-        <v>11533</v>
+        <v>11383</v>
       </c>
     </row>
     <row r="20">
@@ -5417,13 +5417,13 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>5.49</v>
+        <v>5.27</v>
       </c>
       <c r="G22" t="n">
-        <v>1099346102</v>
+        <v>1055292727</v>
       </c>
       <c r="H22" t="n">
-        <v>0</v>
+        <v>2070600</v>
       </c>
       <c r="I22" t="n">
         <v>200245299</v>
@@ -5438,7 +5438,7 @@
         <v>0.27</v>
       </c>
       <c r="M22" t="n">
-        <v>0.09324280714261869</v>
+        <v>0.0895063493140663</v>
       </c>
       <c r="N22" t="n">
         <v>0.08</v>
@@ -5516,7 +5516,7 @@
         <v>378463615.11</v>
       </c>
       <c r="AM22" t="n">
-        <v>249284830.3854875</v>
+        <v>239295402.9478458</v>
       </c>
       <c r="AN22" t="n">
         <v>0</v>
@@ -5566,28 +5566,28 @@
         <v>172.49</v>
       </c>
       <c r="BC22" t="n">
-        <v>441.08</v>
+        <v>463.66</v>
       </c>
       <c r="BD22" t="n">
-        <v>341.79</v>
+        <v>360.23</v>
       </c>
       <c r="BE22" t="n">
         <v>-100</v>
       </c>
       <c r="BF22" t="n">
-        <v>-65.56999999999999</v>
+        <v>-64.14</v>
       </c>
       <c r="BG22" t="n">
-        <v>3041.89</v>
+        <v>3173.05</v>
       </c>
       <c r="BH22" t="n">
         <v>20.75</v>
       </c>
       <c r="BI22" t="n">
-        <v>8.07</v>
+        <v>0</v>
       </c>
       <c r="BJ22" t="n">
-        <v>5.08</v>
+        <v>5.27</v>
       </c>
       <c r="BK22" t="n">
         <v>1.89</v>
@@ -5596,7 +5596,7 @@
         <v>0.67</v>
       </c>
       <c r="BM22" t="n">
-        <v>5.52</v>
+        <v>5.56</v>
       </c>
       <c r="BN22" t="n">
         <v>7.89</v>
@@ -5605,19 +5605,19 @@
         <v>3.37</v>
       </c>
       <c r="BP22" t="n">
-        <v>5.12</v>
+        <v>5.22</v>
       </c>
       <c r="BQ22" t="n">
-        <v>8.18</v>
+        <v>7.85</v>
       </c>
       <c r="BR22" t="n">
-        <v>5.14</v>
+        <v>5.49</v>
       </c>
       <c r="BS22" t="n">
         <v>0.09</v>
       </c>
       <c r="BT22" t="n">
-        <v>1530817</v>
+        <v>1574060</v>
       </c>
     </row>
     <row r="23">
@@ -5877,13 +5877,13 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.99</v>
+        <v>3.09</v>
       </c>
       <c r="G24" t="n">
-        <v>1207567715</v>
+        <v>1247954557</v>
       </c>
       <c r="H24" t="n">
-        <v>0</v>
+        <v>7170800</v>
       </c>
       <c r="I24" t="n">
         <v>403868805</v>
@@ -5898,7 +5898,7 @@
         <v>0.49</v>
       </c>
       <c r="M24" t="n">
-        <v>0.2919184181638287</v>
+        <v>0.3016815667515437</v>
       </c>
       <c r="N24" t="n">
         <v>0.11</v>
@@ -5976,7 +5976,7 @@
         <v>153470145.9</v>
       </c>
       <c r="AM24" t="n">
-        <v>1087898842.342342</v>
+        <v>1124283384.684685</v>
       </c>
       <c r="AN24" t="n">
         <v>0.0813</v>
@@ -6017,7 +6017,7 @@
         <v>5.84</v>
       </c>
       <c r="AZ24" t="n">
-        <v>1.38</v>
+        <v>1.43</v>
       </c>
       <c r="BA24" t="n">
         <v>0.38</v>
@@ -6026,28 +6026,28 @@
         <v>1.46</v>
       </c>
       <c r="BC24" t="n">
-        <v>139.35</v>
+        <v>131.6</v>
       </c>
       <c r="BD24" t="n">
-        <v>95.42</v>
+        <v>89.09999999999999</v>
       </c>
       <c r="BE24" t="n">
         <v>-53.83</v>
       </c>
       <c r="BF24" t="n">
-        <v>-87.29000000000001</v>
+        <v>-87.7</v>
       </c>
       <c r="BG24" t="n">
-        <v>-51.24</v>
+        <v>-52.82</v>
       </c>
       <c r="BH24" t="n">
         <v>5.99</v>
       </c>
       <c r="BI24" t="n">
-        <v>4.55</v>
+        <v>0</v>
       </c>
       <c r="BJ24" t="n">
-        <v>2.86</v>
+        <v>3.09</v>
       </c>
       <c r="BK24" t="n">
         <v>0.38</v>
@@ -6056,7 +6056,7 @@
         <v>0.41</v>
       </c>
       <c r="BM24" t="n">
-        <v>2.99</v>
+        <v>3.1</v>
       </c>
       <c r="BN24" t="n">
         <v>5.29</v>
@@ -6065,19 +6065,19 @@
         <v>1.92</v>
       </c>
       <c r="BP24" t="n">
-        <v>2.85</v>
+        <v>2.94</v>
       </c>
       <c r="BQ24" t="n">
-        <v>7.34</v>
+        <v>7.59</v>
       </c>
       <c r="BR24" t="n">
-        <v>2.89</v>
+        <v>2.99</v>
       </c>
       <c r="BS24" t="n">
         <v>0.29</v>
       </c>
       <c r="BT24" t="n">
-        <v>7235407</v>
+        <v>7341513</v>
       </c>
     </row>
     <row r="25">
@@ -6107,13 +6107,13 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>4.31</v>
+        <v>4.39</v>
       </c>
       <c r="G25" t="n">
-        <v>1493389551</v>
+        <v>1521109052</v>
       </c>
       <c r="H25" t="n">
-        <v>0</v>
+        <v>1186300</v>
       </c>
       <c r="I25" t="n">
         <v>346494097</v>
@@ -6128,7 +6128,7 @@
         <v>0.97</v>
       </c>
       <c r="M25" t="n">
-        <v>0.7446722186967973</v>
+        <v>0.7584944275752618</v>
       </c>
       <c r="N25" t="n">
         <v>0.22</v>
@@ -6206,7 +6206,7 @@
         <v>62368937.46</v>
       </c>
       <c r="AM25" t="n">
-        <v>549040276.1029412</v>
+        <v>559231269.1176471</v>
       </c>
       <c r="AN25" t="n">
         <v>0.4742</v>
@@ -6247,7 +6247,7 @@
         <v>3.27</v>
       </c>
       <c r="AZ25" t="n">
-        <v>10.04</v>
+        <v>10.23</v>
       </c>
       <c r="BA25" t="n">
         <v>0.23</v>
@@ -6256,28 +6256,28 @@
         <v>2.2</v>
       </c>
       <c r="BC25" t="n">
-        <v>-6.97</v>
+        <v>-8.66</v>
       </c>
       <c r="BD25" t="n">
-        <v>-24.04</v>
+        <v>-25.42</v>
       </c>
       <c r="BE25" t="n">
         <v>133</v>
       </c>
       <c r="BF25" t="n">
-        <v>-94.62</v>
+        <v>-94.72</v>
       </c>
       <c r="BG25" t="n">
-        <v>-48.96</v>
+        <v>-49.89</v>
       </c>
       <c r="BH25" t="n">
         <v>3.97</v>
       </c>
       <c r="BI25" t="n">
-        <v>9.390000000000001</v>
+        <v>0</v>
       </c>
       <c r="BJ25" t="n">
-        <v>3.94</v>
+        <v>4.39</v>
       </c>
       <c r="BK25" t="n">
         <v>0.18</v>
@@ -6286,7 +6286,7 @@
         <v>0.24</v>
       </c>
       <c r="BM25" t="n">
-        <v>4.44</v>
+        <v>4.39</v>
       </c>
       <c r="BN25" t="n">
         <v>6.3</v>
@@ -6295,19 +6295,19 @@
         <v>2.64</v>
       </c>
       <c r="BP25" t="n">
-        <v>4.01</v>
+        <v>4.17</v>
       </c>
       <c r="BQ25" t="n">
-        <v>18.21</v>
+        <v>18.55</v>
       </c>
       <c r="BR25" t="n">
-        <v>4.01</v>
+        <v>4.3</v>
       </c>
       <c r="BS25" t="n">
         <v>0.67</v>
       </c>
       <c r="BT25" t="n">
-        <v>1159540</v>
+        <v>1161023</v>
       </c>
     </row>
     <row r="26">
@@ -6337,13 +6337,13 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>10.93</v>
+        <v>11.16</v>
       </c>
       <c r="G26" t="n">
-        <v>14803515903</v>
+        <v>15115025673</v>
       </c>
       <c r="H26" t="n">
-        <v>0</v>
+        <v>16044700</v>
       </c>
       <c r="I26" t="n">
         <v>1354393401</v>
@@ -6358,7 +6358,7 @@
         <v>1.94</v>
       </c>
       <c r="M26" t="n">
-        <v>0.1908900896531577</v>
+        <v>0.1949069818774626</v>
       </c>
       <c r="N26" t="n">
         <v>0.26</v>
@@ -6436,7 +6436,7 @@
         <v>961619314.7099999</v>
       </c>
       <c r="AM26" t="n">
-        <v>5286969965.357143</v>
+        <v>5398223454.642858</v>
       </c>
       <c r="AN26" t="n">
         <v>0.1043</v>
@@ -6477,7 +6477,7 @@
         <v>7.07</v>
       </c>
       <c r="AZ26" t="n">
-        <v>2.09</v>
+        <v>2.14</v>
       </c>
       <c r="BA26" t="n">
         <v>0.66</v>
@@ -6486,28 +6486,28 @@
         <v>1.19</v>
       </c>
       <c r="BC26" t="n">
-        <v>-20.81</v>
+        <v>-22.44</v>
       </c>
       <c r="BD26" t="n">
-        <v>-35.34</v>
+        <v>-36.67</v>
       </c>
       <c r="BE26" t="n">
         <v>-80.83</v>
       </c>
       <c r="BF26" t="n">
-        <v>-93.97</v>
+        <v>-94.09</v>
       </c>
       <c r="BG26" t="n">
-        <v>-89.08</v>
+        <v>-89.31</v>
       </c>
       <c r="BH26" t="n">
         <v>4.69</v>
       </c>
       <c r="BI26" t="n">
-        <v>3.7</v>
+        <v>0</v>
       </c>
       <c r="BJ26" t="n">
-        <v>10.54</v>
+        <v>11.16</v>
       </c>
       <c r="BK26" t="n">
         <v>0.71</v>
@@ -6516,28 +6516,28 @@
         <v>0.72</v>
       </c>
       <c r="BM26" t="n">
-        <v>11</v>
+        <v>11.46</v>
       </c>
       <c r="BN26" t="n">
-        <v>11</v>
+        <v>11.46</v>
       </c>
       <c r="BO26" t="n">
         <v>6.91</v>
       </c>
       <c r="BP26" t="n">
-        <v>10.53</v>
+        <v>10.88</v>
       </c>
       <c r="BQ26" t="n">
-        <v>15.24</v>
+        <v>15.56</v>
       </c>
       <c r="BR26" t="n">
-        <v>10.6</v>
+        <v>11.04</v>
       </c>
       <c r="BS26" t="n">
         <v>0.16</v>
       </c>
       <c r="BT26" t="n">
-        <v>12864177</v>
+        <v>12977910</v>
       </c>
     </row>
     <row r="27">
@@ -8165,13 +8165,13 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>17.38</v>
+        <v>18.6</v>
       </c>
       <c r="G34" t="n">
-        <v>3588790812</v>
+        <v>3840710358</v>
       </c>
       <c r="H34" t="n">
-        <v>0</v>
+        <v>8491200</v>
       </c>
       <c r="I34" t="n">
         <v>206489813</v>
@@ -8186,7 +8186,7 @@
         <v>0.45</v>
       </c>
       <c r="M34" t="n">
-        <v>0.3154966273367283</v>
+        <v>0.3376432977019778</v>
       </c>
       <c r="N34" t="n">
         <v>0.24</v>
@@ -8264,7 +8264,7 @@
         <v>324189006.41</v>
       </c>
       <c r="AM34" t="n">
-        <v>746110355.925156</v>
+        <v>798484481.9126819</v>
       </c>
       <c r="AN34" t="n">
         <v>0</v>
@@ -8305,7 +8305,7 @@
         <v>30.28</v>
       </c>
       <c r="AZ34" t="n">
-        <v>40.55</v>
+        <v>43.4</v>
       </c>
       <c r="BA34" t="n">
         <v>2.29</v>
@@ -8314,28 +8314,28 @@
         <v>25.26</v>
       </c>
       <c r="BC34" t="n">
-        <v>113.4</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="BD34" t="n">
-        <v>74.23999999999999</v>
+        <v>62.81</v>
       </c>
       <c r="BE34" t="n">
         <v>133.33</v>
       </c>
       <c r="BF34" t="n">
-        <v>-86.8</v>
+        <v>-87.66</v>
       </c>
       <c r="BG34" t="n">
-        <v>45.33</v>
+        <v>35.79</v>
       </c>
       <c r="BH34" t="n">
         <v>38.94</v>
       </c>
       <c r="BI34" t="n">
-        <v>1.34</v>
+        <v>0</v>
       </c>
       <c r="BJ34" t="n">
-        <v>17.15</v>
+        <v>18.6</v>
       </c>
       <c r="BK34" t="n">
         <v>1.57</v>
@@ -8344,7 +8344,7 @@
         <v>1.58</v>
       </c>
       <c r="BM34" t="n">
-        <v>18.19</v>
+        <v>19.13</v>
       </c>
       <c r="BN34" t="n">
         <v>28.86</v>
@@ -8353,19 +8353,19 @@
         <v>14.3</v>
       </c>
       <c r="BP34" t="n">
-        <v>16.69</v>
+        <v>17.4</v>
       </c>
       <c r="BQ34" t="n">
-        <v>11.02</v>
+        <v>11.79</v>
       </c>
       <c r="BR34" t="n">
-        <v>17.46</v>
+        <v>17.4</v>
       </c>
       <c r="BS34" t="n">
         <v>0.32</v>
       </c>
       <c r="BT34" t="n">
-        <v>3517930</v>
+        <v>3707453</v>
       </c>
     </row>
     <row r="35">
@@ -8395,13 +8395,13 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>18.34</v>
+        <v>18.51</v>
       </c>
       <c r="G35" t="n">
-        <v>92552792430</v>
+        <v>93410716155</v>
       </c>
       <c r="H35" t="n">
-        <v>0</v>
+        <v>36039100</v>
       </c>
       <c r="I35" t="n">
         <v>5046500000</v>
@@ -8416,7 +8416,7 @@
         <v>4.69</v>
       </c>
       <c r="M35" t="n">
-        <v>7.683766465860515</v>
+        <v>7.754991605322481</v>
       </c>
       <c r="N35" t="n">
         <v>1.79</v>
@@ -8494,7 +8494,7 @@
         <v>5349290000</v>
       </c>
       <c r="AM35" t="n">
-        <v>7648991109.917356</v>
+        <v>7719893897.107438</v>
       </c>
       <c r="AN35" t="n">
         <v>0.5305</v>
@@ -8535,7 +8535,7 @@
         <v>7.68</v>
       </c>
       <c r="AZ35" t="n">
-        <v>10.7</v>
+        <v>10.8</v>
       </c>
       <c r="BA35" t="n">
         <v>1.11</v>
@@ -8544,28 +8544,28 @@
         <v>9.119999999999999</v>
       </c>
       <c r="BC35" t="n">
-        <v>-48.71</v>
+        <v>-49.18</v>
       </c>
       <c r="BD35" t="n">
-        <v>-58.12</v>
+        <v>-58.51</v>
       </c>
       <c r="BE35" t="n">
         <v>-41.67</v>
       </c>
       <c r="BF35" t="n">
-        <v>-93.92</v>
+        <v>-93.98</v>
       </c>
       <c r="BG35" t="n">
-        <v>-50.29</v>
+        <v>-50.75</v>
       </c>
       <c r="BH35" t="n">
         <v>3.71</v>
       </c>
       <c r="BI35" t="n">
-        <v>2.46</v>
+        <v>0</v>
       </c>
       <c r="BJ35" t="n">
-        <v>17.9</v>
+        <v>18.51</v>
       </c>
       <c r="BK35" t="n">
         <v>1.06</v>
@@ -8574,7 +8574,7 @@
         <v>1.04</v>
       </c>
       <c r="BM35" t="n">
-        <v>18.6</v>
+        <v>18.58</v>
       </c>
       <c r="BN35" t="n">
         <v>19.88</v>
@@ -8583,19 +8583,19 @@
         <v>11.58</v>
       </c>
       <c r="BP35" t="n">
-        <v>18.09</v>
+        <v>18.11</v>
       </c>
       <c r="BQ35" t="n">
-        <v>17.55</v>
+        <v>17.71</v>
       </c>
       <c r="BR35" t="n">
-        <v>18.42</v>
+        <v>18.32</v>
       </c>
       <c r="BS35" t="n">
         <v>7.3</v>
       </c>
       <c r="BT35" t="n">
-        <v>40165373</v>
+        <v>40863943</v>
       </c>
     </row>
     <row r="36">
@@ -8858,10 +8858,10 @@
         <v>14.5</v>
       </c>
       <c r="G37" t="n">
-        <v>179073405</v>
+        <v>178849960</v>
       </c>
       <c r="H37" t="n">
-        <v>300</v>
+        <v>1000</v>
       </c>
       <c r="I37" t="n">
         <v>4900000</v>
@@ -8876,7 +8876,7 @@
         <v>0.88</v>
       </c>
       <c r="M37" t="n">
-        <v>1.743430447124304</v>
+        <v>1.741255021821716</v>
       </c>
       <c r="N37" t="n">
         <v>0.5</v>
@@ -8954,7 +8954,7 @@
         <v>11319000</v>
       </c>
       <c r="AM37" t="n">
-        <v>42840527.51196173</v>
+        <v>42787071.77033493</v>
       </c>
       <c r="AN37" t="n">
         <v>0</v>
@@ -9022,10 +9022,10 @@
         <v>17.13</v>
       </c>
       <c r="BI37" t="n">
-        <v>0.21</v>
+        <v>0</v>
       </c>
       <c r="BJ37" t="n">
-        <v>14.47</v>
+        <v>14.5</v>
       </c>
       <c r="BK37" t="n">
         <v>2.31</v>
@@ -9055,7 +9055,7 @@
         <v>0.72</v>
       </c>
       <c r="BT37" t="n">
-        <v>1223</v>
+        <v>1233</v>
       </c>
     </row>
     <row r="38">
@@ -9315,13 +9315,13 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>69.37</v>
+        <v>69.29000000000001</v>
       </c>
       <c r="G39" t="n">
-        <v>3888765118</v>
+        <v>3884280351</v>
       </c>
       <c r="H39" t="n">
-        <v>1200</v>
+        <v>2000</v>
       </c>
       <c r="I39" t="n">
         <v>168174945</v>
@@ -9336,7 +9336,7 @@
         <v>0.53</v>
       </c>
       <c r="M39" t="n">
-        <v>0.1951989513810139</v>
+        <v>0.1949738357494382</v>
       </c>
       <c r="N39" t="n">
         <v>0.06</v>
@@ -9414,7 +9414,7 @@
         <v>2536078170.6</v>
       </c>
       <c r="AM39" t="n">
-        <v>408483730.8823529</v>
+        <v>408012641.9117647</v>
       </c>
       <c r="AN39" t="n">
         <v>11.9435</v>
@@ -9455,7 +9455,7 @@
         <v>170.24</v>
       </c>
       <c r="AZ39" t="n">
-        <v>202.68</v>
+        <v>202.44</v>
       </c>
       <c r="BA39" t="n">
         <v>19.01</v>
@@ -9464,28 +9464,28 @@
         <v>91.72</v>
       </c>
       <c r="BC39" t="n">
-        <v>200.57</v>
+        <v>200.92</v>
       </c>
       <c r="BD39" t="n">
-        <v>145.41</v>
+        <v>145.7</v>
       </c>
       <c r="BE39" t="n">
         <v>192.17</v>
       </c>
       <c r="BF39" t="n">
-        <v>-72.59999999999999</v>
+        <v>-72.56</v>
       </c>
       <c r="BG39" t="n">
-        <v>32.22</v>
+        <v>32.38</v>
       </c>
       <c r="BH39" t="n">
         <v>128.13</v>
       </c>
       <c r="BI39" t="n">
-        <v>1.23</v>
+        <v>0</v>
       </c>
       <c r="BJ39" t="n">
-        <v>68.53</v>
+        <v>69.29000000000001</v>
       </c>
       <c r="BK39" t="n">
         <v>15.08</v>
@@ -9494,7 +9494,7 @@
         <v>15.08</v>
       </c>
       <c r="BM39" t="n">
-        <v>69.41</v>
+        <v>69.37</v>
       </c>
       <c r="BN39" t="n">
         <v>74.56</v>
@@ -9503,19 +9503,19 @@
         <v>54.98</v>
       </c>
       <c r="BP39" t="n">
-        <v>68.51000000000001</v>
+        <v>68.5</v>
       </c>
       <c r="BQ39" t="n">
-        <v>4.6</v>
+        <v>4.59</v>
       </c>
       <c r="BR39" t="n">
-        <v>68.51000000000001</v>
+        <v>69.37</v>
       </c>
       <c r="BS39" t="n">
         <v>0.58</v>
       </c>
       <c r="BT39" t="n">
-        <v>3113</v>
+        <v>3027</v>
       </c>
     </row>
     <row r="40">
@@ -9545,13 +9545,13 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>23.07</v>
+        <v>23.02</v>
       </c>
       <c r="G40" t="n">
-        <v>132210338631</v>
+        <v>131923755263</v>
       </c>
       <c r="H40" t="n">
-        <v>0</v>
+        <v>44611100</v>
       </c>
       <c r="I40" t="n">
         <v>5730834040</v>
@@ -9566,7 +9566,7 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="M40" t="n">
-        <v>0.401142529206861</v>
+        <v>0.4002729998019859</v>
       </c>
       <c r="N40" t="n">
         <v>0.05</v>
@@ -9644,7 +9644,7 @@
         <v>15358635227.2</v>
       </c>
       <c r="AM40" t="n">
-        <v>6857382709.076763</v>
+        <v>6842518426.504149</v>
       </c>
       <c r="AN40" t="n">
         <v>0.5641</v>
@@ -9685,7 +9685,7 @@
         <v>36.13</v>
       </c>
       <c r="AZ40" t="n">
-        <v>11.65</v>
+        <v>11.63</v>
       </c>
       <c r="BA40" t="n">
         <v>2.76</v>
@@ -9694,28 +9694,28 @@
         <v>27.89</v>
       </c>
       <c r="BC40" t="n">
-        <v>91.8</v>
+        <v>92.22</v>
       </c>
       <c r="BD40" t="n">
-        <v>56.61</v>
+        <v>56.95</v>
       </c>
       <c r="BE40" t="n">
         <v>-49.5</v>
       </c>
       <c r="BF40" t="n">
-        <v>-88.04000000000001</v>
+        <v>-88.01000000000001</v>
       </c>
       <c r="BG40" t="n">
-        <v>20.89</v>
+        <v>21.16</v>
       </c>
       <c r="BH40" t="n">
         <v>32.47</v>
       </c>
       <c r="BI40" t="n">
-        <v>4.67</v>
+        <v>0</v>
       </c>
       <c r="BJ40" t="n">
-        <v>22.04</v>
+        <v>23.02</v>
       </c>
       <c r="BK40" t="n">
         <v>2.68</v>
@@ -9724,7 +9724,7 @@
         <v>2.5</v>
       </c>
       <c r="BM40" t="n">
-        <v>23.07</v>
+        <v>23.21</v>
       </c>
       <c r="BN40" t="n">
         <v>27.36</v>
@@ -9733,19 +9733,19 @@
         <v>17.67</v>
       </c>
       <c r="BP40" t="n">
-        <v>22.23</v>
+        <v>22.66</v>
       </c>
       <c r="BQ40" t="n">
-        <v>9.23</v>
+        <v>9.210000000000001</v>
       </c>
       <c r="BR40" t="n">
-        <v>22.5</v>
+        <v>23.07</v>
       </c>
       <c r="BS40" t="n">
         <v>0.39</v>
       </c>
       <c r="BT40" t="n">
-        <v>37410833</v>
+        <v>37951823</v>
       </c>
     </row>
     <row r="41">
@@ -9775,13 +9775,13 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>16.22</v>
+        <v>16.3</v>
       </c>
       <c r="G41" t="n">
-        <v>194821269309</v>
+        <v>195044606494</v>
       </c>
       <c r="H41" t="n">
-        <v>0</v>
+        <v>73450200</v>
       </c>
       <c r="I41" t="n">
         <v>5303870781</v>
@@ -9796,7 +9796,7 @@
         <v>0.92</v>
       </c>
       <c r="M41" t="n">
-        <v>1.298282793487345</v>
+        <v>1.299771105443528</v>
       </c>
       <c r="N41" t="n">
         <v>0.07000000000000001</v>
@@ -9874,7 +9874,7 @@
         <v>12304980211.92</v>
       </c>
       <c r="AM41" t="n">
-        <v>30018685563.79045</v>
+        <v>30053098073.03544</v>
       </c>
       <c r="AN41" t="n">
         <v>1.6841</v>
@@ -9915,7 +9915,7 @@
         <v>24.4</v>
       </c>
       <c r="AZ41" t="n">
-        <v>24.28</v>
+        <v>24.4</v>
       </c>
       <c r="BA41" t="n">
         <v>2.53</v>
@@ -9924,28 +9924,28 @@
         <v>13.77</v>
       </c>
       <c r="BC41" t="n">
-        <v>84.25</v>
+        <v>83.34999999999999</v>
       </c>
       <c r="BD41" t="n">
-        <v>50.44</v>
+        <v>49.7</v>
       </c>
       <c r="BE41" t="n">
         <v>49.67</v>
       </c>
       <c r="BF41" t="n">
-        <v>-84.42</v>
+        <v>-84.5</v>
       </c>
       <c r="BG41" t="n">
-        <v>-15.1</v>
+        <v>-15.52</v>
       </c>
       <c r="BH41" t="n">
         <v>17.11</v>
       </c>
       <c r="BI41" t="n">
-        <v>3.64</v>
+        <v>0.09</v>
       </c>
       <c r="BJ41" t="n">
-        <v>15.65</v>
+        <v>16.29</v>
       </c>
       <c r="BK41" t="n">
         <v>2.32</v>
@@ -9954,28 +9954,28 @@
         <v>2.34</v>
       </c>
       <c r="BM41" t="n">
-        <v>16.31</v>
+        <v>16.42</v>
       </c>
       <c r="BN41" t="n">
-        <v>18.28</v>
+        <v>18.26</v>
       </c>
       <c r="BO41" t="n">
-        <v>13.43</v>
+        <v>13.41</v>
       </c>
       <c r="BP41" t="n">
-        <v>15.87</v>
+        <v>15.93</v>
       </c>
       <c r="BQ41" t="n">
-        <v>6.94</v>
+        <v>6.97</v>
       </c>
       <c r="BR41" t="n">
-        <v>15.98</v>
+        <v>16.23</v>
       </c>
       <c r="BS41" t="n">
         <v>0.5600000000000001</v>
       </c>
       <c r="BT41" t="n">
-        <v>7317057</v>
+        <v>7533983</v>
       </c>
     </row>
     <row r="42">
@@ -10005,13 +10005,13 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>18.51</v>
+        <v>18.57</v>
       </c>
       <c r="G42" t="n">
-        <v>194821269309</v>
+        <v>195044606494</v>
       </c>
       <c r="H42" t="n">
-        <v>0</v>
+        <v>96439600</v>
       </c>
       <c r="I42" t="n">
         <v>5288141247</v>
@@ -10026,7 +10026,7 @@
         <v>1.05</v>
       </c>
       <c r="M42" t="n">
-        <v>1.302144525311048</v>
+        <v>1.303637264239285</v>
       </c>
       <c r="N42" t="n">
         <v>0.08</v>
@@ -10104,7 +10104,7 @@
         <v>12268487693.04</v>
       </c>
       <c r="AM42" t="n">
-        <v>26506295144.08163</v>
+        <v>26536681155.64626</v>
       </c>
       <c r="AN42" t="n">
         <v>1.8491</v>
@@ -10145,7 +10145,7 @@
         <v>24.4</v>
       </c>
       <c r="AZ42" t="n">
-        <v>26.81</v>
+        <v>26.9</v>
       </c>
       <c r="BA42" t="n">
         <v>2.53</v>
@@ -10154,28 +10154,28 @@
         <v>15.11</v>
       </c>
       <c r="BC42" t="n">
-        <v>61.46</v>
+        <v>60.93</v>
       </c>
       <c r="BD42" t="n">
-        <v>31.83</v>
+        <v>31.4</v>
       </c>
       <c r="BE42" t="n">
         <v>44.83</v>
       </c>
       <c r="BF42" t="n">
-        <v>-86.34999999999999</v>
+        <v>-86.39</v>
       </c>
       <c r="BG42" t="n">
-        <v>-18.34</v>
+        <v>-18.61</v>
       </c>
       <c r="BH42" t="n">
         <v>17.11</v>
       </c>
       <c r="BI42" t="n">
-        <v>4.11</v>
+        <v>0.08</v>
       </c>
       <c r="BJ42" t="n">
-        <v>17.78</v>
+        <v>18.55</v>
       </c>
       <c r="BK42" t="n">
         <v>2.32</v>
@@ -10184,28 +10184,28 @@
         <v>2.34</v>
       </c>
       <c r="BM42" t="n">
-        <v>18.54</v>
+        <v>18.72</v>
       </c>
       <c r="BN42" t="n">
-        <v>21.33</v>
+        <v>21.32</v>
       </c>
       <c r="BO42" t="n">
-        <v>15.67</v>
+        <v>15.65</v>
       </c>
       <c r="BP42" t="n">
-        <v>17.97</v>
+        <v>18.1</v>
       </c>
       <c r="BQ42" t="n">
-        <v>7.92</v>
+        <v>7.94</v>
       </c>
       <c r="BR42" t="n">
-        <v>18.15</v>
+        <v>18.44</v>
       </c>
       <c r="BS42" t="n">
         <v>0.63</v>
       </c>
       <c r="BT42" t="n">
-        <v>40003400</v>
+        <v>41125453</v>
       </c>
     </row>
     <row r="43">
@@ -10235,13 +10235,13 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>39.18</v>
+        <v>39.19</v>
       </c>
       <c r="G43" t="n">
-        <v>76064013412</v>
+        <v>76083424143</v>
       </c>
       <c r="H43" t="n">
-        <v>0</v>
+        <v>4510400</v>
       </c>
       <c r="I43" t="n">
         <v>1941400000</v>
@@ -10334,7 +10334,7 @@
         <v>9182822000</v>
       </c>
       <c r="AM43" t="n">
-        <v>9264800659.196102</v>
+        <v>9267164938.24604</v>
       </c>
       <c r="AN43" t="n">
         <v>4.5901</v>
@@ -10375,7 +10375,7 @@
         <v>19.95</v>
       </c>
       <c r="AZ43" t="n">
-        <v>71.11</v>
+        <v>71.13</v>
       </c>
       <c r="BA43" t="n">
         <v>5.63</v>
@@ -10384,28 +10384,28 @@
         <v>48.62</v>
       </c>
       <c r="BC43" t="n">
-        <v>-37.64</v>
+        <v>-37.65</v>
       </c>
       <c r="BD43" t="n">
-        <v>-49.08</v>
+        <v>-49.09</v>
       </c>
       <c r="BE43" t="n">
         <v>81.5</v>
       </c>
       <c r="BF43" t="n">
-        <v>-85.63</v>
+        <v>-85.64</v>
       </c>
       <c r="BG43" t="n">
-        <v>24.09</v>
+        <v>24.06</v>
       </c>
       <c r="BH43" t="n">
         <v>5.61</v>
       </c>
       <c r="BI43" t="n">
-        <v>1.08</v>
+        <v>0</v>
       </c>
       <c r="BJ43" t="n">
-        <v>38.76</v>
+        <v>39.19</v>
       </c>
       <c r="BK43" t="n">
         <v>4.73</v>
@@ -10414,7 +10414,7 @@
         <v>4.73</v>
       </c>
       <c r="BM43" t="n">
-        <v>39.49</v>
+        <v>39.47</v>
       </c>
       <c r="BN43" t="n">
         <v>42.98</v>
@@ -10423,19 +10423,19 @@
         <v>28.06</v>
       </c>
       <c r="BP43" t="n">
-        <v>38.92</v>
+        <v>38.9</v>
       </c>
       <c r="BQ43" t="n">
         <v>8.279999999999999</v>
       </c>
       <c r="BR43" t="n">
-        <v>39.09</v>
+        <v>39.31</v>
       </c>
       <c r="BS43" t="n">
         <v>0</v>
       </c>
       <c r="BT43" t="n">
-        <v>6310687</v>
+        <v>6381763</v>
       </c>
     </row>
     <row r="44">
@@ -10925,13 +10925,13 @@
         </is>
       </c>
       <c r="F46" t="n">
-        <v>3.94</v>
+        <v>3.9</v>
       </c>
       <c r="G46" t="n">
-        <v>3942135537</v>
+        <v>3902113895</v>
       </c>
       <c r="H46" t="n">
-        <v>0</v>
+        <v>22662100</v>
       </c>
       <c r="I46" t="n">
         <v>1000542188</v>
@@ -10946,7 +10946,7 @@
         <v>2.5</v>
       </c>
       <c r="M46" t="n">
-        <v>0.06852172724609572</v>
+        <v>0.06782607586340586</v>
       </c>
       <c r="N46" t="n">
         <v>0.08</v>
@@ -11024,7 +11024,7 @@
         <v>460249406.48</v>
       </c>
       <c r="AM46" t="n">
-        <v>3864838761.764706</v>
+        <v>3825601857.843137</v>
       </c>
       <c r="AN46" t="n">
         <v>0.0311</v>
@@ -11065,7 +11065,7 @@
         <v>3.3</v>
       </c>
       <c r="AZ46" t="n">
-        <v>3.25</v>
+        <v>3.22</v>
       </c>
       <c r="BA46" t="n">
         <v>0.42</v>
@@ -11074,28 +11074,28 @@
         <v>7.38</v>
       </c>
       <c r="BC46" t="n">
-        <v>2.64</v>
+        <v>3.69</v>
       </c>
       <c r="BD46" t="n">
-        <v>-16.2</v>
+        <v>-15.34</v>
       </c>
       <c r="BE46" t="n">
         <v>-17.5</v>
       </c>
       <c r="BF46" t="n">
-        <v>-89.26000000000001</v>
+        <v>-89.15000000000001</v>
       </c>
       <c r="BG46" t="n">
-        <v>87.27</v>
+        <v>89.2</v>
       </c>
       <c r="BH46" t="n">
         <v>1.58</v>
       </c>
       <c r="BI46" t="n">
-        <v>0.51</v>
+        <v>0</v>
       </c>
       <c r="BJ46" t="n">
-        <v>3.92</v>
+        <v>3.9</v>
       </c>
       <c r="BK46" t="n">
         <v>0.46</v>
@@ -11104,7 +11104,7 @@
         <v>0.46</v>
       </c>
       <c r="BM46" t="n">
-        <v>4.06</v>
+        <v>3.99</v>
       </c>
       <c r="BN46" t="n">
         <v>7.31</v>
@@ -11113,19 +11113,19 @@
         <v>2.97</v>
       </c>
       <c r="BP46" t="n">
-        <v>3.91</v>
+        <v>3.82</v>
       </c>
       <c r="BQ46" t="n">
-        <v>8.609999999999999</v>
+        <v>8.529999999999999</v>
       </c>
       <c r="BR46" t="n">
-        <v>3.96</v>
+        <v>3.99</v>
       </c>
       <c r="BS46" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="BT46" t="n">
-        <v>21865118</v>
+        <v>21552368</v>
       </c>
     </row>
     <row r="47">
@@ -11155,13 +11155,13 @@
         </is>
       </c>
       <c r="F47" t="n">
-        <v>9.130000000000001</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="G47" t="n">
-        <v>3179300680</v>
+        <v>3252717846</v>
       </c>
       <c r="H47" t="n">
-        <v>13500</v>
+        <v>27700</v>
       </c>
       <c r="I47" t="n">
         <v>254106600</v>
@@ -11176,7 +11176,7 @@
         <v>1.22</v>
       </c>
       <c r="M47" t="n">
-        <v>0.7497156790251789</v>
+        <v>0.7670282914515677</v>
       </c>
       <c r="N47" t="n">
         <v>0.07000000000000001</v>
@@ -11254,7 +11254,7 @@
         <v>322715382</v>
       </c>
       <c r="AM47" t="n">
-        <v>563705794.3262411</v>
+        <v>576723022.3404256</v>
       </c>
       <c r="AN47" t="n">
         <v>0.4132</v>
@@ -11295,7 +11295,7 @@
         <v>11.74</v>
       </c>
       <c r="AZ47" t="n">
-        <v>11.99</v>
+        <v>12.21</v>
       </c>
       <c r="BA47" t="n">
         <v>1.46</v>
@@ -11304,28 +11304,28 @@
         <v>8.619999999999999</v>
       </c>
       <c r="BC47" t="n">
-        <v>57.43</v>
+        <v>54.55</v>
       </c>
       <c r="BD47" t="n">
-        <v>28.54</v>
+        <v>26.19</v>
       </c>
       <c r="BE47" t="n">
         <v>31.33</v>
       </c>
       <c r="BF47" t="n">
-        <v>-84.03</v>
+        <v>-84.31999999999999</v>
       </c>
       <c r="BG47" t="n">
-        <v>-5.59</v>
+        <v>-7.31</v>
       </c>
       <c r="BH47" t="n">
         <v>7.23</v>
       </c>
       <c r="BI47" t="n">
-        <v>0.77</v>
+        <v>0.92</v>
       </c>
       <c r="BJ47" t="n">
-        <v>9.06</v>
+        <v>9.220000000000001</v>
       </c>
       <c r="BK47" t="n">
         <v>1.27</v>
@@ -11334,28 +11334,28 @@
         <v>1.28</v>
       </c>
       <c r="BM47" t="n">
-        <v>9.199999999999999</v>
+        <v>9.35</v>
       </c>
       <c r="BN47" t="n">
+        <v>9.35</v>
+      </c>
+      <c r="BO47" t="n">
+        <v>7.17</v>
+      </c>
+      <c r="BP47" t="n">
         <v>9.24</v>
       </c>
-      <c r="BO47" t="n">
-        <v>7.19</v>
-      </c>
-      <c r="BP47" t="n">
-        <v>9.06</v>
-      </c>
       <c r="BQ47" t="n">
-        <v>7.12</v>
+        <v>7.25</v>
       </c>
       <c r="BR47" t="n">
-        <v>9.09</v>
+        <v>9.289999999999999</v>
       </c>
       <c r="BS47" t="n">
         <v>0.53</v>
       </c>
       <c r="BT47" t="n">
-        <v>10017</v>
+        <v>10117</v>
       </c>
     </row>
     <row r="48">
@@ -11385,13 +11385,13 @@
         </is>
       </c>
       <c r="F48" t="n">
-        <v>9.35</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="G48" t="n">
-        <v>3179300680</v>
+        <v>3252717846</v>
       </c>
       <c r="H48" t="n">
-        <v>4700</v>
+        <v>6500</v>
       </c>
       <c r="I48" t="n">
         <v>93397546</v>
@@ -11406,7 +11406,7 @@
         <v>1.24</v>
       </c>
       <c r="M48" t="n">
-        <v>2.039750617899313</v>
+        <v>2.086853023360667</v>
       </c>
       <c r="N48" t="n">
         <v>0.07000000000000001</v>
@@ -11484,7 +11484,7 @@
         <v>118614883.42</v>
       </c>
       <c r="AM48" t="n">
-        <v>555821797.2027972</v>
+        <v>568656966.0839161</v>
       </c>
       <c r="AN48" t="n">
         <v>0.4132</v>
@@ -11525,7 +11525,7 @@
         <v>11.74</v>
       </c>
       <c r="AZ48" t="n">
-        <v>12.23</v>
+        <v>12.17</v>
       </c>
       <c r="BA48" t="n">
         <v>1.46</v>
@@ -11534,28 +11534,28 @@
         <v>8.24</v>
       </c>
       <c r="BC48" t="n">
-        <v>53.73</v>
+        <v>54.55</v>
       </c>
       <c r="BD48" t="n">
-        <v>25.52</v>
+        <v>26.19</v>
       </c>
       <c r="BE48" t="n">
         <v>30.83</v>
       </c>
       <c r="BF48" t="n">
-        <v>-84.40000000000001</v>
+        <v>-84.31999999999999</v>
       </c>
       <c r="BG48" t="n">
-        <v>-11.91</v>
+        <v>-11.44</v>
       </c>
       <c r="BH48" t="n">
         <v>7.23</v>
       </c>
       <c r="BI48" t="n">
-        <v>2.41</v>
+        <v>0.92</v>
       </c>
       <c r="BJ48" t="n">
-        <v>9.130000000000001</v>
+        <v>9.220000000000001</v>
       </c>
       <c r="BK48" t="n">
         <v>1.27</v>
@@ -11564,28 +11564,28 @@
         <v>1.28</v>
       </c>
       <c r="BM48" t="n">
-        <v>9.35</v>
+        <v>9.51</v>
       </c>
       <c r="BN48" t="n">
-        <v>9.48</v>
+        <v>9.51</v>
       </c>
       <c r="BO48" t="n">
-        <v>7.2</v>
+        <v>7.18</v>
       </c>
       <c r="BP48" t="n">
-        <v>9.18</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="BQ48" t="n">
-        <v>7.29</v>
+        <v>7.25</v>
       </c>
       <c r="BR48" t="n">
-        <v>9.18</v>
+        <v>9.41</v>
       </c>
       <c r="BS48" t="n">
         <v>0.54</v>
       </c>
       <c r="BT48" t="n">
-        <v>2573</v>
+        <v>2657</v>
       </c>
     </row>
     <row r="49">
@@ -11845,13 +11845,13 @@
         </is>
       </c>
       <c r="F50" t="n">
-        <v>34.6</v>
+        <v>34.14</v>
       </c>
       <c r="G50" t="n">
-        <v>958007600</v>
+        <v>962046900</v>
       </c>
       <c r="H50" t="n">
-        <v>100</v>
+        <v>600</v>
       </c>
       <c r="I50" t="n">
         <v>11540870</v>
@@ -11866,7 +11866,7 @@
         <v>0.8</v>
       </c>
       <c r="M50" t="n">
-        <v>0.9692039320351298</v>
+        <v>0.9732904397441182</v>
       </c>
       <c r="N50" t="n">
         <v>0.06</v>
@@ -11944,7 +11944,7 @@
         <v>84709985.8</v>
       </c>
       <c r="AM50" t="n">
-        <v>326965051.1945392</v>
+        <v>328343651.8771331</v>
       </c>
       <c r="AN50" t="n">
         <v>4.4983</v>
@@ -11985,7 +11985,7 @@
         <v>68.48999999999999</v>
       </c>
       <c r="AZ50" t="n">
-        <v>76.29000000000001</v>
+        <v>75.28</v>
       </c>
       <c r="BA50" t="n">
         <v>9.210000000000001</v>
@@ -11994,28 +11994,28 @@
         <v>30.53</v>
       </c>
       <c r="BC50" t="n">
-        <v>142.42</v>
+        <v>145.69</v>
       </c>
       <c r="BD50" t="n">
-        <v>97.93000000000001</v>
+        <v>100.6</v>
       </c>
       <c r="BE50" t="n">
         <v>120.5</v>
       </c>
       <c r="BF50" t="n">
-        <v>-73.37</v>
+        <v>-73.01000000000001</v>
       </c>
       <c r="BG50" t="n">
-        <v>-11.76</v>
+        <v>-10.57</v>
       </c>
       <c r="BH50" t="n">
         <v>42.6</v>
       </c>
       <c r="BI50" t="n">
-        <v>1.02</v>
+        <v>0</v>
       </c>
       <c r="BJ50" t="n">
-        <v>34.25</v>
+        <v>34.14</v>
       </c>
       <c r="BK50" t="n">
         <v>7.34</v>
@@ -12024,28 +12024,28 @@
         <v>7.6</v>
       </c>
       <c r="BM50" t="n">
-        <v>34.6</v>
+        <v>34.15</v>
       </c>
       <c r="BN50" t="n">
         <v>39.22</v>
       </c>
       <c r="BO50" t="n">
-        <v>23.5</v>
+        <v>23.69</v>
       </c>
       <c r="BP50" t="n">
-        <v>34.6</v>
+        <v>33.65</v>
       </c>
       <c r="BQ50" t="n">
-        <v>4.55</v>
+        <v>4.49</v>
       </c>
       <c r="BR50" t="n">
-        <v>34.6</v>
+        <v>34.15</v>
       </c>
       <c r="BS50" t="n">
         <v>0.4</v>
       </c>
       <c r="BT50" t="n">
-        <v>510</v>
+        <v>513</v>
       </c>
     </row>
     <row r="51">
@@ -12523,13 +12523,13 @@
         </is>
       </c>
       <c r="F53" t="n">
-        <v>6.1</v>
+        <v>6.06</v>
       </c>
       <c r="G53" t="n">
-        <v>834799626</v>
+        <v>829325536</v>
       </c>
       <c r="H53" t="n">
-        <v>55200</v>
+        <v>46800</v>
       </c>
       <c r="I53" t="n">
         <v>136852484</v>
@@ -12544,7 +12544,7 @@
         <v>2.79</v>
       </c>
       <c r="M53" t="n">
-        <v>2.168653804924725</v>
+        <v>2.154433139585088</v>
       </c>
       <c r="N53" t="n">
         <v>1.48</v>
@@ -12622,7 +12622,7 @@
         <v>39687220.36</v>
       </c>
       <c r="AM53" t="n">
-        <v>42526725.7259297</v>
+        <v>42247862.25165563</v>
       </c>
       <c r="AN53" t="n">
         <v>0</v>
@@ -12672,16 +12672,16 @@
         <v>0</v>
       </c>
       <c r="BC53" t="n">
-        <v>-35.4</v>
+        <v>-34.97</v>
       </c>
       <c r="BD53" t="n">
-        <v>-47.25</v>
+        <v>-46.9</v>
       </c>
       <c r="BE53" t="n">
         <v>-100</v>
       </c>
       <c r="BF53" t="n">
-        <v>-95.25</v>
+        <v>-95.20999999999999</v>
       </c>
       <c r="BG53" t="n">
         <v>-100</v>
@@ -12690,10 +12690,10 @@
         <v>2.38</v>
       </c>
       <c r="BI53" t="n">
-        <v>3.74</v>
+        <v>0</v>
       </c>
       <c r="BJ53" t="n">
-        <v>5.88</v>
+        <v>6.06</v>
       </c>
       <c r="BK53" t="n">
         <v>0.29</v>
@@ -12702,7 +12702,7 @@
         <v>0.2</v>
       </c>
       <c r="BM53" t="n">
-        <v>6.1</v>
+        <v>6.15</v>
       </c>
       <c r="BN53" t="n">
         <v>10.39</v>
@@ -12711,19 +12711,19 @@
         <v>4.82</v>
       </c>
       <c r="BP53" t="n">
-        <v>5.78</v>
+        <v>5.84</v>
       </c>
       <c r="BQ53" t="n">
-        <v>29.96</v>
+        <v>29.77</v>
       </c>
       <c r="BR53" t="n">
-        <v>5.98</v>
+        <v>6.11</v>
       </c>
       <c r="BS53" t="n">
         <v>2.36</v>
       </c>
       <c r="BT53" t="n">
-        <v>34733</v>
+        <v>35620</v>
       </c>
     </row>
     <row r="54">
@@ -12753,13 +12753,13 @@
         </is>
       </c>
       <c r="F54" t="n">
-        <v>10.71</v>
+        <v>10.74</v>
       </c>
       <c r="G54" t="n">
-        <v>2497700528</v>
+        <v>2504697900</v>
       </c>
       <c r="H54" t="n">
-        <v>287200</v>
+        <v>131300</v>
       </c>
       <c r="I54" t="n">
         <v>233212121</v>
@@ -12774,7 +12774,7 @@
         <v>0.97</v>
       </c>
       <c r="M54" t="n">
-        <v>1.40193827710696</v>
+        <v>1.405865843096551</v>
       </c>
       <c r="N54" t="n">
         <v>0.5600000000000001</v>
@@ -12852,7 +12852,7 @@
         <v>233212121</v>
       </c>
       <c r="AM54" t="n">
-        <v>341682698.7688099</v>
+        <v>342639931.6005472</v>
       </c>
       <c r="AN54" t="n">
         <v>0.1531</v>
@@ -12893,7 +12893,7 @@
         <v>12.25</v>
       </c>
       <c r="AZ54" t="n">
-        <v>17.05</v>
+        <v>17.09</v>
       </c>
       <c r="BA54" t="n">
         <v>0.98</v>
@@ -12902,28 +12902,28 @@
         <v>6.52</v>
       </c>
       <c r="BC54" t="n">
-        <v>40.13</v>
+        <v>39.73</v>
       </c>
       <c r="BD54" t="n">
-        <v>14.41</v>
+        <v>14.09</v>
       </c>
       <c r="BE54" t="n">
         <v>59.17</v>
       </c>
       <c r="BF54" t="n">
-        <v>-90.81999999999999</v>
+        <v>-90.84</v>
       </c>
       <c r="BG54" t="n">
-        <v>-39.16</v>
+        <v>-39.33</v>
       </c>
       <c r="BH54" t="n">
         <v>10.01</v>
       </c>
       <c r="BI54" t="n">
-        <v>2.51</v>
+        <v>0</v>
       </c>
       <c r="BJ54" t="n">
-        <v>10.45</v>
+        <v>10.74</v>
       </c>
       <c r="BK54" t="n">
         <v>1</v>
@@ -12932,7 +12932,7 @@
         <v>1</v>
       </c>
       <c r="BM54" t="n">
-        <v>10.73</v>
+        <v>10.79</v>
       </c>
       <c r="BN54" t="n">
         <v>11.68</v>
@@ -12941,19 +12941,19 @@
         <v>8.23</v>
       </c>
       <c r="BP54" t="n">
-        <v>10.39</v>
+        <v>10.62</v>
       </c>
       <c r="BQ54" t="n">
-        <v>10.68</v>
+        <v>10.71</v>
       </c>
       <c r="BR54" t="n">
-        <v>10.5</v>
+        <v>10.7</v>
       </c>
       <c r="BS54" t="n">
         <v>1.26</v>
       </c>
       <c r="BT54" t="n">
-        <v>240917</v>
+        <v>244503</v>
       </c>
     </row>
     <row r="55">
@@ -12983,13 +12983,13 @@
         </is>
       </c>
       <c r="F55" t="n">
-        <v>49.48</v>
+        <v>49.42</v>
       </c>
       <c r="G55" t="n">
-        <v>6599884943</v>
+        <v>6429320510</v>
       </c>
       <c r="H55" t="n">
-        <v>2900</v>
+        <v>3900</v>
       </c>
       <c r="I55" t="n">
         <v>84052790</v>
@@ -13004,7 +13004,7 @@
         <v>2</v>
       </c>
       <c r="M55" t="n">
-        <v>1.018831884050305</v>
+        <v>0.9925016549438603</v>
       </c>
       <c r="N55" t="n">
         <v>0.16</v>
@@ -13082,7 +13082,7 @@
         <v>579123723.1</v>
       </c>
       <c r="AM55" t="n">
-        <v>331986164.1348089</v>
+        <v>323406464.2857143</v>
       </c>
       <c r="AN55" t="n">
         <v>3.1953</v>
@@ -13123,7 +13123,7 @@
         <v>51.21</v>
       </c>
       <c r="AZ55" t="n">
-        <v>52.04</v>
+        <v>51.97</v>
       </c>
       <c r="BA55" t="n">
         <v>9.380000000000001</v>
@@ -13132,28 +13132,28 @@
         <v>16.08</v>
       </c>
       <c r="BC55" t="n">
-        <v>26.75</v>
+        <v>26.9</v>
       </c>
       <c r="BD55" t="n">
-        <v>3.49</v>
+        <v>3.61</v>
       </c>
       <c r="BE55" t="n">
         <v>5.17</v>
       </c>
       <c r="BF55" t="n">
-        <v>-81.05</v>
+        <v>-81.02</v>
       </c>
       <c r="BG55" t="n">
-        <v>-67.51000000000001</v>
+        <v>-67.47</v>
       </c>
       <c r="BH55" t="n">
         <v>25.37</v>
       </c>
       <c r="BI55" t="n">
-        <v>0.37</v>
+        <v>0</v>
       </c>
       <c r="BJ55" t="n">
-        <v>49.3</v>
+        <v>49.42</v>
       </c>
       <c r="BK55" t="n">
         <v>6.89</v>
@@ -13162,7 +13162,7 @@
         <v>7.03</v>
       </c>
       <c r="BM55" t="n">
-        <v>49.61</v>
+        <v>49.95</v>
       </c>
       <c r="BN55" t="n">
         <v>73.67</v>
@@ -13171,19 +13171,19 @@
         <v>35.58</v>
       </c>
       <c r="BP55" t="n">
-        <v>49.4</v>
+        <v>49.42</v>
       </c>
       <c r="BQ55" t="n">
-        <v>7.04</v>
+        <v>7.03</v>
       </c>
       <c r="BR55" t="n">
-        <v>49.42</v>
+        <v>49.95</v>
       </c>
       <c r="BS55" t="n">
         <v>0.66</v>
       </c>
       <c r="BT55" t="n">
-        <v>5943</v>
+        <v>5947</v>
       </c>
     </row>
     <row r="56">
@@ -13213,13 +13213,13 @@
         </is>
       </c>
       <c r="F56" t="n">
-        <v>59.65</v>
+        <v>58.77</v>
       </c>
       <c r="G56" t="n">
-        <v>6599884943</v>
+        <v>6429320510</v>
       </c>
       <c r="H56" t="n">
-        <v>17600</v>
+        <v>13300</v>
       </c>
       <c r="I56" t="n">
         <v>39675836</v>
@@ -13234,7 +13234,7 @@
         <v>2.41</v>
       </c>
       <c r="M56" t="n">
-        <v>2.158383314100417</v>
+        <v>2.102603034694689</v>
       </c>
       <c r="N56" t="n">
         <v>0.19</v>
@@ -13312,7 +13312,7 @@
         <v>273366510.04</v>
       </c>
       <c r="AM56" t="n">
-        <v>274537643.2196339</v>
+        <v>267442616.8885191</v>
       </c>
       <c r="AN56" t="n">
         <v>3.5102</v>
@@ -13353,7 +13353,7 @@
         <v>51.21</v>
       </c>
       <c r="AZ56" t="n">
-        <v>56.97</v>
+        <v>56.13</v>
       </c>
       <c r="BA56" t="n">
         <v>9.380000000000001</v>
@@ -13362,28 +13362,28 @@
         <v>17.68</v>
       </c>
       <c r="BC56" t="n">
-        <v>5.14</v>
+        <v>6.71</v>
       </c>
       <c r="BD56" t="n">
-        <v>-14.16</v>
+        <v>-12.87</v>
       </c>
       <c r="BE56" t="n">
         <v>-4.5</v>
       </c>
       <c r="BF56" t="n">
-        <v>-84.28</v>
+        <v>-84.04000000000001</v>
       </c>
       <c r="BG56" t="n">
-        <v>-70.36</v>
+        <v>-69.92</v>
       </c>
       <c r="BH56" t="n">
         <v>25.37</v>
       </c>
       <c r="BI56" t="n">
-        <v>2.16</v>
+        <v>0</v>
       </c>
       <c r="BJ56" t="n">
-        <v>58.39</v>
+        <v>58.77</v>
       </c>
       <c r="BK56" t="n">
         <v>6.89</v>
@@ -13392,7 +13392,7 @@
         <v>7.03</v>
       </c>
       <c r="BM56" t="n">
-        <v>59.94</v>
+        <v>59.74</v>
       </c>
       <c r="BN56" t="n">
         <v>86.77</v>
@@ -13401,19 +13401,19 @@
         <v>46.42</v>
       </c>
       <c r="BP56" t="n">
-        <v>57.57</v>
+        <v>58.75</v>
       </c>
       <c r="BQ56" t="n">
-        <v>8.48</v>
+        <v>8.359999999999999</v>
       </c>
       <c r="BR56" t="n">
-        <v>57.57</v>
+        <v>59.65</v>
       </c>
       <c r="BS56" t="n">
         <v>0.79</v>
       </c>
       <c r="BT56" t="n">
-        <v>29353</v>
+        <v>28630</v>
       </c>
     </row>
     <row r="57">
@@ -13443,13 +13443,13 @@
         </is>
       </c>
       <c r="F57" t="n">
-        <v>6.38</v>
+        <v>6.51</v>
       </c>
       <c r="G57" t="n">
-        <v>1492014066</v>
+        <v>1522414982</v>
       </c>
       <c r="H57" t="n">
-        <v>2314300</v>
+        <v>2748000</v>
       </c>
       <c r="I57" t="n">
         <v>233858065</v>
@@ -13464,7 +13464,7 @@
         <v>0.77</v>
       </c>
       <c r="M57" t="n">
-        <v>0.44659988365165</v>
+        <v>0.4556996943423782</v>
       </c>
       <c r="N57" t="n">
         <v>0.08</v>
@@ -13542,7 +13542,7 @@
         <v>229180903.7</v>
       </c>
       <c r="AM57" t="n">
-        <v>111594170.9798055</v>
+        <v>113867986.6866118</v>
       </c>
       <c r="AN57" t="n">
         <v>0.347</v>
@@ -13583,7 +13583,7 @@
         <v>10.72</v>
       </c>
       <c r="AZ57" t="n">
-        <v>9.73</v>
+        <v>9.93</v>
       </c>
       <c r="BA57" t="n">
         <v>1.13</v>
@@ -13592,28 +13592,28 @@
         <v>6.26</v>
       </c>
       <c r="BC57" t="n">
-        <v>105.82</v>
+        <v>101.71</v>
       </c>
       <c r="BD57" t="n">
-        <v>68.05</v>
+        <v>64.7</v>
       </c>
       <c r="BE57" t="n">
         <v>52.5</v>
       </c>
       <c r="BF57" t="n">
-        <v>-82.33</v>
+        <v>-82.68000000000001</v>
       </c>
       <c r="BG57" t="n">
-        <v>-1.82</v>
+        <v>-3.78</v>
       </c>
       <c r="BH57" t="n">
         <v>7.82</v>
       </c>
       <c r="BI57" t="n">
-        <v>4.93</v>
+        <v>0</v>
       </c>
       <c r="BJ57" t="n">
-        <v>6.08</v>
+        <v>6.51</v>
       </c>
       <c r="BK57" t="n">
         <v>0.98</v>
@@ -13622,28 +13622,28 @@
         <v>1.04</v>
       </c>
       <c r="BM57" t="n">
-        <v>6.38</v>
+        <v>6.52</v>
       </c>
       <c r="BN57" t="n">
-        <v>6.38</v>
+        <v>6.52</v>
       </c>
       <c r="BO57" t="n">
         <v>3.43</v>
       </c>
       <c r="BP57" t="n">
-        <v>6.1</v>
+        <v>6.26</v>
       </c>
       <c r="BQ57" t="n">
-        <v>6.16</v>
+        <v>6.28</v>
       </c>
       <c r="BR57" t="n">
-        <v>6.12</v>
+        <v>6.36</v>
       </c>
       <c r="BS57" t="n">
         <v>0.42</v>
       </c>
       <c r="BT57" t="n">
-        <v>1306047</v>
+        <v>1352800</v>
       </c>
     </row>
     <row r="58">
@@ -13676,7 +13676,7 @@
         <v>19.5</v>
       </c>
       <c r="G58" t="n">
-        <v>91920060</v>
+        <v>91920055</v>
       </c>
       <c r="H58" t="n">
         <v>0</v>
@@ -13694,7 +13694,7 @@
         <v>0.63</v>
       </c>
       <c r="M58" t="n">
-        <v>1.685005660276028</v>
+        <v>1.685005568619992</v>
       </c>
       <c r="N58" t="n">
         <v>0.16</v>
@@ -13772,7 +13772,7 @@
         <v>10904901.05</v>
       </c>
       <c r="AM58" t="n">
-        <v>14995115.82381729</v>
+        <v>14995115.00815661</v>
       </c>
       <c r="AN58" t="n">
         <v>0.5117</v>
@@ -13906,7 +13906,7 @@
         <v>20.45</v>
       </c>
       <c r="G59" t="n">
-        <v>91920060</v>
+        <v>91920055</v>
       </c>
       <c r="H59" t="n">
         <v>100</v>
@@ -13924,7 +13924,7 @@
         <v>0.61</v>
       </c>
       <c r="M59" t="n">
-        <v>9.764081793890091</v>
+        <v>9.764081262771976</v>
       </c>
       <c r="N59" t="n">
         <v>0.15</v>
@@ -14002,7 +14002,7 @@
         <v>1881878.95</v>
       </c>
       <c r="AM59" t="n">
-        <v>15527037.16216216</v>
+        <v>15527036.31756757</v>
       </c>
       <c r="AN59" t="n">
         <v>1.4</v>
@@ -14139,7 +14139,7 @@
         <v>171895500</v>
       </c>
       <c r="H60" t="n">
-        <v>64</v>
+        <v>34</v>
       </c>
       <c r="I60" t="n">
         <v>454750</v>
@@ -14300,10 +14300,10 @@
         <v>454.44</v>
       </c>
       <c r="BI60" t="n">
-        <v>-0.48</v>
+        <v>0</v>
       </c>
       <c r="BJ60" t="n">
-        <v>379.81</v>
+        <v>378</v>
       </c>
       <c r="BK60" t="n">
         <v>130.97</v>
@@ -14327,7 +14327,7 @@
         <v>2.89</v>
       </c>
       <c r="BR60" t="n">
-        <v>379.81</v>
+        <v>380</v>
       </c>
       <c r="BS60" t="n">
         <v>12.82</v>
@@ -14363,13 +14363,13 @@
         </is>
       </c>
       <c r="F61" t="n">
-        <v>28.15</v>
+        <v>27.84</v>
       </c>
       <c r="G61" t="n">
-        <v>2409876145</v>
+        <v>2383337312</v>
       </c>
       <c r="H61" t="n">
-        <v>0</v>
+        <v>769100</v>
       </c>
       <c r="I61" t="n">
         <v>85608392</v>
@@ -14384,7 +14384,7 @@
         <v>2.37</v>
       </c>
       <c r="M61" t="n">
-        <v>1.278040059327848</v>
+        <v>1.263965605015255</v>
       </c>
       <c r="N61" t="n">
         <v>1.1</v>
@@ -14462,7 +14462,7 @@
         <v>160087693.04</v>
       </c>
       <c r="AM61" t="n">
-        <v>189158253.1397174</v>
+        <v>187075142.2291994</v>
       </c>
       <c r="AN61" t="n">
         <v>0.38</v>
@@ -14503,7 +14503,7 @@
         <v>17.56</v>
       </c>
       <c r="AZ61" t="n">
-        <v>35.47</v>
+        <v>35.08</v>
       </c>
       <c r="BA61" t="n">
         <v>2.52</v>
@@ -14512,28 +14512,28 @@
         <v>11.76</v>
       </c>
       <c r="BC61" t="n">
-        <v>-23.61</v>
+        <v>-22.76</v>
       </c>
       <c r="BD61" t="n">
-        <v>-37.63</v>
+        <v>-36.93</v>
       </c>
       <c r="BE61" t="n">
         <v>26</v>
       </c>
       <c r="BF61" t="n">
-        <v>-91.04000000000001</v>
+        <v>-90.94</v>
       </c>
       <c r="BG61" t="n">
-        <v>-58.24</v>
+        <v>-57.77</v>
       </c>
       <c r="BH61" t="n">
         <v>10.99</v>
       </c>
       <c r="BI61" t="n">
-        <v>1.85</v>
+        <v>0</v>
       </c>
       <c r="BJ61" t="n">
-        <v>27.64</v>
+        <v>27.84</v>
       </c>
       <c r="BK61" t="n">
         <v>1.87</v>
@@ -14542,7 +14542,7 @@
         <v>1.86</v>
       </c>
       <c r="BM61" t="n">
-        <v>28.65</v>
+        <v>28.54</v>
       </c>
       <c r="BN61" t="n">
         <v>28.68</v>
@@ -14551,19 +14551,19 @@
         <v>19.35</v>
       </c>
       <c r="BP61" t="n">
-        <v>27.78</v>
+        <v>27.62</v>
       </c>
       <c r="BQ61" t="n">
-        <v>15.12</v>
+        <v>14.95</v>
       </c>
       <c r="BR61" t="n">
-        <v>27.86</v>
+        <v>28.16</v>
       </c>
       <c r="BS61" t="n">
         <v>1.19</v>
       </c>
       <c r="BT61" t="n">
-        <v>642187</v>
+        <v>683753</v>
       </c>
     </row>
     <row r="62">
@@ -14760,7 +14760,7 @@
         <v>170.35</v>
       </c>
       <c r="BI62" t="n">
-        <v>1.83</v>
+        <v>0</v>
       </c>
       <c r="BJ62" t="n">
         <v>108.02</v>
@@ -14823,13 +14823,13 @@
         </is>
       </c>
       <c r="F63" t="n">
-        <v>1.6</v>
+        <v>1.57</v>
       </c>
       <c r="G63" t="n">
-        <v>416815526</v>
+        <v>409000242</v>
       </c>
       <c r="H63" t="n">
-        <v>117200</v>
+        <v>6300</v>
       </c>
       <c r="I63" t="n">
         <v>122894462</v>
@@ -14844,7 +14844,7 @@
         <v>-0.22</v>
       </c>
       <c r="M63" t="n">
-        <v>0.5126615867486239</v>
+        <v>0.5030491907450951</v>
       </c>
       <c r="N63" t="n">
         <v>0.37</v>
@@ -14922,7 +14922,7 @@
         <v>31952560.12</v>
       </c>
       <c r="AM63" t="n">
-        <v>236827003.4090909</v>
+        <v>232386501.1363636</v>
       </c>
       <c r="AN63" t="n">
         <v>0</v>
@@ -14981,7 +14981,7 @@
         <v>-100</v>
       </c>
       <c r="BF63" t="n">
-        <v>-81.93000000000001</v>
+        <v>-81.58</v>
       </c>
       <c r="BG63" t="n">
         <v>-100</v>
@@ -14990,10 +14990,10 @@
         <v>-5.91</v>
       </c>
       <c r="BI63" t="n">
-        <v>11.11</v>
+        <v>0</v>
       </c>
       <c r="BJ63" t="n">
-        <v>1.44</v>
+        <v>1.57</v>
       </c>
       <c r="BK63" t="n">
         <v>0.26</v>
@@ -15011,19 +15011,19 @@
         <v>1.16</v>
       </c>
       <c r="BP63" t="n">
-        <v>1.46</v>
+        <v>1.57</v>
       </c>
       <c r="BQ63" t="n">
-        <v>6.13</v>
+        <v>6.01</v>
       </c>
       <c r="BR63" t="n">
-        <v>1.54</v>
+        <v>1.57</v>
       </c>
       <c r="BS63" t="n">
         <v>0.19</v>
       </c>
       <c r="BT63" t="n">
-        <v>27770</v>
+        <v>31337</v>
       </c>
     </row>
     <row r="64">
@@ -15053,13 +15053,13 @@
         </is>
       </c>
       <c r="F64" t="n">
-        <v>64.09999999999999</v>
+        <v>63.7</v>
       </c>
       <c r="G64" t="n">
-        <v>243047964214</v>
+        <v>241321019190</v>
       </c>
       <c r="H64" t="n">
-        <v>0</v>
+        <v>12951900</v>
       </c>
       <c r="I64" t="n">
         <v>0</v>
@@ -15146,13 +15146,13 @@
         <v>41.22</v>
       </c>
       <c r="AK64" t="n">
-        <v>69685417867.71443</v>
+        <v>69190277387.84583</v>
       </c>
       <c r="AL64" t="n">
-        <v>19428294501.51878</v>
+        <v>19290249335.73141</v>
       </c>
       <c r="AM64" t="n">
-        <v>21642739466.96349</v>
+        <v>21488959856.63401</v>
       </c>
       <c r="AN64" t="n">
         <v>1.4201</v>
@@ -15193,7 +15193,7 @@
         <v>38.98</v>
       </c>
       <c r="AZ64" t="n">
-        <v>25.64</v>
+        <v>25.48</v>
       </c>
       <c r="BA64" t="n">
         <v>6.69</v>
@@ -15202,28 +15202,28 @@
         <v>10.4</v>
       </c>
       <c r="BC64" t="n">
-        <v>-25.52</v>
+        <v>-25.05</v>
       </c>
       <c r="BD64" t="n">
-        <v>-39.19</v>
+        <v>-38.81</v>
       </c>
       <c r="BE64" t="n">
         <v>-60</v>
       </c>
       <c r="BF64" t="n">
-        <v>-89.56</v>
+        <v>-89.48999999999999</v>
       </c>
       <c r="BG64" t="n">
-        <v>-83.78</v>
+        <v>-83.68000000000001</v>
       </c>
       <c r="BH64" t="n">
         <v>21.37</v>
       </c>
       <c r="BI64" t="n">
-        <v>1.99</v>
+        <v>0</v>
       </c>
       <c r="BJ64" t="n">
-        <v>62.85</v>
+        <v>63.7</v>
       </c>
       <c r="BK64" t="n">
         <v>4.74</v>
@@ -15232,28 +15232,28 @@
         <v>1.57</v>
       </c>
       <c r="BM64" t="n">
-        <v>64.64</v>
+        <v>64.79000000000001</v>
       </c>
       <c r="BN64" t="n">
-        <v>64.72</v>
+        <v>64.79000000000001</v>
       </c>
       <c r="BO64" t="n">
         <v>44.12</v>
       </c>
       <c r="BP64" t="n">
-        <v>63.23</v>
+        <v>63.07</v>
       </c>
       <c r="BQ64" t="n">
-        <v>40.83</v>
+        <v>40.57</v>
       </c>
       <c r="BR64" t="n">
-        <v>64</v>
+        <v>63.89</v>
       </c>
       <c r="BS64" t="n">
         <v>3.49</v>
       </c>
       <c r="BT64" t="n">
-        <v>10222830</v>
+        <v>10276677</v>
       </c>
     </row>
     <row r="65">
@@ -15283,13 +15283,13 @@
         </is>
       </c>
       <c r="F65" t="n">
-        <v>24.8</v>
+        <v>24.77</v>
       </c>
       <c r="G65" t="n">
-        <v>243047964214</v>
+        <v>241321019190</v>
       </c>
       <c r="H65" t="n">
-        <v>2800</v>
+        <v>9800</v>
       </c>
       <c r="I65" t="n">
         <v>7298813414</v>
@@ -15304,7 +15304,7 @@
         <v>3.29</v>
       </c>
       <c r="M65" t="n">
-        <v>5.875913700400474</v>
+        <v>5.834163176140064</v>
       </c>
       <c r="N65" t="n">
         <v>0.29</v>
@@ -15382,7 +15382,7 @@
         <v>11532125194.12</v>
       </c>
       <c r="AM65" t="n">
-        <v>18205840016.02996</v>
+        <v>18076480838.20225</v>
       </c>
       <c r="AN65" t="n">
         <v>0.4734</v>
@@ -15423,7 +15423,7 @@
         <v>12.99</v>
       </c>
       <c r="AZ65" t="n">
-        <v>8.35</v>
+        <v>8.34</v>
       </c>
       <c r="BA65" t="n">
         <v>2.23</v>
@@ -15432,28 +15432,28 @@
         <v>3.47</v>
       </c>
       <c r="BC65" t="n">
-        <v>-35.85</v>
+        <v>-35.77</v>
       </c>
       <c r="BD65" t="n">
-        <v>-47.62</v>
+        <v>-47.56</v>
       </c>
       <c r="BE65" t="n">
         <v>-66.33</v>
       </c>
       <c r="BF65" t="n">
-        <v>-91</v>
+        <v>-90.98999999999999</v>
       </c>
       <c r="BG65" t="n">
-        <v>-86.03</v>
+        <v>-86.01000000000001</v>
       </c>
       <c r="BH65" t="n">
         <v>7.12</v>
       </c>
       <c r="BI65" t="n">
-        <v>2.48</v>
+        <v>0</v>
       </c>
       <c r="BJ65" t="n">
-        <v>24.2</v>
+        <v>24.77</v>
       </c>
       <c r="BK65" t="n">
         <v>1.58</v>
@@ -15462,7 +15462,7 @@
         <v>1.57</v>
       </c>
       <c r="BM65" t="n">
-        <v>24.8</v>
+        <v>24.99</v>
       </c>
       <c r="BN65" t="n">
         <v>46.43</v>
@@ -15471,19 +15471,19 @@
         <v>20.44</v>
       </c>
       <c r="BP65" t="n">
-        <v>24.21</v>
+        <v>23.75</v>
       </c>
       <c r="BQ65" t="n">
-        <v>15.8</v>
+        <v>15.78</v>
       </c>
       <c r="BR65" t="n">
-        <v>24.5</v>
+        <v>24.8</v>
       </c>
       <c r="BS65" t="n">
         <v>4.14</v>
       </c>
       <c r="BT65" t="n">
-        <v>8357</v>
+        <v>7957</v>
       </c>
     </row>
     <row r="66">
@@ -15513,13 +15513,13 @@
         </is>
       </c>
       <c r="F66" t="n">
-        <v>20.79</v>
+        <v>20.46</v>
       </c>
       <c r="G66" t="n">
-        <v>243047964214</v>
+        <v>241321019190</v>
       </c>
       <c r="H66" t="n">
-        <v>100</v>
+        <v>3000</v>
       </c>
       <c r="I66" t="n">
         <v>2972355254</v>
@@ -15534,7 +15534,7 @@
         <v>2.75</v>
       </c>
       <c r="M66" t="n">
-        <v>14.42869175152418</v>
+        <v>14.32617059894548</v>
       </c>
       <c r="N66" t="n">
         <v>0.25</v>
@@ -15612,7 +15612,7 @@
         <v>4696321301.320001</v>
       </c>
       <c r="AM66" t="n">
-        <v>21798023696.32287</v>
+        <v>21643140734.52915</v>
       </c>
       <c r="AN66" t="n">
         <v>0.4734</v>
@@ -15653,7 +15653,7 @@
         <v>12.99</v>
       </c>
       <c r="AZ66" t="n">
-        <v>8.35</v>
+        <v>8.220000000000001</v>
       </c>
       <c r="BA66" t="n">
         <v>2.23</v>
@@ -15662,28 +15662,28 @@
         <v>3.47</v>
       </c>
       <c r="BC66" t="n">
-        <v>-23.47</v>
+        <v>-22.24</v>
       </c>
       <c r="BD66" t="n">
-        <v>-37.52</v>
+        <v>-36.51</v>
       </c>
       <c r="BE66" t="n">
         <v>-59.83</v>
       </c>
       <c r="BF66" t="n">
-        <v>-89.27</v>
+        <v>-89.09</v>
       </c>
       <c r="BG66" t="n">
-        <v>-83.33</v>
+        <v>-83.06</v>
       </c>
       <c r="BH66" t="n">
         <v>7.12</v>
       </c>
       <c r="BI66" t="n">
-        <v>0.24</v>
+        <v>0</v>
       </c>
       <c r="BJ66" t="n">
-        <v>20.74</v>
+        <v>20.46</v>
       </c>
       <c r="BK66" t="n">
         <v>1.58</v>
@@ -15692,7 +15692,7 @@
         <v>1.57</v>
       </c>
       <c r="BM66" t="n">
-        <v>20.79</v>
+        <v>20.85</v>
       </c>
       <c r="BN66" t="n">
         <v>21.33</v>
@@ -15701,19 +15701,19 @@
         <v>9.48</v>
       </c>
       <c r="BP66" t="n">
-        <v>20.79</v>
+        <v>20.46</v>
       </c>
       <c r="BQ66" t="n">
-        <v>13.24</v>
+        <v>13.03</v>
       </c>
       <c r="BR66" t="n">
-        <v>20.79</v>
+        <v>20.8</v>
       </c>
       <c r="BS66" t="n">
         <v>3.46</v>
       </c>
       <c r="BT66" t="n">
-        <v>4297</v>
+        <v>4053</v>
       </c>
     </row>
     <row r="67">
@@ -15973,13 +15973,13 @@
         </is>
       </c>
       <c r="F68" t="n">
-        <v>17.98</v>
+        <v>17.91</v>
       </c>
       <c r="G68" t="n">
-        <v>7619953007</v>
+        <v>7660754035</v>
       </c>
       <c r="H68" t="n">
-        <v>82100</v>
+        <v>111100</v>
       </c>
       <c r="I68" t="n">
         <v>137989898</v>
@@ -16072,7 +16072,7 @@
         <v>205604948.02</v>
       </c>
       <c r="AM68" t="n">
-        <v>528429473.4396671</v>
+        <v>531258948.335645</v>
       </c>
       <c r="AN68" t="n">
         <v>0.1911</v>
@@ -16113,7 +16113,7 @@
         <v>21.39</v>
       </c>
       <c r="AZ68" t="n">
-        <v>33.26</v>
+        <v>33.13</v>
       </c>
       <c r="BA68" t="n">
         <v>1.24</v>
@@ -16122,28 +16122,28 @@
         <v>63.25</v>
       </c>
       <c r="BC68" t="n">
-        <v>45.73</v>
+        <v>46.3</v>
       </c>
       <c r="BD68" t="n">
-        <v>18.99</v>
+        <v>19.46</v>
       </c>
       <c r="BE68" t="n">
         <v>85</v>
       </c>
       <c r="BF68" t="n">
-        <v>-93.11</v>
+        <v>-93.08</v>
       </c>
       <c r="BG68" t="n">
-        <v>251.77</v>
+        <v>253.15</v>
       </c>
       <c r="BH68" t="n">
         <v>20.48</v>
       </c>
       <c r="BI68" t="n">
-        <v>0.84</v>
+        <v>0</v>
       </c>
       <c r="BJ68" t="n">
-        <v>17.83</v>
+        <v>17.91</v>
       </c>
       <c r="BK68" t="n">
         <v>1.49</v>
@@ -16152,7 +16152,7 @@
         <v>1.49</v>
       </c>
       <c r="BM68" t="n">
-        <v>18.08</v>
+        <v>18.35</v>
       </c>
       <c r="BN68" t="n">
         <v>22.11</v>
@@ -16161,19 +16161,19 @@
         <v>15.45</v>
       </c>
       <c r="BP68" t="n">
-        <v>17.85</v>
+        <v>17.73</v>
       </c>
       <c r="BQ68" t="n">
-        <v>12.09</v>
+        <v>12.05</v>
       </c>
       <c r="BR68" t="n">
-        <v>17.89</v>
+        <v>18.1</v>
       </c>
       <c r="BS68" t="n">
         <v>0</v>
       </c>
       <c r="BT68" t="n">
-        <v>41707</v>
+        <v>43300</v>
       </c>
     </row>
     <row r="69">
@@ -16203,13 +16203,13 @@
         </is>
       </c>
       <c r="F69" t="n">
-        <v>20.23</v>
+        <v>20.28</v>
       </c>
       <c r="G69" t="n">
-        <v>7619953007</v>
+        <v>7660754035</v>
       </c>
       <c r="H69" t="n">
-        <v>0</v>
+        <v>4260900</v>
       </c>
       <c r="I69" t="n">
         <v>255106712</v>
@@ -16302,7 +16302,7 @@
         <v>380109000.88</v>
       </c>
       <c r="AM69" t="n">
-        <v>453568631.3690476</v>
+        <v>455997263.9880952</v>
       </c>
       <c r="AN69" t="n">
         <v>0.8856000000000001</v>
@@ -16343,7 +16343,7 @@
         <v>21.39</v>
       </c>
       <c r="AZ69" t="n">
-        <v>35.37</v>
+        <v>35.46</v>
       </c>
       <c r="BA69" t="n">
         <v>1.24</v>
@@ -16352,28 +16352,28 @@
         <v>69.59</v>
       </c>
       <c r="BC69" t="n">
-        <v>29.52</v>
+        <v>29.21</v>
       </c>
       <c r="BD69" t="n">
-        <v>5.76</v>
+        <v>5.5</v>
       </c>
       <c r="BE69" t="n">
         <v>74.83</v>
       </c>
       <c r="BF69" t="n">
-        <v>-93.87</v>
+        <v>-93.89</v>
       </c>
       <c r="BG69" t="n">
-        <v>243.98</v>
+        <v>243.13</v>
       </c>
       <c r="BH69" t="n">
         <v>20.48</v>
       </c>
       <c r="BI69" t="n">
-        <v>-0.05</v>
+        <v>0</v>
       </c>
       <c r="BJ69" t="n">
-        <v>20.24</v>
+        <v>20.28</v>
       </c>
       <c r="BK69" t="n">
         <v>1.49</v>
@@ -16382,28 +16382,28 @@
         <v>1.49</v>
       </c>
       <c r="BM69" t="n">
-        <v>20.56</v>
+        <v>20.37</v>
       </c>
       <c r="BN69" t="n">
         <v>25.63</v>
       </c>
       <c r="BO69" t="n">
-        <v>16.97</v>
+        <v>16.99</v>
       </c>
       <c r="BP69" t="n">
-        <v>20.21</v>
+        <v>19.95</v>
       </c>
       <c r="BQ69" t="n">
-        <v>13.61</v>
+        <v>13.64</v>
       </c>
       <c r="BR69" t="n">
-        <v>20.5</v>
+        <v>20.2</v>
       </c>
       <c r="BS69" t="n">
         <v>0</v>
       </c>
       <c r="BT69" t="n">
-        <v>2104557</v>
+        <v>2200057</v>
       </c>
     </row>
     <row r="70">
@@ -16433,13 +16433,13 @@
         </is>
       </c>
       <c r="F70" t="n">
-        <v>18.12</v>
+        <v>18.18</v>
       </c>
       <c r="G70" t="n">
-        <v>8417776853</v>
+        <v>8445650037</v>
       </c>
       <c r="H70" t="n">
-        <v>0</v>
+        <v>5236000</v>
       </c>
       <c r="I70" t="n">
         <v>464557268</v>
@@ -16454,7 +16454,7 @@
         <v>0.68</v>
       </c>
       <c r="M70" t="n">
-        <v>0.6643999334509031</v>
+        <v>0.6665999135546836</v>
       </c>
       <c r="N70" t="n">
         <v>0.2</v>
@@ -16532,7 +16532,7 @@
         <v>55746872.16</v>
       </c>
       <c r="AM70" t="n">
-        <v>2778144175.907591</v>
+        <v>2787343246.534654</v>
       </c>
       <c r="AN70" t="n">
         <v>0.1236</v>
@@ -16573,7 +16573,7 @@
         <v>6.9</v>
       </c>
       <c r="AZ70" t="n">
-        <v>2.08</v>
+        <v>2.09</v>
       </c>
       <c r="BA70" t="n">
         <v>0.12</v>
@@ -16582,10 +16582,10 @@
         <v>1.07</v>
       </c>
       <c r="BC70" t="n">
-        <v>-53.37</v>
+        <v>-53.53</v>
       </c>
       <c r="BD70" t="n">
-        <v>-61.93</v>
+        <v>-62.05</v>
       </c>
       <c r="BE70" t="n">
         <v>-88.5</v>
@@ -16594,16 +16594,16 @@
         <v>-99.34</v>
       </c>
       <c r="BG70" t="n">
-        <v>-94.09999999999999</v>
+        <v>-94.12</v>
       </c>
       <c r="BH70" t="n">
         <v>26.44</v>
       </c>
       <c r="BI70" t="n">
-        <v>-0.6</v>
+        <v>0</v>
       </c>
       <c r="BJ70" t="n">
-        <v>18.23</v>
+        <v>18.18</v>
       </c>
       <c r="BK70" t="n">
         <v>0.12</v>
@@ -16612,7 +16612,7 @@
         <v>0.1</v>
       </c>
       <c r="BM70" t="n">
-        <v>18.59</v>
+        <v>18.5</v>
       </c>
       <c r="BN70" t="n">
         <v>22.15</v>
@@ -16621,19 +16621,19 @@
         <v>13.21</v>
       </c>
       <c r="BP70" t="n">
-        <v>18.12</v>
+        <v>18.13</v>
       </c>
       <c r="BQ70" t="n">
-        <v>181.73</v>
+        <v>182.33</v>
       </c>
       <c r="BR70" t="n">
-        <v>18.49</v>
+        <v>18.26</v>
       </c>
       <c r="BS70" t="n">
         <v>0.67</v>
       </c>
       <c r="BT70" t="n">
-        <v>3798633</v>
+        <v>3755827</v>
       </c>
     </row>
     <row r="71">

</xml_diff>

<commit_message>
📊 Dados atualizados - 2026-10-03 05:56
</commit_message>
<xml_diff>
--- a/data/ativos.xlsx
+++ b/data/ativos.xlsx
@@ -1047,13 +1047,13 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>25.61</v>
+        <v>26.15</v>
       </c>
       <c r="G3" t="n">
-        <v>3425767829</v>
+        <v>3485753109</v>
       </c>
       <c r="H3" t="n">
-        <v>707800</v>
+        <v>1023600</v>
       </c>
       <c r="I3" t="n">
         <v>129510368</v>
@@ -1068,7 +1068,7 @@
         <v>0.88</v>
       </c>
       <c r="M3" t="n">
-        <v>0.8524073325804212</v>
+        <v>0.86733300620198</v>
       </c>
       <c r="N3" t="n">
         <v>0.09</v>
@@ -1146,7 +1146,7 @@
         <v>506385538.88</v>
       </c>
       <c r="AM3" t="n">
-        <v>669095279.1015625</v>
+        <v>680811154.1015625</v>
       </c>
       <c r="AN3" t="n">
         <v>2.7</v>
@@ -1187,7 +1187,7 @@
         <v>40.42</v>
       </c>
       <c r="AZ3" t="n">
-        <v>46.87</v>
+        <v>47.85</v>
       </c>
       <c r="BA3" t="n">
         <v>4.87</v>
@@ -1196,19 +1196,19 @@
         <v>21.14</v>
       </c>
       <c r="BC3" t="n">
-        <v>93.28</v>
+        <v>89.29000000000001</v>
       </c>
       <c r="BD3" t="n">
-        <v>57.81</v>
+        <v>54.55</v>
       </c>
       <c r="BE3" t="n">
         <v>83</v>
       </c>
       <c r="BF3" t="n">
-        <v>-80.98999999999999</v>
+        <v>-81.38</v>
       </c>
       <c r="BG3" t="n">
-        <v>-17.47</v>
+        <v>-19.17</v>
       </c>
       <c r="BH3" t="n">
         <v>27.85</v>
@@ -1217,7 +1217,7 @@
         <v>0</v>
       </c>
       <c r="BJ3" t="n">
-        <v>25.61</v>
+        <v>26.15</v>
       </c>
       <c r="BK3" t="n">
         <v>3.91</v>
@@ -1226,7 +1226,7 @@
         <v>4.39</v>
       </c>
       <c r="BM3" t="n">
-        <v>25.9</v>
+        <v>26.25</v>
       </c>
       <c r="BN3" t="n">
         <v>27.17</v>
@@ -1235,19 +1235,19 @@
         <v>18.72</v>
       </c>
       <c r="BP3" t="n">
-        <v>25.43</v>
+        <v>25.59</v>
       </c>
       <c r="BQ3" t="n">
-        <v>5.83</v>
+        <v>5.95</v>
       </c>
       <c r="BR3" t="n">
-        <v>25.88</v>
+        <v>25.82</v>
       </c>
       <c r="BS3" t="n">
         <v>0.79</v>
       </c>
       <c r="BT3" t="n">
-        <v>551093</v>
+        <v>560080</v>
       </c>
     </row>
     <row r="4">
@@ -1277,13 +1277,13 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>15.42</v>
+        <v>15.84</v>
       </c>
       <c r="G4" t="n">
-        <v>238773458381</v>
+        <v>246074877570</v>
       </c>
       <c r="H4" t="n">
-        <v>25111800</v>
+        <v>36916800</v>
       </c>
       <c r="I4" t="n">
         <v>15484664889</v>
@@ -1298,7 +1298,7 @@
         <v>2.76</v>
       </c>
       <c r="M4" t="n">
-        <v>2.703639159747571</v>
+        <v>2.786313352159752</v>
       </c>
       <c r="N4" t="n">
         <v>1.76</v>
@@ -1376,7 +1376,7 @@
         <v>16258898133.45</v>
       </c>
       <c r="AM4" t="n">
-        <v>23640936473.36634</v>
+        <v>24363849264.35644</v>
       </c>
       <c r="AN4" t="n">
         <v>0.269</v>
@@ -1417,7 +1417,7 @@
         <v>9.470000000000001</v>
       </c>
       <c r="AZ4" t="n">
-        <v>19.25</v>
+        <v>19.77</v>
       </c>
       <c r="BA4" t="n">
         <v>1.13</v>
@@ -1426,19 +1426,19 @@
         <v>11.39</v>
       </c>
       <c r="BC4" t="n">
-        <v>-24.74</v>
+        <v>-26.74</v>
       </c>
       <c r="BD4" t="n">
-        <v>-38.55</v>
+        <v>-40.18</v>
       </c>
       <c r="BE4" t="n">
         <v>24.83</v>
       </c>
       <c r="BF4" t="n">
-        <v>-92.69</v>
+        <v>-92.88</v>
       </c>
       <c r="BG4" t="n">
-        <v>-26.16</v>
+        <v>-28.11</v>
       </c>
       <c r="BH4" t="n">
         <v>5.7</v>
@@ -1447,7 +1447,7 @@
         <v>0</v>
       </c>
       <c r="BJ4" t="n">
-        <v>15.42</v>
+        <v>15.84</v>
       </c>
       <c r="BK4" t="n">
         <v>1.05</v>
@@ -1456,7 +1456,7 @@
         <v>1.04</v>
       </c>
       <c r="BM4" t="n">
-        <v>15.45</v>
+        <v>15.84</v>
       </c>
       <c r="BN4" t="n">
         <v>16.94</v>
@@ -1465,19 +1465,19 @@
         <v>11.04</v>
       </c>
       <c r="BP4" t="n">
-        <v>15.23</v>
+        <v>15.39</v>
       </c>
       <c r="BQ4" t="n">
-        <v>14.87</v>
+        <v>15.28</v>
       </c>
       <c r="BR4" t="n">
-        <v>15.36</v>
+        <v>15.62</v>
       </c>
       <c r="BS4" t="n">
         <v>2.76</v>
       </c>
       <c r="BT4" t="n">
-        <v>26042500</v>
+        <v>26083937</v>
       </c>
     </row>
     <row r="5">
@@ -1737,13 +1737,13 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>7</v>
+        <v>7.17</v>
       </c>
       <c r="G6" t="n">
-        <v>441592830</v>
+        <v>452317303</v>
       </c>
       <c r="H6" t="n">
-        <v>1800</v>
+        <v>100</v>
       </c>
       <c r="I6" t="n">
         <v>63084700</v>
@@ -1758,7 +1758,7 @@
         <v>1.91</v>
       </c>
       <c r="M6" t="n">
-        <v>6.874735752342318</v>
+        <v>7.041694799114273</v>
       </c>
       <c r="N6" t="n">
         <v>1.26</v>
@@ -1836,7 +1836,7 @@
         <v>35958279</v>
       </c>
       <c r="AM6" t="n">
-        <v>42217287.76290631</v>
+        <v>43242571.98852772</v>
       </c>
       <c r="AN6" t="n">
         <v>0.5199</v>
@@ -1877,7 +1877,7 @@
         <v>5.74</v>
       </c>
       <c r="AZ6" t="n">
-        <v>8.210000000000001</v>
+        <v>8.41</v>
       </c>
       <c r="BA6" t="n">
         <v>0.65</v>
@@ -1886,19 +1886,19 @@
         <v>7.95</v>
       </c>
       <c r="BC6" t="n">
-        <v>0.51</v>
+        <v>-1.87</v>
       </c>
       <c r="BD6" t="n">
-        <v>-17.93</v>
+        <v>-19.88</v>
       </c>
       <c r="BE6" t="n">
         <v>17.33</v>
       </c>
       <c r="BF6" t="n">
-        <v>-90.73999999999999</v>
+        <v>-90.95999999999999</v>
       </c>
       <c r="BG6" t="n">
-        <v>13.62</v>
+        <v>10.93</v>
       </c>
       <c r="BH6" t="n">
         <v>3.86</v>
@@ -1907,7 +1907,7 @@
         <v>0</v>
       </c>
       <c r="BJ6" t="n">
-        <v>7</v>
+        <v>7.17</v>
       </c>
       <c r="BK6" t="n">
         <v>0.57</v>
@@ -1916,7 +1916,7 @@
         <v>0.5600000000000001</v>
       </c>
       <c r="BM6" t="n">
-        <v>7.33</v>
+        <v>7.17</v>
       </c>
       <c r="BN6" t="n">
         <v>8.16</v>
@@ -1925,19 +1925,19 @@
         <v>6.22</v>
       </c>
       <c r="BP6" t="n">
-        <v>7</v>
+        <v>7.17</v>
       </c>
       <c r="BQ6" t="n">
-        <v>12.45</v>
+        <v>12.75</v>
       </c>
       <c r="BR6" t="n">
-        <v>7.33</v>
+        <v>7.17</v>
       </c>
       <c r="BS6" t="n">
         <v>7.32</v>
       </c>
       <c r="BT6" t="n">
-        <v>167</v>
+        <v>220</v>
       </c>
     </row>
     <row r="7">
@@ -3117,13 +3117,13 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>5.3</v>
+        <v>5.28</v>
       </c>
       <c r="G12" t="n">
-        <v>508596180</v>
+        <v>505722644</v>
       </c>
       <c r="H12" t="n">
-        <v>1009200</v>
+        <v>1796300</v>
       </c>
       <c r="I12" t="n">
         <v>95961536</v>
@@ -3138,7 +3138,7 @@
         <v>0.32</v>
       </c>
       <c r="M12" t="n">
-        <v>0.09197884306809616</v>
+        <v>0.09145916846732639</v>
       </c>
       <c r="N12" t="n">
         <v>0.14</v>
@@ -3216,7 +3216,7 @@
         <v>362734606.08</v>
       </c>
       <c r="AM12" t="n">
-        <v>546877612.9032258</v>
+        <v>543787789.2473118</v>
       </c>
       <c r="AN12" t="n">
         <v>0.4208</v>
@@ -3257,7 +3257,7 @@
         <v>30.49</v>
       </c>
       <c r="AZ12" t="n">
-        <v>7.16</v>
+        <v>7.14</v>
       </c>
       <c r="BA12" t="n">
         <v>4.41</v>
@@ -3266,19 +3266,19 @@
         <v>18.12</v>
       </c>
       <c r="BC12" t="n">
-        <v>604.67</v>
+        <v>607.34</v>
       </c>
       <c r="BD12" t="n">
-        <v>475.36</v>
+        <v>477.54</v>
       </c>
       <c r="BE12" t="n">
         <v>35.17</v>
       </c>
       <c r="BF12" t="n">
-        <v>-16.76</v>
+        <v>-16.45</v>
       </c>
       <c r="BG12" t="n">
-        <v>241.87</v>
+        <v>243.16</v>
       </c>
       <c r="BH12" t="n">
         <v>16.4</v>
@@ -3287,7 +3287,7 @@
         <v>0</v>
       </c>
       <c r="BJ12" t="n">
-        <v>5.3</v>
+        <v>5.28</v>
       </c>
       <c r="BK12" t="n">
         <v>3.78</v>
@@ -3296,7 +3296,7 @@
         <v>3.63</v>
       </c>
       <c r="BM12" t="n">
-        <v>5.39</v>
+        <v>5.38</v>
       </c>
       <c r="BN12" t="n">
         <v>8.23</v>
@@ -3305,19 +3305,19 @@
         <v>4.42</v>
       </c>
       <c r="BP12" t="n">
-        <v>5.2</v>
+        <v>5.26</v>
       </c>
       <c r="BQ12" t="n">
-        <v>1.46</v>
+        <v>1.45</v>
       </c>
       <c r="BR12" t="n">
-        <v>5.39</v>
+        <v>5.37</v>
       </c>
       <c r="BS12" t="n">
         <v>0.09</v>
       </c>
       <c r="BT12" t="n">
-        <v>560840</v>
+        <v>568933</v>
       </c>
     </row>
     <row r="13">
@@ -3347,13 +3347,13 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>29.73</v>
+        <v>30.51</v>
       </c>
       <c r="G13" t="n">
-        <v>14989595226</v>
+        <v>15424373329</v>
       </c>
       <c r="H13" t="n">
-        <v>5757100</v>
+        <v>10273900</v>
       </c>
       <c r="I13" t="n">
         <v>504190947</v>
@@ -3368,7 +3368,7 @@
         <v>1.13</v>
       </c>
       <c r="M13" t="n">
-        <v>5.184268626025453</v>
+        <v>5.33464002996811</v>
       </c>
       <c r="N13" t="n">
         <v>0.57</v>
@@ -3446,7 +3446,7 @@
         <v>932753251.95</v>
       </c>
       <c r="AM13" t="n">
-        <v>1559791386.680541</v>
+        <v>1605033645.057232</v>
       </c>
       <c r="AN13" t="n">
         <v>2.6301</v>
@@ -3487,7 +3487,7 @@
         <v>26.6</v>
       </c>
       <c r="AZ13" t="n">
-        <v>53.81</v>
+        <v>55.22</v>
       </c>
       <c r="BA13" t="n">
         <v>2.6</v>
@@ -3496,19 +3496,19 @@
         <v>8.69</v>
       </c>
       <c r="BC13" t="n">
-        <v>9.56</v>
+        <v>6.76</v>
       </c>
       <c r="BD13" t="n">
-        <v>-10.54</v>
+        <v>-12.83</v>
       </c>
       <c r="BE13" t="n">
         <v>81</v>
       </c>
       <c r="BF13" t="n">
-        <v>-91.23999999999999</v>
+        <v>-91.45999999999999</v>
       </c>
       <c r="BG13" t="n">
-        <v>-70.76000000000001</v>
+        <v>-71.5</v>
       </c>
       <c r="BH13" t="n">
         <v>25.49</v>
@@ -3517,7 +3517,7 @@
         <v>0</v>
       </c>
       <c r="BJ13" t="n">
-        <v>29.73</v>
+        <v>30.51</v>
       </c>
       <c r="BK13" t="n">
         <v>1.85</v>
@@ -3526,7 +3526,7 @@
         <v>1.96</v>
       </c>
       <c r="BM13" t="n">
-        <v>29.73</v>
+        <v>30.59</v>
       </c>
       <c r="BN13" t="n">
         <v>32.11</v>
@@ -3535,19 +3535,19 @@
         <v>20.85</v>
       </c>
       <c r="BP13" t="n">
-        <v>29.13</v>
+        <v>29.7</v>
       </c>
       <c r="BQ13" t="n">
-        <v>15.19</v>
+        <v>15.59</v>
       </c>
       <c r="BR13" t="n">
-        <v>29.5</v>
+        <v>30.06</v>
       </c>
       <c r="BS13" t="n">
         <v>5.01</v>
       </c>
       <c r="BT13" t="n">
-        <v>5099753</v>
+        <v>5078920</v>
       </c>
     </row>
     <row r="14">
@@ -3577,13 +3577,13 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>10.65</v>
+        <v>11.38</v>
       </c>
       <c r="G14" t="n">
-        <v>8567288036</v>
+        <v>8976365139</v>
       </c>
       <c r="H14" t="n">
-        <v>8900</v>
+        <v>11700</v>
       </c>
       <c r="I14" t="n">
         <v>339510689</v>
@@ -3598,7 +3598,7 @@
         <v>1.92</v>
       </c>
       <c r="M14" t="n">
-        <v>3.557290299083212</v>
+        <v>3.727146384692117</v>
       </c>
       <c r="N14" t="n">
         <v>1.11</v>
@@ -3676,7 +3676,7 @@
         <v>349696009.67</v>
       </c>
       <c r="AM14" t="n">
-        <v>950864376.9145395</v>
+        <v>996266941.0654829</v>
       </c>
       <c r="AN14" t="n">
         <v>0.1489</v>
@@ -3717,7 +3717,7 @@
         <v>9.050000000000001</v>
       </c>
       <c r="AZ14" t="n">
-        <v>8.56</v>
+        <v>9.140000000000001</v>
       </c>
       <c r="BA14" t="n">
         <v>1.42</v>
@@ -3726,19 +3726,19 @@
         <v>5.94</v>
       </c>
       <c r="BC14" t="n">
-        <v>4.06</v>
+        <v>-2.61</v>
       </c>
       <c r="BD14" t="n">
-        <v>-15.03</v>
+        <v>-20.48</v>
       </c>
       <c r="BE14" t="n">
         <v>-19.67</v>
       </c>
       <c r="BF14" t="n">
-        <v>-86.66</v>
+        <v>-87.51000000000001</v>
       </c>
       <c r="BG14" t="n">
-        <v>-44.2</v>
+        <v>-47.78</v>
       </c>
       <c r="BH14" t="n">
         <v>5.3</v>
@@ -3747,7 +3747,7 @@
         <v>0</v>
       </c>
       <c r="BJ14" t="n">
-        <v>10.65</v>
+        <v>11.38</v>
       </c>
       <c r="BK14" t="n">
         <v>1.03</v>
@@ -3756,7 +3756,7 @@
         <v>1.01</v>
       </c>
       <c r="BM14" t="n">
-        <v>10.65</v>
+        <v>11.38</v>
       </c>
       <c r="BN14" t="n">
         <v>13.49</v>
@@ -3765,19 +3765,19 @@
         <v>7.81</v>
       </c>
       <c r="BP14" t="n">
-        <v>10.35</v>
+        <v>10.65</v>
       </c>
       <c r="BQ14" t="n">
-        <v>10.51</v>
+        <v>11.23</v>
       </c>
       <c r="BR14" t="n">
-        <v>10.39</v>
+        <v>10.65</v>
       </c>
       <c r="BS14" t="n">
         <v>1.44</v>
       </c>
       <c r="BT14" t="n">
-        <v>9753</v>
+        <v>9777</v>
       </c>
     </row>
     <row r="15">
@@ -3807,13 +3807,13 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>14.57</v>
+        <v>15.17</v>
       </c>
       <c r="G15" t="n">
-        <v>8567288036</v>
+        <v>8976365139</v>
       </c>
       <c r="H15" t="n">
-        <v>2677700</v>
+        <v>1983600</v>
       </c>
       <c r="I15" t="n">
         <v>343551533</v>
@@ -3828,7 +3828,7 @@
         <v>2.56</v>
       </c>
       <c r="M15" t="n">
-        <v>3.515449545133472</v>
+        <v>3.683307787977996</v>
       </c>
       <c r="N15" t="n">
         <v>1.47</v>
@@ -3906,7 +3906,7 @@
         <v>353858078.99</v>
       </c>
       <c r="AM15" t="n">
-        <v>714536116.4303586</v>
+        <v>748654306.8390325</v>
       </c>
       <c r="AN15" t="n">
         <v>0.1638</v>
@@ -3947,7 +3947,7 @@
         <v>9.050000000000001</v>
       </c>
       <c r="AZ15" t="n">
-        <v>9.69</v>
+        <v>10.09</v>
       </c>
       <c r="BA15" t="n">
         <v>1.42</v>
@@ -3956,19 +3956,19 @@
         <v>6.19</v>
       </c>
       <c r="BC15" t="n">
-        <v>-23.93</v>
+        <v>-26.94</v>
       </c>
       <c r="BD15" t="n">
-        <v>-37.89</v>
+        <v>-40.35</v>
       </c>
       <c r="BE15" t="n">
         <v>-33.5</v>
       </c>
       <c r="BF15" t="n">
-        <v>-90.25</v>
+        <v>-90.63</v>
       </c>
       <c r="BG15" t="n">
-        <v>-57.53</v>
+        <v>-59.21</v>
       </c>
       <c r="BH15" t="n">
         <v>5.3</v>
@@ -3977,7 +3977,7 @@
         <v>0</v>
       </c>
       <c r="BJ15" t="n">
-        <v>14.57</v>
+        <v>15.17</v>
       </c>
       <c r="BK15" t="n">
         <v>1.03</v>
@@ -3986,7 +3986,7 @@
         <v>1.01</v>
       </c>
       <c r="BM15" t="n">
-        <v>14.65</v>
+        <v>15.29</v>
       </c>
       <c r="BN15" t="n">
         <v>16.22</v>
@@ -3995,19 +3995,19 @@
         <v>7.84</v>
       </c>
       <c r="BP15" t="n">
-        <v>14.19</v>
+        <v>14.66</v>
       </c>
       <c r="BQ15" t="n">
-        <v>14.38</v>
+        <v>14.98</v>
       </c>
       <c r="BR15" t="n">
-        <v>14.19</v>
+        <v>14.71</v>
       </c>
       <c r="BS15" t="n">
         <v>1.92</v>
       </c>
       <c r="BT15" t="n">
-        <v>2359873</v>
+        <v>2376813</v>
       </c>
     </row>
     <row r="16">
@@ -4037,13 +4037,13 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>4.49</v>
+        <v>4.6</v>
       </c>
       <c r="G16" t="n">
-        <v>984682542</v>
+        <v>1015591658</v>
       </c>
       <c r="H16" t="n">
-        <v>122500</v>
+        <v>128200</v>
       </c>
       <c r="I16" t="n">
         <v>219305733</v>
@@ -4058,7 +4058,7 @@
         <v>2.69</v>
       </c>
       <c r="M16" t="n">
-        <v>0.46583740577589</v>
+        <v>0.4804600093035415</v>
       </c>
       <c r="N16" t="n">
         <v>0.39</v>
@@ -4136,7 +4136,7 @@
         <v>17544458.64</v>
       </c>
       <c r="AM16" t="n">
-        <v>276596219.6629214</v>
+        <v>285278555.6179775</v>
       </c>
       <c r="AN16" t="n">
         <v>0.0077</v>
@@ -4186,16 +4186,16 @@
         <v>0</v>
       </c>
       <c r="BC16" t="n">
-        <v>-61.27</v>
+        <v>-62.2</v>
       </c>
       <c r="BD16" t="n">
-        <v>-68.38</v>
+        <v>-69.13</v>
       </c>
       <c r="BE16" t="n">
         <v>-97.17</v>
       </c>
       <c r="BF16" t="n">
-        <v>-98.22</v>
+        <v>-98.26000000000001</v>
       </c>
       <c r="BG16" t="n">
         <v>-100</v>
@@ -4207,7 +4207,7 @@
         <v>0</v>
       </c>
       <c r="BJ16" t="n">
-        <v>4.49</v>
+        <v>4.6</v>
       </c>
       <c r="BK16" t="n">
         <v>0.08</v>
@@ -4216,7 +4216,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="BM16" t="n">
-        <v>4.49</v>
+        <v>4.64</v>
       </c>
       <c r="BN16" t="n">
         <v>5.54</v>
@@ -4225,19 +4225,19 @@
         <v>3.22</v>
       </c>
       <c r="BP16" t="n">
-        <v>4.35</v>
+        <v>4.44</v>
       </c>
       <c r="BQ16" t="n">
-        <v>61.27</v>
+        <v>62.77</v>
       </c>
       <c r="BR16" t="n">
-        <v>4.35</v>
+        <v>4.46</v>
       </c>
       <c r="BS16" t="n">
         <v>0.49</v>
       </c>
       <c r="BT16" t="n">
-        <v>129167</v>
+        <v>129907</v>
       </c>
     </row>
     <row r="17">
@@ -4267,13 +4267,13 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>32.66</v>
+        <v>33.51</v>
       </c>
       <c r="G17" t="n">
-        <v>10765611237</v>
+        <v>11015436807</v>
       </c>
       <c r="H17" t="n">
-        <v>940000</v>
+        <v>794100</v>
       </c>
       <c r="I17" t="n">
         <v>0</v>
@@ -4360,13 +4360,13 @@
         <v>8.039999999999999</v>
       </c>
       <c r="AK17" t="n">
-        <v>4861638022.489162</v>
+        <v>4974456650.559971</v>
       </c>
       <c r="AL17" t="n">
-        <v>1345701404.625</v>
+        <v>1376929600.875</v>
       </c>
       <c r="AM17" t="n">
-        <v>3333006574.922601</v>
+        <v>3410351952.631579</v>
       </c>
       <c r="AN17" t="n">
         <v>1.08</v>
@@ -4407,7 +4407,7 @@
         <v>42.98</v>
       </c>
       <c r="AZ17" t="n">
-        <v>17.47</v>
+        <v>17.93</v>
       </c>
       <c r="BA17" t="n">
         <v>4.55</v>
@@ -4416,19 +4416,19 @@
         <v>16.33</v>
       </c>
       <c r="BC17" t="n">
-        <v>61.17</v>
+        <v>57.08</v>
       </c>
       <c r="BD17" t="n">
-        <v>31.59</v>
+        <v>28.26</v>
       </c>
       <c r="BE17" t="n">
         <v>-46.5</v>
       </c>
       <c r="BF17" t="n">
-        <v>-86.06999999999999</v>
+        <v>-86.43000000000001</v>
       </c>
       <c r="BG17" t="n">
-        <v>-49.99</v>
+        <v>-51.26</v>
       </c>
       <c r="BH17" t="n">
         <v>29.25</v>
@@ -4437,7 +4437,7 @@
         <v>0</v>
       </c>
       <c r="BJ17" t="n">
-        <v>32.66</v>
+        <v>33.51</v>
       </c>
       <c r="BK17" t="n">
         <v>4.21</v>
@@ -4446,7 +4446,7 @@
         <v>12.62</v>
       </c>
       <c r="BM17" t="n">
-        <v>32.79</v>
+        <v>33.54</v>
       </c>
       <c r="BN17" t="n">
         <v>36.63</v>
@@ -4455,19 +4455,19 @@
         <v>29.53</v>
       </c>
       <c r="BP17" t="n">
-        <v>32.1</v>
+        <v>32.46</v>
       </c>
       <c r="BQ17" t="n">
-        <v>2.59</v>
+        <v>2.65</v>
       </c>
       <c r="BR17" t="n">
-        <v>32.65</v>
+        <v>32.99</v>
       </c>
       <c r="BS17" t="n">
         <v>2.21</v>
       </c>
       <c r="BT17" t="n">
-        <v>1120500</v>
+        <v>1070423</v>
       </c>
     </row>
     <row r="18">
@@ -4497,13 +4497,13 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>11.5</v>
+        <v>11.75</v>
       </c>
       <c r="G18" t="n">
-        <v>10765611237</v>
+        <v>11015436807</v>
       </c>
       <c r="H18" t="n">
-        <v>7200</v>
+        <v>5000</v>
       </c>
       <c r="I18" t="n">
         <v>671494278</v>
@@ -4518,7 +4518,7 @@
         <v>1.2</v>
       </c>
       <c r="M18" t="n">
-        <v>3.169818724801022</v>
+        <v>3.24337718351616</v>
       </c>
       <c r="N18" t="n">
         <v>0.33</v>
@@ -4596,7 +4596,7 @@
         <v>940091989.1999999</v>
       </c>
       <c r="AM18" t="n">
-        <v>3204050963.392857</v>
+        <v>3278403811.607143</v>
       </c>
       <c r="AN18" t="n">
         <v>0.36</v>
@@ -4637,7 +4637,7 @@
         <v>14.31</v>
       </c>
       <c r="AZ18" t="n">
-        <v>5.92</v>
+        <v>6.05</v>
       </c>
       <c r="BA18" t="n">
         <v>1.51</v>
@@ -4646,19 +4646,19 @@
         <v>5.44</v>
       </c>
       <c r="BC18" t="n">
-        <v>52.39</v>
+        <v>49.15</v>
       </c>
       <c r="BD18" t="n">
-        <v>24.43</v>
+        <v>21.78</v>
       </c>
       <c r="BE18" t="n">
         <v>-48.5</v>
       </c>
       <c r="BF18" t="n">
-        <v>-86.84999999999999</v>
+        <v>-87.13</v>
       </c>
       <c r="BG18" t="n">
-        <v>-52.66</v>
+        <v>-53.66</v>
       </c>
       <c r="BH18" t="n">
         <v>9.75</v>
@@ -4667,7 +4667,7 @@
         <v>0</v>
       </c>
       <c r="BJ18" t="n">
-        <v>11.5</v>
+        <v>11.75</v>
       </c>
       <c r="BK18" t="n">
         <v>1.4</v>
@@ -4676,7 +4676,7 @@
         <v>12.62</v>
       </c>
       <c r="BM18" t="n">
-        <v>11.59</v>
+        <v>11.75</v>
       </c>
       <c r="BN18" t="n">
         <v>13.82</v>
@@ -4685,19 +4685,19 @@
         <v>10.19</v>
       </c>
       <c r="BP18" t="n">
-        <v>11.1</v>
+        <v>11.58</v>
       </c>
       <c r="BQ18" t="n">
-        <v>0.91</v>
+        <v>0.93</v>
       </c>
       <c r="BR18" t="n">
-        <v>11.5</v>
+        <v>11.58</v>
       </c>
       <c r="BS18" t="n">
         <v>2.3</v>
       </c>
       <c r="BT18" t="n">
-        <v>9433</v>
+        <v>8530</v>
       </c>
     </row>
     <row r="19">
@@ -4727,13 +4727,13 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>10.6</v>
+        <v>10.85</v>
       </c>
       <c r="G19" t="n">
-        <v>10765611237</v>
+        <v>11015436807</v>
       </c>
       <c r="H19" t="n">
-        <v>10400</v>
+        <v>11500</v>
       </c>
       <c r="I19" t="n">
         <v>317386323</v>
@@ -4748,7 +4748,7 @@
         <v>1.12</v>
       </c>
       <c r="M19" t="n">
-        <v>6.706385819911789</v>
+        <v>6.862013458994757</v>
       </c>
       <c r="N19" t="n">
         <v>0.3</v>
@@ -4826,7 +4826,7 @@
         <v>444340852.2</v>
       </c>
       <c r="AM19" t="n">
-        <v>3417654360.952381</v>
+        <v>3496964065.714286</v>
       </c>
       <c r="AN19" t="n">
         <v>0.36</v>
@@ -4867,7 +4867,7 @@
         <v>14.31</v>
       </c>
       <c r="AZ19" t="n">
-        <v>5.83</v>
+        <v>5.97</v>
       </c>
       <c r="BA19" t="n">
         <v>1.51</v>
@@ -4876,19 +4876,19 @@
         <v>5.25</v>
       </c>
       <c r="BC19" t="n">
-        <v>65.33</v>
+        <v>61.52</v>
       </c>
       <c r="BD19" t="n">
-        <v>34.99</v>
+        <v>31.88</v>
       </c>
       <c r="BE19" t="n">
         <v>-45</v>
       </c>
       <c r="BF19" t="n">
-        <v>-85.73</v>
+        <v>-86.06</v>
       </c>
       <c r="BG19" t="n">
-        <v>-50.47</v>
+        <v>-51.61</v>
       </c>
       <c r="BH19" t="n">
         <v>9.75</v>
@@ -4897,7 +4897,7 @@
         <v>0</v>
       </c>
       <c r="BJ19" t="n">
-        <v>10.6</v>
+        <v>10.85</v>
       </c>
       <c r="BK19" t="n">
         <v>1.4</v>
@@ -4906,7 +4906,7 @@
         <v>12.62</v>
       </c>
       <c r="BM19" t="n">
-        <v>10.7</v>
+        <v>10.86</v>
       </c>
       <c r="BN19" t="n">
         <v>11.41</v>
@@ -4915,19 +4915,19 @@
         <v>9.19</v>
       </c>
       <c r="BP19" t="n">
-        <v>10.43</v>
+        <v>10.61</v>
       </c>
       <c r="BQ19" t="n">
-        <v>0.84</v>
+        <v>0.86</v>
       </c>
       <c r="BR19" t="n">
-        <v>10.43</v>
+        <v>10.64</v>
       </c>
       <c r="BS19" t="n">
         <v>2.16</v>
       </c>
       <c r="BT19" t="n">
-        <v>11383</v>
+        <v>11387</v>
       </c>
     </row>
     <row r="20">
@@ -5417,13 +5417,13 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>5.27</v>
+        <v>5.48</v>
       </c>
       <c r="G22" t="n">
-        <v>1055292727</v>
+        <v>1095265683</v>
       </c>
       <c r="H22" t="n">
-        <v>2070600</v>
+        <v>3376000</v>
       </c>
       <c r="I22" t="n">
         <v>200245299</v>
@@ -5438,7 +5438,7 @@
         <v>0.27</v>
       </c>
       <c r="M22" t="n">
-        <v>0.0895063493140663</v>
+        <v>0.09289671984473689</v>
       </c>
       <c r="N22" t="n">
         <v>0.08</v>
@@ -5516,7 +5516,7 @@
         <v>378463615.11</v>
       </c>
       <c r="AM22" t="n">
-        <v>239295402.9478458</v>
+        <v>248359565.3061225</v>
       </c>
       <c r="AN22" t="n">
         <v>0</v>
@@ -5566,19 +5566,19 @@
         <v>172.49</v>
       </c>
       <c r="BC22" t="n">
-        <v>463.66</v>
+        <v>442.06</v>
       </c>
       <c r="BD22" t="n">
-        <v>360.23</v>
+        <v>342.59</v>
       </c>
       <c r="BE22" t="n">
         <v>-100</v>
       </c>
       <c r="BF22" t="n">
-        <v>-64.14</v>
+        <v>-65.51000000000001</v>
       </c>
       <c r="BG22" t="n">
-        <v>3173.05</v>
+        <v>3047.62</v>
       </c>
       <c r="BH22" t="n">
         <v>20.75</v>
@@ -5587,7 +5587,7 @@
         <v>0</v>
       </c>
       <c r="BJ22" t="n">
-        <v>5.27</v>
+        <v>5.48</v>
       </c>
       <c r="BK22" t="n">
         <v>1.89</v>
@@ -5605,19 +5605,19 @@
         <v>3.37</v>
       </c>
       <c r="BP22" t="n">
-        <v>5.22</v>
+        <v>5.06</v>
       </c>
       <c r="BQ22" t="n">
-        <v>7.85</v>
+        <v>8.16</v>
       </c>
       <c r="BR22" t="n">
-        <v>5.49</v>
+        <v>5.36</v>
       </c>
       <c r="BS22" t="n">
         <v>0.09</v>
       </c>
       <c r="BT22" t="n">
-        <v>1574060</v>
+        <v>1585160</v>
       </c>
     </row>
     <row r="23">
@@ -5877,13 +5877,13 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>3.09</v>
+        <v>3.34</v>
       </c>
       <c r="G24" t="n">
-        <v>1247954557</v>
+        <v>1353301499</v>
       </c>
       <c r="H24" t="n">
-        <v>7170800</v>
+        <v>9865000</v>
       </c>
       <c r="I24" t="n">
         <v>403868805</v>
@@ -5898,7 +5898,7 @@
         <v>0.49</v>
       </c>
       <c r="M24" t="n">
-        <v>0.3016815667515437</v>
+        <v>0.327148223639631</v>
       </c>
       <c r="N24" t="n">
         <v>0.11</v>
@@ -5976,7 +5976,7 @@
         <v>153470145.9</v>
       </c>
       <c r="AM24" t="n">
-        <v>1124283384.684685</v>
+        <v>1219190539.63964</v>
       </c>
       <c r="AN24" t="n">
         <v>0.0813</v>
@@ -6017,7 +6017,7 @@
         <v>5.84</v>
       </c>
       <c r="AZ24" t="n">
-        <v>1.43</v>
+        <v>1.54</v>
       </c>
       <c r="BA24" t="n">
         <v>0.38</v>
@@ -6026,19 +6026,19 @@
         <v>1.46</v>
       </c>
       <c r="BC24" t="n">
-        <v>131.6</v>
+        <v>114.26</v>
       </c>
       <c r="BD24" t="n">
-        <v>89.09999999999999</v>
+        <v>74.95</v>
       </c>
       <c r="BE24" t="n">
         <v>-53.83</v>
       </c>
       <c r="BF24" t="n">
-        <v>-87.7</v>
+        <v>-88.62</v>
       </c>
       <c r="BG24" t="n">
-        <v>-52.82</v>
+        <v>-56.35</v>
       </c>
       <c r="BH24" t="n">
         <v>5.99</v>
@@ -6047,7 +6047,7 @@
         <v>0</v>
       </c>
       <c r="BJ24" t="n">
-        <v>3.09</v>
+        <v>3.34</v>
       </c>
       <c r="BK24" t="n">
         <v>0.38</v>
@@ -6056,7 +6056,7 @@
         <v>0.41</v>
       </c>
       <c r="BM24" t="n">
-        <v>3.1</v>
+        <v>3.37</v>
       </c>
       <c r="BN24" t="n">
         <v>5.29</v>
@@ -6065,19 +6065,19 @@
         <v>1.92</v>
       </c>
       <c r="BP24" t="n">
-        <v>2.94</v>
+        <v>3.09</v>
       </c>
       <c r="BQ24" t="n">
-        <v>7.59</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="BR24" t="n">
-        <v>2.99</v>
+        <v>3.16</v>
       </c>
       <c r="BS24" t="n">
         <v>0.29</v>
       </c>
       <c r="BT24" t="n">
-        <v>7341513</v>
+        <v>7301783</v>
       </c>
     </row>
     <row r="25">
@@ -6107,13 +6107,13 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>4.39</v>
+        <v>4.46</v>
       </c>
       <c r="G25" t="n">
-        <v>1521109052</v>
+        <v>1570403923</v>
       </c>
       <c r="H25" t="n">
-        <v>1186300</v>
+        <v>1144900</v>
       </c>
       <c r="I25" t="n">
         <v>346494097</v>
@@ -6128,7 +6128,7 @@
         <v>0.97</v>
       </c>
       <c r="M25" t="n">
-        <v>0.7584944275752618</v>
+        <v>0.7830751010729179</v>
       </c>
       <c r="N25" t="n">
         <v>0.22</v>
@@ -6206,7 +6206,7 @@
         <v>62368937.46</v>
       </c>
       <c r="AM25" t="n">
-        <v>559231269.1176471</v>
+        <v>577354383.4558823</v>
       </c>
       <c r="AN25" t="n">
         <v>0.4742</v>
@@ -6247,7 +6247,7 @@
         <v>3.27</v>
       </c>
       <c r="AZ25" t="n">
-        <v>10.23</v>
+        <v>10.39</v>
       </c>
       <c r="BA25" t="n">
         <v>0.23</v>
@@ -6256,19 +6256,19 @@
         <v>2.2</v>
       </c>
       <c r="BC25" t="n">
-        <v>-8.66</v>
+        <v>-10.09</v>
       </c>
       <c r="BD25" t="n">
-        <v>-25.42</v>
+        <v>-26.59</v>
       </c>
       <c r="BE25" t="n">
         <v>133</v>
       </c>
       <c r="BF25" t="n">
-        <v>-94.72</v>
+        <v>-94.8</v>
       </c>
       <c r="BG25" t="n">
-        <v>-49.89</v>
+        <v>-50.68</v>
       </c>
       <c r="BH25" t="n">
         <v>3.97</v>
@@ -6277,7 +6277,7 @@
         <v>0</v>
       </c>
       <c r="BJ25" t="n">
-        <v>4.39</v>
+        <v>4.46</v>
       </c>
       <c r="BK25" t="n">
         <v>0.18</v>
@@ -6286,7 +6286,7 @@
         <v>0.24</v>
       </c>
       <c r="BM25" t="n">
-        <v>4.39</v>
+        <v>4.6</v>
       </c>
       <c r="BN25" t="n">
         <v>6.3</v>
@@ -6295,19 +6295,19 @@
         <v>2.64</v>
       </c>
       <c r="BP25" t="n">
-        <v>4.17</v>
+        <v>4.32</v>
       </c>
       <c r="BQ25" t="n">
-        <v>18.55</v>
+        <v>18.85</v>
       </c>
       <c r="BR25" t="n">
-        <v>4.3</v>
+        <v>4.46</v>
       </c>
       <c r="BS25" t="n">
         <v>0.67</v>
       </c>
       <c r="BT25" t="n">
-        <v>1161023</v>
+        <v>1172900</v>
       </c>
     </row>
     <row r="26">
@@ -6337,13 +6337,13 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>11.16</v>
+        <v>11.15</v>
       </c>
       <c r="G26" t="n">
-        <v>15115025673</v>
+        <v>15101481433</v>
       </c>
       <c r="H26" t="n">
-        <v>16044700</v>
+        <v>31033400</v>
       </c>
       <c r="I26" t="n">
         <v>1354393401</v>
@@ -6358,7 +6358,7 @@
         <v>1.94</v>
       </c>
       <c r="M26" t="n">
-        <v>0.1949069818774626</v>
+        <v>0.1947323300444234</v>
       </c>
       <c r="N26" t="n">
         <v>0.26</v>
@@ -6436,7 +6436,7 @@
         <v>961619314.7099999</v>
       </c>
       <c r="AM26" t="n">
-        <v>5398223454.642858</v>
+        <v>5393386226.071429</v>
       </c>
       <c r="AN26" t="n">
         <v>0.1043</v>
@@ -6486,10 +6486,10 @@
         <v>1.19</v>
       </c>
       <c r="BC26" t="n">
-        <v>-22.44</v>
+        <v>-22.37</v>
       </c>
       <c r="BD26" t="n">
-        <v>-36.67</v>
+        <v>-36.62</v>
       </c>
       <c r="BE26" t="n">
         <v>-80.83</v>
@@ -6498,7 +6498,7 @@
         <v>-94.09</v>
       </c>
       <c r="BG26" t="n">
-        <v>-89.31</v>
+        <v>-89.3</v>
       </c>
       <c r="BH26" t="n">
         <v>4.69</v>
@@ -6507,7 +6507,7 @@
         <v>0</v>
       </c>
       <c r="BJ26" t="n">
-        <v>11.16</v>
+        <v>11.15</v>
       </c>
       <c r="BK26" t="n">
         <v>0.71</v>
@@ -6516,28 +6516,28 @@
         <v>0.72</v>
       </c>
       <c r="BM26" t="n">
-        <v>11.46</v>
+        <v>11.52</v>
       </c>
       <c r="BN26" t="n">
-        <v>11.46</v>
+        <v>11.52</v>
       </c>
       <c r="BO26" t="n">
         <v>6.91</v>
       </c>
       <c r="BP26" t="n">
-        <v>10.88</v>
+        <v>10.85</v>
       </c>
       <c r="BQ26" t="n">
-        <v>15.56</v>
+        <v>15.55</v>
       </c>
       <c r="BR26" t="n">
-        <v>11.04</v>
+        <v>11.52</v>
       </c>
       <c r="BS26" t="n">
         <v>0.16</v>
       </c>
       <c r="BT26" t="n">
-        <v>12977910</v>
+        <v>13317553</v>
       </c>
     </row>
     <row r="27">
@@ -8165,13 +8165,13 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>18.6</v>
+        <v>19.54</v>
       </c>
       <c r="G34" t="n">
-        <v>3840710358</v>
+        <v>4032641940</v>
       </c>
       <c r="H34" t="n">
-        <v>8491200</v>
+        <v>4945600</v>
       </c>
       <c r="I34" t="n">
         <v>206489813</v>
@@ -8186,7 +8186,7 @@
         <v>0.45</v>
       </c>
       <c r="M34" t="n">
-        <v>0.3376432977019778</v>
+        <v>0.3545163254075566</v>
       </c>
       <c r="N34" t="n">
         <v>0.24</v>
@@ -8264,7 +8264,7 @@
         <v>324189006.41</v>
       </c>
       <c r="AM34" t="n">
-        <v>798484481.9126819</v>
+        <v>838387097.7130978</v>
       </c>
       <c r="AN34" t="n">
         <v>0</v>
@@ -8305,7 +8305,7 @@
         <v>30.28</v>
       </c>
       <c r="AZ34" t="n">
-        <v>43.4</v>
+        <v>45.59</v>
       </c>
       <c r="BA34" t="n">
         <v>2.29</v>
@@ -8314,19 +8314,19 @@
         <v>25.26</v>
       </c>
       <c r="BC34" t="n">
-        <v>99.40000000000001</v>
+        <v>89.81</v>
       </c>
       <c r="BD34" t="n">
-        <v>62.81</v>
+        <v>54.98</v>
       </c>
       <c r="BE34" t="n">
         <v>133.33</v>
       </c>
       <c r="BF34" t="n">
-        <v>-87.66</v>
+        <v>-88.26000000000001</v>
       </c>
       <c r="BG34" t="n">
-        <v>35.79</v>
+        <v>29.26</v>
       </c>
       <c r="BH34" t="n">
         <v>38.94</v>
@@ -8335,7 +8335,7 @@
         <v>0</v>
       </c>
       <c r="BJ34" t="n">
-        <v>18.6</v>
+        <v>19.54</v>
       </c>
       <c r="BK34" t="n">
         <v>1.57</v>
@@ -8344,7 +8344,7 @@
         <v>1.58</v>
       </c>
       <c r="BM34" t="n">
-        <v>19.13</v>
+        <v>19.57</v>
       </c>
       <c r="BN34" t="n">
         <v>28.86</v>
@@ -8353,19 +8353,19 @@
         <v>14.3</v>
       </c>
       <c r="BP34" t="n">
-        <v>17.4</v>
+        <v>18.65</v>
       </c>
       <c r="BQ34" t="n">
-        <v>11.79</v>
+        <v>12.39</v>
       </c>
       <c r="BR34" t="n">
-        <v>17.4</v>
+        <v>19.02</v>
       </c>
       <c r="BS34" t="n">
         <v>0.32</v>
       </c>
       <c r="BT34" t="n">
-        <v>3707453</v>
+        <v>3911500</v>
       </c>
     </row>
     <row r="35">
@@ -8395,13 +8395,13 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>18.51</v>
+        <v>19</v>
       </c>
       <c r="G35" t="n">
-        <v>93410716155</v>
+        <v>96299695000</v>
       </c>
       <c r="H35" t="n">
-        <v>36039100</v>
+        <v>40016700</v>
       </c>
       <c r="I35" t="n">
         <v>5046500000</v>
@@ -8416,7 +8416,7 @@
         <v>4.69</v>
       </c>
       <c r="M35" t="n">
-        <v>7.754991605322481</v>
+        <v>7.994835679034039</v>
       </c>
       <c r="N35" t="n">
         <v>1.79</v>
@@ -8494,7 +8494,7 @@
         <v>5349290000</v>
       </c>
       <c r="AM35" t="n">
-        <v>7719893897.107438</v>
+        <v>7958652479.338843</v>
       </c>
       <c r="AN35" t="n">
         <v>0.5305</v>
@@ -8535,7 +8535,7 @@
         <v>7.68</v>
       </c>
       <c r="AZ35" t="n">
-        <v>10.8</v>
+        <v>11.08</v>
       </c>
       <c r="BA35" t="n">
         <v>1.11</v>
@@ -8544,19 +8544,19 @@
         <v>9.119999999999999</v>
       </c>
       <c r="BC35" t="n">
-        <v>-49.18</v>
+        <v>-50.49</v>
       </c>
       <c r="BD35" t="n">
-        <v>-58.51</v>
+        <v>-59.58</v>
       </c>
       <c r="BE35" t="n">
         <v>-41.67</v>
       </c>
       <c r="BF35" t="n">
-        <v>-93.98</v>
+        <v>-94.14</v>
       </c>
       <c r="BG35" t="n">
-        <v>-50.75</v>
+        <v>-52.02</v>
       </c>
       <c r="BH35" t="n">
         <v>3.71</v>
@@ -8565,7 +8565,7 @@
         <v>0</v>
       </c>
       <c r="BJ35" t="n">
-        <v>18.51</v>
+        <v>19</v>
       </c>
       <c r="BK35" t="n">
         <v>1.06</v>
@@ -8574,7 +8574,7 @@
         <v>1.04</v>
       </c>
       <c r="BM35" t="n">
-        <v>18.58</v>
+        <v>19.04</v>
       </c>
       <c r="BN35" t="n">
         <v>19.88</v>
@@ -8583,19 +8583,19 @@
         <v>11.58</v>
       </c>
       <c r="BP35" t="n">
-        <v>18.11</v>
+        <v>18.32</v>
       </c>
       <c r="BQ35" t="n">
-        <v>17.71</v>
+        <v>18.18</v>
       </c>
       <c r="BR35" t="n">
-        <v>18.32</v>
+        <v>18.95</v>
       </c>
       <c r="BS35" t="n">
         <v>7.3</v>
       </c>
       <c r="BT35" t="n">
-        <v>40863943</v>
+        <v>40990940</v>
       </c>
     </row>
     <row r="36">
@@ -8861,7 +8861,7 @@
         <v>178849960</v>
       </c>
       <c r="H37" t="n">
-        <v>1000</v>
+        <v>1400</v>
       </c>
       <c r="I37" t="n">
         <v>4900000</v>
@@ -9043,7 +9043,7 @@
         <v>13.42</v>
       </c>
       <c r="BP37" t="n">
-        <v>14.5</v>
+        <v>14.2</v>
       </c>
       <c r="BQ37" t="n">
         <v>6.27</v>
@@ -9055,7 +9055,7 @@
         <v>0.72</v>
       </c>
       <c r="BT37" t="n">
-        <v>1233</v>
+        <v>1267</v>
       </c>
     </row>
     <row r="38">
@@ -9315,13 +9315,13 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>69.29000000000001</v>
+        <v>69.76000000000001</v>
       </c>
       <c r="G39" t="n">
-        <v>3884280351</v>
+        <v>3910628522</v>
       </c>
       <c r="H39" t="n">
-        <v>2000</v>
+        <v>1700</v>
       </c>
       <c r="I39" t="n">
         <v>168174945</v>
@@ -9336,7 +9336,7 @@
         <v>0.53</v>
       </c>
       <c r="M39" t="n">
-        <v>0.1949738357494382</v>
+        <v>0.1962963983609473</v>
       </c>
       <c r="N39" t="n">
         <v>0.06</v>
@@ -9414,7 +9414,7 @@
         <v>2536078170.6</v>
       </c>
       <c r="AM39" t="n">
-        <v>408012641.9117647</v>
+        <v>410780306.9327731</v>
       </c>
       <c r="AN39" t="n">
         <v>11.9435</v>
@@ -9455,7 +9455,7 @@
         <v>170.24</v>
       </c>
       <c r="AZ39" t="n">
-        <v>202.44</v>
+        <v>203.82</v>
       </c>
       <c r="BA39" t="n">
         <v>19.01</v>
@@ -9464,19 +9464,19 @@
         <v>91.72</v>
       </c>
       <c r="BC39" t="n">
-        <v>200.92</v>
+        <v>198.89</v>
       </c>
       <c r="BD39" t="n">
-        <v>145.7</v>
+        <v>144.04</v>
       </c>
       <c r="BE39" t="n">
         <v>192.17</v>
       </c>
       <c r="BF39" t="n">
-        <v>-72.56</v>
+        <v>-72.75</v>
       </c>
       <c r="BG39" t="n">
-        <v>32.38</v>
+        <v>31.48</v>
       </c>
       <c r="BH39" t="n">
         <v>128.13</v>
@@ -9485,7 +9485,7 @@
         <v>0</v>
       </c>
       <c r="BJ39" t="n">
-        <v>69.29000000000001</v>
+        <v>69.76000000000001</v>
       </c>
       <c r="BK39" t="n">
         <v>15.08</v>
@@ -9494,7 +9494,7 @@
         <v>15.08</v>
       </c>
       <c r="BM39" t="n">
-        <v>69.37</v>
+        <v>69.84999999999999</v>
       </c>
       <c r="BN39" t="n">
         <v>74.56</v>
@@ -9503,19 +9503,19 @@
         <v>54.98</v>
       </c>
       <c r="BP39" t="n">
-        <v>68.5</v>
+        <v>69.29000000000001</v>
       </c>
       <c r="BQ39" t="n">
-        <v>4.59</v>
+        <v>4.63</v>
       </c>
       <c r="BR39" t="n">
-        <v>69.37</v>
+        <v>69.34999999999999</v>
       </c>
       <c r="BS39" t="n">
         <v>0.58</v>
       </c>
       <c r="BT39" t="n">
-        <v>3027</v>
+        <v>3047</v>
       </c>
     </row>
     <row r="40">
@@ -9545,13 +9545,13 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>23.02</v>
+        <v>23.72</v>
       </c>
       <c r="G40" t="n">
-        <v>131923755263</v>
+        <v>135581974275</v>
       </c>
       <c r="H40" t="n">
-        <v>44611100</v>
+        <v>51578000</v>
       </c>
       <c r="I40" t="n">
         <v>5730834040</v>
@@ -9566,7 +9566,7 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="M40" t="n">
-        <v>0.4002729998019859</v>
+        <v>0.4113724890103301</v>
       </c>
       <c r="N40" t="n">
         <v>0.05</v>
@@ -9644,7 +9644,7 @@
         <v>15358635227.2</v>
       </c>
       <c r="AM40" t="n">
-        <v>6842518426.504149</v>
+        <v>7032260076.504149</v>
       </c>
       <c r="AN40" t="n">
         <v>0.5641</v>
@@ -9685,7 +9685,7 @@
         <v>36.13</v>
       </c>
       <c r="AZ40" t="n">
-        <v>11.63</v>
+        <v>11.98</v>
       </c>
       <c r="BA40" t="n">
         <v>2.76</v>
@@ -9694,19 +9694,19 @@
         <v>27.89</v>
       </c>
       <c r="BC40" t="n">
-        <v>92.22</v>
+        <v>86.55</v>
       </c>
       <c r="BD40" t="n">
-        <v>56.95</v>
+        <v>52.31</v>
       </c>
       <c r="BE40" t="n">
         <v>-49.5</v>
       </c>
       <c r="BF40" t="n">
-        <v>-88.01000000000001</v>
+        <v>-88.37</v>
       </c>
       <c r="BG40" t="n">
-        <v>21.16</v>
+        <v>17.58</v>
       </c>
       <c r="BH40" t="n">
         <v>32.47</v>
@@ -9715,7 +9715,7 @@
         <v>0</v>
       </c>
       <c r="BJ40" t="n">
-        <v>23.02</v>
+        <v>23.72</v>
       </c>
       <c r="BK40" t="n">
         <v>2.68</v>
@@ -9724,7 +9724,7 @@
         <v>2.5</v>
       </c>
       <c r="BM40" t="n">
-        <v>23.21</v>
+        <v>23.78</v>
       </c>
       <c r="BN40" t="n">
         <v>27.36</v>
@@ -9733,19 +9733,19 @@
         <v>17.67</v>
       </c>
       <c r="BP40" t="n">
-        <v>22.66</v>
+        <v>22.96</v>
       </c>
       <c r="BQ40" t="n">
-        <v>9.210000000000001</v>
+        <v>9.49</v>
       </c>
       <c r="BR40" t="n">
-        <v>23.07</v>
+        <v>23.36</v>
       </c>
       <c r="BS40" t="n">
         <v>0.39</v>
       </c>
       <c r="BT40" t="n">
-        <v>37951823</v>
+        <v>38498187</v>
       </c>
     </row>
     <row r="41">
@@ -9775,13 +9775,13 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>16.3</v>
+        <v>16.83</v>
       </c>
       <c r="G41" t="n">
-        <v>195044606494</v>
+        <v>202572276577</v>
       </c>
       <c r="H41" t="n">
-        <v>73450200</v>
+        <v>26344000</v>
       </c>
       <c r="I41" t="n">
         <v>5303870781</v>
@@ -9796,7 +9796,7 @@
         <v>0.92</v>
       </c>
       <c r="M41" t="n">
-        <v>1.299771105443528</v>
+        <v>1.34993526143364</v>
       </c>
       <c r="N41" t="n">
         <v>0.07000000000000001</v>
@@ -9874,7 +9874,7 @@
         <v>12304980211.92</v>
       </c>
       <c r="AM41" t="n">
-        <v>30053098073.03544</v>
+        <v>31212985605.08474</v>
       </c>
       <c r="AN41" t="n">
         <v>1.6841</v>
@@ -9915,7 +9915,7 @@
         <v>24.4</v>
       </c>
       <c r="AZ41" t="n">
-        <v>24.4</v>
+        <v>25.19</v>
       </c>
       <c r="BA41" t="n">
         <v>2.53</v>
@@ -9924,28 +9924,28 @@
         <v>13.77</v>
       </c>
       <c r="BC41" t="n">
-        <v>83.34999999999999</v>
+        <v>77.56999999999999</v>
       </c>
       <c r="BD41" t="n">
-        <v>49.7</v>
+        <v>44.99</v>
       </c>
       <c r="BE41" t="n">
         <v>49.67</v>
       </c>
       <c r="BF41" t="n">
-        <v>-84.5</v>
+        <v>-84.98</v>
       </c>
       <c r="BG41" t="n">
-        <v>-15.52</v>
+        <v>-18.18</v>
       </c>
       <c r="BH41" t="n">
         <v>17.11</v>
       </c>
       <c r="BI41" t="n">
-        <v>0.09</v>
+        <v>0</v>
       </c>
       <c r="BJ41" t="n">
-        <v>16.29</v>
+        <v>16.83</v>
       </c>
       <c r="BK41" t="n">
         <v>2.32</v>
@@ -9954,7 +9954,7 @@
         <v>2.34</v>
       </c>
       <c r="BM41" t="n">
-        <v>16.42</v>
+        <v>16.83</v>
       </c>
       <c r="BN41" t="n">
         <v>18.26</v>
@@ -9963,19 +9963,19 @@
         <v>13.41</v>
       </c>
       <c r="BP41" t="n">
-        <v>15.93</v>
+        <v>16.01</v>
       </c>
       <c r="BQ41" t="n">
-        <v>6.97</v>
+        <v>7.2</v>
       </c>
       <c r="BR41" t="n">
-        <v>16.23</v>
+        <v>16.7</v>
       </c>
       <c r="BS41" t="n">
         <v>0.5600000000000001</v>
       </c>
       <c r="BT41" t="n">
-        <v>7533983</v>
+        <v>9832217</v>
       </c>
     </row>
     <row r="42">
@@ -10005,13 +10005,13 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>18.57</v>
+        <v>19.23</v>
       </c>
       <c r="G42" t="n">
-        <v>195044606494</v>
+        <v>202572276577</v>
       </c>
       <c r="H42" t="n">
-        <v>96439600</v>
+        <v>109085500</v>
       </c>
       <c r="I42" t="n">
         <v>5288141247</v>
@@ -10026,7 +10026,7 @@
         <v>1.05</v>
       </c>
       <c r="M42" t="n">
-        <v>1.303637264239285</v>
+        <v>1.35395063311165</v>
       </c>
       <c r="N42" t="n">
         <v>0.08</v>
@@ -10104,7 +10104,7 @@
         <v>12268487693.04</v>
       </c>
       <c r="AM42" t="n">
-        <v>26536681155.64626</v>
+        <v>27560853956.05442</v>
       </c>
       <c r="AN42" t="n">
         <v>1.8491</v>
@@ -10145,7 +10145,7 @@
         <v>24.4</v>
       </c>
       <c r="AZ42" t="n">
-        <v>26.9</v>
+        <v>27.85</v>
       </c>
       <c r="BA42" t="n">
         <v>2.53</v>
@@ -10154,28 +10154,28 @@
         <v>15.11</v>
       </c>
       <c r="BC42" t="n">
-        <v>60.93</v>
+        <v>55.41</v>
       </c>
       <c r="BD42" t="n">
-        <v>31.4</v>
+        <v>26.89</v>
       </c>
       <c r="BE42" t="n">
         <v>44.83</v>
       </c>
       <c r="BF42" t="n">
-        <v>-86.39</v>
+        <v>-86.86</v>
       </c>
       <c r="BG42" t="n">
-        <v>-18.61</v>
+        <v>-21.4</v>
       </c>
       <c r="BH42" t="n">
         <v>17.11</v>
       </c>
       <c r="BI42" t="n">
-        <v>0.08</v>
+        <v>0</v>
       </c>
       <c r="BJ42" t="n">
-        <v>18.55</v>
+        <v>19.23</v>
       </c>
       <c r="BK42" t="n">
         <v>2.32</v>
@@ -10184,7 +10184,7 @@
         <v>2.34</v>
       </c>
       <c r="BM42" t="n">
-        <v>18.72</v>
+        <v>19.3</v>
       </c>
       <c r="BN42" t="n">
         <v>21.32</v>
@@ -10193,19 +10193,19 @@
         <v>15.65</v>
       </c>
       <c r="BP42" t="n">
-        <v>18.1</v>
+        <v>18.19</v>
       </c>
       <c r="BQ42" t="n">
-        <v>7.94</v>
+        <v>8.23</v>
       </c>
       <c r="BR42" t="n">
-        <v>18.44</v>
+        <v>18.94</v>
       </c>
       <c r="BS42" t="n">
         <v>0.63</v>
       </c>
       <c r="BT42" t="n">
-        <v>41125453</v>
+        <v>43064480</v>
       </c>
     </row>
     <row r="43">
@@ -10235,13 +10235,13 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>39.19</v>
+        <v>40.45</v>
       </c>
       <c r="G43" t="n">
-        <v>76083424143</v>
+        <v>78269982926</v>
       </c>
       <c r="H43" t="n">
-        <v>4510400</v>
+        <v>8697900</v>
       </c>
       <c r="I43" t="n">
         <v>1941400000</v>
@@ -10334,7 +10334,7 @@
         <v>9182822000</v>
       </c>
       <c r="AM43" t="n">
-        <v>9267164938.24604</v>
+        <v>9533493657.247259</v>
       </c>
       <c r="AN43" t="n">
         <v>4.5901</v>
@@ -10375,7 +10375,7 @@
         <v>19.95</v>
       </c>
       <c r="AZ43" t="n">
-        <v>71.13</v>
+        <v>73.42</v>
       </c>
       <c r="BA43" t="n">
         <v>5.63</v>
@@ -10384,19 +10384,19 @@
         <v>48.62</v>
       </c>
       <c r="BC43" t="n">
-        <v>-37.65</v>
+        <v>-39.59</v>
       </c>
       <c r="BD43" t="n">
-        <v>-49.09</v>
+        <v>-50.68</v>
       </c>
       <c r="BE43" t="n">
         <v>81.5</v>
       </c>
       <c r="BF43" t="n">
-        <v>-85.64</v>
+        <v>-86.08</v>
       </c>
       <c r="BG43" t="n">
-        <v>24.06</v>
+        <v>20.19</v>
       </c>
       <c r="BH43" t="n">
         <v>5.61</v>
@@ -10405,7 +10405,7 @@
         <v>0</v>
       </c>
       <c r="BJ43" t="n">
-        <v>39.19</v>
+        <v>40.45</v>
       </c>
       <c r="BK43" t="n">
         <v>4.73</v>
@@ -10414,7 +10414,7 @@
         <v>4.73</v>
       </c>
       <c r="BM43" t="n">
-        <v>39.47</v>
+        <v>40.79</v>
       </c>
       <c r="BN43" t="n">
         <v>42.98</v>
@@ -10423,19 +10423,19 @@
         <v>28.06</v>
       </c>
       <c r="BP43" t="n">
-        <v>38.9</v>
+        <v>39.51</v>
       </c>
       <c r="BQ43" t="n">
-        <v>8.279999999999999</v>
+        <v>8.539999999999999</v>
       </c>
       <c r="BR43" t="n">
-        <v>39.31</v>
+        <v>39.58</v>
       </c>
       <c r="BS43" t="n">
         <v>0</v>
       </c>
       <c r="BT43" t="n">
-        <v>6381763</v>
+        <v>6372740</v>
       </c>
     </row>
     <row r="44">
@@ -10925,13 +10925,13 @@
         </is>
       </c>
       <c r="F46" t="n">
-        <v>3.9</v>
+        <v>3.88</v>
       </c>
       <c r="G46" t="n">
-        <v>3902113895</v>
+        <v>3862297613</v>
       </c>
       <c r="H46" t="n">
-        <v>22662100</v>
+        <v>25088000</v>
       </c>
       <c r="I46" t="n">
         <v>1000542188</v>
@@ -10946,7 +10946,7 @@
         <v>2.5</v>
       </c>
       <c r="M46" t="n">
-        <v>0.06782607586340586</v>
+        <v>0.06713399402361354</v>
       </c>
       <c r="N46" t="n">
         <v>0.08</v>
@@ -11024,7 +11024,7 @@
         <v>460249406.48</v>
       </c>
       <c r="AM46" t="n">
-        <v>3825601857.843137</v>
+        <v>3786566287.254902</v>
       </c>
       <c r="AN46" t="n">
         <v>0.0311</v>
@@ -11065,7 +11065,7 @@
         <v>3.3</v>
       </c>
       <c r="AZ46" t="n">
-        <v>3.22</v>
+        <v>3.2</v>
       </c>
       <c r="BA46" t="n">
         <v>0.42</v>
@@ -11074,19 +11074,19 @@
         <v>7.38</v>
       </c>
       <c r="BC46" t="n">
-        <v>3.69</v>
+        <v>4.22</v>
       </c>
       <c r="BD46" t="n">
-        <v>-15.34</v>
+        <v>-14.9</v>
       </c>
       <c r="BE46" t="n">
         <v>-17.5</v>
       </c>
       <c r="BF46" t="n">
-        <v>-89.15000000000001</v>
+        <v>-89.09999999999999</v>
       </c>
       <c r="BG46" t="n">
-        <v>89.2</v>
+        <v>90.17</v>
       </c>
       <c r="BH46" t="n">
         <v>1.58</v>
@@ -11095,7 +11095,7 @@
         <v>0</v>
       </c>
       <c r="BJ46" t="n">
-        <v>3.9</v>
+        <v>3.88</v>
       </c>
       <c r="BK46" t="n">
         <v>0.46</v>
@@ -11104,7 +11104,7 @@
         <v>0.46</v>
       </c>
       <c r="BM46" t="n">
-        <v>3.99</v>
+        <v>3.95</v>
       </c>
       <c r="BN46" t="n">
         <v>7.31</v>
@@ -11113,19 +11113,19 @@
         <v>2.97</v>
       </c>
       <c r="BP46" t="n">
-        <v>3.82</v>
+        <v>3.81</v>
       </c>
       <c r="BQ46" t="n">
-        <v>8.529999999999999</v>
+        <v>8.48</v>
       </c>
       <c r="BR46" t="n">
-        <v>3.99</v>
+        <v>3.95</v>
       </c>
       <c r="BS46" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="BT46" t="n">
-        <v>21552368</v>
+        <v>21389101</v>
       </c>
     </row>
     <row r="47">
@@ -11155,13 +11155,13 @@
         </is>
       </c>
       <c r="F47" t="n">
-        <v>9.300000000000001</v>
+        <v>9.23</v>
       </c>
       <c r="G47" t="n">
-        <v>3252717846</v>
+        <v>3207462683</v>
       </c>
       <c r="H47" t="n">
-        <v>27700</v>
+        <v>21200</v>
       </c>
       <c r="I47" t="n">
         <v>254106600</v>
@@ -11176,7 +11176,7 @@
         <v>1.22</v>
       </c>
       <c r="M47" t="n">
-        <v>0.7670282914515677</v>
+        <v>0.7563566033437477</v>
       </c>
       <c r="N47" t="n">
         <v>0.07000000000000001</v>
@@ -11254,7 +11254,7 @@
         <v>322715382</v>
       </c>
       <c r="AM47" t="n">
-        <v>576723022.3404256</v>
+        <v>568699057.2695036</v>
       </c>
       <c r="AN47" t="n">
         <v>0.4132</v>
@@ -11295,7 +11295,7 @@
         <v>11.74</v>
       </c>
       <c r="AZ47" t="n">
-        <v>12.21</v>
+        <v>12.12</v>
       </c>
       <c r="BA47" t="n">
         <v>1.46</v>
@@ -11304,28 +11304,28 @@
         <v>8.619999999999999</v>
       </c>
       <c r="BC47" t="n">
-        <v>54.55</v>
+        <v>55.73</v>
       </c>
       <c r="BD47" t="n">
-        <v>26.19</v>
+        <v>27.15</v>
       </c>
       <c r="BE47" t="n">
         <v>31.33</v>
       </c>
       <c r="BF47" t="n">
-        <v>-84.31999999999999</v>
+        <v>-84.2</v>
       </c>
       <c r="BG47" t="n">
-        <v>-7.31</v>
+        <v>-6.61</v>
       </c>
       <c r="BH47" t="n">
         <v>7.23</v>
       </c>
       <c r="BI47" t="n">
-        <v>0.92</v>
+        <v>0</v>
       </c>
       <c r="BJ47" t="n">
-        <v>9.220000000000001</v>
+        <v>9.23</v>
       </c>
       <c r="BK47" t="n">
         <v>1.27</v>
@@ -11334,28 +11334,28 @@
         <v>1.28</v>
       </c>
       <c r="BM47" t="n">
-        <v>9.35</v>
+        <v>9.25</v>
       </c>
       <c r="BN47" t="n">
-        <v>9.35</v>
+        <v>9.32</v>
       </c>
       <c r="BO47" t="n">
         <v>7.17</v>
       </c>
       <c r="BP47" t="n">
-        <v>9.24</v>
+        <v>9</v>
       </c>
       <c r="BQ47" t="n">
-        <v>7.25</v>
+        <v>7.2</v>
       </c>
       <c r="BR47" t="n">
-        <v>9.289999999999999</v>
+        <v>9.25</v>
       </c>
       <c r="BS47" t="n">
         <v>0.53</v>
       </c>
       <c r="BT47" t="n">
-        <v>10117</v>
+        <v>10660</v>
       </c>
     </row>
     <row r="48">
@@ -11385,13 +11385,13 @@
         </is>
       </c>
       <c r="F48" t="n">
-        <v>9.300000000000001</v>
+        <v>9.17</v>
       </c>
       <c r="G48" t="n">
-        <v>3252717846</v>
+        <v>3207462683</v>
       </c>
       <c r="H48" t="n">
-        <v>6500</v>
+        <v>2800</v>
       </c>
       <c r="I48" t="n">
         <v>93397546</v>
@@ -11406,7 +11406,7 @@
         <v>1.24</v>
       </c>
       <c r="M48" t="n">
-        <v>2.086853023360667</v>
+        <v>2.05781857334055</v>
       </c>
       <c r="N48" t="n">
         <v>0.07000000000000001</v>
@@ -11484,7 +11484,7 @@
         <v>118614883.42</v>
       </c>
       <c r="AM48" t="n">
-        <v>568656966.0839161</v>
+        <v>560745224.3006994</v>
       </c>
       <c r="AN48" t="n">
         <v>0.4132</v>
@@ -11525,7 +11525,7 @@
         <v>11.74</v>
       </c>
       <c r="AZ48" t="n">
-        <v>12.17</v>
+        <v>12</v>
       </c>
       <c r="BA48" t="n">
         <v>1.46</v>
@@ -11534,28 +11534,28 @@
         <v>8.24</v>
       </c>
       <c r="BC48" t="n">
-        <v>54.55</v>
+        <v>56.74</v>
       </c>
       <c r="BD48" t="n">
-        <v>26.19</v>
+        <v>27.98</v>
       </c>
       <c r="BE48" t="n">
         <v>30.83</v>
       </c>
       <c r="BF48" t="n">
-        <v>-84.31999999999999</v>
+        <v>-84.09999999999999</v>
       </c>
       <c r="BG48" t="n">
-        <v>-11.44</v>
+        <v>-10.18</v>
       </c>
       <c r="BH48" t="n">
         <v>7.23</v>
       </c>
       <c r="BI48" t="n">
-        <v>0.92</v>
+        <v>0</v>
       </c>
       <c r="BJ48" t="n">
-        <v>9.220000000000001</v>
+        <v>9.17</v>
       </c>
       <c r="BK48" t="n">
         <v>1.27</v>
@@ -11564,28 +11564,28 @@
         <v>1.28</v>
       </c>
       <c r="BM48" t="n">
-        <v>9.51</v>
+        <v>9.369999999999999</v>
       </c>
       <c r="BN48" t="n">
-        <v>9.51</v>
+        <v>9.48</v>
       </c>
       <c r="BO48" t="n">
         <v>7.18</v>
       </c>
       <c r="BP48" t="n">
-        <v>9.300000000000001</v>
+        <v>9.140000000000001</v>
       </c>
       <c r="BQ48" t="n">
-        <v>7.25</v>
+        <v>7.15</v>
       </c>
       <c r="BR48" t="n">
-        <v>9.41</v>
+        <v>9.369999999999999</v>
       </c>
       <c r="BS48" t="n">
         <v>0.54</v>
       </c>
       <c r="BT48" t="n">
-        <v>2657</v>
+        <v>2693</v>
       </c>
     </row>
     <row r="49">
@@ -11615,13 +11615,13 @@
         </is>
       </c>
       <c r="F49" t="n">
-        <v>48.76</v>
+        <v>48.07</v>
       </c>
       <c r="G49" t="n">
-        <v>951749820</v>
+        <v>943199249</v>
       </c>
       <c r="H49" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="I49" t="n">
         <v>11540870</v>
@@ -11636,7 +11636,7 @@
         <v>1.09</v>
       </c>
       <c r="M49" t="n">
-        <v>0.9628730167252608</v>
+        <v>0.9542225143343136</v>
       </c>
       <c r="N49" t="n">
         <v>0.08</v>
@@ -11714,7 +11714,7 @@
         <v>84709985.8</v>
       </c>
       <c r="AM49" t="n">
-        <v>237937455</v>
+        <v>235799812.25</v>
       </c>
       <c r="AN49" t="n">
         <v>3.3186</v>
@@ -11755,7 +11755,7 @@
         <v>68.48999999999999</v>
       </c>
       <c r="AZ49" t="n">
-        <v>58.19</v>
+        <v>57.36</v>
       </c>
       <c r="BA49" t="n">
         <v>9.210000000000001</v>
@@ -11764,19 +11764,19 @@
         <v>27.75</v>
       </c>
       <c r="BC49" t="n">
-        <v>72.02</v>
+        <v>74.48999999999999</v>
       </c>
       <c r="BD49" t="n">
-        <v>40.45</v>
+        <v>42.47</v>
       </c>
       <c r="BE49" t="n">
         <v>19.33</v>
       </c>
       <c r="BF49" t="n">
-        <v>-81.09999999999999</v>
+        <v>-80.83</v>
       </c>
       <c r="BG49" t="n">
-        <v>-43.08</v>
+        <v>-42.26</v>
       </c>
       <c r="BH49" t="n">
         <v>42.6</v>
@@ -11785,7 +11785,7 @@
         <v>0</v>
       </c>
       <c r="BJ49" t="n">
-        <v>48.76</v>
+        <v>48.07</v>
       </c>
       <c r="BK49" t="n">
         <v>7.34</v>
@@ -11794,7 +11794,7 @@
         <v>7.6</v>
       </c>
       <c r="BM49" t="n">
-        <v>48.76</v>
+        <v>48.07</v>
       </c>
       <c r="BN49" t="n">
         <v>64.2</v>
@@ -11803,19 +11803,19 @@
         <v>28.48</v>
       </c>
       <c r="BP49" t="n">
-        <v>48.76</v>
+        <v>48.07</v>
       </c>
       <c r="BQ49" t="n">
-        <v>6.42</v>
+        <v>6.32</v>
       </c>
       <c r="BR49" t="n">
-        <v>48.76</v>
+        <v>48.07</v>
       </c>
       <c r="BS49" t="n">
         <v>0.54</v>
       </c>
       <c r="BT49" t="n">
-        <v>367</v>
+        <v>370</v>
       </c>
     </row>
     <row r="50">
@@ -11845,13 +11845,13 @@
         </is>
       </c>
       <c r="F50" t="n">
-        <v>34.14</v>
+        <v>34.1</v>
       </c>
       <c r="G50" t="n">
-        <v>962046900</v>
+        <v>943199249</v>
       </c>
       <c r="H50" t="n">
-        <v>600</v>
+        <v>400</v>
       </c>
       <c r="I50" t="n">
         <v>11540870</v>
@@ -11866,7 +11866,7 @@
         <v>0.8</v>
       </c>
       <c r="M50" t="n">
-        <v>0.9732904397441182</v>
+        <v>0.9542225143343136</v>
       </c>
       <c r="N50" t="n">
         <v>0.06</v>
@@ -11944,7 +11944,7 @@
         <v>84709985.8</v>
       </c>
       <c r="AM50" t="n">
-        <v>328343651.8771331</v>
+        <v>321911006.4846416</v>
       </c>
       <c r="AN50" t="n">
         <v>4.4983</v>
@@ -11985,7 +11985,7 @@
         <v>68.48999999999999</v>
       </c>
       <c r="AZ50" t="n">
-        <v>75.28</v>
+        <v>75.19</v>
       </c>
       <c r="BA50" t="n">
         <v>9.210000000000001</v>
@@ -11994,19 +11994,19 @@
         <v>30.53</v>
       </c>
       <c r="BC50" t="n">
-        <v>145.69</v>
+        <v>145.97</v>
       </c>
       <c r="BD50" t="n">
-        <v>100.6</v>
+        <v>100.84</v>
       </c>
       <c r="BE50" t="n">
         <v>120.5</v>
       </c>
       <c r="BF50" t="n">
-        <v>-73.01000000000001</v>
+        <v>-72.98</v>
       </c>
       <c r="BG50" t="n">
-        <v>-10.57</v>
+        <v>-10.47</v>
       </c>
       <c r="BH50" t="n">
         <v>42.6</v>
@@ -12015,7 +12015,7 @@
         <v>0</v>
       </c>
       <c r="BJ50" t="n">
-        <v>34.14</v>
+        <v>34.1</v>
       </c>
       <c r="BK50" t="n">
         <v>7.34</v>
@@ -12024,28 +12024,28 @@
         <v>7.6</v>
       </c>
       <c r="BM50" t="n">
-        <v>34.15</v>
+        <v>34.13</v>
       </c>
       <c r="BN50" t="n">
         <v>39.22</v>
       </c>
       <c r="BO50" t="n">
-        <v>23.69</v>
+        <v>23.95</v>
       </c>
       <c r="BP50" t="n">
-        <v>33.65</v>
+        <v>33.63</v>
       </c>
       <c r="BQ50" t="n">
         <v>4.49</v>
       </c>
       <c r="BR50" t="n">
-        <v>34.15</v>
+        <v>33.64</v>
       </c>
       <c r="BS50" t="n">
         <v>0.4</v>
       </c>
       <c r="BT50" t="n">
-        <v>513</v>
+        <v>490</v>
       </c>
     </row>
     <row r="51">
@@ -12523,13 +12523,13 @@
         </is>
       </c>
       <c r="F53" t="n">
-        <v>6.06</v>
+        <v>6.45</v>
       </c>
       <c r="G53" t="n">
-        <v>829325536</v>
+        <v>882697953</v>
       </c>
       <c r="H53" t="n">
-        <v>46800</v>
+        <v>57300</v>
       </c>
       <c r="I53" t="n">
         <v>136852484</v>
@@ -12544,7 +12544,7 @@
         <v>2.79</v>
       </c>
       <c r="M53" t="n">
-        <v>2.154433139585088</v>
+        <v>2.293084729260188</v>
       </c>
       <c r="N53" t="n">
         <v>1.48</v>
@@ -12622,7 +12622,7 @@
         <v>39687220.36</v>
       </c>
       <c r="AM53" t="n">
-        <v>42247862.25165563</v>
+        <v>44966783.138054</v>
       </c>
       <c r="AN53" t="n">
         <v>0</v>
@@ -12672,16 +12672,16 @@
         <v>0</v>
       </c>
       <c r="BC53" t="n">
-        <v>-34.97</v>
+        <v>-38.9</v>
       </c>
       <c r="BD53" t="n">
-        <v>-46.9</v>
+        <v>-50.11</v>
       </c>
       <c r="BE53" t="n">
         <v>-100</v>
       </c>
       <c r="BF53" t="n">
-        <v>-95.20999999999999</v>
+        <v>-95.5</v>
       </c>
       <c r="BG53" t="n">
         <v>-100</v>
@@ -12693,7 +12693,7 @@
         <v>0</v>
       </c>
       <c r="BJ53" t="n">
-        <v>6.06</v>
+        <v>6.45</v>
       </c>
       <c r="BK53" t="n">
         <v>0.29</v>
@@ -12702,7 +12702,7 @@
         <v>0.2</v>
       </c>
       <c r="BM53" t="n">
-        <v>6.15</v>
+        <v>6.45</v>
       </c>
       <c r="BN53" t="n">
         <v>10.39</v>
@@ -12711,19 +12711,19 @@
         <v>4.82</v>
       </c>
       <c r="BP53" t="n">
-        <v>5.84</v>
+        <v>5.96</v>
       </c>
       <c r="BQ53" t="n">
-        <v>29.77</v>
+        <v>31.68</v>
       </c>
       <c r="BR53" t="n">
-        <v>6.11</v>
+        <v>6.12</v>
       </c>
       <c r="BS53" t="n">
         <v>2.36</v>
       </c>
       <c r="BT53" t="n">
-        <v>35620</v>
+        <v>37073</v>
       </c>
     </row>
     <row r="54">
@@ -12753,13 +12753,13 @@
         </is>
       </c>
       <c r="F54" t="n">
-        <v>10.74</v>
+        <v>10.82</v>
       </c>
       <c r="G54" t="n">
-        <v>2504697900</v>
+        <v>2535156224</v>
       </c>
       <c r="H54" t="n">
-        <v>131300</v>
+        <v>334700</v>
       </c>
       <c r="I54" t="n">
         <v>233212121</v>
@@ -12774,7 +12774,7 @@
         <v>0.97</v>
       </c>
       <c r="M54" t="n">
-        <v>1.405865843096551</v>
+        <v>1.42296184391548</v>
       </c>
       <c r="N54" t="n">
         <v>0.5600000000000001</v>
@@ -12852,7 +12852,7 @@
         <v>233212121</v>
       </c>
       <c r="AM54" t="n">
-        <v>342639931.6005472</v>
+        <v>346806596.9904241</v>
       </c>
       <c r="AN54" t="n">
         <v>0.1531</v>
@@ -12893,7 +12893,7 @@
         <v>12.25</v>
       </c>
       <c r="AZ54" t="n">
-        <v>17.09</v>
+        <v>17.22</v>
       </c>
       <c r="BA54" t="n">
         <v>0.98</v>
@@ -12902,19 +12902,19 @@
         <v>6.52</v>
       </c>
       <c r="BC54" t="n">
-        <v>39.73</v>
+        <v>38.7</v>
       </c>
       <c r="BD54" t="n">
-        <v>14.09</v>
+        <v>13.25</v>
       </c>
       <c r="BE54" t="n">
         <v>59.17</v>
       </c>
       <c r="BF54" t="n">
-        <v>-90.84</v>
+        <v>-90.91</v>
       </c>
       <c r="BG54" t="n">
-        <v>-39.33</v>
+        <v>-39.77</v>
       </c>
       <c r="BH54" t="n">
         <v>10.01</v>
@@ -12923,7 +12923,7 @@
         <v>0</v>
       </c>
       <c r="BJ54" t="n">
-        <v>10.74</v>
+        <v>10.82</v>
       </c>
       <c r="BK54" t="n">
         <v>1</v>
@@ -12932,7 +12932,7 @@
         <v>1</v>
       </c>
       <c r="BM54" t="n">
-        <v>10.79</v>
+        <v>10.9</v>
       </c>
       <c r="BN54" t="n">
         <v>11.68</v>
@@ -12941,19 +12941,19 @@
         <v>8.23</v>
       </c>
       <c r="BP54" t="n">
-        <v>10.62</v>
+        <v>10.67</v>
       </c>
       <c r="BQ54" t="n">
-        <v>10.71</v>
+        <v>10.79</v>
       </c>
       <c r="BR54" t="n">
-        <v>10.7</v>
+        <v>10.8</v>
       </c>
       <c r="BS54" t="n">
         <v>1.26</v>
       </c>
       <c r="BT54" t="n">
-        <v>244503</v>
+        <v>243630</v>
       </c>
     </row>
     <row r="55">
@@ -12983,13 +12983,13 @@
         </is>
       </c>
       <c r="F55" t="n">
-        <v>49.42</v>
+        <v>50.79</v>
       </c>
       <c r="G55" t="n">
-        <v>6429320510</v>
+        <v>6696691718</v>
       </c>
       <c r="H55" t="n">
-        <v>3900</v>
+        <v>4100</v>
       </c>
       <c r="I55" t="n">
         <v>84052790</v>
@@ -13004,7 +13004,7 @@
         <v>2</v>
       </c>
       <c r="M55" t="n">
-        <v>0.9925016549438603</v>
+        <v>1.033776058049382</v>
       </c>
       <c r="N55" t="n">
         <v>0.16</v>
@@ -13082,7 +13082,7 @@
         <v>579123723.1</v>
       </c>
       <c r="AM55" t="n">
-        <v>323406464.2857143</v>
+        <v>336855720.221328</v>
       </c>
       <c r="AN55" t="n">
         <v>3.1953</v>
@@ -13123,7 +13123,7 @@
         <v>51.21</v>
       </c>
       <c r="AZ55" t="n">
-        <v>51.97</v>
+        <v>53.41</v>
       </c>
       <c r="BA55" t="n">
         <v>9.380000000000001</v>
@@ -13132,19 +13132,19 @@
         <v>16.08</v>
       </c>
       <c r="BC55" t="n">
-        <v>26.9</v>
+        <v>23.48</v>
       </c>
       <c r="BD55" t="n">
-        <v>3.61</v>
+        <v>0.82</v>
       </c>
       <c r="BE55" t="n">
         <v>5.17</v>
       </c>
       <c r="BF55" t="n">
-        <v>-81.02</v>
+        <v>-81.54000000000001</v>
       </c>
       <c r="BG55" t="n">
-        <v>-67.47</v>
+        <v>-68.34999999999999</v>
       </c>
       <c r="BH55" t="n">
         <v>25.37</v>
@@ -13153,7 +13153,7 @@
         <v>0</v>
       </c>
       <c r="BJ55" t="n">
-        <v>49.42</v>
+        <v>50.79</v>
       </c>
       <c r="BK55" t="n">
         <v>6.89</v>
@@ -13162,7 +13162,7 @@
         <v>7.03</v>
       </c>
       <c r="BM55" t="n">
-        <v>49.95</v>
+        <v>50.79</v>
       </c>
       <c r="BN55" t="n">
         <v>73.67</v>
@@ -13171,19 +13171,19 @@
         <v>35.58</v>
       </c>
       <c r="BP55" t="n">
-        <v>49.42</v>
+        <v>49.98</v>
       </c>
       <c r="BQ55" t="n">
-        <v>7.03</v>
+        <v>7.22</v>
       </c>
       <c r="BR55" t="n">
-        <v>49.95</v>
+        <v>49.98</v>
       </c>
       <c r="BS55" t="n">
         <v>0.66</v>
       </c>
       <c r="BT55" t="n">
-        <v>5947</v>
+        <v>5920</v>
       </c>
     </row>
     <row r="56">
@@ -13213,13 +13213,13 @@
         </is>
       </c>
       <c r="F56" t="n">
-        <v>58.77</v>
+        <v>60.92</v>
       </c>
       <c r="G56" t="n">
-        <v>6429320510</v>
+        <v>6696691718</v>
       </c>
       <c r="H56" t="n">
-        <v>13300</v>
+        <v>52300</v>
       </c>
       <c r="I56" t="n">
         <v>39675836</v>
@@ -13234,7 +13234,7 @@
         <v>2.41</v>
       </c>
       <c r="M56" t="n">
-        <v>2.102603034694689</v>
+        <v>2.190042370228885</v>
       </c>
       <c r="N56" t="n">
         <v>0.19</v>
@@ -13312,7 +13312,7 @@
         <v>273366510.04</v>
       </c>
       <c r="AM56" t="n">
-        <v>267442616.8885191</v>
+        <v>278564547.3377704</v>
       </c>
       <c r="AN56" t="n">
         <v>3.5102</v>
@@ -13353,7 +13353,7 @@
         <v>51.21</v>
       </c>
       <c r="AZ56" t="n">
-        <v>56.13</v>
+        <v>58.18</v>
       </c>
       <c r="BA56" t="n">
         <v>9.380000000000001</v>
@@ -13362,19 +13362,19 @@
         <v>17.68</v>
       </c>
       <c r="BC56" t="n">
-        <v>6.71</v>
+        <v>2.94</v>
       </c>
       <c r="BD56" t="n">
-        <v>-12.87</v>
+        <v>-15.95</v>
       </c>
       <c r="BE56" t="n">
         <v>-4.5</v>
       </c>
       <c r="BF56" t="n">
-        <v>-84.04000000000001</v>
+        <v>-84.61</v>
       </c>
       <c r="BG56" t="n">
-        <v>-69.92</v>
+        <v>-70.98</v>
       </c>
       <c r="BH56" t="n">
         <v>25.37</v>
@@ -13383,7 +13383,7 @@
         <v>0</v>
       </c>
       <c r="BJ56" t="n">
-        <v>58.77</v>
+        <v>60.92</v>
       </c>
       <c r="BK56" t="n">
         <v>6.89</v>
@@ -13392,7 +13392,7 @@
         <v>7.03</v>
       </c>
       <c r="BM56" t="n">
-        <v>59.74</v>
+        <v>61.3</v>
       </c>
       <c r="BN56" t="n">
         <v>86.77</v>
@@ -13401,19 +13401,19 @@
         <v>46.42</v>
       </c>
       <c r="BP56" t="n">
-        <v>58.75</v>
+        <v>58.71</v>
       </c>
       <c r="BQ56" t="n">
-        <v>8.359999999999999</v>
+        <v>8.66</v>
       </c>
       <c r="BR56" t="n">
-        <v>59.65</v>
+        <v>58.71</v>
       </c>
       <c r="BS56" t="n">
         <v>0.79</v>
       </c>
       <c r="BT56" t="n">
-        <v>28630</v>
+        <v>28133</v>
       </c>
     </row>
     <row r="57">
@@ -13443,13 +13443,13 @@
         </is>
       </c>
       <c r="F57" t="n">
-        <v>6.51</v>
+        <v>6.59</v>
       </c>
       <c r="G57" t="n">
-        <v>1522414982</v>
+        <v>1543495337</v>
       </c>
       <c r="H57" t="n">
-        <v>2748000</v>
+        <v>2831000</v>
       </c>
       <c r="I57" t="n">
         <v>233858065</v>
@@ -13464,7 +13464,7 @@
         <v>0.77</v>
       </c>
       <c r="M57" t="n">
-        <v>0.4556996943423782</v>
+        <v>0.4620096107867822</v>
       </c>
       <c r="N57" t="n">
         <v>0.08</v>
@@ -13542,7 +13542,7 @@
         <v>229180903.7</v>
       </c>
       <c r="AM57" t="n">
-        <v>113867986.6866118</v>
+        <v>115444677.4121167</v>
       </c>
       <c r="AN57" t="n">
         <v>0.347</v>
@@ -13583,7 +13583,7 @@
         <v>10.72</v>
       </c>
       <c r="AZ57" t="n">
-        <v>9.93</v>
+        <v>10.05</v>
       </c>
       <c r="BA57" t="n">
         <v>1.13</v>
@@ -13592,19 +13592,19 @@
         <v>6.26</v>
       </c>
       <c r="BC57" t="n">
-        <v>101.71</v>
+        <v>99.26000000000001</v>
       </c>
       <c r="BD57" t="n">
-        <v>64.7</v>
+        <v>62.7</v>
       </c>
       <c r="BE57" t="n">
         <v>52.5</v>
       </c>
       <c r="BF57" t="n">
-        <v>-82.68000000000001</v>
+        <v>-82.89</v>
       </c>
       <c r="BG57" t="n">
-        <v>-3.78</v>
+        <v>-4.95</v>
       </c>
       <c r="BH57" t="n">
         <v>7.82</v>
@@ -13613,7 +13613,7 @@
         <v>0</v>
       </c>
       <c r="BJ57" t="n">
-        <v>6.51</v>
+        <v>6.59</v>
       </c>
       <c r="BK57" t="n">
         <v>0.98</v>
@@ -13622,28 +13622,28 @@
         <v>1.04</v>
       </c>
       <c r="BM57" t="n">
-        <v>6.52</v>
+        <v>6.63</v>
       </c>
       <c r="BN57" t="n">
-        <v>6.52</v>
+        <v>6.63</v>
       </c>
       <c r="BO57" t="n">
         <v>3.43</v>
       </c>
       <c r="BP57" t="n">
-        <v>6.26</v>
+        <v>6.47</v>
       </c>
       <c r="BQ57" t="n">
-        <v>6.28</v>
+        <v>6.36</v>
       </c>
       <c r="BR57" t="n">
-        <v>6.36</v>
+        <v>6.52</v>
       </c>
       <c r="BS57" t="n">
         <v>0.42</v>
       </c>
       <c r="BT57" t="n">
-        <v>1352800</v>
+        <v>1422917</v>
       </c>
     </row>
     <row r="58">
@@ -14133,13 +14133,13 @@
         </is>
       </c>
       <c r="F60" t="n">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="G60" t="n">
-        <v>171895500</v>
+        <v>171440750</v>
       </c>
       <c r="H60" t="n">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="I60" t="n">
         <v>454750</v>
@@ -14154,7 +14154,7 @@
         <v>0.83</v>
       </c>
       <c r="M60" t="n">
-        <v>12.85754142169963</v>
+        <v>12.82352676185386</v>
       </c>
       <c r="N60" t="n">
         <v>0.68</v>
@@ -14232,7 +14232,7 @@
         <v>59558607.5</v>
       </c>
       <c r="AM60" t="n">
-        <v>-25204618.76832844</v>
+        <v>-25137939.88269795</v>
       </c>
       <c r="AN60" t="n">
         <v>10.0581</v>
@@ -14273,7 +14273,7 @@
         <v>944.87</v>
       </c>
       <c r="AZ60" t="n">
-        <v>2173.5</v>
+        <v>2167.75</v>
       </c>
       <c r="BA60" t="n">
         <v>231.1</v>
@@ -14282,19 +14282,19 @@
         <v>727.97</v>
       </c>
       <c r="BC60" t="n">
-        <v>206.14</v>
+        <v>206.95</v>
       </c>
       <c r="BD60" t="n">
-        <v>149.96</v>
+        <v>150.63</v>
       </c>
       <c r="BE60" t="n">
         <v>475</v>
       </c>
       <c r="BF60" t="n">
-        <v>-38.86</v>
+        <v>-38.7</v>
       </c>
       <c r="BG60" t="n">
-        <v>92.59</v>
+        <v>93.09999999999999</v>
       </c>
       <c r="BH60" t="n">
         <v>454.44</v>
@@ -14303,7 +14303,7 @@
         <v>0</v>
       </c>
       <c r="BJ60" t="n">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="BK60" t="n">
         <v>130.97</v>
@@ -14312,7 +14312,7 @@
         <v>130.97</v>
       </c>
       <c r="BM60" t="n">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="BN60" t="n">
         <v>405</v>
@@ -14321,13 +14321,13 @@
         <v>309.24</v>
       </c>
       <c r="BP60" t="n">
+        <v>369.23</v>
+      </c>
+      <c r="BQ60" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="BR60" t="n">
         <v>378</v>
-      </c>
-      <c r="BQ60" t="n">
-        <v>2.89</v>
-      </c>
-      <c r="BR60" t="n">
-        <v>380</v>
       </c>
       <c r="BS60" t="n">
         <v>12.82</v>
@@ -14363,13 +14363,13 @@
         </is>
       </c>
       <c r="F61" t="n">
-        <v>27.84</v>
+        <v>28.34</v>
       </c>
       <c r="G61" t="n">
-        <v>2383337312</v>
+        <v>2420924675</v>
       </c>
       <c r="H61" t="n">
-        <v>769100</v>
+        <v>624300</v>
       </c>
       <c r="I61" t="n">
         <v>85608392</v>
@@ -14384,7 +14384,7 @@
         <v>2.37</v>
       </c>
       <c r="M61" t="n">
-        <v>1.263965605015255</v>
+        <v>1.283899474122249</v>
       </c>
       <c r="N61" t="n">
         <v>1.1</v>
@@ -14462,7 +14462,7 @@
         <v>160087693.04</v>
       </c>
       <c r="AM61" t="n">
-        <v>187075142.2291994</v>
+        <v>190025484.6938775</v>
       </c>
       <c r="AN61" t="n">
         <v>0.38</v>
@@ -14503,7 +14503,7 @@
         <v>17.56</v>
       </c>
       <c r="AZ61" t="n">
-        <v>35.08</v>
+        <v>35.71</v>
       </c>
       <c r="BA61" t="n">
         <v>2.52</v>
@@ -14512,19 +14512,19 @@
         <v>11.76</v>
       </c>
       <c r="BC61" t="n">
-        <v>-22.76</v>
+        <v>-24.12</v>
       </c>
       <c r="BD61" t="n">
-        <v>-36.93</v>
+        <v>-38.05</v>
       </c>
       <c r="BE61" t="n">
         <v>26</v>
       </c>
       <c r="BF61" t="n">
-        <v>-90.94</v>
+        <v>-91.09999999999999</v>
       </c>
       <c r="BG61" t="n">
-        <v>-57.77</v>
+        <v>-58.52</v>
       </c>
       <c r="BH61" t="n">
         <v>10.99</v>
@@ -14533,7 +14533,7 @@
         <v>0</v>
       </c>
       <c r="BJ61" t="n">
-        <v>27.84</v>
+        <v>28.34</v>
       </c>
       <c r="BK61" t="n">
         <v>1.87</v>
@@ -14542,7 +14542,7 @@
         <v>1.86</v>
       </c>
       <c r="BM61" t="n">
-        <v>28.54</v>
+        <v>28.35</v>
       </c>
       <c r="BN61" t="n">
         <v>28.68</v>
@@ -14551,19 +14551,19 @@
         <v>19.35</v>
       </c>
       <c r="BP61" t="n">
-        <v>27.62</v>
+        <v>27.65</v>
       </c>
       <c r="BQ61" t="n">
-        <v>14.95</v>
+        <v>15.22</v>
       </c>
       <c r="BR61" t="n">
-        <v>28.16</v>
+        <v>28.35</v>
       </c>
       <c r="BS61" t="n">
         <v>1.19</v>
       </c>
       <c r="BT61" t="n">
-        <v>683753</v>
+        <v>700600</v>
       </c>
     </row>
     <row r="62">
@@ -14593,10 +14593,10 @@
         </is>
       </c>
       <c r="F62" t="n">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="G62" t="n">
-        <v>10856974700</v>
+        <v>11054368640</v>
       </c>
       <c r="H62" t="n">
         <v>100</v>
@@ -14614,7 +14614,7 @@
         <v>0.64</v>
       </c>
       <c r="M62" t="n">
-        <v>1.017716751969055</v>
+        <v>1.036220167978228</v>
       </c>
       <c r="N62" t="n">
         <v>0.13</v>
@@ -14692,7 +14692,7 @@
         <v>2757670987.06</v>
       </c>
       <c r="AM62" t="n">
-        <v>4395536315.789474</v>
+        <v>4475452890.688259</v>
       </c>
       <c r="AN62" t="n">
         <v>6.9319</v>
@@ -14733,7 +14733,7 @@
         <v>267.2</v>
       </c>
       <c r="AZ62" t="n">
-        <v>116.23</v>
+        <v>118.35</v>
       </c>
       <c r="BA62" t="n">
         <v>34.09</v>
@@ -14742,19 +14742,19 @@
         <v>76.01000000000001</v>
       </c>
       <c r="BC62" t="n">
-        <v>197.5</v>
+        <v>192.18</v>
       </c>
       <c r="BD62" t="n">
-        <v>142.91</v>
+        <v>138.57</v>
       </c>
       <c r="BE62" t="n">
         <v>5.67</v>
       </c>
       <c r="BF62" t="n">
-        <v>-69.01000000000001</v>
+        <v>-69.56</v>
       </c>
       <c r="BG62" t="n">
-        <v>-30.9</v>
+        <v>-32.14</v>
       </c>
       <c r="BH62" t="n">
         <v>170.35</v>
@@ -14763,7 +14763,7 @@
         <v>0</v>
       </c>
       <c r="BJ62" t="n">
-        <v>108.02</v>
+        <v>112</v>
       </c>
       <c r="BK62" t="n">
         <v>27.94</v>
@@ -14772,7 +14772,7 @@
         <v>32.73</v>
       </c>
       <c r="BM62" t="n">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="BN62" t="n">
         <v>122.2</v>
@@ -14781,19 +14781,19 @@
         <v>91.84999999999999</v>
       </c>
       <c r="BP62" t="n">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="BQ62" t="n">
-        <v>3.36</v>
+        <v>3.42</v>
       </c>
       <c r="BR62" t="n">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="BS62" t="n">
         <v>1.01</v>
       </c>
       <c r="BT62" t="n">
-        <v>157</v>
+        <v>117</v>
       </c>
     </row>
     <row r="63">
@@ -14823,13 +14823,13 @@
         </is>
       </c>
       <c r="F63" t="n">
-        <v>1.57</v>
+        <v>1.6</v>
       </c>
       <c r="G63" t="n">
-        <v>409000242</v>
+        <v>409000166</v>
       </c>
       <c r="H63" t="n">
-        <v>6300</v>
+        <v>85800</v>
       </c>
       <c r="I63" t="n">
         <v>122894462</v>
@@ -14844,7 +14844,7 @@
         <v>-0.22</v>
       </c>
       <c r="M63" t="n">
-        <v>0.5030491907450951</v>
+        <v>0.5030490972690173</v>
       </c>
       <c r="N63" t="n">
         <v>0.37</v>
@@ -14922,7 +14922,7 @@
         <v>31952560.12</v>
       </c>
       <c r="AM63" t="n">
-        <v>232386501.1363636</v>
+        <v>232386457.9545455</v>
       </c>
       <c r="AN63" t="n">
         <v>0</v>
@@ -14981,7 +14981,7 @@
         <v>-100</v>
       </c>
       <c r="BF63" t="n">
-        <v>-81.58</v>
+        <v>-81.93000000000001</v>
       </c>
       <c r="BG63" t="n">
         <v>-100</v>
@@ -14993,7 +14993,7 @@
         <v>0</v>
       </c>
       <c r="BJ63" t="n">
-        <v>1.57</v>
+        <v>1.6</v>
       </c>
       <c r="BK63" t="n">
         <v>0.26</v>
@@ -15002,7 +15002,7 @@
         <v>0.26</v>
       </c>
       <c r="BM63" t="n">
-        <v>1.6</v>
+        <v>1.7</v>
       </c>
       <c r="BN63" t="n">
         <v>2.12</v>
@@ -15011,19 +15011,19 @@
         <v>1.16</v>
       </c>
       <c r="BP63" t="n">
-        <v>1.57</v>
+        <v>1.59</v>
       </c>
       <c r="BQ63" t="n">
-        <v>6.01</v>
+        <v>6.13</v>
       </c>
       <c r="BR63" t="n">
-        <v>1.57</v>
+        <v>1.59</v>
       </c>
       <c r="BS63" t="n">
         <v>0.19</v>
       </c>
       <c r="BT63" t="n">
-        <v>31337</v>
+        <v>31417</v>
       </c>
     </row>
     <row r="64">
@@ -15053,13 +15053,13 @@
         </is>
       </c>
       <c r="F64" t="n">
-        <v>63.7</v>
+        <v>66.02</v>
       </c>
       <c r="G64" t="n">
-        <v>241321019190</v>
+        <v>250357994349</v>
       </c>
       <c r="H64" t="n">
-        <v>12951900</v>
+        <v>14513200</v>
       </c>
       <c r="I64" t="n">
         <v>0</v>
@@ -15146,13 +15146,13 @@
         <v>41.22</v>
       </c>
       <c r="AK64" t="n">
-        <v>69190277387.84583</v>
+        <v>71781310776.05635</v>
       </c>
       <c r="AL64" t="n">
-        <v>19290249335.73141</v>
+        <v>20012629444.36451</v>
       </c>
       <c r="AM64" t="n">
-        <v>21488959856.63401</v>
+        <v>22293677145.94835</v>
       </c>
       <c r="AN64" t="n">
         <v>1.4201</v>
@@ -15193,7 +15193,7 @@
         <v>38.98</v>
       </c>
       <c r="AZ64" t="n">
-        <v>25.48</v>
+        <v>26.41</v>
       </c>
       <c r="BA64" t="n">
         <v>6.69</v>
@@ -15202,19 +15202,19 @@
         <v>10.4</v>
       </c>
       <c r="BC64" t="n">
-        <v>-25.05</v>
+        <v>-27.69</v>
       </c>
       <c r="BD64" t="n">
-        <v>-38.81</v>
+        <v>-40.96</v>
       </c>
       <c r="BE64" t="n">
         <v>-60</v>
       </c>
       <c r="BF64" t="n">
-        <v>-89.48999999999999</v>
+        <v>-89.86</v>
       </c>
       <c r="BG64" t="n">
-        <v>-83.68000000000001</v>
+        <v>-84.25</v>
       </c>
       <c r="BH64" t="n">
         <v>21.37</v>
@@ -15223,7 +15223,7 @@
         <v>0</v>
       </c>
       <c r="BJ64" t="n">
-        <v>63.7</v>
+        <v>66.02</v>
       </c>
       <c r="BK64" t="n">
         <v>4.74</v>
@@ -15232,28 +15232,28 @@
         <v>1.57</v>
       </c>
       <c r="BM64" t="n">
-        <v>64.79000000000001</v>
+        <v>66.02</v>
       </c>
       <c r="BN64" t="n">
-        <v>64.79000000000001</v>
+        <v>66.02</v>
       </c>
       <c r="BO64" t="n">
         <v>44.12</v>
       </c>
       <c r="BP64" t="n">
-        <v>63.07</v>
+        <v>63.15</v>
       </c>
       <c r="BQ64" t="n">
-        <v>40.57</v>
+        <v>42.05</v>
       </c>
       <c r="BR64" t="n">
-        <v>63.89</v>
+        <v>65.45</v>
       </c>
       <c r="BS64" t="n">
         <v>3.49</v>
       </c>
       <c r="BT64" t="n">
-        <v>10276677</v>
+        <v>10434673</v>
       </c>
     </row>
     <row r="65">
@@ -15283,13 +15283,13 @@
         </is>
       </c>
       <c r="F65" t="n">
-        <v>24.77</v>
+        <v>24.97</v>
       </c>
       <c r="G65" t="n">
-        <v>241321019190</v>
+        <v>250357994349</v>
       </c>
       <c r="H65" t="n">
-        <v>9800</v>
+        <v>6700</v>
       </c>
       <c r="I65" t="n">
         <v>7298813414</v>
@@ -15304,7 +15304,7 @@
         <v>3.29</v>
       </c>
       <c r="M65" t="n">
-        <v>5.834163176140064</v>
+        <v>6.052640571409224</v>
       </c>
       <c r="N65" t="n">
         <v>0.29</v>
@@ -15382,7 +15382,7 @@
         <v>11532125194.12</v>
       </c>
       <c r="AM65" t="n">
-        <v>18076480838.20225</v>
+        <v>18753407816.4045</v>
       </c>
       <c r="AN65" t="n">
         <v>0.4734</v>
@@ -15423,7 +15423,7 @@
         <v>12.99</v>
       </c>
       <c r="AZ65" t="n">
-        <v>8.34</v>
+        <v>8.41</v>
       </c>
       <c r="BA65" t="n">
         <v>2.23</v>
@@ -15432,19 +15432,19 @@
         <v>3.47</v>
       </c>
       <c r="BC65" t="n">
-        <v>-35.77</v>
+        <v>-36.29</v>
       </c>
       <c r="BD65" t="n">
-        <v>-47.56</v>
+        <v>-47.98</v>
       </c>
       <c r="BE65" t="n">
         <v>-66.33</v>
       </c>
       <c r="BF65" t="n">
-        <v>-90.98999999999999</v>
+        <v>-91.06</v>
       </c>
       <c r="BG65" t="n">
-        <v>-86.01000000000001</v>
+        <v>-86.12</v>
       </c>
       <c r="BH65" t="n">
         <v>7.12</v>
@@ -15453,7 +15453,7 @@
         <v>0</v>
       </c>
       <c r="BJ65" t="n">
-        <v>24.77</v>
+        <v>24.97</v>
       </c>
       <c r="BK65" t="n">
         <v>1.58</v>
@@ -15462,7 +15462,7 @@
         <v>1.57</v>
       </c>
       <c r="BM65" t="n">
-        <v>24.99</v>
+        <v>25.2</v>
       </c>
       <c r="BN65" t="n">
         <v>46.43</v>
@@ -15471,19 +15471,19 @@
         <v>20.44</v>
       </c>
       <c r="BP65" t="n">
-        <v>23.75</v>
+        <v>24.69</v>
       </c>
       <c r="BQ65" t="n">
-        <v>15.78</v>
+        <v>15.9</v>
       </c>
       <c r="BR65" t="n">
-        <v>24.8</v>
+        <v>25</v>
       </c>
       <c r="BS65" t="n">
         <v>4.14</v>
       </c>
       <c r="BT65" t="n">
-        <v>7957</v>
+        <v>7647</v>
       </c>
     </row>
     <row r="66">
@@ -15513,13 +15513,13 @@
         </is>
       </c>
       <c r="F66" t="n">
-        <v>20.46</v>
+        <v>20.99</v>
       </c>
       <c r="G66" t="n">
-        <v>241321019190</v>
+        <v>250357994349</v>
       </c>
       <c r="H66" t="n">
-        <v>3000</v>
+        <v>5500</v>
       </c>
       <c r="I66" t="n">
         <v>2972355254</v>
@@ -15534,7 +15534,7 @@
         <v>2.75</v>
       </c>
       <c r="M66" t="n">
-        <v>14.32617059894548</v>
+        <v>14.86265618259178</v>
       </c>
       <c r="N66" t="n">
         <v>0.25</v>
@@ -15612,7 +15612,7 @@
         <v>4696321301.320001</v>
       </c>
       <c r="AM66" t="n">
-        <v>21643140734.52915</v>
+        <v>22453631780.17937</v>
       </c>
       <c r="AN66" t="n">
         <v>0.4734</v>
@@ -15653,7 +15653,7 @@
         <v>12.99</v>
       </c>
       <c r="AZ66" t="n">
-        <v>8.220000000000001</v>
+        <v>8.43</v>
       </c>
       <c r="BA66" t="n">
         <v>2.23</v>
@@ -15662,19 +15662,19 @@
         <v>3.47</v>
       </c>
       <c r="BC66" t="n">
-        <v>-22.24</v>
+        <v>-24.2</v>
       </c>
       <c r="BD66" t="n">
-        <v>-36.51</v>
+        <v>-38.11</v>
       </c>
       <c r="BE66" t="n">
         <v>-59.83</v>
       </c>
       <c r="BF66" t="n">
-        <v>-89.09</v>
+        <v>-89.37</v>
       </c>
       <c r="BG66" t="n">
-        <v>-83.06</v>
+        <v>-83.48999999999999</v>
       </c>
       <c r="BH66" t="n">
         <v>7.12</v>
@@ -15683,7 +15683,7 @@
         <v>0</v>
       </c>
       <c r="BJ66" t="n">
-        <v>20.46</v>
+        <v>20.99</v>
       </c>
       <c r="BK66" t="n">
         <v>1.58</v>
@@ -15692,7 +15692,7 @@
         <v>1.57</v>
       </c>
       <c r="BM66" t="n">
-        <v>20.85</v>
+        <v>21.1</v>
       </c>
       <c r="BN66" t="n">
         <v>21.33</v>
@@ -15701,19 +15701,19 @@
         <v>9.48</v>
       </c>
       <c r="BP66" t="n">
-        <v>20.46</v>
+        <v>20.99</v>
       </c>
       <c r="BQ66" t="n">
-        <v>13.03</v>
+        <v>13.37</v>
       </c>
       <c r="BR66" t="n">
-        <v>20.8</v>
+        <v>20.99</v>
       </c>
       <c r="BS66" t="n">
         <v>3.46</v>
       </c>
       <c r="BT66" t="n">
-        <v>4053</v>
+        <v>3790</v>
       </c>
     </row>
     <row r="67">
@@ -15973,13 +15973,13 @@
         </is>
       </c>
       <c r="F68" t="n">
-        <v>17.91</v>
+        <v>18.13</v>
       </c>
       <c r="G68" t="n">
-        <v>7660754035</v>
+        <v>7806661070</v>
       </c>
       <c r="H68" t="n">
-        <v>111100</v>
+        <v>89800</v>
       </c>
       <c r="I68" t="n">
         <v>137989898</v>
@@ -16072,7 +16072,7 @@
         <v>205604948.02</v>
       </c>
       <c r="AM68" t="n">
-        <v>531258948.335645</v>
+        <v>541377328.0166435</v>
       </c>
       <c r="AN68" t="n">
         <v>0.1911</v>
@@ -16113,7 +16113,7 @@
         <v>21.39</v>
       </c>
       <c r="AZ68" t="n">
-        <v>33.13</v>
+        <v>33.54</v>
       </c>
       <c r="BA68" t="n">
         <v>1.24</v>
@@ -16122,19 +16122,19 @@
         <v>63.25</v>
       </c>
       <c r="BC68" t="n">
-        <v>46.3</v>
+        <v>44.53</v>
       </c>
       <c r="BD68" t="n">
-        <v>19.46</v>
+        <v>18.01</v>
       </c>
       <c r="BE68" t="n">
         <v>85</v>
       </c>
       <c r="BF68" t="n">
-        <v>-93.08</v>
+        <v>-93.16</v>
       </c>
       <c r="BG68" t="n">
-        <v>253.15</v>
+        <v>248.86</v>
       </c>
       <c r="BH68" t="n">
         <v>20.48</v>
@@ -16143,7 +16143,7 @@
         <v>0</v>
       </c>
       <c r="BJ68" t="n">
-        <v>17.91</v>
+        <v>18.13</v>
       </c>
       <c r="BK68" t="n">
         <v>1.49</v>
@@ -16152,7 +16152,7 @@
         <v>1.49</v>
       </c>
       <c r="BM68" t="n">
-        <v>18.35</v>
+        <v>18.24</v>
       </c>
       <c r="BN68" t="n">
         <v>22.11</v>
@@ -16161,19 +16161,19 @@
         <v>15.45</v>
       </c>
       <c r="BP68" t="n">
-        <v>17.73</v>
+        <v>17.85</v>
       </c>
       <c r="BQ68" t="n">
-        <v>12.05</v>
+        <v>12.19</v>
       </c>
       <c r="BR68" t="n">
-        <v>18.1</v>
+        <v>18</v>
       </c>
       <c r="BS68" t="n">
         <v>0</v>
       </c>
       <c r="BT68" t="n">
-        <v>43300</v>
+        <v>45500</v>
       </c>
     </row>
     <row r="69">
@@ -16203,13 +16203,13 @@
         </is>
       </c>
       <c r="F69" t="n">
-        <v>20.28</v>
+        <v>20.76</v>
       </c>
       <c r="G69" t="n">
-        <v>7660754035</v>
+        <v>7806661070</v>
       </c>
       <c r="H69" t="n">
-        <v>4260900</v>
+        <v>2900600</v>
       </c>
       <c r="I69" t="n">
         <v>255106712</v>
@@ -16302,7 +16302,7 @@
         <v>380109000.88</v>
       </c>
       <c r="AM69" t="n">
-        <v>455997263.9880952</v>
+        <v>464682206.547619</v>
       </c>
       <c r="AN69" t="n">
         <v>0.8856000000000001</v>
@@ -16343,7 +16343,7 @@
         <v>21.39</v>
       </c>
       <c r="AZ69" t="n">
-        <v>35.46</v>
+        <v>36.3</v>
       </c>
       <c r="BA69" t="n">
         <v>1.24</v>
@@ -16352,19 +16352,19 @@
         <v>69.59</v>
       </c>
       <c r="BC69" t="n">
-        <v>29.21</v>
+        <v>26.22</v>
       </c>
       <c r="BD69" t="n">
-        <v>5.5</v>
+        <v>3.06</v>
       </c>
       <c r="BE69" t="n">
         <v>74.83</v>
       </c>
       <c r="BF69" t="n">
-        <v>-93.89</v>
+        <v>-94.03</v>
       </c>
       <c r="BG69" t="n">
-        <v>243.13</v>
+        <v>235.2</v>
       </c>
       <c r="BH69" t="n">
         <v>20.48</v>
@@ -16373,7 +16373,7 @@
         <v>0</v>
       </c>
       <c r="BJ69" t="n">
-        <v>20.28</v>
+        <v>20.76</v>
       </c>
       <c r="BK69" t="n">
         <v>1.49</v>
@@ -16382,7 +16382,7 @@
         <v>1.49</v>
       </c>
       <c r="BM69" t="n">
-        <v>20.37</v>
+        <v>20.89</v>
       </c>
       <c r="BN69" t="n">
         <v>25.63</v>
@@ -16391,19 +16391,19 @@
         <v>16.99</v>
       </c>
       <c r="BP69" t="n">
-        <v>19.95</v>
+        <v>20.34</v>
       </c>
       <c r="BQ69" t="n">
-        <v>13.64</v>
+        <v>13.96</v>
       </c>
       <c r="BR69" t="n">
-        <v>20.2</v>
+        <v>20.49</v>
       </c>
       <c r="BS69" t="n">
         <v>0</v>
       </c>
       <c r="BT69" t="n">
-        <v>2200057</v>
+        <v>2277277</v>
       </c>
     </row>
     <row r="70">
@@ -16433,13 +16433,13 @@
         </is>
       </c>
       <c r="F70" t="n">
-        <v>18.18</v>
+        <v>18.9</v>
       </c>
       <c r="G70" t="n">
-        <v>8445650037</v>
+        <v>8746452993</v>
       </c>
       <c r="H70" t="n">
-        <v>5236000</v>
+        <v>3277100</v>
       </c>
       <c r="I70" t="n">
         <v>464557268</v>
@@ -16454,7 +16454,7 @@
         <v>0.68</v>
       </c>
       <c r="M70" t="n">
-        <v>0.6665999135546836</v>
+        <v>0.690341747941397</v>
       </c>
       <c r="N70" t="n">
         <v>0.2</v>
@@ -16532,7 +16532,7 @@
         <v>55746872.16</v>
       </c>
       <c r="AM70" t="n">
-        <v>2787343246.534654</v>
+        <v>2886618149.504951</v>
       </c>
       <c r="AN70" t="n">
         <v>0.1236</v>
@@ -16573,7 +16573,7 @@
         <v>6.9</v>
       </c>
       <c r="AZ70" t="n">
-        <v>2.09</v>
+        <v>2.17</v>
       </c>
       <c r="BA70" t="n">
         <v>0.12</v>
@@ -16582,19 +16582,19 @@
         <v>1.07</v>
       </c>
       <c r="BC70" t="n">
-        <v>-53.53</v>
+        <v>-55.3</v>
       </c>
       <c r="BD70" t="n">
-        <v>-62.05</v>
+        <v>-63.5</v>
       </c>
       <c r="BE70" t="n">
         <v>-88.5</v>
       </c>
       <c r="BF70" t="n">
-        <v>-99.34</v>
+        <v>-99.37</v>
       </c>
       <c r="BG70" t="n">
-        <v>-94.12</v>
+        <v>-94.34</v>
       </c>
       <c r="BH70" t="n">
         <v>26.44</v>
@@ -16603,7 +16603,7 @@
         <v>0</v>
       </c>
       <c r="BJ70" t="n">
-        <v>18.18</v>
+        <v>18.9</v>
       </c>
       <c r="BK70" t="n">
         <v>0.12</v>
@@ -16612,7 +16612,7 @@
         <v>0.1</v>
       </c>
       <c r="BM70" t="n">
-        <v>18.5</v>
+        <v>19</v>
       </c>
       <c r="BN70" t="n">
         <v>22.15</v>
@@ -16621,19 +16621,19 @@
         <v>13.21</v>
       </c>
       <c r="BP70" t="n">
-        <v>18.13</v>
+        <v>18.05</v>
       </c>
       <c r="BQ70" t="n">
-        <v>182.33</v>
+        <v>189.55</v>
       </c>
       <c r="BR70" t="n">
-        <v>18.26</v>
+        <v>18.05</v>
       </c>
       <c r="BS70" t="n">
         <v>0.67</v>
       </c>
       <c r="BT70" t="n">
-        <v>3755827</v>
+        <v>3731647</v>
       </c>
     </row>
     <row r="71">

</xml_diff>

<commit_message>
📊 Dados atualizados - 2026-10-04 06:34
</commit_message>
<xml_diff>
--- a/data/ativos.xlsx
+++ b/data/ativos.xlsx
@@ -5298,22 +5298,22 @@
         <v>0</v>
       </c>
       <c r="AQ21" t="n">
-        <v>0.0134</v>
+        <v>0</v>
       </c>
       <c r="AR21" t="n">
-        <v>0.0303</v>
+        <v>0</v>
       </c>
       <c r="AS21" t="n">
-        <v>0.0094</v>
+        <v>0</v>
       </c>
       <c r="AT21" t="n">
         <v>0</v>
       </c>
       <c r="AU21" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AV21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AW21" t="inlineStr">
         <is>
@@ -5333,7 +5333,7 @@
         <v>-0.15</v>
       </c>
       <c r="BB21" t="n">
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="BC21" t="n">
         <v>-100</v>
@@ -5348,7 +5348,7 @@
         <v>-207.14</v>
       </c>
       <c r="BG21" t="n">
-        <v>5.36</v>
+        <v>-100</v>
       </c>
       <c r="BH21" t="n">
         <v>0.65</v>

</xml_diff>

<commit_message>
📊 Dados atualizados - 2026-10-05 06:28
</commit_message>
<xml_diff>
--- a/data/ativos.xlsx
+++ b/data/ativos.xlsx
@@ -1740,7 +1740,7 @@
         <v>7.17</v>
       </c>
       <c r="G6" t="n">
-        <v>452317303</v>
+        <v>452317300</v>
       </c>
       <c r="H6" t="n">
         <v>100</v>
@@ -1758,7 +1758,7 @@
         <v>1.91</v>
       </c>
       <c r="M6" t="n">
-        <v>7.041694799114273</v>
+        <v>7.041694752410147</v>
       </c>
       <c r="N6" t="n">
         <v>1.26</v>
@@ -1836,7 +1836,7 @@
         <v>35958279</v>
       </c>
       <c r="AM6" t="n">
-        <v>43242571.98852772</v>
+        <v>43242571.70172084</v>
       </c>
       <c r="AN6" t="n">
         <v>0.5199</v>
@@ -5298,22 +5298,22 @@
         <v>0</v>
       </c>
       <c r="AQ21" t="n">
-        <v>0</v>
+        <v>0.0134</v>
       </c>
       <c r="AR21" t="n">
-        <v>0</v>
+        <v>0.0303</v>
       </c>
       <c r="AS21" t="n">
-        <v>0</v>
+        <v>0.0094</v>
       </c>
       <c r="AT21" t="n">
         <v>0</v>
       </c>
       <c r="AU21" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AV21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AW21" t="inlineStr">
         <is>
@@ -5333,7 +5333,7 @@
         <v>-0.15</v>
       </c>
       <c r="BB21" t="n">
-        <v>0</v>
+        <v>0.15</v>
       </c>
       <c r="BC21" t="n">
         <v>-100</v>
@@ -5348,7 +5348,7 @@
         <v>-207.14</v>
       </c>
       <c r="BG21" t="n">
-        <v>-100</v>
+        <v>5.36</v>
       </c>
       <c r="BH21" t="n">
         <v>0.65</v>
@@ -8858,7 +8858,7 @@
         <v>14.5</v>
       </c>
       <c r="G37" t="n">
-        <v>178849960</v>
+        <v>178850000</v>
       </c>
       <c r="H37" t="n">
         <v>1400</v>
@@ -8876,7 +8876,7 @@
         <v>0.88</v>
       </c>
       <c r="M37" t="n">
-        <v>1.741255021821716</v>
+        <v>1.741255411255411</v>
       </c>
       <c r="N37" t="n">
         <v>0.5</v>
@@ -8954,7 +8954,7 @@
         <v>11319000</v>
       </c>
       <c r="AM37" t="n">
-        <v>42787071.77033493</v>
+        <v>42787081.33971293</v>
       </c>
       <c r="AN37" t="n">
         <v>0</v>
@@ -11618,7 +11618,7 @@
         <v>48.07</v>
       </c>
       <c r="G49" t="n">
-        <v>943199249</v>
+        <v>948313300</v>
       </c>
       <c r="H49" t="n">
         <v>200</v>
@@ -11636,7 +11636,7 @@
         <v>1.09</v>
       </c>
       <c r="M49" t="n">
-        <v>0.9542225143343136</v>
+        <v>0.9593963337672996</v>
       </c>
       <c r="N49" t="n">
         <v>0.08</v>
@@ -11714,7 +11714,7 @@
         <v>84709985.8</v>
       </c>
       <c r="AM49" t="n">
-        <v>235799812.25</v>
+        <v>237078325</v>
       </c>
       <c r="AN49" t="n">
         <v>3.3186</v>
@@ -11848,7 +11848,7 @@
         <v>34.1</v>
       </c>
       <c r="G50" t="n">
-        <v>943199249</v>
+        <v>948313300</v>
       </c>
       <c r="H50" t="n">
         <v>400</v>
@@ -11866,7 +11866,7 @@
         <v>0.8</v>
       </c>
       <c r="M50" t="n">
-        <v>0.9542225143343136</v>
+        <v>0.9593963337672996</v>
       </c>
       <c r="N50" t="n">
         <v>0.06</v>
@@ -11944,7 +11944,7 @@
         <v>84709985.8</v>
       </c>
       <c r="AM50" t="n">
-        <v>321911006.4846416</v>
+        <v>323656416.3822525</v>
       </c>
       <c r="AN50" t="n">
         <v>4.4983</v>
@@ -14136,7 +14136,7 @@
         <v>377</v>
       </c>
       <c r="G60" t="n">
-        <v>171440750</v>
+        <v>171440800</v>
       </c>
       <c r="H60" t="n">
         <v>28</v>
@@ -14154,7 +14154,7 @@
         <v>0.83</v>
       </c>
       <c r="M60" t="n">
-        <v>12.82352676185386</v>
+        <v>12.82353050178348</v>
       </c>
       <c r="N60" t="n">
         <v>0.68</v>
@@ -14232,7 +14232,7 @@
         <v>59558607.5</v>
       </c>
       <c r="AM60" t="n">
-        <v>-25137939.88269795</v>
+        <v>-25137947.21407625</v>
       </c>
       <c r="AN60" t="n">
         <v>10.0581</v>
@@ -14596,7 +14596,7 @@
         <v>112</v>
       </c>
       <c r="G62" t="n">
-        <v>11054368640</v>
+        <v>11054370000</v>
       </c>
       <c r="H62" t="n">
         <v>100</v>
@@ -14614,7 +14614,7 @@
         <v>0.64</v>
       </c>
       <c r="M62" t="n">
-        <v>1.036220167978228</v>
+        <v>1.036220295462617</v>
       </c>
       <c r="N62" t="n">
         <v>0.13</v>
@@ -14692,7 +14692,7 @@
         <v>2757670987.06</v>
       </c>
       <c r="AM62" t="n">
-        <v>4475452890.688259</v>
+        <v>4475453441.295547</v>
       </c>
       <c r="AN62" t="n">
         <v>6.9319</v>
@@ -14826,7 +14826,7 @@
         <v>1.6</v>
       </c>
       <c r="G63" t="n">
-        <v>409000166</v>
+        <v>416815600</v>
       </c>
       <c r="H63" t="n">
         <v>85800</v>
@@ -14844,7 +14844,7 @@
         <v>-0.22</v>
       </c>
       <c r="M63" t="n">
-        <v>0.5030490972690173</v>
+        <v>0.5126616777648051</v>
       </c>
       <c r="N63" t="n">
         <v>0.37</v>
@@ -14922,7 +14922,7 @@
         <v>31952560.12</v>
       </c>
       <c r="AM63" t="n">
-        <v>232386457.9545455</v>
+        <v>236827045.4545455</v>
       </c>
       <c r="AN63" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
📊 Dados atualizados - 2026-10-06 07:03
</commit_message>
<xml_diff>
--- a/data/ativos.xlsx
+++ b/data/ativos.xlsx
@@ -1047,13 +1047,13 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>26.15</v>
+        <v>28.24</v>
       </c>
       <c r="G3" t="n">
-        <v>3485753109</v>
+        <v>3777574401</v>
       </c>
       <c r="H3" t="n">
-        <v>1023600</v>
+        <v>2163000</v>
       </c>
       <c r="I3" t="n">
         <v>129510368</v>
@@ -1068,7 +1068,7 @@
         <v>0.88</v>
       </c>
       <c r="M3" t="n">
-        <v>0.86733300620198</v>
+        <v>0.9399446429270828</v>
       </c>
       <c r="N3" t="n">
         <v>0.09</v>
@@ -1146,7 +1146,7 @@
         <v>506385538.88</v>
       </c>
       <c r="AM3" t="n">
-        <v>680811154.1015625</v>
+        <v>737807500.1953125</v>
       </c>
       <c r="AN3" t="n">
         <v>2.7</v>
@@ -1187,7 +1187,7 @@
         <v>40.42</v>
       </c>
       <c r="AZ3" t="n">
-        <v>47.85</v>
+        <v>51.68</v>
       </c>
       <c r="BA3" t="n">
         <v>4.87</v>
@@ -1196,19 +1196,19 @@
         <v>21.14</v>
       </c>
       <c r="BC3" t="n">
-        <v>89.29000000000001</v>
+        <v>75.28</v>
       </c>
       <c r="BD3" t="n">
-        <v>54.55</v>
+        <v>43.11</v>
       </c>
       <c r="BE3" t="n">
         <v>83</v>
       </c>
       <c r="BF3" t="n">
-        <v>-81.38</v>
+        <v>-82.76000000000001</v>
       </c>
       <c r="BG3" t="n">
-        <v>-19.17</v>
+        <v>-25.16</v>
       </c>
       <c r="BH3" t="n">
         <v>27.85</v>
@@ -1217,7 +1217,7 @@
         <v>0</v>
       </c>
       <c r="BJ3" t="n">
-        <v>26.15</v>
+        <v>28.24</v>
       </c>
       <c r="BK3" t="n">
         <v>3.91</v>
@@ -1226,28 +1226,28 @@
         <v>4.39</v>
       </c>
       <c r="BM3" t="n">
-        <v>26.25</v>
+        <v>28.72</v>
       </c>
       <c r="BN3" t="n">
-        <v>27.17</v>
+        <v>28.72</v>
       </c>
       <c r="BO3" t="n">
         <v>18.72</v>
       </c>
       <c r="BP3" t="n">
-        <v>25.59</v>
+        <v>26.48</v>
       </c>
       <c r="BQ3" t="n">
-        <v>5.95</v>
+        <v>6.43</v>
       </c>
       <c r="BR3" t="n">
-        <v>25.82</v>
+        <v>26.5</v>
       </c>
       <c r="BS3" t="n">
         <v>0.79</v>
       </c>
       <c r="BT3" t="n">
-        <v>560080</v>
+        <v>579787</v>
       </c>
     </row>
     <row r="4">
@@ -1277,13 +1277,13 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>15.84</v>
+        <v>16.5</v>
       </c>
       <c r="G4" t="n">
-        <v>246074877570</v>
+        <v>255496890000</v>
       </c>
       <c r="H4" t="n">
-        <v>36916800</v>
+        <v>72356100</v>
       </c>
       <c r="I4" t="n">
         <v>15484664889</v>
@@ -1298,7 +1298,7 @@
         <v>2.76</v>
       </c>
       <c r="M4" t="n">
-        <v>2.786313352159752</v>
+        <v>2.892999086588112</v>
       </c>
       <c r="N4" t="n">
         <v>1.76</v>
@@ -1376,7 +1376,7 @@
         <v>16258898133.45</v>
       </c>
       <c r="AM4" t="n">
-        <v>24363849264.35644</v>
+        <v>25296721782.17822</v>
       </c>
       <c r="AN4" t="n">
         <v>0.269</v>
@@ -1417,7 +1417,7 @@
         <v>9.470000000000001</v>
       </c>
       <c r="AZ4" t="n">
-        <v>19.77</v>
+        <v>20.6</v>
       </c>
       <c r="BA4" t="n">
         <v>1.13</v>
@@ -1426,19 +1426,19 @@
         <v>11.39</v>
       </c>
       <c r="BC4" t="n">
-        <v>-26.74</v>
+        <v>-29.67</v>
       </c>
       <c r="BD4" t="n">
-        <v>-40.18</v>
+        <v>-42.58</v>
       </c>
       <c r="BE4" t="n">
         <v>24.83</v>
       </c>
       <c r="BF4" t="n">
-        <v>-92.88</v>
+        <v>-93.17</v>
       </c>
       <c r="BG4" t="n">
-        <v>-28.11</v>
+        <v>-30.99</v>
       </c>
       <c r="BH4" t="n">
         <v>5.7</v>
@@ -1447,7 +1447,7 @@
         <v>0</v>
       </c>
       <c r="BJ4" t="n">
-        <v>15.84</v>
+        <v>16.5</v>
       </c>
       <c r="BK4" t="n">
         <v>1.05</v>
@@ -1456,7 +1456,7 @@
         <v>1.04</v>
       </c>
       <c r="BM4" t="n">
-        <v>15.84</v>
+        <v>16.86</v>
       </c>
       <c r="BN4" t="n">
         <v>16.94</v>
@@ -1465,19 +1465,19 @@
         <v>11.04</v>
       </c>
       <c r="BP4" t="n">
-        <v>15.39</v>
+        <v>16.23</v>
       </c>
       <c r="BQ4" t="n">
-        <v>15.28</v>
+        <v>15.91</v>
       </c>
       <c r="BR4" t="n">
-        <v>15.62</v>
+        <v>16.45</v>
       </c>
       <c r="BS4" t="n">
         <v>2.76</v>
       </c>
       <c r="BT4" t="n">
-        <v>26083937</v>
+        <v>25944680</v>
       </c>
     </row>
     <row r="5">
@@ -1737,13 +1737,13 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>7.17</v>
+        <v>7.19</v>
       </c>
       <c r="G6" t="n">
-        <v>452317300</v>
+        <v>453578996</v>
       </c>
       <c r="H6" t="n">
-        <v>100</v>
+        <v>800</v>
       </c>
       <c r="I6" t="n">
         <v>63084700</v>
@@ -1758,7 +1758,7 @@
         <v>1.91</v>
       </c>
       <c r="M6" t="n">
-        <v>7.041694752410147</v>
+        <v>7.061336888809389</v>
       </c>
       <c r="N6" t="n">
         <v>1.26</v>
@@ -1836,7 +1836,7 @@
         <v>35958279</v>
       </c>
       <c r="AM6" t="n">
-        <v>43242571.70172084</v>
+        <v>43363192.73422562</v>
       </c>
       <c r="AN6" t="n">
         <v>0.5199</v>
@@ -1877,7 +1877,7 @@
         <v>5.74</v>
       </c>
       <c r="AZ6" t="n">
-        <v>8.41</v>
+        <v>8.44</v>
       </c>
       <c r="BA6" t="n">
         <v>0.65</v>
@@ -1886,19 +1886,19 @@
         <v>7.95</v>
       </c>
       <c r="BC6" t="n">
-        <v>-1.87</v>
+        <v>-2.14</v>
       </c>
       <c r="BD6" t="n">
-        <v>-19.88</v>
+        <v>-20.1</v>
       </c>
       <c r="BE6" t="n">
         <v>17.33</v>
       </c>
       <c r="BF6" t="n">
-        <v>-90.95999999999999</v>
+        <v>-90.98</v>
       </c>
       <c r="BG6" t="n">
-        <v>10.93</v>
+        <v>10.62</v>
       </c>
       <c r="BH6" t="n">
         <v>3.86</v>
@@ -1907,7 +1907,7 @@
         <v>0</v>
       </c>
       <c r="BJ6" t="n">
-        <v>7.17</v>
+        <v>7.19</v>
       </c>
       <c r="BK6" t="n">
         <v>0.57</v>
@@ -1916,7 +1916,7 @@
         <v>0.5600000000000001</v>
       </c>
       <c r="BM6" t="n">
-        <v>7.17</v>
+        <v>7.31</v>
       </c>
       <c r="BN6" t="n">
         <v>8.16</v>
@@ -1928,16 +1928,16 @@
         <v>7.17</v>
       </c>
       <c r="BQ6" t="n">
-        <v>12.75</v>
+        <v>12.79</v>
       </c>
       <c r="BR6" t="n">
-        <v>7.17</v>
+        <v>7.18</v>
       </c>
       <c r="BS6" t="n">
         <v>7.32</v>
       </c>
       <c r="BT6" t="n">
-        <v>220</v>
+        <v>213</v>
       </c>
     </row>
     <row r="7">
@@ -3117,13 +3117,13 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>5.28</v>
+        <v>5.49</v>
       </c>
       <c r="G12" t="n">
-        <v>505722644</v>
+        <v>526828777</v>
       </c>
       <c r="H12" t="n">
-        <v>1796300</v>
+        <v>4403400</v>
       </c>
       <c r="I12" t="n">
         <v>95961536</v>
@@ -3138,7 +3138,7 @@
         <v>0.32</v>
       </c>
       <c r="M12" t="n">
-        <v>0.09145916846732639</v>
+        <v>0.09527618041378137</v>
       </c>
       <c r="N12" t="n">
         <v>0.14</v>
@@ -3216,7 +3216,7 @@
         <v>362734606.08</v>
       </c>
       <c r="AM12" t="n">
-        <v>543787789.2473118</v>
+        <v>566482555.9139785</v>
       </c>
       <c r="AN12" t="n">
         <v>0.4208</v>
@@ -3257,7 +3257,7 @@
         <v>30.49</v>
       </c>
       <c r="AZ12" t="n">
-        <v>7.14</v>
+        <v>7.42</v>
       </c>
       <c r="BA12" t="n">
         <v>4.41</v>
@@ -3266,28 +3266,28 @@
         <v>18.12</v>
       </c>
       <c r="BC12" t="n">
-        <v>607.34</v>
+        <v>580.28</v>
       </c>
       <c r="BD12" t="n">
-        <v>477.54</v>
+        <v>455.45</v>
       </c>
       <c r="BE12" t="n">
         <v>35.17</v>
       </c>
       <c r="BF12" t="n">
-        <v>-16.45</v>
+        <v>-19.64</v>
       </c>
       <c r="BG12" t="n">
-        <v>243.16</v>
+        <v>230.03</v>
       </c>
       <c r="BH12" t="n">
         <v>16.4</v>
       </c>
       <c r="BI12" t="n">
-        <v>0</v>
+        <v>10.37</v>
       </c>
       <c r="BJ12" t="n">
-        <v>5.28</v>
+        <v>4.97</v>
       </c>
       <c r="BK12" t="n">
         <v>3.78</v>
@@ -3296,7 +3296,7 @@
         <v>3.63</v>
       </c>
       <c r="BM12" t="n">
-        <v>5.38</v>
+        <v>5.66</v>
       </c>
       <c r="BN12" t="n">
         <v>8.23</v>
@@ -3305,19 +3305,19 @@
         <v>4.42</v>
       </c>
       <c r="BP12" t="n">
-        <v>5.26</v>
+        <v>5.41</v>
       </c>
       <c r="BQ12" t="n">
-        <v>1.45</v>
+        <v>1.51</v>
       </c>
       <c r="BR12" t="n">
-        <v>5.37</v>
+        <v>5.51</v>
       </c>
       <c r="BS12" t="n">
         <v>0.09</v>
       </c>
       <c r="BT12" t="n">
-        <v>568933</v>
+        <v>614803</v>
       </c>
     </row>
     <row r="13">
@@ -3347,13 +3347,13 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>30.51</v>
+        <v>33.06</v>
       </c>
       <c r="G13" t="n">
-        <v>15424373329</v>
+        <v>16668555152</v>
       </c>
       <c r="H13" t="n">
-        <v>10273900</v>
+        <v>22405900</v>
       </c>
       <c r="I13" t="n">
         <v>504190947</v>
@@ -3368,7 +3368,7 @@
         <v>1.13</v>
       </c>
       <c r="M13" t="n">
-        <v>5.33464002996811</v>
+        <v>5.764950034527939</v>
       </c>
       <c r="N13" t="n">
         <v>0.57</v>
@@ -3446,7 +3446,7 @@
         <v>932753251.95</v>
       </c>
       <c r="AM13" t="n">
-        <v>1605033645.057232</v>
+        <v>1734501056.399584</v>
       </c>
       <c r="AN13" t="n">
         <v>2.6301</v>
@@ -3487,7 +3487,7 @@
         <v>26.6</v>
       </c>
       <c r="AZ13" t="n">
-        <v>55.22</v>
+        <v>59.84</v>
       </c>
       <c r="BA13" t="n">
         <v>2.6</v>
@@ -3496,19 +3496,19 @@
         <v>8.69</v>
       </c>
       <c r="BC13" t="n">
-        <v>6.76</v>
+        <v>-1.47</v>
       </c>
       <c r="BD13" t="n">
-        <v>-12.83</v>
+        <v>-19.55</v>
       </c>
       <c r="BE13" t="n">
         <v>81</v>
       </c>
       <c r="BF13" t="n">
-        <v>-91.45999999999999</v>
+        <v>-92.12</v>
       </c>
       <c r="BG13" t="n">
-        <v>-71.5</v>
+        <v>-73.7</v>
       </c>
       <c r="BH13" t="n">
         <v>25.49</v>
@@ -3517,7 +3517,7 @@
         <v>0</v>
       </c>
       <c r="BJ13" t="n">
-        <v>30.51</v>
+        <v>33.06</v>
       </c>
       <c r="BK13" t="n">
         <v>1.85</v>
@@ -3526,28 +3526,28 @@
         <v>1.96</v>
       </c>
       <c r="BM13" t="n">
-        <v>30.59</v>
+        <v>33.93</v>
       </c>
       <c r="BN13" t="n">
-        <v>32.11</v>
+        <v>33.93</v>
       </c>
       <c r="BO13" t="n">
         <v>20.85</v>
       </c>
       <c r="BP13" t="n">
-        <v>29.7</v>
+        <v>31.8</v>
       </c>
       <c r="BQ13" t="n">
-        <v>15.59</v>
+        <v>16.89</v>
       </c>
       <c r="BR13" t="n">
-        <v>30.06</v>
+        <v>32.41</v>
       </c>
       <c r="BS13" t="n">
         <v>5.01</v>
       </c>
       <c r="BT13" t="n">
-        <v>5078920</v>
+        <v>5305243</v>
       </c>
     </row>
     <row r="14">
@@ -3577,13 +3577,13 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>11.38</v>
+        <v>11.8</v>
       </c>
       <c r="G14" t="n">
-        <v>8976365139</v>
+        <v>9482112153</v>
       </c>
       <c r="H14" t="n">
-        <v>11700</v>
+        <v>90600</v>
       </c>
       <c r="I14" t="n">
         <v>339510689</v>
@@ -3598,7 +3598,7 @@
         <v>1.92</v>
       </c>
       <c r="M14" t="n">
-        <v>3.727146384692117</v>
+        <v>3.937141535915313</v>
       </c>
       <c r="N14" t="n">
         <v>1.11</v>
@@ -3676,7 +3676,7 @@
         <v>349696009.67</v>
       </c>
       <c r="AM14" t="n">
-        <v>996266941.0654829</v>
+        <v>1052398685.127636</v>
       </c>
       <c r="AN14" t="n">
         <v>0.1489</v>
@@ -3717,7 +3717,7 @@
         <v>9.050000000000001</v>
       </c>
       <c r="AZ14" t="n">
-        <v>9.140000000000001</v>
+        <v>9.48</v>
       </c>
       <c r="BA14" t="n">
         <v>1.42</v>
@@ -3726,19 +3726,19 @@
         <v>5.94</v>
       </c>
       <c r="BC14" t="n">
-        <v>-2.61</v>
+        <v>-6.08</v>
       </c>
       <c r="BD14" t="n">
-        <v>-20.48</v>
+        <v>-23.31</v>
       </c>
       <c r="BE14" t="n">
         <v>-19.67</v>
       </c>
       <c r="BF14" t="n">
-        <v>-87.51000000000001</v>
+        <v>-87.95999999999999</v>
       </c>
       <c r="BG14" t="n">
-        <v>-47.78</v>
+        <v>-49.64</v>
       </c>
       <c r="BH14" t="n">
         <v>5.3</v>
@@ -3747,7 +3747,7 @@
         <v>0</v>
       </c>
       <c r="BJ14" t="n">
-        <v>11.38</v>
+        <v>11.8</v>
       </c>
       <c r="BK14" t="n">
         <v>1.03</v>
@@ -3756,7 +3756,7 @@
         <v>1.01</v>
       </c>
       <c r="BM14" t="n">
-        <v>11.38</v>
+        <v>12</v>
       </c>
       <c r="BN14" t="n">
         <v>13.49</v>
@@ -3765,19 +3765,19 @@
         <v>7.81</v>
       </c>
       <c r="BP14" t="n">
-        <v>10.65</v>
+        <v>11.41</v>
       </c>
       <c r="BQ14" t="n">
-        <v>11.23</v>
+        <v>11.65</v>
       </c>
       <c r="BR14" t="n">
-        <v>10.65</v>
+        <v>11.51</v>
       </c>
       <c r="BS14" t="n">
         <v>1.44</v>
       </c>
       <c r="BT14" t="n">
-        <v>9777</v>
+        <v>9933</v>
       </c>
     </row>
     <row r="15">
@@ -3807,13 +3807,13 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>15.17</v>
+        <v>15.85</v>
       </c>
       <c r="G15" t="n">
-        <v>8976365139</v>
+        <v>9482112153</v>
       </c>
       <c r="H15" t="n">
-        <v>1983600</v>
+        <v>4216400</v>
       </c>
       <c r="I15" t="n">
         <v>343551533</v>
@@ -3828,7 +3828,7 @@
         <v>2.56</v>
       </c>
       <c r="M15" t="n">
-        <v>3.683307787977996</v>
+        <v>3.890832981813899</v>
       </c>
       <c r="N15" t="n">
         <v>1.47</v>
@@ -3906,7 +3906,7 @@
         <v>353858078.99</v>
       </c>
       <c r="AM15" t="n">
-        <v>748654306.8390325</v>
+        <v>790835041.9516263</v>
       </c>
       <c r="AN15" t="n">
         <v>0.1638</v>
@@ -3947,7 +3947,7 @@
         <v>9.050000000000001</v>
       </c>
       <c r="AZ15" t="n">
-        <v>10.09</v>
+        <v>10.54</v>
       </c>
       <c r="BA15" t="n">
         <v>1.42</v>
@@ -3956,19 +3956,19 @@
         <v>6.19</v>
       </c>
       <c r="BC15" t="n">
-        <v>-26.94</v>
+        <v>-30.08</v>
       </c>
       <c r="BD15" t="n">
-        <v>-40.35</v>
+        <v>-42.91</v>
       </c>
       <c r="BE15" t="n">
         <v>-33.5</v>
       </c>
       <c r="BF15" t="n">
-        <v>-90.63</v>
+        <v>-91.03</v>
       </c>
       <c r="BG15" t="n">
-        <v>-59.21</v>
+        <v>-60.96</v>
       </c>
       <c r="BH15" t="n">
         <v>5.3</v>
@@ -3977,7 +3977,7 @@
         <v>0</v>
       </c>
       <c r="BJ15" t="n">
-        <v>15.17</v>
+        <v>15.85</v>
       </c>
       <c r="BK15" t="n">
         <v>1.03</v>
@@ -3986,28 +3986,28 @@
         <v>1.01</v>
       </c>
       <c r="BM15" t="n">
-        <v>15.29</v>
+        <v>16.75</v>
       </c>
       <c r="BN15" t="n">
-        <v>16.22</v>
+        <v>16.75</v>
       </c>
       <c r="BO15" t="n">
         <v>7.84</v>
       </c>
       <c r="BP15" t="n">
-        <v>14.66</v>
+        <v>15.57</v>
       </c>
       <c r="BQ15" t="n">
-        <v>14.98</v>
+        <v>15.65</v>
       </c>
       <c r="BR15" t="n">
-        <v>14.71</v>
+        <v>15.89</v>
       </c>
       <c r="BS15" t="n">
         <v>1.92</v>
       </c>
       <c r="BT15" t="n">
-        <v>2376813</v>
+        <v>2405447</v>
       </c>
     </row>
     <row r="16">
@@ -4037,13 +4037,13 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>4.6</v>
+        <v>4.89</v>
       </c>
       <c r="G16" t="n">
-        <v>1015591658</v>
+        <v>1072404354</v>
       </c>
       <c r="H16" t="n">
-        <v>128200</v>
+        <v>297800</v>
       </c>
       <c r="I16" t="n">
         <v>219305733</v>
@@ -4058,7 +4058,7 @@
         <v>2.69</v>
       </c>
       <c r="M16" t="n">
-        <v>0.4804600093035415</v>
+        <v>0.5073371781279424</v>
       </c>
       <c r="N16" t="n">
         <v>0.39</v>
@@ -4136,7 +4136,7 @@
         <v>17544458.64</v>
       </c>
       <c r="AM16" t="n">
-        <v>285278555.6179775</v>
+        <v>301237178.0898876</v>
       </c>
       <c r="AN16" t="n">
         <v>0.0077</v>
@@ -4177,7 +4177,7 @@
         <v>1.42</v>
       </c>
       <c r="AZ16" t="n">
-        <v>0.13</v>
+        <v>0.14</v>
       </c>
       <c r="BA16" t="n">
         <v>0.08</v>
@@ -4186,16 +4186,16 @@
         <v>0</v>
       </c>
       <c r="BC16" t="n">
-        <v>-62.2</v>
+        <v>-64.44</v>
       </c>
       <c r="BD16" t="n">
-        <v>-69.13</v>
+        <v>-70.95999999999999</v>
       </c>
       <c r="BE16" t="n">
         <v>-97.17</v>
       </c>
       <c r="BF16" t="n">
-        <v>-98.26000000000001</v>
+        <v>-98.36</v>
       </c>
       <c r="BG16" t="n">
         <v>-100</v>
@@ -4207,7 +4207,7 @@
         <v>0</v>
       </c>
       <c r="BJ16" t="n">
-        <v>4.6</v>
+        <v>4.89</v>
       </c>
       <c r="BK16" t="n">
         <v>0.08</v>
@@ -4216,7 +4216,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="BM16" t="n">
-        <v>4.64</v>
+        <v>5.09</v>
       </c>
       <c r="BN16" t="n">
         <v>5.54</v>
@@ -4225,19 +4225,19 @@
         <v>3.22</v>
       </c>
       <c r="BP16" t="n">
-        <v>4.44</v>
+        <v>4.71</v>
       </c>
       <c r="BQ16" t="n">
-        <v>62.77</v>
+        <v>66.73</v>
       </c>
       <c r="BR16" t="n">
-        <v>4.46</v>
+        <v>4.71</v>
       </c>
       <c r="BS16" t="n">
         <v>0.49</v>
       </c>
       <c r="BT16" t="n">
-        <v>129907</v>
+        <v>131397</v>
       </c>
     </row>
     <row r="17">
@@ -4267,13 +4267,13 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>33.51</v>
+        <v>36.19</v>
       </c>
       <c r="G17" t="n">
-        <v>11015436807</v>
+        <v>11929197058</v>
       </c>
       <c r="H17" t="n">
-        <v>794100</v>
+        <v>3317100</v>
       </c>
       <c r="I17" t="n">
         <v>0</v>
@@ -4360,13 +4360,13 @@
         <v>8.039999999999999</v>
       </c>
       <c r="AK17" t="n">
-        <v>4974456650.559971</v>
+        <v>5387101272.57948</v>
       </c>
       <c r="AL17" t="n">
-        <v>1376929600.875</v>
+        <v>1491149632.25</v>
       </c>
       <c r="AM17" t="n">
-        <v>3410351952.631579</v>
+        <v>3693249863.157895</v>
       </c>
       <c r="AN17" t="n">
         <v>1.08</v>
@@ -4407,7 +4407,7 @@
         <v>42.98</v>
       </c>
       <c r="AZ17" t="n">
-        <v>17.93</v>
+        <v>19.36</v>
       </c>
       <c r="BA17" t="n">
         <v>4.55</v>
@@ -4416,19 +4416,19 @@
         <v>16.33</v>
       </c>
       <c r="BC17" t="n">
-        <v>57.08</v>
+        <v>45.45</v>
       </c>
       <c r="BD17" t="n">
-        <v>28.26</v>
+        <v>18.76</v>
       </c>
       <c r="BE17" t="n">
         <v>-46.5</v>
       </c>
       <c r="BF17" t="n">
-        <v>-86.43000000000001</v>
+        <v>-87.43000000000001</v>
       </c>
       <c r="BG17" t="n">
-        <v>-51.26</v>
+        <v>-54.87</v>
       </c>
       <c r="BH17" t="n">
         <v>29.25</v>
@@ -4437,7 +4437,7 @@
         <v>0</v>
       </c>
       <c r="BJ17" t="n">
-        <v>33.51</v>
+        <v>36.19</v>
       </c>
       <c r="BK17" t="n">
         <v>4.21</v>
@@ -4446,28 +4446,28 @@
         <v>12.62</v>
       </c>
       <c r="BM17" t="n">
-        <v>33.54</v>
+        <v>37.06</v>
       </c>
       <c r="BN17" t="n">
-        <v>36.63</v>
+        <v>37.06</v>
       </c>
       <c r="BO17" t="n">
         <v>29.53</v>
       </c>
       <c r="BP17" t="n">
-        <v>32.46</v>
+        <v>34.27</v>
       </c>
       <c r="BQ17" t="n">
-        <v>2.65</v>
+        <v>2.87</v>
       </c>
       <c r="BR17" t="n">
-        <v>32.99</v>
+        <v>34.27</v>
       </c>
       <c r="BS17" t="n">
         <v>2.21</v>
       </c>
       <c r="BT17" t="n">
-        <v>1070423</v>
+        <v>1062917</v>
       </c>
     </row>
     <row r="18">
@@ -4497,13 +4497,13 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>11.75</v>
+        <v>12.98</v>
       </c>
       <c r="G18" t="n">
-        <v>11015436807</v>
+        <v>11929197058</v>
       </c>
       <c r="H18" t="n">
-        <v>5000</v>
+        <v>28300</v>
       </c>
       <c r="I18" t="n">
         <v>671494278</v>
@@ -4518,7 +4518,7 @@
         <v>1.2</v>
       </c>
       <c r="M18" t="n">
-        <v>3.24337718351616</v>
+        <v>3.512424085715632</v>
       </c>
       <c r="N18" t="n">
         <v>0.33</v>
@@ -4596,7 +4596,7 @@
         <v>940091989.1999999</v>
       </c>
       <c r="AM18" t="n">
-        <v>3278403811.607143</v>
+        <v>3550356267.261905</v>
       </c>
       <c r="AN18" t="n">
         <v>0.36</v>
@@ -4637,7 +4637,7 @@
         <v>14.31</v>
       </c>
       <c r="AZ18" t="n">
-        <v>6.05</v>
+        <v>6.68</v>
       </c>
       <c r="BA18" t="n">
         <v>1.51</v>
@@ -4646,19 +4646,19 @@
         <v>5.44</v>
       </c>
       <c r="BC18" t="n">
-        <v>49.15</v>
+        <v>35.02</v>
       </c>
       <c r="BD18" t="n">
-        <v>21.78</v>
+        <v>10.24</v>
       </c>
       <c r="BE18" t="n">
         <v>-48.5</v>
       </c>
       <c r="BF18" t="n">
-        <v>-87.13</v>
+        <v>-88.34999999999999</v>
       </c>
       <c r="BG18" t="n">
-        <v>-53.66</v>
+        <v>-58.06</v>
       </c>
       <c r="BH18" t="n">
         <v>9.75</v>
@@ -4667,7 +4667,7 @@
         <v>0</v>
       </c>
       <c r="BJ18" t="n">
-        <v>11.75</v>
+        <v>12.98</v>
       </c>
       <c r="BK18" t="n">
         <v>1.4</v>
@@ -4676,28 +4676,28 @@
         <v>12.62</v>
       </c>
       <c r="BM18" t="n">
-        <v>11.75</v>
+        <v>13.86</v>
       </c>
       <c r="BN18" t="n">
-        <v>13.82</v>
+        <v>13.86</v>
       </c>
       <c r="BO18" t="n">
         <v>10.19</v>
       </c>
       <c r="BP18" t="n">
-        <v>11.58</v>
+        <v>11.75</v>
       </c>
       <c r="BQ18" t="n">
-        <v>0.93</v>
+        <v>1.03</v>
       </c>
       <c r="BR18" t="n">
-        <v>11.58</v>
+        <v>11.9</v>
       </c>
       <c r="BS18" t="n">
         <v>2.3</v>
       </c>
       <c r="BT18" t="n">
-        <v>8530</v>
+        <v>8493</v>
       </c>
     </row>
     <row r="19">
@@ -4727,13 +4727,13 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>10.85</v>
+        <v>11.59</v>
       </c>
       <c r="G19" t="n">
-        <v>11015436807</v>
+        <v>11929197058</v>
       </c>
       <c r="H19" t="n">
-        <v>11500</v>
+        <v>62000</v>
       </c>
       <c r="I19" t="n">
         <v>317386323</v>
@@ -4748,7 +4748,7 @@
         <v>1.12</v>
       </c>
       <c r="M19" t="n">
-        <v>6.862013458994757</v>
+        <v>7.431236019163399</v>
       </c>
       <c r="N19" t="n">
         <v>0.3</v>
@@ -4826,7 +4826,7 @@
         <v>444340852.2</v>
       </c>
       <c r="AM19" t="n">
-        <v>3496964065.714286</v>
+        <v>3787046685.079365</v>
       </c>
       <c r="AN19" t="n">
         <v>0.36</v>
@@ -4867,7 +4867,7 @@
         <v>14.31</v>
       </c>
       <c r="AZ19" t="n">
-        <v>5.97</v>
+        <v>6.37</v>
       </c>
       <c r="BA19" t="n">
         <v>1.51</v>
@@ -4876,19 +4876,19 @@
         <v>5.25</v>
       </c>
       <c r="BC19" t="n">
-        <v>61.52</v>
+        <v>51.21</v>
       </c>
       <c r="BD19" t="n">
-        <v>31.88</v>
+        <v>23.46</v>
       </c>
       <c r="BE19" t="n">
         <v>-45</v>
       </c>
       <c r="BF19" t="n">
-        <v>-86.06</v>
+        <v>-86.95</v>
       </c>
       <c r="BG19" t="n">
-        <v>-51.61</v>
+        <v>-54.7</v>
       </c>
       <c r="BH19" t="n">
         <v>9.75</v>
@@ -4897,7 +4897,7 @@
         <v>0</v>
       </c>
       <c r="BJ19" t="n">
-        <v>10.85</v>
+        <v>11.59</v>
       </c>
       <c r="BK19" t="n">
         <v>1.4</v>
@@ -4906,28 +4906,28 @@
         <v>12.62</v>
       </c>
       <c r="BM19" t="n">
-        <v>10.86</v>
+        <v>11.84</v>
       </c>
       <c r="BN19" t="n">
-        <v>11.41</v>
+        <v>11.84</v>
       </c>
       <c r="BO19" t="n">
         <v>9.19</v>
       </c>
       <c r="BP19" t="n">
-        <v>10.61</v>
+        <v>11.05</v>
       </c>
       <c r="BQ19" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="BR19" t="n">
-        <v>10.64</v>
+        <v>11.5</v>
       </c>
       <c r="BS19" t="n">
         <v>2.16</v>
       </c>
       <c r="BT19" t="n">
-        <v>11387</v>
+        <v>11243</v>
       </c>
     </row>
     <row r="20">
@@ -5417,13 +5417,13 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>5.48</v>
+        <v>5.75</v>
       </c>
       <c r="G22" t="n">
-        <v>1095265683</v>
+        <v>1151409900</v>
       </c>
       <c r="H22" t="n">
-        <v>3376000</v>
+        <v>4550200</v>
       </c>
       <c r="I22" t="n">
         <v>200245299</v>
@@ -5438,7 +5438,7 @@
         <v>0.27</v>
       </c>
       <c r="M22" t="n">
-        <v>0.09289671984473689</v>
+        <v>0.09765868187687618</v>
       </c>
       <c r="N22" t="n">
         <v>0.08</v>
@@ -5516,7 +5516,7 @@
         <v>378463615.11</v>
       </c>
       <c r="AM22" t="n">
-        <v>248359565.3061225</v>
+        <v>261090680.2721088</v>
       </c>
       <c r="AN22" t="n">
         <v>0</v>
@@ -5566,19 +5566,19 @@
         <v>172.49</v>
       </c>
       <c r="BC22" t="n">
-        <v>442.06</v>
+        <v>416.61</v>
       </c>
       <c r="BD22" t="n">
-        <v>342.59</v>
+        <v>321.81</v>
       </c>
       <c r="BE22" t="n">
         <v>-100</v>
       </c>
       <c r="BF22" t="n">
-        <v>-65.51000000000001</v>
+        <v>-67.13</v>
       </c>
       <c r="BG22" t="n">
-        <v>3047.62</v>
+        <v>2899.82</v>
       </c>
       <c r="BH22" t="n">
         <v>20.75</v>
@@ -5587,7 +5587,7 @@
         <v>0</v>
       </c>
       <c r="BJ22" t="n">
-        <v>5.48</v>
+        <v>5.75</v>
       </c>
       <c r="BK22" t="n">
         <v>1.89</v>
@@ -5596,7 +5596,7 @@
         <v>0.67</v>
       </c>
       <c r="BM22" t="n">
-        <v>5.56</v>
+        <v>6.15</v>
       </c>
       <c r="BN22" t="n">
         <v>7.89</v>
@@ -5605,19 +5605,19 @@
         <v>3.37</v>
       </c>
       <c r="BP22" t="n">
-        <v>5.06</v>
+        <v>5.6</v>
       </c>
       <c r="BQ22" t="n">
-        <v>8.16</v>
+        <v>8.56</v>
       </c>
       <c r="BR22" t="n">
-        <v>5.36</v>
+        <v>5.6</v>
       </c>
       <c r="BS22" t="n">
         <v>0.09</v>
       </c>
       <c r="BT22" t="n">
-        <v>1585160</v>
+        <v>1639090</v>
       </c>
     </row>
     <row r="23">
@@ -5877,13 +5877,13 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>3.34</v>
+        <v>3.89</v>
       </c>
       <c r="G24" t="n">
-        <v>1353301499</v>
+        <v>1571049674</v>
       </c>
       <c r="H24" t="n">
-        <v>9865000</v>
+        <v>13516400</v>
       </c>
       <c r="I24" t="n">
         <v>403868805</v>
@@ -5898,7 +5898,7 @@
         <v>0.49</v>
       </c>
       <c r="M24" t="n">
-        <v>0.327148223639631</v>
+        <v>0.3797868475565188</v>
       </c>
       <c r="N24" t="n">
         <v>0.11</v>
@@ -5976,7 +5976,7 @@
         <v>153470145.9</v>
       </c>
       <c r="AM24" t="n">
-        <v>1219190539.63964</v>
+        <v>1415360066.666667</v>
       </c>
       <c r="AN24" t="n">
         <v>0.0813</v>
@@ -6017,7 +6017,7 @@
         <v>5.84</v>
       </c>
       <c r="AZ24" t="n">
-        <v>1.54</v>
+        <v>1.8</v>
       </c>
       <c r="BA24" t="n">
         <v>0.38</v>
@@ -6026,19 +6026,19 @@
         <v>1.46</v>
       </c>
       <c r="BC24" t="n">
-        <v>114.26</v>
+        <v>83.97</v>
       </c>
       <c r="BD24" t="n">
-        <v>74.95</v>
+        <v>50.21</v>
       </c>
       <c r="BE24" t="n">
         <v>-53.83</v>
       </c>
       <c r="BF24" t="n">
-        <v>-88.62</v>
+        <v>-90.23</v>
       </c>
       <c r="BG24" t="n">
-        <v>-56.35</v>
+        <v>-62.52</v>
       </c>
       <c r="BH24" t="n">
         <v>5.99</v>
@@ -6047,7 +6047,7 @@
         <v>0</v>
       </c>
       <c r="BJ24" t="n">
-        <v>3.34</v>
+        <v>3.89</v>
       </c>
       <c r="BK24" t="n">
         <v>0.38</v>
@@ -6056,7 +6056,7 @@
         <v>0.41</v>
       </c>
       <c r="BM24" t="n">
-        <v>3.37</v>
+        <v>3.95</v>
       </c>
       <c r="BN24" t="n">
         <v>5.29</v>
@@ -6065,19 +6065,19 @@
         <v>1.92</v>
       </c>
       <c r="BP24" t="n">
-        <v>3.09</v>
+        <v>3.61</v>
       </c>
       <c r="BQ24" t="n">
-        <v>8.199999999999999</v>
+        <v>9.550000000000001</v>
       </c>
       <c r="BR24" t="n">
-        <v>3.16</v>
+        <v>3.61</v>
       </c>
       <c r="BS24" t="n">
         <v>0.29</v>
       </c>
       <c r="BT24" t="n">
-        <v>7301783</v>
+        <v>7463927</v>
       </c>
     </row>
     <row r="25">
@@ -6107,13 +6107,13 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>4.46</v>
+        <v>5.12</v>
       </c>
       <c r="G25" t="n">
-        <v>1570403923</v>
+        <v>1774049752</v>
       </c>
       <c r="H25" t="n">
-        <v>1144900</v>
+        <v>3447600</v>
       </c>
       <c r="I25" t="n">
         <v>346494097</v>
@@ -6128,7 +6128,7 @@
         <v>0.97</v>
       </c>
       <c r="M25" t="n">
-        <v>0.7830751010729179</v>
+        <v>0.8846222099355932</v>
       </c>
       <c r="N25" t="n">
         <v>0.22</v>
@@ -6206,7 +6206,7 @@
         <v>62368937.46</v>
       </c>
       <c r="AM25" t="n">
-        <v>577354383.4558823</v>
+        <v>652224173.5294117</v>
       </c>
       <c r="AN25" t="n">
         <v>0.4742</v>
@@ -6247,7 +6247,7 @@
         <v>3.27</v>
       </c>
       <c r="AZ25" t="n">
-        <v>10.39</v>
+        <v>11.93</v>
       </c>
       <c r="BA25" t="n">
         <v>0.23</v>
@@ -6256,19 +6256,19 @@
         <v>2.2</v>
       </c>
       <c r="BC25" t="n">
-        <v>-10.09</v>
+        <v>-21.68</v>
       </c>
       <c r="BD25" t="n">
-        <v>-26.59</v>
+        <v>-36.05</v>
       </c>
       <c r="BE25" t="n">
         <v>133</v>
       </c>
       <c r="BF25" t="n">
-        <v>-94.8</v>
+        <v>-95.47</v>
       </c>
       <c r="BG25" t="n">
-        <v>-50.68</v>
+        <v>-57.04</v>
       </c>
       <c r="BH25" t="n">
         <v>3.97</v>
@@ -6277,7 +6277,7 @@
         <v>0</v>
       </c>
       <c r="BJ25" t="n">
-        <v>4.46</v>
+        <v>5.12</v>
       </c>
       <c r="BK25" t="n">
         <v>0.18</v>
@@ -6286,7 +6286,7 @@
         <v>0.24</v>
       </c>
       <c r="BM25" t="n">
-        <v>4.6</v>
+        <v>5.27</v>
       </c>
       <c r="BN25" t="n">
         <v>6.3</v>
@@ -6295,19 +6295,19 @@
         <v>2.64</v>
       </c>
       <c r="BP25" t="n">
-        <v>4.32</v>
+        <v>4.93</v>
       </c>
       <c r="BQ25" t="n">
-        <v>18.85</v>
+        <v>21.64</v>
       </c>
       <c r="BR25" t="n">
-        <v>4.46</v>
+        <v>4.98</v>
       </c>
       <c r="BS25" t="n">
         <v>0.67</v>
       </c>
       <c r="BT25" t="n">
-        <v>1172900</v>
+        <v>1176113</v>
       </c>
     </row>
     <row r="26">
@@ -6337,13 +6337,13 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>11.15</v>
+        <v>12.98</v>
       </c>
       <c r="G26" t="n">
-        <v>15101481433</v>
+        <v>17580020520</v>
       </c>
       <c r="H26" t="n">
-        <v>31033400</v>
+        <v>52209900</v>
       </c>
       <c r="I26" t="n">
         <v>1354393401</v>
@@ -6358,7 +6358,7 @@
         <v>1.94</v>
       </c>
       <c r="M26" t="n">
-        <v>0.1947323300444234</v>
+        <v>0.2266928826338528</v>
       </c>
       <c r="N26" t="n">
         <v>0.26</v>
@@ -6436,7 +6436,7 @@
         <v>961619314.7099999</v>
       </c>
       <c r="AM26" t="n">
-        <v>5393386226.071429</v>
+        <v>6278578757.142858</v>
       </c>
       <c r="AN26" t="n">
         <v>0.1043</v>
@@ -6477,7 +6477,7 @@
         <v>7.07</v>
       </c>
       <c r="AZ26" t="n">
-        <v>2.14</v>
+        <v>2.49</v>
       </c>
       <c r="BA26" t="n">
         <v>0.66</v>
@@ -6486,19 +6486,19 @@
         <v>1.19</v>
       </c>
       <c r="BC26" t="n">
-        <v>-22.37</v>
+        <v>-33.31</v>
       </c>
       <c r="BD26" t="n">
-        <v>-36.62</v>
+        <v>-45.55</v>
       </c>
       <c r="BE26" t="n">
         <v>-80.83</v>
       </c>
       <c r="BF26" t="n">
-        <v>-94.09</v>
+        <v>-94.92</v>
       </c>
       <c r="BG26" t="n">
-        <v>-89.3</v>
+        <v>-90.81</v>
       </c>
       <c r="BH26" t="n">
         <v>4.69</v>
@@ -6507,7 +6507,7 @@
         <v>0</v>
       </c>
       <c r="BJ26" t="n">
-        <v>11.15</v>
+        <v>12.98</v>
       </c>
       <c r="BK26" t="n">
         <v>0.71</v>
@@ -6516,28 +6516,28 @@
         <v>0.72</v>
       </c>
       <c r="BM26" t="n">
-        <v>11.52</v>
+        <v>13.45</v>
       </c>
       <c r="BN26" t="n">
-        <v>11.52</v>
+        <v>13.45</v>
       </c>
       <c r="BO26" t="n">
         <v>6.91</v>
       </c>
       <c r="BP26" t="n">
-        <v>10.85</v>
+        <v>12.62</v>
       </c>
       <c r="BQ26" t="n">
-        <v>15.55</v>
+        <v>18.1</v>
       </c>
       <c r="BR26" t="n">
-        <v>11.52</v>
+        <v>12.82</v>
       </c>
       <c r="BS26" t="n">
         <v>0.16</v>
       </c>
       <c r="BT26" t="n">
-        <v>13317553</v>
+        <v>14118867</v>
       </c>
     </row>
     <row r="27">
@@ -8165,13 +8165,13 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>19.54</v>
+        <v>22.17</v>
       </c>
       <c r="G34" t="n">
-        <v>4032641940</v>
+        <v>4577878881</v>
       </c>
       <c r="H34" t="n">
-        <v>4945600</v>
+        <v>8341600</v>
       </c>
       <c r="I34" t="n">
         <v>206489813</v>
@@ -8186,7 +8186,7 @@
         <v>0.45</v>
       </c>
       <c r="M34" t="n">
-        <v>0.3545163254075566</v>
+        <v>0.4024490205676373</v>
       </c>
       <c r="N34" t="n">
         <v>0.24</v>
@@ -8264,7 +8264,7 @@
         <v>324189006.41</v>
       </c>
       <c r="AM34" t="n">
-        <v>838387097.7130978</v>
+        <v>951741971.1018711</v>
       </c>
       <c r="AN34" t="n">
         <v>0</v>
@@ -8305,7 +8305,7 @@
         <v>30.28</v>
       </c>
       <c r="AZ34" t="n">
-        <v>45.59</v>
+        <v>51.73</v>
       </c>
       <c r="BA34" t="n">
         <v>2.29</v>
@@ -8314,19 +8314,19 @@
         <v>25.26</v>
       </c>
       <c r="BC34" t="n">
-        <v>89.81</v>
+        <v>67.29000000000001</v>
       </c>
       <c r="BD34" t="n">
-        <v>54.98</v>
+        <v>36.59</v>
       </c>
       <c r="BE34" t="n">
         <v>133.33</v>
       </c>
       <c r="BF34" t="n">
-        <v>-88.26000000000001</v>
+        <v>-89.65000000000001</v>
       </c>
       <c r="BG34" t="n">
-        <v>29.26</v>
+        <v>13.93</v>
       </c>
       <c r="BH34" t="n">
         <v>38.94</v>
@@ -8335,7 +8335,7 @@
         <v>0</v>
       </c>
       <c r="BJ34" t="n">
-        <v>19.54</v>
+        <v>22.17</v>
       </c>
       <c r="BK34" t="n">
         <v>1.57</v>
@@ -8344,7 +8344,7 @@
         <v>1.58</v>
       </c>
       <c r="BM34" t="n">
-        <v>19.57</v>
+        <v>22.68</v>
       </c>
       <c r="BN34" t="n">
         <v>28.86</v>
@@ -8353,19 +8353,19 @@
         <v>14.3</v>
       </c>
       <c r="BP34" t="n">
-        <v>18.65</v>
+        <v>21.34</v>
       </c>
       <c r="BQ34" t="n">
-        <v>12.39</v>
+        <v>14.06</v>
       </c>
       <c r="BR34" t="n">
-        <v>19.02</v>
+        <v>21.59</v>
       </c>
       <c r="BS34" t="n">
         <v>0.32</v>
       </c>
       <c r="BT34" t="n">
-        <v>3911500</v>
+        <v>3999757</v>
       </c>
     </row>
     <row r="35">
@@ -8395,13 +8395,13 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>19</v>
+        <v>23.3</v>
       </c>
       <c r="G35" t="n">
-        <v>96299695000</v>
+        <v>117583446149</v>
       </c>
       <c r="H35" t="n">
-        <v>40016700</v>
+        <v>200158200</v>
       </c>
       <c r="I35" t="n">
         <v>5046500000</v>
@@ -8416,7 +8416,7 @@
         <v>4.69</v>
       </c>
       <c r="M35" t="n">
-        <v>7.994835679034039</v>
+        <v>9.761820435005561</v>
       </c>
       <c r="N35" t="n">
         <v>1.79</v>
@@ -8494,7 +8494,7 @@
         <v>5349290000</v>
       </c>
       <c r="AM35" t="n">
-        <v>7958652479.338843</v>
+        <v>9717640177.603306</v>
       </c>
       <c r="AN35" t="n">
         <v>0.5305</v>
@@ -8535,7 +8535,7 @@
         <v>7.68</v>
       </c>
       <c r="AZ35" t="n">
-        <v>11.08</v>
+        <v>13.59</v>
       </c>
       <c r="BA35" t="n">
         <v>1.11</v>
@@ -8544,19 +8544,19 @@
         <v>9.119999999999999</v>
       </c>
       <c r="BC35" t="n">
-        <v>-50.49</v>
+        <v>-59.63</v>
       </c>
       <c r="BD35" t="n">
-        <v>-59.58</v>
+        <v>-67.04000000000001</v>
       </c>
       <c r="BE35" t="n">
         <v>-41.67</v>
       </c>
       <c r="BF35" t="n">
-        <v>-94.14</v>
+        <v>-95.22</v>
       </c>
       <c r="BG35" t="n">
-        <v>-52.02</v>
+        <v>-60.87</v>
       </c>
       <c r="BH35" t="n">
         <v>3.71</v>
@@ -8565,7 +8565,7 @@
         <v>0</v>
       </c>
       <c r="BJ35" t="n">
-        <v>19</v>
+        <v>23.3</v>
       </c>
       <c r="BK35" t="n">
         <v>1.06</v>
@@ -8574,28 +8574,28 @@
         <v>1.04</v>
       </c>
       <c r="BM35" t="n">
-        <v>19.04</v>
+        <v>24.28</v>
       </c>
       <c r="BN35" t="n">
-        <v>19.88</v>
+        <v>24.28</v>
       </c>
       <c r="BO35" t="n">
         <v>11.58</v>
       </c>
       <c r="BP35" t="n">
-        <v>18.32</v>
+        <v>22.03</v>
       </c>
       <c r="BQ35" t="n">
-        <v>18.18</v>
+        <v>22.3</v>
       </c>
       <c r="BR35" t="n">
-        <v>18.95</v>
+        <v>22.1</v>
       </c>
       <c r="BS35" t="n">
         <v>7.3</v>
       </c>
       <c r="BT35" t="n">
-        <v>40990940</v>
+        <v>41530023</v>
       </c>
     </row>
     <row r="36">
@@ -8858,10 +8858,10 @@
         <v>14.5</v>
       </c>
       <c r="G37" t="n">
-        <v>178850000</v>
+        <v>178849960</v>
       </c>
       <c r="H37" t="n">
-        <v>1400</v>
+        <v>5100</v>
       </c>
       <c r="I37" t="n">
         <v>4900000</v>
@@ -8876,7 +8876,7 @@
         <v>0.88</v>
       </c>
       <c r="M37" t="n">
-        <v>1.741255411255411</v>
+        <v>1.741255021821716</v>
       </c>
       <c r="N37" t="n">
         <v>0.5</v>
@@ -8954,7 +8954,7 @@
         <v>11319000</v>
       </c>
       <c r="AM37" t="n">
-        <v>42787081.33971293</v>
+        <v>42787071.77033493</v>
       </c>
       <c r="AN37" t="n">
         <v>0</v>
@@ -9043,7 +9043,7 @@
         <v>13.42</v>
       </c>
       <c r="BP37" t="n">
-        <v>14.2</v>
+        <v>14.22</v>
       </c>
       <c r="BQ37" t="n">
         <v>6.27</v>
@@ -9055,7 +9055,7 @@
         <v>0.72</v>
       </c>
       <c r="BT37" t="n">
-        <v>1267</v>
+        <v>1313</v>
       </c>
     </row>
     <row r="38">
@@ -9085,13 +9085,13 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>93.39</v>
+        <v>95.09999999999999</v>
       </c>
       <c r="G38" t="n">
-        <v>490366600</v>
+        <v>487703300</v>
       </c>
       <c r="H38" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="I38" t="n">
         <v>2375293</v>
@@ -9106,7 +9106,7 @@
         <v>3.18</v>
       </c>
       <c r="M38" t="n">
-        <v>3.695265480220967</v>
+        <v>3.675195596681851</v>
       </c>
       <c r="N38" t="n">
         <v>2.23</v>
@@ -9184,7 +9184,7 @@
         <v>10403783.34</v>
       </c>
       <c r="AM38" t="n">
-        <v>21545105.44815465</v>
+        <v>21428088.75219683</v>
       </c>
       <c r="AN38" t="n">
         <v>0</v>
@@ -9234,19 +9234,19 @@
         <v>11.45</v>
       </c>
       <c r="BC38" t="n">
-        <v>-42.38</v>
+        <v>-43.42</v>
       </c>
       <c r="BD38" t="n">
-        <v>-52.96</v>
+        <v>-53.8</v>
       </c>
       <c r="BE38" t="n">
         <v>-100</v>
       </c>
       <c r="BF38" t="n">
-        <v>-95.33</v>
+        <v>-95.42</v>
       </c>
       <c r="BG38" t="n">
-        <v>-87.73999999999999</v>
+        <v>-87.95999999999999</v>
       </c>
       <c r="BH38" t="n">
         <v>29.38</v>
@@ -9255,7 +9255,7 @@
         <v>0</v>
       </c>
       <c r="BJ38" t="n">
-        <v>93.39</v>
+        <v>95.09999999999999</v>
       </c>
       <c r="BK38" t="n">
         <v>4.38</v>
@@ -9264,22 +9264,22 @@
         <v>4.38</v>
       </c>
       <c r="BM38" t="n">
-        <v>0</v>
+        <v>95.09999999999999</v>
       </c>
       <c r="BN38" t="n">
-        <v>93.90000000000001</v>
+        <v>95.09999999999999</v>
       </c>
       <c r="BO38" t="n">
         <v>70.14</v>
       </c>
       <c r="BP38" t="n">
-        <v>0</v>
+        <v>95.09999999999999</v>
       </c>
       <c r="BQ38" t="n">
-        <v>21.33</v>
+        <v>21.72</v>
       </c>
       <c r="BR38" t="n">
-        <v>0</v>
+        <v>95.09999999999999</v>
       </c>
       <c r="BS38" t="n">
         <v>1.67</v>
@@ -9315,13 +9315,13 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>69.76000000000001</v>
+        <v>71</v>
       </c>
       <c r="G39" t="n">
-        <v>3910628522</v>
+        <v>3980140010</v>
       </c>
       <c r="H39" t="n">
-        <v>1700</v>
+        <v>7200</v>
       </c>
       <c r="I39" t="n">
         <v>168174945</v>
@@ -9336,7 +9336,7 @@
         <v>0.53</v>
       </c>
       <c r="M39" t="n">
-        <v>0.1962963983609473</v>
+        <v>0.1997855701558003</v>
       </c>
       <c r="N39" t="n">
         <v>0.06</v>
@@ -9414,7 +9414,7 @@
         <v>2536078170.6</v>
       </c>
       <c r="AM39" t="n">
-        <v>410780306.9327731</v>
+        <v>418081933.8235294</v>
       </c>
       <c r="AN39" t="n">
         <v>11.9435</v>
@@ -9455,7 +9455,7 @@
         <v>170.24</v>
       </c>
       <c r="AZ39" t="n">
-        <v>203.82</v>
+        <v>207.44</v>
       </c>
       <c r="BA39" t="n">
         <v>19.01</v>
@@ -9464,19 +9464,19 @@
         <v>91.72</v>
       </c>
       <c r="BC39" t="n">
-        <v>198.89</v>
+        <v>193.67</v>
       </c>
       <c r="BD39" t="n">
-        <v>144.04</v>
+        <v>139.78</v>
       </c>
       <c r="BE39" t="n">
         <v>192.17</v>
       </c>
       <c r="BF39" t="n">
-        <v>-72.75</v>
+        <v>-73.23</v>
       </c>
       <c r="BG39" t="n">
-        <v>31.48</v>
+        <v>29.19</v>
       </c>
       <c r="BH39" t="n">
         <v>128.13</v>
@@ -9485,7 +9485,7 @@
         <v>0</v>
       </c>
       <c r="BJ39" t="n">
-        <v>69.76000000000001</v>
+        <v>71</v>
       </c>
       <c r="BK39" t="n">
         <v>15.08</v>
@@ -9494,7 +9494,7 @@
         <v>15.08</v>
       </c>
       <c r="BM39" t="n">
-        <v>69.84999999999999</v>
+        <v>72</v>
       </c>
       <c r="BN39" t="n">
         <v>74.56</v>
@@ -9503,19 +9503,19 @@
         <v>54.98</v>
       </c>
       <c r="BP39" t="n">
-        <v>69.29000000000001</v>
+        <v>70</v>
       </c>
       <c r="BQ39" t="n">
-        <v>4.63</v>
+        <v>4.71</v>
       </c>
       <c r="BR39" t="n">
-        <v>69.34999999999999</v>
+        <v>70.56</v>
       </c>
       <c r="BS39" t="n">
         <v>0.58</v>
       </c>
       <c r="BT39" t="n">
-        <v>3047</v>
+        <v>2857</v>
       </c>
     </row>
     <row r="40">
@@ -9545,13 +9545,13 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>23.72</v>
+        <v>26.33</v>
       </c>
       <c r="G40" t="n">
-        <v>135581974275</v>
+        <v>150892858782</v>
       </c>
       <c r="H40" t="n">
-        <v>51578000</v>
+        <v>147712300</v>
       </c>
       <c r="I40" t="n">
         <v>5730834040</v>
@@ -9566,7 +9566,7 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="M40" t="n">
-        <v>0.4113724890103301</v>
+        <v>0.4578276074158132</v>
       </c>
       <c r="N40" t="n">
         <v>0.05</v>
@@ -9644,7 +9644,7 @@
         <v>15358635227.2</v>
       </c>
       <c r="AM40" t="n">
-        <v>7032260076.504149</v>
+        <v>7826393090.352696</v>
       </c>
       <c r="AN40" t="n">
         <v>0.5641</v>
@@ -9685,7 +9685,7 @@
         <v>36.13</v>
       </c>
       <c r="AZ40" t="n">
-        <v>11.98</v>
+        <v>13.3</v>
       </c>
       <c r="BA40" t="n">
         <v>2.76</v>
@@ -9694,19 +9694,19 @@
         <v>27.89</v>
       </c>
       <c r="BC40" t="n">
-        <v>86.55</v>
+        <v>68.05</v>
       </c>
       <c r="BD40" t="n">
-        <v>52.31</v>
+        <v>37.22</v>
       </c>
       <c r="BE40" t="n">
         <v>-49.5</v>
       </c>
       <c r="BF40" t="n">
-        <v>-88.37</v>
+        <v>-89.52</v>
       </c>
       <c r="BG40" t="n">
-        <v>17.58</v>
+        <v>5.93</v>
       </c>
       <c r="BH40" t="n">
         <v>32.47</v>
@@ -9715,7 +9715,7 @@
         <v>0</v>
       </c>
       <c r="BJ40" t="n">
-        <v>23.72</v>
+        <v>26.33</v>
       </c>
       <c r="BK40" t="n">
         <v>2.68</v>
@@ -9724,7 +9724,7 @@
         <v>2.5</v>
       </c>
       <c r="BM40" t="n">
-        <v>23.78</v>
+        <v>27.19</v>
       </c>
       <c r="BN40" t="n">
         <v>27.36</v>
@@ -9733,19 +9733,19 @@
         <v>17.67</v>
       </c>
       <c r="BP40" t="n">
-        <v>22.96</v>
+        <v>25.19</v>
       </c>
       <c r="BQ40" t="n">
-        <v>9.49</v>
+        <v>10.54</v>
       </c>
       <c r="BR40" t="n">
-        <v>23.36</v>
+        <v>25.19</v>
       </c>
       <c r="BS40" t="n">
         <v>0.39</v>
       </c>
       <c r="BT40" t="n">
-        <v>38498187</v>
+        <v>37487763</v>
       </c>
     </row>
     <row r="41">
@@ -9775,13 +9775,13 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>16.83</v>
+        <v>19.36</v>
       </c>
       <c r="G41" t="n">
-        <v>202572276577</v>
+        <v>229256884001</v>
       </c>
       <c r="H41" t="n">
-        <v>26344000</v>
+        <v>43770400</v>
       </c>
       <c r="I41" t="n">
         <v>5303870781</v>
@@ -9796,7 +9796,7 @@
         <v>0.92</v>
       </c>
       <c r="M41" t="n">
-        <v>1.34993526143364</v>
+        <v>1.52776064360275</v>
       </c>
       <c r="N41" t="n">
         <v>0.07000000000000001</v>
@@ -9874,7 +9874,7 @@
         <v>12304980211.92</v>
       </c>
       <c r="AM41" t="n">
-        <v>31212985605.08474</v>
+        <v>35324635439.29121</v>
       </c>
       <c r="AN41" t="n">
         <v>1.6841</v>
@@ -9915,7 +9915,7 @@
         <v>24.4</v>
       </c>
       <c r="AZ41" t="n">
-        <v>25.19</v>
+        <v>28.98</v>
       </c>
       <c r="BA41" t="n">
         <v>2.53</v>
@@ -9924,19 +9924,19 @@
         <v>13.77</v>
       </c>
       <c r="BC41" t="n">
-        <v>77.56999999999999</v>
+        <v>54.37</v>
       </c>
       <c r="BD41" t="n">
-        <v>44.99</v>
+        <v>26.04</v>
       </c>
       <c r="BE41" t="n">
         <v>49.67</v>
       </c>
       <c r="BF41" t="n">
-        <v>-84.98</v>
+        <v>-86.95</v>
       </c>
       <c r="BG41" t="n">
-        <v>-18.18</v>
+        <v>-28.87</v>
       </c>
       <c r="BH41" t="n">
         <v>17.11</v>
@@ -9945,7 +9945,7 @@
         <v>0</v>
       </c>
       <c r="BJ41" t="n">
-        <v>16.83</v>
+        <v>19.36</v>
       </c>
       <c r="BK41" t="n">
         <v>2.32</v>
@@ -9954,28 +9954,28 @@
         <v>2.34</v>
       </c>
       <c r="BM41" t="n">
-        <v>16.83</v>
+        <v>19.54</v>
       </c>
       <c r="BN41" t="n">
-        <v>18.26</v>
+        <v>19.54</v>
       </c>
       <c r="BO41" t="n">
         <v>13.41</v>
       </c>
       <c r="BP41" t="n">
-        <v>16.01</v>
+        <v>18.04</v>
       </c>
       <c r="BQ41" t="n">
-        <v>7.2</v>
+        <v>8.279999999999999</v>
       </c>
       <c r="BR41" t="n">
-        <v>16.7</v>
+        <v>18.04</v>
       </c>
       <c r="BS41" t="n">
         <v>0.5600000000000001</v>
       </c>
       <c r="BT41" t="n">
-        <v>9832217</v>
+        <v>10457137</v>
       </c>
     </row>
     <row r="42">
@@ -10005,13 +10005,13 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>19.23</v>
+        <v>21.84</v>
       </c>
       <c r="G42" t="n">
-        <v>202572276577</v>
+        <v>229256884001</v>
       </c>
       <c r="H42" t="n">
-        <v>109085500</v>
+        <v>160447100</v>
       </c>
       <c r="I42" t="n">
         <v>5288141247</v>
@@ -10026,7 +10026,7 @@
         <v>1.05</v>
       </c>
       <c r="M42" t="n">
-        <v>1.35395063311165</v>
+        <v>1.532304955462998</v>
       </c>
       <c r="N42" t="n">
         <v>0.08</v>
@@ -10104,7 +10104,7 @@
         <v>12268487693.04</v>
       </c>
       <c r="AM42" t="n">
-        <v>27560853956.05442</v>
+        <v>31191412789.2517</v>
       </c>
       <c r="AN42" t="n">
         <v>1.8491</v>
@@ -10145,7 +10145,7 @@
         <v>24.4</v>
       </c>
       <c r="AZ42" t="n">
-        <v>27.85</v>
+        <v>31.63</v>
       </c>
       <c r="BA42" t="n">
         <v>2.53</v>
@@ -10154,19 +10154,19 @@
         <v>15.11</v>
       </c>
       <c r="BC42" t="n">
-        <v>55.41</v>
+        <v>36.84</v>
       </c>
       <c r="BD42" t="n">
-        <v>26.89</v>
+        <v>11.73</v>
       </c>
       <c r="BE42" t="n">
         <v>44.83</v>
       </c>
       <c r="BF42" t="n">
-        <v>-86.86</v>
+        <v>-88.43000000000001</v>
       </c>
       <c r="BG42" t="n">
-        <v>-21.4</v>
+        <v>-30.79</v>
       </c>
       <c r="BH42" t="n">
         <v>17.11</v>
@@ -10175,7 +10175,7 @@
         <v>0</v>
       </c>
       <c r="BJ42" t="n">
-        <v>19.23</v>
+        <v>21.84</v>
       </c>
       <c r="BK42" t="n">
         <v>2.32</v>
@@ -10184,28 +10184,28 @@
         <v>2.34</v>
       </c>
       <c r="BM42" t="n">
-        <v>19.3</v>
+        <v>22.14</v>
       </c>
       <c r="BN42" t="n">
-        <v>21.32</v>
+        <v>22.14</v>
       </c>
       <c r="BO42" t="n">
         <v>15.65</v>
       </c>
       <c r="BP42" t="n">
-        <v>18.19</v>
+        <v>20.76</v>
       </c>
       <c r="BQ42" t="n">
-        <v>8.23</v>
+        <v>9.34</v>
       </c>
       <c r="BR42" t="n">
-        <v>18.94</v>
+        <v>20.76</v>
       </c>
       <c r="BS42" t="n">
         <v>0.63</v>
       </c>
       <c r="BT42" t="n">
-        <v>43064480</v>
+        <v>45468250</v>
       </c>
     </row>
     <row r="43">
@@ -10235,13 +10235,13 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>40.45</v>
+        <v>40.99</v>
       </c>
       <c r="G43" t="n">
-        <v>78269982926</v>
+        <v>79577948268</v>
       </c>
       <c r="H43" t="n">
-        <v>8697900</v>
+        <v>10011300</v>
       </c>
       <c r="I43" t="n">
         <v>1941400000</v>
@@ -10334,7 +10334,7 @@
         <v>9182822000</v>
       </c>
       <c r="AM43" t="n">
-        <v>9533493657.247259</v>
+        <v>9692807340.803896</v>
       </c>
       <c r="AN43" t="n">
         <v>4.5901</v>
@@ -10375,7 +10375,7 @@
         <v>19.95</v>
       </c>
       <c r="AZ43" t="n">
-        <v>73.42</v>
+        <v>74.40000000000001</v>
       </c>
       <c r="BA43" t="n">
         <v>5.63</v>
@@ -10384,19 +10384,19 @@
         <v>48.62</v>
       </c>
       <c r="BC43" t="n">
-        <v>-39.59</v>
+        <v>-40.39</v>
       </c>
       <c r="BD43" t="n">
-        <v>-50.68</v>
+        <v>-51.33</v>
       </c>
       <c r="BE43" t="n">
         <v>81.5</v>
       </c>
       <c r="BF43" t="n">
-        <v>-86.08</v>
+        <v>-86.27</v>
       </c>
       <c r="BG43" t="n">
-        <v>20.19</v>
+        <v>18.61</v>
       </c>
       <c r="BH43" t="n">
         <v>5.61</v>
@@ -10405,7 +10405,7 @@
         <v>0</v>
       </c>
       <c r="BJ43" t="n">
-        <v>40.45</v>
+        <v>40.99</v>
       </c>
       <c r="BK43" t="n">
         <v>4.73</v>
@@ -10414,7 +10414,7 @@
         <v>4.73</v>
       </c>
       <c r="BM43" t="n">
-        <v>40.79</v>
+        <v>42.42</v>
       </c>
       <c r="BN43" t="n">
         <v>42.98</v>
@@ -10423,19 +10423,19 @@
         <v>28.06</v>
       </c>
       <c r="BP43" t="n">
-        <v>39.51</v>
+        <v>40.88</v>
       </c>
       <c r="BQ43" t="n">
-        <v>8.539999999999999</v>
+        <v>8.66</v>
       </c>
       <c r="BR43" t="n">
-        <v>39.58</v>
+        <v>41.9</v>
       </c>
       <c r="BS43" t="n">
         <v>0</v>
       </c>
       <c r="BT43" t="n">
-        <v>6372740</v>
+        <v>6520643</v>
       </c>
     </row>
     <row r="44">
@@ -10925,13 +10925,13 @@
         </is>
       </c>
       <c r="F46" t="n">
-        <v>3.88</v>
+        <v>4.19</v>
       </c>
       <c r="G46" t="n">
-        <v>3862297613</v>
+        <v>4192271037</v>
       </c>
       <c r="H46" t="n">
-        <v>25088000</v>
+        <v>52029900</v>
       </c>
       <c r="I46" t="n">
         <v>1000542188</v>
@@ -10946,7 +10946,7 @@
         <v>2.5</v>
       </c>
       <c r="M46" t="n">
-        <v>0.06713399402361354</v>
+        <v>0.07286955251610387</v>
       </c>
       <c r="N46" t="n">
         <v>0.08</v>
@@ -11024,7 +11024,7 @@
         <v>460249406.48</v>
       </c>
       <c r="AM46" t="n">
-        <v>3786566287.254902</v>
+        <v>4110069644.117647</v>
       </c>
       <c r="AN46" t="n">
         <v>0.0311</v>
@@ -11065,7 +11065,7 @@
         <v>3.3</v>
       </c>
       <c r="AZ46" t="n">
-        <v>3.2</v>
+        <v>3.46</v>
       </c>
       <c r="BA46" t="n">
         <v>0.42</v>
@@ -11074,19 +11074,19 @@
         <v>7.38</v>
       </c>
       <c r="BC46" t="n">
-        <v>4.22</v>
+        <v>-3.49</v>
       </c>
       <c r="BD46" t="n">
-        <v>-14.9</v>
+        <v>-21.2</v>
       </c>
       <c r="BE46" t="n">
         <v>-17.5</v>
       </c>
       <c r="BF46" t="n">
-        <v>-89.09999999999999</v>
+        <v>-89.90000000000001</v>
       </c>
       <c r="BG46" t="n">
-        <v>90.17</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="BH46" t="n">
         <v>1.58</v>
@@ -11095,7 +11095,7 @@
         <v>0</v>
       </c>
       <c r="BJ46" t="n">
-        <v>3.88</v>
+        <v>4.19</v>
       </c>
       <c r="BK46" t="n">
         <v>0.46</v>
@@ -11104,7 +11104,7 @@
         <v>0.46</v>
       </c>
       <c r="BM46" t="n">
-        <v>3.95</v>
+        <v>4.24</v>
       </c>
       <c r="BN46" t="n">
         <v>7.31</v>
@@ -11113,19 +11113,19 @@
         <v>2.97</v>
       </c>
       <c r="BP46" t="n">
-        <v>3.81</v>
+        <v>4.05</v>
       </c>
       <c r="BQ46" t="n">
-        <v>8.48</v>
+        <v>9.16</v>
       </c>
       <c r="BR46" t="n">
-        <v>3.95</v>
+        <v>4.07</v>
       </c>
       <c r="BS46" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="BT46" t="n">
-        <v>21389101</v>
+        <v>21262804</v>
       </c>
     </row>
     <row r="47">
@@ -11155,13 +11155,13 @@
         </is>
       </c>
       <c r="F47" t="n">
-        <v>9.23</v>
+        <v>9.32</v>
       </c>
       <c r="G47" t="n">
-        <v>3207462683</v>
+        <v>3233079002</v>
       </c>
       <c r="H47" t="n">
-        <v>21200</v>
+        <v>40800</v>
       </c>
       <c r="I47" t="n">
         <v>254106600</v>
@@ -11176,7 +11176,7 @@
         <v>1.22</v>
       </c>
       <c r="M47" t="n">
-        <v>0.7563566033437477</v>
+        <v>0.7623972260863598</v>
       </c>
       <c r="N47" t="n">
         <v>0.07000000000000001</v>
@@ -11254,7 +11254,7 @@
         <v>322715382</v>
       </c>
       <c r="AM47" t="n">
-        <v>568699057.2695036</v>
+        <v>573240957.8014184</v>
       </c>
       <c r="AN47" t="n">
         <v>0.4132</v>
@@ -11295,7 +11295,7 @@
         <v>11.74</v>
       </c>
       <c r="AZ47" t="n">
-        <v>12.12</v>
+        <v>12.24</v>
       </c>
       <c r="BA47" t="n">
         <v>1.46</v>
@@ -11304,19 +11304,19 @@
         <v>8.619999999999999</v>
       </c>
       <c r="BC47" t="n">
-        <v>55.73</v>
+        <v>54.22</v>
       </c>
       <c r="BD47" t="n">
-        <v>27.15</v>
+        <v>25.92</v>
       </c>
       <c r="BE47" t="n">
         <v>31.33</v>
       </c>
       <c r="BF47" t="n">
-        <v>-84.2</v>
+        <v>-84.34999999999999</v>
       </c>
       <c r="BG47" t="n">
-        <v>-6.61</v>
+        <v>-7.51</v>
       </c>
       <c r="BH47" t="n">
         <v>7.23</v>
@@ -11325,7 +11325,7 @@
         <v>0</v>
       </c>
       <c r="BJ47" t="n">
-        <v>9.23</v>
+        <v>9.32</v>
       </c>
       <c r="BK47" t="n">
         <v>1.27</v>
@@ -11334,28 +11334,28 @@
         <v>1.28</v>
       </c>
       <c r="BM47" t="n">
-        <v>9.25</v>
+        <v>9.59</v>
       </c>
       <c r="BN47" t="n">
-        <v>9.32</v>
+        <v>9.59</v>
       </c>
       <c r="BO47" t="n">
-        <v>7.17</v>
+        <v>7.12</v>
       </c>
       <c r="BP47" t="n">
-        <v>9</v>
+        <v>8.83</v>
       </c>
       <c r="BQ47" t="n">
-        <v>7.2</v>
+        <v>7.27</v>
       </c>
       <c r="BR47" t="n">
-        <v>9.25</v>
+        <v>9.5</v>
       </c>
       <c r="BS47" t="n">
         <v>0.53</v>
       </c>
       <c r="BT47" t="n">
-        <v>10660</v>
+        <v>11063</v>
       </c>
     </row>
     <row r="48">
@@ -11385,13 +11385,13 @@
         </is>
       </c>
       <c r="F48" t="n">
-        <v>9.17</v>
+        <v>9.210000000000001</v>
       </c>
       <c r="G48" t="n">
-        <v>3207462683</v>
+        <v>3233079002</v>
       </c>
       <c r="H48" t="n">
-        <v>2800</v>
+        <v>3600</v>
       </c>
       <c r="I48" t="n">
         <v>93397546</v>
@@ -11406,7 +11406,7 @@
         <v>1.24</v>
       </c>
       <c r="M48" t="n">
-        <v>2.05781857334055</v>
+        <v>2.074253288948686</v>
       </c>
       <c r="N48" t="n">
         <v>0.07000000000000001</v>
@@ -11484,7 +11484,7 @@
         <v>118614883.42</v>
       </c>
       <c r="AM48" t="n">
-        <v>560745224.3006994</v>
+        <v>565223601.7482518</v>
       </c>
       <c r="AN48" t="n">
         <v>0.4132</v>
@@ -11525,7 +11525,7 @@
         <v>11.74</v>
       </c>
       <c r="AZ48" t="n">
-        <v>12</v>
+        <v>12.05</v>
       </c>
       <c r="BA48" t="n">
         <v>1.46</v>
@@ -11534,19 +11534,19 @@
         <v>8.24</v>
       </c>
       <c r="BC48" t="n">
-        <v>56.74</v>
+        <v>56.06</v>
       </c>
       <c r="BD48" t="n">
-        <v>27.98</v>
+        <v>27.43</v>
       </c>
       <c r="BE48" t="n">
         <v>30.83</v>
       </c>
       <c r="BF48" t="n">
-        <v>-84.09999999999999</v>
+        <v>-84.16</v>
       </c>
       <c r="BG48" t="n">
-        <v>-10.18</v>
+        <v>-10.57</v>
       </c>
       <c r="BH48" t="n">
         <v>7.23</v>
@@ -11555,7 +11555,7 @@
         <v>0</v>
       </c>
       <c r="BJ48" t="n">
-        <v>9.17</v>
+        <v>9.210000000000001</v>
       </c>
       <c r="BK48" t="n">
         <v>1.27</v>
@@ -11564,28 +11564,28 @@
         <v>1.28</v>
       </c>
       <c r="BM48" t="n">
-        <v>9.369999999999999</v>
+        <v>9.5</v>
       </c>
       <c r="BN48" t="n">
-        <v>9.48</v>
+        <v>9.5</v>
       </c>
       <c r="BO48" t="n">
+        <v>7.13</v>
+      </c>
+      <c r="BP48" t="n">
+        <v>9.17</v>
+      </c>
+      <c r="BQ48" t="n">
         <v>7.18</v>
       </c>
-      <c r="BP48" t="n">
-        <v>9.140000000000001</v>
-      </c>
-      <c r="BQ48" t="n">
-        <v>7.15</v>
-      </c>
       <c r="BR48" t="n">
-        <v>9.369999999999999</v>
+        <v>9.5</v>
       </c>
       <c r="BS48" t="n">
         <v>0.54</v>
       </c>
       <c r="BT48" t="n">
-        <v>2693</v>
+        <v>2677</v>
       </c>
     </row>
     <row r="49">
@@ -11615,10 +11615,10 @@
         </is>
       </c>
       <c r="F49" t="n">
-        <v>48.07</v>
+        <v>47.39</v>
       </c>
       <c r="G49" t="n">
-        <v>948313300</v>
+        <v>934898060</v>
       </c>
       <c r="H49" t="n">
         <v>200</v>
@@ -11636,7 +11636,7 @@
         <v>1.09</v>
       </c>
       <c r="M49" t="n">
-        <v>0.9593963337672996</v>
+        <v>0.9458243084961065</v>
       </c>
       <c r="N49" t="n">
         <v>0.08</v>
@@ -11714,7 +11714,7 @@
         <v>84709985.8</v>
       </c>
       <c r="AM49" t="n">
-        <v>237078325</v>
+        <v>233724515</v>
       </c>
       <c r="AN49" t="n">
         <v>3.3186</v>
@@ -11755,7 +11755,7 @@
         <v>68.48999999999999</v>
       </c>
       <c r="AZ49" t="n">
-        <v>57.36</v>
+        <v>56.55</v>
       </c>
       <c r="BA49" t="n">
         <v>9.210000000000001</v>
@@ -11764,19 +11764,19 @@
         <v>27.75</v>
       </c>
       <c r="BC49" t="n">
-        <v>74.48999999999999</v>
+        <v>76.98999999999999</v>
       </c>
       <c r="BD49" t="n">
-        <v>42.47</v>
+        <v>44.51</v>
       </c>
       <c r="BE49" t="n">
         <v>19.33</v>
       </c>
       <c r="BF49" t="n">
-        <v>-80.83</v>
+        <v>-80.56</v>
       </c>
       <c r="BG49" t="n">
-        <v>-42.26</v>
+        <v>-41.43</v>
       </c>
       <c r="BH49" t="n">
         <v>42.6</v>
@@ -11785,7 +11785,7 @@
         <v>0</v>
       </c>
       <c r="BJ49" t="n">
-        <v>48.07</v>
+        <v>47.39</v>
       </c>
       <c r="BK49" t="n">
         <v>7.34</v>
@@ -11803,10 +11803,10 @@
         <v>28.48</v>
       </c>
       <c r="BP49" t="n">
-        <v>48.07</v>
+        <v>47.39</v>
       </c>
       <c r="BQ49" t="n">
-        <v>6.32</v>
+        <v>6.23</v>
       </c>
       <c r="BR49" t="n">
         <v>48.07</v>
@@ -11815,7 +11815,7 @@
         <v>0.54</v>
       </c>
       <c r="BT49" t="n">
-        <v>370</v>
+        <v>377</v>
       </c>
     </row>
     <row r="50">
@@ -11845,13 +11845,13 @@
         </is>
       </c>
       <c r="F50" t="n">
-        <v>34.1</v>
+        <v>34.01</v>
       </c>
       <c r="G50" t="n">
-        <v>948313300</v>
+        <v>934898060</v>
       </c>
       <c r="H50" t="n">
-        <v>400</v>
+        <v>1400</v>
       </c>
       <c r="I50" t="n">
         <v>11540870</v>
@@ -11866,7 +11866,7 @@
         <v>0.8</v>
       </c>
       <c r="M50" t="n">
-        <v>0.9593963337672996</v>
+        <v>0.9458243084961065</v>
       </c>
       <c r="N50" t="n">
         <v>0.06</v>
@@ -11944,7 +11944,7 @@
         <v>84709985.8</v>
       </c>
       <c r="AM50" t="n">
-        <v>323656416.3822525</v>
+        <v>319077836.1774744</v>
       </c>
       <c r="AN50" t="n">
         <v>4.4983</v>
@@ -11985,7 +11985,7 @@
         <v>68.48999999999999</v>
       </c>
       <c r="AZ50" t="n">
-        <v>75.19</v>
+        <v>74.98999999999999</v>
       </c>
       <c r="BA50" t="n">
         <v>9.210000000000001</v>
@@ -11994,19 +11994,19 @@
         <v>30.53</v>
       </c>
       <c r="BC50" t="n">
-        <v>145.97</v>
+        <v>146.63</v>
       </c>
       <c r="BD50" t="n">
-        <v>100.84</v>
+        <v>101.37</v>
       </c>
       <c r="BE50" t="n">
         <v>120.5</v>
       </c>
       <c r="BF50" t="n">
-        <v>-72.98</v>
+        <v>-72.91</v>
       </c>
       <c r="BG50" t="n">
-        <v>-10.47</v>
+        <v>-10.23</v>
       </c>
       <c r="BH50" t="n">
         <v>42.6</v>
@@ -12015,7 +12015,7 @@
         <v>0</v>
       </c>
       <c r="BJ50" t="n">
-        <v>34.1</v>
+        <v>34.01</v>
       </c>
       <c r="BK50" t="n">
         <v>7.34</v>
@@ -12024,28 +12024,28 @@
         <v>7.6</v>
       </c>
       <c r="BM50" t="n">
-        <v>34.13</v>
+        <v>34.69</v>
       </c>
       <c r="BN50" t="n">
         <v>39.22</v>
       </c>
       <c r="BO50" t="n">
-        <v>23.95</v>
+        <v>24.24</v>
       </c>
       <c r="BP50" t="n">
-        <v>33.63</v>
+        <v>33.14</v>
       </c>
       <c r="BQ50" t="n">
-        <v>4.49</v>
+        <v>4.47</v>
       </c>
       <c r="BR50" t="n">
-        <v>33.64</v>
+        <v>33.14</v>
       </c>
       <c r="BS50" t="n">
         <v>0.4</v>
       </c>
       <c r="BT50" t="n">
-        <v>490</v>
+        <v>483</v>
       </c>
     </row>
     <row r="51">
@@ -12523,13 +12523,13 @@
         </is>
       </c>
       <c r="F53" t="n">
-        <v>6.45</v>
+        <v>6.44</v>
       </c>
       <c r="G53" t="n">
-        <v>882697953</v>
+        <v>881329463</v>
       </c>
       <c r="H53" t="n">
-        <v>57300</v>
+        <v>88100</v>
       </c>
       <c r="I53" t="n">
         <v>136852484</v>
@@ -12544,7 +12544,7 @@
         <v>2.79</v>
       </c>
       <c r="M53" t="n">
-        <v>2.293084729260188</v>
+        <v>2.289529647354219</v>
       </c>
       <c r="N53" t="n">
         <v>1.48</v>
@@ -12622,7 +12622,7 @@
         <v>39687220.36</v>
       </c>
       <c r="AM53" t="n">
-        <v>44966783.138054</v>
+        <v>44897068.92511462</v>
       </c>
       <c r="AN53" t="n">
         <v>0</v>
@@ -12672,10 +12672,10 @@
         <v>0</v>
       </c>
       <c r="BC53" t="n">
-        <v>-38.9</v>
+        <v>-38.81</v>
       </c>
       <c r="BD53" t="n">
-        <v>-50.11</v>
+        <v>-50.04</v>
       </c>
       <c r="BE53" t="n">
         <v>-100</v>
@@ -12693,7 +12693,7 @@
         <v>0</v>
       </c>
       <c r="BJ53" t="n">
-        <v>6.45</v>
+        <v>6.44</v>
       </c>
       <c r="BK53" t="n">
         <v>0.29</v>
@@ -12702,7 +12702,7 @@
         <v>0.2</v>
       </c>
       <c r="BM53" t="n">
-        <v>6.45</v>
+        <v>7.4</v>
       </c>
       <c r="BN53" t="n">
         <v>10.39</v>
@@ -12711,19 +12711,19 @@
         <v>4.82</v>
       </c>
       <c r="BP53" t="n">
-        <v>5.96</v>
+        <v>6.33</v>
       </c>
       <c r="BQ53" t="n">
-        <v>31.68</v>
+        <v>31.63</v>
       </c>
       <c r="BR53" t="n">
-        <v>6.12</v>
+        <v>6.56</v>
       </c>
       <c r="BS53" t="n">
         <v>2.36</v>
       </c>
       <c r="BT53" t="n">
-        <v>37073</v>
+        <v>38407</v>
       </c>
     </row>
     <row r="54">
@@ -12753,13 +12753,13 @@
         </is>
       </c>
       <c r="F54" t="n">
-        <v>10.82</v>
+        <v>11.68</v>
       </c>
       <c r="G54" t="n">
-        <v>2535156224</v>
+        <v>2723917399</v>
       </c>
       <c r="H54" t="n">
-        <v>334700</v>
+        <v>784000</v>
       </c>
       <c r="I54" t="n">
         <v>233212121</v>
@@ -12774,7 +12774,7 @@
         <v>0.97</v>
       </c>
       <c r="M54" t="n">
-        <v>1.42296184391548</v>
+        <v>1.528911902178103</v>
       </c>
       <c r="N54" t="n">
         <v>0.5600000000000001</v>
@@ -12852,7 +12852,7 @@
         <v>233212121</v>
       </c>
       <c r="AM54" t="n">
-        <v>346806596.9904241</v>
+        <v>372628919.1518468</v>
       </c>
       <c r="AN54" t="n">
         <v>0.1531</v>
@@ -12893,7 +12893,7 @@
         <v>12.25</v>
       </c>
       <c r="AZ54" t="n">
-        <v>17.22</v>
+        <v>18.59</v>
       </c>
       <c r="BA54" t="n">
         <v>0.98</v>
@@ -12902,19 +12902,19 @@
         <v>6.52</v>
       </c>
       <c r="BC54" t="n">
-        <v>38.7</v>
+        <v>28.49</v>
       </c>
       <c r="BD54" t="n">
-        <v>13.25</v>
+        <v>4.91</v>
       </c>
       <c r="BE54" t="n">
         <v>59.17</v>
       </c>
       <c r="BF54" t="n">
-        <v>-90.91</v>
+        <v>-91.58</v>
       </c>
       <c r="BG54" t="n">
-        <v>-39.77</v>
+        <v>-44.21</v>
       </c>
       <c r="BH54" t="n">
         <v>10.01</v>
@@ -12923,7 +12923,7 @@
         <v>0</v>
       </c>
       <c r="BJ54" t="n">
-        <v>10.82</v>
+        <v>11.68</v>
       </c>
       <c r="BK54" t="n">
         <v>1</v>
@@ -12932,28 +12932,28 @@
         <v>1</v>
       </c>
       <c r="BM54" t="n">
-        <v>10.9</v>
+        <v>11.95</v>
       </c>
       <c r="BN54" t="n">
-        <v>11.68</v>
+        <v>11.95</v>
       </c>
       <c r="BO54" t="n">
         <v>8.23</v>
       </c>
       <c r="BP54" t="n">
-        <v>10.67</v>
+        <v>11.05</v>
       </c>
       <c r="BQ54" t="n">
-        <v>10.79</v>
+        <v>11.65</v>
       </c>
       <c r="BR54" t="n">
-        <v>10.8</v>
+        <v>11.05</v>
       </c>
       <c r="BS54" t="n">
         <v>1.26</v>
       </c>
       <c r="BT54" t="n">
-        <v>243630</v>
+        <v>248483</v>
       </c>
     </row>
     <row r="55">
@@ -12983,13 +12983,13 @@
         </is>
       </c>
       <c r="F55" t="n">
-        <v>50.79</v>
+        <v>55</v>
       </c>
       <c r="G55" t="n">
-        <v>6696691718</v>
+        <v>7324848245</v>
       </c>
       <c r="H55" t="n">
-        <v>4100</v>
+        <v>16200</v>
       </c>
       <c r="I55" t="n">
         <v>84052790</v>
@@ -13004,7 +13004,7 @@
         <v>2</v>
       </c>
       <c r="M55" t="n">
-        <v>1.033776058049382</v>
+        <v>1.130745308787714</v>
       </c>
       <c r="N55" t="n">
         <v>0.16</v>
@@ -13082,7 +13082,7 @@
         <v>579123723.1</v>
       </c>
       <c r="AM55" t="n">
-        <v>336855720.221328</v>
+        <v>368453131.0362173</v>
       </c>
       <c r="AN55" t="n">
         <v>3.1953</v>
@@ -13123,7 +13123,7 @@
         <v>51.21</v>
       </c>
       <c r="AZ55" t="n">
-        <v>53.41</v>
+        <v>57.84</v>
       </c>
       <c r="BA55" t="n">
         <v>9.380000000000001</v>
@@ -13132,19 +13132,19 @@
         <v>16.08</v>
       </c>
       <c r="BC55" t="n">
-        <v>23.48</v>
+        <v>14.02</v>
       </c>
       <c r="BD55" t="n">
-        <v>0.82</v>
+        <v>-6.9</v>
       </c>
       <c r="BE55" t="n">
         <v>5.17</v>
       </c>
       <c r="BF55" t="n">
-        <v>-81.54000000000001</v>
+        <v>-82.95</v>
       </c>
       <c r="BG55" t="n">
-        <v>-68.34999999999999</v>
+        <v>-70.77</v>
       </c>
       <c r="BH55" t="n">
         <v>25.37</v>
@@ -13153,7 +13153,7 @@
         <v>0</v>
       </c>
       <c r="BJ55" t="n">
-        <v>50.79</v>
+        <v>55</v>
       </c>
       <c r="BK55" t="n">
         <v>6.89</v>
@@ -13162,7 +13162,7 @@
         <v>7.03</v>
       </c>
       <c r="BM55" t="n">
-        <v>50.79</v>
+        <v>55</v>
       </c>
       <c r="BN55" t="n">
         <v>73.67</v>
@@ -13171,19 +13171,19 @@
         <v>35.58</v>
       </c>
       <c r="BP55" t="n">
-        <v>49.98</v>
+        <v>51.21</v>
       </c>
       <c r="BQ55" t="n">
-        <v>7.22</v>
+        <v>7.82</v>
       </c>
       <c r="BR55" t="n">
-        <v>49.98</v>
+        <v>51.21</v>
       </c>
       <c r="BS55" t="n">
         <v>0.66</v>
       </c>
       <c r="BT55" t="n">
-        <v>5920</v>
+        <v>5950</v>
       </c>
     </row>
     <row r="56">
@@ -13213,13 +13213,13 @@
         </is>
       </c>
       <c r="F56" t="n">
-        <v>60.92</v>
+        <v>66.73999999999999</v>
       </c>
       <c r="G56" t="n">
-        <v>6696691718</v>
+        <v>7324848245</v>
       </c>
       <c r="H56" t="n">
-        <v>52300</v>
+        <v>45500</v>
       </c>
       <c r="I56" t="n">
         <v>39675836</v>
@@ -13234,7 +13234,7 @@
         <v>2.41</v>
       </c>
       <c r="M56" t="n">
-        <v>2.190042370228885</v>
+        <v>2.395470582724933</v>
       </c>
       <c r="N56" t="n">
         <v>0.19</v>
@@ -13312,7 +13312,7 @@
         <v>273366510.04</v>
       </c>
       <c r="AM56" t="n">
-        <v>278564547.3377704</v>
+        <v>304694186.5640599</v>
       </c>
       <c r="AN56" t="n">
         <v>3.5102</v>
@@ -13353,7 +13353,7 @@
         <v>51.21</v>
       </c>
       <c r="AZ56" t="n">
-        <v>58.18</v>
+        <v>63.74</v>
       </c>
       <c r="BA56" t="n">
         <v>9.380000000000001</v>
@@ -13362,19 +13362,19 @@
         <v>17.68</v>
       </c>
       <c r="BC56" t="n">
-        <v>2.94</v>
+        <v>-6.03</v>
       </c>
       <c r="BD56" t="n">
-        <v>-15.95</v>
+        <v>-23.28</v>
       </c>
       <c r="BE56" t="n">
         <v>-4.5</v>
       </c>
       <c r="BF56" t="n">
-        <v>-84.61</v>
+        <v>-85.95</v>
       </c>
       <c r="BG56" t="n">
-        <v>-70.98</v>
+        <v>-73.51000000000001</v>
       </c>
       <c r="BH56" t="n">
         <v>25.37</v>
@@ -13383,7 +13383,7 @@
         <v>0</v>
       </c>
       <c r="BJ56" t="n">
-        <v>60.92</v>
+        <v>66.73999999999999</v>
       </c>
       <c r="BK56" t="n">
         <v>6.89</v>
@@ -13392,7 +13392,7 @@
         <v>7.03</v>
       </c>
       <c r="BM56" t="n">
-        <v>61.3</v>
+        <v>68.5</v>
       </c>
       <c r="BN56" t="n">
         <v>86.77</v>
@@ -13401,19 +13401,19 @@
         <v>46.42</v>
       </c>
       <c r="BP56" t="n">
-        <v>58.71</v>
+        <v>61.78</v>
       </c>
       <c r="BQ56" t="n">
-        <v>8.66</v>
+        <v>9.49</v>
       </c>
       <c r="BR56" t="n">
-        <v>58.71</v>
+        <v>61.78</v>
       </c>
       <c r="BS56" t="n">
         <v>0.79</v>
       </c>
       <c r="BT56" t="n">
-        <v>28133</v>
+        <v>28753</v>
       </c>
     </row>
     <row r="57">
@@ -13443,13 +13443,13 @@
         </is>
       </c>
       <c r="F57" t="n">
-        <v>6.59</v>
+        <v>6.9</v>
       </c>
       <c r="G57" t="n">
-        <v>1543495337</v>
+        <v>1613620912</v>
       </c>
       <c r="H57" t="n">
-        <v>2831000</v>
+        <v>3624100</v>
       </c>
       <c r="I57" t="n">
         <v>233858065</v>
@@ -13464,7 +13464,7 @@
         <v>0.77</v>
       </c>
       <c r="M57" t="n">
-        <v>0.4620096107867822</v>
+        <v>0.4830000788726274</v>
       </c>
       <c r="N57" t="n">
         <v>0.08</v>
@@ -13542,7 +13542,7 @@
         <v>229180903.7</v>
       </c>
       <c r="AM57" t="n">
-        <v>115444677.4121167</v>
+        <v>120689671.802543</v>
       </c>
       <c r="AN57" t="n">
         <v>0.347</v>
@@ -13583,7 +13583,7 @@
         <v>10.72</v>
       </c>
       <c r="AZ57" t="n">
-        <v>10.05</v>
+        <v>10.52</v>
       </c>
       <c r="BA57" t="n">
         <v>1.13</v>
@@ -13592,19 +13592,19 @@
         <v>6.26</v>
       </c>
       <c r="BC57" t="n">
-        <v>99.26000000000001</v>
+        <v>90.31</v>
       </c>
       <c r="BD57" t="n">
-        <v>62.7</v>
+        <v>55.39</v>
       </c>
       <c r="BE57" t="n">
         <v>52.5</v>
       </c>
       <c r="BF57" t="n">
-        <v>-82.89</v>
+        <v>-83.66</v>
       </c>
       <c r="BG57" t="n">
-        <v>-4.95</v>
+        <v>-9.220000000000001</v>
       </c>
       <c r="BH57" t="n">
         <v>7.82</v>
@@ -13613,7 +13613,7 @@
         <v>0</v>
       </c>
       <c r="BJ57" t="n">
-        <v>6.59</v>
+        <v>6.9</v>
       </c>
       <c r="BK57" t="n">
         <v>0.98</v>
@@ -13622,28 +13622,28 @@
         <v>1.04</v>
       </c>
       <c r="BM57" t="n">
-        <v>6.63</v>
+        <v>7.03</v>
       </c>
       <c r="BN57" t="n">
-        <v>6.63</v>
+        <v>7.03</v>
       </c>
       <c r="BO57" t="n">
         <v>3.43</v>
       </c>
       <c r="BP57" t="n">
-        <v>6.47</v>
+        <v>6.64</v>
       </c>
       <c r="BQ57" t="n">
-        <v>6.36</v>
+        <v>6.66</v>
       </c>
       <c r="BR57" t="n">
-        <v>6.52</v>
+        <v>6.64</v>
       </c>
       <c r="BS57" t="n">
         <v>0.42</v>
       </c>
       <c r="BT57" t="n">
-        <v>1422917</v>
+        <v>1490457</v>
       </c>
     </row>
     <row r="58">
@@ -13676,10 +13676,10 @@
         <v>19.5</v>
       </c>
       <c r="G58" t="n">
-        <v>91920055</v>
+        <v>94766022</v>
       </c>
       <c r="H58" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="I58" t="n">
         <v>4115057</v>
@@ -13694,7 +13694,7 @@
         <v>0.63</v>
       </c>
       <c r="M58" t="n">
-        <v>1.685005568619992</v>
+        <v>1.737175579213532</v>
       </c>
       <c r="N58" t="n">
         <v>0.16</v>
@@ -13772,7 +13772,7 @@
         <v>10904901.05</v>
       </c>
       <c r="AM58" t="n">
-        <v>14995115.00815661</v>
+        <v>15459383.6867863</v>
       </c>
       <c r="AN58" t="n">
         <v>0.5117</v>
@@ -13873,7 +13873,7 @@
         <v>1.47</v>
       </c>
       <c r="BT58" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="59">
@@ -14136,10 +14136,10 @@
         <v>377</v>
       </c>
       <c r="G60" t="n">
-        <v>171440800</v>
+        <v>171440787</v>
       </c>
       <c r="H60" t="n">
-        <v>28</v>
+        <v>51</v>
       </c>
       <c r="I60" t="n">
         <v>454750</v>
@@ -14154,7 +14154,7 @@
         <v>0.83</v>
       </c>
       <c r="M60" t="n">
-        <v>12.82353050178348</v>
+        <v>12.82352952940177</v>
       </c>
       <c r="N60" t="n">
         <v>0.68</v>
@@ -14232,7 +14232,7 @@
         <v>59558607.5</v>
       </c>
       <c r="AM60" t="n">
-        <v>-25137947.21407625</v>
+        <v>-25137945.30791789</v>
       </c>
       <c r="AN60" t="n">
         <v>10.0581</v>
@@ -14312,7 +14312,7 @@
         <v>130.97</v>
       </c>
       <c r="BM60" t="n">
-        <v>378</v>
+        <v>390</v>
       </c>
       <c r="BN60" t="n">
         <v>405</v>
@@ -14321,13 +14321,13 @@
         <v>309.24</v>
       </c>
       <c r="BP60" t="n">
-        <v>369.23</v>
+        <v>375</v>
       </c>
       <c r="BQ60" t="n">
         <v>2.88</v>
       </c>
       <c r="BR60" t="n">
-        <v>378</v>
+        <v>375</v>
       </c>
       <c r="BS60" t="n">
         <v>12.82</v>
@@ -14363,13 +14363,13 @@
         </is>
       </c>
       <c r="F61" t="n">
-        <v>28.34</v>
+        <v>30.53</v>
       </c>
       <c r="G61" t="n">
-        <v>2420924675</v>
+        <v>2613624205</v>
       </c>
       <c r="H61" t="n">
-        <v>624300</v>
+        <v>2032400</v>
       </c>
       <c r="I61" t="n">
         <v>85608392</v>
@@ -14384,7 +14384,7 @@
         <v>2.37</v>
       </c>
       <c r="M61" t="n">
-        <v>1.283899474122249</v>
+        <v>1.386094650942694</v>
       </c>
       <c r="N61" t="n">
         <v>1.1</v>
@@ -14462,7 +14462,7 @@
         <v>160087693.04</v>
       </c>
       <c r="AM61" t="n">
-        <v>190025484.6938775</v>
+        <v>205151036.4992151</v>
       </c>
       <c r="AN61" t="n">
         <v>0.38</v>
@@ -14503,7 +14503,7 @@
         <v>17.56</v>
       </c>
       <c r="AZ61" t="n">
-        <v>35.71</v>
+        <v>38.47</v>
       </c>
       <c r="BA61" t="n">
         <v>2.52</v>
@@ -14512,19 +14512,19 @@
         <v>11.76</v>
       </c>
       <c r="BC61" t="n">
-        <v>-24.12</v>
+        <v>-29.57</v>
       </c>
       <c r="BD61" t="n">
-        <v>-38.05</v>
+        <v>-42.49</v>
       </c>
       <c r="BE61" t="n">
         <v>26</v>
       </c>
       <c r="BF61" t="n">
-        <v>-91.09999999999999</v>
+        <v>-91.73999999999999</v>
       </c>
       <c r="BG61" t="n">
-        <v>-58.52</v>
+        <v>-61.49</v>
       </c>
       <c r="BH61" t="n">
         <v>10.99</v>
@@ -14533,7 +14533,7 @@
         <v>0</v>
       </c>
       <c r="BJ61" t="n">
-        <v>28.34</v>
+        <v>30.53</v>
       </c>
       <c r="BK61" t="n">
         <v>1.87</v>
@@ -14542,28 +14542,28 @@
         <v>1.86</v>
       </c>
       <c r="BM61" t="n">
-        <v>28.35</v>
+        <v>30.75</v>
       </c>
       <c r="BN61" t="n">
-        <v>28.68</v>
+        <v>30.75</v>
       </c>
       <c r="BO61" t="n">
         <v>19.35</v>
       </c>
       <c r="BP61" t="n">
-        <v>27.65</v>
+        <v>28.82</v>
       </c>
       <c r="BQ61" t="n">
-        <v>15.22</v>
+        <v>16.4</v>
       </c>
       <c r="BR61" t="n">
-        <v>28.35</v>
+        <v>28.82</v>
       </c>
       <c r="BS61" t="n">
         <v>1.19</v>
       </c>
       <c r="BT61" t="n">
-        <v>700600</v>
+        <v>705237</v>
       </c>
     </row>
     <row r="62">
@@ -14593,13 +14593,13 @@
         </is>
       </c>
       <c r="F62" t="n">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G62" t="n">
-        <v>11054370000</v>
+        <v>11251769220</v>
       </c>
       <c r="H62" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="I62" t="n">
         <v>98699749</v>
@@ -14614,7 +14614,7 @@
         <v>0.64</v>
       </c>
       <c r="M62" t="n">
-        <v>1.036220295462617</v>
+        <v>1.054724206411182</v>
       </c>
       <c r="N62" t="n">
         <v>0.13</v>
@@ -14692,7 +14692,7 @@
         <v>2757670987.06</v>
       </c>
       <c r="AM62" t="n">
-        <v>4475453441.295547</v>
+        <v>4555372153.846153</v>
       </c>
       <c r="AN62" t="n">
         <v>6.9319</v>
@@ -14733,7 +14733,7 @@
         <v>267.2</v>
       </c>
       <c r="AZ62" t="n">
-        <v>118.35</v>
+        <v>120.46</v>
       </c>
       <c r="BA62" t="n">
         <v>34.09</v>
@@ -14742,19 +14742,19 @@
         <v>76.01000000000001</v>
       </c>
       <c r="BC62" t="n">
-        <v>192.18</v>
+        <v>187.06</v>
       </c>
       <c r="BD62" t="n">
-        <v>138.57</v>
+        <v>134.38</v>
       </c>
       <c r="BE62" t="n">
         <v>5.67</v>
       </c>
       <c r="BF62" t="n">
-        <v>-69.56</v>
+        <v>-70.09</v>
       </c>
       <c r="BG62" t="n">
-        <v>-32.14</v>
+        <v>-33.33</v>
       </c>
       <c r="BH62" t="n">
         <v>170.35</v>
@@ -14763,7 +14763,7 @@
         <v>0</v>
       </c>
       <c r="BJ62" t="n">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="BK62" t="n">
         <v>27.94</v>
@@ -14772,7 +14772,7 @@
         <v>32.73</v>
       </c>
       <c r="BM62" t="n">
-        <v>112</v>
+        <v>114.45</v>
       </c>
       <c r="BN62" t="n">
         <v>122.2</v>
@@ -14781,19 +14781,19 @@
         <v>91.84999999999999</v>
       </c>
       <c r="BP62" t="n">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="BQ62" t="n">
-        <v>3.42</v>
+        <v>3.48</v>
       </c>
       <c r="BR62" t="n">
-        <v>112</v>
+        <v>114.45</v>
       </c>
       <c r="BS62" t="n">
         <v>1.01</v>
       </c>
       <c r="BT62" t="n">
-        <v>117</v>
+        <v>120</v>
       </c>
     </row>
     <row r="63">
@@ -14823,13 +14823,13 @@
         </is>
       </c>
       <c r="F63" t="n">
-        <v>1.6</v>
+        <v>1.56</v>
       </c>
       <c r="G63" t="n">
-        <v>416815600</v>
+        <v>406395117</v>
       </c>
       <c r="H63" t="n">
-        <v>85800</v>
+        <v>11600</v>
       </c>
       <c r="I63" t="n">
         <v>122894462</v>
@@ -14844,7 +14844,7 @@
         <v>-0.22</v>
       </c>
       <c r="M63" t="n">
-        <v>0.5126616777648051</v>
+        <v>0.4998450214354843</v>
       </c>
       <c r="N63" t="n">
         <v>0.37</v>
@@ -14922,7 +14922,7 @@
         <v>31952560.12</v>
       </c>
       <c r="AM63" t="n">
-        <v>236827045.4545455</v>
+        <v>230906316.4772727</v>
       </c>
       <c r="AN63" t="n">
         <v>0</v>
@@ -14981,7 +14981,7 @@
         <v>-100</v>
       </c>
       <c r="BF63" t="n">
-        <v>-81.93000000000001</v>
+        <v>-81.45999999999999</v>
       </c>
       <c r="BG63" t="n">
         <v>-100</v>
@@ -14993,7 +14993,7 @@
         <v>0</v>
       </c>
       <c r="BJ63" t="n">
-        <v>1.6</v>
+        <v>1.56</v>
       </c>
       <c r="BK63" t="n">
         <v>0.26</v>
@@ -15002,7 +15002,7 @@
         <v>0.26</v>
       </c>
       <c r="BM63" t="n">
-        <v>1.7</v>
+        <v>1.68</v>
       </c>
       <c r="BN63" t="n">
         <v>2.12</v>
@@ -15011,19 +15011,19 @@
         <v>1.16</v>
       </c>
       <c r="BP63" t="n">
-        <v>1.59</v>
+        <v>1.52</v>
       </c>
       <c r="BQ63" t="n">
-        <v>6.13</v>
+        <v>5.98</v>
       </c>
       <c r="BR63" t="n">
-        <v>1.59</v>
+        <v>1.56</v>
       </c>
       <c r="BS63" t="n">
         <v>0.19</v>
       </c>
       <c r="BT63" t="n">
-        <v>31417</v>
+        <v>33890</v>
       </c>
     </row>
     <row r="64">
@@ -15053,13 +15053,13 @@
         </is>
       </c>
       <c r="F64" t="n">
-        <v>66.02</v>
+        <v>80.89</v>
       </c>
       <c r="G64" t="n">
-        <v>250357994349</v>
+        <v>299780602658</v>
       </c>
       <c r="H64" t="n">
-        <v>14513200</v>
+        <v>61965300</v>
       </c>
       <c r="I64" t="n">
         <v>0</v>
@@ -15146,13 +15146,13 @@
         <v>41.22</v>
       </c>
       <c r="AK64" t="n">
-        <v>71781310776.05635</v>
+        <v>85951497814.08733</v>
       </c>
       <c r="AL64" t="n">
-        <v>20012629444.36451</v>
+        <v>23963277590.56755</v>
       </c>
       <c r="AM64" t="n">
-        <v>22293677145.94835</v>
+        <v>26694621786.10863</v>
       </c>
       <c r="AN64" t="n">
         <v>1.4201</v>
@@ -15193,7 +15193,7 @@
         <v>38.98</v>
       </c>
       <c r="AZ64" t="n">
-        <v>26.41</v>
+        <v>32.36</v>
       </c>
       <c r="BA64" t="n">
         <v>6.69</v>
@@ -15202,19 +15202,19 @@
         <v>10.4</v>
       </c>
       <c r="BC64" t="n">
-        <v>-27.69</v>
+        <v>-40.98</v>
       </c>
       <c r="BD64" t="n">
-        <v>-40.96</v>
+        <v>-51.81</v>
       </c>
       <c r="BE64" t="n">
         <v>-60</v>
       </c>
       <c r="BF64" t="n">
-        <v>-89.86</v>
+        <v>-91.72</v>
       </c>
       <c r="BG64" t="n">
-        <v>-84.25</v>
+        <v>-87.15000000000001</v>
       </c>
       <c r="BH64" t="n">
         <v>21.37</v>
@@ -15223,7 +15223,7 @@
         <v>0</v>
       </c>
       <c r="BJ64" t="n">
-        <v>66.02</v>
+        <v>80.89</v>
       </c>
       <c r="BK64" t="n">
         <v>4.74</v>
@@ -15232,28 +15232,28 @@
         <v>1.57</v>
       </c>
       <c r="BM64" t="n">
-        <v>66.02</v>
+        <v>84.59</v>
       </c>
       <c r="BN64" t="n">
-        <v>66.02</v>
+        <v>84.59</v>
       </c>
       <c r="BO64" t="n">
         <v>44.12</v>
       </c>
       <c r="BP64" t="n">
-        <v>63.15</v>
+        <v>75.40000000000001</v>
       </c>
       <c r="BQ64" t="n">
-        <v>42.05</v>
+        <v>51.52</v>
       </c>
       <c r="BR64" t="n">
-        <v>65.45</v>
+        <v>76</v>
       </c>
       <c r="BS64" t="n">
         <v>3.49</v>
       </c>
       <c r="BT64" t="n">
-        <v>10434673</v>
+        <v>10726917</v>
       </c>
     </row>
     <row r="65">
@@ -15283,13 +15283,13 @@
         </is>
       </c>
       <c r="F65" t="n">
-        <v>24.97</v>
+        <v>27.71</v>
       </c>
       <c r="G65" t="n">
-        <v>250357994349</v>
+        <v>299780602658</v>
       </c>
       <c r="H65" t="n">
-        <v>6700</v>
+        <v>64500</v>
       </c>
       <c r="I65" t="n">
         <v>7298813414</v>
@@ -15304,7 +15304,7 @@
         <v>3.29</v>
       </c>
       <c r="M65" t="n">
-        <v>6.052640571409224</v>
+        <v>7.247478726962274</v>
       </c>
       <c r="N65" t="n">
         <v>0.29</v>
@@ -15382,7 +15382,7 @@
         <v>11532125194.12</v>
       </c>
       <c r="AM65" t="n">
-        <v>18753407816.4045</v>
+        <v>22455475854.53184</v>
       </c>
       <c r="AN65" t="n">
         <v>0.4734</v>
@@ -15423,7 +15423,7 @@
         <v>12.99</v>
       </c>
       <c r="AZ65" t="n">
-        <v>8.41</v>
+        <v>9.33</v>
       </c>
       <c r="BA65" t="n">
         <v>2.23</v>
@@ -15432,19 +15432,19 @@
         <v>3.47</v>
       </c>
       <c r="BC65" t="n">
-        <v>-36.29</v>
+        <v>-42.59</v>
       </c>
       <c r="BD65" t="n">
-        <v>-47.98</v>
+        <v>-53.12</v>
       </c>
       <c r="BE65" t="n">
         <v>-66.33</v>
       </c>
       <c r="BF65" t="n">
-        <v>-91.06</v>
+        <v>-91.95</v>
       </c>
       <c r="BG65" t="n">
-        <v>-86.12</v>
+        <v>-87.48999999999999</v>
       </c>
       <c r="BH65" t="n">
         <v>7.12</v>
@@ -15453,7 +15453,7 @@
         <v>0</v>
       </c>
       <c r="BJ65" t="n">
-        <v>24.97</v>
+        <v>27.71</v>
       </c>
       <c r="BK65" t="n">
         <v>1.58</v>
@@ -15462,7 +15462,7 @@
         <v>1.57</v>
       </c>
       <c r="BM65" t="n">
-        <v>25.2</v>
+        <v>28.5</v>
       </c>
       <c r="BN65" t="n">
         <v>46.43</v>
@@ -15471,19 +15471,19 @@
         <v>20.44</v>
       </c>
       <c r="BP65" t="n">
-        <v>24.69</v>
+        <v>26.11</v>
       </c>
       <c r="BQ65" t="n">
-        <v>15.9</v>
+        <v>17.65</v>
       </c>
       <c r="BR65" t="n">
-        <v>25</v>
+        <v>26.11</v>
       </c>
       <c r="BS65" t="n">
         <v>4.14</v>
       </c>
       <c r="BT65" t="n">
-        <v>7647</v>
+        <v>7650</v>
       </c>
     </row>
     <row r="66">
@@ -15513,13 +15513,13 @@
         </is>
       </c>
       <c r="F66" t="n">
-        <v>20.99</v>
+        <v>25.31</v>
       </c>
       <c r="G66" t="n">
-        <v>250357994349</v>
+        <v>299780602658</v>
       </c>
       <c r="H66" t="n">
-        <v>5500</v>
+        <v>24000</v>
       </c>
       <c r="I66" t="n">
         <v>2972355254</v>
@@ -15534,7 +15534,7 @@
         <v>2.75</v>
       </c>
       <c r="M66" t="n">
-        <v>14.86265618259178</v>
+        <v>17.79665969565557</v>
       </c>
       <c r="N66" t="n">
         <v>0.25</v>
@@ -15612,7 +15612,7 @@
         <v>4696321301.320001</v>
       </c>
       <c r="AM66" t="n">
-        <v>22453631780.17937</v>
+        <v>26886152704.75336</v>
       </c>
       <c r="AN66" t="n">
         <v>0.4734</v>
@@ -15653,7 +15653,7 @@
         <v>12.99</v>
       </c>
       <c r="AZ66" t="n">
-        <v>8.43</v>
+        <v>10.17</v>
       </c>
       <c r="BA66" t="n">
         <v>2.23</v>
@@ -15662,19 +15662,19 @@
         <v>3.47</v>
       </c>
       <c r="BC66" t="n">
-        <v>-24.2</v>
+        <v>-37.14</v>
       </c>
       <c r="BD66" t="n">
-        <v>-38.11</v>
+        <v>-48.68</v>
       </c>
       <c r="BE66" t="n">
         <v>-59.83</v>
       </c>
       <c r="BF66" t="n">
-        <v>-89.37</v>
+        <v>-91.18000000000001</v>
       </c>
       <c r="BG66" t="n">
-        <v>-83.48999999999999</v>
+        <v>-86.31</v>
       </c>
       <c r="BH66" t="n">
         <v>7.12</v>
@@ -15683,7 +15683,7 @@
         <v>0</v>
       </c>
       <c r="BJ66" t="n">
-        <v>20.99</v>
+        <v>25.31</v>
       </c>
       <c r="BK66" t="n">
         <v>1.58</v>
@@ -15692,28 +15692,28 @@
         <v>1.57</v>
       </c>
       <c r="BM66" t="n">
-        <v>21.1</v>
+        <v>28.51</v>
       </c>
       <c r="BN66" t="n">
-        <v>21.33</v>
+        <v>28.51</v>
       </c>
       <c r="BO66" t="n">
         <v>9.48</v>
       </c>
       <c r="BP66" t="n">
-        <v>20.99</v>
+        <v>21.13</v>
       </c>
       <c r="BQ66" t="n">
-        <v>13.37</v>
+        <v>16.12</v>
       </c>
       <c r="BR66" t="n">
-        <v>20.99</v>
+        <v>21.13</v>
       </c>
       <c r="BS66" t="n">
         <v>3.46</v>
       </c>
       <c r="BT66" t="n">
-        <v>3790</v>
+        <v>3897</v>
       </c>
     </row>
     <row r="67">
@@ -15973,13 +15973,13 @@
         </is>
       </c>
       <c r="F68" t="n">
-        <v>18.13</v>
+        <v>18.4</v>
       </c>
       <c r="G68" t="n">
-        <v>7806661070</v>
+        <v>7959286288</v>
       </c>
       <c r="H68" t="n">
-        <v>89800</v>
+        <v>144900</v>
       </c>
       <c r="I68" t="n">
         <v>137989898</v>
@@ -16072,7 +16072,7 @@
         <v>205604948.02</v>
       </c>
       <c r="AM68" t="n">
-        <v>541377328.0166435</v>
+        <v>551961601.10957</v>
       </c>
       <c r="AN68" t="n">
         <v>0.1911</v>
@@ -16113,7 +16113,7 @@
         <v>21.39</v>
       </c>
       <c r="AZ68" t="n">
-        <v>33.54</v>
+        <v>34.04</v>
       </c>
       <c r="BA68" t="n">
         <v>1.24</v>
@@ -16122,19 +16122,19 @@
         <v>63.25</v>
       </c>
       <c r="BC68" t="n">
-        <v>44.53</v>
+        <v>42.41</v>
       </c>
       <c r="BD68" t="n">
-        <v>18.01</v>
+        <v>16.27</v>
       </c>
       <c r="BE68" t="n">
         <v>85</v>
       </c>
       <c r="BF68" t="n">
-        <v>-93.16</v>
+        <v>-93.26000000000001</v>
       </c>
       <c r="BG68" t="n">
-        <v>248.86</v>
+        <v>243.74</v>
       </c>
       <c r="BH68" t="n">
         <v>20.48</v>
@@ -16143,7 +16143,7 @@
         <v>0</v>
       </c>
       <c r="BJ68" t="n">
-        <v>18.13</v>
+        <v>18.4</v>
       </c>
       <c r="BK68" t="n">
         <v>1.49</v>
@@ -16152,7 +16152,7 @@
         <v>1.49</v>
       </c>
       <c r="BM68" t="n">
-        <v>18.24</v>
+        <v>18.95</v>
       </c>
       <c r="BN68" t="n">
         <v>22.11</v>
@@ -16161,19 +16161,19 @@
         <v>15.45</v>
       </c>
       <c r="BP68" t="n">
-        <v>17.85</v>
+        <v>18.16</v>
       </c>
       <c r="BQ68" t="n">
-        <v>12.19</v>
+        <v>12.38</v>
       </c>
       <c r="BR68" t="n">
-        <v>18</v>
+        <v>18.52</v>
       </c>
       <c r="BS68" t="n">
         <v>0</v>
       </c>
       <c r="BT68" t="n">
-        <v>45500</v>
+        <v>47700</v>
       </c>
     </row>
     <row r="69">
@@ -16203,13 +16203,13 @@
         </is>
       </c>
       <c r="F69" t="n">
-        <v>20.76</v>
+        <v>21.19</v>
       </c>
       <c r="G69" t="n">
-        <v>7806661070</v>
+        <v>7959286288</v>
       </c>
       <c r="H69" t="n">
-        <v>2900600</v>
+        <v>7534200</v>
       </c>
       <c r="I69" t="n">
         <v>255106712</v>
@@ -16302,7 +16302,7 @@
         <v>380109000.88</v>
       </c>
       <c r="AM69" t="n">
-        <v>464682206.547619</v>
+        <v>473767040.952381</v>
       </c>
       <c r="AN69" t="n">
         <v>0.8856000000000001</v>
@@ -16343,7 +16343,7 @@
         <v>21.39</v>
       </c>
       <c r="AZ69" t="n">
-        <v>36.3</v>
+        <v>37.05</v>
       </c>
       <c r="BA69" t="n">
         <v>1.24</v>
@@ -16352,19 +16352,19 @@
         <v>69.59</v>
       </c>
       <c r="BC69" t="n">
-        <v>26.22</v>
+        <v>23.66</v>
       </c>
       <c r="BD69" t="n">
-        <v>3.06</v>
+        <v>0.97</v>
       </c>
       <c r="BE69" t="n">
         <v>74.83</v>
       </c>
       <c r="BF69" t="n">
-        <v>-94.03</v>
+        <v>-94.15000000000001</v>
       </c>
       <c r="BG69" t="n">
-        <v>235.2</v>
+        <v>228.4</v>
       </c>
       <c r="BH69" t="n">
         <v>20.48</v>
@@ -16373,7 +16373,7 @@
         <v>0</v>
       </c>
       <c r="BJ69" t="n">
-        <v>20.76</v>
+        <v>21.19</v>
       </c>
       <c r="BK69" t="n">
         <v>1.49</v>
@@ -16382,7 +16382,7 @@
         <v>1.49</v>
       </c>
       <c r="BM69" t="n">
-        <v>20.89</v>
+        <v>21.69</v>
       </c>
       <c r="BN69" t="n">
         <v>25.63</v>
@@ -16391,19 +16391,19 @@
         <v>16.99</v>
       </c>
       <c r="BP69" t="n">
-        <v>20.34</v>
+        <v>20.48</v>
       </c>
       <c r="BQ69" t="n">
-        <v>13.96</v>
+        <v>14.25</v>
       </c>
       <c r="BR69" t="n">
-        <v>20.49</v>
+        <v>21.39</v>
       </c>
       <c r="BS69" t="n">
         <v>0</v>
       </c>
       <c r="BT69" t="n">
-        <v>2277277</v>
+        <v>2291533</v>
       </c>
     </row>
     <row r="70">
@@ -16433,13 +16433,13 @@
         </is>
       </c>
       <c r="F70" t="n">
-        <v>18.9</v>
+        <v>19.1</v>
       </c>
       <c r="G70" t="n">
-        <v>8746452993</v>
+        <v>8873044607</v>
       </c>
       <c r="H70" t="n">
-        <v>3277100</v>
+        <v>5137500</v>
       </c>
       <c r="I70" t="n">
         <v>464557268</v>
@@ -16454,7 +16454,7 @@
         <v>0.68</v>
       </c>
       <c r="M70" t="n">
-        <v>0.690341747941397</v>
+        <v>0.7003333955445368</v>
       </c>
       <c r="N70" t="n">
         <v>0.2</v>
@@ -16532,7 +16532,7 @@
         <v>55746872.16</v>
       </c>
       <c r="AM70" t="n">
-        <v>2886618149.504951</v>
+        <v>2928397560.066007</v>
       </c>
       <c r="AN70" t="n">
         <v>0.1236</v>
@@ -16573,7 +16573,7 @@
         <v>6.9</v>
       </c>
       <c r="AZ70" t="n">
-        <v>2.17</v>
+        <v>2.2</v>
       </c>
       <c r="BA70" t="n">
         <v>0.12</v>
@@ -16582,10 +16582,10 @@
         <v>1.07</v>
       </c>
       <c r="BC70" t="n">
-        <v>-55.3</v>
+        <v>-55.76</v>
       </c>
       <c r="BD70" t="n">
-        <v>-63.5</v>
+        <v>-63.88</v>
       </c>
       <c r="BE70" t="n">
         <v>-88.5</v>
@@ -16594,7 +16594,7 @@
         <v>-99.37</v>
       </c>
       <c r="BG70" t="n">
-        <v>-94.34</v>
+        <v>-94.40000000000001</v>
       </c>
       <c r="BH70" t="n">
         <v>26.44</v>
@@ -16603,7 +16603,7 @@
         <v>0</v>
       </c>
       <c r="BJ70" t="n">
-        <v>18.9</v>
+        <v>19.1</v>
       </c>
       <c r="BK70" t="n">
         <v>0.12</v>
@@ -16612,7 +16612,7 @@
         <v>0.1</v>
       </c>
       <c r="BM70" t="n">
-        <v>19</v>
+        <v>19.8</v>
       </c>
       <c r="BN70" t="n">
         <v>22.15</v>
@@ -16621,19 +16621,19 @@
         <v>13.21</v>
       </c>
       <c r="BP70" t="n">
-        <v>18.05</v>
+        <v>18.86</v>
       </c>
       <c r="BQ70" t="n">
-        <v>189.55</v>
+        <v>191.56</v>
       </c>
       <c r="BR70" t="n">
-        <v>18.05</v>
+        <v>19</v>
       </c>
       <c r="BS70" t="n">
         <v>0.67</v>
       </c>
       <c r="BT70" t="n">
-        <v>3731647</v>
+        <v>3682213</v>
       </c>
     </row>
     <row r="71">

</xml_diff>

<commit_message>
📊 Dados atualizados - 2026-10-07 06:45
</commit_message>
<xml_diff>
--- a/data/ativos.xlsx
+++ b/data/ativos.xlsx
@@ -1047,13 +1047,13 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>28.24</v>
+        <v>28.82</v>
       </c>
       <c r="G3" t="n">
-        <v>3777574401</v>
+        <v>3419126949</v>
       </c>
       <c r="H3" t="n">
-        <v>2163000</v>
+        <v>0</v>
       </c>
       <c r="I3" t="n">
         <v>129510368</v>
@@ -1068,7 +1068,7 @@
         <v>0.88</v>
       </c>
       <c r="M3" t="n">
-        <v>0.9399446429270828</v>
+        <v>0.8507549337345721</v>
       </c>
       <c r="N3" t="n">
         <v>0.09</v>
@@ -1146,7 +1146,7 @@
         <v>506385538.88</v>
       </c>
       <c r="AM3" t="n">
-        <v>737807500.1953125</v>
+        <v>667798232.2265625</v>
       </c>
       <c r="AN3" t="n">
         <v>2.7</v>
@@ -1187,7 +1187,7 @@
         <v>40.42</v>
       </c>
       <c r="AZ3" t="n">
-        <v>51.68</v>
+        <v>52.74</v>
       </c>
       <c r="BA3" t="n">
         <v>4.87</v>
@@ -1196,19 +1196,19 @@
         <v>21.14</v>
       </c>
       <c r="BC3" t="n">
-        <v>75.28</v>
+        <v>71.75</v>
       </c>
       <c r="BD3" t="n">
-        <v>43.11</v>
+        <v>40.23</v>
       </c>
       <c r="BE3" t="n">
         <v>83</v>
       </c>
       <c r="BF3" t="n">
-        <v>-82.76000000000001</v>
+        <v>-83.11</v>
       </c>
       <c r="BG3" t="n">
-        <v>-25.16</v>
+        <v>-26.66</v>
       </c>
       <c r="BH3" t="n">
         <v>27.85</v>
@@ -1217,7 +1217,7 @@
         <v>0</v>
       </c>
       <c r="BJ3" t="n">
-        <v>28.24</v>
+        <v>28.82</v>
       </c>
       <c r="BK3" t="n">
         <v>3.91</v>
@@ -1226,28 +1226,28 @@
         <v>4.39</v>
       </c>
       <c r="BM3" t="n">
-        <v>28.72</v>
+        <v>29.2</v>
       </c>
       <c r="BN3" t="n">
-        <v>28.72</v>
+        <v>29.2</v>
       </c>
       <c r="BO3" t="n">
         <v>18.72</v>
       </c>
       <c r="BP3" t="n">
-        <v>26.48</v>
+        <v>28.12</v>
       </c>
       <c r="BQ3" t="n">
-        <v>6.43</v>
+        <v>6.56</v>
       </c>
       <c r="BR3" t="n">
-        <v>26.5</v>
+        <v>28.2</v>
       </c>
       <c r="BS3" t="n">
         <v>0.79</v>
       </c>
       <c r="BT3" t="n">
-        <v>579787</v>
+        <v>634997</v>
       </c>
     </row>
     <row r="4">
@@ -1277,13 +1277,13 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>16.5</v>
+        <v>16.25</v>
       </c>
       <c r="G4" t="n">
-        <v>255496890000</v>
+        <v>231361975000</v>
       </c>
       <c r="H4" t="n">
-        <v>72356100</v>
+        <v>0</v>
       </c>
       <c r="I4" t="n">
         <v>15484664889</v>
@@ -1298,7 +1298,7 @@
         <v>2.76</v>
       </c>
       <c r="M4" t="n">
-        <v>2.892999086588112</v>
+        <v>2.61971870712877</v>
       </c>
       <c r="N4" t="n">
         <v>1.76</v>
@@ -1376,7 +1376,7 @@
         <v>16258898133.45</v>
       </c>
       <c r="AM4" t="n">
-        <v>25296721782.17822</v>
+        <v>22907126237.62376</v>
       </c>
       <c r="AN4" t="n">
         <v>0.269</v>
@@ -1417,7 +1417,7 @@
         <v>9.470000000000001</v>
       </c>
       <c r="AZ4" t="n">
-        <v>20.6</v>
+        <v>20.29</v>
       </c>
       <c r="BA4" t="n">
         <v>1.13</v>
@@ -1426,25 +1426,25 @@
         <v>11.39</v>
       </c>
       <c r="BC4" t="n">
-        <v>-29.67</v>
+        <v>-28.59</v>
       </c>
       <c r="BD4" t="n">
-        <v>-42.58</v>
+        <v>-41.69</v>
       </c>
       <c r="BE4" t="n">
         <v>24.83</v>
       </c>
       <c r="BF4" t="n">
-        <v>-93.17</v>
+        <v>-93.06</v>
       </c>
       <c r="BG4" t="n">
-        <v>-30.99</v>
+        <v>-29.93</v>
       </c>
       <c r="BH4" t="n">
         <v>5.7</v>
       </c>
       <c r="BI4" t="n">
-        <v>0</v>
+        <v>-1.52</v>
       </c>
       <c r="BJ4" t="n">
         <v>16.5</v>
@@ -1456,7 +1456,7 @@
         <v>1.04</v>
       </c>
       <c r="BM4" t="n">
-        <v>16.86</v>
+        <v>16.7</v>
       </c>
       <c r="BN4" t="n">
         <v>16.94</v>
@@ -1465,19 +1465,19 @@
         <v>11.04</v>
       </c>
       <c r="BP4" t="n">
-        <v>16.23</v>
+        <v>16.17</v>
       </c>
       <c r="BQ4" t="n">
-        <v>15.91</v>
+        <v>15.67</v>
       </c>
       <c r="BR4" t="n">
-        <v>16.45</v>
+        <v>16.7</v>
       </c>
       <c r="BS4" t="n">
         <v>2.76</v>
       </c>
       <c r="BT4" t="n">
-        <v>25944680</v>
+        <v>27692800</v>
       </c>
     </row>
     <row r="5">
@@ -1737,13 +1737,13 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>7.19</v>
+        <v>7.49</v>
       </c>
       <c r="G6" t="n">
-        <v>453578996</v>
+        <v>450669691</v>
       </c>
       <c r="H6" t="n">
-        <v>800</v>
+        <v>0</v>
       </c>
       <c r="I6" t="n">
         <v>63084700</v>
@@ -1758,7 +1758,7 @@
         <v>1.91</v>
       </c>
       <c r="M6" t="n">
-        <v>7.061336888809389</v>
+        <v>7.016044706194086</v>
       </c>
       <c r="N6" t="n">
         <v>1.26</v>
@@ -1836,7 +1836,7 @@
         <v>35958279</v>
       </c>
       <c r="AM6" t="n">
-        <v>43363192.73422562</v>
+        <v>43085056.50095602</v>
       </c>
       <c r="AN6" t="n">
         <v>0.5199</v>
@@ -1877,7 +1877,7 @@
         <v>5.74</v>
       </c>
       <c r="AZ6" t="n">
-        <v>8.44</v>
+        <v>8.789999999999999</v>
       </c>
       <c r="BA6" t="n">
         <v>0.65</v>
@@ -1886,25 +1886,25 @@
         <v>7.95</v>
       </c>
       <c r="BC6" t="n">
-        <v>-2.14</v>
+        <v>-6.06</v>
       </c>
       <c r="BD6" t="n">
-        <v>-20.1</v>
+        <v>-23.3</v>
       </c>
       <c r="BE6" t="n">
         <v>17.33</v>
       </c>
       <c r="BF6" t="n">
-        <v>-90.98</v>
+        <v>-91.34</v>
       </c>
       <c r="BG6" t="n">
-        <v>10.62</v>
+        <v>6.19</v>
       </c>
       <c r="BH6" t="n">
         <v>3.86</v>
       </c>
       <c r="BI6" t="n">
-        <v>0</v>
+        <v>4.17</v>
       </c>
       <c r="BJ6" t="n">
         <v>7.19</v>
@@ -1916,7 +1916,7 @@
         <v>0.5600000000000001</v>
       </c>
       <c r="BM6" t="n">
-        <v>7.31</v>
+        <v>7.49</v>
       </c>
       <c r="BN6" t="n">
         <v>8.16</v>
@@ -1925,19 +1925,19 @@
         <v>6.22</v>
       </c>
       <c r="BP6" t="n">
-        <v>7.17</v>
+        <v>7.19</v>
       </c>
       <c r="BQ6" t="n">
-        <v>12.79</v>
+        <v>13.32</v>
       </c>
       <c r="BR6" t="n">
-        <v>7.18</v>
+        <v>7.19</v>
       </c>
       <c r="BS6" t="n">
         <v>7.32</v>
       </c>
       <c r="BT6" t="n">
-        <v>213</v>
+        <v>237</v>
       </c>
     </row>
     <row r="7">
@@ -3117,13 +3117,13 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>5.49</v>
+        <v>5.01</v>
       </c>
       <c r="G12" t="n">
-        <v>526828777</v>
+        <v>442855813</v>
       </c>
       <c r="H12" t="n">
-        <v>4403400</v>
+        <v>0</v>
       </c>
       <c r="I12" t="n">
         <v>95961536</v>
@@ -3138,7 +3138,7 @@
         <v>0.32</v>
       </c>
       <c r="M12" t="n">
-        <v>0.09527618041378137</v>
+        <v>0.08008979801169788</v>
       </c>
       <c r="N12" t="n">
         <v>0.14</v>
@@ -3216,7 +3216,7 @@
         <v>362734606.08</v>
       </c>
       <c r="AM12" t="n">
-        <v>566482555.9139785</v>
+        <v>476189046.2365591</v>
       </c>
       <c r="AN12" t="n">
         <v>0.4208</v>
@@ -3257,7 +3257,7 @@
         <v>30.49</v>
       </c>
       <c r="AZ12" t="n">
-        <v>7.42</v>
+        <v>6.77</v>
       </c>
       <c r="BA12" t="n">
         <v>4.41</v>
@@ -3266,25 +3266,25 @@
         <v>18.12</v>
       </c>
       <c r="BC12" t="n">
-        <v>580.28</v>
+        <v>645.45</v>
       </c>
       <c r="BD12" t="n">
-        <v>455.45</v>
+        <v>508.66</v>
       </c>
       <c r="BE12" t="n">
         <v>35.17</v>
       </c>
       <c r="BF12" t="n">
-        <v>-19.64</v>
+        <v>-11.94</v>
       </c>
       <c r="BG12" t="n">
-        <v>230.03</v>
+        <v>261.65</v>
       </c>
       <c r="BH12" t="n">
         <v>16.4</v>
       </c>
       <c r="BI12" t="n">
-        <v>10.37</v>
+        <v>0.72</v>
       </c>
       <c r="BJ12" t="n">
         <v>4.97</v>
@@ -3296,28 +3296,28 @@
         <v>3.63</v>
       </c>
       <c r="BM12" t="n">
-        <v>5.66</v>
+        <v>5.09</v>
       </c>
       <c r="BN12" t="n">
-        <v>8.23</v>
+        <v>7.43</v>
       </c>
       <c r="BO12" t="n">
-        <v>4.42</v>
+        <v>3.99</v>
       </c>
       <c r="BP12" t="n">
-        <v>5.41</v>
+        <v>4.84</v>
       </c>
       <c r="BQ12" t="n">
-        <v>1.51</v>
+        <v>1.38</v>
       </c>
       <c r="BR12" t="n">
-        <v>5.51</v>
+        <v>5</v>
       </c>
       <c r="BS12" t="n">
         <v>0.09</v>
       </c>
       <c r="BT12" t="n">
-        <v>614803</v>
+        <v>751297</v>
       </c>
     </row>
     <row r="13">
@@ -3347,13 +3347,13 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>33.06</v>
+        <v>34.29</v>
       </c>
       <c r="G13" t="n">
-        <v>16668555152</v>
+        <v>15281565222</v>
       </c>
       <c r="H13" t="n">
-        <v>22405900</v>
+        <v>0</v>
       </c>
       <c r="I13" t="n">
         <v>504190947</v>
@@ -3368,7 +3368,7 @@
         <v>1.13</v>
       </c>
       <c r="M13" t="n">
-        <v>5.764950034527939</v>
+        <v>5.285248730369972</v>
       </c>
       <c r="N13" t="n">
         <v>0.57</v>
@@ -3446,7 +3446,7 @@
         <v>932753251.95</v>
       </c>
       <c r="AM13" t="n">
-        <v>1734501056.399584</v>
+        <v>1590173280.12487</v>
       </c>
       <c r="AN13" t="n">
         <v>2.6301</v>
@@ -3487,7 +3487,7 @@
         <v>26.6</v>
       </c>
       <c r="AZ13" t="n">
-        <v>59.84</v>
+        <v>62.06</v>
       </c>
       <c r="BA13" t="n">
         <v>2.6</v>
@@ -3496,19 +3496,19 @@
         <v>8.69</v>
       </c>
       <c r="BC13" t="n">
-        <v>-1.47</v>
+        <v>-5.01</v>
       </c>
       <c r="BD13" t="n">
-        <v>-19.55</v>
+        <v>-22.44</v>
       </c>
       <c r="BE13" t="n">
         <v>81</v>
       </c>
       <c r="BF13" t="n">
-        <v>-92.12</v>
+        <v>-92.41</v>
       </c>
       <c r="BG13" t="n">
-        <v>-73.7</v>
+        <v>-74.65000000000001</v>
       </c>
       <c r="BH13" t="n">
         <v>25.49</v>
@@ -3517,7 +3517,7 @@
         <v>0</v>
       </c>
       <c r="BJ13" t="n">
-        <v>33.06</v>
+        <v>34.29</v>
       </c>
       <c r="BK13" t="n">
         <v>1.85</v>
@@ -3526,28 +3526,28 @@
         <v>1.96</v>
       </c>
       <c r="BM13" t="n">
-        <v>33.93</v>
+        <v>34.5</v>
       </c>
       <c r="BN13" t="n">
-        <v>33.93</v>
+        <v>34.5</v>
       </c>
       <c r="BO13" t="n">
         <v>20.85</v>
       </c>
       <c r="BP13" t="n">
-        <v>31.8</v>
+        <v>33.16</v>
       </c>
       <c r="BQ13" t="n">
-        <v>16.89</v>
+        <v>17.52</v>
       </c>
       <c r="BR13" t="n">
-        <v>32.41</v>
+        <v>33.32</v>
       </c>
       <c r="BS13" t="n">
         <v>5.01</v>
       </c>
       <c r="BT13" t="n">
-        <v>5305243</v>
+        <v>5913507</v>
       </c>
     </row>
     <row r="14">
@@ -3580,10 +3580,10 @@
         <v>11.8</v>
       </c>
       <c r="G14" t="n">
-        <v>9482112153</v>
+        <v>8768925468</v>
       </c>
       <c r="H14" t="n">
-        <v>90600</v>
+        <v>0</v>
       </c>
       <c r="I14" t="n">
         <v>339510689</v>
@@ -3598,7 +3598,7 @@
         <v>1.92</v>
       </c>
       <c r="M14" t="n">
-        <v>3.937141535915313</v>
+        <v>3.64101374549608</v>
       </c>
       <c r="N14" t="n">
         <v>1.11</v>
@@ -3676,7 +3676,7 @@
         <v>349696009.67</v>
       </c>
       <c r="AM14" t="n">
-        <v>1052398685.127636</v>
+        <v>973243670.1442841</v>
       </c>
       <c r="AN14" t="n">
         <v>0.1489</v>
@@ -3756,7 +3756,7 @@
         <v>1.01</v>
       </c>
       <c r="BM14" t="n">
-        <v>12</v>
+        <v>11.95</v>
       </c>
       <c r="BN14" t="n">
         <v>13.49</v>
@@ -3765,19 +3765,19 @@
         <v>7.81</v>
       </c>
       <c r="BP14" t="n">
-        <v>11.41</v>
+        <v>11.45</v>
       </c>
       <c r="BQ14" t="n">
         <v>11.65</v>
       </c>
       <c r="BR14" t="n">
-        <v>11.51</v>
+        <v>11.8</v>
       </c>
       <c r="BS14" t="n">
         <v>1.44</v>
       </c>
       <c r="BT14" t="n">
-        <v>9933</v>
+        <v>12680</v>
       </c>
     </row>
     <row r="15">
@@ -3807,13 +3807,13 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>15.85</v>
+        <v>15.99</v>
       </c>
       <c r="G15" t="n">
-        <v>9482112153</v>
+        <v>8768925468</v>
       </c>
       <c r="H15" t="n">
-        <v>4216400</v>
+        <v>0</v>
       </c>
       <c r="I15" t="n">
         <v>343551533</v>
@@ -3828,7 +3828,7 @@
         <v>2.56</v>
       </c>
       <c r="M15" t="n">
-        <v>3.890832981813899</v>
+        <v>3.598188238594891</v>
       </c>
       <c r="N15" t="n">
         <v>1.47</v>
@@ -3906,7 +3906,7 @@
         <v>353858078.99</v>
       </c>
       <c r="AM15" t="n">
-        <v>790835041.9516263</v>
+        <v>731353250.0417014</v>
       </c>
       <c r="AN15" t="n">
         <v>0.1638</v>
@@ -3947,7 +3947,7 @@
         <v>9.050000000000001</v>
       </c>
       <c r="AZ15" t="n">
-        <v>10.54</v>
+        <v>10.63</v>
       </c>
       <c r="BA15" t="n">
         <v>1.42</v>
@@ -3956,25 +3956,25 @@
         <v>6.19</v>
       </c>
       <c r="BC15" t="n">
-        <v>-30.08</v>
+        <v>-30.69</v>
       </c>
       <c r="BD15" t="n">
-        <v>-42.91</v>
+        <v>-43.41</v>
       </c>
       <c r="BE15" t="n">
         <v>-33.5</v>
       </c>
       <c r="BF15" t="n">
-        <v>-91.03</v>
+        <v>-91.11</v>
       </c>
       <c r="BG15" t="n">
-        <v>-60.96</v>
+        <v>-61.3</v>
       </c>
       <c r="BH15" t="n">
         <v>5.3</v>
       </c>
       <c r="BI15" t="n">
-        <v>0</v>
+        <v>0.88</v>
       </c>
       <c r="BJ15" t="n">
         <v>15.85</v>
@@ -3986,7 +3986,7 @@
         <v>1.01</v>
       </c>
       <c r="BM15" t="n">
-        <v>16.75</v>
+        <v>16.25</v>
       </c>
       <c r="BN15" t="n">
         <v>16.75</v>
@@ -3995,19 +3995,19 @@
         <v>7.84</v>
       </c>
       <c r="BP15" t="n">
-        <v>15.57</v>
+        <v>15.63</v>
       </c>
       <c r="BQ15" t="n">
-        <v>15.65</v>
+        <v>15.79</v>
       </c>
       <c r="BR15" t="n">
-        <v>15.89</v>
+        <v>15.84</v>
       </c>
       <c r="BS15" t="n">
         <v>1.92</v>
       </c>
       <c r="BT15" t="n">
-        <v>2405447</v>
+        <v>2514247</v>
       </c>
     </row>
     <row r="16">
@@ -4037,13 +4037,13 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>4.89</v>
+        <v>5.07</v>
       </c>
       <c r="G16" t="n">
-        <v>1072404354</v>
+        <v>1001780826</v>
       </c>
       <c r="H16" t="n">
-        <v>297800</v>
+        <v>0</v>
       </c>
       <c r="I16" t="n">
         <v>219305733</v>
@@ -4058,7 +4058,7 @@
         <v>2.69</v>
       </c>
       <c r="M16" t="n">
-        <v>0.5073371781279424</v>
+        <v>0.4739263277604329</v>
       </c>
       <c r="N16" t="n">
         <v>0.39</v>
@@ -4136,7 +4136,7 @@
         <v>17544458.64</v>
       </c>
       <c r="AM16" t="n">
-        <v>301237178.0898876</v>
+        <v>281399108.4269663</v>
       </c>
       <c r="AN16" t="n">
         <v>0.0077</v>
@@ -4186,16 +4186,16 @@
         <v>0</v>
       </c>
       <c r="BC16" t="n">
-        <v>-64.44</v>
+        <v>-65.7</v>
       </c>
       <c r="BD16" t="n">
-        <v>-70.95999999999999</v>
+        <v>-71.98999999999999</v>
       </c>
       <c r="BE16" t="n">
         <v>-97.17</v>
       </c>
       <c r="BF16" t="n">
-        <v>-98.36</v>
+        <v>-98.42</v>
       </c>
       <c r="BG16" t="n">
         <v>-100</v>
@@ -4207,7 +4207,7 @@
         <v>0</v>
       </c>
       <c r="BJ16" t="n">
-        <v>4.89</v>
+        <v>5.07</v>
       </c>
       <c r="BK16" t="n">
         <v>0.08</v>
@@ -4225,19 +4225,19 @@
         <v>3.22</v>
       </c>
       <c r="BP16" t="n">
-        <v>4.71</v>
+        <v>4.91</v>
       </c>
       <c r="BQ16" t="n">
-        <v>66.73</v>
+        <v>69.19</v>
       </c>
       <c r="BR16" t="n">
-        <v>4.71</v>
+        <v>4.91</v>
       </c>
       <c r="BS16" t="n">
         <v>0.49</v>
       </c>
       <c r="BT16" t="n">
-        <v>131397</v>
+        <v>124047</v>
       </c>
     </row>
     <row r="17">
@@ -4267,13 +4267,13 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>36.19</v>
+        <v>37.44</v>
       </c>
       <c r="G17" t="n">
-        <v>11929197058</v>
+        <v>10944861006</v>
       </c>
       <c r="H17" t="n">
-        <v>3317100</v>
+        <v>0</v>
       </c>
       <c r="I17" t="n">
         <v>0</v>
@@ -4360,13 +4360,13 @@
         <v>8.039999999999999</v>
       </c>
       <c r="AK17" t="n">
-        <v>5387101272.57948</v>
+        <v>4942585353.143064</v>
       </c>
       <c r="AL17" t="n">
-        <v>1491149632.25</v>
+        <v>1368107625.75</v>
       </c>
       <c r="AM17" t="n">
-        <v>3693249863.157895</v>
+        <v>3388501859.442725</v>
       </c>
       <c r="AN17" t="n">
         <v>1.08</v>
@@ -4407,7 +4407,7 @@
         <v>42.98</v>
       </c>
       <c r="AZ17" t="n">
-        <v>19.36</v>
+        <v>20.03</v>
       </c>
       <c r="BA17" t="n">
         <v>4.55</v>
@@ -4416,25 +4416,25 @@
         <v>16.33</v>
       </c>
       <c r="BC17" t="n">
-        <v>45.45</v>
+        <v>40.59</v>
       </c>
       <c r="BD17" t="n">
-        <v>18.76</v>
+        <v>14.79</v>
       </c>
       <c r="BE17" t="n">
         <v>-46.5</v>
       </c>
       <c r="BF17" t="n">
-        <v>-87.43000000000001</v>
+        <v>-87.84999999999999</v>
       </c>
       <c r="BG17" t="n">
-        <v>-54.87</v>
+        <v>-56.37</v>
       </c>
       <c r="BH17" t="n">
         <v>29.25</v>
       </c>
       <c r="BI17" t="n">
-        <v>0</v>
+        <v>3.45</v>
       </c>
       <c r="BJ17" t="n">
         <v>36.19</v>
@@ -4446,28 +4446,28 @@
         <v>12.62</v>
       </c>
       <c r="BM17" t="n">
-        <v>37.06</v>
+        <v>38</v>
       </c>
       <c r="BN17" t="n">
-        <v>37.06</v>
+        <v>38</v>
       </c>
       <c r="BO17" t="n">
         <v>29.53</v>
       </c>
       <c r="BP17" t="n">
-        <v>34.27</v>
+        <v>35.96</v>
       </c>
       <c r="BQ17" t="n">
-        <v>2.87</v>
+        <v>2.97</v>
       </c>
       <c r="BR17" t="n">
-        <v>34.27</v>
+        <v>36.1</v>
       </c>
       <c r="BS17" t="n">
         <v>2.21</v>
       </c>
       <c r="BT17" t="n">
-        <v>1062917</v>
+        <v>1131930</v>
       </c>
     </row>
     <row r="18">
@@ -4497,13 +4497,13 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>12.98</v>
+        <v>13.27</v>
       </c>
       <c r="G18" t="n">
-        <v>11929197058</v>
+        <v>10944861006</v>
       </c>
       <c r="H18" t="n">
-        <v>28300</v>
+        <v>0</v>
       </c>
       <c r="I18" t="n">
         <v>671494278</v>
@@ -4518,7 +4518,7 @@
         <v>1.2</v>
       </c>
       <c r="M18" t="n">
-        <v>3.512424085715632</v>
+        <v>3.222596896117451</v>
       </c>
       <c r="N18" t="n">
         <v>0.33</v>
@@ -4596,7 +4596,7 @@
         <v>940091989.1999999</v>
       </c>
       <c r="AM18" t="n">
-        <v>3550356267.261905</v>
+        <v>3257399108.928572</v>
       </c>
       <c r="AN18" t="n">
         <v>0.36</v>
@@ -4637,7 +4637,7 @@
         <v>14.31</v>
       </c>
       <c r="AZ18" t="n">
-        <v>6.68</v>
+        <v>6.83</v>
       </c>
       <c r="BA18" t="n">
         <v>1.51</v>
@@ -4646,19 +4646,19 @@
         <v>5.44</v>
       </c>
       <c r="BC18" t="n">
-        <v>35.02</v>
+        <v>32.06</v>
       </c>
       <c r="BD18" t="n">
-        <v>10.24</v>
+        <v>7.83</v>
       </c>
       <c r="BE18" t="n">
         <v>-48.5</v>
       </c>
       <c r="BF18" t="n">
-        <v>-88.34999999999999</v>
+        <v>-88.59999999999999</v>
       </c>
       <c r="BG18" t="n">
-        <v>-58.06</v>
+        <v>-58.97</v>
       </c>
       <c r="BH18" t="n">
         <v>9.75</v>
@@ -4667,7 +4667,7 @@
         <v>0</v>
       </c>
       <c r="BJ18" t="n">
-        <v>12.98</v>
+        <v>13.27</v>
       </c>
       <c r="BK18" t="n">
         <v>1.4</v>
@@ -4676,7 +4676,7 @@
         <v>12.62</v>
       </c>
       <c r="BM18" t="n">
-        <v>13.86</v>
+        <v>13.56</v>
       </c>
       <c r="BN18" t="n">
         <v>13.86</v>
@@ -4685,19 +4685,19 @@
         <v>10.19</v>
       </c>
       <c r="BP18" t="n">
-        <v>11.75</v>
+        <v>12.5</v>
       </c>
       <c r="BQ18" t="n">
-        <v>1.03</v>
+        <v>1.05</v>
       </c>
       <c r="BR18" t="n">
-        <v>11.9</v>
+        <v>12.5</v>
       </c>
       <c r="BS18" t="n">
         <v>2.3</v>
       </c>
       <c r="BT18" t="n">
-        <v>8493</v>
+        <v>9280</v>
       </c>
     </row>
     <row r="19">
@@ -4727,13 +4727,13 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>11.59</v>
+        <v>11.4</v>
       </c>
       <c r="G19" t="n">
-        <v>11929197058</v>
+        <v>10944861006</v>
       </c>
       <c r="H19" t="n">
-        <v>62000</v>
+        <v>0</v>
       </c>
       <c r="I19" t="n">
         <v>317386323</v>
@@ -4748,7 +4748,7 @@
         <v>1.12</v>
       </c>
       <c r="M19" t="n">
-        <v>7.431236019163399</v>
+        <v>6.81804860269114</v>
       </c>
       <c r="N19" t="n">
         <v>0.3</v>
@@ -4826,7 +4826,7 @@
         <v>444340852.2</v>
       </c>
       <c r="AM19" t="n">
-        <v>3787046685.079365</v>
+        <v>3474559049.523809</v>
       </c>
       <c r="AN19" t="n">
         <v>0.36</v>
@@ -4867,7 +4867,7 @@
         <v>14.31</v>
       </c>
       <c r="AZ19" t="n">
-        <v>6.37</v>
+        <v>6.27</v>
       </c>
       <c r="BA19" t="n">
         <v>1.51</v>
@@ -4876,25 +4876,25 @@
         <v>5.25</v>
       </c>
       <c r="BC19" t="n">
-        <v>51.21</v>
+        <v>53.73</v>
       </c>
       <c r="BD19" t="n">
-        <v>23.46</v>
+        <v>25.52</v>
       </c>
       <c r="BE19" t="n">
         <v>-45</v>
       </c>
       <c r="BF19" t="n">
-        <v>-86.95</v>
+        <v>-86.73</v>
       </c>
       <c r="BG19" t="n">
-        <v>-54.7</v>
+        <v>-53.95</v>
       </c>
       <c r="BH19" t="n">
         <v>9.75</v>
       </c>
       <c r="BI19" t="n">
-        <v>0</v>
+        <v>-1.64</v>
       </c>
       <c r="BJ19" t="n">
         <v>11.59</v>
@@ -4906,28 +4906,28 @@
         <v>12.62</v>
       </c>
       <c r="BM19" t="n">
-        <v>11.84</v>
+        <v>12.3</v>
       </c>
       <c r="BN19" t="n">
-        <v>11.84</v>
+        <v>12.3</v>
       </c>
       <c r="BO19" t="n">
         <v>9.19</v>
       </c>
       <c r="BP19" t="n">
-        <v>11.05</v>
+        <v>11.36</v>
       </c>
       <c r="BQ19" t="n">
-        <v>0.92</v>
+        <v>0.9</v>
       </c>
       <c r="BR19" t="n">
-        <v>11.5</v>
+        <v>11.56</v>
       </c>
       <c r="BS19" t="n">
         <v>2.16</v>
       </c>
       <c r="BT19" t="n">
-        <v>11243</v>
+        <v>12903</v>
       </c>
     </row>
     <row r="20">
@@ -5417,13 +5417,13 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>5.75</v>
+        <v>6.08</v>
       </c>
       <c r="G22" t="n">
-        <v>1151409900</v>
+        <v>1111334002</v>
       </c>
       <c r="H22" t="n">
-        <v>4550200</v>
+        <v>0</v>
       </c>
       <c r="I22" t="n">
         <v>200245299</v>
@@ -5438,7 +5438,7 @@
         <v>0.27</v>
       </c>
       <c r="M22" t="n">
-        <v>0.09765868187687618</v>
+        <v>0.09425958015496799</v>
       </c>
       <c r="N22" t="n">
         <v>0.08</v>
@@ -5516,7 +5516,7 @@
         <v>378463615.11</v>
       </c>
       <c r="AM22" t="n">
-        <v>261090680.2721088</v>
+        <v>252003175.0566893</v>
       </c>
       <c r="AN22" t="n">
         <v>0</v>
@@ -5566,25 +5566,25 @@
         <v>172.49</v>
       </c>
       <c r="BC22" t="n">
-        <v>416.61</v>
+        <v>388.57</v>
       </c>
       <c r="BD22" t="n">
-        <v>321.81</v>
+        <v>298.92</v>
       </c>
       <c r="BE22" t="n">
         <v>-100</v>
       </c>
       <c r="BF22" t="n">
-        <v>-67.13</v>
+        <v>-68.91</v>
       </c>
       <c r="BG22" t="n">
-        <v>2899.82</v>
+        <v>2737</v>
       </c>
       <c r="BH22" t="n">
         <v>20.75</v>
       </c>
       <c r="BI22" t="n">
-        <v>0</v>
+        <v>5.74</v>
       </c>
       <c r="BJ22" t="n">
         <v>5.75</v>
@@ -5596,7 +5596,7 @@
         <v>0.67</v>
       </c>
       <c r="BM22" t="n">
-        <v>6.15</v>
+        <v>6.12</v>
       </c>
       <c r="BN22" t="n">
         <v>7.89</v>
@@ -5605,19 +5605,19 @@
         <v>3.37</v>
       </c>
       <c r="BP22" t="n">
-        <v>5.6</v>
+        <v>5.77</v>
       </c>
       <c r="BQ22" t="n">
-        <v>8.56</v>
+        <v>9.06</v>
       </c>
       <c r="BR22" t="n">
-        <v>5.6</v>
+        <v>5.89</v>
       </c>
       <c r="BS22" t="n">
         <v>0.09</v>
       </c>
       <c r="BT22" t="n">
-        <v>1639090</v>
+        <v>1726780</v>
       </c>
     </row>
     <row r="23">
@@ -5877,13 +5877,13 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>3.89</v>
+        <v>4.08</v>
       </c>
       <c r="G24" t="n">
-        <v>1571049674</v>
+        <v>1355074870</v>
       </c>
       <c r="H24" t="n">
-        <v>13516400</v>
+        <v>0</v>
       </c>
       <c r="I24" t="n">
         <v>403868805</v>
@@ -5898,7 +5898,7 @@
         <v>0.49</v>
       </c>
       <c r="M24" t="n">
-        <v>0.3797868475565188</v>
+        <v>0.3275769198118682</v>
       </c>
       <c r="N24" t="n">
         <v>0.11</v>
@@ -5976,7 +5976,7 @@
         <v>153470145.9</v>
       </c>
       <c r="AM24" t="n">
-        <v>1415360066.666667</v>
+        <v>1220788171.171171</v>
       </c>
       <c r="AN24" t="n">
         <v>0.0813</v>
@@ -6017,7 +6017,7 @@
         <v>5.84</v>
       </c>
       <c r="AZ24" t="n">
-        <v>1.8</v>
+        <v>1.88</v>
       </c>
       <c r="BA24" t="n">
         <v>0.38</v>
@@ -6026,25 +6026,25 @@
         <v>1.46</v>
       </c>
       <c r="BC24" t="n">
-        <v>83.97</v>
+        <v>75.40000000000001</v>
       </c>
       <c r="BD24" t="n">
-        <v>50.21</v>
+        <v>43.22</v>
       </c>
       <c r="BE24" t="n">
         <v>-53.83</v>
       </c>
       <c r="BF24" t="n">
-        <v>-90.23</v>
+        <v>-90.69</v>
       </c>
       <c r="BG24" t="n">
-        <v>-62.52</v>
+        <v>-64.27</v>
       </c>
       <c r="BH24" t="n">
         <v>5.99</v>
       </c>
       <c r="BI24" t="n">
-        <v>0</v>
+        <v>4.88</v>
       </c>
       <c r="BJ24" t="n">
         <v>3.89</v>
@@ -6056,7 +6056,7 @@
         <v>0.41</v>
       </c>
       <c r="BM24" t="n">
-        <v>3.95</v>
+        <v>4.13</v>
       </c>
       <c r="BN24" t="n">
         <v>5.29</v>
@@ -6065,19 +6065,19 @@
         <v>1.92</v>
       </c>
       <c r="BP24" t="n">
-        <v>3.61</v>
+        <v>3.88</v>
       </c>
       <c r="BQ24" t="n">
-        <v>9.550000000000001</v>
+        <v>10.02</v>
       </c>
       <c r="BR24" t="n">
-        <v>3.61</v>
+        <v>4.02</v>
       </c>
       <c r="BS24" t="n">
         <v>0.29</v>
       </c>
       <c r="BT24" t="n">
-        <v>7463927</v>
+        <v>7390317</v>
       </c>
     </row>
     <row r="25">
@@ -6107,13 +6107,13 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>5.12</v>
+        <v>5.33</v>
       </c>
       <c r="G25" t="n">
-        <v>1774049752</v>
+        <v>1540826758</v>
       </c>
       <c r="H25" t="n">
-        <v>3447600</v>
+        <v>0</v>
       </c>
       <c r="I25" t="n">
         <v>346494097</v>
@@ -6128,7 +6128,7 @@
         <v>0.97</v>
       </c>
       <c r="M25" t="n">
-        <v>0.8846222099355932</v>
+        <v>0.7683265761026161</v>
       </c>
       <c r="N25" t="n">
         <v>0.22</v>
@@ -6206,7 +6206,7 @@
         <v>62368937.46</v>
       </c>
       <c r="AM25" t="n">
-        <v>652224173.5294117</v>
+        <v>566480425.7352941</v>
       </c>
       <c r="AN25" t="n">
         <v>0.4742</v>
@@ -6247,7 +6247,7 @@
         <v>3.27</v>
       </c>
       <c r="AZ25" t="n">
-        <v>11.93</v>
+        <v>12.42</v>
       </c>
       <c r="BA25" t="n">
         <v>0.23</v>
@@ -6256,25 +6256,25 @@
         <v>2.2</v>
       </c>
       <c r="BC25" t="n">
-        <v>-21.68</v>
+        <v>-24.77</v>
       </c>
       <c r="BD25" t="n">
-        <v>-36.05</v>
+        <v>-38.57</v>
       </c>
       <c r="BE25" t="n">
         <v>133</v>
       </c>
       <c r="BF25" t="n">
-        <v>-95.47</v>
+        <v>-95.65000000000001</v>
       </c>
       <c r="BG25" t="n">
-        <v>-57.04</v>
+        <v>-58.73</v>
       </c>
       <c r="BH25" t="n">
         <v>3.97</v>
       </c>
       <c r="BI25" t="n">
-        <v>0</v>
+        <v>4.1</v>
       </c>
       <c r="BJ25" t="n">
         <v>5.12</v>
@@ -6286,7 +6286,7 @@
         <v>0.24</v>
       </c>
       <c r="BM25" t="n">
-        <v>5.27</v>
+        <v>5.48</v>
       </c>
       <c r="BN25" t="n">
         <v>6.3</v>
@@ -6295,19 +6295,19 @@
         <v>2.64</v>
       </c>
       <c r="BP25" t="n">
-        <v>4.93</v>
+        <v>5.12</v>
       </c>
       <c r="BQ25" t="n">
-        <v>21.64</v>
+        <v>22.52</v>
       </c>
       <c r="BR25" t="n">
-        <v>4.98</v>
+        <v>5.12</v>
       </c>
       <c r="BS25" t="n">
         <v>0.67</v>
       </c>
       <c r="BT25" t="n">
-        <v>1176113</v>
+        <v>1242380</v>
       </c>
     </row>
     <row r="26">
@@ -6337,13 +6337,13 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>12.98</v>
+        <v>12.63</v>
       </c>
       <c r="G26" t="n">
-        <v>17580020520</v>
+        <v>14073886987</v>
       </c>
       <c r="H26" t="n">
-        <v>52209900</v>
+        <v>0</v>
       </c>
       <c r="I26" t="n">
         <v>1354393401</v>
@@ -6358,7 +6358,7 @@
         <v>1.94</v>
       </c>
       <c r="M26" t="n">
-        <v>0.2266928826338528</v>
+        <v>0.1814815862880517</v>
       </c>
       <c r="N26" t="n">
         <v>0.26</v>
@@ -6436,7 +6436,7 @@
         <v>961619314.7099999</v>
       </c>
       <c r="AM26" t="n">
-        <v>6278578757.142858</v>
+        <v>5026388209.642858</v>
       </c>
       <c r="AN26" t="n">
         <v>0.1043</v>
@@ -6477,7 +6477,7 @@
         <v>7.07</v>
       </c>
       <c r="AZ26" t="n">
-        <v>2.49</v>
+        <v>2.42</v>
       </c>
       <c r="BA26" t="n">
         <v>0.66</v>
@@ -6486,19 +6486,19 @@
         <v>1.19</v>
       </c>
       <c r="BC26" t="n">
-        <v>-33.31</v>
+        <v>-31.47</v>
       </c>
       <c r="BD26" t="n">
-        <v>-45.55</v>
+        <v>-44.04</v>
       </c>
       <c r="BE26" t="n">
         <v>-80.83</v>
       </c>
       <c r="BF26" t="n">
-        <v>-94.92</v>
+        <v>-94.78</v>
       </c>
       <c r="BG26" t="n">
-        <v>-90.81</v>
+        <v>-90.55</v>
       </c>
       <c r="BH26" t="n">
         <v>4.69</v>
@@ -6507,7 +6507,7 @@
         <v>0</v>
       </c>
       <c r="BJ26" t="n">
-        <v>12.98</v>
+        <v>12.63</v>
       </c>
       <c r="BK26" t="n">
         <v>0.71</v>
@@ -6516,7 +6516,7 @@
         <v>0.72</v>
       </c>
       <c r="BM26" t="n">
-        <v>13.45</v>
+        <v>13.31</v>
       </c>
       <c r="BN26" t="n">
         <v>13.45</v>
@@ -6525,19 +6525,19 @@
         <v>6.91</v>
       </c>
       <c r="BP26" t="n">
-        <v>12.62</v>
+        <v>12.57</v>
       </c>
       <c r="BQ26" t="n">
-        <v>18.1</v>
+        <v>17.61</v>
       </c>
       <c r="BR26" t="n">
-        <v>12.82</v>
+        <v>13.03</v>
       </c>
       <c r="BS26" t="n">
         <v>0.16</v>
       </c>
       <c r="BT26" t="n">
-        <v>14118867</v>
+        <v>15567803</v>
       </c>
     </row>
     <row r="27">
@@ -8165,13 +8165,13 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>22.17</v>
+        <v>23.08</v>
       </c>
       <c r="G34" t="n">
-        <v>4577878881</v>
+        <v>4023084018</v>
       </c>
       <c r="H34" t="n">
-        <v>8341600</v>
+        <v>0</v>
       </c>
       <c r="I34" t="n">
         <v>206489813</v>
@@ -8186,7 +8186,7 @@
         <v>0.45</v>
       </c>
       <c r="M34" t="n">
-        <v>0.4024490205676373</v>
+        <v>0.3536760724328598</v>
       </c>
       <c r="N34" t="n">
         <v>0.24</v>
@@ -8264,7 +8264,7 @@
         <v>324189006.41</v>
       </c>
       <c r="AM34" t="n">
-        <v>951741971.1018711</v>
+        <v>836400003.7422038</v>
       </c>
       <c r="AN34" t="n">
         <v>0</v>
@@ -8305,7 +8305,7 @@
         <v>30.28</v>
       </c>
       <c r="AZ34" t="n">
-        <v>51.73</v>
+        <v>53.85</v>
       </c>
       <c r="BA34" t="n">
         <v>2.29</v>
@@ -8314,19 +8314,19 @@
         <v>25.26</v>
       </c>
       <c r="BC34" t="n">
-        <v>67.29000000000001</v>
+        <v>60.7</v>
       </c>
       <c r="BD34" t="n">
-        <v>36.59</v>
+        <v>31.21</v>
       </c>
       <c r="BE34" t="n">
         <v>133.33</v>
       </c>
       <c r="BF34" t="n">
-        <v>-89.65000000000001</v>
+        <v>-90.06</v>
       </c>
       <c r="BG34" t="n">
-        <v>13.93</v>
+        <v>9.44</v>
       </c>
       <c r="BH34" t="n">
         <v>38.94</v>
@@ -8335,7 +8335,7 @@
         <v>0</v>
       </c>
       <c r="BJ34" t="n">
-        <v>22.17</v>
+        <v>23.08</v>
       </c>
       <c r="BK34" t="n">
         <v>1.57</v>
@@ -8344,7 +8344,7 @@
         <v>1.58</v>
       </c>
       <c r="BM34" t="n">
-        <v>22.68</v>
+        <v>23.68</v>
       </c>
       <c r="BN34" t="n">
         <v>28.86</v>
@@ -8353,19 +8353,19 @@
         <v>14.3</v>
       </c>
       <c r="BP34" t="n">
-        <v>21.34</v>
+        <v>22</v>
       </c>
       <c r="BQ34" t="n">
-        <v>14.06</v>
+        <v>14.63</v>
       </c>
       <c r="BR34" t="n">
-        <v>21.59</v>
+        <v>22.17</v>
       </c>
       <c r="BS34" t="n">
         <v>0.32</v>
       </c>
       <c r="BT34" t="n">
-        <v>3999757</v>
+        <v>4140347</v>
       </c>
     </row>
     <row r="35">
@@ -8395,13 +8395,13 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>23.3</v>
+        <v>22.68</v>
       </c>
       <c r="G35" t="n">
-        <v>117583446149</v>
+        <v>89391633602</v>
       </c>
       <c r="H35" t="n">
-        <v>200158200</v>
+        <v>0</v>
       </c>
       <c r="I35" t="n">
         <v>5046500000</v>
@@ -8416,7 +8416,7 @@
         <v>4.69</v>
       </c>
       <c r="M35" t="n">
-        <v>9.761820435005561</v>
+        <v>7.421325911036454</v>
       </c>
       <c r="N35" t="n">
         <v>1.79</v>
@@ -8494,7 +8494,7 @@
         <v>5349290000</v>
       </c>
       <c r="AM35" t="n">
-        <v>9717640177.603306</v>
+        <v>7387738314.214876</v>
       </c>
       <c r="AN35" t="n">
         <v>0.5305</v>
@@ -8535,7 +8535,7 @@
         <v>7.68</v>
       </c>
       <c r="AZ35" t="n">
-        <v>13.59</v>
+        <v>13.23</v>
       </c>
       <c r="BA35" t="n">
         <v>1.11</v>
@@ -8544,19 +8544,19 @@
         <v>9.119999999999999</v>
       </c>
       <c r="BC35" t="n">
-        <v>-59.63</v>
+        <v>-58.52</v>
       </c>
       <c r="BD35" t="n">
-        <v>-67.04000000000001</v>
+        <v>-66.14</v>
       </c>
       <c r="BE35" t="n">
         <v>-41.67</v>
       </c>
       <c r="BF35" t="n">
-        <v>-95.22</v>
+        <v>-95.09</v>
       </c>
       <c r="BG35" t="n">
-        <v>-60.87</v>
+        <v>-59.8</v>
       </c>
       <c r="BH35" t="n">
         <v>3.71</v>
@@ -8565,7 +8565,7 @@
         <v>0</v>
       </c>
       <c r="BJ35" t="n">
-        <v>23.3</v>
+        <v>22.68</v>
       </c>
       <c r="BK35" t="n">
         <v>1.06</v>
@@ -8574,7 +8574,7 @@
         <v>1.04</v>
       </c>
       <c r="BM35" t="n">
-        <v>24.28</v>
+        <v>23.93</v>
       </c>
       <c r="BN35" t="n">
         <v>24.28</v>
@@ -8583,19 +8583,19 @@
         <v>11.58</v>
       </c>
       <c r="BP35" t="n">
-        <v>22.03</v>
+        <v>22.44</v>
       </c>
       <c r="BQ35" t="n">
-        <v>22.3</v>
+        <v>21.7</v>
       </c>
       <c r="BR35" t="n">
-        <v>22.1</v>
+        <v>23.66</v>
       </c>
       <c r="BS35" t="n">
         <v>7.3</v>
       </c>
       <c r="BT35" t="n">
-        <v>41530023</v>
+        <v>46747913</v>
       </c>
     </row>
     <row r="36">
@@ -8858,10 +8858,10 @@
         <v>14.5</v>
       </c>
       <c r="G37" t="n">
-        <v>178849960</v>
+        <v>171417115</v>
       </c>
       <c r="H37" t="n">
-        <v>5100</v>
+        <v>900</v>
       </c>
       <c r="I37" t="n">
         <v>4900000</v>
@@ -8876,7 +8876,7 @@
         <v>0.88</v>
       </c>
       <c r="M37" t="n">
-        <v>1.741255021821716</v>
+        <v>1.668890014400565</v>
       </c>
       <c r="N37" t="n">
         <v>0.5</v>
@@ -8954,7 +8954,7 @@
         <v>11319000</v>
       </c>
       <c r="AM37" t="n">
-        <v>42787071.77033493</v>
+        <v>41008879.18660288</v>
       </c>
       <c r="AN37" t="n">
         <v>0</v>
@@ -9043,7 +9043,7 @@
         <v>13.42</v>
       </c>
       <c r="BP37" t="n">
-        <v>14.22</v>
+        <v>14.33</v>
       </c>
       <c r="BQ37" t="n">
         <v>6.27</v>
@@ -9055,7 +9055,7 @@
         <v>0.72</v>
       </c>
       <c r="BT37" t="n">
-        <v>1313</v>
+        <v>1443</v>
       </c>
     </row>
     <row r="38">
@@ -9315,13 +9315,13 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>71</v>
+        <v>74.91</v>
       </c>
       <c r="G39" t="n">
-        <v>3980140010</v>
+        <v>3951789598</v>
       </c>
       <c r="H39" t="n">
-        <v>7200</v>
+        <v>9000</v>
       </c>
       <c r="I39" t="n">
         <v>168174945</v>
@@ -9336,7 +9336,7 @@
         <v>0.53</v>
       </c>
       <c r="M39" t="n">
-        <v>0.1997855701558003</v>
+        <v>0.1983625038286507</v>
       </c>
       <c r="N39" t="n">
         <v>0.06</v>
@@ -9414,7 +9414,7 @@
         <v>2536078170.6</v>
       </c>
       <c r="AM39" t="n">
-        <v>418081933.8235294</v>
+        <v>415103949.3697479</v>
       </c>
       <c r="AN39" t="n">
         <v>11.9435</v>
@@ -9455,7 +9455,7 @@
         <v>170.24</v>
       </c>
       <c r="AZ39" t="n">
-        <v>207.44</v>
+        <v>218.86</v>
       </c>
       <c r="BA39" t="n">
         <v>19.01</v>
@@ -9464,19 +9464,19 @@
         <v>91.72</v>
       </c>
       <c r="BC39" t="n">
-        <v>193.67</v>
+        <v>178.34</v>
       </c>
       <c r="BD39" t="n">
-        <v>139.78</v>
+        <v>127.26</v>
       </c>
       <c r="BE39" t="n">
         <v>192.17</v>
       </c>
       <c r="BF39" t="n">
-        <v>-73.23</v>
+        <v>-74.62</v>
       </c>
       <c r="BG39" t="n">
-        <v>29.19</v>
+        <v>22.44</v>
       </c>
       <c r="BH39" t="n">
         <v>128.13</v>
@@ -9485,7 +9485,7 @@
         <v>0</v>
       </c>
       <c r="BJ39" t="n">
-        <v>71</v>
+        <v>74.91</v>
       </c>
       <c r="BK39" t="n">
         <v>15.08</v>
@@ -9494,28 +9494,28 @@
         <v>15.08</v>
       </c>
       <c r="BM39" t="n">
-        <v>72</v>
+        <v>77.98</v>
       </c>
       <c r="BN39" t="n">
-        <v>74.56</v>
+        <v>77.98</v>
       </c>
       <c r="BO39" t="n">
         <v>54.98</v>
       </c>
       <c r="BP39" t="n">
-        <v>70</v>
+        <v>71.76000000000001</v>
       </c>
       <c r="BQ39" t="n">
-        <v>4.71</v>
+        <v>4.97</v>
       </c>
       <c r="BR39" t="n">
-        <v>70.56</v>
+        <v>71.76000000000001</v>
       </c>
       <c r="BS39" t="n">
         <v>0.58</v>
       </c>
       <c r="BT39" t="n">
-        <v>2857</v>
+        <v>2993</v>
       </c>
     </row>
     <row r="40">
@@ -9545,13 +9545,13 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>26.33</v>
+        <v>24.64</v>
       </c>
       <c r="G40" t="n">
-        <v>150892858782</v>
+        <v>121839499381</v>
       </c>
       <c r="H40" t="n">
-        <v>147712300</v>
+        <v>0</v>
       </c>
       <c r="I40" t="n">
         <v>5730834040</v>
@@ -9566,7 +9566,7 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="M40" t="n">
-        <v>0.4578276074158132</v>
+        <v>0.3696761194705249</v>
       </c>
       <c r="N40" t="n">
         <v>0.05</v>
@@ -9644,7 +9644,7 @@
         <v>15358635227.2</v>
       </c>
       <c r="AM40" t="n">
-        <v>7826393090.352696</v>
+        <v>6319476108.973029</v>
       </c>
       <c r="AN40" t="n">
         <v>0.5641</v>
@@ -9685,7 +9685,7 @@
         <v>36.13</v>
       </c>
       <c r="AZ40" t="n">
-        <v>13.3</v>
+        <v>12.44</v>
       </c>
       <c r="BA40" t="n">
         <v>2.76</v>
@@ -9694,25 +9694,25 @@
         <v>27.89</v>
       </c>
       <c r="BC40" t="n">
-        <v>68.05</v>
+        <v>79.58</v>
       </c>
       <c r="BD40" t="n">
-        <v>37.22</v>
+        <v>46.63</v>
       </c>
       <c r="BE40" t="n">
         <v>-49.5</v>
       </c>
       <c r="BF40" t="n">
-        <v>-89.52</v>
+        <v>-88.8</v>
       </c>
       <c r="BG40" t="n">
-        <v>5.93</v>
+        <v>13.19</v>
       </c>
       <c r="BH40" t="n">
         <v>32.47</v>
       </c>
       <c r="BI40" t="n">
-        <v>0</v>
+        <v>-6.42</v>
       </c>
       <c r="BJ40" t="n">
         <v>26.33</v>
@@ -9724,7 +9724,7 @@
         <v>2.5</v>
       </c>
       <c r="BM40" t="n">
-        <v>27.19</v>
+        <v>26.29</v>
       </c>
       <c r="BN40" t="n">
         <v>27.36</v>
@@ -9733,19 +9733,19 @@
         <v>17.67</v>
       </c>
       <c r="BP40" t="n">
-        <v>25.19</v>
+        <v>24.37</v>
       </c>
       <c r="BQ40" t="n">
-        <v>10.54</v>
+        <v>9.859999999999999</v>
       </c>
       <c r="BR40" t="n">
-        <v>25.19</v>
+        <v>26.15</v>
       </c>
       <c r="BS40" t="n">
         <v>0.39</v>
       </c>
       <c r="BT40" t="n">
-        <v>37487763</v>
+        <v>40860517</v>
       </c>
     </row>
     <row r="41">
@@ -9775,13 +9775,13 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>19.36</v>
+        <v>19.99</v>
       </c>
       <c r="G41" t="n">
-        <v>229256884001</v>
+        <v>201835420046</v>
       </c>
       <c r="H41" t="n">
-        <v>43770400</v>
+        <v>0</v>
       </c>
       <c r="I41" t="n">
         <v>5303870781</v>
@@ -9796,7 +9796,7 @@
         <v>0.92</v>
       </c>
       <c r="M41" t="n">
-        <v>1.52776064360275</v>
+        <v>1.345024872753497</v>
       </c>
       <c r="N41" t="n">
         <v>0.07000000000000001</v>
@@ -9874,7 +9874,7 @@
         <v>12304980211.92</v>
       </c>
       <c r="AM41" t="n">
-        <v>35324635439.29121</v>
+        <v>31099448389.21418</v>
       </c>
       <c r="AN41" t="n">
         <v>1.6841</v>
@@ -9915,7 +9915,7 @@
         <v>24.4</v>
       </c>
       <c r="AZ41" t="n">
-        <v>28.98</v>
+        <v>29.92</v>
       </c>
       <c r="BA41" t="n">
         <v>2.53</v>
@@ -9924,19 +9924,19 @@
         <v>13.77</v>
       </c>
       <c r="BC41" t="n">
-        <v>54.37</v>
+        <v>49.5</v>
       </c>
       <c r="BD41" t="n">
-        <v>26.04</v>
+        <v>22.07</v>
       </c>
       <c r="BE41" t="n">
         <v>49.67</v>
       </c>
       <c r="BF41" t="n">
-        <v>-86.95</v>
+        <v>-87.36</v>
       </c>
       <c r="BG41" t="n">
-        <v>-28.87</v>
+        <v>-31.12</v>
       </c>
       <c r="BH41" t="n">
         <v>17.11</v>
@@ -9945,7 +9945,7 @@
         <v>0</v>
       </c>
       <c r="BJ41" t="n">
-        <v>19.36</v>
+        <v>19.99</v>
       </c>
       <c r="BK41" t="n">
         <v>2.32</v>
@@ -9954,28 +9954,28 @@
         <v>2.34</v>
       </c>
       <c r="BM41" t="n">
-        <v>19.54</v>
+        <v>20.24</v>
       </c>
       <c r="BN41" t="n">
-        <v>19.54</v>
+        <v>20.24</v>
       </c>
       <c r="BO41" t="n">
         <v>13.41</v>
       </c>
       <c r="BP41" t="n">
-        <v>18.04</v>
+        <v>19.59</v>
       </c>
       <c r="BQ41" t="n">
-        <v>8.279999999999999</v>
+        <v>8.550000000000001</v>
       </c>
       <c r="BR41" t="n">
-        <v>18.04</v>
+        <v>19.7</v>
       </c>
       <c r="BS41" t="n">
         <v>0.5600000000000001</v>
       </c>
       <c r="BT41" t="n">
-        <v>10457137</v>
+        <v>11736093</v>
       </c>
     </row>
     <row r="42">
@@ -10005,13 +10005,13 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>21.84</v>
+        <v>22.8</v>
       </c>
       <c r="G42" t="n">
-        <v>229256884001</v>
+        <v>201835420046</v>
       </c>
       <c r="H42" t="n">
-        <v>160447100</v>
+        <v>0</v>
       </c>
       <c r="I42" t="n">
         <v>5288141247</v>
@@ -10026,7 +10026,7 @@
         <v>1.05</v>
       </c>
       <c r="M42" t="n">
-        <v>1.532304955462998</v>
+        <v>1.349025638519507</v>
       </c>
       <c r="N42" t="n">
         <v>0.08</v>
@@ -10104,7 +10104,7 @@
         <v>12268487693.04</v>
       </c>
       <c r="AM42" t="n">
-        <v>31191412789.2517</v>
+        <v>27460601366.80272</v>
       </c>
       <c r="AN42" t="n">
         <v>1.8491</v>
@@ -10145,7 +10145,7 @@
         <v>24.4</v>
       </c>
       <c r="AZ42" t="n">
-        <v>31.63</v>
+        <v>33.02</v>
       </c>
       <c r="BA42" t="n">
         <v>2.53</v>
@@ -10154,19 +10154,19 @@
         <v>15.11</v>
       </c>
       <c r="BC42" t="n">
-        <v>36.84</v>
+        <v>31.08</v>
       </c>
       <c r="BD42" t="n">
-        <v>11.73</v>
+        <v>7.02</v>
       </c>
       <c r="BE42" t="n">
         <v>44.83</v>
       </c>
       <c r="BF42" t="n">
-        <v>-88.43000000000001</v>
+        <v>-88.92</v>
       </c>
       <c r="BG42" t="n">
-        <v>-30.79</v>
+        <v>-33.71</v>
       </c>
       <c r="BH42" t="n">
         <v>17.11</v>
@@ -10175,7 +10175,7 @@
         <v>0</v>
       </c>
       <c r="BJ42" t="n">
-        <v>21.84</v>
+        <v>22.8</v>
       </c>
       <c r="BK42" t="n">
         <v>2.32</v>
@@ -10184,28 +10184,28 @@
         <v>2.34</v>
       </c>
       <c r="BM42" t="n">
-        <v>22.14</v>
+        <v>23</v>
       </c>
       <c r="BN42" t="n">
-        <v>22.14</v>
+        <v>23</v>
       </c>
       <c r="BO42" t="n">
         <v>15.65</v>
       </c>
       <c r="BP42" t="n">
-        <v>20.76</v>
+        <v>22.14</v>
       </c>
       <c r="BQ42" t="n">
-        <v>9.34</v>
+        <v>9.75</v>
       </c>
       <c r="BR42" t="n">
-        <v>20.76</v>
+        <v>22.26</v>
       </c>
       <c r="BS42" t="n">
         <v>0.63</v>
       </c>
       <c r="BT42" t="n">
-        <v>45468250</v>
+        <v>49436283</v>
       </c>
     </row>
     <row r="43">
@@ -10235,13 +10235,13 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>40.99</v>
+        <v>40.08</v>
       </c>
       <c r="G43" t="n">
-        <v>79577948268</v>
+        <v>73544318399</v>
       </c>
       <c r="H43" t="n">
-        <v>10011300</v>
+        <v>0</v>
       </c>
       <c r="I43" t="n">
         <v>1941400000</v>
@@ -10334,7 +10334,7 @@
         <v>9182822000</v>
       </c>
       <c r="AM43" t="n">
-        <v>9692807340.803896</v>
+        <v>8957895054.689402</v>
       </c>
       <c r="AN43" t="n">
         <v>4.5901</v>
@@ -10375,7 +10375,7 @@
         <v>19.95</v>
       </c>
       <c r="AZ43" t="n">
-        <v>74.40000000000001</v>
+        <v>72.75</v>
       </c>
       <c r="BA43" t="n">
         <v>5.63</v>
@@ -10384,19 +10384,19 @@
         <v>48.62</v>
       </c>
       <c r="BC43" t="n">
-        <v>-40.39</v>
+        <v>-39.04</v>
       </c>
       <c r="BD43" t="n">
-        <v>-51.33</v>
+        <v>-50.22</v>
       </c>
       <c r="BE43" t="n">
         <v>81.5</v>
       </c>
       <c r="BF43" t="n">
-        <v>-86.27</v>
+        <v>-85.95999999999999</v>
       </c>
       <c r="BG43" t="n">
-        <v>18.61</v>
+        <v>21.3</v>
       </c>
       <c r="BH43" t="n">
         <v>5.61</v>
@@ -10405,7 +10405,7 @@
         <v>0</v>
       </c>
       <c r="BJ43" t="n">
-        <v>40.99</v>
+        <v>40.08</v>
       </c>
       <c r="BK43" t="n">
         <v>4.73</v>
@@ -10414,7 +10414,7 @@
         <v>4.73</v>
       </c>
       <c r="BM43" t="n">
-        <v>42.42</v>
+        <v>41.7</v>
       </c>
       <c r="BN43" t="n">
         <v>42.98</v>
@@ -10423,19 +10423,19 @@
         <v>28.06</v>
       </c>
       <c r="BP43" t="n">
-        <v>40.88</v>
+        <v>39.8</v>
       </c>
       <c r="BQ43" t="n">
-        <v>8.66</v>
+        <v>8.470000000000001</v>
       </c>
       <c r="BR43" t="n">
-        <v>41.9</v>
+        <v>40.99</v>
       </c>
       <c r="BS43" t="n">
         <v>0</v>
       </c>
       <c r="BT43" t="n">
-        <v>6520643</v>
+        <v>6328787</v>
       </c>
     </row>
     <row r="44">
@@ -10925,13 +10925,13 @@
         </is>
       </c>
       <c r="F46" t="n">
-        <v>4.19</v>
+        <v>4.5</v>
       </c>
       <c r="G46" t="n">
-        <v>4192271037</v>
+        <v>3993295500</v>
       </c>
       <c r="H46" t="n">
-        <v>52029900</v>
+        <v>0</v>
       </c>
       <c r="I46" t="n">
         <v>1000542188</v>
@@ -10946,7 +10946,7 @@
         <v>2.5</v>
       </c>
       <c r="M46" t="n">
-        <v>0.07286955251610387</v>
+        <v>0.06941098358893423</v>
       </c>
       <c r="N46" t="n">
         <v>0.08</v>
@@ -11024,7 +11024,7 @@
         <v>460249406.48</v>
       </c>
       <c r="AM46" t="n">
-        <v>4110069644.117647</v>
+        <v>3914995588.235294</v>
       </c>
       <c r="AN46" t="n">
         <v>0.0311</v>
@@ -11065,7 +11065,7 @@
         <v>3.3</v>
       </c>
       <c r="AZ46" t="n">
-        <v>3.46</v>
+        <v>3.71</v>
       </c>
       <c r="BA46" t="n">
         <v>0.42</v>
@@ -11074,19 +11074,19 @@
         <v>7.38</v>
       </c>
       <c r="BC46" t="n">
-        <v>-3.49</v>
+        <v>-10.14</v>
       </c>
       <c r="BD46" t="n">
-        <v>-21.2</v>
+        <v>-26.63</v>
       </c>
       <c r="BE46" t="n">
         <v>-17.5</v>
       </c>
       <c r="BF46" t="n">
-        <v>-89.90000000000001</v>
+        <v>-90.59999999999999</v>
       </c>
       <c r="BG46" t="n">
-        <v>76.09999999999999</v>
+        <v>63.97</v>
       </c>
       <c r="BH46" t="n">
         <v>1.58</v>
@@ -11095,7 +11095,7 @@
         <v>0</v>
       </c>
       <c r="BJ46" t="n">
-        <v>4.19</v>
+        <v>4.5</v>
       </c>
       <c r="BK46" t="n">
         <v>0.46</v>
@@ -11104,7 +11104,7 @@
         <v>0.46</v>
       </c>
       <c r="BM46" t="n">
-        <v>4.24</v>
+        <v>4.5</v>
       </c>
       <c r="BN46" t="n">
         <v>7.31</v>
@@ -11113,19 +11113,19 @@
         <v>2.97</v>
       </c>
       <c r="BP46" t="n">
-        <v>4.05</v>
+        <v>4.18</v>
       </c>
       <c r="BQ46" t="n">
-        <v>9.16</v>
+        <v>9.84</v>
       </c>
       <c r="BR46" t="n">
-        <v>4.07</v>
+        <v>4.21</v>
       </c>
       <c r="BS46" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="BT46" t="n">
-        <v>21262804</v>
+        <v>22262314</v>
       </c>
     </row>
     <row r="47">
@@ -11155,13 +11155,13 @@
         </is>
       </c>
       <c r="F47" t="n">
-        <v>9.32</v>
+        <v>9.289999999999999</v>
       </c>
       <c r="G47" t="n">
-        <v>3233079002</v>
+        <v>3056806670</v>
       </c>
       <c r="H47" t="n">
-        <v>40800</v>
+        <v>0</v>
       </c>
       <c r="I47" t="n">
         <v>254106600</v>
@@ -11176,7 +11176,7 @@
         <v>1.22</v>
       </c>
       <c r="M47" t="n">
-        <v>0.7623972260863598</v>
+        <v>0.7208301821417362</v>
       </c>
       <c r="N47" t="n">
         <v>0.07000000000000001</v>
@@ -11254,7 +11254,7 @@
         <v>322715382</v>
       </c>
       <c r="AM47" t="n">
-        <v>573240957.8014184</v>
+        <v>541986998.2269504</v>
       </c>
       <c r="AN47" t="n">
         <v>0.4132</v>
@@ -11295,7 +11295,7 @@
         <v>11.74</v>
       </c>
       <c r="AZ47" t="n">
-        <v>12.24</v>
+        <v>12.2</v>
       </c>
       <c r="BA47" t="n">
         <v>1.46</v>
@@ -11304,25 +11304,25 @@
         <v>8.619999999999999</v>
       </c>
       <c r="BC47" t="n">
-        <v>54.22</v>
+        <v>54.72</v>
       </c>
       <c r="BD47" t="n">
-        <v>25.92</v>
+        <v>26.33</v>
       </c>
       <c r="BE47" t="n">
         <v>31.33</v>
       </c>
       <c r="BF47" t="n">
-        <v>-84.34999999999999</v>
+        <v>-84.3</v>
       </c>
       <c r="BG47" t="n">
-        <v>-7.51</v>
+        <v>-7.22</v>
       </c>
       <c r="BH47" t="n">
         <v>7.23</v>
       </c>
       <c r="BI47" t="n">
-        <v>0</v>
+        <v>-0.32</v>
       </c>
       <c r="BJ47" t="n">
         <v>9.32</v>
@@ -11334,28 +11334,28 @@
         <v>1.28</v>
       </c>
       <c r="BM47" t="n">
-        <v>9.59</v>
+        <v>9.6</v>
       </c>
       <c r="BN47" t="n">
-        <v>9.59</v>
+        <v>9.6</v>
       </c>
       <c r="BO47" t="n">
         <v>7.12</v>
       </c>
       <c r="BP47" t="n">
-        <v>8.83</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="BQ47" t="n">
-        <v>7.27</v>
+        <v>7.24</v>
       </c>
       <c r="BR47" t="n">
-        <v>9.5</v>
+        <v>9.27</v>
       </c>
       <c r="BS47" t="n">
         <v>0.53</v>
       </c>
       <c r="BT47" t="n">
-        <v>11063</v>
+        <v>12140</v>
       </c>
     </row>
     <row r="48">
@@ -11385,13 +11385,13 @@
         </is>
       </c>
       <c r="F48" t="n">
-        <v>9.210000000000001</v>
+        <v>9.19</v>
       </c>
       <c r="G48" t="n">
-        <v>3233079002</v>
+        <v>3056806670</v>
       </c>
       <c r="H48" t="n">
-        <v>3600</v>
+        <v>0</v>
       </c>
       <c r="I48" t="n">
         <v>93397546</v>
@@ -11406,7 +11406,7 @@
         <v>1.24</v>
       </c>
       <c r="M48" t="n">
-        <v>2.074253288948686</v>
+        <v>1.961161878508214</v>
       </c>
       <c r="N48" t="n">
         <v>0.07000000000000001</v>
@@ -11484,7 +11484,7 @@
         <v>118614883.42</v>
       </c>
       <c r="AM48" t="n">
-        <v>565223601.7482518</v>
+        <v>534406760.4895105</v>
       </c>
       <c r="AN48" t="n">
         <v>0.4132</v>
@@ -11525,7 +11525,7 @@
         <v>11.74</v>
       </c>
       <c r="AZ48" t="n">
-        <v>12.05</v>
+        <v>12.02</v>
       </c>
       <c r="BA48" t="n">
         <v>1.46</v>
@@ -11534,25 +11534,25 @@
         <v>8.24</v>
       </c>
       <c r="BC48" t="n">
-        <v>56.06</v>
+        <v>56.4</v>
       </c>
       <c r="BD48" t="n">
-        <v>27.43</v>
+        <v>27.7</v>
       </c>
       <c r="BE48" t="n">
         <v>30.83</v>
       </c>
       <c r="BF48" t="n">
-        <v>-84.16</v>
+        <v>-84.13</v>
       </c>
       <c r="BG48" t="n">
-        <v>-10.57</v>
+        <v>-10.38</v>
       </c>
       <c r="BH48" t="n">
         <v>7.23</v>
       </c>
       <c r="BI48" t="n">
-        <v>0</v>
+        <v>-0.22</v>
       </c>
       <c r="BJ48" t="n">
         <v>9.210000000000001</v>
@@ -11564,28 +11564,28 @@
         <v>1.28</v>
       </c>
       <c r="BM48" t="n">
-        <v>9.5</v>
+        <v>9.529999999999999</v>
       </c>
       <c r="BN48" t="n">
-        <v>9.5</v>
+        <v>9.529999999999999</v>
       </c>
       <c r="BO48" t="n">
         <v>7.13</v>
       </c>
       <c r="BP48" t="n">
-        <v>9.17</v>
+        <v>9.19</v>
       </c>
       <c r="BQ48" t="n">
-        <v>7.18</v>
+        <v>7.16</v>
       </c>
       <c r="BR48" t="n">
-        <v>9.5</v>
+        <v>9.529999999999999</v>
       </c>
       <c r="BS48" t="n">
         <v>0.54</v>
       </c>
       <c r="BT48" t="n">
-        <v>2677</v>
+        <v>2763</v>
       </c>
     </row>
     <row r="49">
@@ -11845,13 +11845,13 @@
         </is>
       </c>
       <c r="F50" t="n">
-        <v>34.01</v>
+        <v>34.41</v>
       </c>
       <c r="G50" t="n">
-        <v>934898060</v>
+        <v>908275800</v>
       </c>
       <c r="H50" t="n">
-        <v>1400</v>
+        <v>0</v>
       </c>
       <c r="I50" t="n">
         <v>11540870</v>
@@ -11866,7 +11866,7 @@
         <v>0.8</v>
       </c>
       <c r="M50" t="n">
-        <v>0.9458243084961065</v>
+        <v>0.9188909114419898</v>
       </c>
       <c r="N50" t="n">
         <v>0.06</v>
@@ -11944,7 +11944,7 @@
         <v>84709985.8</v>
       </c>
       <c r="AM50" t="n">
-        <v>319077836.1774744</v>
+        <v>309991740.6143345</v>
       </c>
       <c r="AN50" t="n">
         <v>4.4983</v>
@@ -11985,7 +11985,7 @@
         <v>68.48999999999999</v>
       </c>
       <c r="AZ50" t="n">
-        <v>74.98999999999999</v>
+        <v>75.87</v>
       </c>
       <c r="BA50" t="n">
         <v>9.210000000000001</v>
@@ -11994,25 +11994,25 @@
         <v>30.53</v>
       </c>
       <c r="BC50" t="n">
-        <v>146.63</v>
+        <v>143.76</v>
       </c>
       <c r="BD50" t="n">
-        <v>101.37</v>
+        <v>99.03</v>
       </c>
       <c r="BE50" t="n">
         <v>120.5</v>
       </c>
       <c r="BF50" t="n">
-        <v>-72.91</v>
+        <v>-73.22</v>
       </c>
       <c r="BG50" t="n">
-        <v>-10.23</v>
+        <v>-11.27</v>
       </c>
       <c r="BH50" t="n">
         <v>42.6</v>
       </c>
       <c r="BI50" t="n">
-        <v>0</v>
+        <v>1.18</v>
       </c>
       <c r="BJ50" t="n">
         <v>34.01</v>
@@ -12024,28 +12024,28 @@
         <v>7.6</v>
       </c>
       <c r="BM50" t="n">
-        <v>34.69</v>
+        <v>34.42</v>
       </c>
       <c r="BN50" t="n">
         <v>39.22</v>
       </c>
       <c r="BO50" t="n">
-        <v>24.24</v>
+        <v>24.28</v>
       </c>
       <c r="BP50" t="n">
-        <v>33.14</v>
+        <v>33.92</v>
       </c>
       <c r="BQ50" t="n">
-        <v>4.47</v>
+        <v>4.53</v>
       </c>
       <c r="BR50" t="n">
-        <v>33.14</v>
+        <v>33.92</v>
       </c>
       <c r="BS50" t="n">
         <v>0.4</v>
       </c>
       <c r="BT50" t="n">
-        <v>483</v>
+        <v>517</v>
       </c>
     </row>
     <row r="51">
@@ -12523,13 +12523,13 @@
         </is>
       </c>
       <c r="F53" t="n">
-        <v>6.44</v>
+        <v>6.86</v>
       </c>
       <c r="G53" t="n">
-        <v>881329463</v>
+        <v>900567783</v>
       </c>
       <c r="H53" t="n">
-        <v>88100</v>
+        <v>0</v>
       </c>
       <c r="I53" t="n">
         <v>136852484</v>
@@ -12544,7 +12544,7 @@
         <v>2.79</v>
       </c>
       <c r="M53" t="n">
-        <v>2.289529647354219</v>
+        <v>2.339507216304831</v>
       </c>
       <c r="N53" t="n">
         <v>1.48</v>
@@ -12622,7 +12622,7 @@
         <v>39687220.36</v>
       </c>
       <c r="AM53" t="n">
-        <v>44897068.92511462</v>
+        <v>45877115.79215487</v>
       </c>
       <c r="AN53" t="n">
         <v>0</v>
@@ -12672,16 +12672,16 @@
         <v>0</v>
       </c>
       <c r="BC53" t="n">
-        <v>-38.81</v>
+        <v>-42.55</v>
       </c>
       <c r="BD53" t="n">
-        <v>-50.04</v>
+        <v>-53.1</v>
       </c>
       <c r="BE53" t="n">
         <v>-100</v>
       </c>
       <c r="BF53" t="n">
-        <v>-95.5</v>
+        <v>-95.77</v>
       </c>
       <c r="BG53" t="n">
         <v>-100</v>
@@ -12693,7 +12693,7 @@
         <v>0</v>
       </c>
       <c r="BJ53" t="n">
-        <v>6.44</v>
+        <v>6.86</v>
       </c>
       <c r="BK53" t="n">
         <v>0.29</v>
@@ -12702,7 +12702,7 @@
         <v>0.2</v>
       </c>
       <c r="BM53" t="n">
-        <v>7.4</v>
+        <v>6.86</v>
       </c>
       <c r="BN53" t="n">
         <v>10.39</v>
@@ -12711,19 +12711,19 @@
         <v>4.82</v>
       </c>
       <c r="BP53" t="n">
-        <v>6.33</v>
+        <v>6.43</v>
       </c>
       <c r="BQ53" t="n">
-        <v>31.63</v>
+        <v>33.7</v>
       </c>
       <c r="BR53" t="n">
-        <v>6.56</v>
+        <v>6.43</v>
       </c>
       <c r="BS53" t="n">
         <v>2.36</v>
       </c>
       <c r="BT53" t="n">
-        <v>38407</v>
+        <v>40470</v>
       </c>
     </row>
     <row r="54">
@@ -12753,13 +12753,13 @@
         </is>
       </c>
       <c r="F54" t="n">
-        <v>11.68</v>
+        <v>11.95</v>
       </c>
       <c r="G54" t="n">
-        <v>2723917399</v>
+        <v>2472687985</v>
       </c>
       <c r="H54" t="n">
-        <v>784000</v>
+        <v>0</v>
       </c>
       <c r="I54" t="n">
         <v>233212121</v>
@@ -12774,7 +12774,7 @@
         <v>0.97</v>
       </c>
       <c r="M54" t="n">
-        <v>1.528911902178103</v>
+        <v>1.387898947312863</v>
       </c>
       <c r="N54" t="n">
         <v>0.5600000000000001</v>
@@ -12852,7 +12852,7 @@
         <v>233212121</v>
       </c>
       <c r="AM54" t="n">
-        <v>372628919.1518468</v>
+        <v>338261010.2599179</v>
       </c>
       <c r="AN54" t="n">
         <v>0.1531</v>
@@ -12893,7 +12893,7 @@
         <v>12.25</v>
       </c>
       <c r="AZ54" t="n">
-        <v>18.59</v>
+        <v>19.02</v>
       </c>
       <c r="BA54" t="n">
         <v>0.98</v>
@@ -12902,25 +12902,25 @@
         <v>6.52</v>
       </c>
       <c r="BC54" t="n">
-        <v>28.49</v>
+        <v>25.59</v>
       </c>
       <c r="BD54" t="n">
-        <v>4.91</v>
+        <v>2.54</v>
       </c>
       <c r="BE54" t="n">
         <v>59.17</v>
       </c>
       <c r="BF54" t="n">
-        <v>-91.58</v>
+        <v>-91.77</v>
       </c>
       <c r="BG54" t="n">
-        <v>-44.21</v>
+        <v>-45.47</v>
       </c>
       <c r="BH54" t="n">
         <v>10.01</v>
       </c>
       <c r="BI54" t="n">
-        <v>0</v>
+        <v>2.31</v>
       </c>
       <c r="BJ54" t="n">
         <v>11.68</v>
@@ -12932,28 +12932,28 @@
         <v>1</v>
       </c>
       <c r="BM54" t="n">
-        <v>11.95</v>
+        <v>12.15</v>
       </c>
       <c r="BN54" t="n">
-        <v>11.95</v>
+        <v>12.15</v>
       </c>
       <c r="BO54" t="n">
         <v>8.23</v>
       </c>
       <c r="BP54" t="n">
-        <v>11.05</v>
+        <v>11.54</v>
       </c>
       <c r="BQ54" t="n">
-        <v>11.65</v>
+        <v>11.92</v>
       </c>
       <c r="BR54" t="n">
-        <v>11.05</v>
+        <v>11.59</v>
       </c>
       <c r="BS54" t="n">
         <v>1.26</v>
       </c>
       <c r="BT54" t="n">
-        <v>248483</v>
+        <v>267900</v>
       </c>
     </row>
     <row r="55">
@@ -12983,13 +12983,13 @@
         </is>
       </c>
       <c r="F55" t="n">
-        <v>55</v>
+        <v>55.44</v>
       </c>
       <c r="G55" t="n">
-        <v>7324848245</v>
+        <v>6835589641</v>
       </c>
       <c r="H55" t="n">
-        <v>16200</v>
+        <v>0</v>
       </c>
       <c r="I55" t="n">
         <v>84052790</v>
@@ -13004,7 +13004,7 @@
         <v>2</v>
       </c>
       <c r="M55" t="n">
-        <v>1.130745308787714</v>
+        <v>1.055217891324197</v>
       </c>
       <c r="N55" t="n">
         <v>0.16</v>
@@ -13082,7 +13082,7 @@
         <v>579123723.1</v>
       </c>
       <c r="AM55" t="n">
-        <v>368453131.0362173</v>
+        <v>343842537.2736419</v>
       </c>
       <c r="AN55" t="n">
         <v>3.1953</v>
@@ -13123,7 +13123,7 @@
         <v>51.21</v>
       </c>
       <c r="AZ55" t="n">
-        <v>57.84</v>
+        <v>58.3</v>
       </c>
       <c r="BA55" t="n">
         <v>9.380000000000001</v>
@@ -13132,19 +13132,19 @@
         <v>16.08</v>
       </c>
       <c r="BC55" t="n">
-        <v>14.02</v>
+        <v>13.12</v>
       </c>
       <c r="BD55" t="n">
-        <v>-6.9</v>
+        <v>-7.64</v>
       </c>
       <c r="BE55" t="n">
         <v>5.17</v>
       </c>
       <c r="BF55" t="n">
-        <v>-82.95</v>
+        <v>-83.08</v>
       </c>
       <c r="BG55" t="n">
-        <v>-70.77</v>
+        <v>-71</v>
       </c>
       <c r="BH55" t="n">
         <v>25.37</v>
@@ -13153,7 +13153,7 @@
         <v>0</v>
       </c>
       <c r="BJ55" t="n">
-        <v>55</v>
+        <v>55.44</v>
       </c>
       <c r="BK55" t="n">
         <v>6.89</v>
@@ -13162,7 +13162,7 @@
         <v>7.03</v>
       </c>
       <c r="BM55" t="n">
-        <v>55</v>
+        <v>56.39</v>
       </c>
       <c r="BN55" t="n">
         <v>73.67</v>
@@ -13171,19 +13171,19 @@
         <v>35.58</v>
       </c>
       <c r="BP55" t="n">
-        <v>51.21</v>
+        <v>54.42</v>
       </c>
       <c r="BQ55" t="n">
-        <v>7.82</v>
+        <v>7.89</v>
       </c>
       <c r="BR55" t="n">
-        <v>51.21</v>
+        <v>54.92</v>
       </c>
       <c r="BS55" t="n">
         <v>0.66</v>
       </c>
       <c r="BT55" t="n">
-        <v>5950</v>
+        <v>6290</v>
       </c>
     </row>
     <row r="56">
@@ -13213,13 +13213,13 @@
         </is>
       </c>
       <c r="F56" t="n">
-        <v>66.73999999999999</v>
+        <v>71.23999999999999</v>
       </c>
       <c r="G56" t="n">
-        <v>7324848245</v>
+        <v>6835589641</v>
       </c>
       <c r="H56" t="n">
-        <v>45500</v>
+        <v>35700</v>
       </c>
       <c r="I56" t="n">
         <v>39675836</v>
@@ -13234,7 +13234,7 @@
         <v>2.41</v>
       </c>
       <c r="M56" t="n">
-        <v>2.395470582724933</v>
+        <v>2.235466640796568</v>
       </c>
       <c r="N56" t="n">
         <v>0.19</v>
@@ -13312,7 +13312,7 @@
         <v>273366510.04</v>
       </c>
       <c r="AM56" t="n">
-        <v>304694186.5640599</v>
+        <v>284342331.156406</v>
       </c>
       <c r="AN56" t="n">
         <v>3.5102</v>
@@ -13353,7 +13353,7 @@
         <v>51.21</v>
       </c>
       <c r="AZ56" t="n">
-        <v>63.74</v>
+        <v>68.03</v>
       </c>
       <c r="BA56" t="n">
         <v>9.380000000000001</v>
@@ -13362,19 +13362,19 @@
         <v>17.68</v>
       </c>
       <c r="BC56" t="n">
-        <v>-6.03</v>
+        <v>-11.97</v>
       </c>
       <c r="BD56" t="n">
-        <v>-23.28</v>
+        <v>-28.12</v>
       </c>
       <c r="BE56" t="n">
         <v>-4.5</v>
       </c>
       <c r="BF56" t="n">
-        <v>-85.95</v>
+        <v>-86.84</v>
       </c>
       <c r="BG56" t="n">
-        <v>-73.51000000000001</v>
+        <v>-75.19</v>
       </c>
       <c r="BH56" t="n">
         <v>25.37</v>
@@ -13383,7 +13383,7 @@
         <v>0</v>
       </c>
       <c r="BJ56" t="n">
-        <v>66.73999999999999</v>
+        <v>71.23999999999999</v>
       </c>
       <c r="BK56" t="n">
         <v>6.89</v>
@@ -13392,7 +13392,7 @@
         <v>7.03</v>
       </c>
       <c r="BM56" t="n">
-        <v>68.5</v>
+        <v>71.37</v>
       </c>
       <c r="BN56" t="n">
         <v>86.77</v>
@@ -13401,19 +13401,19 @@
         <v>46.42</v>
       </c>
       <c r="BP56" t="n">
-        <v>61.78</v>
+        <v>67.36</v>
       </c>
       <c r="BQ56" t="n">
-        <v>9.49</v>
+        <v>10.13</v>
       </c>
       <c r="BR56" t="n">
-        <v>61.78</v>
+        <v>67.36</v>
       </c>
       <c r="BS56" t="n">
         <v>0.79</v>
       </c>
       <c r="BT56" t="n">
-        <v>28753</v>
+        <v>27717</v>
       </c>
     </row>
     <row r="57">
@@ -13443,13 +13443,13 @@
         </is>
       </c>
       <c r="F57" t="n">
-        <v>6.9</v>
+        <v>6.87</v>
       </c>
       <c r="G57" t="n">
-        <v>1613620912</v>
+        <v>1469640680</v>
       </c>
       <c r="H57" t="n">
-        <v>3624100</v>
+        <v>1858700</v>
       </c>
       <c r="I57" t="n">
         <v>233858065</v>
@@ -13464,7 +13464,7 @@
         <v>0.77</v>
       </c>
       <c r="M57" t="n">
-        <v>0.4830000788726274</v>
+        <v>0.4399029282996933</v>
       </c>
       <c r="N57" t="n">
         <v>0.08</v>
@@ -13542,7 +13542,7 @@
         <v>229180903.7</v>
       </c>
       <c r="AM57" t="n">
-        <v>120689671.802543</v>
+        <v>109920768.8855647</v>
       </c>
       <c r="AN57" t="n">
         <v>0.347</v>
@@ -13583,7 +13583,7 @@
         <v>10.72</v>
       </c>
       <c r="AZ57" t="n">
-        <v>10.52</v>
+        <v>10.48</v>
       </c>
       <c r="BA57" t="n">
         <v>1.13</v>
@@ -13592,19 +13592,19 @@
         <v>6.26</v>
       </c>
       <c r="BC57" t="n">
-        <v>90.31</v>
+        <v>91.14</v>
       </c>
       <c r="BD57" t="n">
-        <v>55.39</v>
+        <v>56.06</v>
       </c>
       <c r="BE57" t="n">
         <v>52.5</v>
       </c>
       <c r="BF57" t="n">
-        <v>-83.66</v>
+        <v>-83.59</v>
       </c>
       <c r="BG57" t="n">
-        <v>-9.220000000000001</v>
+        <v>-8.82</v>
       </c>
       <c r="BH57" t="n">
         <v>7.82</v>
@@ -13613,7 +13613,7 @@
         <v>0</v>
       </c>
       <c r="BJ57" t="n">
-        <v>6.9</v>
+        <v>6.87</v>
       </c>
       <c r="BK57" t="n">
         <v>0.98</v>
@@ -13622,7 +13622,7 @@
         <v>1.04</v>
       </c>
       <c r="BM57" t="n">
-        <v>7.03</v>
+        <v>6.98</v>
       </c>
       <c r="BN57" t="n">
         <v>7.03</v>
@@ -13631,19 +13631,19 @@
         <v>3.43</v>
       </c>
       <c r="BP57" t="n">
-        <v>6.64</v>
+        <v>6.78</v>
       </c>
       <c r="BQ57" t="n">
-        <v>6.66</v>
+        <v>6.63</v>
       </c>
       <c r="BR57" t="n">
-        <v>6.64</v>
+        <v>6.9</v>
       </c>
       <c r="BS57" t="n">
         <v>0.42</v>
       </c>
       <c r="BT57" t="n">
-        <v>1490457</v>
+        <v>1582530</v>
       </c>
     </row>
     <row r="58">
@@ -14133,13 +14133,13 @@
         </is>
       </c>
       <c r="F60" t="n">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="G60" t="n">
-        <v>171440787</v>
+        <v>159992274</v>
       </c>
       <c r="H60" t="n">
-        <v>51</v>
+        <v>0</v>
       </c>
       <c r="I60" t="n">
         <v>454750</v>
@@ -14154,7 +14154,7 @@
         <v>0.83</v>
       </c>
       <c r="M60" t="n">
-        <v>12.82352952940177</v>
+        <v>11.96719687314046</v>
       </c>
       <c r="N60" t="n">
         <v>0.68</v>
@@ -14232,7 +14232,7 @@
         <v>59558607.5</v>
       </c>
       <c r="AM60" t="n">
-        <v>-25137945.30791789</v>
+        <v>-23459277.71260997</v>
       </c>
       <c r="AN60" t="n">
         <v>10.0581</v>
@@ -14273,7 +14273,7 @@
         <v>944.87</v>
       </c>
       <c r="AZ60" t="n">
-        <v>2167.75</v>
+        <v>2185</v>
       </c>
       <c r="BA60" t="n">
         <v>231.1</v>
@@ -14282,25 +14282,25 @@
         <v>727.97</v>
       </c>
       <c r="BC60" t="n">
-        <v>206.95</v>
+        <v>204.53</v>
       </c>
       <c r="BD60" t="n">
-        <v>150.63</v>
+        <v>148.65</v>
       </c>
       <c r="BE60" t="n">
         <v>475</v>
       </c>
       <c r="BF60" t="n">
-        <v>-38.7</v>
+        <v>-39.19</v>
       </c>
       <c r="BG60" t="n">
-        <v>93.09999999999999</v>
+        <v>91.56999999999999</v>
       </c>
       <c r="BH60" t="n">
         <v>454.44</v>
       </c>
       <c r="BI60" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="BJ60" t="n">
         <v>377</v>
@@ -14321,19 +14321,19 @@
         <v>309.24</v>
       </c>
       <c r="BP60" t="n">
-        <v>375</v>
+        <v>380</v>
       </c>
       <c r="BQ60" t="n">
-        <v>2.88</v>
+        <v>2.9</v>
       </c>
       <c r="BR60" t="n">
-        <v>375</v>
+        <v>390</v>
       </c>
       <c r="BS60" t="n">
         <v>12.82</v>
       </c>
       <c r="BT60" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="61">
@@ -14366,10 +14366,10 @@
         <v>30.53</v>
       </c>
       <c r="G61" t="n">
-        <v>2613624205</v>
+        <v>2323711013</v>
       </c>
       <c r="H61" t="n">
-        <v>2032400</v>
+        <v>0</v>
       </c>
       <c r="I61" t="n">
         <v>85608392</v>
@@ -14384,7 +14384,7 @@
         <v>2.37</v>
       </c>
       <c r="M61" t="n">
-        <v>1.386094650942694</v>
+        <v>1.232343731472264</v>
       </c>
       <c r="N61" t="n">
         <v>1.1</v>
@@ -14462,7 +14462,7 @@
         <v>160087693.04</v>
       </c>
       <c r="AM61" t="n">
-        <v>205151036.4992151</v>
+        <v>182394898.9795918</v>
       </c>
       <c r="AN61" t="n">
         <v>0.38</v>
@@ -14542,7 +14542,7 @@
         <v>1.86</v>
       </c>
       <c r="BM61" t="n">
-        <v>30.75</v>
+        <v>30.65</v>
       </c>
       <c r="BN61" t="n">
         <v>30.75</v>
@@ -14551,19 +14551,19 @@
         <v>19.35</v>
       </c>
       <c r="BP61" t="n">
-        <v>28.82</v>
+        <v>30.14</v>
       </c>
       <c r="BQ61" t="n">
         <v>16.4</v>
       </c>
       <c r="BR61" t="n">
-        <v>28.82</v>
+        <v>30.51</v>
       </c>
       <c r="BS61" t="n">
         <v>1.19</v>
       </c>
       <c r="BT61" t="n">
-        <v>705237</v>
+        <v>763527</v>
       </c>
     </row>
     <row r="62">
@@ -14593,13 +14593,13 @@
         </is>
       </c>
       <c r="F62" t="n">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="G62" t="n">
-        <v>11251769220</v>
+        <v>10494785730</v>
       </c>
       <c r="H62" t="n">
-        <v>200</v>
+        <v>500</v>
       </c>
       <c r="I62" t="n">
         <v>98699749</v>
@@ -14614,7 +14614,7 @@
         <v>0.64</v>
       </c>
       <c r="M62" t="n">
-        <v>1.054724206411182</v>
+        <v>0.9837656935634919</v>
       </c>
       <c r="N62" t="n">
         <v>0.13</v>
@@ -14692,7 +14692,7 @@
         <v>2757670987.06</v>
       </c>
       <c r="AM62" t="n">
-        <v>4555372153.846153</v>
+        <v>4248901105.263157</v>
       </c>
       <c r="AN62" t="n">
         <v>6.9319</v>
@@ -14733,7 +14733,7 @@
         <v>267.2</v>
       </c>
       <c r="AZ62" t="n">
-        <v>120.46</v>
+        <v>119.4</v>
       </c>
       <c r="BA62" t="n">
         <v>34.09</v>
@@ -14742,19 +14742,19 @@
         <v>76.01000000000001</v>
       </c>
       <c r="BC62" t="n">
-        <v>187.06</v>
+        <v>189.6</v>
       </c>
       <c r="BD62" t="n">
-        <v>134.38</v>
+        <v>136.46</v>
       </c>
       <c r="BE62" t="n">
         <v>5.67</v>
       </c>
       <c r="BF62" t="n">
-        <v>-70.09</v>
+        <v>-69.83</v>
       </c>
       <c r="BG62" t="n">
-        <v>-33.33</v>
+        <v>-32.74</v>
       </c>
       <c r="BH62" t="n">
         <v>170.35</v>
@@ -14763,7 +14763,7 @@
         <v>0</v>
       </c>
       <c r="BJ62" t="n">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="BK62" t="n">
         <v>27.94</v>
@@ -14772,7 +14772,7 @@
         <v>32.73</v>
       </c>
       <c r="BM62" t="n">
-        <v>114.45</v>
+        <v>114.25</v>
       </c>
       <c r="BN62" t="n">
         <v>122.2</v>
@@ -14781,19 +14781,19 @@
         <v>91.84999999999999</v>
       </c>
       <c r="BP62" t="n">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="BQ62" t="n">
-        <v>3.48</v>
+        <v>3.45</v>
       </c>
       <c r="BR62" t="n">
-        <v>114.45</v>
+        <v>114.25</v>
       </c>
       <c r="BS62" t="n">
         <v>1.01</v>
       </c>
       <c r="BT62" t="n">
-        <v>120</v>
+        <v>123</v>
       </c>
     </row>
     <row r="63">
@@ -14823,13 +14823,13 @@
         </is>
       </c>
       <c r="F63" t="n">
-        <v>1.56</v>
+        <v>1.62</v>
       </c>
       <c r="G63" t="n">
-        <v>406395117</v>
+        <v>414572257</v>
       </c>
       <c r="H63" t="n">
-        <v>11600</v>
+        <v>81700</v>
       </c>
       <c r="I63" t="n">
         <v>122894462</v>
@@ -14844,7 +14844,7 @@
         <v>-0.22</v>
       </c>
       <c r="M63" t="n">
-        <v>0.4998450214354843</v>
+        <v>0.5099024816450295</v>
       </c>
       <c r="N63" t="n">
         <v>0.37</v>
@@ -14922,7 +14922,7 @@
         <v>31952560.12</v>
       </c>
       <c r="AM63" t="n">
-        <v>230906316.4772727</v>
+        <v>235552418.75</v>
       </c>
       <c r="AN63" t="n">
         <v>0</v>
@@ -14981,7 +14981,7 @@
         <v>-100</v>
       </c>
       <c r="BF63" t="n">
-        <v>-81.45999999999999</v>
+        <v>-82.15000000000001</v>
       </c>
       <c r="BG63" t="n">
         <v>-100</v>
@@ -14993,7 +14993,7 @@
         <v>0</v>
       </c>
       <c r="BJ63" t="n">
-        <v>1.56</v>
+        <v>1.62</v>
       </c>
       <c r="BK63" t="n">
         <v>0.26</v>
@@ -15002,7 +15002,7 @@
         <v>0.26</v>
       </c>
       <c r="BM63" t="n">
-        <v>1.68</v>
+        <v>1.7</v>
       </c>
       <c r="BN63" t="n">
         <v>2.12</v>
@@ -15011,19 +15011,19 @@
         <v>1.16</v>
       </c>
       <c r="BP63" t="n">
-        <v>1.52</v>
+        <v>1.58</v>
       </c>
       <c r="BQ63" t="n">
-        <v>5.98</v>
+        <v>6.21</v>
       </c>
       <c r="BR63" t="n">
-        <v>1.56</v>
+        <v>1.58</v>
       </c>
       <c r="BS63" t="n">
         <v>0.19</v>
       </c>
       <c r="BT63" t="n">
-        <v>33890</v>
+        <v>33517</v>
       </c>
     </row>
     <row r="64">
@@ -15053,13 +15053,13 @@
         </is>
       </c>
       <c r="F64" t="n">
-        <v>80.89</v>
+        <v>78.62</v>
       </c>
       <c r="G64" t="n">
-        <v>299780602658</v>
+        <v>227765685856</v>
       </c>
       <c r="H64" t="n">
-        <v>61965300</v>
+        <v>0</v>
       </c>
       <c r="I64" t="n">
         <v>0</v>
@@ -15146,13 +15146,13 @@
         <v>41.22</v>
       </c>
       <c r="AK64" t="n">
-        <v>85951497814.08733</v>
+        <v>65303764407.6991</v>
       </c>
       <c r="AL64" t="n">
-        <v>23963277590.56755</v>
+        <v>18206689516.86651</v>
       </c>
       <c r="AM64" t="n">
-        <v>26694621786.10863</v>
+        <v>20281895445.77026</v>
       </c>
       <c r="AN64" t="n">
         <v>1.4201</v>
@@ -15193,7 +15193,7 @@
         <v>38.98</v>
       </c>
       <c r="AZ64" t="n">
-        <v>32.36</v>
+        <v>31.45</v>
       </c>
       <c r="BA64" t="n">
         <v>6.69</v>
@@ -15202,25 +15202,25 @@
         <v>10.4</v>
       </c>
       <c r="BC64" t="n">
-        <v>-40.98</v>
+        <v>-39.28</v>
       </c>
       <c r="BD64" t="n">
-        <v>-51.81</v>
+        <v>-50.42</v>
       </c>
       <c r="BE64" t="n">
         <v>-60</v>
       </c>
       <c r="BF64" t="n">
-        <v>-91.72</v>
+        <v>-91.48999999999999</v>
       </c>
       <c r="BG64" t="n">
-        <v>-87.15000000000001</v>
+        <v>-86.77</v>
       </c>
       <c r="BH64" t="n">
         <v>21.37</v>
       </c>
       <c r="BI64" t="n">
-        <v>0</v>
+        <v>-2.81</v>
       </c>
       <c r="BJ64" t="n">
         <v>80.89</v>
@@ -15232,7 +15232,7 @@
         <v>1.57</v>
       </c>
       <c r="BM64" t="n">
-        <v>84.59</v>
+        <v>82.5</v>
       </c>
       <c r="BN64" t="n">
         <v>84.59</v>
@@ -15241,19 +15241,19 @@
         <v>44.12</v>
       </c>
       <c r="BP64" t="n">
-        <v>75.40000000000001</v>
+        <v>76.70999999999999</v>
       </c>
       <c r="BQ64" t="n">
-        <v>51.52</v>
+        <v>50.07</v>
       </c>
       <c r="BR64" t="n">
-        <v>76</v>
+        <v>81.26000000000001</v>
       </c>
       <c r="BS64" t="n">
         <v>3.49</v>
       </c>
       <c r="BT64" t="n">
-        <v>10726917</v>
+        <v>12347880</v>
       </c>
     </row>
     <row r="65">
@@ -15283,13 +15283,13 @@
         </is>
       </c>
       <c r="F65" t="n">
-        <v>27.71</v>
+        <v>27</v>
       </c>
       <c r="G65" t="n">
-        <v>299780602658</v>
+        <v>227765685856</v>
       </c>
       <c r="H65" t="n">
-        <v>64500</v>
+        <v>41100</v>
       </c>
       <c r="I65" t="n">
         <v>7298813414</v>
@@ -15304,7 +15304,7 @@
         <v>3.29</v>
       </c>
       <c r="M65" t="n">
-        <v>7.247478726962274</v>
+        <v>5.506450211712123</v>
       </c>
       <c r="N65" t="n">
         <v>0.29</v>
@@ -15382,7 +15382,7 @@
         <v>11532125194.12</v>
       </c>
       <c r="AM65" t="n">
-        <v>22455475854.53184</v>
+        <v>17061100064.11985</v>
       </c>
       <c r="AN65" t="n">
         <v>0.4734</v>
@@ -15423,7 +15423,7 @@
         <v>12.99</v>
       </c>
       <c r="AZ65" t="n">
-        <v>9.33</v>
+        <v>9.09</v>
       </c>
       <c r="BA65" t="n">
         <v>2.23</v>
@@ -15432,19 +15432,19 @@
         <v>3.47</v>
       </c>
       <c r="BC65" t="n">
-        <v>-42.59</v>
+        <v>-41.08</v>
       </c>
       <c r="BD65" t="n">
-        <v>-53.12</v>
+        <v>-51.89</v>
       </c>
       <c r="BE65" t="n">
         <v>-66.33</v>
       </c>
       <c r="BF65" t="n">
-        <v>-91.95</v>
+        <v>-91.73999999999999</v>
       </c>
       <c r="BG65" t="n">
-        <v>-87.48999999999999</v>
+        <v>-87.16</v>
       </c>
       <c r="BH65" t="n">
         <v>7.12</v>
@@ -15453,7 +15453,7 @@
         <v>0</v>
       </c>
       <c r="BJ65" t="n">
-        <v>27.71</v>
+        <v>27</v>
       </c>
       <c r="BK65" t="n">
         <v>1.58</v>
@@ -15462,7 +15462,7 @@
         <v>1.57</v>
       </c>
       <c r="BM65" t="n">
-        <v>28.5</v>
+        <v>28.72</v>
       </c>
       <c r="BN65" t="n">
         <v>46.43</v>
@@ -15471,19 +15471,19 @@
         <v>20.44</v>
       </c>
       <c r="BP65" t="n">
-        <v>26.11</v>
+        <v>26.13</v>
       </c>
       <c r="BQ65" t="n">
-        <v>17.65</v>
+        <v>17.2</v>
       </c>
       <c r="BR65" t="n">
-        <v>26.11</v>
+        <v>27.99</v>
       </c>
       <c r="BS65" t="n">
         <v>4.14</v>
       </c>
       <c r="BT65" t="n">
-        <v>7650</v>
+        <v>9137</v>
       </c>
     </row>
     <row r="66">
@@ -15513,13 +15513,13 @@
         </is>
       </c>
       <c r="F66" t="n">
-        <v>25.31</v>
+        <v>25.99</v>
       </c>
       <c r="G66" t="n">
-        <v>299780602658</v>
+        <v>227765685856</v>
       </c>
       <c r="H66" t="n">
-        <v>24000</v>
+        <v>17200</v>
       </c>
       <c r="I66" t="n">
         <v>2972355254</v>
@@ -15534,7 +15534,7 @@
         <v>2.75</v>
       </c>
       <c r="M66" t="n">
-        <v>17.79665969565557</v>
+        <v>13.5214499056537</v>
       </c>
       <c r="N66" t="n">
         <v>0.25</v>
@@ -15612,7 +15612,7 @@
         <v>4696321301.320001</v>
       </c>
       <c r="AM66" t="n">
-        <v>26886152704.75336</v>
+        <v>20427415771.83857</v>
       </c>
       <c r="AN66" t="n">
         <v>0.4734</v>
@@ -15653,7 +15653,7 @@
         <v>12.99</v>
       </c>
       <c r="AZ66" t="n">
-        <v>10.17</v>
+        <v>10.44</v>
       </c>
       <c r="BA66" t="n">
         <v>2.23</v>
@@ -15662,19 +15662,19 @@
         <v>3.47</v>
       </c>
       <c r="BC66" t="n">
-        <v>-37.14</v>
+        <v>-38.79</v>
       </c>
       <c r="BD66" t="n">
-        <v>-48.68</v>
+        <v>-50.02</v>
       </c>
       <c r="BE66" t="n">
         <v>-59.83</v>
       </c>
       <c r="BF66" t="n">
-        <v>-91.18000000000001</v>
+        <v>-91.41</v>
       </c>
       <c r="BG66" t="n">
-        <v>-86.31</v>
+        <v>-86.67</v>
       </c>
       <c r="BH66" t="n">
         <v>7.12</v>
@@ -15683,7 +15683,7 @@
         <v>0</v>
       </c>
       <c r="BJ66" t="n">
-        <v>25.31</v>
+        <v>25.99</v>
       </c>
       <c r="BK66" t="n">
         <v>1.58</v>
@@ -15692,7 +15692,7 @@
         <v>1.57</v>
       </c>
       <c r="BM66" t="n">
-        <v>28.51</v>
+        <v>27.2</v>
       </c>
       <c r="BN66" t="n">
         <v>28.51</v>
@@ -15701,19 +15701,19 @@
         <v>9.48</v>
       </c>
       <c r="BP66" t="n">
-        <v>21.13</v>
+        <v>25.34</v>
       </c>
       <c r="BQ66" t="n">
-        <v>16.12</v>
+        <v>16.55</v>
       </c>
       <c r="BR66" t="n">
-        <v>21.13</v>
+        <v>25.52</v>
       </c>
       <c r="BS66" t="n">
         <v>3.46</v>
       </c>
       <c r="BT66" t="n">
-        <v>3897</v>
+        <v>4520</v>
       </c>
     </row>
     <row r="67">
@@ -15973,13 +15973,13 @@
         </is>
       </c>
       <c r="F68" t="n">
-        <v>18.4</v>
+        <v>18.46</v>
       </c>
       <c r="G68" t="n">
-        <v>7959286288</v>
+        <v>7503797078</v>
       </c>
       <c r="H68" t="n">
-        <v>144900</v>
+        <v>74600</v>
       </c>
       <c r="I68" t="n">
         <v>137989898</v>
@@ -16072,7 +16072,7 @@
         <v>205604948.02</v>
       </c>
       <c r="AM68" t="n">
-        <v>551961601.10957</v>
+        <v>520374277.2538142</v>
       </c>
       <c r="AN68" t="n">
         <v>0.1911</v>
@@ -16113,7 +16113,7 @@
         <v>21.39</v>
       </c>
       <c r="AZ68" t="n">
-        <v>34.04</v>
+        <v>34.15</v>
       </c>
       <c r="BA68" t="n">
         <v>1.24</v>
@@ -16122,19 +16122,19 @@
         <v>63.25</v>
       </c>
       <c r="BC68" t="n">
-        <v>42.41</v>
+        <v>41.94</v>
       </c>
       <c r="BD68" t="n">
-        <v>16.27</v>
+        <v>15.9</v>
       </c>
       <c r="BE68" t="n">
         <v>85</v>
       </c>
       <c r="BF68" t="n">
-        <v>-93.26000000000001</v>
+        <v>-93.29000000000001</v>
       </c>
       <c r="BG68" t="n">
-        <v>243.74</v>
+        <v>242.63</v>
       </c>
       <c r="BH68" t="n">
         <v>20.48</v>
@@ -16143,7 +16143,7 @@
         <v>0</v>
       </c>
       <c r="BJ68" t="n">
-        <v>18.4</v>
+        <v>18.46</v>
       </c>
       <c r="BK68" t="n">
         <v>1.49</v>
@@ -16152,7 +16152,7 @@
         <v>1.49</v>
       </c>
       <c r="BM68" t="n">
-        <v>18.95</v>
+        <v>18.8</v>
       </c>
       <c r="BN68" t="n">
         <v>22.11</v>
@@ -16161,19 +16161,19 @@
         <v>15.45</v>
       </c>
       <c r="BP68" t="n">
-        <v>18.16</v>
+        <v>18.2</v>
       </c>
       <c r="BQ68" t="n">
-        <v>12.38</v>
+        <v>12.42</v>
       </c>
       <c r="BR68" t="n">
-        <v>18.52</v>
+        <v>18.4</v>
       </c>
       <c r="BS68" t="n">
         <v>0</v>
       </c>
       <c r="BT68" t="n">
-        <v>47700</v>
+        <v>51903</v>
       </c>
     </row>
     <row r="69">
@@ -16203,13 +16203,13 @@
         </is>
       </c>
       <c r="F69" t="n">
-        <v>21.19</v>
+        <v>21.29</v>
       </c>
       <c r="G69" t="n">
-        <v>7959286288</v>
+        <v>7503797078</v>
       </c>
       <c r="H69" t="n">
-        <v>7534200</v>
+        <v>0</v>
       </c>
       <c r="I69" t="n">
         <v>255106712</v>
@@ -16302,7 +16302,7 @@
         <v>380109000.88</v>
       </c>
       <c r="AM69" t="n">
-        <v>473767040.952381</v>
+        <v>446654587.9761904</v>
       </c>
       <c r="AN69" t="n">
         <v>0.8856000000000001</v>
@@ -16343,7 +16343,7 @@
         <v>21.39</v>
       </c>
       <c r="AZ69" t="n">
-        <v>37.05</v>
+        <v>37.22</v>
       </c>
       <c r="BA69" t="n">
         <v>1.24</v>
@@ -16352,19 +16352,19 @@
         <v>69.59</v>
       </c>
       <c r="BC69" t="n">
-        <v>23.66</v>
+        <v>23.08</v>
       </c>
       <c r="BD69" t="n">
-        <v>0.97</v>
+        <v>0.49</v>
       </c>
       <c r="BE69" t="n">
         <v>74.83</v>
       </c>
       <c r="BF69" t="n">
-        <v>-94.15000000000001</v>
+        <v>-94.18000000000001</v>
       </c>
       <c r="BG69" t="n">
-        <v>228.4</v>
+        <v>226.85</v>
       </c>
       <c r="BH69" t="n">
         <v>20.48</v>
@@ -16373,7 +16373,7 @@
         <v>0</v>
       </c>
       <c r="BJ69" t="n">
-        <v>21.19</v>
+        <v>21.29</v>
       </c>
       <c r="BK69" t="n">
         <v>1.49</v>
@@ -16382,7 +16382,7 @@
         <v>1.49</v>
       </c>
       <c r="BM69" t="n">
-        <v>21.69</v>
+        <v>21.43</v>
       </c>
       <c r="BN69" t="n">
         <v>25.63</v>
@@ -16391,19 +16391,19 @@
         <v>16.99</v>
       </c>
       <c r="BP69" t="n">
-        <v>20.48</v>
+        <v>20.78</v>
       </c>
       <c r="BQ69" t="n">
-        <v>14.25</v>
+        <v>14.32</v>
       </c>
       <c r="BR69" t="n">
-        <v>21.39</v>
+        <v>21.42</v>
       </c>
       <c r="BS69" t="n">
         <v>0</v>
       </c>
       <c r="BT69" t="n">
-        <v>2291533</v>
+        <v>2495197</v>
       </c>
     </row>
     <row r="70">
@@ -16433,13 +16433,13 @@
         </is>
       </c>
       <c r="F70" t="n">
-        <v>19.1</v>
+        <v>19.25</v>
       </c>
       <c r="G70" t="n">
-        <v>8873044607</v>
+        <v>8475480475</v>
       </c>
       <c r="H70" t="n">
-        <v>5137500</v>
+        <v>0</v>
       </c>
       <c r="I70" t="n">
         <v>464557268</v>
@@ -16454,7 +16454,7 @@
         <v>0.68</v>
       </c>
       <c r="M70" t="n">
-        <v>0.7003333955445368</v>
+        <v>0.6689543761839642</v>
       </c>
       <c r="N70" t="n">
         <v>0.2</v>
@@ -16532,7 +16532,7 @@
         <v>55746872.16</v>
       </c>
       <c r="AM70" t="n">
-        <v>2928397560.066007</v>
+        <v>2797188275.577558</v>
       </c>
       <c r="AN70" t="n">
         <v>0.1236</v>
@@ -16573,7 +16573,7 @@
         <v>6.9</v>
       </c>
       <c r="AZ70" t="n">
-        <v>2.2</v>
+        <v>2.21</v>
       </c>
       <c r="BA70" t="n">
         <v>0.12</v>
@@ -16582,25 +16582,25 @@
         <v>1.07</v>
       </c>
       <c r="BC70" t="n">
-        <v>-55.76</v>
+        <v>-56.11</v>
       </c>
       <c r="BD70" t="n">
-        <v>-63.88</v>
+        <v>-64.16</v>
       </c>
       <c r="BE70" t="n">
         <v>-88.5</v>
       </c>
       <c r="BF70" t="n">
-        <v>-99.37</v>
+        <v>-99.38</v>
       </c>
       <c r="BG70" t="n">
-        <v>-94.40000000000001</v>
+        <v>-94.44</v>
       </c>
       <c r="BH70" t="n">
         <v>26.44</v>
       </c>
       <c r="BI70" t="n">
-        <v>0</v>
+        <v>0.79</v>
       </c>
       <c r="BJ70" t="n">
         <v>19.1</v>
@@ -16612,7 +16612,7 @@
         <v>0.1</v>
       </c>
       <c r="BM70" t="n">
-        <v>19.8</v>
+        <v>19.51</v>
       </c>
       <c r="BN70" t="n">
         <v>22.15</v>
@@ -16621,10 +16621,10 @@
         <v>13.21</v>
       </c>
       <c r="BP70" t="n">
-        <v>18.86</v>
+        <v>18.9</v>
       </c>
       <c r="BQ70" t="n">
-        <v>191.56</v>
+        <v>193.06</v>
       </c>
       <c r="BR70" t="n">
         <v>19</v>
@@ -16633,7 +16633,7 @@
         <v>0.67</v>
       </c>
       <c r="BT70" t="n">
-        <v>3682213</v>
+        <v>3709903</v>
       </c>
     </row>
     <row r="71">

</xml_diff>

<commit_message>
📊 Dados atualizados - 2026-10-08 06:53
</commit_message>
<xml_diff>
--- a/data/ativos.xlsx
+++ b/data/ativos.xlsx
@@ -1047,13 +1047,13 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>28.82</v>
+        <v>28.06</v>
       </c>
       <c r="G3" t="n">
-        <v>3419126949</v>
+        <v>3753496336</v>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>1032800</v>
       </c>
       <c r="I3" t="n">
         <v>129510368</v>
@@ -1068,7 +1068,7 @@
         <v>0.88</v>
       </c>
       <c r="M3" t="n">
-        <v>0.8507549337345721</v>
+        <v>0.9339534841023065</v>
       </c>
       <c r="N3" t="n">
         <v>0.09</v>
@@ -1146,7 +1146,7 @@
         <v>506385538.88</v>
       </c>
       <c r="AM3" t="n">
-        <v>667798232.2265625</v>
+        <v>733104753.125</v>
       </c>
       <c r="AN3" t="n">
         <v>2.7</v>
@@ -1187,7 +1187,7 @@
         <v>40.42</v>
       </c>
       <c r="AZ3" t="n">
-        <v>52.74</v>
+        <v>51.35</v>
       </c>
       <c r="BA3" t="n">
         <v>4.87</v>
@@ -1196,19 +1196,19 @@
         <v>21.14</v>
       </c>
       <c r="BC3" t="n">
-        <v>71.75</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="BD3" t="n">
-        <v>40.23</v>
+        <v>44.03</v>
       </c>
       <c r="BE3" t="n">
         <v>83</v>
       </c>
       <c r="BF3" t="n">
-        <v>-83.11</v>
+        <v>-82.65000000000001</v>
       </c>
       <c r="BG3" t="n">
-        <v>-26.66</v>
+        <v>-24.68</v>
       </c>
       <c r="BH3" t="n">
         <v>27.85</v>
@@ -1217,7 +1217,7 @@
         <v>0</v>
       </c>
       <c r="BJ3" t="n">
-        <v>28.82</v>
+        <v>28.06</v>
       </c>
       <c r="BK3" t="n">
         <v>3.91</v>
@@ -1226,7 +1226,7 @@
         <v>4.39</v>
       </c>
       <c r="BM3" t="n">
-        <v>29.2</v>
+        <v>28.82</v>
       </c>
       <c r="BN3" t="n">
         <v>29.2</v>
@@ -1235,19 +1235,19 @@
         <v>18.72</v>
       </c>
       <c r="BP3" t="n">
-        <v>28.12</v>
+        <v>28.06</v>
       </c>
       <c r="BQ3" t="n">
-        <v>6.56</v>
+        <v>6.39</v>
       </c>
       <c r="BR3" t="n">
-        <v>28.2</v>
+        <v>28.77</v>
       </c>
       <c r="BS3" t="n">
         <v>0.79</v>
       </c>
       <c r="BT3" t="n">
-        <v>634997</v>
+        <v>657713</v>
       </c>
     </row>
     <row r="4">
@@ -1277,13 +1277,13 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>16.25</v>
+        <v>15.97</v>
       </c>
       <c r="G4" t="n">
-        <v>231361975000</v>
+        <v>247290024334</v>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
+        <v>46954500</v>
       </c>
       <c r="I4" t="n">
         <v>15484664889</v>
@@ -1298,7 +1298,7 @@
         <v>2.76</v>
       </c>
       <c r="M4" t="n">
-        <v>2.61971870712877</v>
+        <v>2.80007249607075</v>
       </c>
       <c r="N4" t="n">
         <v>1.76</v>
@@ -1376,7 +1376,7 @@
         <v>16258898133.45</v>
       </c>
       <c r="AM4" t="n">
-        <v>22907126237.62376</v>
+        <v>24484160825.14852</v>
       </c>
       <c r="AN4" t="n">
         <v>0.269</v>
@@ -1417,7 +1417,7 @@
         <v>9.470000000000001</v>
       </c>
       <c r="AZ4" t="n">
-        <v>20.29</v>
+        <v>19.94</v>
       </c>
       <c r="BA4" t="n">
         <v>1.13</v>
@@ -1426,28 +1426,28 @@
         <v>11.39</v>
       </c>
       <c r="BC4" t="n">
-        <v>-28.59</v>
+        <v>-27.34</v>
       </c>
       <c r="BD4" t="n">
-        <v>-41.69</v>
+        <v>-40.67</v>
       </c>
       <c r="BE4" t="n">
         <v>24.83</v>
       </c>
       <c r="BF4" t="n">
-        <v>-93.06</v>
+        <v>-92.94</v>
       </c>
       <c r="BG4" t="n">
-        <v>-29.93</v>
+        <v>-28.7</v>
       </c>
       <c r="BH4" t="n">
         <v>5.7</v>
       </c>
       <c r="BI4" t="n">
-        <v>-1.52</v>
+        <v>0</v>
       </c>
       <c r="BJ4" t="n">
-        <v>16.5</v>
+        <v>15.97</v>
       </c>
       <c r="BK4" t="n">
         <v>1.05</v>
@@ -1456,7 +1456,7 @@
         <v>1.04</v>
       </c>
       <c r="BM4" t="n">
-        <v>16.7</v>
+        <v>16.18</v>
       </c>
       <c r="BN4" t="n">
         <v>16.94</v>
@@ -1465,19 +1465,19 @@
         <v>11.04</v>
       </c>
       <c r="BP4" t="n">
-        <v>16.17</v>
+        <v>15.71</v>
       </c>
       <c r="BQ4" t="n">
-        <v>15.67</v>
+        <v>15.4</v>
       </c>
       <c r="BR4" t="n">
-        <v>16.7</v>
+        <v>16.05</v>
       </c>
       <c r="BS4" t="n">
         <v>2.76</v>
       </c>
       <c r="BT4" t="n">
-        <v>27692800</v>
+        <v>27898513</v>
       </c>
     </row>
     <row r="5">
@@ -1737,13 +1737,13 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>7.49</v>
+        <v>7</v>
       </c>
       <c r="G6" t="n">
-        <v>450669691</v>
+        <v>441592830</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>3700</v>
       </c>
       <c r="I6" t="n">
         <v>63084700</v>
@@ -1758,7 +1758,7 @@
         <v>1.91</v>
       </c>
       <c r="M6" t="n">
-        <v>7.016044706194086</v>
+        <v>6.874735752342318</v>
       </c>
       <c r="N6" t="n">
         <v>1.26</v>
@@ -1836,7 +1836,7 @@
         <v>35958279</v>
       </c>
       <c r="AM6" t="n">
-        <v>43085056.50095602</v>
+        <v>42217287.76290631</v>
       </c>
       <c r="AN6" t="n">
         <v>0.5199</v>
@@ -1877,7 +1877,7 @@
         <v>5.74</v>
       </c>
       <c r="AZ6" t="n">
-        <v>8.789999999999999</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="BA6" t="n">
         <v>0.65</v>
@@ -1886,28 +1886,28 @@
         <v>7.95</v>
       </c>
       <c r="BC6" t="n">
-        <v>-6.06</v>
+        <v>0.51</v>
       </c>
       <c r="BD6" t="n">
-        <v>-23.3</v>
+        <v>-17.93</v>
       </c>
       <c r="BE6" t="n">
         <v>17.33</v>
       </c>
       <c r="BF6" t="n">
-        <v>-91.34</v>
+        <v>-90.73999999999999</v>
       </c>
       <c r="BG6" t="n">
-        <v>6.19</v>
+        <v>13.62</v>
       </c>
       <c r="BH6" t="n">
         <v>3.86</v>
       </c>
       <c r="BI6" t="n">
-        <v>4.17</v>
+        <v>0</v>
       </c>
       <c r="BJ6" t="n">
-        <v>7.19</v>
+        <v>7</v>
       </c>
       <c r="BK6" t="n">
         <v>0.57</v>
@@ -1916,7 +1916,7 @@
         <v>0.5600000000000001</v>
       </c>
       <c r="BM6" t="n">
-        <v>7.49</v>
+        <v>7.33</v>
       </c>
       <c r="BN6" t="n">
         <v>8.16</v>
@@ -1925,19 +1925,19 @@
         <v>6.22</v>
       </c>
       <c r="BP6" t="n">
-        <v>7.19</v>
+        <v>7</v>
       </c>
       <c r="BQ6" t="n">
-        <v>13.32</v>
+        <v>12.45</v>
       </c>
       <c r="BR6" t="n">
-        <v>7.19</v>
+        <v>7.22</v>
       </c>
       <c r="BS6" t="n">
         <v>7.32</v>
       </c>
       <c r="BT6" t="n">
-        <v>237</v>
+        <v>327</v>
       </c>
     </row>
     <row r="7">
@@ -3117,13 +3117,13 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>5.01</v>
+        <v>5.09</v>
       </c>
       <c r="G12" t="n">
-        <v>442855813</v>
+        <v>488444202</v>
       </c>
       <c r="H12" t="n">
-        <v>0</v>
+        <v>5760900</v>
       </c>
       <c r="I12" t="n">
         <v>95961536</v>
@@ -3138,7 +3138,7 @@
         <v>0.32</v>
       </c>
       <c r="M12" t="n">
-        <v>0.08008979801169788</v>
+        <v>0.0883343885974123</v>
       </c>
       <c r="N12" t="n">
         <v>0.14</v>
@@ -3216,7 +3216,7 @@
         <v>362734606.08</v>
       </c>
       <c r="AM12" t="n">
-        <v>476189046.2365591</v>
+        <v>525208819.3548387</v>
       </c>
       <c r="AN12" t="n">
         <v>0.4208</v>
@@ -3257,7 +3257,7 @@
         <v>30.49</v>
       </c>
       <c r="AZ12" t="n">
-        <v>6.77</v>
+        <v>6.88</v>
       </c>
       <c r="BA12" t="n">
         <v>4.41</v>
@@ -3266,28 +3266,28 @@
         <v>18.12</v>
       </c>
       <c r="BC12" t="n">
-        <v>645.45</v>
+        <v>633.74</v>
       </c>
       <c r="BD12" t="n">
-        <v>508.66</v>
+        <v>499.09</v>
       </c>
       <c r="BE12" t="n">
         <v>35.17</v>
       </c>
       <c r="BF12" t="n">
-        <v>-11.94</v>
+        <v>-13.33</v>
       </c>
       <c r="BG12" t="n">
-        <v>261.65</v>
+        <v>255.97</v>
       </c>
       <c r="BH12" t="n">
         <v>16.4</v>
       </c>
       <c r="BI12" t="n">
-        <v>0.72</v>
+        <v>0</v>
       </c>
       <c r="BJ12" t="n">
-        <v>4.97</v>
+        <v>5.09</v>
       </c>
       <c r="BK12" t="n">
         <v>3.78</v>
@@ -3296,28 +3296,28 @@
         <v>3.63</v>
       </c>
       <c r="BM12" t="n">
-        <v>5.09</v>
+        <v>5.2</v>
       </c>
       <c r="BN12" t="n">
-        <v>7.43</v>
+        <v>7.46</v>
       </c>
       <c r="BO12" t="n">
-        <v>3.99</v>
+        <v>4</v>
       </c>
       <c r="BP12" t="n">
-        <v>4.84</v>
+        <v>4.95</v>
       </c>
       <c r="BQ12" t="n">
-        <v>1.38</v>
+        <v>1.4</v>
       </c>
       <c r="BR12" t="n">
-        <v>5</v>
+        <v>5.04</v>
       </c>
       <c r="BS12" t="n">
         <v>0.09</v>
       </c>
       <c r="BT12" t="n">
-        <v>751297</v>
+        <v>827680</v>
       </c>
     </row>
     <row r="13">
@@ -3347,13 +3347,13 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>34.29</v>
+        <v>34.46</v>
       </c>
       <c r="G13" t="n">
-        <v>15281565222</v>
+        <v>17374421398</v>
       </c>
       <c r="H13" t="n">
-        <v>0</v>
+        <v>10041700</v>
       </c>
       <c r="I13" t="n">
         <v>504190947</v>
@@ -3368,7 +3368,7 @@
         <v>1.13</v>
       </c>
       <c r="M13" t="n">
-        <v>5.285248730369972</v>
+        <v>6.009079390800402</v>
       </c>
       <c r="N13" t="n">
         <v>0.57</v>
@@ -3446,7 +3446,7 @@
         <v>932753251.95</v>
       </c>
       <c r="AM13" t="n">
-        <v>1590173280.12487</v>
+        <v>1807952278.668054</v>
       </c>
       <c r="AN13" t="n">
         <v>2.6301</v>
@@ -3487,7 +3487,7 @@
         <v>26.6</v>
       </c>
       <c r="AZ13" t="n">
-        <v>62.06</v>
+        <v>62.37</v>
       </c>
       <c r="BA13" t="n">
         <v>2.6</v>
@@ -3496,19 +3496,19 @@
         <v>8.69</v>
       </c>
       <c r="BC13" t="n">
-        <v>-5.01</v>
+        <v>-5.47</v>
       </c>
       <c r="BD13" t="n">
-        <v>-22.44</v>
+        <v>-22.82</v>
       </c>
       <c r="BE13" t="n">
         <v>81</v>
       </c>
       <c r="BF13" t="n">
-        <v>-92.41</v>
+        <v>-92.44</v>
       </c>
       <c r="BG13" t="n">
-        <v>-74.65000000000001</v>
+        <v>-74.77</v>
       </c>
       <c r="BH13" t="n">
         <v>25.49</v>
@@ -3517,7 +3517,7 @@
         <v>0</v>
       </c>
       <c r="BJ13" t="n">
-        <v>34.29</v>
+        <v>34.46</v>
       </c>
       <c r="BK13" t="n">
         <v>1.85</v>
@@ -3526,28 +3526,28 @@
         <v>1.96</v>
       </c>
       <c r="BM13" t="n">
-        <v>34.5</v>
+        <v>34.63</v>
       </c>
       <c r="BN13" t="n">
-        <v>34.5</v>
+        <v>34.63</v>
       </c>
       <c r="BO13" t="n">
         <v>20.85</v>
       </c>
       <c r="BP13" t="n">
-        <v>33.16</v>
+        <v>33.91</v>
       </c>
       <c r="BQ13" t="n">
-        <v>17.52</v>
+        <v>17.61</v>
       </c>
       <c r="BR13" t="n">
-        <v>33.32</v>
+        <v>34.3</v>
       </c>
       <c r="BS13" t="n">
         <v>5.01</v>
       </c>
       <c r="BT13" t="n">
-        <v>5913507</v>
+        <v>6161573</v>
       </c>
     </row>
     <row r="14">
@@ -3577,13 +3577,13 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>11.8</v>
+        <v>11.16</v>
       </c>
       <c r="G14" t="n">
-        <v>8768925468</v>
+        <v>9065923407</v>
       </c>
       <c r="H14" t="n">
-        <v>0</v>
+        <v>15200</v>
       </c>
       <c r="I14" t="n">
         <v>339510689</v>
@@ -3598,7 +3598,7 @@
         <v>1.92</v>
       </c>
       <c r="M14" t="n">
-        <v>3.64101374549608</v>
+        <v>3.764332569704269</v>
       </c>
       <c r="N14" t="n">
         <v>1.11</v>
@@ -3676,7 +3676,7 @@
         <v>349696009.67</v>
       </c>
       <c r="AM14" t="n">
-        <v>973243670.1442841</v>
+        <v>1006206815.427303</v>
       </c>
       <c r="AN14" t="n">
         <v>0.1489</v>
@@ -3717,7 +3717,7 @@
         <v>9.050000000000001</v>
       </c>
       <c r="AZ14" t="n">
-        <v>9.48</v>
+        <v>8.970000000000001</v>
       </c>
       <c r="BA14" t="n">
         <v>1.42</v>
@@ -3726,19 +3726,19 @@
         <v>5.94</v>
       </c>
       <c r="BC14" t="n">
-        <v>-6.08</v>
+        <v>-0.6899999999999999</v>
       </c>
       <c r="BD14" t="n">
-        <v>-23.31</v>
+        <v>-18.92</v>
       </c>
       <c r="BE14" t="n">
         <v>-19.67</v>
       </c>
       <c r="BF14" t="n">
-        <v>-87.95999999999999</v>
+        <v>-87.27</v>
       </c>
       <c r="BG14" t="n">
-        <v>-49.64</v>
+        <v>-46.75</v>
       </c>
       <c r="BH14" t="n">
         <v>5.3</v>
@@ -3747,7 +3747,7 @@
         <v>0</v>
       </c>
       <c r="BJ14" t="n">
-        <v>11.8</v>
+        <v>11.16</v>
       </c>
       <c r="BK14" t="n">
         <v>1.03</v>
@@ -3756,7 +3756,7 @@
         <v>1.01</v>
       </c>
       <c r="BM14" t="n">
-        <v>11.95</v>
+        <v>11.62</v>
       </c>
       <c r="BN14" t="n">
         <v>13.49</v>
@@ -3765,19 +3765,19 @@
         <v>7.81</v>
       </c>
       <c r="BP14" t="n">
-        <v>11.45</v>
+        <v>11.16</v>
       </c>
       <c r="BQ14" t="n">
-        <v>11.65</v>
+        <v>11.02</v>
       </c>
       <c r="BR14" t="n">
-        <v>11.8</v>
+        <v>11.57</v>
       </c>
       <c r="BS14" t="n">
         <v>1.44</v>
       </c>
       <c r="BT14" t="n">
-        <v>12680</v>
+        <v>12770</v>
       </c>
     </row>
     <row r="15">
@@ -3807,13 +3807,13 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>15.99</v>
+        <v>15.26</v>
       </c>
       <c r="G15" t="n">
-        <v>8768925468</v>
+        <v>9065923407</v>
       </c>
       <c r="H15" t="n">
-        <v>0</v>
+        <v>2290000</v>
       </c>
       <c r="I15" t="n">
         <v>343551533</v>
@@ -3828,7 +3828,7 @@
         <v>2.56</v>
       </c>
       <c r="M15" t="n">
-        <v>3.598188238594891</v>
+        <v>3.720056590070395</v>
       </c>
       <c r="N15" t="n">
         <v>1.47</v>
@@ -3906,7 +3906,7 @@
         <v>353858078.99</v>
       </c>
       <c r="AM15" t="n">
-        <v>731353250.0417014</v>
+        <v>756123720.3502918</v>
       </c>
       <c r="AN15" t="n">
         <v>0.1638</v>
@@ -3947,7 +3947,7 @@
         <v>9.050000000000001</v>
       </c>
       <c r="AZ15" t="n">
-        <v>10.63</v>
+        <v>10.15</v>
       </c>
       <c r="BA15" t="n">
         <v>1.42</v>
@@ -3956,28 +3956,28 @@
         <v>6.19</v>
       </c>
       <c r="BC15" t="n">
-        <v>-30.69</v>
+        <v>-27.37</v>
       </c>
       <c r="BD15" t="n">
-        <v>-43.41</v>
+        <v>-40.7</v>
       </c>
       <c r="BE15" t="n">
         <v>-33.5</v>
       </c>
       <c r="BF15" t="n">
-        <v>-91.11</v>
+        <v>-90.69</v>
       </c>
       <c r="BG15" t="n">
-        <v>-61.3</v>
+        <v>-59.45</v>
       </c>
       <c r="BH15" t="n">
         <v>5.3</v>
       </c>
       <c r="BI15" t="n">
-        <v>0.88</v>
+        <v>0</v>
       </c>
       <c r="BJ15" t="n">
-        <v>15.85</v>
+        <v>15.26</v>
       </c>
       <c r="BK15" t="n">
         <v>1.03</v>
@@ -3986,28 +3986,28 @@
         <v>1.01</v>
       </c>
       <c r="BM15" t="n">
-        <v>16.25</v>
+        <v>16.09</v>
       </c>
       <c r="BN15" t="n">
         <v>16.75</v>
       </c>
       <c r="BO15" t="n">
-        <v>7.84</v>
+        <v>7.96</v>
       </c>
       <c r="BP15" t="n">
-        <v>15.63</v>
+        <v>15.26</v>
       </c>
       <c r="BQ15" t="n">
-        <v>15.79</v>
+        <v>15.07</v>
       </c>
       <c r="BR15" t="n">
-        <v>15.84</v>
+        <v>15.98</v>
       </c>
       <c r="BS15" t="n">
         <v>1.92</v>
       </c>
       <c r="BT15" t="n">
-        <v>2514247</v>
+        <v>2578723</v>
       </c>
     </row>
     <row r="16">
@@ -4037,13 +4037,13 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>5.07</v>
+        <v>5.61</v>
       </c>
       <c r="G16" t="n">
-        <v>1001780826</v>
+        <v>1230305006</v>
       </c>
       <c r="H16" t="n">
-        <v>0</v>
+        <v>671300</v>
       </c>
       <c r="I16" t="n">
         <v>219305733</v>
@@ -4058,7 +4058,7 @@
         <v>2.69</v>
       </c>
       <c r="M16" t="n">
-        <v>0.4739263277604329</v>
+        <v>0.5820374261374188</v>
       </c>
       <c r="N16" t="n">
         <v>0.39</v>
@@ -4136,7 +4136,7 @@
         <v>17544458.64</v>
       </c>
       <c r="AM16" t="n">
-        <v>281399108.4269663</v>
+        <v>345591293.8202247</v>
       </c>
       <c r="AN16" t="n">
         <v>0.0077</v>
@@ -4177,7 +4177,7 @@
         <v>1.42</v>
       </c>
       <c r="AZ16" t="n">
-        <v>0.14</v>
+        <v>0.16</v>
       </c>
       <c r="BA16" t="n">
         <v>0.08</v>
@@ -4186,16 +4186,16 @@
         <v>0</v>
       </c>
       <c r="BC16" t="n">
-        <v>-65.7</v>
+        <v>-69</v>
       </c>
       <c r="BD16" t="n">
-        <v>-71.98999999999999</v>
+        <v>-74.69</v>
       </c>
       <c r="BE16" t="n">
         <v>-97.17</v>
       </c>
       <c r="BF16" t="n">
-        <v>-98.42</v>
+        <v>-98.56999999999999</v>
       </c>
       <c r="BG16" t="n">
         <v>-100</v>
@@ -4207,7 +4207,7 @@
         <v>0</v>
       </c>
       <c r="BJ16" t="n">
-        <v>5.07</v>
+        <v>5.61</v>
       </c>
       <c r="BK16" t="n">
         <v>0.08</v>
@@ -4216,28 +4216,28 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="BM16" t="n">
-        <v>5.09</v>
+        <v>5.61</v>
       </c>
       <c r="BN16" t="n">
-        <v>5.54</v>
+        <v>5.61</v>
       </c>
       <c r="BO16" t="n">
-        <v>3.22</v>
+        <v>3.31</v>
       </c>
       <c r="BP16" t="n">
-        <v>4.91</v>
+        <v>4.97</v>
       </c>
       <c r="BQ16" t="n">
-        <v>69.19</v>
+        <v>76.56</v>
       </c>
       <c r="BR16" t="n">
-        <v>4.91</v>
+        <v>4.97</v>
       </c>
       <c r="BS16" t="n">
         <v>0.49</v>
       </c>
       <c r="BT16" t="n">
-        <v>124047</v>
+        <v>124510</v>
       </c>
     </row>
     <row r="17">
@@ -4267,13 +4267,13 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>37.44</v>
+        <v>38.18</v>
       </c>
       <c r="G17" t="n">
-        <v>10944861006</v>
+        <v>12585151324</v>
       </c>
       <c r="H17" t="n">
-        <v>0</v>
+        <v>1457900</v>
       </c>
       <c r="I17" t="n">
         <v>0</v>
@@ -4360,13 +4360,13 @@
         <v>8.039999999999999</v>
       </c>
       <c r="AK17" t="n">
-        <v>4942585353.143064</v>
+        <v>5683323394.147399</v>
       </c>
       <c r="AL17" t="n">
-        <v>1368107625.75</v>
+        <v>1573143915.5</v>
       </c>
       <c r="AM17" t="n">
-        <v>3388501859.442725</v>
+        <v>3896331679.256966</v>
       </c>
       <c r="AN17" t="n">
         <v>1.08</v>
@@ -4407,7 +4407,7 @@
         <v>42.98</v>
       </c>
       <c r="AZ17" t="n">
-        <v>20.03</v>
+        <v>20.43</v>
       </c>
       <c r="BA17" t="n">
         <v>4.55</v>
@@ -4416,28 +4416,28 @@
         <v>16.33</v>
       </c>
       <c r="BC17" t="n">
-        <v>40.59</v>
+        <v>37.87</v>
       </c>
       <c r="BD17" t="n">
-        <v>14.79</v>
+        <v>12.57</v>
       </c>
       <c r="BE17" t="n">
         <v>-46.5</v>
       </c>
       <c r="BF17" t="n">
-        <v>-87.84999999999999</v>
+        <v>-88.09</v>
       </c>
       <c r="BG17" t="n">
-        <v>-56.37</v>
+        <v>-57.22</v>
       </c>
       <c r="BH17" t="n">
         <v>29.25</v>
       </c>
       <c r="BI17" t="n">
-        <v>3.45</v>
+        <v>0</v>
       </c>
       <c r="BJ17" t="n">
-        <v>36.19</v>
+        <v>38.18</v>
       </c>
       <c r="BK17" t="n">
         <v>4.21</v>
@@ -4446,28 +4446,28 @@
         <v>12.62</v>
       </c>
       <c r="BM17" t="n">
-        <v>38</v>
+        <v>38.69</v>
       </c>
       <c r="BN17" t="n">
-        <v>38</v>
+        <v>38.69</v>
       </c>
       <c r="BO17" t="n">
         <v>29.53</v>
       </c>
       <c r="BP17" t="n">
-        <v>35.96</v>
+        <v>37.2</v>
       </c>
       <c r="BQ17" t="n">
-        <v>2.97</v>
+        <v>3.03</v>
       </c>
       <c r="BR17" t="n">
-        <v>36.1</v>
+        <v>37.36</v>
       </c>
       <c r="BS17" t="n">
         <v>2.21</v>
       </c>
       <c r="BT17" t="n">
-        <v>1131930</v>
+        <v>1183480</v>
       </c>
     </row>
     <row r="18">
@@ -4497,13 +4497,13 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>13.27</v>
+        <v>14.03</v>
       </c>
       <c r="G18" t="n">
-        <v>10944861006</v>
+        <v>12585151324</v>
       </c>
       <c r="H18" t="n">
-        <v>0</v>
+        <v>21300</v>
       </c>
       <c r="I18" t="n">
         <v>671494278</v>
@@ -4518,7 +4518,7 @@
         <v>1.2</v>
       </c>
       <c r="M18" t="n">
-        <v>3.222596896117451</v>
+        <v>3.70556278162486</v>
       </c>
       <c r="N18" t="n">
         <v>0.33</v>
@@ -4596,7 +4596,7 @@
         <v>940091989.1999999</v>
       </c>
       <c r="AM18" t="n">
-        <v>3257399108.928572</v>
+        <v>3745580751.190476</v>
       </c>
       <c r="AN18" t="n">
         <v>0.36</v>
@@ -4637,7 +4637,7 @@
         <v>14.31</v>
       </c>
       <c r="AZ18" t="n">
-        <v>6.83</v>
+        <v>7.23</v>
       </c>
       <c r="BA18" t="n">
         <v>1.51</v>
@@ -4646,19 +4646,19 @@
         <v>5.44</v>
       </c>
       <c r="BC18" t="n">
-        <v>32.06</v>
+        <v>24.91</v>
       </c>
       <c r="BD18" t="n">
-        <v>7.83</v>
+        <v>1.99</v>
       </c>
       <c r="BE18" t="n">
         <v>-48.5</v>
       </c>
       <c r="BF18" t="n">
-        <v>-88.59999999999999</v>
+        <v>-89.22</v>
       </c>
       <c r="BG18" t="n">
-        <v>-58.97</v>
+        <v>-61.19</v>
       </c>
       <c r="BH18" t="n">
         <v>9.75</v>
@@ -4667,7 +4667,7 @@
         <v>0</v>
       </c>
       <c r="BJ18" t="n">
-        <v>13.27</v>
+        <v>14.03</v>
       </c>
       <c r="BK18" t="n">
         <v>1.4</v>
@@ -4676,28 +4676,28 @@
         <v>12.62</v>
       </c>
       <c r="BM18" t="n">
-        <v>13.56</v>
+        <v>14.07</v>
       </c>
       <c r="BN18" t="n">
-        <v>13.86</v>
+        <v>14.07</v>
       </c>
       <c r="BO18" t="n">
         <v>10.19</v>
       </c>
       <c r="BP18" t="n">
-        <v>12.5</v>
+        <v>13.27</v>
       </c>
       <c r="BQ18" t="n">
-        <v>1.05</v>
+        <v>1.11</v>
       </c>
       <c r="BR18" t="n">
-        <v>12.5</v>
+        <v>13.27</v>
       </c>
       <c r="BS18" t="n">
         <v>2.3</v>
       </c>
       <c r="BT18" t="n">
-        <v>9280</v>
+        <v>9507</v>
       </c>
     </row>
     <row r="19">
@@ -4727,13 +4727,13 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>11.4</v>
+        <v>12.3</v>
       </c>
       <c r="G19" t="n">
-        <v>10944861006</v>
+        <v>12585151324</v>
       </c>
       <c r="H19" t="n">
-        <v>0</v>
+        <v>40100</v>
       </c>
       <c r="I19" t="n">
         <v>317386323</v>
@@ -4748,7 +4748,7 @@
         <v>1.12</v>
       </c>
       <c r="M19" t="n">
-        <v>6.81804860269114</v>
+        <v>7.839859579049527</v>
       </c>
       <c r="N19" t="n">
         <v>0.3</v>
@@ -4826,7 +4826,7 @@
         <v>444340852.2</v>
       </c>
       <c r="AM19" t="n">
-        <v>3474559049.523809</v>
+        <v>3995286134.603175</v>
       </c>
       <c r="AN19" t="n">
         <v>0.36</v>
@@ -4867,7 +4867,7 @@
         <v>14.31</v>
       </c>
       <c r="AZ19" t="n">
-        <v>6.27</v>
+        <v>6.76</v>
       </c>
       <c r="BA19" t="n">
         <v>1.51</v>
@@ -4876,28 +4876,28 @@
         <v>5.25</v>
       </c>
       <c r="BC19" t="n">
-        <v>53.73</v>
+        <v>42.48</v>
       </c>
       <c r="BD19" t="n">
-        <v>25.52</v>
+        <v>16.33</v>
       </c>
       <c r="BE19" t="n">
         <v>-45</v>
       </c>
       <c r="BF19" t="n">
-        <v>-86.73</v>
+        <v>-87.7</v>
       </c>
       <c r="BG19" t="n">
-        <v>-53.95</v>
+        <v>-57.32</v>
       </c>
       <c r="BH19" t="n">
         <v>9.75</v>
       </c>
       <c r="BI19" t="n">
-        <v>-1.64</v>
+        <v>0</v>
       </c>
       <c r="BJ19" t="n">
-        <v>11.59</v>
+        <v>12.3</v>
       </c>
       <c r="BK19" t="n">
         <v>1.4</v>
@@ -4906,28 +4906,28 @@
         <v>12.62</v>
       </c>
       <c r="BM19" t="n">
-        <v>12.3</v>
+        <v>12.33</v>
       </c>
       <c r="BN19" t="n">
-        <v>12.3</v>
+        <v>12.33</v>
       </c>
       <c r="BO19" t="n">
         <v>9.19</v>
       </c>
       <c r="BP19" t="n">
-        <v>11.36</v>
+        <v>11.48</v>
       </c>
       <c r="BQ19" t="n">
-        <v>0.9</v>
+        <v>0.97</v>
       </c>
       <c r="BR19" t="n">
-        <v>11.56</v>
+        <v>11.5</v>
       </c>
       <c r="BS19" t="n">
         <v>2.16</v>
       </c>
       <c r="BT19" t="n">
-        <v>12903</v>
+        <v>13970</v>
       </c>
     </row>
     <row r="20">
@@ -5417,13 +5417,13 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>6.08</v>
+        <v>5.94</v>
       </c>
       <c r="G22" t="n">
-        <v>1111334002</v>
+        <v>1189456499</v>
       </c>
       <c r="H22" t="n">
-        <v>0</v>
+        <v>2520600</v>
       </c>
       <c r="I22" t="n">
         <v>200245299</v>
@@ -5438,7 +5438,7 @@
         <v>0.27</v>
       </c>
       <c r="M22" t="n">
-        <v>0.09425958015496799</v>
+        <v>0.1008856653414426</v>
       </c>
       <c r="N22" t="n">
         <v>0.08</v>
@@ -5516,7 +5516,7 @@
         <v>378463615.11</v>
       </c>
       <c r="AM22" t="n">
-        <v>252003175.0566893</v>
+        <v>269718026.984127</v>
       </c>
       <c r="AN22" t="n">
         <v>0</v>
@@ -5566,28 +5566,28 @@
         <v>172.49</v>
       </c>
       <c r="BC22" t="n">
-        <v>388.57</v>
+        <v>400.09</v>
       </c>
       <c r="BD22" t="n">
-        <v>298.92</v>
+        <v>308.32</v>
       </c>
       <c r="BE22" t="n">
         <v>-100</v>
       </c>
       <c r="BF22" t="n">
-        <v>-68.91</v>
+        <v>-68.18000000000001</v>
       </c>
       <c r="BG22" t="n">
-        <v>2737</v>
+        <v>2803.87</v>
       </c>
       <c r="BH22" t="n">
         <v>20.75</v>
       </c>
       <c r="BI22" t="n">
-        <v>5.74</v>
+        <v>0</v>
       </c>
       <c r="BJ22" t="n">
-        <v>5.75</v>
+        <v>5.94</v>
       </c>
       <c r="BK22" t="n">
         <v>1.89</v>
@@ -5596,7 +5596,7 @@
         <v>0.67</v>
       </c>
       <c r="BM22" t="n">
-        <v>6.12</v>
+        <v>6.29</v>
       </c>
       <c r="BN22" t="n">
         <v>7.89</v>
@@ -5605,19 +5605,19 @@
         <v>3.37</v>
       </c>
       <c r="BP22" t="n">
-        <v>5.77</v>
+        <v>5.94</v>
       </c>
       <c r="BQ22" t="n">
-        <v>9.06</v>
+        <v>8.85</v>
       </c>
       <c r="BR22" t="n">
-        <v>5.89</v>
+        <v>6.02</v>
       </c>
       <c r="BS22" t="n">
         <v>0.09</v>
       </c>
       <c r="BT22" t="n">
-        <v>1726780</v>
+        <v>1764637</v>
       </c>
     </row>
     <row r="23">
@@ -5877,13 +5877,13 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>4.08</v>
+        <v>4.18</v>
       </c>
       <c r="G24" t="n">
-        <v>1355074870</v>
+        <v>1688171514</v>
       </c>
       <c r="H24" t="n">
-        <v>0</v>
+        <v>5866700</v>
       </c>
       <c r="I24" t="n">
         <v>403868805</v>
@@ -5898,7 +5898,7 @@
         <v>0.49</v>
       </c>
       <c r="M24" t="n">
-        <v>0.3275769198118682</v>
+        <v>0.4080999780257588</v>
       </c>
       <c r="N24" t="n">
         <v>0.11</v>
@@ -5976,7 +5976,7 @@
         <v>153470145.9</v>
       </c>
       <c r="AM24" t="n">
-        <v>1220788171.171171</v>
+        <v>1520875237.837838</v>
       </c>
       <c r="AN24" t="n">
         <v>0.0813</v>
@@ -6017,7 +6017,7 @@
         <v>5.84</v>
       </c>
       <c r="AZ24" t="n">
-        <v>1.88</v>
+        <v>1.93</v>
       </c>
       <c r="BA24" t="n">
         <v>0.38</v>
@@ -6026,28 +6026,28 @@
         <v>1.46</v>
       </c>
       <c r="BC24" t="n">
-        <v>75.40000000000001</v>
+        <v>71.20999999999999</v>
       </c>
       <c r="BD24" t="n">
-        <v>43.22</v>
+        <v>39.79</v>
       </c>
       <c r="BE24" t="n">
         <v>-53.83</v>
       </c>
       <c r="BF24" t="n">
-        <v>-90.69</v>
+        <v>-90.91</v>
       </c>
       <c r="BG24" t="n">
-        <v>-64.27</v>
+        <v>-65.12</v>
       </c>
       <c r="BH24" t="n">
         <v>5.99</v>
       </c>
       <c r="BI24" t="n">
-        <v>4.88</v>
+        <v>0</v>
       </c>
       <c r="BJ24" t="n">
-        <v>3.89</v>
+        <v>4.18</v>
       </c>
       <c r="BK24" t="n">
         <v>0.38</v>
@@ -6056,7 +6056,7 @@
         <v>0.41</v>
       </c>
       <c r="BM24" t="n">
-        <v>4.13</v>
+        <v>4.23</v>
       </c>
       <c r="BN24" t="n">
         <v>5.29</v>
@@ -6065,19 +6065,19 @@
         <v>1.92</v>
       </c>
       <c r="BP24" t="n">
-        <v>3.88</v>
+        <v>4.06</v>
       </c>
       <c r="BQ24" t="n">
-        <v>10.02</v>
+        <v>10.27</v>
       </c>
       <c r="BR24" t="n">
-        <v>4.02</v>
+        <v>4.08</v>
       </c>
       <c r="BS24" t="n">
         <v>0.29</v>
       </c>
       <c r="BT24" t="n">
-        <v>7390317</v>
+        <v>7367390</v>
       </c>
     </row>
     <row r="25">
@@ -6107,13 +6107,13 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>5.33</v>
+        <v>5.62</v>
       </c>
       <c r="G25" t="n">
-        <v>1540826758</v>
+        <v>1947296802</v>
       </c>
       <c r="H25" t="n">
-        <v>0</v>
+        <v>1996000</v>
       </c>
       <c r="I25" t="n">
         <v>346494097</v>
@@ -6128,7 +6128,7 @@
         <v>0.97</v>
       </c>
       <c r="M25" t="n">
-        <v>0.7683265761026161</v>
+        <v>0.9710110995724505</v>
       </c>
       <c r="N25" t="n">
         <v>0.22</v>
@@ -6206,7 +6206,7 @@
         <v>62368937.46</v>
       </c>
       <c r="AM25" t="n">
-        <v>566480425.7352941</v>
+        <v>715917941.9117646</v>
       </c>
       <c r="AN25" t="n">
         <v>0.4742</v>
@@ -6247,7 +6247,7 @@
         <v>3.27</v>
       </c>
       <c r="AZ25" t="n">
-        <v>12.42</v>
+        <v>13.09</v>
       </c>
       <c r="BA25" t="n">
         <v>0.23</v>
@@ -6256,28 +6256,28 @@
         <v>2.2</v>
       </c>
       <c r="BC25" t="n">
-        <v>-24.77</v>
+        <v>-28.65</v>
       </c>
       <c r="BD25" t="n">
-        <v>-38.57</v>
+        <v>-41.74</v>
       </c>
       <c r="BE25" t="n">
         <v>133</v>
       </c>
       <c r="BF25" t="n">
-        <v>-95.65000000000001</v>
+        <v>-95.88</v>
       </c>
       <c r="BG25" t="n">
-        <v>-58.73</v>
+        <v>-60.86</v>
       </c>
       <c r="BH25" t="n">
         <v>3.97</v>
       </c>
       <c r="BI25" t="n">
-        <v>4.1</v>
+        <v>0</v>
       </c>
       <c r="BJ25" t="n">
-        <v>5.12</v>
+        <v>5.62</v>
       </c>
       <c r="BK25" t="n">
         <v>0.18</v>
@@ -6286,7 +6286,7 @@
         <v>0.24</v>
       </c>
       <c r="BM25" t="n">
-        <v>5.48</v>
+        <v>5.79</v>
       </c>
       <c r="BN25" t="n">
         <v>6.3</v>
@@ -6295,19 +6295,19 @@
         <v>2.64</v>
       </c>
       <c r="BP25" t="n">
-        <v>5.12</v>
+        <v>5.35</v>
       </c>
       <c r="BQ25" t="n">
-        <v>22.52</v>
+        <v>23.75</v>
       </c>
       <c r="BR25" t="n">
-        <v>5.12</v>
+        <v>5.35</v>
       </c>
       <c r="BS25" t="n">
         <v>0.67</v>
       </c>
       <c r="BT25" t="n">
-        <v>1242380</v>
+        <v>1241470</v>
       </c>
     </row>
     <row r="26">
@@ -6337,13 +6337,13 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>12.63</v>
+        <v>12.07</v>
       </c>
       <c r="G26" t="n">
-        <v>14073886987</v>
+        <v>16347523096</v>
       </c>
       <c r="H26" t="n">
-        <v>0</v>
+        <v>35799200</v>
       </c>
       <c r="I26" t="n">
         <v>1354393401</v>
@@ -6358,7 +6358,7 @@
         <v>1.94</v>
       </c>
       <c r="M26" t="n">
-        <v>0.1814815862880517</v>
+        <v>0.2107999322492103</v>
       </c>
       <c r="N26" t="n">
         <v>0.26</v>
@@ -6436,7 +6436,7 @@
         <v>961619314.7099999</v>
       </c>
       <c r="AM26" t="n">
-        <v>5026388209.642858</v>
+        <v>5838401105.714286</v>
       </c>
       <c r="AN26" t="n">
         <v>0.1043</v>
@@ -6477,7 +6477,7 @@
         <v>7.07</v>
       </c>
       <c r="AZ26" t="n">
-        <v>2.42</v>
+        <v>2.31</v>
       </c>
       <c r="BA26" t="n">
         <v>0.66</v>
@@ -6486,19 +6486,19 @@
         <v>1.19</v>
       </c>
       <c r="BC26" t="n">
-        <v>-31.47</v>
+        <v>-28.29</v>
       </c>
       <c r="BD26" t="n">
-        <v>-44.04</v>
+        <v>-41.45</v>
       </c>
       <c r="BE26" t="n">
         <v>-80.83</v>
       </c>
       <c r="BF26" t="n">
-        <v>-94.78</v>
+        <v>-94.54000000000001</v>
       </c>
       <c r="BG26" t="n">
-        <v>-90.55</v>
+        <v>-90.11</v>
       </c>
       <c r="BH26" t="n">
         <v>4.69</v>
@@ -6507,7 +6507,7 @@
         <v>0</v>
       </c>
       <c r="BJ26" t="n">
-        <v>12.63</v>
+        <v>12.07</v>
       </c>
       <c r="BK26" t="n">
         <v>0.71</v>
@@ -6516,7 +6516,7 @@
         <v>0.72</v>
       </c>
       <c r="BM26" t="n">
-        <v>13.31</v>
+        <v>12.8</v>
       </c>
       <c r="BN26" t="n">
         <v>13.45</v>
@@ -6525,19 +6525,19 @@
         <v>6.91</v>
       </c>
       <c r="BP26" t="n">
-        <v>12.57</v>
+        <v>12</v>
       </c>
       <c r="BQ26" t="n">
-        <v>17.61</v>
+        <v>16.83</v>
       </c>
       <c r="BR26" t="n">
-        <v>13.03</v>
+        <v>12.77</v>
       </c>
       <c r="BS26" t="n">
         <v>0.16</v>
       </c>
       <c r="BT26" t="n">
-        <v>15567803</v>
+        <v>16362283</v>
       </c>
     </row>
     <row r="27">
@@ -8165,13 +8165,13 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>23.08</v>
+        <v>23.47</v>
       </c>
       <c r="G34" t="n">
-        <v>4023084018</v>
+        <v>4846315464</v>
       </c>
       <c r="H34" t="n">
-        <v>0</v>
+        <v>8378300</v>
       </c>
       <c r="I34" t="n">
         <v>206489813</v>
@@ -8186,7 +8186,7 @@
         <v>0.45</v>
       </c>
       <c r="M34" t="n">
-        <v>0.3536760724328598</v>
+        <v>0.426047731394446</v>
       </c>
       <c r="N34" t="n">
         <v>0.24</v>
@@ -8264,7 +8264,7 @@
         <v>324189006.41</v>
       </c>
       <c r="AM34" t="n">
-        <v>836400003.7422038</v>
+        <v>1007549992.515593</v>
       </c>
       <c r="AN34" t="n">
         <v>0</v>
@@ -8305,7 +8305,7 @@
         <v>30.28</v>
       </c>
       <c r="AZ34" t="n">
-        <v>53.85</v>
+        <v>54.76</v>
       </c>
       <c r="BA34" t="n">
         <v>2.29</v>
@@ -8314,19 +8314,19 @@
         <v>25.26</v>
       </c>
       <c r="BC34" t="n">
-        <v>60.7</v>
+        <v>58.03</v>
       </c>
       <c r="BD34" t="n">
-        <v>31.21</v>
+        <v>29.03</v>
       </c>
       <c r="BE34" t="n">
         <v>133.33</v>
       </c>
       <c r="BF34" t="n">
-        <v>-90.06</v>
+        <v>-90.22</v>
       </c>
       <c r="BG34" t="n">
-        <v>9.44</v>
+        <v>7.62</v>
       </c>
       <c r="BH34" t="n">
         <v>38.94</v>
@@ -8335,7 +8335,7 @@
         <v>0</v>
       </c>
       <c r="BJ34" t="n">
-        <v>23.08</v>
+        <v>23.47</v>
       </c>
       <c r="BK34" t="n">
         <v>1.57</v>
@@ -8344,7 +8344,7 @@
         <v>1.58</v>
       </c>
       <c r="BM34" t="n">
-        <v>23.68</v>
+        <v>24.6</v>
       </c>
       <c r="BN34" t="n">
         <v>28.86</v>
@@ -8353,19 +8353,19 @@
         <v>14.3</v>
       </c>
       <c r="BP34" t="n">
-        <v>22</v>
+        <v>22.99</v>
       </c>
       <c r="BQ34" t="n">
-        <v>14.63</v>
+        <v>14.88</v>
       </c>
       <c r="BR34" t="n">
-        <v>22.17</v>
+        <v>23</v>
       </c>
       <c r="BS34" t="n">
         <v>0.32</v>
       </c>
       <c r="BT34" t="n">
-        <v>4140347</v>
+        <v>4258470</v>
       </c>
     </row>
     <row r="35">
@@ -8395,13 +8395,13 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>22.68</v>
+        <v>22.33</v>
       </c>
       <c r="G35" t="n">
-        <v>89391633602</v>
+        <v>112688322284</v>
       </c>
       <c r="H35" t="n">
-        <v>0</v>
+        <v>70151300</v>
       </c>
       <c r="I35" t="n">
         <v>5046500000</v>
@@ -8416,7 +8416,7 @@
         <v>4.69</v>
       </c>
       <c r="M35" t="n">
-        <v>7.421325911036454</v>
+        <v>9.355425472599988</v>
       </c>
       <c r="N35" t="n">
         <v>1.79</v>
@@ -8494,7 +8494,7 @@
         <v>5349290000</v>
       </c>
       <c r="AM35" t="n">
-        <v>7387738314.214876</v>
+        <v>9313084486.280993</v>
       </c>
       <c r="AN35" t="n">
         <v>0.5305</v>
@@ -8535,7 +8535,7 @@
         <v>7.68</v>
       </c>
       <c r="AZ35" t="n">
-        <v>13.23</v>
+        <v>13.03</v>
       </c>
       <c r="BA35" t="n">
         <v>1.11</v>
@@ -8544,19 +8544,19 @@
         <v>9.119999999999999</v>
       </c>
       <c r="BC35" t="n">
-        <v>-58.52</v>
+        <v>-57.87</v>
       </c>
       <c r="BD35" t="n">
-        <v>-66.14</v>
+        <v>-65.59999999999999</v>
       </c>
       <c r="BE35" t="n">
         <v>-41.67</v>
       </c>
       <c r="BF35" t="n">
-        <v>-95.09</v>
+        <v>-95.01000000000001</v>
       </c>
       <c r="BG35" t="n">
-        <v>-59.8</v>
+        <v>-59.17</v>
       </c>
       <c r="BH35" t="n">
         <v>3.71</v>
@@ -8565,7 +8565,7 @@
         <v>0</v>
       </c>
       <c r="BJ35" t="n">
-        <v>22.68</v>
+        <v>22.33</v>
       </c>
       <c r="BK35" t="n">
         <v>1.06</v>
@@ -8574,28 +8574,28 @@
         <v>1.04</v>
       </c>
       <c r="BM35" t="n">
-        <v>23.93</v>
+        <v>23.05</v>
       </c>
       <c r="BN35" t="n">
         <v>24.28</v>
       </c>
       <c r="BO35" t="n">
-        <v>11.58</v>
+        <v>11.67</v>
       </c>
       <c r="BP35" t="n">
-        <v>22.44</v>
+        <v>22.2</v>
       </c>
       <c r="BQ35" t="n">
-        <v>21.7</v>
+        <v>21.37</v>
       </c>
       <c r="BR35" t="n">
-        <v>23.66</v>
+        <v>22.9</v>
       </c>
       <c r="BS35" t="n">
         <v>7.3</v>
       </c>
       <c r="BT35" t="n">
-        <v>46747913</v>
+        <v>48311877</v>
       </c>
     </row>
     <row r="36">
@@ -8628,10 +8628,10 @@
         <v>22</v>
       </c>
       <c r="G36" t="n">
-        <v>197807652</v>
+        <v>178849960</v>
       </c>
       <c r="H36" t="n">
-        <v>4600</v>
+        <v>100</v>
       </c>
       <c r="I36" t="n">
         <v>4900000</v>
@@ -8646,7 +8646,7 @@
         <v>1.52</v>
       </c>
       <c r="M36" t="n">
-        <v>1.925824123191094</v>
+        <v>1.741255021821716</v>
       </c>
       <c r="N36" t="n">
         <v>0.87</v>
@@ -8724,7 +8724,7 @@
         <v>11319000</v>
       </c>
       <c r="AM36" t="n">
-        <v>27246233.05785124</v>
+        <v>24634980.71625344</v>
       </c>
       <c r="AN36" t="n">
         <v>0</v>
@@ -8810,7 +8810,7 @@
         <v>29.05</v>
       </c>
       <c r="BO36" t="n">
-        <v>17.14</v>
+        <v>18.36</v>
       </c>
       <c r="BP36" t="n">
         <v>22</v>
@@ -8825,7 +8825,7 @@
         <v>1.24</v>
       </c>
       <c r="BT36" t="n">
-        <v>300</v>
+        <v>297</v>
       </c>
     </row>
     <row r="37">
@@ -8858,10 +8858,10 @@
         <v>14.5</v>
       </c>
       <c r="G37" t="n">
-        <v>171417115</v>
+        <v>178849960</v>
       </c>
       <c r="H37" t="n">
-        <v>900</v>
+        <v>400</v>
       </c>
       <c r="I37" t="n">
         <v>4900000</v>
@@ -8876,7 +8876,7 @@
         <v>0.88</v>
       </c>
       <c r="M37" t="n">
-        <v>1.668890014400565</v>
+        <v>1.741255021821716</v>
       </c>
       <c r="N37" t="n">
         <v>0.5</v>
@@ -8954,7 +8954,7 @@
         <v>11319000</v>
       </c>
       <c r="AM37" t="n">
-        <v>41008879.18660288</v>
+        <v>42787071.77033493</v>
       </c>
       <c r="AN37" t="n">
         <v>0</v>
@@ -9043,7 +9043,7 @@
         <v>13.42</v>
       </c>
       <c r="BP37" t="n">
-        <v>14.33</v>
+        <v>14.39</v>
       </c>
       <c r="BQ37" t="n">
         <v>6.27</v>
@@ -9055,7 +9055,7 @@
         <v>0.72</v>
       </c>
       <c r="BT37" t="n">
-        <v>1443</v>
+        <v>1460</v>
       </c>
     </row>
     <row r="38">
@@ -9315,13 +9315,13 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>74.91</v>
+        <v>76</v>
       </c>
       <c r="G39" t="n">
-        <v>3951789598</v>
+        <v>4260432320</v>
       </c>
       <c r="H39" t="n">
-        <v>9000</v>
+        <v>10800</v>
       </c>
       <c r="I39" t="n">
         <v>168174945</v>
@@ -9336,7 +9336,7 @@
         <v>0.53</v>
       </c>
       <c r="M39" t="n">
-        <v>0.1983625038286507</v>
+        <v>0.2138550146534667</v>
       </c>
       <c r="N39" t="n">
         <v>0.06</v>
@@ -9414,7 +9414,7 @@
         <v>2536078170.6</v>
       </c>
       <c r="AM39" t="n">
-        <v>415103949.3697479</v>
+        <v>447524403.3613446</v>
       </c>
       <c r="AN39" t="n">
         <v>11.9435</v>
@@ -9455,7 +9455,7 @@
         <v>170.24</v>
       </c>
       <c r="AZ39" t="n">
-        <v>218.86</v>
+        <v>222.05</v>
       </c>
       <c r="BA39" t="n">
         <v>19.01</v>
@@ -9464,19 +9464,19 @@
         <v>91.72</v>
       </c>
       <c r="BC39" t="n">
-        <v>178.34</v>
+        <v>174.35</v>
       </c>
       <c r="BD39" t="n">
-        <v>127.26</v>
+        <v>124.01</v>
       </c>
       <c r="BE39" t="n">
         <v>192.17</v>
       </c>
       <c r="BF39" t="n">
-        <v>-74.62</v>
+        <v>-74.98999999999999</v>
       </c>
       <c r="BG39" t="n">
-        <v>22.44</v>
+        <v>20.69</v>
       </c>
       <c r="BH39" t="n">
         <v>128.13</v>
@@ -9485,7 +9485,7 @@
         <v>0</v>
       </c>
       <c r="BJ39" t="n">
-        <v>74.91</v>
+        <v>76</v>
       </c>
       <c r="BK39" t="n">
         <v>15.08</v>
@@ -9494,7 +9494,7 @@
         <v>15.08</v>
       </c>
       <c r="BM39" t="n">
-        <v>77.98</v>
+        <v>77</v>
       </c>
       <c r="BN39" t="n">
         <v>77.98</v>
@@ -9503,19 +9503,19 @@
         <v>54.98</v>
       </c>
       <c r="BP39" t="n">
-        <v>71.76000000000001</v>
+        <v>74.5</v>
       </c>
       <c r="BQ39" t="n">
-        <v>4.97</v>
+        <v>5.04</v>
       </c>
       <c r="BR39" t="n">
-        <v>71.76000000000001</v>
+        <v>74.84999999999999</v>
       </c>
       <c r="BS39" t="n">
         <v>0.58</v>
       </c>
       <c r="BT39" t="n">
-        <v>2993</v>
+        <v>3140</v>
       </c>
     </row>
     <row r="40">
@@ -9545,13 +9545,13 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>24.64</v>
+        <v>24.18</v>
       </c>
       <c r="G40" t="n">
-        <v>121839499381</v>
+        <v>138571616228</v>
       </c>
       <c r="H40" t="n">
-        <v>0</v>
+        <v>57292200</v>
       </c>
       <c r="I40" t="n">
         <v>5730834040</v>
@@ -9566,7 +9566,7 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="M40" t="n">
-        <v>0.3696761194705249</v>
+        <v>0.4204434326813582</v>
       </c>
       <c r="N40" t="n">
         <v>0.05</v>
@@ -9644,7 +9644,7 @@
         <v>15358635227.2</v>
       </c>
       <c r="AM40" t="n">
-        <v>6319476108.973029</v>
+        <v>7187324493.153526</v>
       </c>
       <c r="AN40" t="n">
         <v>0.5641</v>
@@ -9685,7 +9685,7 @@
         <v>36.13</v>
       </c>
       <c r="AZ40" t="n">
-        <v>12.44</v>
+        <v>12.21</v>
       </c>
       <c r="BA40" t="n">
         <v>2.76</v>
@@ -9694,28 +9694,28 @@
         <v>27.89</v>
       </c>
       <c r="BC40" t="n">
-        <v>79.58</v>
+        <v>83</v>
       </c>
       <c r="BD40" t="n">
-        <v>46.63</v>
+        <v>49.42</v>
       </c>
       <c r="BE40" t="n">
         <v>-49.5</v>
       </c>
       <c r="BF40" t="n">
-        <v>-88.8</v>
+        <v>-88.59</v>
       </c>
       <c r="BG40" t="n">
-        <v>13.19</v>
+        <v>15.34</v>
       </c>
       <c r="BH40" t="n">
         <v>32.47</v>
       </c>
       <c r="BI40" t="n">
-        <v>-6.42</v>
+        <v>0</v>
       </c>
       <c r="BJ40" t="n">
-        <v>26.33</v>
+        <v>24.18</v>
       </c>
       <c r="BK40" t="n">
         <v>2.68</v>
@@ -9724,7 +9724,7 @@
         <v>2.5</v>
       </c>
       <c r="BM40" t="n">
-        <v>26.29</v>
+        <v>24.78</v>
       </c>
       <c r="BN40" t="n">
         <v>27.36</v>
@@ -9733,19 +9733,19 @@
         <v>17.67</v>
       </c>
       <c r="BP40" t="n">
-        <v>24.37</v>
+        <v>24.1</v>
       </c>
       <c r="BQ40" t="n">
-        <v>9.859999999999999</v>
+        <v>9.68</v>
       </c>
       <c r="BR40" t="n">
-        <v>26.15</v>
+        <v>24.5</v>
       </c>
       <c r="BS40" t="n">
         <v>0.39</v>
       </c>
       <c r="BT40" t="n">
-        <v>40860517</v>
+        <v>43555470</v>
       </c>
     </row>
     <row r="41">
@@ -9775,13 +9775,13 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>19.99</v>
+        <v>19.29</v>
       </c>
       <c r="G41" t="n">
-        <v>201835420046</v>
+        <v>230708456381</v>
       </c>
       <c r="H41" t="n">
-        <v>0</v>
+        <v>19042200</v>
       </c>
       <c r="I41" t="n">
         <v>5303870781</v>
@@ -9796,7 +9796,7 @@
         <v>0.92</v>
       </c>
       <c r="M41" t="n">
-        <v>1.345024872753497</v>
+        <v>1.537433876156565</v>
       </c>
       <c r="N41" t="n">
         <v>0.07000000000000001</v>
@@ -9874,7 +9874,7 @@
         <v>12304980211.92</v>
       </c>
       <c r="AM41" t="n">
-        <v>31099448389.21418</v>
+        <v>35548298363.79044</v>
       </c>
       <c r="AN41" t="n">
         <v>1.6841</v>
@@ -9915,7 +9915,7 @@
         <v>24.4</v>
       </c>
       <c r="AZ41" t="n">
-        <v>29.92</v>
+        <v>28.87</v>
       </c>
       <c r="BA41" t="n">
         <v>2.53</v>
@@ -9924,19 +9924,19 @@
         <v>13.77</v>
       </c>
       <c r="BC41" t="n">
-        <v>49.5</v>
+        <v>54.93</v>
       </c>
       <c r="BD41" t="n">
-        <v>22.07</v>
+        <v>26.5</v>
       </c>
       <c r="BE41" t="n">
         <v>49.67</v>
       </c>
       <c r="BF41" t="n">
-        <v>-87.36</v>
+        <v>-86.90000000000001</v>
       </c>
       <c r="BG41" t="n">
-        <v>-31.12</v>
+        <v>-28.62</v>
       </c>
       <c r="BH41" t="n">
         <v>17.11</v>
@@ -9945,7 +9945,7 @@
         <v>0</v>
       </c>
       <c r="BJ41" t="n">
-        <v>19.99</v>
+        <v>19.29</v>
       </c>
       <c r="BK41" t="n">
         <v>2.32</v>
@@ -9954,28 +9954,28 @@
         <v>2.34</v>
       </c>
       <c r="BM41" t="n">
-        <v>20.24</v>
+        <v>19.95</v>
       </c>
       <c r="BN41" t="n">
         <v>20.24</v>
       </c>
       <c r="BO41" t="n">
-        <v>13.41</v>
+        <v>13.44</v>
       </c>
       <c r="BP41" t="n">
-        <v>19.59</v>
+        <v>19.19</v>
       </c>
       <c r="BQ41" t="n">
-        <v>8.550000000000001</v>
+        <v>8.25</v>
       </c>
       <c r="BR41" t="n">
-        <v>19.7</v>
+        <v>19.95</v>
       </c>
       <c r="BS41" t="n">
         <v>0.5600000000000001</v>
       </c>
       <c r="BT41" t="n">
-        <v>11736093</v>
+        <v>12591443</v>
       </c>
     </row>
     <row r="42">
@@ -10005,13 +10005,13 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>22.8</v>
+        <v>21.96</v>
       </c>
       <c r="G42" t="n">
-        <v>201835420046</v>
+        <v>230708456381</v>
       </c>
       <c r="H42" t="n">
-        <v>0</v>
+        <v>119596100</v>
       </c>
       <c r="I42" t="n">
         <v>5288141247</v>
@@ -10026,7 +10026,7 @@
         <v>1.05</v>
       </c>
       <c r="M42" t="n">
-        <v>1.349025638519507</v>
+        <v>1.542006960969963</v>
       </c>
       <c r="N42" t="n">
         <v>0.08</v>
@@ -10104,7 +10104,7 @@
         <v>12268487693.04</v>
       </c>
       <c r="AM42" t="n">
-        <v>27460601366.80272</v>
+        <v>31388905630.06803</v>
       </c>
       <c r="AN42" t="n">
         <v>1.8491</v>
@@ -10145,7 +10145,7 @@
         <v>24.4</v>
       </c>
       <c r="AZ42" t="n">
-        <v>33.02</v>
+        <v>31.81</v>
       </c>
       <c r="BA42" t="n">
         <v>2.53</v>
@@ -10154,19 +10154,19 @@
         <v>15.11</v>
       </c>
       <c r="BC42" t="n">
-        <v>31.08</v>
+        <v>36.09</v>
       </c>
       <c r="BD42" t="n">
-        <v>7.02</v>
+        <v>11.12</v>
       </c>
       <c r="BE42" t="n">
         <v>44.83</v>
       </c>
       <c r="BF42" t="n">
-        <v>-88.92</v>
+        <v>-88.48999999999999</v>
       </c>
       <c r="BG42" t="n">
-        <v>-33.71</v>
+        <v>-31.17</v>
       </c>
       <c r="BH42" t="n">
         <v>17.11</v>
@@ -10175,7 +10175,7 @@
         <v>0</v>
       </c>
       <c r="BJ42" t="n">
-        <v>22.8</v>
+        <v>21.96</v>
       </c>
       <c r="BK42" t="n">
         <v>2.32</v>
@@ -10184,7 +10184,7 @@
         <v>2.34</v>
       </c>
       <c r="BM42" t="n">
-        <v>23</v>
+        <v>22.81</v>
       </c>
       <c r="BN42" t="n">
         <v>23</v>
@@ -10193,19 +10193,19 @@
         <v>15.65</v>
       </c>
       <c r="BP42" t="n">
-        <v>22.14</v>
+        <v>21.91</v>
       </c>
       <c r="BQ42" t="n">
-        <v>9.75</v>
+        <v>9.390000000000001</v>
       </c>
       <c r="BR42" t="n">
-        <v>22.26</v>
+        <v>22.77</v>
       </c>
       <c r="BS42" t="n">
         <v>0.63</v>
       </c>
       <c r="BT42" t="n">
-        <v>49436283</v>
+        <v>52453280</v>
       </c>
     </row>
     <row r="43">
@@ -10235,13 +10235,13 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>40.08</v>
+        <v>40.28</v>
       </c>
       <c r="G43" t="n">
-        <v>73544318399</v>
+        <v>78199549350</v>
       </c>
       <c r="H43" t="n">
-        <v>0</v>
+        <v>6291500</v>
       </c>
       <c r="I43" t="n">
         <v>1941400000</v>
@@ -10334,7 +10334,7 @@
         <v>9182822000</v>
       </c>
       <c r="AM43" t="n">
-        <v>8957895054.689402</v>
+        <v>9524914658.952496</v>
       </c>
       <c r="AN43" t="n">
         <v>4.5901</v>
@@ -10375,7 +10375,7 @@
         <v>19.95</v>
       </c>
       <c r="AZ43" t="n">
-        <v>72.75</v>
+        <v>73.11</v>
       </c>
       <c r="BA43" t="n">
         <v>5.63</v>
@@ -10384,19 +10384,19 @@
         <v>48.62</v>
       </c>
       <c r="BC43" t="n">
-        <v>-39.04</v>
+        <v>-39.34</v>
       </c>
       <c r="BD43" t="n">
-        <v>-50.22</v>
+        <v>-50.47</v>
       </c>
       <c r="BE43" t="n">
         <v>81.5</v>
       </c>
       <c r="BF43" t="n">
-        <v>-85.95999999999999</v>
+        <v>-86.03</v>
       </c>
       <c r="BG43" t="n">
-        <v>21.3</v>
+        <v>20.7</v>
       </c>
       <c r="BH43" t="n">
         <v>5.61</v>
@@ -10405,7 +10405,7 @@
         <v>0</v>
       </c>
       <c r="BJ43" t="n">
-        <v>40.08</v>
+        <v>40.28</v>
       </c>
       <c r="BK43" t="n">
         <v>4.73</v>
@@ -10414,7 +10414,7 @@
         <v>4.73</v>
       </c>
       <c r="BM43" t="n">
-        <v>41.7</v>
+        <v>40.58</v>
       </c>
       <c r="BN43" t="n">
         <v>42.98</v>
@@ -10423,19 +10423,19 @@
         <v>28.06</v>
       </c>
       <c r="BP43" t="n">
-        <v>39.8</v>
+        <v>39.93</v>
       </c>
       <c r="BQ43" t="n">
-        <v>8.470000000000001</v>
+        <v>8.51</v>
       </c>
       <c r="BR43" t="n">
-        <v>40.99</v>
+        <v>40.1</v>
       </c>
       <c r="BS43" t="n">
         <v>0</v>
       </c>
       <c r="BT43" t="n">
-        <v>6328787</v>
+        <v>6393540</v>
       </c>
     </row>
     <row r="44">
@@ -10925,13 +10925,13 @@
         </is>
       </c>
       <c r="F46" t="n">
-        <v>4.5</v>
+        <v>4.6</v>
       </c>
       <c r="G46" t="n">
-        <v>3993295500</v>
+        <v>4602493104</v>
       </c>
       <c r="H46" t="n">
-        <v>0</v>
+        <v>33100300</v>
       </c>
       <c r="I46" t="n">
         <v>1000542188</v>
@@ -10946,7 +10946,7 @@
         <v>2.5</v>
       </c>
       <c r="M46" t="n">
-        <v>0.06941098358893423</v>
+        <v>0.0799999832994896</v>
       </c>
       <c r="N46" t="n">
         <v>0.08</v>
@@ -11024,7 +11024,7 @@
         <v>460249406.48</v>
       </c>
       <c r="AM46" t="n">
-        <v>3914995588.235294</v>
+        <v>4512248141.176471</v>
       </c>
       <c r="AN46" t="n">
         <v>0.0311</v>
@@ -11065,7 +11065,7 @@
         <v>3.3</v>
       </c>
       <c r="AZ46" t="n">
-        <v>3.71</v>
+        <v>3.8</v>
       </c>
       <c r="BA46" t="n">
         <v>0.42</v>
@@ -11074,19 +11074,19 @@
         <v>7.38</v>
       </c>
       <c r="BC46" t="n">
-        <v>-10.14</v>
+        <v>-12.09</v>
       </c>
       <c r="BD46" t="n">
-        <v>-26.63</v>
+        <v>-28.22</v>
       </c>
       <c r="BE46" t="n">
         <v>-17.5</v>
       </c>
       <c r="BF46" t="n">
-        <v>-90.59999999999999</v>
+        <v>-90.8</v>
       </c>
       <c r="BG46" t="n">
-        <v>63.97</v>
+        <v>60.4</v>
       </c>
       <c r="BH46" t="n">
         <v>1.58</v>
@@ -11095,7 +11095,7 @@
         <v>0</v>
       </c>
       <c r="BJ46" t="n">
-        <v>4.5</v>
+        <v>4.6</v>
       </c>
       <c r="BK46" t="n">
         <v>0.46</v>
@@ -11104,7 +11104,7 @@
         <v>0.46</v>
       </c>
       <c r="BM46" t="n">
-        <v>4.5</v>
+        <v>4.69</v>
       </c>
       <c r="BN46" t="n">
         <v>7.31</v>
@@ -11113,19 +11113,19 @@
         <v>2.97</v>
       </c>
       <c r="BP46" t="n">
-        <v>4.18</v>
+        <v>4.45</v>
       </c>
       <c r="BQ46" t="n">
-        <v>9.84</v>
+        <v>10.06</v>
       </c>
       <c r="BR46" t="n">
-        <v>4.21</v>
+        <v>4.49</v>
       </c>
       <c r="BS46" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="BT46" t="n">
-        <v>22262314</v>
+        <v>23078354</v>
       </c>
     </row>
     <row r="47">
@@ -11155,13 +11155,13 @@
         </is>
       </c>
       <c r="F47" t="n">
-        <v>9.289999999999999</v>
+        <v>9.460000000000001</v>
       </c>
       <c r="G47" t="n">
-        <v>3056806670</v>
+        <v>3277878661</v>
       </c>
       <c r="H47" t="n">
-        <v>0</v>
+        <v>9400</v>
       </c>
       <c r="I47" t="n">
         <v>254106600</v>
@@ -11176,7 +11176,7 @@
         <v>1.22</v>
       </c>
       <c r="M47" t="n">
-        <v>0.7208301821417362</v>
+        <v>0.7729615011102879</v>
       </c>
       <c r="N47" t="n">
         <v>0.07000000000000001</v>
@@ -11254,7 +11254,7 @@
         <v>322715382</v>
       </c>
       <c r="AM47" t="n">
-        <v>541986998.2269504</v>
+        <v>581184159.7517731</v>
       </c>
       <c r="AN47" t="n">
         <v>0.4132</v>
@@ -11295,7 +11295,7 @@
         <v>11.74</v>
       </c>
       <c r="AZ47" t="n">
-        <v>12.2</v>
+        <v>12.42</v>
       </c>
       <c r="BA47" t="n">
         <v>1.46</v>
@@ -11304,28 +11304,28 @@
         <v>8.619999999999999</v>
       </c>
       <c r="BC47" t="n">
-        <v>54.72</v>
+        <v>51.94</v>
       </c>
       <c r="BD47" t="n">
-        <v>26.33</v>
+        <v>24.06</v>
       </c>
       <c r="BE47" t="n">
         <v>31.33</v>
       </c>
       <c r="BF47" t="n">
-        <v>-84.3</v>
+        <v>-84.58</v>
       </c>
       <c r="BG47" t="n">
-        <v>-7.22</v>
+        <v>-8.880000000000001</v>
       </c>
       <c r="BH47" t="n">
         <v>7.23</v>
       </c>
       <c r="BI47" t="n">
-        <v>-0.32</v>
+        <v>0</v>
       </c>
       <c r="BJ47" t="n">
-        <v>9.32</v>
+        <v>9.460000000000001</v>
       </c>
       <c r="BK47" t="n">
         <v>1.27</v>
@@ -11334,7 +11334,7 @@
         <v>1.28</v>
       </c>
       <c r="BM47" t="n">
-        <v>9.6</v>
+        <v>9.5</v>
       </c>
       <c r="BN47" t="n">
         <v>9.6</v>
@@ -11343,19 +11343,19 @@
         <v>7.12</v>
       </c>
       <c r="BP47" t="n">
-        <v>9.199999999999999</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="BQ47" t="n">
-        <v>7.24</v>
+        <v>7.38</v>
       </c>
       <c r="BR47" t="n">
-        <v>9.27</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="BS47" t="n">
         <v>0.53</v>
       </c>
       <c r="BT47" t="n">
-        <v>12140</v>
+        <v>12533</v>
       </c>
     </row>
     <row r="48">
@@ -11385,13 +11385,13 @@
         </is>
       </c>
       <c r="F48" t="n">
-        <v>9.19</v>
+        <v>9.41</v>
       </c>
       <c r="G48" t="n">
-        <v>3056806670</v>
+        <v>3277878661</v>
       </c>
       <c r="H48" t="n">
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="I48" t="n">
         <v>93397546</v>
@@ -11406,7 +11406,7 @@
         <v>1.24</v>
       </c>
       <c r="M48" t="n">
-        <v>1.961161878508214</v>
+        <v>2.102995500310378</v>
       </c>
       <c r="N48" t="n">
         <v>0.07000000000000001</v>
@@ -11484,7 +11484,7 @@
         <v>118614883.42</v>
       </c>
       <c r="AM48" t="n">
-        <v>534406760.4895105</v>
+        <v>573055709.965035</v>
       </c>
       <c r="AN48" t="n">
         <v>0.4132</v>
@@ -11525,7 +11525,7 @@
         <v>11.74</v>
       </c>
       <c r="AZ48" t="n">
-        <v>12.02</v>
+        <v>12.31</v>
       </c>
       <c r="BA48" t="n">
         <v>1.46</v>
@@ -11534,28 +11534,28 @@
         <v>8.24</v>
       </c>
       <c r="BC48" t="n">
-        <v>56.4</v>
+        <v>52.75</v>
       </c>
       <c r="BD48" t="n">
-        <v>27.7</v>
+        <v>24.72</v>
       </c>
       <c r="BE48" t="n">
         <v>30.83</v>
       </c>
       <c r="BF48" t="n">
-        <v>-84.13</v>
+        <v>-84.5</v>
       </c>
       <c r="BG48" t="n">
-        <v>-10.38</v>
+        <v>-12.47</v>
       </c>
       <c r="BH48" t="n">
         <v>7.23</v>
       </c>
       <c r="BI48" t="n">
-        <v>-0.22</v>
+        <v>0</v>
       </c>
       <c r="BJ48" t="n">
-        <v>9.210000000000001</v>
+        <v>9.41</v>
       </c>
       <c r="BK48" t="n">
         <v>1.27</v>
@@ -11564,28 +11564,28 @@
         <v>1.28</v>
       </c>
       <c r="BM48" t="n">
-        <v>9.529999999999999</v>
+        <v>9.57</v>
       </c>
       <c r="BN48" t="n">
-        <v>9.529999999999999</v>
+        <v>9.57</v>
       </c>
       <c r="BO48" t="n">
         <v>7.13</v>
       </c>
       <c r="BP48" t="n">
-        <v>9.19</v>
+        <v>9.369999999999999</v>
       </c>
       <c r="BQ48" t="n">
-        <v>7.16</v>
+        <v>7.34</v>
       </c>
       <c r="BR48" t="n">
-        <v>9.529999999999999</v>
+        <v>9.460000000000001</v>
       </c>
       <c r="BS48" t="n">
         <v>0.54</v>
       </c>
       <c r="BT48" t="n">
-        <v>2763</v>
+        <v>2903</v>
       </c>
     </row>
     <row r="49">
@@ -11615,13 +11615,13 @@
         </is>
       </c>
       <c r="F49" t="n">
-        <v>47.39</v>
+        <v>48.06</v>
       </c>
       <c r="G49" t="n">
-        <v>934898060</v>
+        <v>957389830</v>
       </c>
       <c r="H49" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="I49" t="n">
         <v>11540870</v>
@@ -11636,7 +11636,7 @@
         <v>1.09</v>
       </c>
       <c r="M49" t="n">
-        <v>0.9458243084961065</v>
+        <v>0.9685789420944515</v>
       </c>
       <c r="N49" t="n">
         <v>0.08</v>
@@ -11714,7 +11714,7 @@
         <v>84709985.8</v>
       </c>
       <c r="AM49" t="n">
-        <v>233724515</v>
+        <v>239347457.5</v>
       </c>
       <c r="AN49" t="n">
         <v>3.3186</v>
@@ -11755,7 +11755,7 @@
         <v>68.48999999999999</v>
       </c>
       <c r="AZ49" t="n">
-        <v>56.55</v>
+        <v>57.35</v>
       </c>
       <c r="BA49" t="n">
         <v>9.210000000000001</v>
@@ -11764,19 +11764,19 @@
         <v>27.75</v>
       </c>
       <c r="BC49" t="n">
-        <v>76.98999999999999</v>
+        <v>74.53</v>
       </c>
       <c r="BD49" t="n">
-        <v>44.51</v>
+        <v>42.5</v>
       </c>
       <c r="BE49" t="n">
         <v>19.33</v>
       </c>
       <c r="BF49" t="n">
-        <v>-80.56</v>
+        <v>-80.83</v>
       </c>
       <c r="BG49" t="n">
-        <v>-41.43</v>
+        <v>-42.25</v>
       </c>
       <c r="BH49" t="n">
         <v>42.6</v>
@@ -11785,7 +11785,7 @@
         <v>0</v>
       </c>
       <c r="BJ49" t="n">
-        <v>47.39</v>
+        <v>48.06</v>
       </c>
       <c r="BK49" t="n">
         <v>7.34</v>
@@ -11794,7 +11794,7 @@
         <v>7.6</v>
       </c>
       <c r="BM49" t="n">
-        <v>48.07</v>
+        <v>48.06</v>
       </c>
       <c r="BN49" t="n">
         <v>64.2</v>
@@ -11803,19 +11803,19 @@
         <v>28.48</v>
       </c>
       <c r="BP49" t="n">
-        <v>47.39</v>
+        <v>48.06</v>
       </c>
       <c r="BQ49" t="n">
-        <v>6.23</v>
+        <v>6.32</v>
       </c>
       <c r="BR49" t="n">
-        <v>48.07</v>
+        <v>48.06</v>
       </c>
       <c r="BS49" t="n">
         <v>0.54</v>
       </c>
       <c r="BT49" t="n">
-        <v>377</v>
+        <v>383</v>
       </c>
     </row>
     <row r="50">
@@ -11845,13 +11845,13 @@
         </is>
       </c>
       <c r="F50" t="n">
-        <v>34.41</v>
+        <v>35.11</v>
       </c>
       <c r="G50" t="n">
-        <v>908275800</v>
+        <v>957389830</v>
       </c>
       <c r="H50" t="n">
-        <v>0</v>
+        <v>500</v>
       </c>
       <c r="I50" t="n">
         <v>11540870</v>
@@ -11866,7 +11866,7 @@
         <v>0.8</v>
       </c>
       <c r="M50" t="n">
-        <v>0.9188909114419898</v>
+        <v>0.9685789420944515</v>
       </c>
       <c r="N50" t="n">
         <v>0.06</v>
@@ -11944,7 +11944,7 @@
         <v>84709985.8</v>
       </c>
       <c r="AM50" t="n">
-        <v>309991740.6143345</v>
+        <v>326754208.1911263</v>
       </c>
       <c r="AN50" t="n">
         <v>4.4983</v>
@@ -11985,7 +11985,7 @@
         <v>68.48999999999999</v>
       </c>
       <c r="AZ50" t="n">
-        <v>75.87</v>
+        <v>77.42</v>
       </c>
       <c r="BA50" t="n">
         <v>9.210000000000001</v>
@@ -11994,28 +11994,28 @@
         <v>30.53</v>
       </c>
       <c r="BC50" t="n">
-        <v>143.76</v>
+        <v>138.9</v>
       </c>
       <c r="BD50" t="n">
-        <v>99.03</v>
+        <v>95.06</v>
       </c>
       <c r="BE50" t="n">
         <v>120.5</v>
       </c>
       <c r="BF50" t="n">
-        <v>-73.22</v>
+        <v>-73.76000000000001</v>
       </c>
       <c r="BG50" t="n">
-        <v>-11.27</v>
+        <v>-13.04</v>
       </c>
       <c r="BH50" t="n">
         <v>42.6</v>
       </c>
       <c r="BI50" t="n">
-        <v>1.18</v>
+        <v>0</v>
       </c>
       <c r="BJ50" t="n">
-        <v>34.01</v>
+        <v>35.11</v>
       </c>
       <c r="BK50" t="n">
         <v>7.34</v>
@@ -12024,28 +12024,28 @@
         <v>7.6</v>
       </c>
       <c r="BM50" t="n">
-        <v>34.42</v>
+        <v>35.11</v>
       </c>
       <c r="BN50" t="n">
         <v>39.22</v>
       </c>
       <c r="BO50" t="n">
-        <v>24.28</v>
+        <v>24.3</v>
       </c>
       <c r="BP50" t="n">
-        <v>33.92</v>
+        <v>34.7</v>
       </c>
       <c r="BQ50" t="n">
-        <v>4.53</v>
+        <v>4.62</v>
       </c>
       <c r="BR50" t="n">
-        <v>33.92</v>
+        <v>34.7</v>
       </c>
       <c r="BS50" t="n">
         <v>0.4</v>
       </c>
       <c r="BT50" t="n">
-        <v>517</v>
+        <v>523</v>
       </c>
     </row>
     <row r="51">
@@ -12523,13 +12523,13 @@
         </is>
       </c>
       <c r="F53" t="n">
-        <v>6.86</v>
+        <v>6.9</v>
       </c>
       <c r="G53" t="n">
-        <v>900567783</v>
+        <v>944281573</v>
       </c>
       <c r="H53" t="n">
-        <v>0</v>
+        <v>184700</v>
       </c>
       <c r="I53" t="n">
         <v>136852484</v>
@@ -12544,7 +12544,7 @@
         <v>2.79</v>
       </c>
       <c r="M53" t="n">
-        <v>2.339507216304831</v>
+        <v>2.453067493596067</v>
       </c>
       <c r="N53" t="n">
         <v>1.48</v>
@@ -12622,7 +12622,7 @@
         <v>39687220.36</v>
       </c>
       <c r="AM53" t="n">
-        <v>45877115.79215487</v>
+        <v>48104002.69994906</v>
       </c>
       <c r="AN53" t="n">
         <v>0</v>
@@ -12672,16 +12672,16 @@
         <v>0</v>
       </c>
       <c r="BC53" t="n">
-        <v>-42.55</v>
+        <v>-42.89</v>
       </c>
       <c r="BD53" t="n">
-        <v>-53.1</v>
+        <v>-53.37</v>
       </c>
       <c r="BE53" t="n">
         <v>-100</v>
       </c>
       <c r="BF53" t="n">
-        <v>-95.77</v>
+        <v>-95.8</v>
       </c>
       <c r="BG53" t="n">
         <v>-100</v>
@@ -12693,7 +12693,7 @@
         <v>0</v>
       </c>
       <c r="BJ53" t="n">
-        <v>6.86</v>
+        <v>6.9</v>
       </c>
       <c r="BK53" t="n">
         <v>0.29</v>
@@ -12702,7 +12702,7 @@
         <v>0.2</v>
       </c>
       <c r="BM53" t="n">
-        <v>6.86</v>
+        <v>7.1</v>
       </c>
       <c r="BN53" t="n">
         <v>10.39</v>
@@ -12711,19 +12711,19 @@
         <v>4.82</v>
       </c>
       <c r="BP53" t="n">
-        <v>6.43</v>
+        <v>6.61</v>
       </c>
       <c r="BQ53" t="n">
-        <v>33.7</v>
+        <v>33.89</v>
       </c>
       <c r="BR53" t="n">
-        <v>6.43</v>
+        <v>6.85</v>
       </c>
       <c r="BS53" t="n">
         <v>2.36</v>
       </c>
       <c r="BT53" t="n">
-        <v>40470</v>
+        <v>42107</v>
       </c>
     </row>
     <row r="54">
@@ -12753,13 +12753,13 @@
         </is>
       </c>
       <c r="F54" t="n">
-        <v>11.95</v>
+        <v>11.97</v>
       </c>
       <c r="G54" t="n">
-        <v>2472687985</v>
+        <v>2791548899</v>
       </c>
       <c r="H54" t="n">
-        <v>0</v>
+        <v>318100</v>
       </c>
       <c r="I54" t="n">
         <v>233212121</v>
@@ -12774,7 +12774,7 @@
         <v>0.97</v>
       </c>
       <c r="M54" t="n">
-        <v>1.387898947312863</v>
+        <v>1.566872893708213</v>
       </c>
       <c r="N54" t="n">
         <v>0.5600000000000001</v>
@@ -12852,7 +12852,7 @@
         <v>233212121</v>
       </c>
       <c r="AM54" t="n">
-        <v>338261010.2599179</v>
+        <v>381880834.3365253</v>
       </c>
       <c r="AN54" t="n">
         <v>0.1531</v>
@@ -12893,7 +12893,7 @@
         <v>12.25</v>
       </c>
       <c r="AZ54" t="n">
-        <v>19.02</v>
+        <v>19.05</v>
       </c>
       <c r="BA54" t="n">
         <v>0.98</v>
@@ -12902,28 +12902,28 @@
         <v>6.52</v>
       </c>
       <c r="BC54" t="n">
-        <v>25.59</v>
+        <v>25.38</v>
       </c>
       <c r="BD54" t="n">
-        <v>2.54</v>
+        <v>2.37</v>
       </c>
       <c r="BE54" t="n">
         <v>59.17</v>
       </c>
       <c r="BF54" t="n">
-        <v>-91.77</v>
+        <v>-91.79000000000001</v>
       </c>
       <c r="BG54" t="n">
-        <v>-45.47</v>
+        <v>-45.56</v>
       </c>
       <c r="BH54" t="n">
         <v>10.01</v>
       </c>
       <c r="BI54" t="n">
-        <v>2.31</v>
+        <v>0</v>
       </c>
       <c r="BJ54" t="n">
-        <v>11.68</v>
+        <v>11.97</v>
       </c>
       <c r="BK54" t="n">
         <v>1</v>
@@ -12932,7 +12932,7 @@
         <v>1</v>
       </c>
       <c r="BM54" t="n">
-        <v>12.15</v>
+        <v>12.11</v>
       </c>
       <c r="BN54" t="n">
         <v>12.15</v>
@@ -12941,19 +12941,19 @@
         <v>8.23</v>
       </c>
       <c r="BP54" t="n">
-        <v>11.54</v>
+        <v>11.86</v>
       </c>
       <c r="BQ54" t="n">
-        <v>11.92</v>
+        <v>11.94</v>
       </c>
       <c r="BR54" t="n">
-        <v>11.59</v>
+        <v>11.88</v>
       </c>
       <c r="BS54" t="n">
         <v>1.26</v>
       </c>
       <c r="BT54" t="n">
-        <v>267900</v>
+        <v>275960</v>
       </c>
     </row>
     <row r="55">
@@ -12983,13 +12983,13 @@
         </is>
       </c>
       <c r="F55" t="n">
-        <v>55.44</v>
+        <v>57</v>
       </c>
       <c r="G55" t="n">
-        <v>6835589641</v>
+        <v>7809007282</v>
       </c>
       <c r="H55" t="n">
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="I55" t="n">
         <v>84052790</v>
@@ -13004,7 +13004,7 @@
         <v>2</v>
       </c>
       <c r="M55" t="n">
-        <v>1.055217891324197</v>
+        <v>1.205485500186031</v>
       </c>
       <c r="N55" t="n">
         <v>0.16</v>
@@ -13082,7 +13082,7 @@
         <v>579123723.1</v>
       </c>
       <c r="AM55" t="n">
-        <v>343842537.2736419</v>
+        <v>392807207.3440644</v>
       </c>
       <c r="AN55" t="n">
         <v>3.1953</v>
@@ -13123,7 +13123,7 @@
         <v>51.21</v>
       </c>
       <c r="AZ55" t="n">
-        <v>58.3</v>
+        <v>59.94</v>
       </c>
       <c r="BA55" t="n">
         <v>9.380000000000001</v>
@@ -13132,19 +13132,19 @@
         <v>16.08</v>
       </c>
       <c r="BC55" t="n">
-        <v>13.12</v>
+        <v>10.02</v>
       </c>
       <c r="BD55" t="n">
-        <v>-7.64</v>
+        <v>-10.17</v>
       </c>
       <c r="BE55" t="n">
         <v>5.17</v>
       </c>
       <c r="BF55" t="n">
-        <v>-83.08</v>
+        <v>-83.55</v>
       </c>
       <c r="BG55" t="n">
-        <v>-71</v>
+        <v>-71.8</v>
       </c>
       <c r="BH55" t="n">
         <v>25.37</v>
@@ -13153,7 +13153,7 @@
         <v>0</v>
       </c>
       <c r="BJ55" t="n">
-        <v>55.44</v>
+        <v>57</v>
       </c>
       <c r="BK55" t="n">
         <v>6.89</v>
@@ -13162,7 +13162,7 @@
         <v>7.03</v>
       </c>
       <c r="BM55" t="n">
-        <v>56.39</v>
+        <v>58.09</v>
       </c>
       <c r="BN55" t="n">
         <v>73.67</v>
@@ -13171,19 +13171,19 @@
         <v>35.58</v>
       </c>
       <c r="BP55" t="n">
-        <v>54.42</v>
+        <v>55.8</v>
       </c>
       <c r="BQ55" t="n">
-        <v>7.89</v>
+        <v>8.109999999999999</v>
       </c>
       <c r="BR55" t="n">
-        <v>54.92</v>
+        <v>56.46</v>
       </c>
       <c r="BS55" t="n">
         <v>0.66</v>
       </c>
       <c r="BT55" t="n">
-        <v>6290</v>
+        <v>6437</v>
       </c>
     </row>
     <row r="56">
@@ -13213,13 +13213,13 @@
         </is>
       </c>
       <c r="F56" t="n">
-        <v>71.23999999999999</v>
+        <v>74.31</v>
       </c>
       <c r="G56" t="n">
-        <v>6835589641</v>
+        <v>7809007282</v>
       </c>
       <c r="H56" t="n">
-        <v>35700</v>
+        <v>44700</v>
       </c>
       <c r="I56" t="n">
         <v>39675836</v>
@@ -13234,7 +13234,7 @@
         <v>2.41</v>
       </c>
       <c r="M56" t="n">
-        <v>2.235466640796568</v>
+        <v>2.5538067955312</v>
       </c>
       <c r="N56" t="n">
         <v>0.19</v>
@@ -13312,7 +13312,7 @@
         <v>273366510.04</v>
       </c>
       <c r="AM56" t="n">
-        <v>284342331.156406</v>
+        <v>324833913.5607321</v>
       </c>
       <c r="AN56" t="n">
         <v>3.5102</v>
@@ -13353,7 +13353,7 @@
         <v>51.21</v>
       </c>
       <c r="AZ56" t="n">
-        <v>68.03</v>
+        <v>70.97</v>
       </c>
       <c r="BA56" t="n">
         <v>9.380000000000001</v>
@@ -13362,19 +13362,19 @@
         <v>17.68</v>
       </c>
       <c r="BC56" t="n">
-        <v>-11.97</v>
+        <v>-15.61</v>
       </c>
       <c r="BD56" t="n">
-        <v>-28.12</v>
+        <v>-31.09</v>
       </c>
       <c r="BE56" t="n">
         <v>-4.5</v>
       </c>
       <c r="BF56" t="n">
-        <v>-86.84</v>
+        <v>-87.38</v>
       </c>
       <c r="BG56" t="n">
-        <v>-75.19</v>
+        <v>-76.20999999999999</v>
       </c>
       <c r="BH56" t="n">
         <v>25.37</v>
@@ -13383,7 +13383,7 @@
         <v>0</v>
       </c>
       <c r="BJ56" t="n">
-        <v>71.23999999999999</v>
+        <v>74.31</v>
       </c>
       <c r="BK56" t="n">
         <v>6.89</v>
@@ -13392,7 +13392,7 @@
         <v>7.03</v>
       </c>
       <c r="BM56" t="n">
-        <v>71.37</v>
+        <v>74.98</v>
       </c>
       <c r="BN56" t="n">
         <v>86.77</v>
@@ -13401,19 +13401,19 @@
         <v>46.42</v>
       </c>
       <c r="BP56" t="n">
-        <v>67.36</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="BQ56" t="n">
-        <v>10.13</v>
+        <v>10.57</v>
       </c>
       <c r="BR56" t="n">
-        <v>67.36</v>
+        <v>71</v>
       </c>
       <c r="BS56" t="n">
         <v>0.79</v>
       </c>
       <c r="BT56" t="n">
-        <v>27717</v>
+        <v>27680</v>
       </c>
     </row>
     <row r="57">
@@ -13443,13 +13443,13 @@
         </is>
       </c>
       <c r="F57" t="n">
-        <v>6.87</v>
+        <v>6.73</v>
       </c>
       <c r="G57" t="n">
-        <v>1469640680</v>
+        <v>1573864344</v>
       </c>
       <c r="H57" t="n">
-        <v>1858700</v>
+        <v>990800</v>
       </c>
       <c r="I57" t="n">
         <v>233858065</v>
@@ -13464,7 +13464,7 @@
         <v>0.77</v>
       </c>
       <c r="M57" t="n">
-        <v>0.4399029282996933</v>
+        <v>0.4710998702567731</v>
       </c>
       <c r="N57" t="n">
         <v>0.08</v>
@@ -13542,7 +13542,7 @@
         <v>229180903.7</v>
       </c>
       <c r="AM57" t="n">
-        <v>109920768.8855647</v>
+        <v>117716106.5071055</v>
       </c>
       <c r="AN57" t="n">
         <v>0.347</v>
@@ -13583,7 +13583,7 @@
         <v>10.72</v>
       </c>
       <c r="AZ57" t="n">
-        <v>10.48</v>
+        <v>10.26</v>
       </c>
       <c r="BA57" t="n">
         <v>1.13</v>
@@ -13592,19 +13592,19 @@
         <v>6.26</v>
       </c>
       <c r="BC57" t="n">
-        <v>91.14</v>
+        <v>95.12</v>
       </c>
       <c r="BD57" t="n">
-        <v>56.06</v>
+        <v>59.31</v>
       </c>
       <c r="BE57" t="n">
         <v>52.5</v>
       </c>
       <c r="BF57" t="n">
-        <v>-83.59</v>
+        <v>-83.25</v>
       </c>
       <c r="BG57" t="n">
-        <v>-8.82</v>
+        <v>-6.93</v>
       </c>
       <c r="BH57" t="n">
         <v>7.82</v>
@@ -13613,7 +13613,7 @@
         <v>0</v>
       </c>
       <c r="BJ57" t="n">
-        <v>6.87</v>
+        <v>6.73</v>
       </c>
       <c r="BK57" t="n">
         <v>0.98</v>
@@ -13622,7 +13622,7 @@
         <v>1.04</v>
       </c>
       <c r="BM57" t="n">
-        <v>6.98</v>
+        <v>6.88</v>
       </c>
       <c r="BN57" t="n">
         <v>7.03</v>
@@ -13631,19 +13631,19 @@
         <v>3.43</v>
       </c>
       <c r="BP57" t="n">
-        <v>6.78</v>
+        <v>6.73</v>
       </c>
       <c r="BQ57" t="n">
-        <v>6.63</v>
+        <v>6.5</v>
       </c>
       <c r="BR57" t="n">
-        <v>6.9</v>
+        <v>6.88</v>
       </c>
       <c r="BS57" t="n">
         <v>0.42</v>
       </c>
       <c r="BT57" t="n">
-        <v>1582530</v>
+        <v>1603800</v>
       </c>
     </row>
     <row r="58">
@@ -14133,13 +14133,13 @@
         </is>
       </c>
       <c r="F60" t="n">
-        <v>380</v>
+        <v>388.46</v>
       </c>
       <c r="G60" t="n">
-        <v>159992274</v>
+        <v>176652181</v>
       </c>
       <c r="H60" t="n">
-        <v>0</v>
+        <v>227</v>
       </c>
       <c r="I60" t="n">
         <v>454750</v>
@@ -14154,7 +14154,7 @@
         <v>0.83</v>
       </c>
       <c r="M60" t="n">
-        <v>11.96719687314046</v>
+        <v>13.21333446449197</v>
       </c>
       <c r="N60" t="n">
         <v>0.68</v>
@@ -14232,7 +14232,7 @@
         <v>59558607.5</v>
       </c>
       <c r="AM60" t="n">
-        <v>-23459277.71260997</v>
+        <v>-25902079.3255132</v>
       </c>
       <c r="AN60" t="n">
         <v>10.0581</v>
@@ -14273,7 +14273,7 @@
         <v>944.87</v>
       </c>
       <c r="AZ60" t="n">
-        <v>2185</v>
+        <v>2233.64</v>
       </c>
       <c r="BA60" t="n">
         <v>231.1</v>
@@ -14282,28 +14282,28 @@
         <v>727.97</v>
       </c>
       <c r="BC60" t="n">
-        <v>204.53</v>
+        <v>197.9</v>
       </c>
       <c r="BD60" t="n">
-        <v>148.65</v>
+        <v>143.23</v>
       </c>
       <c r="BE60" t="n">
         <v>475</v>
       </c>
       <c r="BF60" t="n">
-        <v>-39.19</v>
+        <v>-40.51</v>
       </c>
       <c r="BG60" t="n">
-        <v>91.56999999999999</v>
+        <v>87.40000000000001</v>
       </c>
       <c r="BH60" t="n">
         <v>454.44</v>
       </c>
       <c r="BI60" t="n">
-        <v>0.8</v>
+        <v>0</v>
       </c>
       <c r="BJ60" t="n">
-        <v>377</v>
+        <v>388.46</v>
       </c>
       <c r="BK60" t="n">
         <v>130.97</v>
@@ -14312,7 +14312,7 @@
         <v>130.97</v>
       </c>
       <c r="BM60" t="n">
-        <v>390</v>
+        <v>388.98</v>
       </c>
       <c r="BN60" t="n">
         <v>405</v>
@@ -14321,19 +14321,19 @@
         <v>309.24</v>
       </c>
       <c r="BP60" t="n">
-        <v>380</v>
+        <v>356</v>
       </c>
       <c r="BQ60" t="n">
-        <v>2.9</v>
+        <v>2.97</v>
       </c>
       <c r="BR60" t="n">
-        <v>390</v>
+        <v>379</v>
       </c>
       <c r="BS60" t="n">
         <v>12.82</v>
       </c>
       <c r="BT60" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="61">
@@ -14363,13 +14363,13 @@
         </is>
       </c>
       <c r="F61" t="n">
-        <v>30.53</v>
+        <v>30.92</v>
       </c>
       <c r="G61" t="n">
-        <v>2323711013</v>
+        <v>2647011116</v>
       </c>
       <c r="H61" t="n">
-        <v>0</v>
+        <v>1249100</v>
       </c>
       <c r="I61" t="n">
         <v>85608392</v>
@@ -14384,7 +14384,7 @@
         <v>2.37</v>
       </c>
       <c r="M61" t="n">
-        <v>1.232343731472264</v>
+        <v>1.403800876137605</v>
       </c>
       <c r="N61" t="n">
         <v>1.1</v>
@@ -14462,7 +14462,7 @@
         <v>160087693.04</v>
       </c>
       <c r="AM61" t="n">
-        <v>182394898.9795918</v>
+        <v>207771673.155416</v>
       </c>
       <c r="AN61" t="n">
         <v>0.38</v>
@@ -14503,7 +14503,7 @@
         <v>17.56</v>
       </c>
       <c r="AZ61" t="n">
-        <v>38.47</v>
+        <v>38.96</v>
       </c>
       <c r="BA61" t="n">
         <v>2.52</v>
@@ -14512,19 +14512,19 @@
         <v>11.76</v>
       </c>
       <c r="BC61" t="n">
-        <v>-29.57</v>
+        <v>-30.45</v>
       </c>
       <c r="BD61" t="n">
-        <v>-42.49</v>
+        <v>-43.22</v>
       </c>
       <c r="BE61" t="n">
         <v>26</v>
       </c>
       <c r="BF61" t="n">
-        <v>-91.73999999999999</v>
+        <v>-91.84</v>
       </c>
       <c r="BG61" t="n">
-        <v>-61.49</v>
+        <v>-61.98</v>
       </c>
       <c r="BH61" t="n">
         <v>10.99</v>
@@ -14533,7 +14533,7 @@
         <v>0</v>
       </c>
       <c r="BJ61" t="n">
-        <v>30.53</v>
+        <v>30.92</v>
       </c>
       <c r="BK61" t="n">
         <v>1.87</v>
@@ -14542,28 +14542,28 @@
         <v>1.86</v>
       </c>
       <c r="BM61" t="n">
-        <v>30.65</v>
+        <v>31.28</v>
       </c>
       <c r="BN61" t="n">
-        <v>30.75</v>
+        <v>31.28</v>
       </c>
       <c r="BO61" t="n">
         <v>19.35</v>
       </c>
       <c r="BP61" t="n">
-        <v>30.14</v>
+        <v>30.35</v>
       </c>
       <c r="BQ61" t="n">
-        <v>16.4</v>
+        <v>16.61</v>
       </c>
       <c r="BR61" t="n">
-        <v>30.51</v>
+        <v>30.35</v>
       </c>
       <c r="BS61" t="n">
         <v>1.19</v>
       </c>
       <c r="BT61" t="n">
-        <v>763527</v>
+        <v>806107</v>
       </c>
     </row>
     <row r="62">
@@ -14593,13 +14593,13 @@
         </is>
       </c>
       <c r="F62" t="n">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="G62" t="n">
-        <v>10494785730</v>
+        <v>11350468950</v>
       </c>
       <c r="H62" t="n">
-        <v>500</v>
+        <v>100</v>
       </c>
       <c r="I62" t="n">
         <v>98699749</v>
@@ -14614,7 +14614,7 @@
         <v>0.64</v>
       </c>
       <c r="M62" t="n">
-        <v>0.9837656935634919</v>
+        <v>1.063976173134087</v>
       </c>
       <c r="N62" t="n">
         <v>0.13</v>
@@ -14692,7 +14692,7 @@
         <v>2757670987.06</v>
       </c>
       <c r="AM62" t="n">
-        <v>4248901105.263157</v>
+        <v>4595331558.704453</v>
       </c>
       <c r="AN62" t="n">
         <v>6.9319</v>
@@ -14733,7 +14733,7 @@
         <v>267.2</v>
       </c>
       <c r="AZ62" t="n">
-        <v>119.4</v>
+        <v>121.52</v>
       </c>
       <c r="BA62" t="n">
         <v>34.09</v>
@@ -14742,19 +14742,19 @@
         <v>76.01000000000001</v>
       </c>
       <c r="BC62" t="n">
-        <v>189.6</v>
+        <v>184.56</v>
       </c>
       <c r="BD62" t="n">
-        <v>136.46</v>
+        <v>132.34</v>
       </c>
       <c r="BE62" t="n">
         <v>5.67</v>
       </c>
       <c r="BF62" t="n">
-        <v>-69.83</v>
+        <v>-70.34999999999999</v>
       </c>
       <c r="BG62" t="n">
-        <v>-32.74</v>
+        <v>-33.91</v>
       </c>
       <c r="BH62" t="n">
         <v>170.35</v>
@@ -14763,7 +14763,7 @@
         <v>0</v>
       </c>
       <c r="BJ62" t="n">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="BK62" t="n">
         <v>27.94</v>
@@ -14772,7 +14772,7 @@
         <v>32.73</v>
       </c>
       <c r="BM62" t="n">
-        <v>114.25</v>
+        <v>115</v>
       </c>
       <c r="BN62" t="n">
         <v>122.2</v>
@@ -14781,19 +14781,19 @@
         <v>91.84999999999999</v>
       </c>
       <c r="BP62" t="n">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="BQ62" t="n">
-        <v>3.45</v>
+        <v>3.51</v>
       </c>
       <c r="BR62" t="n">
-        <v>114.25</v>
+        <v>115</v>
       </c>
       <c r="BS62" t="n">
         <v>1.01</v>
       </c>
       <c r="BT62" t="n">
-        <v>123</v>
+        <v>137</v>
       </c>
     </row>
     <row r="63">
@@ -14823,13 +14823,13 @@
         </is>
       </c>
       <c r="F63" t="n">
-        <v>1.62</v>
+        <v>1.58</v>
       </c>
       <c r="G63" t="n">
-        <v>414572257</v>
+        <v>411605337</v>
       </c>
       <c r="H63" t="n">
-        <v>81700</v>
+        <v>7200</v>
       </c>
       <c r="I63" t="n">
         <v>122894462</v>
@@ -14844,7 +14844,7 @@
         <v>-0.22</v>
       </c>
       <c r="M63" t="n">
-        <v>0.5099024816450295</v>
+        <v>0.5062533231562543</v>
       </c>
       <c r="N63" t="n">
         <v>0.37</v>
@@ -14922,7 +14922,7 @@
         <v>31952560.12</v>
       </c>
       <c r="AM63" t="n">
-        <v>235552418.75</v>
+        <v>233866668.75</v>
       </c>
       <c r="AN63" t="n">
         <v>0</v>
@@ -14981,7 +14981,7 @@
         <v>-100</v>
       </c>
       <c r="BF63" t="n">
-        <v>-82.15000000000001</v>
+        <v>-81.7</v>
       </c>
       <c r="BG63" t="n">
         <v>-100</v>
@@ -14993,7 +14993,7 @@
         <v>0</v>
       </c>
       <c r="BJ63" t="n">
-        <v>1.62</v>
+        <v>1.58</v>
       </c>
       <c r="BK63" t="n">
         <v>0.26</v>
@@ -15002,7 +15002,7 @@
         <v>0.26</v>
       </c>
       <c r="BM63" t="n">
-        <v>1.7</v>
+        <v>1.68</v>
       </c>
       <c r="BN63" t="n">
         <v>2.12</v>
@@ -15011,19 +15011,19 @@
         <v>1.16</v>
       </c>
       <c r="BP63" t="n">
-        <v>1.58</v>
+        <v>1.53</v>
       </c>
       <c r="BQ63" t="n">
-        <v>6.21</v>
+        <v>6.05</v>
       </c>
       <c r="BR63" t="n">
-        <v>1.58</v>
+        <v>1.6</v>
       </c>
       <c r="BS63" t="n">
         <v>0.19</v>
       </c>
       <c r="BT63" t="n">
-        <v>33517</v>
+        <v>35820</v>
       </c>
     </row>
     <row r="64">
@@ -15053,13 +15053,13 @@
         </is>
       </c>
       <c r="F64" t="n">
-        <v>78.62</v>
+        <v>76.64</v>
       </c>
       <c r="G64" t="n">
-        <v>227765685856</v>
+        <v>267448153390</v>
       </c>
       <c r="H64" t="n">
-        <v>0</v>
+        <v>25964600</v>
       </c>
       <c r="I64" t="n">
         <v>0</v>
@@ -15146,13 +15146,13 @@
         <v>41.22</v>
       </c>
       <c r="AK64" t="n">
-        <v>65303764407.6991</v>
+        <v>76681310157.03937</v>
       </c>
       <c r="AL64" t="n">
-        <v>18206689516.86651</v>
+        <v>21378749271.78257</v>
       </c>
       <c r="AM64" t="n">
-        <v>20281895445.77026</v>
+        <v>23815507870.88157</v>
       </c>
       <c r="AN64" t="n">
         <v>1.4201</v>
@@ -15193,7 +15193,7 @@
         <v>38.98</v>
       </c>
       <c r="AZ64" t="n">
-        <v>31.45</v>
+        <v>30.66</v>
       </c>
       <c r="BA64" t="n">
         <v>6.69</v>
@@ -15202,28 +15202,28 @@
         <v>10.4</v>
       </c>
       <c r="BC64" t="n">
-        <v>-39.28</v>
+        <v>-37.71</v>
       </c>
       <c r="BD64" t="n">
-        <v>-50.42</v>
+        <v>-49.14</v>
       </c>
       <c r="BE64" t="n">
         <v>-60</v>
       </c>
       <c r="BF64" t="n">
-        <v>-91.48999999999999</v>
+        <v>-91.27</v>
       </c>
       <c r="BG64" t="n">
-        <v>-86.77</v>
+        <v>-86.43000000000001</v>
       </c>
       <c r="BH64" t="n">
         <v>21.37</v>
       </c>
       <c r="BI64" t="n">
-        <v>-2.81</v>
+        <v>0</v>
       </c>
       <c r="BJ64" t="n">
-        <v>80.89</v>
+        <v>76.64</v>
       </c>
       <c r="BK64" t="n">
         <v>4.74</v>
@@ -15232,7 +15232,7 @@
         <v>1.57</v>
       </c>
       <c r="BM64" t="n">
-        <v>82.5</v>
+        <v>78.76000000000001</v>
       </c>
       <c r="BN64" t="n">
         <v>84.59</v>
@@ -15241,19 +15241,19 @@
         <v>44.12</v>
       </c>
       <c r="BP64" t="n">
-        <v>76.70999999999999</v>
+        <v>76.56999999999999</v>
       </c>
       <c r="BQ64" t="n">
-        <v>50.07</v>
+        <v>48.81</v>
       </c>
       <c r="BR64" t="n">
-        <v>81.26000000000001</v>
+        <v>78.76000000000001</v>
       </c>
       <c r="BS64" t="n">
         <v>3.49</v>
       </c>
       <c r="BT64" t="n">
-        <v>12347880</v>
+        <v>12971537</v>
       </c>
     </row>
     <row r="65">
@@ -15283,13 +15283,13 @@
         </is>
       </c>
       <c r="F65" t="n">
-        <v>27</v>
+        <v>26.5</v>
       </c>
       <c r="G65" t="n">
-        <v>227765685856</v>
+        <v>267448153390</v>
       </c>
       <c r="H65" t="n">
-        <v>41100</v>
+        <v>29700</v>
       </c>
       <c r="I65" t="n">
         <v>7298813414</v>
@@ -15304,7 +15304,7 @@
         <v>3.29</v>
       </c>
       <c r="M65" t="n">
-        <v>5.506450211712123</v>
+        <v>6.465811280227078</v>
       </c>
       <c r="N65" t="n">
         <v>0.29</v>
@@ -15382,7 +15382,7 @@
         <v>11532125194.12</v>
       </c>
       <c r="AM65" t="n">
-        <v>17061100064.11985</v>
+        <v>20033569542.3221</v>
       </c>
       <c r="AN65" t="n">
         <v>0.4734</v>
@@ -15423,7 +15423,7 @@
         <v>12.99</v>
       </c>
       <c r="AZ65" t="n">
-        <v>9.09</v>
+        <v>8.92</v>
       </c>
       <c r="BA65" t="n">
         <v>2.23</v>
@@ -15432,19 +15432,19 @@
         <v>3.47</v>
       </c>
       <c r="BC65" t="n">
-        <v>-41.08</v>
+        <v>-39.96</v>
       </c>
       <c r="BD65" t="n">
-        <v>-51.89</v>
+        <v>-50.98</v>
       </c>
       <c r="BE65" t="n">
         <v>-66.33</v>
       </c>
       <c r="BF65" t="n">
-        <v>-91.73999999999999</v>
+        <v>-91.58</v>
       </c>
       <c r="BG65" t="n">
-        <v>-87.16</v>
+        <v>-86.92</v>
       </c>
       <c r="BH65" t="n">
         <v>7.12</v>
@@ -15453,7 +15453,7 @@
         <v>0</v>
       </c>
       <c r="BJ65" t="n">
-        <v>27</v>
+        <v>26.5</v>
       </c>
       <c r="BK65" t="n">
         <v>1.58</v>
@@ -15462,7 +15462,7 @@
         <v>1.57</v>
       </c>
       <c r="BM65" t="n">
-        <v>28.72</v>
+        <v>27</v>
       </c>
       <c r="BN65" t="n">
         <v>46.43</v>
@@ -15471,19 +15471,19 @@
         <v>20.44</v>
       </c>
       <c r="BP65" t="n">
-        <v>26.13</v>
+        <v>26.5</v>
       </c>
       <c r="BQ65" t="n">
-        <v>17.2</v>
+        <v>16.88</v>
       </c>
       <c r="BR65" t="n">
-        <v>27.99</v>
+        <v>27</v>
       </c>
       <c r="BS65" t="n">
         <v>4.14</v>
       </c>
       <c r="BT65" t="n">
-        <v>9137</v>
+        <v>10330</v>
       </c>
     </row>
     <row r="66">
@@ -15513,13 +15513,13 @@
         </is>
       </c>
       <c r="F66" t="n">
-        <v>25.99</v>
+        <v>25.5</v>
       </c>
       <c r="G66" t="n">
-        <v>227765685856</v>
+        <v>267448153390</v>
       </c>
       <c r="H66" t="n">
-        <v>17200</v>
+        <v>3700</v>
       </c>
       <c r="I66" t="n">
         <v>2972355254</v>
@@ -15534,7 +15534,7 @@
         <v>2.75</v>
       </c>
       <c r="M66" t="n">
-        <v>13.5214499056537</v>
+        <v>15.87722397617345</v>
       </c>
       <c r="N66" t="n">
         <v>0.25</v>
@@ -15612,7 +15612,7 @@
         <v>4696321301.320001</v>
       </c>
       <c r="AM66" t="n">
-        <v>20427415771.83857</v>
+        <v>23986381469.95515</v>
       </c>
       <c r="AN66" t="n">
         <v>0.4734</v>
@@ -15653,7 +15653,7 @@
         <v>12.99</v>
       </c>
       <c r="AZ66" t="n">
-        <v>10.44</v>
+        <v>10.24</v>
       </c>
       <c r="BA66" t="n">
         <v>2.23</v>
@@ -15662,19 +15662,19 @@
         <v>3.47</v>
       </c>
       <c r="BC66" t="n">
-        <v>-38.79</v>
+        <v>-37.61</v>
       </c>
       <c r="BD66" t="n">
-        <v>-50.02</v>
+        <v>-49.06</v>
       </c>
       <c r="BE66" t="n">
         <v>-59.83</v>
       </c>
       <c r="BF66" t="n">
-        <v>-91.41</v>
+        <v>-91.25</v>
       </c>
       <c r="BG66" t="n">
-        <v>-86.67</v>
+        <v>-86.41</v>
       </c>
       <c r="BH66" t="n">
         <v>7.12</v>
@@ -15683,7 +15683,7 @@
         <v>0</v>
       </c>
       <c r="BJ66" t="n">
-        <v>25.99</v>
+        <v>25.5</v>
       </c>
       <c r="BK66" t="n">
         <v>1.58</v>
@@ -15692,7 +15692,7 @@
         <v>1.57</v>
       </c>
       <c r="BM66" t="n">
-        <v>27.2</v>
+        <v>26</v>
       </c>
       <c r="BN66" t="n">
         <v>28.51</v>
@@ -15701,10 +15701,10 @@
         <v>9.48</v>
       </c>
       <c r="BP66" t="n">
-        <v>25.34</v>
+        <v>25.5</v>
       </c>
       <c r="BQ66" t="n">
-        <v>16.55</v>
+        <v>16.24</v>
       </c>
       <c r="BR66" t="n">
         <v>25.52</v>
@@ -15713,7 +15713,7 @@
         <v>3.46</v>
       </c>
       <c r="BT66" t="n">
-        <v>4520</v>
+        <v>5077</v>
       </c>
     </row>
     <row r="67">
@@ -15973,13 +15973,13 @@
         </is>
       </c>
       <c r="F68" t="n">
-        <v>18.46</v>
+        <v>18.63</v>
       </c>
       <c r="G68" t="n">
-        <v>7503797078</v>
+        <v>7888573519</v>
       </c>
       <c r="H68" t="n">
-        <v>74600</v>
+        <v>83000</v>
       </c>
       <c r="I68" t="n">
         <v>137989898</v>
@@ -16072,7 +16072,7 @@
         <v>205604948.02</v>
       </c>
       <c r="AM68" t="n">
-        <v>520374277.2538142</v>
+        <v>547057802.9819695</v>
       </c>
       <c r="AN68" t="n">
         <v>0.1911</v>
@@ -16113,7 +16113,7 @@
         <v>21.39</v>
       </c>
       <c r="AZ68" t="n">
-        <v>34.15</v>
+        <v>34.47</v>
       </c>
       <c r="BA68" t="n">
         <v>1.24</v>
@@ -16122,19 +16122,19 @@
         <v>63.25</v>
       </c>
       <c r="BC68" t="n">
-        <v>41.94</v>
+        <v>40.65</v>
       </c>
       <c r="BD68" t="n">
-        <v>15.9</v>
+        <v>14.84</v>
       </c>
       <c r="BE68" t="n">
         <v>85</v>
       </c>
       <c r="BF68" t="n">
-        <v>-93.29000000000001</v>
+        <v>-93.34999999999999</v>
       </c>
       <c r="BG68" t="n">
-        <v>242.63</v>
+        <v>239.5</v>
       </c>
       <c r="BH68" t="n">
         <v>20.48</v>
@@ -16143,7 +16143,7 @@
         <v>0</v>
       </c>
       <c r="BJ68" t="n">
-        <v>18.46</v>
+        <v>18.63</v>
       </c>
       <c r="BK68" t="n">
         <v>1.49</v>
@@ -16152,28 +16152,28 @@
         <v>1.49</v>
       </c>
       <c r="BM68" t="n">
-        <v>18.8</v>
+        <v>18.63</v>
       </c>
       <c r="BN68" t="n">
         <v>22.11</v>
       </c>
       <c r="BO68" t="n">
-        <v>15.45</v>
+        <v>15.51</v>
       </c>
       <c r="BP68" t="n">
-        <v>18.2</v>
+        <v>18.27</v>
       </c>
       <c r="BQ68" t="n">
-        <v>12.42</v>
+        <v>12.53</v>
       </c>
       <c r="BR68" t="n">
-        <v>18.4</v>
+        <v>18.45</v>
       </c>
       <c r="BS68" t="n">
         <v>0</v>
       </c>
       <c r="BT68" t="n">
-        <v>51903</v>
+        <v>53610</v>
       </c>
     </row>
     <row r="69">
@@ -16203,13 +16203,13 @@
         </is>
       </c>
       <c r="F69" t="n">
-        <v>21.29</v>
+        <v>21.05</v>
       </c>
       <c r="G69" t="n">
-        <v>7503797078</v>
+        <v>7888573519</v>
       </c>
       <c r="H69" t="n">
-        <v>0</v>
+        <v>3855000</v>
       </c>
       <c r="I69" t="n">
         <v>255106712</v>
@@ -16302,7 +16302,7 @@
         <v>380109000.88</v>
       </c>
       <c r="AM69" t="n">
-        <v>446654587.9761904</v>
+        <v>469557947.5595238</v>
       </c>
       <c r="AN69" t="n">
         <v>0.8856000000000001</v>
@@ -16343,7 +16343,7 @@
         <v>21.39</v>
       </c>
       <c r="AZ69" t="n">
-        <v>37.22</v>
+        <v>36.8</v>
       </c>
       <c r="BA69" t="n">
         <v>1.24</v>
@@ -16352,19 +16352,19 @@
         <v>69.59</v>
       </c>
       <c r="BC69" t="n">
-        <v>23.08</v>
+        <v>24.48</v>
       </c>
       <c r="BD69" t="n">
-        <v>0.49</v>
+        <v>1.64</v>
       </c>
       <c r="BE69" t="n">
         <v>74.83</v>
       </c>
       <c r="BF69" t="n">
-        <v>-94.18000000000001</v>
+        <v>-94.11</v>
       </c>
       <c r="BG69" t="n">
-        <v>226.85</v>
+        <v>230.58</v>
       </c>
       <c r="BH69" t="n">
         <v>20.48</v>
@@ -16373,7 +16373,7 @@
         <v>0</v>
       </c>
       <c r="BJ69" t="n">
-        <v>21.29</v>
+        <v>21.05</v>
       </c>
       <c r="BK69" t="n">
         <v>1.49</v>
@@ -16382,7 +16382,7 @@
         <v>1.49</v>
       </c>
       <c r="BM69" t="n">
-        <v>21.43</v>
+        <v>21.26</v>
       </c>
       <c r="BN69" t="n">
         <v>25.63</v>
@@ -16391,19 +16391,19 @@
         <v>16.99</v>
       </c>
       <c r="BP69" t="n">
-        <v>20.78</v>
+        <v>20.7</v>
       </c>
       <c r="BQ69" t="n">
-        <v>14.32</v>
+        <v>14.16</v>
       </c>
       <c r="BR69" t="n">
-        <v>21.42</v>
+        <v>21.26</v>
       </c>
       <c r="BS69" t="n">
         <v>0</v>
       </c>
       <c r="BT69" t="n">
-        <v>2495197</v>
+        <v>2612180</v>
       </c>
     </row>
     <row r="70">
@@ -16433,13 +16433,13 @@
         </is>
       </c>
       <c r="F70" t="n">
-        <v>19.25</v>
+        <v>19.89</v>
       </c>
       <c r="G70" t="n">
-        <v>8475480475</v>
+        <v>9240042424</v>
       </c>
       <c r="H70" t="n">
-        <v>0</v>
+        <v>4890000</v>
       </c>
       <c r="I70" t="n">
         <v>464557268</v>
@@ -16454,7 +16454,7 @@
         <v>0.68</v>
       </c>
       <c r="M70" t="n">
-        <v>0.6689543761839642</v>
+        <v>0.7292998708324303</v>
       </c>
       <c r="N70" t="n">
         <v>0.2</v>
@@ -16532,7 +16532,7 @@
         <v>55746872.16</v>
       </c>
       <c r="AM70" t="n">
-        <v>2797188275.577558</v>
+        <v>3049518951.815182</v>
       </c>
       <c r="AN70" t="n">
         <v>0.1236</v>
@@ -16573,7 +16573,7 @@
         <v>6.9</v>
       </c>
       <c r="AZ70" t="n">
-        <v>2.21</v>
+        <v>2.29</v>
       </c>
       <c r="BA70" t="n">
         <v>0.12</v>
@@ -16582,28 +16582,28 @@
         <v>1.07</v>
       </c>
       <c r="BC70" t="n">
-        <v>-56.11</v>
+        <v>-57.52</v>
       </c>
       <c r="BD70" t="n">
-        <v>-64.16</v>
+        <v>-65.31999999999999</v>
       </c>
       <c r="BE70" t="n">
         <v>-88.5</v>
       </c>
       <c r="BF70" t="n">
-        <v>-99.38</v>
+        <v>-99.40000000000001</v>
       </c>
       <c r="BG70" t="n">
-        <v>-94.44</v>
+        <v>-94.62</v>
       </c>
       <c r="BH70" t="n">
         <v>26.44</v>
       </c>
       <c r="BI70" t="n">
-        <v>0.79</v>
+        <v>0</v>
       </c>
       <c r="BJ70" t="n">
-        <v>19.1</v>
+        <v>19.89</v>
       </c>
       <c r="BK70" t="n">
         <v>0.12</v>
@@ -16612,7 +16612,7 @@
         <v>0.1</v>
       </c>
       <c r="BM70" t="n">
-        <v>19.51</v>
+        <v>19.99</v>
       </c>
       <c r="BN70" t="n">
         <v>22.15</v>
@@ -16621,19 +16621,19 @@
         <v>13.21</v>
       </c>
       <c r="BP70" t="n">
-        <v>18.9</v>
+        <v>19.4</v>
       </c>
       <c r="BQ70" t="n">
-        <v>193.06</v>
+        <v>199.48</v>
       </c>
       <c r="BR70" t="n">
-        <v>19</v>
+        <v>19.44</v>
       </c>
       <c r="BS70" t="n">
         <v>0.67</v>
       </c>
       <c r="BT70" t="n">
-        <v>3709903</v>
+        <v>3669280</v>
       </c>
     </row>
     <row r="71">

</xml_diff>

<commit_message>
📊 Dados atualizados - 2026-10-12 06:50
</commit_message>
<xml_diff>
--- a/data/ativos.xlsx
+++ b/data/ativos.xlsx
@@ -2430,7 +2430,7 @@
         <v>23</v>
       </c>
       <c r="G9" t="n">
-        <v>200993895</v>
+        <v>195992400</v>
       </c>
       <c r="H9" t="n">
         <v>200</v>
@@ -2448,7 +2448,7 @@
         <v>0.68</v>
       </c>
       <c r="M9" t="n">
-        <v>0.4028958973501266</v>
+        <v>0.392870310174371</v>
       </c>
       <c r="N9" t="n">
         <v>0.36</v>
@@ -2526,7 +2526,7 @@
         <v>49438316.76</v>
       </c>
       <c r="AM9" t="n">
-        <v>59998177.61194029</v>
+        <v>58505194.02985074</v>
       </c>
       <c r="AN9" t="n">
         <v>0</v>
@@ -8858,7 +8858,7 @@
         <v>15.93</v>
       </c>
       <c r="G37" t="n">
-        <v>196488270</v>
+        <v>185857000</v>
       </c>
       <c r="H37" t="n">
         <v>200</v>
@@ -8876,7 +8876,7 @@
         <v>0.88</v>
       </c>
       <c r="M37" t="n">
-        <v>1.912978827988338</v>
+        <v>1.809474458874459</v>
       </c>
       <c r="N37" t="n">
         <v>0.5</v>
@@ -8954,7 +8954,7 @@
         <v>11319000</v>
       </c>
       <c r="AM37" t="n">
-        <v>47006763.15789474</v>
+        <v>44463397.12918661</v>
       </c>
       <c r="AN37" t="n">
         <v>0</v>
@@ -9784,7 +9784,7 @@
         <v>24469000</v>
       </c>
       <c r="I41" t="n">
-        <v>5303870781</v>
+        <v>5606747177</v>
       </c>
       <c r="J41" t="n">
         <v>8.98</v>
@@ -9796,7 +9796,7 @@
         <v>0.92</v>
       </c>
       <c r="M41" t="n">
-        <v>1.516347572867865</v>
+        <v>1.434434500375928</v>
       </c>
       <c r="N41" t="n">
         <v>0.07000000000000001</v>
@@ -9868,10 +9868,10 @@
         <v>8.93</v>
       </c>
       <c r="AK41" t="n">
-        <v>150060734291.7073</v>
+        <v>158629920129.7561</v>
       </c>
       <c r="AL41" t="n">
-        <v>12304980211.92</v>
+        <v>13007653450.64</v>
       </c>
       <c r="AM41" t="n">
         <v>35060744256.70262</v>
@@ -10014,7 +10014,7 @@
         <v>77677000</v>
       </c>
       <c r="I42" t="n">
-        <v>5288141247</v>
+        <v>5590117604</v>
       </c>
       <c r="J42" t="n">
         <v>8.69</v>
@@ -10026,7 +10026,7 @@
         <v>1.05</v>
       </c>
       <c r="M42" t="n">
-        <v>1.520857936640159</v>
+        <v>1.43870167951732</v>
       </c>
       <c r="N42" t="n">
         <v>0.08</v>
@@ -10098,10 +10098,10 @@
         <v>8.93</v>
       </c>
       <c r="AK42" t="n">
-        <v>149615703573.6585</v>
+        <v>158159424893.6585</v>
       </c>
       <c r="AL42" t="n">
-        <v>12268487693.04</v>
+        <v>12969072841.28</v>
       </c>
       <c r="AM42" t="n">
         <v>30958398670.20408</v>
@@ -11158,7 +11158,7 @@
         <v>9.66</v>
       </c>
       <c r="G47" t="n">
-        <v>3352181269</v>
+        <v>3346616000</v>
       </c>
       <c r="H47" t="n">
         <v>13600</v>
@@ -11176,7 +11176,7 @@
         <v>1.22</v>
       </c>
       <c r="M47" t="n">
-        <v>0.7904829109475172</v>
+        <v>0.7891705564874499</v>
       </c>
       <c r="N47" t="n">
         <v>0.07000000000000001</v>
@@ -11254,7 +11254,7 @@
         <v>322715382</v>
       </c>
       <c r="AM47" t="n">
-        <v>594358381.0283688</v>
+        <v>593371631.2056738</v>
       </c>
       <c r="AN47" t="n">
         <v>0.4132</v>
@@ -11388,7 +11388,7 @@
         <v>9.550000000000001</v>
       </c>
       <c r="G48" t="n">
-        <v>3352181269</v>
+        <v>3346616000</v>
       </c>
       <c r="H48" t="n">
         <v>4700</v>
@@ -11406,7 +11406,7 @@
         <v>1.24</v>
       </c>
       <c r="M48" t="n">
-        <v>2.150665980656241</v>
+        <v>2.147095459329669</v>
       </c>
       <c r="N48" t="n">
         <v>0.07000000000000001</v>
@@ -11484,7 +11484,7 @@
         <v>118614883.42</v>
       </c>
       <c r="AM48" t="n">
-        <v>586045676.3986014</v>
+        <v>585072727.2727273</v>
       </c>
       <c r="AN48" t="n">
         <v>0.4132</v>
@@ -11618,7 +11618,7 @@
         <v>48.74</v>
       </c>
       <c r="G49" t="n">
-        <v>985490178</v>
+        <v>979589100</v>
       </c>
       <c r="H49" t="n">
         <v>100</v>
@@ -11636,7 +11636,7 @@
         <v>1.09</v>
       </c>
       <c r="M49" t="n">
-        <v>0.9970077017130135</v>
+        <v>0.9910376572156149</v>
       </c>
       <c r="N49" t="n">
         <v>0.08</v>
@@ -11714,7 +11714,7 @@
         <v>84709985.8</v>
       </c>
       <c r="AM49" t="n">
-        <v>246372544.5</v>
+        <v>244897275</v>
       </c>
       <c r="AN49" t="n">
         <v>3.3186</v>
@@ -11848,7 +11848,7 @@
         <v>36.14</v>
       </c>
       <c r="G50" t="n">
-        <v>985490178</v>
+        <v>979589100</v>
       </c>
       <c r="H50" t="n">
         <v>800</v>
@@ -11866,7 +11866,7 @@
         <v>0.8</v>
       </c>
       <c r="M50" t="n">
-        <v>0.9970077017130135</v>
+        <v>0.9910376572156149</v>
       </c>
       <c r="N50" t="n">
         <v>0.06</v>
@@ -11944,7 +11944,7 @@
         <v>84709985.8</v>
       </c>
       <c r="AM50" t="n">
-        <v>336344770.6484641</v>
+        <v>334330750.8532423</v>
       </c>
       <c r="AN50" t="n">
         <v>4.4983</v>
@@ -14136,7 +14136,7 @@
         <v>414.99</v>
       </c>
       <c r="G60" t="n">
-        <v>188716698</v>
+        <v>188716700</v>
       </c>
       <c r="H60" t="n">
         <v>511</v>
@@ -14154,7 +14154,7 @@
         <v>0.83</v>
       </c>
       <c r="M60" t="n">
-        <v>14.11574335280085</v>
+        <v>14.11574350239804</v>
       </c>
       <c r="N60" t="n">
         <v>0.68</v>
@@ -14232,7 +14232,7 @@
         <v>59558607.5</v>
       </c>
       <c r="AM60" t="n">
-        <v>-27671070.08797654</v>
+        <v>-27671070.38123167</v>
       </c>
       <c r="AN60" t="n">
         <v>10.0581</v>
@@ -14596,7 +14596,7 @@
         <v>115.24</v>
       </c>
       <c r="G62" t="n">
-        <v>11374162436</v>
+        <v>11374160000</v>
       </c>
       <c r="H62" t="n">
         <v>200</v>
@@ -14614,7 +14614,7 @@
         <v>0.64</v>
       </c>
       <c r="M62" t="n">
-        <v>1.066197165471367</v>
+        <v>1.06619693712433</v>
       </c>
       <c r="N62" t="n">
         <v>0.13</v>
@@ -14692,7 +14692,7 @@
         <v>2757670987.06</v>
       </c>
       <c r="AM62" t="n">
-        <v>4604924063.157894</v>
+        <v>4604923076.923077</v>
       </c>
       <c r="AN62" t="n">
         <v>6.9319</v>
@@ -14826,7 +14826,7 @@
         <v>1.65</v>
       </c>
       <c r="G63" t="n">
-        <v>429840998</v>
+        <v>429841100</v>
       </c>
       <c r="H63" t="n">
         <v>36400</v>
@@ -14844,7 +14844,7 @@
         <v>-0.22</v>
       </c>
       <c r="M63" t="n">
-        <v>0.528682245114574</v>
+        <v>0.5286823705693101</v>
       </c>
       <c r="N63" t="n">
         <v>0.37</v>
@@ -14922,7 +14922,7 @@
         <v>31952560.12</v>
       </c>
       <c r="AM63" t="n">
-        <v>244227839.7727273</v>
+        <v>244227897.7272727</v>
       </c>
       <c r="AN63" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
📊 Dados atualizados - 2026-10-13 07:16
</commit_message>
<xml_diff>
--- a/data/ativos.xlsx
+++ b/data/ativos.xlsx
@@ -1280,7 +1280,7 @@
         <v>15.99</v>
       </c>
       <c r="G4" t="n">
-        <v>247599709855</v>
+        <v>50272592396</v>
       </c>
       <c r="H4" t="n">
         <v>41224400</v>
@@ -1298,7 +1298,7 @@
         <v>2.76</v>
       </c>
       <c r="M4" t="n">
-        <v>2.803579074680699</v>
+        <v>0.5692380986791833</v>
       </c>
       <c r="N4" t="n">
         <v>1.76</v>
@@ -1376,7 +1376,7 @@
         <v>16258898133.45</v>
       </c>
       <c r="AM4" t="n">
-        <v>24514822757.92079</v>
+        <v>4977484395.643564</v>
       </c>
       <c r="AN4" t="n">
         <v>0.269</v>
@@ -6340,7 +6340,7 @@
         <v>13.27</v>
       </c>
       <c r="G26" t="n">
-        <v>17972795729</v>
+        <v>3622941765</v>
       </c>
       <c r="H26" t="n">
         <v>27967800</v>
@@ -6358,7 +6358,7 @@
         <v>1.94</v>
       </c>
       <c r="M26" t="n">
-        <v>0.231757685843498</v>
+        <v>0.04671752865066785</v>
       </c>
       <c r="N26" t="n">
         <v>0.26</v>
@@ -6436,7 +6436,7 @@
         <v>961619314.7099999</v>
       </c>
       <c r="AM26" t="n">
-        <v>6418855617.5</v>
+        <v>1293907773.214286</v>
       </c>
       <c r="AN26" t="n">
         <v>0.1043</v>
@@ -9778,7 +9778,7 @@
         <v>19.02</v>
       </c>
       <c r="G41" t="n">
-        <v>227544230226</v>
+        <v>45395907825</v>
       </c>
       <c r="H41" t="n">
         <v>24469000</v>
@@ -9796,7 +9796,7 @@
         <v>0.92</v>
       </c>
       <c r="M41" t="n">
-        <v>1.434434500375928</v>
+        <v>0.2861749396826718</v>
       </c>
       <c r="N41" t="n">
         <v>0.07000000000000001</v>
@@ -9874,7 +9874,7 @@
         <v>13007653450.64</v>
       </c>
       <c r="AM41" t="n">
-        <v>35060744256.70262</v>
+        <v>6994746968.412943</v>
       </c>
       <c r="AN41" t="n">
         <v>1.6841</v>
@@ -10008,7 +10008,7 @@
         <v>21.61</v>
       </c>
       <c r="G42" t="n">
-        <v>227544230226</v>
+        <v>45395907825</v>
       </c>
       <c r="H42" t="n">
         <v>77677000</v>
@@ -10026,7 +10026,7 @@
         <v>1.05</v>
       </c>
       <c r="M42" t="n">
-        <v>1.43870167951732</v>
+        <v>0.2870262575595656</v>
       </c>
       <c r="N42" t="n">
         <v>0.08</v>
@@ -10104,7 +10104,7 @@
         <v>12969072841.28</v>
       </c>
       <c r="AM42" t="n">
-        <v>30958398670.20408</v>
+        <v>6176313989.795918</v>
       </c>
       <c r="AN42" t="n">
         <v>1.8491</v>

</xml_diff>

<commit_message>
📊 Dados atualizados - 2026-10-14 05:40
</commit_message>
<xml_diff>
--- a/data/ativos.xlsx
+++ b/data/ativos.xlsx
@@ -1047,13 +1047,13 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>29.56</v>
+        <v>29.15</v>
       </c>
       <c r="G3" t="n">
-        <v>3954146536</v>
+        <v>3899302168</v>
       </c>
       <c r="H3" t="n">
-        <v>1055800</v>
+        <v>791200</v>
       </c>
       <c r="I3" t="n">
         <v>129510368</v>
@@ -1068,7 +1068,7 @@
         <v>0.88</v>
       </c>
       <c r="M3" t="n">
-        <v>0.9838797226278327</v>
+        <v>0.970233222407301</v>
       </c>
       <c r="N3" t="n">
         <v>0.09</v>
@@ -1146,7 +1146,7 @@
         <v>506385538.88</v>
       </c>
       <c r="AM3" t="n">
-        <v>772294245.3125</v>
+        <v>761582454.6875</v>
       </c>
       <c r="AN3" t="n">
         <v>2.7</v>
@@ -1187,7 +1187,7 @@
         <v>40.42</v>
       </c>
       <c r="AZ3" t="n">
-        <v>54.09</v>
+        <v>53.34</v>
       </c>
       <c r="BA3" t="n">
         <v>4.87</v>
@@ -1196,19 +1196,19 @@
         <v>21.14</v>
       </c>
       <c r="BC3" t="n">
-        <v>67.45</v>
+        <v>69.81</v>
       </c>
       <c r="BD3" t="n">
-        <v>36.72</v>
+        <v>38.65</v>
       </c>
       <c r="BE3" t="n">
         <v>83</v>
       </c>
       <c r="BF3" t="n">
-        <v>-83.53</v>
+        <v>-83.3</v>
       </c>
       <c r="BG3" t="n">
-        <v>-28.5</v>
+        <v>-27.49</v>
       </c>
       <c r="BH3" t="n">
         <v>27.85</v>
@@ -1217,7 +1217,7 @@
         <v>0</v>
       </c>
       <c r="BJ3" t="n">
-        <v>29.56</v>
+        <v>29.15</v>
       </c>
       <c r="BK3" t="n">
         <v>3.91</v>
@@ -1226,7 +1226,7 @@
         <v>4.39</v>
       </c>
       <c r="BM3" t="n">
-        <v>29.56</v>
+        <v>29.44</v>
       </c>
       <c r="BN3" t="n">
         <v>29.56</v>
@@ -1235,19 +1235,19 @@
         <v>18.72</v>
       </c>
       <c r="BP3" t="n">
-        <v>28.68</v>
+        <v>28.79</v>
       </c>
       <c r="BQ3" t="n">
-        <v>6.73</v>
+        <v>6.64</v>
       </c>
       <c r="BR3" t="n">
-        <v>28.77</v>
+        <v>29.37</v>
       </c>
       <c r="BS3" t="n">
         <v>0.79</v>
       </c>
       <c r="BT3" t="n">
-        <v>678733</v>
+        <v>701093</v>
       </c>
     </row>
     <row r="4">
@@ -1277,13 +1277,13 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>15.99</v>
+        <v>16.32</v>
       </c>
       <c r="G4" t="n">
-        <v>50272592396</v>
+        <v>252709646474</v>
       </c>
       <c r="H4" t="n">
-        <v>41224400</v>
+        <v>56978500</v>
       </c>
       <c r="I4" t="n">
         <v>15484664889</v>
@@ -1298,7 +1298,7 @@
         <v>2.76</v>
       </c>
       <c r="M4" t="n">
-        <v>0.5692380986791833</v>
+        <v>2.861439043039963</v>
       </c>
       <c r="N4" t="n">
         <v>1.76</v>
@@ -1376,7 +1376,7 @@
         <v>16258898133.45</v>
       </c>
       <c r="AM4" t="n">
-        <v>4977484395.643564</v>
+        <v>25020757076.63366</v>
       </c>
       <c r="AN4" t="n">
         <v>0.269</v>
@@ -1417,7 +1417,7 @@
         <v>9.470000000000001</v>
       </c>
       <c r="AZ4" t="n">
-        <v>19.96</v>
+        <v>20.37</v>
       </c>
       <c r="BA4" t="n">
         <v>1.13</v>
@@ -1426,19 +1426,19 @@
         <v>11.39</v>
       </c>
       <c r="BC4" t="n">
-        <v>-27.43</v>
+        <v>-28.89</v>
       </c>
       <c r="BD4" t="n">
-        <v>-40.74</v>
+        <v>-41.94</v>
       </c>
       <c r="BE4" t="n">
         <v>24.83</v>
       </c>
       <c r="BF4" t="n">
-        <v>-92.95</v>
+        <v>-93.09</v>
       </c>
       <c r="BG4" t="n">
-        <v>-28.79</v>
+        <v>-30.23</v>
       </c>
       <c r="BH4" t="n">
         <v>5.7</v>
@@ -1447,7 +1447,7 @@
         <v>0</v>
       </c>
       <c r="BJ4" t="n">
-        <v>15.99</v>
+        <v>16.32</v>
       </c>
       <c r="BK4" t="n">
         <v>1.05</v>
@@ -1456,28 +1456,28 @@
         <v>1.04</v>
       </c>
       <c r="BM4" t="n">
-        <v>16.24</v>
+        <v>16.32</v>
       </c>
       <c r="BN4" t="n">
         <v>16.94</v>
       </c>
       <c r="BO4" t="n">
-        <v>11.04</v>
+        <v>11.11</v>
       </c>
       <c r="BP4" t="n">
         <v>15.88</v>
       </c>
       <c r="BQ4" t="n">
-        <v>15.42</v>
+        <v>15.74</v>
       </c>
       <c r="BR4" t="n">
-        <v>16.21</v>
+        <v>16</v>
       </c>
       <c r="BS4" t="n">
         <v>2.76</v>
       </c>
       <c r="BT4" t="n">
-        <v>30775123</v>
+        <v>31361613</v>
       </c>
     </row>
     <row r="5">
@@ -1737,13 +1737,13 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>7</v>
+        <v>7.07</v>
       </c>
       <c r="G6" t="n">
-        <v>441592900</v>
+        <v>446008839</v>
       </c>
       <c r="H6" t="n">
-        <v>4200</v>
+        <v>1100</v>
       </c>
       <c r="I6" t="n">
         <v>63084700</v>
@@ -1758,7 +1758,7 @@
         <v>1.91</v>
       </c>
       <c r="M6" t="n">
-        <v>6.874736842105262</v>
+        <v>6.943484366206736</v>
       </c>
       <c r="N6" t="n">
         <v>1.26</v>
@@ -1836,7 +1836,7 @@
         <v>35958279</v>
       </c>
       <c r="AM6" t="n">
-        <v>42217294.45506692</v>
+        <v>42639468.35564053</v>
       </c>
       <c r="AN6" t="n">
         <v>0.5199</v>
@@ -1877,7 +1877,7 @@
         <v>5.74</v>
       </c>
       <c r="AZ6" t="n">
-        <v>8.210000000000001</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="BA6" t="n">
         <v>0.65</v>
@@ -1886,19 +1886,19 @@
         <v>7.95</v>
       </c>
       <c r="BC6" t="n">
-        <v>0.51</v>
+        <v>-0.48</v>
       </c>
       <c r="BD6" t="n">
-        <v>-17.93</v>
+        <v>-18.74</v>
       </c>
       <c r="BE6" t="n">
         <v>17.33</v>
       </c>
       <c r="BF6" t="n">
-        <v>-90.73999999999999</v>
+        <v>-90.83</v>
       </c>
       <c r="BG6" t="n">
-        <v>13.62</v>
+        <v>12.5</v>
       </c>
       <c r="BH6" t="n">
         <v>3.86</v>
@@ -1907,7 +1907,7 @@
         <v>0</v>
       </c>
       <c r="BJ6" t="n">
-        <v>7</v>
+        <v>7.07</v>
       </c>
       <c r="BK6" t="n">
         <v>0.57</v>
@@ -1916,7 +1916,7 @@
         <v>0.5600000000000001</v>
       </c>
       <c r="BM6" t="n">
-        <v>7.21</v>
+        <v>7.08</v>
       </c>
       <c r="BN6" t="n">
         <v>8.16</v>
@@ -1925,19 +1925,19 @@
         <v>6.22</v>
       </c>
       <c r="BP6" t="n">
-        <v>7</v>
+        <v>7.03</v>
       </c>
       <c r="BQ6" t="n">
-        <v>12.45</v>
+        <v>12.57</v>
       </c>
       <c r="BR6" t="n">
-        <v>7.1</v>
+        <v>7.03</v>
       </c>
       <c r="BS6" t="n">
         <v>7.32</v>
       </c>
       <c r="BT6" t="n">
-        <v>507</v>
+        <v>647</v>
       </c>
     </row>
     <row r="7">
@@ -2433,7 +2433,7 @@
         <v>195992400</v>
       </c>
       <c r="H9" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="I9" t="n">
         <v>8407877</v>
@@ -3117,13 +3117,13 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>6.22</v>
+        <v>6.5</v>
       </c>
       <c r="G12" t="n">
-        <v>596880758</v>
+        <v>623749880</v>
       </c>
       <c r="H12" t="n">
-        <v>16099900</v>
+        <v>2954700</v>
       </c>
       <c r="I12" t="n">
         <v>95961536</v>
@@ -3138,7 +3138,7 @@
         <v>0.32</v>
       </c>
       <c r="M12" t="n">
-        <v>0.1079449742828353</v>
+        <v>0.1128042139959915</v>
       </c>
       <c r="N12" t="n">
         <v>0.14</v>
@@ -3216,7 +3216,7 @@
         <v>362734606.08</v>
       </c>
       <c r="AM12" t="n">
-        <v>641807266.6666666</v>
+        <v>670698795.6989247</v>
       </c>
       <c r="AN12" t="n">
         <v>0.4208</v>
@@ -3257,7 +3257,7 @@
         <v>30.49</v>
       </c>
       <c r="AZ12" t="n">
-        <v>8.41</v>
+        <v>8.789999999999999</v>
       </c>
       <c r="BA12" t="n">
         <v>4.41</v>
@@ -3266,19 +3266,19 @@
         <v>18.12</v>
       </c>
       <c r="BC12" t="n">
-        <v>500.44</v>
+        <v>474.57</v>
       </c>
       <c r="BD12" t="n">
-        <v>390.26</v>
+        <v>369.14</v>
       </c>
       <c r="BE12" t="n">
         <v>35.17</v>
       </c>
       <c r="BF12" t="n">
-        <v>-29.07</v>
+        <v>-32.13</v>
       </c>
       <c r="BG12" t="n">
-        <v>191.3</v>
+        <v>178.75</v>
       </c>
       <c r="BH12" t="n">
         <v>16.4</v>
@@ -3287,7 +3287,7 @@
         <v>0</v>
       </c>
       <c r="BJ12" t="n">
-        <v>6.22</v>
+        <v>6.5</v>
       </c>
       <c r="BK12" t="n">
         <v>3.78</v>
@@ -3296,7 +3296,7 @@
         <v>3.63</v>
       </c>
       <c r="BM12" t="n">
-        <v>6.39</v>
+        <v>6.62</v>
       </c>
       <c r="BN12" t="n">
         <v>7.3</v>
@@ -3305,19 +3305,19 @@
         <v>3.92</v>
       </c>
       <c r="BP12" t="n">
-        <v>5.48</v>
+        <v>6.25</v>
       </c>
       <c r="BQ12" t="n">
-        <v>1.71</v>
+        <v>1.79</v>
       </c>
       <c r="BR12" t="n">
-        <v>5.5</v>
+        <v>6.5</v>
       </c>
       <c r="BS12" t="n">
         <v>0.09</v>
       </c>
       <c r="BT12" t="n">
-        <v>1123930</v>
+        <v>1637133</v>
       </c>
     </row>
     <row r="13">
@@ -3347,13 +3347,13 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>35.83</v>
+        <v>34.8</v>
       </c>
       <c r="G13" t="n">
-        <v>18065164453</v>
+        <v>17545842935</v>
       </c>
       <c r="H13" t="n">
-        <v>9069000</v>
+        <v>6433900</v>
       </c>
       <c r="I13" t="n">
         <v>504190947</v>
@@ -3368,7 +3368,7 @@
         <v>1.13</v>
       </c>
       <c r="M13" t="n">
-        <v>6.247978273304588</v>
+        <v>6.06836686872727</v>
       </c>
       <c r="N13" t="n">
         <v>0.57</v>
@@ -3446,7 +3446,7 @@
         <v>932753251.95</v>
       </c>
       <c r="AM13" t="n">
-        <v>1879829807.804371</v>
+        <v>1825790107.700312</v>
       </c>
       <c r="AN13" t="n">
         <v>2.6301</v>
@@ -3487,7 +3487,7 @@
         <v>26.6</v>
       </c>
       <c r="AZ13" t="n">
-        <v>64.84999999999999</v>
+        <v>62.99</v>
       </c>
       <c r="BA13" t="n">
         <v>2.6</v>
@@ -3496,19 +3496,19 @@
         <v>8.69</v>
       </c>
       <c r="BC13" t="n">
-        <v>-9.09</v>
+        <v>-6.4</v>
       </c>
       <c r="BD13" t="n">
-        <v>-25.77</v>
+        <v>-23.57</v>
       </c>
       <c r="BE13" t="n">
         <v>81</v>
       </c>
       <c r="BF13" t="n">
-        <v>-92.73</v>
+        <v>-92.52</v>
       </c>
       <c r="BG13" t="n">
-        <v>-75.73999999999999</v>
+        <v>-75.02</v>
       </c>
       <c r="BH13" t="n">
         <v>25.49</v>
@@ -3517,7 +3517,7 @@
         <v>0</v>
       </c>
       <c r="BJ13" t="n">
-        <v>35.83</v>
+        <v>34.8</v>
       </c>
       <c r="BK13" t="n">
         <v>1.85</v>
@@ -3526,7 +3526,7 @@
         <v>1.96</v>
       </c>
       <c r="BM13" t="n">
-        <v>36.1</v>
+        <v>35.6</v>
       </c>
       <c r="BN13" t="n">
         <v>36.1</v>
@@ -3535,19 +3535,19 @@
         <v>20.85</v>
       </c>
       <c r="BP13" t="n">
-        <v>35.27</v>
+        <v>34.64</v>
       </c>
       <c r="BQ13" t="n">
-        <v>18.31</v>
+        <v>17.78</v>
       </c>
       <c r="BR13" t="n">
-        <v>35.4</v>
+        <v>35.6</v>
       </c>
       <c r="BS13" t="n">
         <v>5.01</v>
       </c>
       <c r="BT13" t="n">
-        <v>6608540</v>
+        <v>6800837</v>
       </c>
     </row>
     <row r="14">
@@ -3577,13 +3577,13 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>11.82</v>
+        <v>12.2</v>
       </c>
       <c r="G14" t="n">
-        <v>9851888362</v>
+        <v>10143177540</v>
       </c>
       <c r="H14" t="n">
-        <v>11300</v>
+        <v>19900</v>
       </c>
       <c r="I14" t="n">
         <v>339510689</v>
@@ -3598,7 +3598,7 @@
         <v>1.92</v>
       </c>
       <c r="M14" t="n">
-        <v>4.09067919165656</v>
+        <v>4.211627636809002</v>
       </c>
       <c r="N14" t="n">
         <v>1.11</v>
@@ -3676,7 +3676,7 @@
         <v>349696009.67</v>
       </c>
       <c r="AM14" t="n">
-        <v>1093439329.855716</v>
+        <v>1125768872.36404</v>
       </c>
       <c r="AN14" t="n">
         <v>0.1489</v>
@@ -3717,7 +3717,7 @@
         <v>9.050000000000001</v>
       </c>
       <c r="AZ14" t="n">
-        <v>9.5</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="BA14" t="n">
         <v>1.42</v>
@@ -3726,19 +3726,19 @@
         <v>5.94</v>
       </c>
       <c r="BC14" t="n">
-        <v>-6.24</v>
+        <v>-9.16</v>
       </c>
       <c r="BD14" t="n">
-        <v>-23.44</v>
+        <v>-25.83</v>
       </c>
       <c r="BE14" t="n">
         <v>-19.67</v>
       </c>
       <c r="BF14" t="n">
-        <v>-87.98</v>
+        <v>-88.34999999999999</v>
       </c>
       <c r="BG14" t="n">
-        <v>-49.73</v>
+        <v>-51.29</v>
       </c>
       <c r="BH14" t="n">
         <v>5.3</v>
@@ -3747,7 +3747,7 @@
         <v>0</v>
       </c>
       <c r="BJ14" t="n">
-        <v>11.82</v>
+        <v>12.2</v>
       </c>
       <c r="BK14" t="n">
         <v>1.03</v>
@@ -3756,7 +3756,7 @@
         <v>1.01</v>
       </c>
       <c r="BM14" t="n">
-        <v>12.23</v>
+        <v>12.55</v>
       </c>
       <c r="BN14" t="n">
         <v>13.49</v>
@@ -3765,19 +3765,19 @@
         <v>7.81</v>
       </c>
       <c r="BP14" t="n">
-        <v>11.78</v>
+        <v>11.97</v>
       </c>
       <c r="BQ14" t="n">
-        <v>11.67</v>
+        <v>12.04</v>
       </c>
       <c r="BR14" t="n">
-        <v>11.78</v>
+        <v>11.97</v>
       </c>
       <c r="BS14" t="n">
         <v>1.44</v>
       </c>
       <c r="BT14" t="n">
-        <v>12543</v>
+        <v>12397</v>
       </c>
     </row>
     <row r="15">
@@ -3807,13 +3807,13 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>16.67</v>
+        <v>17.36</v>
       </c>
       <c r="G15" t="n">
-        <v>9851888362</v>
+        <v>10143177540</v>
       </c>
       <c r="H15" t="n">
-        <v>4471100</v>
+        <v>6142200</v>
       </c>
       <c r="I15" t="n">
         <v>343551533</v>
@@ -3828,7 +3828,7 @@
         <v>2.56</v>
       </c>
       <c r="M15" t="n">
-        <v>4.042564731729144</v>
+        <v>4.162090584484354</v>
       </c>
       <c r="N15" t="n">
         <v>1.47</v>
@@ -3906,7 +3906,7 @@
         <v>353858078.99</v>
       </c>
       <c r="AM15" t="n">
-        <v>821675426.355296</v>
+        <v>845969769.8081734</v>
       </c>
       <c r="AN15" t="n">
         <v>0.1638</v>
@@ -3947,7 +3947,7 @@
         <v>9.050000000000001</v>
       </c>
       <c r="AZ15" t="n">
-        <v>11.09</v>
+        <v>11.54</v>
       </c>
       <c r="BA15" t="n">
         <v>1.42</v>
@@ -3956,19 +3956,19 @@
         <v>6.19</v>
       </c>
       <c r="BC15" t="n">
-        <v>-33.52</v>
+        <v>-36.16</v>
       </c>
       <c r="BD15" t="n">
-        <v>-45.72</v>
+        <v>-47.87</v>
       </c>
       <c r="BE15" t="n">
         <v>-33.5</v>
       </c>
       <c r="BF15" t="n">
-        <v>-91.47</v>
+        <v>-91.81</v>
       </c>
       <c r="BG15" t="n">
-        <v>-62.88</v>
+        <v>-64.34999999999999</v>
       </c>
       <c r="BH15" t="n">
         <v>5.3</v>
@@ -3977,7 +3977,7 @@
         <v>0</v>
       </c>
       <c r="BJ15" t="n">
-        <v>16.67</v>
+        <v>17.36</v>
       </c>
       <c r="BK15" t="n">
         <v>1.03</v>
@@ -3986,28 +3986,28 @@
         <v>1.01</v>
       </c>
       <c r="BM15" t="n">
-        <v>16.88</v>
+        <v>17.36</v>
       </c>
       <c r="BN15" t="n">
-        <v>16.88</v>
+        <v>17.36</v>
       </c>
       <c r="BO15" t="n">
-        <v>7.96</v>
+        <v>7.97</v>
       </c>
       <c r="BP15" t="n">
-        <v>15.98</v>
+        <v>16.34</v>
       </c>
       <c r="BQ15" t="n">
-        <v>16.46</v>
+        <v>17.14</v>
       </c>
       <c r="BR15" t="n">
-        <v>16.01</v>
+        <v>16.72</v>
       </c>
       <c r="BS15" t="n">
         <v>1.92</v>
       </c>
       <c r="BT15" t="n">
-        <v>2676027</v>
+        <v>2734313</v>
       </c>
     </row>
     <row r="16">
@@ -4037,13 +4037,13 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>6.05</v>
+        <v>5.65</v>
       </c>
       <c r="G16" t="n">
-        <v>1326798921</v>
+        <v>1239077225</v>
       </c>
       <c r="H16" t="n">
-        <v>281800</v>
+        <v>275800</v>
       </c>
       <c r="I16" t="n">
         <v>219305733</v>
@@ -4058,7 +4058,7 @@
         <v>2.69</v>
       </c>
       <c r="M16" t="n">
-        <v>0.6276871387295196</v>
+        <v>0.5861874212551935</v>
       </c>
       <c r="N16" t="n">
         <v>0.39</v>
@@ -4136,7 +4136,7 @@
         <v>17544458.64</v>
       </c>
       <c r="AM16" t="n">
-        <v>372696326.1235955</v>
+        <v>348055400.2808989</v>
       </c>
       <c r="AN16" t="n">
         <v>0.0077</v>
@@ -4177,7 +4177,7 @@
         <v>1.42</v>
       </c>
       <c r="AZ16" t="n">
-        <v>0.17</v>
+        <v>0.16</v>
       </c>
       <c r="BA16" t="n">
         <v>0.08</v>
@@ -4186,16 +4186,16 @@
         <v>0</v>
       </c>
       <c r="BC16" t="n">
-        <v>-71.26000000000001</v>
+        <v>-69.22</v>
       </c>
       <c r="BD16" t="n">
-        <v>-76.53</v>
+        <v>-74.87</v>
       </c>
       <c r="BE16" t="n">
         <v>-97.17</v>
       </c>
       <c r="BF16" t="n">
-        <v>-98.68000000000001</v>
+        <v>-98.58</v>
       </c>
       <c r="BG16" t="n">
         <v>-100</v>
@@ -4207,7 +4207,7 @@
         <v>0</v>
       </c>
       <c r="BJ16" t="n">
-        <v>6.05</v>
+        <v>5.65</v>
       </c>
       <c r="BK16" t="n">
         <v>0.08</v>
@@ -4216,28 +4216,28 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="BM16" t="n">
-        <v>6.05</v>
+        <v>6.06</v>
       </c>
       <c r="BN16" t="n">
-        <v>6.05</v>
+        <v>6.06</v>
       </c>
       <c r="BO16" t="n">
         <v>3.31</v>
       </c>
       <c r="BP16" t="n">
-        <v>5.65</v>
+        <v>5.41</v>
       </c>
       <c r="BQ16" t="n">
-        <v>82.56</v>
+        <v>77.09999999999999</v>
       </c>
       <c r="BR16" t="n">
-        <v>5.75</v>
+        <v>6.06</v>
       </c>
       <c r="BS16" t="n">
         <v>0.49</v>
       </c>
       <c r="BT16" t="n">
-        <v>144000</v>
+        <v>144287</v>
       </c>
     </row>
     <row r="17">
@@ -4267,13 +4267,13 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>39.72</v>
+        <v>39.65</v>
       </c>
       <c r="G17" t="n">
-        <v>13092772926</v>
+        <v>13069703122</v>
       </c>
       <c r="H17" t="n">
-        <v>3435300</v>
+        <v>1352700</v>
       </c>
       <c r="I17" t="n">
         <v>0</v>
@@ -4360,13 +4360,13 @@
         <v>8.039999999999999</v>
       </c>
       <c r="AK17" t="n">
-        <v>5912560027.998555</v>
+        <v>5902141944.544798</v>
       </c>
       <c r="AL17" t="n">
-        <v>1636596615.75</v>
+        <v>1633712890.25</v>
       </c>
       <c r="AM17" t="n">
-        <v>4053490069.96904</v>
+        <v>4046347715.789474</v>
       </c>
       <c r="AN17" t="n">
         <v>1.08</v>
@@ -4407,7 +4407,7 @@
         <v>42.98</v>
       </c>
       <c r="AZ17" t="n">
-        <v>21.25</v>
+        <v>21.21</v>
       </c>
       <c r="BA17" t="n">
         <v>4.55</v>
@@ -4416,19 +4416,19 @@
         <v>16.33</v>
       </c>
       <c r="BC17" t="n">
-        <v>32.52</v>
+        <v>32.76</v>
       </c>
       <c r="BD17" t="n">
-        <v>8.199999999999999</v>
+        <v>8.390000000000001</v>
       </c>
       <c r="BE17" t="n">
         <v>-46.5</v>
       </c>
       <c r="BF17" t="n">
-        <v>-88.55</v>
+        <v>-88.53</v>
       </c>
       <c r="BG17" t="n">
-        <v>-58.88</v>
+        <v>-58.81</v>
       </c>
       <c r="BH17" t="n">
         <v>29.25</v>
@@ -4437,7 +4437,7 @@
         <v>0</v>
       </c>
       <c r="BJ17" t="n">
-        <v>39.72</v>
+        <v>39.65</v>
       </c>
       <c r="BK17" t="n">
         <v>4.21</v>
@@ -4446,28 +4446,28 @@
         <v>12.62</v>
       </c>
       <c r="BM17" t="n">
-        <v>40.95</v>
+        <v>39.99</v>
       </c>
       <c r="BN17" t="n">
         <v>40.95</v>
       </c>
       <c r="BO17" t="n">
-        <v>29.53</v>
+        <v>29.59</v>
       </c>
       <c r="BP17" t="n">
-        <v>39.23</v>
+        <v>39.09</v>
       </c>
       <c r="BQ17" t="n">
-        <v>3.15</v>
+        <v>3.14</v>
       </c>
       <c r="BR17" t="n">
-        <v>39.23</v>
+        <v>39.66</v>
       </c>
       <c r="BS17" t="n">
         <v>2.21</v>
       </c>
       <c r="BT17" t="n">
-        <v>1216523</v>
+        <v>1307063</v>
       </c>
     </row>
     <row r="18">
@@ -4497,13 +4497,13 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>14.19</v>
+        <v>13.74</v>
       </c>
       <c r="G18" t="n">
-        <v>13092772926</v>
+        <v>13069703122</v>
       </c>
       <c r="H18" t="n">
-        <v>6700</v>
+        <v>5200</v>
       </c>
       <c r="I18" t="n">
         <v>671494278</v>
@@ -4518,7 +4518,7 @@
         <v>1.2</v>
       </c>
       <c r="M18" t="n">
-        <v>3.855026516076178</v>
+        <v>3.848233859803642</v>
       </c>
       <c r="N18" t="n">
         <v>0.33</v>
@@ -4596,7 +4596,7 @@
         <v>940091989.1999999</v>
       </c>
       <c r="AM18" t="n">
-        <v>3896658608.928572</v>
+        <v>3889792595.833333</v>
       </c>
       <c r="AN18" t="n">
         <v>0.36</v>
@@ -4637,7 +4637,7 @@
         <v>14.31</v>
       </c>
       <c r="AZ18" t="n">
-        <v>7.31</v>
+        <v>7.08</v>
       </c>
       <c r="BA18" t="n">
         <v>1.51</v>
@@ -4646,19 +4646,19 @@
         <v>5.44</v>
       </c>
       <c r="BC18" t="n">
-        <v>23.5</v>
+        <v>27.55</v>
       </c>
       <c r="BD18" t="n">
-        <v>0.84</v>
+        <v>4.14</v>
       </c>
       <c r="BE18" t="n">
         <v>-48.5</v>
       </c>
       <c r="BF18" t="n">
-        <v>-89.34</v>
+        <v>-88.98999999999999</v>
       </c>
       <c r="BG18" t="n">
-        <v>-61.63</v>
+        <v>-60.38</v>
       </c>
       <c r="BH18" t="n">
         <v>9.75</v>
@@ -4667,7 +4667,7 @@
         <v>0</v>
       </c>
       <c r="BJ18" t="n">
-        <v>14.19</v>
+        <v>13.74</v>
       </c>
       <c r="BK18" t="n">
         <v>1.4</v>
@@ -4676,7 +4676,7 @@
         <v>12.62</v>
       </c>
       <c r="BM18" t="n">
-        <v>14.62</v>
+        <v>14.19</v>
       </c>
       <c r="BN18" t="n">
         <v>14.62</v>
@@ -4685,19 +4685,19 @@
         <v>10.19</v>
       </c>
       <c r="BP18" t="n">
-        <v>13.8</v>
+        <v>13.62</v>
       </c>
       <c r="BQ18" t="n">
-        <v>1.12</v>
+        <v>1.09</v>
       </c>
       <c r="BR18" t="n">
-        <v>14.09</v>
+        <v>14.19</v>
       </c>
       <c r="BS18" t="n">
         <v>2.3</v>
       </c>
       <c r="BT18" t="n">
-        <v>8560</v>
+        <v>7873</v>
       </c>
     </row>
     <row r="19">
@@ -4727,13 +4727,13 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>12.6</v>
+        <v>12.7</v>
       </c>
       <c r="G19" t="n">
-        <v>13092772926</v>
+        <v>13069703122</v>
       </c>
       <c r="H19" t="n">
-        <v>15100</v>
+        <v>5800</v>
       </c>
       <c r="I19" t="n">
         <v>317386323</v>
@@ -4748,7 +4748,7 @@
         <v>1.12</v>
       </c>
       <c r="M19" t="n">
-        <v>8.156080018241456</v>
+        <v>8.14170879462881</v>
       </c>
       <c r="N19" t="n">
         <v>0.3</v>
@@ -4826,7 +4826,7 @@
         <v>444340852.2</v>
       </c>
       <c r="AM19" t="n">
-        <v>4156435849.523809</v>
+        <v>4149112102.222222</v>
       </c>
       <c r="AN19" t="n">
         <v>0.36</v>
@@ -4867,7 +4867,7 @@
         <v>14.31</v>
       </c>
       <c r="AZ19" t="n">
-        <v>6.93</v>
+        <v>6.98</v>
       </c>
       <c r="BA19" t="n">
         <v>1.51</v>
@@ -4876,19 +4876,19 @@
         <v>5.25</v>
       </c>
       <c r="BC19" t="n">
-        <v>39.09</v>
+        <v>37.99</v>
       </c>
       <c r="BD19" t="n">
-        <v>13.56</v>
+        <v>12.67</v>
       </c>
       <c r="BE19" t="n">
         <v>-45</v>
       </c>
       <c r="BF19" t="n">
-        <v>-88</v>
+        <v>-88.09</v>
       </c>
       <c r="BG19" t="n">
-        <v>-58.33</v>
+        <v>-58.66</v>
       </c>
       <c r="BH19" t="n">
         <v>9.75</v>
@@ -4897,7 +4897,7 @@
         <v>0</v>
       </c>
       <c r="BJ19" t="n">
-        <v>12.6</v>
+        <v>12.7</v>
       </c>
       <c r="BK19" t="n">
         <v>1.4</v>
@@ -4906,28 +4906,28 @@
         <v>12.62</v>
       </c>
       <c r="BM19" t="n">
-        <v>13.26</v>
+        <v>12.9</v>
       </c>
       <c r="BN19" t="n">
         <v>13.26</v>
       </c>
       <c r="BO19" t="n">
-        <v>9.19</v>
+        <v>9.279999999999999</v>
       </c>
       <c r="BP19" t="n">
-        <v>12.4</v>
+        <v>12.6</v>
       </c>
       <c r="BQ19" t="n">
-        <v>1</v>
+        <v>1.01</v>
       </c>
       <c r="BR19" t="n">
-        <v>12.4</v>
+        <v>12.6</v>
       </c>
       <c r="BS19" t="n">
         <v>2.16</v>
       </c>
       <c r="BT19" t="n">
-        <v>14383</v>
+        <v>14447</v>
       </c>
     </row>
     <row r="20">
@@ -5417,13 +5417,13 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>6.6</v>
+        <v>6.4</v>
       </c>
       <c r="G22" t="n">
-        <v>1321618300</v>
+        <v>1281569939</v>
       </c>
       <c r="H22" t="n">
-        <v>2173700</v>
+        <v>1365200</v>
       </c>
       <c r="I22" t="n">
         <v>200245299</v>
@@ -5438,7 +5438,7 @@
         <v>0.27</v>
       </c>
       <c r="M22" t="n">
-        <v>0.1120951809797344</v>
+        <v>0.1086984148527545</v>
       </c>
       <c r="N22" t="n">
         <v>0.08</v>
@@ -5516,7 +5516,7 @@
         <v>378463615.11</v>
       </c>
       <c r="AM22" t="n">
-        <v>299686689.3424036</v>
+        <v>290605428.3446712</v>
       </c>
       <c r="AN22" t="n">
         <v>0</v>
@@ -5566,19 +5566,19 @@
         <v>172.49</v>
       </c>
       <c r="BC22" t="n">
-        <v>350.08</v>
+        <v>364.14</v>
       </c>
       <c r="BD22" t="n">
-        <v>267.49</v>
+        <v>278.97</v>
       </c>
       <c r="BE22" t="n">
         <v>-100</v>
       </c>
       <c r="BF22" t="n">
-        <v>-71.36</v>
+        <v>-70.47</v>
       </c>
       <c r="BG22" t="n">
-        <v>2513.48</v>
+        <v>2595.15</v>
       </c>
       <c r="BH22" t="n">
         <v>20.75</v>
@@ -5587,7 +5587,7 @@
         <v>0</v>
       </c>
       <c r="BJ22" t="n">
-        <v>6.6</v>
+        <v>6.4</v>
       </c>
       <c r="BK22" t="n">
         <v>1.89</v>
@@ -5596,7 +5596,7 @@
         <v>0.67</v>
       </c>
       <c r="BM22" t="n">
-        <v>6.6</v>
+        <v>6.65</v>
       </c>
       <c r="BN22" t="n">
         <v>7.89</v>
@@ -5605,19 +5605,19 @@
         <v>3.37</v>
       </c>
       <c r="BP22" t="n">
-        <v>6.11</v>
+        <v>6.36</v>
       </c>
       <c r="BQ22" t="n">
-        <v>9.83</v>
+        <v>9.529999999999999</v>
       </c>
       <c r="BR22" t="n">
-        <v>6.17</v>
+        <v>6.6</v>
       </c>
       <c r="BS22" t="n">
         <v>0.09</v>
       </c>
       <c r="BT22" t="n">
-        <v>1741010</v>
+        <v>1773507</v>
       </c>
     </row>
     <row r="23">
@@ -5877,13 +5877,13 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>5.29</v>
+        <v>5.03</v>
       </c>
       <c r="G24" t="n">
-        <v>2136465407</v>
+        <v>2031460148</v>
       </c>
       <c r="H24" t="n">
-        <v>19448300</v>
+        <v>22258800</v>
       </c>
       <c r="I24" t="n">
         <v>403868805</v>
@@ -5898,7 +5898,7 @@
         <v>0.49</v>
       </c>
       <c r="M24" t="n">
-        <v>0.5164709144887834</v>
+        <v>0.4910868563317108</v>
       </c>
       <c r="N24" t="n">
         <v>0.11</v>
@@ -5976,7 +5976,7 @@
         <v>153470145.9</v>
       </c>
       <c r="AM24" t="n">
-        <v>1924743609.90991</v>
+        <v>1830144277.477477</v>
       </c>
       <c r="AN24" t="n">
         <v>0.0813</v>
@@ -6017,7 +6017,7 @@
         <v>5.84</v>
       </c>
       <c r="AZ24" t="n">
-        <v>2.44</v>
+        <v>2.32</v>
       </c>
       <c r="BA24" t="n">
         <v>0.38</v>
@@ -6026,19 +6026,19 @@
         <v>1.46</v>
       </c>
       <c r="BC24" t="n">
-        <v>35.28</v>
+        <v>42.27</v>
       </c>
       <c r="BD24" t="n">
-        <v>10.46</v>
+        <v>16.17</v>
       </c>
       <c r="BE24" t="n">
         <v>-53.83</v>
       </c>
       <c r="BF24" t="n">
-        <v>-92.81999999999999</v>
+        <v>-92.45</v>
       </c>
       <c r="BG24" t="n">
-        <v>-72.44</v>
+        <v>-71.02</v>
       </c>
       <c r="BH24" t="n">
         <v>5.99</v>
@@ -6047,7 +6047,7 @@
         <v>0</v>
       </c>
       <c r="BJ24" t="n">
-        <v>5.29</v>
+        <v>5.03</v>
       </c>
       <c r="BK24" t="n">
         <v>0.38</v>
@@ -6056,28 +6056,28 @@
         <v>0.41</v>
       </c>
       <c r="BM24" t="n">
-        <v>5.3</v>
+        <v>5.45</v>
       </c>
       <c r="BN24" t="n">
-        <v>5.3</v>
+        <v>5.45</v>
       </c>
       <c r="BO24" t="n">
         <v>1.92</v>
       </c>
       <c r="BP24" t="n">
-        <v>4.7</v>
+        <v>4.97</v>
       </c>
       <c r="BQ24" t="n">
-        <v>12.99</v>
+        <v>12.36</v>
       </c>
       <c r="BR24" t="n">
-        <v>4.7</v>
+        <v>5.06</v>
       </c>
       <c r="BS24" t="n">
         <v>0.29</v>
       </c>
       <c r="BT24" t="n">
-        <v>7192340</v>
+        <v>7501063</v>
       </c>
     </row>
     <row r="25">
@@ -6107,13 +6107,13 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>6.48</v>
+        <v>6.05</v>
       </c>
       <c r="G25" t="n">
-        <v>2245281126</v>
+        <v>2096289371</v>
       </c>
       <c r="H25" t="n">
-        <v>3244700</v>
+        <v>1601000</v>
       </c>
       <c r="I25" t="n">
         <v>346494097</v>
@@ -6128,7 +6128,7 @@
         <v>0.97</v>
       </c>
       <c r="M25" t="n">
-        <v>1.119599689563158</v>
+        <v>1.045305597516588</v>
       </c>
       <c r="N25" t="n">
         <v>0.22</v>
@@ -6206,7 +6206,7 @@
         <v>62368937.46</v>
       </c>
       <c r="AM25" t="n">
-        <v>825471002.2058823</v>
+        <v>770694621.6911764</v>
       </c>
       <c r="AN25" t="n">
         <v>0.4742</v>
@@ -6247,7 +6247,7 @@
         <v>3.27</v>
       </c>
       <c r="AZ25" t="n">
-        <v>15.1</v>
+        <v>14.1</v>
       </c>
       <c r="BA25" t="n">
         <v>0.23</v>
@@ -6256,19 +6256,19 @@
         <v>2.2</v>
       </c>
       <c r="BC25" t="n">
-        <v>-38.12</v>
+        <v>-33.72</v>
       </c>
       <c r="BD25" t="n">
-        <v>-49.48</v>
+        <v>-45.88</v>
       </c>
       <c r="BE25" t="n">
         <v>133</v>
       </c>
       <c r="BF25" t="n">
-        <v>-96.42</v>
+        <v>-96.17</v>
       </c>
       <c r="BG25" t="n">
-        <v>-66.05</v>
+        <v>-63.64</v>
       </c>
       <c r="BH25" t="n">
         <v>3.97</v>
@@ -6277,7 +6277,7 @@
         <v>0</v>
       </c>
       <c r="BJ25" t="n">
-        <v>6.48</v>
+        <v>6.05</v>
       </c>
       <c r="BK25" t="n">
         <v>0.18</v>
@@ -6286,7 +6286,7 @@
         <v>0.24</v>
       </c>
       <c r="BM25" t="n">
-        <v>6.79</v>
+        <v>6.52</v>
       </c>
       <c r="BN25" t="n">
         <v>6.79</v>
@@ -6295,19 +6295,19 @@
         <v>2.64</v>
       </c>
       <c r="BP25" t="n">
-        <v>5.95</v>
+        <v>5.97</v>
       </c>
       <c r="BQ25" t="n">
-        <v>27.38</v>
+        <v>25.57</v>
       </c>
       <c r="BR25" t="n">
-        <v>5.95</v>
+        <v>6.49</v>
       </c>
       <c r="BS25" t="n">
         <v>0.67</v>
       </c>
       <c r="BT25" t="n">
-        <v>1322247</v>
+        <v>1417033</v>
       </c>
     </row>
     <row r="26">
@@ -6337,13 +6337,13 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>13.27</v>
+        <v>12.64</v>
       </c>
       <c r="G26" t="n">
-        <v>3622941765</v>
+        <v>17119527984</v>
       </c>
       <c r="H26" t="n">
-        <v>27967800</v>
+        <v>17064100</v>
       </c>
       <c r="I26" t="n">
         <v>1354393401</v>
@@ -6358,7 +6358,7 @@
         <v>1.94</v>
       </c>
       <c r="M26" t="n">
-        <v>0.04671752865066785</v>
+        <v>0.2207548702010202</v>
       </c>
       <c r="N26" t="n">
         <v>0.26</v>
@@ -6436,7 +6436,7 @@
         <v>961619314.7099999</v>
       </c>
       <c r="AM26" t="n">
-        <v>1293907773.214286</v>
+        <v>6114117137.142858</v>
       </c>
       <c r="AN26" t="n">
         <v>0.1043</v>
@@ -6477,7 +6477,7 @@
         <v>7.07</v>
       </c>
       <c r="AZ26" t="n">
-        <v>2.54</v>
+        <v>2.42</v>
       </c>
       <c r="BA26" t="n">
         <v>0.66</v>
@@ -6486,19 +6486,19 @@
         <v>1.19</v>
       </c>
       <c r="BC26" t="n">
-        <v>-34.77</v>
+        <v>-31.52</v>
       </c>
       <c r="BD26" t="n">
-        <v>-46.74</v>
+        <v>-44.09</v>
       </c>
       <c r="BE26" t="n">
         <v>-80.83</v>
       </c>
       <c r="BF26" t="n">
-        <v>-95.03</v>
+        <v>-94.78</v>
       </c>
       <c r="BG26" t="n">
-        <v>-91.01000000000001</v>
+        <v>-90.56</v>
       </c>
       <c r="BH26" t="n">
         <v>4.69</v>
@@ -6507,7 +6507,7 @@
         <v>0</v>
       </c>
       <c r="BJ26" t="n">
-        <v>13.27</v>
+        <v>12.64</v>
       </c>
       <c r="BK26" t="n">
         <v>0.71</v>
@@ -6516,7 +6516,7 @@
         <v>0.72</v>
       </c>
       <c r="BM26" t="n">
-        <v>13.8</v>
+        <v>13.06</v>
       </c>
       <c r="BN26" t="n">
         <v>13.8</v>
@@ -6525,19 +6525,19 @@
         <v>6.91</v>
       </c>
       <c r="BP26" t="n">
-        <v>13.26</v>
+        <v>12.53</v>
       </c>
       <c r="BQ26" t="n">
-        <v>18.5</v>
+        <v>17.62</v>
       </c>
       <c r="BR26" t="n">
-        <v>13.4</v>
+        <v>13.03</v>
       </c>
       <c r="BS26" t="n">
         <v>0.16</v>
       </c>
       <c r="BT26" t="n">
-        <v>16922083</v>
+        <v>17325813</v>
       </c>
     </row>
     <row r="27">
@@ -8165,13 +8165,13 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>26.2</v>
+        <v>25.3</v>
       </c>
       <c r="G34" t="n">
-        <v>5410032917</v>
+        <v>5224191782</v>
       </c>
       <c r="H34" t="n">
-        <v>5260900</v>
+        <v>5400600</v>
       </c>
       <c r="I34" t="n">
         <v>206489813</v>
@@ -8186,7 +8186,7 @@
         <v>0.45</v>
       </c>
       <c r="M34" t="n">
-        <v>0.4756050794008169</v>
+        <v>0.4592674731193702</v>
       </c>
       <c r="N34" t="n">
         <v>0.24</v>
@@ -8264,7 +8264,7 @@
         <v>324189006.41</v>
       </c>
       <c r="AM34" t="n">
-        <v>1124746968.191268</v>
+        <v>1086110557.588358</v>
       </c>
       <c r="AN34" t="n">
         <v>0</v>
@@ -8305,7 +8305,7 @@
         <v>30.28</v>
       </c>
       <c r="AZ34" t="n">
-        <v>61.13</v>
+        <v>59.03</v>
       </c>
       <c r="BA34" t="n">
         <v>2.29</v>
@@ -8314,19 +8314,19 @@
         <v>25.26</v>
       </c>
       <c r="BC34" t="n">
-        <v>41.56</v>
+        <v>46.59</v>
       </c>
       <c r="BD34" t="n">
-        <v>15.58</v>
+        <v>19.69</v>
       </c>
       <c r="BE34" t="n">
         <v>133.33</v>
       </c>
       <c r="BF34" t="n">
-        <v>-91.23999999999999</v>
+        <v>-90.93000000000001</v>
       </c>
       <c r="BG34" t="n">
-        <v>-3.6</v>
+        <v>-0.17</v>
       </c>
       <c r="BH34" t="n">
         <v>38.94</v>
@@ -8335,7 +8335,7 @@
         <v>0</v>
       </c>
       <c r="BJ34" t="n">
-        <v>26.2</v>
+        <v>25.3</v>
       </c>
       <c r="BK34" t="n">
         <v>1.57</v>
@@ -8344,7 +8344,7 @@
         <v>1.58</v>
       </c>
       <c r="BM34" t="n">
-        <v>26.58</v>
+        <v>26.21</v>
       </c>
       <c r="BN34" t="n">
         <v>28.86</v>
@@ -8353,19 +8353,19 @@
         <v>14.3</v>
       </c>
       <c r="BP34" t="n">
-        <v>24.98</v>
+        <v>24.85</v>
       </c>
       <c r="BQ34" t="n">
-        <v>16.61</v>
+        <v>16.04</v>
       </c>
       <c r="BR34" t="n">
-        <v>25.61</v>
+        <v>26</v>
       </c>
       <c r="BS34" t="n">
         <v>0.32</v>
       </c>
       <c r="BT34" t="n">
-        <v>4641020</v>
+        <v>4774720</v>
       </c>
     </row>
     <row r="35">
@@ -8395,13 +8395,13 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>23.35</v>
+        <v>22.76</v>
       </c>
       <c r="G35" t="n">
-        <v>117835753575</v>
+        <v>114858363915</v>
       </c>
       <c r="H35" t="n">
-        <v>63980100</v>
+        <v>64385800</v>
       </c>
       <c r="I35" t="n">
         <v>5046500000</v>
@@ -8416,7 +8416,7 @@
         <v>4.69</v>
       </c>
       <c r="M35" t="n">
-        <v>9.782767089213239</v>
+        <v>9.535583117507462</v>
       </c>
       <c r="N35" t="n">
         <v>1.79</v>
@@ -8494,7 +8494,7 @@
         <v>5349290000</v>
       </c>
       <c r="AM35" t="n">
-        <v>9738492030.991735</v>
+        <v>9492426769.834711</v>
       </c>
       <c r="AN35" t="n">
         <v>0.5305</v>
@@ -8535,7 +8535,7 @@
         <v>7.68</v>
       </c>
       <c r="AZ35" t="n">
-        <v>13.62</v>
+        <v>13.28</v>
       </c>
       <c r="BA35" t="n">
         <v>1.11</v>
@@ -8544,19 +8544,19 @@
         <v>9.119999999999999</v>
       </c>
       <c r="BC35" t="n">
-        <v>-59.71</v>
+        <v>-58.67</v>
       </c>
       <c r="BD35" t="n">
-        <v>-67.11</v>
+        <v>-66.25</v>
       </c>
       <c r="BE35" t="n">
         <v>-41.67</v>
       </c>
       <c r="BF35" t="n">
-        <v>-95.23</v>
+        <v>-95.09999999999999</v>
       </c>
       <c r="BG35" t="n">
-        <v>-60.96</v>
+        <v>-59.94</v>
       </c>
       <c r="BH35" t="n">
         <v>3.71</v>
@@ -8565,7 +8565,7 @@
         <v>0</v>
       </c>
       <c r="BJ35" t="n">
-        <v>23.35</v>
+        <v>22.76</v>
       </c>
       <c r="BK35" t="n">
         <v>1.06</v>
@@ -8574,7 +8574,7 @@
         <v>1.04</v>
       </c>
       <c r="BM35" t="n">
-        <v>23.53</v>
+        <v>23.26</v>
       </c>
       <c r="BN35" t="n">
         <v>24.28</v>
@@ -8583,19 +8583,19 @@
         <v>11.71</v>
       </c>
       <c r="BP35" t="n">
-        <v>22.98</v>
+        <v>22.67</v>
       </c>
       <c r="BQ35" t="n">
-        <v>22.35</v>
+        <v>21.78</v>
       </c>
       <c r="BR35" t="n">
-        <v>23</v>
+        <v>23.26</v>
       </c>
       <c r="BS35" t="n">
         <v>7.3</v>
       </c>
       <c r="BT35" t="n">
-        <v>50368047</v>
+        <v>51944770</v>
       </c>
     </row>
     <row r="36">
@@ -8855,13 +8855,13 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>15.93</v>
+        <v>15.11</v>
       </c>
       <c r="G37" t="n">
-        <v>185857000</v>
+        <v>176289876</v>
       </c>
       <c r="H37" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="I37" t="n">
         <v>4900000</v>
@@ -8876,7 +8876,7 @@
         <v>0.88</v>
       </c>
       <c r="M37" t="n">
-        <v>1.809474458874459</v>
+        <v>1.716330447495362</v>
       </c>
       <c r="N37" t="n">
         <v>0.5</v>
@@ -8954,7 +8954,7 @@
         <v>11319000</v>
       </c>
       <c r="AM37" t="n">
-        <v>44463397.12918661</v>
+        <v>42174611.48325359</v>
       </c>
       <c r="AN37" t="n">
         <v>0</v>
@@ -8995,7 +8995,7 @@
         <v>24.36</v>
       </c>
       <c r="AZ37" t="n">
-        <v>70.84</v>
+        <v>67.19</v>
       </c>
       <c r="BA37" t="n">
         <v>2.44</v>
@@ -9004,19 +9004,19 @@
         <v>15.53</v>
       </c>
       <c r="BC37" t="n">
-        <v>87.31</v>
+        <v>97.47</v>
       </c>
       <c r="BD37" t="n">
-        <v>52.94</v>
+        <v>61.24</v>
       </c>
       <c r="BE37" t="n">
         <v>344.67</v>
       </c>
       <c r="BF37" t="n">
-        <v>-84.65000000000001</v>
+        <v>-83.81999999999999</v>
       </c>
       <c r="BG37" t="n">
-        <v>-2.49</v>
+        <v>2.8</v>
       </c>
       <c r="BH37" t="n">
         <v>17.13</v>
@@ -9025,7 +9025,7 @@
         <v>0</v>
       </c>
       <c r="BJ37" t="n">
-        <v>15.93</v>
+        <v>15.11</v>
       </c>
       <c r="BK37" t="n">
         <v>2.31</v>
@@ -9034,7 +9034,7 @@
         <v>2.31</v>
       </c>
       <c r="BM37" t="n">
-        <v>15.93</v>
+        <v>15.11</v>
       </c>
       <c r="BN37" t="n">
         <v>20.9</v>
@@ -9043,19 +9043,19 @@
         <v>13.42</v>
       </c>
       <c r="BP37" t="n">
-        <v>14.9</v>
+        <v>15.11</v>
       </c>
       <c r="BQ37" t="n">
-        <v>6.89</v>
+        <v>6.54</v>
       </c>
       <c r="BR37" t="n">
-        <v>14.9</v>
+        <v>15.11</v>
       </c>
       <c r="BS37" t="n">
         <v>0.72</v>
       </c>
       <c r="BT37" t="n">
-        <v>1197</v>
+        <v>1187</v>
       </c>
     </row>
     <row r="38">
@@ -9315,13 +9315,13 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>77.7</v>
+        <v>76.31999999999999</v>
       </c>
       <c r="G39" t="n">
-        <v>4355730515</v>
+        <v>4278370202</v>
       </c>
       <c r="H39" t="n">
-        <v>5800</v>
+        <v>6300</v>
       </c>
       <c r="I39" t="n">
         <v>168174945</v>
@@ -9336,7 +9336,7 @@
         <v>0.53</v>
       </c>
       <c r="M39" t="n">
-        <v>0.2186385660298148</v>
+        <v>0.2147554176477718</v>
       </c>
       <c r="N39" t="n">
         <v>0.06</v>
@@ -9414,7 +9414,7 @@
         <v>2536078170.6</v>
       </c>
       <c r="AM39" t="n">
-        <v>457534717.9621849</v>
+        <v>449408634.6638656</v>
       </c>
       <c r="AN39" t="n">
         <v>11.9435</v>
@@ -9455,7 +9455,7 @@
         <v>170.24</v>
       </c>
       <c r="AZ39" t="n">
-        <v>227.01</v>
+        <v>222.98</v>
       </c>
       <c r="BA39" t="n">
         <v>19.01</v>
@@ -9464,19 +9464,19 @@
         <v>91.72</v>
       </c>
       <c r="BC39" t="n">
-        <v>168.35</v>
+        <v>173.2</v>
       </c>
       <c r="BD39" t="n">
-        <v>119.1</v>
+        <v>123.07</v>
       </c>
       <c r="BE39" t="n">
         <v>192.17</v>
       </c>
       <c r="BF39" t="n">
-        <v>-75.53</v>
+        <v>-75.09</v>
       </c>
       <c r="BG39" t="n">
-        <v>18.05</v>
+        <v>20.18</v>
       </c>
       <c r="BH39" t="n">
         <v>128.13</v>
@@ -9485,7 +9485,7 @@
         <v>0</v>
       </c>
       <c r="BJ39" t="n">
-        <v>77.7</v>
+        <v>76.31999999999999</v>
       </c>
       <c r="BK39" t="n">
         <v>15.08</v>
@@ -9494,7 +9494,7 @@
         <v>15.08</v>
       </c>
       <c r="BM39" t="n">
-        <v>78.62</v>
+        <v>78.5</v>
       </c>
       <c r="BN39" t="n">
         <v>78.62</v>
@@ -9503,19 +9503,19 @@
         <v>54.98</v>
       </c>
       <c r="BP39" t="n">
-        <v>77</v>
+        <v>76.3</v>
       </c>
       <c r="BQ39" t="n">
-        <v>5.15</v>
+        <v>5.06</v>
       </c>
       <c r="BR39" t="n">
-        <v>78.47</v>
+        <v>77.03</v>
       </c>
       <c r="BS39" t="n">
         <v>0.58</v>
       </c>
       <c r="BT39" t="n">
-        <v>3303</v>
+        <v>3460</v>
       </c>
     </row>
     <row r="40">
@@ -9545,13 +9545,13 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>24.64</v>
+        <v>24.25</v>
       </c>
       <c r="G40" t="n">
-        <v>141207696982</v>
+        <v>138972773000</v>
       </c>
       <c r="H40" t="n">
-        <v>38595900</v>
+        <v>29035000</v>
       </c>
       <c r="I40" t="n">
         <v>5730834040</v>
@@ -9566,7 +9566,7 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="M40" t="n">
-        <v>0.4284416279193602</v>
+        <v>0.4216605919730961</v>
       </c>
       <c r="N40" t="n">
         <v>0.05</v>
@@ -9644,7 +9644,7 @@
         <v>15358635227.2</v>
       </c>
       <c r="AM40" t="n">
-        <v>7324050673.340248</v>
+        <v>7208131379.66805</v>
       </c>
       <c r="AN40" t="n">
         <v>0.5641</v>
@@ -9685,7 +9685,7 @@
         <v>36.13</v>
       </c>
       <c r="AZ40" t="n">
-        <v>12.44</v>
+        <v>12.25</v>
       </c>
       <c r="BA40" t="n">
         <v>2.76</v>
@@ -9694,19 +9694,19 @@
         <v>27.89</v>
       </c>
       <c r="BC40" t="n">
-        <v>79.58</v>
+        <v>82.47</v>
       </c>
       <c r="BD40" t="n">
-        <v>46.63</v>
+        <v>48.98</v>
       </c>
       <c r="BE40" t="n">
         <v>-49.5</v>
       </c>
       <c r="BF40" t="n">
-        <v>-88.8</v>
+        <v>-88.62</v>
       </c>
       <c r="BG40" t="n">
-        <v>13.19</v>
+        <v>15.01</v>
       </c>
       <c r="BH40" t="n">
         <v>32.47</v>
@@ -9715,7 +9715,7 @@
         <v>0</v>
       </c>
       <c r="BJ40" t="n">
-        <v>24.64</v>
+        <v>24.25</v>
       </c>
       <c r="BK40" t="n">
         <v>2.68</v>
@@ -9724,7 +9724,7 @@
         <v>2.5</v>
       </c>
       <c r="BM40" t="n">
-        <v>24.85</v>
+        <v>24.69</v>
       </c>
       <c r="BN40" t="n">
         <v>27.36</v>
@@ -9733,19 +9733,19 @@
         <v>17.67</v>
       </c>
       <c r="BP40" t="n">
-        <v>24.28</v>
+        <v>24.12</v>
       </c>
       <c r="BQ40" t="n">
-        <v>9.859999999999999</v>
+        <v>9.710000000000001</v>
       </c>
       <c r="BR40" t="n">
-        <v>24.47</v>
+        <v>24.51</v>
       </c>
       <c r="BS40" t="n">
         <v>0.39</v>
       </c>
       <c r="BT40" t="n">
-        <v>44532087</v>
+        <v>44941167</v>
       </c>
     </row>
     <row r="41">
@@ -9775,13 +9775,13 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>19.02</v>
+        <v>18.84</v>
       </c>
       <c r="G41" t="n">
-        <v>45395907825</v>
+        <v>225232427985</v>
       </c>
       <c r="H41" t="n">
-        <v>24469000</v>
+        <v>13597300</v>
       </c>
       <c r="I41" t="n">
         <v>5606747177</v>
@@ -9796,7 +9796,7 @@
         <v>0.92</v>
       </c>
       <c r="M41" t="n">
-        <v>0.2861749396826718</v>
+        <v>1.41986094300977</v>
       </c>
       <c r="N41" t="n">
         <v>0.07000000000000001</v>
@@ -9874,7 +9874,7 @@
         <v>13007653450.64</v>
       </c>
       <c r="AM41" t="n">
-        <v>6994746968.412943</v>
+        <v>34704534358.24345</v>
       </c>
       <c r="AN41" t="n">
         <v>1.6841</v>
@@ -9915,7 +9915,7 @@
         <v>24.4</v>
       </c>
       <c r="AZ41" t="n">
-        <v>28.47</v>
+        <v>28.2</v>
       </c>
       <c r="BA41" t="n">
         <v>2.53</v>
@@ -9924,28 +9924,28 @@
         <v>13.77</v>
       </c>
       <c r="BC41" t="n">
-        <v>57.13</v>
+        <v>58.63</v>
       </c>
       <c r="BD41" t="n">
-        <v>28.29</v>
+        <v>29.52</v>
       </c>
       <c r="BE41" t="n">
         <v>49.67</v>
       </c>
       <c r="BF41" t="n">
-        <v>-86.70999999999999</v>
+        <v>-86.59</v>
       </c>
       <c r="BG41" t="n">
-        <v>-27.6</v>
+        <v>-26.91</v>
       </c>
       <c r="BH41" t="n">
         <v>17.11</v>
       </c>
       <c r="BI41" t="n">
-        <v>0</v>
+        <v>1.44</v>
       </c>
       <c r="BJ41" t="n">
-        <v>19.02</v>
+        <v>18.57</v>
       </c>
       <c r="BK41" t="n">
         <v>2.32</v>
@@ -9954,28 +9954,28 @@
         <v>2.34</v>
       </c>
       <c r="BM41" t="n">
-        <v>19.21</v>
+        <v>18.85</v>
       </c>
       <c r="BN41" t="n">
         <v>20.24</v>
       </c>
       <c r="BO41" t="n">
-        <v>13.44</v>
+        <v>13.56</v>
       </c>
       <c r="BP41" t="n">
-        <v>18.7</v>
+        <v>18.56</v>
       </c>
       <c r="BQ41" t="n">
-        <v>8.140000000000001</v>
+        <v>8.06</v>
       </c>
       <c r="BR41" t="n">
-        <v>19.09</v>
+        <v>18.83</v>
       </c>
       <c r="BS41" t="n">
         <v>0.5600000000000001</v>
       </c>
       <c r="BT41" t="n">
-        <v>13246460</v>
+        <v>13878950</v>
       </c>
     </row>
     <row r="42">
@@ -10005,13 +10005,13 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>21.61</v>
+        <v>21.4</v>
       </c>
       <c r="G42" t="n">
-        <v>45395907825</v>
+        <v>225232427985</v>
       </c>
       <c r="H42" t="n">
-        <v>77677000</v>
+        <v>65583300</v>
       </c>
       <c r="I42" t="n">
         <v>5590117604</v>
@@ -10026,7 +10026,7 @@
         <v>1.05</v>
       </c>
       <c r="M42" t="n">
-        <v>0.2870262575595656</v>
+        <v>1.424084768495075</v>
       </c>
       <c r="N42" t="n">
         <v>0.08</v>
@@ -10104,7 +10104,7 @@
         <v>12969072841.28</v>
       </c>
       <c r="AM42" t="n">
-        <v>6176313989.795918</v>
+        <v>30643867753.06123</v>
       </c>
       <c r="AN42" t="n">
         <v>1.8491</v>
@@ -10145,7 +10145,7 @@
         <v>24.4</v>
       </c>
       <c r="AZ42" t="n">
-        <v>31.3</v>
+        <v>30.99</v>
       </c>
       <c r="BA42" t="n">
         <v>2.53</v>
@@ -10154,28 +10154,28 @@
         <v>15.11</v>
       </c>
       <c r="BC42" t="n">
-        <v>38.29</v>
+        <v>39.65</v>
       </c>
       <c r="BD42" t="n">
-        <v>12.92</v>
+        <v>14.03</v>
       </c>
       <c r="BE42" t="n">
         <v>44.83</v>
       </c>
       <c r="BF42" t="n">
-        <v>-88.31</v>
+        <v>-88.19</v>
       </c>
       <c r="BG42" t="n">
-        <v>-30.06</v>
+        <v>-29.37</v>
       </c>
       <c r="BH42" t="n">
         <v>17.11</v>
       </c>
       <c r="BI42" t="n">
-        <v>0</v>
+        <v>1.39</v>
       </c>
       <c r="BJ42" t="n">
-        <v>21.61</v>
+        <v>21.11</v>
       </c>
       <c r="BK42" t="n">
         <v>2.32</v>
@@ -10184,7 +10184,7 @@
         <v>2.34</v>
       </c>
       <c r="BM42" t="n">
-        <v>21.82</v>
+        <v>21.49</v>
       </c>
       <c r="BN42" t="n">
         <v>23</v>
@@ -10193,19 +10193,19 @@
         <v>15.65</v>
       </c>
       <c r="BP42" t="n">
-        <v>21.31</v>
+        <v>21.11</v>
       </c>
       <c r="BQ42" t="n">
-        <v>9.24</v>
+        <v>9.16</v>
       </c>
       <c r="BR42" t="n">
-        <v>21.7</v>
+        <v>21.45</v>
       </c>
       <c r="BS42" t="n">
         <v>0.63</v>
       </c>
       <c r="BT42" t="n">
-        <v>56664260</v>
+        <v>58456720</v>
       </c>
     </row>
     <row r="43">
@@ -10235,13 +10235,13 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>40.82</v>
+        <v>41.18</v>
       </c>
       <c r="G43" t="n">
-        <v>79247906587</v>
+        <v>79946852592</v>
       </c>
       <c r="H43" t="n">
-        <v>19587400</v>
+        <v>7350000</v>
       </c>
       <c r="I43" t="n">
         <v>1941400000</v>
@@ -10334,7 +10334,7 @@
         <v>9182822000</v>
       </c>
       <c r="AM43" t="n">
-        <v>9652607379.658951</v>
+        <v>9737740876.004871</v>
       </c>
       <c r="AN43" t="n">
         <v>4.5901</v>
@@ -10375,7 +10375,7 @@
         <v>19.95</v>
       </c>
       <c r="AZ43" t="n">
-        <v>74.09</v>
+        <v>74.73999999999999</v>
       </c>
       <c r="BA43" t="n">
         <v>5.63</v>
@@ -10384,19 +10384,19 @@
         <v>48.62</v>
       </c>
       <c r="BC43" t="n">
-        <v>-40.14</v>
+        <v>-40.66</v>
       </c>
       <c r="BD43" t="n">
-        <v>-51.13</v>
+        <v>-51.55</v>
       </c>
       <c r="BE43" t="n">
         <v>81.5</v>
       </c>
       <c r="BF43" t="n">
-        <v>-86.20999999999999</v>
+        <v>-86.33</v>
       </c>
       <c r="BG43" t="n">
-        <v>19.1</v>
+        <v>18.06</v>
       </c>
       <c r="BH43" t="n">
         <v>5.61</v>
@@ -10405,7 +10405,7 @@
         <v>0</v>
       </c>
       <c r="BJ43" t="n">
-        <v>40.82</v>
+        <v>41.18</v>
       </c>
       <c r="BK43" t="n">
         <v>4.73</v>
@@ -10414,7 +10414,7 @@
         <v>4.73</v>
       </c>
       <c r="BM43" t="n">
-        <v>41.39</v>
+        <v>41.29</v>
       </c>
       <c r="BN43" t="n">
         <v>42.98</v>
@@ -10423,19 +10423,19 @@
         <v>28.06</v>
       </c>
       <c r="BP43" t="n">
-        <v>40.62</v>
+        <v>40.07</v>
       </c>
       <c r="BQ43" t="n">
-        <v>8.619999999999999</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="BR43" t="n">
-        <v>40.95</v>
+        <v>40.6</v>
       </c>
       <c r="BS43" t="n">
         <v>0</v>
       </c>
       <c r="BT43" t="n">
-        <v>6525553</v>
+        <v>7031567</v>
       </c>
     </row>
     <row r="44">
@@ -10925,13 +10925,13 @@
         </is>
       </c>
       <c r="F46" t="n">
-        <v>4.5</v>
+        <v>4.36</v>
       </c>
       <c r="G46" t="n">
-        <v>4502439000</v>
+        <v>4362363253</v>
       </c>
       <c r="H46" t="n">
-        <v>33699600</v>
+        <v>22976000</v>
       </c>
       <c r="I46" t="n">
         <v>1000542188</v>
@@ -10946,7 +10946,7 @@
         <v>2.5</v>
       </c>
       <c r="M46" t="n">
-        <v>0.07826085486014682</v>
+        <v>0.07582607502073231</v>
       </c>
       <c r="N46" t="n">
         <v>0.08</v>
@@ -11024,7 +11024,7 @@
         <v>460249406.48</v>
       </c>
       <c r="AM46" t="n">
-        <v>4414155882.352942</v>
+        <v>4276826718.627451</v>
       </c>
       <c r="AN46" t="n">
         <v>0.0311</v>
@@ -11065,7 +11065,7 @@
         <v>3.3</v>
       </c>
       <c r="AZ46" t="n">
-        <v>3.71</v>
+        <v>3.6</v>
       </c>
       <c r="BA46" t="n">
         <v>0.42</v>
@@ -11074,19 +11074,19 @@
         <v>7.38</v>
       </c>
       <c r="BC46" t="n">
-        <v>-10.14</v>
+        <v>-7.25</v>
       </c>
       <c r="BD46" t="n">
-        <v>-26.63</v>
+        <v>-24.27</v>
       </c>
       <c r="BE46" t="n">
         <v>-17.5</v>
       </c>
       <c r="BF46" t="n">
-        <v>-90.59999999999999</v>
+        <v>-90.3</v>
       </c>
       <c r="BG46" t="n">
-        <v>63.97</v>
+        <v>69.23</v>
       </c>
       <c r="BH46" t="n">
         <v>1.58</v>
@@ -11095,7 +11095,7 @@
         <v>0</v>
       </c>
       <c r="BJ46" t="n">
-        <v>4.5</v>
+        <v>4.36</v>
       </c>
       <c r="BK46" t="n">
         <v>0.46</v>
@@ -11104,7 +11104,7 @@
         <v>0.46</v>
       </c>
       <c r="BM46" t="n">
-        <v>4.5</v>
+        <v>4.58</v>
       </c>
       <c r="BN46" t="n">
         <v>7.31</v>
@@ -11113,19 +11113,19 @@
         <v>2.97</v>
       </c>
       <c r="BP46" t="n">
-        <v>4.33</v>
+        <v>4.36</v>
       </c>
       <c r="BQ46" t="n">
-        <v>9.84</v>
+        <v>9.529999999999999</v>
       </c>
       <c r="BR46" t="n">
-        <v>4.46</v>
+        <v>4.53</v>
       </c>
       <c r="BS46" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="BT46" t="n">
-        <v>24364274</v>
+        <v>25110798</v>
       </c>
     </row>
     <row r="47">
@@ -11155,13 +11155,13 @@
         </is>
       </c>
       <c r="F47" t="n">
-        <v>9.66</v>
+        <v>9.77</v>
       </c>
       <c r="G47" t="n">
-        <v>3346616000</v>
+        <v>3384723843</v>
       </c>
       <c r="H47" t="n">
-        <v>13600</v>
+        <v>8000</v>
       </c>
       <c r="I47" t="n">
         <v>254106600</v>
@@ -11176,7 +11176,7 @@
         <v>1.22</v>
       </c>
       <c r="M47" t="n">
-        <v>0.7891705564874499</v>
+        <v>0.7981568243074946</v>
       </c>
       <c r="N47" t="n">
         <v>0.07000000000000001</v>
@@ -11254,7 +11254,7 @@
         <v>322715382</v>
       </c>
       <c r="AM47" t="n">
-        <v>593371631.2056738</v>
+        <v>600128340.9574468</v>
       </c>
       <c r="AN47" t="n">
         <v>0.4132</v>
@@ -11295,7 +11295,7 @@
         <v>11.74</v>
       </c>
       <c r="AZ47" t="n">
-        <v>12.69</v>
+        <v>12.83</v>
       </c>
       <c r="BA47" t="n">
         <v>1.46</v>
@@ -11304,19 +11304,19 @@
         <v>8.619999999999999</v>
       </c>
       <c r="BC47" t="n">
-        <v>48.79</v>
+        <v>47.12</v>
       </c>
       <c r="BD47" t="n">
-        <v>21.49</v>
+        <v>20.12</v>
       </c>
       <c r="BE47" t="n">
         <v>31.33</v>
       </c>
       <c r="BF47" t="n">
-        <v>-84.90000000000001</v>
+        <v>-85.06999999999999</v>
       </c>
       <c r="BG47" t="n">
-        <v>-10.77</v>
+        <v>-11.77</v>
       </c>
       <c r="BH47" t="n">
         <v>7.23</v>
@@ -11325,7 +11325,7 @@
         <v>0</v>
       </c>
       <c r="BJ47" t="n">
-        <v>9.66</v>
+        <v>9.77</v>
       </c>
       <c r="BK47" t="n">
         <v>1.27</v>
@@ -11334,7 +11334,7 @@
         <v>1.28</v>
       </c>
       <c r="BM47" t="n">
-        <v>9.9</v>
+        <v>9.869999999999999</v>
       </c>
       <c r="BN47" t="n">
         <v>9.9</v>
@@ -11343,19 +11343,19 @@
         <v>7.13</v>
       </c>
       <c r="BP47" t="n">
-        <v>9.460000000000001</v>
+        <v>9.6</v>
       </c>
       <c r="BQ47" t="n">
-        <v>7.53</v>
+        <v>7.62</v>
       </c>
       <c r="BR47" t="n">
-        <v>9.58</v>
+        <v>9.67</v>
       </c>
       <c r="BS47" t="n">
         <v>0.53</v>
       </c>
       <c r="BT47" t="n">
-        <v>12817</v>
+        <v>13063</v>
       </c>
     </row>
     <row r="48">
@@ -11385,13 +11385,13 @@
         </is>
       </c>
       <c r="F48" t="n">
-        <v>9.550000000000001</v>
+        <v>9.69</v>
       </c>
       <c r="G48" t="n">
-        <v>3346616000</v>
+        <v>3384723843</v>
       </c>
       <c r="H48" t="n">
-        <v>4700</v>
+        <v>7100</v>
       </c>
       <c r="I48" t="n">
         <v>93397546</v>
@@ -11406,7 +11406,7 @@
         <v>1.24</v>
       </c>
       <c r="M48" t="n">
-        <v>2.147095459329669</v>
+        <v>2.171544388238796</v>
       </c>
       <c r="N48" t="n">
         <v>0.07000000000000001</v>
@@ -11484,7 +11484,7 @@
         <v>118614883.42</v>
       </c>
       <c r="AM48" t="n">
-        <v>585072727.2727273</v>
+        <v>591734937.5874126</v>
       </c>
       <c r="AN48" t="n">
         <v>0.4132</v>
@@ -11525,7 +11525,7 @@
         <v>11.74</v>
       </c>
       <c r="AZ48" t="n">
-        <v>12.49</v>
+        <v>12.68</v>
       </c>
       <c r="BA48" t="n">
         <v>1.46</v>
@@ -11534,19 +11534,19 @@
         <v>8.24</v>
       </c>
       <c r="BC48" t="n">
-        <v>50.51</v>
+        <v>48.33</v>
       </c>
       <c r="BD48" t="n">
-        <v>22.89</v>
+        <v>21.11</v>
       </c>
       <c r="BE48" t="n">
         <v>30.83</v>
       </c>
       <c r="BF48" t="n">
-        <v>-84.73</v>
+        <v>-84.95</v>
       </c>
       <c r="BG48" t="n">
-        <v>-13.76</v>
+        <v>-15</v>
       </c>
       <c r="BH48" t="n">
         <v>7.23</v>
@@ -11555,7 +11555,7 @@
         <v>0</v>
       </c>
       <c r="BJ48" t="n">
-        <v>9.550000000000001</v>
+        <v>9.69</v>
       </c>
       <c r="BK48" t="n">
         <v>1.27</v>
@@ -11564,7 +11564,7 @@
         <v>1.28</v>
       </c>
       <c r="BM48" t="n">
-        <v>9.99</v>
+        <v>9.93</v>
       </c>
       <c r="BN48" t="n">
         <v>9.99</v>
@@ -11573,19 +11573,19 @@
         <v>7.13</v>
       </c>
       <c r="BP48" t="n">
-        <v>9.539999999999999</v>
+        <v>9.43</v>
       </c>
       <c r="BQ48" t="n">
-        <v>7.45</v>
+        <v>7.55</v>
       </c>
       <c r="BR48" t="n">
-        <v>9.539999999999999</v>
+        <v>9.5</v>
       </c>
       <c r="BS48" t="n">
         <v>0.54</v>
       </c>
       <c r="BT48" t="n">
-        <v>2980</v>
+        <v>3053</v>
       </c>
     </row>
     <row r="49">
@@ -11621,7 +11621,7 @@
         <v>979589100</v>
       </c>
       <c r="H49" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I49" t="n">
         <v>11540870</v>
@@ -11845,7 +11845,7 @@
         </is>
       </c>
       <c r="F50" t="n">
-        <v>36.14</v>
+        <v>36.67</v>
       </c>
       <c r="G50" t="n">
         <v>979589100</v>
@@ -11985,7 +11985,7 @@
         <v>68.48999999999999</v>
       </c>
       <c r="AZ50" t="n">
-        <v>79.69</v>
+        <v>80.86</v>
       </c>
       <c r="BA50" t="n">
         <v>9.210000000000001</v>
@@ -11994,19 +11994,19 @@
         <v>30.53</v>
       </c>
       <c r="BC50" t="n">
-        <v>132.09</v>
+        <v>128.74</v>
       </c>
       <c r="BD50" t="n">
-        <v>89.5</v>
+        <v>86.76000000000001</v>
       </c>
       <c r="BE50" t="n">
         <v>120.5</v>
       </c>
       <c r="BF50" t="n">
-        <v>-74.5</v>
+        <v>-74.87</v>
       </c>
       <c r="BG50" t="n">
-        <v>-15.52</v>
+        <v>-16.74</v>
       </c>
       <c r="BH50" t="n">
         <v>42.6</v>
@@ -12015,7 +12015,7 @@
         <v>0</v>
       </c>
       <c r="BJ50" t="n">
-        <v>36.14</v>
+        <v>36.67</v>
       </c>
       <c r="BK50" t="n">
         <v>7.34</v>
@@ -12024,7 +12024,7 @@
         <v>7.6</v>
       </c>
       <c r="BM50" t="n">
-        <v>36.14</v>
+        <v>36.68</v>
       </c>
       <c r="BN50" t="n">
         <v>39.22</v>
@@ -12033,19 +12033,19 @@
         <v>24.3</v>
       </c>
       <c r="BP50" t="n">
-        <v>35.01</v>
+        <v>36.14</v>
       </c>
       <c r="BQ50" t="n">
-        <v>4.75</v>
+        <v>4.82</v>
       </c>
       <c r="BR50" t="n">
-        <v>35.88</v>
+        <v>36.14</v>
       </c>
       <c r="BS50" t="n">
         <v>0.4</v>
       </c>
       <c r="BT50" t="n">
-        <v>477</v>
+        <v>493</v>
       </c>
     </row>
     <row r="51">
@@ -12523,13 +12523,13 @@
         </is>
       </c>
       <c r="F53" t="n">
-        <v>7.34</v>
+        <v>6.61</v>
       </c>
       <c r="G53" t="n">
-        <v>1004496636</v>
+        <v>904594382</v>
       </c>
       <c r="H53" t="n">
-        <v>134800</v>
+        <v>65300</v>
       </c>
       <c r="I53" t="n">
         <v>136852484</v>
@@ -12544,7 +12544,7 @@
         <v>2.79</v>
       </c>
       <c r="M53" t="n">
-        <v>2.609495001972469</v>
+        <v>2.349967569867874</v>
       </c>
       <c r="N53" t="n">
         <v>1.48</v>
@@ -12622,7 +12622,7 @@
         <v>39687220.36</v>
       </c>
       <c r="AM53" t="n">
-        <v>51171504.63576159</v>
+        <v>46082240.5501783</v>
       </c>
       <c r="AN53" t="n">
         <v>0</v>
@@ -12672,16 +12672,16 @@
         <v>0</v>
       </c>
       <c r="BC53" t="n">
-        <v>-46.31</v>
+        <v>-40.38</v>
       </c>
       <c r="BD53" t="n">
-        <v>-56.16</v>
+        <v>-51.32</v>
       </c>
       <c r="BE53" t="n">
         <v>-100</v>
       </c>
       <c r="BF53" t="n">
-        <v>-96.05</v>
+        <v>-95.61</v>
       </c>
       <c r="BG53" t="n">
         <v>-100</v>
@@ -12693,7 +12693,7 @@
         <v>0</v>
       </c>
       <c r="BJ53" t="n">
-        <v>7.34</v>
+        <v>6.61</v>
       </c>
       <c r="BK53" t="n">
         <v>0.29</v>
@@ -12702,19 +12702,19 @@
         <v>0.2</v>
       </c>
       <c r="BM53" t="n">
-        <v>7.6</v>
+        <v>7.44</v>
       </c>
       <c r="BN53" t="n">
-        <v>10.32</v>
+        <v>10.29</v>
       </c>
       <c r="BO53" t="n">
         <v>4.82</v>
       </c>
       <c r="BP53" t="n">
-        <v>7.14</v>
+        <v>6.61</v>
       </c>
       <c r="BQ53" t="n">
-        <v>36.05</v>
+        <v>32.47</v>
       </c>
       <c r="BR53" t="n">
         <v>7.15</v>
@@ -12723,7 +12723,7 @@
         <v>2.36</v>
       </c>
       <c r="BT53" t="n">
-        <v>47210</v>
+        <v>51363</v>
       </c>
     </row>
     <row r="54">
@@ -12753,13 +12753,13 @@
         </is>
       </c>
       <c r="F54" t="n">
-        <v>12.61</v>
+        <v>12.3</v>
       </c>
       <c r="G54" t="n">
-        <v>2940803239</v>
+        <v>2868508874</v>
       </c>
       <c r="H54" t="n">
-        <v>228800</v>
+        <v>193600</v>
       </c>
       <c r="I54" t="n">
         <v>233212121</v>
@@ -12774,7 +12774,7 @@
         <v>0.97</v>
       </c>
       <c r="M54" t="n">
-        <v>1.650648098111075</v>
+        <v>1.610069879715214</v>
       </c>
       <c r="N54" t="n">
         <v>0.5600000000000001</v>
@@ -12852,7 +12852,7 @@
         <v>233212121</v>
       </c>
       <c r="AM54" t="n">
-        <v>402298664.7058824</v>
+        <v>392408874.6922025</v>
       </c>
       <c r="AN54" t="n">
         <v>0.1531</v>
@@ -12893,7 +12893,7 @@
         <v>12.25</v>
       </c>
       <c r="AZ54" t="n">
-        <v>20.07</v>
+        <v>19.58</v>
       </c>
       <c r="BA54" t="n">
         <v>0.98</v>
@@ -12902,19 +12902,19 @@
         <v>6.52</v>
       </c>
       <c r="BC54" t="n">
-        <v>19.01</v>
+        <v>22.01</v>
       </c>
       <c r="BD54" t="n">
-        <v>-2.83</v>
+        <v>-0.38</v>
       </c>
       <c r="BE54" t="n">
         <v>59.17</v>
       </c>
       <c r="BF54" t="n">
-        <v>-92.2</v>
+        <v>-92.01000000000001</v>
       </c>
       <c r="BG54" t="n">
-        <v>-48.32</v>
+        <v>-47.02</v>
       </c>
       <c r="BH54" t="n">
         <v>10.01</v>
@@ -12923,7 +12923,7 @@
         <v>0</v>
       </c>
       <c r="BJ54" t="n">
-        <v>12.61</v>
+        <v>12.3</v>
       </c>
       <c r="BK54" t="n">
         <v>1</v>
@@ -12932,7 +12932,7 @@
         <v>1</v>
       </c>
       <c r="BM54" t="n">
-        <v>12.89</v>
+        <v>12.67</v>
       </c>
       <c r="BN54" t="n">
         <v>12.89</v>
@@ -12941,19 +12941,19 @@
         <v>8.220000000000001</v>
       </c>
       <c r="BP54" t="n">
-        <v>12.47</v>
+        <v>12.29</v>
       </c>
       <c r="BQ54" t="n">
-        <v>12.58</v>
+        <v>12.27</v>
       </c>
       <c r="BR54" t="n">
-        <v>12.68</v>
+        <v>12.67</v>
       </c>
       <c r="BS54" t="n">
         <v>1.26</v>
       </c>
       <c r="BT54" t="n">
-        <v>285567</v>
+        <v>290450</v>
       </c>
     </row>
     <row r="55">
@@ -12983,13 +12983,13 @@
         </is>
       </c>
       <c r="F55" t="n">
-        <v>58.74</v>
+        <v>59.83</v>
       </c>
       <c r="G55" t="n">
-        <v>8110932223</v>
+        <v>6145354876</v>
       </c>
       <c r="H55" t="n">
-        <v>19100</v>
+        <v>4600</v>
       </c>
       <c r="I55" t="n">
         <v>84052790</v>
@@ -13004,7 +13004,7 @@
         <v>2</v>
       </c>
       <c r="M55" t="n">
-        <v>1.252094003082292</v>
+        <v>0.9486655510735024</v>
       </c>
       <c r="N55" t="n">
         <v>0.16</v>
@@ -13082,7 +13082,7 @@
         <v>579123723.1</v>
       </c>
       <c r="AM55" t="n">
-        <v>407994578.6217304</v>
+        <v>309122478.6720322</v>
       </c>
       <c r="AN55" t="n">
         <v>3.1953</v>
@@ -13123,7 +13123,7 @@
         <v>51.21</v>
       </c>
       <c r="AZ55" t="n">
-        <v>61.77</v>
+        <v>62.92</v>
       </c>
       <c r="BA55" t="n">
         <v>9.380000000000001</v>
@@ -13132,19 +13132,19 @@
         <v>16.08</v>
       </c>
       <c r="BC55" t="n">
-        <v>6.76</v>
+        <v>4.82</v>
       </c>
       <c r="BD55" t="n">
-        <v>-12.83</v>
+        <v>-14.42</v>
       </c>
       <c r="BE55" t="n">
         <v>5.17</v>
       </c>
       <c r="BF55" t="n">
-        <v>-84.03</v>
+        <v>-84.33</v>
       </c>
       <c r="BG55" t="n">
-        <v>-72.63</v>
+        <v>-73.13</v>
       </c>
       <c r="BH55" t="n">
         <v>25.37</v>
@@ -13153,7 +13153,7 @@
         <v>0</v>
       </c>
       <c r="BJ55" t="n">
-        <v>58.74</v>
+        <v>59.83</v>
       </c>
       <c r="BK55" t="n">
         <v>6.89</v>
@@ -13162,28 +13162,28 @@
         <v>7.03</v>
       </c>
       <c r="BM55" t="n">
-        <v>60.39</v>
+        <v>60</v>
       </c>
       <c r="BN55" t="n">
         <v>73.67</v>
       </c>
       <c r="BO55" t="n">
-        <v>35.58</v>
+        <v>36.14</v>
       </c>
       <c r="BP55" t="n">
-        <v>58.42</v>
+        <v>57.55</v>
       </c>
       <c r="BQ55" t="n">
-        <v>8.35</v>
+        <v>8.51</v>
       </c>
       <c r="BR55" t="n">
-        <v>60.39</v>
+        <v>58</v>
       </c>
       <c r="BS55" t="n">
         <v>0.66</v>
       </c>
       <c r="BT55" t="n">
-        <v>6240</v>
+        <v>6727</v>
       </c>
     </row>
     <row r="56">
@@ -13213,13 +13213,13 @@
         </is>
       </c>
       <c r="F56" t="n">
-        <v>75.90000000000001</v>
+        <v>78.98999999999999</v>
       </c>
       <c r="G56" t="n">
-        <v>8110932223</v>
+        <v>6145354876</v>
       </c>
       <c r="H56" t="n">
-        <v>84600</v>
+        <v>55700</v>
       </c>
       <c r="I56" t="n">
         <v>39675836</v>
@@ -13234,7 +13234,7 @@
         <v>2.41</v>
       </c>
       <c r="M56" t="n">
-        <v>2.652546358477116</v>
+        <v>2.009736766343509</v>
       </c>
       <c r="N56" t="n">
         <v>0.19</v>
@@ -13312,7 +13312,7 @@
         <v>273366510.04</v>
       </c>
       <c r="AM56" t="n">
-        <v>337393187.312812</v>
+        <v>255630402.4958403</v>
       </c>
       <c r="AN56" t="n">
         <v>3.5102</v>
@@ -13353,7 +13353,7 @@
         <v>51.21</v>
       </c>
       <c r="AZ56" t="n">
-        <v>72.48</v>
+        <v>75.44</v>
       </c>
       <c r="BA56" t="n">
         <v>9.380000000000001</v>
@@ -13362,19 +13362,19 @@
         <v>17.68</v>
       </c>
       <c r="BC56" t="n">
-        <v>-17.37</v>
+        <v>-20.61</v>
       </c>
       <c r="BD56" t="n">
-        <v>-32.54</v>
+        <v>-35.17</v>
       </c>
       <c r="BE56" t="n">
         <v>-4.5</v>
       </c>
       <c r="BF56" t="n">
-        <v>-87.64</v>
+        <v>-88.13</v>
       </c>
       <c r="BG56" t="n">
-        <v>-76.70999999999999</v>
+        <v>-77.62</v>
       </c>
       <c r="BH56" t="n">
         <v>25.37</v>
@@ -13383,7 +13383,7 @@
         <v>0</v>
       </c>
       <c r="BJ56" t="n">
-        <v>75.90000000000001</v>
+        <v>78.98999999999999</v>
       </c>
       <c r="BK56" t="n">
         <v>6.89</v>
@@ -13392,7 +13392,7 @@
         <v>7.03</v>
       </c>
       <c r="BM56" t="n">
-        <v>76</v>
+        <v>79.86</v>
       </c>
       <c r="BN56" t="n">
         <v>86.77</v>
@@ -13401,19 +13401,19 @@
         <v>46.42</v>
       </c>
       <c r="BP56" t="n">
-        <v>73.09999999999999</v>
+        <v>74.23</v>
       </c>
       <c r="BQ56" t="n">
-        <v>10.8</v>
+        <v>11.23</v>
       </c>
       <c r="BR56" t="n">
-        <v>74.98</v>
+        <v>76.11</v>
       </c>
       <c r="BS56" t="n">
         <v>0.79</v>
       </c>
       <c r="BT56" t="n">
-        <v>27547</v>
+        <v>29900</v>
       </c>
     </row>
     <row r="57">
@@ -13443,13 +13443,13 @@
         </is>
       </c>
       <c r="F57" t="n">
-        <v>7</v>
+        <v>7.05</v>
       </c>
       <c r="G57" t="n">
-        <v>1637006000</v>
+        <v>1648698944</v>
       </c>
       <c r="H57" t="n">
-        <v>1478600</v>
+        <v>1900200</v>
       </c>
       <c r="I57" t="n">
         <v>233858065</v>
@@ -13464,7 +13464,7 @@
         <v>0.77</v>
       </c>
       <c r="M57" t="n">
-        <v>0.4899998638062793</v>
+        <v>0.4934998760038488</v>
       </c>
       <c r="N57" t="n">
         <v>0.08</v>
@@ -13542,7 +13542,7 @@
         <v>229180903.7</v>
       </c>
       <c r="AM57" t="n">
-        <v>122438743.4554974</v>
+        <v>123313309.1997008</v>
       </c>
       <c r="AN57" t="n">
         <v>0.347</v>
@@ -13583,7 +13583,7 @@
         <v>10.72</v>
       </c>
       <c r="AZ57" t="n">
-        <v>10.68</v>
+        <v>10.75</v>
       </c>
       <c r="BA57" t="n">
         <v>1.13</v>
@@ -13592,19 +13592,19 @@
         <v>6.26</v>
       </c>
       <c r="BC57" t="n">
-        <v>87.59</v>
+        <v>86.26000000000001</v>
       </c>
       <c r="BD57" t="n">
-        <v>53.17</v>
+        <v>52.08</v>
       </c>
       <c r="BE57" t="n">
         <v>52.5</v>
       </c>
       <c r="BF57" t="n">
-        <v>-83.89</v>
+        <v>-84.01000000000001</v>
       </c>
       <c r="BG57" t="n">
-        <v>-10.52</v>
+        <v>-11.15</v>
       </c>
       <c r="BH57" t="n">
         <v>7.82</v>
@@ -13613,7 +13613,7 @@
         <v>0</v>
       </c>
       <c r="BJ57" t="n">
-        <v>7</v>
+        <v>7.05</v>
       </c>
       <c r="BK57" t="n">
         <v>0.98</v>
@@ -13622,28 +13622,28 @@
         <v>1.04</v>
       </c>
       <c r="BM57" t="n">
-        <v>7.07</v>
+        <v>7.09</v>
       </c>
       <c r="BN57" t="n">
-        <v>7.07</v>
+        <v>7.09</v>
       </c>
       <c r="BO57" t="n">
-        <v>3.43</v>
+        <v>3.45</v>
       </c>
       <c r="BP57" t="n">
-        <v>6.8</v>
+        <v>6.84</v>
       </c>
       <c r="BQ57" t="n">
-        <v>6.76</v>
+        <v>6.81</v>
       </c>
       <c r="BR57" t="n">
-        <v>6.81</v>
+        <v>7</v>
       </c>
       <c r="BS57" t="n">
         <v>0.42</v>
       </c>
       <c r="BT57" t="n">
-        <v>1629150</v>
+        <v>1663980</v>
       </c>
     </row>
     <row r="58">
@@ -14133,13 +14133,13 @@
         </is>
       </c>
       <c r="F60" t="n">
-        <v>414.99</v>
+        <v>410</v>
       </c>
       <c r="G60" t="n">
-        <v>188716700</v>
+        <v>190914532</v>
       </c>
       <c r="H60" t="n">
-        <v>511</v>
+        <v>80</v>
       </c>
       <c r="I60" t="n">
         <v>454750</v>
@@ -14154,7 +14154,7 @@
         <v>0.83</v>
       </c>
       <c r="M60" t="n">
-        <v>14.11574350239804</v>
+        <v>14.28013824209708</v>
       </c>
       <c r="N60" t="n">
         <v>0.68</v>
@@ -14232,7 +14232,7 @@
         <v>59558607.5</v>
       </c>
       <c r="AM60" t="n">
-        <v>-27671070.38123167</v>
+        <v>-27993333.13782991</v>
       </c>
       <c r="AN60" t="n">
         <v>10.0581</v>
@@ -14273,7 +14273,7 @@
         <v>944.87</v>
       </c>
       <c r="AZ60" t="n">
-        <v>2386.19</v>
+        <v>2357.5</v>
       </c>
       <c r="BA60" t="n">
         <v>231.1</v>
@@ -14282,19 +14282,19 @@
         <v>727.97</v>
       </c>
       <c r="BC60" t="n">
-        <v>178.85</v>
+        <v>182.25</v>
       </c>
       <c r="BD60" t="n">
-        <v>127.68</v>
+        <v>130.45</v>
       </c>
       <c r="BE60" t="n">
         <v>475</v>
       </c>
       <c r="BF60" t="n">
-        <v>-44.31</v>
+        <v>-43.63</v>
       </c>
       <c r="BG60" t="n">
-        <v>75.42</v>
+        <v>77.55</v>
       </c>
       <c r="BH60" t="n">
         <v>454.44</v>
@@ -14303,7 +14303,7 @@
         <v>0</v>
       </c>
       <c r="BJ60" t="n">
-        <v>414.99</v>
+        <v>410</v>
       </c>
       <c r="BK60" t="n">
         <v>130.97</v>
@@ -14312,28 +14312,28 @@
         <v>130.97</v>
       </c>
       <c r="BM60" t="n">
-        <v>415</v>
+        <v>414.99</v>
       </c>
       <c r="BN60" t="n">
         <v>415</v>
       </c>
       <c r="BO60" t="n">
-        <v>309.24</v>
+        <v>310.74</v>
       </c>
       <c r="BP60" t="n">
-        <v>370</v>
+        <v>382.1</v>
       </c>
       <c r="BQ60" t="n">
-        <v>3.17</v>
+        <v>3.13</v>
       </c>
       <c r="BR60" t="n">
-        <v>382.08</v>
+        <v>414.99</v>
       </c>
       <c r="BS60" t="n">
         <v>12.82</v>
       </c>
       <c r="BT60" t="n">
-        <v>36</v>
+        <v>50</v>
       </c>
     </row>
     <row r="61">
@@ -14363,13 +14363,13 @@
         </is>
       </c>
       <c r="F61" t="n">
-        <v>34.55</v>
+        <v>33</v>
       </c>
       <c r="G61" t="n">
-        <v>2957769118</v>
+        <v>2825076870</v>
       </c>
       <c r="H61" t="n">
-        <v>1402700</v>
+        <v>1731200</v>
       </c>
       <c r="I61" t="n">
         <v>85608392</v>
@@ -14384,7 +14384,7 @@
         <v>2.37</v>
       </c>
       <c r="M61" t="n">
-        <v>1.568606514027632</v>
+        <v>1.498235259115581</v>
       </c>
       <c r="N61" t="n">
         <v>1.1</v>
@@ -14462,7 +14462,7 @@
         <v>160087693.04</v>
       </c>
       <c r="AM61" t="n">
-        <v>232163981.0047096</v>
+        <v>221748576.9230769</v>
       </c>
       <c r="AN61" t="n">
         <v>0.38</v>
@@ -14503,7 +14503,7 @@
         <v>17.56</v>
       </c>
       <c r="AZ61" t="n">
-        <v>43.53</v>
+        <v>41.58</v>
       </c>
       <c r="BA61" t="n">
         <v>2.52</v>
@@ -14512,19 +14512,19 @@
         <v>11.76</v>
       </c>
       <c r="BC61" t="n">
-        <v>-37.76</v>
+        <v>-34.84</v>
       </c>
       <c r="BD61" t="n">
-        <v>-49.18</v>
+        <v>-46.8</v>
       </c>
       <c r="BE61" t="n">
         <v>26</v>
       </c>
       <c r="BF61" t="n">
-        <v>-92.7</v>
+        <v>-92.36</v>
       </c>
       <c r="BG61" t="n">
-        <v>-65.97</v>
+        <v>-64.37</v>
       </c>
       <c r="BH61" t="n">
         <v>10.99</v>
@@ -14533,7 +14533,7 @@
         <v>0</v>
       </c>
       <c r="BJ61" t="n">
-        <v>34.55</v>
+        <v>33</v>
       </c>
       <c r="BK61" t="n">
         <v>1.87</v>
@@ -14542,7 +14542,7 @@
         <v>1.86</v>
       </c>
       <c r="BM61" t="n">
-        <v>34.8</v>
+        <v>34.53</v>
       </c>
       <c r="BN61" t="n">
         <v>34.8</v>
@@ -14551,19 +14551,19 @@
         <v>19.35</v>
       </c>
       <c r="BP61" t="n">
-        <v>32.4</v>
+        <v>32.93</v>
       </c>
       <c r="BQ61" t="n">
-        <v>18.56</v>
+        <v>17.72</v>
       </c>
       <c r="BR61" t="n">
-        <v>32.4</v>
+        <v>34.29</v>
       </c>
       <c r="BS61" t="n">
         <v>1.19</v>
       </c>
       <c r="BT61" t="n">
-        <v>924077</v>
+        <v>958630</v>
       </c>
     </row>
     <row r="62">
@@ -14599,7 +14599,7 @@
         <v>11374160000</v>
       </c>
       <c r="H62" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="I62" t="n">
         <v>98699749</v>
@@ -14823,13 +14823,13 @@
         </is>
       </c>
       <c r="F63" t="n">
-        <v>1.65</v>
+        <v>1.55</v>
       </c>
       <c r="G63" t="n">
-        <v>429841100</v>
+        <v>403790022</v>
       </c>
       <c r="H63" t="n">
-        <v>36400</v>
+        <v>4100</v>
       </c>
       <c r="I63" t="n">
         <v>122894462</v>
@@ -14844,7 +14844,7 @@
         <v>-0.22</v>
       </c>
       <c r="M63" t="n">
-        <v>0.5286823705693101</v>
+        <v>0.4966408890243252</v>
       </c>
       <c r="N63" t="n">
         <v>0.37</v>
@@ -14922,7 +14922,7 @@
         <v>31952560.12</v>
       </c>
       <c r="AM63" t="n">
-        <v>244227897.7272727</v>
+        <v>229426148.8636364</v>
       </c>
       <c r="AN63" t="n">
         <v>0</v>
@@ -14981,7 +14981,7 @@
         <v>-100</v>
       </c>
       <c r="BF63" t="n">
-        <v>-82.47</v>
+        <v>-81.34</v>
       </c>
       <c r="BG63" t="n">
         <v>-100</v>
@@ -14993,7 +14993,7 @@
         <v>0</v>
       </c>
       <c r="BJ63" t="n">
-        <v>1.65</v>
+        <v>1.55</v>
       </c>
       <c r="BK63" t="n">
         <v>0.26</v>
@@ -15002,7 +15002,7 @@
         <v>0.26</v>
       </c>
       <c r="BM63" t="n">
-        <v>1.7</v>
+        <v>1.65</v>
       </c>
       <c r="BN63" t="n">
         <v>2.12</v>
@@ -15011,19 +15011,19 @@
         <v>1.16</v>
       </c>
       <c r="BP63" t="n">
-        <v>1.6</v>
+        <v>1.53</v>
       </c>
       <c r="BQ63" t="n">
-        <v>6.32</v>
+        <v>5.94</v>
       </c>
       <c r="BR63" t="n">
-        <v>1.63</v>
+        <v>1.65</v>
       </c>
       <c r="BS63" t="n">
         <v>0.19</v>
       </c>
       <c r="BT63" t="n">
-        <v>35890</v>
+        <v>36440</v>
       </c>
     </row>
     <row r="64">
@@ -15053,13 +15053,13 @@
         </is>
       </c>
       <c r="F64" t="n">
-        <v>81.5</v>
+        <v>80.56</v>
       </c>
       <c r="G64" t="n">
-        <v>284816094000</v>
+        <v>279340502574</v>
       </c>
       <c r="H64" t="n">
-        <v>15111300</v>
+        <v>17541000</v>
       </c>
       <c r="I64" t="n">
         <v>0</v>
@@ -15146,13 +15146,13 @@
         <v>41.22</v>
       </c>
       <c r="AK64" t="n">
-        <v>81660953590.06912</v>
+        <v>80091021178.46613</v>
       </c>
       <c r="AL64" t="n">
-        <v>22767073860.91127</v>
+        <v>22329376704.55635</v>
       </c>
       <c r="AM64" t="n">
-        <v>25362074265.36064</v>
+        <v>24874488207.83615</v>
       </c>
       <c r="AN64" t="n">
         <v>1.4201</v>
@@ -15193,7 +15193,7 @@
         <v>38.98</v>
       </c>
       <c r="AZ64" t="n">
-        <v>32.6</v>
+        <v>32.22</v>
       </c>
       <c r="BA64" t="n">
         <v>6.69</v>
@@ -15202,19 +15202,19 @@
         <v>10.4</v>
       </c>
       <c r="BC64" t="n">
-        <v>-41.42</v>
+        <v>-40.74</v>
       </c>
       <c r="BD64" t="n">
-        <v>-52.17</v>
+        <v>-51.61</v>
       </c>
       <c r="BE64" t="n">
         <v>-60</v>
       </c>
       <c r="BF64" t="n">
-        <v>-91.79000000000001</v>
+        <v>-91.69</v>
       </c>
       <c r="BG64" t="n">
-        <v>-87.23999999999999</v>
+        <v>-87.09</v>
       </c>
       <c r="BH64" t="n">
         <v>21.37</v>
@@ -15223,7 +15223,7 @@
         <v>0</v>
       </c>
       <c r="BJ64" t="n">
-        <v>81.5</v>
+        <v>80.56</v>
       </c>
       <c r="BK64" t="n">
         <v>4.74</v>
@@ -15232,7 +15232,7 @@
         <v>1.57</v>
       </c>
       <c r="BM64" t="n">
-        <v>81.5</v>
+        <v>82</v>
       </c>
       <c r="BN64" t="n">
         <v>84.59</v>
@@ -15241,19 +15241,19 @@
         <v>44.12</v>
       </c>
       <c r="BP64" t="n">
-        <v>78.34999999999999</v>
+        <v>79.2</v>
       </c>
       <c r="BQ64" t="n">
-        <v>51.91</v>
+        <v>51.31</v>
       </c>
       <c r="BR64" t="n">
-        <v>78.54000000000001</v>
+        <v>81.08</v>
       </c>
       <c r="BS64" t="n">
         <v>3.49</v>
       </c>
       <c r="BT64" t="n">
-        <v>13647857</v>
+        <v>13684580</v>
       </c>
     </row>
     <row r="65">
@@ -15283,13 +15283,13 @@
         </is>
       </c>
       <c r="F65" t="n">
-        <v>27.95</v>
+        <v>26.7</v>
       </c>
       <c r="G65" t="n">
-        <v>284816094000</v>
+        <v>279340502574</v>
       </c>
       <c r="H65" t="n">
-        <v>29100</v>
+        <v>49500</v>
       </c>
       <c r="I65" t="n">
         <v>7298813414</v>
@@ -15304,7 +15304,7 @@
         <v>3.29</v>
       </c>
       <c r="M65" t="n">
-        <v>6.885697620390723</v>
+        <v>6.753320034831109</v>
       </c>
       <c r="N65" t="n">
         <v>0.29</v>
@@ -15382,7 +15382,7 @@
         <v>11532125194.12</v>
       </c>
       <c r="AM65" t="n">
-        <v>21334538876.4045</v>
+        <v>20924382215.2809</v>
       </c>
       <c r="AN65" t="n">
         <v>0.4734</v>
@@ -15423,7 +15423,7 @@
         <v>12.99</v>
       </c>
       <c r="AZ65" t="n">
-        <v>9.41</v>
+        <v>8.99</v>
       </c>
       <c r="BA65" t="n">
         <v>2.23</v>
@@ -15432,19 +15432,19 @@
         <v>3.47</v>
       </c>
       <c r="BC65" t="n">
-        <v>-43.08</v>
+        <v>-40.41</v>
       </c>
       <c r="BD65" t="n">
-        <v>-53.52</v>
+        <v>-51.35</v>
       </c>
       <c r="BE65" t="n">
         <v>-66.33</v>
       </c>
       <c r="BF65" t="n">
-        <v>-92.02</v>
+        <v>-91.64</v>
       </c>
       <c r="BG65" t="n">
-        <v>-87.59999999999999</v>
+        <v>-87.02</v>
       </c>
       <c r="BH65" t="n">
         <v>7.12</v>
@@ -15453,7 +15453,7 @@
         <v>0</v>
       </c>
       <c r="BJ65" t="n">
-        <v>27.95</v>
+        <v>26.7</v>
       </c>
       <c r="BK65" t="n">
         <v>1.58</v>
@@ -15462,7 +15462,7 @@
         <v>1.57</v>
       </c>
       <c r="BM65" t="n">
-        <v>27.96</v>
+        <v>29.3</v>
       </c>
       <c r="BN65" t="n">
         <v>46.43</v>
@@ -15471,19 +15471,19 @@
         <v>20.44</v>
       </c>
       <c r="BP65" t="n">
-        <v>26.56</v>
+        <v>26.7</v>
       </c>
       <c r="BQ65" t="n">
-        <v>17.8</v>
+        <v>17.01</v>
       </c>
       <c r="BR65" t="n">
-        <v>26.56</v>
+        <v>27.95</v>
       </c>
       <c r="BS65" t="n">
         <v>4.14</v>
       </c>
       <c r="BT65" t="n">
-        <v>11217</v>
+        <v>11510</v>
       </c>
     </row>
     <row r="66">
@@ -15513,13 +15513,13 @@
         </is>
       </c>
       <c r="F66" t="n">
-        <v>26.43</v>
+        <v>26.7</v>
       </c>
       <c r="G66" t="n">
-        <v>284816094000</v>
+        <v>279340502574</v>
       </c>
       <c r="H66" t="n">
-        <v>28900</v>
+        <v>26500</v>
       </c>
       <c r="I66" t="n">
         <v>2972355254</v>
@@ -15534,7 +15534,7 @@
         <v>2.75</v>
       </c>
       <c r="M66" t="n">
-        <v>16.90828244329898</v>
+        <v>16.58322059347629</v>
       </c>
       <c r="N66" t="n">
         <v>0.25</v>
@@ -15612,7 +15612,7 @@
         <v>4696321301.320001</v>
       </c>
       <c r="AM66" t="n">
-        <v>25544044304.93274</v>
+        <v>25052959872.10762</v>
       </c>
       <c r="AN66" t="n">
         <v>0.4734</v>
@@ -15653,7 +15653,7 @@
         <v>12.99</v>
       </c>
       <c r="AZ66" t="n">
-        <v>10.62</v>
+        <v>10.72</v>
       </c>
       <c r="BA66" t="n">
         <v>2.23</v>
@@ -15662,19 +15662,19 @@
         <v>3.47</v>
       </c>
       <c r="BC66" t="n">
-        <v>-39.8</v>
+        <v>-40.41</v>
       </c>
       <c r="BD66" t="n">
-        <v>-50.85</v>
+        <v>-51.35</v>
       </c>
       <c r="BE66" t="n">
         <v>-59.83</v>
       </c>
       <c r="BF66" t="n">
-        <v>-91.56</v>
+        <v>-91.64</v>
       </c>
       <c r="BG66" t="n">
-        <v>-86.89</v>
+        <v>-87.02</v>
       </c>
       <c r="BH66" t="n">
         <v>7.12</v>
@@ -15683,7 +15683,7 @@
         <v>0</v>
       </c>
       <c r="BJ66" t="n">
-        <v>26.43</v>
+        <v>26.7</v>
       </c>
       <c r="BK66" t="n">
         <v>1.58</v>
@@ -15692,7 +15692,7 @@
         <v>1.57</v>
       </c>
       <c r="BM66" t="n">
-        <v>26.67</v>
+        <v>28.5</v>
       </c>
       <c r="BN66" t="n">
         <v>28.51</v>
@@ -15701,19 +15701,19 @@
         <v>9.48</v>
       </c>
       <c r="BP66" t="n">
-        <v>26.01</v>
+        <v>25.11</v>
       </c>
       <c r="BQ66" t="n">
-        <v>16.83</v>
+        <v>17.01</v>
       </c>
       <c r="BR66" t="n">
-        <v>26.01</v>
+        <v>26.2</v>
       </c>
       <c r="BS66" t="n">
         <v>3.46</v>
       </c>
       <c r="BT66" t="n">
-        <v>5083</v>
+        <v>4857</v>
       </c>
     </row>
     <row r="67">
@@ -15973,13 +15973,13 @@
         </is>
       </c>
       <c r="F68" t="n">
-        <v>18.55</v>
+        <v>18.28</v>
       </c>
       <c r="G68" t="n">
-        <v>7841351237</v>
+        <v>7736577455</v>
       </c>
       <c r="H68" t="n">
-        <v>166800</v>
+        <v>119200</v>
       </c>
       <c r="I68" t="n">
         <v>137989898</v>
@@ -16072,7 +16072,7 @@
         <v>205604948.02</v>
       </c>
       <c r="AM68" t="n">
-        <v>543783026.1442441</v>
+        <v>536517160.5409154</v>
       </c>
       <c r="AN68" t="n">
         <v>0.1911</v>
@@ -16113,7 +16113,7 @@
         <v>21.39</v>
       </c>
       <c r="AZ68" t="n">
-        <v>34.32</v>
+        <v>33.82</v>
       </c>
       <c r="BA68" t="n">
         <v>1.24</v>
@@ -16122,19 +16122,19 @@
         <v>63.25</v>
       </c>
       <c r="BC68" t="n">
-        <v>41.26</v>
+        <v>43.34</v>
       </c>
       <c r="BD68" t="n">
-        <v>15.33</v>
+        <v>17.04</v>
       </c>
       <c r="BE68" t="n">
         <v>85</v>
       </c>
       <c r="BF68" t="n">
-        <v>-93.31999999999999</v>
+        <v>-93.22</v>
       </c>
       <c r="BG68" t="n">
-        <v>240.96</v>
+        <v>246</v>
       </c>
       <c r="BH68" t="n">
         <v>20.48</v>
@@ -16143,7 +16143,7 @@
         <v>0</v>
       </c>
       <c r="BJ68" t="n">
-        <v>18.55</v>
+        <v>18.28</v>
       </c>
       <c r="BK68" t="n">
         <v>1.49</v>
@@ -16152,28 +16152,28 @@
         <v>1.49</v>
       </c>
       <c r="BM68" t="n">
-        <v>18.91</v>
+        <v>18.67</v>
       </c>
       <c r="BN68" t="n">
         <v>22.11</v>
       </c>
       <c r="BO68" t="n">
-        <v>15.51</v>
+        <v>15.57</v>
       </c>
       <c r="BP68" t="n">
-        <v>18.5</v>
+        <v>18.27</v>
       </c>
       <c r="BQ68" t="n">
-        <v>12.48</v>
+        <v>12.3</v>
       </c>
       <c r="BR68" t="n">
-        <v>18.91</v>
+        <v>18.65</v>
       </c>
       <c r="BS68" t="n">
         <v>0</v>
       </c>
       <c r="BT68" t="n">
-        <v>58130</v>
+        <v>62987</v>
       </c>
     </row>
     <row r="69">
@@ -16203,13 +16203,13 @@
         </is>
       </c>
       <c r="F69" t="n">
-        <v>20.62</v>
+        <v>20.4</v>
       </c>
       <c r="G69" t="n">
-        <v>7841351237</v>
+        <v>7736577455</v>
       </c>
       <c r="H69" t="n">
-        <v>5307500</v>
+        <v>3769700</v>
       </c>
       <c r="I69" t="n">
         <v>255106712</v>
@@ -16302,7 +16302,7 @@
         <v>380109000.88</v>
       </c>
       <c r="AM69" t="n">
-        <v>466747097.4404762</v>
+        <v>460510562.797619</v>
       </c>
       <c r="AN69" t="n">
         <v>0.8856000000000001</v>
@@ -16343,7 +16343,7 @@
         <v>21.39</v>
       </c>
       <c r="AZ69" t="n">
-        <v>36.05</v>
+        <v>35.67</v>
       </c>
       <c r="BA69" t="n">
         <v>1.24</v>
@@ -16352,19 +16352,19 @@
         <v>69.59</v>
       </c>
       <c r="BC69" t="n">
-        <v>27.08</v>
+        <v>28.45</v>
       </c>
       <c r="BD69" t="n">
-        <v>3.76</v>
+        <v>4.88</v>
       </c>
       <c r="BE69" t="n">
         <v>74.83</v>
       </c>
       <c r="BF69" t="n">
-        <v>-93.98999999999999</v>
+        <v>-93.92</v>
       </c>
       <c r="BG69" t="n">
-        <v>237.47</v>
+        <v>241.11</v>
       </c>
       <c r="BH69" t="n">
         <v>20.48</v>
@@ -16373,7 +16373,7 @@
         <v>0</v>
       </c>
       <c r="BJ69" t="n">
-        <v>20.62</v>
+        <v>20.4</v>
       </c>
       <c r="BK69" t="n">
         <v>1.49</v>
@@ -16382,28 +16382,28 @@
         <v>1.49</v>
       </c>
       <c r="BM69" t="n">
-        <v>20.91</v>
+        <v>20.62</v>
       </c>
       <c r="BN69" t="n">
         <v>25.63</v>
       </c>
       <c r="BO69" t="n">
-        <v>16.99</v>
+        <v>17.11</v>
       </c>
       <c r="BP69" t="n">
-        <v>20.52</v>
+        <v>20.25</v>
       </c>
       <c r="BQ69" t="n">
-        <v>13.87</v>
+        <v>13.72</v>
       </c>
       <c r="BR69" t="n">
-        <v>20.88</v>
+        <v>20.62</v>
       </c>
       <c r="BS69" t="n">
         <v>0</v>
       </c>
       <c r="BT69" t="n">
-        <v>2907200</v>
+        <v>3038073</v>
       </c>
     </row>
     <row r="70">
@@ -16433,13 +16433,13 @@
         </is>
       </c>
       <c r="F70" t="n">
-        <v>20.57</v>
+        <v>20.91</v>
       </c>
       <c r="G70" t="n">
-        <v>9555941462</v>
+        <v>9713890981</v>
       </c>
       <c r="H70" t="n">
-        <v>6335300</v>
+        <v>4828200</v>
       </c>
       <c r="I70" t="n">
         <v>464557268</v>
@@ -16454,7 +16454,7 @@
         <v>0.68</v>
       </c>
       <c r="M70" t="n">
-        <v>0.7542332117239275</v>
+        <v>0.7666998821696762</v>
       </c>
       <c r="N70" t="n">
         <v>0.2</v>
@@ -16532,7 +16532,7 @@
         <v>55746872.16</v>
       </c>
       <c r="AM70" t="n">
-        <v>3153776060.066007</v>
+        <v>3205904614.191419</v>
       </c>
       <c r="AN70" t="n">
         <v>0.1236</v>
@@ -16573,7 +16573,7 @@
         <v>6.9</v>
       </c>
       <c r="AZ70" t="n">
-        <v>2.37</v>
+        <v>2.4</v>
       </c>
       <c r="BA70" t="n">
         <v>0.12</v>
@@ -16582,19 +16582,19 @@
         <v>1.07</v>
       </c>
       <c r="BC70" t="n">
-        <v>-58.92</v>
+        <v>-59.59</v>
       </c>
       <c r="BD70" t="n">
-        <v>-66.45999999999999</v>
+        <v>-67.01000000000001</v>
       </c>
       <c r="BE70" t="n">
         <v>-88.5</v>
       </c>
       <c r="BF70" t="n">
-        <v>-99.42</v>
+        <v>-99.43000000000001</v>
       </c>
       <c r="BG70" t="n">
-        <v>-94.8</v>
+        <v>-94.89</v>
       </c>
       <c r="BH70" t="n">
         <v>26.44</v>
@@ -16603,7 +16603,7 @@
         <v>0</v>
       </c>
       <c r="BJ70" t="n">
-        <v>20.57</v>
+        <v>20.91</v>
       </c>
       <c r="BK70" t="n">
         <v>0.12</v>
@@ -16612,7 +16612,7 @@
         <v>0.1</v>
       </c>
       <c r="BM70" t="n">
-        <v>21</v>
+        <v>21.08</v>
       </c>
       <c r="BN70" t="n">
         <v>22.15</v>
@@ -16621,19 +16621,19 @@
         <v>13.21</v>
       </c>
       <c r="BP70" t="n">
-        <v>20.36</v>
+        <v>20</v>
       </c>
       <c r="BQ70" t="n">
-        <v>206.3</v>
+        <v>209.71</v>
       </c>
       <c r="BR70" t="n">
-        <v>20.62</v>
+        <v>20.5</v>
       </c>
       <c r="BS70" t="n">
         <v>0.67</v>
       </c>
       <c r="BT70" t="n">
-        <v>3724413</v>
+        <v>3823463</v>
       </c>
     </row>
     <row r="71">

</xml_diff>

<commit_message>
📊 Dados atualizados - 2026-10-15 05:27
</commit_message>
<xml_diff>
--- a/data/ativos.xlsx
+++ b/data/ativos.xlsx
@@ -1047,13 +1047,13 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>29.15</v>
+        <v>28.51</v>
       </c>
       <c r="G3" t="n">
-        <v>3899302168</v>
+        <v>3813691498</v>
       </c>
       <c r="H3" t="n">
-        <v>791200</v>
+        <v>666900</v>
       </c>
       <c r="I3" t="n">
         <v>129510368</v>
@@ -1068,7 +1068,7 @@
         <v>0.88</v>
       </c>
       <c r="M3" t="n">
-        <v>0.970233222407301</v>
+        <v>0.9489313810398361</v>
       </c>
       <c r="N3" t="n">
         <v>0.09</v>
@@ -1146,7 +1146,7 @@
         <v>506385538.88</v>
       </c>
       <c r="AM3" t="n">
-        <v>761582454.6875</v>
+        <v>744861620.703125</v>
       </c>
       <c r="AN3" t="n">
         <v>2.7</v>
@@ -1187,7 +1187,7 @@
         <v>40.42</v>
       </c>
       <c r="AZ3" t="n">
-        <v>53.34</v>
+        <v>52.17</v>
       </c>
       <c r="BA3" t="n">
         <v>4.87</v>
@@ -1196,19 +1196,19 @@
         <v>21.14</v>
       </c>
       <c r="BC3" t="n">
-        <v>69.81</v>
+        <v>73.62</v>
       </c>
       <c r="BD3" t="n">
-        <v>38.65</v>
+        <v>41.76</v>
       </c>
       <c r="BE3" t="n">
         <v>83</v>
       </c>
       <c r="BF3" t="n">
-        <v>-83.3</v>
+        <v>-82.92</v>
       </c>
       <c r="BG3" t="n">
-        <v>-27.49</v>
+        <v>-25.87</v>
       </c>
       <c r="BH3" t="n">
         <v>27.85</v>
@@ -1217,7 +1217,7 @@
         <v>0</v>
       </c>
       <c r="BJ3" t="n">
-        <v>29.15</v>
+        <v>28.51</v>
       </c>
       <c r="BK3" t="n">
         <v>3.91</v>
@@ -1226,7 +1226,7 @@
         <v>4.39</v>
       </c>
       <c r="BM3" t="n">
-        <v>29.44</v>
+        <v>28.83</v>
       </c>
       <c r="BN3" t="n">
         <v>29.56</v>
@@ -1235,19 +1235,19 @@
         <v>18.72</v>
       </c>
       <c r="BP3" t="n">
-        <v>28.79</v>
+        <v>27.89</v>
       </c>
       <c r="BQ3" t="n">
-        <v>6.64</v>
+        <v>6.49</v>
       </c>
       <c r="BR3" t="n">
-        <v>29.37</v>
+        <v>28.72</v>
       </c>
       <c r="BS3" t="n">
         <v>0.79</v>
       </c>
       <c r="BT3" t="n">
-        <v>701093</v>
+        <v>712993</v>
       </c>
     </row>
     <row r="4">
@@ -1277,13 +1277,13 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>16.32</v>
+        <v>16.52</v>
       </c>
       <c r="G4" t="n">
-        <v>252709646474</v>
+        <v>255806590288</v>
       </c>
       <c r="H4" t="n">
-        <v>56978500</v>
+        <v>43431300</v>
       </c>
       <c r="I4" t="n">
         <v>15484664889</v>
@@ -1298,7 +1298,7 @@
         <v>2.76</v>
       </c>
       <c r="M4" t="n">
-        <v>2.861439043039963</v>
+        <v>2.896505832405253</v>
       </c>
       <c r="N4" t="n">
         <v>1.76</v>
@@ -1376,7 +1376,7 @@
         <v>16258898133.45</v>
       </c>
       <c r="AM4" t="n">
-        <v>25020757076.63366</v>
+        <v>25327385177.02971</v>
       </c>
       <c r="AN4" t="n">
         <v>0.269</v>
@@ -1417,7 +1417,7 @@
         <v>9.470000000000001</v>
       </c>
       <c r="AZ4" t="n">
-        <v>20.37</v>
+        <v>20.62</v>
       </c>
       <c r="BA4" t="n">
         <v>1.13</v>
@@ -1426,19 +1426,19 @@
         <v>11.39</v>
       </c>
       <c r="BC4" t="n">
-        <v>-28.89</v>
+        <v>-29.76</v>
       </c>
       <c r="BD4" t="n">
-        <v>-41.94</v>
+        <v>-42.65</v>
       </c>
       <c r="BE4" t="n">
         <v>24.83</v>
       </c>
       <c r="BF4" t="n">
-        <v>-93.09</v>
+        <v>-93.18000000000001</v>
       </c>
       <c r="BG4" t="n">
-        <v>-30.23</v>
+        <v>-31.07</v>
       </c>
       <c r="BH4" t="n">
         <v>5.7</v>
@@ -1447,7 +1447,7 @@
         <v>0</v>
       </c>
       <c r="BJ4" t="n">
-        <v>16.32</v>
+        <v>16.52</v>
       </c>
       <c r="BK4" t="n">
         <v>1.05</v>
@@ -1456,28 +1456,28 @@
         <v>1.04</v>
       </c>
       <c r="BM4" t="n">
-        <v>16.32</v>
+        <v>16.55</v>
       </c>
       <c r="BN4" t="n">
         <v>16.94</v>
       </c>
       <c r="BO4" t="n">
-        <v>11.11</v>
+        <v>11.26</v>
       </c>
       <c r="BP4" t="n">
-        <v>15.88</v>
+        <v>16.12</v>
       </c>
       <c r="BQ4" t="n">
-        <v>15.74</v>
+        <v>15.93</v>
       </c>
       <c r="BR4" t="n">
-        <v>16</v>
+        <v>16.23</v>
       </c>
       <c r="BS4" t="n">
         <v>2.76</v>
       </c>
       <c r="BT4" t="n">
-        <v>31361613</v>
+        <v>32705670</v>
       </c>
     </row>
     <row r="5">
@@ -1737,13 +1737,13 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>7.07</v>
+        <v>7</v>
       </c>
       <c r="G6" t="n">
-        <v>446008839</v>
+        <v>441592830</v>
       </c>
       <c r="H6" t="n">
-        <v>1100</v>
+        <v>1400</v>
       </c>
       <c r="I6" t="n">
         <v>63084700</v>
@@ -1758,7 +1758,7 @@
         <v>1.91</v>
       </c>
       <c r="M6" t="n">
-        <v>6.943484366206736</v>
+        <v>6.874735752342318</v>
       </c>
       <c r="N6" t="n">
         <v>1.26</v>
@@ -1836,7 +1836,7 @@
         <v>35958279</v>
       </c>
       <c r="AM6" t="n">
-        <v>42639468.35564053</v>
+        <v>42217287.76290631</v>
       </c>
       <c r="AN6" t="n">
         <v>0.5199</v>
@@ -1877,7 +1877,7 @@
         <v>5.74</v>
       </c>
       <c r="AZ6" t="n">
-        <v>8.300000000000001</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="BA6" t="n">
         <v>0.65</v>
@@ -1886,19 +1886,19 @@
         <v>7.95</v>
       </c>
       <c r="BC6" t="n">
-        <v>-0.48</v>
+        <v>0.51</v>
       </c>
       <c r="BD6" t="n">
-        <v>-18.74</v>
+        <v>-17.93</v>
       </c>
       <c r="BE6" t="n">
         <v>17.33</v>
       </c>
       <c r="BF6" t="n">
-        <v>-90.83</v>
+        <v>-90.73999999999999</v>
       </c>
       <c r="BG6" t="n">
-        <v>12.5</v>
+        <v>13.62</v>
       </c>
       <c r="BH6" t="n">
         <v>3.86</v>
@@ -1907,7 +1907,7 @@
         <v>0</v>
       </c>
       <c r="BJ6" t="n">
-        <v>7.07</v>
+        <v>7</v>
       </c>
       <c r="BK6" t="n">
         <v>0.57</v>
@@ -1916,7 +1916,7 @@
         <v>0.5600000000000001</v>
       </c>
       <c r="BM6" t="n">
-        <v>7.08</v>
+        <v>7.05</v>
       </c>
       <c r="BN6" t="n">
         <v>8.16</v>
@@ -1925,19 +1925,19 @@
         <v>6.22</v>
       </c>
       <c r="BP6" t="n">
-        <v>7.03</v>
+        <v>7</v>
       </c>
       <c r="BQ6" t="n">
-        <v>12.57</v>
+        <v>12.45</v>
       </c>
       <c r="BR6" t="n">
-        <v>7.03</v>
+        <v>7.05</v>
       </c>
       <c r="BS6" t="n">
         <v>7.32</v>
       </c>
       <c r="BT6" t="n">
-        <v>647</v>
+        <v>683</v>
       </c>
     </row>
     <row r="7">
@@ -3117,13 +3117,13 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>6.5</v>
+        <v>6.35</v>
       </c>
       <c r="G12" t="n">
-        <v>623749880</v>
+        <v>609355706</v>
       </c>
       <c r="H12" t="n">
-        <v>2954700</v>
+        <v>1748400</v>
       </c>
       <c r="I12" t="n">
         <v>95961536</v>
@@ -3138,7 +3138,7 @@
         <v>0.32</v>
       </c>
       <c r="M12" t="n">
-        <v>0.1128042139959915</v>
+        <v>0.1102010495926708</v>
       </c>
       <c r="N12" t="n">
         <v>0.14</v>
@@ -3216,7 +3216,7 @@
         <v>362734606.08</v>
       </c>
       <c r="AM12" t="n">
-        <v>670698795.6989247</v>
+        <v>655221189.2473118</v>
       </c>
       <c r="AN12" t="n">
         <v>0.4208</v>
@@ -3257,7 +3257,7 @@
         <v>30.49</v>
       </c>
       <c r="AZ12" t="n">
-        <v>8.789999999999999</v>
+        <v>8.58</v>
       </c>
       <c r="BA12" t="n">
         <v>4.41</v>
@@ -3266,19 +3266,19 @@
         <v>18.12</v>
       </c>
       <c r="BC12" t="n">
-        <v>474.57</v>
+        <v>488.15</v>
       </c>
       <c r="BD12" t="n">
-        <v>369.14</v>
+        <v>380.22</v>
       </c>
       <c r="BE12" t="n">
         <v>35.17</v>
       </c>
       <c r="BF12" t="n">
-        <v>-32.13</v>
+        <v>-30.53</v>
       </c>
       <c r="BG12" t="n">
-        <v>178.75</v>
+        <v>185.34</v>
       </c>
       <c r="BH12" t="n">
         <v>16.4</v>
@@ -3287,7 +3287,7 @@
         <v>0</v>
       </c>
       <c r="BJ12" t="n">
-        <v>6.5</v>
+        <v>6.35</v>
       </c>
       <c r="BK12" t="n">
         <v>3.78</v>
@@ -3296,7 +3296,7 @@
         <v>3.63</v>
       </c>
       <c r="BM12" t="n">
-        <v>6.62</v>
+        <v>6.47</v>
       </c>
       <c r="BN12" t="n">
         <v>7.3</v>
@@ -3305,19 +3305,19 @@
         <v>3.92</v>
       </c>
       <c r="BP12" t="n">
-        <v>6.25</v>
+        <v>6.11</v>
       </c>
       <c r="BQ12" t="n">
-        <v>1.79</v>
+        <v>1.75</v>
       </c>
       <c r="BR12" t="n">
-        <v>6.5</v>
+        <v>6.47</v>
       </c>
       <c r="BS12" t="n">
         <v>0.09</v>
       </c>
       <c r="BT12" t="n">
-        <v>1637133</v>
+        <v>1724353</v>
       </c>
     </row>
     <row r="13">
@@ -3347,13 +3347,13 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>34.8</v>
+        <v>34.71</v>
       </c>
       <c r="G13" t="n">
-        <v>17545842935</v>
+        <v>17500469148</v>
       </c>
       <c r="H13" t="n">
-        <v>6433900</v>
+        <v>7036100</v>
       </c>
       <c r="I13" t="n">
         <v>504190947</v>
@@ -3368,7 +3368,7 @@
         <v>1.13</v>
       </c>
       <c r="M13" t="n">
-        <v>6.06836686872727</v>
+        <v>6.052673989977612</v>
       </c>
       <c r="N13" t="n">
         <v>0.57</v>
@@ -3446,7 +3446,7 @@
         <v>932753251.95</v>
       </c>
       <c r="AM13" t="n">
-        <v>1825790107.700312</v>
+        <v>1821068589.802289</v>
       </c>
       <c r="AN13" t="n">
         <v>2.6301</v>
@@ -3487,7 +3487,7 @@
         <v>26.6</v>
       </c>
       <c r="AZ13" t="n">
-        <v>62.99</v>
+        <v>62.83</v>
       </c>
       <c r="BA13" t="n">
         <v>2.6</v>
@@ -3496,19 +3496,19 @@
         <v>8.69</v>
       </c>
       <c r="BC13" t="n">
-        <v>-6.4</v>
+        <v>-6.16</v>
       </c>
       <c r="BD13" t="n">
-        <v>-23.57</v>
+        <v>-23.38</v>
       </c>
       <c r="BE13" t="n">
         <v>81</v>
       </c>
       <c r="BF13" t="n">
-        <v>-92.52</v>
+        <v>-92.5</v>
       </c>
       <c r="BG13" t="n">
-        <v>-75.02</v>
+        <v>-74.95</v>
       </c>
       <c r="BH13" t="n">
         <v>25.49</v>
@@ -3517,7 +3517,7 @@
         <v>0</v>
       </c>
       <c r="BJ13" t="n">
-        <v>34.8</v>
+        <v>34.71</v>
       </c>
       <c r="BK13" t="n">
         <v>1.85</v>
@@ -3526,7 +3526,7 @@
         <v>1.96</v>
       </c>
       <c r="BM13" t="n">
-        <v>35.6</v>
+        <v>34.94</v>
       </c>
       <c r="BN13" t="n">
         <v>36.1</v>
@@ -3535,19 +3535,19 @@
         <v>20.85</v>
       </c>
       <c r="BP13" t="n">
-        <v>34.64</v>
+        <v>33.76</v>
       </c>
       <c r="BQ13" t="n">
-        <v>17.78</v>
+        <v>17.73</v>
       </c>
       <c r="BR13" t="n">
-        <v>35.6</v>
+        <v>34.27</v>
       </c>
       <c r="BS13" t="n">
         <v>5.01</v>
       </c>
       <c r="BT13" t="n">
-        <v>6800837</v>
+        <v>6937150</v>
       </c>
     </row>
     <row r="14">
@@ -3577,13 +3577,13 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>12.2</v>
+        <v>12.5</v>
       </c>
       <c r="G14" t="n">
-        <v>10143177540</v>
+        <v>10298187816</v>
       </c>
       <c r="H14" t="n">
-        <v>19900</v>
+        <v>14600</v>
       </c>
       <c r="I14" t="n">
         <v>339510689</v>
@@ -3598,7 +3598,7 @@
         <v>1.92</v>
       </c>
       <c r="M14" t="n">
-        <v>4.211627636809002</v>
+        <v>4.275990659127843</v>
       </c>
       <c r="N14" t="n">
         <v>1.11</v>
@@ -3676,7 +3676,7 @@
         <v>349696009.67</v>
       </c>
       <c r="AM14" t="n">
-        <v>1125768872.36404</v>
+        <v>1142973120.532741</v>
       </c>
       <c r="AN14" t="n">
         <v>0.1489</v>
@@ -3717,7 +3717,7 @@
         <v>9.050000000000001</v>
       </c>
       <c r="AZ14" t="n">
-        <v>9.800000000000001</v>
+        <v>10.04</v>
       </c>
       <c r="BA14" t="n">
         <v>1.42</v>
@@ -3726,19 +3726,19 @@
         <v>5.94</v>
       </c>
       <c r="BC14" t="n">
-        <v>-9.16</v>
+        <v>-11.34</v>
       </c>
       <c r="BD14" t="n">
-        <v>-25.83</v>
+        <v>-27.61</v>
       </c>
       <c r="BE14" t="n">
         <v>-19.67</v>
       </c>
       <c r="BF14" t="n">
-        <v>-88.34999999999999</v>
+        <v>-88.63</v>
       </c>
       <c r="BG14" t="n">
-        <v>-51.29</v>
+        <v>-52.46</v>
       </c>
       <c r="BH14" t="n">
         <v>5.3</v>
@@ -3747,7 +3747,7 @@
         <v>0</v>
       </c>
       <c r="BJ14" t="n">
-        <v>12.2</v>
+        <v>12.5</v>
       </c>
       <c r="BK14" t="n">
         <v>1.03</v>
@@ -3756,28 +3756,28 @@
         <v>1.01</v>
       </c>
       <c r="BM14" t="n">
-        <v>12.55</v>
+        <v>12.58</v>
       </c>
       <c r="BN14" t="n">
         <v>13.49</v>
       </c>
       <c r="BO14" t="n">
-        <v>7.81</v>
+        <v>7.92</v>
       </c>
       <c r="BP14" t="n">
-        <v>11.97</v>
+        <v>12.03</v>
       </c>
       <c r="BQ14" t="n">
-        <v>12.04</v>
+        <v>12.34</v>
       </c>
       <c r="BR14" t="n">
-        <v>11.97</v>
+        <v>12.2</v>
       </c>
       <c r="BS14" t="n">
         <v>1.44</v>
       </c>
       <c r="BT14" t="n">
-        <v>12397</v>
+        <v>12947</v>
       </c>
     </row>
     <row r="15">
@@ -3807,13 +3807,13 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>17.36</v>
+        <v>17.69</v>
       </c>
       <c r="G15" t="n">
-        <v>10143177540</v>
+        <v>10298187816</v>
       </c>
       <c r="H15" t="n">
-        <v>6142200</v>
+        <v>5280400</v>
       </c>
       <c r="I15" t="n">
         <v>343551533</v>
@@ -3828,7 +3828,7 @@
         <v>2.56</v>
       </c>
       <c r="M15" t="n">
-        <v>4.162090584484354</v>
+        <v>4.225696570645366</v>
       </c>
       <c r="N15" t="n">
         <v>1.47</v>
@@ -3906,7 +3906,7 @@
         <v>353858078.99</v>
       </c>
       <c r="AM15" t="n">
-        <v>845969769.8081734</v>
+        <v>858898066.3886572</v>
       </c>
       <c r="AN15" t="n">
         <v>0.1638</v>
@@ -3947,7 +3947,7 @@
         <v>9.050000000000001</v>
       </c>
       <c r="AZ15" t="n">
-        <v>11.54</v>
+        <v>11.76</v>
       </c>
       <c r="BA15" t="n">
         <v>1.42</v>
@@ -3956,19 +3956,19 @@
         <v>6.19</v>
       </c>
       <c r="BC15" t="n">
-        <v>-36.16</v>
+        <v>-37.35</v>
       </c>
       <c r="BD15" t="n">
-        <v>-47.87</v>
+        <v>-48.85</v>
       </c>
       <c r="BE15" t="n">
         <v>-33.5</v>
       </c>
       <c r="BF15" t="n">
-        <v>-91.81</v>
+        <v>-91.97</v>
       </c>
       <c r="BG15" t="n">
-        <v>-64.34999999999999</v>
+        <v>-65.02</v>
       </c>
       <c r="BH15" t="n">
         <v>5.3</v>
@@ -3977,7 +3977,7 @@
         <v>0</v>
       </c>
       <c r="BJ15" t="n">
-        <v>17.36</v>
+        <v>17.69</v>
       </c>
       <c r="BK15" t="n">
         <v>1.03</v>
@@ -3986,28 +3986,28 @@
         <v>1.01</v>
       </c>
       <c r="BM15" t="n">
-        <v>17.36</v>
+        <v>17.8</v>
       </c>
       <c r="BN15" t="n">
-        <v>17.36</v>
+        <v>17.8</v>
       </c>
       <c r="BO15" t="n">
         <v>7.97</v>
       </c>
       <c r="BP15" t="n">
-        <v>16.34</v>
+        <v>16.87</v>
       </c>
       <c r="BQ15" t="n">
-        <v>17.14</v>
+        <v>17.46</v>
       </c>
       <c r="BR15" t="n">
-        <v>16.72</v>
+        <v>17.21</v>
       </c>
       <c r="BS15" t="n">
         <v>1.92</v>
       </c>
       <c r="BT15" t="n">
-        <v>2734313</v>
+        <v>2822340</v>
       </c>
     </row>
     <row r="16">
@@ -4037,13 +4037,13 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>5.65</v>
+        <v>5.55</v>
       </c>
       <c r="G16" t="n">
-        <v>1239077225</v>
+        <v>1217146121</v>
       </c>
       <c r="H16" t="n">
-        <v>275800</v>
+        <v>214600</v>
       </c>
       <c r="I16" t="n">
         <v>219305733</v>
@@ -4058,7 +4058,7 @@
         <v>2.69</v>
       </c>
       <c r="M16" t="n">
-        <v>0.5861874212551935</v>
+        <v>0.5758121701895955</v>
       </c>
       <c r="N16" t="n">
         <v>0.39</v>
@@ -4136,7 +4136,7 @@
         <v>17544458.64</v>
       </c>
       <c r="AM16" t="n">
-        <v>348055400.2808989</v>
+        <v>341894977.8089887</v>
       </c>
       <c r="AN16" t="n">
         <v>0.0077</v>
@@ -4186,16 +4186,16 @@
         <v>0</v>
       </c>
       <c r="BC16" t="n">
-        <v>-69.22</v>
+        <v>-68.67</v>
       </c>
       <c r="BD16" t="n">
-        <v>-74.87</v>
+        <v>-74.42</v>
       </c>
       <c r="BE16" t="n">
         <v>-97.17</v>
       </c>
       <c r="BF16" t="n">
-        <v>-98.58</v>
+        <v>-98.56</v>
       </c>
       <c r="BG16" t="n">
         <v>-100</v>
@@ -4207,7 +4207,7 @@
         <v>0</v>
       </c>
       <c r="BJ16" t="n">
-        <v>5.65</v>
+        <v>5.55</v>
       </c>
       <c r="BK16" t="n">
         <v>0.08</v>
@@ -4216,7 +4216,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="BM16" t="n">
-        <v>6.06</v>
+        <v>5.64</v>
       </c>
       <c r="BN16" t="n">
         <v>6.06</v>
@@ -4225,19 +4225,19 @@
         <v>3.31</v>
       </c>
       <c r="BP16" t="n">
-        <v>5.41</v>
+        <v>5.26</v>
       </c>
       <c r="BQ16" t="n">
-        <v>77.09999999999999</v>
+        <v>75.73999999999999</v>
       </c>
       <c r="BR16" t="n">
-        <v>6.06</v>
+        <v>5.56</v>
       </c>
       <c r="BS16" t="n">
         <v>0.49</v>
       </c>
       <c r="BT16" t="n">
-        <v>144287</v>
+        <v>149017</v>
       </c>
     </row>
     <row r="17">
@@ -4267,13 +4267,13 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>39.65</v>
+        <v>39.08</v>
       </c>
       <c r="G17" t="n">
-        <v>13069703122</v>
+        <v>12881819855</v>
       </c>
       <c r="H17" t="n">
-        <v>1352700</v>
+        <v>1896600</v>
       </c>
       <c r="I17" t="n">
         <v>0</v>
@@ -4360,13 +4360,13 @@
         <v>8.039999999999999</v>
       </c>
       <c r="AK17" t="n">
-        <v>5902141944.544798</v>
+        <v>5817295816.022399</v>
       </c>
       <c r="AL17" t="n">
-        <v>1633712890.25</v>
+        <v>1610227481.875</v>
       </c>
       <c r="AM17" t="n">
-        <v>4046347715.789474</v>
+        <v>3988179521.671827</v>
       </c>
       <c r="AN17" t="n">
         <v>1.08</v>
@@ -4407,7 +4407,7 @@
         <v>42.98</v>
       </c>
       <c r="AZ17" t="n">
-        <v>21.21</v>
+        <v>20.91</v>
       </c>
       <c r="BA17" t="n">
         <v>4.55</v>
@@ -4416,19 +4416,19 @@
         <v>16.33</v>
       </c>
       <c r="BC17" t="n">
-        <v>32.76</v>
+        <v>34.69</v>
       </c>
       <c r="BD17" t="n">
-        <v>8.390000000000001</v>
+        <v>9.98</v>
       </c>
       <c r="BE17" t="n">
         <v>-46.5</v>
       </c>
       <c r="BF17" t="n">
-        <v>-88.53</v>
+        <v>-88.36</v>
       </c>
       <c r="BG17" t="n">
-        <v>-58.81</v>
+        <v>-58.21</v>
       </c>
       <c r="BH17" t="n">
         <v>29.25</v>
@@ -4437,7 +4437,7 @@
         <v>0</v>
       </c>
       <c r="BJ17" t="n">
-        <v>39.65</v>
+        <v>39.08</v>
       </c>
       <c r="BK17" t="n">
         <v>4.21</v>
@@ -4446,7 +4446,7 @@
         <v>12.62</v>
       </c>
       <c r="BM17" t="n">
-        <v>39.99</v>
+        <v>39.65</v>
       </c>
       <c r="BN17" t="n">
         <v>40.95</v>
@@ -4455,19 +4455,19 @@
         <v>29.59</v>
       </c>
       <c r="BP17" t="n">
-        <v>39.09</v>
+        <v>38.99</v>
       </c>
       <c r="BQ17" t="n">
-        <v>3.14</v>
+        <v>3.1</v>
       </c>
       <c r="BR17" t="n">
-        <v>39.66</v>
+        <v>39.46</v>
       </c>
       <c r="BS17" t="n">
         <v>2.21</v>
       </c>
       <c r="BT17" t="n">
-        <v>1307063</v>
+        <v>1340323</v>
       </c>
     </row>
     <row r="18">
@@ -4497,13 +4497,13 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>13.74</v>
+        <v>13.86</v>
       </c>
       <c r="G18" t="n">
-        <v>13069703122</v>
+        <v>12881819855</v>
       </c>
       <c r="H18" t="n">
-        <v>5200</v>
+        <v>3500</v>
       </c>
       <c r="I18" t="n">
         <v>671494278</v>
@@ -4518,7 +4518,7 @@
         <v>1.2</v>
       </c>
       <c r="M18" t="n">
-        <v>3.848233859803642</v>
+        <v>3.792913647629665</v>
       </c>
       <c r="N18" t="n">
         <v>0.33</v>
@@ -4596,7 +4596,7 @@
         <v>940091989.1999999</v>
       </c>
       <c r="AM18" t="n">
-        <v>3889792595.833333</v>
+        <v>3833874956.845238</v>
       </c>
       <c r="AN18" t="n">
         <v>0.36</v>
@@ -4637,7 +4637,7 @@
         <v>14.31</v>
       </c>
       <c r="AZ18" t="n">
-        <v>7.08</v>
+        <v>7.14</v>
       </c>
       <c r="BA18" t="n">
         <v>1.51</v>
@@ -4646,19 +4646,19 @@
         <v>5.44</v>
       </c>
       <c r="BC18" t="n">
-        <v>27.55</v>
+        <v>26.44</v>
       </c>
       <c r="BD18" t="n">
-        <v>4.14</v>
+        <v>3.24</v>
       </c>
       <c r="BE18" t="n">
         <v>-48.5</v>
       </c>
       <c r="BF18" t="n">
-        <v>-88.98999999999999</v>
+        <v>-89.09</v>
       </c>
       <c r="BG18" t="n">
-        <v>-60.38</v>
+        <v>-60.72</v>
       </c>
       <c r="BH18" t="n">
         <v>9.75</v>
@@ -4667,7 +4667,7 @@
         <v>0</v>
       </c>
       <c r="BJ18" t="n">
-        <v>13.74</v>
+        <v>13.86</v>
       </c>
       <c r="BK18" t="n">
         <v>1.4</v>
@@ -4676,7 +4676,7 @@
         <v>12.62</v>
       </c>
       <c r="BM18" t="n">
-        <v>14.19</v>
+        <v>13.87</v>
       </c>
       <c r="BN18" t="n">
         <v>14.62</v>
@@ -4685,19 +4685,19 @@
         <v>10.19</v>
       </c>
       <c r="BP18" t="n">
-        <v>13.62</v>
+        <v>13.63</v>
       </c>
       <c r="BQ18" t="n">
-        <v>1.09</v>
+        <v>1.1</v>
       </c>
       <c r="BR18" t="n">
-        <v>14.19</v>
+        <v>13.74</v>
       </c>
       <c r="BS18" t="n">
         <v>2.3</v>
       </c>
       <c r="BT18" t="n">
-        <v>7873</v>
+        <v>7753</v>
       </c>
     </row>
     <row r="19">
@@ -4727,13 +4727,13 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>12.7</v>
+        <v>12.84</v>
       </c>
       <c r="G19" t="n">
-        <v>13069703122</v>
+        <v>12881819855</v>
       </c>
       <c r="H19" t="n">
-        <v>5800</v>
+        <v>9500</v>
       </c>
       <c r="I19" t="n">
         <v>317386323</v>
@@ -4748,7 +4748,7 @@
         <v>1.12</v>
       </c>
       <c r="M19" t="n">
-        <v>8.14170879462881</v>
+        <v>8.024667815731394</v>
       </c>
       <c r="N19" t="n">
         <v>0.3</v>
@@ -4826,7 +4826,7 @@
         <v>444340852.2</v>
       </c>
       <c r="AM19" t="n">
-        <v>4149112102.222222</v>
+        <v>4089466620.634921</v>
       </c>
       <c r="AN19" t="n">
         <v>0.36</v>
@@ -4867,7 +4867,7 @@
         <v>14.31</v>
       </c>
       <c r="AZ19" t="n">
-        <v>6.98</v>
+        <v>7.06</v>
       </c>
       <c r="BA19" t="n">
         <v>1.51</v>
@@ -4876,19 +4876,19 @@
         <v>5.25</v>
       </c>
       <c r="BC19" t="n">
-        <v>37.99</v>
+        <v>36.49</v>
       </c>
       <c r="BD19" t="n">
-        <v>12.67</v>
+        <v>11.44</v>
       </c>
       <c r="BE19" t="n">
         <v>-45</v>
       </c>
       <c r="BF19" t="n">
-        <v>-88.09</v>
+        <v>-88.22</v>
       </c>
       <c r="BG19" t="n">
-        <v>-58.66</v>
+        <v>-59.11</v>
       </c>
       <c r="BH19" t="n">
         <v>9.75</v>
@@ -4897,7 +4897,7 @@
         <v>0</v>
       </c>
       <c r="BJ19" t="n">
-        <v>12.7</v>
+        <v>12.84</v>
       </c>
       <c r="BK19" t="n">
         <v>1.4</v>
@@ -4906,7 +4906,7 @@
         <v>12.62</v>
       </c>
       <c r="BM19" t="n">
-        <v>12.9</v>
+        <v>12.95</v>
       </c>
       <c r="BN19" t="n">
         <v>13.26</v>
@@ -4915,13 +4915,13 @@
         <v>9.279999999999999</v>
       </c>
       <c r="BP19" t="n">
-        <v>12.6</v>
+        <v>12.64</v>
       </c>
       <c r="BQ19" t="n">
-        <v>1.01</v>
+        <v>1.02</v>
       </c>
       <c r="BR19" t="n">
-        <v>12.6</v>
+        <v>12.7</v>
       </c>
       <c r="BS19" t="n">
         <v>2.16</v>
@@ -5417,13 +5417,13 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>6.4</v>
+        <v>5.71</v>
       </c>
       <c r="G22" t="n">
-        <v>1281569939</v>
+        <v>1143400670</v>
       </c>
       <c r="H22" t="n">
-        <v>1365200</v>
+        <v>2926800</v>
       </c>
       <c r="I22" t="n">
         <v>200245299</v>
@@ -5438,7 +5438,7 @@
         <v>0.27</v>
       </c>
       <c r="M22" t="n">
-        <v>0.1086984148527545</v>
+        <v>0.09697936615738417</v>
       </c>
       <c r="N22" t="n">
         <v>0.08</v>
@@ -5516,7 +5516,7 @@
         <v>378463615.11</v>
       </c>
       <c r="AM22" t="n">
-        <v>290605428.3446712</v>
+        <v>259274528.3446712</v>
       </c>
       <c r="AN22" t="n">
         <v>0</v>
@@ -5566,19 +5566,19 @@
         <v>172.49</v>
       </c>
       <c r="BC22" t="n">
-        <v>364.14</v>
+        <v>420.23</v>
       </c>
       <c r="BD22" t="n">
-        <v>278.97</v>
+        <v>324.77</v>
       </c>
       <c r="BE22" t="n">
         <v>-100</v>
       </c>
       <c r="BF22" t="n">
-        <v>-70.47</v>
+        <v>-66.90000000000001</v>
       </c>
       <c r="BG22" t="n">
-        <v>2595.15</v>
+        <v>2920.84</v>
       </c>
       <c r="BH22" t="n">
         <v>20.75</v>
@@ -5587,7 +5587,7 @@
         <v>0</v>
       </c>
       <c r="BJ22" t="n">
-        <v>6.4</v>
+        <v>5.71</v>
       </c>
       <c r="BK22" t="n">
         <v>1.89</v>
@@ -5596,7 +5596,7 @@
         <v>0.67</v>
       </c>
       <c r="BM22" t="n">
-        <v>6.65</v>
+        <v>6.31</v>
       </c>
       <c r="BN22" t="n">
         <v>7.89</v>
@@ -5605,19 +5605,19 @@
         <v>3.37</v>
       </c>
       <c r="BP22" t="n">
-        <v>6.36</v>
+        <v>5.71</v>
       </c>
       <c r="BQ22" t="n">
-        <v>9.529999999999999</v>
+        <v>8.5</v>
       </c>
       <c r="BR22" t="n">
-        <v>6.6</v>
+        <v>6.27</v>
       </c>
       <c r="BS22" t="n">
         <v>0.09</v>
       </c>
       <c r="BT22" t="n">
-        <v>1773507</v>
+        <v>1760240</v>
       </c>
     </row>
     <row r="23">
@@ -5877,13 +5877,13 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>5.03</v>
+        <v>5.22</v>
       </c>
       <c r="G24" t="n">
-        <v>2031460148</v>
+        <v>2108194529</v>
       </c>
       <c r="H24" t="n">
-        <v>22258800</v>
+        <v>13061000</v>
       </c>
       <c r="I24" t="n">
         <v>403868805</v>
@@ -5898,7 +5898,7 @@
         <v>0.49</v>
       </c>
       <c r="M24" t="n">
-        <v>0.4910868563317108</v>
+        <v>0.5096366890591456</v>
       </c>
       <c r="N24" t="n">
         <v>0.11</v>
@@ -5976,7 +5976,7 @@
         <v>153470145.9</v>
       </c>
       <c r="AM24" t="n">
-        <v>1830144277.477477</v>
+        <v>1899274350.45045</v>
       </c>
       <c r="AN24" t="n">
         <v>0.0813</v>
@@ -6017,7 +6017,7 @@
         <v>5.84</v>
       </c>
       <c r="AZ24" t="n">
-        <v>2.32</v>
+        <v>2.41</v>
       </c>
       <c r="BA24" t="n">
         <v>0.38</v>
@@ -6026,19 +6026,19 @@
         <v>1.46</v>
       </c>
       <c r="BC24" t="n">
-        <v>42.27</v>
+        <v>37.1</v>
       </c>
       <c r="BD24" t="n">
-        <v>16.17</v>
+        <v>11.94</v>
       </c>
       <c r="BE24" t="n">
         <v>-53.83</v>
       </c>
       <c r="BF24" t="n">
-        <v>-92.45</v>
+        <v>-92.72</v>
       </c>
       <c r="BG24" t="n">
-        <v>-71.02</v>
+        <v>-72.06999999999999</v>
       </c>
       <c r="BH24" t="n">
         <v>5.99</v>
@@ -6047,7 +6047,7 @@
         <v>0</v>
       </c>
       <c r="BJ24" t="n">
-        <v>5.03</v>
+        <v>5.22</v>
       </c>
       <c r="BK24" t="n">
         <v>0.38</v>
@@ -6056,7 +6056,7 @@
         <v>0.41</v>
       </c>
       <c r="BM24" t="n">
-        <v>5.45</v>
+        <v>5.29</v>
       </c>
       <c r="BN24" t="n">
         <v>5.45</v>
@@ -6065,19 +6065,19 @@
         <v>1.92</v>
       </c>
       <c r="BP24" t="n">
-        <v>4.97</v>
+        <v>4.71</v>
       </c>
       <c r="BQ24" t="n">
-        <v>12.36</v>
+        <v>12.82</v>
       </c>
       <c r="BR24" t="n">
-        <v>5.06</v>
+        <v>4.92</v>
       </c>
       <c r="BS24" t="n">
         <v>0.29</v>
       </c>
       <c r="BT24" t="n">
-        <v>7501063</v>
+        <v>7945810</v>
       </c>
     </row>
     <row r="25">
@@ -6107,13 +6107,13 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>6.05</v>
+        <v>6.04</v>
       </c>
       <c r="G25" t="n">
-        <v>2096289371</v>
+        <v>2092823746</v>
       </c>
       <c r="H25" t="n">
-        <v>1601000</v>
+        <v>1260400</v>
       </c>
       <c r="I25" t="n">
         <v>346494097</v>
@@ -6128,7 +6128,7 @@
         <v>0.97</v>
       </c>
       <c r="M25" t="n">
-        <v>1.045305597516588</v>
+        <v>1.043577478650219</v>
       </c>
       <c r="N25" t="n">
         <v>0.22</v>
@@ -6206,7 +6206,7 @@
         <v>62368937.46</v>
       </c>
       <c r="AM25" t="n">
-        <v>770694621.6911764</v>
+        <v>769420494.8529412</v>
       </c>
       <c r="AN25" t="n">
         <v>0.4742</v>
@@ -6247,7 +6247,7 @@
         <v>3.27</v>
       </c>
       <c r="AZ25" t="n">
-        <v>14.1</v>
+        <v>14.07</v>
       </c>
       <c r="BA25" t="n">
         <v>0.23</v>
@@ -6256,19 +6256,19 @@
         <v>2.2</v>
       </c>
       <c r="BC25" t="n">
-        <v>-33.72</v>
+        <v>-33.61</v>
       </c>
       <c r="BD25" t="n">
-        <v>-45.88</v>
+        <v>-45.79</v>
       </c>
       <c r="BE25" t="n">
         <v>133</v>
       </c>
       <c r="BF25" t="n">
-        <v>-96.17</v>
+        <v>-96.16</v>
       </c>
       <c r="BG25" t="n">
-        <v>-63.64</v>
+        <v>-63.58</v>
       </c>
       <c r="BH25" t="n">
         <v>3.97</v>
@@ -6277,7 +6277,7 @@
         <v>0</v>
       </c>
       <c r="BJ25" t="n">
-        <v>6.05</v>
+        <v>6.04</v>
       </c>
       <c r="BK25" t="n">
         <v>0.18</v>
@@ -6286,7 +6286,7 @@
         <v>0.24</v>
       </c>
       <c r="BM25" t="n">
-        <v>6.52</v>
+        <v>6.15</v>
       </c>
       <c r="BN25" t="n">
         <v>6.79</v>
@@ -6295,19 +6295,19 @@
         <v>2.64</v>
       </c>
       <c r="BP25" t="n">
-        <v>5.97</v>
+        <v>5.7</v>
       </c>
       <c r="BQ25" t="n">
-        <v>25.57</v>
+        <v>25.52</v>
       </c>
       <c r="BR25" t="n">
-        <v>6.49</v>
+        <v>5.82</v>
       </c>
       <c r="BS25" t="n">
         <v>0.67</v>
       </c>
       <c r="BT25" t="n">
-        <v>1417033</v>
+        <v>1456860</v>
       </c>
     </row>
     <row r="26">
@@ -6337,13 +6337,13 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>12.64</v>
+        <v>12.72</v>
       </c>
       <c r="G26" t="n">
-        <v>17119527984</v>
+        <v>17227879321</v>
       </c>
       <c r="H26" t="n">
-        <v>17064100</v>
+        <v>18266900</v>
       </c>
       <c r="I26" t="n">
         <v>1354393401</v>
@@ -6358,7 +6358,7 @@
         <v>1.94</v>
       </c>
       <c r="M26" t="n">
-        <v>0.2207548702010202</v>
+        <v>0.2221520515577665</v>
       </c>
       <c r="N26" t="n">
         <v>0.26</v>
@@ -6436,7 +6436,7 @@
         <v>961619314.7099999</v>
       </c>
       <c r="AM26" t="n">
-        <v>6114117137.142858</v>
+        <v>6152814043.214286</v>
       </c>
       <c r="AN26" t="n">
         <v>0.1043</v>
@@ -6477,7 +6477,7 @@
         <v>7.07</v>
       </c>
       <c r="AZ26" t="n">
-        <v>2.42</v>
+        <v>2.44</v>
       </c>
       <c r="BA26" t="n">
         <v>0.66</v>
@@ -6486,19 +6486,19 @@
         <v>1.19</v>
       </c>
       <c r="BC26" t="n">
-        <v>-31.52</v>
+        <v>-31.95</v>
       </c>
       <c r="BD26" t="n">
-        <v>-44.09</v>
+        <v>-44.44</v>
       </c>
       <c r="BE26" t="n">
         <v>-80.83</v>
       </c>
       <c r="BF26" t="n">
-        <v>-94.78</v>
+        <v>-94.81999999999999</v>
       </c>
       <c r="BG26" t="n">
-        <v>-90.56</v>
+        <v>-90.62</v>
       </c>
       <c r="BH26" t="n">
         <v>4.69</v>
@@ -6507,7 +6507,7 @@
         <v>0</v>
       </c>
       <c r="BJ26" t="n">
-        <v>12.64</v>
+        <v>12.72</v>
       </c>
       <c r="BK26" t="n">
         <v>0.71</v>
@@ -6516,7 +6516,7 @@
         <v>0.72</v>
       </c>
       <c r="BM26" t="n">
-        <v>13.06</v>
+        <v>12.8</v>
       </c>
       <c r="BN26" t="n">
         <v>13.8</v>
@@ -6525,19 +6525,19 @@
         <v>6.91</v>
       </c>
       <c r="BP26" t="n">
-        <v>12.53</v>
+        <v>12.06</v>
       </c>
       <c r="BQ26" t="n">
-        <v>17.62</v>
+        <v>17.73</v>
       </c>
       <c r="BR26" t="n">
-        <v>13.03</v>
+        <v>12.36</v>
       </c>
       <c r="BS26" t="n">
         <v>0.16</v>
       </c>
       <c r="BT26" t="n">
-        <v>17325813</v>
+        <v>17619293</v>
       </c>
     </row>
     <row r="27">
@@ -8165,13 +8165,13 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>25.3</v>
+        <v>24.31</v>
       </c>
       <c r="G34" t="n">
-        <v>5224191782</v>
+        <v>5019766927</v>
       </c>
       <c r="H34" t="n">
-        <v>5400600</v>
+        <v>5518700</v>
       </c>
       <c r="I34" t="n">
         <v>206489813</v>
@@ -8186,7 +8186,7 @@
         <v>0.45</v>
       </c>
       <c r="M34" t="n">
-        <v>0.4592674731193702</v>
+        <v>0.4412961408030246</v>
       </c>
       <c r="N34" t="n">
         <v>0.24</v>
@@ -8264,7 +8264,7 @@
         <v>324189006.41</v>
       </c>
       <c r="AM34" t="n">
-        <v>1086110557.588358</v>
+        <v>1043610587.733888</v>
       </c>
       <c r="AN34" t="n">
         <v>0</v>
@@ -8305,7 +8305,7 @@
         <v>30.28</v>
       </c>
       <c r="AZ34" t="n">
-        <v>59.03</v>
+        <v>56.72</v>
       </c>
       <c r="BA34" t="n">
         <v>2.29</v>
@@ -8314,19 +8314,19 @@
         <v>25.26</v>
       </c>
       <c r="BC34" t="n">
-        <v>46.59</v>
+        <v>52.56</v>
       </c>
       <c r="BD34" t="n">
-        <v>19.69</v>
+        <v>24.57</v>
       </c>
       <c r="BE34" t="n">
         <v>133.33</v>
       </c>
       <c r="BF34" t="n">
-        <v>-90.93000000000001</v>
+        <v>-90.56</v>
       </c>
       <c r="BG34" t="n">
-        <v>-0.17</v>
+        <v>3.9</v>
       </c>
       <c r="BH34" t="n">
         <v>38.94</v>
@@ -8335,7 +8335,7 @@
         <v>0</v>
       </c>
       <c r="BJ34" t="n">
-        <v>25.3</v>
+        <v>24.31</v>
       </c>
       <c r="BK34" t="n">
         <v>1.57</v>
@@ -8344,7 +8344,7 @@
         <v>1.58</v>
       </c>
       <c r="BM34" t="n">
-        <v>26.21</v>
+        <v>24.93</v>
       </c>
       <c r="BN34" t="n">
         <v>28.86</v>
@@ -8353,19 +8353,19 @@
         <v>14.3</v>
       </c>
       <c r="BP34" t="n">
-        <v>24.85</v>
+        <v>23.44</v>
       </c>
       <c r="BQ34" t="n">
-        <v>16.04</v>
+        <v>15.41</v>
       </c>
       <c r="BR34" t="n">
-        <v>26</v>
+        <v>24.93</v>
       </c>
       <c r="BS34" t="n">
         <v>0.32</v>
       </c>
       <c r="BT34" t="n">
-        <v>4774720</v>
+        <v>4869843</v>
       </c>
     </row>
     <row r="35">
@@ -8395,13 +8395,13 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>22.76</v>
+        <v>22.33</v>
       </c>
       <c r="G35" t="n">
-        <v>114858363915</v>
+        <v>112688299954</v>
       </c>
       <c r="H35" t="n">
-        <v>64385800</v>
+        <v>69936900</v>
       </c>
       <c r="I35" t="n">
         <v>5046500000</v>
@@ -8416,7 +8416,7 @@
         <v>4.69</v>
       </c>
       <c r="M35" t="n">
-        <v>9.535583117507462</v>
+        <v>9.355423618755273</v>
       </c>
       <c r="N35" t="n">
         <v>1.79</v>
@@ -8494,7 +8494,7 @@
         <v>5349290000</v>
       </c>
       <c r="AM35" t="n">
-        <v>9492426769.834711</v>
+        <v>9313082640.826447</v>
       </c>
       <c r="AN35" t="n">
         <v>0.5305</v>
@@ -8535,7 +8535,7 @@
         <v>7.68</v>
       </c>
       <c r="AZ35" t="n">
-        <v>13.28</v>
+        <v>13.03</v>
       </c>
       <c r="BA35" t="n">
         <v>1.11</v>
@@ -8544,19 +8544,19 @@
         <v>9.119999999999999</v>
       </c>
       <c r="BC35" t="n">
-        <v>-58.67</v>
+        <v>-57.87</v>
       </c>
       <c r="BD35" t="n">
-        <v>-66.25</v>
+        <v>-65.59999999999999</v>
       </c>
       <c r="BE35" t="n">
         <v>-41.67</v>
       </c>
       <c r="BF35" t="n">
-        <v>-95.09999999999999</v>
+        <v>-95.01000000000001</v>
       </c>
       <c r="BG35" t="n">
-        <v>-59.94</v>
+        <v>-59.17</v>
       </c>
       <c r="BH35" t="n">
         <v>3.71</v>
@@ -8565,7 +8565,7 @@
         <v>0</v>
       </c>
       <c r="BJ35" t="n">
-        <v>22.76</v>
+        <v>22.33</v>
       </c>
       <c r="BK35" t="n">
         <v>1.06</v>
@@ -8574,7 +8574,7 @@
         <v>1.04</v>
       </c>
       <c r="BM35" t="n">
-        <v>23.26</v>
+        <v>22.35</v>
       </c>
       <c r="BN35" t="n">
         <v>24.28</v>
@@ -8583,19 +8583,19 @@
         <v>11.71</v>
       </c>
       <c r="BP35" t="n">
-        <v>22.67</v>
+        <v>21.66</v>
       </c>
       <c r="BQ35" t="n">
-        <v>21.78</v>
+        <v>21.37</v>
       </c>
       <c r="BR35" t="n">
-        <v>23.26</v>
+        <v>22.3</v>
       </c>
       <c r="BS35" t="n">
         <v>7.3</v>
       </c>
       <c r="BT35" t="n">
-        <v>51944770</v>
+        <v>53251573</v>
       </c>
     </row>
     <row r="36">
@@ -8628,10 +8628,10 @@
         <v>22</v>
       </c>
       <c r="G36" t="n">
-        <v>178849960</v>
+        <v>177987888</v>
       </c>
       <c r="H36" t="n">
-        <v>100</v>
+        <v>2500</v>
       </c>
       <c r="I36" t="n">
         <v>4900000</v>
@@ -8646,7 +8646,7 @@
         <v>1.52</v>
       </c>
       <c r="M36" t="n">
-        <v>1.741255021821716</v>
+        <v>1.732862024701829</v>
       </c>
       <c r="N36" t="n">
         <v>0.87</v>
@@ -8724,7 +8724,7 @@
         <v>11319000</v>
       </c>
       <c r="AM36" t="n">
-        <v>24634980.71625344</v>
+        <v>24516238.01652893</v>
       </c>
       <c r="AN36" t="n">
         <v>0</v>
@@ -8825,7 +8825,7 @@
         <v>1.24</v>
       </c>
       <c r="BT36" t="n">
-        <v>297</v>
+        <v>170</v>
       </c>
     </row>
     <row r="37">
@@ -8855,13 +8855,13 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>15.11</v>
+        <v>14.79</v>
       </c>
       <c r="G37" t="n">
-        <v>176289876</v>
+        <v>177987888</v>
       </c>
       <c r="H37" t="n">
-        <v>100</v>
+        <v>1300</v>
       </c>
       <c r="I37" t="n">
         <v>4900000</v>
@@ -8876,7 +8876,7 @@
         <v>0.88</v>
       </c>
       <c r="M37" t="n">
-        <v>1.716330447495362</v>
+        <v>1.732862024701829</v>
       </c>
       <c r="N37" t="n">
         <v>0.5</v>
@@ -8954,7 +8954,7 @@
         <v>11319000</v>
       </c>
       <c r="AM37" t="n">
-        <v>42174611.48325359</v>
+        <v>42580834.44976076</v>
       </c>
       <c r="AN37" t="n">
         <v>0</v>
@@ -8995,7 +8995,7 @@
         <v>24.36</v>
       </c>
       <c r="AZ37" t="n">
-        <v>67.19</v>
+        <v>65.77</v>
       </c>
       <c r="BA37" t="n">
         <v>2.44</v>
@@ -9004,19 +9004,19 @@
         <v>15.53</v>
       </c>
       <c r="BC37" t="n">
-        <v>97.47</v>
+        <v>101.75</v>
       </c>
       <c r="BD37" t="n">
-        <v>61.24</v>
+        <v>64.73</v>
       </c>
       <c r="BE37" t="n">
         <v>344.67</v>
       </c>
       <c r="BF37" t="n">
-        <v>-83.81999999999999</v>
+        <v>-83.47</v>
       </c>
       <c r="BG37" t="n">
-        <v>2.8</v>
+        <v>5.03</v>
       </c>
       <c r="BH37" t="n">
         <v>17.13</v>
@@ -9025,7 +9025,7 @@
         <v>0</v>
       </c>
       <c r="BJ37" t="n">
-        <v>15.11</v>
+        <v>14.79</v>
       </c>
       <c r="BK37" t="n">
         <v>2.31</v>
@@ -9034,7 +9034,7 @@
         <v>2.31</v>
       </c>
       <c r="BM37" t="n">
-        <v>15.11</v>
+        <v>15.89</v>
       </c>
       <c r="BN37" t="n">
         <v>20.9</v>
@@ -9043,19 +9043,19 @@
         <v>13.42</v>
       </c>
       <c r="BP37" t="n">
-        <v>15.11</v>
+        <v>14.76</v>
       </c>
       <c r="BQ37" t="n">
-        <v>6.54</v>
+        <v>6.4</v>
       </c>
       <c r="BR37" t="n">
-        <v>15.11</v>
+        <v>15.89</v>
       </c>
       <c r="BS37" t="n">
         <v>0.72</v>
       </c>
       <c r="BT37" t="n">
-        <v>1187</v>
+        <v>1190</v>
       </c>
     </row>
     <row r="38">
@@ -9315,13 +9315,13 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>76.31999999999999</v>
+        <v>75.51000000000001</v>
       </c>
       <c r="G39" t="n">
-        <v>4278370202</v>
+        <v>4232963862</v>
       </c>
       <c r="H39" t="n">
-        <v>6300</v>
+        <v>4400</v>
       </c>
       <c r="I39" t="n">
         <v>168174945</v>
@@ -9336,7 +9336,7 @@
         <v>0.53</v>
       </c>
       <c r="M39" t="n">
-        <v>0.2147554176477718</v>
+        <v>0.2124762185485451</v>
       </c>
       <c r="N39" t="n">
         <v>0.06</v>
@@ -9414,7 +9414,7 @@
         <v>2536078170.6</v>
       </c>
       <c r="AM39" t="n">
-        <v>449408634.6638656</v>
+        <v>444639061.1344538</v>
       </c>
       <c r="AN39" t="n">
         <v>11.9435</v>
@@ -9455,7 +9455,7 @@
         <v>170.24</v>
       </c>
       <c r="AZ39" t="n">
-        <v>222.98</v>
+        <v>220.62</v>
       </c>
       <c r="BA39" t="n">
         <v>19.01</v>
@@ -9464,19 +9464,19 @@
         <v>91.72</v>
       </c>
       <c r="BC39" t="n">
-        <v>173.2</v>
+        <v>176.13</v>
       </c>
       <c r="BD39" t="n">
-        <v>123.07</v>
+        <v>125.46</v>
       </c>
       <c r="BE39" t="n">
         <v>192.17</v>
       </c>
       <c r="BF39" t="n">
-        <v>-75.09</v>
+        <v>-74.81999999999999</v>
       </c>
       <c r="BG39" t="n">
-        <v>20.18</v>
+        <v>21.47</v>
       </c>
       <c r="BH39" t="n">
         <v>128.13</v>
@@ -9485,7 +9485,7 @@
         <v>0</v>
       </c>
       <c r="BJ39" t="n">
-        <v>76.31999999999999</v>
+        <v>75.51000000000001</v>
       </c>
       <c r="BK39" t="n">
         <v>15.08</v>
@@ -9494,7 +9494,7 @@
         <v>15.08</v>
       </c>
       <c r="BM39" t="n">
-        <v>78.5</v>
+        <v>76.72</v>
       </c>
       <c r="BN39" t="n">
         <v>78.62</v>
@@ -9503,19 +9503,19 @@
         <v>54.98</v>
       </c>
       <c r="BP39" t="n">
-        <v>76.3</v>
+        <v>74.5</v>
       </c>
       <c r="BQ39" t="n">
-        <v>5.06</v>
+        <v>5.01</v>
       </c>
       <c r="BR39" t="n">
-        <v>77.03</v>
+        <v>75.84999999999999</v>
       </c>
       <c r="BS39" t="n">
         <v>0.58</v>
       </c>
       <c r="BT39" t="n">
-        <v>3460</v>
+        <v>3527</v>
       </c>
     </row>
     <row r="40">
@@ -9545,13 +9545,13 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>24.25</v>
+        <v>24.19</v>
       </c>
       <c r="G40" t="n">
-        <v>138972773000</v>
+        <v>138628829140</v>
       </c>
       <c r="H40" t="n">
-        <v>29035000</v>
+        <v>46494500</v>
       </c>
       <c r="I40" t="n">
         <v>5730834040</v>
@@ -9566,7 +9566,7 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="M40" t="n">
-        <v>0.4216605919730961</v>
+        <v>0.4206170237367977</v>
       </c>
       <c r="N40" t="n">
         <v>0.05</v>
@@ -9644,7 +9644,7 @@
         <v>15358635227.2</v>
       </c>
       <c r="AM40" t="n">
-        <v>7208131379.66805</v>
+        <v>7190291967.842323</v>
       </c>
       <c r="AN40" t="n">
         <v>0.5641</v>
@@ -9685,7 +9685,7 @@
         <v>36.13</v>
       </c>
       <c r="AZ40" t="n">
-        <v>12.25</v>
+        <v>12.22</v>
       </c>
       <c r="BA40" t="n">
         <v>2.76</v>
@@ -9694,19 +9694,19 @@
         <v>27.89</v>
       </c>
       <c r="BC40" t="n">
-        <v>82.47</v>
+        <v>82.92</v>
       </c>
       <c r="BD40" t="n">
-        <v>48.98</v>
+        <v>49.35</v>
       </c>
       <c r="BE40" t="n">
         <v>-49.5</v>
       </c>
       <c r="BF40" t="n">
-        <v>-88.62</v>
+        <v>-88.59</v>
       </c>
       <c r="BG40" t="n">
-        <v>15.01</v>
+        <v>15.3</v>
       </c>
       <c r="BH40" t="n">
         <v>32.47</v>
@@ -9715,7 +9715,7 @@
         <v>0</v>
       </c>
       <c r="BJ40" t="n">
-        <v>24.25</v>
+        <v>24.19</v>
       </c>
       <c r="BK40" t="n">
         <v>2.68</v>
@@ -9724,7 +9724,7 @@
         <v>2.5</v>
       </c>
       <c r="BM40" t="n">
-        <v>24.69</v>
+        <v>24.45</v>
       </c>
       <c r="BN40" t="n">
         <v>27.36</v>
@@ -9733,19 +9733,19 @@
         <v>17.67</v>
       </c>
       <c r="BP40" t="n">
-        <v>24.12</v>
+        <v>23.5</v>
       </c>
       <c r="BQ40" t="n">
-        <v>9.710000000000001</v>
+        <v>9.68</v>
       </c>
       <c r="BR40" t="n">
-        <v>24.51</v>
+        <v>24.11</v>
       </c>
       <c r="BS40" t="n">
         <v>0.39</v>
       </c>
       <c r="BT40" t="n">
-        <v>44941167</v>
+        <v>45187290</v>
       </c>
     </row>
     <row r="41">
@@ -9775,13 +9775,13 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>18.84</v>
+        <v>18.38</v>
       </c>
       <c r="G41" t="n">
-        <v>225232427985</v>
+        <v>219680550633</v>
       </c>
       <c r="H41" t="n">
-        <v>13597300</v>
+        <v>11239900</v>
       </c>
       <c r="I41" t="n">
         <v>5606747177</v>
@@ -9796,7 +9796,7 @@
         <v>0.92</v>
       </c>
       <c r="M41" t="n">
-        <v>1.41986094300977</v>
+        <v>1.384862013756961</v>
       </c>
       <c r="N41" t="n">
         <v>0.07000000000000001</v>
@@ -9874,7 +9874,7 @@
         <v>13007653450.64</v>
       </c>
       <c r="AM41" t="n">
-        <v>34704534358.24345</v>
+        <v>33849083302.46533</v>
       </c>
       <c r="AN41" t="n">
         <v>1.6841</v>
@@ -9915,7 +9915,7 @@
         <v>24.4</v>
       </c>
       <c r="AZ41" t="n">
-        <v>28.2</v>
+        <v>27.51</v>
       </c>
       <c r="BA41" t="n">
         <v>2.53</v>
@@ -9924,28 +9924,28 @@
         <v>13.77</v>
       </c>
       <c r="BC41" t="n">
-        <v>58.63</v>
+        <v>62.6</v>
       </c>
       <c r="BD41" t="n">
-        <v>29.52</v>
+        <v>32.76</v>
       </c>
       <c r="BE41" t="n">
         <v>49.67</v>
       </c>
       <c r="BF41" t="n">
-        <v>-86.59</v>
+        <v>-86.25</v>
       </c>
       <c r="BG41" t="n">
-        <v>-26.91</v>
+        <v>-25.08</v>
       </c>
       <c r="BH41" t="n">
         <v>17.11</v>
       </c>
       <c r="BI41" t="n">
-        <v>1.44</v>
+        <v>0</v>
       </c>
       <c r="BJ41" t="n">
-        <v>18.57</v>
+        <v>18.38</v>
       </c>
       <c r="BK41" t="n">
         <v>2.32</v>
@@ -9954,28 +9954,28 @@
         <v>2.34</v>
       </c>
       <c r="BM41" t="n">
-        <v>18.85</v>
+        <v>18.51</v>
       </c>
       <c r="BN41" t="n">
         <v>20.24</v>
       </c>
       <c r="BO41" t="n">
-        <v>13.56</v>
+        <v>13.57</v>
       </c>
       <c r="BP41" t="n">
-        <v>18.56</v>
+        <v>17.94</v>
       </c>
       <c r="BQ41" t="n">
-        <v>8.06</v>
+        <v>7.86</v>
       </c>
       <c r="BR41" t="n">
-        <v>18.83</v>
+        <v>18.3</v>
       </c>
       <c r="BS41" t="n">
         <v>0.5600000000000001</v>
       </c>
       <c r="BT41" t="n">
-        <v>13878950</v>
+        <v>14206333</v>
       </c>
     </row>
     <row r="42">
@@ -10005,13 +10005,13 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>21.4</v>
+        <v>20.87</v>
       </c>
       <c r="G42" t="n">
-        <v>225232427985</v>
+        <v>219680550633</v>
       </c>
       <c r="H42" t="n">
-        <v>65583300</v>
+        <v>48274900</v>
       </c>
       <c r="I42" t="n">
         <v>5590117604</v>
@@ -10026,7 +10026,7 @@
         <v>1.05</v>
       </c>
       <c r="M42" t="n">
-        <v>1.424084768495075</v>
+        <v>1.388981723856838</v>
       </c>
       <c r="N42" t="n">
         <v>0.08</v>
@@ -10104,7 +10104,7 @@
         <v>12969072841.28</v>
       </c>
       <c r="AM42" t="n">
-        <v>30643867753.06123</v>
+        <v>29888510290.20408</v>
       </c>
       <c r="AN42" t="n">
         <v>1.8491</v>
@@ -10145,7 +10145,7 @@
         <v>24.4</v>
       </c>
       <c r="AZ42" t="n">
-        <v>30.99</v>
+        <v>30.23</v>
       </c>
       <c r="BA42" t="n">
         <v>2.53</v>
@@ -10154,28 +10154,28 @@
         <v>15.11</v>
       </c>
       <c r="BC42" t="n">
-        <v>39.65</v>
+        <v>43.2</v>
       </c>
       <c r="BD42" t="n">
-        <v>14.03</v>
+        <v>16.92</v>
       </c>
       <c r="BE42" t="n">
         <v>44.83</v>
       </c>
       <c r="BF42" t="n">
-        <v>-88.19</v>
+        <v>-87.89</v>
       </c>
       <c r="BG42" t="n">
-        <v>-29.37</v>
+        <v>-27.58</v>
       </c>
       <c r="BH42" t="n">
         <v>17.11</v>
       </c>
       <c r="BI42" t="n">
-        <v>1.39</v>
+        <v>0</v>
       </c>
       <c r="BJ42" t="n">
-        <v>21.11</v>
+        <v>20.87</v>
       </c>
       <c r="BK42" t="n">
         <v>2.32</v>
@@ -10184,7 +10184,7 @@
         <v>2.34</v>
       </c>
       <c r="BM42" t="n">
-        <v>21.49</v>
+        <v>21.02</v>
       </c>
       <c r="BN42" t="n">
         <v>23</v>
@@ -10193,19 +10193,19 @@
         <v>15.65</v>
       </c>
       <c r="BP42" t="n">
-        <v>21.11</v>
+        <v>20.48</v>
       </c>
       <c r="BQ42" t="n">
-        <v>9.16</v>
+        <v>8.93</v>
       </c>
       <c r="BR42" t="n">
-        <v>21.45</v>
+        <v>20.86</v>
       </c>
       <c r="BS42" t="n">
         <v>0.63</v>
       </c>
       <c r="BT42" t="n">
-        <v>58456720</v>
+        <v>59613200</v>
       </c>
     </row>
     <row r="43">
@@ -10235,13 +10235,13 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>41.18</v>
+        <v>41.68</v>
       </c>
       <c r="G43" t="n">
-        <v>79946852592</v>
+        <v>80917510912</v>
       </c>
       <c r="H43" t="n">
-        <v>7350000</v>
+        <v>8059000</v>
       </c>
       <c r="I43" t="n">
         <v>1941400000</v>
@@ -10334,7 +10334,7 @@
         <v>9182822000</v>
       </c>
       <c r="AM43" t="n">
-        <v>9737740876.004871</v>
+        <v>9855969660.414127</v>
       </c>
       <c r="AN43" t="n">
         <v>4.5901</v>
@@ -10375,7 +10375,7 @@
         <v>19.95</v>
       </c>
       <c r="AZ43" t="n">
-        <v>74.73999999999999</v>
+        <v>75.65000000000001</v>
       </c>
       <c r="BA43" t="n">
         <v>5.63</v>
@@ -10384,19 +10384,19 @@
         <v>48.62</v>
       </c>
       <c r="BC43" t="n">
-        <v>-40.66</v>
+        <v>-41.38</v>
       </c>
       <c r="BD43" t="n">
-        <v>-51.55</v>
+        <v>-52.13</v>
       </c>
       <c r="BE43" t="n">
         <v>81.5</v>
       </c>
       <c r="BF43" t="n">
-        <v>-86.33</v>
+        <v>-86.5</v>
       </c>
       <c r="BG43" t="n">
-        <v>18.06</v>
+        <v>16.64</v>
       </c>
       <c r="BH43" t="n">
         <v>5.61</v>
@@ -10405,7 +10405,7 @@
         <v>0</v>
       </c>
       <c r="BJ43" t="n">
-        <v>41.18</v>
+        <v>41.68</v>
       </c>
       <c r="BK43" t="n">
         <v>4.73</v>
@@ -10414,7 +10414,7 @@
         <v>4.73</v>
       </c>
       <c r="BM43" t="n">
-        <v>41.29</v>
+        <v>41.83</v>
       </c>
       <c r="BN43" t="n">
         <v>42.98</v>
@@ -10423,19 +10423,19 @@
         <v>28.06</v>
       </c>
       <c r="BP43" t="n">
-        <v>40.07</v>
+        <v>40.56</v>
       </c>
       <c r="BQ43" t="n">
-        <v>8.699999999999999</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="BR43" t="n">
-        <v>40.6</v>
+        <v>41.49</v>
       </c>
       <c r="BS43" t="n">
         <v>0</v>
       </c>
       <c r="BT43" t="n">
-        <v>7031567</v>
+        <v>7106710</v>
       </c>
     </row>
     <row r="44">
@@ -10925,13 +10925,13 @@
         </is>
       </c>
       <c r="F46" t="n">
-        <v>4.36</v>
+        <v>4.18</v>
       </c>
       <c r="G46" t="n">
-        <v>4362363253</v>
+        <v>4182265388</v>
       </c>
       <c r="H46" t="n">
-        <v>22976000</v>
+        <v>29495100</v>
       </c>
       <c r="I46" t="n">
         <v>1000542188</v>
@@ -10946,7 +10946,7 @@
         <v>2.5</v>
       </c>
       <c r="M46" t="n">
-        <v>0.07582607502073231</v>
+        <v>0.072695635524853</v>
       </c>
       <c r="N46" t="n">
         <v>0.08</v>
@@ -11024,7 +11024,7 @@
         <v>460249406.48</v>
       </c>
       <c r="AM46" t="n">
-        <v>4276826718.627451</v>
+        <v>4100260184.313725</v>
       </c>
       <c r="AN46" t="n">
         <v>0.0311</v>
@@ -11065,7 +11065,7 @@
         <v>3.3</v>
       </c>
       <c r="AZ46" t="n">
-        <v>3.6</v>
+        <v>3.45</v>
       </c>
       <c r="BA46" t="n">
         <v>0.42</v>
@@ -11074,19 +11074,19 @@
         <v>7.38</v>
       </c>
       <c r="BC46" t="n">
-        <v>-7.25</v>
+        <v>-3.26</v>
       </c>
       <c r="BD46" t="n">
-        <v>-24.27</v>
+        <v>-21.01</v>
       </c>
       <c r="BE46" t="n">
         <v>-17.5</v>
       </c>
       <c r="BF46" t="n">
-        <v>-90.3</v>
+        <v>-89.88</v>
       </c>
       <c r="BG46" t="n">
-        <v>69.23</v>
+        <v>76.52</v>
       </c>
       <c r="BH46" t="n">
         <v>1.58</v>
@@ -11095,7 +11095,7 @@
         <v>0</v>
       </c>
       <c r="BJ46" t="n">
-        <v>4.36</v>
+        <v>4.18</v>
       </c>
       <c r="BK46" t="n">
         <v>0.46</v>
@@ -11104,7 +11104,7 @@
         <v>0.46</v>
       </c>
       <c r="BM46" t="n">
-        <v>4.58</v>
+        <v>4.38</v>
       </c>
       <c r="BN46" t="n">
         <v>7.31</v>
@@ -11113,19 +11113,19 @@
         <v>2.97</v>
       </c>
       <c r="BP46" t="n">
-        <v>4.36</v>
+        <v>4.15</v>
       </c>
       <c r="BQ46" t="n">
-        <v>9.529999999999999</v>
+        <v>9.140000000000001</v>
       </c>
       <c r="BR46" t="n">
-        <v>4.53</v>
+        <v>4.35</v>
       </c>
       <c r="BS46" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="BT46" t="n">
-        <v>25110798</v>
+        <v>25600101</v>
       </c>
     </row>
     <row r="47">
@@ -11155,13 +11155,13 @@
         </is>
       </c>
       <c r="F47" t="n">
-        <v>9.77</v>
+        <v>9.57</v>
       </c>
       <c r="G47" t="n">
-        <v>3384723843</v>
+        <v>3318295952</v>
       </c>
       <c r="H47" t="n">
-        <v>8000</v>
+        <v>20500</v>
       </c>
       <c r="I47" t="n">
         <v>254106600</v>
@@ -11176,7 +11176,7 @@
         <v>1.22</v>
       </c>
       <c r="M47" t="n">
-        <v>0.7981568243074946</v>
+        <v>0.7824923633395324</v>
       </c>
       <c r="N47" t="n">
         <v>0.07000000000000001</v>
@@ -11254,7 +11254,7 @@
         <v>322715382</v>
       </c>
       <c r="AM47" t="n">
-        <v>600128340.9574468</v>
+        <v>588350346.0992908</v>
       </c>
       <c r="AN47" t="n">
         <v>0.4132</v>
@@ -11295,7 +11295,7 @@
         <v>11.74</v>
       </c>
       <c r="AZ47" t="n">
-        <v>12.83</v>
+        <v>12.57</v>
       </c>
       <c r="BA47" t="n">
         <v>1.46</v>
@@ -11304,19 +11304,19 @@
         <v>8.619999999999999</v>
       </c>
       <c r="BC47" t="n">
-        <v>47.12</v>
+        <v>50.19</v>
       </c>
       <c r="BD47" t="n">
-        <v>20.12</v>
+        <v>22.63</v>
       </c>
       <c r="BE47" t="n">
         <v>31.33</v>
       </c>
       <c r="BF47" t="n">
-        <v>-85.06999999999999</v>
+        <v>-84.76000000000001</v>
       </c>
       <c r="BG47" t="n">
-        <v>-11.77</v>
+        <v>-9.93</v>
       </c>
       <c r="BH47" t="n">
         <v>7.23</v>
@@ -11325,7 +11325,7 @@
         <v>0</v>
       </c>
       <c r="BJ47" t="n">
-        <v>9.77</v>
+        <v>9.57</v>
       </c>
       <c r="BK47" t="n">
         <v>1.27</v>
@@ -11334,7 +11334,7 @@
         <v>1.28</v>
       </c>
       <c r="BM47" t="n">
-        <v>9.869999999999999</v>
+        <v>9.6</v>
       </c>
       <c r="BN47" t="n">
         <v>9.9</v>
@@ -11343,19 +11343,19 @@
         <v>7.13</v>
       </c>
       <c r="BP47" t="n">
+        <v>9.359999999999999</v>
+      </c>
+      <c r="BQ47" t="n">
+        <v>7.46</v>
+      </c>
+      <c r="BR47" t="n">
         <v>9.6</v>
-      </c>
-      <c r="BQ47" t="n">
-        <v>7.62</v>
-      </c>
-      <c r="BR47" t="n">
-        <v>9.67</v>
       </c>
       <c r="BS47" t="n">
         <v>0.53</v>
       </c>
       <c r="BT47" t="n">
-        <v>13063</v>
+        <v>13090</v>
       </c>
     </row>
     <row r="48">
@@ -11385,13 +11385,13 @@
         </is>
       </c>
       <c r="F48" t="n">
-        <v>9.69</v>
+        <v>9.92</v>
       </c>
       <c r="G48" t="n">
-        <v>3384723843</v>
+        <v>3318295952</v>
       </c>
       <c r="H48" t="n">
-        <v>7100</v>
+        <v>6200</v>
       </c>
       <c r="I48" t="n">
         <v>93397546</v>
@@ -11406,7 +11406,7 @@
         <v>1.24</v>
       </c>
       <c r="M48" t="n">
-        <v>2.171544388238796</v>
+        <v>2.128926106625684</v>
       </c>
       <c r="N48" t="n">
         <v>0.07000000000000001</v>
@@ -11484,7 +11484,7 @@
         <v>118614883.42</v>
       </c>
       <c r="AM48" t="n">
-        <v>591734937.5874126</v>
+        <v>580121669.9300699</v>
       </c>
       <c r="AN48" t="n">
         <v>0.4132</v>
@@ -11525,7 +11525,7 @@
         <v>11.74</v>
       </c>
       <c r="AZ48" t="n">
-        <v>12.68</v>
+        <v>12.98</v>
       </c>
       <c r="BA48" t="n">
         <v>1.46</v>
@@ -11534,19 +11534,19 @@
         <v>8.24</v>
       </c>
       <c r="BC48" t="n">
-        <v>48.33</v>
+        <v>44.89</v>
       </c>
       <c r="BD48" t="n">
-        <v>21.11</v>
+        <v>18.31</v>
       </c>
       <c r="BE48" t="n">
         <v>30.83</v>
       </c>
       <c r="BF48" t="n">
-        <v>-84.95</v>
+        <v>-85.3</v>
       </c>
       <c r="BG48" t="n">
-        <v>-15</v>
+        <v>-16.97</v>
       </c>
       <c r="BH48" t="n">
         <v>7.23</v>
@@ -11555,7 +11555,7 @@
         <v>0</v>
       </c>
       <c r="BJ48" t="n">
-        <v>9.69</v>
+        <v>9.92</v>
       </c>
       <c r="BK48" t="n">
         <v>1.27</v>
@@ -11564,7 +11564,7 @@
         <v>1.28</v>
       </c>
       <c r="BM48" t="n">
-        <v>9.93</v>
+        <v>9.92</v>
       </c>
       <c r="BN48" t="n">
         <v>9.99</v>
@@ -11573,19 +11573,19 @@
         <v>7.13</v>
       </c>
       <c r="BP48" t="n">
-        <v>9.43</v>
+        <v>9.69</v>
       </c>
       <c r="BQ48" t="n">
-        <v>7.55</v>
+        <v>7.73</v>
       </c>
       <c r="BR48" t="n">
-        <v>9.5</v>
+        <v>9.720000000000001</v>
       </c>
       <c r="BS48" t="n">
         <v>0.54</v>
       </c>
       <c r="BT48" t="n">
-        <v>3053</v>
+        <v>3230</v>
       </c>
     </row>
     <row r="49">
@@ -11615,13 +11615,13 @@
         </is>
       </c>
       <c r="F49" t="n">
-        <v>48.74</v>
+        <v>49.46</v>
       </c>
       <c r="G49" t="n">
-        <v>979589100</v>
+        <v>1000266656</v>
       </c>
       <c r="H49" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="I49" t="n">
         <v>11540870</v>
@@ -11636,7 +11636,7 @@
         <v>1.09</v>
       </c>
       <c r="M49" t="n">
-        <v>0.9910376572156149</v>
+        <v>1.011956873910844</v>
       </c>
       <c r="N49" t="n">
         <v>0.08</v>
@@ -11714,7 +11714,7 @@
         <v>84709985.8</v>
       </c>
       <c r="AM49" t="n">
-        <v>244897275</v>
+        <v>250066664</v>
       </c>
       <c r="AN49" t="n">
         <v>3.3186</v>
@@ -11755,7 +11755,7 @@
         <v>68.48999999999999</v>
       </c>
       <c r="AZ49" t="n">
-        <v>58.16</v>
+        <v>59.02</v>
       </c>
       <c r="BA49" t="n">
         <v>9.210000000000001</v>
@@ -11764,19 +11764,19 @@
         <v>27.75</v>
       </c>
       <c r="BC49" t="n">
-        <v>72.09</v>
+        <v>69.59</v>
       </c>
       <c r="BD49" t="n">
-        <v>40.51</v>
+        <v>38.47</v>
       </c>
       <c r="BE49" t="n">
         <v>19.33</v>
       </c>
       <c r="BF49" t="n">
-        <v>-81.09999999999999</v>
+        <v>-81.37</v>
       </c>
       <c r="BG49" t="n">
-        <v>-43.06</v>
+        <v>-43.88</v>
       </c>
       <c r="BH49" t="n">
         <v>42.6</v>
@@ -11785,7 +11785,7 @@
         <v>0</v>
       </c>
       <c r="BJ49" t="n">
-        <v>48.74</v>
+        <v>49.46</v>
       </c>
       <c r="BK49" t="n">
         <v>7.34</v>
@@ -11794,7 +11794,7 @@
         <v>7.6</v>
       </c>
       <c r="BM49" t="n">
-        <v>48.74</v>
+        <v>49.46</v>
       </c>
       <c r="BN49" t="n">
         <v>64.2</v>
@@ -11803,19 +11803,19 @@
         <v>28.48</v>
       </c>
       <c r="BP49" t="n">
-        <v>48.74</v>
+        <v>49.46</v>
       </c>
       <c r="BQ49" t="n">
-        <v>6.41</v>
+        <v>6.51</v>
       </c>
       <c r="BR49" t="n">
-        <v>48.74</v>
+        <v>49.46</v>
       </c>
       <c r="BS49" t="n">
         <v>0.54</v>
       </c>
       <c r="BT49" t="n">
-        <v>387</v>
+        <v>390</v>
       </c>
     </row>
     <row r="50">
@@ -11845,13 +11845,13 @@
         </is>
       </c>
       <c r="F50" t="n">
-        <v>36.67</v>
+        <v>35.6</v>
       </c>
       <c r="G50" t="n">
-        <v>979589100</v>
+        <v>1000266656</v>
       </c>
       <c r="H50" t="n">
-        <v>800</v>
+        <v>1100</v>
       </c>
       <c r="I50" t="n">
         <v>11540870</v>
@@ -11866,7 +11866,7 @@
         <v>0.8</v>
       </c>
       <c r="M50" t="n">
-        <v>0.9910376572156149</v>
+        <v>1.011956873910844</v>
       </c>
       <c r="N50" t="n">
         <v>0.06</v>
@@ -11944,7 +11944,7 @@
         <v>84709985.8</v>
       </c>
       <c r="AM50" t="n">
-        <v>334330750.8532423</v>
+        <v>341387937.2013652</v>
       </c>
       <c r="AN50" t="n">
         <v>4.4983</v>
@@ -11985,7 +11985,7 @@
         <v>68.48999999999999</v>
       </c>
       <c r="AZ50" t="n">
-        <v>80.86</v>
+        <v>78.5</v>
       </c>
       <c r="BA50" t="n">
         <v>9.210000000000001</v>
@@ -11994,19 +11994,19 @@
         <v>30.53</v>
       </c>
       <c r="BC50" t="n">
-        <v>128.74</v>
+        <v>135.61</v>
       </c>
       <c r="BD50" t="n">
-        <v>86.76000000000001</v>
+        <v>92.37</v>
       </c>
       <c r="BE50" t="n">
         <v>120.5</v>
       </c>
       <c r="BF50" t="n">
-        <v>-74.87</v>
+        <v>-74.12</v>
       </c>
       <c r="BG50" t="n">
-        <v>-16.74</v>
+        <v>-14.24</v>
       </c>
       <c r="BH50" t="n">
         <v>42.6</v>
@@ -12015,7 +12015,7 @@
         <v>0</v>
       </c>
       <c r="BJ50" t="n">
-        <v>36.67</v>
+        <v>35.6</v>
       </c>
       <c r="BK50" t="n">
         <v>7.34</v>
@@ -12024,28 +12024,28 @@
         <v>7.6</v>
       </c>
       <c r="BM50" t="n">
-        <v>36.68</v>
+        <v>36.1</v>
       </c>
       <c r="BN50" t="n">
         <v>39.22</v>
       </c>
       <c r="BO50" t="n">
-        <v>24.3</v>
+        <v>24.32</v>
       </c>
       <c r="BP50" t="n">
-        <v>36.14</v>
+        <v>35.6</v>
       </c>
       <c r="BQ50" t="n">
-        <v>4.82</v>
+        <v>4.68</v>
       </c>
       <c r="BR50" t="n">
-        <v>36.14</v>
+        <v>35.6</v>
       </c>
       <c r="BS50" t="n">
         <v>0.4</v>
       </c>
       <c r="BT50" t="n">
-        <v>493</v>
+        <v>477</v>
       </c>
     </row>
     <row r="51">
@@ -12523,13 +12523,13 @@
         </is>
       </c>
       <c r="F53" t="n">
-        <v>6.61</v>
+        <v>6.31</v>
       </c>
       <c r="G53" t="n">
-        <v>904594382</v>
+        <v>863538636</v>
       </c>
       <c r="H53" t="n">
-        <v>65300</v>
+        <v>79100</v>
       </c>
       <c r="I53" t="n">
         <v>136852484</v>
@@ -12544,7 +12544,7 @@
         <v>2.79</v>
       </c>
       <c r="M53" t="n">
-        <v>2.349967569867874</v>
+        <v>2.24331239537583</v>
       </c>
       <c r="N53" t="n">
         <v>1.48</v>
@@ -12622,7 +12622,7 @@
         <v>39687220.36</v>
       </c>
       <c r="AM53" t="n">
-        <v>46082240.5501783</v>
+        <v>43990760.87620988</v>
       </c>
       <c r="AN53" t="n">
         <v>0</v>
@@ -12672,16 +12672,16 @@
         <v>0</v>
       </c>
       <c r="BC53" t="n">
-        <v>-40.38</v>
+        <v>-37.55</v>
       </c>
       <c r="BD53" t="n">
-        <v>-51.32</v>
+        <v>-49.01</v>
       </c>
       <c r="BE53" t="n">
         <v>-100</v>
       </c>
       <c r="BF53" t="n">
-        <v>-95.61</v>
+        <v>-95.40000000000001</v>
       </c>
       <c r="BG53" t="n">
         <v>-100</v>
@@ -12693,7 +12693,7 @@
         <v>0</v>
       </c>
       <c r="BJ53" t="n">
-        <v>6.61</v>
+        <v>6.31</v>
       </c>
       <c r="BK53" t="n">
         <v>0.29</v>
@@ -12702,7 +12702,7 @@
         <v>0.2</v>
       </c>
       <c r="BM53" t="n">
-        <v>7.44</v>
+        <v>6.63</v>
       </c>
       <c r="BN53" t="n">
         <v>10.29</v>
@@ -12711,19 +12711,19 @@
         <v>4.82</v>
       </c>
       <c r="BP53" t="n">
-        <v>6.61</v>
+        <v>6.31</v>
       </c>
       <c r="BQ53" t="n">
-        <v>32.47</v>
+        <v>30.99</v>
       </c>
       <c r="BR53" t="n">
-        <v>7.15</v>
+        <v>6.53</v>
       </c>
       <c r="BS53" t="n">
         <v>2.36</v>
       </c>
       <c r="BT53" t="n">
-        <v>51363</v>
+        <v>52797</v>
       </c>
     </row>
     <row r="54">
@@ -12753,13 +12753,13 @@
         </is>
       </c>
       <c r="F54" t="n">
-        <v>12.3</v>
+        <v>12.51</v>
       </c>
       <c r="G54" t="n">
-        <v>2868508874</v>
+        <v>2917483424</v>
       </c>
       <c r="H54" t="n">
-        <v>193600</v>
+        <v>418500</v>
       </c>
       <c r="I54" t="n">
         <v>233212121</v>
@@ -12774,7 +12774,7 @@
         <v>0.97</v>
       </c>
       <c r="M54" t="n">
-        <v>1.610069879715214</v>
+        <v>1.637558882291543</v>
       </c>
       <c r="N54" t="n">
         <v>0.5600000000000001</v>
@@ -12852,7 +12852,7 @@
         <v>233212121</v>
       </c>
       <c r="AM54" t="n">
-        <v>392408874.6922025</v>
+        <v>399108539.5348837</v>
       </c>
       <c r="AN54" t="n">
         <v>0.1531</v>
@@ -12893,7 +12893,7 @@
         <v>12.25</v>
       </c>
       <c r="AZ54" t="n">
-        <v>19.58</v>
+        <v>19.91</v>
       </c>
       <c r="BA54" t="n">
         <v>0.98</v>
@@ -12902,19 +12902,19 @@
         <v>6.52</v>
       </c>
       <c r="BC54" t="n">
-        <v>22.01</v>
+        <v>19.96</v>
       </c>
       <c r="BD54" t="n">
-        <v>-0.38</v>
+        <v>-2.05</v>
       </c>
       <c r="BE54" t="n">
         <v>59.17</v>
       </c>
       <c r="BF54" t="n">
-        <v>-92.01000000000001</v>
+        <v>-92.14</v>
       </c>
       <c r="BG54" t="n">
-        <v>-47.02</v>
+        <v>-47.91</v>
       </c>
       <c r="BH54" t="n">
         <v>10.01</v>
@@ -12923,7 +12923,7 @@
         <v>0</v>
       </c>
       <c r="BJ54" t="n">
-        <v>12.3</v>
+        <v>12.51</v>
       </c>
       <c r="BK54" t="n">
         <v>1</v>
@@ -12932,7 +12932,7 @@
         <v>1</v>
       </c>
       <c r="BM54" t="n">
-        <v>12.67</v>
+        <v>12.83</v>
       </c>
       <c r="BN54" t="n">
         <v>12.89</v>
@@ -12941,19 +12941,19 @@
         <v>8.220000000000001</v>
       </c>
       <c r="BP54" t="n">
-        <v>12.29</v>
+        <v>12.01</v>
       </c>
       <c r="BQ54" t="n">
-        <v>12.27</v>
+        <v>12.48</v>
       </c>
       <c r="BR54" t="n">
-        <v>12.67</v>
+        <v>12.33</v>
       </c>
       <c r="BS54" t="n">
         <v>1.26</v>
       </c>
       <c r="BT54" t="n">
-        <v>290450</v>
+        <v>292480</v>
       </c>
     </row>
     <row r="55">
@@ -12983,13 +12983,13 @@
         </is>
       </c>
       <c r="F55" t="n">
-        <v>59.83</v>
+        <v>60.2</v>
       </c>
       <c r="G55" t="n">
-        <v>6145354876</v>
+        <v>7956184874</v>
       </c>
       <c r="H55" t="n">
-        <v>4600</v>
+        <v>1600</v>
       </c>
       <c r="I55" t="n">
         <v>84052790</v>
@@ -13004,7 +13004,7 @@
         <v>2</v>
       </c>
       <c r="M55" t="n">
-        <v>0.9486655510735024</v>
+        <v>1.22820547555566</v>
       </c>
       <c r="N55" t="n">
         <v>0.16</v>
@@ -13082,7 +13082,7 @@
         <v>579123723.1</v>
       </c>
       <c r="AM55" t="n">
-        <v>309122478.6720322</v>
+        <v>400210506.7404427</v>
       </c>
       <c r="AN55" t="n">
         <v>3.1953</v>
@@ -13123,7 +13123,7 @@
         <v>51.21</v>
       </c>
       <c r="AZ55" t="n">
-        <v>62.92</v>
+        <v>63.31</v>
       </c>
       <c r="BA55" t="n">
         <v>9.380000000000001</v>
@@ -13132,19 +13132,19 @@
         <v>16.08</v>
       </c>
       <c r="BC55" t="n">
-        <v>4.82</v>
+        <v>4.18</v>
       </c>
       <c r="BD55" t="n">
-        <v>-14.42</v>
+        <v>-14.94</v>
       </c>
       <c r="BE55" t="n">
         <v>5.17</v>
       </c>
       <c r="BF55" t="n">
-        <v>-84.33</v>
+        <v>-84.42</v>
       </c>
       <c r="BG55" t="n">
-        <v>-73.13</v>
+        <v>-73.3</v>
       </c>
       <c r="BH55" t="n">
         <v>25.37</v>
@@ -13153,7 +13153,7 @@
         <v>0</v>
       </c>
       <c r="BJ55" t="n">
-        <v>59.83</v>
+        <v>60.2</v>
       </c>
       <c r="BK55" t="n">
         <v>6.89</v>
@@ -13162,7 +13162,7 @@
         <v>7.03</v>
       </c>
       <c r="BM55" t="n">
-        <v>60</v>
+        <v>60.2</v>
       </c>
       <c r="BN55" t="n">
         <v>73.67</v>
@@ -13171,19 +13171,19 @@
         <v>36.14</v>
       </c>
       <c r="BP55" t="n">
-        <v>57.55</v>
+        <v>58.35</v>
       </c>
       <c r="BQ55" t="n">
-        <v>8.51</v>
+        <v>8.56</v>
       </c>
       <c r="BR55" t="n">
-        <v>58</v>
+        <v>59.03</v>
       </c>
       <c r="BS55" t="n">
         <v>0.66</v>
       </c>
       <c r="BT55" t="n">
-        <v>6727</v>
+        <v>6847</v>
       </c>
     </row>
     <row r="56">
@@ -13213,13 +13213,13 @@
         </is>
       </c>
       <c r="F56" t="n">
-        <v>78.98999999999999</v>
+        <v>76.98999999999999</v>
       </c>
       <c r="G56" t="n">
-        <v>6145354876</v>
+        <v>7956184874</v>
       </c>
       <c r="H56" t="n">
-        <v>55700</v>
+        <v>34500</v>
       </c>
       <c r="I56" t="n">
         <v>39675836</v>
@@ -13234,7 +13234,7 @@
         <v>2.41</v>
       </c>
       <c r="M56" t="n">
-        <v>2.009736766343509</v>
+        <v>2.60193879503207</v>
       </c>
       <c r="N56" t="n">
         <v>0.19</v>
@@ -13312,7 +13312,7 @@
         <v>273366510.04</v>
       </c>
       <c r="AM56" t="n">
-        <v>255630402.4958403</v>
+        <v>330956109.5673877</v>
       </c>
       <c r="AN56" t="n">
         <v>3.5102</v>
@@ -13353,7 +13353,7 @@
         <v>51.21</v>
       </c>
       <c r="AZ56" t="n">
-        <v>75.44</v>
+        <v>73.53</v>
       </c>
       <c r="BA56" t="n">
         <v>9.380000000000001</v>
@@ -13362,19 +13362,19 @@
         <v>17.68</v>
       </c>
       <c r="BC56" t="n">
-        <v>-20.61</v>
+        <v>-18.54</v>
       </c>
       <c r="BD56" t="n">
-        <v>-35.17</v>
+        <v>-33.49</v>
       </c>
       <c r="BE56" t="n">
         <v>-4.5</v>
       </c>
       <c r="BF56" t="n">
-        <v>-88.13</v>
+        <v>-87.81999999999999</v>
       </c>
       <c r="BG56" t="n">
-        <v>-77.62</v>
+        <v>-77.04000000000001</v>
       </c>
       <c r="BH56" t="n">
         <v>25.37</v>
@@ -13383,7 +13383,7 @@
         <v>0</v>
       </c>
       <c r="BJ56" t="n">
-        <v>78.98999999999999</v>
+        <v>76.98999999999999</v>
       </c>
       <c r="BK56" t="n">
         <v>6.89</v>
@@ -13392,7 +13392,7 @@
         <v>7.03</v>
       </c>
       <c r="BM56" t="n">
-        <v>79.86</v>
+        <v>78.98</v>
       </c>
       <c r="BN56" t="n">
         <v>86.77</v>
@@ -13401,19 +13401,19 @@
         <v>46.42</v>
       </c>
       <c r="BP56" t="n">
-        <v>74.23</v>
+        <v>75.84999999999999</v>
       </c>
       <c r="BQ56" t="n">
-        <v>11.23</v>
+        <v>10.95</v>
       </c>
       <c r="BR56" t="n">
-        <v>76.11</v>
+        <v>78.98</v>
       </c>
       <c r="BS56" t="n">
         <v>0.79</v>
       </c>
       <c r="BT56" t="n">
-        <v>29900</v>
+        <v>31147</v>
       </c>
     </row>
     <row r="57">
@@ -13443,13 +13443,13 @@
         </is>
       </c>
       <c r="F57" t="n">
-        <v>7.05</v>
+        <v>6.97</v>
       </c>
       <c r="G57" t="n">
-        <v>1648698944</v>
+        <v>1629990210</v>
       </c>
       <c r="H57" t="n">
-        <v>1900200</v>
+        <v>1071800</v>
       </c>
       <c r="I57" t="n">
         <v>233858065</v>
@@ -13464,7 +13464,7 @@
         <v>0.77</v>
       </c>
       <c r="M57" t="n">
-        <v>0.4934998760038488</v>
+        <v>0.4878998494236237</v>
       </c>
       <c r="N57" t="n">
         <v>0.08</v>
@@ -13542,7 +13542,7 @@
         <v>229180903.7</v>
       </c>
       <c r="AM57" t="n">
-        <v>123313309.1997008</v>
+        <v>121914002.2438295</v>
       </c>
       <c r="AN57" t="n">
         <v>0.347</v>
@@ -13583,7 +13583,7 @@
         <v>10.72</v>
       </c>
       <c r="AZ57" t="n">
-        <v>10.75</v>
+        <v>10.63</v>
       </c>
       <c r="BA57" t="n">
         <v>1.13</v>
@@ -13592,19 +13592,19 @@
         <v>6.26</v>
       </c>
       <c r="BC57" t="n">
-        <v>86.26000000000001</v>
+        <v>88.40000000000001</v>
       </c>
       <c r="BD57" t="n">
-        <v>52.08</v>
+        <v>53.83</v>
       </c>
       <c r="BE57" t="n">
         <v>52.5</v>
       </c>
       <c r="BF57" t="n">
-        <v>-84.01000000000001</v>
+        <v>-83.81999999999999</v>
       </c>
       <c r="BG57" t="n">
-        <v>-11.15</v>
+        <v>-10.13</v>
       </c>
       <c r="BH57" t="n">
         <v>7.82</v>
@@ -13613,7 +13613,7 @@
         <v>0</v>
       </c>
       <c r="BJ57" t="n">
-        <v>7.05</v>
+        <v>6.97</v>
       </c>
       <c r="BK57" t="n">
         <v>0.98</v>
@@ -13622,19 +13622,19 @@
         <v>1.04</v>
       </c>
       <c r="BM57" t="n">
-        <v>7.09</v>
+        <v>7</v>
       </c>
       <c r="BN57" t="n">
         <v>7.09</v>
       </c>
       <c r="BO57" t="n">
-        <v>3.45</v>
+        <v>3.48</v>
       </c>
       <c r="BP57" t="n">
-        <v>6.84</v>
+        <v>6.78</v>
       </c>
       <c r="BQ57" t="n">
-        <v>6.81</v>
+        <v>6.73</v>
       </c>
       <c r="BR57" t="n">
         <v>7</v>
@@ -13643,7 +13643,7 @@
         <v>0.42</v>
       </c>
       <c r="BT57" t="n">
-        <v>1663980</v>
+        <v>1707633</v>
       </c>
     </row>
     <row r="58">
@@ -14133,13 +14133,13 @@
         </is>
       </c>
       <c r="F60" t="n">
-        <v>410</v>
+        <v>382.11</v>
       </c>
       <c r="G60" t="n">
-        <v>190914532</v>
+        <v>173764515</v>
       </c>
       <c r="H60" t="n">
-        <v>80</v>
+        <v>54</v>
       </c>
       <c r="I60" t="n">
         <v>454750</v>
@@ -14154,7 +14154,7 @@
         <v>0.83</v>
       </c>
       <c r="M60" t="n">
-        <v>14.28013824209708</v>
+        <v>12.99734111267628</v>
       </c>
       <c r="N60" t="n">
         <v>0.68</v>
@@ -14232,7 +14232,7 @@
         <v>59558607.5</v>
       </c>
       <c r="AM60" t="n">
-        <v>-27993333.13782991</v>
+        <v>-25478667.88856305</v>
       </c>
       <c r="AN60" t="n">
         <v>10.0581</v>
@@ -14273,7 +14273,7 @@
         <v>944.87</v>
       </c>
       <c r="AZ60" t="n">
-        <v>2357.5</v>
+        <v>2197.13</v>
       </c>
       <c r="BA60" t="n">
         <v>231.1</v>
@@ -14282,19 +14282,19 @@
         <v>727.97</v>
       </c>
       <c r="BC60" t="n">
-        <v>182.25</v>
+        <v>202.85</v>
       </c>
       <c r="BD60" t="n">
-        <v>130.45</v>
+        <v>147.28</v>
       </c>
       <c r="BE60" t="n">
         <v>475</v>
       </c>
       <c r="BF60" t="n">
-        <v>-43.63</v>
+        <v>-39.52</v>
       </c>
       <c r="BG60" t="n">
-        <v>77.55</v>
+        <v>90.51000000000001</v>
       </c>
       <c r="BH60" t="n">
         <v>454.44</v>
@@ -14303,7 +14303,7 @@
         <v>0</v>
       </c>
       <c r="BJ60" t="n">
-        <v>410</v>
+        <v>382.11</v>
       </c>
       <c r="BK60" t="n">
         <v>130.97</v>
@@ -14312,7 +14312,7 @@
         <v>130.97</v>
       </c>
       <c r="BM60" t="n">
-        <v>414.99</v>
+        <v>382.57</v>
       </c>
       <c r="BN60" t="n">
         <v>415</v>
@@ -14321,19 +14321,19 @@
         <v>310.74</v>
       </c>
       <c r="BP60" t="n">
-        <v>382.1</v>
+        <v>382.11</v>
       </c>
       <c r="BQ60" t="n">
-        <v>3.13</v>
+        <v>2.92</v>
       </c>
       <c r="BR60" t="n">
-        <v>414.99</v>
+        <v>382.57</v>
       </c>
       <c r="BS60" t="n">
         <v>12.82</v>
       </c>
       <c r="BT60" t="n">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="61">
@@ -14363,13 +14363,13 @@
         </is>
       </c>
       <c r="F61" t="n">
-        <v>33</v>
+        <v>32.45</v>
       </c>
       <c r="G61" t="n">
-        <v>2825076870</v>
+        <v>2777992320</v>
       </c>
       <c r="H61" t="n">
-        <v>1731200</v>
+        <v>889100</v>
       </c>
       <c r="I61" t="n">
         <v>85608392</v>
@@ -14384,7 +14384,7 @@
         <v>2.37</v>
       </c>
       <c r="M61" t="n">
-        <v>1.498235259115581</v>
+        <v>1.473264705670219</v>
       </c>
       <c r="N61" t="n">
         <v>1.1</v>
@@ -14462,7 +14462,7 @@
         <v>160087693.04</v>
       </c>
       <c r="AM61" t="n">
-        <v>221748576.9230769</v>
+        <v>218052772.3704866</v>
       </c>
       <c r="AN61" t="n">
         <v>0.38</v>
@@ -14503,7 +14503,7 @@
         <v>17.56</v>
       </c>
       <c r="AZ61" t="n">
-        <v>41.58</v>
+        <v>40.89</v>
       </c>
       <c r="BA61" t="n">
         <v>2.52</v>
@@ -14512,19 +14512,19 @@
         <v>11.76</v>
       </c>
       <c r="BC61" t="n">
-        <v>-34.84</v>
+        <v>-33.73</v>
       </c>
       <c r="BD61" t="n">
-        <v>-46.8</v>
+        <v>-45.89</v>
       </c>
       <c r="BE61" t="n">
         <v>26</v>
       </c>
       <c r="BF61" t="n">
-        <v>-92.36</v>
+        <v>-92.23</v>
       </c>
       <c r="BG61" t="n">
-        <v>-64.37</v>
+        <v>-63.77</v>
       </c>
       <c r="BH61" t="n">
         <v>10.99</v>
@@ -14533,7 +14533,7 @@
         <v>0</v>
       </c>
       <c r="BJ61" t="n">
-        <v>33</v>
+        <v>32.45</v>
       </c>
       <c r="BK61" t="n">
         <v>1.87</v>
@@ -14542,7 +14542,7 @@
         <v>1.86</v>
       </c>
       <c r="BM61" t="n">
-        <v>34.53</v>
+        <v>32.84</v>
       </c>
       <c r="BN61" t="n">
         <v>34.8</v>
@@ -14551,19 +14551,19 @@
         <v>19.35</v>
       </c>
       <c r="BP61" t="n">
-        <v>32.93</v>
+        <v>31.87</v>
       </c>
       <c r="BQ61" t="n">
-        <v>17.72</v>
+        <v>17.43</v>
       </c>
       <c r="BR61" t="n">
-        <v>34.29</v>
+        <v>32.84</v>
       </c>
       <c r="BS61" t="n">
         <v>1.19</v>
       </c>
       <c r="BT61" t="n">
-        <v>958630</v>
+        <v>1001953</v>
       </c>
     </row>
     <row r="62">
@@ -14593,13 +14593,13 @@
         </is>
       </c>
       <c r="F62" t="n">
-        <v>115.24</v>
+        <v>114.01</v>
       </c>
       <c r="G62" t="n">
-        <v>11374160000</v>
+        <v>11252758708</v>
       </c>
       <c r="H62" t="n">
-        <v>0</v>
+        <v>1100</v>
       </c>
       <c r="I62" t="n">
         <v>98699749</v>
@@ -14614,7 +14614,7 @@
         <v>0.64</v>
       </c>
       <c r="M62" t="n">
-        <v>1.06619693712433</v>
+        <v>1.054816959552946</v>
       </c>
       <c r="N62" t="n">
         <v>0.13</v>
@@ -14692,7 +14692,7 @@
         <v>2757670987.06</v>
       </c>
       <c r="AM62" t="n">
-        <v>4604923076.923077</v>
+        <v>4555772756.275303</v>
       </c>
       <c r="AN62" t="n">
         <v>6.9319</v>
@@ -14733,7 +14733,7 @@
         <v>267.2</v>
       </c>
       <c r="AZ62" t="n">
-        <v>121.77</v>
+        <v>120.47</v>
       </c>
       <c r="BA62" t="n">
         <v>34.09</v>
@@ -14742,19 +14742,19 @@
         <v>76.01000000000001</v>
       </c>
       <c r="BC62" t="n">
-        <v>183.97</v>
+        <v>187.03</v>
       </c>
       <c r="BD62" t="n">
-        <v>131.86</v>
+        <v>134.36</v>
       </c>
       <c r="BE62" t="n">
         <v>5.67</v>
       </c>
       <c r="BF62" t="n">
-        <v>-70.42</v>
+        <v>-70.09999999999999</v>
       </c>
       <c r="BG62" t="n">
-        <v>-34.04</v>
+        <v>-33.33</v>
       </c>
       <c r="BH62" t="n">
         <v>170.35</v>
@@ -14763,7 +14763,7 @@
         <v>0</v>
       </c>
       <c r="BJ62" t="n">
-        <v>115.24</v>
+        <v>114.01</v>
       </c>
       <c r="BK62" t="n">
         <v>27.94</v>
@@ -14772,28 +14772,28 @@
         <v>32.73</v>
       </c>
       <c r="BM62" t="n">
-        <v>115.24</v>
+        <v>121.5</v>
       </c>
       <c r="BN62" t="n">
         <v>122.2</v>
       </c>
       <c r="BO62" t="n">
-        <v>91.84999999999999</v>
+        <v>94.19</v>
       </c>
       <c r="BP62" t="n">
-        <v>115</v>
+        <v>114.01</v>
       </c>
       <c r="BQ62" t="n">
-        <v>3.52</v>
+        <v>3.48</v>
       </c>
       <c r="BR62" t="n">
-        <v>115</v>
+        <v>120.99</v>
       </c>
       <c r="BS62" t="n">
         <v>1.01</v>
       </c>
       <c r="BT62" t="n">
-        <v>137</v>
+        <v>123</v>
       </c>
     </row>
     <row r="63">
@@ -14826,10 +14826,10 @@
         <v>1.55</v>
       </c>
       <c r="G63" t="n">
-        <v>403790022</v>
+        <v>403790177</v>
       </c>
       <c r="H63" t="n">
-        <v>4100</v>
+        <v>3200</v>
       </c>
       <c r="I63" t="n">
         <v>122894462</v>
@@ -14844,7 +14844,7 @@
         <v>-0.22</v>
       </c>
       <c r="M63" t="n">
-        <v>0.4966408890243252</v>
+        <v>0.4966410796663263</v>
       </c>
       <c r="N63" t="n">
         <v>0.37</v>
@@ -14922,7 +14922,7 @@
         <v>31952560.12</v>
       </c>
       <c r="AM63" t="n">
-        <v>229426148.8636364</v>
+        <v>229426236.9318182</v>
       </c>
       <c r="AN63" t="n">
         <v>0</v>
@@ -15017,13 +15017,13 @@
         <v>5.94</v>
       </c>
       <c r="BR63" t="n">
-        <v>1.65</v>
+        <v>1.55</v>
       </c>
       <c r="BS63" t="n">
         <v>0.19</v>
       </c>
       <c r="BT63" t="n">
-        <v>36440</v>
+        <v>34910</v>
       </c>
     </row>
     <row r="64">
@@ -15053,13 +15053,13 @@
         </is>
       </c>
       <c r="F64" t="n">
-        <v>80.56</v>
+        <v>78.08</v>
       </c>
       <c r="G64" t="n">
-        <v>279340502574</v>
+        <v>265835780954</v>
       </c>
       <c r="H64" t="n">
-        <v>17541000</v>
+        <v>15024110</v>
       </c>
       <c r="I64" t="n">
         <v>0</v>
@@ -15146,13 +15146,13 @@
         <v>41.22</v>
       </c>
       <c r="AK64" t="n">
-        <v>80091021178.46613</v>
+        <v>76219019319.40817</v>
       </c>
       <c r="AL64" t="n">
-        <v>22329376704.55635</v>
+        <v>21249862586.251</v>
       </c>
       <c r="AM64" t="n">
-        <v>24874488207.83615</v>
+        <v>23671930628.13891</v>
       </c>
       <c r="AN64" t="n">
         <v>1.4201</v>
@@ -15193,7 +15193,7 @@
         <v>38.98</v>
       </c>
       <c r="AZ64" t="n">
-        <v>32.22</v>
+        <v>31.23</v>
       </c>
       <c r="BA64" t="n">
         <v>6.69</v>
@@ -15202,28 +15202,28 @@
         <v>10.4</v>
       </c>
       <c r="BC64" t="n">
-        <v>-40.74</v>
+        <v>-38.86</v>
       </c>
       <c r="BD64" t="n">
-        <v>-51.61</v>
+        <v>-50.08</v>
       </c>
       <c r="BE64" t="n">
         <v>-60</v>
       </c>
       <c r="BF64" t="n">
-        <v>-91.69</v>
+        <v>-91.43000000000001</v>
       </c>
       <c r="BG64" t="n">
-        <v>-87.09</v>
+        <v>-86.68000000000001</v>
       </c>
       <c r="BH64" t="n">
         <v>21.37</v>
       </c>
       <c r="BI64" t="n">
-        <v>0</v>
+        <v>-0.28</v>
       </c>
       <c r="BJ64" t="n">
-        <v>80.56</v>
+        <v>78.3</v>
       </c>
       <c r="BK64" t="n">
         <v>4.74</v>
@@ -15232,7 +15232,7 @@
         <v>1.57</v>
       </c>
       <c r="BM64" t="n">
-        <v>82</v>
+        <v>79.40000000000001</v>
       </c>
       <c r="BN64" t="n">
         <v>84.59</v>
@@ -15241,19 +15241,19 @@
         <v>44.12</v>
       </c>
       <c r="BP64" t="n">
-        <v>79.2</v>
+        <v>77.03</v>
       </c>
       <c r="BQ64" t="n">
-        <v>51.31</v>
+        <v>49.73</v>
       </c>
       <c r="BR64" t="n">
-        <v>81.08</v>
+        <v>78.7</v>
       </c>
       <c r="BS64" t="n">
         <v>3.49</v>
       </c>
       <c r="BT64" t="n">
-        <v>13684580</v>
+        <v>14027903</v>
       </c>
     </row>
     <row r="65">
@@ -15283,13 +15283,13 @@
         </is>
       </c>
       <c r="F65" t="n">
-        <v>26.7</v>
+        <v>26.53</v>
       </c>
       <c r="G65" t="n">
-        <v>279340502574</v>
+        <v>265835780954</v>
       </c>
       <c r="H65" t="n">
-        <v>49500</v>
+        <v>17200</v>
       </c>
       <c r="I65" t="n">
         <v>7298813414</v>
@@ -15304,7 +15304,7 @@
         <v>3.29</v>
       </c>
       <c r="M65" t="n">
-        <v>6.753320034831109</v>
+        <v>6.426830656309988</v>
       </c>
       <c r="N65" t="n">
         <v>0.29</v>
@@ -15382,7 +15382,7 @@
         <v>11532125194.12</v>
       </c>
       <c r="AM65" t="n">
-        <v>20924382215.2809</v>
+        <v>19912792580.82397</v>
       </c>
       <c r="AN65" t="n">
         <v>0.4734</v>
@@ -15423,7 +15423,7 @@
         <v>12.99</v>
       </c>
       <c r="AZ65" t="n">
-        <v>8.99</v>
+        <v>8.93</v>
       </c>
       <c r="BA65" t="n">
         <v>2.23</v>
@@ -15432,19 +15432,19 @@
         <v>3.47</v>
       </c>
       <c r="BC65" t="n">
-        <v>-40.41</v>
+        <v>-40.03</v>
       </c>
       <c r="BD65" t="n">
-        <v>-51.35</v>
+        <v>-51.04</v>
       </c>
       <c r="BE65" t="n">
         <v>-66.33</v>
       </c>
       <c r="BF65" t="n">
-        <v>-91.64</v>
+        <v>-91.59</v>
       </c>
       <c r="BG65" t="n">
-        <v>-87.02</v>
+        <v>-86.94</v>
       </c>
       <c r="BH65" t="n">
         <v>7.12</v>
@@ -15453,7 +15453,7 @@
         <v>0</v>
       </c>
       <c r="BJ65" t="n">
-        <v>26.7</v>
+        <v>26.53</v>
       </c>
       <c r="BK65" t="n">
         <v>1.58</v>
@@ -15462,7 +15462,7 @@
         <v>1.57</v>
       </c>
       <c r="BM65" t="n">
-        <v>29.3</v>
+        <v>26.74</v>
       </c>
       <c r="BN65" t="n">
         <v>46.43</v>
@@ -15471,19 +15471,19 @@
         <v>20.44</v>
       </c>
       <c r="BP65" t="n">
+        <v>26.1</v>
+      </c>
+      <c r="BQ65" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="BR65" t="n">
         <v>26.7</v>
-      </c>
-      <c r="BQ65" t="n">
-        <v>17.01</v>
-      </c>
-      <c r="BR65" t="n">
-        <v>27.95</v>
       </c>
       <c r="BS65" t="n">
         <v>4.14</v>
       </c>
       <c r="BT65" t="n">
-        <v>11510</v>
+        <v>13000</v>
       </c>
     </row>
     <row r="66">
@@ -15513,13 +15513,13 @@
         </is>
       </c>
       <c r="F66" t="n">
-        <v>26.7</v>
+        <v>26</v>
       </c>
       <c r="G66" t="n">
-        <v>279340502574</v>
+        <v>265835780954</v>
       </c>
       <c r="H66" t="n">
-        <v>26500</v>
+        <v>5000</v>
       </c>
       <c r="I66" t="n">
         <v>2972355254</v>
@@ -15534,7 +15534,7 @@
         <v>2.75</v>
       </c>
       <c r="M66" t="n">
-        <v>16.58322059347629</v>
+        <v>15.78150449568763</v>
       </c>
       <c r="N66" t="n">
         <v>0.25</v>
@@ -15612,7 +15612,7 @@
         <v>4696321301.320001</v>
       </c>
       <c r="AM66" t="n">
-        <v>25052959872.10762</v>
+        <v>23841774076.59193</v>
       </c>
       <c r="AN66" t="n">
         <v>0.4734</v>
@@ -15653,7 +15653,7 @@
         <v>12.99</v>
       </c>
       <c r="AZ66" t="n">
-        <v>10.72</v>
+        <v>10.44</v>
       </c>
       <c r="BA66" t="n">
         <v>2.23</v>
@@ -15662,19 +15662,19 @@
         <v>3.47</v>
       </c>
       <c r="BC66" t="n">
-        <v>-40.41</v>
+        <v>-38.81</v>
       </c>
       <c r="BD66" t="n">
-        <v>-51.35</v>
+        <v>-50.04</v>
       </c>
       <c r="BE66" t="n">
         <v>-59.83</v>
       </c>
       <c r="BF66" t="n">
-        <v>-91.64</v>
+        <v>-91.42</v>
       </c>
       <c r="BG66" t="n">
-        <v>-87.02</v>
+        <v>-86.67</v>
       </c>
       <c r="BH66" t="n">
         <v>7.12</v>
@@ -15683,7 +15683,7 @@
         <v>0</v>
       </c>
       <c r="BJ66" t="n">
-        <v>26.7</v>
+        <v>26</v>
       </c>
       <c r="BK66" t="n">
         <v>1.58</v>
@@ -15692,7 +15692,7 @@
         <v>1.57</v>
       </c>
       <c r="BM66" t="n">
-        <v>28.5</v>
+        <v>26.72</v>
       </c>
       <c r="BN66" t="n">
         <v>28.51</v>
@@ -15701,19 +15701,19 @@
         <v>9.48</v>
       </c>
       <c r="BP66" t="n">
-        <v>25.11</v>
+        <v>25.7</v>
       </c>
       <c r="BQ66" t="n">
-        <v>17.01</v>
+        <v>16.56</v>
       </c>
       <c r="BR66" t="n">
-        <v>26.2</v>
+        <v>26.71</v>
       </c>
       <c r="BS66" t="n">
         <v>3.46</v>
       </c>
       <c r="BT66" t="n">
-        <v>4857</v>
+        <v>5660</v>
       </c>
     </row>
     <row r="67">
@@ -15973,13 +15973,13 @@
         </is>
       </c>
       <c r="F68" t="n">
-        <v>18.28</v>
+        <v>17.9</v>
       </c>
       <c r="G68" t="n">
-        <v>7736577455</v>
+        <v>7631941315</v>
       </c>
       <c r="H68" t="n">
-        <v>119200</v>
+        <v>256800</v>
       </c>
       <c r="I68" t="n">
         <v>137989898</v>
@@ -16072,7 +16072,7 @@
         <v>205604948.02</v>
       </c>
       <c r="AM68" t="n">
-        <v>536517160.5409154</v>
+        <v>529260840.1525659</v>
       </c>
       <c r="AN68" t="n">
         <v>0.1911</v>
@@ -16113,7 +16113,7 @@
         <v>21.39</v>
       </c>
       <c r="AZ68" t="n">
-        <v>33.82</v>
+        <v>33.11</v>
       </c>
       <c r="BA68" t="n">
         <v>1.24</v>
@@ -16122,19 +16122,19 @@
         <v>63.25</v>
       </c>
       <c r="BC68" t="n">
-        <v>43.34</v>
+        <v>46.38</v>
       </c>
       <c r="BD68" t="n">
-        <v>17.04</v>
+        <v>19.52</v>
       </c>
       <c r="BE68" t="n">
         <v>85</v>
       </c>
       <c r="BF68" t="n">
-        <v>-93.22</v>
+        <v>-93.08</v>
       </c>
       <c r="BG68" t="n">
-        <v>246</v>
+        <v>253.34</v>
       </c>
       <c r="BH68" t="n">
         <v>20.48</v>
@@ -16143,7 +16143,7 @@
         <v>0</v>
       </c>
       <c r="BJ68" t="n">
-        <v>18.28</v>
+        <v>17.9</v>
       </c>
       <c r="BK68" t="n">
         <v>1.49</v>
@@ -16152,28 +16152,28 @@
         <v>1.49</v>
       </c>
       <c r="BM68" t="n">
-        <v>18.67</v>
+        <v>18.27</v>
       </c>
       <c r="BN68" t="n">
         <v>22.11</v>
       </c>
       <c r="BO68" t="n">
-        <v>15.57</v>
+        <v>15.6</v>
       </c>
       <c r="BP68" t="n">
+        <v>17.79</v>
+      </c>
+      <c r="BQ68" t="n">
+        <v>12.04</v>
+      </c>
+      <c r="BR68" t="n">
         <v>18.27</v>
       </c>
-      <c r="BQ68" t="n">
-        <v>12.3</v>
-      </c>
-      <c r="BR68" t="n">
-        <v>18.65</v>
-      </c>
       <c r="BS68" t="n">
         <v>0</v>
       </c>
       <c r="BT68" t="n">
-        <v>62987</v>
+        <v>65980</v>
       </c>
     </row>
     <row r="69">
@@ -16203,13 +16203,13 @@
         </is>
       </c>
       <c r="F69" t="n">
-        <v>20.4</v>
+        <v>20.15</v>
       </c>
       <c r="G69" t="n">
-        <v>7736577455</v>
+        <v>7631941315</v>
       </c>
       <c r="H69" t="n">
-        <v>3769700</v>
+        <v>4189900</v>
       </c>
       <c r="I69" t="n">
         <v>255106712</v>
@@ -16302,7 +16302,7 @@
         <v>380109000.88</v>
       </c>
       <c r="AM69" t="n">
-        <v>460510562.797619</v>
+        <v>454282221.1309524</v>
       </c>
       <c r="AN69" t="n">
         <v>0.8856000000000001</v>
@@ -16343,7 +16343,7 @@
         <v>21.39</v>
       </c>
       <c r="AZ69" t="n">
-        <v>35.67</v>
+        <v>35.23</v>
       </c>
       <c r="BA69" t="n">
         <v>1.24</v>
@@ -16352,19 +16352,19 @@
         <v>69.59</v>
       </c>
       <c r="BC69" t="n">
-        <v>28.45</v>
+        <v>30.04</v>
       </c>
       <c r="BD69" t="n">
-        <v>4.88</v>
+        <v>6.18</v>
       </c>
       <c r="BE69" t="n">
         <v>74.83</v>
       </c>
       <c r="BF69" t="n">
-        <v>-93.92</v>
+        <v>-93.84999999999999</v>
       </c>
       <c r="BG69" t="n">
-        <v>241.11</v>
+        <v>245.34</v>
       </c>
       <c r="BH69" t="n">
         <v>20.48</v>
@@ -16373,7 +16373,7 @@
         <v>0</v>
       </c>
       <c r="BJ69" t="n">
-        <v>20.4</v>
+        <v>20.15</v>
       </c>
       <c r="BK69" t="n">
         <v>1.49</v>
@@ -16382,7 +16382,7 @@
         <v>1.49</v>
       </c>
       <c r="BM69" t="n">
-        <v>20.62</v>
+        <v>20.4</v>
       </c>
       <c r="BN69" t="n">
         <v>25.63</v>
@@ -16391,19 +16391,19 @@
         <v>17.11</v>
       </c>
       <c r="BP69" t="n">
-        <v>20.25</v>
+        <v>19.88</v>
       </c>
       <c r="BQ69" t="n">
-        <v>13.72</v>
+        <v>13.55</v>
       </c>
       <c r="BR69" t="n">
-        <v>20.62</v>
+        <v>20.33</v>
       </c>
       <c r="BS69" t="n">
         <v>0</v>
       </c>
       <c r="BT69" t="n">
-        <v>3038073</v>
+        <v>3082490</v>
       </c>
     </row>
     <row r="70">
@@ -16433,13 +16433,13 @@
         </is>
       </c>
       <c r="F70" t="n">
-        <v>20.91</v>
+        <v>20.55</v>
       </c>
       <c r="G70" t="n">
-        <v>9713890981</v>
+        <v>9546650105</v>
       </c>
       <c r="H70" t="n">
-        <v>4828200</v>
+        <v>4186100</v>
       </c>
       <c r="I70" t="n">
         <v>464557268</v>
@@ -16454,7 +16454,7 @@
         <v>0.68</v>
       </c>
       <c r="M70" t="n">
-        <v>0.7666998821696762</v>
+        <v>0.7534998616862311</v>
       </c>
       <c r="N70" t="n">
         <v>0.2</v>
@@ -16532,7 +16532,7 @@
         <v>55746872.16</v>
       </c>
       <c r="AM70" t="n">
-        <v>3205904614.191419</v>
+        <v>3150709605.610561</v>
       </c>
       <c r="AN70" t="n">
         <v>0.1236</v>
@@ -16573,7 +16573,7 @@
         <v>6.9</v>
       </c>
       <c r="AZ70" t="n">
-        <v>2.4</v>
+        <v>2.36</v>
       </c>
       <c r="BA70" t="n">
         <v>0.12</v>
@@ -16582,19 +16582,19 @@
         <v>1.07</v>
       </c>
       <c r="BC70" t="n">
-        <v>-59.59</v>
+        <v>-58.88</v>
       </c>
       <c r="BD70" t="n">
-        <v>-67.01000000000001</v>
+        <v>-66.43000000000001</v>
       </c>
       <c r="BE70" t="n">
         <v>-88.5</v>
       </c>
       <c r="BF70" t="n">
-        <v>-99.43000000000001</v>
+        <v>-99.42</v>
       </c>
       <c r="BG70" t="n">
-        <v>-94.89</v>
+        <v>-94.8</v>
       </c>
       <c r="BH70" t="n">
         <v>26.44</v>
@@ -16603,7 +16603,7 @@
         <v>0</v>
       </c>
       <c r="BJ70" t="n">
-        <v>20.91</v>
+        <v>20.55</v>
       </c>
       <c r="BK70" t="n">
         <v>0.12</v>
@@ -16612,7 +16612,7 @@
         <v>0.1</v>
       </c>
       <c r="BM70" t="n">
-        <v>21.08</v>
+        <v>20.92</v>
       </c>
       <c r="BN70" t="n">
         <v>22.15</v>
@@ -16621,19 +16621,19 @@
         <v>13.21</v>
       </c>
       <c r="BP70" t="n">
-        <v>20</v>
+        <v>20.4</v>
       </c>
       <c r="BQ70" t="n">
-        <v>209.71</v>
+        <v>206.1</v>
       </c>
       <c r="BR70" t="n">
-        <v>20.5</v>
+        <v>20.8</v>
       </c>
       <c r="BS70" t="n">
         <v>0.67</v>
       </c>
       <c r="BT70" t="n">
-        <v>3823463</v>
+        <v>3882937</v>
       </c>
     </row>
     <row r="71">

</xml_diff>

<commit_message>
📊 Dados atualizados - 2026-10-16 05:19
</commit_message>
<xml_diff>
--- a/data/ativos.xlsx
+++ b/data/ativos.xlsx
@@ -1047,13 +1047,13 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>28.51</v>
+        <v>28.94</v>
       </c>
       <c r="G3" t="n">
-        <v>3813691498</v>
+        <v>3871211263</v>
       </c>
       <c r="H3" t="n">
-        <v>666900</v>
+        <v>0</v>
       </c>
       <c r="I3" t="n">
         <v>129510368</v>
@@ -1068,7 +1068,7 @@
         <v>0.88</v>
       </c>
       <c r="M3" t="n">
-        <v>0.9489313810398361</v>
+        <v>0.9632435796188668</v>
       </c>
       <c r="N3" t="n">
         <v>0.09</v>
@@ -1146,7 +1146,7 @@
         <v>506385538.88</v>
       </c>
       <c r="AM3" t="n">
-        <v>744861620.703125</v>
+        <v>756095949.8046875</v>
       </c>
       <c r="AN3" t="n">
         <v>2.7</v>
@@ -1187,7 +1187,7 @@
         <v>40.42</v>
       </c>
       <c r="AZ3" t="n">
-        <v>52.17</v>
+        <v>52.96</v>
       </c>
       <c r="BA3" t="n">
         <v>4.87</v>
@@ -1196,19 +1196,19 @@
         <v>21.14</v>
       </c>
       <c r="BC3" t="n">
-        <v>73.62</v>
+        <v>71.04000000000001</v>
       </c>
       <c r="BD3" t="n">
-        <v>41.76</v>
+        <v>39.65</v>
       </c>
       <c r="BE3" t="n">
         <v>83</v>
       </c>
       <c r="BF3" t="n">
-        <v>-82.92</v>
+        <v>-83.18000000000001</v>
       </c>
       <c r="BG3" t="n">
-        <v>-25.87</v>
+        <v>-26.97</v>
       </c>
       <c r="BH3" t="n">
         <v>27.85</v>
@@ -1217,7 +1217,7 @@
         <v>0</v>
       </c>
       <c r="BJ3" t="n">
-        <v>28.51</v>
+        <v>28.94</v>
       </c>
       <c r="BK3" t="n">
         <v>3.91</v>
@@ -1226,7 +1226,7 @@
         <v>4.39</v>
       </c>
       <c r="BM3" t="n">
-        <v>28.83</v>
+        <v>29.26</v>
       </c>
       <c r="BN3" t="n">
         <v>29.56</v>
@@ -1235,19 +1235,19 @@
         <v>18.72</v>
       </c>
       <c r="BP3" t="n">
-        <v>27.89</v>
+        <v>28.18</v>
       </c>
       <c r="BQ3" t="n">
-        <v>6.49</v>
+        <v>6.59</v>
       </c>
       <c r="BR3" t="n">
-        <v>28.72</v>
+        <v>28.27</v>
       </c>
       <c r="BS3" t="n">
         <v>0.79</v>
       </c>
       <c r="BT3" t="n">
-        <v>712993</v>
+        <v>718217</v>
       </c>
     </row>
     <row r="4">
@@ -1277,13 +1277,13 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>16.52</v>
+        <v>16.69</v>
       </c>
       <c r="G4" t="n">
-        <v>255806590288</v>
+        <v>258438983669</v>
       </c>
       <c r="H4" t="n">
-        <v>43431300</v>
+        <v>0</v>
       </c>
       <c r="I4" t="n">
         <v>15484664889</v>
@@ -1298,7 +1298,7 @@
         <v>2.76</v>
       </c>
       <c r="M4" t="n">
-        <v>2.896505832405253</v>
+        <v>2.926312503033508</v>
       </c>
       <c r="N4" t="n">
         <v>1.76</v>
@@ -1376,7 +1376,7 @@
         <v>16258898133.45</v>
       </c>
       <c r="AM4" t="n">
-        <v>25327385177.02971</v>
+        <v>25588018185.04951</v>
       </c>
       <c r="AN4" t="n">
         <v>0.269</v>
@@ -1417,7 +1417,7 @@
         <v>9.470000000000001</v>
       </c>
       <c r="AZ4" t="n">
-        <v>20.62</v>
+        <v>20.83</v>
       </c>
       <c r="BA4" t="n">
         <v>1.13</v>
@@ -1426,19 +1426,19 @@
         <v>11.39</v>
       </c>
       <c r="BC4" t="n">
-        <v>-29.76</v>
+        <v>-30.47</v>
       </c>
       <c r="BD4" t="n">
-        <v>-42.65</v>
+        <v>-43.23</v>
       </c>
       <c r="BE4" t="n">
         <v>24.83</v>
       </c>
       <c r="BF4" t="n">
-        <v>-93.18000000000001</v>
+        <v>-93.23999999999999</v>
       </c>
       <c r="BG4" t="n">
-        <v>-31.07</v>
+        <v>-31.78</v>
       </c>
       <c r="BH4" t="n">
         <v>5.7</v>
@@ -1447,7 +1447,7 @@
         <v>0</v>
       </c>
       <c r="BJ4" t="n">
-        <v>16.52</v>
+        <v>16.69</v>
       </c>
       <c r="BK4" t="n">
         <v>1.05</v>
@@ -1456,7 +1456,7 @@
         <v>1.04</v>
       </c>
       <c r="BM4" t="n">
-        <v>16.55</v>
+        <v>16.82</v>
       </c>
       <c r="BN4" t="n">
         <v>16.94</v>
@@ -1465,19 +1465,19 @@
         <v>11.26</v>
       </c>
       <c r="BP4" t="n">
-        <v>16.12</v>
+        <v>16.33</v>
       </c>
       <c r="BQ4" t="n">
-        <v>15.93</v>
+        <v>16.1</v>
       </c>
       <c r="BR4" t="n">
-        <v>16.23</v>
+        <v>16.38</v>
       </c>
       <c r="BS4" t="n">
         <v>2.76</v>
       </c>
       <c r="BT4" t="n">
-        <v>32705670</v>
+        <v>32464360</v>
       </c>
     </row>
     <row r="5">
@@ -1743,7 +1743,7 @@
         <v>441592830</v>
       </c>
       <c r="H6" t="n">
-        <v>1400</v>
+        <v>0</v>
       </c>
       <c r="I6" t="n">
         <v>63084700</v>
@@ -1916,7 +1916,7 @@
         <v>0.5600000000000001</v>
       </c>
       <c r="BM6" t="n">
-        <v>7.05</v>
+        <v>7.07</v>
       </c>
       <c r="BN6" t="n">
         <v>8.16</v>
@@ -1931,13 +1931,13 @@
         <v>12.45</v>
       </c>
       <c r="BR6" t="n">
-        <v>7.05</v>
+        <v>7.07</v>
       </c>
       <c r="BS6" t="n">
         <v>7.32</v>
       </c>
       <c r="BT6" t="n">
-        <v>683</v>
+        <v>713</v>
       </c>
     </row>
     <row r="7">
@@ -3117,13 +3117,13 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>6.35</v>
+        <v>6.3</v>
       </c>
       <c r="G12" t="n">
-        <v>609355706</v>
+        <v>604557657</v>
       </c>
       <c r="H12" t="n">
-        <v>1748400</v>
+        <v>0</v>
       </c>
       <c r="I12" t="n">
         <v>95961536</v>
@@ -3138,7 +3138,7 @@
         <v>0.32</v>
       </c>
       <c r="M12" t="n">
-        <v>0.1102010495926708</v>
+        <v>0.1093333297525335</v>
       </c>
       <c r="N12" t="n">
         <v>0.14</v>
@@ -3216,7 +3216,7 @@
         <v>362734606.08</v>
       </c>
       <c r="AM12" t="n">
-        <v>655221189.2473118</v>
+        <v>650061996.7741935</v>
       </c>
       <c r="AN12" t="n">
         <v>0.4208</v>
@@ -3257,7 +3257,7 @@
         <v>30.49</v>
       </c>
       <c r="AZ12" t="n">
-        <v>8.58</v>
+        <v>8.52</v>
       </c>
       <c r="BA12" t="n">
         <v>4.41</v>
@@ -3266,19 +3266,19 @@
         <v>18.12</v>
       </c>
       <c r="BC12" t="n">
-        <v>488.15</v>
+        <v>492.81</v>
       </c>
       <c r="BD12" t="n">
-        <v>380.22</v>
+        <v>384.03</v>
       </c>
       <c r="BE12" t="n">
         <v>35.17</v>
       </c>
       <c r="BF12" t="n">
-        <v>-30.53</v>
+        <v>-29.97</v>
       </c>
       <c r="BG12" t="n">
-        <v>185.34</v>
+        <v>187.6</v>
       </c>
       <c r="BH12" t="n">
         <v>16.4</v>
@@ -3287,7 +3287,7 @@
         <v>0</v>
       </c>
       <c r="BJ12" t="n">
-        <v>6.35</v>
+        <v>6.3</v>
       </c>
       <c r="BK12" t="n">
         <v>3.78</v>
@@ -3296,7 +3296,7 @@
         <v>3.63</v>
       </c>
       <c r="BM12" t="n">
-        <v>6.47</v>
+        <v>6.48</v>
       </c>
       <c r="BN12" t="n">
         <v>7.3</v>
@@ -3308,16 +3308,16 @@
         <v>6.11</v>
       </c>
       <c r="BQ12" t="n">
-        <v>1.75</v>
+        <v>1.73</v>
       </c>
       <c r="BR12" t="n">
-        <v>6.47</v>
+        <v>6.26</v>
       </c>
       <c r="BS12" t="n">
         <v>0.09</v>
       </c>
       <c r="BT12" t="n">
-        <v>1724353</v>
+        <v>1766893</v>
       </c>
     </row>
     <row r="13">
@@ -3347,13 +3347,13 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>34.71</v>
+        <v>34.64</v>
       </c>
       <c r="G13" t="n">
-        <v>17500469148</v>
+        <v>17465175932</v>
       </c>
       <c r="H13" t="n">
-        <v>7036100</v>
+        <v>0</v>
       </c>
       <c r="I13" t="n">
         <v>504190947</v>
@@ -3368,7 +3368,7 @@
         <v>1.13</v>
       </c>
       <c r="M13" t="n">
-        <v>6.052673989977612</v>
+        <v>6.040467555470097</v>
       </c>
       <c r="N13" t="n">
         <v>0.57</v>
@@ -3446,7 +3446,7 @@
         <v>932753251.95</v>
       </c>
       <c r="AM13" t="n">
-        <v>1821068589.802289</v>
+        <v>1817396038.709677</v>
       </c>
       <c r="AN13" t="n">
         <v>2.6301</v>
@@ -3487,7 +3487,7 @@
         <v>26.6</v>
       </c>
       <c r="AZ13" t="n">
-        <v>62.83</v>
+        <v>62.7</v>
       </c>
       <c r="BA13" t="n">
         <v>2.6</v>
@@ -3496,19 +3496,19 @@
         <v>8.69</v>
       </c>
       <c r="BC13" t="n">
-        <v>-6.16</v>
+        <v>-5.97</v>
       </c>
       <c r="BD13" t="n">
-        <v>-23.38</v>
+        <v>-23.22</v>
       </c>
       <c r="BE13" t="n">
         <v>81</v>
       </c>
       <c r="BF13" t="n">
-        <v>-92.5</v>
+        <v>-92.48</v>
       </c>
       <c r="BG13" t="n">
-        <v>-74.95</v>
+        <v>-74.90000000000001</v>
       </c>
       <c r="BH13" t="n">
         <v>25.49</v>
@@ -3517,7 +3517,7 @@
         <v>0</v>
       </c>
       <c r="BJ13" t="n">
-        <v>34.71</v>
+        <v>34.64</v>
       </c>
       <c r="BK13" t="n">
         <v>1.85</v>
@@ -3526,7 +3526,7 @@
         <v>1.96</v>
       </c>
       <c r="BM13" t="n">
-        <v>34.94</v>
+        <v>34.92</v>
       </c>
       <c r="BN13" t="n">
         <v>36.1</v>
@@ -3535,19 +3535,19 @@
         <v>20.85</v>
       </c>
       <c r="BP13" t="n">
-        <v>33.76</v>
+        <v>33.91</v>
       </c>
       <c r="BQ13" t="n">
-        <v>17.73</v>
+        <v>17.7</v>
       </c>
       <c r="BR13" t="n">
-        <v>34.27</v>
+        <v>34.07</v>
       </c>
       <c r="BS13" t="n">
         <v>5.01</v>
       </c>
       <c r="BT13" t="n">
-        <v>6937150</v>
+        <v>7014540</v>
       </c>
     </row>
     <row r="14">
@@ -3577,13 +3577,13 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>12.5</v>
+        <v>12.55</v>
       </c>
       <c r="G14" t="n">
-        <v>10298187816</v>
+        <v>10565975087</v>
       </c>
       <c r="H14" t="n">
-        <v>14600</v>
+        <v>0</v>
       </c>
       <c r="I14" t="n">
         <v>339510689</v>
@@ -3598,7 +3598,7 @@
         <v>1.92</v>
       </c>
       <c r="M14" t="n">
-        <v>4.275990659127843</v>
+        <v>4.387180694684419</v>
       </c>
       <c r="N14" t="n">
         <v>1.11</v>
@@ -3676,7 +3676,7 @@
         <v>349696009.67</v>
       </c>
       <c r="AM14" t="n">
-        <v>1142973120.532741</v>
+        <v>1172694238.290788</v>
       </c>
       <c r="AN14" t="n">
         <v>0.1489</v>
@@ -3717,7 +3717,7 @@
         <v>9.050000000000001</v>
       </c>
       <c r="AZ14" t="n">
-        <v>10.04</v>
+        <v>10.08</v>
       </c>
       <c r="BA14" t="n">
         <v>1.42</v>
@@ -3726,19 +3726,19 @@
         <v>5.94</v>
       </c>
       <c r="BC14" t="n">
-        <v>-11.34</v>
+        <v>-11.69</v>
       </c>
       <c r="BD14" t="n">
-        <v>-27.61</v>
+        <v>-27.9</v>
       </c>
       <c r="BE14" t="n">
         <v>-19.67</v>
       </c>
       <c r="BF14" t="n">
-        <v>-88.63</v>
+        <v>-88.68000000000001</v>
       </c>
       <c r="BG14" t="n">
-        <v>-52.46</v>
+        <v>-52.65</v>
       </c>
       <c r="BH14" t="n">
         <v>5.3</v>
@@ -3747,7 +3747,7 @@
         <v>0</v>
       </c>
       <c r="BJ14" t="n">
-        <v>12.5</v>
+        <v>12.55</v>
       </c>
       <c r="BK14" t="n">
         <v>1.03</v>
@@ -3756,7 +3756,7 @@
         <v>1.01</v>
       </c>
       <c r="BM14" t="n">
-        <v>12.58</v>
+        <v>12.89</v>
       </c>
       <c r="BN14" t="n">
         <v>13.49</v>
@@ -3765,19 +3765,19 @@
         <v>7.92</v>
       </c>
       <c r="BP14" t="n">
-        <v>12.03</v>
+        <v>12.1</v>
       </c>
       <c r="BQ14" t="n">
-        <v>12.34</v>
+        <v>12.39</v>
       </c>
       <c r="BR14" t="n">
-        <v>12.2</v>
+        <v>12.73</v>
       </c>
       <c r="BS14" t="n">
         <v>1.44</v>
       </c>
       <c r="BT14" t="n">
-        <v>12947</v>
+        <v>12927</v>
       </c>
     </row>
     <row r="15">
@@ -3807,13 +3807,13 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>17.69</v>
+        <v>18.15</v>
       </c>
       <c r="G15" t="n">
-        <v>10298187816</v>
+        <v>10565975087</v>
       </c>
       <c r="H15" t="n">
-        <v>5280400</v>
+        <v>0</v>
       </c>
       <c r="I15" t="n">
         <v>343551533</v>
@@ -3828,7 +3828,7 @@
         <v>2.56</v>
       </c>
       <c r="M15" t="n">
-        <v>4.225696570645366</v>
+        <v>4.335578791959009</v>
       </c>
       <c r="N15" t="n">
         <v>1.47</v>
@@ -3906,7 +3906,7 @@
         <v>353858078.99</v>
       </c>
       <c r="AM15" t="n">
-        <v>858898066.3886572</v>
+        <v>881232284.1534612</v>
       </c>
       <c r="AN15" t="n">
         <v>0.1638</v>
@@ -3947,7 +3947,7 @@
         <v>9.050000000000001</v>
       </c>
       <c r="AZ15" t="n">
-        <v>11.76</v>
+        <v>12.07</v>
       </c>
       <c r="BA15" t="n">
         <v>1.42</v>
@@ -3956,19 +3956,19 @@
         <v>6.19</v>
       </c>
       <c r="BC15" t="n">
-        <v>-37.35</v>
+        <v>-38.94</v>
       </c>
       <c r="BD15" t="n">
-        <v>-48.85</v>
+        <v>-50.14</v>
       </c>
       <c r="BE15" t="n">
         <v>-33.5</v>
       </c>
       <c r="BF15" t="n">
-        <v>-91.97</v>
+        <v>-92.17</v>
       </c>
       <c r="BG15" t="n">
-        <v>-65.02</v>
+        <v>-65.90000000000001</v>
       </c>
       <c r="BH15" t="n">
         <v>5.3</v>
@@ -3977,7 +3977,7 @@
         <v>0</v>
       </c>
       <c r="BJ15" t="n">
-        <v>17.69</v>
+        <v>18.15</v>
       </c>
       <c r="BK15" t="n">
         <v>1.03</v>
@@ -3986,28 +3986,28 @@
         <v>1.01</v>
       </c>
       <c r="BM15" t="n">
-        <v>17.8</v>
+        <v>18.33</v>
       </c>
       <c r="BN15" t="n">
-        <v>17.8</v>
+        <v>18.33</v>
       </c>
       <c r="BO15" t="n">
         <v>7.97</v>
       </c>
       <c r="BP15" t="n">
-        <v>16.87</v>
+        <v>17.17</v>
       </c>
       <c r="BQ15" t="n">
-        <v>17.46</v>
+        <v>17.92</v>
       </c>
       <c r="BR15" t="n">
-        <v>17.21</v>
+        <v>17.32</v>
       </c>
       <c r="BS15" t="n">
         <v>1.92</v>
       </c>
       <c r="BT15" t="n">
-        <v>2822340</v>
+        <v>2917280</v>
       </c>
     </row>
     <row r="16">
@@ -4037,13 +4037,13 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>5.55</v>
+        <v>5.37</v>
       </c>
       <c r="G16" t="n">
-        <v>1217146121</v>
+        <v>1177671046</v>
       </c>
       <c r="H16" t="n">
-        <v>214600</v>
+        <v>0</v>
       </c>
       <c r="I16" t="n">
         <v>219305733</v>
@@ -4058,7 +4058,7 @@
         <v>2.69</v>
       </c>
       <c r="M16" t="n">
-        <v>0.5758121701895955</v>
+        <v>0.5571371498186051</v>
       </c>
       <c r="N16" t="n">
         <v>0.39</v>
@@ -4136,7 +4136,7 @@
         <v>17544458.64</v>
       </c>
       <c r="AM16" t="n">
-        <v>341894977.8089887</v>
+        <v>330806473.5955056</v>
       </c>
       <c r="AN16" t="n">
         <v>0.0077</v>
@@ -4177,7 +4177,7 @@
         <v>1.42</v>
       </c>
       <c r="AZ16" t="n">
-        <v>0.16</v>
+        <v>0.15</v>
       </c>
       <c r="BA16" t="n">
         <v>0.08</v>
@@ -4186,16 +4186,16 @@
         <v>0</v>
       </c>
       <c r="BC16" t="n">
-        <v>-68.67</v>
+        <v>-67.62</v>
       </c>
       <c r="BD16" t="n">
-        <v>-74.42</v>
+        <v>-73.56</v>
       </c>
       <c r="BE16" t="n">
         <v>-97.17</v>
       </c>
       <c r="BF16" t="n">
-        <v>-98.56</v>
+        <v>-98.51000000000001</v>
       </c>
       <c r="BG16" t="n">
         <v>-100</v>
@@ -4207,7 +4207,7 @@
         <v>0</v>
       </c>
       <c r="BJ16" t="n">
-        <v>5.55</v>
+        <v>5.37</v>
       </c>
       <c r="BK16" t="n">
         <v>0.08</v>
@@ -4225,19 +4225,19 @@
         <v>3.31</v>
       </c>
       <c r="BP16" t="n">
-        <v>5.26</v>
+        <v>5.37</v>
       </c>
       <c r="BQ16" t="n">
-        <v>75.73999999999999</v>
+        <v>73.28</v>
       </c>
       <c r="BR16" t="n">
-        <v>5.56</v>
+        <v>5.43</v>
       </c>
       <c r="BS16" t="n">
         <v>0.49</v>
       </c>
       <c r="BT16" t="n">
-        <v>149017</v>
+        <v>152730</v>
       </c>
     </row>
     <row r="17">
@@ -4267,13 +4267,13 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>39.08</v>
+        <v>38.37</v>
       </c>
       <c r="G17" t="n">
-        <v>12881819855</v>
+        <v>12647783800</v>
       </c>
       <c r="H17" t="n">
-        <v>1896600</v>
+        <v>0</v>
       </c>
       <c r="I17" t="n">
         <v>0</v>
@@ -4360,13 +4360,13 @@
         <v>8.039999999999999</v>
       </c>
       <c r="AK17" t="n">
-        <v>5817295816.022399</v>
+        <v>5711607568.641619</v>
       </c>
       <c r="AL17" t="n">
-        <v>1610227481.875</v>
+        <v>1580972975</v>
       </c>
       <c r="AM17" t="n">
-        <v>3988179521.671827</v>
+        <v>3915722538.69969</v>
       </c>
       <c r="AN17" t="n">
         <v>1.08</v>
@@ -4407,7 +4407,7 @@
         <v>42.98</v>
       </c>
       <c r="AZ17" t="n">
-        <v>20.91</v>
+        <v>20.53</v>
       </c>
       <c r="BA17" t="n">
         <v>4.55</v>
@@ -4416,19 +4416,19 @@
         <v>16.33</v>
       </c>
       <c r="BC17" t="n">
-        <v>34.69</v>
+        <v>37.18</v>
       </c>
       <c r="BD17" t="n">
-        <v>9.98</v>
+        <v>12.01</v>
       </c>
       <c r="BE17" t="n">
         <v>-46.5</v>
       </c>
       <c r="BF17" t="n">
-        <v>-88.36</v>
+        <v>-88.15000000000001</v>
       </c>
       <c r="BG17" t="n">
-        <v>-58.21</v>
+        <v>-57.43</v>
       </c>
       <c r="BH17" t="n">
         <v>29.25</v>
@@ -4437,7 +4437,7 @@
         <v>0</v>
       </c>
       <c r="BJ17" t="n">
-        <v>39.08</v>
+        <v>38.37</v>
       </c>
       <c r="BK17" t="n">
         <v>4.21</v>
@@ -4446,7 +4446,7 @@
         <v>12.62</v>
       </c>
       <c r="BM17" t="n">
-        <v>39.65</v>
+        <v>39.24</v>
       </c>
       <c r="BN17" t="n">
         <v>40.95</v>
@@ -4455,19 +4455,19 @@
         <v>29.59</v>
       </c>
       <c r="BP17" t="n">
-        <v>38.99</v>
+        <v>38.16</v>
       </c>
       <c r="BQ17" t="n">
-        <v>3.1</v>
+        <v>3.04</v>
       </c>
       <c r="BR17" t="n">
-        <v>39.46</v>
+        <v>38.37</v>
       </c>
       <c r="BS17" t="n">
         <v>2.21</v>
       </c>
       <c r="BT17" t="n">
-        <v>1340323</v>
+        <v>1361140</v>
       </c>
     </row>
     <row r="18">
@@ -4497,13 +4497,13 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>13.86</v>
+        <v>13.69</v>
       </c>
       <c r="G18" t="n">
-        <v>12881819855</v>
+        <v>12647783800</v>
       </c>
       <c r="H18" t="n">
-        <v>3500</v>
+        <v>0</v>
       </c>
       <c r="I18" t="n">
         <v>671494278</v>
@@ -4518,7 +4518,7 @@
         <v>1.2</v>
       </c>
       <c r="M18" t="n">
-        <v>3.792913647629665</v>
+        <v>3.724004242201025</v>
       </c>
       <c r="N18" t="n">
         <v>0.33</v>
@@ -4596,7 +4596,7 @@
         <v>940091989.1999999</v>
       </c>
       <c r="AM18" t="n">
-        <v>3833874956.845238</v>
+        <v>3764221369.047619</v>
       </c>
       <c r="AN18" t="n">
         <v>0.36</v>
@@ -4637,7 +4637,7 @@
         <v>14.31</v>
       </c>
       <c r="AZ18" t="n">
-        <v>7.14</v>
+        <v>7.05</v>
       </c>
       <c r="BA18" t="n">
         <v>1.51</v>
@@ -4646,19 +4646,19 @@
         <v>5.44</v>
       </c>
       <c r="BC18" t="n">
-        <v>26.44</v>
+        <v>28.01</v>
       </c>
       <c r="BD18" t="n">
-        <v>3.24</v>
+        <v>4.52</v>
       </c>
       <c r="BE18" t="n">
         <v>-48.5</v>
       </c>
       <c r="BF18" t="n">
-        <v>-89.09</v>
+        <v>-88.95</v>
       </c>
       <c r="BG18" t="n">
-        <v>-60.72</v>
+        <v>-60.23</v>
       </c>
       <c r="BH18" t="n">
         <v>9.75</v>
@@ -4667,7 +4667,7 @@
         <v>0</v>
       </c>
       <c r="BJ18" t="n">
-        <v>13.86</v>
+        <v>13.69</v>
       </c>
       <c r="BK18" t="n">
         <v>1.4</v>
@@ -4676,7 +4676,7 @@
         <v>12.62</v>
       </c>
       <c r="BM18" t="n">
-        <v>13.87</v>
+        <v>13.92</v>
       </c>
       <c r="BN18" t="n">
         <v>14.62</v>
@@ -4685,19 +4685,19 @@
         <v>10.19</v>
       </c>
       <c r="BP18" t="n">
-        <v>13.63</v>
+        <v>13.24</v>
       </c>
       <c r="BQ18" t="n">
-        <v>1.1</v>
+        <v>1.08</v>
       </c>
       <c r="BR18" t="n">
-        <v>13.74</v>
+        <v>13.56</v>
       </c>
       <c r="BS18" t="n">
         <v>2.3</v>
       </c>
       <c r="BT18" t="n">
-        <v>7753</v>
+        <v>7770</v>
       </c>
     </row>
     <row r="19">
@@ -4727,13 +4727,13 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>12.84</v>
+        <v>12.3</v>
       </c>
       <c r="G19" t="n">
-        <v>12881819855</v>
+        <v>12647783800</v>
       </c>
       <c r="H19" t="n">
-        <v>9500</v>
+        <v>0</v>
       </c>
       <c r="I19" t="n">
         <v>317386323</v>
@@ -4748,7 +4748,7 @@
         <v>1.12</v>
       </c>
       <c r="M19" t="n">
-        <v>8.024667815731394</v>
+        <v>7.87887617919098</v>
       </c>
       <c r="N19" t="n">
         <v>0.3</v>
@@ -4826,7 +4826,7 @@
         <v>444340852.2</v>
       </c>
       <c r="AM19" t="n">
-        <v>4089466620.634921</v>
+        <v>4015169460.317461</v>
       </c>
       <c r="AN19" t="n">
         <v>0.36</v>
@@ -4867,7 +4867,7 @@
         <v>14.31</v>
       </c>
       <c r="AZ19" t="n">
-        <v>7.06</v>
+        <v>6.76</v>
       </c>
       <c r="BA19" t="n">
         <v>1.51</v>
@@ -4876,19 +4876,19 @@
         <v>5.25</v>
       </c>
       <c r="BC19" t="n">
-        <v>36.49</v>
+        <v>42.48</v>
       </c>
       <c r="BD19" t="n">
-        <v>11.44</v>
+        <v>16.33</v>
       </c>
       <c r="BE19" t="n">
         <v>-45</v>
       </c>
       <c r="BF19" t="n">
-        <v>-88.22</v>
+        <v>-87.7</v>
       </c>
       <c r="BG19" t="n">
-        <v>-59.11</v>
+        <v>-57.32</v>
       </c>
       <c r="BH19" t="n">
         <v>9.75</v>
@@ -4897,7 +4897,7 @@
         <v>0</v>
       </c>
       <c r="BJ19" t="n">
-        <v>12.84</v>
+        <v>12.3</v>
       </c>
       <c r="BK19" t="n">
         <v>1.4</v>
@@ -4906,7 +4906,7 @@
         <v>12.62</v>
       </c>
       <c r="BM19" t="n">
-        <v>12.95</v>
+        <v>12.78</v>
       </c>
       <c r="BN19" t="n">
         <v>13.26</v>
@@ -4915,19 +4915,19 @@
         <v>9.279999999999999</v>
       </c>
       <c r="BP19" t="n">
-        <v>12.64</v>
+        <v>12.3</v>
       </c>
       <c r="BQ19" t="n">
-        <v>1.02</v>
+        <v>0.97</v>
       </c>
       <c r="BR19" t="n">
-        <v>12.7</v>
+        <v>12.6</v>
       </c>
       <c r="BS19" t="n">
         <v>2.16</v>
       </c>
       <c r="BT19" t="n">
-        <v>14447</v>
+        <v>14493</v>
       </c>
     </row>
     <row r="20">
@@ -5417,13 +5417,13 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>5.71</v>
+        <v>5.64</v>
       </c>
       <c r="G22" t="n">
-        <v>1143400670</v>
+        <v>1129383465</v>
       </c>
       <c r="H22" t="n">
-        <v>2926800</v>
+        <v>0</v>
       </c>
       <c r="I22" t="n">
         <v>200245299</v>
@@ -5438,7 +5438,7 @@
         <v>0.27</v>
       </c>
       <c r="M22" t="n">
-        <v>0.09697936615738417</v>
+        <v>0.09579047437879346</v>
       </c>
       <c r="N22" t="n">
         <v>0.08</v>
@@ -5516,7 +5516,7 @@
         <v>378463615.11</v>
       </c>
       <c r="AM22" t="n">
-        <v>259274528.3446712</v>
+        <v>256096023.8095238</v>
       </c>
       <c r="AN22" t="n">
         <v>0</v>
@@ -5566,19 +5566,19 @@
         <v>172.49</v>
       </c>
       <c r="BC22" t="n">
-        <v>420.23</v>
+        <v>426.69</v>
       </c>
       <c r="BD22" t="n">
-        <v>324.77</v>
+        <v>330.04</v>
       </c>
       <c r="BE22" t="n">
         <v>-100</v>
       </c>
       <c r="BF22" t="n">
-        <v>-66.90000000000001</v>
+        <v>-66.48999999999999</v>
       </c>
       <c r="BG22" t="n">
-        <v>2920.84</v>
+        <v>2958.33</v>
       </c>
       <c r="BH22" t="n">
         <v>20.75</v>
@@ -5587,7 +5587,7 @@
         <v>0</v>
       </c>
       <c r="BJ22" t="n">
-        <v>5.71</v>
+        <v>5.64</v>
       </c>
       <c r="BK22" t="n">
         <v>1.89</v>
@@ -5596,7 +5596,7 @@
         <v>0.67</v>
       </c>
       <c r="BM22" t="n">
-        <v>6.31</v>
+        <v>5.9</v>
       </c>
       <c r="BN22" t="n">
         <v>7.89</v>
@@ -5605,19 +5605,19 @@
         <v>3.37</v>
       </c>
       <c r="BP22" t="n">
-        <v>5.71</v>
+        <v>5.45</v>
       </c>
       <c r="BQ22" t="n">
-        <v>8.5</v>
+        <v>8.4</v>
       </c>
       <c r="BR22" t="n">
-        <v>6.27</v>
+        <v>5.67</v>
       </c>
       <c r="BS22" t="n">
         <v>0.09</v>
       </c>
       <c r="BT22" t="n">
-        <v>1760240</v>
+        <v>1799793</v>
       </c>
     </row>
     <row r="23">
@@ -5877,13 +5877,13 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>5.22</v>
+        <v>5.25</v>
       </c>
       <c r="G24" t="n">
-        <v>2108194529</v>
+        <v>2120310675</v>
       </c>
       <c r="H24" t="n">
-        <v>13061000</v>
+        <v>0</v>
       </c>
       <c r="I24" t="n">
         <v>403868805</v>
@@ -5898,7 +5898,7 @@
         <v>0.49</v>
       </c>
       <c r="M24" t="n">
-        <v>0.5096366890591456</v>
+        <v>0.5125656562140534</v>
       </c>
       <c r="N24" t="n">
         <v>0.11</v>
@@ -5976,7 +5976,7 @@
         <v>153470145.9</v>
       </c>
       <c r="AM24" t="n">
-        <v>1899274350.45045</v>
+        <v>1910189797.297297</v>
       </c>
       <c r="AN24" t="n">
         <v>0.0813</v>
@@ -6017,7 +6017,7 @@
         <v>5.84</v>
       </c>
       <c r="AZ24" t="n">
-        <v>2.41</v>
+        <v>2.42</v>
       </c>
       <c r="BA24" t="n">
         <v>0.38</v>
@@ -6026,19 +6026,19 @@
         <v>1.46</v>
       </c>
       <c r="BC24" t="n">
-        <v>37.1</v>
+        <v>36.31</v>
       </c>
       <c r="BD24" t="n">
-        <v>11.94</v>
+        <v>11.3</v>
       </c>
       <c r="BE24" t="n">
         <v>-53.83</v>
       </c>
       <c r="BF24" t="n">
-        <v>-92.72</v>
+        <v>-92.76000000000001</v>
       </c>
       <c r="BG24" t="n">
-        <v>-72.06999999999999</v>
+        <v>-72.23</v>
       </c>
       <c r="BH24" t="n">
         <v>5.99</v>
@@ -6047,7 +6047,7 @@
         <v>0</v>
       </c>
       <c r="BJ24" t="n">
-        <v>5.22</v>
+        <v>5.25</v>
       </c>
       <c r="BK24" t="n">
         <v>0.38</v>
@@ -6056,28 +6056,28 @@
         <v>0.41</v>
       </c>
       <c r="BM24" t="n">
-        <v>5.29</v>
+        <v>5.49</v>
       </c>
       <c r="BN24" t="n">
-        <v>5.45</v>
+        <v>5.49</v>
       </c>
       <c r="BO24" t="n">
         <v>1.92</v>
       </c>
       <c r="BP24" t="n">
-        <v>4.71</v>
+        <v>4.98</v>
       </c>
       <c r="BQ24" t="n">
-        <v>12.82</v>
+        <v>12.9</v>
       </c>
       <c r="BR24" t="n">
-        <v>4.92</v>
+        <v>5.09</v>
       </c>
       <c r="BS24" t="n">
         <v>0.29</v>
       </c>
       <c r="BT24" t="n">
-        <v>7945810</v>
+        <v>8033663</v>
       </c>
     </row>
     <row r="25">
@@ -6107,13 +6107,13 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>6.04</v>
+        <v>5.91</v>
       </c>
       <c r="G25" t="n">
-        <v>2092823746</v>
+        <v>2047779487</v>
       </c>
       <c r="H25" t="n">
-        <v>1260400</v>
+        <v>0</v>
       </c>
       <c r="I25" t="n">
         <v>346494097</v>
@@ -6128,7 +6128,7 @@
         <v>0.97</v>
       </c>
       <c r="M25" t="n">
-        <v>1.043577478650219</v>
+        <v>1.021116354379849</v>
       </c>
       <c r="N25" t="n">
         <v>0.22</v>
@@ -6206,7 +6206,7 @@
         <v>62368937.46</v>
       </c>
       <c r="AM25" t="n">
-        <v>769420494.8529412</v>
+        <v>752860105.5147058</v>
       </c>
       <c r="AN25" t="n">
         <v>0.4742</v>
@@ -6247,7 +6247,7 @@
         <v>3.27</v>
       </c>
       <c r="AZ25" t="n">
-        <v>14.07</v>
+        <v>13.77</v>
       </c>
       <c r="BA25" t="n">
         <v>0.23</v>
@@ -6256,19 +6256,19 @@
         <v>2.2</v>
       </c>
       <c r="BC25" t="n">
-        <v>-33.61</v>
+        <v>-32.15</v>
       </c>
       <c r="BD25" t="n">
-        <v>-45.79</v>
+        <v>-44.6</v>
       </c>
       <c r="BE25" t="n">
         <v>133</v>
       </c>
       <c r="BF25" t="n">
-        <v>-96.16</v>
+        <v>-96.08</v>
       </c>
       <c r="BG25" t="n">
-        <v>-63.58</v>
+        <v>-62.78</v>
       </c>
       <c r="BH25" t="n">
         <v>3.97</v>
@@ -6277,7 +6277,7 @@
         <v>0</v>
       </c>
       <c r="BJ25" t="n">
-        <v>6.04</v>
+        <v>5.91</v>
       </c>
       <c r="BK25" t="n">
         <v>0.18</v>
@@ -6286,7 +6286,7 @@
         <v>0.24</v>
       </c>
       <c r="BM25" t="n">
-        <v>6.15</v>
+        <v>6.18</v>
       </c>
       <c r="BN25" t="n">
         <v>6.79</v>
@@ -6295,19 +6295,19 @@
         <v>2.64</v>
       </c>
       <c r="BP25" t="n">
-        <v>5.7</v>
+        <v>5.72</v>
       </c>
       <c r="BQ25" t="n">
-        <v>25.52</v>
+        <v>24.97</v>
       </c>
       <c r="BR25" t="n">
-        <v>5.82</v>
+        <v>5.89</v>
       </c>
       <c r="BS25" t="n">
         <v>0.67</v>
       </c>
       <c r="BT25" t="n">
-        <v>1456860</v>
+        <v>1488093</v>
       </c>
     </row>
     <row r="26">
@@ -6337,13 +6337,13 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>12.72</v>
+        <v>12.32</v>
       </c>
       <c r="G26" t="n">
-        <v>17227879321</v>
+        <v>16686121346</v>
       </c>
       <c r="H26" t="n">
-        <v>18266900</v>
+        <v>0</v>
       </c>
       <c r="I26" t="n">
         <v>1354393401</v>
@@ -6358,7 +6358,7 @@
         <v>1.94</v>
       </c>
       <c r="M26" t="n">
-        <v>0.2221520515577665</v>
+        <v>0.2151661281395936</v>
       </c>
       <c r="N26" t="n">
         <v>0.26</v>
@@ -6436,7 +6436,7 @@
         <v>961619314.7099999</v>
       </c>
       <c r="AM26" t="n">
-        <v>6152814043.214286</v>
+        <v>5959329052.142858</v>
       </c>
       <c r="AN26" t="n">
         <v>0.1043</v>
@@ -6477,7 +6477,7 @@
         <v>7.07</v>
       </c>
       <c r="AZ26" t="n">
-        <v>2.44</v>
+        <v>2.36</v>
       </c>
       <c r="BA26" t="n">
         <v>0.66</v>
@@ -6486,19 +6486,19 @@
         <v>1.19</v>
       </c>
       <c r="BC26" t="n">
-        <v>-31.95</v>
+        <v>-29.74</v>
       </c>
       <c r="BD26" t="n">
-        <v>-44.44</v>
+        <v>-42.63</v>
       </c>
       <c r="BE26" t="n">
         <v>-80.83</v>
       </c>
       <c r="BF26" t="n">
-        <v>-94.81999999999999</v>
+        <v>-94.65000000000001</v>
       </c>
       <c r="BG26" t="n">
-        <v>-90.62</v>
+        <v>-90.31</v>
       </c>
       <c r="BH26" t="n">
         <v>4.69</v>
@@ -6507,7 +6507,7 @@
         <v>0</v>
       </c>
       <c r="BJ26" t="n">
-        <v>12.72</v>
+        <v>12.32</v>
       </c>
       <c r="BK26" t="n">
         <v>0.71</v>
@@ -6516,7 +6516,7 @@
         <v>0.72</v>
       </c>
       <c r="BM26" t="n">
-        <v>12.8</v>
+        <v>12.82</v>
       </c>
       <c r="BN26" t="n">
         <v>13.8</v>
@@ -6525,19 +6525,19 @@
         <v>6.91</v>
       </c>
       <c r="BP26" t="n">
-        <v>12.06</v>
+        <v>12.22</v>
       </c>
       <c r="BQ26" t="n">
-        <v>17.73</v>
+        <v>17.18</v>
       </c>
       <c r="BR26" t="n">
-        <v>12.36</v>
+        <v>12.32</v>
       </c>
       <c r="BS26" t="n">
         <v>0.16</v>
       </c>
       <c r="BT26" t="n">
-        <v>17619293</v>
+        <v>17631313</v>
       </c>
     </row>
     <row r="27">
@@ -8165,13 +8165,13 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>24.31</v>
+        <v>23.61</v>
       </c>
       <c r="G34" t="n">
-        <v>5019766927</v>
+        <v>4875224304</v>
       </c>
       <c r="H34" t="n">
-        <v>5518700</v>
+        <v>0</v>
       </c>
       <c r="I34" t="n">
         <v>206489813</v>
@@ -8186,7 +8186,7 @@
         <v>0.45</v>
       </c>
       <c r="M34" t="n">
-        <v>0.4412961408030246</v>
+        <v>0.4285891560686622</v>
       </c>
       <c r="N34" t="n">
         <v>0.24</v>
@@ -8264,7 +8264,7 @@
         <v>324189006.41</v>
       </c>
       <c r="AM34" t="n">
-        <v>1043610587.733888</v>
+        <v>1013560146.361746</v>
       </c>
       <c r="AN34" t="n">
         <v>0</v>
@@ -8305,7 +8305,7 @@
         <v>30.28</v>
       </c>
       <c r="AZ34" t="n">
-        <v>56.72</v>
+        <v>55.09</v>
       </c>
       <c r="BA34" t="n">
         <v>2.29</v>
@@ -8314,19 +8314,19 @@
         <v>25.26</v>
       </c>
       <c r="BC34" t="n">
-        <v>52.56</v>
+        <v>57.09</v>
       </c>
       <c r="BD34" t="n">
-        <v>24.57</v>
+        <v>28.26</v>
       </c>
       <c r="BE34" t="n">
         <v>133.33</v>
       </c>
       <c r="BF34" t="n">
-        <v>-90.56</v>
+        <v>-90.28</v>
       </c>
       <c r="BG34" t="n">
-        <v>3.9</v>
+        <v>6.98</v>
       </c>
       <c r="BH34" t="n">
         <v>38.94</v>
@@ -8335,7 +8335,7 @@
         <v>0</v>
       </c>
       <c r="BJ34" t="n">
-        <v>24.31</v>
+        <v>23.61</v>
       </c>
       <c r="BK34" t="n">
         <v>1.57</v>
@@ -8344,7 +8344,7 @@
         <v>1.58</v>
       </c>
       <c r="BM34" t="n">
-        <v>24.93</v>
+        <v>24.36</v>
       </c>
       <c r="BN34" t="n">
         <v>28.86</v>
@@ -8353,19 +8353,19 @@
         <v>14.3</v>
       </c>
       <c r="BP34" t="n">
-        <v>23.44</v>
+        <v>23.22</v>
       </c>
       <c r="BQ34" t="n">
-        <v>15.41</v>
+        <v>14.97</v>
       </c>
       <c r="BR34" t="n">
-        <v>24.93</v>
+        <v>23.5</v>
       </c>
       <c r="BS34" t="n">
         <v>0.32</v>
       </c>
       <c r="BT34" t="n">
-        <v>4869843</v>
+        <v>4982620</v>
       </c>
     </row>
     <row r="35">
@@ -8395,13 +8395,13 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>22.33</v>
+        <v>22.22</v>
       </c>
       <c r="G35" t="n">
-        <v>112688299954</v>
+        <v>112133182094</v>
       </c>
       <c r="H35" t="n">
-        <v>69936900</v>
+        <v>0</v>
       </c>
       <c r="I35" t="n">
         <v>5046500000</v>
@@ -8416,7 +8416,7 @@
         <v>4.69</v>
       </c>
       <c r="M35" t="n">
-        <v>9.355423618755273</v>
+        <v>9.309337532260429</v>
       </c>
       <c r="N35" t="n">
         <v>1.79</v>
@@ -8494,7 +8494,7 @@
         <v>5349290000</v>
       </c>
       <c r="AM35" t="n">
-        <v>9313082640.826447</v>
+        <v>9267205131.735537</v>
       </c>
       <c r="AN35" t="n">
         <v>0.5305</v>
@@ -8535,7 +8535,7 @@
         <v>7.68</v>
       </c>
       <c r="AZ35" t="n">
-        <v>13.03</v>
+        <v>12.96</v>
       </c>
       <c r="BA35" t="n">
         <v>1.11</v>
@@ -8544,19 +8544,19 @@
         <v>9.119999999999999</v>
       </c>
       <c r="BC35" t="n">
-        <v>-57.87</v>
+        <v>-57.67</v>
       </c>
       <c r="BD35" t="n">
-        <v>-65.59999999999999</v>
+        <v>-65.43000000000001</v>
       </c>
       <c r="BE35" t="n">
         <v>-41.67</v>
       </c>
       <c r="BF35" t="n">
-        <v>-95.01000000000001</v>
+        <v>-94.98999999999999</v>
       </c>
       <c r="BG35" t="n">
-        <v>-59.17</v>
+        <v>-58.97</v>
       </c>
       <c r="BH35" t="n">
         <v>3.71</v>
@@ -8565,7 +8565,7 @@
         <v>0</v>
       </c>
       <c r="BJ35" t="n">
-        <v>22.33</v>
+        <v>22.22</v>
       </c>
       <c r="BK35" t="n">
         <v>1.06</v>
@@ -8574,7 +8574,7 @@
         <v>1.04</v>
       </c>
       <c r="BM35" t="n">
-        <v>22.35</v>
+        <v>22.45</v>
       </c>
       <c r="BN35" t="n">
         <v>24.28</v>
@@ -8583,19 +8583,19 @@
         <v>11.71</v>
       </c>
       <c r="BP35" t="n">
-        <v>21.66</v>
+        <v>21.73</v>
       </c>
       <c r="BQ35" t="n">
-        <v>21.37</v>
+        <v>21.26</v>
       </c>
       <c r="BR35" t="n">
-        <v>22.3</v>
+        <v>21.87</v>
       </c>
       <c r="BS35" t="n">
         <v>7.3</v>
       </c>
       <c r="BT35" t="n">
-        <v>53251573</v>
+        <v>54499020</v>
       </c>
     </row>
     <row r="36">
@@ -8628,10 +8628,10 @@
         <v>22</v>
       </c>
       <c r="G36" t="n">
-        <v>177987888</v>
+        <v>191346001</v>
       </c>
       <c r="H36" t="n">
-        <v>2500</v>
+        <v>0</v>
       </c>
       <c r="I36" t="n">
         <v>4900000</v>
@@ -8646,7 +8646,7 @@
         <v>1.52</v>
       </c>
       <c r="M36" t="n">
-        <v>1.732862024701829</v>
+        <v>1.862914507482993</v>
       </c>
       <c r="N36" t="n">
         <v>0.87</v>
@@ -8724,7 +8724,7 @@
         <v>11319000</v>
       </c>
       <c r="AM36" t="n">
-        <v>24516238.01652893</v>
+        <v>26356198.48484848</v>
       </c>
       <c r="AN36" t="n">
         <v>0</v>
@@ -8825,7 +8825,7 @@
         <v>1.24</v>
       </c>
       <c r="BT36" t="n">
-        <v>170</v>
+        <v>253</v>
       </c>
     </row>
     <row r="37">
@@ -8855,13 +8855,13 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>14.79</v>
+        <v>15.9</v>
       </c>
       <c r="G37" t="n">
-        <v>177987888</v>
+        <v>191346001</v>
       </c>
       <c r="H37" t="n">
-        <v>1300</v>
+        <v>0</v>
       </c>
       <c r="I37" t="n">
         <v>4900000</v>
@@ -8876,7 +8876,7 @@
         <v>0.88</v>
       </c>
       <c r="M37" t="n">
-        <v>1.732862024701829</v>
+        <v>1.862914507482993</v>
       </c>
       <c r="N37" t="n">
         <v>0.5</v>
@@ -8954,7 +8954,7 @@
         <v>11319000</v>
       </c>
       <c r="AM37" t="n">
-        <v>42580834.44976076</v>
+        <v>45776555.2631579</v>
       </c>
       <c r="AN37" t="n">
         <v>0</v>
@@ -8995,7 +8995,7 @@
         <v>24.36</v>
       </c>
       <c r="AZ37" t="n">
-        <v>65.77</v>
+        <v>70.7</v>
       </c>
       <c r="BA37" t="n">
         <v>2.44</v>
@@ -9004,19 +9004,19 @@
         <v>15.53</v>
       </c>
       <c r="BC37" t="n">
-        <v>101.75</v>
+        <v>87.66</v>
       </c>
       <c r="BD37" t="n">
-        <v>64.73</v>
+        <v>53.23</v>
       </c>
       <c r="BE37" t="n">
         <v>344.67</v>
       </c>
       <c r="BF37" t="n">
-        <v>-83.47</v>
+        <v>-84.62</v>
       </c>
       <c r="BG37" t="n">
-        <v>5.03</v>
+        <v>-2.31</v>
       </c>
       <c r="BH37" t="n">
         <v>17.13</v>
@@ -9025,7 +9025,7 @@
         <v>0</v>
       </c>
       <c r="BJ37" t="n">
-        <v>14.79</v>
+        <v>15.9</v>
       </c>
       <c r="BK37" t="n">
         <v>2.31</v>
@@ -9034,7 +9034,7 @@
         <v>2.31</v>
       </c>
       <c r="BM37" t="n">
-        <v>15.89</v>
+        <v>15.9</v>
       </c>
       <c r="BN37" t="n">
         <v>20.9</v>
@@ -9043,19 +9043,19 @@
         <v>13.42</v>
       </c>
       <c r="BP37" t="n">
-        <v>14.76</v>
+        <v>14.9</v>
       </c>
       <c r="BQ37" t="n">
-        <v>6.4</v>
+        <v>6.88</v>
       </c>
       <c r="BR37" t="n">
-        <v>15.89</v>
+        <v>14.9</v>
       </c>
       <c r="BS37" t="n">
         <v>0.72</v>
       </c>
       <c r="BT37" t="n">
-        <v>1190</v>
+        <v>1233</v>
       </c>
     </row>
     <row r="38">
@@ -9315,13 +9315,13 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>75.51000000000001</v>
+        <v>76.51000000000001</v>
       </c>
       <c r="G39" t="n">
-        <v>4232963862</v>
+        <v>4289022182</v>
       </c>
       <c r="H39" t="n">
-        <v>4400</v>
+        <v>0</v>
       </c>
       <c r="I39" t="n">
         <v>168174945</v>
@@ -9336,7 +9336,7 @@
         <v>0.53</v>
       </c>
       <c r="M39" t="n">
-        <v>0.2124762185485451</v>
+        <v>0.2152901003203012</v>
       </c>
       <c r="N39" t="n">
         <v>0.06</v>
@@ -9414,7 +9414,7 @@
         <v>2536078170.6</v>
       </c>
       <c r="AM39" t="n">
-        <v>444639061.1344538</v>
+        <v>450527540.1260504</v>
       </c>
       <c r="AN39" t="n">
         <v>11.9435</v>
@@ -9455,7 +9455,7 @@
         <v>170.24</v>
       </c>
       <c r="AZ39" t="n">
-        <v>220.62</v>
+        <v>223.54</v>
       </c>
       <c r="BA39" t="n">
         <v>19.01</v>
@@ -9464,19 +9464,19 @@
         <v>91.72</v>
       </c>
       <c r="BC39" t="n">
-        <v>176.13</v>
+        <v>172.52</v>
       </c>
       <c r="BD39" t="n">
-        <v>125.46</v>
+        <v>122.51</v>
       </c>
       <c r="BE39" t="n">
         <v>192.17</v>
       </c>
       <c r="BF39" t="n">
-        <v>-74.81999999999999</v>
+        <v>-75.15000000000001</v>
       </c>
       <c r="BG39" t="n">
-        <v>21.47</v>
+        <v>19.88</v>
       </c>
       <c r="BH39" t="n">
         <v>128.13</v>
@@ -9485,7 +9485,7 @@
         <v>0</v>
       </c>
       <c r="BJ39" t="n">
-        <v>75.51000000000001</v>
+        <v>76.51000000000001</v>
       </c>
       <c r="BK39" t="n">
         <v>15.08</v>
@@ -9494,7 +9494,7 @@
         <v>15.08</v>
       </c>
       <c r="BM39" t="n">
-        <v>76.72</v>
+        <v>77.12</v>
       </c>
       <c r="BN39" t="n">
         <v>78.62</v>
@@ -9503,19 +9503,19 @@
         <v>54.98</v>
       </c>
       <c r="BP39" t="n">
-        <v>74.5</v>
+        <v>75.61</v>
       </c>
       <c r="BQ39" t="n">
-        <v>5.01</v>
+        <v>5.07</v>
       </c>
       <c r="BR39" t="n">
-        <v>75.84999999999999</v>
+        <v>75.62</v>
       </c>
       <c r="BS39" t="n">
         <v>0.58</v>
       </c>
       <c r="BT39" t="n">
-        <v>3527</v>
+        <v>3437</v>
       </c>
     </row>
     <row r="40">
@@ -9545,13 +9545,13 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>24.19</v>
+        <v>23.76</v>
       </c>
       <c r="G40" t="n">
-        <v>138628829140</v>
+        <v>136164569631</v>
       </c>
       <c r="H40" t="n">
-        <v>46494500</v>
+        <v>0</v>
       </c>
       <c r="I40" t="n">
         <v>5730834040</v>
@@ -9566,7 +9566,7 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="M40" t="n">
-        <v>0.4206170237367977</v>
+        <v>0.4131401554200068</v>
       </c>
       <c r="N40" t="n">
         <v>0.05</v>
@@ -9644,7 +9644,7 @@
         <v>15358635227.2</v>
       </c>
       <c r="AM40" t="n">
-        <v>7190291967.842323</v>
+        <v>7062477677.956431</v>
       </c>
       <c r="AN40" t="n">
         <v>0.5641</v>
@@ -9685,7 +9685,7 @@
         <v>36.13</v>
       </c>
       <c r="AZ40" t="n">
-        <v>12.22</v>
+        <v>12</v>
       </c>
       <c r="BA40" t="n">
         <v>2.76</v>
@@ -9694,19 +9694,19 @@
         <v>27.89</v>
       </c>
       <c r="BC40" t="n">
-        <v>82.92</v>
+        <v>86.23</v>
       </c>
       <c r="BD40" t="n">
-        <v>49.35</v>
+        <v>52.06</v>
       </c>
       <c r="BE40" t="n">
         <v>-49.5</v>
       </c>
       <c r="BF40" t="n">
-        <v>-88.59</v>
+        <v>-88.39</v>
       </c>
       <c r="BG40" t="n">
-        <v>15.3</v>
+        <v>17.38</v>
       </c>
       <c r="BH40" t="n">
         <v>32.47</v>
@@ -9715,7 +9715,7 @@
         <v>0</v>
       </c>
       <c r="BJ40" t="n">
-        <v>24.19</v>
+        <v>23.76</v>
       </c>
       <c r="BK40" t="n">
         <v>2.68</v>
@@ -9724,7 +9724,7 @@
         <v>2.5</v>
       </c>
       <c r="BM40" t="n">
-        <v>24.45</v>
+        <v>24.15</v>
       </c>
       <c r="BN40" t="n">
         <v>27.36</v>
@@ -9733,19 +9733,19 @@
         <v>17.67</v>
       </c>
       <c r="BP40" t="n">
-        <v>23.5</v>
+        <v>23.53</v>
       </c>
       <c r="BQ40" t="n">
-        <v>9.68</v>
+        <v>9.51</v>
       </c>
       <c r="BR40" t="n">
-        <v>24.11</v>
+        <v>23.75</v>
       </c>
       <c r="BS40" t="n">
         <v>0.39</v>
       </c>
       <c r="BT40" t="n">
-        <v>45187290</v>
+        <v>45234997</v>
       </c>
     </row>
     <row r="41">
@@ -9775,13 +9775,13 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>18.38</v>
+        <v>18.15</v>
       </c>
       <c r="G41" t="n">
-        <v>219680550633</v>
+        <v>218206877381</v>
       </c>
       <c r="H41" t="n">
-        <v>11239900</v>
+        <v>0</v>
       </c>
       <c r="I41" t="n">
         <v>5606747177</v>
@@ -9796,7 +9796,7 @@
         <v>0.92</v>
       </c>
       <c r="M41" t="n">
-        <v>1.384862013756961</v>
+        <v>1.375572005599644</v>
       </c>
       <c r="N41" t="n">
         <v>0.07000000000000001</v>
@@ -9874,7 +9874,7 @@
         <v>13007653450.64</v>
       </c>
       <c r="AM41" t="n">
-        <v>33849083302.46533</v>
+        <v>33622015004.77658</v>
       </c>
       <c r="AN41" t="n">
         <v>1.6841</v>
@@ -9915,7 +9915,7 @@
         <v>24.4</v>
       </c>
       <c r="AZ41" t="n">
-        <v>27.51</v>
+        <v>27.16</v>
       </c>
       <c r="BA41" t="n">
         <v>2.53</v>
@@ -9924,19 +9924,19 @@
         <v>13.77</v>
       </c>
       <c r="BC41" t="n">
-        <v>62.6</v>
+        <v>64.66</v>
       </c>
       <c r="BD41" t="n">
-        <v>32.76</v>
+        <v>34.44</v>
       </c>
       <c r="BE41" t="n">
         <v>49.67</v>
       </c>
       <c r="BF41" t="n">
-        <v>-86.25</v>
+        <v>-86.08</v>
       </c>
       <c r="BG41" t="n">
-        <v>-25.08</v>
+        <v>-24.13</v>
       </c>
       <c r="BH41" t="n">
         <v>17.11</v>
@@ -9945,7 +9945,7 @@
         <v>0</v>
       </c>
       <c r="BJ41" t="n">
-        <v>18.38</v>
+        <v>18.15</v>
       </c>
       <c r="BK41" t="n">
         <v>2.32</v>
@@ -9954,7 +9954,7 @@
         <v>2.34</v>
       </c>
       <c r="BM41" t="n">
-        <v>18.51</v>
+        <v>18.5</v>
       </c>
       <c r="BN41" t="n">
         <v>20.24</v>
@@ -9963,19 +9963,19 @@
         <v>13.57</v>
       </c>
       <c r="BP41" t="n">
-        <v>17.94</v>
+        <v>17.91</v>
       </c>
       <c r="BQ41" t="n">
-        <v>7.86</v>
+        <v>7.76</v>
       </c>
       <c r="BR41" t="n">
-        <v>18.3</v>
+        <v>18.03</v>
       </c>
       <c r="BS41" t="n">
         <v>0.5600000000000001</v>
       </c>
       <c r="BT41" t="n">
-        <v>14206333</v>
+        <v>14240297</v>
       </c>
     </row>
     <row r="42">
@@ -10005,13 +10005,13 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>20.87</v>
+        <v>20.73</v>
       </c>
       <c r="G42" t="n">
-        <v>219680550633</v>
+        <v>218206877381</v>
       </c>
       <c r="H42" t="n">
-        <v>48274900</v>
+        <v>0</v>
       </c>
       <c r="I42" t="n">
         <v>5590117604</v>
@@ -10026,7 +10026,7 @@
         <v>1.05</v>
       </c>
       <c r="M42" t="n">
-        <v>1.388981723856838</v>
+        <v>1.379664079631773</v>
       </c>
       <c r="N42" t="n">
         <v>0.08</v>
@@ -10104,7 +10104,7 @@
         <v>12969072841.28</v>
       </c>
       <c r="AM42" t="n">
-        <v>29888510290.20408</v>
+        <v>29688010528.02721</v>
       </c>
       <c r="AN42" t="n">
         <v>1.8491</v>
@@ -10145,7 +10145,7 @@
         <v>24.4</v>
       </c>
       <c r="AZ42" t="n">
-        <v>30.23</v>
+        <v>30.02</v>
       </c>
       <c r="BA42" t="n">
         <v>2.53</v>
@@ -10154,19 +10154,19 @@
         <v>15.11</v>
       </c>
       <c r="BC42" t="n">
-        <v>43.2</v>
+        <v>44.17</v>
       </c>
       <c r="BD42" t="n">
-        <v>16.92</v>
+        <v>17.71</v>
       </c>
       <c r="BE42" t="n">
         <v>44.83</v>
       </c>
       <c r="BF42" t="n">
-        <v>-87.89</v>
+        <v>-87.81</v>
       </c>
       <c r="BG42" t="n">
-        <v>-27.58</v>
+        <v>-27.09</v>
       </c>
       <c r="BH42" t="n">
         <v>17.11</v>
@@ -10175,7 +10175,7 @@
         <v>0</v>
       </c>
       <c r="BJ42" t="n">
-        <v>20.87</v>
+        <v>20.73</v>
       </c>
       <c r="BK42" t="n">
         <v>2.32</v>
@@ -10193,19 +10193,19 @@
         <v>15.65</v>
       </c>
       <c r="BP42" t="n">
-        <v>20.48</v>
+        <v>20.37</v>
       </c>
       <c r="BQ42" t="n">
-        <v>8.93</v>
+        <v>8.869999999999999</v>
       </c>
       <c r="BR42" t="n">
-        <v>20.86</v>
+        <v>20.54</v>
       </c>
       <c r="BS42" t="n">
         <v>0.63</v>
       </c>
       <c r="BT42" t="n">
-        <v>59613200</v>
+        <v>59879917</v>
       </c>
     </row>
     <row r="43">
@@ -10235,13 +10235,13 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>41.68</v>
+        <v>41.57</v>
       </c>
       <c r="G43" t="n">
-        <v>80917510912</v>
+        <v>80703955837</v>
       </c>
       <c r="H43" t="n">
-        <v>8059000</v>
+        <v>0</v>
       </c>
       <c r="I43" t="n">
         <v>1941400000</v>
@@ -10334,7 +10334,7 @@
         <v>9182822000</v>
       </c>
       <c r="AM43" t="n">
-        <v>9855969660.414127</v>
+        <v>9829958080.024359</v>
       </c>
       <c r="AN43" t="n">
         <v>4.5901</v>
@@ -10375,7 +10375,7 @@
         <v>19.95</v>
       </c>
       <c r="AZ43" t="n">
-        <v>75.65000000000001</v>
+        <v>75.45</v>
       </c>
       <c r="BA43" t="n">
         <v>5.63</v>
@@ -10384,19 +10384,19 @@
         <v>48.62</v>
       </c>
       <c r="BC43" t="n">
-        <v>-41.38</v>
+        <v>-41.22</v>
       </c>
       <c r="BD43" t="n">
-        <v>-52.13</v>
+        <v>-52.01</v>
       </c>
       <c r="BE43" t="n">
         <v>81.5</v>
       </c>
       <c r="BF43" t="n">
-        <v>-86.5</v>
+        <v>-86.45999999999999</v>
       </c>
       <c r="BG43" t="n">
-        <v>16.64</v>
+        <v>16.95</v>
       </c>
       <c r="BH43" t="n">
         <v>5.61</v>
@@ -10405,7 +10405,7 @@
         <v>0</v>
       </c>
       <c r="BJ43" t="n">
-        <v>41.68</v>
+        <v>41.57</v>
       </c>
       <c r="BK43" t="n">
         <v>4.73</v>
@@ -10414,7 +10414,7 @@
         <v>4.73</v>
       </c>
       <c r="BM43" t="n">
-        <v>41.83</v>
+        <v>41.92</v>
       </c>
       <c r="BN43" t="n">
         <v>42.98</v>
@@ -10423,19 +10423,19 @@
         <v>28.06</v>
       </c>
       <c r="BP43" t="n">
-        <v>40.56</v>
+        <v>41.11</v>
       </c>
       <c r="BQ43" t="n">
-        <v>8.800000000000001</v>
+        <v>8.779999999999999</v>
       </c>
       <c r="BR43" t="n">
-        <v>41.49</v>
+        <v>41.11</v>
       </c>
       <c r="BS43" t="n">
         <v>0</v>
       </c>
       <c r="BT43" t="n">
-        <v>7106710</v>
+        <v>7043740</v>
       </c>
     </row>
     <row r="44">
@@ -10925,13 +10925,13 @@
         </is>
       </c>
       <c r="F46" t="n">
-        <v>4.18</v>
+        <v>4.1</v>
       </c>
       <c r="G46" t="n">
-        <v>4182265388</v>
+        <v>4102222104</v>
       </c>
       <c r="H46" t="n">
-        <v>29495100</v>
+        <v>0</v>
       </c>
       <c r="I46" t="n">
         <v>1000542188</v>
@@ -10946,7 +10946,7 @@
         <v>2.5</v>
       </c>
       <c r="M46" t="n">
-        <v>0.072695635524853</v>
+        <v>0.07130433275947329</v>
       </c>
       <c r="N46" t="n">
         <v>0.08</v>
@@ -11024,7 +11024,7 @@
         <v>460249406.48</v>
       </c>
       <c r="AM46" t="n">
-        <v>4100260184.313725</v>
+        <v>4021786376.470588</v>
       </c>
       <c r="AN46" t="n">
         <v>0.0311</v>
@@ -11065,7 +11065,7 @@
         <v>3.3</v>
       </c>
       <c r="AZ46" t="n">
-        <v>3.45</v>
+        <v>3.38</v>
       </c>
       <c r="BA46" t="n">
         <v>0.42</v>
@@ -11074,19 +11074,19 @@
         <v>7.38</v>
       </c>
       <c r="BC46" t="n">
-        <v>-3.26</v>
+        <v>-1.37</v>
       </c>
       <c r="BD46" t="n">
-        <v>-21.01</v>
+        <v>-19.47</v>
       </c>
       <c r="BE46" t="n">
         <v>-17.5</v>
       </c>
       <c r="BF46" t="n">
-        <v>-89.88</v>
+        <v>-89.68000000000001</v>
       </c>
       <c r="BG46" t="n">
-        <v>76.52</v>
+        <v>79.97</v>
       </c>
       <c r="BH46" t="n">
         <v>1.58</v>
@@ -11095,7 +11095,7 @@
         <v>0</v>
       </c>
       <c r="BJ46" t="n">
-        <v>4.18</v>
+        <v>4.1</v>
       </c>
       <c r="BK46" t="n">
         <v>0.46</v>
@@ -11104,7 +11104,7 @@
         <v>0.46</v>
       </c>
       <c r="BM46" t="n">
-        <v>4.38</v>
+        <v>4.3</v>
       </c>
       <c r="BN46" t="n">
         <v>7.31</v>
@@ -11113,19 +11113,19 @@
         <v>2.97</v>
       </c>
       <c r="BP46" t="n">
+        <v>4.06</v>
+      </c>
+      <c r="BQ46" t="n">
+        <v>8.960000000000001</v>
+      </c>
+      <c r="BR46" t="n">
         <v>4.15</v>
-      </c>
-      <c r="BQ46" t="n">
-        <v>9.140000000000001</v>
-      </c>
-      <c r="BR46" t="n">
-        <v>4.35</v>
       </c>
       <c r="BS46" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="BT46" t="n">
-        <v>25600101</v>
+        <v>26093158</v>
       </c>
     </row>
     <row r="47">
@@ -11155,13 +11155,13 @@
         </is>
       </c>
       <c r="F47" t="n">
-        <v>9.57</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="G47" t="n">
-        <v>3318295952</v>
+        <v>3450056963</v>
       </c>
       <c r="H47" t="n">
-        <v>20500</v>
+        <v>0</v>
       </c>
       <c r="I47" t="n">
         <v>254106600</v>
@@ -11176,7 +11176,7 @@
         <v>1.22</v>
       </c>
       <c r="M47" t="n">
-        <v>0.7824923633395324</v>
+        <v>0.8135631256780317</v>
       </c>
       <c r="N47" t="n">
         <v>0.07000000000000001</v>
@@ -11254,7 +11254,7 @@
         <v>322715382</v>
       </c>
       <c r="AM47" t="n">
-        <v>588350346.0992908</v>
+        <v>611712227.4822695</v>
       </c>
       <c r="AN47" t="n">
         <v>0.4132</v>
@@ -11295,7 +11295,7 @@
         <v>11.74</v>
       </c>
       <c r="AZ47" t="n">
-        <v>12.57</v>
+        <v>13.07</v>
       </c>
       <c r="BA47" t="n">
         <v>1.46</v>
@@ -11304,19 +11304,19 @@
         <v>8.619999999999999</v>
       </c>
       <c r="BC47" t="n">
-        <v>50.19</v>
+        <v>44.46</v>
       </c>
       <c r="BD47" t="n">
-        <v>22.63</v>
+        <v>17.95</v>
       </c>
       <c r="BE47" t="n">
         <v>31.33</v>
       </c>
       <c r="BF47" t="n">
-        <v>-84.76000000000001</v>
+        <v>-85.34</v>
       </c>
       <c r="BG47" t="n">
-        <v>-9.93</v>
+        <v>-13.37</v>
       </c>
       <c r="BH47" t="n">
         <v>7.23</v>
@@ -11325,7 +11325,7 @@
         <v>0</v>
       </c>
       <c r="BJ47" t="n">
-        <v>9.57</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="BK47" t="n">
         <v>1.27</v>
@@ -11334,28 +11334,28 @@
         <v>1.28</v>
       </c>
       <c r="BM47" t="n">
-        <v>9.6</v>
+        <v>9.98</v>
       </c>
       <c r="BN47" t="n">
-        <v>9.9</v>
+        <v>9.98</v>
       </c>
       <c r="BO47" t="n">
         <v>7.13</v>
       </c>
       <c r="BP47" t="n">
-        <v>9.359999999999999</v>
+        <v>9.6</v>
       </c>
       <c r="BQ47" t="n">
-        <v>7.46</v>
+        <v>7.76</v>
       </c>
       <c r="BR47" t="n">
-        <v>9.6</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="BS47" t="n">
         <v>0.53</v>
       </c>
       <c r="BT47" t="n">
-        <v>13090</v>
+        <v>12677</v>
       </c>
     </row>
     <row r="48">
@@ -11385,13 +11385,13 @@
         </is>
       </c>
       <c r="F48" t="n">
-        <v>9.92</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="G48" t="n">
-        <v>3318295952</v>
+        <v>3450056963</v>
       </c>
       <c r="H48" t="n">
-        <v>6200</v>
+        <v>0</v>
       </c>
       <c r="I48" t="n">
         <v>93397546</v>
@@ -11406,7 +11406,7 @@
         <v>1.24</v>
       </c>
       <c r="M48" t="n">
-        <v>2.128926106625684</v>
+        <v>2.213460295321007</v>
       </c>
       <c r="N48" t="n">
         <v>0.07000000000000001</v>
@@ -11484,7 +11484,7 @@
         <v>118614883.42</v>
       </c>
       <c r="AM48" t="n">
-        <v>580121669.9300699</v>
+        <v>603156811.7132868</v>
       </c>
       <c r="AN48" t="n">
         <v>0.4132</v>
@@ -11525,7 +11525,7 @@
         <v>11.74</v>
       </c>
       <c r="AZ48" t="n">
-        <v>12.98</v>
+        <v>12.82</v>
       </c>
       <c r="BA48" t="n">
         <v>1.46</v>
@@ -11534,19 +11534,19 @@
         <v>8.24</v>
       </c>
       <c r="BC48" t="n">
-        <v>44.89</v>
+        <v>46.67</v>
       </c>
       <c r="BD48" t="n">
-        <v>18.31</v>
+        <v>19.75</v>
       </c>
       <c r="BE48" t="n">
         <v>30.83</v>
       </c>
       <c r="BF48" t="n">
-        <v>-85.3</v>
+        <v>-85.12</v>
       </c>
       <c r="BG48" t="n">
-        <v>-16.97</v>
+        <v>-15.96</v>
       </c>
       <c r="BH48" t="n">
         <v>7.23</v>
@@ -11555,7 +11555,7 @@
         <v>0</v>
       </c>
       <c r="BJ48" t="n">
-        <v>9.92</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="BK48" t="n">
         <v>1.27</v>
@@ -11564,7 +11564,7 @@
         <v>1.28</v>
       </c>
       <c r="BM48" t="n">
-        <v>9.92</v>
+        <v>9.98</v>
       </c>
       <c r="BN48" t="n">
         <v>9.99</v>
@@ -11573,19 +11573,19 @@
         <v>7.13</v>
       </c>
       <c r="BP48" t="n">
-        <v>9.69</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="BQ48" t="n">
-        <v>7.73</v>
+        <v>7.64</v>
       </c>
       <c r="BR48" t="n">
-        <v>9.720000000000001</v>
+        <v>9.92</v>
       </c>
       <c r="BS48" t="n">
         <v>0.54</v>
       </c>
       <c r="BT48" t="n">
-        <v>3230</v>
+        <v>3417</v>
       </c>
     </row>
     <row r="49">
@@ -11815,7 +11815,7 @@
         <v>0.54</v>
       </c>
       <c r="BT49" t="n">
-        <v>390</v>
+        <v>397</v>
       </c>
     </row>
     <row r="50">
@@ -11845,13 +11845,13 @@
         </is>
       </c>
       <c r="F50" t="n">
-        <v>35.6</v>
+        <v>36.12</v>
       </c>
       <c r="G50" t="n">
         <v>1000266656</v>
       </c>
       <c r="H50" t="n">
-        <v>1100</v>
+        <v>0</v>
       </c>
       <c r="I50" t="n">
         <v>11540870</v>
@@ -11985,7 +11985,7 @@
         <v>68.48999999999999</v>
       </c>
       <c r="AZ50" t="n">
-        <v>78.5</v>
+        <v>79.64</v>
       </c>
       <c r="BA50" t="n">
         <v>9.210000000000001</v>
@@ -11994,19 +11994,19 @@
         <v>30.53</v>
       </c>
       <c r="BC50" t="n">
-        <v>135.61</v>
+        <v>132.22</v>
       </c>
       <c r="BD50" t="n">
-        <v>92.37</v>
+        <v>89.61</v>
       </c>
       <c r="BE50" t="n">
         <v>120.5</v>
       </c>
       <c r="BF50" t="n">
-        <v>-74.12</v>
+        <v>-74.48999999999999</v>
       </c>
       <c r="BG50" t="n">
-        <v>-14.24</v>
+        <v>-15.48</v>
       </c>
       <c r="BH50" t="n">
         <v>42.6</v>
@@ -12015,7 +12015,7 @@
         <v>0</v>
       </c>
       <c r="BJ50" t="n">
-        <v>35.6</v>
+        <v>36.12</v>
       </c>
       <c r="BK50" t="n">
         <v>7.34</v>
@@ -12024,7 +12024,7 @@
         <v>7.6</v>
       </c>
       <c r="BM50" t="n">
-        <v>36.1</v>
+        <v>36.12</v>
       </c>
       <c r="BN50" t="n">
         <v>39.22</v>
@@ -12033,19 +12033,19 @@
         <v>24.32</v>
       </c>
       <c r="BP50" t="n">
-        <v>35.6</v>
+        <v>36.12</v>
       </c>
       <c r="BQ50" t="n">
-        <v>4.68</v>
+        <v>4.75</v>
       </c>
       <c r="BR50" t="n">
-        <v>35.6</v>
+        <v>36.12</v>
       </c>
       <c r="BS50" t="n">
         <v>0.4</v>
       </c>
       <c r="BT50" t="n">
-        <v>477</v>
+        <v>493</v>
       </c>
     </row>
     <row r="51">
@@ -12523,13 +12523,13 @@
         </is>
       </c>
       <c r="F53" t="n">
-        <v>6.31</v>
+        <v>6.1</v>
       </c>
       <c r="G53" t="n">
-        <v>863538636</v>
+        <v>834799626</v>
       </c>
       <c r="H53" t="n">
-        <v>79100</v>
+        <v>0</v>
       </c>
       <c r="I53" t="n">
         <v>136852484</v>
@@ -12544,7 +12544,7 @@
         <v>2.79</v>
       </c>
       <c r="M53" t="n">
-        <v>2.24331239537583</v>
+        <v>2.168653804924725</v>
       </c>
       <c r="N53" t="n">
         <v>1.48</v>
@@ -12622,7 +12622,7 @@
         <v>39687220.36</v>
       </c>
       <c r="AM53" t="n">
-        <v>43990760.87620988</v>
+        <v>42526725.7259297</v>
       </c>
       <c r="AN53" t="n">
         <v>0</v>
@@ -12672,16 +12672,16 @@
         <v>0</v>
       </c>
       <c r="BC53" t="n">
-        <v>-37.55</v>
+        <v>-35.4</v>
       </c>
       <c r="BD53" t="n">
-        <v>-49.01</v>
+        <v>-47.25</v>
       </c>
       <c r="BE53" t="n">
         <v>-100</v>
       </c>
       <c r="BF53" t="n">
-        <v>-95.40000000000001</v>
+        <v>-95.25</v>
       </c>
       <c r="BG53" t="n">
         <v>-100</v>
@@ -12693,7 +12693,7 @@
         <v>0</v>
       </c>
       <c r="BJ53" t="n">
-        <v>6.31</v>
+        <v>6.1</v>
       </c>
       <c r="BK53" t="n">
         <v>0.29</v>
@@ -12702,7 +12702,7 @@
         <v>0.2</v>
       </c>
       <c r="BM53" t="n">
-        <v>6.63</v>
+        <v>6.23</v>
       </c>
       <c r="BN53" t="n">
         <v>10.29</v>
@@ -12711,19 +12711,19 @@
         <v>4.82</v>
       </c>
       <c r="BP53" t="n">
-        <v>6.31</v>
+        <v>5.9</v>
       </c>
       <c r="BQ53" t="n">
-        <v>30.99</v>
+        <v>29.96</v>
       </c>
       <c r="BR53" t="n">
-        <v>6.53</v>
+        <v>6.23</v>
       </c>
       <c r="BS53" t="n">
         <v>2.36</v>
       </c>
       <c r="BT53" t="n">
-        <v>52797</v>
+        <v>55073</v>
       </c>
     </row>
     <row r="54">
@@ -12753,13 +12753,13 @@
         </is>
       </c>
       <c r="F54" t="n">
-        <v>12.51</v>
+        <v>12.5</v>
       </c>
       <c r="G54" t="n">
-        <v>2917483424</v>
+        <v>2915151250</v>
       </c>
       <c r="H54" t="n">
-        <v>418500</v>
+        <v>0</v>
       </c>
       <c r="I54" t="n">
         <v>233212121</v>
@@ -12774,7 +12774,7 @@
         <v>0.97</v>
       </c>
       <c r="M54" t="n">
-        <v>1.637558882291543</v>
+        <v>1.63624985266096</v>
       </c>
       <c r="N54" t="n">
         <v>0.5600000000000001</v>
@@ -12852,7 +12852,7 @@
         <v>233212121</v>
       </c>
       <c r="AM54" t="n">
-        <v>399108539.5348837</v>
+        <v>398789500.6839945</v>
       </c>
       <c r="AN54" t="n">
         <v>0.1531</v>
@@ -12893,7 +12893,7 @@
         <v>12.25</v>
       </c>
       <c r="AZ54" t="n">
-        <v>19.91</v>
+        <v>19.9</v>
       </c>
       <c r="BA54" t="n">
         <v>0.98</v>
@@ -12902,19 +12902,19 @@
         <v>6.52</v>
       </c>
       <c r="BC54" t="n">
-        <v>19.96</v>
+        <v>20.06</v>
       </c>
       <c r="BD54" t="n">
-        <v>-2.05</v>
+        <v>-1.97</v>
       </c>
       <c r="BE54" t="n">
         <v>59.17</v>
       </c>
       <c r="BF54" t="n">
-        <v>-92.14</v>
+        <v>-92.13</v>
       </c>
       <c r="BG54" t="n">
-        <v>-47.91</v>
+        <v>-47.87</v>
       </c>
       <c r="BH54" t="n">
         <v>10.01</v>
@@ -12923,7 +12923,7 @@
         <v>0</v>
       </c>
       <c r="BJ54" t="n">
-        <v>12.51</v>
+        <v>12.5</v>
       </c>
       <c r="BK54" t="n">
         <v>1</v>
@@ -12932,28 +12932,28 @@
         <v>1</v>
       </c>
       <c r="BM54" t="n">
-        <v>12.83</v>
+        <v>13.06</v>
       </c>
       <c r="BN54" t="n">
-        <v>12.89</v>
+        <v>13.06</v>
       </c>
       <c r="BO54" t="n">
         <v>8.220000000000001</v>
       </c>
       <c r="BP54" t="n">
-        <v>12.01</v>
+        <v>12.25</v>
       </c>
       <c r="BQ54" t="n">
-        <v>12.48</v>
+        <v>12.47</v>
       </c>
       <c r="BR54" t="n">
-        <v>12.33</v>
+        <v>12.25</v>
       </c>
       <c r="BS54" t="n">
         <v>1.26</v>
       </c>
       <c r="BT54" t="n">
-        <v>292480</v>
+        <v>300683</v>
       </c>
     </row>
     <row r="55">
@@ -12983,13 +12983,13 @@
         </is>
       </c>
       <c r="F55" t="n">
-        <v>60.2</v>
+        <v>59.74</v>
       </c>
       <c r="G55" t="n">
-        <v>7956184874</v>
+        <v>7934483463</v>
       </c>
       <c r="H55" t="n">
-        <v>1600</v>
+        <v>0</v>
       </c>
       <c r="I55" t="n">
         <v>84052790</v>
@@ -13004,7 +13004,7 @@
         <v>2</v>
       </c>
       <c r="M55" t="n">
-        <v>1.22820547555566</v>
+        <v>1.224855403600371</v>
       </c>
       <c r="N55" t="n">
         <v>0.16</v>
@@ -13082,7 +13082,7 @@
         <v>579123723.1</v>
       </c>
       <c r="AM55" t="n">
-        <v>400210506.7404427</v>
+        <v>399118886.4688129</v>
       </c>
       <c r="AN55" t="n">
         <v>3.1953</v>
@@ -13123,7 +13123,7 @@
         <v>51.21</v>
       </c>
       <c r="AZ55" t="n">
-        <v>63.31</v>
+        <v>62.83</v>
       </c>
       <c r="BA55" t="n">
         <v>9.380000000000001</v>
@@ -13132,19 +13132,19 @@
         <v>16.08</v>
       </c>
       <c r="BC55" t="n">
-        <v>4.18</v>
+        <v>4.98</v>
       </c>
       <c r="BD55" t="n">
-        <v>-14.94</v>
+        <v>-14.29</v>
       </c>
       <c r="BE55" t="n">
         <v>5.17</v>
       </c>
       <c r="BF55" t="n">
-        <v>-84.42</v>
+        <v>-84.3</v>
       </c>
       <c r="BG55" t="n">
-        <v>-73.3</v>
+        <v>-73.09</v>
       </c>
       <c r="BH55" t="n">
         <v>25.37</v>
@@ -13153,7 +13153,7 @@
         <v>0</v>
       </c>
       <c r="BJ55" t="n">
-        <v>60.2</v>
+        <v>59.74</v>
       </c>
       <c r="BK55" t="n">
         <v>6.89</v>
@@ -13162,7 +13162,7 @@
         <v>7.03</v>
       </c>
       <c r="BM55" t="n">
-        <v>60.2</v>
+        <v>59.74</v>
       </c>
       <c r="BN55" t="n">
         <v>73.67</v>
@@ -13171,19 +13171,19 @@
         <v>36.14</v>
       </c>
       <c r="BP55" t="n">
-        <v>58.35</v>
+        <v>58.3</v>
       </c>
       <c r="BQ55" t="n">
-        <v>8.56</v>
+        <v>8.5</v>
       </c>
       <c r="BR55" t="n">
-        <v>59.03</v>
+        <v>59.01</v>
       </c>
       <c r="BS55" t="n">
         <v>0.66</v>
       </c>
       <c r="BT55" t="n">
-        <v>6847</v>
+        <v>6297</v>
       </c>
     </row>
     <row r="56">
@@ -13213,13 +13213,13 @@
         </is>
       </c>
       <c r="F56" t="n">
-        <v>76.98999999999999</v>
+        <v>76.78</v>
       </c>
       <c r="G56" t="n">
-        <v>7956184874</v>
+        <v>7934483463</v>
       </c>
       <c r="H56" t="n">
-        <v>34500</v>
+        <v>0</v>
       </c>
       <c r="I56" t="n">
         <v>39675836</v>
@@ -13234,7 +13234,7 @@
         <v>2.41</v>
       </c>
       <c r="M56" t="n">
-        <v>2.60193879503207</v>
+        <v>2.594841707158666</v>
       </c>
       <c r="N56" t="n">
         <v>0.19</v>
@@ -13312,7 +13312,7 @@
         <v>273366510.04</v>
       </c>
       <c r="AM56" t="n">
-        <v>330956109.5673877</v>
+        <v>330053388.6439268</v>
       </c>
       <c r="AN56" t="n">
         <v>3.5102</v>
@@ -13353,7 +13353,7 @@
         <v>51.21</v>
       </c>
       <c r="AZ56" t="n">
-        <v>73.53</v>
+        <v>73.31999999999999</v>
       </c>
       <c r="BA56" t="n">
         <v>9.380000000000001</v>
@@ -13362,19 +13362,19 @@
         <v>17.68</v>
       </c>
       <c r="BC56" t="n">
-        <v>-18.54</v>
+        <v>-18.32</v>
       </c>
       <c r="BD56" t="n">
-        <v>-33.49</v>
+        <v>-33.31</v>
       </c>
       <c r="BE56" t="n">
         <v>-4.5</v>
       </c>
       <c r="BF56" t="n">
-        <v>-87.81999999999999</v>
+        <v>-87.79000000000001</v>
       </c>
       <c r="BG56" t="n">
-        <v>-77.04000000000001</v>
+        <v>-76.98</v>
       </c>
       <c r="BH56" t="n">
         <v>25.37</v>
@@ -13383,7 +13383,7 @@
         <v>0</v>
       </c>
       <c r="BJ56" t="n">
-        <v>76.98999999999999</v>
+        <v>76.78</v>
       </c>
       <c r="BK56" t="n">
         <v>6.89</v>
@@ -13392,7 +13392,7 @@
         <v>7.03</v>
       </c>
       <c r="BM56" t="n">
-        <v>78.98</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="BN56" t="n">
         <v>86.77</v>
@@ -13401,19 +13401,19 @@
         <v>46.42</v>
       </c>
       <c r="BP56" t="n">
-        <v>75.84999999999999</v>
+        <v>72.23999999999999</v>
       </c>
       <c r="BQ56" t="n">
-        <v>10.95</v>
+        <v>10.92</v>
       </c>
       <c r="BR56" t="n">
-        <v>78.98</v>
+        <v>76.98999999999999</v>
       </c>
       <c r="BS56" t="n">
         <v>0.79</v>
       </c>
       <c r="BT56" t="n">
-        <v>31147</v>
+        <v>30973</v>
       </c>
     </row>
     <row r="57">
@@ -13443,13 +13443,13 @@
         </is>
       </c>
       <c r="F57" t="n">
-        <v>6.97</v>
+        <v>7.07</v>
       </c>
       <c r="G57" t="n">
-        <v>1629990210</v>
+        <v>1653376100</v>
       </c>
       <c r="H57" t="n">
-        <v>1071800</v>
+        <v>0</v>
       </c>
       <c r="I57" t="n">
         <v>233858065</v>
@@ -13464,7 +13464,7 @@
         <v>0.77</v>
       </c>
       <c r="M57" t="n">
-        <v>0.4878998494236237</v>
+        <v>0.4948998744174165</v>
       </c>
       <c r="N57" t="n">
         <v>0.08</v>
@@ -13542,7 +13542,7 @@
         <v>229180903.7</v>
       </c>
       <c r="AM57" t="n">
-        <v>121914002.2438295</v>
+        <v>123663133.881825</v>
       </c>
       <c r="AN57" t="n">
         <v>0.347</v>
@@ -13583,7 +13583,7 @@
         <v>10.72</v>
       </c>
       <c r="AZ57" t="n">
-        <v>10.63</v>
+        <v>10.78</v>
       </c>
       <c r="BA57" t="n">
         <v>1.13</v>
@@ -13592,19 +13592,19 @@
         <v>6.26</v>
       </c>
       <c r="BC57" t="n">
-        <v>88.40000000000001</v>
+        <v>85.73</v>
       </c>
       <c r="BD57" t="n">
-        <v>53.83</v>
+        <v>51.65</v>
       </c>
       <c r="BE57" t="n">
         <v>52.5</v>
       </c>
       <c r="BF57" t="n">
-        <v>-83.81999999999999</v>
+        <v>-84.05</v>
       </c>
       <c r="BG57" t="n">
-        <v>-10.13</v>
+        <v>-11.4</v>
       </c>
       <c r="BH57" t="n">
         <v>7.82</v>
@@ -13613,7 +13613,7 @@
         <v>0</v>
       </c>
       <c r="BJ57" t="n">
-        <v>6.97</v>
+        <v>7.07</v>
       </c>
       <c r="BK57" t="n">
         <v>0.98</v>
@@ -13622,28 +13622,28 @@
         <v>1.04</v>
       </c>
       <c r="BM57" t="n">
-        <v>7</v>
+        <v>7.15</v>
       </c>
       <c r="BN57" t="n">
-        <v>7.09</v>
+        <v>7.15</v>
       </c>
       <c r="BO57" t="n">
         <v>3.48</v>
       </c>
       <c r="BP57" t="n">
-        <v>6.78</v>
+        <v>6.81</v>
       </c>
       <c r="BQ57" t="n">
-        <v>6.73</v>
+        <v>6.83</v>
       </c>
       <c r="BR57" t="n">
-        <v>7</v>
+        <v>6.92</v>
       </c>
       <c r="BS57" t="n">
         <v>0.42</v>
       </c>
       <c r="BT57" t="n">
-        <v>1707633</v>
+        <v>1701807</v>
       </c>
     </row>
     <row r="58">
@@ -14133,13 +14133,13 @@
         </is>
       </c>
       <c r="F60" t="n">
-        <v>382.11</v>
+        <v>389</v>
       </c>
       <c r="G60" t="n">
-        <v>173764515</v>
+        <v>176897750</v>
       </c>
       <c r="H60" t="n">
-        <v>54</v>
+        <v>0</v>
       </c>
       <c r="I60" t="n">
         <v>454750</v>
@@ -14154,7 +14154,7 @@
         <v>0.83</v>
       </c>
       <c r="M60" t="n">
-        <v>12.99734111267628</v>
+        <v>13.23170268000306</v>
       </c>
       <c r="N60" t="n">
         <v>0.68</v>
@@ -14232,7 +14232,7 @@
         <v>59558607.5</v>
       </c>
       <c r="AM60" t="n">
-        <v>-25478667.88856305</v>
+        <v>-25938086.51026393</v>
       </c>
       <c r="AN60" t="n">
         <v>10.0581</v>
@@ -14273,7 +14273,7 @@
         <v>944.87</v>
       </c>
       <c r="AZ60" t="n">
-        <v>2197.13</v>
+        <v>2236.75</v>
       </c>
       <c r="BA60" t="n">
         <v>231.1</v>
@@ -14282,19 +14282,19 @@
         <v>727.97</v>
       </c>
       <c r="BC60" t="n">
-        <v>202.85</v>
+        <v>197.49</v>
       </c>
       <c r="BD60" t="n">
-        <v>147.28</v>
+        <v>142.9</v>
       </c>
       <c r="BE60" t="n">
         <v>475</v>
       </c>
       <c r="BF60" t="n">
-        <v>-39.52</v>
+        <v>-40.59</v>
       </c>
       <c r="BG60" t="n">
-        <v>90.51000000000001</v>
+        <v>87.14</v>
       </c>
       <c r="BH60" t="n">
         <v>454.44</v>
@@ -14303,7 +14303,7 @@
         <v>0</v>
       </c>
       <c r="BJ60" t="n">
-        <v>382.11</v>
+        <v>389</v>
       </c>
       <c r="BK60" t="n">
         <v>130.97</v>
@@ -14312,7 +14312,7 @@
         <v>130.97</v>
       </c>
       <c r="BM60" t="n">
-        <v>382.57</v>
+        <v>389</v>
       </c>
       <c r="BN60" t="n">
         <v>415</v>
@@ -14321,19 +14321,19 @@
         <v>310.74</v>
       </c>
       <c r="BP60" t="n">
-        <v>382.11</v>
+        <v>380</v>
       </c>
       <c r="BQ60" t="n">
-        <v>2.92</v>
+        <v>2.97</v>
       </c>
       <c r="BR60" t="n">
-        <v>382.57</v>
+        <v>380</v>
       </c>
       <c r="BS60" t="n">
         <v>12.82</v>
       </c>
       <c r="BT60" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="61">
@@ -14369,7 +14369,7 @@
         <v>2777992320</v>
       </c>
       <c r="H61" t="n">
-        <v>889100</v>
+        <v>0</v>
       </c>
       <c r="I61" t="n">
         <v>85608392</v>
@@ -14542,7 +14542,7 @@
         <v>1.86</v>
       </c>
       <c r="BM61" t="n">
-        <v>32.84</v>
+        <v>33.1</v>
       </c>
       <c r="BN61" t="n">
         <v>34.8</v>
@@ -14551,19 +14551,19 @@
         <v>19.35</v>
       </c>
       <c r="BP61" t="n">
-        <v>31.87</v>
+        <v>31.42</v>
       </c>
       <c r="BQ61" t="n">
         <v>17.43</v>
       </c>
       <c r="BR61" t="n">
-        <v>32.84</v>
+        <v>31.87</v>
       </c>
       <c r="BS61" t="n">
         <v>1.19</v>
       </c>
       <c r="BT61" t="n">
-        <v>1001953</v>
+        <v>996783</v>
       </c>
     </row>
     <row r="62">
@@ -14823,13 +14823,13 @@
         </is>
       </c>
       <c r="F63" t="n">
-        <v>1.55</v>
+        <v>1.66</v>
       </c>
       <c r="G63" t="n">
-        <v>403790177</v>
+        <v>432446259</v>
       </c>
       <c r="H63" t="n">
-        <v>3200</v>
+        <v>0</v>
       </c>
       <c r="I63" t="n">
         <v>122894462</v>
@@ -14844,7 +14844,7 @@
         <v>-0.22</v>
       </c>
       <c r="M63" t="n">
-        <v>0.4966410796663263</v>
+        <v>0.5318865816971664</v>
       </c>
       <c r="N63" t="n">
         <v>0.37</v>
@@ -14922,7 +14922,7 @@
         <v>31952560.12</v>
       </c>
       <c r="AM63" t="n">
-        <v>229426236.9318182</v>
+        <v>245708101.7045455</v>
       </c>
       <c r="AN63" t="n">
         <v>0</v>
@@ -14981,7 +14981,7 @@
         <v>-100</v>
       </c>
       <c r="BF63" t="n">
-        <v>-81.34</v>
+        <v>-82.58</v>
       </c>
       <c r="BG63" t="n">
         <v>-100</v>
@@ -14993,7 +14993,7 @@
         <v>0</v>
       </c>
       <c r="BJ63" t="n">
-        <v>1.55</v>
+        <v>1.66</v>
       </c>
       <c r="BK63" t="n">
         <v>0.26</v>
@@ -15002,7 +15002,7 @@
         <v>0.26</v>
       </c>
       <c r="BM63" t="n">
-        <v>1.65</v>
+        <v>1.69</v>
       </c>
       <c r="BN63" t="n">
         <v>2.12</v>
@@ -15011,19 +15011,19 @@
         <v>1.16</v>
       </c>
       <c r="BP63" t="n">
-        <v>1.53</v>
+        <v>1.56</v>
       </c>
       <c r="BQ63" t="n">
-        <v>5.94</v>
+        <v>6.36</v>
       </c>
       <c r="BR63" t="n">
-        <v>1.55</v>
+        <v>1.56</v>
       </c>
       <c r="BS63" t="n">
         <v>0.19</v>
       </c>
       <c r="BT63" t="n">
-        <v>34910</v>
+        <v>30850</v>
       </c>
     </row>
     <row r="64">
@@ -15053,13 +15053,13 @@
         </is>
       </c>
       <c r="F64" t="n">
-        <v>78.08</v>
+        <v>77.13</v>
       </c>
       <c r="G64" t="n">
-        <v>265835780954</v>
+        <v>262601339318</v>
       </c>
       <c r="H64" t="n">
-        <v>15024110</v>
+        <v>0</v>
       </c>
       <c r="I64" t="n">
         <v>0</v>
@@ -15146,13 +15146,13 @@
         <v>41.22</v>
       </c>
       <c r="AK64" t="n">
-        <v>76219019319.40817</v>
+        <v>75291657439.61502</v>
       </c>
       <c r="AL64" t="n">
-        <v>21249862586.251</v>
+        <v>20991314094.16467</v>
       </c>
       <c r="AM64" t="n">
-        <v>23671930628.13891</v>
+        <v>23383912673.0187</v>
       </c>
       <c r="AN64" t="n">
         <v>1.4201</v>
@@ -15193,7 +15193,7 @@
         <v>38.98</v>
       </c>
       <c r="AZ64" t="n">
-        <v>31.23</v>
+        <v>30.85</v>
       </c>
       <c r="BA64" t="n">
         <v>6.69</v>
@@ -15202,28 +15202,28 @@
         <v>10.4</v>
       </c>
       <c r="BC64" t="n">
-        <v>-38.86</v>
+        <v>-38.1</v>
       </c>
       <c r="BD64" t="n">
-        <v>-50.08</v>
+        <v>-49.46</v>
       </c>
       <c r="BE64" t="n">
         <v>-60</v>
       </c>
       <c r="BF64" t="n">
-        <v>-91.43000000000001</v>
+        <v>-91.31999999999999</v>
       </c>
       <c r="BG64" t="n">
-        <v>-86.68000000000001</v>
+        <v>-86.52</v>
       </c>
       <c r="BH64" t="n">
         <v>21.37</v>
       </c>
       <c r="BI64" t="n">
-        <v>-0.28</v>
+        <v>0</v>
       </c>
       <c r="BJ64" t="n">
-        <v>78.3</v>
+        <v>77.13</v>
       </c>
       <c r="BK64" t="n">
         <v>4.74</v>
@@ -15232,7 +15232,7 @@
         <v>1.57</v>
       </c>
       <c r="BM64" t="n">
-        <v>79.40000000000001</v>
+        <v>78.48</v>
       </c>
       <c r="BN64" t="n">
         <v>84.59</v>
@@ -15241,19 +15241,19 @@
         <v>44.12</v>
       </c>
       <c r="BP64" t="n">
-        <v>77.03</v>
+        <v>76.53</v>
       </c>
       <c r="BQ64" t="n">
-        <v>49.73</v>
+        <v>49.12</v>
       </c>
       <c r="BR64" t="n">
-        <v>78.7</v>
+        <v>77.40000000000001</v>
       </c>
       <c r="BS64" t="n">
         <v>3.49</v>
       </c>
       <c r="BT64" t="n">
-        <v>14027903</v>
+        <v>14281497</v>
       </c>
     </row>
     <row r="65">
@@ -15283,13 +15283,13 @@
         </is>
       </c>
       <c r="F65" t="n">
-        <v>26.53</v>
+        <v>25.89</v>
       </c>
       <c r="G65" t="n">
-        <v>265835780954</v>
+        <v>262601339318</v>
       </c>
       <c r="H65" t="n">
-        <v>17200</v>
+        <v>0</v>
       </c>
       <c r="I65" t="n">
         <v>7298813414</v>
@@ -15304,7 +15304,7 @@
         <v>3.29</v>
       </c>
       <c r="M65" t="n">
-        <v>6.426830656309988</v>
+        <v>6.348634980063203</v>
       </c>
       <c r="N65" t="n">
         <v>0.29</v>
@@ -15382,7 +15382,7 @@
         <v>11532125194.12</v>
       </c>
       <c r="AM65" t="n">
-        <v>19912792580.82397</v>
+        <v>19670512308.46442</v>
       </c>
       <c r="AN65" t="n">
         <v>0.4734</v>
@@ -15423,7 +15423,7 @@
         <v>12.99</v>
       </c>
       <c r="AZ65" t="n">
-        <v>8.93</v>
+        <v>8.720000000000001</v>
       </c>
       <c r="BA65" t="n">
         <v>2.23</v>
@@ -15432,19 +15432,19 @@
         <v>3.47</v>
       </c>
       <c r="BC65" t="n">
-        <v>-40.03</v>
+        <v>-38.55</v>
       </c>
       <c r="BD65" t="n">
-        <v>-51.04</v>
+        <v>-49.83</v>
       </c>
       <c r="BE65" t="n">
         <v>-66.33</v>
       </c>
       <c r="BF65" t="n">
-        <v>-91.59</v>
+        <v>-91.38</v>
       </c>
       <c r="BG65" t="n">
-        <v>-86.94</v>
+        <v>-86.61</v>
       </c>
       <c r="BH65" t="n">
         <v>7.12</v>
@@ -15453,7 +15453,7 @@
         <v>0</v>
       </c>
       <c r="BJ65" t="n">
-        <v>26.53</v>
+        <v>25.89</v>
       </c>
       <c r="BK65" t="n">
         <v>1.58</v>
@@ -15462,7 +15462,7 @@
         <v>1.57</v>
       </c>
       <c r="BM65" t="n">
-        <v>26.74</v>
+        <v>26.53</v>
       </c>
       <c r="BN65" t="n">
         <v>46.43</v>
@@ -15471,19 +15471,19 @@
         <v>20.44</v>
       </c>
       <c r="BP65" t="n">
-        <v>26.1</v>
+        <v>25.8</v>
       </c>
       <c r="BQ65" t="n">
-        <v>16.9</v>
+        <v>16.49</v>
       </c>
       <c r="BR65" t="n">
-        <v>26.7</v>
+        <v>26.53</v>
       </c>
       <c r="BS65" t="n">
         <v>4.14</v>
       </c>
       <c r="BT65" t="n">
-        <v>13000</v>
+        <v>13427</v>
       </c>
     </row>
     <row r="66">
@@ -15513,13 +15513,13 @@
         </is>
       </c>
       <c r="F66" t="n">
-        <v>26</v>
+        <v>25.98</v>
       </c>
       <c r="G66" t="n">
-        <v>265835780954</v>
+        <v>262601339318</v>
       </c>
       <c r="H66" t="n">
-        <v>5000</v>
+        <v>0</v>
       </c>
       <c r="I66" t="n">
         <v>2972355254</v>
@@ -15534,7 +15534,7 @@
         <v>2.75</v>
       </c>
       <c r="M66" t="n">
-        <v>15.78150449568763</v>
+        <v>15.58948988036237</v>
       </c>
       <c r="N66" t="n">
         <v>0.25</v>
@@ -15612,7 +15612,7 @@
         <v>4696321301.320001</v>
       </c>
       <c r="AM66" t="n">
-        <v>23841774076.59193</v>
+        <v>23551689624.93274</v>
       </c>
       <c r="AN66" t="n">
         <v>0.4734</v>
@@ -15662,19 +15662,19 @@
         <v>3.47</v>
       </c>
       <c r="BC66" t="n">
-        <v>-38.81</v>
+        <v>-38.76</v>
       </c>
       <c r="BD66" t="n">
-        <v>-50.04</v>
+        <v>-50</v>
       </c>
       <c r="BE66" t="n">
         <v>-59.83</v>
       </c>
       <c r="BF66" t="n">
-        <v>-91.42</v>
+        <v>-91.41</v>
       </c>
       <c r="BG66" t="n">
-        <v>-86.67</v>
+        <v>-86.66</v>
       </c>
       <c r="BH66" t="n">
         <v>7.12</v>
@@ -15683,7 +15683,7 @@
         <v>0</v>
       </c>
       <c r="BJ66" t="n">
-        <v>26</v>
+        <v>25.98</v>
       </c>
       <c r="BK66" t="n">
         <v>1.58</v>
@@ -15692,7 +15692,7 @@
         <v>1.57</v>
       </c>
       <c r="BM66" t="n">
-        <v>26.72</v>
+        <v>28.11</v>
       </c>
       <c r="BN66" t="n">
         <v>28.51</v>
@@ -15701,19 +15701,19 @@
         <v>9.48</v>
       </c>
       <c r="BP66" t="n">
-        <v>25.7</v>
+        <v>25.27</v>
       </c>
       <c r="BQ66" t="n">
-        <v>16.56</v>
+        <v>16.55</v>
       </c>
       <c r="BR66" t="n">
-        <v>26.71</v>
+        <v>26.01</v>
       </c>
       <c r="BS66" t="n">
         <v>3.46</v>
       </c>
       <c r="BT66" t="n">
-        <v>5660</v>
+        <v>5743</v>
       </c>
     </row>
     <row r="67">
@@ -15973,13 +15973,13 @@
         </is>
       </c>
       <c r="F68" t="n">
-        <v>17.9</v>
+        <v>17.92</v>
       </c>
       <c r="G68" t="n">
-        <v>7631941315</v>
+        <v>7590278602</v>
       </c>
       <c r="H68" t="n">
-        <v>256800</v>
+        <v>0</v>
       </c>
       <c r="I68" t="n">
         <v>137989898</v>
@@ -16072,7 +16072,7 @@
         <v>205604948.02</v>
       </c>
       <c r="AM68" t="n">
-        <v>529260840.1525659</v>
+        <v>526371609.0152566</v>
       </c>
       <c r="AN68" t="n">
         <v>0.1911</v>
@@ -16113,7 +16113,7 @@
         <v>21.39</v>
       </c>
       <c r="AZ68" t="n">
-        <v>33.11</v>
+        <v>33.15</v>
       </c>
       <c r="BA68" t="n">
         <v>1.24</v>
@@ -16122,10 +16122,10 @@
         <v>63.25</v>
       </c>
       <c r="BC68" t="n">
-        <v>46.38</v>
+        <v>46.22</v>
       </c>
       <c r="BD68" t="n">
-        <v>19.52</v>
+        <v>19.39</v>
       </c>
       <c r="BE68" t="n">
         <v>85</v>
@@ -16134,7 +16134,7 @@
         <v>-93.08</v>
       </c>
       <c r="BG68" t="n">
-        <v>253.34</v>
+        <v>252.95</v>
       </c>
       <c r="BH68" t="n">
         <v>20.48</v>
@@ -16143,7 +16143,7 @@
         <v>0</v>
       </c>
       <c r="BJ68" t="n">
-        <v>17.9</v>
+        <v>17.92</v>
       </c>
       <c r="BK68" t="n">
         <v>1.49</v>
@@ -16152,7 +16152,7 @@
         <v>1.49</v>
       </c>
       <c r="BM68" t="n">
-        <v>18.27</v>
+        <v>18.16</v>
       </c>
       <c r="BN68" t="n">
         <v>22.11</v>
@@ -16164,16 +16164,16 @@
         <v>17.79</v>
       </c>
       <c r="BQ68" t="n">
-        <v>12.04</v>
+        <v>12.05</v>
       </c>
       <c r="BR68" t="n">
-        <v>18.27</v>
+        <v>17.9</v>
       </c>
       <c r="BS68" t="n">
         <v>0</v>
       </c>
       <c r="BT68" t="n">
-        <v>65980</v>
+        <v>73153</v>
       </c>
     </row>
     <row r="69">
@@ -16203,13 +16203,13 @@
         </is>
       </c>
       <c r="F69" t="n">
-        <v>20.15</v>
+        <v>20.04</v>
       </c>
       <c r="G69" t="n">
-        <v>7631941315</v>
+        <v>7590278602</v>
       </c>
       <c r="H69" t="n">
-        <v>4189900</v>
+        <v>0</v>
       </c>
       <c r="I69" t="n">
         <v>255106712</v>
@@ -16302,7 +16302,7 @@
         <v>380109000.88</v>
       </c>
       <c r="AM69" t="n">
-        <v>454282221.1309524</v>
+        <v>451802297.7380952</v>
       </c>
       <c r="AN69" t="n">
         <v>0.8856000000000001</v>
@@ -16343,7 +16343,7 @@
         <v>21.39</v>
       </c>
       <c r="AZ69" t="n">
-        <v>35.23</v>
+        <v>35.04</v>
       </c>
       <c r="BA69" t="n">
         <v>1.24</v>
@@ -16352,19 +16352,19 @@
         <v>69.59</v>
       </c>
       <c r="BC69" t="n">
-        <v>30.04</v>
+        <v>30.75</v>
       </c>
       <c r="BD69" t="n">
-        <v>6.18</v>
+        <v>6.76</v>
       </c>
       <c r="BE69" t="n">
         <v>74.83</v>
       </c>
       <c r="BF69" t="n">
-        <v>-93.84999999999999</v>
+        <v>-93.81</v>
       </c>
       <c r="BG69" t="n">
-        <v>245.34</v>
+        <v>247.24</v>
       </c>
       <c r="BH69" t="n">
         <v>20.48</v>
@@ -16373,7 +16373,7 @@
         <v>0</v>
       </c>
       <c r="BJ69" t="n">
-        <v>20.15</v>
+        <v>20.04</v>
       </c>
       <c r="BK69" t="n">
         <v>1.49</v>
@@ -16382,7 +16382,7 @@
         <v>1.49</v>
       </c>
       <c r="BM69" t="n">
-        <v>20.4</v>
+        <v>20.25</v>
       </c>
       <c r="BN69" t="n">
         <v>25.63</v>
@@ -16391,19 +16391,19 @@
         <v>17.11</v>
       </c>
       <c r="BP69" t="n">
-        <v>19.88</v>
+        <v>19.82</v>
       </c>
       <c r="BQ69" t="n">
-        <v>13.55</v>
+        <v>13.48</v>
       </c>
       <c r="BR69" t="n">
-        <v>20.33</v>
+        <v>19.91</v>
       </c>
       <c r="BS69" t="n">
         <v>0</v>
       </c>
       <c r="BT69" t="n">
-        <v>3082490</v>
+        <v>3146667</v>
       </c>
     </row>
     <row r="70">
@@ -16433,13 +16433,13 @@
         </is>
       </c>
       <c r="F70" t="n">
-        <v>20.55</v>
+        <v>20.69</v>
       </c>
       <c r="G70" t="n">
-        <v>9546650105</v>
+        <v>9611688716</v>
       </c>
       <c r="H70" t="n">
-        <v>4186100</v>
+        <v>0</v>
       </c>
       <c r="I70" t="n">
         <v>464557268</v>
@@ -16454,7 +16454,7 @@
         <v>0.68</v>
       </c>
       <c r="M70" t="n">
-        <v>0.7534998616862311</v>
+        <v>0.7586332418618695</v>
       </c>
       <c r="N70" t="n">
         <v>0.2</v>
@@ -16532,7 +16532,7 @@
         <v>55746872.16</v>
       </c>
       <c r="AM70" t="n">
-        <v>3150709605.610561</v>
+        <v>3172174493.729373</v>
       </c>
       <c r="AN70" t="n">
         <v>0.1236</v>
@@ -16573,7 +16573,7 @@
         <v>6.9</v>
       </c>
       <c r="AZ70" t="n">
-        <v>2.36</v>
+        <v>2.38</v>
       </c>
       <c r="BA70" t="n">
         <v>0.12</v>
@@ -16582,10 +16582,10 @@
         <v>1.07</v>
       </c>
       <c r="BC70" t="n">
-        <v>-58.88</v>
+        <v>-59.16</v>
       </c>
       <c r="BD70" t="n">
-        <v>-66.43000000000001</v>
+        <v>-66.66</v>
       </c>
       <c r="BE70" t="n">
         <v>-88.5</v>
@@ -16594,7 +16594,7 @@
         <v>-99.42</v>
       </c>
       <c r="BG70" t="n">
-        <v>-94.8</v>
+        <v>-94.83</v>
       </c>
       <c r="BH70" t="n">
         <v>26.44</v>
@@ -16603,7 +16603,7 @@
         <v>0</v>
       </c>
       <c r="BJ70" t="n">
-        <v>20.55</v>
+        <v>20.69</v>
       </c>
       <c r="BK70" t="n">
         <v>0.12</v>
@@ -16612,7 +16612,7 @@
         <v>0.1</v>
       </c>
       <c r="BM70" t="n">
-        <v>20.92</v>
+        <v>20.78</v>
       </c>
       <c r="BN70" t="n">
         <v>22.15</v>
@@ -16621,19 +16621,19 @@
         <v>13.21</v>
       </c>
       <c r="BP70" t="n">
-        <v>20.4</v>
+        <v>20.15</v>
       </c>
       <c r="BQ70" t="n">
-        <v>206.1</v>
+        <v>207.5</v>
       </c>
       <c r="BR70" t="n">
-        <v>20.8</v>
+        <v>20.2</v>
       </c>
       <c r="BS70" t="n">
         <v>0.67</v>
       </c>
       <c r="BT70" t="n">
-        <v>3882937</v>
+        <v>3900647</v>
       </c>
     </row>
     <row r="71">

</xml_diff>

<commit_message>
📊 Dados atualizados - 2026-10-17 05:14
</commit_message>
<xml_diff>
--- a/data/ativos.xlsx
+++ b/data/ativos.xlsx
@@ -1047,13 +1047,13 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>28.94</v>
+        <v>28.66</v>
       </c>
       <c r="G3" t="n">
-        <v>3871211263</v>
+        <v>3833756467</v>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>491900</v>
       </c>
       <c r="I3" t="n">
         <v>129510368</v>
@@ -1068,7 +1068,7 @@
         <v>0.88</v>
       </c>
       <c r="M3" t="n">
-        <v>0.9632435796188668</v>
+        <v>0.9539239922024528</v>
       </c>
       <c r="N3" t="n">
         <v>0.09</v>
@@ -1146,7 +1146,7 @@
         <v>506385538.88</v>
       </c>
       <c r="AM3" t="n">
-        <v>756095949.8046875</v>
+        <v>748780559.9609375</v>
       </c>
       <c r="AN3" t="n">
         <v>2.7</v>
@@ -1187,7 +1187,7 @@
         <v>40.42</v>
       </c>
       <c r="AZ3" t="n">
-        <v>52.96</v>
+        <v>52.45</v>
       </c>
       <c r="BA3" t="n">
         <v>4.87</v>
@@ -1196,19 +1196,19 @@
         <v>21.14</v>
       </c>
       <c r="BC3" t="n">
-        <v>71.04000000000001</v>
+        <v>72.70999999999999</v>
       </c>
       <c r="BD3" t="n">
-        <v>39.65</v>
+        <v>41.02</v>
       </c>
       <c r="BE3" t="n">
         <v>83</v>
       </c>
       <c r="BF3" t="n">
-        <v>-83.18000000000001</v>
+        <v>-83.01000000000001</v>
       </c>
       <c r="BG3" t="n">
-        <v>-26.97</v>
+        <v>-26.25</v>
       </c>
       <c r="BH3" t="n">
         <v>27.85</v>
@@ -1217,7 +1217,7 @@
         <v>0</v>
       </c>
       <c r="BJ3" t="n">
-        <v>28.94</v>
+        <v>28.66</v>
       </c>
       <c r="BK3" t="n">
         <v>3.91</v>
@@ -1226,7 +1226,7 @@
         <v>4.39</v>
       </c>
       <c r="BM3" t="n">
-        <v>29.26</v>
+        <v>29.04</v>
       </c>
       <c r="BN3" t="n">
         <v>29.56</v>
@@ -1235,19 +1235,19 @@
         <v>18.72</v>
       </c>
       <c r="BP3" t="n">
-        <v>28.18</v>
+        <v>28.3</v>
       </c>
       <c r="BQ3" t="n">
-        <v>6.59</v>
+        <v>6.52</v>
       </c>
       <c r="BR3" t="n">
-        <v>28.27</v>
+        <v>28.94</v>
       </c>
       <c r="BS3" t="n">
         <v>0.79</v>
       </c>
       <c r="BT3" t="n">
-        <v>718217</v>
+        <v>713560</v>
       </c>
     </row>
     <row r="4">
@@ -1277,13 +1277,13 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>16.69</v>
+        <v>16.84</v>
       </c>
       <c r="G4" t="n">
-        <v>258438983669</v>
+        <v>260761676762</v>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
+        <v>33731100</v>
       </c>
       <c r="I4" t="n">
         <v>15484664889</v>
@@ -1298,7 +1298,7 @@
         <v>2.76</v>
       </c>
       <c r="M4" t="n">
-        <v>2.926312503033508</v>
+        <v>2.952612427844623</v>
       </c>
       <c r="N4" t="n">
         <v>1.76</v>
@@ -1376,7 +1376,7 @@
         <v>16258898133.45</v>
       </c>
       <c r="AM4" t="n">
-        <v>25588018185.04951</v>
+        <v>25817987798.21782</v>
       </c>
       <c r="AN4" t="n">
         <v>0.269</v>
@@ -1417,7 +1417,7 @@
         <v>9.470000000000001</v>
       </c>
       <c r="AZ4" t="n">
-        <v>20.83</v>
+        <v>21.02</v>
       </c>
       <c r="BA4" t="n">
         <v>1.13</v>
@@ -1426,19 +1426,19 @@
         <v>11.39</v>
       </c>
       <c r="BC4" t="n">
-        <v>-30.47</v>
+        <v>-31.09</v>
       </c>
       <c r="BD4" t="n">
-        <v>-43.23</v>
+        <v>-43.74</v>
       </c>
       <c r="BE4" t="n">
         <v>24.83</v>
       </c>
       <c r="BF4" t="n">
-        <v>-93.23999999999999</v>
+        <v>-93.3</v>
       </c>
       <c r="BG4" t="n">
-        <v>-31.78</v>
+        <v>-32.38</v>
       </c>
       <c r="BH4" t="n">
         <v>5.7</v>
@@ -1447,7 +1447,7 @@
         <v>0</v>
       </c>
       <c r="BJ4" t="n">
-        <v>16.69</v>
+        <v>16.84</v>
       </c>
       <c r="BK4" t="n">
         <v>1.05</v>
@@ -1456,28 +1456,28 @@
         <v>1.04</v>
       </c>
       <c r="BM4" t="n">
-        <v>16.82</v>
+        <v>16.93</v>
       </c>
       <c r="BN4" t="n">
         <v>16.94</v>
       </c>
       <c r="BO4" t="n">
-        <v>11.26</v>
+        <v>11.33</v>
       </c>
       <c r="BP4" t="n">
-        <v>16.33</v>
+        <v>16.66</v>
       </c>
       <c r="BQ4" t="n">
-        <v>16.1</v>
+        <v>16.24</v>
       </c>
       <c r="BR4" t="n">
-        <v>16.38</v>
+        <v>16.7</v>
       </c>
       <c r="BS4" t="n">
         <v>2.76</v>
       </c>
       <c r="BT4" t="n">
-        <v>32464360</v>
+        <v>32465157</v>
       </c>
     </row>
     <row r="5">
@@ -1737,13 +1737,13 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>7</v>
+        <v>6.8</v>
       </c>
       <c r="G6" t="n">
-        <v>441592830</v>
+        <v>428975972</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>1400</v>
       </c>
       <c r="I6" t="n">
         <v>63084700</v>
@@ -1758,7 +1758,7 @@
         <v>1.91</v>
       </c>
       <c r="M6" t="n">
-        <v>6.874735752342318</v>
+        <v>6.678315976290189</v>
       </c>
       <c r="N6" t="n">
         <v>1.26</v>
@@ -1836,7 +1836,7 @@
         <v>35958279</v>
       </c>
       <c r="AM6" t="n">
-        <v>42217287.76290631</v>
+        <v>41011087.18929254</v>
       </c>
       <c r="AN6" t="n">
         <v>0.5199</v>
@@ -1877,7 +1877,7 @@
         <v>5.74</v>
       </c>
       <c r="AZ6" t="n">
-        <v>8.210000000000001</v>
+        <v>7.98</v>
       </c>
       <c r="BA6" t="n">
         <v>0.65</v>
@@ -1886,19 +1886,19 @@
         <v>7.95</v>
       </c>
       <c r="BC6" t="n">
-        <v>0.51</v>
+        <v>3.47</v>
       </c>
       <c r="BD6" t="n">
-        <v>-17.93</v>
+        <v>-15.52</v>
       </c>
       <c r="BE6" t="n">
         <v>17.33</v>
       </c>
       <c r="BF6" t="n">
-        <v>-90.73999999999999</v>
+        <v>-90.45999999999999</v>
       </c>
       <c r="BG6" t="n">
-        <v>13.62</v>
+        <v>16.96</v>
       </c>
       <c r="BH6" t="n">
         <v>3.86</v>
@@ -1907,7 +1907,7 @@
         <v>0</v>
       </c>
       <c r="BJ6" t="n">
-        <v>7</v>
+        <v>6.8</v>
       </c>
       <c r="BK6" t="n">
         <v>0.57</v>
@@ -1916,7 +1916,7 @@
         <v>0.5600000000000001</v>
       </c>
       <c r="BM6" t="n">
-        <v>7.07</v>
+        <v>6.85</v>
       </c>
       <c r="BN6" t="n">
         <v>8.16</v>
@@ -1925,19 +1925,19 @@
         <v>6.22</v>
       </c>
       <c r="BP6" t="n">
-        <v>7</v>
+        <v>6.8</v>
       </c>
       <c r="BQ6" t="n">
-        <v>12.45</v>
+        <v>12.09</v>
       </c>
       <c r="BR6" t="n">
-        <v>7.07</v>
+        <v>6.85</v>
       </c>
       <c r="BS6" t="n">
         <v>7.32</v>
       </c>
       <c r="BT6" t="n">
-        <v>713</v>
+        <v>737</v>
       </c>
     </row>
     <row r="7">
@@ -3117,13 +3117,13 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>6.3</v>
+        <v>6.59</v>
       </c>
       <c r="G12" t="n">
-        <v>604557657</v>
+        <v>632386497</v>
       </c>
       <c r="H12" t="n">
-        <v>0</v>
+        <v>1624200</v>
       </c>
       <c r="I12" t="n">
         <v>95961536</v>
@@ -3138,7 +3138,7 @@
         <v>0.32</v>
       </c>
       <c r="M12" t="n">
-        <v>0.1093333297525335</v>
+        <v>0.1143661330015221</v>
       </c>
       <c r="N12" t="n">
         <v>0.14</v>
@@ -3216,7 +3216,7 @@
         <v>362734606.08</v>
       </c>
       <c r="AM12" t="n">
-        <v>650061996.7741935</v>
+        <v>679985480.6451613</v>
       </c>
       <c r="AN12" t="n">
         <v>0.4208</v>
@@ -3257,7 +3257,7 @@
         <v>30.49</v>
       </c>
       <c r="AZ12" t="n">
-        <v>8.52</v>
+        <v>8.91</v>
       </c>
       <c r="BA12" t="n">
         <v>4.41</v>
@@ -3266,19 +3266,19 @@
         <v>18.12</v>
       </c>
       <c r="BC12" t="n">
-        <v>492.81</v>
+        <v>466.73</v>
       </c>
       <c r="BD12" t="n">
-        <v>384.03</v>
+        <v>362.73</v>
       </c>
       <c r="BE12" t="n">
         <v>35.17</v>
       </c>
       <c r="BF12" t="n">
-        <v>-29.97</v>
+        <v>-33.06</v>
       </c>
       <c r="BG12" t="n">
-        <v>187.6</v>
+        <v>174.95</v>
       </c>
       <c r="BH12" t="n">
         <v>16.4</v>
@@ -3287,7 +3287,7 @@
         <v>0</v>
       </c>
       <c r="BJ12" t="n">
-        <v>6.3</v>
+        <v>6.59</v>
       </c>
       <c r="BK12" t="n">
         <v>3.78</v>
@@ -3296,7 +3296,7 @@
         <v>3.63</v>
       </c>
       <c r="BM12" t="n">
-        <v>6.48</v>
+        <v>6.59</v>
       </c>
       <c r="BN12" t="n">
         <v>7.3</v>
@@ -3305,19 +3305,19 @@
         <v>3.92</v>
       </c>
       <c r="BP12" t="n">
-        <v>6.11</v>
+        <v>6.24</v>
       </c>
       <c r="BQ12" t="n">
-        <v>1.73</v>
+        <v>1.81</v>
       </c>
       <c r="BR12" t="n">
-        <v>6.26</v>
+        <v>6.29</v>
       </c>
       <c r="BS12" t="n">
         <v>0.09</v>
       </c>
       <c r="BT12" t="n">
-        <v>1766893</v>
+        <v>1831757</v>
       </c>
     </row>
     <row r="13">
@@ -3347,13 +3347,13 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>34.64</v>
+        <v>34.5</v>
       </c>
       <c r="G13" t="n">
-        <v>17465175932</v>
+        <v>17394589500</v>
       </c>
       <c r="H13" t="n">
-        <v>0</v>
+        <v>10880000</v>
       </c>
       <c r="I13" t="n">
         <v>504190947</v>
@@ -3368,7 +3368,7 @@
         <v>1.13</v>
       </c>
       <c r="M13" t="n">
-        <v>6.040467555470097</v>
+        <v>6.016054686455066</v>
       </c>
       <c r="N13" t="n">
         <v>0.57</v>
@@ -3446,7 +3446,7 @@
         <v>932753251.95</v>
       </c>
       <c r="AM13" t="n">
-        <v>1817396038.709677</v>
+        <v>1810050936.524454</v>
       </c>
       <c r="AN13" t="n">
         <v>2.6301</v>
@@ -3487,7 +3487,7 @@
         <v>26.6</v>
       </c>
       <c r="AZ13" t="n">
-        <v>62.7</v>
+        <v>62.44</v>
       </c>
       <c r="BA13" t="n">
         <v>2.6</v>
@@ -3496,19 +3496,19 @@
         <v>8.69</v>
       </c>
       <c r="BC13" t="n">
-        <v>-5.97</v>
+        <v>-5.58</v>
       </c>
       <c r="BD13" t="n">
-        <v>-23.22</v>
+        <v>-22.91</v>
       </c>
       <c r="BE13" t="n">
         <v>81</v>
       </c>
       <c r="BF13" t="n">
-        <v>-92.48</v>
+        <v>-92.45</v>
       </c>
       <c r="BG13" t="n">
-        <v>-74.90000000000001</v>
+        <v>-74.8</v>
       </c>
       <c r="BH13" t="n">
         <v>25.49</v>
@@ -3517,7 +3517,7 @@
         <v>0</v>
       </c>
       <c r="BJ13" t="n">
-        <v>34.64</v>
+        <v>34.5</v>
       </c>
       <c r="BK13" t="n">
         <v>1.85</v>
@@ -3526,28 +3526,28 @@
         <v>1.96</v>
       </c>
       <c r="BM13" t="n">
-        <v>34.92</v>
+        <v>35.02</v>
       </c>
       <c r="BN13" t="n">
         <v>36.1</v>
       </c>
       <c r="BO13" t="n">
-        <v>20.85</v>
+        <v>20.98</v>
       </c>
       <c r="BP13" t="n">
-        <v>33.91</v>
+        <v>34.03</v>
       </c>
       <c r="BQ13" t="n">
-        <v>17.7</v>
+        <v>17.63</v>
       </c>
       <c r="BR13" t="n">
-        <v>34.07</v>
+        <v>34.69</v>
       </c>
       <c r="BS13" t="n">
         <v>5.01</v>
       </c>
       <c r="BT13" t="n">
-        <v>7014540</v>
+        <v>7190477</v>
       </c>
     </row>
     <row r="14">
@@ -3577,13 +3577,13 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>12.55</v>
+        <v>12.9</v>
       </c>
       <c r="G14" t="n">
-        <v>10565975087</v>
+        <v>10408795023</v>
       </c>
       <c r="H14" t="n">
-        <v>0</v>
+        <v>8100</v>
       </c>
       <c r="I14" t="n">
         <v>339510689</v>
@@ -3598,7 +3598,7 @@
         <v>1.92</v>
       </c>
       <c r="M14" t="n">
-        <v>4.387180694684419</v>
+        <v>4.321916737814173</v>
       </c>
       <c r="N14" t="n">
         <v>1.11</v>
@@ -3676,7 +3676,7 @@
         <v>349696009.67</v>
       </c>
       <c r="AM14" t="n">
-        <v>1172694238.290788</v>
+        <v>1155249170.144284</v>
       </c>
       <c r="AN14" t="n">
         <v>0.1489</v>
@@ -3717,7 +3717,7 @@
         <v>9.050000000000001</v>
       </c>
       <c r="AZ14" t="n">
-        <v>10.08</v>
+        <v>10.36</v>
       </c>
       <c r="BA14" t="n">
         <v>1.42</v>
@@ -3726,19 +3726,19 @@
         <v>5.94</v>
       </c>
       <c r="BC14" t="n">
-        <v>-11.69</v>
+        <v>-14.09</v>
       </c>
       <c r="BD14" t="n">
-        <v>-27.9</v>
+        <v>-29.85</v>
       </c>
       <c r="BE14" t="n">
         <v>-19.67</v>
       </c>
       <c r="BF14" t="n">
-        <v>-88.68000000000001</v>
+        <v>-88.98</v>
       </c>
       <c r="BG14" t="n">
-        <v>-52.65</v>
+        <v>-53.94</v>
       </c>
       <c r="BH14" t="n">
         <v>5.3</v>
@@ -3747,7 +3747,7 @@
         <v>0</v>
       </c>
       <c r="BJ14" t="n">
-        <v>12.55</v>
+        <v>12.9</v>
       </c>
       <c r="BK14" t="n">
         <v>1.03</v>
@@ -3756,28 +3756,28 @@
         <v>1.01</v>
       </c>
       <c r="BM14" t="n">
-        <v>12.89</v>
+        <v>12.95</v>
       </c>
       <c r="BN14" t="n">
         <v>13.49</v>
       </c>
       <c r="BO14" t="n">
-        <v>7.92</v>
+        <v>7.98</v>
       </c>
       <c r="BP14" t="n">
-        <v>12.1</v>
+        <v>12.32</v>
       </c>
       <c r="BQ14" t="n">
-        <v>12.39</v>
+        <v>12.74</v>
       </c>
       <c r="BR14" t="n">
-        <v>12.73</v>
+        <v>12.55</v>
       </c>
       <c r="BS14" t="n">
         <v>1.44</v>
       </c>
       <c r="BT14" t="n">
-        <v>12927</v>
+        <v>13457</v>
       </c>
     </row>
     <row r="15">
@@ -3807,13 +3807,13 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>18.15</v>
+        <v>17.88</v>
       </c>
       <c r="G15" t="n">
-        <v>10565975087</v>
+        <v>10408795023</v>
       </c>
       <c r="H15" t="n">
-        <v>0</v>
+        <v>2465400</v>
       </c>
       <c r="I15" t="n">
         <v>343551533</v>
@@ -3828,7 +3828,7 @@
         <v>2.56</v>
       </c>
       <c r="M15" t="n">
-        <v>4.335578791959009</v>
+        <v>4.271082468014842</v>
       </c>
       <c r="N15" t="n">
         <v>1.47</v>
@@ -3906,7 +3906,7 @@
         <v>353858078.99</v>
       </c>
       <c r="AM15" t="n">
-        <v>881232284.1534612</v>
+        <v>868123021.1009175</v>
       </c>
       <c r="AN15" t="n">
         <v>0.1638</v>
@@ -3947,7 +3947,7 @@
         <v>9.050000000000001</v>
       </c>
       <c r="AZ15" t="n">
-        <v>12.07</v>
+        <v>11.89</v>
       </c>
       <c r="BA15" t="n">
         <v>1.42</v>
@@ -3956,19 +3956,19 @@
         <v>6.19</v>
       </c>
       <c r="BC15" t="n">
-        <v>-38.94</v>
+        <v>-38.02</v>
       </c>
       <c r="BD15" t="n">
-        <v>-50.14</v>
+        <v>-49.39</v>
       </c>
       <c r="BE15" t="n">
         <v>-33.5</v>
       </c>
       <c r="BF15" t="n">
-        <v>-92.17</v>
+        <v>-92.05</v>
       </c>
       <c r="BG15" t="n">
-        <v>-65.90000000000001</v>
+        <v>-65.39</v>
       </c>
       <c r="BH15" t="n">
         <v>5.3</v>
@@ -3977,7 +3977,7 @@
         <v>0</v>
       </c>
       <c r="BJ15" t="n">
-        <v>18.15</v>
+        <v>17.88</v>
       </c>
       <c r="BK15" t="n">
         <v>1.03</v>
@@ -3986,28 +3986,28 @@
         <v>1.01</v>
       </c>
       <c r="BM15" t="n">
-        <v>18.33</v>
+        <v>18.27</v>
       </c>
       <c r="BN15" t="n">
         <v>18.33</v>
       </c>
       <c r="BO15" t="n">
-        <v>7.97</v>
+        <v>8.15</v>
       </c>
       <c r="BP15" t="n">
-        <v>17.17</v>
+        <v>17.45</v>
       </c>
       <c r="BQ15" t="n">
-        <v>17.92</v>
+        <v>17.65</v>
       </c>
       <c r="BR15" t="n">
-        <v>17.32</v>
+        <v>18.15</v>
       </c>
       <c r="BS15" t="n">
         <v>1.92</v>
       </c>
       <c r="BT15" t="n">
-        <v>2917280</v>
+        <v>2884317</v>
       </c>
     </row>
     <row r="16">
@@ -4037,13 +4037,13 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>5.37</v>
+        <v>5.52</v>
       </c>
       <c r="G16" t="n">
-        <v>1177671046</v>
+        <v>1210567459</v>
       </c>
       <c r="H16" t="n">
-        <v>0</v>
+        <v>87100</v>
       </c>
       <c r="I16" t="n">
         <v>219305733</v>
@@ -4058,7 +4058,7 @@
         <v>2.69</v>
       </c>
       <c r="M16" t="n">
-        